<commit_message>
Search box without focus ring; /the-index fits the screen; /supplier-intake real page again; status block, spreadsheet regenerated
- Search modal and /search: no extra focus ring (owner asked)
- /the-index: results grid no longer runs past the screen (crawl found it)
- /supplier-intake: page served again (redirect to RampRate removed; Stage 2 and vendor-intake paths still go there)
- Fraunces 500 loaded for Kava quote text
- NEXTJS-MIGRATION-TODO.md: 2026-10-07 status block, decisions list, open item for redesign group 2
- Migration-Status-Report.xlsx: rebuilt by scripts/build-migration-status-report.py

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Migration-Status-Report.xlsx
+++ b/Migration-Status-Report.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Remaining Work" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Full Detail'!$A$1:$D$317</definedName>
-    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">'Remaining Work'!$A$1:$D$31</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Full Detail'!$A$1:$D$318</definedName>
+    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">'Remaining Work'!$A$1:$D$32</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1331" uniqueCount="606">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1339" uniqueCount="608">
   <si>
     <t xml:space="preserve">Tony Greenberg site — Next.js migration status</t>
   </si>
@@ -904,6 +904,759 @@
     <t xml:space="preserve">Discourse comments (shown straight away like live, honeypot and a 5-per-10-minutes limit, Tony emailed for each), reactions, Rate this thinking, Micro-commitment: supabase/migrations/0002_blog_engagement.sql, server actions src/app/blog/[slug]/engagement-actions.ts; essays stay prebuilt (the blocks load after the page). Needs the 0002 script run in Supabase (Phase 2) and Resend for the emails; until then the forms say "isn't available just now".</t>
   </si>
   <si>
+    <t xml:space="preserve">/brewsoul</t>
+  </si>
+  <si>
+    <t xml:space="preserve">welcome/landing gate (built, not yet pushed — pending local review), along with the shared foundation the rest of Phase 6 depends on. Ported BrewSoulLayout.tsx → app/brewsoul/layout.tsx + components/brewsoul/brewsoul-nav.tsx (BrewSoulNav/BrewSoulFooter), CategoryBadge.tsx → components/brewsoul/category-badge.tsx, brewsoul-config.ts → lib/content/brewsoul-config.ts, and BrewSoulDirectory.tsx's CATEGORIES/PAGE_CATEGORY_MAP data (not the page itself yet) → lib/content/brewsoul-directory.ts. Real architecture decision: BrewSoul is a self-contained sub-site with its own nav/footer/coffee-brown palette, same as legacy — but this app has one flat root layout with no route groups, so the main site's SiteHeader/SiteFooter needed to be suppressed for this one subtree without restructuring every existing route. Added components/site-chrome.tsx (SiteChrome, a small client wrapper checking pathname.startsWith("/brewsoul")) around both in app/layout.tsx — verified via literal &lt;header&gt;/&lt;footer&gt;/&lt;nav&gt; tag counts in real SSR HTML (not text search, which false-positives on Next dev mode's RSC debug payload) that /brewsoul gets zero main-site chrome and its own real nav+footer, while / still gets exactly one of each. Dropped TonyAvatarTrigger (FauxTony chatbot widget — Phase 10, no backend yet, same "don't fake it" call made elsewhere) from the nav. Ported BrewSoulWelcome.tsx → components/brewsoul/brewsoul-welcome-quiz.tsx (8-screen onboarding quiz, real identity-scoring logic, palate questions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/brewsoul/first-sip</t>
+  </si>
+  <si>
+    <t xml:space="preserve">onboarding intro (built, not yet pushed — pending local review). Ported "The First Sip Is a Vote" in full — the complete manifesto essay (5 sections, 3 pullquotes, the couplets block, the disclosure-demands grid), the 5-tool journey map, 6 related-essay links (real slugs, cross-checked against this session's already-verified corpus), the closing + sources, and the email capture. Built as a Server Component (all static except the email form) + components/brewsoul/next-steps.tsx (shared "what's next" CTA, itself a Server Component — legacy's hover effects were plain CSS-able, no JS state needed) + components/brewsoul/first-sip-email-capture.tsx (client island, mailto: fallback since no subscribe backend exists, same pattern as newsletter-popup.tsx). Dropped the canvas CoffeeDust decoration and the confirmed-dead hero photo (/api/img/brewsoul-orig_84eb4bc9.jpg, 404, same Manus proxy) — with no image left, the scroll-linked parallax that moved it went too. The 5 tool-card links (prescription/health/pairings/economics/compare) point at later Phase 6 routes not built yet — same forward-reference pattern as /find-my. Verified live: 200 OK, full essay text present, CategoryBadge correctly shows "Start Here" (from PAGE_CATEGORY_MAP), zero main-site chrome leaking in, typecheck/lint clean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/brewsoul/home</t>
+  </si>
+  <si>
+    <t xml:space="preserve">the real BrewSoul dashboard (distinct from /brewsoul's identity-quiz welcome gate and /brewsoul/first-sip's manifesto): hero + stats, Follow the Dollar teaser, Top QPR coffees (computed live via computeQPR), the 2025 crisis callout, New Drops, a Wall of Shame preview (SHAME_ENTRIES), the research-hub card grid, and a cyclable health-fact ticker (components/brewsoul/health-ticker.tsx, its own small client island so the rest of the page stays a Server Component). Canvas WarmParticles/ParallaxBg decorations and the dead hero photo (/api/img/brewsoul-orig_84eb4bc9.jpg, same confirmed-404 Manus proxy used elsewhere in Phase 6) dropped for CSS gradients. Stats use the real live BREWSOUL_COFFEES.length (107) in place of legacy's stale "103". Verified live: 200 OK.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/brewsoul/browse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">coffee listing (components/brewsoul/browse-explorer.tsx), real filter/search over the full BREWSOUL_COFFEES catalog. Verified live: 200 OK.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/brewsoul/coffee/[id]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">coffee detail page (breadcrumb, QPR + tier header, quick stats, tasting notes, flavor-profile bars, the 4 intelligence scores, transparency/ethics data, buy links, competition wins, similar-coffees cross-links, journey CTAs), server-rendered with generateStaticParams over all 107 real coffees (this repo's bounded-dynamic-route convention, same as /blog/[slug]) instead of legacy's client-side useParams lookup. Verified live: 200 OK.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/brewsoul/quiz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">matching quiz (built, not yet pushed — pending local review), along with the real data/engine foundation most of the rest of Phase 6 depends on. Ported lib/intelligence-engine/{types,scoring}.ts verbatim (generic scoring engine — QPR/availability/scarcity/wow/tier/freshness — reusable beyond BrewSoul) and the full coffee catalog (legacy's 3 files: brewsoul-coffees.ts + -expanded.ts + -expanded2.ts, merged at import time) → one lib/content/brewsoul-coffees.ts, extracted via tsx (not hand-typed — 107 real entries, ~6.5K lines). Caught a real stale count: legacy's own file header claimed "105" and its UI copy said "103", but the actual merged arrays contain 107 — this migration shows the live BREWSOUL_COFFEES.length everywhere instead of a repeated hardcoded number. Ported JourneyBar.tsx (components/brewsoul/journey-bar.tsx) — the fixed bottom "what's next" bar shown on every BrewSoul content page except the identity quiz — and retrofitted it onto /brewsoul/first-sip too (built before JourneyBar existed). Built components/brewsoul/brewsoul-quiz.tsx: real 7-question taste quiz scored against each coffee's real flavorProfile via the real scoring engine, ranking the full catalog by match. Legacy's useMarkVisited was renamed to markVisited (it's a plain localStorage write, not a hook — its old use-prefixed name tripped React's rules-of-hooks lint when called from inside a useEffect). Dropped the canvas WarmParticles decoration and the dead hero photo (same confirmed-404 Manus proxy,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/brewsoul/wall-of-shame</t>
+  </si>
+  <si>
+    <t xml:space="preserve">content page. Real 13 entries (brand/category/evidence/severity/response) from SHAME_ENTRIES, unchanged. Category filter buttons extracted into components/brewsoul/shame-explorer.tsx (the only interactive piece) so the page itself stays a Server Component. Verified live: 200 OK.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/brewsoul/follow-the-dollar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">supply-chain essay. Real DOLLAR_BREAKDOWNS segment bars (farmer/exporter/importer/roaster/retailer %, real commentary), unchanged. The farmer-segment bar's data-driven color (green/gold/red by threshold) is a small known set of variants — precomposed as 3 literal Tailwind classes rather than an inline style background, per this repo's dynamic-class rule; only the genuinely per-item width stays as style. Fully static, Server Component. Verified live: 200 OK.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/brewsoul/farms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sourcing content ("Farm Passports"). Real FARMS entries (country/region/producer/altitude/story/varieties/certifications), unchanged. Fully static. Verified live: 200 OK.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/brewsoul/mold-free</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mycotoxin content. Real verified/claims/untested split computed live over the full BREWSOUL_COFFEES catalog by moldTestStatus. Fully static. Verified live: 200 OK.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/brewsoul/experiences</t>
+  </si>
+  <si>
+    <t xml:space="preserve">experiential content ("Experience Map"). Real EXPERIENCES entries (farm tours, cafés, cupping labs, roastery visits), unchanged. Country filter buttons extracted into components/brewsoul/experiences-explorer.tsx, same split-out-the-interactive-bit pattern as wall-of-shame. Verified live: 200 OK.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/brewsoul/health</t>
+  </si>
+  <si>
+    <t xml:space="preserve">health deep-dive, ported from BrewSoulHealthFull.tsx (the file legacy's own router actually uses for this route — BrewSoulContent.tsx's same-named BrewSoulHealth export is real but genuinely dead/unrouted code in legacy, shadowed by this one). Real 8 longevity findings with real citations/participant counts, 7 real risks with severity ratings, CYP1A2 caffeine-metabolism genetics, a 6-step chronobiology timing schedule, 8 real bioactive compounds, 3 real mycotoxin threats, and a 3-step "simplification protocol," all ported unchanged and verbatim. Dead Manus hero image dropped for a CSS gradient. Legacy's own redundant BrewSoulLayout wrapper dropped — app/brewsoul/layout.tsx already wraps every route. The two real interactive pieces (show-all-risks toggle, per-compound click-to-expand) split into components/brewsoul/health-{risks,compounds}.tsx client islands so the rest stays a Server Component. Legacy's bespoke earthy "science" palette (soil/clay/sage/moss — distinct from the rest of BrewSoul's amber/gold commercial palette) kept as a deliberate one-off sub-identity for this one page, same reasoning as /attention-theft's own "crusade" palette elsewhere in this migration. Verified live: 200 OK, typecheck/lint clean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/brewsoul/varieties</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reference: varieties. Real VARIETIES encyclopedia entries (species/origin/genetics/cup profile/yield/disease resistance), unchanged. Search extracted into components/brewsoul/varieties-explorer.tsx. Verified live: 200 OK.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/brewsoul/processing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reference: processing. Real PROCESSING_METHODS entries (description/flavor impact/complexity/controversy), unchanged. Fully static. Verified live: 200 OK.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/brewsoul/roasters</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reference: roaster directory. Real ROASTERS entries (philosophy/quality/transparency/farmer-equity scores), unchanged. Search + tier filter extracted into components/brewsoul/roasters-explorer.tsx. Verified live: 200 OK.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/brewsoul/glossary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reference: glossary. Real GLOSSARY terms, unchanged. Search + alphabetical grouping extracted into components/brewsoul/glossary-explorer.tsx. Verified live: 200 OK.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/brewsoul/pairings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reference: pairings. Real PAIRINGS (food/drink pairings by origin) and 3 real curated FLIGHTS (each linking to real coffees in the catalog), unchanged. Fully static. Verified live: 200 OK.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/brewsoul/economics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reference: economics. Real live-computed stats (coffee/origin/roaster/variety counts, average price, average farmer share via DOLLAR_BREAKDOWNS), a real price-distribution histogram, and a real top-origins ranking — all computed directly from BREWSOUL_COFFEES at render time, unchanged. Fully static. Verified live: 200 OK.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/brewsoul/compare</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tool: compare coffees. Real side-by-side comparison of up to 4 coffees across origin/producer/variety/process/price/cupping and the 4 intelligence scores (QPR/availability/wow/overall), unchanged. Interactivity in components/brewsoul/compare-explorer.tsx. Verified live: 200 OK.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/brewsoul/blend-builder</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tool: blend builder. Real combine-up-to-5-coffees ratio calculator with weighted-average QPR/Wow/Overall scores via range sliders, unchanged (never persisted anywhere in legacy either — a pure in-session calculator). Interactivity in components/brewsoul/blend-builder-explorer.tsx. Verified live: 200 OK.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/brewsoul/drops</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tool: product drops ("Latest Drops"). Real top-12-by-overall-score coffees. No client-side state at all (legacy's own useMemo had no changing dependencies — a pure derived list), so this ships as a plain Server Component. Verified live: 200 OK.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/brewsoul/collection</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tool: personal collection tracker ("My Collection"). Real save/toggle-to-collection behavior, unchanged. Real bug found and fixed: legacy read localStorage directly inside a useState initializer — unsafe during SSR, same hydration-mismatch class already fixed in journey-bar.tsx/journey-tracker.tsx — rebuilt around a module-level external store fed through useSyncExternalStore in components/brewsoul/collection-explorer.tsx. Also found and fixed: the already-ported brewsoul-directory.ts listed this page's path as /brewsoul/my-coffees — a real dead link in legacy's own directory (legacy's actual router only ever served this at /brewsoul/collection, /brewsoul/my-coffees never existed) — corrected to the real path. Verified live: 200 OK.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/brewsoul/submit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tool: submit a coffee ("Submit or Appeal"). Real submit-a-coffee / appeal-a-score form, unchanged in structure. Real bug found and fixed: legacy's own comment admitted "In production this would POST to a tRPC endpoint" but in the meantime wrote the submission to localStorage and showed "Received. We'll review your submission" regardless — actively misleading, since nobody would ever see a localStorage-only write. Replaced with a real mailto: fallback pre-filled with the form fields, same honest-degradation pattern as first-sip-email-capture.tsx — no fake success state. Verified live: 200 OK.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/brewsoul/prescription</t>
+  </si>
+  <si>
+    <t xml:space="preserve">personalized "prescription", ported from BrewSoulPrescriptionFull.tsx (the file legacy's router actually uses — BrewSoulTools.tsx's same-named export is dead/unrouted, same shadowed-file trap as /brewsoul/health). Real 5-step questionnaire (genetics/timing/health/flavor/budget) generating a real, deterministic prescription (generatePrescription — real roast/cup-count/brand/pricing/warning logic), all ported unchanged and verbatim. Legacy's trpc.coffeePrescription.generate AI-enhancement mutation doesn't exist in this migration — dropped along with its "AI ANALYSIS LOADING..." block, which would otherwise spin forever and never resolve; the real prescription itself never depended on that call, it's already fully computed client-side. Same bespoke earthy "science" palette as /brewsoul/health kept as the same deliberate sub-identity. Verified live: 200 OK, typecheck/lint clean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/brewsoul/chains</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Top 100 Coffee Chains" ranking (not supply-chain visualization — that's /brewsoul/economics//brewsoul/follow-the-dollar; this is chain rankings). Real 100-chain dataset extracted from legacy's computed CHAIN_RANKINGS export (5 real weighted dimensions → aggregate → S-F tier) via a one-off tsx script (same approach as brewsoul-coffees.ts) into lib/content/brewsoul-chains.ts, with a new ChainEntry type added to intelligence-engine/types.ts. Real tier/type filters, search, and per-chain expand, unchanged, extracted into components/brewsoul/chains-explorer.tsx. Verified live: 200 OK, typecheck/lint clean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/brewsoul/biodynamic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">biodynamic content. The complete real census of Demeter-certified biodynamic coffee: 3 real source farms, 6 real roasters/brands with real product tables and pricing, real nutritional-science compounds, a real cost calculator, and a real impact/tokenization section, all ported unchanged and verbatim. Dead Manus hero image dropped for a CSS gradient. The 3 genuinely interactive pieces (click-to-expand farms/roasters, cups-per-day cost slider) split into components/brewsoul/{biodynamic-farms,biodynamic-roasters,cost-calculator}.tsx client islands so the rest stays a Server Component. Same bespoke earthy "science" palette as /brewsoul/health and /brewsoul/prescription kept as the same deliberate sub-identity. Verified live: 200 OK, typecheck/lint clean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/brewsoul/decaf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">decaf content ("Paint Stripper or Pure Water?"). Real 3-process breakdown (methylene chloride/Swiss Water/supercritical CO₂), 13 real clean-decaf brands ("Hall of Fame"), 10 real methylene-chloride brands ("Wall of Shame," with real Clean Label Project lawsuit citations), a real carbon footprint comparison, real decaf health science, and a real price-comparison table, all ported unchanged and verbatim. Legacy's manual document.title/&lt;meta keywords&gt; mutation in a useEffect (a real anti-pattern — Next's generateMetadata already owns the head) dropped for the real metadata export. Real bug found and fixed: the 13-brand FAME dataset was initially exported from the "use client" decaf-fame.tsx component file and imported into the Server Component page for its price-comparison table — non-component exports from a client module aren't available across the RSC boundary, which threw FAME is not iterable at runtime (only caught by live verification, not typecheck/lint). Moved the data to a plain lib/content/brewsoul-decaf.ts module instead. The 2 genuinely interactive pieces (click-to-expand Hall of Fame, reveal-toggle Wall of Shame) split into components/brewsoul/decaf-{fame,shame}.tsx client islands. Same bespoke earthy "science" palette as the other /brewsoul deep-dive pages kept as the same deliberate sub-identity. Verified live: 200 OK, typecheck/lint clean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/brewsoul/esoteric</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rare-coffee content ("Esoteric Coffee Index"). Real 9-coffee index across 2 tiers (Panama Geisha, Yemen Mokha, Liberica, Eugenioides, Wush Wush, Sidra, Pink Bourbon, Bourbon Aji, Sudan Rume) with real tasting notes, rarity scores, and real named buy sources, plus a real acquisition-priority list and explorer scorecard, all ported unchanged and verbatim. Real content gap found, not fixed: legacy's own "Top 10 Acquisition Priority" list and scorecard table both reference "Laurina" as a 10th entry, but no coffee card for it exists anywhere in the source dataset — ported as-is rather than inventing card content that was never written. Zero client-side state anywhere in this page (only CSS-able hover) — ships entirely as a Server Component. Verified live: 200 OK, typecheck/lint clean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/brewsoul/cities + /brewsoul/cities/[slug]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">city directory + detail ("City Intelligence Module"). Real 25-city leaderboard (name/state/grade/score/tagline/verdict/live stats), a real 7-dimension scoring methodology, and real national + universal/nuanced chain report cards, all ported unchanged and verbatim into lib/content/brewsoul-cities.ts. Real data-completeness note, not a bug: legacy's own comment admits only Portland has full shop-by-shop data (25 real best + 5 real worst shops with real blurbs/scores/order-this/skip-this) — the other 24 cities have real city-level stats but empty shop/chain/bridge-drink/non-coffee arrays; legacy's own UI already handles this honestly (a real "Full data coming soon" state on both the card and detail page, not fake data) — preserved exactly, verified for both Portland (full tabs) and Seattle (coming-soon state). Grade filter, methodology modal, and chain-toggle interactivity in components/brewsoul/cities-explorer.tsx; per-city tab switching and per-shop expand in components/brewsoul/city-detail-tabs.tsx. Detail route uses generateStaticParams over all 25 real slugs. Scroll-linked parallax and floating-particle backgrounds dropped, same decoration call made throughout this migration. Real image-hosting gap flagged, not silently worked around: the 25 city hero photos are real, live Unsplash URLs (not a dead Manus proxy) but aren't yet uploaded to Sanity per this repo's own image convention — added images.unsplash.com to next.config.ts's remotePatterns as an interim measure rather th</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/brewsoul/directory</t>
+  </si>
+  <si>
+    <t xml:space="preserve">real master page index ("Everything Inside BrewSoul," not a roaster directory — that's /brewsoul/roasters). Real 6 categories with real page descriptions/icons, unchanged; the underlying data already lived in lib/content/brewsoul-directory.ts (built earlier this phase to power CategoryBadge) — this route is where it finally becomes a real browsable page. Category filter extracted into components/brewsoul/directory-explorer.tsx. Fixed the stale "Browse All 103 Coffees" label (real count is 107) by dropping the hardcoded number from the shared data module — benefits every other consumer of that module too. Verified live: 200 OK, typecheck/lint clean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/brewsoul/guest + /brewsoul/guest/shanita-nicholas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">guest series index + profile ("Tony G Guest Series"). Real single guest entry (Shanita Nicholas — real headline/teaser/tags) on the index, and the real 10-question interview on the detail page (Fair Trade economics, roasting mythology, the C Market, regenerative vs. sustainable, origin-roasting economics vs. Fair Trade, blockchain traceability, pre-harvest financing — real substantive answers with real citations), all ported unchanged and verbatim into components/brewsoul/shanita-interview.tsx. Legacy's guest photo (/api/img/brewsoul-orig_84eb4bc9.jpg) was the same dead Manus proxy confirmed 404 throughout this migration — dropped for a plain initial avatar on both pages rather than a broken headshot. Per-question expand/collapse, "Expand/Collapse All," and the real Twitter/LinkedIn/copy-link share row are genuinely interactive, split into client islands. Verified live: 200 OK on both, typecheck/lint clean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shared: port BrewSoulLayout, CategoryBadge, JourneyBar, NextSteps as Next.js layout/components</t>
+  </si>
+  <si>
+    <t xml:space="preserve">app/brewsoul/layout.tsx + components/brewsoul/{brewsoul-nav,category-badge,journey-bar,next-steps}.tsx, all built and reused by every /brewsoul/* route above.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kava shared foundation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">app/kava/layout.tsx + components/kava/kava-nav.tsx (KavaNav/KavaFooter, 10 real nav items) + components/kava/kava-ui.tsx (KavaHero/KavaSection/KavaSectionTitle/KavaCard/KavaBadge/KavaDivider/KavaDisclaimer, converted from legacy inline style={} to Tailwind + new --kava-* tokens in globals.css). Added /kava to site-chrome.tsx's SUPPRESSED_PREFIXES (self-contained sub-site, same pattern as BrewSoul and /attention-theft). Real dead link fixed: legacy nav pointed at /pri, which legacy's own App.tsx never routed (only /psychedelic-readiness-index exists) — corrected.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/kava (home)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9 module cards, "Threshold Doctrine," "Sacred Masculine Triad" (Mezcal/Kava/Peyote), 4 market stats, all ported unchanged. Verified live: 200 OK, exactly 1 header/1 footer (chrome suppression confirmed), typecheck/lint clean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/kava/origins</t>
+  </si>
+  <si>
+    <t xml:space="preserve">real migration timeline (6 Pacific nations, ~3000 BCE–1000 CE), real 6-island selector (Vanuatu/Fiji/Tonga/Samoa/Hawaii/Pohnpei, each with real facts/ceremony/cultivar/safety content), and the real Noble vs. Tudei safety comparison, all ported unchanged and verbatim. Island-selector interactivity in components/kava/origins-explorer.tsx. Verified live: 200 OK, typecheck/lint clean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/kava/interactions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">real 24-substance drug interaction database (real severity ratings across an 11-value scale, real pharmacological mechanisms, real PRI protocol guidance) and real 5-enzyme CYP450 inhibition profile, ported unchanged and verbatim. Search + severity-filter interactivity in components/kava/interactions-explorer.tsx, using a precomposed SEVERITY_CONFIG class lookup (not string-built classes — same Tailwind static-scanner rule enforced elsewhere this migration). Legacy's unused Download icon import (dead code, no export feature attached to it) not ported. Verified live: 200 OK, typecheck/lint clean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/kava/science</t>
+  </si>
+  <si>
+    <t xml:space="preserve">real 6 major kavalactones (real receptor mechanisms, real PRI relevance) and real 11-item combined pharmacological profile, ported unchanged into lib/content/kava-science.ts. RSC-boundary bug caught proactively before shipping: initially drafted KAVALACTONES as an export of the "use client" chemotype-decoder.tsx, which would have thrown the same TypeError: X is not iterable already hit once this migration on /brewsoul/decaf when the Server Component page tried to import it — moved to the plain data module before ever running it. Chemotype decoder tool (enter e.g. 4-2-6-5-3-1, see dominant kavalactones) kept as the real interactive client island. Verified live: 200 OK, typecheck/lint clean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/kava/assessment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">real 5-domain, 20-question PRI readiness assessment (somatic/psychological/relational/cultural/integration), real per-domain point weights, and real 4-band recommendation scoring (CLEARED/CONDITIONAL/DEFER/NOT READY), all ported unchanged into components/kava/assessment-quiz.tsx. Fully stateful (domain navigation, per-question answers, results view), so kept as a single client island per this migration's established pattern for multi-step assessments. Domain and recommendation accent colors (5 + 4 distinct hexes, none matching the --kava-* brand palette) precomposed into literal DOMAIN_STYLES/RECOMMENDATION_STYLES lookup objects rather than style={}, avoiding the dynamic-class bug already caught twice this migration (chains-explorer.tsx, biodynamic/page.tsx). Real backend gap, handled honestly: legacy's AssessmentResultActions took sessionId/serialized-answers props feeding a trpc.assessments.submit mutation this migration never built — used the already-simplified, print-only AssessmentResultActions (components/assessments/result-actions.tsx, built during Phase 9) instead of reproducing a submit call with no backend. Verified live: 200 OK, real domain/question content confirmed in rendered HTML, typecheck/lint clean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/kava/hawaii</t>
+  </si>
+  <si>
+    <t xml:space="preserve">real ICE/meth crisis statistics (Quest Diagnostics 410% figure, Hawaii DOH conviction rates, law enforcement seizure data), real dual crisis/revival timeline (1985–present), the real (explicitly-labeled hypothesis, not proven) pharmacological alignment table, and real recovery resource listings, all ported unchanged and verbatim. Fully static, no client island needed. Verified live: 200 OK, typecheck/lint clean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/kava/myths</t>
+  </si>
+  <si>
+    <t xml:space="preserve">real 7-myth evidence review (2002/2014 European kava ban and reversal, WHO findings, CYP2D6 metabolism differences by population, chemotype/preparation distinctions) and the real closing takeaway, ported unchanged. Expand/collapse interactivity in components/kava/myths-explorer.tsx, verdict colors (3-value enum) precomposed into a literal VERDICT_CLASS lookup. Extended shared KavaCard (kava-ui.tsx) with an optional onClick prop to support this — first Kava page needing a clickable card. Verified live: 200 OK, typecheck/lint clean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/kava/caffeine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">real CYP1A2 inhibition mechanism (56%, the same pathway grapefruit juice uses on medications), real caffeine cutoff protocol, and the real kava-vs-coffee comparison table, ported unchanged. Fully static, no client island needed. Verified live: 200 OK, typecheck/lint clean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/kava/products</t>
+  </si>
+  <si>
+    <t xml:space="preserve">real 5-category product index (ceremonial powder, fresh frozen, RTD beverages, supplements, kava bars) with real named vendors/cultivars/chemotypes/pricing/PRI ratings and real outbound buy links (all live vendor domains, not Manus proxies — no image assets on this page to check), ported unchanged into components/kava/products-explorer.tsx. Category-tab interactivity kept as the client island. Verified live: 200 OK, typecheck/lint clean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/kava/certification</t>
+  </si>
+  <si>
+    <t xml:space="preserve">real 12-module, 80-hour facilitator curriculum, real 3-tier certification structure (Practitioner/Threshold Facilitator/Master Facilitator), and real prerequisites list, ported unchanged. Fully static, no client island needed; legacy's wouter cross-links replaced with next/link. Verified live: 200 OK, typecheck/lint clean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PRI shared data: lib/content/pri-data.ts (copied verbatim from legacy pri/data.ts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">real 39-medicine pharmacopoeia, 50+ questions across 6 domains, MAO-B interaction matrix, medication interaction guide, crisis/integration resources, pathway questions), lib/content/pri-safety-data.ts (verbatim safety data merge source), lib/content/pri-medicine-images.ts (verbatim real CloudFront hero-image map, all spot-checked 200 OK — RampRate's own CDN, already whitelisted, not Manus), lib/content/pri-shared.ts (the real scoring engine — computeScores/READINESS_LEVELS/getMedicineWithSafety — extracted to a plain module per the RSC-boundary lesson from /brewsoul/decaf and /kava/science). Added --pri-* CSS custom properties to globals.css (this subsystem's own purple/parchment/near-black palette, same pattern as --kava-/--crusade-) since Phase 7's PRI section spans 9 more routes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/psychedelic-readiness-index (core tool)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">the real hero, 39-medicine grid with compare/save/bookmark tooling, MAO-B interaction matrix, medication interaction guide, crisis resources, the real 5-state assessment flow (philosophy intro → readiness quiz → pathway &amp; access questions → legal disclaimer gate → results), medicine detail modal (overview/safety/correction tabs), testimonials, and ImpactSoul cross-promotion, all ported unchanged and verbatim into components/pri/psychedelic-readiness-index.tsx plus supporting client islands (disclaimer-gate.tsx, medicine-modal.tsx, safety-section.tsx, correction-form.tsx, share-bar.tsx, cinematic-band.tsx). Kept as one client island — a single state machine drives which section renders, same call made for other large multi-step assessments this migration. Real hero/section photography (8 CloudFront images) kept via next/image; legacy's purely decorative glitch-scanline overlay divs and CSS shimmer/glow @keyframes dropped (no framer-motion — CONTRIBUTING.md rule 5 — and "decoration not worth the cost," same call made throughout this migration).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PRI: /peyote-mescaline</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MescalineDeepDive, real receptor pharmacology table, the real "Latuda Mirror" same-target-opposite-action comparison, real clinical outcomes (Agin-Liebes et al. 2021, n=452), the real 16-row pharma-to-plant alternatives table, real supplement protocol (pre/day-of/post-integration), real mescaline-specific PRI dimension scores, the real medicine-selector comparison table, and real sources, all ported unchanged and verbatim into lib/content/pri-mescaline-module.ts (copied verbatim) + app/peyote-mescaline/page.tsx. Fully static except the pharma-table expand toggle, extracted into components/pri/pharma-table.tsx; shared PriSection/PriEyebrow wrapper (components/pri/pri-section.tsx) introduced here for reuse by the remaining PRI deep-dive modules. All 8 real section photos (CloudFront) spot-checked live before use; legacy's purely decorative glitch-scanline overlays dropped. Verified live: 200 OK, real content confirmed in rendered HTML, exactly 1 header/1 footer, typecheck/lint clean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PRI: /iboga-ibogaine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IbogaDeepDive, "The Plant vs The Isolate": real alkaloid-profile comparison, real receptor pharmacology, real head-to-head iboga-vs-ibogaine table, real clinical outcomes (Mash/Noller/Schenberg/Brown &amp; Alper/Cherian/Williams — including the 2024 Stanford Nature Medicine SOF-veteran data and the 2026 19,071-patient safety analysis), real pharma-to-plant alternatives, real supplement protocol, real dimension thresholds, real medicine selector, Tony's real first-hand account of sitting ibogaine at The Mission Within, real hard-stop contraindications, a real 9-facility directory (with the 2 facilities legacy explicitly removed and why), real Nagoya Protocol / extractive-capitalism argument, real 2026 US legal-status rundown, the embedded Iboga Compass v2 documentation section (components/pri/iboga-compass-section.tsx, its own client island for the question-group toggles), and real sources — all ported unchanged and verbatim into lib/content/pri-iboga-module.ts + lib/content/pri-iboga-compass-data.ts (both copied verbatim) + app/iboga-ibogaine/page.tsx. Fully static except the pharma-table expand toggle (components/pri/iboga-pharma-table.tsx) and the compass section's toggles; reused the shared PriSection/PriEyebrow wrapper from the mescaline module. All 5 real hero/section photos (CloudFront) spot-checked live before use. Verified live: 200 OK, real content confirmed in rendered HTML, exactly 1 header/1 footer, typecheck/lint clean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PRI: /iboga-compass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IbogaCompassAssessment, the real interactive 28-question / 7-section compass (outcome/medical/approach/logistics/geography/personal/aftercare), the real drag-or-arrow priority-rank step (top dimension ×2.0, bottom ×0.5), the real facility-scoring engine, and the real results view (matched facilities with real "why this matched" reasoning and real elimination reasons), all ported unchanged and verbatim. lib/content/pri-iboga-compass-engine.ts (real scoring logic — weight deltas, hard filters, substance bonuses, priority-rank application, facility scoring) and lib/content/pri-iboga-facility-data.ts (real facility directory + substance-bonus data) both copied verbatim from legacy rather than hand-transcribed, given this is the actual matching algorithm — correctness matters more here than anywhere else in this migration. Uses this site's own brand-gold/foreground/muted-foreground design tokens rather than the pri-* palette — legacy's own hex here (#8B6914) is an exact match for brand-gold, confirming this one page always used the main site identity, not a PRI-specific one. Real backend gap handled honestly: legacy's lead-capture gate posted a rich structured payload (question-by-question answers, top facility matches, primary goal, budget range) to trpc.assessments.submit (no backend built for this migration) — replaced with a mailto: to Tony carrying the same structured summary, same pattern used throughout this migration; the meaningless "Submitting..." pending state and its e</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PRI: /pri-calibration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">forced-rank calibration study, the real Bradley-Terry pairwise-comparison model (all 15 unique pairs of the 6 PRI dimensions), the real drag-or-arrow full ranking step, real methodology copy (acquiescence-bias explanation, the 4 headline validation stats), and the real Monte Carlo validation metrics (lib/content/pri-efficacy-data.json, copied verbatim from legacy — also feeds /pri-efficacy below), all ported unchanged into components/pri/calibration-assessment.tsx. Real backend gap, handled honestly: legacy's "Contribute to Research?" opt-in phase posted to trpc.priCalibration.submit (no backend built for this migration), and the results view's "Community Data" section read a live trpc.priCalibration.stats aggregate query showing other users' scores — neither has an honest backend-free equivalent (a cross-user aggregate can't be faked locally, and a research opt-in toggle with nothing behind it would be dishonest UI, the same call already made dropping the main PRI results page's inert research-pool checkbox). Both dropped; the flow goes straight from ranking to results. Verified live: 200 OK, real content confirmed in rendered HTML, exactly 1 header/1 footer, typecheck/lint clean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PRI: /pri-efficacy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">psychometric validation dashboard, the real Monte Carlo simulation results (10,000 synthetic respondents), real classification-accuracy comparison, real dimension-priority distribution (the real first-dimension-inflation finding), real test-retest reliability and entropy metrics, and the real methodology writeup, all ported unchanged into app/pri-efficacy/page.tsx, reading the same lib/content/pri-efficacy-data.json also used by /pri-calibration. Real backend gap, handled honestly: legacy's "Live Calibrations" tab read a live trpc.priCalibration.stats query — since /pri-calibration's own submit call was already dropped (no backend, see that page's port note), this tab would permanently render "0 total calibrations, no data yet," a dead feature masquerading as a live one. Dropped entirely rather than ship a perpetually-empty tab; only the real, fully-populated Simulation view ships — which also means this page has no state left at all, so it's a plain Server Component now instead of a client one. Verified live: 200 OK, real content confirmed in rendered HTML, exactly 1 header/1 footer, typecheck/lint clean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PRI: /pri-research Built 2026-10-06 behind the login: admins are the emails in ADMIN_EMAILS; everyone else gets live's "Access Denied"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Totals, anonymized opt-in table, admin-only CSV export (/pri-research/export). /pri-calibration regained legacy's "Contribute to Research?" step and now saves every calibration anonymously to pri_calibrations (opt-ins flagged). Was: — Deferred, not skipped (access-model question resolved by inspection). Read the real legacy source: this is a genuine admin-only dashboard (useAuth() gated to role === "admin") showing trpc.priCalibration.researchData — the same calibration-submission backend already confirmed absent and intentionally not built for /pri-calibration and /pri-efficacy (see their port notes). No admin-auth system exists anywhere in this Next.js migration yet either. So this isn't just an access-control decision — even fully wired up, the page would have zero real data to show, forever. Not worth building an admin dashboard against a backend this migration has twice already decided not to build. Added to "Explicitly deferred" below alongside the other admin dashboards; revisit only if/when both a real admin-auth system and a real calibration-submission backend exist.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PRI: /facilitator-index</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"The Facilitator Index: Know Who You Go With," the real 15-question quick-intake archetype quiz (real Bradley-Terry-style axis derivation, fully client-computed via deriveArchetype()), the real 108-item, 12-band (plus Band 0) practitioner self-assessment instrument, and the real methodology prose (rationale, code/tier system, data-handling policy, Reciprocity Gate, Corroboration token system), all ported unchanged and verbatim into lib/content/facilitator-index-data.ts (single authoritative content source) + components/facilitator/* + app/facilitator-index/page.tsx. Real content-drift bug found and fixed: legacy shipped two divergent copies of the same "108 items" — the on-page JSX and a separate printFacilitatorQuestions() print/PDF export using an older, different set of item numbers and band groupings (missing the on-page "Twenty-Five Traditions and Protocols" band entirely) — the print export was never updated when the on-page instrument was revised. Used the on-page version (the one actually shown to visitors) as the single source of truth and rebuilt the print export to generate from that same data, so the two can never diverge again. Real fake-data found and dropped: legacy's PeerStats component's own comment admits its numbers ("163 practitioners mapped so far," etc.) are "seeded, realistic-feeling" — fabricated, not real — dropped entirely, same principle as BrewSoul's stale "reads" counts; UsageCounter's hardcoded 160-practitioner fallback (shown forever since no ba</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Port shared safety/medicine data modules (safety-data.ts, medicine-images.ts) as typed .ts content in the new codebase</t>
+  </si>
+  <si>
+    <t xml:space="preserve">done as part of the main PRI page above (lib/content/pri-safety-data.ts, lib/content/pri-medicine-images.ts, both copied verbatim).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/attention-theft</t>
+  </si>
+  <si>
+    <t xml:space="preserve">consolidated mega-page. Real content ported in full across all 9 sections (hero, The Sacred, The Heresy economics data + full breakdown table + sources, the 10 Weapons, Legal Arsenal w/ filter + letter template, AI Blocker Finder quiz, Report a Spammer, closing vow + related reading) — AttentionTheft.tsx used as the single source, the 5 pre-consolidation sub-pages not resurrected (they never existed in this codebase anyway). Section "glamour" photography is real, live imagery on RampRate's own CloudFront (already whitelisted in next.config.ts as a non-Manus, permanent host — confirmed all 7 URLs 200 before using them), rendered via next/image. Real backend gap found and handled honestly: legacy's Wall of Shame (a live trpc.spam.wallOfShame ranked list) and the Report form's trpc.spam.submit both depended on a spam-tracking backend that this migration explicitly defers (see "Explicitly deferred" list below: "/youve-been-reported, /spamtoast, admin spam tooling") — rather than fake a public database with no real data behind it, the report form now composes a mailto: to Tony (same honest non-fake-success pattern as newsletter-popup.tsx), and the ranked Wall of Shame list isn't reproduced. Two simplifications matching precedent set elsewhere in this migration: legacy's "Fraunces" serif (loaded for this one page only) was dropped for font-heading (Playfair Display, already loaded — same call made on /akbar), and the glitch/VHS/ember-particle/shattered-glass decoration layer was dr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Legacy anchor redirects</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/attention-theft/economics, /blocker-finder, /legal, /weapons, /report → /attention-theft#&lt;anchor&gt; via next.config.ts redirects(). Verified live: all return real 308s to the correct anchor.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Port ManifestoLayout scroll-tracking wrapper behavior</t>
+  </si>
+  <si>
+    <t xml:space="preserve">components/manifesto/manifesto-nav.tsx tracks which section is in view on scroll and highlights the matching nav pill (desktop + mobile), real behavior kept per this line item rather than simplified away.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HumanOS section</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/humanos, /humanos/philosophy, /humanos/ecosystem, /humanos/resources, /humanos/connect, /humanos/path-to-here, ported from _legacy-manus-app/client/src/pages/HumanOS.tsx + humanos/*.tsx. The top-level HumanOS.tsx (an iframe embed of an external manus.space site) turned out to be dead code, never wired into legacy's router — the real, routed implementation is HumanosHome/HumanosPhilosophy/HumanosEcosystem/HumanosResources/HumanosConnect/HumanosPathToHere behind HumanosLayout, which is what got ported, with its own nested layout.tsx (route now added to site-chrome.tsx's SUPPRESSED_PREFIXES so the main SiteHeader/SiteFooter don't double up around HumanOS's own nav/footer). Real content in full: the Maximizer-vs-Satisficer framework and "Boiling the Human"/"Maximizer Trap"/"Conscious Satisficer" philosophy sections, the full ecosystem roster (1 mentor, 8 advisors, 3 partners, 29 clients), all 4 transformation playbooks + 3 daily-practice protocols + 8-book reading list, all 4 connect channels, and the 6-entry "Path to Here" timeline (2010 H+ Summit through 2025). Real bugs fixed: every "Take the Diagnostic" CTA site-wide pointed at /assessment, an 8-question Maximizer/Satisficer quiz that was never actually built anywhere (legacy's real /assessment and /assessments routes are two different, unrelated quiz sets) — redirected to /humanos/philosophy, which delivers the actual promised content; Connect's "Read the Living Declaration" pointed at /manifesto, a dead redirect stub in le</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/find-your-me (+ /find-my-me, /discover)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Find My — To Find Your We," the ecosystem hub assessment and by far the largest page in Phase 9. Real 5 NLP-driven questions, 6 dimensions (relationships/purpose/body/truth/tribe/consciousness), and 6 real archetypes (each with a real description, real blog article links, real satellite-site links, real "go deeper" forward-references, and a real share text) ported unchanged and verbatim into a new lib/content/find-your-me.ts data module (kept separate from the component given the file's exceptional size, same pattern as brewsoul-directory.ts). All 17 unique blog article slugs referenced across the 6 archetypes were individually verified live (200 OK) against this migration's real Sanity blog before porting — zero dead article links. Real accuracy fix: legacy's "Full Ecosystem Directory" (26 items across 5 categories, with a real LIVE/COMING pill UI already built for exactly this purpose) marked everything "live," including several routes that don't exist anywhere in this migration yet (/find-my, /the-mirror, /assessments/dharma-finder, /assessments/consciousness-scale, /assessments/grant-study, /flow-circuit) — corrected each item's status to this app's actual current build state rather than shipping false LIVE labels on what would be 404s. Real completeness fix: added Find Your Peptide and Find Your Sexuality to the directory (Body &amp; Temple and Love &amp; Belonging) — both are real, fully-built assessments elsewhere in this migration that didn't exist yet when legacy was writte</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/find-your-therapy (+ /find-my-therapy)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Real 25 questions across 6 dimensions (Cognitive/Somatic/Relational/Depth-Unconscious/Altered States/Integrative), 6 real therapeutic modalities (each with a real description, "how it works," best-for/not-ideal-for lists, real named pioneers, and real book/directory resources), and the real archetype-matching logic (highest-scoring dimension wins) ported unchanged and verbatim. Three real stale-count bugs found and fixed: legacy's own file-header comment claimed "10 questions," its AssessmentIntro stats prop claimed 20 — neither matches the real 25-item array (the scoring code's own maxPossible = 30 // rough max per dimension with 25 questions comment confirms 25 is correct) — replaced both with live QUESTIONS.length. Real dead-link bug fixed: legacy's "Journey Continues" grid linked "Find Your Spirit"/"Find Your Religion" to external findmyassess-9eekxcob.manus.space stub URLs (dead Manus domain) despite this migration already having real, fully-built internal pages at /find-your-spirit and /find-your-religion — repointed to the real internal routes, and corrected Religion's stale "15 Questions" badge to the real 20. Real accent-color inconsistency fixed: legacy passed accentColor="#7B1FA2" only to the landing screen, then hardcoded brand-gold everywhere on the results screen instead — threaded one ACCENT constant through intro/radar/result-actions consistently, matching every other assessment in this migration. The "Also Worth Exploring" related-modality cards were dropped </t>
+  </si>
+  <si>
+    <t xml:space="preserve">/find-your-sake</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Real 20 questions across 5 dimensions (Palate/Ritual/Terroir/Philosophy/Season) and the real 5 sake profiles (each with real Japanese name, tasting notes, food pairings, serving temperature, named producers with region/note, and further-reading resources) ported unchanged and verbatim. Legacy's own AssessmentIntro stats prop claimed "15 questions, 6 dimensions" — didn't match the real 20/5 implementation — replaced with live QUESTIONS.length/DIMENSIONS.length counts, same fix pattern already applied on /find-your-attachment-style and /find-your-sexuality. Two real bugs found and fixed: (1) legacy's "Journey Continues" list read "Find Myzcal" — a literal typo for "Find Your Mezcal" — corrected. (2) legacy's JSX rendered &lt;WhatsNext /&gt; (a full page section) nested inside the small "Retake the Tasting" &lt;button&gt; element — moved to a proper top-level section, same class of nested-interactive-content bug already fixed on /find-your-religion. The dark GlassPanel treatment (near-black translucent cards with light cream text, sitting on the page's own light parchment ThemedBackground) was kept as a real, intentional design choice rather than "fixed" to this migration's usual light-card convention — unlike the light-text-directly-on-light-background contrast bugs found on Style/Sexuality/Peptide/Religion, the text here sits inside its own correctly-contrasted dark card. SacredGeometryBg's canvas-based floating rice-grain particles dropped (same decoration-not-worth-the-JS-cost call made</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/find-your-spirit (+ /find-my-spirit), along with a shared PDF-export component the rest of Phase 9 can reuse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Real 35 questions, 10 dimensions, and the 6 real spiritual traditions (each with real description/practices/key texts/figures/modern expressions/growth edge) ported unchanged and verbatim — legacy's own file-header comment claimed "12 archetypes," but only 6 TRADITIONS actually exist in the code; ported the real 6, not the stale doc comment. The real weighted tradition-matching logic (top 3 dimensions per tradition, weighted 3/2/1) is unchanged. Ported components/assessments/result-actions.tsx from legacy's AssessmentResultActions — kept only the real, backend-free "Download PDF" action (browser print); the "Send to Tony"/"Keep Private" buttons posted to an unbuilt trpc.assessments.submit and weren't reproduced, same honest-degradation pattern used throughout this migration. Verified live: 200 OK, redirect confirmed 308, typecheck/lint clean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/find-your-religion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Real 20 questions across 8 dimensions, 8 real spiritual/philosophical archetypes (each with real description/practices/key texts/figures/resonant traditions/growth-edge tensions), and the real scoring/matching logic ported unchanged and verbatim. Real bug found and fixed: legacy's own JSX rendered &lt;AssessmentResultActions&gt; nested inside the "Retake Assessment" &lt;button&gt; element — a button inside a button, invalid HTML — fixed by rendering it as a sibling instead, same fix pattern already applied on /find-your-spirit. Verified live: 200 OK, typecheck/lint clean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/find-your-diet (+ /find-my-diet)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Real 15 questions, 6 real archetypes (with descriptions), and the real nearest-neighbor archetype-matching logic ported unchanged. Legacy's dead JourneyTracker import wired in for real (see journey-tracker.tsx). /find-my-diet → /find-your-diet redirect added. Verified live: 200 OK, full quiz flow, redirect confirmed 308, typecheck/lint clean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/find-your-movement (+ /find-my-movement), along with the shared assessment foundation the rest of Phase 9 depends on</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ported components/assessments/{themed-background,assessment-intro,email-gate,whats-next}.tsx from legacy's ThemedBackground/AssessmentIntro/EmailGate/WhatsNext — real content/behavior unchanged, with 2 real fixes along the way: (1) EmailGate now posts to the real /api/subscribe Route Handler (built earlier this migration) using the exact find-your-&lt;slug&gt; source keys already defined in lib/content/kit-source-tags.ts's KIT_TAG_MAP — legacy's own assessment-gate:&lt;slug&gt; prefix didn't match any tag in that map, so this is a genuine improvement, not just a port. (2) ThemedBackground's per-theme decorative particle field + SVG sacred-geometry overlay + 2 extra radial-glow layers dropped (same "not worth the cost" call made repeatedly elsewhere) — the real per-theme base gradient (16 themes) is kept, precomposed as one literal Tailwind class per theme rather than assembled from fragments. find-your-movement-quiz.tsx ports all 15 real questions and the real 6-dimension (Strength/Flexibility/Endurance/Mindfulness/Community/Adventure) scoring unchanged; the legacy JourneyTracker/useJourneyProgress import in the source file was dead code (imported, never rendered) and not ported. /find-my-movement → /find-your-movement redirect added (next.config.ts), same duplicate-route pattern as /find-my-tribe. Verified live: 200 OK, full quiz flow renders, redirect confirmed 308, typecheck/lint clean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/find-your-sleep (+ /find-my-sleep)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Real 15 questions, 6 real archetypes, and the real cascading archetype-match logic ported unchanged, including legacy's own real behavioral quirk of rendering JourneyTracker on every phase (not just results). One real duplicate-destination "Journey Continues" link pair dropped (see file's own port note), the one real distinct link (Find Your Diet) kept. /find-my-sleep → /find-your-sleep redirect added. Verified live: 200 OK, redirect confirmed 308, typecheck/lint clean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/find-your-coffee (+ /find-my-coffee)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Real 15 questions, 6 dimensions (Roast Preference/Origin Curiosity/Brewing Ritual/Social Context/Caffeine Sensitivity/Flavor Complexity), 6 real archetypes (each with a real description and 5 real named coffee recommendations — roaster, origin, roast level, tasting notes, real "why" rationale), and the real archetype-matching logic (sum of each archetype's 2 primary dimensions, highest wins) ported unchanged and verbatim. This legacy page predates the shared ThemedBackground/AssessmentIntro component system the rest of Phase 9 is built on — it hand-rolled its own hero-image page shell — so it needed more normalization than most: its hero image (/api/img/coffee-orig_a935f111.jpg) was a dead Manus asset, dropped for the standard ThemedBackground light theme (added a new "coffee" warm-cream entry) instead of reproducing a broken background; the canvas bean-particle field, floating steam-wisp divs, and SVG sacred-geometry overlay all dropped (same decoration-not-worth-the-JS-cost call made repeatedly elsewhere). Real bug found and fixed: legacy read window.innerWidth directly during render (twice — to pick grid columns and flex direction), unsafe during SSR and a real hydration-mismatch source — replaced with responsive Tailwind classes. EmailGate's prop was legacy's assessmentName; ported using this repo's real assessmentSlug="coffee" to match find-your-coffee in KIT_TAG_MAP. Legacy imported useJourneyProgress for markComplete but never rendered a visible JourneyTracker, and nev</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/find-your-kitchen. Real 15 questions (all rendered on one page at once</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a genuinely different, legacy-intentional UX from the other paginated quizzes, kept as-is) and the real dual-tracking scoring (answer score keys split into archetype tallies vs. 6 separate radar-chart dimensions) ported unchanged, including the 3 real "Journey Continues" links (one to already-built /find-your-diet, one forward-reference to /find-your-style). Verified live: 200 OK, typecheck/lint clean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/find-your-style. Real 15 questions, 6 real archetypes, and the real (if crude</t>
+  </si>
+  <si>
+    <t xml:space="preserve">legacy's own comment admits "Simple mapping for demonstration") threshold-based archetype match ported unchanged. Two real inconsistencies found and normalized: legacy's own inline styles used near-illegible light text on ThemedBackground's actual light pastel "style" theme (inconsistent with every other assessment in this migration); and legacy rendered &lt;JourneyTracker /&gt; defaulting to variant="dark" on a light results screen instead of the variant="light" every other assessment passes. Verified live: 200 OK, typecheck/lint clean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/find-your-attachment-style (+ /find-my-attachment-style, /find-my-we)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Real 18 questions (legacy's own AssessmentIntro stats prop under-reported this as "15" — used the live QUESTIONS.length instead of repeating the stale number, same live-count discipline used elsewhere in this migration), the 4 real archetypes, and the real scoring/selection logic all ported unchanged, including the real closing note on attachment theory. Both alt-path redirects added. Verified live: 200 OK, both redirects confirmed 308, typecheck/lint clean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/find-your-love-language</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Real 15 questions (incl. the negative-score "disconnect" question), 5 real archetypes with descriptions/tips, and Dr. Gary Chapman's real attribution note all ported unchanged. Verified live: 200 OK, full quiz flow, typecheck/lint clean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/find-your-peptide (+ /find-my-peptide)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"The Peptide Clarity Index™." A real, evidence-cited 10-question assessment across 7 clinical axes, mapping to 16 real peptide archetype profiles — every question (with its real PubMed/journal citation), every profile's real primary/secondary peptides with mechanisms and evidence, suggested lab work, red flags, and stacking notes ported unchanged and verbatim (clinical-adjacent content, not paraphrased). The real Peptide Readiness Score, contraindication-flag screening, share buttons (Twitter/LinkedIn/email/copy — real, backend-free), and the real medical disclaimer are all preserved. Real hero image (CloudFront, confirmed live) kept via next/image. Reused the simplified AssessmentResultActions (PDF-only) built for /find-your-spirit. Same light-text-on-light-background contrast bug already caught elsewhere was fixed here too. Verified live: 200 OK, redirect confirmed 308, typecheck/lint clean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/find-your-sexuality (+ /find-my-sexuality)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A research-informed assessment across 6 real dimensions, grounded in real cited research (Klein Sexual Orientation Grid 1978, Kinsey Scale 1948, Lisa Diamond 2008, Sari van Anders 2015) — real 16 questions (with per-question research context notes), real 12 archetypes (each with a real description + research note), and the real scoring/selection logic all ported unchanged and verbatim, including the real closing disclaimer. Legacy's own AssessmentIntro stats prop claimed "20 questions, 7 dimensions" — didn't match the real 16/6 implementation, used the live counts instead. Legacy's results screen also used light grey text on the real light pastel theme background (same low-contrast bug already caught on /find-your-style) — normalized to dark ink. Verified live: 200 OK, redirect confirmed 308, typecheck/lint clean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/find-my</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Find What's Yours," the real destination of the homepage's "Diagnose" door (confirmed by grepping lib/content/home-doors.ts's /find-my href) and of whats-next.tsx's "Take Another Assessment" link, both already pointing here as forward-references before this page existed. Legacy's 26-item ALL_LINKS directory (Featured + 6 categories) ported unchanged and verbatim into lib/content/find-my-directory.ts. Real accuracy fix, same pattern as /find-your-me's own port note: cross-checked all 26 destinations against the real route list — /find-your-ev, /life-assessment, and /soulscore (at the time) didn't exist yet, rendered as real "Coming Soon" cards instead of links that would 404 (dharma-finder/consciousness-scale/grant-study have since shipped and now flip to live — see below). Real reuse, not re-derivation: every item whose destination already exists in find-your-me.ts's audited DIRECTORY pulls that entry's real hook text and status at build time via a lookup helper, instead of hand-copying a second, driftable copy of the same facts. Two real live destinations added that legacy linked but find-your-me.ts's directory didn't track: /brewsoul (confirmed 200) and the external findmystem-s3lknc4h.manus.space sibling tool (confirmed live), both using the same "real external sibling product" trust already established for the other manus.space tools. Legacy's dead Manus hero image dropped for ThemedBackground (theme="ecosystem"), same call as /find-your-me. AssessmentProgressBar (never </t>
+  </si>
+  <si>
+    <t xml:space="preserve">/assessments</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Three Maps. One Journey," confirmed genuinely distinct from /find-my rather than a duplicate: /find-my is the wide 26-item ecosystem directory, /assessments is its own page for exactly 3 long research-grounded instruments (Dharma Finder / Consciousness Scale / Grant Study) that also happen to appear as one category inside /find-my's directory — legacy kept these as two separate pages, so the port does too. Real title/subtitle/description/time/icon/accent content for all 3 instruments ported unchanged and verbatim into lib/content/assessments-hub.ts, including the full "Why These Three" closing essay (Schmachtenberger/Hawkins/Harvard Grant Study triangulation). All 3 instrument cards now link live (dharma-finder/consciousness-scale/grant-study shipped alongside this page). Legacy's footer claim "Results saved for your return" was dropped — replaced with an honest line since nothing persists results yet. Added a real cross-link to /find-my. JourneyTracker reused unchanged; no EmailGate/AssessmentResultActions — pure preview/hub page with no quiz or results step of its own. Verified live: 200 OK, exactly 1 header/footer, real content in all 3 cards, typecheck/lint clean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/dharma-finder (+ /assessments/dharma-finder redirect). Structurally different from every other Phase 9 quiz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">legacy's real 25 questions are open-text reflection prompts, not multiple choice, distilled from Daniel Schmachtenberger's Dharma Inquiry and grouped into 4 real sections (Capacities/Values/Propensities/The Shadow Inquiry), each with a real framing quote, plus 3 real interstitial quotes shown between sections with the original 4-second auto-advance. All 25 questions, all quotes, and legacy's own keyword-matching generateDharmaProfile (deriving up to 3 archetypal roles and up to 4 core values from free-text answers, plus a completion-depth percentage) are ported unchanged and verbatim into a new dharma-finder-quiz.tsx. Real bug found and fixed: legacy's result-screen JSX rendered &lt;AssessmentResultActions&gt; nested inside the "Retake Assessment" &lt;button&gt; element — a button inside a button, invalid HTML — fixed the same way as /find-your-religion. Real dead-link bug fixed: "Journey Continues" linked to /assessments/consciousness-scale (repointed to the real /consciousness-scale) and /assessments/grant-study (dropped at the time, now live too). EmailGate (new here; legacy had none) is a real ecosystem-consistency addition. find-your-me.ts's ecosystem-directory status flipped from "coming" to "live" now that this page ships. Verified live: 200 OK, typecheck/lint clean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/consciousness-scale (+ /assessments/consciousness-scale redirect)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Real 25 questions, each scored against David R. Hawkins' real 17-level Map of Consciousness (Shame 20 through Enlightenment 700+, final score = average of all 25 answers) — every question/option, every level's name/emotion/threshold, and getInsight's exact 6 tiers of interpretive copy ported unchanged and verbatim into a new consciousness-scale-quiz.tsx, along with the real live running-average indicator, visual scale gauge, full 17-level map, 6-month reminder, and X/LinkedIn/copy share. Since this assessment produces one composite score on a single axis rather than independent dimensions, a bespoke single-axis gauge replaces AssessmentRadarChart; per-level colors (17 known-at-build-time values) are precomposed literal Tailwind classes rather than assembled from hex fragments. Real Manus-dependency bug found and fixed: legacy's cinematic Q1 hero used a /api/img/consciousness-scale-hero-v2_085e0746.jpg Manus-proxied image — forbidden even temporarily per this migration's Zero-Manus rule — dropped for the plain question-card layout every other assessment uses; a real Sanity-hosted replacement is a tracked follow-up (see BLOG-IMAGE-BRIEFS.md-style tracking). find-your-me.ts's ecosystem-directory status flipped from "coming" to "live" now that this page ships. Verified live: 200 OK, typecheck/lint clean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/grant-study (+ /assessments/grant-study redirect)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Find Your Score," the real 25-question (5 per factor), 5-factor Harvard Grant Study life-satisfaction assessment (724 men, 1938–present, 85+ years — the longest-running study of human happiness). Every question, the 5 real factors (Warm Relationships/Adaptive Coping/Generativity/Career Satisfaction/Physical Vitality), every per-factor/per-tier insight (real named findings — Vaillant's "mature defenses," Erikson's generativity, Waldinger's quote), and the closing "Tony's Note" (Vaillant's "Happiness is love. Full stop." + Waldinger's "good relationships keep us happier and healthier") all ported unchanged and verbatim. Real nested-interactive-element bug found and fixed: legacy rendered &lt;AssessmentResultActions&gt; (its own &lt;button&gt;) literally inside the "Retake Assessment" &lt;button&gt; — same bug class already caught on /find-your-religion//find-your-sake — split into siblings. Real dead-link fix: "Journey Continues" pointed "Find Your Spirit" at a dead external Manus stub despite the real internal /find-your-spirit existing — repointed. Real ecosystem-consistency normalization: unlike every sibling "Find Your X" quiz, legacy skipped EmailGate entirely and went straight to results — added for consistency, plus new find-your-grant-study/find-your-dharma-finder/find-your-consciousness-scale alias keys in kit-source-tags.ts's KIT_TAG_MAP so EmailGate's fixed find-your-&lt;slug&gt; source prefix actually resolves to the intended tag instead of a generic fallback. resultSlug="grant-study" pas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/soulscore</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SoulScore™, ImpactSoul's 12-dimension impact measurement engine (1231-line legacy file, the largest remaining port). Unlike the quiz-style "Find Your X" assessments, this is a live interactive calculator, not a Q&amp;A flow: entity-type picker, 12 weighted dimension sliders (Hawkins-scale Consciousness + 11 others), real-time score/grade/radar/auto-diagnosis, a benchmark table against 7 real entities (Patagonia, BP, Fortune 500 Avg, etc.), a 6-tier/30-factor supply chain drill-down, 20 "why every impact system failed" entries, a real Consciousness-Adjusted NPV calculator, and the gig-economy 5-layer stack comparison — all real content/formulas ported verbatim. Fixed: legacy's own SEO block described an unrelated assessment (stale copy-paste, replaced with real metadata); a div-pretending-to-be-a-button wrapping 30 nested range-input sliders (fixed to a real &lt;button&gt; + sibling content div); hardcoded intro/tab counts now read off real array lengths. No EmailGate (legacy never had one here — it's an open calculator, not a report unlock), matching /find-your-peptide's precedent. AssessmentResultActions wired with resultSlug="soulscore". journey-tracker.tsx's JOURNEY_MAP and /impact-dashboard's "Launch SoulScore Engine"/"Launch C-NPV Calculator" links (previously a disabled "Coming Soon" note) now point at the real page. This closes the real dead-end referenced from site-nav-data.ts (/soulscore appears twice in nav) and from /impact-dashboard — the last item in the STATUS.md dead-end</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/self-portrait</t>
+  </si>
+  <si>
+    <t xml:space="preserve">composite of completed assessments. Decision made: local-only (a real cookie, not Supabase — Phase 2 isn't provisioned yet). AssessmentResultActions (components/assessments/result-actions.tsx) takes an optional resultSlug and logs completions to a tg_assessment_results cookie via lib/assessments/result-log.ts, the same real-cookie-read-via-next/headers pattern already established by returning-visitor-hero.tsx/track-last-blog-visit.tsx — the page itself is a Server Component reading that cookie with zero client hydration step. Real, deliberate scope cut, not a silent one: legacy's SelfPortrait.tsx combined each assessment's own per-dimension scores (16 separate localStorage keys) into one composite radar chart across 15 unified dimensions, gated behind "5+ completed." This migration's result log only ever records that an assessment was completed, not its actual scored answers — building the real composite radar would mean threading a second, much larger data channel through every quiz. Shipped the honest subset instead: a real completed-assessments list (title, real completion date, retake link) plus a real "X of N completed" count and a "Still to Explore" section for the rest, via a new lib/content/self-portrait-catalog.ts. Wired resultSlug into the 7 remaining older "Find Your X" quizzes that already call AssessmentResultActions but hadn't been threaded yet (spirit/therapy/religion/sake/coffee/peptide/me) — /self-portrait now tracks 13 real assessments total. /find-my's "Sel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/the-mirror (+ /life-assessment)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">uses mirrorData.json, real 6-dimension/18-question life assessment ("The Mirror") ported into a typed lib/content/mirror-data.ts. Legacy served the identical component at both paths; /the-mirror is canonical (it's the only URL every existing internal link already pointed to — nav, journey tracker, Find Your Me), /life-assessment permanently redirects there. Real dimension-averaged scoring, radar chart via the shared AssessmentRadarChart, and weakest-dimension article/satellite-site recommendations ported unchanged. A live Sanity check found only 27 of 85 legacy article slugs still resolve; recommendations now resolve server-side and defensively skip missing ones, matching legacy's own behavior. Fixed: a hydration-unsafe typeof window branch computing the share URL, three stale manus.space satellite URLs superseded by their current live counterparts already used elsewhere in this migration, and dead /assessments/*/external-stub links in the "Journey Continues" grid. Added find-your-mirror to kit-source-tags.ts's KIT_TAG_MAP and reconciled journey-tracker.tsx's stale 10-minute estimate to legacy's real "~4 minutes" claim. find-your-me.ts's ecosystem-directory status flipped to "live." Verified live: 200 OK on both paths, redirect confirmed, typecheck/lint clean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/assessment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">confirmed via full legacy read this is not a "Find Your X" quiz (it predates that convention): it's Tony's own 3-way reader-path diagnostic — Builder / Crusader / Investor — 5 real questions, one point per matching answer, highest tally wins. Real questions and real archetype copy ported unchanged, reused from lib/content/archetypes.ts (already ported for /essays's archetype filter) rather than duplicated — added the page's ASSESSMENT_QUESTIONS to that same module since both come from the identical legacy source file. Preserved the real, distinct UX (no landing screen, no ThemedBackground/JourneyTracker — this page sits outside that ecosystem). Real bugs fixed: JS onMouseEnter/onMouseLeave inline-style hover hack replaced with Tailwind hover: classes; literal "..." pending-state text replaced with a real Loader2 spinner per house rule; dead trpc.subscribe.add replaced with a real POST /api/subscribe call. Real link audit: kept /impact-dashboard, /find-your-me, /living-declaration, and the real /blog/boiling-the-human-summit-harvard-kurzweil article as live links; /soulscore and /humanos are established forward-references used repeatedly elsewhere in this migration and both now ship too. The Human OS CTA reuses the border-red-800/30 text-red-800 treatment /living-declaration already established for the identical button instead of a new one-off raw-hex pair. AssessmentResultActions resultSlug="assessment" added (didn't exist when legacy was written). Added assessment-builder/as</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fix dead-end pages flagged in STATUS.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sake, therapy, and love-language all got real next-step navigation (WhatsNext + real "Journey Continues" links) during their ports — the last remaining one, soulscore, is now built (see above), closing this out.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Port shared radar-chart / PDF-export / email-gate components used across assessments</t>
+  </si>
+  <si>
+    <t xml:space="preserve">components/assessments/{radar-chart,result-actions,email-gate}.tsx, built during Phase 9 and reused unchanged by all 15 "Find Your X" quizzes plus /find-your-me.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">src/lib/admin/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">guardrails (fixes the removed version's proxy.ts pattern, which missed the real src/proxy.ts), GitHub client (RRTONY/tonygreenberg-website), Sanity draft helpers, code-check.ts (ESLint + CONTRIBUTING.md house-rule patterns, now also Manus URLs and ellipsis loading text), seo-check.ts, tools.ts, mcp-server.ts, mcp-handler.ts, mcp-tool-context.ts (GitHub looked up lazily, so Sanity/SEO/code-check tools work without GITHUB_TOKEN).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Per-person access via MCP_ADMIN_USERS (read/edit/write roles, tools filtered per role, calls logged, commits stamped [by &lt;name&gt;])</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mcp-auth.ts.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rules gate: get_project_rules serves CONTRIBUTING.md + AGENTS.md + docs/ai/ guides with a rulesVersion; all 6 write tools require it</t>
+  </si>
+  <si>
+    <t xml:space="preserve">project-rules.ts.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">src/app/api/mcp/route.ts (header auth) + src/app/api/mcp/[token]/route.ts (token in URL).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">docs/ai/ knowledge base (README, TASK_GUIDE, PROJECT_STRUCTURE, project_mcp_server), linked from CONTRIBUTING.md.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">@modelcontextprotocol/sdk ^1.30.0 re-added (approved 2026-09-29); GITHUB_TOKEN/MCP_ADMIN_USERS/MCP_SITE_ORIGIN documented in .env.local.example.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verified locally</t>
+  </si>
+  <si>
+    <t xml:space="preserve">auth (401/405), role filtering, rules-gate markers, token-in-URL route, code check, Sanity query, SEO check.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sign-in for the MCP server (OAuth 2.1, ported from ramprate-ui, 2026-09-30)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/oauth/authorize sign-in page + /.well-known metadata + register/authorize/token endpoints, stateless (signed tokens, no database), no new dependency. Verified end to end on a local production build. See docs/ai/project_mcp_server.md.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Set GITHUB_TOKEN, MCP_ADMIN_USERS, MCP_LOGIN_PASSWORD, MCP_OAUTH_SECRET, MCP_SITE_ORIGIN, MCP_PUBLIC_ORIGIN in Netlify (done) (checked 2026-…</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10-07: all already set in Netlify). Left: connect Claude.ai to /api/mcp for real, and verify the GitHub flow end to end (branch → PR → deploy preview → publish_changes) against a real PR.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Commit a team-wide .mcp.json (URL only) once the production URL is settled.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Google read-only tools added (2026-10-02)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">check_analytics (GA4), search_console_sites / _performance / _inspect_url / _sitemaps (list only, no submit or delete), lighthouse_check_page (PageSpeed Insights). New files google-auth.ts, ga4-client.ts, gsc-client.ts, lighthouse-check.ts; no new dependency. Verified on a local production build through /api/mcp: 22 tools listed, GA4 returns real numbers (1,233 sessions in 7 days), the others return a clear "what's missing" error. Env vars added to .env.local.example.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">publish_changes fixed (2026-10-02)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">it published every draft in Sanity (31 waiting for review today), so any one-line fix would have pushed them all live. Now it publishes only the drafts named in draft_ids; unknown ids are refused before anything happens (verified).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">seo_check_page decoded &amp;#39; but not React's &amp;#x27;, so descriptions showed Tony Greenberg&amp;#x27;s and the length was off</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fixed and verified (2026-10-02).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Search Console access for the service account added by the team (2026-10-02); all four search_console_* tools verified with real tonygreenbe…</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rg.com data (99 clicks / 1,663 impressions in 28 days, homepage indexed, sitemap 284 URLs, 0 errors, 82 warnings).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GOOGLE_GA_CLIENT_EMAIL, GOOGLE_GA_PRIVATE_KEY, GA4_PROPERTY_ID_TONYGREENBERG set in Netlify (2026-10-02, via the Netlify API, values checked…</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> equal to .env.local; this plan can't limit a variable's scopes, so they're available to builds and functions). Used from the next deploy.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Per-request change system ported from ramprate-ui (2026-10-02, owner said yes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">, covering the 10 review points the team raised for RampRate's setup: (1) discard_change; (2) one request = one change with its own branch, PR and drafts, so publishing never takes another request live; (3) a review with pages affected, a server-written "what's included" line and preview links; (4) publish needs the review's reviewToken, and the rules make the AI ask "You are about to publish these changes to the live tonygreenberg.com website. Are you sure you want to continue?"; (5) list_change_history, also visible read-only in Studio under "Website change history" (new adminChange type); (6) undo_change; (7) before/after (automatic for Sanity, given by the AI for code); (8) preview_on_devices phone + laptop screenshots (needs GOOGLE_API_KEY); (9) the AI's plain summary plus the server's facts line; (10) Draft → Ready for review → Published / Discarded. Files: change-sets.ts, change-describe.ts, device-preview.ts, mcp-tool-context.ts, mcp-server.ts, github-client.ts (RampRate's full version), src/sanity/schemas/adminChange.ts, sanity.config.ts. Tested end to end with a real throwaway change, then discarded (see docs/ai/project_mcp_server.md).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Merge the CI fix into main</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(done with PR #3; checked 2026-10-06: main's pr-lint.yml runs Node 22 and next typegen before the type check). The test change's GitHub check failed because main still has the old pr-lint.yml (Node 20 crash). Every MCP change will fail its site check, and so can't be published, until this branch's work (or at least .github/workflows/pr-lint.yml) is on main. Then test a real publish and undo_change.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blocked on you (Google)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">create a GOOGLE_API_KEY in Google Cloud (project of the vcos-ga4-reader service account, where the PageSpeed Insights API is already on), restricted to the PageSpeed Insights API, then add it to .env.local and Netlify. Creating it from here was blocked by the session's safety check (it would use the service account's credentials to change the Cloud project). Note lighthouse_check_page may time out on Netlify (10 s function limit on the free plan).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Per-page generateMetadata (title, description, OG, Twitter Card, canonical) for every ported route, sourced from Sanity seo object where con…</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tent is CMS-backed, static otherwise. Audited all 140 page.tsx files: only /studio has none (correct — it's robots.txt-disallowed, not public content). Real gap found and fixed: /blog/category/[slug] had no alternates.canonical at all, and no page-aware title for its own real pagination (?page=N) — every paginated page was serving an identical title with no canonical, a real duplicate-content signal. Fixed: generateMetadata now reads searchParams too, self-canonicals each page (?page=N pages canonical to themselves, not consolidated to page 1 — genuinely different posts per page, matching Google's current pagination guidance) and appends "— Page N" to the title past page 1. Verified live: page 1 canonicals to the bare URL, ?page=2 canonicals to ?page=2 with a distinct title.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sitemap.ts generated from real Sanity content + static route list, auto-updates on publish</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extended from the Phase 5-era version (homepage + blog posts only, 122 URLs) to every real route: the full static route list (130 routes, generated from find src/app -name page.tsx, excluding /studio (robots.txt-disallowed), /(auth)/login (noindex via its own metadata), and /life-assessment (a pure redirect, not distinct content)) plus all 5 real dynamic sources — blog categories (allCategorySlugsQuery), BrewSoul cities (25), BrewSoul coffees (107), and charity-scorecard entries (103) — each pulled from the exact same data source its own page's generateStaticParams already uses, not re-derived. Auto-updates on publish for anything Sanity-backed (blog posts/categories) since it's a live client.fetch on every build; the static route list itself needs a one-line addition whenever a new page ships (same as any other route-registration step). Verified live: 496 real &lt;loc&gt; entries, spot-checked a coffee/city/charity/category URL each, typecheck/lint clean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">llms.txt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fetched verbatim from the still-live site and saved to web/public/llms.txt (real content: Tony's bio, expertise, full article index by category, every product/tool section) — do this before Manus goes away, it won't be recoverable after</t>
+  </si>
+  <si>
+    <t xml:space="preserve">robots.txt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">same approach: fetched the real live file (not my earlier guessed robots.ts, which has been removed) and saved verbatim to web/public/robots.txt, plus added Disallow: /studio for the new Sanity Studio route. Confirmed live: real AI-crawler allowlist (GPTBot, Claude-Web, PerplexityBot, etc.), scraper blocklist, and the site's non-standard LLMs: directive all intact</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JSON-LD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WebSite + Person schema ported verbatim from the live homepage's actual &lt;script type="application/ld+json"&gt; tags (not reconstructed from memory) — rendered site-wide from src/lib/structured-data.ts in the root layout. The Person image was hardcoded to a /api/img/... legacy proxy path on the live site — rescued that headshot (downloaded it while still live, uploaded to Sanity as the author-tony-greenberg document's avatar) so the new site's JSON-LD has zero Manus dependency instead of just copying the fragile path forward</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Article JSON-LD on /blog/[slug], built from real per-post Sanity data (headline, image, datePublished/dateModified, author, canonical URL)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">verified live on a real post</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/path/:archetype (src/app/path/[archetype]/page.tsx)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">per-archetype landing page for /assessment's Builder/Crusader/Investor result, reusing lib/content/archetypes.ts. Real content ported in full (top-5 essential-reading list per archetype via allPostsForArchiveQuery, real PathSubscribeForm posting to /api/subscribe, AUTHORITY_ITEMS strip). Real bug fixed vs. legacy: replaced a hand-rolled inline-styled "Path not found" div with a real notFound() (this route's generateStaticParams only ever produces the 3 real keys). Verified live: all 3 archetype routes 200 OK, typecheck/lint clean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/my-journey (src/app/my-journey/page.tsx + components/assessments/my-journey-dashboard.tsx)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"My Journey Dashboard," real grid/timeline views across all 28 JOURNEY_MAP experiences, category/status filters, phase progress ring, recommended-next card, using the same real useJourneyProgress/JOURNEY_MAP completion tracking every "Find Your X" quiz already writes to (not the narrower tg_assessment_results cookie built for /self-portrait). Legacy's per-quiz scored-result caching (RESULT_KEYS, feeding a mini radar chart) was not ported — no quiz in this migration writes that data either, same honest-degradation call already made for /self-portrait's own composite radar. Fixed a real legacy dead link (/ecosystem-map, a still-unbuilt page) to /self-portrait. Verified live: 200 OK, real content confirmed, typecheck/lint clean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/the-open-door (src/app/the-open-door/page.tsx)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">real press/credibility content: all 10 "Magic Genie" client-pitch prompts (real named targets — Marco Argenti/Goldman Sachs, Adam Smith/Disney, etc.), 18 real client testimonials, all 8 explicitly-labeled satirical "parody" quotes (kept with disclaimers, not presented as real). Real overlap found and reconciled: this page's publications/speaking/podcasts arrays substantially duplicate the already-shipped /published's fuller bibliography — kept only what /published doesn't cover (Forbes + Business Insider bylines, the Clinton Global Initiative keynote, 4 of 5 podcast appearances) and cross-linked to /published for the rest, same reconciliation pattern as /assessments vs /find-my. Real bugs fixed: 3 genie/keynote links pointed externally at tonygreenberg.com/&lt;slug&gt; for posts that are real internal posts in this migration — relinked to /blog/psychedelics-could-become-extractive-capitalism, /blog/boiling-the-human-summit-harvard-kurzweil, /blog/return-on-investment-going-green-going-green-2 (all verified 200); a bare self-link to tonygreenberg.com remapped to /. Ships as a pure Server Component (legacy's FadeIn/Section/editorial-component dependencies don't exist here and weren't needed). Verified live: 200 OK, real content in raw SSR HTML, typecheck/lint clean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Homepage "Recent Updates" band (2026-09-29)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">on the live site (a newer Blog.tsx than _legacy-manus-app/, so rebuilt from the live page's markup), replacing the older "Latest Thinking" pair. Found while doing it: two live essays are missing from Sanity, the-tollbooth-and-the-alternative (Aug 18, 2026, the live site's newest) and what-quest-could-fix. Both were published on live after the legacy snapshot and need importing.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Re-sync the legacy reference</t>
+  </si>
+  <si>
+    <t xml:space="preserve">_legacy-manus-app/ is older than what's live (Recent Updates proves it), so visual diffs should be against the live site, not only that folder.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Visual diff pass: every ported page vs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">legacy page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Padding / spacing on the story pages matched to live (2026-10-01)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Measured margins, text column and spacing on 31 pages, live vs a production build, at 375px and 1280px. The "door" story pages were the clear mismatch: live's text column is ~546px (ours was 720px), 20px side margins on phones / 40px on desktop, body text 19px/1.8 on phones and 18px/1.85 on desktop (ours 16px/1.5). Fixed on /the-body, /engine-room, /under-nda, /the-nightstand, /the-web, /the-territory, /about, /intel (Intel uses live's 16.8px/1.9; About's hero line 480px max, 18.4px/1.8). Re-measured: all 8 match live to within 2px (About's column 28px narrower), no sideways scroll at 375px.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Header-to-title spacing re-checked (2026-10-02)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The 2026-10-01 note compared different things: live's header wasn't measured (it showed 0), so "96px vs 168px" was really 161px vs 168px from the top of the page. Measured again from the top of the page, live vs a production build, at 375px and 1280px: most pages were already within 10px. Fixed the real gaps: /the-open-door (now live's dark centered hero band, 56px title, 546px text column; title was 72px too high), /start-here (live's 48px/96px top padding; 25px too high on desktop), /invest and /engage (label spacing and live's 32px/51px title; /invest's desktop title was 36px), /impact-dashboard on phones (card edge to edge under the header like live; title was 89px too low). Re-measured: all within 8px of live, no sideways scroll at 375px, no JS errors.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HumanOS headings in capitals like live (2026-10-02, owner said yes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">the 4 headings live capitalises on /humanos (title, "Are you a Maximizer...", "Take the Diagnostic", "The Diagnostic") get uppercase; the words are unchanged. The subpages already matched.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">More layout gaps matched to live (2026-10-02)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/series (live's centered 546px column, and a bug fixed: every card kept an empty 240px picture column, squeezing the text; live's per-series picture is one generic placeholder on the Manus proxy, so not copied), /humanos (middle section 900px like live), homepage desktop widths (hero text 804px, Four Doors 1000px, Editor's Picks 1168px, GemSpark edge, section title sizes; live's /blog now shows the homepage), /find-my (photo undimmed and plain background, like live; our site header kept). Re-measured: headings within 3px (/series) to 20px (homepage) of live, no sideways scroll, no JS errors. Note: live's "New here?" tour bar sits over its header and doesn't move the page, so it doesn't affect these numbers.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Full sweep vs live (2026-10-02)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">142 pages (every non-blog page, 3 of each templated set) at 375px and 1280px, title position, text column, title size. Fixed the shared causes: BrewSoul (live wraps most pages in its frame twice, so a second 52px offset plus the category badge; the landing, cities, directory and quiz pages have neither: src/components/brewsoul/brewsoul-main.tsx; intro paragraphs uncapped like live; 38px titles), Kava (live's extra 52px offset), /the-body, /the-nightstand, /the-web (405px top photo like live), the 6 peptide pages (live's 768/896px intro column), /journeys, /pick-up-the-phone, /published, /ecosystem (546px story column and live's text size). Re-measured: 110 of 120 within 40px / 60px of live.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sweep leftovers fixed (2026-10-06)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ported legacy's exact title sizes, margins and column widths. Measured live vs a production build at 375px and 1280px (H1 distance from the top, H1 size, intro and table widths). Now within 8px and the same title size on /published, /brewsoul/first-sip, /brewsoul/home, /brewsoul/chains (intro 912px like live), /brewsoul/browse, /brewsoul/directory (3-column 952px grid like live), /brewsoul and /brewsoul/quiz (intro 520px), /amplifier (546px column), /diamond-cut, /speaking, /living-declaration, /spirits, /protecting-your-business (tables 730px), and the 5 HumanOS subpages (titles smaller like live, 752px column). No sideways scroll at 375px. Left on purpose: /self-portrait (font matches; our page has a different title and no back link, so it sits 23-57px higher), BrewSoul pages 3-6px off (the shared journey bar row), and the different-layout pages /dharma-finder, /grant-study, /search, /quiz_25q, /soulscore. Also: /brewsoul/quiz rebuilt as a step registry (src/components/brewsoul/brewsoul-quiz/: parent + hook/ + components/step-* + data/), same questions, scoring and look; Back/Skip/Retake use lucide icons. New CONTRIBUTING rule 19 (multi-step flows, FydoPartner pattern). brewsoul-welcome-quiz.tsx (/brewsoul) still has the old shape and text arrows.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Match live's redesigned pages (2026-10-06, owner said go)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/self-portrait (live: dark page, progress ring, "N more brushstrokes" lock until 5 assessments), /grant-study and /dharma-finder (live opens straight on question 1, no intro screen), /quiz_25q (live adds a hero picture above the title; rescue it into Sanity first), /search (live: one search box across essays, BrewSoul, peptides, HumanOS, assessments, kava and pages with filter chips). Measure live vs a production build at 375px and 1280px when done. Done 2026-10-06: /grant-study and /dharma-finder open straight on question 1 like live (title block / part header above the first question, live's 546px column, plain page, credit under every question), both rebuilt as step registries (rule 19); measured within 3px of live at the top (dharma's question block within 7px). /quiz_25q's hero rescued into Sanity and placed like live (within 2px). Found and fixed on the way: on the deployed copy /grant-study's answer buttons could not be clicked (the themed page background was fixed z-0, painted over the quiz); ThemedBackground is now -z-10 pointer-events-none (backgrounds unchanged on all 21 pages that use it), and the shared email gate no longer scrolls sideways on phones. Both quizzes clicked through to results in Chrome and Safari. /self-portrait restyled to live (dark page, "The Composite You", progress ring, "N More Brushstrokes Needed" lock until 5 done, live's copy) on our real cookie data; within 3px of live at both widths; tested with 0, 2 and 6 completed. Counts are ours (13 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Still different from live (needs a yes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">blog posts (done) (done 2026-10-07, see Phase 5); /find-my on live hides the site header. /walk-through is a 404 on live now.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Design change on live, needs a decision</t>
+  </si>
+  <si>
+    <t xml:space="preserve">live's story pages now use Cormorant Garamond for titles (ours: Playfair Display), a lighter title weight (400 vs our 700), and a red eyebrow label (#8E1E25, wider letter spacing) instead of our gold. A site-wide font swap is a design call, so not done.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Link check across all ported pages (no 404s, no broken internal cross-references)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">First full pass done 2026-09-29 (510 pages crawled from the sitemap plus every internal link, on a production build). Fixed in code: /brewsoul/coffee/…-tarrazú 404 (the route got the id still percent-encoded), 30+ links that went through the /assessments/* redirects, /find-your-me's dead Homeaglow link, the two root-level Iboga essay links, and the dead FauxTony nav item. Fixed as Sanity drafts (scripts/fix-blog-body-links.ts, 14 posts): broken post links, leaked !… placeholder text, Energy Is Money's split author bio, and scraped WordPress furniture ("Share this / Related / You Might Also Like / Copyright", "Show More / Top News", [mc4wp_form]). Left for a decision: /framework's "Ask FauxTony" button, when-healing-becomes-extraction's two links to a Dr. Lee case file that doesn't exist, and the-clock-keeper-chronicles-part-1's link to the deferred /clock-keeper-part-2. Re-run after the drafts are published. 2026-10-01 re-run (local production build, all 498 sitemap URLs load; 440 unique internal links): 5 broken. Fixed as a Sanity draft: molecule-as-mirror-10-what-the-pioneers-know's "Final installment" link pointed at a non-existent part-10 slug (now part 11; live also shows that line twice, kept). Already fixed in a waiting draft: forever-chemicals-... → /blog/psychedelic-readiness-index. Still the 3 known decisions: /fauxtony (from /framework), /clock-keeper-part-2, /blog/the-case-file-dr-samuel-lee.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lighthouse pass (performance/accessibility/SEO) on top 20 pages by traffic 2026-09-30, 20 key pages (no traffic data yet), local production …</t>
+  </si>
+  <si>
+    <t xml:space="preserve">build, mobile: averages performance 87, accessibility 99→100, best practices 100, SEO 92→100, CLS 0 everywhere. Fixed: public/robots.txt had an LLMs: line (not a real directive) that made Google treat the whole file as invalid, now a comment; h3/h4 headings skipping a level on /assessments, /kava, /peptide-watch (same look, right tag); the Kava and /attention-theft back-arrow links had no accessible name on phones; two small phone-width contrast misses. Left: performance is local-machine only (±10-15 points, see CONTRIBUTING.md); the slowest were / 76 (LCP 5.2 s), /psychedelic-readiness-index 82, /iboga-ibogaine 83. Re-run against the Netlify deploy before launch. 2026-10-06 re-run against the Netlify deploy (14 key pages, mobile): accessibility 100 and CLS 0 on every page, SEO clean (only the expected netlify.app noindex), performance 77-97 held back by 3-4 s LCP. Fixed: all 21 hero images moved off the deprecated priority prop to fetchPriority="high" + loading="eager" (Next 16); /iboga-ibogaine hero and the first card on /blog and category pages no longer lazy-loaded; sizes on the Four Doors cards (~150 KiB per page), /humanos diagram (~100 KiB) and /about headshot; urlFor no longer imports the Sanity client, so ~115 KB of Sanity client code stopped loading on / and /blog; React hydration error #418 on / and /blog (post dates) gone, checked in two time zones; /blog is static again; empty icon &lt;th&gt;s on /iboga-ibogaine labelled; category page reads use sanityFetch(). Left: se</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SEO audit fixes (2026-10-06)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Checked an outside audit point by point against the code. Fixed: Core Themes cards linked to /?theme=…#essays-archive (not crawlable, counts from a stale hand-kept list) and now link to /blog/category/&lt;slug&gt; with real counts (21/25/20/14, matching the archive pills; THEME_MAP and the ?theme= filter removed); Four Doors cards were &lt;button&gt;s, now real links that still open the modal on a plain click; "DIAGNOSE · ENGAGE" now link to /find-my and /engage; one shared formatPostDate (Asia/Kolkata, src/lib/format-post-date.ts) so a post no longer shows two different dates; the title repeated as the first body paragraph is dropped at render time (legacyBodyLayout); essay cards are h3 under a section h2 (archive, Read next), h2 only on category/search; heading glyphs (◆ ✦) hidden from screen readers; posts send BlogPosting with the author tied to the site Person (@id) plus a BreadcrumbList; descriptive alt on the homepage and BrewSoul heroes; homepage OG image cropped to 1200x630 JPEG. Already fine (audit could not see it): Person/Article schema, Netlify noindex, robots.txt, sitemap, header nav and search, Amazon links carry no affiliate tag. Checked on a production build: type check, lint, build, status codes, browser click test at 375px, no console errors. Implementation pack (Mohammad Danish, 2026-10-05) checked the same day: added og:type/og:site_name back on the 6 pages with their own openGraph (a page-level openGraph replaces the layout one), twitter:creator, and on posts og:url</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SEO audit items needing a yes (2026-10-06)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">the pack's new copy (homepage title/description, five-cups title, description, short answer, FAQ, heading rewrites, entity statement, newsletter block, author box, health disclaimer, COA wording); "Further Reading" shown twice on posts (merge the lists?); long post title (84 chars), homepage description length and obsolete keywords tag, slugs (/blog/five-cups, the -2 slug; would need redirects), "Six lenses" over four cards, sources for health claims and proof for "$10B+", "Certified B Corp", "Validity: 91", legal review of the homepage Case File banner, ABIT waitlist disclosures, one contact email, the two one-post categories, fewer homepage CTAs / email signup / table of contents / explaining "COA".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Connect Google Search Console + GA4 to the new deployment on day one of cutover</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Restore/adapt the manus.space triple-layer noindex lockdown pattern for any remaining staging URLs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-01: the Netlify copy (tonygreenberg-website.netlify.app) and every deploy preview had no noindex at all, so Google could index a duplicate of the site. next.config.ts headers() now sends X-Robots-Tag: noindex, nofollow on any *.netlify.app host only; tonygreenberg.com is unaffected, so nothing to remove at cutover. Tested with Host headers on a production build.</t>
+  </si>
+  <si>
     <t xml:space="preserve">"Keep going" strip above the footer on every page (2026-10-07)</t>
   </si>
   <si>
@@ -940,757 +1693,10 @@
     <t xml:space="preserve">dark top sections, narrow single text column, short red section rules and dark call-to-action bands on /invest, /amplifier, /community (now "Sign In to Join the Community", linking our real sign-in; live's made-up counters left out), /framework, /the-letter (daily provocation with "Share this thought" and "Search past provocations"), /engage, /diamond-cut, /ecosystem and the homepage's "The thinking doesn't stop here" band. Kept on purpose: AA-contrast colours where live's fail, "Enter the Gate" instead of live's $5,000 checkout on /diamond-cut.</t>
   </si>
   <si>
-    <t xml:space="preserve">/brewsoul</t>
-  </si>
-  <si>
-    <t xml:space="preserve">welcome/landing gate (built, not yet pushed — pending local review), along with the shared foundation the rest of Phase 6 depends on. Ported BrewSoulLayout.tsx → app/brewsoul/layout.tsx + components/brewsoul/brewsoul-nav.tsx (BrewSoulNav/BrewSoulFooter), CategoryBadge.tsx → components/brewsoul/category-badge.tsx, brewsoul-config.ts → lib/content/brewsoul-config.ts, and BrewSoulDirectory.tsx's CATEGORIES/PAGE_CATEGORY_MAP data (not the page itself yet) → lib/content/brewsoul-directory.ts. Real architecture decision: BrewSoul is a self-contained sub-site with its own nav/footer/coffee-brown palette, same as legacy — but this app has one flat root layout with no route groups, so the main site's SiteHeader/SiteFooter needed to be suppressed for this one subtree without restructuring every existing route. Added components/site-chrome.tsx (SiteChrome, a small client wrapper checking pathname.startsWith("/brewsoul")) around both in app/layout.tsx — verified via literal &lt;header&gt;/&lt;footer&gt;/&lt;nav&gt; tag counts in real SSR HTML (not text search, which false-positives on Next dev mode's RSC debug payload) that /brewsoul gets zero main-site chrome and its own real nav+footer, while / still gets exactly one of each. Dropped TonyAvatarTrigger (FauxTony chatbot widget — Phase 10, no backend yet, same "don't fake it" call made elsewhere) from the nav. Ported BrewSoulWelcome.tsx → components/brewsoul/brewsoul-welcome-quiz.tsx (8-screen onboarding quiz, real identity-scoring logic, palate questions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/brewsoul/first-sip</t>
-  </si>
-  <si>
-    <t xml:space="preserve">onboarding intro (built, not yet pushed — pending local review). Ported "The First Sip Is a Vote" in full — the complete manifesto essay (5 sections, 3 pullquotes, the couplets block, the disclosure-demands grid), the 5-tool journey map, 6 related-essay links (real slugs, cross-checked against this session's already-verified corpus), the closing + sources, and the email capture. Built as a Server Component (all static except the email form) + components/brewsoul/next-steps.tsx (shared "what's next" CTA, itself a Server Component — legacy's hover effects were plain CSS-able, no JS state needed) + components/brewsoul/first-sip-email-capture.tsx (client island, mailto: fallback since no subscribe backend exists, same pattern as newsletter-popup.tsx). Dropped the canvas CoffeeDust decoration and the confirmed-dead hero photo (/api/img/brewsoul-orig_84eb4bc9.jpg, 404, same Manus proxy) — with no image left, the scroll-linked parallax that moved it went too. The 5 tool-card links (prescription/health/pairings/economics/compare) point at later Phase 6 routes not built yet — same forward-reference pattern as /find-my. Verified live: 200 OK, full essay text present, CategoryBadge correctly shows "Start Here" (from PAGE_CATEGORY_MAP), zero main-site chrome leaking in, typecheck/lint clean.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/brewsoul/home</t>
-  </si>
-  <si>
-    <t xml:space="preserve">the real BrewSoul dashboard (distinct from /brewsoul's identity-quiz welcome gate and /brewsoul/first-sip's manifesto): hero + stats, Follow the Dollar teaser, Top QPR coffees (computed live via computeQPR), the 2025 crisis callout, New Drops, a Wall of Shame preview (SHAME_ENTRIES), the research-hub card grid, and a cyclable health-fact ticker (components/brewsoul/health-ticker.tsx, its own small client island so the rest of the page stays a Server Component). Canvas WarmParticles/ParallaxBg decorations and the dead hero photo (/api/img/brewsoul-orig_84eb4bc9.jpg, same confirmed-404 Manus proxy used elsewhere in Phase 6) dropped for CSS gradients. Stats use the real live BREWSOUL_COFFEES.length (107) in place of legacy's stale "103". Verified live: 200 OK.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/brewsoul/browse</t>
-  </si>
-  <si>
-    <t xml:space="preserve">coffee listing (components/brewsoul/browse-explorer.tsx), real filter/search over the full BREWSOUL_COFFEES catalog. Verified live: 200 OK.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/brewsoul/coffee/[id]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">coffee detail page (breadcrumb, QPR + tier header, quick stats, tasting notes, flavor-profile bars, the 4 intelligence scores, transparency/ethics data, buy links, competition wins, similar-coffees cross-links, journey CTAs), server-rendered with generateStaticParams over all 107 real coffees (this repo's bounded-dynamic-route convention, same as /blog/[slug]) instead of legacy's client-side useParams lookup. Verified live: 200 OK.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/brewsoul/quiz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">matching quiz (built, not yet pushed — pending local review), along with the real data/engine foundation most of the rest of Phase 6 depends on. Ported lib/intelligence-engine/{types,scoring}.ts verbatim (generic scoring engine — QPR/availability/scarcity/wow/tier/freshness — reusable beyond BrewSoul) and the full coffee catalog (legacy's 3 files: brewsoul-coffees.ts + -expanded.ts + -expanded2.ts, merged at import time) → one lib/content/brewsoul-coffees.ts, extracted via tsx (not hand-typed — 107 real entries, ~6.5K lines). Caught a real stale count: legacy's own file header claimed "105" and its UI copy said "103", but the actual merged arrays contain 107 — this migration shows the live BREWSOUL_COFFEES.length everywhere instead of a repeated hardcoded number. Ported JourneyBar.tsx (components/brewsoul/journey-bar.tsx) — the fixed bottom "what's next" bar shown on every BrewSoul content page except the identity quiz — and retrofitted it onto /brewsoul/first-sip too (built before JourneyBar existed). Built components/brewsoul/brewsoul-quiz.tsx: real 7-question taste quiz scored against each coffee's real flavorProfile via the real scoring engine, ranking the full catalog by match. Legacy's useMarkVisited was renamed to markVisited (it's a plain localStorage write, not a hook — its old use-prefixed name tripped React's rules-of-hooks lint when called from inside a useEffect). Dropped the canvas WarmParticles decoration and the dead hero photo (same confirmed-404 Manus proxy,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/brewsoul/wall-of-shame</t>
-  </si>
-  <si>
-    <t xml:space="preserve">content page. Real 13 entries (brand/category/evidence/severity/response) from SHAME_ENTRIES, unchanged. Category filter buttons extracted into components/brewsoul/shame-explorer.tsx (the only interactive piece) so the page itself stays a Server Component. Verified live: 200 OK.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/brewsoul/follow-the-dollar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">supply-chain essay. Real DOLLAR_BREAKDOWNS segment bars (farmer/exporter/importer/roaster/retailer %, real commentary), unchanged. The farmer-segment bar's data-driven color (green/gold/red by threshold) is a small known set of variants — precomposed as 3 literal Tailwind classes rather than an inline style background, per this repo's dynamic-class rule; only the genuinely per-item width stays as style. Fully static, Server Component. Verified live: 200 OK.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/brewsoul/farms</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sourcing content ("Farm Passports"). Real FARMS entries (country/region/producer/altitude/story/varieties/certifications), unchanged. Fully static. Verified live: 200 OK.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/brewsoul/mold-free</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mycotoxin content. Real verified/claims/untested split computed live over the full BREWSOUL_COFFEES catalog by moldTestStatus. Fully static. Verified live: 200 OK.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/brewsoul/experiences</t>
-  </si>
-  <si>
-    <t xml:space="preserve">experiential content ("Experience Map"). Real EXPERIENCES entries (farm tours, cafés, cupping labs, roastery visits), unchanged. Country filter buttons extracted into components/brewsoul/experiences-explorer.tsx, same split-out-the-interactive-bit pattern as wall-of-shame. Verified live: 200 OK.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/brewsoul/health</t>
-  </si>
-  <si>
-    <t xml:space="preserve">health deep-dive, ported from BrewSoulHealthFull.tsx (the file legacy's own router actually uses for this route — BrewSoulContent.tsx's same-named BrewSoulHealth export is real but genuinely dead/unrouted code in legacy, shadowed by this one). Real 8 longevity findings with real citations/participant counts, 7 real risks with severity ratings, CYP1A2 caffeine-metabolism genetics, a 6-step chronobiology timing schedule, 8 real bioactive compounds, 3 real mycotoxin threats, and a 3-step "simplification protocol," all ported unchanged and verbatim. Dead Manus hero image dropped for a CSS gradient. Legacy's own redundant BrewSoulLayout wrapper dropped — app/brewsoul/layout.tsx already wraps every route. The two real interactive pieces (show-all-risks toggle, per-compound click-to-expand) split into components/brewsoul/health-{risks,compounds}.tsx client islands so the rest stays a Server Component. Legacy's bespoke earthy "science" palette (soil/clay/sage/moss — distinct from the rest of BrewSoul's amber/gold commercial palette) kept as a deliberate one-off sub-identity for this one page, same reasoning as /attention-theft's own "crusade" palette elsewhere in this migration. Verified live: 200 OK, typecheck/lint clean.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/brewsoul/varieties</t>
-  </si>
-  <si>
-    <t xml:space="preserve">reference: varieties. Real VARIETIES encyclopedia entries (species/origin/genetics/cup profile/yield/disease resistance), unchanged. Search extracted into components/brewsoul/varieties-explorer.tsx. Verified live: 200 OK.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/brewsoul/processing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">reference: processing. Real PROCESSING_METHODS entries (description/flavor impact/complexity/controversy), unchanged. Fully static. Verified live: 200 OK.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/brewsoul/roasters</t>
-  </si>
-  <si>
-    <t xml:space="preserve">reference: roaster directory. Real ROASTERS entries (philosophy/quality/transparency/farmer-equity scores), unchanged. Search + tier filter extracted into components/brewsoul/roasters-explorer.tsx. Verified live: 200 OK.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/brewsoul/glossary</t>
-  </si>
-  <si>
-    <t xml:space="preserve">reference: glossary. Real GLOSSARY terms, unchanged. Search + alphabetical grouping extracted into components/brewsoul/glossary-explorer.tsx. Verified live: 200 OK.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/brewsoul/pairings</t>
-  </si>
-  <si>
-    <t xml:space="preserve">reference: pairings. Real PAIRINGS (food/drink pairings by origin) and 3 real curated FLIGHTS (each linking to real coffees in the catalog), unchanged. Fully static. Verified live: 200 OK.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/brewsoul/economics</t>
-  </si>
-  <si>
-    <t xml:space="preserve">reference: economics. Real live-computed stats (coffee/origin/roaster/variety counts, average price, average farmer share via DOLLAR_BREAKDOWNS), a real price-distribution histogram, and a real top-origins ranking — all computed directly from BREWSOUL_COFFEES at render time, unchanged. Fully static. Verified live: 200 OK.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/brewsoul/compare</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tool: compare coffees. Real side-by-side comparison of up to 4 coffees across origin/producer/variety/process/price/cupping and the 4 intelligence scores (QPR/availability/wow/overall), unchanged. Interactivity in components/brewsoul/compare-explorer.tsx. Verified live: 200 OK.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/brewsoul/blend-builder</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tool: blend builder. Real combine-up-to-5-coffees ratio calculator with weighted-average QPR/Wow/Overall scores via range sliders, unchanged (never persisted anywhere in legacy either — a pure in-session calculator). Interactivity in components/brewsoul/blend-builder-explorer.tsx. Verified live: 200 OK.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/brewsoul/drops</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tool: product drops ("Latest Drops"). Real top-12-by-overall-score coffees. No client-side state at all (legacy's own useMemo had no changing dependencies — a pure derived list), so this ships as a plain Server Component. Verified live: 200 OK.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/brewsoul/collection</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tool: personal collection tracker ("My Collection"). Real save/toggle-to-collection behavior, unchanged. Real bug found and fixed: legacy read localStorage directly inside a useState initializer — unsafe during SSR, same hydration-mismatch class already fixed in journey-bar.tsx/journey-tracker.tsx — rebuilt around a module-level external store fed through useSyncExternalStore in components/brewsoul/collection-explorer.tsx. Also found and fixed: the already-ported brewsoul-directory.ts listed this page's path as /brewsoul/my-coffees — a real dead link in legacy's own directory (legacy's actual router only ever served this at /brewsoul/collection, /brewsoul/my-coffees never existed) — corrected to the real path. Verified live: 200 OK.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/brewsoul/submit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tool: submit a coffee ("Submit or Appeal"). Real submit-a-coffee / appeal-a-score form, unchanged in structure. Real bug found and fixed: legacy's own comment admitted "In production this would POST to a tRPC endpoint" but in the meantime wrote the submission to localStorage and showed "Received. We'll review your submission" regardless — actively misleading, since nobody would ever see a localStorage-only write. Replaced with a real mailto: fallback pre-filled with the form fields, same honest-degradation pattern as first-sip-email-capture.tsx — no fake success state. Verified live: 200 OK.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/brewsoul/prescription</t>
-  </si>
-  <si>
-    <t xml:space="preserve">personalized "prescription", ported from BrewSoulPrescriptionFull.tsx (the file legacy's router actually uses — BrewSoulTools.tsx's same-named export is dead/unrouted, same shadowed-file trap as /brewsoul/health). Real 5-step questionnaire (genetics/timing/health/flavor/budget) generating a real, deterministic prescription (generatePrescription — real roast/cup-count/brand/pricing/warning logic), all ported unchanged and verbatim. Legacy's trpc.coffeePrescription.generate AI-enhancement mutation doesn't exist in this migration — dropped along with its "AI ANALYSIS LOADING..." block, which would otherwise spin forever and never resolve; the real prescription itself never depended on that call, it's already fully computed client-side. Same bespoke earthy "science" palette as /brewsoul/health kept as the same deliberate sub-identity. Verified live: 200 OK, typecheck/lint clean.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/brewsoul/chains</t>
-  </si>
-  <si>
-    <t xml:space="preserve">"Top 100 Coffee Chains" ranking (not supply-chain visualization — that's /brewsoul/economics//brewsoul/follow-the-dollar; this is chain rankings). Real 100-chain dataset extracted from legacy's computed CHAIN_RANKINGS export (5 real weighted dimensions → aggregate → S-F tier) via a one-off tsx script (same approach as brewsoul-coffees.ts) into lib/content/brewsoul-chains.ts, with a new ChainEntry type added to intelligence-engine/types.ts. Real tier/type filters, search, and per-chain expand, unchanged, extracted into components/brewsoul/chains-explorer.tsx. Verified live: 200 OK, typecheck/lint clean.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/brewsoul/biodynamic</t>
-  </si>
-  <si>
-    <t xml:space="preserve">biodynamic content. The complete real census of Demeter-certified biodynamic coffee: 3 real source farms, 6 real roasters/brands with real product tables and pricing, real nutritional-science compounds, a real cost calculator, and a real impact/tokenization section, all ported unchanged and verbatim. Dead Manus hero image dropped for a CSS gradient. The 3 genuinely interactive pieces (click-to-expand farms/roasters, cups-per-day cost slider) split into components/brewsoul/{biodynamic-farms,biodynamic-roasters,cost-calculator}.tsx client islands so the rest stays a Server Component. Same bespoke earthy "science" palette as /brewsoul/health and /brewsoul/prescription kept as the same deliberate sub-identity. Verified live: 200 OK, typecheck/lint clean.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/brewsoul/decaf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">decaf content ("Paint Stripper or Pure Water?"). Real 3-process breakdown (methylene chloride/Swiss Water/supercritical CO₂), 13 real clean-decaf brands ("Hall of Fame"), 10 real methylene-chloride brands ("Wall of Shame," with real Clean Label Project lawsuit citations), a real carbon footprint comparison, real decaf health science, and a real price-comparison table, all ported unchanged and verbatim. Legacy's manual document.title/&lt;meta keywords&gt; mutation in a useEffect (a real anti-pattern — Next's generateMetadata already owns the head) dropped for the real metadata export. Real bug found and fixed: the 13-brand FAME dataset was initially exported from the "use client" decaf-fame.tsx component file and imported into the Server Component page for its price-comparison table — non-component exports from a client module aren't available across the RSC boundary, which threw FAME is not iterable at runtime (only caught by live verification, not typecheck/lint). Moved the data to a plain lib/content/brewsoul-decaf.ts module instead. The 2 genuinely interactive pieces (click-to-expand Hall of Fame, reveal-toggle Wall of Shame) split into components/brewsoul/decaf-{fame,shame}.tsx client islands. Same bespoke earthy "science" palette as the other /brewsoul deep-dive pages kept as the same deliberate sub-identity. Verified live: 200 OK, typecheck/lint clean.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/brewsoul/esoteric</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rare-coffee content ("Esoteric Coffee Index"). Real 9-coffee index across 2 tiers (Panama Geisha, Yemen Mokha, Liberica, Eugenioides, Wush Wush, Sidra, Pink Bourbon, Bourbon Aji, Sudan Rume) with real tasting notes, rarity scores, and real named buy sources, plus a real acquisition-priority list and explorer scorecard, all ported unchanged and verbatim. Real content gap found, not fixed: legacy's own "Top 10 Acquisition Priority" list and scorecard table both reference "Laurina" as a 10th entry, but no coffee card for it exists anywhere in the source dataset — ported as-is rather than inventing card content that was never written. Zero client-side state anywhere in this page (only CSS-able hover) — ships entirely as a Server Component. Verified live: 200 OK, typecheck/lint clean.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/brewsoul/cities + /brewsoul/cities/[slug]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">city directory + detail ("City Intelligence Module"). Real 25-city leaderboard (name/state/grade/score/tagline/verdict/live stats), a real 7-dimension scoring methodology, and real national + universal/nuanced chain report cards, all ported unchanged and verbatim into lib/content/brewsoul-cities.ts. Real data-completeness note, not a bug: legacy's own comment admits only Portland has full shop-by-shop data (25 real best + 5 real worst shops with real blurbs/scores/order-this/skip-this) — the other 24 cities have real city-level stats but empty shop/chain/bridge-drink/non-coffee arrays; legacy's own UI already handles this honestly (a real "Full data coming soon" state on both the card and detail page, not fake data) — preserved exactly, verified for both Portland (full tabs) and Seattle (coming-soon state). Grade filter, methodology modal, and chain-toggle interactivity in components/brewsoul/cities-explorer.tsx; per-city tab switching and per-shop expand in components/brewsoul/city-detail-tabs.tsx. Detail route uses generateStaticParams over all 25 real slugs. Scroll-linked parallax and floating-particle backgrounds dropped, same decoration call made throughout this migration. Real image-hosting gap flagged, not silently worked around: the 25 city hero photos are real, live Unsplash URLs (not a dead Manus proxy) but aren't yet uploaded to Sanity per this repo's own image convention — added images.unsplash.com to next.config.ts's remotePatterns as an interim measure rather th</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/brewsoul/directory</t>
-  </si>
-  <si>
-    <t xml:space="preserve">real master page index ("Everything Inside BrewSoul," not a roaster directory — that's /brewsoul/roasters). Real 6 categories with real page descriptions/icons, unchanged; the underlying data already lived in lib/content/brewsoul-directory.ts (built earlier this phase to power CategoryBadge) — this route is where it finally becomes a real browsable page. Category filter extracted into components/brewsoul/directory-explorer.tsx. Fixed the stale "Browse All 103 Coffees" label (real count is 107) by dropping the hardcoded number from the shared data module — benefits every other consumer of that module too. Verified live: 200 OK, typecheck/lint clean.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/brewsoul/guest + /brewsoul/guest/shanita-nicholas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">guest series index + profile ("Tony G Guest Series"). Real single guest entry (Shanita Nicholas — real headline/teaser/tags) on the index, and the real 10-question interview on the detail page (Fair Trade economics, roasting mythology, the C Market, regenerative vs. sustainable, origin-roasting economics vs. Fair Trade, blockchain traceability, pre-harvest financing — real substantive answers with real citations), all ported unchanged and verbatim into components/brewsoul/shanita-interview.tsx. Legacy's guest photo (/api/img/brewsoul-orig_84eb4bc9.jpg) was the same dead Manus proxy confirmed 404 throughout this migration — dropped for a plain initial avatar on both pages rather than a broken headshot. Per-question expand/collapse, "Expand/Collapse All," and the real Twitter/LinkedIn/copy-link share row are genuinely interactive, split into client islands. Verified live: 200 OK on both, typecheck/lint clean.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shared: port BrewSoulLayout, CategoryBadge, JourneyBar, NextSteps as Next.js layout/components</t>
-  </si>
-  <si>
-    <t xml:space="preserve">app/brewsoul/layout.tsx + components/brewsoul/{brewsoul-nav,category-badge,journey-bar,next-steps}.tsx, all built and reused by every /brewsoul/* route above.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kava shared foundation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">app/kava/layout.tsx + components/kava/kava-nav.tsx (KavaNav/KavaFooter, 10 real nav items) + components/kava/kava-ui.tsx (KavaHero/KavaSection/KavaSectionTitle/KavaCard/KavaBadge/KavaDivider/KavaDisclaimer, converted from legacy inline style={} to Tailwind + new --kava-* tokens in globals.css). Added /kava to site-chrome.tsx's SUPPRESSED_PREFIXES (self-contained sub-site, same pattern as BrewSoul and /attention-theft). Real dead link fixed: legacy nav pointed at /pri, which legacy's own App.tsx never routed (only /psychedelic-readiness-index exists) — corrected.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/kava (home)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9 module cards, "Threshold Doctrine," "Sacred Masculine Triad" (Mezcal/Kava/Peyote), 4 market stats, all ported unchanged. Verified live: 200 OK, exactly 1 header/1 footer (chrome suppression confirmed), typecheck/lint clean.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/kava/origins</t>
-  </si>
-  <si>
-    <t xml:space="preserve">real migration timeline (6 Pacific nations, ~3000 BCE–1000 CE), real 6-island selector (Vanuatu/Fiji/Tonga/Samoa/Hawaii/Pohnpei, each with real facts/ceremony/cultivar/safety content), and the real Noble vs. Tudei safety comparison, all ported unchanged and verbatim. Island-selector interactivity in components/kava/origins-explorer.tsx. Verified live: 200 OK, typecheck/lint clean.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/kava/interactions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">real 24-substance drug interaction database (real severity ratings across an 11-value scale, real pharmacological mechanisms, real PRI protocol guidance) and real 5-enzyme CYP450 inhibition profile, ported unchanged and verbatim. Search + severity-filter interactivity in components/kava/interactions-explorer.tsx, using a precomposed SEVERITY_CONFIG class lookup (not string-built classes — same Tailwind static-scanner rule enforced elsewhere this migration). Legacy's unused Download icon import (dead code, no export feature attached to it) not ported. Verified live: 200 OK, typecheck/lint clean.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/kava/science</t>
-  </si>
-  <si>
-    <t xml:space="preserve">real 6 major kavalactones (real receptor mechanisms, real PRI relevance) and real 11-item combined pharmacological profile, ported unchanged into lib/content/kava-science.ts. RSC-boundary bug caught proactively before shipping: initially drafted KAVALACTONES as an export of the "use client" chemotype-decoder.tsx, which would have thrown the same TypeError: X is not iterable already hit once this migration on /brewsoul/decaf when the Server Component page tried to import it — moved to the plain data module before ever running it. Chemotype decoder tool (enter e.g. 4-2-6-5-3-1, see dominant kavalactones) kept as the real interactive client island. Verified live: 200 OK, typecheck/lint clean.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/kava/assessment</t>
-  </si>
-  <si>
-    <t xml:space="preserve">real 5-domain, 20-question PRI readiness assessment (somatic/psychological/relational/cultural/integration), real per-domain point weights, and real 4-band recommendation scoring (CLEARED/CONDITIONAL/DEFER/NOT READY), all ported unchanged into components/kava/assessment-quiz.tsx. Fully stateful (domain navigation, per-question answers, results view), so kept as a single client island per this migration's established pattern for multi-step assessments. Domain and recommendation accent colors (5 + 4 distinct hexes, none matching the --kava-* brand palette) precomposed into literal DOMAIN_STYLES/RECOMMENDATION_STYLES lookup objects rather than style={}, avoiding the dynamic-class bug already caught twice this migration (chains-explorer.tsx, biodynamic/page.tsx). Real backend gap, handled honestly: legacy's AssessmentResultActions took sessionId/serialized-answers props feeding a trpc.assessments.submit mutation this migration never built — used the already-simplified, print-only AssessmentResultActions (components/assessments/result-actions.tsx, built during Phase 9) instead of reproducing a submit call with no backend. Verified live: 200 OK, real domain/question content confirmed in rendered HTML, typecheck/lint clean.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/kava/hawaii</t>
-  </si>
-  <si>
-    <t xml:space="preserve">real ICE/meth crisis statistics (Quest Diagnostics 410% figure, Hawaii DOH conviction rates, law enforcement seizure data), real dual crisis/revival timeline (1985–present), the real (explicitly-labeled hypothesis, not proven) pharmacological alignment table, and real recovery resource listings, all ported unchanged and verbatim. Fully static, no client island needed. Verified live: 200 OK, typecheck/lint clean.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/kava/myths</t>
-  </si>
-  <si>
-    <t xml:space="preserve">real 7-myth evidence review (2002/2014 European kava ban and reversal, WHO findings, CYP2D6 metabolism differences by population, chemotype/preparation distinctions) and the real closing takeaway, ported unchanged. Expand/collapse interactivity in components/kava/myths-explorer.tsx, verdict colors (3-value enum) precomposed into a literal VERDICT_CLASS lookup. Extended shared KavaCard (kava-ui.tsx) with an optional onClick prop to support this — first Kava page needing a clickable card. Verified live: 200 OK, typecheck/lint clean.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/kava/caffeine</t>
-  </si>
-  <si>
-    <t xml:space="preserve">real CYP1A2 inhibition mechanism (56%, the same pathway grapefruit juice uses on medications), real caffeine cutoff protocol, and the real kava-vs-coffee comparison table, ported unchanged. Fully static, no client island needed. Verified live: 200 OK, typecheck/lint clean.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/kava/products</t>
-  </si>
-  <si>
-    <t xml:space="preserve">real 5-category product index (ceremonial powder, fresh frozen, RTD beverages, supplements, kava bars) with real named vendors/cultivars/chemotypes/pricing/PRI ratings and real outbound buy links (all live vendor domains, not Manus proxies — no image assets on this page to check), ported unchanged into components/kava/products-explorer.tsx. Category-tab interactivity kept as the client island. Verified live: 200 OK, typecheck/lint clean.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/kava/certification</t>
-  </si>
-  <si>
-    <t xml:space="preserve">real 12-module, 80-hour facilitator curriculum, real 3-tier certification structure (Practitioner/Threshold Facilitator/Master Facilitator), and real prerequisites list, ported unchanged. Fully static, no client island needed; legacy's wouter cross-links replaced with next/link. Verified live: 200 OK, typecheck/lint clean.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PRI shared data: lib/content/pri-data.ts (copied verbatim from legacy pri/data.ts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">real 39-medicine pharmacopoeia, 50+ questions across 6 domains, MAO-B interaction matrix, medication interaction guide, crisis/integration resources, pathway questions), lib/content/pri-safety-data.ts (verbatim safety data merge source), lib/content/pri-medicine-images.ts (verbatim real CloudFront hero-image map, all spot-checked 200 OK — RampRate's own CDN, already whitelisted, not Manus), lib/content/pri-shared.ts (the real scoring engine — computeScores/READINESS_LEVELS/getMedicineWithSafety — extracted to a plain module per the RSC-boundary lesson from /brewsoul/decaf and /kava/science). Added --pri-* CSS custom properties to globals.css (this subsystem's own purple/parchment/near-black palette, same pattern as --kava-/--crusade-) since Phase 7's PRI section spans 9 more routes.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/psychedelic-readiness-index (core tool)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">the real hero, 39-medicine grid with compare/save/bookmark tooling, MAO-B interaction matrix, medication interaction guide, crisis resources, the real 5-state assessment flow (philosophy intro → readiness quiz → pathway &amp; access questions → legal disclaimer gate → results), medicine detail modal (overview/safety/correction tabs), testimonials, and ImpactSoul cross-promotion, all ported unchanged and verbatim into components/pri/psychedelic-readiness-index.tsx plus supporting client islands (disclaimer-gate.tsx, medicine-modal.tsx, safety-section.tsx, correction-form.tsx, share-bar.tsx, cinematic-band.tsx). Kept as one client island — a single state machine drives which section renders, same call made for other large multi-step assessments this migration. Real hero/section photography (8 CloudFront images) kept via next/image; legacy's purely decorative glitch-scanline overlay divs and CSS shimmer/glow @keyframes dropped (no framer-motion — CONTRIBUTING.md rule 5 — and "decoration not worth the cost," same call made throughout this migration).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PRI: /peyote-mescaline</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MescalineDeepDive, real receptor pharmacology table, the real "Latuda Mirror" same-target-opposite-action comparison, real clinical outcomes (Agin-Liebes et al. 2021, n=452), the real 16-row pharma-to-plant alternatives table, real supplement protocol (pre/day-of/post-integration), real mescaline-specific PRI dimension scores, the real medicine-selector comparison table, and real sources, all ported unchanged and verbatim into lib/content/pri-mescaline-module.ts (copied verbatim) + app/peyote-mescaline/page.tsx. Fully static except the pharma-table expand toggle, extracted into components/pri/pharma-table.tsx; shared PriSection/PriEyebrow wrapper (components/pri/pri-section.tsx) introduced here for reuse by the remaining PRI deep-dive modules. All 8 real section photos (CloudFront) spot-checked live before use; legacy's purely decorative glitch-scanline overlays dropped. Verified live: 200 OK, real content confirmed in rendered HTML, exactly 1 header/1 footer, typecheck/lint clean.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PRI: /iboga-ibogaine</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IbogaDeepDive, "The Plant vs The Isolate": real alkaloid-profile comparison, real receptor pharmacology, real head-to-head iboga-vs-ibogaine table, real clinical outcomes (Mash/Noller/Schenberg/Brown &amp; Alper/Cherian/Williams — including the 2024 Stanford Nature Medicine SOF-veteran data and the 2026 19,071-patient safety analysis), real pharma-to-plant alternatives, real supplement protocol, real dimension thresholds, real medicine selector, Tony's real first-hand account of sitting ibogaine at The Mission Within, real hard-stop contraindications, a real 9-facility directory (with the 2 facilities legacy explicitly removed and why), real Nagoya Protocol / extractive-capitalism argument, real 2026 US legal-status rundown, the embedded Iboga Compass v2 documentation section (components/pri/iboga-compass-section.tsx, its own client island for the question-group toggles), and real sources — all ported unchanged and verbatim into lib/content/pri-iboga-module.ts + lib/content/pri-iboga-compass-data.ts (both copied verbatim) + app/iboga-ibogaine/page.tsx. Fully static except the pharma-table expand toggle (components/pri/iboga-pharma-table.tsx) and the compass section's toggles; reused the shared PriSection/PriEyebrow wrapper from the mescaline module. All 5 real hero/section photos (CloudFront) spot-checked live before use. Verified live: 200 OK, real content confirmed in rendered HTML, exactly 1 header/1 footer, typecheck/lint clean.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PRI: /iboga-compass</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IbogaCompassAssessment, the real interactive 28-question / 7-section compass (outcome/medical/approach/logistics/geography/personal/aftercare), the real drag-or-arrow priority-rank step (top dimension ×2.0, bottom ×0.5), the real facility-scoring engine, and the real results view (matched facilities with real "why this matched" reasoning and real elimination reasons), all ported unchanged and verbatim. lib/content/pri-iboga-compass-engine.ts (real scoring logic — weight deltas, hard filters, substance bonuses, priority-rank application, facility scoring) and lib/content/pri-iboga-facility-data.ts (real facility directory + substance-bonus data) both copied verbatim from legacy rather than hand-transcribed, given this is the actual matching algorithm — correctness matters more here than anywhere else in this migration. Uses this site's own brand-gold/foreground/muted-foreground design tokens rather than the pri-* palette — legacy's own hex here (#8B6914) is an exact match for brand-gold, confirming this one page always used the main site identity, not a PRI-specific one. Real backend gap handled honestly: legacy's lead-capture gate posted a rich structured payload (question-by-question answers, top facility matches, primary goal, budget range) to trpc.assessments.submit (no backend built for this migration) — replaced with a mailto: to Tony carrying the same structured summary, same pattern used throughout this migration; the meaningless "Submitting..." pending state and its e</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PRI: /pri-calibration</t>
-  </si>
-  <si>
-    <t xml:space="preserve">forced-rank calibration study, the real Bradley-Terry pairwise-comparison model (all 15 unique pairs of the 6 PRI dimensions), the real drag-or-arrow full ranking step, real methodology copy (acquiescence-bias explanation, the 4 headline validation stats), and the real Monte Carlo validation metrics (lib/content/pri-efficacy-data.json, copied verbatim from legacy — also feeds /pri-efficacy below), all ported unchanged into components/pri/calibration-assessment.tsx. Real backend gap, handled honestly: legacy's "Contribute to Research?" opt-in phase posted to trpc.priCalibration.submit (no backend built for this migration), and the results view's "Community Data" section read a live trpc.priCalibration.stats aggregate query showing other users' scores — neither has an honest backend-free equivalent (a cross-user aggregate can't be faked locally, and a research opt-in toggle with nothing behind it would be dishonest UI, the same call already made dropping the main PRI results page's inert research-pool checkbox). Both dropped; the flow goes straight from ranking to results. Verified live: 200 OK, real content confirmed in rendered HTML, exactly 1 header/1 footer, typecheck/lint clean.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PRI: /pri-efficacy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">psychometric validation dashboard, the real Monte Carlo simulation results (10,000 synthetic respondents), real classification-accuracy comparison, real dimension-priority distribution (the real first-dimension-inflation finding), real test-retest reliability and entropy metrics, and the real methodology writeup, all ported unchanged into app/pri-efficacy/page.tsx, reading the same lib/content/pri-efficacy-data.json also used by /pri-calibration. Real backend gap, handled honestly: legacy's "Live Calibrations" tab read a live trpc.priCalibration.stats query — since /pri-calibration's own submit call was already dropped (no backend, see that page's port note), this tab would permanently render "0 total calibrations, no data yet," a dead feature masquerading as a live one. Dropped entirely rather than ship a perpetually-empty tab; only the real, fully-populated Simulation view ships — which also means this page has no state left at all, so it's a plain Server Component now instead of a client one. Verified live: 200 OK, real content confirmed in rendered HTML, exactly 1 header/1 footer, typecheck/lint clean.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PRI: /pri-research Built 2026-10-06 behind the login: admins are the emails in ADMIN_EMAILS; everyone else gets live's "Access Denied"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Totals, anonymized opt-in table, admin-only CSV export (/pri-research/export). /pri-calibration regained legacy's "Contribute to Research?" step and now saves every calibration anonymously to pri_calibrations (opt-ins flagged). Was: — Deferred, not skipped (access-model question resolved by inspection). Read the real legacy source: this is a genuine admin-only dashboard (useAuth() gated to role === "admin") showing trpc.priCalibration.researchData — the same calibration-submission backend already confirmed absent and intentionally not built for /pri-calibration and /pri-efficacy (see their port notes). No admin-auth system exists anywhere in this Next.js migration yet either. So this isn't just an access-control decision — even fully wired up, the page would have zero real data to show, forever. Not worth building an admin dashboard against a backend this migration has twice already decided not to build. Added to "Explicitly deferred" below alongside the other admin dashboards; revisit only if/when both a real admin-auth system and a real calibration-submission backend exist.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PRI: /facilitator-index</t>
-  </si>
-  <si>
-    <t xml:space="preserve">"The Facilitator Index: Know Who You Go With," the real 15-question quick-intake archetype quiz (real Bradley-Terry-style axis derivation, fully client-computed via deriveArchetype()), the real 108-item, 12-band (plus Band 0) practitioner self-assessment instrument, and the real methodology prose (rationale, code/tier system, data-handling policy, Reciprocity Gate, Corroboration token system), all ported unchanged and verbatim into lib/content/facilitator-index-data.ts (single authoritative content source) + components/facilitator/* + app/facilitator-index/page.tsx. Real content-drift bug found and fixed: legacy shipped two divergent copies of the same "108 items" — the on-page JSX and a separate printFacilitatorQuestions() print/PDF export using an older, different set of item numbers and band groupings (missing the on-page "Twenty-Five Traditions and Protocols" band entirely) — the print export was never updated when the on-page instrument was revised. Used the on-page version (the one actually shown to visitors) as the single source of truth and rebuilt the print export to generate from that same data, so the two can never diverge again. Real fake-data found and dropped: legacy's PeerStats component's own comment admits its numbers ("163 practitioners mapped so far," etc.) are "seeded, realistic-feeling" — fabricated, not real — dropped entirely, same principle as BrewSoul's stale "reads" counts; UsageCounter's hardcoded 160-practitioner fallback (shown forever since no ba</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Port shared safety/medicine data modules (safety-data.ts, medicine-images.ts) as typed .ts content in the new codebase</t>
-  </si>
-  <si>
-    <t xml:space="preserve">done as part of the main PRI page above (lib/content/pri-safety-data.ts, lib/content/pri-medicine-images.ts, both copied verbatim).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/attention-theft</t>
-  </si>
-  <si>
-    <t xml:space="preserve">consolidated mega-page. Real content ported in full across all 9 sections (hero, The Sacred, The Heresy economics data + full breakdown table + sources, the 10 Weapons, Legal Arsenal w/ filter + letter template, AI Blocker Finder quiz, Report a Spammer, closing vow + related reading) — AttentionTheft.tsx used as the single source, the 5 pre-consolidation sub-pages not resurrected (they never existed in this codebase anyway). Section "glamour" photography is real, live imagery on RampRate's own CloudFront (already whitelisted in next.config.ts as a non-Manus, permanent host — confirmed all 7 URLs 200 before using them), rendered via next/image. Real backend gap found and handled honestly: legacy's Wall of Shame (a live trpc.spam.wallOfShame ranked list) and the Report form's trpc.spam.submit both depended on a spam-tracking backend that this migration explicitly defers (see "Explicitly deferred" list below: "/youve-been-reported, /spamtoast, admin spam tooling") — rather than fake a public database with no real data behind it, the report form now composes a mailto: to Tony (same honest non-fake-success pattern as newsletter-popup.tsx), and the ranked Wall of Shame list isn't reproduced. Two simplifications matching precedent set elsewhere in this migration: legacy's "Fraunces" serif (loaded for this one page only) was dropped for font-heading (Playfair Display, already loaded — same call made on /akbar), and the glitch/VHS/ember-particle/shattered-glass decoration layer was dr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Legacy anchor redirects</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/attention-theft/economics, /blocker-finder, /legal, /weapons, /report → /attention-theft#&lt;anchor&gt; via next.config.ts redirects(). Verified live: all return real 308s to the correct anchor.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Port ManifestoLayout scroll-tracking wrapper behavior</t>
-  </si>
-  <si>
-    <t xml:space="preserve">components/manifesto/manifesto-nav.tsx tracks which section is in view on scroll and highlights the matching nav pill (desktop + mobile), real behavior kept per this line item rather than simplified away.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HumanOS section</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/humanos, /humanos/philosophy, /humanos/ecosystem, /humanos/resources, /humanos/connect, /humanos/path-to-here, ported from _legacy-manus-app/client/src/pages/HumanOS.tsx + humanos/*.tsx. The top-level HumanOS.tsx (an iframe embed of an external manus.space site) turned out to be dead code, never wired into legacy's router — the real, routed implementation is HumanosHome/HumanosPhilosophy/HumanosEcosystem/HumanosResources/HumanosConnect/HumanosPathToHere behind HumanosLayout, which is what got ported, with its own nested layout.tsx (route now added to site-chrome.tsx's SUPPRESSED_PREFIXES so the main SiteHeader/SiteFooter don't double up around HumanOS's own nav/footer). Real content in full: the Maximizer-vs-Satisficer framework and "Boiling the Human"/"Maximizer Trap"/"Conscious Satisficer" philosophy sections, the full ecosystem roster (1 mentor, 8 advisors, 3 partners, 29 clients), all 4 transformation playbooks + 3 daily-practice protocols + 8-book reading list, all 4 connect channels, and the 6-entry "Path to Here" timeline (2010 H+ Summit through 2025). Real bugs fixed: every "Take the Diagnostic" CTA site-wide pointed at /assessment, an 8-question Maximizer/Satisficer quiz that was never actually built anywhere (legacy's real /assessment and /assessments routes are two different, unrelated quiz sets) — redirected to /humanos/philosophy, which delivers the actual promised content; Connect's "Read the Living Declaration" pointed at /manifesto, a dead redirect stub in le</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/find-your-me (+ /find-my-me, /discover)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">"Find My — To Find Your We," the ecosystem hub assessment and by far the largest page in Phase 9. Real 5 NLP-driven questions, 6 dimensions (relationships/purpose/body/truth/tribe/consciousness), and 6 real archetypes (each with a real description, real blog article links, real satellite-site links, real "go deeper" forward-references, and a real share text) ported unchanged and verbatim into a new lib/content/find-your-me.ts data module (kept separate from the component given the file's exceptional size, same pattern as brewsoul-directory.ts). All 17 unique blog article slugs referenced across the 6 archetypes were individually verified live (200 OK) against this migration's real Sanity blog before porting — zero dead article links. Real accuracy fix: legacy's "Full Ecosystem Directory" (26 items across 5 categories, with a real LIVE/COMING pill UI already built for exactly this purpose) marked everything "live," including several routes that don't exist anywhere in this migration yet (/find-my, /the-mirror, /assessments/dharma-finder, /assessments/consciousness-scale, /assessments/grant-study, /flow-circuit) — corrected each item's status to this app's actual current build state rather than shipping false LIVE labels on what would be 404s. Real completeness fix: added Find Your Peptide and Find Your Sexuality to the directory (Body &amp; Temple and Love &amp; Belonging) — both are real, fully-built assessments elsewhere in this migration that didn't exist yet when legacy was writte</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/find-your-therapy (+ /find-my-therapy)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Real 25 questions across 6 dimensions (Cognitive/Somatic/Relational/Depth-Unconscious/Altered States/Integrative), 6 real therapeutic modalities (each with a real description, "how it works," best-for/not-ideal-for lists, real named pioneers, and real book/directory resources), and the real archetype-matching logic (highest-scoring dimension wins) ported unchanged and verbatim. Three real stale-count bugs found and fixed: legacy's own file-header comment claimed "10 questions," its AssessmentIntro stats prop claimed 20 — neither matches the real 25-item array (the scoring code's own maxPossible = 30 // rough max per dimension with 25 questions comment confirms 25 is correct) — replaced both with live QUESTIONS.length. Real dead-link bug fixed: legacy's "Journey Continues" grid linked "Find Your Spirit"/"Find Your Religion" to external findmyassess-9eekxcob.manus.space stub URLs (dead Manus domain) despite this migration already having real, fully-built internal pages at /find-your-spirit and /find-your-religion — repointed to the real internal routes, and corrected Religion's stale "15 Questions" badge to the real 20. Real accent-color inconsistency fixed: legacy passed accentColor="#7B1FA2" only to the landing screen, then hardcoded brand-gold everywhere on the results screen instead — threaded one ACCENT constant through intro/radar/result-actions consistently, matching every other assessment in this migration. The "Also Worth Exploring" related-modality cards were dropped </t>
-  </si>
-  <si>
-    <t xml:space="preserve">/find-your-sake</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Real 20 questions across 5 dimensions (Palate/Ritual/Terroir/Philosophy/Season) and the real 5 sake profiles (each with real Japanese name, tasting notes, food pairings, serving temperature, named producers with region/note, and further-reading resources) ported unchanged and verbatim. Legacy's own AssessmentIntro stats prop claimed "15 questions, 6 dimensions" — didn't match the real 20/5 implementation — replaced with live QUESTIONS.length/DIMENSIONS.length counts, same fix pattern already applied on /find-your-attachment-style and /find-your-sexuality. Two real bugs found and fixed: (1) legacy's "Journey Continues" list read "Find Myzcal" — a literal typo for "Find Your Mezcal" — corrected. (2) legacy's JSX rendered &lt;WhatsNext /&gt; (a full page section) nested inside the small "Retake the Tasting" &lt;button&gt; element — moved to a proper top-level section, same class of nested-interactive-content bug already fixed on /find-your-religion. The dark GlassPanel treatment (near-black translucent cards with light cream text, sitting on the page's own light parchment ThemedBackground) was kept as a real, intentional design choice rather than "fixed" to this migration's usual light-card convention — unlike the light-text-directly-on-light-background contrast bugs found on Style/Sexuality/Peptide/Religion, the text here sits inside its own correctly-contrasted dark card. SacredGeometryBg's canvas-based floating rice-grain particles dropped (same decoration-not-worth-the-JS-cost call made</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/find-your-spirit (+ /find-my-spirit), along with a shared PDF-export component the rest of Phase 9 can reuse</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Real 35 questions, 10 dimensions, and the 6 real spiritual traditions (each with real description/practices/key texts/figures/modern expressions/growth edge) ported unchanged and verbatim — legacy's own file-header comment claimed "12 archetypes," but only 6 TRADITIONS actually exist in the code; ported the real 6, not the stale doc comment. The real weighted tradition-matching logic (top 3 dimensions per tradition, weighted 3/2/1) is unchanged. Ported components/assessments/result-actions.tsx from legacy's AssessmentResultActions — kept only the real, backend-free "Download PDF" action (browser print); the "Send to Tony"/"Keep Private" buttons posted to an unbuilt trpc.assessments.submit and weren't reproduced, same honest-degradation pattern used throughout this migration. Verified live: 200 OK, redirect confirmed 308, typecheck/lint clean.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/find-your-religion</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Real 20 questions across 8 dimensions, 8 real spiritual/philosophical archetypes (each with real description/practices/key texts/figures/resonant traditions/growth-edge tensions), and the real scoring/matching logic ported unchanged and verbatim. Real bug found and fixed: legacy's own JSX rendered &lt;AssessmentResultActions&gt; nested inside the "Retake Assessment" &lt;button&gt; element — a button inside a button, invalid HTML — fixed by rendering it as a sibling instead, same fix pattern already applied on /find-your-spirit. Verified live: 200 OK, typecheck/lint clean.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/find-your-diet (+ /find-my-diet)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Real 15 questions, 6 real archetypes (with descriptions), and the real nearest-neighbor archetype-matching logic ported unchanged. Legacy's dead JourneyTracker import wired in for real (see journey-tracker.tsx). /find-my-diet → /find-your-diet redirect added. Verified live: 200 OK, full quiz flow, redirect confirmed 308, typecheck/lint clean.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/find-your-movement (+ /find-my-movement), along with the shared assessment foundation the rest of Phase 9 depends on</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ported components/assessments/{themed-background,assessment-intro,email-gate,whats-next}.tsx from legacy's ThemedBackground/AssessmentIntro/EmailGate/WhatsNext — real content/behavior unchanged, with 2 real fixes along the way: (1) EmailGate now posts to the real /api/subscribe Route Handler (built earlier this migration) using the exact find-your-&lt;slug&gt; source keys already defined in lib/content/kit-source-tags.ts's KIT_TAG_MAP — legacy's own assessment-gate:&lt;slug&gt; prefix didn't match any tag in that map, so this is a genuine improvement, not just a port. (2) ThemedBackground's per-theme decorative particle field + SVG sacred-geometry overlay + 2 extra radial-glow layers dropped (same "not worth the cost" call made repeatedly elsewhere) — the real per-theme base gradient (16 themes) is kept, precomposed as one literal Tailwind class per theme rather than assembled from fragments. find-your-movement-quiz.tsx ports all 15 real questions and the real 6-dimension (Strength/Flexibility/Endurance/Mindfulness/Community/Adventure) scoring unchanged; the legacy JourneyTracker/useJourneyProgress import in the source file was dead code (imported, never rendered) and not ported. /find-my-movement → /find-your-movement redirect added (next.config.ts), same duplicate-route pattern as /find-my-tribe. Verified live: 200 OK, full quiz flow renders, redirect confirmed 308, typecheck/lint clean.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/find-your-sleep (+ /find-my-sleep)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Real 15 questions, 6 real archetypes, and the real cascading archetype-match logic ported unchanged, including legacy's own real behavioral quirk of rendering JourneyTracker on every phase (not just results). One real duplicate-destination "Journey Continues" link pair dropped (see file's own port note), the one real distinct link (Find Your Diet) kept. /find-my-sleep → /find-your-sleep redirect added. Verified live: 200 OK, redirect confirmed 308, typecheck/lint clean.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/find-your-coffee (+ /find-my-coffee)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Real 15 questions, 6 dimensions (Roast Preference/Origin Curiosity/Brewing Ritual/Social Context/Caffeine Sensitivity/Flavor Complexity), 6 real archetypes (each with a real description and 5 real named coffee recommendations — roaster, origin, roast level, tasting notes, real "why" rationale), and the real archetype-matching logic (sum of each archetype's 2 primary dimensions, highest wins) ported unchanged and verbatim. This legacy page predates the shared ThemedBackground/AssessmentIntro component system the rest of Phase 9 is built on — it hand-rolled its own hero-image page shell — so it needed more normalization than most: its hero image (/api/img/coffee-orig_a935f111.jpg) was a dead Manus asset, dropped for the standard ThemedBackground light theme (added a new "coffee" warm-cream entry) instead of reproducing a broken background; the canvas bean-particle field, floating steam-wisp divs, and SVG sacred-geometry overlay all dropped (same decoration-not-worth-the-JS-cost call made repeatedly elsewhere). Real bug found and fixed: legacy read window.innerWidth directly during render (twice — to pick grid columns and flex direction), unsafe during SSR and a real hydration-mismatch source — replaced with responsive Tailwind classes. EmailGate's prop was legacy's assessmentName; ported using this repo's real assessmentSlug="coffee" to match find-your-coffee in KIT_TAG_MAP. Legacy imported useJourneyProgress for markComplete but never rendered a visible JourneyTracker, and nev</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/find-your-kitchen. Real 15 questions (all rendered on one page at once</t>
-  </si>
-  <si>
-    <t xml:space="preserve">a genuinely different, legacy-intentional UX from the other paginated quizzes, kept as-is) and the real dual-tracking scoring (answer score keys split into archetype tallies vs. 6 separate radar-chart dimensions) ported unchanged, including the 3 real "Journey Continues" links (one to already-built /find-your-diet, one forward-reference to /find-your-style). Verified live: 200 OK, typecheck/lint clean.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/find-your-style. Real 15 questions, 6 real archetypes, and the real (if crude</t>
-  </si>
-  <si>
-    <t xml:space="preserve">legacy's own comment admits "Simple mapping for demonstration") threshold-based archetype match ported unchanged. Two real inconsistencies found and normalized: legacy's own inline styles used near-illegible light text on ThemedBackground's actual light pastel "style" theme (inconsistent with every other assessment in this migration); and legacy rendered &lt;JourneyTracker /&gt; defaulting to variant="dark" on a light results screen instead of the variant="light" every other assessment passes. Verified live: 200 OK, typecheck/lint clean.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/find-your-attachment-style (+ /find-my-attachment-style, /find-my-we)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Real 18 questions (legacy's own AssessmentIntro stats prop under-reported this as "15" — used the live QUESTIONS.length instead of repeating the stale number, same live-count discipline used elsewhere in this migration), the 4 real archetypes, and the real scoring/selection logic all ported unchanged, including the real closing note on attachment theory. Both alt-path redirects added. Verified live: 200 OK, both redirects confirmed 308, typecheck/lint clean.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/find-your-love-language</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Real 15 questions (incl. the negative-score "disconnect" question), 5 real archetypes with descriptions/tips, and Dr. Gary Chapman's real attribution note all ported unchanged. Verified live: 200 OK, full quiz flow, typecheck/lint clean.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/find-your-peptide (+ /find-my-peptide)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">"The Peptide Clarity Index™." A real, evidence-cited 10-question assessment across 7 clinical axes, mapping to 16 real peptide archetype profiles — every question (with its real PubMed/journal citation), every profile's real primary/secondary peptides with mechanisms and evidence, suggested lab work, red flags, and stacking notes ported unchanged and verbatim (clinical-adjacent content, not paraphrased). The real Peptide Readiness Score, contraindication-flag screening, share buttons (Twitter/LinkedIn/email/copy — real, backend-free), and the real medical disclaimer are all preserved. Real hero image (CloudFront, confirmed live) kept via next/image. Reused the simplified AssessmentResultActions (PDF-only) built for /find-your-spirit. Same light-text-on-light-background contrast bug already caught elsewhere was fixed here too. Verified live: 200 OK, redirect confirmed 308, typecheck/lint clean.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/find-your-sexuality (+ /find-my-sexuality)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A research-informed assessment across 6 real dimensions, grounded in real cited research (Klein Sexual Orientation Grid 1978, Kinsey Scale 1948, Lisa Diamond 2008, Sari van Anders 2015) — real 16 questions (with per-question research context notes), real 12 archetypes (each with a real description + research note), and the real scoring/selection logic all ported unchanged and verbatim, including the real closing disclaimer. Legacy's own AssessmentIntro stats prop claimed "20 questions, 7 dimensions" — didn't match the real 16/6 implementation, used the live counts instead. Legacy's results screen also used light grey text on the real light pastel theme background (same low-contrast bug already caught on /find-your-style) — normalized to dark ink. Verified live: 200 OK, redirect confirmed 308, typecheck/lint clean.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/find-my</t>
-  </si>
-  <si>
-    <t xml:space="preserve">"Find What's Yours," the real destination of the homepage's "Diagnose" door (confirmed by grepping lib/content/home-doors.ts's /find-my href) and of whats-next.tsx's "Take Another Assessment" link, both already pointing here as forward-references before this page existed. Legacy's 26-item ALL_LINKS directory (Featured + 6 categories) ported unchanged and verbatim into lib/content/find-my-directory.ts. Real accuracy fix, same pattern as /find-your-me's own port note: cross-checked all 26 destinations against the real route list — /find-your-ev, /life-assessment, and /soulscore (at the time) didn't exist yet, rendered as real "Coming Soon" cards instead of links that would 404 (dharma-finder/consciousness-scale/grant-study have since shipped and now flip to live — see below). Real reuse, not re-derivation: every item whose destination already exists in find-your-me.ts's audited DIRECTORY pulls that entry's real hook text and status at build time via a lookup helper, instead of hand-copying a second, driftable copy of the same facts. Two real live destinations added that legacy linked but find-your-me.ts's directory didn't track: /brewsoul (confirmed 200) and the external findmystem-s3lknc4h.manus.space sibling tool (confirmed live), both using the same "real external sibling product" trust already established for the other manus.space tools. Legacy's dead Manus hero image dropped for ThemedBackground (theme="ecosystem"), same call as /find-your-me. AssessmentProgressBar (never </t>
-  </si>
-  <si>
-    <t xml:space="preserve">/assessments</t>
-  </si>
-  <si>
-    <t xml:space="preserve">"Three Maps. One Journey," confirmed genuinely distinct from /find-my rather than a duplicate: /find-my is the wide 26-item ecosystem directory, /assessments is its own page for exactly 3 long research-grounded instruments (Dharma Finder / Consciousness Scale / Grant Study) that also happen to appear as one category inside /find-my's directory — legacy kept these as two separate pages, so the port does too. Real title/subtitle/description/time/icon/accent content for all 3 instruments ported unchanged and verbatim into lib/content/assessments-hub.ts, including the full "Why These Three" closing essay (Schmachtenberger/Hawkins/Harvard Grant Study triangulation). All 3 instrument cards now link live (dharma-finder/consciousness-scale/grant-study shipped alongside this page). Legacy's footer claim "Results saved for your return" was dropped — replaced with an honest line since nothing persists results yet. Added a real cross-link to /find-my. JourneyTracker reused unchanged; no EmailGate/AssessmentResultActions — pure preview/hub page with no quiz or results step of its own. Verified live: 200 OK, exactly 1 header/footer, real content in all 3 cards, typecheck/lint clean.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/dharma-finder (+ /assessments/dharma-finder redirect). Structurally different from every other Phase 9 quiz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">legacy's real 25 questions are open-text reflection prompts, not multiple choice, distilled from Daniel Schmachtenberger's Dharma Inquiry and grouped into 4 real sections (Capacities/Values/Propensities/The Shadow Inquiry), each with a real framing quote, plus 3 real interstitial quotes shown between sections with the original 4-second auto-advance. All 25 questions, all quotes, and legacy's own keyword-matching generateDharmaProfile (deriving up to 3 archetypal roles and up to 4 core values from free-text answers, plus a completion-depth percentage) are ported unchanged and verbatim into a new dharma-finder-quiz.tsx. Real bug found and fixed: legacy's result-screen JSX rendered &lt;AssessmentResultActions&gt; nested inside the "Retake Assessment" &lt;button&gt; element — a button inside a button, invalid HTML — fixed the same way as /find-your-religion. Real dead-link bug fixed: "Journey Continues" linked to /assessments/consciousness-scale (repointed to the real /consciousness-scale) and /assessments/grant-study (dropped at the time, now live too). EmailGate (new here; legacy had none) is a real ecosystem-consistency addition. find-your-me.ts's ecosystem-directory status flipped from "coming" to "live" now that this page ships. Verified live: 200 OK, typecheck/lint clean.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/consciousness-scale (+ /assessments/consciousness-scale redirect)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Real 25 questions, each scored against David R. Hawkins' real 17-level Map of Consciousness (Shame 20 through Enlightenment 700+, final score = average of all 25 answers) — every question/option, every level's name/emotion/threshold, and getInsight's exact 6 tiers of interpretive copy ported unchanged and verbatim into a new consciousness-scale-quiz.tsx, along with the real live running-average indicator, visual scale gauge, full 17-level map, 6-month reminder, and X/LinkedIn/copy share. Since this assessment produces one composite score on a single axis rather than independent dimensions, a bespoke single-axis gauge replaces AssessmentRadarChart; per-level colors (17 known-at-build-time values) are precomposed literal Tailwind classes rather than assembled from hex fragments. Real Manus-dependency bug found and fixed: legacy's cinematic Q1 hero used a /api/img/consciousness-scale-hero-v2_085e0746.jpg Manus-proxied image — forbidden even temporarily per this migration's Zero-Manus rule — dropped for the plain question-card layout every other assessment uses; a real Sanity-hosted replacement is a tracked follow-up (see BLOG-IMAGE-BRIEFS.md-style tracking). find-your-me.ts's ecosystem-directory status flipped from "coming" to "live" now that this page ships. Verified live: 200 OK, typecheck/lint clean.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/grant-study (+ /assessments/grant-study redirect)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">"Find Your Score," the real 25-question (5 per factor), 5-factor Harvard Grant Study life-satisfaction assessment (724 men, 1938–present, 85+ years — the longest-running study of human happiness). Every question, the 5 real factors (Warm Relationships/Adaptive Coping/Generativity/Career Satisfaction/Physical Vitality), every per-factor/per-tier insight (real named findings — Vaillant's "mature defenses," Erikson's generativity, Waldinger's quote), and the closing "Tony's Note" (Vaillant's "Happiness is love. Full stop." + Waldinger's "good relationships keep us happier and healthier") all ported unchanged and verbatim. Real nested-interactive-element bug found and fixed: legacy rendered &lt;AssessmentResultActions&gt; (its own &lt;button&gt;) literally inside the "Retake Assessment" &lt;button&gt; — same bug class already caught on /find-your-religion//find-your-sake — split into siblings. Real dead-link fix: "Journey Continues" pointed "Find Your Spirit" at a dead external Manus stub despite the real internal /find-your-spirit existing — repointed. Real ecosystem-consistency normalization: unlike every sibling "Find Your X" quiz, legacy skipped EmailGate entirely and went straight to results — added for consistency, plus new find-your-grant-study/find-your-dharma-finder/find-your-consciousness-scale alias keys in kit-source-tags.ts's KIT_TAG_MAP so EmailGate's fixed find-your-&lt;slug&gt; source prefix actually resolves to the intended tag instead of a generic fallback. resultSlug="grant-study" pas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/soulscore</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SoulScore™, ImpactSoul's 12-dimension impact measurement engine (1231-line legacy file, the largest remaining port). Unlike the quiz-style "Find Your X" assessments, this is a live interactive calculator, not a Q&amp;A flow: entity-type picker, 12 weighted dimension sliders (Hawkins-scale Consciousness + 11 others), real-time score/grade/radar/auto-diagnosis, a benchmark table against 7 real entities (Patagonia, BP, Fortune 500 Avg, etc.), a 6-tier/30-factor supply chain drill-down, 20 "why every impact system failed" entries, a real Consciousness-Adjusted NPV calculator, and the gig-economy 5-layer stack comparison — all real content/formulas ported verbatim. Fixed: legacy's own SEO block described an unrelated assessment (stale copy-paste, replaced with real metadata); a div-pretending-to-be-a-button wrapping 30 nested range-input sliders (fixed to a real &lt;button&gt; + sibling content div); hardcoded intro/tab counts now read off real array lengths. No EmailGate (legacy never had one here — it's an open calculator, not a report unlock), matching /find-your-peptide's precedent. AssessmentResultActions wired with resultSlug="soulscore". journey-tracker.tsx's JOURNEY_MAP and /impact-dashboard's "Launch SoulScore Engine"/"Launch C-NPV Calculator" links (previously a disabled "Coming Soon" note) now point at the real page. This closes the real dead-end referenced from site-nav-data.ts (/soulscore appears twice in nav) and from /impact-dashboard — the last item in the STATUS.md dead-end</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/self-portrait</t>
-  </si>
-  <si>
-    <t xml:space="preserve">composite of completed assessments. Decision made: local-only (a real cookie, not Supabase — Phase 2 isn't provisioned yet). AssessmentResultActions (components/assessments/result-actions.tsx) takes an optional resultSlug and logs completions to a tg_assessment_results cookie via lib/assessments/result-log.ts, the same real-cookie-read-via-next/headers pattern already established by returning-visitor-hero.tsx/track-last-blog-visit.tsx — the page itself is a Server Component reading that cookie with zero client hydration step. Real, deliberate scope cut, not a silent one: legacy's SelfPortrait.tsx combined each assessment's own per-dimension scores (16 separate localStorage keys) into one composite radar chart across 15 unified dimensions, gated behind "5+ completed." This migration's result log only ever records that an assessment was completed, not its actual scored answers — building the real composite radar would mean threading a second, much larger data channel through every quiz. Shipped the honest subset instead: a real completed-assessments list (title, real completion date, retake link) plus a real "X of N completed" count and a "Still to Explore" section for the rest, via a new lib/content/self-portrait-catalog.ts. Wired resultSlug into the 7 remaining older "Find Your X" quizzes that already call AssessmentResultActions but hadn't been threaded yet (spirit/therapy/religion/sake/coffee/peptide/me) — /self-portrait now tracks 13 real assessments total. /find-my's "Sel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/the-mirror (+ /life-assessment)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">uses mirrorData.json, real 6-dimension/18-question life assessment ("The Mirror") ported into a typed lib/content/mirror-data.ts. Legacy served the identical component at both paths; /the-mirror is canonical (it's the only URL every existing internal link already pointed to — nav, journey tracker, Find Your Me), /life-assessment permanently redirects there. Real dimension-averaged scoring, radar chart via the shared AssessmentRadarChart, and weakest-dimension article/satellite-site recommendations ported unchanged. A live Sanity check found only 27 of 85 legacy article slugs still resolve; recommendations now resolve server-side and defensively skip missing ones, matching legacy's own behavior. Fixed: a hydration-unsafe typeof window branch computing the share URL, three stale manus.space satellite URLs superseded by their current live counterparts already used elsewhere in this migration, and dead /assessments/*/external-stub links in the "Journey Continues" grid. Added find-your-mirror to kit-source-tags.ts's KIT_TAG_MAP and reconciled journey-tracker.tsx's stale 10-minute estimate to legacy's real "~4 minutes" claim. find-your-me.ts's ecosystem-directory status flipped to "live." Verified live: 200 OK on both paths, redirect confirmed, typecheck/lint clean.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/assessment</t>
-  </si>
-  <si>
-    <t xml:space="preserve">confirmed via full legacy read this is not a "Find Your X" quiz (it predates that convention): it's Tony's own 3-way reader-path diagnostic — Builder / Crusader / Investor — 5 real questions, one point per matching answer, highest tally wins. Real questions and real archetype copy ported unchanged, reused from lib/content/archetypes.ts (already ported for /essays's archetype filter) rather than duplicated — added the page's ASSESSMENT_QUESTIONS to that same module since both come from the identical legacy source file. Preserved the real, distinct UX (no landing screen, no ThemedBackground/JourneyTracker — this page sits outside that ecosystem). Real bugs fixed: JS onMouseEnter/onMouseLeave inline-style hover hack replaced with Tailwind hover: classes; literal "..." pending-state text replaced with a real Loader2 spinner per house rule; dead trpc.subscribe.add replaced with a real POST /api/subscribe call. Real link audit: kept /impact-dashboard, /find-your-me, /living-declaration, and the real /blog/boiling-the-human-summit-harvard-kurzweil article as live links; /soulscore and /humanos are established forward-references used repeatedly elsewhere in this migration and both now ship too. The Human OS CTA reuses the border-red-800/30 text-red-800 treatment /living-declaration already established for the identical button instead of a new one-off raw-hex pair. AssessmentResultActions resultSlug="assessment" added (didn't exist when legacy was written). Added assessment-builder/as</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fix dead-end pages flagged in STATUS.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sake, therapy, and love-language all got real next-step navigation (WhatsNext + real "Journey Continues" links) during their ports — the last remaining one, soulscore, is now built (see above), closing this out.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Port shared radar-chart / PDF-export / email-gate components used across assessments</t>
-  </si>
-  <si>
-    <t xml:space="preserve">components/assessments/{radar-chart,result-actions,email-gate}.tsx, built during Phase 9 and reused unchanged by all 15 "Find Your X" quizzes plus /find-your-me.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">src/lib/admin/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">guardrails (fixes the removed version's proxy.ts pattern, which missed the real src/proxy.ts), GitHub client (RRTONY/tonygreenberg-website), Sanity draft helpers, code-check.ts (ESLint + CONTRIBUTING.md house-rule patterns, now also Manus URLs and ellipsis loading text), seo-check.ts, tools.ts, mcp-server.ts, mcp-handler.ts, mcp-tool-context.ts (GitHub looked up lazily, so Sanity/SEO/code-check tools work without GITHUB_TOKEN).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Per-person access via MCP_ADMIN_USERS (read/edit/write roles, tools filtered per role, calls logged, commits stamped [by &lt;name&gt;])</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mcp-auth.ts.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rules gate: get_project_rules serves CONTRIBUTING.md + AGENTS.md + docs/ai/ guides with a rulesVersion; all 6 write tools require it</t>
-  </si>
-  <si>
-    <t xml:space="preserve">project-rules.ts.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">src/app/api/mcp/route.ts (header auth) + src/app/api/mcp/[token]/route.ts (token in URL).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">docs/ai/ knowledge base (README, TASK_GUIDE, PROJECT_STRUCTURE, project_mcp_server), linked from CONTRIBUTING.md.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">@modelcontextprotocol/sdk ^1.30.0 re-added (approved 2026-09-29); GITHUB_TOKEN/MCP_ADMIN_USERS/MCP_SITE_ORIGIN documented in .env.local.example.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verified locally</t>
-  </si>
-  <si>
-    <t xml:space="preserve">auth (401/405), role filtering, rules-gate markers, token-in-URL route, code check, Sanity query, SEO check.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sign-in for the MCP server (OAuth 2.1, ported from ramprate-ui, 2026-09-30)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/oauth/authorize sign-in page + /.well-known metadata + register/authorize/token endpoints, stateless (signed tokens, no database), no new dependency. Verified end to end on a local production build. See docs/ai/project_mcp_server.md.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Set GITHUB_TOKEN, MCP_ADMIN_USERS, MCP_LOGIN_PASSWORD, MCP_OAUTH_SECRET, MCP_SITE_ORIGIN, MCP_PUBLIC_ORIGIN in Netlify (done) (checked 2026-…</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10-07: all already set in Netlify). Left: connect Claude.ai to /api/mcp for real, and verify the GitHub flow end to end (branch → PR → deploy preview → publish_changes) against a real PR.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Commit a team-wide .mcp.json (URL only) once the production URL is settled.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Google read-only tools added (2026-10-02)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">check_analytics (GA4), search_console_sites / _performance / _inspect_url / _sitemaps (list only, no submit or delete), lighthouse_check_page (PageSpeed Insights). New files google-auth.ts, ga4-client.ts, gsc-client.ts, lighthouse-check.ts; no new dependency. Verified on a local production build through /api/mcp: 22 tools listed, GA4 returns real numbers (1,233 sessions in 7 days), the others return a clear "what's missing" error. Env vars added to .env.local.example.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">publish_changes fixed (2026-10-02)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">it published every draft in Sanity (31 waiting for review today), so any one-line fix would have pushed them all live. Now it publishes only the drafts named in draft_ids; unknown ids are refused before anything happens (verified).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">seo_check_page decoded &amp;#39; but not React's &amp;#x27;, so descriptions showed Tony Greenberg&amp;#x27;s and the length was off</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fixed and verified (2026-10-02).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Search Console access for the service account added by the team (2026-10-02); all four search_console_* tools verified with real tonygreenbe…</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rg.com data (99 clicks / 1,663 impressions in 28 days, homepage indexed, sitemap 284 URLs, 0 errors, 82 warnings).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GOOGLE_GA_CLIENT_EMAIL, GOOGLE_GA_PRIVATE_KEY, GA4_PROPERTY_ID_TONYGREENBERG set in Netlify (2026-10-02, via the Netlify API, values checked…</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> equal to .env.local; this plan can't limit a variable's scopes, so they're available to builds and functions). Used from the next deploy.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Per-request change system ported from ramprate-ui (2026-10-02, owner said yes)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">, covering the 10 review points the team raised for RampRate's setup: (1) discard_change; (2) one request = one change with its own branch, PR and drafts, so publishing never takes another request live; (3) a review with pages affected, a server-written "what's included" line and preview links; (4) publish needs the review's reviewToken, and the rules make the AI ask "You are about to publish these changes to the live tonygreenberg.com website. Are you sure you want to continue?"; (5) list_change_history, also visible read-only in Studio under "Website change history" (new adminChange type); (6) undo_change; (7) before/after (automatic for Sanity, given by the AI for code); (8) preview_on_devices phone + laptop screenshots (needs GOOGLE_API_KEY); (9) the AI's plain summary plus the server's facts line; (10) Draft → Ready for review → Published / Discarded. Files: change-sets.ts, change-describe.ts, device-preview.ts, mcp-tool-context.ts, mcp-server.ts, github-client.ts (RampRate's full version), src/sanity/schemas/adminChange.ts, sanity.config.ts. Tested end to end with a real throwaway change, then discarded (see docs/ai/project_mcp_server.md).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Merge the CI fix into main</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(done with PR #3; checked 2026-10-06: main's pr-lint.yml runs Node 22 and next typegen before the type check). The test change's GitHub check failed because main still has the old pr-lint.yml (Node 20 crash). Every MCP change will fail its site check, and so can't be published, until this branch's work (or at least .github/workflows/pr-lint.yml) is on main. Then test a real publish and undo_change.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Blocked on you (Google)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">create a GOOGLE_API_KEY in Google Cloud (project of the vcos-ga4-reader service account, where the PageSpeed Insights API is already on), restricted to the PageSpeed Insights API, then add it to .env.local and Netlify. Creating it from here was blocked by the session's safety check (it would use the service account's credentials to change the Cloud project). Note lighthouse_check_page may time out on Netlify (10 s function limit on the free plan).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Per-page generateMetadata (title, description, OG, Twitter Card, canonical) for every ported route, sourced from Sanity seo object where con…</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tent is CMS-backed, static otherwise. Audited all 140 page.tsx files: only /studio has none (correct — it's robots.txt-disallowed, not public content). Real gap found and fixed: /blog/category/[slug] had no alternates.canonical at all, and no page-aware title for its own real pagination (?page=N) — every paginated page was serving an identical title with no canonical, a real duplicate-content signal. Fixed: generateMetadata now reads searchParams too, self-canonicals each page (?page=N pages canonical to themselves, not consolidated to page 1 — genuinely different posts per page, matching Google's current pagination guidance) and appends "— Page N" to the title past page 1. Verified live: page 1 canonicals to the bare URL, ?page=2 canonicals to ?page=2 with a distinct title.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sitemap.ts generated from real Sanity content + static route list, auto-updates on publish</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Extended from the Phase 5-era version (homepage + blog posts only, 122 URLs) to every real route: the full static route list (130 routes, generated from find src/app -name page.tsx, excluding /studio (robots.txt-disallowed), /(auth)/login (noindex via its own metadata), and /life-assessment (a pure redirect, not distinct content)) plus all 5 real dynamic sources — blog categories (allCategorySlugsQuery), BrewSoul cities (25), BrewSoul coffees (107), and charity-scorecard entries (103) — each pulled from the exact same data source its own page's generateStaticParams already uses, not re-derived. Auto-updates on publish for anything Sanity-backed (blog posts/categories) since it's a live client.fetch on every build; the static route list itself needs a one-line addition whenever a new page ships (same as any other route-registration step). Verified live: 496 real &lt;loc&gt; entries, spot-checked a coffee/city/charity/category URL each, typecheck/lint clean.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">llms.txt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fetched verbatim from the still-live site and saved to web/public/llms.txt (real content: Tony's bio, expertise, full article index by category, every product/tool section) — do this before Manus goes away, it won't be recoverable after</t>
-  </si>
-  <si>
-    <t xml:space="preserve">robots.txt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">same approach: fetched the real live file (not my earlier guessed robots.ts, which has been removed) and saved verbatim to web/public/robots.txt, plus added Disallow: /studio for the new Sanity Studio route. Confirmed live: real AI-crawler allowlist (GPTBot, Claude-Web, PerplexityBot, etc.), scraper blocklist, and the site's non-standard LLMs: directive all intact</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JSON-LD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WebSite + Person schema ported verbatim from the live homepage's actual &lt;script type="application/ld+json"&gt; tags (not reconstructed from memory) — rendered site-wide from src/lib/structured-data.ts in the root layout. The Person image was hardcoded to a /api/img/... legacy proxy path on the live site — rescued that headshot (downloaded it while still live, uploaded to Sanity as the author-tony-greenberg document's avatar) so the new site's JSON-LD has zero Manus dependency instead of just copying the fragile path forward</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Article JSON-LD on /blog/[slug], built from real per-post Sanity data (headline, image, datePublished/dateModified, author, canonical URL)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">verified live on a real post</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/path/:archetype (src/app/path/[archetype]/page.tsx)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">per-archetype landing page for /assessment's Builder/Crusader/Investor result, reusing lib/content/archetypes.ts. Real content ported in full (top-5 essential-reading list per archetype via allPostsForArchiveQuery, real PathSubscribeForm posting to /api/subscribe, AUTHORITY_ITEMS strip). Real bug fixed vs. legacy: replaced a hand-rolled inline-styled "Path not found" div with a real notFound() (this route's generateStaticParams only ever produces the 3 real keys). Verified live: all 3 archetype routes 200 OK, typecheck/lint clean.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/my-journey (src/app/my-journey/page.tsx + components/assessments/my-journey-dashboard.tsx)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">"My Journey Dashboard," real grid/timeline views across all 28 JOURNEY_MAP experiences, category/status filters, phase progress ring, recommended-next card, using the same real useJourneyProgress/JOURNEY_MAP completion tracking every "Find Your X" quiz already writes to (not the narrower tg_assessment_results cookie built for /self-portrait). Legacy's per-quiz scored-result caching (RESULT_KEYS, feeding a mini radar chart) was not ported — no quiz in this migration writes that data either, same honest-degradation call already made for /self-portrait's own composite radar. Fixed a real legacy dead link (/ecosystem-map, a still-unbuilt page) to /self-portrait. Verified live: 200 OK, real content confirmed, typecheck/lint clean.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/the-open-door (src/app/the-open-door/page.tsx)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">real press/credibility content: all 10 "Magic Genie" client-pitch prompts (real named targets — Marco Argenti/Goldman Sachs, Adam Smith/Disney, etc.), 18 real client testimonials, all 8 explicitly-labeled satirical "parody" quotes (kept with disclaimers, not presented as real). Real overlap found and reconciled: this page's publications/speaking/podcasts arrays substantially duplicate the already-shipped /published's fuller bibliography — kept only what /published doesn't cover (Forbes + Business Insider bylines, the Clinton Global Initiative keynote, 4 of 5 podcast appearances) and cross-linked to /published for the rest, same reconciliation pattern as /assessments vs /find-my. Real bugs fixed: 3 genie/keynote links pointed externally at tonygreenberg.com/&lt;slug&gt; for posts that are real internal posts in this migration — relinked to /blog/psychedelics-could-become-extractive-capitalism, /blog/boiling-the-human-summit-harvard-kurzweil, /blog/return-on-investment-going-green-going-green-2 (all verified 200); a bare self-link to tonygreenberg.com remapped to /. Ships as a pure Server Component (legacy's FadeIn/Section/editorial-component dependencies don't exist here and weren't needed). Verified live: 200 OK, real content in raw SSR HTML, typecheck/lint clean.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Homepage "Recent Updates" band (2026-09-29)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">on the live site (a newer Blog.tsx than _legacy-manus-app/, so rebuilt from the live page's markup), replacing the older "Latest Thinking" pair. Found while doing it: two live essays are missing from Sanity, the-tollbooth-and-the-alternative (Aug 18, 2026, the live site's newest) and what-quest-could-fix. Both were published on live after the legacy snapshot and need importing.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Re-sync the legacy reference</t>
-  </si>
-  <si>
-    <t xml:space="preserve">_legacy-manus-app/ is older than what's live (Recent Updates proves it), so visual diffs should be against the live site, not only that folder.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Visual diff pass: every ported page vs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">legacy page</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Padding / spacing on the story pages matched to live (2026-10-01)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Measured margins, text column and spacing on 31 pages, live vs a production build, at 375px and 1280px. The "door" story pages were the clear mismatch: live's text column is ~546px (ours was 720px), 20px side margins on phones / 40px on desktop, body text 19px/1.8 on phones and 18px/1.85 on desktop (ours 16px/1.5). Fixed on /the-body, /engine-room, /under-nda, /the-nightstand, /the-web, /the-territory, /about, /intel (Intel uses live's 16.8px/1.9; About's hero line 480px max, 18.4px/1.8). Re-measured: all 8 match live to within 2px (About's column 28px narrower), no sideways scroll at 375px.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Header-to-title spacing re-checked (2026-10-02)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The 2026-10-01 note compared different things: live's header wasn't measured (it showed 0), so "96px vs 168px" was really 161px vs 168px from the top of the page. Measured again from the top of the page, live vs a production build, at 375px and 1280px: most pages were already within 10px. Fixed the real gaps: /the-open-door (now live's dark centered hero band, 56px title, 546px text column; title was 72px too high), /start-here (live's 48px/96px top padding; 25px too high on desktop), /invest and /engage (label spacing and live's 32px/51px title; /invest's desktop title was 36px), /impact-dashboard on phones (card edge to edge under the header like live; title was 89px too low). Re-measured: all within 8px of live, no sideways scroll at 375px, no JS errors.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HumanOS headings in capitals like live (2026-10-02, owner said yes)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">the 4 headings live capitalises on /humanos (title, "Are you a Maximizer...", "Take the Diagnostic", "The Diagnostic") get uppercase; the words are unchanged. The subpages already matched.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">More layout gaps matched to live (2026-10-02)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/series (live's centered 546px column, and a bug fixed: every card kept an empty 240px picture column, squeezing the text; live's per-series picture is one generic placeholder on the Manus proxy, so not copied), /humanos (middle section 900px like live), homepage desktop widths (hero text 804px, Four Doors 1000px, Editor's Picks 1168px, GemSpark edge, section title sizes; live's /blog now shows the homepage), /find-my (photo undimmed and plain background, like live; our site header kept). Re-measured: headings within 3px (/series) to 20px (homepage) of live, no sideways scroll, no JS errors. Note: live's "New here?" tour bar sits over its header and doesn't move the page, so it doesn't affect these numbers.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Full sweep vs live (2026-10-02)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">142 pages (every non-blog page, 3 of each templated set) at 375px and 1280px, title position, text column, title size. Fixed the shared causes: BrewSoul (live wraps most pages in its frame twice, so a second 52px offset plus the category badge; the landing, cities, directory and quiz pages have neither: src/components/brewsoul/brewsoul-main.tsx; intro paragraphs uncapped like live; 38px titles), Kava (live's extra 52px offset), /the-body, /the-nightstand, /the-web (405px top photo like live), the 6 peptide pages (live's 768/896px intro column), /journeys, /pick-up-the-phone, /published, /ecosystem (546px story column and live's text size). Re-measured: 110 of 120 within 40px / 60px of live.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sweep leftovers fixed (2026-10-06)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ported legacy's exact title sizes, margins and column widths. Measured live vs a production build at 375px and 1280px (H1 distance from the top, H1 size, intro and table widths). Now within 8px and the same title size on /published, /brewsoul/first-sip, /brewsoul/home, /brewsoul/chains (intro 912px like live), /brewsoul/browse, /brewsoul/directory (3-column 952px grid like live), /brewsoul and /brewsoul/quiz (intro 520px), /amplifier (546px column), /diamond-cut, /speaking, /living-declaration, /spirits, /protecting-your-business (tables 730px), and the 5 HumanOS subpages (titles smaller like live, 752px column). No sideways scroll at 375px. Left on purpose: /self-portrait (font matches; our page has a different title and no back link, so it sits 23-57px higher), BrewSoul pages 3-6px off (the shared journey bar row), and the different-layout pages /dharma-finder, /grant-study, /search, /quiz_25q, /soulscore. Also: /brewsoul/quiz rebuilt as a step registry (src/components/brewsoul/brewsoul-quiz/: parent + hook/ + components/step-* + data/), same questions, scoring and look; Back/Skip/Retake use lucide icons. New CONTRIBUTING rule 19 (multi-step flows, FydoPartner pattern). brewsoul-welcome-quiz.tsx (/brewsoul) still has the old shape and text arrows.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Match live's redesigned pages (2026-10-06, owner said go)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/self-portrait (live: dark page, progress ring, "N more brushstrokes" lock until 5 assessments), /grant-study and /dharma-finder (live opens straight on question 1, no intro screen), /quiz_25q (live adds a hero picture above the title; rescue it into Sanity first), /search (live: one search box across essays, BrewSoul, peptides, HumanOS, assessments, kava and pages with filter chips). Measure live vs a production build at 375px and 1280px when done. Done 2026-10-06: /grant-study and /dharma-finder open straight on question 1 like live (title block / part header above the first question, live's 546px column, plain page, credit under every question), both rebuilt as step registries (rule 19); measured within 3px of live at the top (dharma's question block within 7px). /quiz_25q's hero rescued into Sanity and placed like live (within 2px). Found and fixed on the way: on the deployed copy /grant-study's answer buttons could not be clicked (the themed page background was fixed z-0, painted over the quiz); ThemedBackground is now -z-10 pointer-events-none (backgrounds unchanged on all 21 pages that use it), and the shared email gate no longer scrolls sideways on phones. Both quizzes clicked through to results in Chrome and Safari. /self-portrait restyled to live (dark page, "The Composite You", progress ring, "N More Brushstrokes Needed" lock until 5 done, live's copy) on our real cookie data; within 3px of live at both widths; tested with 0, 2 and 6 completed. Counts are ours (13 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Still different from live (needs a yes)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">blog posts (done) (done 2026-10-07, see Phase 5); /find-my on live hides the site header. /walk-through is a 404 on live now.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Design change on live, needs a decision</t>
-  </si>
-  <si>
-    <t xml:space="preserve">live's story pages now use Cormorant Garamond for titles (ours: Playfair Display), a lighter title weight (400 vs our 700), and a red eyebrow label (#8E1E25, wider letter spacing) instead of our gold. A site-wide font swap is a design call, so not done.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Link check across all ported pages (no 404s, no broken internal cross-references)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">First full pass done 2026-09-29 (510 pages crawled from the sitemap plus every internal link, on a production build). Fixed in code: /brewsoul/coffee/…-tarrazú 404 (the route got the id still percent-encoded), 30+ links that went through the /assessments/* redirects, /find-your-me's dead Homeaglow link, the two root-level Iboga essay links, and the dead FauxTony nav item. Fixed as Sanity drafts (scripts/fix-blog-body-links.ts, 14 posts): broken post links, leaked !… placeholder text, Energy Is Money's split author bio, and scraped WordPress furniture ("Share this / Related / You Might Also Like / Copyright", "Show More / Top News", [mc4wp_form]). Left for a decision: /framework's "Ask FauxTony" button, when-healing-becomes-extraction's two links to a Dr. Lee case file that doesn't exist, and the-clock-keeper-chronicles-part-1's link to the deferred /clock-keeper-part-2. Re-run after the drafts are published. 2026-10-01 re-run (local production build, all 498 sitemap URLs load; 440 unique internal links): 5 broken. Fixed as a Sanity draft: molecule-as-mirror-10-what-the-pioneers-know's "Final installment" link pointed at a non-existent part-10 slug (now part 11; live also shows that line twice, kept). Already fixed in a waiting draft: forever-chemicals-... → /blog/psychedelic-readiness-index. Still the 3 known decisions: /fauxtony (from /framework), /clock-keeper-part-2, /blog/the-case-file-dr-samuel-lee.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lighthouse pass (performance/accessibility/SEO) on top 20 pages by traffic 2026-09-30, 20 key pages (no traffic data yet), local production …</t>
-  </si>
-  <si>
-    <t xml:space="preserve">build, mobile: averages performance 87, accessibility 99→100, best practices 100, SEO 92→100, CLS 0 everywhere. Fixed: public/robots.txt had an LLMs: line (not a real directive) that made Google treat the whole file as invalid, now a comment; h3/h4 headings skipping a level on /assessments, /kava, /peptide-watch (same look, right tag); the Kava and /attention-theft back-arrow links had no accessible name on phones; two small phone-width contrast misses. Left: performance is local-machine only (±10-15 points, see CONTRIBUTING.md); the slowest were / 76 (LCP 5.2 s), /psychedelic-readiness-index 82, /iboga-ibogaine 83. Re-run against the Netlify deploy before launch. 2026-10-06 re-run against the Netlify deploy (14 key pages, mobile): accessibility 100 and CLS 0 on every page, SEO clean (only the expected netlify.app noindex), performance 77-97 held back by 3-4 s LCP. Fixed: all 21 hero images moved off the deprecated priority prop to fetchPriority="high" + loading="eager" (Next 16); /iboga-ibogaine hero and the first card on /blog and category pages no longer lazy-loaded; sizes on the Four Doors cards (~150 KiB per page), /humanos diagram (~100 KiB) and /about headshot; urlFor no longer imports the Sanity client, so ~115 KB of Sanity client code stopped loading on / and /blog; React hydration error #418 on / and /blog (post dates) gone, checked in two time zones; /blog is static again; empty icon &lt;th&gt;s on /iboga-ibogaine labelled; category page reads use sanityFetch(). Left: se</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SEO audit fixes (2026-10-06)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Checked an outside audit point by point against the code. Fixed: Core Themes cards linked to /?theme=…#essays-archive (not crawlable, counts from a stale hand-kept list) and now link to /blog/category/&lt;slug&gt; with real counts (21/25/20/14, matching the archive pills; THEME_MAP and the ?theme= filter removed); Four Doors cards were &lt;button&gt;s, now real links that still open the modal on a plain click; "DIAGNOSE · ENGAGE" now link to /find-my and /engage; one shared formatPostDate (Asia/Kolkata, src/lib/format-post-date.ts) so a post no longer shows two different dates; the title repeated as the first body paragraph is dropped at render time (legacyBodyLayout); essay cards are h3 under a section h2 (archive, Read next), h2 only on category/search; heading glyphs (◆ ✦) hidden from screen readers; posts send BlogPosting with the author tied to the site Person (@id) plus a BreadcrumbList; descriptive alt on the homepage and BrewSoul heroes; homepage OG image cropped to 1200x630 JPEG. Already fine (audit could not see it): Person/Article schema, Netlify noindex, robots.txt, sitemap, header nav and search, Amazon links carry no affiliate tag. Checked on a production build: type check, lint, build, status codes, browser click test at 375px, no console errors. Implementation pack (Mohammad Danish, 2026-10-05) checked the same day: added og:type/og:site_name back on the 6 pages with their own openGraph (a page-level openGraph replaces the layout one), twitter:creator, and on posts og:url</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SEO audit items needing a yes (2026-10-06)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">the pack's new copy (homepage title/description, five-cups title, description, short answer, FAQ, heading rewrites, entity statement, newsletter block, author box, health disclaimer, COA wording); "Further Reading" shown twice on posts (merge the lists?); long post title (84 chars), homepage description length and obsolete keywords tag, slugs (/blog/five-cups, the -2 slug; would need redirects), "Six lenses" over four cards, sources for health claims and proof for "$10B+", "Certified B Corp", "Validity: 91", legal review of the homepage Case File banner, ABIT waitlist disclosures, one contact email, the two one-post categories, fewer homepage CTAs / email signup / table of contents / explaining "COA".</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Connect Google Search Console + GA4 to the new deployment on day one of cutover</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Restore/adapt the manus.space triple-layer noindex lockdown pattern for any remaining staging URLs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-01: the Netlify copy (tonygreenberg-website.netlify.app) and every deploy preview had no noindex at all, so Google could index a duplicate of the site. next.config.ts headers() now sends X-Robots-Tag: noindex, nofollow on any *.netlify.app host only; tonygreenberg.com is unaffected, so nothing to remove at cutover. Tested with Host headers on a production build.</t>
+    <t xml:space="preserve">Live's redesign, second group (started 2026-10-07, cut off by the usage limit)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/living-declaration is done (dark bands, Cormorant title; all of live's text checked present). Still to match live: /the-web, /spirits, /iboga-ibogaine (title weight 800), /find-your-journey (64px title, red label), /impact-dashboard (64px title), red labels on /published and /speaking, label colours on /recent-creations and /soulscore, /pri-calibration (title weight 900), /quiz_25q; /pri-efficacy's "Simulation / Live Calibrations" switch (counts from the pri_calibrations table); live's BrewSoul photo (already in Sanity: 1c8cf85c…-1200x670.webp) on the BrewSoul hero, first-sip, guest and browse pages; the page re-check of /clients, /humanos/connect, /peptide-hall-of-shame (its hero is rescued, not wired) and the blend-builder / biodynamic pages.</t>
   </si>
   <si>
     <t xml:space="preserve">Manus media rescue (2026-09-29)</t>
@@ -2494,15 +2500,15 @@
         <v>8</v>
       </c>
       <c r="B5" s="5" t="n">
-        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$317,$A5,'Full Detail'!$C$2:$C$317,"Done")</f>
+        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$318,$A5,'Full Detail'!$C$2:$C$318,"Done")</f>
         <v>12</v>
       </c>
       <c r="C5" s="5" t="n">
-        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$317,$A5,'Full Detail'!$C$2:$C$317,"Remaining")</f>
+        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$318,$A5,'Full Detail'!$C$2:$C$318,"Remaining")</f>
         <v>0</v>
       </c>
       <c r="D5" s="5" t="n">
-        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$317,$A5,'Full Detail'!$C$2:$C$317,"Deferred")</f>
+        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$318,$A5,'Full Detail'!$C$2:$C$318,"Deferred")</f>
         <v>0</v>
       </c>
       <c r="E5" s="5" t="n">
@@ -2519,15 +2525,15 @@
         <v>9</v>
       </c>
       <c r="B6" s="5" t="n">
-        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$317,$A6,'Full Detail'!$C$2:$C$317,"Done")</f>
+        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$318,$A6,'Full Detail'!$C$2:$C$318,"Done")</f>
         <v>16</v>
       </c>
       <c r="C6" s="5" t="n">
-        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$317,$A6,'Full Detail'!$C$2:$C$317,"Remaining")</f>
+        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$318,$A6,'Full Detail'!$C$2:$C$318,"Remaining")</f>
         <v>0</v>
       </c>
       <c r="D6" s="5" t="n">
-        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$317,$A6,'Full Detail'!$C$2:$C$317,"Deferred")</f>
+        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$318,$A6,'Full Detail'!$C$2:$C$318,"Deferred")</f>
         <v>0</v>
       </c>
       <c r="E6" s="5" t="n">
@@ -2544,15 +2550,15 @@
         <v>10</v>
       </c>
       <c r="B7" s="5" t="n">
-        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$317,$A7,'Full Detail'!$C$2:$C$317,"Done")</f>
+        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$318,$A7,'Full Detail'!$C$2:$C$318,"Done")</f>
         <v>8</v>
       </c>
       <c r="C7" s="5" t="n">
-        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$317,$A7,'Full Detail'!$C$2:$C$317,"Remaining")</f>
+        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$318,$A7,'Full Detail'!$C$2:$C$318,"Remaining")</f>
         <v>2</v>
       </c>
       <c r="D7" s="5" t="n">
-        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$317,$A7,'Full Detail'!$C$2:$C$317,"Deferred")</f>
+        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$318,$A7,'Full Detail'!$C$2:$C$318,"Deferred")</f>
         <v>0</v>
       </c>
       <c r="E7" s="5" t="n">
@@ -2569,15 +2575,15 @@
         <v>11</v>
       </c>
       <c r="B8" s="5" t="n">
-        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$317,$A8,'Full Detail'!$C$2:$C$317,"Done")</f>
+        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$318,$A8,'Full Detail'!$C$2:$C$318,"Done")</f>
         <v>14</v>
       </c>
       <c r="C8" s="5" t="n">
-        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$317,$A8,'Full Detail'!$C$2:$C$317,"Remaining")</f>
+        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$318,$A8,'Full Detail'!$C$2:$C$318,"Remaining")</f>
         <v>0</v>
       </c>
       <c r="D8" s="5" t="n">
-        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$317,$A8,'Full Detail'!$C$2:$C$317,"Deferred")</f>
+        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$318,$A8,'Full Detail'!$C$2:$C$318,"Deferred")</f>
         <v>0</v>
       </c>
       <c r="E8" s="5" t="n">
@@ -2594,15 +2600,15 @@
         <v>12</v>
       </c>
       <c r="B9" s="5" t="n">
-        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$317,$A9,'Full Detail'!$C$2:$C$317,"Done")</f>
+        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$318,$A9,'Full Detail'!$C$2:$C$318,"Done")</f>
         <v>63</v>
       </c>
       <c r="C9" s="5" t="n">
-        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$317,$A9,'Full Detail'!$C$2:$C$317,"Remaining")</f>
+        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$318,$A9,'Full Detail'!$C$2:$C$318,"Remaining")</f>
         <v>0</v>
       </c>
       <c r="D9" s="5" t="n">
-        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$317,$A9,'Full Detail'!$C$2:$C$317,"Deferred")</f>
+        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$318,$A9,'Full Detail'!$C$2:$C$318,"Deferred")</f>
         <v>1</v>
       </c>
       <c r="E9" s="5" t="n">
@@ -2619,20 +2625,20 @@
         <v>13</v>
       </c>
       <c r="B10" s="5" t="n">
-        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$317,$A10,'Full Detail'!$C$2:$C$317,"Done")</f>
-        <v>32</v>
+        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$318,$A10,'Full Detail'!$C$2:$C$318,"Done")</f>
+        <v>26</v>
       </c>
       <c r="C10" s="5" t="n">
-        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$317,$A10,'Full Detail'!$C$2:$C$317,"Remaining")</f>
+        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$318,$A10,'Full Detail'!$C$2:$C$318,"Remaining")</f>
         <v>0</v>
       </c>
       <c r="D10" s="5" t="n">
-        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$317,$A10,'Full Detail'!$C$2:$C$317,"Deferred")</f>
+        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$318,$A10,'Full Detail'!$C$2:$C$318,"Deferred")</f>
         <v>0</v>
       </c>
       <c r="E10" s="5" t="n">
         <f aca="false">SUM(B10:D10)</f>
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F10" s="6" t="n">
         <f aca="false">IF(E10=0,0,B10/E10)</f>
@@ -2644,15 +2650,15 @@
         <v>14</v>
       </c>
       <c r="B11" s="5" t="n">
-        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$317,$A11,'Full Detail'!$C$2:$C$317,"Done")</f>
+        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$318,$A11,'Full Detail'!$C$2:$C$318,"Done")</f>
         <v>32</v>
       </c>
       <c r="C11" s="5" t="n">
-        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$317,$A11,'Full Detail'!$C$2:$C$317,"Remaining")</f>
+        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$318,$A11,'Full Detail'!$C$2:$C$318,"Remaining")</f>
         <v>0</v>
       </c>
       <c r="D11" s="5" t="n">
-        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$317,$A11,'Full Detail'!$C$2:$C$317,"Deferred")</f>
+        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$318,$A11,'Full Detail'!$C$2:$C$318,"Deferred")</f>
         <v>0</v>
       </c>
       <c r="E11" s="5" t="n">
@@ -2669,15 +2675,15 @@
         <v>15</v>
       </c>
       <c r="B12" s="5" t="n">
-        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$317,$A12,'Full Detail'!$C$2:$C$317,"Done")</f>
+        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$318,$A12,'Full Detail'!$C$2:$C$318,"Done")</f>
         <v>21</v>
       </c>
       <c r="C12" s="5" t="n">
-        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$317,$A12,'Full Detail'!$C$2:$C$317,"Remaining")</f>
+        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$318,$A12,'Full Detail'!$C$2:$C$318,"Remaining")</f>
         <v>0</v>
       </c>
       <c r="D12" s="5" t="n">
-        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$317,$A12,'Full Detail'!$C$2:$C$317,"Deferred")</f>
+        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$318,$A12,'Full Detail'!$C$2:$C$318,"Deferred")</f>
         <v>0</v>
       </c>
       <c r="E12" s="5" t="n">
@@ -2694,15 +2700,15 @@
         <v>16</v>
       </c>
       <c r="B13" s="5" t="n">
-        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$317,$A13,'Full Detail'!$C$2:$C$317,"Done")</f>
+        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$318,$A13,'Full Detail'!$C$2:$C$318,"Done")</f>
         <v>3</v>
       </c>
       <c r="C13" s="5" t="n">
-        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$317,$A13,'Full Detail'!$C$2:$C$317,"Remaining")</f>
+        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$318,$A13,'Full Detail'!$C$2:$C$318,"Remaining")</f>
         <v>0</v>
       </c>
       <c r="D13" s="5" t="n">
-        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$317,$A13,'Full Detail'!$C$2:$C$317,"Deferred")</f>
+        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$318,$A13,'Full Detail'!$C$2:$C$318,"Deferred")</f>
         <v>0</v>
       </c>
       <c r="E13" s="5" t="n">
@@ -2719,15 +2725,15 @@
         <v>17</v>
       </c>
       <c r="B14" s="5" t="n">
-        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$317,$A14,'Full Detail'!$C$2:$C$317,"Done")</f>
+        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$318,$A14,'Full Detail'!$C$2:$C$318,"Done")</f>
         <v>27</v>
       </c>
       <c r="C14" s="5" t="n">
-        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$317,$A14,'Full Detail'!$C$2:$C$317,"Remaining")</f>
+        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$318,$A14,'Full Detail'!$C$2:$C$318,"Remaining")</f>
         <v>0</v>
       </c>
       <c r="D14" s="5" t="n">
-        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$317,$A14,'Full Detail'!$C$2:$C$317,"Deferred")</f>
+        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$318,$A14,'Full Detail'!$C$2:$C$318,"Deferred")</f>
         <v>0</v>
       </c>
       <c r="E14" s="5" t="n">
@@ -2744,15 +2750,15 @@
         <v>18</v>
       </c>
       <c r="B15" s="5" t="n">
-        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$317,$A15,'Full Detail'!$C$2:$C$317,"Done")</f>
+        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$318,$A15,'Full Detail'!$C$2:$C$318,"Done")</f>
         <v>0</v>
       </c>
       <c r="C15" s="5" t="n">
-        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$317,$A15,'Full Detail'!$C$2:$C$317,"Remaining")</f>
+        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$318,$A15,'Full Detail'!$C$2:$C$318,"Remaining")</f>
         <v>0</v>
       </c>
       <c r="D15" s="5" t="n">
-        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$317,$A15,'Full Detail'!$C$2:$C$317,"Deferred")</f>
+        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$318,$A15,'Full Detail'!$C$2:$C$318,"Deferred")</f>
         <v>0</v>
       </c>
       <c r="E15" s="5" t="n">
@@ -2769,15 +2775,15 @@
         <v>19</v>
       </c>
       <c r="B16" s="5" t="n">
-        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$317,$A16,'Full Detail'!$C$2:$C$317,"Done")</f>
+        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$318,$A16,'Full Detail'!$C$2:$C$318,"Done")</f>
         <v>15</v>
       </c>
       <c r="C16" s="5" t="n">
-        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$317,$A16,'Full Detail'!$C$2:$C$317,"Remaining")</f>
+        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$318,$A16,'Full Detail'!$C$2:$C$318,"Remaining")</f>
         <v>3</v>
       </c>
       <c r="D16" s="5" t="n">
-        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$317,$A16,'Full Detail'!$C$2:$C$317,"Deferred")</f>
+        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$318,$A16,'Full Detail'!$C$2:$C$318,"Deferred")</f>
         <v>0</v>
       </c>
       <c r="E16" s="5" t="n">
@@ -2794,24 +2800,24 @@
         <v>20</v>
       </c>
       <c r="B17" s="5" t="n">
-        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$317,$A17,'Full Detail'!$C$2:$C$317,"Done")</f>
-        <v>19</v>
+        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$318,$A17,'Full Detail'!$C$2:$C$318,"Done")</f>
+        <v>25</v>
       </c>
       <c r="C17" s="5" t="n">
-        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$317,$A17,'Full Detail'!$C$2:$C$317,"Remaining")</f>
-        <v>7</v>
+        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$318,$A17,'Full Detail'!$C$2:$C$318,"Remaining")</f>
+        <v>8</v>
       </c>
       <c r="D17" s="5" t="n">
-        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$317,$A17,'Full Detail'!$C$2:$C$317,"Deferred")</f>
+        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$318,$A17,'Full Detail'!$C$2:$C$318,"Deferred")</f>
         <v>1</v>
       </c>
       <c r="E17" s="5" t="n">
         <f aca="false">SUM(B17:D17)</f>
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="F17" s="6" t="n">
         <f aca="false">IF(E17=0,0,B17/E17)</f>
-        <v>0.703703703703704</v>
+        <v>0.735294117647059</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2819,15 +2825,15 @@
         <v>21</v>
       </c>
       <c r="B18" s="5" t="n">
-        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$317,$A18,'Full Detail'!$C$2:$C$317,"Done")</f>
+        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$318,$A18,'Full Detail'!$C$2:$C$318,"Done")</f>
         <v>16</v>
       </c>
       <c r="C18" s="5" t="n">
-        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$317,$A18,'Full Detail'!$C$2:$C$317,"Remaining")</f>
+        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$318,$A18,'Full Detail'!$C$2:$C$318,"Remaining")</f>
         <v>3</v>
       </c>
       <c r="D18" s="5" t="n">
-        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$317,$A18,'Full Detail'!$C$2:$C$317,"Deferred")</f>
+        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$318,$A18,'Full Detail'!$C$2:$C$318,"Deferred")</f>
         <v>0</v>
       </c>
       <c r="E18" s="5" t="n">
@@ -2844,15 +2850,15 @@
         <v>22</v>
       </c>
       <c r="B19" s="5" t="n">
-        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$317,$A19,'Full Detail'!$C$2:$C$317,"Done")</f>
+        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$318,$A19,'Full Detail'!$C$2:$C$318,"Done")</f>
         <v>0</v>
       </c>
       <c r="C19" s="5" t="n">
-        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$317,$A19,'Full Detail'!$C$2:$C$317,"Remaining")</f>
+        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$318,$A19,'Full Detail'!$C$2:$C$318,"Remaining")</f>
         <v>7</v>
       </c>
       <c r="D19" s="5" t="n">
-        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$317,$A19,'Full Detail'!$C$2:$C$317,"Deferred")</f>
+        <f aca="false">COUNTIFS('Full Detail'!$E$2:$E$318,$A19,'Full Detail'!$C$2:$C$318,"Deferred")</f>
         <v>0</v>
       </c>
       <c r="E19" s="5" t="n">
@@ -2874,7 +2880,7 @@
       </c>
       <c r="C20" s="8" t="n">
         <f aca="false">SUM(C5:C19)</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D20" s="8" t="n">
         <f aca="false">SUM(D5:D19)</f>
@@ -2882,11 +2888,11 @@
       </c>
       <c r="E20" s="8" t="n">
         <f aca="false">SUM(E5:E19)</f>
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="F20" s="9" t="n">
         <f aca="false">IF(E20=0,0,B20/E20)</f>
-        <v>0.920529801324503</v>
+        <v>0.917491749174918</v>
       </c>
     </row>
   </sheetData>
@@ -2905,7 +2911,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E317"/>
+  <dimension ref="A1:E318"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
@@ -5078,105 +5084,105 @@
         <v>13</v>
       </c>
     </row>
-    <row r="150" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A150" s="4"/>
-      <c r="B150" s="4" t="s">
-        <v>292</v>
-      </c>
-      <c r="C150" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="D150" s="4" t="s">
-        <v>293</v>
-      </c>
-      <c r="E150" s="12" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="151" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="150" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A150" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B150" s="10"/>
+      <c r="C150" s="10"/>
+      <c r="D150" s="10"/>
+    </row>
+    <row r="151" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="4"/>
       <c r="B151" s="4" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="C151" s="11" t="s">
         <v>3</v>
       </c>
       <c r="D151" s="4" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="E151" s="12" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="152" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="152" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A152" s="4"/>
       <c r="B152" s="4" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="C152" s="11" t="s">
         <v>3</v>
       </c>
       <c r="D152" s="4" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="E152" s="12" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="153" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="153" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="4"/>
       <c r="B153" s="4" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="C153" s="11" t="s">
         <v>3</v>
       </c>
       <c r="D153" s="4" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="E153" s="12" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="4"/>
       <c r="B154" s="4" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="C154" s="11" t="s">
         <v>3</v>
       </c>
       <c r="D154" s="4" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="E154" s="12" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="155" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="155" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A155" s="4"/>
       <c r="B155" s="4" t="s">
+        <v>300</v>
+      </c>
+      <c r="C155" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="D155" s="4" t="s">
+        <v>301</v>
+      </c>
+      <c r="E155" s="12" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="156" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A156" s="4"/>
+      <c r="B156" s="4" t="s">
         <v>302</v>
       </c>
-      <c r="C155" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="D155" s="4" t="s">
+      <c r="C156" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="D156" s="4" t="s">
         <v>303</v>
       </c>
-      <c r="E155" s="12" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="156" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A156" s="10" t="s">
+      <c r="E156" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="B156" s="10"/>
-      <c r="C156" s="10"/>
-      <c r="D156" s="10"/>
-    </row>
-    <row r="157" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="157" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="4"/>
       <c r="B157" s="4" t="s">
         <v>304</v>
@@ -5191,7 +5197,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="158" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="158" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="4"/>
       <c r="B158" s="4" t="s">
         <v>306</v>
@@ -5206,7 +5212,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="159" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="159" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="4"/>
       <c r="B159" s="4" t="s">
         <v>308</v>
@@ -5236,7 +5242,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="161" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="161" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A161" s="4"/>
       <c r="B161" s="4" t="s">
         <v>312</v>
@@ -5251,7 +5257,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="162" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="162" customFormat="false" ht="124.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A162" s="4"/>
       <c r="B162" s="4" t="s">
         <v>314</v>
@@ -5266,7 +5272,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="163" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="163" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="4"/>
       <c r="B163" s="4" t="s">
         <v>316</v>
@@ -5281,7 +5287,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="164" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="164" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A164" s="4"/>
       <c r="B164" s="4" t="s">
         <v>318</v>
@@ -5326,7 +5332,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="167" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="167" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A167" s="4"/>
       <c r="B167" s="4" t="s">
         <v>324</v>
@@ -5341,7 +5347,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="168" customFormat="false" ht="124.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="168" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A168" s="4"/>
       <c r="B168" s="4" t="s">
         <v>326</v>
@@ -5356,7 +5362,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="169" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="169" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A169" s="4"/>
       <c r="B169" s="4" t="s">
         <v>328</v>
@@ -5371,7 +5377,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="170" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="170" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A170" s="4"/>
       <c r="B170" s="4" t="s">
         <v>330</v>
@@ -5386,7 +5392,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="171" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="171" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A171" s="4"/>
       <c r="B171" s="4" t="s">
         <v>332</v>
@@ -5401,7 +5407,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="172" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="172" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A172" s="4"/>
       <c r="B172" s="4" t="s">
         <v>334</v>
@@ -5416,7 +5422,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="173" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="173" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A173" s="4"/>
       <c r="B173" s="4" t="s">
         <v>336</v>
@@ -5431,7 +5437,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="174" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="174" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A174" s="4"/>
       <c r="B174" s="4" t="s">
         <v>338</v>
@@ -5446,7 +5452,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="175" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="175" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A175" s="4"/>
       <c r="B175" s="4" t="s">
         <v>340</v>
@@ -5461,7 +5467,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="176" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="176" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A176" s="4"/>
       <c r="B176" s="4" t="s">
         <v>342</v>
@@ -5476,7 +5482,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="177" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="177" customFormat="false" ht="147" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A177" s="4"/>
       <c r="B177" s="4" t="s">
         <v>344</v>
@@ -5506,7 +5512,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="179" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="179" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A179" s="4"/>
       <c r="B179" s="4" t="s">
         <v>348</v>
@@ -5521,7 +5527,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="180" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="180" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A180" s="4"/>
       <c r="B180" s="4" t="s">
         <v>350</v>
@@ -5536,7 +5542,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="181" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="181" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A181" s="4"/>
       <c r="B181" s="4" t="s">
         <v>352</v>
@@ -5551,7 +5557,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="182" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="182" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A182" s="4"/>
       <c r="B182" s="4" t="s">
         <v>354</v>
@@ -5566,105 +5572,105 @@
         <v>14</v>
       </c>
     </row>
-    <row r="183" customFormat="false" ht="147" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A183" s="4"/>
-      <c r="B183" s="4" t="s">
-        <v>356</v>
-      </c>
-      <c r="C183" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="D183" s="4" t="s">
-        <v>357</v>
-      </c>
-      <c r="E183" s="12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="184" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="183" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A183" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B183" s="10"/>
+      <c r="C183" s="10"/>
+      <c r="D183" s="10"/>
+    </row>
+    <row r="184" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A184" s="4"/>
       <c r="B184" s="4" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="C184" s="11" t="s">
         <v>3</v>
       </c>
       <c r="D184" s="4" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="E184" s="12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="185" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="185" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A185" s="4"/>
       <c r="B185" s="4" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="C185" s="11" t="s">
         <v>3</v>
       </c>
       <c r="D185" s="4" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="E185" s="12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="186" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="186" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A186" s="4"/>
       <c r="B186" s="4" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="C186" s="11" t="s">
         <v>3</v>
       </c>
       <c r="D186" s="4" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="E186" s="12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="187" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="187" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A187" s="4"/>
       <c r="B187" s="4" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="C187" s="11" t="s">
         <v>3</v>
       </c>
       <c r="D187" s="4" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="E187" s="12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="188" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="188" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A188" s="4"/>
       <c r="B188" s="4" t="s">
+        <v>364</v>
+      </c>
+      <c r="C188" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="D188" s="4" t="s">
+        <v>365</v>
+      </c>
+      <c r="E188" s="12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="189" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A189" s="4"/>
+      <c r="B189" s="4" t="s">
         <v>366</v>
       </c>
-      <c r="C188" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="D188" s="4" t="s">
+      <c r="C189" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="D189" s="4" t="s">
         <v>367</v>
       </c>
-      <c r="E188" s="12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="189" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A189" s="10" t="s">
+      <c r="E189" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B189" s="10"/>
-      <c r="C189" s="10"/>
-      <c r="D189" s="10"/>
-    </row>
-    <row r="190" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="190" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A190" s="4"/>
       <c r="B190" s="4" t="s">
         <v>368</v>
@@ -5679,7 +5685,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="191" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="191" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A191" s="4"/>
       <c r="B191" s="4" t="s">
         <v>370</v>
@@ -5694,7 +5700,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="192" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="192" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A192" s="4"/>
       <c r="B192" s="4" t="s">
         <v>372</v>
@@ -5709,7 +5715,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="193" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="193" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A193" s="4"/>
       <c r="B193" s="4" t="s">
         <v>374</v>
@@ -5724,7 +5730,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="194" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="194" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A194" s="4"/>
       <c r="B194" s="4" t="s">
         <v>376</v>
@@ -5739,7 +5745,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="195" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="195" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A195" s="4"/>
       <c r="B195" s="4" t="s">
         <v>378</v>
@@ -5754,7 +5760,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="196" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="196" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A196" s="4"/>
       <c r="B196" s="4" t="s">
         <v>380</v>
@@ -5769,7 +5775,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="197" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="197" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A197" s="4"/>
       <c r="B197" s="4" t="s">
         <v>382</v>
@@ -5784,7 +5790,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="198" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="198" customFormat="false" ht="147" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A198" s="4"/>
       <c r="B198" s="4" t="s">
         <v>384</v>
@@ -5799,7 +5805,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="199" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="199" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A199" s="4"/>
       <c r="B199" s="4" t="s">
         <v>386</v>
@@ -5814,7 +5820,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="200" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="200" customFormat="false" ht="124.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A200" s="4"/>
       <c r="B200" s="4" t="s">
         <v>388</v>
@@ -5829,7 +5835,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="201" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="201" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A201" s="4"/>
       <c r="B201" s="4" t="s">
         <v>390</v>
@@ -5859,7 +5865,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="203" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="203" customFormat="false" ht="147" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A203" s="4"/>
       <c r="B203" s="4" t="s">
         <v>394</v>
@@ -5874,7 +5880,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="204" customFormat="false" ht="147" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="204" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A204" s="4"/>
       <c r="B204" s="4" t="s">
         <v>396</v>
@@ -5889,158 +5895,158 @@
         <v>15</v>
       </c>
     </row>
-    <row r="205" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A205" s="4"/>
-      <c r="B205" s="4" t="s">
-        <v>398</v>
-      </c>
-      <c r="C205" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="D205" s="4" t="s">
-        <v>399</v>
-      </c>
-      <c r="E205" s="12" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="206" customFormat="false" ht="124.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="205" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A205" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B205" s="10"/>
+      <c r="C205" s="10"/>
+      <c r="D205" s="10"/>
+    </row>
+    <row r="206" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A206" s="4"/>
       <c r="B206" s="4" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="C206" s="11" t="s">
         <v>3</v>
       </c>
       <c r="D206" s="4" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="E206" s="12" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="207" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="207" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A207" s="4"/>
       <c r="B207" s="4" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="C207" s="11" t="s">
         <v>3</v>
       </c>
       <c r="D207" s="4" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="E207" s="12" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="208" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="208" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A208" s="4"/>
       <c r="B208" s="4" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="C208" s="11" t="s">
         <v>3</v>
       </c>
       <c r="D208" s="4" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="E208" s="12" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="209" customFormat="false" ht="147" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A209" s="4"/>
-      <c r="B209" s="4" t="s">
-        <v>406</v>
-      </c>
-      <c r="C209" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="D209" s="4" t="s">
-        <v>407</v>
-      </c>
-      <c r="E209" s="12" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="210" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="209" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A209" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B209" s="10"/>
+      <c r="C209" s="10"/>
+      <c r="D209" s="10"/>
+    </row>
+    <row r="210" customFormat="false" ht="169.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A210" s="4"/>
       <c r="B210" s="4" t="s">
-        <v>408</v>
+        <v>404</v>
       </c>
       <c r="C210" s="11" t="s">
         <v>3</v>
       </c>
       <c r="D210" s="4" t="s">
-        <v>409</v>
+        <v>405</v>
       </c>
       <c r="E210" s="12" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="211" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A211" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="B211" s="10"/>
-      <c r="C211" s="10"/>
-      <c r="D211" s="10"/>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="211" customFormat="false" ht="147" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A211" s="4"/>
+      <c r="B211" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C211" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="D211" s="4" t="s">
+        <v>407</v>
+      </c>
+      <c r="E211" s="12" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="212" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A212" s="4"/>
       <c r="B212" s="4" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="C212" s="11" t="s">
         <v>3</v>
       </c>
       <c r="D212" s="4" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="E212" s="12" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="213" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="213" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A213" s="4"/>
       <c r="B213" s="4" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="C213" s="11" t="s">
         <v>3</v>
       </c>
       <c r="D213" s="4" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="E213" s="12" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="214" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="214" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A214" s="4"/>
       <c r="B214" s="4" t="s">
+        <v>412</v>
+      </c>
+      <c r="C214" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="D214" s="4" t="s">
+        <v>413</v>
+      </c>
+      <c r="E214" s="12" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="215" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A215" s="4"/>
+      <c r="B215" s="4" t="s">
         <v>414</v>
       </c>
-      <c r="C214" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="D214" s="4" t="s">
+      <c r="C215" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="D215" s="4" t="s">
         <v>415</v>
       </c>
-      <c r="E214" s="12" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="215" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A215" s="10" t="s">
+      <c r="E215" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="B215" s="10"/>
-      <c r="C215" s="10"/>
-      <c r="D215" s="10"/>
-    </row>
-    <row r="216" customFormat="false" ht="169.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="216" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A216" s="4"/>
       <c r="B216" s="4" t="s">
         <v>416</v>
@@ -6070,7 +6076,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="218" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="218" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A218" s="4"/>
       <c r="B218" s="4" t="s">
         <v>420</v>
@@ -6100,7 +6106,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="220" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="220" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A220" s="4"/>
       <c r="B220" s="4" t="s">
         <v>424</v>
@@ -6115,7 +6121,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="221" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="221" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A221" s="4"/>
       <c r="B221" s="4" t="s">
         <v>426</v>
@@ -6130,7 +6136,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="222" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="222" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A222" s="4"/>
       <c r="B222" s="4" t="s">
         <v>428</v>
@@ -6145,7 +6151,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="223" customFormat="false" ht="147" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="223" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A223" s="4"/>
       <c r="B223" s="4" t="s">
         <v>430</v>
@@ -6160,7 +6166,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="224" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="224" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A224" s="4"/>
       <c r="B224" s="4" t="s">
         <v>432</v>
@@ -6175,7 +6181,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="225" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="225" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A225" s="4"/>
       <c r="B225" s="4" t="s">
         <v>434</v>
@@ -6190,7 +6196,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="226" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="226" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A226" s="4"/>
       <c r="B226" s="4" t="s">
         <v>436</v>
@@ -6205,7 +6211,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="227" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="227" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A227" s="4"/>
       <c r="B227" s="4" t="s">
         <v>438</v>
@@ -6220,7 +6226,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="228" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="228" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A228" s="4"/>
       <c r="B228" s="4" t="s">
         <v>440</v>
@@ -6235,7 +6241,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="229" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="229" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A229" s="4"/>
       <c r="B229" s="4" t="s">
         <v>442</v>
@@ -6250,7 +6256,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="230" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="230" customFormat="false" ht="147" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A230" s="4"/>
       <c r="B230" s="4" t="s">
         <v>444</v>
@@ -6265,7 +6271,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="231" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="231" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A231" s="4"/>
       <c r="B231" s="4" t="s">
         <v>446</v>
@@ -6280,7 +6286,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="232" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="232" customFormat="false" ht="147" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A232" s="4"/>
       <c r="B232" s="4" t="s">
         <v>448</v>
@@ -6310,7 +6316,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="234" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="234" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A234" s="4"/>
       <c r="B234" s="4" t="s">
         <v>452</v>
@@ -6325,7 +6331,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="235" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="235" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A235" s="4"/>
       <c r="B235" s="4" t="s">
         <v>454</v>
@@ -6340,7 +6346,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="236" customFormat="false" ht="147" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="236" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A236" s="4"/>
       <c r="B236" s="4" t="s">
         <v>456</v>
@@ -6355,114 +6361,108 @@
         <v>17</v>
       </c>
     </row>
-    <row r="237" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A237" s="4"/>
-      <c r="B237" s="4" t="s">
-        <v>458</v>
-      </c>
-      <c r="C237" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="D237" s="4" t="s">
-        <v>459</v>
-      </c>
-      <c r="E237" s="12" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="238" customFormat="false" ht="147" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="237" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A237" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B237" s="10"/>
+      <c r="C237" s="10"/>
+      <c r="D237" s="10"/>
+    </row>
+    <row r="238" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A238" s="4"/>
       <c r="B238" s="4" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="C238" s="11" t="s">
         <v>3</v>
       </c>
       <c r="D238" s="4" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="E238" s="12" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="239" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="239" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A239" s="4"/>
       <c r="B239" s="4" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="C239" s="11" t="s">
         <v>3</v>
       </c>
       <c r="D239" s="4" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="E239" s="12" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="240" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="240" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A240" s="4"/>
       <c r="B240" s="4" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="C240" s="11" t="s">
         <v>3</v>
       </c>
       <c r="D240" s="4" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="E240" s="12" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="241" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A241" s="4"/>
       <c r="B241" s="4" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="C241" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="D241" s="4" t="s">
-        <v>467</v>
-      </c>
+      <c r="D241" s="4"/>
       <c r="E241" s="12" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="242" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="242" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A242" s="4"/>
       <c r="B242" s="4" t="s">
-        <v>468</v>
+        <v>465</v>
       </c>
       <c r="C242" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="D242" s="4" t="s">
-        <v>469</v>
-      </c>
+      <c r="D242" s="4"/>
       <c r="E242" s="12" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="243" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A243" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="B243" s="10"/>
-      <c r="C243" s="10"/>
-      <c r="D243" s="10"/>
-    </row>
-    <row r="244" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="243" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A243" s="4"/>
+      <c r="B243" s="4" t="s">
+        <v>466</v>
+      </c>
+      <c r="C243" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="D243" s="4"/>
+      <c r="E243" s="12" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="244" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A244" s="4"/>
       <c r="B244" s="4" t="s">
-        <v>470</v>
+        <v>467</v>
       </c>
       <c r="C244" s="11" t="s">
         <v>3</v>
       </c>
       <c r="D244" s="4" t="s">
-        <v>471</v>
+        <v>468</v>
       </c>
       <c r="E244" s="12" t="s">
         <v>19</v>
@@ -6471,28 +6471,28 @@
     <row r="245" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A245" s="4"/>
       <c r="B245" s="4" t="s">
-        <v>472</v>
+        <v>469</v>
       </c>
       <c r="C245" s="11" t="s">
         <v>3</v>
       </c>
       <c r="D245" s="4" t="s">
-        <v>473</v>
+        <v>470</v>
       </c>
       <c r="E245" s="12" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="246" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="246" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A246" s="4"/>
       <c r="B246" s="4" t="s">
-        <v>474</v>
-      </c>
-      <c r="C246" s="11" t="s">
-        <v>3</v>
+        <v>471</v>
+      </c>
+      <c r="C246" s="13" t="s">
+        <v>4</v>
       </c>
       <c r="D246" s="4" t="s">
-        <v>475</v>
+        <v>472</v>
       </c>
       <c r="E246" s="12" t="s">
         <v>19</v>
@@ -6501,67 +6501,71 @@
     <row r="247" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A247" s="4"/>
       <c r="B247" s="4" t="s">
-        <v>476</v>
-      </c>
-      <c r="C247" s="11" t="s">
-        <v>3</v>
+        <v>473</v>
+      </c>
+      <c r="C247" s="13" t="s">
+        <v>4</v>
       </c>
       <c r="D247" s="4"/>
       <c r="E247" s="12" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="248" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="248" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A248" s="4"/>
       <c r="B248" s="4" t="s">
-        <v>477</v>
+        <v>474</v>
       </c>
       <c r="C248" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="D248" s="4"/>
+      <c r="D248" s="4" t="s">
+        <v>475</v>
+      </c>
       <c r="E248" s="12" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="249" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="249" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A249" s="4"/>
       <c r="B249" s="4" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="C249" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="D249" s="4"/>
+      <c r="D249" s="4" t="s">
+        <v>477</v>
+      </c>
       <c r="E249" s="12" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="250" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="250" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A250" s="4"/>
       <c r="B250" s="4" t="s">
+        <v>478</v>
+      </c>
+      <c r="C250" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="D250" s="4" t="s">
         <v>479</v>
-      </c>
-      <c r="C250" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="D250" s="4" t="s">
-        <v>480</v>
       </c>
       <c r="E250" s="12" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="251" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="251" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A251" s="4"/>
       <c r="B251" s="4" t="s">
+        <v>480</v>
+      </c>
+      <c r="C251" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="D251" s="4" t="s">
         <v>481</v>
-      </c>
-      <c r="C251" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="D251" s="4" t="s">
-        <v>482</v>
       </c>
       <c r="E251" s="12" t="s">
         <v>19</v>
@@ -6570,32 +6574,34 @@
     <row r="252" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A252" s="4"/>
       <c r="B252" s="4" t="s">
+        <v>482</v>
+      </c>
+      <c r="C252" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="D252" s="4" t="s">
         <v>483</v>
-      </c>
-      <c r="C252" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="D252" s="4" t="s">
-        <v>484</v>
       </c>
       <c r="E252" s="12" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="253" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="253" customFormat="false" ht="124.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A253" s="4"/>
       <c r="B253" s="4" t="s">
+        <v>484</v>
+      </c>
+      <c r="C253" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="D253" s="4" t="s">
         <v>485</v>
       </c>
-      <c r="C253" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="D253" s="4"/>
       <c r="E253" s="12" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="254" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="254" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A254" s="4"/>
       <c r="B254" s="4" t="s">
         <v>486</v>
@@ -6610,13 +6616,13 @@
         <v>19</v>
       </c>
     </row>
-    <row r="255" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="255" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A255" s="4"/>
       <c r="B255" s="4" t="s">
         <v>488</v>
       </c>
-      <c r="C255" s="11" t="s">
-        <v>3</v>
+      <c r="C255" s="13" t="s">
+        <v>4</v>
       </c>
       <c r="D255" s="4" t="s">
         <v>489</v>
@@ -6625,105 +6631,105 @@
         <v>19</v>
       </c>
     </row>
-    <row r="256" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A256" s="4"/>
-      <c r="B256" s="4" t="s">
-        <v>490</v>
-      </c>
-      <c r="C256" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="D256" s="4" t="s">
-        <v>491</v>
-      </c>
-      <c r="E256" s="12" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="257" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="256" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A256" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="B256" s="10"/>
+      <c r="C256" s="10"/>
+      <c r="D256" s="10"/>
+    </row>
+    <row r="257" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A257" s="4"/>
       <c r="B257" s="4" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="C257" s="11" t="s">
         <v>3</v>
       </c>
       <c r="D257" s="4" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="E257" s="12" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="258" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="258" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A258" s="4"/>
       <c r="B258" s="4" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="C258" s="11" t="s">
         <v>3</v>
       </c>
       <c r="D258" s="4" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
       <c r="E258" s="12" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="259" customFormat="false" ht="124.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="259" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A259" s="4"/>
       <c r="B259" s="4" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="C259" s="11" t="s">
         <v>3</v>
       </c>
       <c r="D259" s="4" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
       <c r="E259" s="12" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="260" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A260" s="4"/>
       <c r="B260" s="4" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="C260" s="11" t="s">
         <v>3</v>
       </c>
       <c r="D260" s="4" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="E260" s="12" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="261" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="261" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A261" s="4"/>
       <c r="B261" s="4" t="s">
+        <v>498</v>
+      </c>
+      <c r="C261" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="D261" s="4" t="s">
+        <v>499</v>
+      </c>
+      <c r="E261" s="12" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="262" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A262" s="4"/>
+      <c r="B262" s="4" t="s">
         <v>500</v>
       </c>
-      <c r="C261" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="D261" s="4" t="s">
+      <c r="C262" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="D262" s="4" t="s">
         <v>501</v>
       </c>
-      <c r="E261" s="12" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="262" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A262" s="10" t="s">
+      <c r="E262" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="B262" s="10"/>
-      <c r="C262" s="10"/>
-      <c r="D262" s="10"/>
-    </row>
-    <row r="263" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="263" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A263" s="4"/>
       <c r="B263" s="4" t="s">
         <v>502</v>
@@ -6738,7 +6744,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="264" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="264" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A264" s="4"/>
       <c r="B264" s="4" t="s">
         <v>504</v>
@@ -6753,7 +6759,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="265" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="265" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A265" s="4"/>
       <c r="B265" s="4" t="s">
         <v>506</v>
@@ -6783,13 +6789,13 @@
         <v>20</v>
       </c>
     </row>
-    <row r="267" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="267" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A267" s="4"/>
       <c r="B267" s="4" t="s">
         <v>510</v>
       </c>
-      <c r="C267" s="11" t="s">
-        <v>3</v>
+      <c r="C267" s="13" t="s">
+        <v>4</v>
       </c>
       <c r="D267" s="4" t="s">
         <v>511</v>
@@ -6798,13 +6804,13 @@
         <v>20</v>
       </c>
     </row>
-    <row r="268" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="268" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A268" s="4"/>
       <c r="B268" s="4" t="s">
         <v>512</v>
       </c>
-      <c r="C268" s="11" t="s">
-        <v>3</v>
+      <c r="C268" s="13" t="s">
+        <v>4</v>
       </c>
       <c r="D268" s="4" t="s">
         <v>513</v>
@@ -6813,7 +6819,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="269" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="269" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A269" s="4"/>
       <c r="B269" s="4" t="s">
         <v>514</v>
@@ -6843,7 +6849,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="271" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="271" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A271" s="4"/>
       <c r="B271" s="4" t="s">
         <v>518</v>
@@ -6858,7 +6864,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="272" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="272" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A272" s="4"/>
       <c r="B272" s="4" t="s">
         <v>520</v>
@@ -6873,13 +6879,13 @@
         <v>20</v>
       </c>
     </row>
-    <row r="273" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="273" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A273" s="4"/>
       <c r="B273" s="4" t="s">
         <v>522</v>
       </c>
-      <c r="C273" s="13" t="s">
-        <v>4</v>
+      <c r="C273" s="11" t="s">
+        <v>3</v>
       </c>
       <c r="D273" s="4" t="s">
         <v>523</v>
@@ -6888,13 +6894,13 @@
         <v>20</v>
       </c>
     </row>
-    <row r="274" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="274" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A274" s="4"/>
       <c r="B274" s="4" t="s">
         <v>524</v>
       </c>
-      <c r="C274" s="13" t="s">
-        <v>4</v>
+      <c r="C274" s="11" t="s">
+        <v>3</v>
       </c>
       <c r="D274" s="4" t="s">
         <v>525</v>
@@ -6903,7 +6909,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="275" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="275" customFormat="false" ht="147" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A275" s="4"/>
       <c r="B275" s="4" t="s">
         <v>526</v>
@@ -6918,13 +6924,13 @@
         <v>20</v>
       </c>
     </row>
-    <row r="276" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="276" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A276" s="4"/>
       <c r="B276" s="4" t="s">
         <v>528</v>
       </c>
-      <c r="C276" s="11" t="s">
-        <v>3</v>
+      <c r="C276" s="13" t="s">
+        <v>4</v>
       </c>
       <c r="D276" s="4" t="s">
         <v>529</v>
@@ -6933,13 +6939,13 @@
         <v>20</v>
       </c>
     </row>
-    <row r="277" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="277" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A277" s="4"/>
       <c r="B277" s="4" t="s">
         <v>530</v>
       </c>
-      <c r="C277" s="11" t="s">
-        <v>3</v>
+      <c r="C277" s="13" t="s">
+        <v>4</v>
       </c>
       <c r="D277" s="4" t="s">
         <v>531</v>
@@ -6948,13 +6954,13 @@
         <v>20</v>
       </c>
     </row>
-    <row r="278" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="278" customFormat="false" ht="147" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A278" s="4"/>
       <c r="B278" s="4" t="s">
         <v>532</v>
       </c>
-      <c r="C278" s="11" t="s">
-        <v>3</v>
+      <c r="C278" s="14" t="s">
+        <v>5</v>
       </c>
       <c r="D278" s="4" t="s">
         <v>533</v>
@@ -6963,13 +6969,13 @@
         <v>20</v>
       </c>
     </row>
-    <row r="279" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="279" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A279" s="4"/>
       <c r="B279" s="4" t="s">
         <v>534</v>
       </c>
-      <c r="C279" s="11" t="s">
-        <v>3</v>
+      <c r="C279" s="13" t="s">
+        <v>4</v>
       </c>
       <c r="D279" s="4" t="s">
         <v>535</v>
@@ -6978,7 +6984,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="280" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="280" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A280" s="4"/>
       <c r="B280" s="4" t="s">
         <v>536</v>
@@ -6993,13 +6999,13 @@
         <v>20</v>
       </c>
     </row>
-    <row r="281" customFormat="false" ht="147" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="281" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A281" s="4"/>
       <c r="B281" s="4" t="s">
         <v>538</v>
       </c>
-      <c r="C281" s="11" t="s">
-        <v>3</v>
+      <c r="C281" s="13" t="s">
+        <v>4</v>
       </c>
       <c r="D281" s="4" t="s">
         <v>539</v>
@@ -7016,83 +7022,81 @@
       <c r="C282" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="D282" s="4" t="s">
-        <v>541</v>
-      </c>
+      <c r="D282" s="4"/>
       <c r="E282" s="12" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="283" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="283" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A283" s="4"/>
       <c r="B283" s="4" t="s">
+        <v>541</v>
+      </c>
+      <c r="C283" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="D283" s="4" t="s">
         <v>542</v>
-      </c>
-      <c r="C283" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="D283" s="4" t="s">
-        <v>543</v>
       </c>
       <c r="E283" s="12" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="284" customFormat="false" ht="147" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="284" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A284" s="4"/>
       <c r="B284" s="4" t="s">
+        <v>543</v>
+      </c>
+      <c r="C284" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="D284" s="4" t="s">
         <v>544</v>
-      </c>
-      <c r="C284" s="14" t="s">
-        <v>5</v>
-      </c>
-      <c r="D284" s="4" t="s">
-        <v>545</v>
       </c>
       <c r="E284" s="12" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="285" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="285" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A285" s="4"/>
       <c r="B285" s="4" t="s">
+        <v>545</v>
+      </c>
+      <c r="C285" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="D285" s="4" t="s">
         <v>546</v>
-      </c>
-      <c r="C285" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="D285" s="4" t="s">
-        <v>547</v>
       </c>
       <c r="E285" s="12" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="286" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="286" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A286" s="4"/>
       <c r="B286" s="4" t="s">
+        <v>547</v>
+      </c>
+      <c r="C286" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="D286" s="4" t="s">
         <v>548</v>
-      </c>
-      <c r="C286" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="D286" s="4" t="s">
-        <v>549</v>
       </c>
       <c r="E286" s="12" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="287" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="287" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A287" s="4"/>
       <c r="B287" s="4" t="s">
+        <v>549</v>
+      </c>
+      <c r="C287" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="D287" s="4" t="s">
         <v>550</v>
-      </c>
-      <c r="C287" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="D287" s="4" t="s">
-        <v>551</v>
       </c>
       <c r="E287" s="12" t="s">
         <v>20</v>
@@ -7101,17 +7105,19 @@
     <row r="288" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A288" s="4"/>
       <c r="B288" s="4" t="s">
+        <v>551</v>
+      </c>
+      <c r="C288" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="D288" s="4" t="s">
         <v>552</v>
       </c>
-      <c r="C288" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="D288" s="4"/>
       <c r="E288" s="12" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="289" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="289" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A289" s="4"/>
       <c r="B289" s="4" t="s">
         <v>553</v>
@@ -7126,30 +7132,30 @@
         <v>20</v>
       </c>
     </row>
-    <row r="290" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A290" s="10" t="s">
+    <row r="290" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A290" s="4"/>
+      <c r="B290" s="4" t="s">
+        <v>555</v>
+      </c>
+      <c r="C290" s="13" t="s">
+        <v>4</v>
+      </c>
+      <c r="D290" s="4" t="s">
+        <v>556</v>
+      </c>
+      <c r="E290" s="12" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="291" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A291" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B290" s="10"/>
-      <c r="C290" s="10"/>
-      <c r="D290" s="10"/>
-    </row>
-    <row r="291" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A291" s="4"/>
-      <c r="B291" s="4" t="s">
-        <v>555</v>
-      </c>
-      <c r="C291" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="D291" s="4" t="s">
-        <v>556</v>
-      </c>
-      <c r="E291" s="12" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="292" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B291" s="10"/>
+      <c r="C291" s="10"/>
+      <c r="D291" s="10"/>
+    </row>
+    <row r="292" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A292" s="4"/>
       <c r="B292" s="4" t="s">
         <v>557</v>
@@ -7164,13 +7170,13 @@
         <v>21</v>
       </c>
     </row>
-    <row r="293" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="293" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A293" s="4"/>
       <c r="B293" s="4" t="s">
         <v>559</v>
       </c>
-      <c r="C293" s="13" t="s">
-        <v>4</v>
+      <c r="C293" s="11" t="s">
+        <v>3</v>
       </c>
       <c r="D293" s="4" t="s">
         <v>560</v>
@@ -7184,8 +7190,8 @@
       <c r="B294" s="4" t="s">
         <v>561</v>
       </c>
-      <c r="C294" s="11" t="s">
-        <v>3</v>
+      <c r="C294" s="13" t="s">
+        <v>4</v>
       </c>
       <c r="D294" s="4" t="s">
         <v>562</v>
@@ -7194,7 +7200,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="295" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="295" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A295" s="4"/>
       <c r="B295" s="4" t="s">
         <v>563</v>
@@ -7209,7 +7215,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="296" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="296" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A296" s="4"/>
       <c r="B296" s="4" t="s">
         <v>565</v>
@@ -7239,13 +7245,13 @@
         <v>21</v>
       </c>
     </row>
-    <row r="298" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="298" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A298" s="4"/>
       <c r="B298" s="4" t="s">
         <v>569</v>
       </c>
-      <c r="C298" s="13" t="s">
-        <v>4</v>
+      <c r="C298" s="11" t="s">
+        <v>3</v>
       </c>
       <c r="D298" s="4" t="s">
         <v>570</v>
@@ -7254,13 +7260,13 @@
         <v>21</v>
       </c>
     </row>
-    <row r="299" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="299" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A299" s="4"/>
       <c r="B299" s="4" t="s">
         <v>571</v>
       </c>
-      <c r="C299" s="11" t="s">
-        <v>3</v>
+      <c r="C299" s="13" t="s">
+        <v>4</v>
       </c>
       <c r="D299" s="4" t="s">
         <v>572</v>
@@ -7269,7 +7275,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="300" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="300" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A300" s="4"/>
       <c r="B300" s="4" t="s">
         <v>573</v>
@@ -7284,7 +7290,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="301" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="301" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A301" s="4"/>
       <c r="B301" s="4" t="s">
         <v>575</v>
@@ -7299,7 +7305,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="302" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="302" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A302" s="4"/>
       <c r="B302" s="4" t="s">
         <v>577</v>
@@ -7314,7 +7320,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="303" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="303" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A303" s="4"/>
       <c r="B303" s="4" t="s">
         <v>579</v>
@@ -7329,7 +7335,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="304" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="304" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A304" s="4"/>
       <c r="B304" s="4" t="s">
         <v>581</v>
@@ -7344,7 +7350,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="305" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="305" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A305" s="4"/>
       <c r="B305" s="4" t="s">
         <v>583</v>
@@ -7379,8 +7385,8 @@
       <c r="B307" s="4" t="s">
         <v>587</v>
       </c>
-      <c r="C307" s="13" t="s">
-        <v>4</v>
+      <c r="C307" s="11" t="s">
+        <v>3</v>
       </c>
       <c r="D307" s="4" t="s">
         <v>588</v>
@@ -7389,13 +7395,13 @@
         <v>21</v>
       </c>
     </row>
-    <row r="308" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="308" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A308" s="4"/>
       <c r="B308" s="4" t="s">
         <v>589</v>
       </c>
-      <c r="C308" s="11" t="s">
-        <v>3</v>
+      <c r="C308" s="13" t="s">
+        <v>4</v>
       </c>
       <c r="D308" s="4" t="s">
         <v>590</v>
@@ -7404,7 +7410,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="309" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="309" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A309" s="4"/>
       <c r="B309" s="4" t="s">
         <v>591</v>
@@ -7419,30 +7425,30 @@
         <v>21</v>
       </c>
     </row>
-    <row r="310" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A310" s="10" t="s">
+    <row r="310" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A310" s="4"/>
+      <c r="B310" s="4" t="s">
+        <v>593</v>
+      </c>
+      <c r="C310" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="D310" s="4" t="s">
+        <v>594</v>
+      </c>
+      <c r="E310" s="12" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="311" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A311" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="B310" s="10"/>
-      <c r="C310" s="10"/>
-      <c r="D310" s="10"/>
-    </row>
-    <row r="311" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A311" s="4"/>
-      <c r="B311" s="4" t="s">
-        <v>593</v>
-      </c>
-      <c r="C311" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="D311" s="4" t="s">
-        <v>594</v>
-      </c>
-      <c r="E311" s="12" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="312" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B311" s="10"/>
+      <c r="C311" s="10"/>
+      <c r="D311" s="10"/>
+    </row>
+    <row r="312" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A312" s="4"/>
       <c r="B312" s="4" t="s">
         <v>595</v>
@@ -7457,7 +7463,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="313" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="313" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A313" s="4"/>
       <c r="B313" s="4" t="s">
         <v>597</v>
@@ -7472,7 +7478,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="314" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="314" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A314" s="4"/>
       <c r="B314" s="4" t="s">
         <v>599</v>
@@ -7487,7 +7493,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="315" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="315" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A315" s="4"/>
       <c r="B315" s="4" t="s">
         <v>601</v>
@@ -7510,7 +7516,9 @@
       <c r="C316" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="D316" s="4"/>
+      <c r="D316" s="4" t="s">
+        <v>604</v>
+      </c>
       <c r="E316" s="12" t="s">
         <v>22</v>
       </c>
@@ -7518,7 +7526,7 @@
     <row r="317" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A317" s="4"/>
       <c r="B317" s="4" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="C317" s="13" t="s">
         <v>4</v>
@@ -7528,8 +7536,21 @@
         <v>22</v>
       </c>
     </row>
+    <row r="318" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A318" s="4"/>
+      <c r="B318" s="4" t="s">
+        <v>606</v>
+      </c>
+      <c r="C318" s="13" t="s">
+        <v>4</v>
+      </c>
+      <c r="D318" s="4"/>
+      <c r="E318" s="12" t="s">
+        <v>22</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D317"/>
+  <autoFilter ref="A1:D318"/>
   <mergeCells count="14">
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A15:D15"/>
@@ -7537,14 +7558,14 @@
     <mergeCell ref="A43:D43"/>
     <mergeCell ref="A58:D58"/>
     <mergeCell ref="A123:D123"/>
-    <mergeCell ref="A156:D156"/>
-    <mergeCell ref="A189:D189"/>
-    <mergeCell ref="A211:D211"/>
-    <mergeCell ref="A215:D215"/>
-    <mergeCell ref="A243:D243"/>
-    <mergeCell ref="A262:D262"/>
-    <mergeCell ref="A290:D290"/>
-    <mergeCell ref="A310:D310"/>
+    <mergeCell ref="A150:D150"/>
+    <mergeCell ref="A183:D183"/>
+    <mergeCell ref="A205:D205"/>
+    <mergeCell ref="A209:D209"/>
+    <mergeCell ref="A237:D237"/>
+    <mergeCell ref="A256:D256"/>
+    <mergeCell ref="A291:D291"/>
+    <mergeCell ref="A311:D311"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -7562,7 +7583,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
@@ -7583,7 +7604,7 @@
         <v>25</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>27</v>
@@ -7661,13 +7682,13 @@
     <row r="8" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4"/>
       <c r="B8" s="4" t="s">
-        <v>483</v>
+        <v>471</v>
       </c>
       <c r="C8" s="13" t="s">
         <v>4</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>484</v>
+        <v>472</v>
       </c>
       <c r="E8" s="12" t="s">
         <v>19</v>
@@ -7676,7 +7697,7 @@
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4"/>
       <c r="B9" s="4" t="s">
-        <v>485</v>
+        <v>473</v>
       </c>
       <c r="C9" s="13" t="s">
         <v>4</v>
@@ -7689,13 +7710,13 @@
     <row r="10" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4"/>
       <c r="B10" s="4" t="s">
-        <v>500</v>
+        <v>488</v>
       </c>
       <c r="C10" s="13" t="s">
         <v>4</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>501</v>
+        <v>489</v>
       </c>
       <c r="E10" s="12" t="s">
         <v>19</v>
@@ -7712,13 +7733,13 @@
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4"/>
       <c r="B12" s="4" t="s">
-        <v>522</v>
+        <v>510</v>
       </c>
       <c r="C12" s="13" t="s">
         <v>4</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>523</v>
+        <v>511</v>
       </c>
       <c r="E12" s="12" t="s">
         <v>20</v>
@@ -7727,13 +7748,13 @@
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4"/>
       <c r="B13" s="4" t="s">
-        <v>524</v>
+        <v>512</v>
       </c>
       <c r="C13" s="13" t="s">
         <v>4</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>525</v>
+        <v>513</v>
       </c>
       <c r="E13" s="12" t="s">
         <v>20</v>
@@ -7742,13 +7763,13 @@
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4"/>
       <c r="B14" s="4" t="s">
-        <v>540</v>
+        <v>528</v>
       </c>
       <c r="C14" s="13" t="s">
         <v>4</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>541</v>
+        <v>529</v>
       </c>
       <c r="E14" s="12" t="s">
         <v>20</v>
@@ -7757,13 +7778,13 @@
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4"/>
       <c r="B15" s="4" t="s">
-        <v>542</v>
+        <v>530</v>
       </c>
       <c r="C15" s="13" t="s">
         <v>4</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>543</v>
+        <v>531</v>
       </c>
       <c r="E15" s="12" t="s">
         <v>20</v>
@@ -7772,13 +7793,13 @@
     <row r="16" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4"/>
       <c r="B16" s="4" t="s">
-        <v>544</v>
+        <v>532</v>
       </c>
       <c r="C16" s="14" t="s">
         <v>5</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>545</v>
+        <v>533</v>
       </c>
       <c r="E16" s="12" t="s">
         <v>20</v>
@@ -7787,13 +7808,13 @@
     <row r="17" customFormat="false" ht="147" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4"/>
       <c r="B17" s="4" t="s">
-        <v>546</v>
+        <v>534</v>
       </c>
       <c r="C17" s="13" t="s">
         <v>4</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>547</v>
+        <v>535</v>
       </c>
       <c r="E17" s="12" t="s">
         <v>20</v>
@@ -7802,13 +7823,13 @@
     <row r="18" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4"/>
       <c r="B18" s="4" t="s">
-        <v>550</v>
+        <v>538</v>
       </c>
       <c r="C18" s="13" t="s">
         <v>4</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>551</v>
+        <v>539</v>
       </c>
       <c r="E18" s="12" t="s">
         <v>20</v>
@@ -7817,7 +7838,7 @@
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4"/>
       <c r="B19" s="4" t="s">
-        <v>552</v>
+        <v>540</v>
       </c>
       <c r="C19" s="13" t="s">
         <v>4</v>
@@ -7827,83 +7848,83 @@
         <v>20</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="10" t="s">
+    <row r="20" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4"/>
+      <c r="B20" s="4" t="s">
+        <v>555</v>
+      </c>
+      <c r="C20" s="13" t="s">
+        <v>4</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>556</v>
+      </c>
+      <c r="E20" s="12" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B20" s="10"/>
-      <c r="C20" s="10"/>
-      <c r="D20" s="10"/>
-    </row>
-    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4"/>
-      <c r="B21" s="4" t="s">
-        <v>559</v>
-      </c>
-      <c r="C21" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="D21" s="4" t="s">
-        <v>560</v>
-      </c>
-      <c r="E21" s="12" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B21" s="10"/>
+      <c r="C21" s="10"/>
+      <c r="D21" s="10"/>
+    </row>
+    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4"/>
       <c r="B22" s="4" t="s">
-        <v>569</v>
+        <v>561</v>
       </c>
       <c r="C22" s="13" t="s">
         <v>4</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>570</v>
+        <v>562</v>
       </c>
       <c r="E22" s="12" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4"/>
       <c r="B23" s="4" t="s">
-        <v>587</v>
+        <v>571</v>
       </c>
       <c r="C23" s="13" t="s">
         <v>4</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>588</v>
+        <v>572</v>
       </c>
       <c r="E23" s="12" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="10" t="s">
+    <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4"/>
+      <c r="B24" s="4" t="s">
+        <v>589</v>
+      </c>
+      <c r="C24" s="13" t="s">
+        <v>4</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>590</v>
+      </c>
+      <c r="E24" s="12" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="B24" s="10"/>
-      <c r="C24" s="10"/>
-      <c r="D24" s="10"/>
-    </row>
-    <row r="25" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="4"/>
-      <c r="B25" s="4" t="s">
-        <v>593</v>
-      </c>
-      <c r="C25" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="D25" s="4" t="s">
-        <v>594</v>
-      </c>
-      <c r="E25" s="12" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="147" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B25" s="10"/>
+      <c r="C25" s="10"/>
+      <c r="D25" s="10"/>
+    </row>
+    <row r="26" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4"/>
       <c r="B26" s="4" t="s">
         <v>595</v>
@@ -7918,7 +7939,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="147" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4"/>
       <c r="B27" s="4" t="s">
         <v>597</v>
@@ -7933,7 +7954,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4"/>
       <c r="B28" s="4" t="s">
         <v>599</v>
@@ -7948,7 +7969,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4"/>
       <c r="B29" s="4" t="s">
         <v>601</v>
@@ -7971,7 +7992,9 @@
       <c r="C30" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="D30" s="4"/>
+      <c r="D30" s="4" t="s">
+        <v>604</v>
+      </c>
       <c r="E30" s="12" t="s">
         <v>22</v>
       </c>
@@ -7979,7 +8002,7 @@
     <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4"/>
       <c r="B31" s="4" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="C31" s="13" t="s">
         <v>4</v>
@@ -7989,15 +8012,28 @@
         <v>22</v>
       </c>
     </row>
+    <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="4"/>
+      <c r="B32" s="4" t="s">
+        <v>606</v>
+      </c>
+      <c r="C32" s="13" t="s">
+        <v>4</v>
+      </c>
+      <c r="D32" s="4"/>
+      <c r="E32" s="12" t="s">
+        <v>22</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D31"/>
+  <autoFilter ref="A1:D32"/>
   <mergeCells count="6">
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A5:D5"/>
     <mergeCell ref="A7:D7"/>
     <mergeCell ref="A11:D11"/>
-    <mergeCell ref="A20:D20"/>
-    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A21:D21"/>
+    <mergeCell ref="A25:D25"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Redirect map: send old addresses Google still shows to the right page
Pulled every tonygreenberg.com address with Search Console impressions in
the last 16 months (429) and checked each against a production build: 91
ended in a 404, including the old About page
(/transforming-industries-and-perceptions-tonyg/, 80 clicks) and 18 old
WordPress-era essay addresses. Live shows its own 404 page for all of them.

- src/lib/content/search-console-redirects.ts (read by next.config.ts):
  essays matched by title, About, 4 moved pages, old category/tag/paging
  addresses to their category or /blog. All 308, at most 2 hops.
- Result: 409 of 429 end on a working page, 3 external on purpose, 17
  stay 404 on purpose (404 on live too, or documented deferrals).
- scripts/check-search-console-urls.ts re-runs the check (for cutover).
- Phase 12 redirect-map item checked off; inventory and docs updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Migration-Status-Report.xlsx
+++ b/Migration-Status-Report.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Remaining Work" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Full Detail'!$A$1:$D$325</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Full Detail'!$A$1:$D$326</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Remaining Work'!$A$1:$D$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -639,15 +639,15 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$325,$A5,'Full Detail'!$C$2:$C$325,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A5,'Full Detail'!$C$2:$C$326,"Done")</f>
         <v/>
       </c>
       <c r="C5" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$325,$A5,'Full Detail'!$C$2:$C$325,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A5,'Full Detail'!$C$2:$C$326,"Remaining")</f>
         <v/>
       </c>
       <c r="D5" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$325,$A5,'Full Detail'!$C$2:$C$325,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A5,'Full Detail'!$C$2:$C$326,"Deferred")</f>
         <v/>
       </c>
       <c r="E5" s="5">
@@ -666,15 +666,15 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$325,$A6,'Full Detail'!$C$2:$C$325,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A6,'Full Detail'!$C$2:$C$326,"Done")</f>
         <v/>
       </c>
       <c r="C6" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$325,$A6,'Full Detail'!$C$2:$C$325,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A6,'Full Detail'!$C$2:$C$326,"Remaining")</f>
         <v/>
       </c>
       <c r="D6" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$325,$A6,'Full Detail'!$C$2:$C$325,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A6,'Full Detail'!$C$2:$C$326,"Deferred")</f>
         <v/>
       </c>
       <c r="E6" s="5">
@@ -693,15 +693,15 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$325,$A7,'Full Detail'!$C$2:$C$325,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A7,'Full Detail'!$C$2:$C$326,"Done")</f>
         <v/>
       </c>
       <c r="C7" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$325,$A7,'Full Detail'!$C$2:$C$325,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A7,'Full Detail'!$C$2:$C$326,"Remaining")</f>
         <v/>
       </c>
       <c r="D7" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$325,$A7,'Full Detail'!$C$2:$C$325,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A7,'Full Detail'!$C$2:$C$326,"Deferred")</f>
         <v/>
       </c>
       <c r="E7" s="5">
@@ -720,15 +720,15 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$325,$A8,'Full Detail'!$C$2:$C$325,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A8,'Full Detail'!$C$2:$C$326,"Done")</f>
         <v/>
       </c>
       <c r="C8" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$325,$A8,'Full Detail'!$C$2:$C$325,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A8,'Full Detail'!$C$2:$C$326,"Remaining")</f>
         <v/>
       </c>
       <c r="D8" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$325,$A8,'Full Detail'!$C$2:$C$325,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A8,'Full Detail'!$C$2:$C$326,"Deferred")</f>
         <v/>
       </c>
       <c r="E8" s="5">
@@ -747,15 +747,15 @@
         </is>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$325,$A9,'Full Detail'!$C$2:$C$325,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A9,'Full Detail'!$C$2:$C$326,"Done")</f>
         <v/>
       </c>
       <c r="C9" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$325,$A9,'Full Detail'!$C$2:$C$325,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A9,'Full Detail'!$C$2:$C$326,"Remaining")</f>
         <v/>
       </c>
       <c r="D9" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$325,$A9,'Full Detail'!$C$2:$C$325,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A9,'Full Detail'!$C$2:$C$326,"Deferred")</f>
         <v/>
       </c>
       <c r="E9" s="5">
@@ -774,15 +774,15 @@
         </is>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$325,$A10,'Full Detail'!$C$2:$C$325,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A10,'Full Detail'!$C$2:$C$326,"Done")</f>
         <v/>
       </c>
       <c r="C10" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$325,$A10,'Full Detail'!$C$2:$C$325,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A10,'Full Detail'!$C$2:$C$326,"Remaining")</f>
         <v/>
       </c>
       <c r="D10" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$325,$A10,'Full Detail'!$C$2:$C$325,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A10,'Full Detail'!$C$2:$C$326,"Deferred")</f>
         <v/>
       </c>
       <c r="E10" s="5">
@@ -801,15 +801,15 @@
         </is>
       </c>
       <c r="B11" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$325,$A11,'Full Detail'!$C$2:$C$325,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A11,'Full Detail'!$C$2:$C$326,"Done")</f>
         <v/>
       </c>
       <c r="C11" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$325,$A11,'Full Detail'!$C$2:$C$325,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A11,'Full Detail'!$C$2:$C$326,"Remaining")</f>
         <v/>
       </c>
       <c r="D11" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$325,$A11,'Full Detail'!$C$2:$C$325,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A11,'Full Detail'!$C$2:$C$326,"Deferred")</f>
         <v/>
       </c>
       <c r="E11" s="5">
@@ -828,15 +828,15 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$325,$A12,'Full Detail'!$C$2:$C$325,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A12,'Full Detail'!$C$2:$C$326,"Done")</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$325,$A12,'Full Detail'!$C$2:$C$325,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A12,'Full Detail'!$C$2:$C$326,"Remaining")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$325,$A12,'Full Detail'!$C$2:$C$325,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A12,'Full Detail'!$C$2:$C$326,"Deferred")</f>
         <v/>
       </c>
       <c r="E12" s="5">
@@ -855,15 +855,15 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$325,$A13,'Full Detail'!$C$2:$C$325,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A13,'Full Detail'!$C$2:$C$326,"Done")</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$325,$A13,'Full Detail'!$C$2:$C$325,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A13,'Full Detail'!$C$2:$C$326,"Remaining")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$325,$A13,'Full Detail'!$C$2:$C$325,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A13,'Full Detail'!$C$2:$C$326,"Deferred")</f>
         <v/>
       </c>
       <c r="E13" s="5">
@@ -882,15 +882,15 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$325,$A14,'Full Detail'!$C$2:$C$325,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A14,'Full Detail'!$C$2:$C$326,"Done")</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$325,$A14,'Full Detail'!$C$2:$C$325,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A14,'Full Detail'!$C$2:$C$326,"Remaining")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$325,$A14,'Full Detail'!$C$2:$C$325,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A14,'Full Detail'!$C$2:$C$326,"Deferred")</f>
         <v/>
       </c>
       <c r="E14" s="5">
@@ -909,15 +909,15 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$325,$A15,'Full Detail'!$C$2:$C$325,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A15,'Full Detail'!$C$2:$C$326,"Done")</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$325,$A15,'Full Detail'!$C$2:$C$325,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A15,'Full Detail'!$C$2:$C$326,"Remaining")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$325,$A15,'Full Detail'!$C$2:$C$325,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A15,'Full Detail'!$C$2:$C$326,"Deferred")</f>
         <v/>
       </c>
       <c r="E15" s="5">
@@ -936,15 +936,15 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$325,$A16,'Full Detail'!$C$2:$C$325,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A16,'Full Detail'!$C$2:$C$326,"Done")</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$325,$A16,'Full Detail'!$C$2:$C$325,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A16,'Full Detail'!$C$2:$C$326,"Remaining")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$325,$A16,'Full Detail'!$C$2:$C$325,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A16,'Full Detail'!$C$2:$C$326,"Deferred")</f>
         <v/>
       </c>
       <c r="E16" s="5">
@@ -963,15 +963,15 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$325,$A17,'Full Detail'!$C$2:$C$325,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A17,'Full Detail'!$C$2:$C$326,"Done")</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$325,$A17,'Full Detail'!$C$2:$C$325,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A17,'Full Detail'!$C$2:$C$326,"Remaining")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$325,$A17,'Full Detail'!$C$2:$C$325,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A17,'Full Detail'!$C$2:$C$326,"Deferred")</f>
         <v/>
       </c>
       <c r="E17" s="5">
@@ -990,15 +990,15 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$325,$A18,'Full Detail'!$C$2:$C$325,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A18,'Full Detail'!$C$2:$C$326,"Done")</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$325,$A18,'Full Detail'!$C$2:$C$325,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A18,'Full Detail'!$C$2:$C$326,"Remaining")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$325,$A18,'Full Detail'!$C$2:$C$325,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A18,'Full Detail'!$C$2:$C$326,"Deferred")</f>
         <v/>
       </c>
       <c r="E18" s="5">
@@ -1017,15 +1017,15 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$325,$A19,'Full Detail'!$C$2:$C$325,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A19,'Full Detail'!$C$2:$C$326,"Done")</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$325,$A19,'Full Detail'!$C$2:$C$325,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A19,'Full Detail'!$C$2:$C$326,"Remaining")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$325,$A19,'Full Detail'!$C$2:$C$325,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A19,'Full Detail'!$C$2:$C$326,"Deferred")</f>
         <v/>
       </c>
       <c r="E19" s="5">
@@ -1075,7 +1075,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E325"/>
+  <dimension ref="A1:E326"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -6929,7 +6929,7 @@
       <c r="A265" s="4" t="n"/>
       <c r="B265" s="4" t="inlineStr">
         <is>
-          <t>/path/:archetype (src/app/path/[archetype]/page.tsx)</t>
+          <t>Build the full Manus/legacy-URL → Next.js-URL 301 redirect map (next.config.ts redirects() or Sanity redirect documents)</t>
         </is>
       </c>
       <c r="C265" s="13" t="inlineStr">
@@ -6939,7 +6939,7 @@
       </c>
       <c r="D265" s="4" t="inlineStr">
         <is>
-          <t>per-archetype landing page for /assessment's Builder/Crusader/Investor result, reusing lib/content/archetypes.ts. Real content ported in full (top-5 essential-reading list per archetype via allPostsForArchiveQuery, real PathSubscribeForm posting to /api/subscribe, AUTHORITY_ITEMS strip). Real bug fixed vs. legacy: replaced a hand-rolled inline-styled "Path not found" div with a real notFound() (this route's generateStaticParams only ever produces the 3 real keys). Verified live: all 3 archetype routes 200 OK, typecheck/lint clean.</t>
+          <t>hard QA gate, nothing proceeds to DNS cutover until this is complete and tested. First real pass done: extracted all 197 real path= routes from legacy's App.tsx router (not guessed — the actual route table), diffed against this app's real current routes (find src/app -maxdepth 1 -name page.tsx) + next.config.ts's existing redirect sources, normalizing :param/[param] syntax to compare like-for-like. Started at 41 real gaps, closed 10 with new redirects: /attention-theft/{blocker-finder,legal,report,weapons} (legacy registered both a bare AND a /attention-theft/-nested path for each, only the bare ones had redirects before), /find-my-car → /find-my, /the-index → /search (matching the fix already applied to other pages' dead links to it), /supplier-intake-long (bare) + /vendor-intake + /vendor-intake-long (+/:token) → the same real ramprate.com/biochain/supplier-intake destination the token'd path already redirected to, and /spamtoast + /youve-been-reported → / (the live half of legacy's "report a spammer" confrontation flow — a fake IP-fingerprinting/countdown-timer page; the other half, ReportSpammer.tsx, was already a documented drop in Phase 4, this is the same call for its sequel). 21 of the remaining 31 gaps need no redirect — they're /admin/*//analytics//edit/frqncy (internal tools never meant for public discovery) or already-documented intentional defers from Phase 4/7/10 (/clock-keeper-part-2, /ecosystem-map, /friend-gate, /friend-survey/:token, /medicine-sequencing, /m</t>
         </is>
       </c>
       <c r="E265" s="14" t="inlineStr">
@@ -6952,7 +6952,7 @@
       <c r="A266" s="4" t="n"/>
       <c r="B266" s="4" t="inlineStr">
         <is>
-          <t>/my-journey (src/app/my-journey/page.tsx + components/assessments/my-journey-dashboard.tsx)</t>
+          <t>/path/:archetype (src/app/path/[archetype]/page.tsx)</t>
         </is>
       </c>
       <c r="C266" s="13" t="inlineStr">
@@ -6962,7 +6962,7 @@
       </c>
       <c r="D266" s="4" t="inlineStr">
         <is>
-          <t>"My Journey Dashboard," real grid/timeline views across all 28 JOURNEY_MAP experiences, category/status filters, phase progress ring, recommended-next card, using the same real useJourneyProgress/JOURNEY_MAP completion tracking every "Find Your X" quiz already writes to (not the narrower tg_assessment_results cookie built for /self-portrait). Legacy's per-quiz scored-result caching (RESULT_KEYS, feeding a mini radar chart) was not ported — no quiz in this migration writes that data either, same honest-degradation call already made for /self-portrait's own composite radar. Fixed a real legacy dead link (/ecosystem-map, a still-unbuilt page) to /self-portrait. Verified live: 200 OK, real content confirmed, typecheck/lint clean.</t>
+          <t>per-archetype landing page for /assessment's Builder/Crusader/Investor result, reusing lib/content/archetypes.ts. Real content ported in full (top-5 essential-reading list per archetype via allPostsForArchiveQuery, real PathSubscribeForm posting to /api/subscribe, AUTHORITY_ITEMS strip). Real bug fixed vs. legacy: replaced a hand-rolled inline-styled "Path not found" div with a real notFound() (this route's generateStaticParams only ever produces the 3 real keys). Verified live: all 3 archetype routes 200 OK, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E266" s="14" t="inlineStr">
@@ -6975,7 +6975,7 @@
       <c r="A267" s="4" t="n"/>
       <c r="B267" s="4" t="inlineStr">
         <is>
-          <t>/the-open-door (src/app/the-open-door/page.tsx)</t>
+          <t>/my-journey (src/app/my-journey/page.tsx + components/assessments/my-journey-dashboard.tsx)</t>
         </is>
       </c>
       <c r="C267" s="13" t="inlineStr">
@@ -6985,7 +6985,7 @@
       </c>
       <c r="D267" s="4" t="inlineStr">
         <is>
-          <t>real press/credibility content: all 10 "Magic Genie" client-pitch prompts (real named targets — Marco Argenti/Goldman Sachs, Adam Smith/Disney, etc.), 18 real client testimonials, all 8 explicitly-labeled satirical "parody" quotes (kept with disclaimers, not presented as real). Real overlap found and reconciled: this page's publications/speaking/podcasts arrays substantially duplicate the already-shipped /published's fuller bibliography — kept only what /published doesn't cover (Forbes + Business Insider bylines, the Clinton Global Initiative keynote, 4 of 5 podcast appearances) and cross-linked to /published for the rest, same reconciliation pattern as /assessments vs /find-my. Real bugs fixed: 3 genie/keynote links pointed externally at tonygreenberg.com/&lt;slug&gt; for posts that are real internal posts in this migration — relinked to /blog/psychedelics-could-become-extractive-capitalism, /blog/boiling-the-human-summit-harvard-kurzweil, /blog/return-on-investment-going-green-going-green-2 (all verified 200); a bare self-link to tonygreenberg.com remapped to /. Ships as a pure Server Component (legacy's FadeIn/Section/editorial-component dependencies don't exist here and weren't needed). Verified live: 200 OK, real content in raw SSR HTML, typecheck/lint clean.</t>
+          <t>"My Journey Dashboard," real grid/timeline views across all 28 JOURNEY_MAP experiences, category/status filters, phase progress ring, recommended-next card, using the same real useJourneyProgress/JOURNEY_MAP completion tracking every "Find Your X" quiz already writes to (not the narrower tg_assessment_results cookie built for /self-portrait). Legacy's per-quiz scored-result caching (RESULT_KEYS, feeding a mini radar chart) was not ported — no quiz in this migration writes that data either, same honest-degradation call already made for /self-portrait's own composite radar. Fixed a real legacy dead link (/ecosystem-map, a still-unbuilt page) to /self-portrait. Verified live: 200 OK, real content confirmed, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E267" s="14" t="inlineStr">
@@ -6998,7 +6998,7 @@
       <c r="A268" s="4" t="n"/>
       <c r="B268" s="4" t="inlineStr">
         <is>
-          <t>Homepage "Recent Updates" band (2026-09-29)</t>
+          <t>/the-open-door (src/app/the-open-door/page.tsx)</t>
         </is>
       </c>
       <c r="C268" s="13" t="inlineStr">
@@ -7008,7 +7008,7 @@
       </c>
       <c r="D268" s="4" t="inlineStr">
         <is>
-          <t>on the live site (a newer Blog.tsx than _legacy-manus-app/, so rebuilt from the live page's markup), replacing the older "Latest Thinking" pair. Found while doing it: two live essays are missing from Sanity, the-tollbooth-and-the-alternative (Aug 18, 2026, the live site's newest) and what-quest-could-fix. Both were published on live after the legacy snapshot and need importing.</t>
+          <t>real press/credibility content: all 10 "Magic Genie" client-pitch prompts (real named targets — Marco Argenti/Goldman Sachs, Adam Smith/Disney, etc.), 18 real client testimonials, all 8 explicitly-labeled satirical "parody" quotes (kept with disclaimers, not presented as real). Real overlap found and reconciled: this page's publications/speaking/podcasts arrays substantially duplicate the already-shipped /published's fuller bibliography — kept only what /published doesn't cover (Forbes + Business Insider bylines, the Clinton Global Initiative keynote, 4 of 5 podcast appearances) and cross-linked to /published for the rest, same reconciliation pattern as /assessments vs /find-my. Real bugs fixed: 3 genie/keynote links pointed externally at tonygreenberg.com/&lt;slug&gt; for posts that are real internal posts in this migration — relinked to /blog/psychedelics-could-become-extractive-capitalism, /blog/boiling-the-human-summit-harvard-kurzweil, /blog/return-on-investment-going-green-going-green-2 (all verified 200); a bare self-link to tonygreenberg.com remapped to /. Ships as a pure Server Component (legacy's FadeIn/Section/editorial-component dependencies don't exist here and weren't needed). Verified live: 200 OK, real content in raw SSR HTML, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E268" s="14" t="inlineStr">
@@ -7021,7 +7021,7 @@
       <c r="A269" s="4" t="n"/>
       <c r="B269" s="4" t="inlineStr">
         <is>
-          <t>Re-sync the legacy reference</t>
+          <t>Homepage "Recent Updates" band (2026-09-29)</t>
         </is>
       </c>
       <c r="C269" s="13" t="inlineStr">
@@ -7031,7 +7031,7 @@
       </c>
       <c r="D269" s="4" t="inlineStr">
         <is>
-          <t>_legacy-manus-app/ is older than what's live (Recent Updates proves it), so visual diffs should be against the live site, not only that folder. Closed 2026-10-08: done the way this item suggests: every comparison since 2026-10-01 is against the live site itself (163 pages + 121 posts on 2026-10-01, 188 pages on 2026-10-07, 18 redesigned pages on 2026-10-08), with _legacy-manus-app/ used only as the code reference.</t>
+          <t>on the live site (a newer Blog.tsx than _legacy-manus-app/, so rebuilt from the live page's markup), replacing the older "Latest Thinking" pair. Found while doing it: two live essays are missing from Sanity, the-tollbooth-and-the-alternative (Aug 18, 2026, the live site's newest) and what-quest-could-fix. Both were published on live after the legacy snapshot and need importing.</t>
         </is>
       </c>
       <c r="E269" s="14" t="inlineStr">
@@ -7044,7 +7044,7 @@
       <c r="A270" s="4" t="n"/>
       <c r="B270" s="4" t="inlineStr">
         <is>
-          <t>Visual diff pass: every ported page vs</t>
+          <t>Re-sync the legacy reference</t>
         </is>
       </c>
       <c r="C270" s="13" t="inlineStr">
@@ -7054,7 +7054,7 @@
       </c>
       <c r="D270" s="4" t="inlineStr">
         <is>
-          <t>legacy page Closed 2026-10-08: covered by the live-site sweeps above (screenshots and measured title/label/spacing per page, see the 2026-10-01, 10-02, 10-07 and 10-08 entries in this phase). Remaining differences are listed as decisions (Cormorant titles, /find-my header) or deliberate (CONTRIBUTING rule 20).</t>
+          <t>_legacy-manus-app/ is older than what's live (Recent Updates proves it), so visual diffs should be against the live site, not only that folder. Closed 2026-10-08: done the way this item suggests: every comparison since 2026-10-01 is against the live site itself (163 pages + 121 posts on 2026-10-01, 188 pages on 2026-10-07, 18 redesigned pages on 2026-10-08), with _legacy-manus-app/ used only as the code reference.</t>
         </is>
       </c>
       <c r="E270" s="14" t="inlineStr">
@@ -7067,7 +7067,7 @@
       <c r="A271" s="4" t="n"/>
       <c r="B271" s="4" t="inlineStr">
         <is>
-          <t>Padding / spacing on the story pages matched to live (2026-10-01)</t>
+          <t>Visual diff pass: every ported page vs</t>
         </is>
       </c>
       <c r="C271" s="13" t="inlineStr">
@@ -7077,7 +7077,7 @@
       </c>
       <c r="D271" s="4" t="inlineStr">
         <is>
-          <t>Measured margins, text column and spacing on 31 pages, live vs a production build, at 375px and 1280px. The "door" story pages were the clear mismatch: live's text column is ~546px (ours was 720px), 20px side margins on phones / 40px on desktop, body text 19px/1.8 on phones and 18px/1.85 on desktop (ours 16px/1.5). Fixed on /the-body, /engine-room, /under-nda, /the-nightstand, /the-web, /the-territory, /about, /intel (Intel uses live's 16.8px/1.9; About's hero line 480px max, 18.4px/1.8). Re-measured: all 8 match live to within 2px (About's column 28px narrower), no sideways scroll at 375px.</t>
+          <t>legacy page Closed 2026-10-08: covered by the live-site sweeps above (screenshots and measured title/label/spacing per page, see the 2026-10-01, 10-02, 10-07 and 10-08 entries in this phase). Remaining differences are listed as decisions (Cormorant titles, /find-my header) or deliberate (CONTRIBUTING rule 20).</t>
         </is>
       </c>
       <c r="E271" s="14" t="inlineStr">
@@ -7090,7 +7090,7 @@
       <c r="A272" s="4" t="n"/>
       <c r="B272" s="4" t="inlineStr">
         <is>
-          <t>Header-to-title spacing re-checked (2026-10-02)</t>
+          <t>Padding / spacing on the story pages matched to live (2026-10-01)</t>
         </is>
       </c>
       <c r="C272" s="13" t="inlineStr">
@@ -7100,7 +7100,7 @@
       </c>
       <c r="D272" s="4" t="inlineStr">
         <is>
-          <t>The 2026-10-01 note compared different things: live's header wasn't measured (it showed 0), so "96px vs 168px" was really 161px vs 168px from the top of the page. Measured again from the top of the page, live vs a production build, at 375px and 1280px: most pages were already within 10px. Fixed the real gaps: /the-open-door (now live's dark centered hero band, 56px title, 546px text column; title was 72px too high), /start-here (live's 48px/96px top padding; 25px too high on desktop), /invest and /engage (label spacing and live's 32px/51px title; /invest's desktop title was 36px), /impact-dashboard on phones (card edge to edge under the header like live; title was 89px too low). Re-measured: all within 8px of live, no sideways scroll at 375px, no JS errors.</t>
+          <t>Measured margins, text column and spacing on 31 pages, live vs a production build, at 375px and 1280px. The "door" story pages were the clear mismatch: live's text column is ~546px (ours was 720px), 20px side margins on phones / 40px on desktop, body text 19px/1.8 on phones and 18px/1.85 on desktop (ours 16px/1.5). Fixed on /the-body, /engine-room, /under-nda, /the-nightstand, /the-web, /the-territory, /about, /intel (Intel uses live's 16.8px/1.9; About's hero line 480px max, 18.4px/1.8). Re-measured: all 8 match live to within 2px (About's column 28px narrower), no sideways scroll at 375px.</t>
         </is>
       </c>
       <c r="E272" s="14" t="inlineStr">
@@ -7113,7 +7113,7 @@
       <c r="A273" s="4" t="n"/>
       <c r="B273" s="4" t="inlineStr">
         <is>
-          <t>HumanOS headings in capitals like live (2026-10-02, owner said yes)</t>
+          <t>Header-to-title spacing re-checked (2026-10-02)</t>
         </is>
       </c>
       <c r="C273" s="13" t="inlineStr">
@@ -7123,7 +7123,7 @@
       </c>
       <c r="D273" s="4" t="inlineStr">
         <is>
-          <t>the 4 headings live capitalises on /humanos (title, "Are you a Maximizer...", "Take the Diagnostic", "The Diagnostic") get uppercase; the words are unchanged. The subpages already matched.</t>
+          <t>The 2026-10-01 note compared different things: live's header wasn't measured (it showed 0), so "96px vs 168px" was really 161px vs 168px from the top of the page. Measured again from the top of the page, live vs a production build, at 375px and 1280px: most pages were already within 10px. Fixed the real gaps: /the-open-door (now live's dark centered hero band, 56px title, 546px text column; title was 72px too high), /start-here (live's 48px/96px top padding; 25px too high on desktop), /invest and /engage (label spacing and live's 32px/51px title; /invest's desktop title was 36px), /impact-dashboard on phones (card edge to edge under the header like live; title was 89px too low). Re-measured: all within 8px of live, no sideways scroll at 375px, no JS errors.</t>
         </is>
       </c>
       <c r="E273" s="14" t="inlineStr">
@@ -7136,7 +7136,7 @@
       <c r="A274" s="4" t="n"/>
       <c r="B274" s="4" t="inlineStr">
         <is>
-          <t>More layout gaps matched to live (2026-10-02)</t>
+          <t>HumanOS headings in capitals like live (2026-10-02, owner said yes)</t>
         </is>
       </c>
       <c r="C274" s="13" t="inlineStr">
@@ -7146,7 +7146,7 @@
       </c>
       <c r="D274" s="4" t="inlineStr">
         <is>
-          <t>/series (live's centered 546px column, and a bug fixed: every card kept an empty 240px picture column, squeezing the text; live's per-series picture is one generic placeholder on the Manus proxy, so not copied), /humanos (middle section 900px like live), homepage desktop widths (hero text 804px, Four Doors 1000px, Editor's Picks 1168px, GemSpark edge, section title sizes; live's /blog now shows the homepage), /find-my (photo undimmed and plain background, like live; our site header kept). Re-measured: headings within 3px (/series) to 20px (homepage) of live, no sideways scroll, no JS errors. Note: live's "New here?" tour bar sits over its header and doesn't move the page, so it doesn't affect these numbers.</t>
+          <t>the 4 headings live capitalises on /humanos (title, "Are you a Maximizer...", "Take the Diagnostic", "The Diagnostic") get uppercase; the words are unchanged. The subpages already matched.</t>
         </is>
       </c>
       <c r="E274" s="14" t="inlineStr">
@@ -7159,7 +7159,7 @@
       <c r="A275" s="4" t="n"/>
       <c r="B275" s="4" t="inlineStr">
         <is>
-          <t>Full sweep vs live (2026-10-02)</t>
+          <t>More layout gaps matched to live (2026-10-02)</t>
         </is>
       </c>
       <c r="C275" s="13" t="inlineStr">
@@ -7169,7 +7169,7 @@
       </c>
       <c r="D275" s="4" t="inlineStr">
         <is>
-          <t>142 pages (every non-blog page, 3 of each templated set) at 375px and 1280px, title position, text column, title size. Fixed the shared causes: BrewSoul (live wraps most pages in its frame twice, so a second 52px offset plus the category badge; the landing, cities, directory and quiz pages have neither: src/components/brewsoul/brewsoul-main.tsx; intro paragraphs uncapped like live; 38px titles), Kava (live's extra 52px offset), /the-body, /the-nightstand, /the-web (405px top photo like live), the 6 peptide pages (live's 768/896px intro column), /journeys, /pick-up-the-phone, /published, /ecosystem (546px story column and live's text size). Re-measured: 110 of 120 within 40px / 60px of live.</t>
+          <t>/series (live's centered 546px column, and a bug fixed: every card kept an empty 240px picture column, squeezing the text; live's per-series picture is one generic placeholder on the Manus proxy, so not copied), /humanos (middle section 900px like live), homepage desktop widths (hero text 804px, Four Doors 1000px, Editor's Picks 1168px, GemSpark edge, section title sizes; live's /blog now shows the homepage), /find-my (photo undimmed and plain background, like live; our site header kept). Re-measured: headings within 3px (/series) to 20px (homepage) of live, no sideways scroll, no JS errors. Note: live's "New here?" tour bar sits over its header and doesn't move the page, so it doesn't affect these numbers.</t>
         </is>
       </c>
       <c r="E275" s="14" t="inlineStr">
@@ -7182,7 +7182,7 @@
       <c r="A276" s="4" t="n"/>
       <c r="B276" s="4" t="inlineStr">
         <is>
-          <t>Sweep leftovers fixed (2026-10-06)</t>
+          <t>Full sweep vs live (2026-10-02)</t>
         </is>
       </c>
       <c r="C276" s="13" t="inlineStr">
@@ -7192,7 +7192,7 @@
       </c>
       <c r="D276" s="4" t="inlineStr">
         <is>
-          <t>Ported legacy's exact title sizes, margins and column widths. Measured live vs a production build at 375px and 1280px (H1 distance from the top, H1 size, intro and table widths). Now within 8px and the same title size on /published, /brewsoul/first-sip, /brewsoul/home, /brewsoul/chains (intro 912px like live), /brewsoul/browse, /brewsoul/directory (3-column 952px grid like live), /brewsoul and /brewsoul/quiz (intro 520px), /amplifier (546px column), /diamond-cut, /speaking, /living-declaration, /spirits, /protecting-your-business (tables 730px), and the 5 HumanOS subpages (titles smaller like live, 752px column). No sideways scroll at 375px. Left on purpose: /self-portrait (font matches; our page has a different title and no back link, so it sits 23-57px higher), BrewSoul pages 3-6px off (the shared journey bar row), and the different-layout pages /dharma-finder, /grant-study, /search, /quiz_25q, /soulscore. Also: /brewsoul/quiz rebuilt as a step registry (src/components/brewsoul/brewsoul-quiz/: parent + hook/ + components/step-* + data/), same questions, scoring and look; Back/Skip/Retake use lucide icons. New CONTRIBUTING rule 19 (multi-step flows, FydoPartner pattern). brewsoul-welcome-quiz.tsx (/brewsoul) still has the old shape and text arrows.</t>
+          <t>142 pages (every non-blog page, 3 of each templated set) at 375px and 1280px, title position, text column, title size. Fixed the shared causes: BrewSoul (live wraps most pages in its frame twice, so a second 52px offset plus the category badge; the landing, cities, directory and quiz pages have neither: src/components/brewsoul/brewsoul-main.tsx; intro paragraphs uncapped like live; 38px titles), Kava (live's extra 52px offset), /the-body, /the-nightstand, /the-web (405px top photo like live), the 6 peptide pages (live's 768/896px intro column), /journeys, /pick-up-the-phone, /published, /ecosystem (546px story column and live's text size). Re-measured: 110 of 120 within 40px / 60px of live.</t>
         </is>
       </c>
       <c r="E276" s="14" t="inlineStr">
@@ -7205,7 +7205,7 @@
       <c r="A277" s="4" t="n"/>
       <c r="B277" s="4" t="inlineStr">
         <is>
-          <t>Match live's redesigned pages (2026-10-06, owner said go)</t>
+          <t>Sweep leftovers fixed (2026-10-06)</t>
         </is>
       </c>
       <c r="C277" s="13" t="inlineStr">
@@ -7215,7 +7215,7 @@
       </c>
       <c r="D277" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">/self-portrait (live: dark page, progress ring, "N more brushstrokes" lock until 5 assessments), /grant-study and /dharma-finder (live opens straight on question 1, no intro screen), /quiz_25q (live adds a hero picture above the title; rescue it into Sanity first), /search (live: one search box across essays, BrewSoul, peptides, HumanOS, assessments, kava and pages with filter chips). Measure live vs a production build at 375px and 1280px when done. Done 2026-10-06: /grant-study and /dharma-finder open straight on question 1 like live (title block / part header above the first question, live's 546px column, plain page, credit under every question), both rebuilt as step registries (rule 19); measured within 3px of live at the top (dharma's question block within 7px). /quiz_25q's hero rescued into Sanity and placed like live (within 2px). Found and fixed on the way: on the deployed copy /grant-study's answer buttons could not be clicked (the themed page background was fixed z-0, painted over the quiz); ThemedBackground is now -z-10 pointer-events-none (backgrounds unchanged on all 21 pages that use it), and the shared email gate no longer scrolls sideways on phones. Both quizzes clicked through to results in Chrome and Safari. /self-portrait restyled to live (dark page, "The Composite You", progress ring, "N More Brushstrokes Needed" lock until 5 done, live's copy) on our real cookie data; within 3px of live at both widths; tested with 0, 2 and 6 completed. Counts are ours (13 </t>
+          <t>Ported legacy's exact title sizes, margins and column widths. Measured live vs a production build at 375px and 1280px (H1 distance from the top, H1 size, intro and table widths). Now within 8px and the same title size on /published, /brewsoul/first-sip, /brewsoul/home, /brewsoul/chains (intro 912px like live), /brewsoul/browse, /brewsoul/directory (3-column 952px grid like live), /brewsoul and /brewsoul/quiz (intro 520px), /amplifier (546px column), /diamond-cut, /speaking, /living-declaration, /spirits, /protecting-your-business (tables 730px), and the 5 HumanOS subpages (titles smaller like live, 752px column). No sideways scroll at 375px. Left on purpose: /self-portrait (font matches; our page has a different title and no back link, so it sits 23-57px higher), BrewSoul pages 3-6px off (the shared journey bar row), and the different-layout pages /dharma-finder, /grant-study, /search, /quiz_25q, /soulscore. Also: /brewsoul/quiz rebuilt as a step registry (src/components/brewsoul/brewsoul-quiz/: parent + hook/ + components/step-* + data/), same questions, scoring and look; Back/Skip/Retake use lucide icons. New CONTRIBUTING rule 19 (multi-step flows, FydoPartner pattern). brewsoul-welcome-quiz.tsx (/brewsoul) still has the old shape and text arrows.</t>
         </is>
       </c>
       <c r="E277" s="14" t="inlineStr">
@@ -7228,17 +7228,17 @@
       <c r="A278" s="4" t="n"/>
       <c r="B278" s="4" t="inlineStr">
         <is>
-          <t>Still different from live (needs a yes)</t>
-        </is>
-      </c>
-      <c r="C278" s="15" t="inlineStr">
-        <is>
-          <t>Remaining</t>
+          <t>Match live's redesigned pages (2026-10-06, owner said go)</t>
+        </is>
+      </c>
+      <c r="C278" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D278" s="4" t="inlineStr">
         <is>
-          <t>blog posts (done) (done 2026-10-07, see Phase 5); /find-my on live hides the site header. /walk-through is a 404 on live now.</t>
+          <t xml:space="preserve">/self-portrait (live: dark page, progress ring, "N more brushstrokes" lock until 5 assessments), /grant-study and /dharma-finder (live opens straight on question 1, no intro screen), /quiz_25q (live adds a hero picture above the title; rescue it into Sanity first), /search (live: one search box across essays, BrewSoul, peptides, HumanOS, assessments, kava and pages with filter chips). Measure live vs a production build at 375px and 1280px when done. Done 2026-10-06: /grant-study and /dharma-finder open straight on question 1 like live (title block / part header above the first question, live's 546px column, plain page, credit under every question), both rebuilt as step registries (rule 19); measured within 3px of live at the top (dharma's question block within 7px). /quiz_25q's hero rescued into Sanity and placed like live (within 2px). Found and fixed on the way: on the deployed copy /grant-study's answer buttons could not be clicked (the themed page background was fixed z-0, painted over the quiz); ThemedBackground is now -z-10 pointer-events-none (backgrounds unchanged on all 21 pages that use it), and the shared email gate no longer scrolls sideways on phones. Both quizzes clicked through to results in Chrome and Safari. /self-portrait restyled to live (dark page, "The Composite You", progress ring, "N More Brushstrokes Needed" lock until 5 done, live's copy) on our real cookie data; within 3px of live at both widths; tested with 0, 2 and 6 completed. Counts are ours (13 </t>
         </is>
       </c>
       <c r="E278" s="14" t="inlineStr">
@@ -7251,7 +7251,7 @@
       <c r="A279" s="4" t="n"/>
       <c r="B279" s="4" t="inlineStr">
         <is>
-          <t>Design change on live, needs a decision</t>
+          <t>Still different from live (needs a yes)</t>
         </is>
       </c>
       <c r="C279" s="15" t="inlineStr">
@@ -7261,7 +7261,7 @@
       </c>
       <c r="D279" s="4" t="inlineStr">
         <is>
-          <t>live's story pages now use Cormorant Garamond for titles (ours: Playfair Display), a lighter title weight (400 vs our 700), and a red eyebrow label (#8E1E25, wider letter spacing) instead of our gold. A site-wide font swap is a design call, so not done.</t>
+          <t>blog posts (done) (done 2026-10-07, see Phase 5); /find-my on live hides the site header. /walk-through is a 404 on live now.</t>
         </is>
       </c>
       <c r="E279" s="14" t="inlineStr">
@@ -7274,17 +7274,17 @@
       <c r="A280" s="4" t="n"/>
       <c r="B280" s="4" t="inlineStr">
         <is>
-          <t>Link check across all ported pages (no 404s, no broken internal cross-references)</t>
-        </is>
-      </c>
-      <c r="C280" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Design change on live, needs a decision</t>
+        </is>
+      </c>
+      <c r="C280" s="15" t="inlineStr">
+        <is>
+          <t>Remaining</t>
         </is>
       </c>
       <c r="D280" s="4" t="inlineStr">
         <is>
-          <t>First full pass done 2026-09-29 (510 pages crawled from the sitemap plus every internal link, on a production build). Fixed in code: /brewsoul/coffee/…-tarrazú 404 (the route got the id still percent-encoded), 30+ links that went through the /assessments/* redirects, /find-your-me's dead Homeaglow link, the two root-level Iboga essay links, and the dead FauxTony nav item. Fixed as Sanity drafts (scripts/fix-blog-body-links.ts, 14 posts): broken post links, leaked !… placeholder text, Energy Is Money's split author bio, and scraped WordPress furniture ("Share this / Related / You Might Also Like / Copyright", "Show More / Top News", [mc4wp_form]). Left for a decision: /framework's "Ask FauxTony" button, when-healing-becomes-extraction's two links to a Dr. Lee case file that doesn't exist, and the-clock-keeper-chronicles-part-1's link to the deferred /clock-keeper-part-2. Re-run after the drafts are published. 2026-10-01 re-run (local production build, all 498 sitemap URLs load; 440 unique internal links): 5 broken. Fixed as a Sanity draft: molecule-as-mirror-10-what-the-pioneers-know's "Final installment" link pointed at a non-existent part-10 slug (now part 11; live also shows that line twice, kept). Already fixed in a waiting draft: forever-chemicals-... → /blog/psychedelic-readiness-index. Still the 3 known decisions: /fauxtony (from /framework), /clock-keeper-part-2, /blog/the-case-file-dr-samuel-lee. 2026-10-08 re-run (production build, all 497 sitemap pages, 453 unique i</t>
+          <t>live's story pages now use Cormorant Garamond for titles (ours: Playfair Display), a lighter title weight (400 vs our 700), and a red eyebrow label (#8E1E25, wider letter spacing) instead of our gold. A site-wide font swap is a design call, so not done.</t>
         </is>
       </c>
       <c r="E280" s="14" t="inlineStr">
@@ -7297,7 +7297,7 @@
       <c r="A281" s="4" t="n"/>
       <c r="B281" s="4" t="inlineStr">
         <is>
-          <t>Sitemap: no noindex pages (2026-10-08)</t>
+          <t>Link check across all ported pages (no 404s, no broken internal cross-references)</t>
         </is>
       </c>
       <c r="C281" s="13" t="inlineStr">
@@ -7307,7 +7307,7 @@
       </c>
       <c r="D281" s="4" t="inlineStr">
         <is>
-          <t>the password-locked /blog/you-are-the-moat was in the sitemap while telling Google not to index it (a Search Console sitemap warning). Gated posts and posts that redirect are now left out (src/app/sitemap.ts); all 497 sitemap addresses return 200 with a matching canonical and no noindex. The 82 warnings Search Console shows are for the old live sitemap, so re-check them after cutover.</t>
+          <t>First full pass done 2026-09-29 (510 pages crawled from the sitemap plus every internal link, on a production build). Fixed in code: /brewsoul/coffee/…-tarrazú 404 (the route got the id still percent-encoded), 30+ links that went through the /assessments/* redirects, /find-your-me's dead Homeaglow link, the two root-level Iboga essay links, and the dead FauxTony nav item. Fixed as Sanity drafts (scripts/fix-blog-body-links.ts, 14 posts): broken post links, leaked !… placeholder text, Energy Is Money's split author bio, and scraped WordPress furniture ("Share this / Related / You Might Also Like / Copyright", "Show More / Top News", [mc4wp_form]). Left for a decision: /framework's "Ask FauxTony" button, when-healing-becomes-extraction's two links to a Dr. Lee case file that doesn't exist, and the-clock-keeper-chronicles-part-1's link to the deferred /clock-keeper-part-2. Re-run after the drafts are published. 2026-10-01 re-run (local production build, all 498 sitemap URLs load; 440 unique internal links): 5 broken. Fixed as a Sanity draft: molecule-as-mirror-10-what-the-pioneers-know's "Final installment" link pointed at a non-existent part-10 slug (now part 11; live also shows that line twice, kept). Already fixed in a waiting draft: forever-chemicals-... → /blog/psychedelic-readiness-index. Still the 3 known decisions: /fauxtony (from /framework), /clock-keeper-part-2, /blog/the-case-file-dr-samuel-lee. 2026-10-08 re-run (production build, all 497 sitemap pages, 453 unique i</t>
         </is>
       </c>
       <c r="E281" s="14" t="inlineStr">
@@ -7320,17 +7320,17 @@
       <c r="A282" s="4" t="n"/>
       <c r="B282" s="4" t="inlineStr">
         <is>
-          <t>Lighthouse pass (performance/accessibility/SEO) on top 20 pages by traffic 2026-09-30, 20 key pages (no traffic data yet), local production …</t>
-        </is>
-      </c>
-      <c r="C282" s="15" t="inlineStr">
-        <is>
-          <t>Remaining</t>
+          <t>Sitemap: no noindex pages (2026-10-08)</t>
+        </is>
+      </c>
+      <c r="C282" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D282" s="4" t="inlineStr">
         <is>
-          <t>build, mobile: averages performance 87, accessibility 99→100, best practices 100, SEO 92→100, CLS 0 everywhere. Fixed: public/robots.txt had an LLMs: line (not a real directive) that made Google treat the whole file as invalid, now a comment; h3/h4 headings skipping a level on /assessments, /kava, /peptide-watch (same look, right tag); the Kava and /attention-theft back-arrow links had no accessible name on phones; two small phone-width contrast misses. Left: performance is local-machine only (±10-15 points, see CONTRIBUTING.md); the slowest were / 76 (LCP 5.2 s), /psychedelic-readiness-index 82, /iboga-ibogaine 83. Re-run against the Netlify deploy before launch. 2026-10-06 re-run against the Netlify deploy (14 key pages, mobile): accessibility 100 and CLS 0 on every page, SEO clean (only the expected netlify.app noindex), performance 77-97 held back by 3-4 s LCP. Fixed: all 21 hero images moved off the deprecated priority prop to fetchPriority="high" + loading="eager" (Next 16); /iboga-ibogaine hero and the first card on /blog and category pages no longer lazy-loaded; sizes on the Four Doors cards (~150 KiB per page), /humanos diagram (~100 KiB) and /about headshot; urlFor no longer imports the Sanity client, so ~115 KB of Sanity client code stopped loading on / and /blog; React hydration error #418 on / and /blog (post dates) gone, checked in two time zones; /blog is static again; empty icon &lt;th&gt;s on /iboga-ibogaine labelled; category page reads use sanityFetch(). Left: se</t>
+          <t>the password-locked /blog/you-are-the-moat was in the sitemap while telling Google not to index it (a Search Console sitemap warning). Gated posts and posts that redirect are now left out (src/app/sitemap.ts); all 497 sitemap addresses return 200 with a matching canonical and no noindex. The 82 warnings Search Console shows are for the old live sitemap, so re-check them after cutover.</t>
         </is>
       </c>
       <c r="E282" s="14" t="inlineStr">
@@ -7343,17 +7343,17 @@
       <c r="A283" s="4" t="n"/>
       <c r="B283" s="4" t="inlineStr">
         <is>
-          <t>Error pages (2026-10-09, owner asked)</t>
-        </is>
-      </c>
-      <c r="C283" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Lighthouse pass (performance/accessibility/SEO) on top 20 pages by traffic 2026-09-30, 20 key pages (no traffic data yet), local production …</t>
+        </is>
+      </c>
+      <c r="C283" s="15" t="inlineStr">
+        <is>
+          <t>Remaining</t>
         </is>
       </c>
       <c r="D283" s="4" t="inlineStr">
         <is>
-          <t>404 page now sets its own title ("Page not found") as a server page around live's 3-second redirect (not-found.tsx + components/not-found-redirect.tsx), arrow as an icon; page error screen (error.tsx) uses Next 16's retry (re-fetches), shows a reference code for the server logs, links home and to the site index; new global-error.tsx for failures in the root layout itself (own &lt;html&gt;, plain links). Verified on a production build: missing page, missing essay and missing Kava page return 404 with the right title; a test page that throws returns 500 with the error screen, "Try again" re-fetches; phone and laptop, no sideways scroll (test page removed).</t>
+          <t>build, mobile: averages performance 87, accessibility 99→100, best practices 100, SEO 92→100, CLS 0 everywhere. Fixed: public/robots.txt had an LLMs: line (not a real directive) that made Google treat the whole file as invalid, now a comment; h3/h4 headings skipping a level on /assessments, /kava, /peptide-watch (same look, right tag); the Kava and /attention-theft back-arrow links had no accessible name on phones; two small phone-width contrast misses. Left: performance is local-machine only (±10-15 points, see CONTRIBUTING.md); the slowest were / 76 (LCP 5.2 s), /psychedelic-readiness-index 82, /iboga-ibogaine 83. Re-run against the Netlify deploy before launch. 2026-10-06 re-run against the Netlify deploy (14 key pages, mobile): accessibility 100 and CLS 0 on every page, SEO clean (only the expected netlify.app noindex), performance 77-97 held back by 3-4 s LCP. Fixed: all 21 hero images moved off the deprecated priority prop to fetchPriority="high" + loading="eager" (Next 16); /iboga-ibogaine hero and the first card on /blog and category pages no longer lazy-loaded; sizes on the Four Doors cards (~150 KiB per page), /humanos diagram (~100 KiB) and /about headshot; urlFor no longer imports the Sanity client, so ~115 KB of Sanity client code stopped loading on / and /blog; React hydration error #418 on / and /blog (post dates) gone, checked in two time zones; /blog is static again; empty icon &lt;th&gt;s on /iboga-ibogaine labelled; category page reads use sanityFetch(). Left: se</t>
         </is>
       </c>
       <c r="E283" s="14" t="inlineStr">
@@ -7366,7 +7366,7 @@
       <c r="A284" s="4" t="n"/>
       <c r="B284" s="4" t="inlineStr">
         <is>
-          <t>SEO audit fixes (2026-10-06)</t>
+          <t>Error pages (2026-10-09, owner asked)</t>
         </is>
       </c>
       <c r="C284" s="13" t="inlineStr">
@@ -7376,7 +7376,7 @@
       </c>
       <c r="D284" s="4" t="inlineStr">
         <is>
-          <t>Checked an outside audit point by point against the code. Fixed: Core Themes cards linked to /?theme=…#essays-archive (not crawlable, counts from a stale hand-kept list) and now link to /blog/category/&lt;slug&gt; with real counts (21/25/20/14, matching the archive pills; THEME_MAP and the ?theme= filter removed); Four Doors cards were &lt;button&gt;s, now real links that still open the modal on a plain click; "DIAGNOSE · ENGAGE" now link to /find-my and /engage; one shared formatPostDate (Asia/Kolkata, src/lib/format-post-date.ts) so a post no longer shows two different dates; the title repeated as the first body paragraph is dropped at render time (legacyBodyLayout); essay cards are h3 under a section h2 (archive, Read next), h2 only on category/search; heading glyphs (◆ ✦) hidden from screen readers; posts send BlogPosting with the author tied to the site Person (@id) plus a BreadcrumbList; descriptive alt on the homepage and BrewSoul heroes; homepage OG image cropped to 1200x630 JPEG. Already fine (audit could not see it): Person/Article schema, Netlify noindex, robots.txt, sitemap, header nav and search, Amazon links carry no affiliate tag. Checked on a production build: type check, lint, build, status codes, browser click test at 375px, no console errors. Implementation pack (Mohammad Danish, 2026-10-05) checked the same day: added og:type/og:site_name back on the 6 pages with their own openGraph (a page-level openGraph replaces the layout one), twitter:creator, and on posts og:url</t>
+          <t>404 page now sets its own title ("Page not found") as a server page around live's 3-second redirect (not-found.tsx + components/not-found-redirect.tsx), arrow as an icon; page error screen (error.tsx) uses Next 16's retry (re-fetches), shows a reference code for the server logs, links home and to the site index; new global-error.tsx for failures in the root layout itself (own &lt;html&gt;, plain links). Verified on a production build: missing page, missing essay and missing Kava page return 404 with the right title; a test page that throws returns 500 with the error screen, "Try again" re-fetches; phone and laptop, no sideways scroll (test page removed).</t>
         </is>
       </c>
       <c r="E284" s="14" t="inlineStr">
@@ -7389,17 +7389,17 @@
       <c r="A285" s="4" t="n"/>
       <c r="B285" s="4" t="inlineStr">
         <is>
-          <t>SEO audit items needing a yes (2026-10-06)</t>
-        </is>
-      </c>
-      <c r="C285" s="15" t="inlineStr">
-        <is>
-          <t>Remaining</t>
+          <t>SEO audit fixes (2026-10-06)</t>
+        </is>
+      </c>
+      <c r="C285" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D285" s="4" t="inlineStr">
         <is>
-          <t>the pack's new copy (homepage title/description, five-cups title, description, short answer, FAQ, heading rewrites, entity statement, newsletter block, author box, health disclaimer, COA wording); "Further Reading" shown twice on posts (merge the lists?); long post title (84 chars), homepage description length and obsolete keywords tag, slugs (/blog/five-cups, the -2 slug; would need redirects), "Six lenses" over four cards, sources for health claims and proof for "$10B+", "Certified B Corp", "Validity: 91", legal review of the homepage Case File banner, ABIT waitlist disclosures, one contact email, the two one-post categories, fewer homepage CTAs / email signup / table of contents / explaining "COA".</t>
+          <t>Checked an outside audit point by point against the code. Fixed: Core Themes cards linked to /?theme=…#essays-archive (not crawlable, counts from a stale hand-kept list) and now link to /blog/category/&lt;slug&gt; with real counts (21/25/20/14, matching the archive pills; THEME_MAP and the ?theme= filter removed); Four Doors cards were &lt;button&gt;s, now real links that still open the modal on a plain click; "DIAGNOSE · ENGAGE" now link to /find-my and /engage; one shared formatPostDate (Asia/Kolkata, src/lib/format-post-date.ts) so a post no longer shows two different dates; the title repeated as the first body paragraph is dropped at render time (legacyBodyLayout); essay cards are h3 under a section h2 (archive, Read next), h2 only on category/search; heading glyphs (◆ ✦) hidden from screen readers; posts send BlogPosting with the author tied to the site Person (@id) plus a BreadcrumbList; descriptive alt on the homepage and BrewSoul heroes; homepage OG image cropped to 1200x630 JPEG. Already fine (audit could not see it): Person/Article schema, Netlify noindex, robots.txt, sitemap, header nav and search, Amazon links carry no affiliate tag. Checked on a production build: type check, lint, build, status codes, browser click test at 375px, no console errors. Implementation pack (Mohammad Danish, 2026-10-05) checked the same day: added og:type/og:site_name back on the 6 pages with their own openGraph (a page-level openGraph replaces the layout one), twitter:creator, and on posts og:url</t>
         </is>
       </c>
       <c r="E285" s="14" t="inlineStr">
@@ -7412,7 +7412,7 @@
       <c r="A286" s="4" t="n"/>
       <c r="B286" s="4" t="inlineStr">
         <is>
-          <t>Connect Google Search Console + GA4 to the new deployment on day one of cutover</t>
+          <t>SEO audit items needing a yes (2026-10-06)</t>
         </is>
       </c>
       <c r="C286" s="15" t="inlineStr">
@@ -7420,7 +7420,11 @@
           <t>Remaining</t>
         </is>
       </c>
-      <c r="D286" s="4" t="inlineStr"/>
+      <c r="D286" s="4" t="inlineStr">
+        <is>
+          <t>the pack's new copy (homepage title/description, five-cups title, description, short answer, FAQ, heading rewrites, entity statement, newsletter block, author box, health disclaimer, COA wording); "Further Reading" shown twice on posts (merge the lists?); long post title (84 chars), homepage description length and obsolete keywords tag, slugs (/blog/five-cups, the -2 slug; would need redirects), "Six lenses" over four cards, sources for health claims and proof for "$10B+", "Certified B Corp", "Validity: 91", legal review of the homepage Case File banner, ABIT waitlist disclosures, one contact email, the two one-post categories, fewer homepage CTAs / email signup / table of contents / explaining "COA".</t>
+        </is>
+      </c>
       <c r="E286" s="14" t="inlineStr">
         <is>
           <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
@@ -7431,19 +7435,15 @@
       <c r="A287" s="4" t="n"/>
       <c r="B287" s="4" t="inlineStr">
         <is>
-          <t>Restore/adapt the manus.space triple-layer noindex lockdown pattern for any remaining staging URLs</t>
-        </is>
-      </c>
-      <c r="C287" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D287" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-01: the Netlify copy (tonygreenberg-website.netlify.app) and every deploy preview had no noindex at all, so Google could index a duplicate of the site. next.config.ts headers() now sends X-Robots-Tag: noindex, nofollow on any *.netlify.app host only; tonygreenberg.com is unaffected, so nothing to remove at cutover. Tested with Host headers on a production build.</t>
-        </is>
-      </c>
+          <t>Connect Google Search Console + GA4 to the new deployment on day one of cutover</t>
+        </is>
+      </c>
+      <c r="C287" s="15" t="inlineStr">
+        <is>
+          <t>Remaining</t>
+        </is>
+      </c>
+      <c r="D287" s="4" t="inlineStr"/>
       <c r="E287" s="14" t="inlineStr">
         <is>
           <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
@@ -7454,7 +7454,7 @@
       <c r="A288" s="4" t="n"/>
       <c r="B288" s="4" t="inlineStr">
         <is>
-          <t>"Keep going" strip above the footer on every page (2026-10-07)</t>
+          <t>Restore/adapt the manus.space triple-layer noindex lockdown pattern for any remaining staging URLs</t>
         </is>
       </c>
       <c r="C288" s="13" t="inlineStr">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="D288" s="4" t="inlineStr">
         <is>
-          <t>legacy's WhereNext (deferred in Phase 3, never picked up) with its per-page suggestions, Home · Site Index · All Assessments; links pointed at current routes.</t>
+          <t>2026-10-01: the Netlify copy (tonygreenberg-website.netlify.app) and every deploy preview had no noindex at all, so Google could index a duplicate of the site. next.config.ts headers() now sends X-Robots-Tag: noindex, nofollow on any *.netlify.app host only; tonygreenberg.com is unaffected, so nothing to remove at cutover. Tested with Host headers on a production build.</t>
         </is>
       </c>
       <c r="E288" s="14" t="inlineStr">
@@ -7477,7 +7477,7 @@
       <c r="A289" s="4" t="n"/>
       <c r="B289" s="4" t="inlineStr">
         <is>
-          <t>Live-only and redesigned pages from the 2026-10-07 page sweep (188 pages compared with live)</t>
+          <t>"Keep going" strip above the footer on every page (2026-10-07)</t>
         </is>
       </c>
       <c r="C289" s="13" t="inlineStr">
@@ -7487,7 +7487,7 @@
       </c>
       <c r="D289" s="4" t="inlineStr">
         <is>
-          <t>/the-index rebuilt from live's code (20 concepts, related-word search across essays and site pages, full-text search on the server, "three related places to go next"; the old redirect to /search removed and its links, including the "Site Index" link in "Keep going", point at it again); /the-mirror (and /life-assessment) opens on live's intro (dark hero, "What We Measure" with the six areas, "The Ecosystem"), rebuilt as a step registry (rule 19); /essays header, order and column like live; /about "What They Say" styled like live (live picks 3 of the same 19 quotes at random; ours shows a fixed 3 so they're in the server HTML); /impact-futurism list titles and subtitles; /supplier-intake is a real page again with live's Stage 1 form; /seven-doors and /projects redirect home like live; /impact, /health, /library, /built-on-manus, /heroes are 404 on live too. Left as is on purpose: /blog stays our archive page (on live it repeats the homepage), the email gates on /framework and /peptide-supply-chain, the attention-theft Wall of Shame.</t>
+          <t>legacy's WhereNext (deferred in Phase 3, never picked up) with its per-page suggestions, Home · Site Index · All Assessments; links pointed at current routes.</t>
         </is>
       </c>
       <c r="E289" s="14" t="inlineStr">
@@ -7500,7 +7500,7 @@
       <c r="A290" s="4" t="n"/>
       <c r="B290" s="4" t="inlineStr">
         <is>
-          <t>/alex-azzi locked like live (2026-10-07, owner said match it)</t>
+          <t>Live-only and redesigned pages from the 2026-10-07 page sweep (188 pages compared with live)</t>
         </is>
       </c>
       <c r="C290" s="13" t="inlineStr">
@@ -7510,7 +7510,7 @@
       </c>
       <c r="D290" s="4" t="inlineStr">
         <is>
-          <t>same server-checked password as the locked essay (GATED_POST_PASSWORD, now also set in Netlify), live's "Restricted Access" screen, the report not in the page until unlocked, out of search and the sitemap.</t>
+          <t>/the-index rebuilt from live's code (20 concepts, related-word search across essays and site pages, full-text search on the server, "three related places to go next"; the old redirect to /search removed and its links, including the "Site Index" link in "Keep going", point at it again); /the-mirror (and /life-assessment) opens on live's intro (dark hero, "What We Measure" with the six areas, "The Ecosystem"), rebuilt as a step registry (rule 19); /essays header, order and column like live; /about "What They Say" styled like live (live picks 3 of the same 19 quotes at random; ours shows a fixed 3 so they're in the server HTML); /impact-futurism list titles and subtitles; /supplier-intake is a real page again with live's Stage 1 form; /seven-doors and /projects redirect home like live; /impact, /health, /library, /built-on-manus, /heroes are 404 on live too. Left as is on purpose: /blog stays our archive page (on live it repeats the homepage), the email gates on /framework and /peptide-supply-chain, the attention-theft Wall of Shame.</t>
         </is>
       </c>
       <c r="E290" s="14" t="inlineStr">
@@ -7523,7 +7523,7 @@
       <c r="A291" s="4" t="n"/>
       <c r="B291" s="4" t="inlineStr">
         <is>
-          <t>Live's title fonts and sizes (2026-10-07, "fix the style")</t>
+          <t>/alex-azzi locked like live (2026-10-07, owner said match it)</t>
         </is>
       </c>
       <c r="C291" s="13" t="inlineStr">
@@ -7533,7 +7533,7 @@
       </c>
       <c r="D291" s="4" t="inlineStr">
         <is>
-          <t>measured every page's title font, weight, size and label colour on live vs ours (136 pages). Now like live: Kava headings in Fraunces, HumanOS in Space Grotesk, the peptide tools / charity scorecard / thesis threads in the system serif, America Unbundled in the Iowan Old Style stack at live's size, /akbar in Fraunces 900, friend-gate and post-intervention in Georgia, and live's title sizes on peptide-matrix, peptide-supply-chain, rip-peptide-sciences and the HumanOS pages. Fonts load only on the pages that use them (src/lib/fonts/page-fonts.ts). Label colours stay the darker AA-contrast versions where live's lighter ones fail on a light background.</t>
+          <t>same server-checked password as the locked essay (GATED_POST_PASSWORD, now also set in Netlify), live's "Restricted Access" screen, the report not in the page until unlocked, out of search and the sitemap.</t>
         </is>
       </c>
       <c r="E291" s="14" t="inlineStr">
@@ -7546,7 +7546,7 @@
       <c r="A292" s="4" t="n"/>
       <c r="B292" s="4" t="inlineStr">
         <is>
-          <t>Peptide page images rescued into Sanity and wired (2026-10-07)</t>
+          <t>Live's title fonts and sizes (2026-10-07, "fix the style")</t>
         </is>
       </c>
       <c r="C292" s="13" t="inlineStr">
@@ -7556,7 +7556,7 @@
       </c>
       <c r="D292" s="4" t="inlineStr">
         <is>
-          <t>/peptide-watch hero plus its 11 section banners, /peptide-matrix and /peptide-supply-chain heroes, the /peptide-hall-of-shame hero (scripts/rescue-2026-10-07-peptide-images.ts, logged in docs/ai/manus-media-rescue.md).</t>
+          <t>measured every page's title font, weight, size and label colour on live vs ours (136 pages). Now like live: Kava headings in Fraunces, HumanOS in Space Grotesk, the peptide tools / charity scorecard / thesis threads in the system serif, America Unbundled in the Iowan Old Style stack at live's size, /akbar in Fraunces 900, friend-gate and post-intervention in Georgia, and live's title sizes on peptide-matrix, peptide-supply-chain, rip-peptide-sciences and the HumanOS pages. Fonts load only on the pages that use them (src/lib/fonts/page-fonts.ts). Label colours stay the darker AA-contrast versions where live's lighter ones fail on a light background.</t>
         </is>
       </c>
       <c r="E292" s="14" t="inlineStr">
@@ -7569,7 +7569,7 @@
       <c r="A293" s="4" t="n"/>
       <c r="B293" s="4" t="inlineStr">
         <is>
-          <t>Live's editorial redesign, first group (2026-10-07)</t>
+          <t>Peptide page images rescued into Sanity and wired (2026-10-07)</t>
         </is>
       </c>
       <c r="C293" s="13" t="inlineStr">
@@ -7579,7 +7579,7 @@
       </c>
       <c r="D293" s="4" t="inlineStr">
         <is>
-          <t>dark top sections, narrow single text column, short red section rules and dark call-to-action bands on /invest, /amplifier, /community (now "Sign In to Join the Community", linking our real sign-in; live's made-up counters left out), /framework, /the-letter (daily provocation with "Share this thought" and "Search past provocations"), /engage, /diamond-cut, /ecosystem and the homepage's "The thinking doesn't stop here" band. Kept on purpose: AA-contrast colours where live's fail, "Enter the Gate" instead of live's $5,000 checkout on /diamond-cut.</t>
+          <t>/peptide-watch hero plus its 11 section banners, /peptide-matrix and /peptide-supply-chain heroes, the /peptide-hall-of-shame hero (scripts/rescue-2026-10-07-peptide-images.ts, logged in docs/ai/manus-media-rescue.md).</t>
         </is>
       </c>
       <c r="E293" s="14" t="inlineStr">
@@ -7592,7 +7592,7 @@
       <c r="A294" s="4" t="n"/>
       <c r="B294" s="4" t="inlineStr">
         <is>
-          <t>Live's redesign, second group (done 2026-10-08)</t>
+          <t>Live's editorial redesign, first group (2026-10-07)</t>
         </is>
       </c>
       <c r="C294" s="13" t="inlineStr">
@@ -7602,7 +7602,7 @@
       </c>
       <c r="D294" s="4" t="inlineStr">
         <is>
-          <t>re-measured all 18 pages on live vs a fresh production build (title font/size/weight/colour, labels, hero images). Already matching from 2026-10-07: /the-web, /spirits, /iboga-ibogaine (weight 800), /living-declaration, BrewSoul photo on /brewsoul, /brewsoul/browse, /brewsoul/first-sip (live has none there either), /quiz_25q, /recent-creations. Fixed today: /find-your-journey (64px title, red label), /impact-dashboard (64px title in essay ink, label spacing), red labels on /published and /speaking (plus its "rooms" chips), /soulscore "by ImpactSoul" label, /pri-calibration title (weight 900, solid cream, was a purple gradient), /clients (live's narrow 546px column for the whole page, 56px title, roomier stats band, cards 2 per row; two static inline styles moved to classes), /brewsoul/guest (live's BrewSoul photo on the guest card instead of "SN" initials, labels in capitals), /humanos/connect (cards line up with the title), /peptide-hall-of-shame (stats and label readable light gold; were dark gold on dark). Typed arrows on the touched links are icons now (rule 18). Deliberately not copied from live (new CONTRIBUTING rule 20, owner 2026-10-08): red labels on dark bands use #E07A80 (live's #8E1E25 on black is about 2:1, unreadable); /recent-creations keeps our darker label colours (live's fail contrast on white); /humanos/connect keeps "Start Reading" (that card links to the philosophy page, the quiz live's "Start the Assessment" implies doesn't exist). Checked: type check, l</t>
+          <t>dark top sections, narrow single text column, short red section rules and dark call-to-action bands on /invest, /amplifier, /community (now "Sign In to Join the Community", linking our real sign-in; live's made-up counters left out), /framework, /the-letter (daily provocation with "Share this thought" and "Search past provocations"), /engage, /diamond-cut, /ecosystem and the homepage's "The thinking doesn't stop here" band. Kept on purpose: AA-contrast colours where live's fail, "Enter the Gate" instead of live's $5,000 checkout on /diamond-cut.</t>
         </is>
       </c>
       <c r="E294" s="14" t="inlineStr">
@@ -7615,7 +7615,7 @@
       <c r="A295" s="4" t="n"/>
       <c r="B295" s="4" t="inlineStr">
         <is>
-          <t>BrewSoul top of page (2026-10-08, owner: "button in the center at the top doesn't look good")</t>
+          <t>Live's redesign, second group (done 2026-10-08)</t>
         </is>
       </c>
       <c r="C295" s="13" t="inlineStr">
@@ -7625,7 +7625,7 @@
       </c>
       <c r="D295" s="4" t="inlineStr">
         <is>
-          <t>the category badge ("Deep Research" etc.) sat centred in an empty strip, squeezed against the hero, because we copied live's doubled 52px top gap. Now one gap everywhere and the badge floats in the top-left corner, lined up with the BrewSoul logo (brewsoul-main.tsx, category-badge.tsx); checked on all 26 badge pages at 3 widths that it covers nothing. BrewSoul menu: on tablets (768-1023px) the links were cut off and "More" was hidden with no menu button at all; now the menu button shows below 1024px, 5 links + "More" from 1024px, all 8 from 1280px, "More" always visible.</t>
+          <t>re-measured all 18 pages on live vs a fresh production build (title font/size/weight/colour, labels, hero images). Already matching from 2026-10-07: /the-web, /spirits, /iboga-ibogaine (weight 800), /living-declaration, BrewSoul photo on /brewsoul, /brewsoul/browse, /brewsoul/first-sip (live has none there either), /quiz_25q, /recent-creations. Fixed today: /find-your-journey (64px title, red label), /impact-dashboard (64px title in essay ink, label spacing), red labels on /published and /speaking (plus its "rooms" chips), /soulscore "by ImpactSoul" label, /pri-calibration title (weight 900, solid cream, was a purple gradient), /clients (live's narrow 546px column for the whole page, 56px title, roomier stats band, cards 2 per row; two static inline styles moved to classes), /brewsoul/guest (live's BrewSoul photo on the guest card instead of "SN" initials, labels in capitals), /humanos/connect (cards line up with the title), /peptide-hall-of-shame (stats and label readable light gold; were dark gold on dark). Typed arrows on the touched links are icons now (rule 18). Deliberately not copied from live (new CONTRIBUTING rule 20, owner 2026-10-08): red labels on dark bands use #E07A80 (live's #8E1E25 on black is about 2:1, unreadable); /recent-creations keeps our darker label colours (live's fail contrast on white); /humanos/connect keeps "Start Reading" (that card links to the philosophy page, the quiz live's "Start the Assessment" implies doesn't exist). Checked: type check, l</t>
         </is>
       </c>
       <c r="E295" s="14" t="inlineStr">
@@ -7638,7 +7638,7 @@
       <c r="A296" s="4" t="n"/>
       <c r="B296" s="4" t="inlineStr">
         <is>
-          <t>/pri-efficacy's "Simulation / Live Calibrations" switch like live (2026-10-08)</t>
+          <t>BrewSoul top of page (2026-10-08, owner: "button in the center at the top doesn't look good")</t>
         </is>
       </c>
       <c r="C296" s="13" t="inlineStr">
@@ -7648,7 +7648,7 @@
       </c>
       <c r="D296" s="4" t="inlineStr">
         <is>
-          <t>shadcn Tabs, both panels in the server HTML (forceMount). The Live tab reads real aggregate numbers from pri_calibrations (getPriLiveStats() in src/lib/pri-research.ts: totals, opt-ins, average score per dimension; no rows leave the server), page stays static and refreshes every 10 minutes. Until the Supabase scripts are run (Phase 2) it says the numbers "aren't available just now" instead of a fake zero. Checked: build (○, 10m), server HTML has both tabs, tab switch at 390/1280px, no JS errors. Re-check with real numbers once the table exists.</t>
+          <t>the category badge ("Deep Research" etc.) sat centred in an empty strip, squeezed against the hero, because we copied live's doubled 52px top gap. Now one gap everywhere and the badge floats in the top-left corner, lined up with the BrewSoul logo (brewsoul-main.tsx, category-badge.tsx); checked on all 26 badge pages at 3 widths that it covers nothing. BrewSoul menu: on tablets (768-1023px) the links were cut off and "More" was hidden with no menu button at all; now the menu button shows below 1024px, 5 links + "More" from 1024px, all 8 from 1280px, "More" always visible.</t>
         </is>
       </c>
       <c r="E296" s="14" t="inlineStr">
@@ -7661,63 +7661,63 @@
       <c r="A297" s="4" t="n"/>
       <c r="B297" s="4" t="inlineStr">
         <is>
+          <t>/pri-efficacy's "Simulation / Live Calibrations" switch like live (2026-10-08)</t>
+        </is>
+      </c>
+      <c r="C297" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D297" s="4" t="inlineStr">
+        <is>
+          <t>shadcn Tabs, both panels in the server HTML (forceMount). The Live tab reads real aggregate numbers from pri_calibrations (getPriLiveStats() in src/lib/pri-research.ts: totals, opt-ins, average score per dimension; no rows leave the server), page stays static and refreshes every 10 minutes. Until the Supabase scripts are run (Phase 2) it says the numbers "aren't available just now" instead of a fake zero. Checked: build (○, 10m), server HTML has both tabs, tab switch at 390/1280px, no JS errors. Re-check with real numbers once the table exists.</t>
+        </is>
+      </c>
+      <c r="E297" s="14" t="inlineStr">
+        <is>
+          <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" s="4" t="n"/>
+      <c r="B298" s="4" t="inlineStr">
+        <is>
           <t>/brewsoul/browse hero readable (2026-10-08, owner said go ahead)</t>
         </is>
       </c>
-      <c r="C297" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D297" s="4" t="inlineStr">
+      <c r="C298" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D298" s="4" t="inlineStr">
         <is>
           <t>a soft cream glow behind the title block so "The Catalog", the subtitle and the stat labels read clearly over the coffee photo (live is hard to read there too; rule 20). Photo still shows around the edges. Checked at 390/1280px.</t>
         </is>
       </c>
-      <c r="E297" s="14" t="inlineStr">
+      <c r="E298" s="14" t="inlineStr">
         <is>
           <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
         </is>
       </c>
     </row>
-    <row r="298">
-      <c r="A298" s="10" t="inlineStr">
+    <row r="299">
+      <c r="A299" s="10" t="inlineStr">
         <is>
           <t>Phase 13 — Images Needed in Sanity</t>
         </is>
       </c>
-      <c r="B298" s="11" t="n"/>
-      <c r="C298" s="11" t="n"/>
-      <c r="D298" s="12" t="n"/>
-    </row>
-    <row r="299">
-      <c r="A299" s="4" t="n"/>
-      <c r="B299" s="4" t="inlineStr">
-        <is>
-          <t>Manus media rescue (2026-09-29)</t>
-        </is>
-      </c>
-      <c r="C299" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D299" s="4" t="inlineStr">
-        <is>
-          <t>all 94 Manus-hosted image/video references in the legacy source (/api/img/, /manus-storage/) were checked live. 91 were still downloadable, including the /akbar photos the entry below calls "permanently lost", and all 91 are now Sanity assets (scripts/rescue-manus-media.ts; Sanity dedupes by SHA-1). 3 were gone (HTTP 502). The manifest docs/ai/manus-media-rescue.md maps each one to the legacy files that used it and its Sanity URL. They are not wired into pages yet: go page by page, with real alt text. /facilitator-index's two diagrams are done (scripts/rescue-facilitator-images.ts).</t>
-        </is>
-      </c>
-      <c r="E299" s="14" t="inlineStr">
-        <is>
-          <t>Phase 13 — Images Needed in Sanity</t>
-        </is>
-      </c>
+      <c r="B299" s="11" t="n"/>
+      <c r="C299" s="11" t="n"/>
+      <c r="D299" s="12" t="n"/>
     </row>
     <row r="300">
       <c r="A300" s="4" t="n"/>
       <c r="B300" s="4" t="inlineStr">
         <is>
-          <t>Favicon</t>
+          <t>Manus media rescue (2026-09-29)</t>
         </is>
       </c>
       <c r="C300" s="13" t="inlineStr">
@@ -7727,7 +7727,7 @@
       </c>
       <c r="D300" s="4" t="inlineStr">
         <is>
-          <t>real "G" brand mark generated from the header's actual wordmark treatment (src/app/icon.tsx), see Phase 3</t>
+          <t>all 94 Manus-hosted image/video references in the legacy source (/api/img/, /manus-storage/) were checked live. 91 were still downloadable, including the /akbar photos the entry below calls "permanently lost", and all 91 are now Sanity assets (scripts/rescue-manus-media.ts; Sanity dedupes by SHA-1). 3 were gone (HTTP 502). The manifest docs/ai/manus-media-rescue.md maps each one to the legacy files that used it and its Sanity URL. They are not wired into pages yet: go page by page, with real alt text. /facilitator-index's two diagrams are done (scripts/rescue-facilitator-images.ts).</t>
         </is>
       </c>
       <c r="E300" s="14" t="inlineStr">
@@ -7740,17 +7740,17 @@
       <c r="A301" s="4" t="n"/>
       <c r="B301" s="4" t="inlineStr">
         <is>
-          <t>Site-wide: logo (light + dark) beyond the current text wordmark</t>
-        </is>
-      </c>
-      <c r="C301" s="15" t="inlineStr">
-        <is>
-          <t>Remaining</t>
+          <t>Favicon</t>
+        </is>
+      </c>
+      <c r="C301" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D301" s="4" t="inlineStr">
         <is>
-          <t>(Default/fallback OG image 1200×630 exists: public/images/default-og.png, checked 2026-10-02.)</t>
+          <t>real "G" brand mark generated from the header's actual wordmark treatment (src/app/icon.tsx), see Phase 3</t>
         </is>
       </c>
       <c r="E301" s="14" t="inlineStr">
@@ -7763,17 +7763,17 @@
       <c r="A302" s="4" t="n"/>
       <c r="B302" s="4" t="inlineStr">
         <is>
-          <t>Author photo(s) for blog author schema (Tony Greenberg headshot at minimum)</t>
-        </is>
-      </c>
-      <c r="C302" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Site-wide: logo (light + dark) beyond the current text wordmark</t>
+        </is>
+      </c>
+      <c r="C302" s="15" t="inlineStr">
+        <is>
+          <t>Remaining</t>
         </is>
       </c>
       <c r="D302" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02: the rescued headshot is already the author avatar in Sanity; now also in every post's Article JSON-LD (author image + url /about). The JSON-LD publisher logo pointed at /favicon.ico, a 404 here; now /icon.</t>
+          <t>(Default/fallback OG image 1200×630 exists: public/images/default-og.png, checked 2026-10-02.)</t>
         </is>
       </c>
       <c r="E302" s="14" t="inlineStr">
@@ -7786,7 +7786,7 @@
       <c r="A303" s="4" t="n"/>
       <c r="B303" s="4" t="inlineStr">
         <is>
-          <t>Blog hero images</t>
+          <t>Author photo(s) for blog author schema (Tony Greenberg headshot at minimum)</t>
         </is>
       </c>
       <c r="C303" s="13" t="inlineStr">
@@ -7796,7 +7796,7 @@
       </c>
       <c r="D303" s="4" t="inlineStr">
         <is>
-          <t>audited, then migrated. Final state:</t>
+          <t>2026-10-02: the rescued headshot is already the author avatar in Sanity; now also in every post's Article JSON-LD (author image + url /about). The JSON-LD publisher logo pointed at /favicon.ico, a 404 here; now /icon.</t>
         </is>
       </c>
       <c r="E303" s="14" t="inlineStr">
@@ -7809,7 +7809,7 @@
       <c r="A304" s="4" t="n"/>
       <c r="B304" s="4" t="inlineStr">
         <is>
-          <t>22 posts have a real hero image, now live in Sanity (17 already on RampRate's own CloudFront + 4 rescued from the legacy /api/img/ proxy + 1…</t>
+          <t>Blog hero images</t>
         </is>
       </c>
       <c r="C304" s="13" t="inlineStr">
@@ -7819,7 +7819,7 @@
       </c>
       <c r="D304" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> rescued from /manus-storage/, all pulled over by migrate-blog-posts.ts before Manus is decommissioned)</t>
+          <t>audited, then migrated. Final state:</t>
         </is>
       </c>
       <c r="E304" s="14" t="inlineStr">
@@ -7832,7 +7832,7 @@
       <c r="A305" s="4" t="n"/>
       <c r="B305" s="4" t="inlineStr">
         <is>
-          <t>7 more posts got a real, unique hero image rescued from the live legacy site's newly-added art this pass (scripts/rescue-2026-09-blog-images…</t>
+          <t>22 posts have a real hero image, now live in Sanity (17 already on RampRate's own CloudFront + 4 rescued from the legacy /api/img/ proxy + 1…</t>
         </is>
       </c>
       <c r="C305" s="13" t="inlineStr">
@@ -7842,7 +7842,7 @@
       </c>
       <c r="D305" s="4" t="inlineStr">
         <is>
-          <t>.ts — see the correction note above): california-toll-roads-legalized-scam, the-1000-hour-hold, conscious-capital-partnership-ecosystem, the-peptide-truth-65m-fraud-industry-vs-life-changing-medicine, clear-communication, building-services-market-transhuman-era, heart-protocol-addendum.</t>
+          <t xml:space="preserve"> rescued from /manus-storage/, all pulled over by migrate-blog-posts.ts before Manus is decommissioned)</t>
         </is>
       </c>
       <c r="E305" s="14" t="inlineStr">
@@ -7855,17 +7855,17 @@
       <c r="A306" s="4" t="n"/>
       <c r="B306" s="4" t="inlineStr">
         <is>
-          <t>92 posts still need a real, unique hero image</t>
-        </is>
-      </c>
-      <c r="C306" s="15" t="inlineStr">
-        <is>
-          <t>Remaining</t>
+          <t>7 more posts got a real, unique hero image rescued from the live legacy site's newly-added art this pass (scripts/rescue-2026-09-blog-images…</t>
+        </is>
+      </c>
+      <c r="C306" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D306" s="4" t="inlineStr">
         <is>
-          <t>(down from 99). Tracked one row per post, with a suggested image-generation prompt, in BLOG-IMAGE-BRIEFS.md — work through that file and check items off there, not here. No image-generation tool was connected in this environment as of this writing; either connect one (e.g. an MCP image-gen extension), source these manually/with a designer then upload via Sanity Studio (/studio), or re-check the live legacy site periodically per the correction note above.</t>
+          <t>.ts — see the correction note above): california-toll-roads-legalized-scam, the-1000-hour-hold, conscious-capital-partnership-ecosystem, the-peptide-truth-65m-fraud-industry-vs-life-changing-medicine, clear-communication, building-services-market-transhuman-era, heart-protocol-addendum.</t>
         </is>
       </c>
       <c r="E306" s="14" t="inlineStr">
@@ -7878,17 +7878,17 @@
       <c r="A307" s="4" t="n"/>
       <c r="B307" s="4" t="inlineStr">
         <is>
-          <t>Blog: per-post OG image if different from hero (many posts can reuse hero as OG)</t>
-        </is>
-      </c>
-      <c r="C307" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>92 posts still need a real, unique hero image</t>
+        </is>
+      </c>
+      <c r="C307" s="15" t="inlineStr">
+        <is>
+          <t>Remaining</t>
         </is>
       </c>
       <c r="D307" s="4" t="inlineStr">
         <is>
-          <t>Confirmed 2026-10-02: generateMetadata uses seo.ogImage, else the hero, else the default OG image.</t>
+          <t>(down from 99). Tracked one row per post, with a suggested image-generation prompt, in BLOG-IMAGE-BRIEFS.md — work through that file and check items off there, not here. No image-generation tool was connected in this environment as of this writing; either connect one (e.g. an MCP image-gen extension), source these manually/with a designer then upload via Sanity Studio (/studio), or re-check the live legacy site periodically per the correction note above.</t>
         </is>
       </c>
       <c r="E307" s="14" t="inlineStr">
@@ -7901,7 +7901,7 @@
       <c r="A308" s="4" t="n"/>
       <c r="B308" s="4" t="inlineStr">
         <is>
-          <t>Marketing pages</t>
+          <t>Blog: per-post OG image if different from hero (many posts can reuse hero as OG)</t>
         </is>
       </c>
       <c r="C308" s="13" t="inlineStr">
@@ -7911,7 +7911,7 @@
       </c>
       <c r="D308" s="4" t="inlineStr">
         <is>
-          <t>hero/section images for /the-letter, /the-territory, /engine-room, /the-body, /the-nightstand, /recent-creations (portfolio thumbnails), /published (publication logos), /clients (client logos — confirm licensing before re-hosting). Checked against live 2026-10-02: same image count on every one; /the-territory, /engine-room, /recent-creations, /published, /clients have no images on live either.</t>
+          <t>Confirmed 2026-10-02: generateMetadata uses seo.ogImage, else the hero, else the default OG image.</t>
         </is>
       </c>
       <c r="E308" s="14" t="inlineStr">
@@ -7924,7 +7924,7 @@
       <c r="A309" s="4" t="n"/>
       <c r="B309" s="4" t="inlineStr">
         <is>
-          <t>/akbar essay images</t>
+          <t>Marketing pages</t>
         </is>
       </c>
       <c r="C309" s="13" t="inlineStr">
@@ -7934,7 +7934,7 @@
       </c>
       <c r="D309" s="4" t="inlineStr">
         <is>
-          <t>not lost after all: 20 of the 21 were rescued into Sanity by scripts/rescue-manus-media.ts (2026-09-28) and are wired back in legacy's layout (hero mosaic, JC portrait, 2x2 grid, 3 full-bleeds, 3-up strip, footer gallery) as of 2026-09-29. Only slider-3 was gone (HTTP 502); the hero mosaic is 4 tiles instead of 5.</t>
+          <t>hero/section images for /the-letter, /the-territory, /engine-room, /the-body, /the-nightstand, /recent-creations (portfolio thumbnails), /published (publication logos), /clients (client logos — confirm licensing before re-hosting). Checked against live 2026-10-02: same image count on every one; /the-territory, /engine-room, /recent-creations, /published, /clients have no images on live either.</t>
         </is>
       </c>
       <c r="E309" s="14" t="inlineStr">
@@ -7947,7 +7947,7 @@
       <c r="A310" s="4" t="n"/>
       <c r="B310" s="4" t="inlineStr">
         <is>
-          <t>Rescued page images wired back in (2026-09-29)</t>
+          <t>/akbar essay images</t>
         </is>
       </c>
       <c r="C310" s="13" t="inlineStr">
@@ -7957,7 +7957,7 @@
       </c>
       <c r="D310" s="4" t="inlineStr">
         <is>
-          <t>/living-declaration hero, hand image and Clarisse Abelarde artwork; /impact-dashboard earth hero; /find-my banner; /find-your-coffee dark photo landing (legacy copy restored, replacing an intro that wasn't in legacy). Also wired (second pass): /consciousness-scale (legacy's hero-first flow restored, the invented intro screen removed), /find-your-me hero, /humanos hero, the HumanOS nav logo, and all 12 HumanOS people headshots (/humanos/ecosystem, /humanos/philosophy). Blog-body images (2026-09-29): all 19 the migration dropped are restored by scripts/restore-blog-body-images.ts as Sanity drafts on 4 posts (Clarisse Abelarde 7, You Are the Moat 4, FRQNCY 6, Energy Is Money 2), waiting to be published in Studio; the other blog-listed assets were heroes already set. Still unwired from docs/ai/manus-media-rescue.md: and /alex-azzi's subject photo (a photo of a real person on an accusation page: needs Tony's yes first).</t>
+          <t>not lost after all: 20 of the 21 were rescued into Sanity by scripts/rescue-manus-media.ts (2026-09-28) and are wired back in legacy's layout (hero mosaic, JC portrait, 2x2 grid, 3 full-bleeds, 3-up strip, footer gallery) as of 2026-09-29. Only slider-3 was gone (HTTP 502); the hero mosaic is 4 tiles instead of 5.</t>
         </is>
       </c>
       <c r="E310" s="14" t="inlineStr">
@@ -7970,7 +7970,7 @@
       <c r="A311" s="4" t="n"/>
       <c r="B311" s="4" t="inlineStr">
         <is>
-          <t>BrewSoul: coffee/product images (brewsoul-coffees-expanded.ts likely has image refs</t>
+          <t>Rescued page images wired back in (2026-09-29)</t>
         </is>
       </c>
       <c r="C311" s="13" t="inlineStr">
@@ -7980,7 +7980,7 @@
       </c>
       <c r="D311" s="4" t="inlineStr">
         <is>
-          <t>audit), city guide header images, roaster directory photos. Audited 2026-09-09 (status spreadsheet), confirmed 2026-10-02: city guides already have photos; coffees, chains and roasters have no image field in legacy or here (text-only by design); farms got real photos.</t>
+          <t>/living-declaration hero, hand image and Clarisse Abelarde artwork; /impact-dashboard earth hero; /find-my banner; /find-your-coffee dark photo landing (legacy copy restored, replacing an intro that wasn't in legacy). Also wired (second pass): /consciousness-scale (legacy's hero-first flow restored, the invented intro screen removed), /find-your-me hero, /humanos hero, the HumanOS nav logo, and all 12 HumanOS people headshots (/humanos/ecosystem, /humanos/philosophy). Blog-body images (2026-09-29): all 19 the migration dropped are restored by scripts/restore-blog-body-images.ts as Sanity drafts on 4 posts (Clarisse Abelarde 7, You Are the Moat 4, FRQNCY 6, Energy Is Money 2), waiting to be published in Studio; the other blog-listed assets were heroes already set. Still unwired from docs/ai/manus-media-rescue.md: and /alex-azzi's subject photo (a photo of a real person on an accusation page: needs Tony's yes first).</t>
         </is>
       </c>
       <c r="E311" s="14" t="inlineStr">
@@ -7993,7 +7993,7 @@
       <c r="A312" s="4" t="n"/>
       <c r="B312" s="4" t="inlineStr">
         <is>
-          <t>65 page images moved off the Manus storage copy into Sanity (2026-10-02)</t>
+          <t>BrewSoul: coffee/product images (brewsoul-coffees-expanded.ts likely has image refs</t>
         </is>
       </c>
       <c r="C312" s="13" t="inlineStr">
@@ -8003,7 +8003,7 @@
       </c>
       <c r="D312" s="4" t="inlineStr">
         <is>
-          <t>every image the code loaded from d2xsxph8kpxj0f.cloudfront.net (PRI medicine images, Iboga module, facilitator index, /attention-theft, /alex-azzi, /protecting-your-business, /peyote-mescaline, HumanOS, the peptide quiz). Notes called it "RampRate's own CloudFront", but every file sits in the legacy Manus project's folder and its owner couldn't be confirmed. All 65 uploaded (scripts/rescue-cloudfront-images.ts), code rewritten, host removed from images.remotePatterns, no Sanity document used it. Table in docs/ai/manus-media-rescue.md.</t>
+          <t>audit), city guide header images, roaster directory photos. Audited 2026-09-09 (status spreadsheet), confirmed 2026-10-02: city guides already have photos; coffees, chains and roasters have no image field in legacy or here (text-only by design); farms got real photos.</t>
         </is>
       </c>
       <c r="E312" s="14" t="inlineStr">
@@ -8016,7 +8016,7 @@
       <c r="A313" s="4" t="n"/>
       <c r="B313" s="4" t="inlineStr">
         <is>
-          <t>PRI/Kava: medicine reference images (medicine-images.ts), facility images for /facilitator-index</t>
+          <t>65 page images moved off the Manus storage copy into Sanity (2026-10-02)</t>
         </is>
       </c>
       <c r="C313" s="13" t="inlineStr">
@@ -8026,7 +8026,7 @@
       </c>
       <c r="D313" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02: all in Sanity; image counts match live on PRI, Kava, Iboga, Peyote, facilitator pages.</t>
+          <t>every image the code loaded from d2xsxph8kpxj0f.cloudfront.net (PRI medicine images, Iboga module, facilitator index, /attention-theft, /alex-azzi, /protecting-your-business, /peyote-mescaline, HumanOS, the peptide quiz). Notes called it "RampRate's own CloudFront", but every file sits in the legacy Manus project's folder and its owner couldn't be confirmed. All 65 uploaded (scripts/rescue-cloudfront-images.ts), code rewritten, host removed from images.remotePatterns, no Sanity document used it. Table in docs/ai/manus-media-rescue.md.</t>
         </is>
       </c>
       <c r="E313" s="14" t="inlineStr">
@@ -8039,7 +8039,7 @@
       <c r="A314" s="4" t="n"/>
       <c r="B314" s="4" t="inlineStr">
         <is>
-          <t>Manifesto/Attention Theft: any diagram/illustration assets used on the mega-page</t>
+          <t>PRI/Kava: medicine reference images (medicine-images.ts), facility images for /facilitator-index</t>
         </is>
       </c>
       <c r="C314" s="13" t="inlineStr">
@@ -8049,7 +8049,7 @@
       </c>
       <c r="D314" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02: 6 of live's 7 are in (now in Sanity); the 7th belongs to the Wall of Shame section left out on purpose.</t>
+          <t>2026-10-02: all in Sanity; image counts match live on PRI, Kava, Iboga, Peyote, facilitator pages.</t>
         </is>
       </c>
       <c r="E314" s="14" t="inlineStr">
@@ -8062,17 +8062,17 @@
       <c r="A315" s="4" t="n"/>
       <c r="B315" s="4" t="inlineStr">
         <is>
-          <t>Assessment result-screen background art (flagged in STATUS.md as a known gap</t>
-        </is>
-      </c>
-      <c r="C315" s="15" t="inlineStr">
-        <is>
-          <t>Remaining</t>
+          <t>Manifesto/Attention Theft: any diagram/illustration assets used on the mega-page</t>
+        </is>
+      </c>
+      <c r="C315" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D315" s="4" t="inlineStr">
         <is>
-          <t>18/20 assessments currently have plain black backgrounds; sourcing themed art here also closes that gap)</t>
+          <t>2026-10-02: 6 of live's 7 are in (now in Sanity); the 7th belongs to the Wall of Shame section left out on purpose.</t>
         </is>
       </c>
       <c r="E315" s="14" t="inlineStr">
@@ -8085,17 +8085,17 @@
       <c r="A316" s="4" t="n"/>
       <c r="B316" s="4" t="inlineStr">
         <is>
-          <t>Chatbot: FauxTony avatar/icon</t>
-        </is>
-      </c>
-      <c r="C316" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Assessment result-screen background art (flagged in STATUS.md as a known gap</t>
+        </is>
+      </c>
+      <c r="C316" s="15" t="inlineStr">
+        <is>
+          <t>Remaining</t>
         </is>
       </c>
       <c r="D316" s="4" t="inlineStr">
         <is>
-          <t>Not needed (2026-10-02): the chatbot phase (Phase 10) was cancelled.</t>
+          <t>18/20 assessments currently have plain black backgrounds; sourcing themed art here also closes that gap)</t>
         </is>
       </c>
       <c r="E316" s="14" t="inlineStr">
@@ -8108,73 +8108,73 @@
       <c r="A317" s="4" t="n"/>
       <c r="B317" s="4" t="inlineStr">
         <is>
+          <t>Chatbot: FauxTony avatar/icon</t>
+        </is>
+      </c>
+      <c r="C317" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D317" s="4" t="inlineStr">
+        <is>
+          <t>Not needed (2026-10-02): the chatbot phase (Phase 10) was cancelled.</t>
+        </is>
+      </c>
+      <c r="E317" s="14" t="inlineStr">
+        <is>
+          <t>Phase 13 — Images Needed in Sanity</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" s="4" t="n"/>
+      <c r="B318" s="4" t="inlineStr">
+        <is>
           <t>Audit client/public/ (including alex-azzi/, brewsoul/ subfolders) for any static assets already sitting there unused that should be pulled i…</t>
         </is>
       </c>
-      <c r="C317" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D317" s="4" t="inlineStr">
+      <c r="C318" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D318" s="4" t="inlineStr">
         <is>
           <t>n rather than re-created. Done 2026-10-02: no images there at all (only llms.txt, a BrewSoul catalog, Manus debug files, design-options.html). Found and fixed a cutover risk instead: live serves two Google site-verification files (/google6881a0411c48b301.html, /alex-azzi/googleedff0185753a4a1f.html) that the new site returned 404 for, so Search Console could lose verification at DNS cutover. Both copied to public/ byte for byte. Not copied: site.webmanifest (its icons don't exist here; Next's app/icon.tsx covers the favicon).</t>
         </is>
       </c>
-      <c r="E317" s="14" t="inlineStr">
+      <c r="E318" s="14" t="inlineStr">
         <is>
           <t>Phase 13 — Images Needed in Sanity</t>
         </is>
       </c>
     </row>
-    <row r="318">
-      <c r="A318" s="10" t="inlineStr">
+    <row r="319">
+      <c r="A319" s="10" t="inlineStr">
         <is>
           <t>Phase 14 — QA &amp; Launch</t>
         </is>
       </c>
-      <c r="B318" s="11" t="n"/>
-      <c r="C318" s="11" t="n"/>
-      <c r="D318" s="12" t="n"/>
-    </row>
-    <row r="319">
-      <c r="A319" s="4" t="n"/>
-      <c r="B319" s="4" t="inlineStr">
-        <is>
-          <t>Mobile responsive pass on every ported section</t>
-        </is>
-      </c>
-      <c r="C319" s="15" t="inlineStr">
-        <is>
-          <t>Remaining</t>
-        </is>
-      </c>
-      <c r="D319" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-29: no page scrolls sideways at 375px any more (114 pages checked in Chrome: every unique page plus 3 of each templated set like blog posts and coffees). Fixed: BrewSoul NextSteps forced 3 columns (and used an inline style), charity-scorecard tab row, /brewsoul/browse filter dropdowns, /the-philosophy hero glow. Still to check by hand: 44px tap targets and Safari iOS. 2026-09-30: 44px tap targets on phones for the shared header, footer, BrewSoul/Kava/HumanOS menus and ~100 standalone links (undersized targets 1,904 → 578; the rest are 24-43px pills/chips that meet WCAG 2.2 AA). axe target-size (WCAG 2.2 AA, with its spacing exception): 0 failures on 114 pages. Safari/iPhone (WebKit, iPhone 14 emulation): all 114 pages load, no sideways scroll, no JS errors; form fields under 16px (iOS zoom-on-tap) fixed site-wide in globals.css. Still to check on a real iPhone: BrewSoul's bottom journey bar showed page text through it in headless WebKit only (taps hit the bar correctly; Chrome renders it solid).</t>
-        </is>
-      </c>
-      <c r="E319" s="14" t="inlineStr">
-        <is>
-          <t>Phase 14 — QA &amp; Launch</t>
-        </is>
-      </c>
+      <c r="B319" s="11" t="n"/>
+      <c r="C319" s="11" t="n"/>
+      <c r="D319" s="12" t="n"/>
     </row>
     <row r="320">
       <c r="A320" s="4" t="n"/>
       <c r="B320" s="4" t="inlineStr">
         <is>
-          <t>Accessibility pass (WCAG AA contrast, 44px touch targets, keyboard nav)</t>
-        </is>
-      </c>
-      <c r="C320" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Mobile responsive pass on every ported section</t>
+        </is>
+      </c>
+      <c r="C320" s="15" t="inlineStr">
+        <is>
+          <t>Remaining</t>
         </is>
       </c>
       <c r="D320" s="4" t="inlineStr">
         <is>
-          <t>same bar as legacy QA_MASTER_PROMPT.md. 2026-09-29 axe-core pass (WCAG 2.1 AA, same 114 pages, production build): all unlabeled dropdowns/inputs and unnamed links fixed; contrast down from 1,453 failing items on 106 pages to 1,038 on 70 (43 pages fully clean). Shared fixes: brand gold #8b6914 → #836311 site-wide (was 4.3:1 on cream, AA needs 4.5), header "⌘K"/social icons, BrewSoul nav and footer, HumanOS footer, Kava footer, assessment intro footnote, post-card image links. 2026-09-30: contrast finished, 0 axe color-contrast failures left on the same 114 pages (production build). Token changes: --kava-saffron #b86a28 → #8e521f, --pri-purple-light #a855f7 → #b87bf9 (on-dark purple only), --crusade-teal #0e7c7c → #0d7373; PriEyebrow goes light purple inside a dark PriSection via group-data-dark/pri; /find-your-me and the journey tracker's dark glass panels 60-70% → 90% (legacy's own 60% glass on beige rendered gray, cream text failed). Everything else: nearest passing shade of the same hue, or gold ↔ gold-light on the wrong background. Left: 18 links inside text marked only by color (need an underline), 44px tap targets, keyboard nav. 2026-09-30: 18 color-only in-text links underlined (axe link-in-text-block: 0 left); keyboard focus visible on every focusable item on 8 sampled pages (two form fields had none, fixed). 2026-10-02 re-run (axe WCAG 2.2 AA, 142 pages × 375/1280px, production build, plus Tab through 40 stops per page): found 1,370 contrast failures (mostly BrewSoul'</t>
+          <t>2026-09-29: no page scrolls sideways at 375px any more (114 pages checked in Chrome: every unique page plus 3 of each templated set like blog posts and coffees). Fixed: BrewSoul NextSteps forced 3 columns (and used an inline style), charity-scorecard tab row, /brewsoul/browse filter dropdowns, /the-philosophy hero glow. Still to check by hand: 44px tap targets and Safari iOS. 2026-09-30: 44px tap targets on phones for the shared header, footer, BrewSoul/Kava/HumanOS menus and ~100 standalone links (undersized targets 1,904 → 578; the rest are 24-43px pills/chips that meet WCAG 2.2 AA). axe target-size (WCAG 2.2 AA, with its spacing exception): 0 failures on 114 pages. Safari/iPhone (WebKit, iPhone 14 emulation): all 114 pages load, no sideways scroll, no JS errors; form fields under 16px (iOS zoom-on-tap) fixed site-wide in globals.css. Still to check on a real iPhone: BrewSoul's bottom journey bar showed page text through it in headless WebKit only (taps hit the bar correctly; Chrome renders it solid).</t>
         </is>
       </c>
       <c r="E320" s="14" t="inlineStr">
@@ -8187,17 +8187,17 @@
       <c r="A321" s="4" t="n"/>
       <c r="B321" s="4" t="inlineStr">
         <is>
-          <t>No dead-end pages (every page links to 2+ others)</t>
-        </is>
-      </c>
-      <c r="C321" s="15" t="inlineStr">
-        <is>
-          <t>Remaining</t>
+          <t>Accessibility pass (WCAG AA contrast, 44px touch targets, keyboard nav)</t>
+        </is>
+      </c>
+      <c r="C321" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D321" s="4" t="inlineStr">
         <is>
-          <t>same bar as legacy MASTER_QUALITY_PROMPT.md 2026-09-30 scan (496 sitemap pages, header/footer links not counted): every page has a way home (the 6 HumanOS pages had none, in legacy too; added a "← TonyGreenberg.com" footer link). ~17 quiz pages only look like dead ends on their intro screen; their result screens link to related assessments. Left for a content decision: ~20 marketing pages (/akbar, /amplifier, /diamond-cut, /ecosystem, /engage, /engine-room, /intel, /invest, /pick-up-the-phone, /protecting-your-business, /published, /speaking, /the-nightstand, /the-territory, /the-web, /under-nda, /pri-calibration, /charity-scorecard and its detail pages) link to only 0-1 other page in their content. The port matches legacy there (legacy was just as sparse), so adding related links is new content and needs the owner's yes.</t>
+          <t>same bar as legacy QA_MASTER_PROMPT.md. 2026-09-29 axe-core pass (WCAG 2.1 AA, same 114 pages, production build): all unlabeled dropdowns/inputs and unnamed links fixed; contrast down from 1,453 failing items on 106 pages to 1,038 on 70 (43 pages fully clean). Shared fixes: brand gold #8b6914 → #836311 site-wide (was 4.3:1 on cream, AA needs 4.5), header "⌘K"/social icons, BrewSoul nav and footer, HumanOS footer, Kava footer, assessment intro footnote, post-card image links. 2026-09-30: contrast finished, 0 axe color-contrast failures left on the same 114 pages (production build). Token changes: --kava-saffron #b86a28 → #8e521f, --pri-purple-light #a855f7 → #b87bf9 (on-dark purple only), --crusade-teal #0e7c7c → #0d7373; PriEyebrow goes light purple inside a dark PriSection via group-data-dark/pri; /find-your-me and the journey tracker's dark glass panels 60-70% → 90% (legacy's own 60% glass on beige rendered gray, cream text failed). Everything else: nearest passing shade of the same hue, or gold ↔ gold-light on the wrong background. Left: 18 links inside text marked only by color (need an underline), 44px tap targets, keyboard nav. 2026-09-30: 18 color-only in-text links underlined (axe link-in-text-block: 0 left); keyboard focus visible on every focusable item on 8 sampled pages (two form fields had none, fixed). 2026-10-02 re-run (axe WCAG 2.2 AA, 142 pages × 375/1280px, production build, plus Tab through 40 stops per page): found 1,370 contrast failures (mostly BrewSoul'</t>
         </is>
       </c>
       <c r="E321" s="14" t="inlineStr">
@@ -8210,7 +8210,7 @@
       <c r="A322" s="4" t="n"/>
       <c r="B322" s="4" t="inlineStr">
         <is>
-          <t>Cross-browser check (Safari iOS in particular, per legacy performance notes) 2026-10-06 WebKit pass (Playwright WebKit, iPhone 13 profile, 1…</t>
+          <t>No dead-end pages (every page links to 2+ others)</t>
         </is>
       </c>
       <c r="C322" s="15" t="inlineStr">
@@ -8220,7 +8220,7 @@
       </c>
       <c r="D322" s="4" t="inlineStr">
         <is>
-          <t>52 pages: every unique page plus 3 of each templated set, production build): no page pans sideways, no failed requests, no JS errors. Found and fixed on the way: upgrade-insecure-requests in the new CSP made Safari fetch every stylesheet and font over https on localhost (dropped; the site is HTTPS-only via HSTS anyway), and .toLocaleString() without a locale caused a hydration error on /brewsoul/chains in Safari (all number formatting now en-US). Left: a check on a real iPhone (Phase 14).</t>
+          <t>same bar as legacy MASTER_QUALITY_PROMPT.md 2026-09-30 scan (496 sitemap pages, header/footer links not counted): every page has a way home (the 6 HumanOS pages had none, in legacy too; added a "← TonyGreenberg.com" footer link). ~17 quiz pages only look like dead ends on their intro screen; their result screens link to related assessments. Left for a content decision: ~20 marketing pages (/akbar, /amplifier, /diamond-cut, /ecosystem, /engage, /engine-room, /intel, /invest, /pick-up-the-phone, /protecting-your-business, /published, /speaking, /the-nightstand, /the-territory, /the-web, /under-nda, /pri-calibration, /charity-scorecard and its detail pages) link to only 0-1 other page in their content. The port matches legacy there (legacy was just as sparse), so adding related links is new content and needs the owner's yes.</t>
         </is>
       </c>
       <c r="E322" s="14" t="inlineStr">
@@ -8233,7 +8233,7 @@
       <c r="A323" s="4" t="n"/>
       <c r="B323" s="4" t="inlineStr">
         <is>
-          <t>Remove noindex only when sign-off is given</t>
+          <t>Cross-browser check (Safari iOS in particular, per legacy performance notes) 2026-10-06 WebKit pass (Playwright WebKit, iPhone 13 profile, 1…</t>
         </is>
       </c>
       <c r="C323" s="15" t="inlineStr">
@@ -8243,7 +8243,7 @@
       </c>
       <c r="D323" s="4" t="inlineStr">
         <is>
-          <t>do not launch indexable by accident (The only noindex is the host-based one for *.netlify.app above, so the real domain is indexable as soon as DNS points at it: sign-off must come before DNS.)</t>
+          <t>52 pages: every unique page plus 3 of each templated set, production build): no page pans sideways, no failed requests, no JS errors. Found and fixed on the way: upgrade-insecure-requests in the new CSP made Safari fetch every stylesheet and font over https on localhost (dropped; the site is HTTPS-only via HSTS anyway), and .toLocaleString() without a locale caused a hydration error on /brewsoul/chains in Safari (all number formatting now en-US). Left: a check on a real iPhone (Phase 14).</t>
         </is>
       </c>
       <c r="E323" s="14" t="inlineStr">
@@ -8256,7 +8256,7 @@
       <c r="A324" s="4" t="n"/>
       <c r="B324" s="4" t="inlineStr">
         <is>
-          <t>Final stakeholder sign-off (Tony/Darryl/Kimberly) on the ported site before DNS cutover</t>
+          <t>Remove noindex only when sign-off is given</t>
         </is>
       </c>
       <c r="C324" s="15" t="inlineStr">
@@ -8264,7 +8264,11 @@
           <t>Remaining</t>
         </is>
       </c>
-      <c r="D324" s="4" t="inlineStr"/>
+      <c r="D324" s="4" t="inlineStr">
+        <is>
+          <t>do not launch indexable by accident (The only noindex is the host-based one for *.netlify.app above, so the real domain is indexable as soon as DNS points at it: sign-off must come before DNS.)</t>
+        </is>
+      </c>
       <c r="E324" s="14" t="inlineStr">
         <is>
           <t>Phase 14 — QA &amp; Launch</t>
@@ -8275,7 +8279,7 @@
       <c r="A325" s="4" t="n"/>
       <c r="B325" s="4" t="inlineStr">
         <is>
-          <t>DNS cutover, legacy app decommissioned only after a stable overlap window</t>
+          <t>Final stakeholder sign-off (Tony/Darryl/Kimberly) on the ported site before DNS cutover</t>
         </is>
       </c>
       <c r="C325" s="15" t="inlineStr">
@@ -8290,23 +8294,42 @@
         </is>
       </c>
     </row>
+    <row r="326">
+      <c r="A326" s="4" t="n"/>
+      <c r="B326" s="4" t="inlineStr">
+        <is>
+          <t>DNS cutover, legacy app decommissioned only after a stable overlap window</t>
+        </is>
+      </c>
+      <c r="C326" s="15" t="inlineStr">
+        <is>
+          <t>Remaining</t>
+        </is>
+      </c>
+      <c r="D326" s="4" t="inlineStr"/>
+      <c r="E326" s="14" t="inlineStr">
+        <is>
+          <t>Phase 14 — QA &amp; Launch</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D325"/>
+  <autoFilter ref="A1:D326"/>
   <mergeCells count="14">
     <mergeCell ref="A150:D150"/>
     <mergeCell ref="A237:D237"/>
     <mergeCell ref="A58:D58"/>
     <mergeCell ref="A258:D258"/>
+    <mergeCell ref="A319:D319"/>
     <mergeCell ref="A209:D209"/>
     <mergeCell ref="A205:D205"/>
     <mergeCell ref="A15:D15"/>
-    <mergeCell ref="A318:D318"/>
     <mergeCell ref="A43:D43"/>
     <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A299:D299"/>
     <mergeCell ref="A183:D183"/>
     <mergeCell ref="A32:D32"/>
     <mergeCell ref="A123:D123"/>
-    <mergeCell ref="A298:D298"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Category pages pre-built (/page/N instead of ?page=N); solid BrewSoul bar
- /blog/category/[slug] read searchParams, so every category page rendered
  per request. Shared CategoryListing + categoryMetadata; page 1 at the
  plain address, pages 2+ at /page/[n] (generateStaticParams,
  dynamicParams = false). Old ?page=N 308s to /page/N (2+ only), /page/1
  308s back, out-of-range is 404. "All essays" arrow is an icon.
- BrewSoul journey bar: solid bg instead of 92% + backdrop-blur, so text
  can't show through where the blur isn't drawn (WebKit); z-9990 canonical.
- Checked: build route table (all category pages SSG), redirects, 404s,
  titles/canonicals, Previous/Next; bar in WebKit + Chrome.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Migration-Status-Report.xlsx
+++ b/Migration-Status-Report.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Remaining Work" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Full Detail'!$A$1:$D$326</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Full Detail'!$A$1:$D$327</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Remaining Work'!$A$1:$D$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -639,15 +639,15 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A5,'Full Detail'!$C$2:$C$326,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A5,'Full Detail'!$C$2:$C$327,"Done")</f>
         <v/>
       </c>
       <c r="C5" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A5,'Full Detail'!$C$2:$C$326,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A5,'Full Detail'!$C$2:$C$327,"Remaining")</f>
         <v/>
       </c>
       <c r="D5" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A5,'Full Detail'!$C$2:$C$326,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A5,'Full Detail'!$C$2:$C$327,"Deferred")</f>
         <v/>
       </c>
       <c r="E5" s="5">
@@ -666,15 +666,15 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A6,'Full Detail'!$C$2:$C$326,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A6,'Full Detail'!$C$2:$C$327,"Done")</f>
         <v/>
       </c>
       <c r="C6" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A6,'Full Detail'!$C$2:$C$326,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A6,'Full Detail'!$C$2:$C$327,"Remaining")</f>
         <v/>
       </c>
       <c r="D6" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A6,'Full Detail'!$C$2:$C$326,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A6,'Full Detail'!$C$2:$C$327,"Deferred")</f>
         <v/>
       </c>
       <c r="E6" s="5">
@@ -693,15 +693,15 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A7,'Full Detail'!$C$2:$C$326,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A7,'Full Detail'!$C$2:$C$327,"Done")</f>
         <v/>
       </c>
       <c r="C7" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A7,'Full Detail'!$C$2:$C$326,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A7,'Full Detail'!$C$2:$C$327,"Remaining")</f>
         <v/>
       </c>
       <c r="D7" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A7,'Full Detail'!$C$2:$C$326,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A7,'Full Detail'!$C$2:$C$327,"Deferred")</f>
         <v/>
       </c>
       <c r="E7" s="5">
@@ -720,15 +720,15 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A8,'Full Detail'!$C$2:$C$326,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A8,'Full Detail'!$C$2:$C$327,"Done")</f>
         <v/>
       </c>
       <c r="C8" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A8,'Full Detail'!$C$2:$C$326,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A8,'Full Detail'!$C$2:$C$327,"Remaining")</f>
         <v/>
       </c>
       <c r="D8" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A8,'Full Detail'!$C$2:$C$326,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A8,'Full Detail'!$C$2:$C$327,"Deferred")</f>
         <v/>
       </c>
       <c r="E8" s="5">
@@ -747,15 +747,15 @@
         </is>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A9,'Full Detail'!$C$2:$C$326,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A9,'Full Detail'!$C$2:$C$327,"Done")</f>
         <v/>
       </c>
       <c r="C9" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A9,'Full Detail'!$C$2:$C$326,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A9,'Full Detail'!$C$2:$C$327,"Remaining")</f>
         <v/>
       </c>
       <c r="D9" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A9,'Full Detail'!$C$2:$C$326,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A9,'Full Detail'!$C$2:$C$327,"Deferred")</f>
         <v/>
       </c>
       <c r="E9" s="5">
@@ -774,15 +774,15 @@
         </is>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A10,'Full Detail'!$C$2:$C$326,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A10,'Full Detail'!$C$2:$C$327,"Done")</f>
         <v/>
       </c>
       <c r="C10" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A10,'Full Detail'!$C$2:$C$326,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A10,'Full Detail'!$C$2:$C$327,"Remaining")</f>
         <v/>
       </c>
       <c r="D10" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A10,'Full Detail'!$C$2:$C$326,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A10,'Full Detail'!$C$2:$C$327,"Deferred")</f>
         <v/>
       </c>
       <c r="E10" s="5">
@@ -801,15 +801,15 @@
         </is>
       </c>
       <c r="B11" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A11,'Full Detail'!$C$2:$C$326,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A11,'Full Detail'!$C$2:$C$327,"Done")</f>
         <v/>
       </c>
       <c r="C11" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A11,'Full Detail'!$C$2:$C$326,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A11,'Full Detail'!$C$2:$C$327,"Remaining")</f>
         <v/>
       </c>
       <c r="D11" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A11,'Full Detail'!$C$2:$C$326,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A11,'Full Detail'!$C$2:$C$327,"Deferred")</f>
         <v/>
       </c>
       <c r="E11" s="5">
@@ -828,15 +828,15 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A12,'Full Detail'!$C$2:$C$326,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A12,'Full Detail'!$C$2:$C$327,"Done")</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A12,'Full Detail'!$C$2:$C$326,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A12,'Full Detail'!$C$2:$C$327,"Remaining")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A12,'Full Detail'!$C$2:$C$326,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A12,'Full Detail'!$C$2:$C$327,"Deferred")</f>
         <v/>
       </c>
       <c r="E12" s="5">
@@ -855,15 +855,15 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A13,'Full Detail'!$C$2:$C$326,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A13,'Full Detail'!$C$2:$C$327,"Done")</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A13,'Full Detail'!$C$2:$C$326,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A13,'Full Detail'!$C$2:$C$327,"Remaining")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A13,'Full Detail'!$C$2:$C$326,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A13,'Full Detail'!$C$2:$C$327,"Deferred")</f>
         <v/>
       </c>
       <c r="E13" s="5">
@@ -882,15 +882,15 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A14,'Full Detail'!$C$2:$C$326,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A14,'Full Detail'!$C$2:$C$327,"Done")</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A14,'Full Detail'!$C$2:$C$326,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A14,'Full Detail'!$C$2:$C$327,"Remaining")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A14,'Full Detail'!$C$2:$C$326,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A14,'Full Detail'!$C$2:$C$327,"Deferred")</f>
         <v/>
       </c>
       <c r="E14" s="5">
@@ -909,15 +909,15 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A15,'Full Detail'!$C$2:$C$326,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A15,'Full Detail'!$C$2:$C$327,"Done")</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A15,'Full Detail'!$C$2:$C$326,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A15,'Full Detail'!$C$2:$C$327,"Remaining")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A15,'Full Detail'!$C$2:$C$326,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A15,'Full Detail'!$C$2:$C$327,"Deferred")</f>
         <v/>
       </c>
       <c r="E15" s="5">
@@ -936,15 +936,15 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A16,'Full Detail'!$C$2:$C$326,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A16,'Full Detail'!$C$2:$C$327,"Done")</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A16,'Full Detail'!$C$2:$C$326,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A16,'Full Detail'!$C$2:$C$327,"Remaining")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A16,'Full Detail'!$C$2:$C$326,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A16,'Full Detail'!$C$2:$C$327,"Deferred")</f>
         <v/>
       </c>
       <c r="E16" s="5">
@@ -963,15 +963,15 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A17,'Full Detail'!$C$2:$C$326,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A17,'Full Detail'!$C$2:$C$327,"Done")</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A17,'Full Detail'!$C$2:$C$326,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A17,'Full Detail'!$C$2:$C$327,"Remaining")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A17,'Full Detail'!$C$2:$C$326,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A17,'Full Detail'!$C$2:$C$327,"Deferred")</f>
         <v/>
       </c>
       <c r="E17" s="5">
@@ -990,15 +990,15 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A18,'Full Detail'!$C$2:$C$326,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A18,'Full Detail'!$C$2:$C$327,"Done")</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A18,'Full Detail'!$C$2:$C$326,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A18,'Full Detail'!$C$2:$C$327,"Remaining")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A18,'Full Detail'!$C$2:$C$326,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A18,'Full Detail'!$C$2:$C$327,"Deferred")</f>
         <v/>
       </c>
       <c r="E18" s="5">
@@ -1017,15 +1017,15 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A19,'Full Detail'!$C$2:$C$326,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A19,'Full Detail'!$C$2:$C$327,"Done")</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A19,'Full Detail'!$C$2:$C$326,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A19,'Full Detail'!$C$2:$C$327,"Remaining")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$326,$A19,'Full Detail'!$C$2:$C$326,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A19,'Full Detail'!$C$2:$C$327,"Deferred")</f>
         <v/>
       </c>
       <c r="E19" s="5">
@@ -1075,7 +1075,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E326"/>
+  <dimension ref="A1:E327"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -7366,7 +7366,7 @@
       <c r="A284" s="4" t="n"/>
       <c r="B284" s="4" t="inlineStr">
         <is>
-          <t>Error pages (2026-10-09, owner asked)</t>
+          <t>Category pages pre-built (2026-10-09)</t>
         </is>
       </c>
       <c r="C284" s="13" t="inlineStr">
@@ -7376,7 +7376,7 @@
       </c>
       <c r="D284" s="4" t="inlineStr">
         <is>
-          <t>404 page now sets its own title ("Page not found") as a server page around live's 3-second redirect (not-found.tsx + components/not-found-redirect.tsx), arrow as an icon; page error screen (error.tsx) uses Next 16's retry (re-fetches), shows a reference code for the server logs, links home and to the site index; new global-error.tsx for failures in the root layout itself (own &lt;html&gt;, plain links). Verified on a production build: missing page, missing essay and missing Kava page return 404 with the right title; a test page that throws returns 500 with the error screen, "Try again" re-fetches; phone and laptop, no sideways scroll (test page removed).</t>
+          <t>/blog/category/[slug] read ?page=N, so every category page was rendered on each request (slower first byte, flagged in the Lighthouse notes). Page numbers are now part of the address (/blog/category/&lt;slug&gt;/page/&lt;n&gt;, generateStaticParams, dynamicParams = false), shared code in src/components/blog/category-listing.tsx; old ?page=N links 308 to the new address (pages 2+ only, so no loop), /page/1 308s to the plain address, a page past the end is a 404; "All essays" back link uses an icon. Verified on a production build: route table shows every category page as pre-built (9 page-1s, 7 later pages), titles and canonicals per page, Previous/Next links, the redirects and the 404s.</t>
         </is>
       </c>
       <c r="E284" s="14" t="inlineStr">
@@ -7389,7 +7389,7 @@
       <c r="A285" s="4" t="n"/>
       <c r="B285" s="4" t="inlineStr">
         <is>
-          <t>SEO audit fixes (2026-10-06)</t>
+          <t>Error pages (2026-10-09, owner asked)</t>
         </is>
       </c>
       <c r="C285" s="13" t="inlineStr">
@@ -7399,7 +7399,7 @@
       </c>
       <c r="D285" s="4" t="inlineStr">
         <is>
-          <t>Checked an outside audit point by point against the code. Fixed: Core Themes cards linked to /?theme=…#essays-archive (not crawlable, counts from a stale hand-kept list) and now link to /blog/category/&lt;slug&gt; with real counts (21/25/20/14, matching the archive pills; THEME_MAP and the ?theme= filter removed); Four Doors cards were &lt;button&gt;s, now real links that still open the modal on a plain click; "DIAGNOSE · ENGAGE" now link to /find-my and /engage; one shared formatPostDate (Asia/Kolkata, src/lib/format-post-date.ts) so a post no longer shows two different dates; the title repeated as the first body paragraph is dropped at render time (legacyBodyLayout); essay cards are h3 under a section h2 (archive, Read next), h2 only on category/search; heading glyphs (◆ ✦) hidden from screen readers; posts send BlogPosting with the author tied to the site Person (@id) plus a BreadcrumbList; descriptive alt on the homepage and BrewSoul heroes; homepage OG image cropped to 1200x630 JPEG. Already fine (audit could not see it): Person/Article schema, Netlify noindex, robots.txt, sitemap, header nav and search, Amazon links carry no affiliate tag. Checked on a production build: type check, lint, build, status codes, browser click test at 375px, no console errors. Implementation pack (Mohammad Danish, 2026-10-05) checked the same day: added og:type/og:site_name back on the 6 pages with their own openGraph (a page-level openGraph replaces the layout one), twitter:creator, and on posts og:url</t>
+          <t>404 page now sets its own title ("Page not found") as a server page around live's 3-second redirect (not-found.tsx + components/not-found-redirect.tsx), arrow as an icon; page error screen (error.tsx) uses Next 16's retry (re-fetches), shows a reference code for the server logs, links home and to the site index; new global-error.tsx for failures in the root layout itself (own &lt;html&gt;, plain links). Verified on a production build: missing page, missing essay and missing Kava page return 404 with the right title; a test page that throws returns 500 with the error screen, "Try again" re-fetches; phone and laptop, no sideways scroll (test page removed).</t>
         </is>
       </c>
       <c r="E285" s="14" t="inlineStr">
@@ -7412,17 +7412,17 @@
       <c r="A286" s="4" t="n"/>
       <c r="B286" s="4" t="inlineStr">
         <is>
-          <t>SEO audit items needing a yes (2026-10-06)</t>
-        </is>
-      </c>
-      <c r="C286" s="15" t="inlineStr">
-        <is>
-          <t>Remaining</t>
+          <t>SEO audit fixes (2026-10-06)</t>
+        </is>
+      </c>
+      <c r="C286" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D286" s="4" t="inlineStr">
         <is>
-          <t>the pack's new copy (homepage title/description, five-cups title, description, short answer, FAQ, heading rewrites, entity statement, newsletter block, author box, health disclaimer, COA wording); "Further Reading" shown twice on posts (merge the lists?); long post title (84 chars), homepage description length and obsolete keywords tag, slugs (/blog/five-cups, the -2 slug; would need redirects), "Six lenses" over four cards, sources for health claims and proof for "$10B+", "Certified B Corp", "Validity: 91", legal review of the homepage Case File banner, ABIT waitlist disclosures, one contact email, the two one-post categories, fewer homepage CTAs / email signup / table of contents / explaining "COA".</t>
+          <t>Checked an outside audit point by point against the code. Fixed: Core Themes cards linked to /?theme=…#essays-archive (not crawlable, counts from a stale hand-kept list) and now link to /blog/category/&lt;slug&gt; with real counts (21/25/20/14, matching the archive pills; THEME_MAP and the ?theme= filter removed); Four Doors cards were &lt;button&gt;s, now real links that still open the modal on a plain click; "DIAGNOSE · ENGAGE" now link to /find-my and /engage; one shared formatPostDate (Asia/Kolkata, src/lib/format-post-date.ts) so a post no longer shows two different dates; the title repeated as the first body paragraph is dropped at render time (legacyBodyLayout); essay cards are h3 under a section h2 (archive, Read next), h2 only on category/search; heading glyphs (◆ ✦) hidden from screen readers; posts send BlogPosting with the author tied to the site Person (@id) plus a BreadcrumbList; descriptive alt on the homepage and BrewSoul heroes; homepage OG image cropped to 1200x630 JPEG. Already fine (audit could not see it): Person/Article schema, Netlify noindex, robots.txt, sitemap, header nav and search, Amazon links carry no affiliate tag. Checked on a production build: type check, lint, build, status codes, browser click test at 375px, no console errors. Implementation pack (Mohammad Danish, 2026-10-05) checked the same day: added og:type/og:site_name back on the 6 pages with their own openGraph (a page-level openGraph replaces the layout one), twitter:creator, and on posts og:url</t>
         </is>
       </c>
       <c r="E286" s="14" t="inlineStr">
@@ -7435,7 +7435,7 @@
       <c r="A287" s="4" t="n"/>
       <c r="B287" s="4" t="inlineStr">
         <is>
-          <t>Connect Google Search Console + GA4 to the new deployment on day one of cutover</t>
+          <t>SEO audit items needing a yes (2026-10-06)</t>
         </is>
       </c>
       <c r="C287" s="15" t="inlineStr">
@@ -7443,7 +7443,11 @@
           <t>Remaining</t>
         </is>
       </c>
-      <c r="D287" s="4" t="inlineStr"/>
+      <c r="D287" s="4" t="inlineStr">
+        <is>
+          <t>the pack's new copy (homepage title/description, five-cups title, description, short answer, FAQ, heading rewrites, entity statement, newsletter block, author box, health disclaimer, COA wording); "Further Reading" shown twice on posts (merge the lists?); long post title (84 chars), homepage description length and obsolete keywords tag, slugs (/blog/five-cups, the -2 slug; would need redirects), "Six lenses" over four cards, sources for health claims and proof for "$10B+", "Certified B Corp", "Validity: 91", legal review of the homepage Case File banner, ABIT waitlist disclosures, one contact email, the two one-post categories, fewer homepage CTAs / email signup / table of contents / explaining "COA".</t>
+        </is>
+      </c>
       <c r="E287" s="14" t="inlineStr">
         <is>
           <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
@@ -7454,19 +7458,15 @@
       <c r="A288" s="4" t="n"/>
       <c r="B288" s="4" t="inlineStr">
         <is>
-          <t>Restore/adapt the manus.space triple-layer noindex lockdown pattern for any remaining staging URLs</t>
-        </is>
-      </c>
-      <c r="C288" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D288" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-01: the Netlify copy (tonygreenberg-website.netlify.app) and every deploy preview had no noindex at all, so Google could index a duplicate of the site. next.config.ts headers() now sends X-Robots-Tag: noindex, nofollow on any *.netlify.app host only; tonygreenberg.com is unaffected, so nothing to remove at cutover. Tested with Host headers on a production build.</t>
-        </is>
-      </c>
+          <t>Connect Google Search Console + GA4 to the new deployment on day one of cutover</t>
+        </is>
+      </c>
+      <c r="C288" s="15" t="inlineStr">
+        <is>
+          <t>Remaining</t>
+        </is>
+      </c>
+      <c r="D288" s="4" t="inlineStr"/>
       <c r="E288" s="14" t="inlineStr">
         <is>
           <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
@@ -7477,7 +7477,7 @@
       <c r="A289" s="4" t="n"/>
       <c r="B289" s="4" t="inlineStr">
         <is>
-          <t>"Keep going" strip above the footer on every page (2026-10-07)</t>
+          <t>Restore/adapt the manus.space triple-layer noindex lockdown pattern for any remaining staging URLs</t>
         </is>
       </c>
       <c r="C289" s="13" t="inlineStr">
@@ -7487,7 +7487,7 @@
       </c>
       <c r="D289" s="4" t="inlineStr">
         <is>
-          <t>legacy's WhereNext (deferred in Phase 3, never picked up) with its per-page suggestions, Home · Site Index · All Assessments; links pointed at current routes.</t>
+          <t>2026-10-01: the Netlify copy (tonygreenberg-website.netlify.app) and every deploy preview had no noindex at all, so Google could index a duplicate of the site. next.config.ts headers() now sends X-Robots-Tag: noindex, nofollow on any *.netlify.app host only; tonygreenberg.com is unaffected, so nothing to remove at cutover. Tested with Host headers on a production build.</t>
         </is>
       </c>
       <c r="E289" s="14" t="inlineStr">
@@ -7500,7 +7500,7 @@
       <c r="A290" s="4" t="n"/>
       <c r="B290" s="4" t="inlineStr">
         <is>
-          <t>Live-only and redesigned pages from the 2026-10-07 page sweep (188 pages compared with live)</t>
+          <t>"Keep going" strip above the footer on every page (2026-10-07)</t>
         </is>
       </c>
       <c r="C290" s="13" t="inlineStr">
@@ -7510,7 +7510,7 @@
       </c>
       <c r="D290" s="4" t="inlineStr">
         <is>
-          <t>/the-index rebuilt from live's code (20 concepts, related-word search across essays and site pages, full-text search on the server, "three related places to go next"; the old redirect to /search removed and its links, including the "Site Index" link in "Keep going", point at it again); /the-mirror (and /life-assessment) opens on live's intro (dark hero, "What We Measure" with the six areas, "The Ecosystem"), rebuilt as a step registry (rule 19); /essays header, order and column like live; /about "What They Say" styled like live (live picks 3 of the same 19 quotes at random; ours shows a fixed 3 so they're in the server HTML); /impact-futurism list titles and subtitles; /supplier-intake is a real page again with live's Stage 1 form; /seven-doors and /projects redirect home like live; /impact, /health, /library, /built-on-manus, /heroes are 404 on live too. Left as is on purpose: /blog stays our archive page (on live it repeats the homepage), the email gates on /framework and /peptide-supply-chain, the attention-theft Wall of Shame.</t>
+          <t>legacy's WhereNext (deferred in Phase 3, never picked up) with its per-page suggestions, Home · Site Index · All Assessments; links pointed at current routes.</t>
         </is>
       </c>
       <c r="E290" s="14" t="inlineStr">
@@ -7523,7 +7523,7 @@
       <c r="A291" s="4" t="n"/>
       <c r="B291" s="4" t="inlineStr">
         <is>
-          <t>/alex-azzi locked like live (2026-10-07, owner said match it)</t>
+          <t>Live-only and redesigned pages from the 2026-10-07 page sweep (188 pages compared with live)</t>
         </is>
       </c>
       <c r="C291" s="13" t="inlineStr">
@@ -7533,7 +7533,7 @@
       </c>
       <c r="D291" s="4" t="inlineStr">
         <is>
-          <t>same server-checked password as the locked essay (GATED_POST_PASSWORD, now also set in Netlify), live's "Restricted Access" screen, the report not in the page until unlocked, out of search and the sitemap.</t>
+          <t>/the-index rebuilt from live's code (20 concepts, related-word search across essays and site pages, full-text search on the server, "three related places to go next"; the old redirect to /search removed and its links, including the "Site Index" link in "Keep going", point at it again); /the-mirror (and /life-assessment) opens on live's intro (dark hero, "What We Measure" with the six areas, "The Ecosystem"), rebuilt as a step registry (rule 19); /essays header, order and column like live; /about "What They Say" styled like live (live picks 3 of the same 19 quotes at random; ours shows a fixed 3 so they're in the server HTML); /impact-futurism list titles and subtitles; /supplier-intake is a real page again with live's Stage 1 form; /seven-doors and /projects redirect home like live; /impact, /health, /library, /built-on-manus, /heroes are 404 on live too. Left as is on purpose: /blog stays our archive page (on live it repeats the homepage), the email gates on /framework and /peptide-supply-chain, the attention-theft Wall of Shame.</t>
         </is>
       </c>
       <c r="E291" s="14" t="inlineStr">
@@ -7546,7 +7546,7 @@
       <c r="A292" s="4" t="n"/>
       <c r="B292" s="4" t="inlineStr">
         <is>
-          <t>Live's title fonts and sizes (2026-10-07, "fix the style")</t>
+          <t>/alex-azzi locked like live (2026-10-07, owner said match it)</t>
         </is>
       </c>
       <c r="C292" s="13" t="inlineStr">
@@ -7556,7 +7556,7 @@
       </c>
       <c r="D292" s="4" t="inlineStr">
         <is>
-          <t>measured every page's title font, weight, size and label colour on live vs ours (136 pages). Now like live: Kava headings in Fraunces, HumanOS in Space Grotesk, the peptide tools / charity scorecard / thesis threads in the system serif, America Unbundled in the Iowan Old Style stack at live's size, /akbar in Fraunces 900, friend-gate and post-intervention in Georgia, and live's title sizes on peptide-matrix, peptide-supply-chain, rip-peptide-sciences and the HumanOS pages. Fonts load only on the pages that use them (src/lib/fonts/page-fonts.ts). Label colours stay the darker AA-contrast versions where live's lighter ones fail on a light background.</t>
+          <t>same server-checked password as the locked essay (GATED_POST_PASSWORD, now also set in Netlify), live's "Restricted Access" screen, the report not in the page until unlocked, out of search and the sitemap.</t>
         </is>
       </c>
       <c r="E292" s="14" t="inlineStr">
@@ -7569,7 +7569,7 @@
       <c r="A293" s="4" t="n"/>
       <c r="B293" s="4" t="inlineStr">
         <is>
-          <t>Peptide page images rescued into Sanity and wired (2026-10-07)</t>
+          <t>Live's title fonts and sizes (2026-10-07, "fix the style")</t>
         </is>
       </c>
       <c r="C293" s="13" t="inlineStr">
@@ -7579,7 +7579,7 @@
       </c>
       <c r="D293" s="4" t="inlineStr">
         <is>
-          <t>/peptide-watch hero plus its 11 section banners, /peptide-matrix and /peptide-supply-chain heroes, the /peptide-hall-of-shame hero (scripts/rescue-2026-10-07-peptide-images.ts, logged in docs/ai/manus-media-rescue.md).</t>
+          <t>measured every page's title font, weight, size and label colour on live vs ours (136 pages). Now like live: Kava headings in Fraunces, HumanOS in Space Grotesk, the peptide tools / charity scorecard / thesis threads in the system serif, America Unbundled in the Iowan Old Style stack at live's size, /akbar in Fraunces 900, friend-gate and post-intervention in Georgia, and live's title sizes on peptide-matrix, peptide-supply-chain, rip-peptide-sciences and the HumanOS pages. Fonts load only on the pages that use them (src/lib/fonts/page-fonts.ts). Label colours stay the darker AA-contrast versions where live's lighter ones fail on a light background.</t>
         </is>
       </c>
       <c r="E293" s="14" t="inlineStr">
@@ -7592,7 +7592,7 @@
       <c r="A294" s="4" t="n"/>
       <c r="B294" s="4" t="inlineStr">
         <is>
-          <t>Live's editorial redesign, first group (2026-10-07)</t>
+          <t>Peptide page images rescued into Sanity and wired (2026-10-07)</t>
         </is>
       </c>
       <c r="C294" s="13" t="inlineStr">
@@ -7602,7 +7602,7 @@
       </c>
       <c r="D294" s="4" t="inlineStr">
         <is>
-          <t>dark top sections, narrow single text column, short red section rules and dark call-to-action bands on /invest, /amplifier, /community (now "Sign In to Join the Community", linking our real sign-in; live's made-up counters left out), /framework, /the-letter (daily provocation with "Share this thought" and "Search past provocations"), /engage, /diamond-cut, /ecosystem and the homepage's "The thinking doesn't stop here" band. Kept on purpose: AA-contrast colours where live's fail, "Enter the Gate" instead of live's $5,000 checkout on /diamond-cut.</t>
+          <t>/peptide-watch hero plus its 11 section banners, /peptide-matrix and /peptide-supply-chain heroes, the /peptide-hall-of-shame hero (scripts/rescue-2026-10-07-peptide-images.ts, logged in docs/ai/manus-media-rescue.md).</t>
         </is>
       </c>
       <c r="E294" s="14" t="inlineStr">
@@ -7615,7 +7615,7 @@
       <c r="A295" s="4" t="n"/>
       <c r="B295" s="4" t="inlineStr">
         <is>
-          <t>Live's redesign, second group (done 2026-10-08)</t>
+          <t>Live's editorial redesign, first group (2026-10-07)</t>
         </is>
       </c>
       <c r="C295" s="13" t="inlineStr">
@@ -7625,7 +7625,7 @@
       </c>
       <c r="D295" s="4" t="inlineStr">
         <is>
-          <t>re-measured all 18 pages on live vs a fresh production build (title font/size/weight/colour, labels, hero images). Already matching from 2026-10-07: /the-web, /spirits, /iboga-ibogaine (weight 800), /living-declaration, BrewSoul photo on /brewsoul, /brewsoul/browse, /brewsoul/first-sip (live has none there either), /quiz_25q, /recent-creations. Fixed today: /find-your-journey (64px title, red label), /impact-dashboard (64px title in essay ink, label spacing), red labels on /published and /speaking (plus its "rooms" chips), /soulscore "by ImpactSoul" label, /pri-calibration title (weight 900, solid cream, was a purple gradient), /clients (live's narrow 546px column for the whole page, 56px title, roomier stats band, cards 2 per row; two static inline styles moved to classes), /brewsoul/guest (live's BrewSoul photo on the guest card instead of "SN" initials, labels in capitals), /humanos/connect (cards line up with the title), /peptide-hall-of-shame (stats and label readable light gold; were dark gold on dark). Typed arrows on the touched links are icons now (rule 18). Deliberately not copied from live (new CONTRIBUTING rule 20, owner 2026-10-08): red labels on dark bands use #E07A80 (live's #8E1E25 on black is about 2:1, unreadable); /recent-creations keeps our darker label colours (live's fail contrast on white); /humanos/connect keeps "Start Reading" (that card links to the philosophy page, the quiz live's "Start the Assessment" implies doesn't exist). Checked: type check, l</t>
+          <t>dark top sections, narrow single text column, short red section rules and dark call-to-action bands on /invest, /amplifier, /community (now "Sign In to Join the Community", linking our real sign-in; live's made-up counters left out), /framework, /the-letter (daily provocation with "Share this thought" and "Search past provocations"), /engage, /diamond-cut, /ecosystem and the homepage's "The thinking doesn't stop here" band. Kept on purpose: AA-contrast colours where live's fail, "Enter the Gate" instead of live's $5,000 checkout on /diamond-cut.</t>
         </is>
       </c>
       <c r="E295" s="14" t="inlineStr">
@@ -7638,7 +7638,7 @@
       <c r="A296" s="4" t="n"/>
       <c r="B296" s="4" t="inlineStr">
         <is>
-          <t>BrewSoul top of page (2026-10-08, owner: "button in the center at the top doesn't look good")</t>
+          <t>Live's redesign, second group (done 2026-10-08)</t>
         </is>
       </c>
       <c r="C296" s="13" t="inlineStr">
@@ -7648,7 +7648,7 @@
       </c>
       <c r="D296" s="4" t="inlineStr">
         <is>
-          <t>the category badge ("Deep Research" etc.) sat centred in an empty strip, squeezed against the hero, because we copied live's doubled 52px top gap. Now one gap everywhere and the badge floats in the top-left corner, lined up with the BrewSoul logo (brewsoul-main.tsx, category-badge.tsx); checked on all 26 badge pages at 3 widths that it covers nothing. BrewSoul menu: on tablets (768-1023px) the links were cut off and "More" was hidden with no menu button at all; now the menu button shows below 1024px, 5 links + "More" from 1024px, all 8 from 1280px, "More" always visible.</t>
+          <t>re-measured all 18 pages on live vs a fresh production build (title font/size/weight/colour, labels, hero images). Already matching from 2026-10-07: /the-web, /spirits, /iboga-ibogaine (weight 800), /living-declaration, BrewSoul photo on /brewsoul, /brewsoul/browse, /brewsoul/first-sip (live has none there either), /quiz_25q, /recent-creations. Fixed today: /find-your-journey (64px title, red label), /impact-dashboard (64px title in essay ink, label spacing), red labels on /published and /speaking (plus its "rooms" chips), /soulscore "by ImpactSoul" label, /pri-calibration title (weight 900, solid cream, was a purple gradient), /clients (live's narrow 546px column for the whole page, 56px title, roomier stats band, cards 2 per row; two static inline styles moved to classes), /brewsoul/guest (live's BrewSoul photo on the guest card instead of "SN" initials, labels in capitals), /humanos/connect (cards line up with the title), /peptide-hall-of-shame (stats and label readable light gold; were dark gold on dark). Typed arrows on the touched links are icons now (rule 18). Deliberately not copied from live (new CONTRIBUTING rule 20, owner 2026-10-08): red labels on dark bands use #E07A80 (live's #8E1E25 on black is about 2:1, unreadable); /recent-creations keeps our darker label colours (live's fail contrast on white); /humanos/connect keeps "Start Reading" (that card links to the philosophy page, the quiz live's "Start the Assessment" implies doesn't exist). Checked: type check, l</t>
         </is>
       </c>
       <c r="E296" s="14" t="inlineStr">
@@ -7661,7 +7661,7 @@
       <c r="A297" s="4" t="n"/>
       <c r="B297" s="4" t="inlineStr">
         <is>
-          <t>/pri-efficacy's "Simulation / Live Calibrations" switch like live (2026-10-08)</t>
+          <t>BrewSoul top of page (2026-10-08, owner: "button in the center at the top doesn't look good")</t>
         </is>
       </c>
       <c r="C297" s="13" t="inlineStr">
@@ -7671,7 +7671,7 @@
       </c>
       <c r="D297" s="4" t="inlineStr">
         <is>
-          <t>shadcn Tabs, both panels in the server HTML (forceMount). The Live tab reads real aggregate numbers from pri_calibrations (getPriLiveStats() in src/lib/pri-research.ts: totals, opt-ins, average score per dimension; no rows leave the server), page stays static and refreshes every 10 minutes. Until the Supabase scripts are run (Phase 2) it says the numbers "aren't available just now" instead of a fake zero. Checked: build (○, 10m), server HTML has both tabs, tab switch at 390/1280px, no JS errors. Re-check with real numbers once the table exists.</t>
+          <t>the category badge ("Deep Research" etc.) sat centred in an empty strip, squeezed against the hero, because we copied live's doubled 52px top gap. Now one gap everywhere and the badge floats in the top-left corner, lined up with the BrewSoul logo (brewsoul-main.tsx, category-badge.tsx); checked on all 26 badge pages at 3 widths that it covers nothing. BrewSoul menu: on tablets (768-1023px) the links were cut off and "More" was hidden with no menu button at all; now the menu button shows below 1024px, 5 links + "More" from 1024px, all 8 from 1280px, "More" always visible.</t>
         </is>
       </c>
       <c r="E297" s="14" t="inlineStr">
@@ -7684,63 +7684,63 @@
       <c r="A298" s="4" t="n"/>
       <c r="B298" s="4" t="inlineStr">
         <is>
+          <t>/pri-efficacy's "Simulation / Live Calibrations" switch like live (2026-10-08)</t>
+        </is>
+      </c>
+      <c r="C298" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D298" s="4" t="inlineStr">
+        <is>
+          <t>shadcn Tabs, both panels in the server HTML (forceMount). The Live tab reads real aggregate numbers from pri_calibrations (getPriLiveStats() in src/lib/pri-research.ts: totals, opt-ins, average score per dimension; no rows leave the server), page stays static and refreshes every 10 minutes. Until the Supabase scripts are run (Phase 2) it says the numbers "aren't available just now" instead of a fake zero. Checked: build (○, 10m), server HTML has both tabs, tab switch at 390/1280px, no JS errors. Re-check with real numbers once the table exists.</t>
+        </is>
+      </c>
+      <c r="E298" s="14" t="inlineStr">
+        <is>
+          <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" s="4" t="n"/>
+      <c r="B299" s="4" t="inlineStr">
+        <is>
           <t>/brewsoul/browse hero readable (2026-10-08, owner said go ahead)</t>
         </is>
       </c>
-      <c r="C298" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D298" s="4" t="inlineStr">
+      <c r="C299" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D299" s="4" t="inlineStr">
         <is>
           <t>a soft cream glow behind the title block so "The Catalog", the subtitle and the stat labels read clearly over the coffee photo (live is hard to read there too; rule 20). Photo still shows around the edges. Checked at 390/1280px.</t>
         </is>
       </c>
-      <c r="E298" s="14" t="inlineStr">
+      <c r="E299" s="14" t="inlineStr">
         <is>
           <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
         </is>
       </c>
     </row>
-    <row r="299">
-      <c r="A299" s="10" t="inlineStr">
+    <row r="300">
+      <c r="A300" s="10" t="inlineStr">
         <is>
           <t>Phase 13 — Images Needed in Sanity</t>
         </is>
       </c>
-      <c r="B299" s="11" t="n"/>
-      <c r="C299" s="11" t="n"/>
-      <c r="D299" s="12" t="n"/>
-    </row>
-    <row r="300">
-      <c r="A300" s="4" t="n"/>
-      <c r="B300" s="4" t="inlineStr">
-        <is>
-          <t>Manus media rescue (2026-09-29)</t>
-        </is>
-      </c>
-      <c r="C300" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D300" s="4" t="inlineStr">
-        <is>
-          <t>all 94 Manus-hosted image/video references in the legacy source (/api/img/, /manus-storage/) were checked live. 91 were still downloadable, including the /akbar photos the entry below calls "permanently lost", and all 91 are now Sanity assets (scripts/rescue-manus-media.ts; Sanity dedupes by SHA-1). 3 were gone (HTTP 502). The manifest docs/ai/manus-media-rescue.md maps each one to the legacy files that used it and its Sanity URL. They are not wired into pages yet: go page by page, with real alt text. /facilitator-index's two diagrams are done (scripts/rescue-facilitator-images.ts).</t>
-        </is>
-      </c>
-      <c r="E300" s="14" t="inlineStr">
-        <is>
-          <t>Phase 13 — Images Needed in Sanity</t>
-        </is>
-      </c>
+      <c r="B300" s="11" t="n"/>
+      <c r="C300" s="11" t="n"/>
+      <c r="D300" s="12" t="n"/>
     </row>
     <row r="301">
       <c r="A301" s="4" t="n"/>
       <c r="B301" s="4" t="inlineStr">
         <is>
-          <t>Favicon</t>
+          <t>Manus media rescue (2026-09-29)</t>
         </is>
       </c>
       <c r="C301" s="13" t="inlineStr">
@@ -7750,7 +7750,7 @@
       </c>
       <c r="D301" s="4" t="inlineStr">
         <is>
-          <t>real "G" brand mark generated from the header's actual wordmark treatment (src/app/icon.tsx), see Phase 3</t>
+          <t>all 94 Manus-hosted image/video references in the legacy source (/api/img/, /manus-storage/) were checked live. 91 were still downloadable, including the /akbar photos the entry below calls "permanently lost", and all 91 are now Sanity assets (scripts/rescue-manus-media.ts; Sanity dedupes by SHA-1). 3 were gone (HTTP 502). The manifest docs/ai/manus-media-rescue.md maps each one to the legacy files that used it and its Sanity URL. They are not wired into pages yet: go page by page, with real alt text. /facilitator-index's two diagrams are done (scripts/rescue-facilitator-images.ts).</t>
         </is>
       </c>
       <c r="E301" s="14" t="inlineStr">
@@ -7763,17 +7763,17 @@
       <c r="A302" s="4" t="n"/>
       <c r="B302" s="4" t="inlineStr">
         <is>
-          <t>Site-wide: logo (light + dark) beyond the current text wordmark</t>
-        </is>
-      </c>
-      <c r="C302" s="15" t="inlineStr">
-        <is>
-          <t>Remaining</t>
+          <t>Favicon</t>
+        </is>
+      </c>
+      <c r="C302" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D302" s="4" t="inlineStr">
         <is>
-          <t>(Default/fallback OG image 1200×630 exists: public/images/default-og.png, checked 2026-10-02.)</t>
+          <t>real "G" brand mark generated from the header's actual wordmark treatment (src/app/icon.tsx), see Phase 3</t>
         </is>
       </c>
       <c r="E302" s="14" t="inlineStr">
@@ -7786,17 +7786,17 @@
       <c r="A303" s="4" t="n"/>
       <c r="B303" s="4" t="inlineStr">
         <is>
-          <t>Author photo(s) for blog author schema (Tony Greenberg headshot at minimum)</t>
-        </is>
-      </c>
-      <c r="C303" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Site-wide: logo (light + dark) beyond the current text wordmark</t>
+        </is>
+      </c>
+      <c r="C303" s="15" t="inlineStr">
+        <is>
+          <t>Remaining</t>
         </is>
       </c>
       <c r="D303" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02: the rescued headshot is already the author avatar in Sanity; now also in every post's Article JSON-LD (author image + url /about). The JSON-LD publisher logo pointed at /favicon.ico, a 404 here; now /icon.</t>
+          <t>(Default/fallback OG image 1200×630 exists: public/images/default-og.png, checked 2026-10-02.)</t>
         </is>
       </c>
       <c r="E303" s="14" t="inlineStr">
@@ -7809,7 +7809,7 @@
       <c r="A304" s="4" t="n"/>
       <c r="B304" s="4" t="inlineStr">
         <is>
-          <t>Blog hero images</t>
+          <t>Author photo(s) for blog author schema (Tony Greenberg headshot at minimum)</t>
         </is>
       </c>
       <c r="C304" s="13" t="inlineStr">
@@ -7819,7 +7819,7 @@
       </c>
       <c r="D304" s="4" t="inlineStr">
         <is>
-          <t>audited, then migrated. Final state:</t>
+          <t>2026-10-02: the rescued headshot is already the author avatar in Sanity; now also in every post's Article JSON-LD (author image + url /about). The JSON-LD publisher logo pointed at /favicon.ico, a 404 here; now /icon.</t>
         </is>
       </c>
       <c r="E304" s="14" t="inlineStr">
@@ -7832,7 +7832,7 @@
       <c r="A305" s="4" t="n"/>
       <c r="B305" s="4" t="inlineStr">
         <is>
-          <t>22 posts have a real hero image, now live in Sanity (17 already on RampRate's own CloudFront + 4 rescued from the legacy /api/img/ proxy + 1…</t>
+          <t>Blog hero images</t>
         </is>
       </c>
       <c r="C305" s="13" t="inlineStr">
@@ -7842,7 +7842,7 @@
       </c>
       <c r="D305" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> rescued from /manus-storage/, all pulled over by migrate-blog-posts.ts before Manus is decommissioned)</t>
+          <t>audited, then migrated. Final state:</t>
         </is>
       </c>
       <c r="E305" s="14" t="inlineStr">
@@ -7855,7 +7855,7 @@
       <c r="A306" s="4" t="n"/>
       <c r="B306" s="4" t="inlineStr">
         <is>
-          <t>7 more posts got a real, unique hero image rescued from the live legacy site's newly-added art this pass (scripts/rescue-2026-09-blog-images…</t>
+          <t>22 posts have a real hero image, now live in Sanity (17 already on RampRate's own CloudFront + 4 rescued from the legacy /api/img/ proxy + 1…</t>
         </is>
       </c>
       <c r="C306" s="13" t="inlineStr">
@@ -7865,7 +7865,7 @@
       </c>
       <c r="D306" s="4" t="inlineStr">
         <is>
-          <t>.ts — see the correction note above): california-toll-roads-legalized-scam, the-1000-hour-hold, conscious-capital-partnership-ecosystem, the-peptide-truth-65m-fraud-industry-vs-life-changing-medicine, clear-communication, building-services-market-transhuman-era, heart-protocol-addendum.</t>
+          <t xml:space="preserve"> rescued from /manus-storage/, all pulled over by migrate-blog-posts.ts before Manus is decommissioned)</t>
         </is>
       </c>
       <c r="E306" s="14" t="inlineStr">
@@ -7878,17 +7878,17 @@
       <c r="A307" s="4" t="n"/>
       <c r="B307" s="4" t="inlineStr">
         <is>
-          <t>92 posts still need a real, unique hero image</t>
-        </is>
-      </c>
-      <c r="C307" s="15" t="inlineStr">
-        <is>
-          <t>Remaining</t>
+          <t>7 more posts got a real, unique hero image rescued from the live legacy site's newly-added art this pass (scripts/rescue-2026-09-blog-images…</t>
+        </is>
+      </c>
+      <c r="C307" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D307" s="4" t="inlineStr">
         <is>
-          <t>(down from 99). Tracked one row per post, with a suggested image-generation prompt, in BLOG-IMAGE-BRIEFS.md — work through that file and check items off there, not here. No image-generation tool was connected in this environment as of this writing; either connect one (e.g. an MCP image-gen extension), source these manually/with a designer then upload via Sanity Studio (/studio), or re-check the live legacy site periodically per the correction note above.</t>
+          <t>.ts — see the correction note above): california-toll-roads-legalized-scam, the-1000-hour-hold, conscious-capital-partnership-ecosystem, the-peptide-truth-65m-fraud-industry-vs-life-changing-medicine, clear-communication, building-services-market-transhuman-era, heart-protocol-addendum.</t>
         </is>
       </c>
       <c r="E307" s="14" t="inlineStr">
@@ -7901,17 +7901,17 @@
       <c r="A308" s="4" t="n"/>
       <c r="B308" s="4" t="inlineStr">
         <is>
-          <t>Blog: per-post OG image if different from hero (many posts can reuse hero as OG)</t>
-        </is>
-      </c>
-      <c r="C308" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>92 posts still need a real, unique hero image</t>
+        </is>
+      </c>
+      <c r="C308" s="15" t="inlineStr">
+        <is>
+          <t>Remaining</t>
         </is>
       </c>
       <c r="D308" s="4" t="inlineStr">
         <is>
-          <t>Confirmed 2026-10-02: generateMetadata uses seo.ogImage, else the hero, else the default OG image.</t>
+          <t>(down from 99). Tracked one row per post, with a suggested image-generation prompt, in BLOG-IMAGE-BRIEFS.md — work through that file and check items off there, not here. No image-generation tool was connected in this environment as of this writing; either connect one (e.g. an MCP image-gen extension), source these manually/with a designer then upload via Sanity Studio (/studio), or re-check the live legacy site periodically per the correction note above.</t>
         </is>
       </c>
       <c r="E308" s="14" t="inlineStr">
@@ -7924,7 +7924,7 @@
       <c r="A309" s="4" t="n"/>
       <c r="B309" s="4" t="inlineStr">
         <is>
-          <t>Marketing pages</t>
+          <t>Blog: per-post OG image if different from hero (many posts can reuse hero as OG)</t>
         </is>
       </c>
       <c r="C309" s="13" t="inlineStr">
@@ -7934,7 +7934,7 @@
       </c>
       <c r="D309" s="4" t="inlineStr">
         <is>
-          <t>hero/section images for /the-letter, /the-territory, /engine-room, /the-body, /the-nightstand, /recent-creations (portfolio thumbnails), /published (publication logos), /clients (client logos — confirm licensing before re-hosting). Checked against live 2026-10-02: same image count on every one; /the-territory, /engine-room, /recent-creations, /published, /clients have no images on live either.</t>
+          <t>Confirmed 2026-10-02: generateMetadata uses seo.ogImage, else the hero, else the default OG image.</t>
         </is>
       </c>
       <c r="E309" s="14" t="inlineStr">
@@ -7947,7 +7947,7 @@
       <c r="A310" s="4" t="n"/>
       <c r="B310" s="4" t="inlineStr">
         <is>
-          <t>/akbar essay images</t>
+          <t>Marketing pages</t>
         </is>
       </c>
       <c r="C310" s="13" t="inlineStr">
@@ -7957,7 +7957,7 @@
       </c>
       <c r="D310" s="4" t="inlineStr">
         <is>
-          <t>not lost after all: 20 of the 21 were rescued into Sanity by scripts/rescue-manus-media.ts (2026-09-28) and are wired back in legacy's layout (hero mosaic, JC portrait, 2x2 grid, 3 full-bleeds, 3-up strip, footer gallery) as of 2026-09-29. Only slider-3 was gone (HTTP 502); the hero mosaic is 4 tiles instead of 5.</t>
+          <t>hero/section images for /the-letter, /the-territory, /engine-room, /the-body, /the-nightstand, /recent-creations (portfolio thumbnails), /published (publication logos), /clients (client logos — confirm licensing before re-hosting). Checked against live 2026-10-02: same image count on every one; /the-territory, /engine-room, /recent-creations, /published, /clients have no images on live either.</t>
         </is>
       </c>
       <c r="E310" s="14" t="inlineStr">
@@ -7970,7 +7970,7 @@
       <c r="A311" s="4" t="n"/>
       <c r="B311" s="4" t="inlineStr">
         <is>
-          <t>Rescued page images wired back in (2026-09-29)</t>
+          <t>/akbar essay images</t>
         </is>
       </c>
       <c r="C311" s="13" t="inlineStr">
@@ -7980,7 +7980,7 @@
       </c>
       <c r="D311" s="4" t="inlineStr">
         <is>
-          <t>/living-declaration hero, hand image and Clarisse Abelarde artwork; /impact-dashboard earth hero; /find-my banner; /find-your-coffee dark photo landing (legacy copy restored, replacing an intro that wasn't in legacy). Also wired (second pass): /consciousness-scale (legacy's hero-first flow restored, the invented intro screen removed), /find-your-me hero, /humanos hero, the HumanOS nav logo, and all 12 HumanOS people headshots (/humanos/ecosystem, /humanos/philosophy). Blog-body images (2026-09-29): all 19 the migration dropped are restored by scripts/restore-blog-body-images.ts as Sanity drafts on 4 posts (Clarisse Abelarde 7, You Are the Moat 4, FRQNCY 6, Energy Is Money 2), waiting to be published in Studio; the other blog-listed assets were heroes already set. Still unwired from docs/ai/manus-media-rescue.md: and /alex-azzi's subject photo (a photo of a real person on an accusation page: needs Tony's yes first).</t>
+          <t>not lost after all: 20 of the 21 were rescued into Sanity by scripts/rescue-manus-media.ts (2026-09-28) and are wired back in legacy's layout (hero mosaic, JC portrait, 2x2 grid, 3 full-bleeds, 3-up strip, footer gallery) as of 2026-09-29. Only slider-3 was gone (HTTP 502); the hero mosaic is 4 tiles instead of 5.</t>
         </is>
       </c>
       <c r="E311" s="14" t="inlineStr">
@@ -7993,7 +7993,7 @@
       <c r="A312" s="4" t="n"/>
       <c r="B312" s="4" t="inlineStr">
         <is>
-          <t>BrewSoul: coffee/product images (brewsoul-coffees-expanded.ts likely has image refs</t>
+          <t>Rescued page images wired back in (2026-09-29)</t>
         </is>
       </c>
       <c r="C312" s="13" t="inlineStr">
@@ -8003,7 +8003,7 @@
       </c>
       <c r="D312" s="4" t="inlineStr">
         <is>
-          <t>audit), city guide header images, roaster directory photos. Audited 2026-09-09 (status spreadsheet), confirmed 2026-10-02: city guides already have photos; coffees, chains and roasters have no image field in legacy or here (text-only by design); farms got real photos.</t>
+          <t>/living-declaration hero, hand image and Clarisse Abelarde artwork; /impact-dashboard earth hero; /find-my banner; /find-your-coffee dark photo landing (legacy copy restored, replacing an intro that wasn't in legacy). Also wired (second pass): /consciousness-scale (legacy's hero-first flow restored, the invented intro screen removed), /find-your-me hero, /humanos hero, the HumanOS nav logo, and all 12 HumanOS people headshots (/humanos/ecosystem, /humanos/philosophy). Blog-body images (2026-09-29): all 19 the migration dropped are restored by scripts/restore-blog-body-images.ts as Sanity drafts on 4 posts (Clarisse Abelarde 7, You Are the Moat 4, FRQNCY 6, Energy Is Money 2), waiting to be published in Studio; the other blog-listed assets were heroes already set. Still unwired from docs/ai/manus-media-rescue.md: and /alex-azzi's subject photo (a photo of a real person on an accusation page: needs Tony's yes first).</t>
         </is>
       </c>
       <c r="E312" s="14" t="inlineStr">
@@ -8016,7 +8016,7 @@
       <c r="A313" s="4" t="n"/>
       <c r="B313" s="4" t="inlineStr">
         <is>
-          <t>65 page images moved off the Manus storage copy into Sanity (2026-10-02)</t>
+          <t>BrewSoul: coffee/product images (brewsoul-coffees-expanded.ts likely has image refs</t>
         </is>
       </c>
       <c r="C313" s="13" t="inlineStr">
@@ -8026,7 +8026,7 @@
       </c>
       <c r="D313" s="4" t="inlineStr">
         <is>
-          <t>every image the code loaded from d2xsxph8kpxj0f.cloudfront.net (PRI medicine images, Iboga module, facilitator index, /attention-theft, /alex-azzi, /protecting-your-business, /peyote-mescaline, HumanOS, the peptide quiz). Notes called it "RampRate's own CloudFront", but every file sits in the legacy Manus project's folder and its owner couldn't be confirmed. All 65 uploaded (scripts/rescue-cloudfront-images.ts), code rewritten, host removed from images.remotePatterns, no Sanity document used it. Table in docs/ai/manus-media-rescue.md.</t>
+          <t>audit), city guide header images, roaster directory photos. Audited 2026-09-09 (status spreadsheet), confirmed 2026-10-02: city guides already have photos; coffees, chains and roasters have no image field in legacy or here (text-only by design); farms got real photos.</t>
         </is>
       </c>
       <c r="E313" s="14" t="inlineStr">
@@ -8039,7 +8039,7 @@
       <c r="A314" s="4" t="n"/>
       <c r="B314" s="4" t="inlineStr">
         <is>
-          <t>PRI/Kava: medicine reference images (medicine-images.ts), facility images for /facilitator-index</t>
+          <t>65 page images moved off the Manus storage copy into Sanity (2026-10-02)</t>
         </is>
       </c>
       <c r="C314" s="13" t="inlineStr">
@@ -8049,7 +8049,7 @@
       </c>
       <c r="D314" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02: all in Sanity; image counts match live on PRI, Kava, Iboga, Peyote, facilitator pages.</t>
+          <t>every image the code loaded from d2xsxph8kpxj0f.cloudfront.net (PRI medicine images, Iboga module, facilitator index, /attention-theft, /alex-azzi, /protecting-your-business, /peyote-mescaline, HumanOS, the peptide quiz). Notes called it "RampRate's own CloudFront", but every file sits in the legacy Manus project's folder and its owner couldn't be confirmed. All 65 uploaded (scripts/rescue-cloudfront-images.ts), code rewritten, host removed from images.remotePatterns, no Sanity document used it. Table in docs/ai/manus-media-rescue.md.</t>
         </is>
       </c>
       <c r="E314" s="14" t="inlineStr">
@@ -8062,7 +8062,7 @@
       <c r="A315" s="4" t="n"/>
       <c r="B315" s="4" t="inlineStr">
         <is>
-          <t>Manifesto/Attention Theft: any diagram/illustration assets used on the mega-page</t>
+          <t>PRI/Kava: medicine reference images (medicine-images.ts), facility images for /facilitator-index</t>
         </is>
       </c>
       <c r="C315" s="13" t="inlineStr">
@@ -8072,7 +8072,7 @@
       </c>
       <c r="D315" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02: 6 of live's 7 are in (now in Sanity); the 7th belongs to the Wall of Shame section left out on purpose.</t>
+          <t>2026-10-02: all in Sanity; image counts match live on PRI, Kava, Iboga, Peyote, facilitator pages.</t>
         </is>
       </c>
       <c r="E315" s="14" t="inlineStr">
@@ -8085,17 +8085,17 @@
       <c r="A316" s="4" t="n"/>
       <c r="B316" s="4" t="inlineStr">
         <is>
-          <t>Assessment result-screen background art (flagged in STATUS.md as a known gap</t>
-        </is>
-      </c>
-      <c r="C316" s="15" t="inlineStr">
-        <is>
-          <t>Remaining</t>
+          <t>Manifesto/Attention Theft: any diagram/illustration assets used on the mega-page</t>
+        </is>
+      </c>
+      <c r="C316" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D316" s="4" t="inlineStr">
         <is>
-          <t>18/20 assessments currently have plain black backgrounds; sourcing themed art here also closes that gap)</t>
+          <t>2026-10-02: 6 of live's 7 are in (now in Sanity); the 7th belongs to the Wall of Shame section left out on purpose.</t>
         </is>
       </c>
       <c r="E316" s="14" t="inlineStr">
@@ -8108,17 +8108,17 @@
       <c r="A317" s="4" t="n"/>
       <c r="B317" s="4" t="inlineStr">
         <is>
-          <t>Chatbot: FauxTony avatar/icon</t>
-        </is>
-      </c>
-      <c r="C317" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Assessment result-screen background art (flagged in STATUS.md as a known gap</t>
+        </is>
+      </c>
+      <c r="C317" s="15" t="inlineStr">
+        <is>
+          <t>Remaining</t>
         </is>
       </c>
       <c r="D317" s="4" t="inlineStr">
         <is>
-          <t>Not needed (2026-10-02): the chatbot phase (Phase 10) was cancelled.</t>
+          <t>18/20 assessments currently have plain black backgrounds; sourcing themed art here also closes that gap)</t>
         </is>
       </c>
       <c r="E317" s="14" t="inlineStr">
@@ -8131,73 +8131,73 @@
       <c r="A318" s="4" t="n"/>
       <c r="B318" s="4" t="inlineStr">
         <is>
+          <t>Chatbot: FauxTony avatar/icon</t>
+        </is>
+      </c>
+      <c r="C318" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D318" s="4" t="inlineStr">
+        <is>
+          <t>Not needed (2026-10-02): the chatbot phase (Phase 10) was cancelled.</t>
+        </is>
+      </c>
+      <c r="E318" s="14" t="inlineStr">
+        <is>
+          <t>Phase 13 — Images Needed in Sanity</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" s="4" t="n"/>
+      <c r="B319" s="4" t="inlineStr">
+        <is>
           <t>Audit client/public/ (including alex-azzi/, brewsoul/ subfolders) for any static assets already sitting there unused that should be pulled i…</t>
         </is>
       </c>
-      <c r="C318" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D318" s="4" t="inlineStr">
+      <c r="C319" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D319" s="4" t="inlineStr">
         <is>
           <t>n rather than re-created. Done 2026-10-02: no images there at all (only llms.txt, a BrewSoul catalog, Manus debug files, design-options.html). Found and fixed a cutover risk instead: live serves two Google site-verification files (/google6881a0411c48b301.html, /alex-azzi/googleedff0185753a4a1f.html) that the new site returned 404 for, so Search Console could lose verification at DNS cutover. Both copied to public/ byte for byte. Not copied: site.webmanifest (its icons don't exist here; Next's app/icon.tsx covers the favicon).</t>
         </is>
       </c>
-      <c r="E318" s="14" t="inlineStr">
+      <c r="E319" s="14" t="inlineStr">
         <is>
           <t>Phase 13 — Images Needed in Sanity</t>
         </is>
       </c>
     </row>
-    <row r="319">
-      <c r="A319" s="10" t="inlineStr">
+    <row r="320">
+      <c r="A320" s="10" t="inlineStr">
         <is>
           <t>Phase 14 — QA &amp; Launch</t>
         </is>
       </c>
-      <c r="B319" s="11" t="n"/>
-      <c r="C319" s="11" t="n"/>
-      <c r="D319" s="12" t="n"/>
-    </row>
-    <row r="320">
-      <c r="A320" s="4" t="n"/>
-      <c r="B320" s="4" t="inlineStr">
-        <is>
-          <t>Mobile responsive pass on every ported section</t>
-        </is>
-      </c>
-      <c r="C320" s="15" t="inlineStr">
-        <is>
-          <t>Remaining</t>
-        </is>
-      </c>
-      <c r="D320" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-29: no page scrolls sideways at 375px any more (114 pages checked in Chrome: every unique page plus 3 of each templated set like blog posts and coffees). Fixed: BrewSoul NextSteps forced 3 columns (and used an inline style), charity-scorecard tab row, /brewsoul/browse filter dropdowns, /the-philosophy hero glow. Still to check by hand: 44px tap targets and Safari iOS. 2026-09-30: 44px tap targets on phones for the shared header, footer, BrewSoul/Kava/HumanOS menus and ~100 standalone links (undersized targets 1,904 → 578; the rest are 24-43px pills/chips that meet WCAG 2.2 AA). axe target-size (WCAG 2.2 AA, with its spacing exception): 0 failures on 114 pages. Safari/iPhone (WebKit, iPhone 14 emulation): all 114 pages load, no sideways scroll, no JS errors; form fields under 16px (iOS zoom-on-tap) fixed site-wide in globals.css. Still to check on a real iPhone: BrewSoul's bottom journey bar showed page text through it in headless WebKit only (taps hit the bar correctly; Chrome renders it solid).</t>
-        </is>
-      </c>
-      <c r="E320" s="14" t="inlineStr">
-        <is>
-          <t>Phase 14 — QA &amp; Launch</t>
-        </is>
-      </c>
+      <c r="B320" s="11" t="n"/>
+      <c r="C320" s="11" t="n"/>
+      <c r="D320" s="12" t="n"/>
     </row>
     <row r="321">
       <c r="A321" s="4" t="n"/>
       <c r="B321" s="4" t="inlineStr">
         <is>
-          <t>Accessibility pass (WCAG AA contrast, 44px touch targets, keyboard nav)</t>
-        </is>
-      </c>
-      <c r="C321" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Mobile responsive pass on every ported section</t>
+        </is>
+      </c>
+      <c r="C321" s="15" t="inlineStr">
+        <is>
+          <t>Remaining</t>
         </is>
       </c>
       <c r="D321" s="4" t="inlineStr">
         <is>
-          <t>same bar as legacy QA_MASTER_PROMPT.md. 2026-09-29 axe-core pass (WCAG 2.1 AA, same 114 pages, production build): all unlabeled dropdowns/inputs and unnamed links fixed; contrast down from 1,453 failing items on 106 pages to 1,038 on 70 (43 pages fully clean). Shared fixes: brand gold #8b6914 → #836311 site-wide (was 4.3:1 on cream, AA needs 4.5), header "⌘K"/social icons, BrewSoul nav and footer, HumanOS footer, Kava footer, assessment intro footnote, post-card image links. 2026-09-30: contrast finished, 0 axe color-contrast failures left on the same 114 pages (production build). Token changes: --kava-saffron #b86a28 → #8e521f, --pri-purple-light #a855f7 → #b87bf9 (on-dark purple only), --crusade-teal #0e7c7c → #0d7373; PriEyebrow goes light purple inside a dark PriSection via group-data-dark/pri; /find-your-me and the journey tracker's dark glass panels 60-70% → 90% (legacy's own 60% glass on beige rendered gray, cream text failed). Everything else: nearest passing shade of the same hue, or gold ↔ gold-light on the wrong background. Left: 18 links inside text marked only by color (need an underline), 44px tap targets, keyboard nav. 2026-09-30: 18 color-only in-text links underlined (axe link-in-text-block: 0 left); keyboard focus visible on every focusable item on 8 sampled pages (two form fields had none, fixed). 2026-10-02 re-run (axe WCAG 2.2 AA, 142 pages × 375/1280px, production build, plus Tab through 40 stops per page): found 1,370 contrast failures (mostly BrewSoul'</t>
+          <t>2026-09-29: no page scrolls sideways at 375px any more (114 pages checked in Chrome: every unique page plus 3 of each templated set like blog posts and coffees). Fixed: BrewSoul NextSteps forced 3 columns (and used an inline style), charity-scorecard tab row, /brewsoul/browse filter dropdowns, /the-philosophy hero glow. Still to check by hand: 44px tap targets and Safari iOS. 2026-09-30: 44px tap targets on phones for the shared header, footer, BrewSoul/Kava/HumanOS menus and ~100 standalone links (undersized targets 1,904 → 578; the rest are 24-43px pills/chips that meet WCAG 2.2 AA). axe target-size (WCAG 2.2 AA, with its spacing exception): 0 failures on 114 pages. Safari/iPhone (WebKit, iPhone 14 emulation): all 114 pages load, no sideways scroll, no JS errors; form fields under 16px (iOS zoom-on-tap) fixed site-wide in globals.css. Still to check on a real iPhone: BrewSoul's bottom journey bar showed page text through it in headless WebKit only (taps hit the bar correctly; Chrome renders it solid). Fixed 2026-10-09: the bar is now solid (bg-[#2C1810], was 92% plus backdrop-blur-md), so nothing can show through even where the blur isn't drawn; checked in WebKit (iPhone 13 profile) and Chrome: background rgb(44, 24, 16), no text behind the buttons. A real iPhone check is still part of Phase 14.</t>
         </is>
       </c>
       <c r="E321" s="14" t="inlineStr">
@@ -8210,17 +8210,17 @@
       <c r="A322" s="4" t="n"/>
       <c r="B322" s="4" t="inlineStr">
         <is>
-          <t>No dead-end pages (every page links to 2+ others)</t>
-        </is>
-      </c>
-      <c r="C322" s="15" t="inlineStr">
-        <is>
-          <t>Remaining</t>
+          <t>Accessibility pass (WCAG AA contrast, 44px touch targets, keyboard nav)</t>
+        </is>
+      </c>
+      <c r="C322" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D322" s="4" t="inlineStr">
         <is>
-          <t>same bar as legacy MASTER_QUALITY_PROMPT.md 2026-09-30 scan (496 sitemap pages, header/footer links not counted): every page has a way home (the 6 HumanOS pages had none, in legacy too; added a "← TonyGreenberg.com" footer link). ~17 quiz pages only look like dead ends on their intro screen; their result screens link to related assessments. Left for a content decision: ~20 marketing pages (/akbar, /amplifier, /diamond-cut, /ecosystem, /engage, /engine-room, /intel, /invest, /pick-up-the-phone, /protecting-your-business, /published, /speaking, /the-nightstand, /the-territory, /the-web, /under-nda, /pri-calibration, /charity-scorecard and its detail pages) link to only 0-1 other page in their content. The port matches legacy there (legacy was just as sparse), so adding related links is new content and needs the owner's yes.</t>
+          <t>same bar as legacy QA_MASTER_PROMPT.md. 2026-09-29 axe-core pass (WCAG 2.1 AA, same 114 pages, production build): all unlabeled dropdowns/inputs and unnamed links fixed; contrast down from 1,453 failing items on 106 pages to 1,038 on 70 (43 pages fully clean). Shared fixes: brand gold #8b6914 → #836311 site-wide (was 4.3:1 on cream, AA needs 4.5), header "⌘K"/social icons, BrewSoul nav and footer, HumanOS footer, Kava footer, assessment intro footnote, post-card image links. 2026-09-30: contrast finished, 0 axe color-contrast failures left on the same 114 pages (production build). Token changes: --kava-saffron #b86a28 → #8e521f, --pri-purple-light #a855f7 → #b87bf9 (on-dark purple only), --crusade-teal #0e7c7c → #0d7373; PriEyebrow goes light purple inside a dark PriSection via group-data-dark/pri; /find-your-me and the journey tracker's dark glass panels 60-70% → 90% (legacy's own 60% glass on beige rendered gray, cream text failed). Everything else: nearest passing shade of the same hue, or gold ↔ gold-light on the wrong background. Left: 18 links inside text marked only by color (need an underline), 44px tap targets, keyboard nav. 2026-09-30: 18 color-only in-text links underlined (axe link-in-text-block: 0 left); keyboard focus visible on every focusable item on 8 sampled pages (two form fields had none, fixed). 2026-10-02 re-run (axe WCAG 2.2 AA, 142 pages × 375/1280px, production build, plus Tab through 40 stops per page): found 1,370 contrast failures (mostly BrewSoul'</t>
         </is>
       </c>
       <c r="E322" s="14" t="inlineStr">
@@ -8233,7 +8233,7 @@
       <c r="A323" s="4" t="n"/>
       <c r="B323" s="4" t="inlineStr">
         <is>
-          <t>Cross-browser check (Safari iOS in particular, per legacy performance notes) 2026-10-06 WebKit pass (Playwright WebKit, iPhone 13 profile, 1…</t>
+          <t>No dead-end pages (every page links to 2+ others)</t>
         </is>
       </c>
       <c r="C323" s="15" t="inlineStr">
@@ -8243,7 +8243,7 @@
       </c>
       <c r="D323" s="4" t="inlineStr">
         <is>
-          <t>52 pages: every unique page plus 3 of each templated set, production build): no page pans sideways, no failed requests, no JS errors. Found and fixed on the way: upgrade-insecure-requests in the new CSP made Safari fetch every stylesheet and font over https on localhost (dropped; the site is HTTPS-only via HSTS anyway), and .toLocaleString() without a locale caused a hydration error on /brewsoul/chains in Safari (all number formatting now en-US). Left: a check on a real iPhone (Phase 14).</t>
+          <t>same bar as legacy MASTER_QUALITY_PROMPT.md 2026-09-30 scan (496 sitemap pages, header/footer links not counted): every page has a way home (the 6 HumanOS pages had none, in legacy too; added a "← TonyGreenberg.com" footer link). ~17 quiz pages only look like dead ends on their intro screen; their result screens link to related assessments. Left for a content decision: ~20 marketing pages (/akbar, /amplifier, /diamond-cut, /ecosystem, /engage, /engine-room, /intel, /invest, /pick-up-the-phone, /protecting-your-business, /published, /speaking, /the-nightstand, /the-territory, /the-web, /under-nda, /pri-calibration, /charity-scorecard and its detail pages) link to only 0-1 other page in their content. The port matches legacy there (legacy was just as sparse), so adding related links is new content and needs the owner's yes.</t>
         </is>
       </c>
       <c r="E323" s="14" t="inlineStr">
@@ -8256,7 +8256,7 @@
       <c r="A324" s="4" t="n"/>
       <c r="B324" s="4" t="inlineStr">
         <is>
-          <t>Remove noindex only when sign-off is given</t>
+          <t>Cross-browser check (Safari iOS in particular, per legacy performance notes) 2026-10-06 WebKit pass (Playwright WebKit, iPhone 13 profile, 1…</t>
         </is>
       </c>
       <c r="C324" s="15" t="inlineStr">
@@ -8266,7 +8266,7 @@
       </c>
       <c r="D324" s="4" t="inlineStr">
         <is>
-          <t>do not launch indexable by accident (The only noindex is the host-based one for *.netlify.app above, so the real domain is indexable as soon as DNS points at it: sign-off must come before DNS.)</t>
+          <t>52 pages: every unique page plus 3 of each templated set, production build): no page pans sideways, no failed requests, no JS errors. Found and fixed on the way: upgrade-insecure-requests in the new CSP made Safari fetch every stylesheet and font over https on localhost (dropped; the site is HTTPS-only via HSTS anyway), and .toLocaleString() without a locale caused a hydration error on /brewsoul/chains in Safari (all number formatting now en-US). Left: a check on a real iPhone (Phase 14).</t>
         </is>
       </c>
       <c r="E324" s="14" t="inlineStr">
@@ -8279,7 +8279,7 @@
       <c r="A325" s="4" t="n"/>
       <c r="B325" s="4" t="inlineStr">
         <is>
-          <t>Final stakeholder sign-off (Tony/Darryl/Kimberly) on the ported site before DNS cutover</t>
+          <t>Remove noindex only when sign-off is given</t>
         </is>
       </c>
       <c r="C325" s="15" t="inlineStr">
@@ -8287,7 +8287,11 @@
           <t>Remaining</t>
         </is>
       </c>
-      <c r="D325" s="4" t="inlineStr"/>
+      <c r="D325" s="4" t="inlineStr">
+        <is>
+          <t>do not launch indexable by accident (The only noindex is the host-based one for *.netlify.app above, so the real domain is indexable as soon as DNS points at it: sign-off must come before DNS.)</t>
+        </is>
+      </c>
       <c r="E325" s="14" t="inlineStr">
         <is>
           <t>Phase 14 — QA &amp; Launch</t>
@@ -8298,7 +8302,7 @@
       <c r="A326" s="4" t="n"/>
       <c r="B326" s="4" t="inlineStr">
         <is>
-          <t>DNS cutover, legacy app decommissioned only after a stable overlap window</t>
+          <t>Final stakeholder sign-off (Tony/Darryl/Kimberly) on the ported site before DNS cutover</t>
         </is>
       </c>
       <c r="C326" s="15" t="inlineStr">
@@ -8313,21 +8317,40 @@
         </is>
       </c>
     </row>
+    <row r="327">
+      <c r="A327" s="4" t="n"/>
+      <c r="B327" s="4" t="inlineStr">
+        <is>
+          <t>DNS cutover, legacy app decommissioned only after a stable overlap window</t>
+        </is>
+      </c>
+      <c r="C327" s="15" t="inlineStr">
+        <is>
+          <t>Remaining</t>
+        </is>
+      </c>
+      <c r="D327" s="4" t="inlineStr"/>
+      <c r="E327" s="14" t="inlineStr">
+        <is>
+          <t>Phase 14 — QA &amp; Launch</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D326"/>
+  <autoFilter ref="A1:D327"/>
   <mergeCells count="14">
     <mergeCell ref="A150:D150"/>
+    <mergeCell ref="A320:D320"/>
     <mergeCell ref="A237:D237"/>
     <mergeCell ref="A58:D58"/>
     <mergeCell ref="A258:D258"/>
-    <mergeCell ref="A319:D319"/>
     <mergeCell ref="A209:D209"/>
     <mergeCell ref="A205:D205"/>
     <mergeCell ref="A15:D15"/>
     <mergeCell ref="A43:D43"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A299:D299"/>
     <mergeCell ref="A183:D183"/>
+    <mergeCell ref="A300:D300"/>
     <mergeCell ref="A32:D32"/>
     <mergeCell ref="A123:D123"/>
   </mergeCells>
@@ -8789,7 +8812,7 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>2026-09-29: no page scrolls sideways at 375px any more (114 pages checked in Chrome: every unique page plus 3 of each templated set like blog posts and coffees). Fixed: BrewSoul NextSteps forced 3 columns (and used an inline style), charity-scorecard tab row, /brewsoul/browse filter dropdowns, /the-philosophy hero glow. Still to check by hand: 44px tap targets and Safari iOS. 2026-09-30: 44px tap targets on phones for the shared header, footer, BrewSoul/Kava/HumanOS menus and ~100 standalone links (undersized targets 1,904 → 578; the rest are 24-43px pills/chips that meet WCAG 2.2 AA). axe target-size (WCAG 2.2 AA, with its spacing exception): 0 failures on 114 pages. Safari/iPhone (WebKit, iPhone 14 emulation): all 114 pages load, no sideways scroll, no JS errors; form fields under 16px (iOS zoom-on-tap) fixed site-wide in globals.css. Still to check on a real iPhone: BrewSoul's bottom journey bar showed page text through it in headless WebKit only (taps hit the bar correctly; Chrome renders it solid).</t>
+          <t>2026-09-29: no page scrolls sideways at 375px any more (114 pages checked in Chrome: every unique page plus 3 of each templated set like blog posts and coffees). Fixed: BrewSoul NextSteps forced 3 columns (and used an inline style), charity-scorecard tab row, /brewsoul/browse filter dropdowns, /the-philosophy hero glow. Still to check by hand: 44px tap targets and Safari iOS. 2026-09-30: 44px tap targets on phones for the shared header, footer, BrewSoul/Kava/HumanOS menus and ~100 standalone links (undersized targets 1,904 → 578; the rest are 24-43px pills/chips that meet WCAG 2.2 AA). axe target-size (WCAG 2.2 AA, with its spacing exception): 0 failures on 114 pages. Safari/iPhone (WebKit, iPhone 14 emulation): all 114 pages load, no sideways scroll, no JS errors; form fields under 16px (iOS zoom-on-tap) fixed site-wide in globals.css. Still to check on a real iPhone: BrewSoul's bottom journey bar showed page text through it in headless WebKit only (taps hit the bar correctly; Chrome renders it solid). Fixed 2026-10-09: the bar is now solid (bg-[#2C1810], was 92% plus backdrop-blur-md), so nothing can show through even where the blur isn't drawn; checked in WebKit (iPhone 13 profile) and Chrome: background rgb(44, 24, 16), no text behind the buttons. A real iPhone check is still part of Phase 14.</t>
         </is>
       </c>
       <c r="E23" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Arrows in buttons and links are icons; record owner's design answers
Owner said yes (2026-10-09) to switching typed arrows in buttons/links to
icons. 113 arrows in 52 files -> lucide ArrowRight/ArrowLeft (size-[1em],
wrapped in inline-flex items-center gap-1.5 so parent layout is
untouched): JSX labels (codemod), Next/See My Results toggles, decorative
arrow spans, walk-through deeperLabel data, the Letter's "I'm in" button
(NewsletterSignupForm buttonLabel is now ReactNode). Content arrows (Tony's
text, data, process flows, share text, <option> labels, "<- you" marker)
left as they are.

Checked: type check, lint, build; 16 pages at 375/1280 have no typed arrow
in any link/button, no sideways scroll, no JS errors; icon close-ups.

Also records the owner's answers: title font "match live" (done in the
previous commit), keep the menu on /find-my, keep the "117" box.
CONTRIBUTING rule 18 notes the switch.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Migration-Status-Report.xlsx
+++ b/Migration-Status-Report.xlsx
@@ -12,8 +12,8 @@
     <sheet name="Remaining Work" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Full Detail'!$A$1:$D$327</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Remaining Work'!$A$1:$D$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Full Detail'!$A$1:$D$328</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Remaining Work'!$A$1:$D$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -639,15 +639,15 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A5,'Full Detail'!$C$2:$C$327,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A5,'Full Detail'!$C$2:$C$328,"Done")</f>
         <v/>
       </c>
       <c r="C5" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A5,'Full Detail'!$C$2:$C$327,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A5,'Full Detail'!$C$2:$C$328,"Remaining")</f>
         <v/>
       </c>
       <c r="D5" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A5,'Full Detail'!$C$2:$C$327,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A5,'Full Detail'!$C$2:$C$328,"Deferred")</f>
         <v/>
       </c>
       <c r="E5" s="5">
@@ -666,15 +666,15 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A6,'Full Detail'!$C$2:$C$327,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A6,'Full Detail'!$C$2:$C$328,"Done")</f>
         <v/>
       </c>
       <c r="C6" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A6,'Full Detail'!$C$2:$C$327,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A6,'Full Detail'!$C$2:$C$328,"Remaining")</f>
         <v/>
       </c>
       <c r="D6" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A6,'Full Detail'!$C$2:$C$327,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A6,'Full Detail'!$C$2:$C$328,"Deferred")</f>
         <v/>
       </c>
       <c r="E6" s="5">
@@ -693,15 +693,15 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A7,'Full Detail'!$C$2:$C$327,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A7,'Full Detail'!$C$2:$C$328,"Done")</f>
         <v/>
       </c>
       <c r="C7" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A7,'Full Detail'!$C$2:$C$327,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A7,'Full Detail'!$C$2:$C$328,"Remaining")</f>
         <v/>
       </c>
       <c r="D7" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A7,'Full Detail'!$C$2:$C$327,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A7,'Full Detail'!$C$2:$C$328,"Deferred")</f>
         <v/>
       </c>
       <c r="E7" s="5">
@@ -720,15 +720,15 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A8,'Full Detail'!$C$2:$C$327,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A8,'Full Detail'!$C$2:$C$328,"Done")</f>
         <v/>
       </c>
       <c r="C8" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A8,'Full Detail'!$C$2:$C$327,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A8,'Full Detail'!$C$2:$C$328,"Remaining")</f>
         <v/>
       </c>
       <c r="D8" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A8,'Full Detail'!$C$2:$C$327,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A8,'Full Detail'!$C$2:$C$328,"Deferred")</f>
         <v/>
       </c>
       <c r="E8" s="5">
@@ -747,15 +747,15 @@
         </is>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A9,'Full Detail'!$C$2:$C$327,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A9,'Full Detail'!$C$2:$C$328,"Done")</f>
         <v/>
       </c>
       <c r="C9" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A9,'Full Detail'!$C$2:$C$327,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A9,'Full Detail'!$C$2:$C$328,"Remaining")</f>
         <v/>
       </c>
       <c r="D9" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A9,'Full Detail'!$C$2:$C$327,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A9,'Full Detail'!$C$2:$C$328,"Deferred")</f>
         <v/>
       </c>
       <c r="E9" s="5">
@@ -774,15 +774,15 @@
         </is>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A10,'Full Detail'!$C$2:$C$327,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A10,'Full Detail'!$C$2:$C$328,"Done")</f>
         <v/>
       </c>
       <c r="C10" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A10,'Full Detail'!$C$2:$C$327,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A10,'Full Detail'!$C$2:$C$328,"Remaining")</f>
         <v/>
       </c>
       <c r="D10" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A10,'Full Detail'!$C$2:$C$327,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A10,'Full Detail'!$C$2:$C$328,"Deferred")</f>
         <v/>
       </c>
       <c r="E10" s="5">
@@ -801,15 +801,15 @@
         </is>
       </c>
       <c r="B11" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A11,'Full Detail'!$C$2:$C$327,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A11,'Full Detail'!$C$2:$C$328,"Done")</f>
         <v/>
       </c>
       <c r="C11" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A11,'Full Detail'!$C$2:$C$327,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A11,'Full Detail'!$C$2:$C$328,"Remaining")</f>
         <v/>
       </c>
       <c r="D11" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A11,'Full Detail'!$C$2:$C$327,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A11,'Full Detail'!$C$2:$C$328,"Deferred")</f>
         <v/>
       </c>
       <c r="E11" s="5">
@@ -828,15 +828,15 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A12,'Full Detail'!$C$2:$C$327,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A12,'Full Detail'!$C$2:$C$328,"Done")</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A12,'Full Detail'!$C$2:$C$327,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A12,'Full Detail'!$C$2:$C$328,"Remaining")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A12,'Full Detail'!$C$2:$C$327,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A12,'Full Detail'!$C$2:$C$328,"Deferred")</f>
         <v/>
       </c>
       <c r="E12" s="5">
@@ -855,15 +855,15 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A13,'Full Detail'!$C$2:$C$327,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A13,'Full Detail'!$C$2:$C$328,"Done")</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A13,'Full Detail'!$C$2:$C$327,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A13,'Full Detail'!$C$2:$C$328,"Remaining")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A13,'Full Detail'!$C$2:$C$327,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A13,'Full Detail'!$C$2:$C$328,"Deferred")</f>
         <v/>
       </c>
       <c r="E13" s="5">
@@ -882,15 +882,15 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A14,'Full Detail'!$C$2:$C$327,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A14,'Full Detail'!$C$2:$C$328,"Done")</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A14,'Full Detail'!$C$2:$C$327,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A14,'Full Detail'!$C$2:$C$328,"Remaining")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A14,'Full Detail'!$C$2:$C$327,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A14,'Full Detail'!$C$2:$C$328,"Deferred")</f>
         <v/>
       </c>
       <c r="E14" s="5">
@@ -909,15 +909,15 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A15,'Full Detail'!$C$2:$C$327,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A15,'Full Detail'!$C$2:$C$328,"Done")</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A15,'Full Detail'!$C$2:$C$327,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A15,'Full Detail'!$C$2:$C$328,"Remaining")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A15,'Full Detail'!$C$2:$C$327,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A15,'Full Detail'!$C$2:$C$328,"Deferred")</f>
         <v/>
       </c>
       <c r="E15" s="5">
@@ -936,15 +936,15 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A16,'Full Detail'!$C$2:$C$327,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A16,'Full Detail'!$C$2:$C$328,"Done")</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A16,'Full Detail'!$C$2:$C$327,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A16,'Full Detail'!$C$2:$C$328,"Remaining")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A16,'Full Detail'!$C$2:$C$327,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A16,'Full Detail'!$C$2:$C$328,"Deferred")</f>
         <v/>
       </c>
       <c r="E16" s="5">
@@ -963,15 +963,15 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A17,'Full Detail'!$C$2:$C$327,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A17,'Full Detail'!$C$2:$C$328,"Done")</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A17,'Full Detail'!$C$2:$C$327,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A17,'Full Detail'!$C$2:$C$328,"Remaining")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A17,'Full Detail'!$C$2:$C$327,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A17,'Full Detail'!$C$2:$C$328,"Deferred")</f>
         <v/>
       </c>
       <c r="E17" s="5">
@@ -990,15 +990,15 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A18,'Full Detail'!$C$2:$C$327,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A18,'Full Detail'!$C$2:$C$328,"Done")</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A18,'Full Detail'!$C$2:$C$327,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A18,'Full Detail'!$C$2:$C$328,"Remaining")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A18,'Full Detail'!$C$2:$C$327,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A18,'Full Detail'!$C$2:$C$328,"Deferred")</f>
         <v/>
       </c>
       <c r="E18" s="5">
@@ -1017,15 +1017,15 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A19,'Full Detail'!$C$2:$C$327,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A19,'Full Detail'!$C$2:$C$328,"Done")</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A19,'Full Detail'!$C$2:$C$327,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A19,'Full Detail'!$C$2:$C$328,"Remaining")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$327,$A19,'Full Detail'!$C$2:$C$327,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A19,'Full Detail'!$C$2:$C$328,"Deferred")</f>
         <v/>
       </c>
       <c r="E19" s="5">
@@ -1075,7 +1075,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E327"/>
+  <dimension ref="A1:E328"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -7251,17 +7251,17 @@
       <c r="A279" s="4" t="n"/>
       <c r="B279" s="4" t="inlineStr">
         <is>
-          <t>Still different from live (needs a yes)</t>
-        </is>
-      </c>
-      <c r="C279" s="15" t="inlineStr">
-        <is>
-          <t>Remaining</t>
+          <t>Still different from live (decided 2026-10-09)</t>
+        </is>
+      </c>
+      <c r="C279" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D279" s="4" t="inlineStr">
         <is>
-          <t>blog posts (done) (done 2026-10-07, see Phase 5); /find-my on live hides the site header. /walk-through is a 404 on live now.</t>
+          <t>blog posts (done) (done 2026-10-07, see Phase 5); /find-my on live hides the site header. /walk-through is a 404 on live now. Owner: keep our site menu on /find-my (visitors can still reach the rest of the site); nothing left to change.</t>
         </is>
       </c>
       <c r="E279" s="14" t="inlineStr">
@@ -7274,17 +7274,17 @@
       <c r="A280" s="4" t="n"/>
       <c r="B280" s="4" t="inlineStr">
         <is>
-          <t>Design change on live, needs a decision</t>
-        </is>
-      </c>
-      <c r="C280" s="15" t="inlineStr">
-        <is>
-          <t>Remaining</t>
+          <t>Design change on live (owner: "match live", 2026-10-09)</t>
+        </is>
+      </c>
+      <c r="C280" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D280" s="4" t="inlineStr">
         <is>
-          <t>live's story pages now use Cormorant Garamond for titles (ours: Playfair Display), a lighter title weight (400 vs our 700), and a red eyebrow label (#8E1E25, wider letter spacing) instead of our gold. A site-wide font swap is a design call, so not done.</t>
+          <t>live's story pages now use Cormorant Garamond for titles (ours: Playfair Display), a lighter title weight (400 vs our 700), and a red eyebrow label (#8E1E25, wider letter spacing) instead of our gold. A site-wide font swap is a design call, so not done. Done 2026-10-09: a fresh sweep of 163 live pages found live has since dropped Cormorant from the story pages (only /living-declaration uses it, ours already matched) and mostly uses Playfair; the real differences were fixed: every heading on /attention-theft in Fraunces 700 (section-wide, like Kava), /supplier-intake title in the system serif, and live's fluid title sizes on /about, /articles, /the-letter, /the-philosophy, /clock-keeper-part-2, /living-declaration (measured at 375/640/820/1024/1280, now identical). Label colours stay darker than live on purpose (contrast, rule 20).</t>
         </is>
       </c>
       <c r="E280" s="14" t="inlineStr">
@@ -7366,7 +7366,7 @@
       <c r="A284" s="4" t="n"/>
       <c r="B284" s="4" t="inlineStr">
         <is>
-          <t>Category pages pre-built (2026-10-09)</t>
+          <t>Arrows in buttons and links are icons (2026-10-09, owner said yes)</t>
         </is>
       </c>
       <c r="C284" s="13" t="inlineStr">
@@ -7376,7 +7376,7 @@
       </c>
       <c r="D284" s="4" t="inlineStr">
         <is>
-          <t>/blog/category/[slug] read ?page=N, so every category page was rendered on each request (slower first byte, flagged in the Lighthouse notes). Page numbers are now part of the address (/blog/category/&lt;slug&gt;/page/&lt;n&gt;, generateStaticParams, dynamicParams = false), shared code in src/components/blog/category-listing.tsx; old ?page=N links 308 to the new address (pages 2+ only, so no loop), /page/1 308s to the plain address, a page past the end is a 404; "All essays" back link uses an icon. Verified on a production build: route table shows every category page as pre-built (9 page-1s, 7 later pages), titles and canonicals per page, Previous/Next links, the redirects and the 404s.</t>
+          <t>113 typed arrows in 52 files (button and link labels, "Next"/"See My Results" toggles, decorative arrow spans, the walk-through "See the..." labels, the Letter's "I'm in" button) replaced with lucide ArrowRight/ArrowLeft (size-[1em], inside inline-flex items-center gap-1.5, so the parent layout is untouched). Left as content on purpose: arrows inside Tony's text and data (health findings, origins, iboga compass options, process flows like "Inherit → Wake → Choose → Act", share text), the "← you" marker on the consciousness scale, and &lt;option&gt; sort labels (an option can't hold an icon). Checked on 16 pages at 375 and 1280: no typed arrow left in any link or button, no sideways scroll, no JS errors; close-up screenshots of the new icons.</t>
         </is>
       </c>
       <c r="E284" s="14" t="inlineStr">
@@ -7389,7 +7389,7 @@
       <c r="A285" s="4" t="n"/>
       <c r="B285" s="4" t="inlineStr">
         <is>
-          <t>Error pages (2026-10-09, owner asked)</t>
+          <t>Category pages pre-built (2026-10-09)</t>
         </is>
       </c>
       <c r="C285" s="13" t="inlineStr">
@@ -7399,7 +7399,7 @@
       </c>
       <c r="D285" s="4" t="inlineStr">
         <is>
-          <t>404 page now sets its own title ("Page not found") as a server page around live's 3-second redirect (not-found.tsx + components/not-found-redirect.tsx), arrow as an icon; page error screen (error.tsx) uses Next 16's retry (re-fetches), shows a reference code for the server logs, links home and to the site index; new global-error.tsx for failures in the root layout itself (own &lt;html&gt;, plain links). Verified on a production build: missing page, missing essay and missing Kava page return 404 with the right title; a test page that throws returns 500 with the error screen, "Try again" re-fetches; phone and laptop, no sideways scroll (test page removed).</t>
+          <t>/blog/category/[slug] read ?page=N, so every category page was rendered on each request (slower first byte, flagged in the Lighthouse notes). Page numbers are now part of the address (/blog/category/&lt;slug&gt;/page/&lt;n&gt;, generateStaticParams, dynamicParams = false), shared code in src/components/blog/category-listing.tsx; old ?page=N links 308 to the new address (pages 2+ only, so no loop), /page/1 308s to the plain address, a page past the end is a 404; "All essays" back link uses an icon. Verified on a production build: route table shows every category page as pre-built (9 page-1s, 7 later pages), titles and canonicals per page, Previous/Next links, the redirects and the 404s.</t>
         </is>
       </c>
       <c r="E285" s="14" t="inlineStr">
@@ -7412,7 +7412,7 @@
       <c r="A286" s="4" t="n"/>
       <c r="B286" s="4" t="inlineStr">
         <is>
-          <t>SEO audit fixes (2026-10-06)</t>
+          <t>Error pages (2026-10-09, owner asked)</t>
         </is>
       </c>
       <c r="C286" s="13" t="inlineStr">
@@ -7422,7 +7422,7 @@
       </c>
       <c r="D286" s="4" t="inlineStr">
         <is>
-          <t>Checked an outside audit point by point against the code. Fixed: Core Themes cards linked to /?theme=…#essays-archive (not crawlable, counts from a stale hand-kept list) and now link to /blog/category/&lt;slug&gt; with real counts (21/25/20/14, matching the archive pills; THEME_MAP and the ?theme= filter removed); Four Doors cards were &lt;button&gt;s, now real links that still open the modal on a plain click; "DIAGNOSE · ENGAGE" now link to /find-my and /engage; one shared formatPostDate (Asia/Kolkata, src/lib/format-post-date.ts) so a post no longer shows two different dates; the title repeated as the first body paragraph is dropped at render time (legacyBodyLayout); essay cards are h3 under a section h2 (archive, Read next), h2 only on category/search; heading glyphs (◆ ✦) hidden from screen readers; posts send BlogPosting with the author tied to the site Person (@id) plus a BreadcrumbList; descriptive alt on the homepage and BrewSoul heroes; homepage OG image cropped to 1200x630 JPEG. Already fine (audit could not see it): Person/Article schema, Netlify noindex, robots.txt, sitemap, header nav and search, Amazon links carry no affiliate tag. Checked on a production build: type check, lint, build, status codes, browser click test at 375px, no console errors. Implementation pack (Mohammad Danish, 2026-10-05) checked the same day: added og:type/og:site_name back on the 6 pages with their own openGraph (a page-level openGraph replaces the layout one), twitter:creator, and on posts og:url</t>
+          <t>404 page now sets its own title ("Page not found") as a server page around live's 3-second redirect (not-found.tsx + components/not-found-redirect.tsx), arrow as an icon; page error screen (error.tsx) uses Next 16's retry (re-fetches), shows a reference code for the server logs, links home and to the site index; new global-error.tsx for failures in the root layout itself (own &lt;html&gt;, plain links). Verified on a production build: missing page, missing essay and missing Kava page return 404 with the right title; a test page that throws returns 500 with the error screen, "Try again" re-fetches; phone and laptop, no sideways scroll (test page removed).</t>
         </is>
       </c>
       <c r="E286" s="14" t="inlineStr">
@@ -7435,17 +7435,17 @@
       <c r="A287" s="4" t="n"/>
       <c r="B287" s="4" t="inlineStr">
         <is>
-          <t>SEO audit items needing a yes (2026-10-06)</t>
-        </is>
-      </c>
-      <c r="C287" s="15" t="inlineStr">
-        <is>
-          <t>Remaining</t>
+          <t>SEO audit fixes (2026-10-06)</t>
+        </is>
+      </c>
+      <c r="C287" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D287" s="4" t="inlineStr">
         <is>
-          <t>the pack's new copy (homepage title/description, five-cups title, description, short answer, FAQ, heading rewrites, entity statement, newsletter block, author box, health disclaimer, COA wording); "Further Reading" shown twice on posts (merge the lists?); long post title (84 chars), homepage description length and obsolete keywords tag, slugs (/blog/five-cups, the -2 slug; would need redirects), "Six lenses" over four cards, sources for health claims and proof for "$10B+", "Certified B Corp", "Validity: 91", legal review of the homepage Case File banner, ABIT waitlist disclosures, one contact email, the two one-post categories, fewer homepage CTAs / email signup / table of contents / explaining "COA".</t>
+          <t>Checked an outside audit point by point against the code. Fixed: Core Themes cards linked to /?theme=…#essays-archive (not crawlable, counts from a stale hand-kept list) and now link to /blog/category/&lt;slug&gt; with real counts (21/25/20/14, matching the archive pills; THEME_MAP and the ?theme= filter removed); Four Doors cards were &lt;button&gt;s, now real links that still open the modal on a plain click; "DIAGNOSE · ENGAGE" now link to /find-my and /engage; one shared formatPostDate (Asia/Kolkata, src/lib/format-post-date.ts) so a post no longer shows two different dates; the title repeated as the first body paragraph is dropped at render time (legacyBodyLayout); essay cards are h3 under a section h2 (archive, Read next), h2 only on category/search; heading glyphs (◆ ✦) hidden from screen readers; posts send BlogPosting with the author tied to the site Person (@id) plus a BreadcrumbList; descriptive alt on the homepage and BrewSoul heroes; homepage OG image cropped to 1200x630 JPEG. Already fine (audit could not see it): Person/Article schema, Netlify noindex, robots.txt, sitemap, header nav and search, Amazon links carry no affiliate tag. Checked on a production build: type check, lint, build, status codes, browser click test at 375px, no console errors. Implementation pack (Mohammad Danish, 2026-10-05) checked the same day: added og:type/og:site_name back on the 6 pages with their own openGraph (a page-level openGraph replaces the layout one), twitter:creator, and on posts og:url</t>
         </is>
       </c>
       <c r="E287" s="14" t="inlineStr">
@@ -7458,7 +7458,7 @@
       <c r="A288" s="4" t="n"/>
       <c r="B288" s="4" t="inlineStr">
         <is>
-          <t>Connect Google Search Console + GA4 to the new deployment on day one of cutover</t>
+          <t>SEO audit items needing a yes (2026-10-06)</t>
         </is>
       </c>
       <c r="C288" s="15" t="inlineStr">
@@ -7466,7 +7466,11 @@
           <t>Remaining</t>
         </is>
       </c>
-      <c r="D288" s="4" t="inlineStr"/>
+      <c r="D288" s="4" t="inlineStr">
+        <is>
+          <t>the pack's new copy (homepage title/description, five-cups title, description, short answer, FAQ, heading rewrites, entity statement, newsletter block, author box, health disclaimer, COA wording); "Further Reading" shown twice on posts (merge the lists?); long post title (84 chars), homepage description length and obsolete keywords tag, slugs (/blog/five-cups, the -2 slug; would need redirects), "Six lenses" over four cards, sources for health claims and proof for "$10B+", "Certified B Corp", "Validity: 91", legal review of the homepage Case File banner, ABIT waitlist disclosures, one contact email, the two one-post categories, fewer homepage CTAs / email signup / table of contents / explaining "COA".</t>
+        </is>
+      </c>
       <c r="E288" s="14" t="inlineStr">
         <is>
           <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
@@ -7477,19 +7481,15 @@
       <c r="A289" s="4" t="n"/>
       <c r="B289" s="4" t="inlineStr">
         <is>
-          <t>Restore/adapt the manus.space triple-layer noindex lockdown pattern for any remaining staging URLs</t>
-        </is>
-      </c>
-      <c r="C289" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D289" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-01: the Netlify copy (tonygreenberg-website.netlify.app) and every deploy preview had no noindex at all, so Google could index a duplicate of the site. next.config.ts headers() now sends X-Robots-Tag: noindex, nofollow on any *.netlify.app host only; tonygreenberg.com is unaffected, so nothing to remove at cutover. Tested with Host headers on a production build.</t>
-        </is>
-      </c>
+          <t>Connect Google Search Console + GA4 to the new deployment on day one of cutover</t>
+        </is>
+      </c>
+      <c r="C289" s="15" t="inlineStr">
+        <is>
+          <t>Remaining</t>
+        </is>
+      </c>
+      <c r="D289" s="4" t="inlineStr"/>
       <c r="E289" s="14" t="inlineStr">
         <is>
           <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
@@ -7500,7 +7500,7 @@
       <c r="A290" s="4" t="n"/>
       <c r="B290" s="4" t="inlineStr">
         <is>
-          <t>"Keep going" strip above the footer on every page (2026-10-07)</t>
+          <t>Restore/adapt the manus.space triple-layer noindex lockdown pattern for any remaining staging URLs</t>
         </is>
       </c>
       <c r="C290" s="13" t="inlineStr">
@@ -7510,7 +7510,7 @@
       </c>
       <c r="D290" s="4" t="inlineStr">
         <is>
-          <t>legacy's WhereNext (deferred in Phase 3, never picked up) with its per-page suggestions, Home · Site Index · All Assessments; links pointed at current routes.</t>
+          <t>2026-10-01: the Netlify copy (tonygreenberg-website.netlify.app) and every deploy preview had no noindex at all, so Google could index a duplicate of the site. next.config.ts headers() now sends X-Robots-Tag: noindex, nofollow on any *.netlify.app host only; tonygreenberg.com is unaffected, so nothing to remove at cutover. Tested with Host headers on a production build.</t>
         </is>
       </c>
       <c r="E290" s="14" t="inlineStr">
@@ -7523,7 +7523,7 @@
       <c r="A291" s="4" t="n"/>
       <c r="B291" s="4" t="inlineStr">
         <is>
-          <t>Live-only and redesigned pages from the 2026-10-07 page sweep (188 pages compared with live)</t>
+          <t>"Keep going" strip above the footer on every page (2026-10-07)</t>
         </is>
       </c>
       <c r="C291" s="13" t="inlineStr">
@@ -7533,7 +7533,7 @@
       </c>
       <c r="D291" s="4" t="inlineStr">
         <is>
-          <t>/the-index rebuilt from live's code (20 concepts, related-word search across essays and site pages, full-text search on the server, "three related places to go next"; the old redirect to /search removed and its links, including the "Site Index" link in "Keep going", point at it again); /the-mirror (and /life-assessment) opens on live's intro (dark hero, "What We Measure" with the six areas, "The Ecosystem"), rebuilt as a step registry (rule 19); /essays header, order and column like live; /about "What They Say" styled like live (live picks 3 of the same 19 quotes at random; ours shows a fixed 3 so they're in the server HTML); /impact-futurism list titles and subtitles; /supplier-intake is a real page again with live's Stage 1 form; /seven-doors and /projects redirect home like live; /impact, /health, /library, /built-on-manus, /heroes are 404 on live too. Left as is on purpose: /blog stays our archive page (on live it repeats the homepage), the email gates on /framework and /peptide-supply-chain, the attention-theft Wall of Shame.</t>
+          <t>legacy's WhereNext (deferred in Phase 3, never picked up) with its per-page suggestions, Home · Site Index · All Assessments; links pointed at current routes.</t>
         </is>
       </c>
       <c r="E291" s="14" t="inlineStr">
@@ -7546,7 +7546,7 @@
       <c r="A292" s="4" t="n"/>
       <c r="B292" s="4" t="inlineStr">
         <is>
-          <t>/alex-azzi locked like live (2026-10-07, owner said match it)</t>
+          <t>Live-only and redesigned pages from the 2026-10-07 page sweep (188 pages compared with live)</t>
         </is>
       </c>
       <c r="C292" s="13" t="inlineStr">
@@ -7556,7 +7556,7 @@
       </c>
       <c r="D292" s="4" t="inlineStr">
         <is>
-          <t>same server-checked password as the locked essay (GATED_POST_PASSWORD, now also set in Netlify), live's "Restricted Access" screen, the report not in the page until unlocked, out of search and the sitemap.</t>
+          <t>/the-index rebuilt from live's code (20 concepts, related-word search across essays and site pages, full-text search on the server, "three related places to go next"; the old redirect to /search removed and its links, including the "Site Index" link in "Keep going", point at it again); /the-mirror (and /life-assessment) opens on live's intro (dark hero, "What We Measure" with the six areas, "The Ecosystem"), rebuilt as a step registry (rule 19); /essays header, order and column like live; /about "What They Say" styled like live (live picks 3 of the same 19 quotes at random; ours shows a fixed 3 so they're in the server HTML); /impact-futurism list titles and subtitles; /supplier-intake is a real page again with live's Stage 1 form; /seven-doors and /projects redirect home like live; /impact, /health, /library, /built-on-manus, /heroes are 404 on live too. Left as is on purpose: /blog stays our archive page (on live it repeats the homepage), the email gates on /framework and /peptide-supply-chain, the attention-theft Wall of Shame.</t>
         </is>
       </c>
       <c r="E292" s="14" t="inlineStr">
@@ -7569,7 +7569,7 @@
       <c r="A293" s="4" t="n"/>
       <c r="B293" s="4" t="inlineStr">
         <is>
-          <t>Live's title fonts and sizes (2026-10-07, "fix the style")</t>
+          <t>/alex-azzi locked like live (2026-10-07, owner said match it)</t>
         </is>
       </c>
       <c r="C293" s="13" t="inlineStr">
@@ -7579,7 +7579,7 @@
       </c>
       <c r="D293" s="4" t="inlineStr">
         <is>
-          <t>measured every page's title font, weight, size and label colour on live vs ours (136 pages). Now like live: Kava headings in Fraunces, HumanOS in Space Grotesk, the peptide tools / charity scorecard / thesis threads in the system serif, America Unbundled in the Iowan Old Style stack at live's size, /akbar in Fraunces 900, friend-gate and post-intervention in Georgia, and live's title sizes on peptide-matrix, peptide-supply-chain, rip-peptide-sciences and the HumanOS pages. Fonts load only on the pages that use them (src/lib/fonts/page-fonts.ts). Label colours stay the darker AA-contrast versions where live's lighter ones fail on a light background.</t>
+          <t>same server-checked password as the locked essay (GATED_POST_PASSWORD, now also set in Netlify), live's "Restricted Access" screen, the report not in the page until unlocked, out of search and the sitemap.</t>
         </is>
       </c>
       <c r="E293" s="14" t="inlineStr">
@@ -7592,7 +7592,7 @@
       <c r="A294" s="4" t="n"/>
       <c r="B294" s="4" t="inlineStr">
         <is>
-          <t>Peptide page images rescued into Sanity and wired (2026-10-07)</t>
+          <t>Live's title fonts and sizes (2026-10-07, "fix the style")</t>
         </is>
       </c>
       <c r="C294" s="13" t="inlineStr">
@@ -7602,7 +7602,7 @@
       </c>
       <c r="D294" s="4" t="inlineStr">
         <is>
-          <t>/peptide-watch hero plus its 11 section banners, /peptide-matrix and /peptide-supply-chain heroes, the /peptide-hall-of-shame hero (scripts/rescue-2026-10-07-peptide-images.ts, logged in docs/ai/manus-media-rescue.md).</t>
+          <t>measured every page's title font, weight, size and label colour on live vs ours (136 pages). Now like live: Kava headings in Fraunces, HumanOS in Space Grotesk, the peptide tools / charity scorecard / thesis threads in the system serif, America Unbundled in the Iowan Old Style stack at live's size, /akbar in Fraunces 900, friend-gate and post-intervention in Georgia, and live's title sizes on peptide-matrix, peptide-supply-chain, rip-peptide-sciences and the HumanOS pages. Fonts load only on the pages that use them (src/lib/fonts/page-fonts.ts). Label colours stay the darker AA-contrast versions where live's lighter ones fail on a light background.</t>
         </is>
       </c>
       <c r="E294" s="14" t="inlineStr">
@@ -7615,7 +7615,7 @@
       <c r="A295" s="4" t="n"/>
       <c r="B295" s="4" t="inlineStr">
         <is>
-          <t>Live's editorial redesign, first group (2026-10-07)</t>
+          <t>Peptide page images rescued into Sanity and wired (2026-10-07)</t>
         </is>
       </c>
       <c r="C295" s="13" t="inlineStr">
@@ -7625,7 +7625,7 @@
       </c>
       <c r="D295" s="4" t="inlineStr">
         <is>
-          <t>dark top sections, narrow single text column, short red section rules and dark call-to-action bands on /invest, /amplifier, /community (now "Sign In to Join the Community", linking our real sign-in; live's made-up counters left out), /framework, /the-letter (daily provocation with "Share this thought" and "Search past provocations"), /engage, /diamond-cut, /ecosystem and the homepage's "The thinking doesn't stop here" band. Kept on purpose: AA-contrast colours where live's fail, "Enter the Gate" instead of live's $5,000 checkout on /diamond-cut.</t>
+          <t>/peptide-watch hero plus its 11 section banners, /peptide-matrix and /peptide-supply-chain heroes, the /peptide-hall-of-shame hero (scripts/rescue-2026-10-07-peptide-images.ts, logged in docs/ai/manus-media-rescue.md).</t>
         </is>
       </c>
       <c r="E295" s="14" t="inlineStr">
@@ -7638,7 +7638,7 @@
       <c r="A296" s="4" t="n"/>
       <c r="B296" s="4" t="inlineStr">
         <is>
-          <t>Live's redesign, second group (done 2026-10-08)</t>
+          <t>Live's editorial redesign, first group (2026-10-07)</t>
         </is>
       </c>
       <c r="C296" s="13" t="inlineStr">
@@ -7648,7 +7648,7 @@
       </c>
       <c r="D296" s="4" t="inlineStr">
         <is>
-          <t>re-measured all 18 pages on live vs a fresh production build (title font/size/weight/colour, labels, hero images). Already matching from 2026-10-07: /the-web, /spirits, /iboga-ibogaine (weight 800), /living-declaration, BrewSoul photo on /brewsoul, /brewsoul/browse, /brewsoul/first-sip (live has none there either), /quiz_25q, /recent-creations. Fixed today: /find-your-journey (64px title, red label), /impact-dashboard (64px title in essay ink, label spacing), red labels on /published and /speaking (plus its "rooms" chips), /soulscore "by ImpactSoul" label, /pri-calibration title (weight 900, solid cream, was a purple gradient), /clients (live's narrow 546px column for the whole page, 56px title, roomier stats band, cards 2 per row; two static inline styles moved to classes), /brewsoul/guest (live's BrewSoul photo on the guest card instead of "SN" initials, labels in capitals), /humanos/connect (cards line up with the title), /peptide-hall-of-shame (stats and label readable light gold; were dark gold on dark). Typed arrows on the touched links are icons now (rule 18). Deliberately not copied from live (new CONTRIBUTING rule 20, owner 2026-10-08): red labels on dark bands use #E07A80 (live's #8E1E25 on black is about 2:1, unreadable); /recent-creations keeps our darker label colours (live's fail contrast on white); /humanos/connect keeps "Start Reading" (that card links to the philosophy page, the quiz live's "Start the Assessment" implies doesn't exist). Checked: type check, l</t>
+          <t>dark top sections, narrow single text column, short red section rules and dark call-to-action bands on /invest, /amplifier, /community (now "Sign In to Join the Community", linking our real sign-in; live's made-up counters left out), /framework, /the-letter (daily provocation with "Share this thought" and "Search past provocations"), /engage, /diamond-cut, /ecosystem and the homepage's "The thinking doesn't stop here" band. Kept on purpose: AA-contrast colours where live's fail, "Enter the Gate" instead of live's $5,000 checkout on /diamond-cut.</t>
         </is>
       </c>
       <c r="E296" s="14" t="inlineStr">
@@ -7661,7 +7661,7 @@
       <c r="A297" s="4" t="n"/>
       <c r="B297" s="4" t="inlineStr">
         <is>
-          <t>BrewSoul top of page (2026-10-08, owner: "button in the center at the top doesn't look good")</t>
+          <t>Live's redesign, second group (done 2026-10-08)</t>
         </is>
       </c>
       <c r="C297" s="13" t="inlineStr">
@@ -7671,7 +7671,7 @@
       </c>
       <c r="D297" s="4" t="inlineStr">
         <is>
-          <t>the category badge ("Deep Research" etc.) sat centred in an empty strip, squeezed against the hero, because we copied live's doubled 52px top gap. Now one gap everywhere and the badge floats in the top-left corner, lined up with the BrewSoul logo (brewsoul-main.tsx, category-badge.tsx); checked on all 26 badge pages at 3 widths that it covers nothing. BrewSoul menu: on tablets (768-1023px) the links were cut off and "More" was hidden with no menu button at all; now the menu button shows below 1024px, 5 links + "More" from 1024px, all 8 from 1280px, "More" always visible.</t>
+          <t>re-measured all 18 pages on live vs a fresh production build (title font/size/weight/colour, labels, hero images). Already matching from 2026-10-07: /the-web, /spirits, /iboga-ibogaine (weight 800), /living-declaration, BrewSoul photo on /brewsoul, /brewsoul/browse, /brewsoul/first-sip (live has none there either), /quiz_25q, /recent-creations. Fixed today: /find-your-journey (64px title, red label), /impact-dashboard (64px title in essay ink, label spacing), red labels on /published and /speaking (plus its "rooms" chips), /soulscore "by ImpactSoul" label, /pri-calibration title (weight 900, solid cream, was a purple gradient), /clients (live's narrow 546px column for the whole page, 56px title, roomier stats band, cards 2 per row; two static inline styles moved to classes), /brewsoul/guest (live's BrewSoul photo on the guest card instead of "SN" initials, labels in capitals), /humanos/connect (cards line up with the title), /peptide-hall-of-shame (stats and label readable light gold; were dark gold on dark). Typed arrows on the touched links are icons now (rule 18). Deliberately not copied from live (new CONTRIBUTING rule 20, owner 2026-10-08): red labels on dark bands use #E07A80 (live's #8E1E25 on black is about 2:1, unreadable); /recent-creations keeps our darker label colours (live's fail contrast on white); /humanos/connect keeps "Start Reading" (that card links to the philosophy page, the quiz live's "Start the Assessment" implies doesn't exist). Checked: type check, l</t>
         </is>
       </c>
       <c r="E297" s="14" t="inlineStr">
@@ -7684,7 +7684,7 @@
       <c r="A298" s="4" t="n"/>
       <c r="B298" s="4" t="inlineStr">
         <is>
-          <t>/pri-efficacy's "Simulation / Live Calibrations" switch like live (2026-10-08)</t>
+          <t>BrewSoul top of page (2026-10-08, owner: "button in the center at the top doesn't look good")</t>
         </is>
       </c>
       <c r="C298" s="13" t="inlineStr">
@@ -7694,7 +7694,7 @@
       </c>
       <c r="D298" s="4" t="inlineStr">
         <is>
-          <t>shadcn Tabs, both panels in the server HTML (forceMount). The Live tab reads real aggregate numbers from pri_calibrations (getPriLiveStats() in src/lib/pri-research.ts: totals, opt-ins, average score per dimension; no rows leave the server), page stays static and refreshes every 10 minutes. Until the Supabase scripts are run (Phase 2) it says the numbers "aren't available just now" instead of a fake zero. Checked: build (○, 10m), server HTML has both tabs, tab switch at 390/1280px, no JS errors. Re-check with real numbers once the table exists.</t>
+          <t>the category badge ("Deep Research" etc.) sat centred in an empty strip, squeezed against the hero, because we copied live's doubled 52px top gap. Now one gap everywhere and the badge floats in the top-left corner, lined up with the BrewSoul logo (brewsoul-main.tsx, category-badge.tsx); checked on all 26 badge pages at 3 widths that it covers nothing. BrewSoul menu: on tablets (768-1023px) the links were cut off and "More" was hidden with no menu button at all; now the menu button shows below 1024px, 5 links + "More" from 1024px, all 8 from 1280px, "More" always visible.</t>
         </is>
       </c>
       <c r="E298" s="14" t="inlineStr">
@@ -7707,63 +7707,63 @@
       <c r="A299" s="4" t="n"/>
       <c r="B299" s="4" t="inlineStr">
         <is>
+          <t>/pri-efficacy's "Simulation / Live Calibrations" switch like live (2026-10-08)</t>
+        </is>
+      </c>
+      <c r="C299" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D299" s="4" t="inlineStr">
+        <is>
+          <t>shadcn Tabs, both panels in the server HTML (forceMount). The Live tab reads real aggregate numbers from pri_calibrations (getPriLiveStats() in src/lib/pri-research.ts: totals, opt-ins, average score per dimension; no rows leave the server), page stays static and refreshes every 10 minutes. Until the Supabase scripts are run (Phase 2) it says the numbers "aren't available just now" instead of a fake zero. Checked: build (○, 10m), server HTML has both tabs, tab switch at 390/1280px, no JS errors. Re-check with real numbers once the table exists.</t>
+        </is>
+      </c>
+      <c r="E299" s="14" t="inlineStr">
+        <is>
+          <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" s="4" t="n"/>
+      <c r="B300" s="4" t="inlineStr">
+        <is>
           <t>/brewsoul/browse hero readable (2026-10-08, owner said go ahead)</t>
         </is>
       </c>
-      <c r="C299" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D299" s="4" t="inlineStr">
+      <c r="C300" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D300" s="4" t="inlineStr">
         <is>
           <t>a soft cream glow behind the title block so "The Catalog", the subtitle and the stat labels read clearly over the coffee photo (live is hard to read there too; rule 20). Photo still shows around the edges. Checked at 390/1280px.</t>
         </is>
       </c>
-      <c r="E299" s="14" t="inlineStr">
+      <c r="E300" s="14" t="inlineStr">
         <is>
           <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
         </is>
       </c>
     </row>
-    <row r="300">
-      <c r="A300" s="10" t="inlineStr">
+    <row r="301">
+      <c r="A301" s="10" t="inlineStr">
         <is>
           <t>Phase 13 — Images Needed in Sanity</t>
         </is>
       </c>
-      <c r="B300" s="11" t="n"/>
-      <c r="C300" s="11" t="n"/>
-      <c r="D300" s="12" t="n"/>
-    </row>
-    <row r="301">
-      <c r="A301" s="4" t="n"/>
-      <c r="B301" s="4" t="inlineStr">
-        <is>
-          <t>Manus media rescue (2026-09-29)</t>
-        </is>
-      </c>
-      <c r="C301" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D301" s="4" t="inlineStr">
-        <is>
-          <t>all 94 Manus-hosted image/video references in the legacy source (/api/img/, /manus-storage/) were checked live. 91 were still downloadable, including the /akbar photos the entry below calls "permanently lost", and all 91 are now Sanity assets (scripts/rescue-manus-media.ts; Sanity dedupes by SHA-1). 3 were gone (HTTP 502). The manifest docs/ai/manus-media-rescue.md maps each one to the legacy files that used it and its Sanity URL. They are not wired into pages yet: go page by page, with real alt text. /facilitator-index's two diagrams are done (scripts/rescue-facilitator-images.ts).</t>
-        </is>
-      </c>
-      <c r="E301" s="14" t="inlineStr">
-        <is>
-          <t>Phase 13 — Images Needed in Sanity</t>
-        </is>
-      </c>
+      <c r="B301" s="11" t="n"/>
+      <c r="C301" s="11" t="n"/>
+      <c r="D301" s="12" t="n"/>
     </row>
     <row r="302">
       <c r="A302" s="4" t="n"/>
       <c r="B302" s="4" t="inlineStr">
         <is>
-          <t>Favicon</t>
+          <t>Manus media rescue (2026-09-29)</t>
         </is>
       </c>
       <c r="C302" s="13" t="inlineStr">
@@ -7773,7 +7773,7 @@
       </c>
       <c r="D302" s="4" t="inlineStr">
         <is>
-          <t>real "G" brand mark generated from the header's actual wordmark treatment (src/app/icon.tsx), see Phase 3</t>
+          <t>all 94 Manus-hosted image/video references in the legacy source (/api/img/, /manus-storage/) were checked live. 91 were still downloadable, including the /akbar photos the entry below calls "permanently lost", and all 91 are now Sanity assets (scripts/rescue-manus-media.ts; Sanity dedupes by SHA-1). 3 were gone (HTTP 502). The manifest docs/ai/manus-media-rescue.md maps each one to the legacy files that used it and its Sanity URL. They are not wired into pages yet: go page by page, with real alt text. /facilitator-index's two diagrams are done (scripts/rescue-facilitator-images.ts).</t>
         </is>
       </c>
       <c r="E302" s="14" t="inlineStr">
@@ -7786,17 +7786,17 @@
       <c r="A303" s="4" t="n"/>
       <c r="B303" s="4" t="inlineStr">
         <is>
-          <t>Site-wide: logo (light + dark) beyond the current text wordmark</t>
-        </is>
-      </c>
-      <c r="C303" s="15" t="inlineStr">
-        <is>
-          <t>Remaining</t>
+          <t>Favicon</t>
+        </is>
+      </c>
+      <c r="C303" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D303" s="4" t="inlineStr">
         <is>
-          <t>(Default/fallback OG image 1200×630 exists: public/images/default-og.png, checked 2026-10-02.)</t>
+          <t>real "G" brand mark generated from the header's actual wordmark treatment (src/app/icon.tsx), see Phase 3</t>
         </is>
       </c>
       <c r="E303" s="14" t="inlineStr">
@@ -7809,17 +7809,17 @@
       <c r="A304" s="4" t="n"/>
       <c r="B304" s="4" t="inlineStr">
         <is>
-          <t>Author photo(s) for blog author schema (Tony Greenberg headshot at minimum)</t>
-        </is>
-      </c>
-      <c r="C304" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Site-wide: logo (light + dark) beyond the current text wordmark</t>
+        </is>
+      </c>
+      <c r="C304" s="15" t="inlineStr">
+        <is>
+          <t>Remaining</t>
         </is>
       </c>
       <c r="D304" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02: the rescued headshot is already the author avatar in Sanity; now also in every post's Article JSON-LD (author image + url /about). The JSON-LD publisher logo pointed at /favicon.ico, a 404 here; now /icon.</t>
+          <t>(Default/fallback OG image 1200×630 exists: public/images/default-og.png, checked 2026-10-02.)</t>
         </is>
       </c>
       <c r="E304" s="14" t="inlineStr">
@@ -7832,7 +7832,7 @@
       <c r="A305" s="4" t="n"/>
       <c r="B305" s="4" t="inlineStr">
         <is>
-          <t>Blog hero images</t>
+          <t>Author photo(s) for blog author schema (Tony Greenberg headshot at minimum)</t>
         </is>
       </c>
       <c r="C305" s="13" t="inlineStr">
@@ -7842,7 +7842,7 @@
       </c>
       <c r="D305" s="4" t="inlineStr">
         <is>
-          <t>audited, then migrated. Final state:</t>
+          <t>2026-10-02: the rescued headshot is already the author avatar in Sanity; now also in every post's Article JSON-LD (author image + url /about). The JSON-LD publisher logo pointed at /favicon.ico, a 404 here; now /icon.</t>
         </is>
       </c>
       <c r="E305" s="14" t="inlineStr">
@@ -7855,7 +7855,7 @@
       <c r="A306" s="4" t="n"/>
       <c r="B306" s="4" t="inlineStr">
         <is>
-          <t>22 posts have a real hero image, now live in Sanity (17 already on RampRate's own CloudFront + 4 rescued from the legacy /api/img/ proxy + 1…</t>
+          <t>Blog hero images</t>
         </is>
       </c>
       <c r="C306" s="13" t="inlineStr">
@@ -7865,7 +7865,7 @@
       </c>
       <c r="D306" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> rescued from /manus-storage/, all pulled over by migrate-blog-posts.ts before Manus is decommissioned)</t>
+          <t>audited, then migrated. Final state:</t>
         </is>
       </c>
       <c r="E306" s="14" t="inlineStr">
@@ -7878,7 +7878,7 @@
       <c r="A307" s="4" t="n"/>
       <c r="B307" s="4" t="inlineStr">
         <is>
-          <t>7 more posts got a real, unique hero image rescued from the live legacy site's newly-added art this pass (scripts/rescue-2026-09-blog-images…</t>
+          <t>22 posts have a real hero image, now live in Sanity (17 already on RampRate's own CloudFront + 4 rescued from the legacy /api/img/ proxy + 1…</t>
         </is>
       </c>
       <c r="C307" s="13" t="inlineStr">
@@ -7888,7 +7888,7 @@
       </c>
       <c r="D307" s="4" t="inlineStr">
         <is>
-          <t>.ts — see the correction note above): california-toll-roads-legalized-scam, the-1000-hour-hold, conscious-capital-partnership-ecosystem, the-peptide-truth-65m-fraud-industry-vs-life-changing-medicine, clear-communication, building-services-market-transhuman-era, heart-protocol-addendum.</t>
+          <t xml:space="preserve"> rescued from /manus-storage/, all pulled over by migrate-blog-posts.ts before Manus is decommissioned)</t>
         </is>
       </c>
       <c r="E307" s="14" t="inlineStr">
@@ -7901,17 +7901,17 @@
       <c r="A308" s="4" t="n"/>
       <c r="B308" s="4" t="inlineStr">
         <is>
-          <t>92 posts still need a real, unique hero image</t>
-        </is>
-      </c>
-      <c r="C308" s="15" t="inlineStr">
-        <is>
-          <t>Remaining</t>
+          <t>7 more posts got a real, unique hero image rescued from the live legacy site's newly-added art this pass (scripts/rescue-2026-09-blog-images…</t>
+        </is>
+      </c>
+      <c r="C308" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D308" s="4" t="inlineStr">
         <is>
-          <t>(down from 99). Tracked one row per post, with a suggested image-generation prompt, in BLOG-IMAGE-BRIEFS.md — work through that file and check items off there, not here. No image-generation tool was connected in this environment as of this writing; either connect one (e.g. an MCP image-gen extension), source these manually/with a designer then upload via Sanity Studio (/studio), or re-check the live legacy site periodically per the correction note above.</t>
+          <t>.ts — see the correction note above): california-toll-roads-legalized-scam, the-1000-hour-hold, conscious-capital-partnership-ecosystem, the-peptide-truth-65m-fraud-industry-vs-life-changing-medicine, clear-communication, building-services-market-transhuman-era, heart-protocol-addendum.</t>
         </is>
       </c>
       <c r="E308" s="14" t="inlineStr">
@@ -7924,17 +7924,17 @@
       <c r="A309" s="4" t="n"/>
       <c r="B309" s="4" t="inlineStr">
         <is>
-          <t>Blog: per-post OG image if different from hero (many posts can reuse hero as OG)</t>
-        </is>
-      </c>
-      <c r="C309" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>92 posts still need a real, unique hero image</t>
+        </is>
+      </c>
+      <c r="C309" s="15" t="inlineStr">
+        <is>
+          <t>Remaining</t>
         </is>
       </c>
       <c r="D309" s="4" t="inlineStr">
         <is>
-          <t>Confirmed 2026-10-02: generateMetadata uses seo.ogImage, else the hero, else the default OG image.</t>
+          <t>(down from 99). Tracked one row per post, with a suggested image-generation prompt, in BLOG-IMAGE-BRIEFS.md — work through that file and check items off there, not here. No image-generation tool was connected in this environment as of this writing; either connect one (e.g. an MCP image-gen extension), source these manually/with a designer then upload via Sanity Studio (/studio), or re-check the live legacy site periodically per the correction note above.</t>
         </is>
       </c>
       <c r="E309" s="14" t="inlineStr">
@@ -7947,7 +7947,7 @@
       <c r="A310" s="4" t="n"/>
       <c r="B310" s="4" t="inlineStr">
         <is>
-          <t>Marketing pages</t>
+          <t>Blog: per-post OG image if different from hero (many posts can reuse hero as OG)</t>
         </is>
       </c>
       <c r="C310" s="13" t="inlineStr">
@@ -7957,7 +7957,7 @@
       </c>
       <c r="D310" s="4" t="inlineStr">
         <is>
-          <t>hero/section images for /the-letter, /the-territory, /engine-room, /the-body, /the-nightstand, /recent-creations (portfolio thumbnails), /published (publication logos), /clients (client logos — confirm licensing before re-hosting). Checked against live 2026-10-02: same image count on every one; /the-territory, /engine-room, /recent-creations, /published, /clients have no images on live either.</t>
+          <t>Confirmed 2026-10-02: generateMetadata uses seo.ogImage, else the hero, else the default OG image.</t>
         </is>
       </c>
       <c r="E310" s="14" t="inlineStr">
@@ -7970,7 +7970,7 @@
       <c r="A311" s="4" t="n"/>
       <c r="B311" s="4" t="inlineStr">
         <is>
-          <t>/akbar essay images</t>
+          <t>Marketing pages</t>
         </is>
       </c>
       <c r="C311" s="13" t="inlineStr">
@@ -7980,7 +7980,7 @@
       </c>
       <c r="D311" s="4" t="inlineStr">
         <is>
-          <t>not lost after all: 20 of the 21 were rescued into Sanity by scripts/rescue-manus-media.ts (2026-09-28) and are wired back in legacy's layout (hero mosaic, JC portrait, 2x2 grid, 3 full-bleeds, 3-up strip, footer gallery) as of 2026-09-29. Only slider-3 was gone (HTTP 502); the hero mosaic is 4 tiles instead of 5.</t>
+          <t>hero/section images for /the-letter, /the-territory, /engine-room, /the-body, /the-nightstand, /recent-creations (portfolio thumbnails), /published (publication logos), /clients (client logos — confirm licensing before re-hosting). Checked against live 2026-10-02: same image count on every one; /the-territory, /engine-room, /recent-creations, /published, /clients have no images on live either.</t>
         </is>
       </c>
       <c r="E311" s="14" t="inlineStr">
@@ -7993,7 +7993,7 @@
       <c r="A312" s="4" t="n"/>
       <c r="B312" s="4" t="inlineStr">
         <is>
-          <t>Rescued page images wired back in (2026-09-29)</t>
+          <t>/akbar essay images</t>
         </is>
       </c>
       <c r="C312" s="13" t="inlineStr">
@@ -8003,7 +8003,7 @@
       </c>
       <c r="D312" s="4" t="inlineStr">
         <is>
-          <t>/living-declaration hero, hand image and Clarisse Abelarde artwork; /impact-dashboard earth hero; /find-my banner; /find-your-coffee dark photo landing (legacy copy restored, replacing an intro that wasn't in legacy). Also wired (second pass): /consciousness-scale (legacy's hero-first flow restored, the invented intro screen removed), /find-your-me hero, /humanos hero, the HumanOS nav logo, and all 12 HumanOS people headshots (/humanos/ecosystem, /humanos/philosophy). Blog-body images (2026-09-29): all 19 the migration dropped are restored by scripts/restore-blog-body-images.ts as Sanity drafts on 4 posts (Clarisse Abelarde 7, You Are the Moat 4, FRQNCY 6, Energy Is Money 2), waiting to be published in Studio; the other blog-listed assets were heroes already set. Still unwired from docs/ai/manus-media-rescue.md: and /alex-azzi's subject photo (a photo of a real person on an accusation page: needs Tony's yes first).</t>
+          <t>not lost after all: 20 of the 21 were rescued into Sanity by scripts/rescue-manus-media.ts (2026-09-28) and are wired back in legacy's layout (hero mosaic, JC portrait, 2x2 grid, 3 full-bleeds, 3-up strip, footer gallery) as of 2026-09-29. Only slider-3 was gone (HTTP 502); the hero mosaic is 4 tiles instead of 5.</t>
         </is>
       </c>
       <c r="E312" s="14" t="inlineStr">
@@ -8016,7 +8016,7 @@
       <c r="A313" s="4" t="n"/>
       <c r="B313" s="4" t="inlineStr">
         <is>
-          <t>BrewSoul: coffee/product images (brewsoul-coffees-expanded.ts likely has image refs</t>
+          <t>Rescued page images wired back in (2026-09-29)</t>
         </is>
       </c>
       <c r="C313" s="13" t="inlineStr">
@@ -8026,7 +8026,7 @@
       </c>
       <c r="D313" s="4" t="inlineStr">
         <is>
-          <t>audit), city guide header images, roaster directory photos. Audited 2026-09-09 (status spreadsheet), confirmed 2026-10-02: city guides already have photos; coffees, chains and roasters have no image field in legacy or here (text-only by design); farms got real photos.</t>
+          <t>/living-declaration hero, hand image and Clarisse Abelarde artwork; /impact-dashboard earth hero; /find-my banner; /find-your-coffee dark photo landing (legacy copy restored, replacing an intro that wasn't in legacy). Also wired (second pass): /consciousness-scale (legacy's hero-first flow restored, the invented intro screen removed), /find-your-me hero, /humanos hero, the HumanOS nav logo, and all 12 HumanOS people headshots (/humanos/ecosystem, /humanos/philosophy). Blog-body images (2026-09-29): all 19 the migration dropped are restored by scripts/restore-blog-body-images.ts as Sanity drafts on 4 posts (Clarisse Abelarde 7, You Are the Moat 4, FRQNCY 6, Energy Is Money 2), waiting to be published in Studio; the other blog-listed assets were heroes already set. Still unwired from docs/ai/manus-media-rescue.md: and /alex-azzi's subject photo (a photo of a real person on an accusation page: needs Tony's yes first).</t>
         </is>
       </c>
       <c r="E313" s="14" t="inlineStr">
@@ -8039,7 +8039,7 @@
       <c r="A314" s="4" t="n"/>
       <c r="B314" s="4" t="inlineStr">
         <is>
-          <t>65 page images moved off the Manus storage copy into Sanity (2026-10-02)</t>
+          <t>BrewSoul: coffee/product images (brewsoul-coffees-expanded.ts likely has image refs</t>
         </is>
       </c>
       <c r="C314" s="13" t="inlineStr">
@@ -8049,7 +8049,7 @@
       </c>
       <c r="D314" s="4" t="inlineStr">
         <is>
-          <t>every image the code loaded from d2xsxph8kpxj0f.cloudfront.net (PRI medicine images, Iboga module, facilitator index, /attention-theft, /alex-azzi, /protecting-your-business, /peyote-mescaline, HumanOS, the peptide quiz). Notes called it "RampRate's own CloudFront", but every file sits in the legacy Manus project's folder and its owner couldn't be confirmed. All 65 uploaded (scripts/rescue-cloudfront-images.ts), code rewritten, host removed from images.remotePatterns, no Sanity document used it. Table in docs/ai/manus-media-rescue.md.</t>
+          <t>audit), city guide header images, roaster directory photos. Audited 2026-09-09 (status spreadsheet), confirmed 2026-10-02: city guides already have photos; coffees, chains and roasters have no image field in legacy or here (text-only by design); farms got real photos.</t>
         </is>
       </c>
       <c r="E314" s="14" t="inlineStr">
@@ -8062,7 +8062,7 @@
       <c r="A315" s="4" t="n"/>
       <c r="B315" s="4" t="inlineStr">
         <is>
-          <t>PRI/Kava: medicine reference images (medicine-images.ts), facility images for /facilitator-index</t>
+          <t>65 page images moved off the Manus storage copy into Sanity (2026-10-02)</t>
         </is>
       </c>
       <c r="C315" s="13" t="inlineStr">
@@ -8072,7 +8072,7 @@
       </c>
       <c r="D315" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02: all in Sanity; image counts match live on PRI, Kava, Iboga, Peyote, facilitator pages.</t>
+          <t>every image the code loaded from d2xsxph8kpxj0f.cloudfront.net (PRI medicine images, Iboga module, facilitator index, /attention-theft, /alex-azzi, /protecting-your-business, /peyote-mescaline, HumanOS, the peptide quiz). Notes called it "RampRate's own CloudFront", but every file sits in the legacy Manus project's folder and its owner couldn't be confirmed. All 65 uploaded (scripts/rescue-cloudfront-images.ts), code rewritten, host removed from images.remotePatterns, no Sanity document used it. Table in docs/ai/manus-media-rescue.md.</t>
         </is>
       </c>
       <c r="E315" s="14" t="inlineStr">
@@ -8085,7 +8085,7 @@
       <c r="A316" s="4" t="n"/>
       <c r="B316" s="4" t="inlineStr">
         <is>
-          <t>Manifesto/Attention Theft: any diagram/illustration assets used on the mega-page</t>
+          <t>PRI/Kava: medicine reference images (medicine-images.ts), facility images for /facilitator-index</t>
         </is>
       </c>
       <c r="C316" s="13" t="inlineStr">
@@ -8095,7 +8095,7 @@
       </c>
       <c r="D316" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02: 6 of live's 7 are in (now in Sanity); the 7th belongs to the Wall of Shame section left out on purpose.</t>
+          <t>2026-10-02: all in Sanity; image counts match live on PRI, Kava, Iboga, Peyote, facilitator pages.</t>
         </is>
       </c>
       <c r="E316" s="14" t="inlineStr">
@@ -8108,17 +8108,17 @@
       <c r="A317" s="4" t="n"/>
       <c r="B317" s="4" t="inlineStr">
         <is>
-          <t>Assessment result-screen background art (flagged in STATUS.md as a known gap</t>
-        </is>
-      </c>
-      <c r="C317" s="15" t="inlineStr">
-        <is>
-          <t>Remaining</t>
+          <t>Manifesto/Attention Theft: any diagram/illustration assets used on the mega-page</t>
+        </is>
+      </c>
+      <c r="C317" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D317" s="4" t="inlineStr">
         <is>
-          <t>18/20 assessments currently have plain black backgrounds; sourcing themed art here also closes that gap)</t>
+          <t>2026-10-02: 6 of live's 7 are in (now in Sanity); the 7th belongs to the Wall of Shame section left out on purpose.</t>
         </is>
       </c>
       <c r="E317" s="14" t="inlineStr">
@@ -8131,17 +8131,17 @@
       <c r="A318" s="4" t="n"/>
       <c r="B318" s="4" t="inlineStr">
         <is>
-          <t>Chatbot: FauxTony avatar/icon</t>
-        </is>
-      </c>
-      <c r="C318" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Assessment result-screen background art (flagged in STATUS.md as a known gap</t>
+        </is>
+      </c>
+      <c r="C318" s="15" t="inlineStr">
+        <is>
+          <t>Remaining</t>
         </is>
       </c>
       <c r="D318" s="4" t="inlineStr">
         <is>
-          <t>Not needed (2026-10-02): the chatbot phase (Phase 10) was cancelled.</t>
+          <t>18/20 assessments currently have plain black backgrounds; sourcing themed art here also closes that gap)</t>
         </is>
       </c>
       <c r="E318" s="14" t="inlineStr">
@@ -8154,73 +8154,73 @@
       <c r="A319" s="4" t="n"/>
       <c r="B319" s="4" t="inlineStr">
         <is>
+          <t>Chatbot: FauxTony avatar/icon</t>
+        </is>
+      </c>
+      <c r="C319" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D319" s="4" t="inlineStr">
+        <is>
+          <t>Not needed (2026-10-02): the chatbot phase (Phase 10) was cancelled.</t>
+        </is>
+      </c>
+      <c r="E319" s="14" t="inlineStr">
+        <is>
+          <t>Phase 13 — Images Needed in Sanity</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" s="4" t="n"/>
+      <c r="B320" s="4" t="inlineStr">
+        <is>
           <t>Audit client/public/ (including alex-azzi/, brewsoul/ subfolders) for any static assets already sitting there unused that should be pulled i…</t>
         </is>
       </c>
-      <c r="C319" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D319" s="4" t="inlineStr">
+      <c r="C320" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D320" s="4" t="inlineStr">
         <is>
           <t>n rather than re-created. Done 2026-10-02: no images there at all (only llms.txt, a BrewSoul catalog, Manus debug files, design-options.html). Found and fixed a cutover risk instead: live serves two Google site-verification files (/google6881a0411c48b301.html, /alex-azzi/googleedff0185753a4a1f.html) that the new site returned 404 for, so Search Console could lose verification at DNS cutover. Both copied to public/ byte for byte. Not copied: site.webmanifest (its icons don't exist here; Next's app/icon.tsx covers the favicon).</t>
         </is>
       </c>
-      <c r="E319" s="14" t="inlineStr">
+      <c r="E320" s="14" t="inlineStr">
         <is>
           <t>Phase 13 — Images Needed in Sanity</t>
         </is>
       </c>
     </row>
-    <row r="320">
-      <c r="A320" s="10" t="inlineStr">
+    <row r="321">
+      <c r="A321" s="10" t="inlineStr">
         <is>
           <t>Phase 14 — QA &amp; Launch</t>
         </is>
       </c>
-      <c r="B320" s="11" t="n"/>
-      <c r="C320" s="11" t="n"/>
-      <c r="D320" s="12" t="n"/>
-    </row>
-    <row r="321">
-      <c r="A321" s="4" t="n"/>
-      <c r="B321" s="4" t="inlineStr">
-        <is>
-          <t>Mobile responsive pass on every ported section</t>
-        </is>
-      </c>
-      <c r="C321" s="15" t="inlineStr">
-        <is>
-          <t>Remaining</t>
-        </is>
-      </c>
-      <c r="D321" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-29: no page scrolls sideways at 375px any more (114 pages checked in Chrome: every unique page plus 3 of each templated set like blog posts and coffees). Fixed: BrewSoul NextSteps forced 3 columns (and used an inline style), charity-scorecard tab row, /brewsoul/browse filter dropdowns, /the-philosophy hero glow. Still to check by hand: 44px tap targets and Safari iOS. 2026-09-30: 44px tap targets on phones for the shared header, footer, BrewSoul/Kava/HumanOS menus and ~100 standalone links (undersized targets 1,904 → 578; the rest are 24-43px pills/chips that meet WCAG 2.2 AA). axe target-size (WCAG 2.2 AA, with its spacing exception): 0 failures on 114 pages. Safari/iPhone (WebKit, iPhone 14 emulation): all 114 pages load, no sideways scroll, no JS errors; form fields under 16px (iOS zoom-on-tap) fixed site-wide in globals.css. Still to check on a real iPhone: BrewSoul's bottom journey bar showed page text through it in headless WebKit only (taps hit the bar correctly; Chrome renders it solid). Fixed 2026-10-09: the bar is now solid (bg-[#2C1810], was 92% plus backdrop-blur-md), so nothing can show through even where the blur isn't drawn; checked in WebKit (iPhone 13 profile) and Chrome: background rgb(44, 24, 16), no text behind the buttons. A real iPhone check is still part of Phase 14.</t>
-        </is>
-      </c>
-      <c r="E321" s="14" t="inlineStr">
-        <is>
-          <t>Phase 14 — QA &amp; Launch</t>
-        </is>
-      </c>
+      <c r="B321" s="11" t="n"/>
+      <c r="C321" s="11" t="n"/>
+      <c r="D321" s="12" t="n"/>
     </row>
     <row r="322">
       <c r="A322" s="4" t="n"/>
       <c r="B322" s="4" t="inlineStr">
         <is>
-          <t>Accessibility pass (WCAG AA contrast, 44px touch targets, keyboard nav)</t>
-        </is>
-      </c>
-      <c r="C322" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Mobile responsive pass on every ported section</t>
+        </is>
+      </c>
+      <c r="C322" s="15" t="inlineStr">
+        <is>
+          <t>Remaining</t>
         </is>
       </c>
       <c r="D322" s="4" t="inlineStr">
         <is>
-          <t>same bar as legacy QA_MASTER_PROMPT.md. 2026-09-29 axe-core pass (WCAG 2.1 AA, same 114 pages, production build): all unlabeled dropdowns/inputs and unnamed links fixed; contrast down from 1,453 failing items on 106 pages to 1,038 on 70 (43 pages fully clean). Shared fixes: brand gold #8b6914 → #836311 site-wide (was 4.3:1 on cream, AA needs 4.5), header "⌘K"/social icons, BrewSoul nav and footer, HumanOS footer, Kava footer, assessment intro footnote, post-card image links. 2026-09-30: contrast finished, 0 axe color-contrast failures left on the same 114 pages (production build). Token changes: --kava-saffron #b86a28 → #8e521f, --pri-purple-light #a855f7 → #b87bf9 (on-dark purple only), --crusade-teal #0e7c7c → #0d7373; PriEyebrow goes light purple inside a dark PriSection via group-data-dark/pri; /find-your-me and the journey tracker's dark glass panels 60-70% → 90% (legacy's own 60% glass on beige rendered gray, cream text failed). Everything else: nearest passing shade of the same hue, or gold ↔ gold-light on the wrong background. Left: 18 links inside text marked only by color (need an underline), 44px tap targets, keyboard nav. 2026-09-30: 18 color-only in-text links underlined (axe link-in-text-block: 0 left); keyboard focus visible on every focusable item on 8 sampled pages (two form fields had none, fixed). 2026-10-02 re-run (axe WCAG 2.2 AA, 142 pages × 375/1280px, production build, plus Tab through 40 stops per page): found 1,370 contrast failures (mostly BrewSoul'</t>
+          <t>2026-09-29: no page scrolls sideways at 375px any more (114 pages checked in Chrome: every unique page plus 3 of each templated set like blog posts and coffees). Fixed: BrewSoul NextSteps forced 3 columns (and used an inline style), charity-scorecard tab row, /brewsoul/browse filter dropdowns, /the-philosophy hero glow. Still to check by hand: 44px tap targets and Safari iOS. 2026-09-30: 44px tap targets on phones for the shared header, footer, BrewSoul/Kava/HumanOS menus and ~100 standalone links (undersized targets 1,904 → 578; the rest are 24-43px pills/chips that meet WCAG 2.2 AA). axe target-size (WCAG 2.2 AA, with its spacing exception): 0 failures on 114 pages. Safari/iPhone (WebKit, iPhone 14 emulation): all 114 pages load, no sideways scroll, no JS errors; form fields under 16px (iOS zoom-on-tap) fixed site-wide in globals.css. Still to check on a real iPhone: BrewSoul's bottom journey bar showed page text through it in headless WebKit only (taps hit the bar correctly; Chrome renders it solid). Fixed 2026-10-09: the bar is now solid (bg-[#2C1810], was 92% plus backdrop-blur-md), so nothing can show through even where the blur isn't drawn; checked in WebKit (iPhone 13 profile) and Chrome: background rgb(44, 24, 16), no text behind the buttons. A real iPhone check is still part of Phase 14.</t>
         </is>
       </c>
       <c r="E322" s="14" t="inlineStr">
@@ -8233,17 +8233,17 @@
       <c r="A323" s="4" t="n"/>
       <c r="B323" s="4" t="inlineStr">
         <is>
-          <t>No dead-end pages (every page links to 2+ others)</t>
-        </is>
-      </c>
-      <c r="C323" s="15" t="inlineStr">
-        <is>
-          <t>Remaining</t>
+          <t>Accessibility pass (WCAG AA contrast, 44px touch targets, keyboard nav)</t>
+        </is>
+      </c>
+      <c r="C323" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D323" s="4" t="inlineStr">
         <is>
-          <t>same bar as legacy MASTER_QUALITY_PROMPT.md 2026-09-30 scan (496 sitemap pages, header/footer links not counted): every page has a way home (the 6 HumanOS pages had none, in legacy too; added a "← TonyGreenberg.com" footer link). ~17 quiz pages only look like dead ends on their intro screen; their result screens link to related assessments. Left for a content decision: ~20 marketing pages (/akbar, /amplifier, /diamond-cut, /ecosystem, /engage, /engine-room, /intel, /invest, /pick-up-the-phone, /protecting-your-business, /published, /speaking, /the-nightstand, /the-territory, /the-web, /under-nda, /pri-calibration, /charity-scorecard and its detail pages) link to only 0-1 other page in their content. The port matches legacy there (legacy was just as sparse), so adding related links is new content and needs the owner's yes.</t>
+          <t>same bar as legacy QA_MASTER_PROMPT.md. 2026-09-29 axe-core pass (WCAG 2.1 AA, same 114 pages, production build): all unlabeled dropdowns/inputs and unnamed links fixed; contrast down from 1,453 failing items on 106 pages to 1,038 on 70 (43 pages fully clean). Shared fixes: brand gold #8b6914 → #836311 site-wide (was 4.3:1 on cream, AA needs 4.5), header "⌘K"/social icons, BrewSoul nav and footer, HumanOS footer, Kava footer, assessment intro footnote, post-card image links. 2026-09-30: contrast finished, 0 axe color-contrast failures left on the same 114 pages (production build). Token changes: --kava-saffron #b86a28 → #8e521f, --pri-purple-light #a855f7 → #b87bf9 (on-dark purple only), --crusade-teal #0e7c7c → #0d7373; PriEyebrow goes light purple inside a dark PriSection via group-data-dark/pri; /find-your-me and the journey tracker's dark glass panels 60-70% → 90% (legacy's own 60% glass on beige rendered gray, cream text failed). Everything else: nearest passing shade of the same hue, or gold ↔ gold-light on the wrong background. Left: 18 links inside text marked only by color (need an underline), 44px tap targets, keyboard nav. 2026-09-30: 18 color-only in-text links underlined (axe link-in-text-block: 0 left); keyboard focus visible on every focusable item on 8 sampled pages (two form fields had none, fixed). 2026-10-02 re-run (axe WCAG 2.2 AA, 142 pages × 375/1280px, production build, plus Tab through 40 stops per page): found 1,370 contrast failures (mostly BrewSoul'</t>
         </is>
       </c>
       <c r="E323" s="14" t="inlineStr">
@@ -8256,7 +8256,7 @@
       <c r="A324" s="4" t="n"/>
       <c r="B324" s="4" t="inlineStr">
         <is>
-          <t>Cross-browser check (Safari iOS in particular, per legacy performance notes) 2026-10-06 WebKit pass (Playwright WebKit, iPhone 13 profile, 1…</t>
+          <t>No dead-end pages (every page links to 2+ others)</t>
         </is>
       </c>
       <c r="C324" s="15" t="inlineStr">
@@ -8266,7 +8266,7 @@
       </c>
       <c r="D324" s="4" t="inlineStr">
         <is>
-          <t>52 pages: every unique page plus 3 of each templated set, production build): no page pans sideways, no failed requests, no JS errors. Found and fixed on the way: upgrade-insecure-requests in the new CSP made Safari fetch every stylesheet and font over https on localhost (dropped; the site is HTTPS-only via HSTS anyway), and .toLocaleString() without a locale caused a hydration error on /brewsoul/chains in Safari (all number formatting now en-US). Left: a check on a real iPhone (Phase 14).</t>
+          <t>same bar as legacy MASTER_QUALITY_PROMPT.md 2026-09-30 scan (496 sitemap pages, header/footer links not counted): every page has a way home (the 6 HumanOS pages had none, in legacy too; added a "← TonyGreenberg.com" footer link). ~17 quiz pages only look like dead ends on their intro screen; their result screens link to related assessments. Left for a content decision: ~20 marketing pages (/akbar, /amplifier, /diamond-cut, /ecosystem, /engage, /engine-room, /intel, /invest, /pick-up-the-phone, /protecting-your-business, /published, /speaking, /the-nightstand, /the-territory, /the-web, /under-nda, /pri-calibration, /charity-scorecard and its detail pages) link to only 0-1 other page in their content. The port matches legacy there (legacy was just as sparse), so adding related links is new content and needs the owner's yes.</t>
         </is>
       </c>
       <c r="E324" s="14" t="inlineStr">
@@ -8279,7 +8279,7 @@
       <c r="A325" s="4" t="n"/>
       <c r="B325" s="4" t="inlineStr">
         <is>
-          <t>Remove noindex only when sign-off is given</t>
+          <t>Cross-browser check (Safari iOS in particular, per legacy performance notes) 2026-10-06 WebKit pass (Playwright WebKit, iPhone 13 profile, 1…</t>
         </is>
       </c>
       <c r="C325" s="15" t="inlineStr">
@@ -8289,7 +8289,7 @@
       </c>
       <c r="D325" s="4" t="inlineStr">
         <is>
-          <t>do not launch indexable by accident (The only noindex is the host-based one for *.netlify.app above, so the real domain is indexable as soon as DNS points at it: sign-off must come before DNS.)</t>
+          <t>52 pages: every unique page plus 3 of each templated set, production build): no page pans sideways, no failed requests, no JS errors. Found and fixed on the way: upgrade-insecure-requests in the new CSP made Safari fetch every stylesheet and font over https on localhost (dropped; the site is HTTPS-only via HSTS anyway), and .toLocaleString() without a locale caused a hydration error on /brewsoul/chains in Safari (all number formatting now en-US). Left: a check on a real iPhone (Phase 14).</t>
         </is>
       </c>
       <c r="E325" s="14" t="inlineStr">
@@ -8302,7 +8302,7 @@
       <c r="A326" s="4" t="n"/>
       <c r="B326" s="4" t="inlineStr">
         <is>
-          <t>Final stakeholder sign-off (Tony/Darryl/Kimberly) on the ported site before DNS cutover</t>
+          <t>Remove noindex only when sign-off is given</t>
         </is>
       </c>
       <c r="C326" s="15" t="inlineStr">
@@ -8310,7 +8310,11 @@
           <t>Remaining</t>
         </is>
       </c>
-      <c r="D326" s="4" t="inlineStr"/>
+      <c r="D326" s="4" t="inlineStr">
+        <is>
+          <t>do not launch indexable by accident (The only noindex is the host-based one for *.netlify.app above, so the real domain is indexable as soon as DNS points at it: sign-off must come before DNS.)</t>
+        </is>
+      </c>
       <c r="E326" s="14" t="inlineStr">
         <is>
           <t>Phase 14 — QA &amp; Launch</t>
@@ -8321,7 +8325,7 @@
       <c r="A327" s="4" t="n"/>
       <c r="B327" s="4" t="inlineStr">
         <is>
-          <t>DNS cutover, legacy app decommissioned only after a stable overlap window</t>
+          <t>Final stakeholder sign-off (Tony/Darryl/Kimberly) on the ported site before DNS cutover</t>
         </is>
       </c>
       <c r="C327" s="15" t="inlineStr">
@@ -8336,21 +8340,40 @@
         </is>
       </c>
     </row>
+    <row r="328">
+      <c r="A328" s="4" t="n"/>
+      <c r="B328" s="4" t="inlineStr">
+        <is>
+          <t>DNS cutover, legacy app decommissioned only after a stable overlap window</t>
+        </is>
+      </c>
+      <c r="C328" s="15" t="inlineStr">
+        <is>
+          <t>Remaining</t>
+        </is>
+      </c>
+      <c r="D328" s="4" t="inlineStr"/>
+      <c r="E328" s="14" t="inlineStr">
+        <is>
+          <t>Phase 14 — QA &amp; Launch</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D327"/>
+  <autoFilter ref="A1:D328"/>
   <mergeCells count="14">
     <mergeCell ref="A150:D150"/>
-    <mergeCell ref="A320:D320"/>
+    <mergeCell ref="A321:D321"/>
     <mergeCell ref="A237:D237"/>
     <mergeCell ref="A58:D58"/>
     <mergeCell ref="A258:D258"/>
     <mergeCell ref="A209:D209"/>
     <mergeCell ref="A205:D205"/>
     <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A301:D301"/>
     <mergeCell ref="A43:D43"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A183:D183"/>
-    <mergeCell ref="A300:D300"/>
     <mergeCell ref="A32:D32"/>
     <mergeCell ref="A123:D123"/>
   </mergeCells>
@@ -8364,7 +8387,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -8602,7 +8625,7 @@
       <c r="A13" s="4" t="n"/>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Still different from live (needs a yes)</t>
+          <t>Lighthouse pass (performance/accessibility/SEO) on top 20 pages by traffic 2026-09-30, 20 key pages (no traffic data yet), local production …</t>
         </is>
       </c>
       <c r="C13" s="15" t="inlineStr">
@@ -8612,7 +8635,7 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>blog posts (done) (done 2026-10-07, see Phase 5); /find-my on live hides the site header. /walk-through is a 404 on live now.</t>
+          <t>build, mobile: averages performance 87, accessibility 99→100, best practices 100, SEO 92→100, CLS 0 everywhere. Fixed: public/robots.txt had an LLMs: line (not a real directive) that made Google treat the whole file as invalid, now a comment; h3/h4 headings skipping a level on /assessments, /kava, /peptide-watch (same look, right tag); the Kava and /attention-theft back-arrow links had no accessible name on phones; two small phone-width contrast misses. Left: performance is local-machine only (±10-15 points, see CONTRIBUTING.md); the slowest were / 76 (LCP 5.2 s), /psychedelic-readiness-index 82, /iboga-ibogaine 83. Re-run against the Netlify deploy before launch. 2026-10-06 re-run against the Netlify deploy (14 key pages, mobile): accessibility 100 and CLS 0 on every page, SEO clean (only the expected netlify.app noindex), performance 77-97 held back by 3-4 s LCP. Fixed: all 21 hero images moved off the deprecated priority prop to fetchPriority="high" + loading="eager" (Next 16); /iboga-ibogaine hero and the first card on /blog and category pages no longer lazy-loaded; sizes on the Four Doors cards (~150 KiB per page), /humanos diagram (~100 KiB) and /about headshot; urlFor no longer imports the Sanity client, so ~115 KB of Sanity client code stopped loading on / and /blog; React hydration error #418 on / and /blog (post dates) gone, checked in two time zones; /blog is static again; empty icon &lt;th&gt;s on /iboga-ibogaine labelled; category page reads use sanityFetch(). Left: se</t>
         </is>
       </c>
       <c r="E13" s="14" t="inlineStr">
@@ -8625,7 +8648,7 @@
       <c r="A14" s="4" t="n"/>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Design change on live, needs a decision</t>
+          <t>SEO audit items needing a yes (2026-10-06)</t>
         </is>
       </c>
       <c r="C14" s="15" t="inlineStr">
@@ -8635,7 +8658,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>live's story pages now use Cormorant Garamond for titles (ours: Playfair Display), a lighter title weight (400 vs our 700), and a red eyebrow label (#8E1E25, wider letter spacing) instead of our gold. A site-wide font swap is a design call, so not done.</t>
+          <t>the pack's new copy (homepage title/description, five-cups title, description, short answer, FAQ, heading rewrites, entity statement, newsletter block, author box, health disclaimer, COA wording); "Further Reading" shown twice on posts (merge the lists?); long post title (84 chars), homepage description length and obsolete keywords tag, slugs (/blog/five-cups, the -2 slug; would need redirects), "Six lenses" over four cards, sources for health claims and proof for "$10B+", "Certified B Corp", "Validity: 91", legal review of the homepage Case File banner, ABIT waitlist disclosures, one contact email, the two one-post categories, fewer homepage CTAs / email signup / table of contents / explaining "COA".</t>
         </is>
       </c>
       <c r="E14" s="14" t="inlineStr">
@@ -8648,7 +8671,7 @@
       <c r="A15" s="4" t="n"/>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Lighthouse pass (performance/accessibility/SEO) on top 20 pages by traffic 2026-09-30, 20 key pages (no traffic data yet), local production …</t>
+          <t>Connect Google Search Console + GA4 to the new deployment on day one of cutover</t>
         </is>
       </c>
       <c r="C15" s="15" t="inlineStr">
@@ -8656,11 +8679,7 @@
           <t>Remaining</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>build, mobile: averages performance 87, accessibility 99→100, best practices 100, SEO 92→100, CLS 0 everywhere. Fixed: public/robots.txt had an LLMs: line (not a real directive) that made Google treat the whole file as invalid, now a comment; h3/h4 headings skipping a level on /assessments, /kava, /peptide-watch (same look, right tag); the Kava and /attention-theft back-arrow links had no accessible name on phones; two small phone-width contrast misses. Left: performance is local-machine only (±10-15 points, see CONTRIBUTING.md); the slowest were / 76 (LCP 5.2 s), /psychedelic-readiness-index 82, /iboga-ibogaine 83. Re-run against the Netlify deploy before launch. 2026-10-06 re-run against the Netlify deploy (14 key pages, mobile): accessibility 100 and CLS 0 on every page, SEO clean (only the expected netlify.app noindex), performance 77-97 held back by 3-4 s LCP. Fixed: all 21 hero images moved off the deprecated priority prop to fetchPriority="high" + loading="eager" (Next 16); /iboga-ibogaine hero and the first card on /blog and category pages no longer lazy-loaded; sizes on the Four Doors cards (~150 KiB per page), /humanos diagram (~100 KiB) and /about headshot; urlFor no longer imports the Sanity client, so ~115 KB of Sanity client code stopped loading on / and /blog; React hydration error #418 on / and /blog (post dates) gone, checked in two time zones; /blog is static again; empty icon &lt;th&gt;s on /iboga-ibogaine labelled; category page reads use sanityFetch(). Left: se</t>
-        </is>
-      </c>
+      <c r="D15" s="4" t="inlineStr"/>
       <c r="E15" s="14" t="inlineStr">
         <is>
           <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
@@ -8668,33 +8687,20 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="n"/>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>SEO audit items needing a yes (2026-10-06)</t>
-        </is>
-      </c>
-      <c r="C16" s="15" t="inlineStr">
-        <is>
-          <t>Remaining</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>the pack's new copy (homepage title/description, five-cups title, description, short answer, FAQ, heading rewrites, entity statement, newsletter block, author box, health disclaimer, COA wording); "Further Reading" shown twice on posts (merge the lists?); long post title (84 chars), homepage description length and obsolete keywords tag, slugs (/blog/five-cups, the -2 slug; would need redirects), "Six lenses" over four cards, sources for health claims and proof for "$10B+", "Certified B Corp", "Validity: 91", legal review of the homepage Case File banner, ABIT waitlist disclosures, one contact email, the two one-post categories, fewer homepage CTAs / email signup / table of contents / explaining "COA".</t>
-        </is>
-      </c>
-      <c r="E16" s="14" t="inlineStr">
-        <is>
-          <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
-        </is>
-      </c>
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>Phase 13 — Images Needed in Sanity</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="n"/>
+      <c r="C16" s="11" t="n"/>
+      <c r="D16" s="12" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n"/>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Connect Google Search Console + GA4 to the new deployment on day one of cutover</t>
+          <t>Site-wide: logo (light + dark) beyond the current text wordmark</t>
         </is>
       </c>
       <c r="C17" s="15" t="inlineStr">
@@ -8702,28 +8708,45 @@
           <t>Remaining</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr"/>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>(Default/fallback OG image 1200×630 exists: public/images/default-og.png, checked 2026-10-02.)</t>
+        </is>
+      </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
-          <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
+          <t>Phase 13 — Images Needed in Sanity</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="inlineStr">
+      <c r="A18" s="4" t="n"/>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>92 posts still need a real, unique hero image</t>
+        </is>
+      </c>
+      <c r="C18" s="15" t="inlineStr">
+        <is>
+          <t>Remaining</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>(down from 99). Tracked one row per post, with a suggested image-generation prompt, in BLOG-IMAGE-BRIEFS.md — work through that file and check items off there, not here. No image-generation tool was connected in this environment as of this writing; either connect one (e.g. an MCP image-gen extension), source these manually/with a designer then upload via Sanity Studio (/studio), or re-check the live legacy site periodically per the correction note above.</t>
+        </is>
+      </c>
+      <c r="E18" s="14" t="inlineStr">
         <is>
           <t>Phase 13 — Images Needed in Sanity</t>
         </is>
       </c>
-      <c r="B18" s="11" t="n"/>
-      <c r="C18" s="11" t="n"/>
-      <c r="D18" s="12" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n"/>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Site-wide: logo (light + dark) beyond the current text wordmark</t>
+          <t>Assessment result-screen background art (flagged in STATUS.md as a known gap</t>
         </is>
       </c>
       <c r="C19" s="15" t="inlineStr">
@@ -8733,7 +8756,7 @@
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>(Default/fallback OG image 1200×630 exists: public/images/default-og.png, checked 2026-10-02.)</t>
+          <t>18/20 assessments currently have plain black backgrounds; sourcing themed art here also closes that gap)</t>
         </is>
       </c>
       <c r="E19" s="14" t="inlineStr">
@@ -8743,33 +8766,20 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="n"/>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>92 posts still need a real, unique hero image</t>
-        </is>
-      </c>
-      <c r="C20" s="15" t="inlineStr">
-        <is>
-          <t>Remaining</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>(down from 99). Tracked one row per post, with a suggested image-generation prompt, in BLOG-IMAGE-BRIEFS.md — work through that file and check items off there, not here. No image-generation tool was connected in this environment as of this writing; either connect one (e.g. an MCP image-gen extension), source these manually/with a designer then upload via Sanity Studio (/studio), or re-check the live legacy site periodically per the correction note above.</t>
-        </is>
-      </c>
-      <c r="E20" s="14" t="inlineStr">
-        <is>
-          <t>Phase 13 — Images Needed in Sanity</t>
-        </is>
-      </c>
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>Phase 14 — QA &amp; Launch</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="n"/>
+      <c r="C20" s="11" t="n"/>
+      <c r="D20" s="12" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n"/>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Assessment result-screen background art (flagged in STATUS.md as a known gap</t>
+          <t>Mobile responsive pass on every ported section</t>
         </is>
       </c>
       <c r="C21" s="15" t="inlineStr">
@@ -8779,30 +8789,43 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>18/20 assessments currently have plain black backgrounds; sourcing themed art here also closes that gap)</t>
+          <t>2026-09-29: no page scrolls sideways at 375px any more (114 pages checked in Chrome: every unique page plus 3 of each templated set like blog posts and coffees). Fixed: BrewSoul NextSteps forced 3 columns (and used an inline style), charity-scorecard tab row, /brewsoul/browse filter dropdowns, /the-philosophy hero glow. Still to check by hand: 44px tap targets and Safari iOS. 2026-09-30: 44px tap targets on phones for the shared header, footer, BrewSoul/Kava/HumanOS menus and ~100 standalone links (undersized targets 1,904 → 578; the rest are 24-43px pills/chips that meet WCAG 2.2 AA). axe target-size (WCAG 2.2 AA, with its spacing exception): 0 failures on 114 pages. Safari/iPhone (WebKit, iPhone 14 emulation): all 114 pages load, no sideways scroll, no JS errors; form fields under 16px (iOS zoom-on-tap) fixed site-wide in globals.css. Still to check on a real iPhone: BrewSoul's bottom journey bar showed page text through it in headless WebKit only (taps hit the bar correctly; Chrome renders it solid). Fixed 2026-10-09: the bar is now solid (bg-[#2C1810], was 92% plus backdrop-blur-md), so nothing can show through even where the blur isn't drawn; checked in WebKit (iPhone 13 profile) and Chrome: background rgb(44, 24, 16), no text behind the buttons. A real iPhone check is still part of Phase 14.</t>
         </is>
       </c>
       <c r="E21" s="14" t="inlineStr">
         <is>
-          <t>Phase 13 — Images Needed in Sanity</t>
+          <t>Phase 14 — QA &amp; Launch</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="10" t="inlineStr">
+      <c r="A22" s="4" t="n"/>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>No dead-end pages (every page links to 2+ others)</t>
+        </is>
+      </c>
+      <c r="C22" s="15" t="inlineStr">
+        <is>
+          <t>Remaining</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>same bar as legacy MASTER_QUALITY_PROMPT.md 2026-09-30 scan (496 sitemap pages, header/footer links not counted): every page has a way home (the 6 HumanOS pages had none, in legacy too; added a "← TonyGreenberg.com" footer link). ~17 quiz pages only look like dead ends on their intro screen; their result screens link to related assessments. Left for a content decision: ~20 marketing pages (/akbar, /amplifier, /diamond-cut, /ecosystem, /engage, /engine-room, /intel, /invest, /pick-up-the-phone, /protecting-your-business, /published, /speaking, /the-nightstand, /the-territory, /the-web, /under-nda, /pri-calibration, /charity-scorecard and its detail pages) link to only 0-1 other page in their content. The port matches legacy there (legacy was just as sparse), so adding related links is new content and needs the owner's yes.</t>
+        </is>
+      </c>
+      <c r="E22" s="14" t="inlineStr">
         <is>
           <t>Phase 14 — QA &amp; Launch</t>
         </is>
       </c>
-      <c r="B22" s="11" t="n"/>
-      <c r="C22" s="11" t="n"/>
-      <c r="D22" s="12" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n"/>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Mobile responsive pass on every ported section</t>
+          <t>Cross-browser check (Safari iOS in particular, per legacy performance notes) 2026-10-06 WebKit pass (Playwright WebKit, iPhone 13 profile, 1…</t>
         </is>
       </c>
       <c r="C23" s="15" t="inlineStr">
@@ -8812,7 +8835,7 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>2026-09-29: no page scrolls sideways at 375px any more (114 pages checked in Chrome: every unique page plus 3 of each templated set like blog posts and coffees). Fixed: BrewSoul NextSteps forced 3 columns (and used an inline style), charity-scorecard tab row, /brewsoul/browse filter dropdowns, /the-philosophy hero glow. Still to check by hand: 44px tap targets and Safari iOS. 2026-09-30: 44px tap targets on phones for the shared header, footer, BrewSoul/Kava/HumanOS menus and ~100 standalone links (undersized targets 1,904 → 578; the rest are 24-43px pills/chips that meet WCAG 2.2 AA). axe target-size (WCAG 2.2 AA, with its spacing exception): 0 failures on 114 pages. Safari/iPhone (WebKit, iPhone 14 emulation): all 114 pages load, no sideways scroll, no JS errors; form fields under 16px (iOS zoom-on-tap) fixed site-wide in globals.css. Still to check on a real iPhone: BrewSoul's bottom journey bar showed page text through it in headless WebKit only (taps hit the bar correctly; Chrome renders it solid). Fixed 2026-10-09: the bar is now solid (bg-[#2C1810], was 92% plus backdrop-blur-md), so nothing can show through even where the blur isn't drawn; checked in WebKit (iPhone 13 profile) and Chrome: background rgb(44, 24, 16), no text behind the buttons. A real iPhone check is still part of Phase 14.</t>
+          <t>52 pages: every unique page plus 3 of each templated set, production build): no page pans sideways, no failed requests, no JS errors. Found and fixed on the way: upgrade-insecure-requests in the new CSP made Safari fetch every stylesheet and font over https on localhost (dropped; the site is HTTPS-only via HSTS anyway), and .toLocaleString() without a locale caused a hydration error on /brewsoul/chains in Safari (all number formatting now en-US). Left: a check on a real iPhone (Phase 14).</t>
         </is>
       </c>
       <c r="E23" s="14" t="inlineStr">
@@ -8825,7 +8848,7 @@
       <c r="A24" s="4" t="n"/>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>No dead-end pages (every page links to 2+ others)</t>
+          <t>Remove noindex only when sign-off is given</t>
         </is>
       </c>
       <c r="C24" s="15" t="inlineStr">
@@ -8835,7 +8858,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>same bar as legacy MASTER_QUALITY_PROMPT.md 2026-09-30 scan (496 sitemap pages, header/footer links not counted): every page has a way home (the 6 HumanOS pages had none, in legacy too; added a "← TonyGreenberg.com" footer link). ~17 quiz pages only look like dead ends on their intro screen; their result screens link to related assessments. Left for a content decision: ~20 marketing pages (/akbar, /amplifier, /diamond-cut, /ecosystem, /engage, /engine-room, /intel, /invest, /pick-up-the-phone, /protecting-your-business, /published, /speaking, /the-nightstand, /the-territory, /the-web, /under-nda, /pri-calibration, /charity-scorecard and its detail pages) link to only 0-1 other page in their content. The port matches legacy there (legacy was just as sparse), so adding related links is new content and needs the owner's yes.</t>
+          <t>do not launch indexable by accident (The only noindex is the host-based one for *.netlify.app above, so the real domain is indexable as soon as DNS points at it: sign-off must come before DNS.)</t>
         </is>
       </c>
       <c r="E24" s="14" t="inlineStr">
@@ -8848,7 +8871,7 @@
       <c r="A25" s="4" t="n"/>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Cross-browser check (Safari iOS in particular, per legacy performance notes) 2026-10-06 WebKit pass (Playwright WebKit, iPhone 13 profile, 1…</t>
+          <t>Final stakeholder sign-off (Tony/Darryl/Kimberly) on the ported site before DNS cutover</t>
         </is>
       </c>
       <c r="C25" s="15" t="inlineStr">
@@ -8856,11 +8879,7 @@
           <t>Remaining</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
-        <is>
-          <t>52 pages: every unique page plus 3 of each templated set, production build): no page pans sideways, no failed requests, no JS errors. Found and fixed on the way: upgrade-insecure-requests in the new CSP made Safari fetch every stylesheet and font over https on localhost (dropped; the site is HTTPS-only via HSTS anyway), and .toLocaleString() without a locale caused a hydration error on /brewsoul/chains in Safari (all number formatting now en-US). Left: a check on a real iPhone (Phase 14).</t>
-        </is>
-      </c>
+      <c r="D25" s="4" t="inlineStr"/>
       <c r="E25" s="14" t="inlineStr">
         <is>
           <t>Phase 14 — QA &amp; Launch</t>
@@ -8871,7 +8890,7 @@
       <c r="A26" s="4" t="n"/>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Remove noindex only when sign-off is given</t>
+          <t>DNS cutover, legacy app decommissioned only after a stable overlap window</t>
         </is>
       </c>
       <c r="C26" s="15" t="inlineStr">
@@ -8879,64 +8898,22 @@
           <t>Remaining</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
-          <t>do not launch indexable by accident (The only noindex is the host-based one for *.netlify.app above, so the real domain is indexable as soon as DNS points at it: sign-off must come before DNS.)</t>
-        </is>
-      </c>
+      <c r="D26" s="4" t="inlineStr"/>
       <c r="E26" s="14" t="inlineStr">
         <is>
           <t>Phase 14 — QA &amp; Launch</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="4" t="n"/>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>Final stakeholder sign-off (Tony/Darryl/Kimberly) on the ported site before DNS cutover</t>
-        </is>
-      </c>
-      <c r="C27" s="15" t="inlineStr">
-        <is>
-          <t>Remaining</t>
-        </is>
-      </c>
-      <c r="D27" s="4" t="inlineStr"/>
-      <c r="E27" s="14" t="inlineStr">
-        <is>
-          <t>Phase 14 — QA &amp; Launch</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="4" t="n"/>
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>DNS cutover, legacy app decommissioned only after a stable overlap window</t>
-        </is>
-      </c>
-      <c r="C28" s="15" t="inlineStr">
-        <is>
-          <t>Remaining</t>
-        </is>
-      </c>
-      <c r="D28" s="4" t="inlineStr"/>
-      <c r="E28" s="14" t="inlineStr">
-        <is>
-          <t>Phase 14 — QA &amp; Launch</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:D28"/>
+  <autoFilter ref="A1:D26"/>
   <mergeCells count="6">
     <mergeCell ref="A5:D5"/>
-    <mergeCell ref="A18:D18"/>
-    <mergeCell ref="A22:D22"/>
     <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A20:D20"/>
     <mergeCell ref="A7:D7"/>
     <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A16:D16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Owner answers round 2: real counts, Mirror Manus links, dead links
- Real counts (owner: "show the real counts"): /charity-scorecard intro and
  meta description use STATS.totalCharities (103, was "98"/"Ninety-eight");
  /impact-dashboard and /the-index explorers get the count as a prop (no
  charity list in the browser bundle); search directory coffees 103 -> 107.
- The Mirror: 4 *.manus.space partner apps removed from "Explore further"
  (owner: drop all 4; the section hides when empty).
- /framework: "Ask FauxTony" button and lead-in removed (chatbot cancelled).
- Essay links to /blog/the-case-file-dr-samuel-lee (never published) render
  as plain text via DEAD_INTERNAL_LINKS in portable-text.tsx; no Sanity
  draft needed.
- B Corp notes: checked live; neither site displays them. No change.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Migration-Status-Report.xlsx
+++ b/Migration-Status-Report.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Remaining Work" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Full Detail'!$A$1:$D$328</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Full Detail'!$A$1:$D$329</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Remaining Work'!$A$1:$D$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -639,15 +639,15 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A5,'Full Detail'!$C$2:$C$328,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$329,$A5,'Full Detail'!$C$2:$C$329,"Done")</f>
         <v/>
       </c>
       <c r="C5" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A5,'Full Detail'!$C$2:$C$328,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$329,$A5,'Full Detail'!$C$2:$C$329,"Remaining")</f>
         <v/>
       </c>
       <c r="D5" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A5,'Full Detail'!$C$2:$C$328,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$329,$A5,'Full Detail'!$C$2:$C$329,"Deferred")</f>
         <v/>
       </c>
       <c r="E5" s="5">
@@ -666,15 +666,15 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A6,'Full Detail'!$C$2:$C$328,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$329,$A6,'Full Detail'!$C$2:$C$329,"Done")</f>
         <v/>
       </c>
       <c r="C6" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A6,'Full Detail'!$C$2:$C$328,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$329,$A6,'Full Detail'!$C$2:$C$329,"Remaining")</f>
         <v/>
       </c>
       <c r="D6" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A6,'Full Detail'!$C$2:$C$328,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$329,$A6,'Full Detail'!$C$2:$C$329,"Deferred")</f>
         <v/>
       </c>
       <c r="E6" s="5">
@@ -693,15 +693,15 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A7,'Full Detail'!$C$2:$C$328,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$329,$A7,'Full Detail'!$C$2:$C$329,"Done")</f>
         <v/>
       </c>
       <c r="C7" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A7,'Full Detail'!$C$2:$C$328,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$329,$A7,'Full Detail'!$C$2:$C$329,"Remaining")</f>
         <v/>
       </c>
       <c r="D7" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A7,'Full Detail'!$C$2:$C$328,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$329,$A7,'Full Detail'!$C$2:$C$329,"Deferred")</f>
         <v/>
       </c>
       <c r="E7" s="5">
@@ -720,15 +720,15 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A8,'Full Detail'!$C$2:$C$328,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$329,$A8,'Full Detail'!$C$2:$C$329,"Done")</f>
         <v/>
       </c>
       <c r="C8" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A8,'Full Detail'!$C$2:$C$328,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$329,$A8,'Full Detail'!$C$2:$C$329,"Remaining")</f>
         <v/>
       </c>
       <c r="D8" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A8,'Full Detail'!$C$2:$C$328,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$329,$A8,'Full Detail'!$C$2:$C$329,"Deferred")</f>
         <v/>
       </c>
       <c r="E8" s="5">
@@ -747,15 +747,15 @@
         </is>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A9,'Full Detail'!$C$2:$C$328,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$329,$A9,'Full Detail'!$C$2:$C$329,"Done")</f>
         <v/>
       </c>
       <c r="C9" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A9,'Full Detail'!$C$2:$C$328,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$329,$A9,'Full Detail'!$C$2:$C$329,"Remaining")</f>
         <v/>
       </c>
       <c r="D9" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A9,'Full Detail'!$C$2:$C$328,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$329,$A9,'Full Detail'!$C$2:$C$329,"Deferred")</f>
         <v/>
       </c>
       <c r="E9" s="5">
@@ -774,15 +774,15 @@
         </is>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A10,'Full Detail'!$C$2:$C$328,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$329,$A10,'Full Detail'!$C$2:$C$329,"Done")</f>
         <v/>
       </c>
       <c r="C10" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A10,'Full Detail'!$C$2:$C$328,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$329,$A10,'Full Detail'!$C$2:$C$329,"Remaining")</f>
         <v/>
       </c>
       <c r="D10" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A10,'Full Detail'!$C$2:$C$328,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$329,$A10,'Full Detail'!$C$2:$C$329,"Deferred")</f>
         <v/>
       </c>
       <c r="E10" s="5">
@@ -801,15 +801,15 @@
         </is>
       </c>
       <c r="B11" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A11,'Full Detail'!$C$2:$C$328,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$329,$A11,'Full Detail'!$C$2:$C$329,"Done")</f>
         <v/>
       </c>
       <c r="C11" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A11,'Full Detail'!$C$2:$C$328,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$329,$A11,'Full Detail'!$C$2:$C$329,"Remaining")</f>
         <v/>
       </c>
       <c r="D11" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A11,'Full Detail'!$C$2:$C$328,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$329,$A11,'Full Detail'!$C$2:$C$329,"Deferred")</f>
         <v/>
       </c>
       <c r="E11" s="5">
@@ -828,15 +828,15 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A12,'Full Detail'!$C$2:$C$328,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$329,$A12,'Full Detail'!$C$2:$C$329,"Done")</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A12,'Full Detail'!$C$2:$C$328,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$329,$A12,'Full Detail'!$C$2:$C$329,"Remaining")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A12,'Full Detail'!$C$2:$C$328,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$329,$A12,'Full Detail'!$C$2:$C$329,"Deferred")</f>
         <v/>
       </c>
       <c r="E12" s="5">
@@ -855,15 +855,15 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A13,'Full Detail'!$C$2:$C$328,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$329,$A13,'Full Detail'!$C$2:$C$329,"Done")</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A13,'Full Detail'!$C$2:$C$328,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$329,$A13,'Full Detail'!$C$2:$C$329,"Remaining")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A13,'Full Detail'!$C$2:$C$328,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$329,$A13,'Full Detail'!$C$2:$C$329,"Deferred")</f>
         <v/>
       </c>
       <c r="E13" s="5">
@@ -882,15 +882,15 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A14,'Full Detail'!$C$2:$C$328,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$329,$A14,'Full Detail'!$C$2:$C$329,"Done")</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A14,'Full Detail'!$C$2:$C$328,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$329,$A14,'Full Detail'!$C$2:$C$329,"Remaining")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A14,'Full Detail'!$C$2:$C$328,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$329,$A14,'Full Detail'!$C$2:$C$329,"Deferred")</f>
         <v/>
       </c>
       <c r="E14" s="5">
@@ -909,15 +909,15 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A15,'Full Detail'!$C$2:$C$328,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$329,$A15,'Full Detail'!$C$2:$C$329,"Done")</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A15,'Full Detail'!$C$2:$C$328,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$329,$A15,'Full Detail'!$C$2:$C$329,"Remaining")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A15,'Full Detail'!$C$2:$C$328,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$329,$A15,'Full Detail'!$C$2:$C$329,"Deferred")</f>
         <v/>
       </c>
       <c r="E15" s="5">
@@ -936,15 +936,15 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A16,'Full Detail'!$C$2:$C$328,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$329,$A16,'Full Detail'!$C$2:$C$329,"Done")</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A16,'Full Detail'!$C$2:$C$328,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$329,$A16,'Full Detail'!$C$2:$C$329,"Remaining")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A16,'Full Detail'!$C$2:$C$328,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$329,$A16,'Full Detail'!$C$2:$C$329,"Deferred")</f>
         <v/>
       </c>
       <c r="E16" s="5">
@@ -963,15 +963,15 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A17,'Full Detail'!$C$2:$C$328,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$329,$A17,'Full Detail'!$C$2:$C$329,"Done")</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A17,'Full Detail'!$C$2:$C$328,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$329,$A17,'Full Detail'!$C$2:$C$329,"Remaining")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A17,'Full Detail'!$C$2:$C$328,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$329,$A17,'Full Detail'!$C$2:$C$329,"Deferred")</f>
         <v/>
       </c>
       <c r="E17" s="5">
@@ -990,15 +990,15 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A18,'Full Detail'!$C$2:$C$328,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$329,$A18,'Full Detail'!$C$2:$C$329,"Done")</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A18,'Full Detail'!$C$2:$C$328,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$329,$A18,'Full Detail'!$C$2:$C$329,"Remaining")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A18,'Full Detail'!$C$2:$C$328,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$329,$A18,'Full Detail'!$C$2:$C$329,"Deferred")</f>
         <v/>
       </c>
       <c r="E18" s="5">
@@ -1017,15 +1017,15 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A19,'Full Detail'!$C$2:$C$328,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$329,$A19,'Full Detail'!$C$2:$C$329,"Done")</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A19,'Full Detail'!$C$2:$C$328,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$329,$A19,'Full Detail'!$C$2:$C$329,"Remaining")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$328,$A19,'Full Detail'!$C$2:$C$328,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$329,$A19,'Full Detail'!$C$2:$C$329,"Deferred")</f>
         <v/>
       </c>
       <c r="E19" s="5">
@@ -1075,7 +1075,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E328"/>
+  <dimension ref="A1:E329"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -7366,7 +7366,7 @@
       <c r="A284" s="4" t="n"/>
       <c r="B284" s="4" t="inlineStr">
         <is>
-          <t>Arrows in buttons and links are icons (2026-10-09, owner said yes)</t>
+          <t>Owner answers, round 2 (2026-10-09)</t>
         </is>
       </c>
       <c r="C284" s="13" t="inlineStr">
@@ -7376,7 +7376,7 @@
       </c>
       <c r="D284" s="4" t="inlineStr">
         <is>
-          <t>113 typed arrows in 52 files (button and link labels, "Next"/"See My Results" toggles, decorative arrow spans, the walk-through "See the..." labels, the Letter's "I'm in" button) replaced with lucide ArrowRight/ArrowLeft (size-[1em], inside inline-flex items-center gap-1.5, so the parent layout is untouched). Left as content on purpose: arrows inside Tony's text and data (health findings, origins, iboga compass options, process flows like "Inherit → Wake → Choose → Act", share text), the "← you" marker on the consciousness scale, and &lt;option&gt; sort labels (an option can't hold an icon). Checked on 16 pages at 375 and 1280: no typed arrow left in any link or button, no sideways scroll, no JS errors; close-up screenshots of the new icons.</t>
+          <t>(1) real counts instead of live's typed numbers: /charity-scorecard intro and description ("98"/"Ninety-eight" → STATS.totalCharities = 103), /impact-dashboard ("100" → passed in from the page so the browser doesn't load the charity list), /the-index (prop), search directory coffees 103 → 107 (typed, with a note, since it ships to the search pop-up); (2) The Mirror results no longer list the 4 *.manus.space apps (the "Explore further" section hides when empty); (3) /framework's "Ask FauxTony" button and its lead-in line removed; the Dr. Lee case-file link (4 places in when-healing-becomes-extraction, original and updated versions) renders as plain text through a DEAD_INTERNAL_LINKS list in lib/sanity/portable-text.tsx (no Sanity draft needed); (4) B Corp: checked live, nothing shown on either site, no change. Verified on a production build: the counts read 103, /framework has no FauxTony block, the essay has 0 links to the case file and keeps the words, /the-index shows "103 charities" when searching "charity".</t>
         </is>
       </c>
       <c r="E284" s="14" t="inlineStr">
@@ -7389,7 +7389,7 @@
       <c r="A285" s="4" t="n"/>
       <c r="B285" s="4" t="inlineStr">
         <is>
-          <t>Category pages pre-built (2026-10-09)</t>
+          <t>Arrows in buttons and links are icons (2026-10-09, owner said yes)</t>
         </is>
       </c>
       <c r="C285" s="13" t="inlineStr">
@@ -7399,7 +7399,7 @@
       </c>
       <c r="D285" s="4" t="inlineStr">
         <is>
-          <t>/blog/category/[slug] read ?page=N, so every category page was rendered on each request (slower first byte, flagged in the Lighthouse notes). Page numbers are now part of the address (/blog/category/&lt;slug&gt;/page/&lt;n&gt;, generateStaticParams, dynamicParams = false), shared code in src/components/blog/category-listing.tsx; old ?page=N links 308 to the new address (pages 2+ only, so no loop), /page/1 308s to the plain address, a page past the end is a 404; "All essays" back link uses an icon. Verified on a production build: route table shows every category page as pre-built (9 page-1s, 7 later pages), titles and canonicals per page, Previous/Next links, the redirects and the 404s.</t>
+          <t>113 typed arrows in 52 files (button and link labels, "Next"/"See My Results" toggles, decorative arrow spans, the walk-through "See the..." labels, the Letter's "I'm in" button) replaced with lucide ArrowRight/ArrowLeft (size-[1em], inside inline-flex items-center gap-1.5, so the parent layout is untouched). Left as content on purpose: arrows inside Tony's text and data (health findings, origins, iboga compass options, process flows like "Inherit → Wake → Choose → Act", share text), the "← you" marker on the consciousness scale, and &lt;option&gt; sort labels (an option can't hold an icon). Checked on 16 pages at 375 and 1280: no typed arrow left in any link or button, no sideways scroll, no JS errors; close-up screenshots of the new icons.</t>
         </is>
       </c>
       <c r="E285" s="14" t="inlineStr">
@@ -7412,7 +7412,7 @@
       <c r="A286" s="4" t="n"/>
       <c r="B286" s="4" t="inlineStr">
         <is>
-          <t>Error pages (2026-10-09, owner asked)</t>
+          <t>Category pages pre-built (2026-10-09)</t>
         </is>
       </c>
       <c r="C286" s="13" t="inlineStr">
@@ -7422,7 +7422,7 @@
       </c>
       <c r="D286" s="4" t="inlineStr">
         <is>
-          <t>404 page now sets its own title ("Page not found") as a server page around live's 3-second redirect (not-found.tsx + components/not-found-redirect.tsx), arrow as an icon; page error screen (error.tsx) uses Next 16's retry (re-fetches), shows a reference code for the server logs, links home and to the site index; new global-error.tsx for failures in the root layout itself (own &lt;html&gt;, plain links). Verified on a production build: missing page, missing essay and missing Kava page return 404 with the right title; a test page that throws returns 500 with the error screen, "Try again" re-fetches; phone and laptop, no sideways scroll (test page removed).</t>
+          <t>/blog/category/[slug] read ?page=N, so every category page was rendered on each request (slower first byte, flagged in the Lighthouse notes). Page numbers are now part of the address (/blog/category/&lt;slug&gt;/page/&lt;n&gt;, generateStaticParams, dynamicParams = false), shared code in src/components/blog/category-listing.tsx; old ?page=N links 308 to the new address (pages 2+ only, so no loop), /page/1 308s to the plain address, a page past the end is a 404; "All essays" back link uses an icon. Verified on a production build: route table shows every category page as pre-built (9 page-1s, 7 later pages), titles and canonicals per page, Previous/Next links, the redirects and the 404s.</t>
         </is>
       </c>
       <c r="E286" s="14" t="inlineStr">
@@ -7435,7 +7435,7 @@
       <c r="A287" s="4" t="n"/>
       <c r="B287" s="4" t="inlineStr">
         <is>
-          <t>SEO audit fixes (2026-10-06)</t>
+          <t>Error pages (2026-10-09, owner asked)</t>
         </is>
       </c>
       <c r="C287" s="13" t="inlineStr">
@@ -7445,7 +7445,7 @@
       </c>
       <c r="D287" s="4" t="inlineStr">
         <is>
-          <t>Checked an outside audit point by point against the code. Fixed: Core Themes cards linked to /?theme=…#essays-archive (not crawlable, counts from a stale hand-kept list) and now link to /blog/category/&lt;slug&gt; with real counts (21/25/20/14, matching the archive pills; THEME_MAP and the ?theme= filter removed); Four Doors cards were &lt;button&gt;s, now real links that still open the modal on a plain click; "DIAGNOSE · ENGAGE" now link to /find-my and /engage; one shared formatPostDate (Asia/Kolkata, src/lib/format-post-date.ts) so a post no longer shows two different dates; the title repeated as the first body paragraph is dropped at render time (legacyBodyLayout); essay cards are h3 under a section h2 (archive, Read next), h2 only on category/search; heading glyphs (◆ ✦) hidden from screen readers; posts send BlogPosting with the author tied to the site Person (@id) plus a BreadcrumbList; descriptive alt on the homepage and BrewSoul heroes; homepage OG image cropped to 1200x630 JPEG. Already fine (audit could not see it): Person/Article schema, Netlify noindex, robots.txt, sitemap, header nav and search, Amazon links carry no affiliate tag. Checked on a production build: type check, lint, build, status codes, browser click test at 375px, no console errors. Implementation pack (Mohammad Danish, 2026-10-05) checked the same day: added og:type/og:site_name back on the 6 pages with their own openGraph (a page-level openGraph replaces the layout one), twitter:creator, and on posts og:url</t>
+          <t>404 page now sets its own title ("Page not found") as a server page around live's 3-second redirect (not-found.tsx + components/not-found-redirect.tsx), arrow as an icon; page error screen (error.tsx) uses Next 16's retry (re-fetches), shows a reference code for the server logs, links home and to the site index; new global-error.tsx for failures in the root layout itself (own &lt;html&gt;, plain links). Verified on a production build: missing page, missing essay and missing Kava page return 404 with the right title; a test page that throws returns 500 with the error screen, "Try again" re-fetches; phone and laptop, no sideways scroll (test page removed).</t>
         </is>
       </c>
       <c r="E287" s="14" t="inlineStr">
@@ -7458,17 +7458,17 @@
       <c r="A288" s="4" t="n"/>
       <c r="B288" s="4" t="inlineStr">
         <is>
-          <t>SEO audit items needing a yes (2026-10-06)</t>
-        </is>
-      </c>
-      <c r="C288" s="15" t="inlineStr">
-        <is>
-          <t>Remaining</t>
+          <t>SEO audit fixes (2026-10-06)</t>
+        </is>
+      </c>
+      <c r="C288" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D288" s="4" t="inlineStr">
         <is>
-          <t>the pack's new copy (homepage title/description, five-cups title, description, short answer, FAQ, heading rewrites, entity statement, newsletter block, author box, health disclaimer, COA wording); "Further Reading" shown twice on posts (merge the lists?); long post title (84 chars), homepage description length and obsolete keywords tag, slugs (/blog/five-cups, the -2 slug; would need redirects), "Six lenses" over four cards, sources for health claims and proof for "$10B+", "Certified B Corp", "Validity: 91", legal review of the homepage Case File banner, ABIT waitlist disclosures, one contact email, the two one-post categories, fewer homepage CTAs / email signup / table of contents / explaining "COA".</t>
+          <t>Checked an outside audit point by point against the code. Fixed: Core Themes cards linked to /?theme=…#essays-archive (not crawlable, counts from a stale hand-kept list) and now link to /blog/category/&lt;slug&gt; with real counts (21/25/20/14, matching the archive pills; THEME_MAP and the ?theme= filter removed); Four Doors cards were &lt;button&gt;s, now real links that still open the modal on a plain click; "DIAGNOSE · ENGAGE" now link to /find-my and /engage; one shared formatPostDate (Asia/Kolkata, src/lib/format-post-date.ts) so a post no longer shows two different dates; the title repeated as the first body paragraph is dropped at render time (legacyBodyLayout); essay cards are h3 under a section h2 (archive, Read next), h2 only on category/search; heading glyphs (◆ ✦) hidden from screen readers; posts send BlogPosting with the author tied to the site Person (@id) plus a BreadcrumbList; descriptive alt on the homepage and BrewSoul heroes; homepage OG image cropped to 1200x630 JPEG. Already fine (audit could not see it): Person/Article schema, Netlify noindex, robots.txt, sitemap, header nav and search, Amazon links carry no affiliate tag. Checked on a production build: type check, lint, build, status codes, browser click test at 375px, no console errors. Implementation pack (Mohammad Danish, 2026-10-05) checked the same day: added og:type/og:site_name back on the 6 pages with their own openGraph (a page-level openGraph replaces the layout one), twitter:creator, and on posts og:url</t>
         </is>
       </c>
       <c r="E288" s="14" t="inlineStr">
@@ -7481,7 +7481,7 @@
       <c r="A289" s="4" t="n"/>
       <c r="B289" s="4" t="inlineStr">
         <is>
-          <t>Connect Google Search Console + GA4 to the new deployment on day one of cutover</t>
+          <t>SEO audit items needing a yes (2026-10-06)</t>
         </is>
       </c>
       <c r="C289" s="15" t="inlineStr">
@@ -7489,7 +7489,11 @@
           <t>Remaining</t>
         </is>
       </c>
-      <c r="D289" s="4" t="inlineStr"/>
+      <c r="D289" s="4" t="inlineStr">
+        <is>
+          <t>the pack's new copy (homepage title/description, five-cups title, description, short answer, FAQ, heading rewrites, entity statement, newsletter block, author box, health disclaimer, COA wording); "Further Reading" shown twice on posts (merge the lists?); long post title (84 chars), homepage description length and obsolete keywords tag, slugs (/blog/five-cups, the -2 slug; would need redirects), "Six lenses" over four cards, sources for health claims and proof for "$10B+", "Certified B Corp", "Validity: 91", legal review of the homepage Case File banner, ABIT waitlist disclosures, one contact email, the two one-post categories, fewer homepage CTAs / email signup / table of contents / explaining "COA".</t>
+        </is>
+      </c>
       <c r="E289" s="14" t="inlineStr">
         <is>
           <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
@@ -7500,19 +7504,15 @@
       <c r="A290" s="4" t="n"/>
       <c r="B290" s="4" t="inlineStr">
         <is>
-          <t>Restore/adapt the manus.space triple-layer noindex lockdown pattern for any remaining staging URLs</t>
-        </is>
-      </c>
-      <c r="C290" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D290" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-01: the Netlify copy (tonygreenberg-website.netlify.app) and every deploy preview had no noindex at all, so Google could index a duplicate of the site. next.config.ts headers() now sends X-Robots-Tag: noindex, nofollow on any *.netlify.app host only; tonygreenberg.com is unaffected, so nothing to remove at cutover. Tested with Host headers on a production build.</t>
-        </is>
-      </c>
+          <t>Connect Google Search Console + GA4 to the new deployment on day one of cutover</t>
+        </is>
+      </c>
+      <c r="C290" s="15" t="inlineStr">
+        <is>
+          <t>Remaining</t>
+        </is>
+      </c>
+      <c r="D290" s="4" t="inlineStr"/>
       <c r="E290" s="14" t="inlineStr">
         <is>
           <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
@@ -7523,7 +7523,7 @@
       <c r="A291" s="4" t="n"/>
       <c r="B291" s="4" t="inlineStr">
         <is>
-          <t>"Keep going" strip above the footer on every page (2026-10-07)</t>
+          <t>Restore/adapt the manus.space triple-layer noindex lockdown pattern for any remaining staging URLs</t>
         </is>
       </c>
       <c r="C291" s="13" t="inlineStr">
@@ -7533,7 +7533,7 @@
       </c>
       <c r="D291" s="4" t="inlineStr">
         <is>
-          <t>legacy's WhereNext (deferred in Phase 3, never picked up) with its per-page suggestions, Home · Site Index · All Assessments; links pointed at current routes.</t>
+          <t>2026-10-01: the Netlify copy (tonygreenberg-website.netlify.app) and every deploy preview had no noindex at all, so Google could index a duplicate of the site. next.config.ts headers() now sends X-Robots-Tag: noindex, nofollow on any *.netlify.app host only; tonygreenberg.com is unaffected, so nothing to remove at cutover. Tested with Host headers on a production build.</t>
         </is>
       </c>
       <c r="E291" s="14" t="inlineStr">
@@ -7546,7 +7546,7 @@
       <c r="A292" s="4" t="n"/>
       <c r="B292" s="4" t="inlineStr">
         <is>
-          <t>Live-only and redesigned pages from the 2026-10-07 page sweep (188 pages compared with live)</t>
+          <t>"Keep going" strip above the footer on every page (2026-10-07)</t>
         </is>
       </c>
       <c r="C292" s="13" t="inlineStr">
@@ -7556,7 +7556,7 @@
       </c>
       <c r="D292" s="4" t="inlineStr">
         <is>
-          <t>/the-index rebuilt from live's code (20 concepts, related-word search across essays and site pages, full-text search on the server, "three related places to go next"; the old redirect to /search removed and its links, including the "Site Index" link in "Keep going", point at it again); /the-mirror (and /life-assessment) opens on live's intro (dark hero, "What We Measure" with the six areas, "The Ecosystem"), rebuilt as a step registry (rule 19); /essays header, order and column like live; /about "What They Say" styled like live (live picks 3 of the same 19 quotes at random; ours shows a fixed 3 so they're in the server HTML); /impact-futurism list titles and subtitles; /supplier-intake is a real page again with live's Stage 1 form; /seven-doors and /projects redirect home like live; /impact, /health, /library, /built-on-manus, /heroes are 404 on live too. Left as is on purpose: /blog stays our archive page (on live it repeats the homepage), the email gates on /framework and /peptide-supply-chain, the attention-theft Wall of Shame.</t>
+          <t>legacy's WhereNext (deferred in Phase 3, never picked up) with its per-page suggestions, Home · Site Index · All Assessments; links pointed at current routes.</t>
         </is>
       </c>
       <c r="E292" s="14" t="inlineStr">
@@ -7569,7 +7569,7 @@
       <c r="A293" s="4" t="n"/>
       <c r="B293" s="4" t="inlineStr">
         <is>
-          <t>/alex-azzi locked like live (2026-10-07, owner said match it)</t>
+          <t>Live-only and redesigned pages from the 2026-10-07 page sweep (188 pages compared with live)</t>
         </is>
       </c>
       <c r="C293" s="13" t="inlineStr">
@@ -7579,7 +7579,7 @@
       </c>
       <c r="D293" s="4" t="inlineStr">
         <is>
-          <t>same server-checked password as the locked essay (GATED_POST_PASSWORD, now also set in Netlify), live's "Restricted Access" screen, the report not in the page until unlocked, out of search and the sitemap.</t>
+          <t>/the-index rebuilt from live's code (20 concepts, related-word search across essays and site pages, full-text search on the server, "three related places to go next"; the old redirect to /search removed and its links, including the "Site Index" link in "Keep going", point at it again); /the-mirror (and /life-assessment) opens on live's intro (dark hero, "What We Measure" with the six areas, "The Ecosystem"), rebuilt as a step registry (rule 19); /essays header, order and column like live; /about "What They Say" styled like live (live picks 3 of the same 19 quotes at random; ours shows a fixed 3 so they're in the server HTML); /impact-futurism list titles and subtitles; /supplier-intake is a real page again with live's Stage 1 form; /seven-doors and /projects redirect home like live; /impact, /health, /library, /built-on-manus, /heroes are 404 on live too. Left as is on purpose: /blog stays our archive page (on live it repeats the homepage), the email gates on /framework and /peptide-supply-chain, the attention-theft Wall of Shame.</t>
         </is>
       </c>
       <c r="E293" s="14" t="inlineStr">
@@ -7592,7 +7592,7 @@
       <c r="A294" s="4" t="n"/>
       <c r="B294" s="4" t="inlineStr">
         <is>
-          <t>Live's title fonts and sizes (2026-10-07, "fix the style")</t>
+          <t>/alex-azzi locked like live (2026-10-07, owner said match it)</t>
         </is>
       </c>
       <c r="C294" s="13" t="inlineStr">
@@ -7602,7 +7602,7 @@
       </c>
       <c r="D294" s="4" t="inlineStr">
         <is>
-          <t>measured every page's title font, weight, size and label colour on live vs ours (136 pages). Now like live: Kava headings in Fraunces, HumanOS in Space Grotesk, the peptide tools / charity scorecard / thesis threads in the system serif, America Unbundled in the Iowan Old Style stack at live's size, /akbar in Fraunces 900, friend-gate and post-intervention in Georgia, and live's title sizes on peptide-matrix, peptide-supply-chain, rip-peptide-sciences and the HumanOS pages. Fonts load only on the pages that use them (src/lib/fonts/page-fonts.ts). Label colours stay the darker AA-contrast versions where live's lighter ones fail on a light background.</t>
+          <t>same server-checked password as the locked essay (GATED_POST_PASSWORD, now also set in Netlify), live's "Restricted Access" screen, the report not in the page until unlocked, out of search and the sitemap.</t>
         </is>
       </c>
       <c r="E294" s="14" t="inlineStr">
@@ -7615,7 +7615,7 @@
       <c r="A295" s="4" t="n"/>
       <c r="B295" s="4" t="inlineStr">
         <is>
-          <t>Peptide page images rescued into Sanity and wired (2026-10-07)</t>
+          <t>Live's title fonts and sizes (2026-10-07, "fix the style")</t>
         </is>
       </c>
       <c r="C295" s="13" t="inlineStr">
@@ -7625,7 +7625,7 @@
       </c>
       <c r="D295" s="4" t="inlineStr">
         <is>
-          <t>/peptide-watch hero plus its 11 section banners, /peptide-matrix and /peptide-supply-chain heroes, the /peptide-hall-of-shame hero (scripts/rescue-2026-10-07-peptide-images.ts, logged in docs/ai/manus-media-rescue.md).</t>
+          <t>measured every page's title font, weight, size and label colour on live vs ours (136 pages). Now like live: Kava headings in Fraunces, HumanOS in Space Grotesk, the peptide tools / charity scorecard / thesis threads in the system serif, America Unbundled in the Iowan Old Style stack at live's size, /akbar in Fraunces 900, friend-gate and post-intervention in Georgia, and live's title sizes on peptide-matrix, peptide-supply-chain, rip-peptide-sciences and the HumanOS pages. Fonts load only on the pages that use them (src/lib/fonts/page-fonts.ts). Label colours stay the darker AA-contrast versions where live's lighter ones fail on a light background.</t>
         </is>
       </c>
       <c r="E295" s="14" t="inlineStr">
@@ -7638,7 +7638,7 @@
       <c r="A296" s="4" t="n"/>
       <c r="B296" s="4" t="inlineStr">
         <is>
-          <t>Live's editorial redesign, first group (2026-10-07)</t>
+          <t>Peptide page images rescued into Sanity and wired (2026-10-07)</t>
         </is>
       </c>
       <c r="C296" s="13" t="inlineStr">
@@ -7648,7 +7648,7 @@
       </c>
       <c r="D296" s="4" t="inlineStr">
         <is>
-          <t>dark top sections, narrow single text column, short red section rules and dark call-to-action bands on /invest, /amplifier, /community (now "Sign In to Join the Community", linking our real sign-in; live's made-up counters left out), /framework, /the-letter (daily provocation with "Share this thought" and "Search past provocations"), /engage, /diamond-cut, /ecosystem and the homepage's "The thinking doesn't stop here" band. Kept on purpose: AA-contrast colours where live's fail, "Enter the Gate" instead of live's $5,000 checkout on /diamond-cut.</t>
+          <t>/peptide-watch hero plus its 11 section banners, /peptide-matrix and /peptide-supply-chain heroes, the /peptide-hall-of-shame hero (scripts/rescue-2026-10-07-peptide-images.ts, logged in docs/ai/manus-media-rescue.md).</t>
         </is>
       </c>
       <c r="E296" s="14" t="inlineStr">
@@ -7661,7 +7661,7 @@
       <c r="A297" s="4" t="n"/>
       <c r="B297" s="4" t="inlineStr">
         <is>
-          <t>Live's redesign, second group (done 2026-10-08)</t>
+          <t>Live's editorial redesign, first group (2026-10-07)</t>
         </is>
       </c>
       <c r="C297" s="13" t="inlineStr">
@@ -7671,7 +7671,7 @@
       </c>
       <c r="D297" s="4" t="inlineStr">
         <is>
-          <t>re-measured all 18 pages on live vs a fresh production build (title font/size/weight/colour, labels, hero images). Already matching from 2026-10-07: /the-web, /spirits, /iboga-ibogaine (weight 800), /living-declaration, BrewSoul photo on /brewsoul, /brewsoul/browse, /brewsoul/first-sip (live has none there either), /quiz_25q, /recent-creations. Fixed today: /find-your-journey (64px title, red label), /impact-dashboard (64px title in essay ink, label spacing), red labels on /published and /speaking (plus its "rooms" chips), /soulscore "by ImpactSoul" label, /pri-calibration title (weight 900, solid cream, was a purple gradient), /clients (live's narrow 546px column for the whole page, 56px title, roomier stats band, cards 2 per row; two static inline styles moved to classes), /brewsoul/guest (live's BrewSoul photo on the guest card instead of "SN" initials, labels in capitals), /humanos/connect (cards line up with the title), /peptide-hall-of-shame (stats and label readable light gold; were dark gold on dark). Typed arrows on the touched links are icons now (rule 18). Deliberately not copied from live (new CONTRIBUTING rule 20, owner 2026-10-08): red labels on dark bands use #E07A80 (live's #8E1E25 on black is about 2:1, unreadable); /recent-creations keeps our darker label colours (live's fail contrast on white); /humanos/connect keeps "Start Reading" (that card links to the philosophy page, the quiz live's "Start the Assessment" implies doesn't exist). Checked: type check, l</t>
+          <t>dark top sections, narrow single text column, short red section rules and dark call-to-action bands on /invest, /amplifier, /community (now "Sign In to Join the Community", linking our real sign-in; live's made-up counters left out), /framework, /the-letter (daily provocation with "Share this thought" and "Search past provocations"), /engage, /diamond-cut, /ecosystem and the homepage's "The thinking doesn't stop here" band. Kept on purpose: AA-contrast colours where live's fail, "Enter the Gate" instead of live's $5,000 checkout on /diamond-cut.</t>
         </is>
       </c>
       <c r="E297" s="14" t="inlineStr">
@@ -7684,7 +7684,7 @@
       <c r="A298" s="4" t="n"/>
       <c r="B298" s="4" t="inlineStr">
         <is>
-          <t>BrewSoul top of page (2026-10-08, owner: "button in the center at the top doesn't look good")</t>
+          <t>Live's redesign, second group (done 2026-10-08)</t>
         </is>
       </c>
       <c r="C298" s="13" t="inlineStr">
@@ -7694,7 +7694,7 @@
       </c>
       <c r="D298" s="4" t="inlineStr">
         <is>
-          <t>the category badge ("Deep Research" etc.) sat centred in an empty strip, squeezed against the hero, because we copied live's doubled 52px top gap. Now one gap everywhere and the badge floats in the top-left corner, lined up with the BrewSoul logo (brewsoul-main.tsx, category-badge.tsx); checked on all 26 badge pages at 3 widths that it covers nothing. BrewSoul menu: on tablets (768-1023px) the links were cut off and "More" was hidden with no menu button at all; now the menu button shows below 1024px, 5 links + "More" from 1024px, all 8 from 1280px, "More" always visible.</t>
+          <t>re-measured all 18 pages on live vs a fresh production build (title font/size/weight/colour, labels, hero images). Already matching from 2026-10-07: /the-web, /spirits, /iboga-ibogaine (weight 800), /living-declaration, BrewSoul photo on /brewsoul, /brewsoul/browse, /brewsoul/first-sip (live has none there either), /quiz_25q, /recent-creations. Fixed today: /find-your-journey (64px title, red label), /impact-dashboard (64px title in essay ink, label spacing), red labels on /published and /speaking (plus its "rooms" chips), /soulscore "by ImpactSoul" label, /pri-calibration title (weight 900, solid cream, was a purple gradient), /clients (live's narrow 546px column for the whole page, 56px title, roomier stats band, cards 2 per row; two static inline styles moved to classes), /brewsoul/guest (live's BrewSoul photo on the guest card instead of "SN" initials, labels in capitals), /humanos/connect (cards line up with the title), /peptide-hall-of-shame (stats and label readable light gold; were dark gold on dark). Typed arrows on the touched links are icons now (rule 18). Deliberately not copied from live (new CONTRIBUTING rule 20, owner 2026-10-08): red labels on dark bands use #E07A80 (live's #8E1E25 on black is about 2:1, unreadable); /recent-creations keeps our darker label colours (live's fail contrast on white); /humanos/connect keeps "Start Reading" (that card links to the philosophy page, the quiz live's "Start the Assessment" implies doesn't exist). Checked: type check, l</t>
         </is>
       </c>
       <c r="E298" s="14" t="inlineStr">
@@ -7707,7 +7707,7 @@
       <c r="A299" s="4" t="n"/>
       <c r="B299" s="4" t="inlineStr">
         <is>
-          <t>/pri-efficacy's "Simulation / Live Calibrations" switch like live (2026-10-08)</t>
+          <t>BrewSoul top of page (2026-10-08, owner: "button in the center at the top doesn't look good")</t>
         </is>
       </c>
       <c r="C299" s="13" t="inlineStr">
@@ -7717,7 +7717,7 @@
       </c>
       <c r="D299" s="4" t="inlineStr">
         <is>
-          <t>shadcn Tabs, both panels in the server HTML (forceMount). The Live tab reads real aggregate numbers from pri_calibrations (getPriLiveStats() in src/lib/pri-research.ts: totals, opt-ins, average score per dimension; no rows leave the server), page stays static and refreshes every 10 minutes. Until the Supabase scripts are run (Phase 2) it says the numbers "aren't available just now" instead of a fake zero. Checked: build (○, 10m), server HTML has both tabs, tab switch at 390/1280px, no JS errors. Re-check with real numbers once the table exists.</t>
+          <t>the category badge ("Deep Research" etc.) sat centred in an empty strip, squeezed against the hero, because we copied live's doubled 52px top gap. Now one gap everywhere and the badge floats in the top-left corner, lined up with the BrewSoul logo (brewsoul-main.tsx, category-badge.tsx); checked on all 26 badge pages at 3 widths that it covers nothing. BrewSoul menu: on tablets (768-1023px) the links were cut off and "More" was hidden with no menu button at all; now the menu button shows below 1024px, 5 links + "More" from 1024px, all 8 from 1280px, "More" always visible.</t>
         </is>
       </c>
       <c r="E299" s="14" t="inlineStr">
@@ -7730,63 +7730,63 @@
       <c r="A300" s="4" t="n"/>
       <c r="B300" s="4" t="inlineStr">
         <is>
+          <t>/pri-efficacy's "Simulation / Live Calibrations" switch like live (2026-10-08)</t>
+        </is>
+      </c>
+      <c r="C300" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D300" s="4" t="inlineStr">
+        <is>
+          <t>shadcn Tabs, both panels in the server HTML (forceMount). The Live tab reads real aggregate numbers from pri_calibrations (getPriLiveStats() in src/lib/pri-research.ts: totals, opt-ins, average score per dimension; no rows leave the server), page stays static and refreshes every 10 minutes. Until the Supabase scripts are run (Phase 2) it says the numbers "aren't available just now" instead of a fake zero. Checked: build (○, 10m), server HTML has both tabs, tab switch at 390/1280px, no JS errors. Re-check with real numbers once the table exists.</t>
+        </is>
+      </c>
+      <c r="E300" s="14" t="inlineStr">
+        <is>
+          <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" s="4" t="n"/>
+      <c r="B301" s="4" t="inlineStr">
+        <is>
           <t>/brewsoul/browse hero readable (2026-10-08, owner said go ahead)</t>
         </is>
       </c>
-      <c r="C300" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D300" s="4" t="inlineStr">
+      <c r="C301" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D301" s="4" t="inlineStr">
         <is>
           <t>a soft cream glow behind the title block so "The Catalog", the subtitle and the stat labels read clearly over the coffee photo (live is hard to read there too; rule 20). Photo still shows around the edges. Checked at 390/1280px.</t>
         </is>
       </c>
-      <c r="E300" s="14" t="inlineStr">
+      <c r="E301" s="14" t="inlineStr">
         <is>
           <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
         </is>
       </c>
     </row>
-    <row r="301">
-      <c r="A301" s="10" t="inlineStr">
+    <row r="302">
+      <c r="A302" s="10" t="inlineStr">
         <is>
           <t>Phase 13 — Images Needed in Sanity</t>
         </is>
       </c>
-      <c r="B301" s="11" t="n"/>
-      <c r="C301" s="11" t="n"/>
-      <c r="D301" s="12" t="n"/>
-    </row>
-    <row r="302">
-      <c r="A302" s="4" t="n"/>
-      <c r="B302" s="4" t="inlineStr">
-        <is>
-          <t>Manus media rescue (2026-09-29)</t>
-        </is>
-      </c>
-      <c r="C302" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D302" s="4" t="inlineStr">
-        <is>
-          <t>all 94 Manus-hosted image/video references in the legacy source (/api/img/, /manus-storage/) were checked live. 91 were still downloadable, including the /akbar photos the entry below calls "permanently lost", and all 91 are now Sanity assets (scripts/rescue-manus-media.ts; Sanity dedupes by SHA-1). 3 were gone (HTTP 502). The manifest docs/ai/manus-media-rescue.md maps each one to the legacy files that used it and its Sanity URL. They are not wired into pages yet: go page by page, with real alt text. /facilitator-index's two diagrams are done (scripts/rescue-facilitator-images.ts).</t>
-        </is>
-      </c>
-      <c r="E302" s="14" t="inlineStr">
-        <is>
-          <t>Phase 13 — Images Needed in Sanity</t>
-        </is>
-      </c>
+      <c r="B302" s="11" t="n"/>
+      <c r="C302" s="11" t="n"/>
+      <c r="D302" s="12" t="n"/>
     </row>
     <row r="303">
       <c r="A303" s="4" t="n"/>
       <c r="B303" s="4" t="inlineStr">
         <is>
-          <t>Favicon</t>
+          <t>Manus media rescue (2026-09-29)</t>
         </is>
       </c>
       <c r="C303" s="13" t="inlineStr">
@@ -7796,7 +7796,7 @@
       </c>
       <c r="D303" s="4" t="inlineStr">
         <is>
-          <t>real "G" brand mark generated from the header's actual wordmark treatment (src/app/icon.tsx), see Phase 3</t>
+          <t>all 94 Manus-hosted image/video references in the legacy source (/api/img/, /manus-storage/) were checked live. 91 were still downloadable, including the /akbar photos the entry below calls "permanently lost", and all 91 are now Sanity assets (scripts/rescue-manus-media.ts; Sanity dedupes by SHA-1). 3 were gone (HTTP 502). The manifest docs/ai/manus-media-rescue.md maps each one to the legacy files that used it and its Sanity URL. They are not wired into pages yet: go page by page, with real alt text. /facilitator-index's two diagrams are done (scripts/rescue-facilitator-images.ts).</t>
         </is>
       </c>
       <c r="E303" s="14" t="inlineStr">
@@ -7809,17 +7809,17 @@
       <c r="A304" s="4" t="n"/>
       <c r="B304" s="4" t="inlineStr">
         <is>
-          <t>Site-wide: logo (light + dark) beyond the current text wordmark</t>
-        </is>
-      </c>
-      <c r="C304" s="15" t="inlineStr">
-        <is>
-          <t>Remaining</t>
+          <t>Favicon</t>
+        </is>
+      </c>
+      <c r="C304" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D304" s="4" t="inlineStr">
         <is>
-          <t>(Default/fallback OG image 1200×630 exists: public/images/default-og.png, checked 2026-10-02.)</t>
+          <t>real "G" brand mark generated from the header's actual wordmark treatment (src/app/icon.tsx), see Phase 3</t>
         </is>
       </c>
       <c r="E304" s="14" t="inlineStr">
@@ -7832,17 +7832,17 @@
       <c r="A305" s="4" t="n"/>
       <c r="B305" s="4" t="inlineStr">
         <is>
-          <t>Author photo(s) for blog author schema (Tony Greenberg headshot at minimum)</t>
-        </is>
-      </c>
-      <c r="C305" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Site-wide: logo (light + dark) beyond the current text wordmark</t>
+        </is>
+      </c>
+      <c r="C305" s="15" t="inlineStr">
+        <is>
+          <t>Remaining</t>
         </is>
       </c>
       <c r="D305" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02: the rescued headshot is already the author avatar in Sanity; now also in every post's Article JSON-LD (author image + url /about). The JSON-LD publisher logo pointed at /favicon.ico, a 404 here; now /icon.</t>
+          <t>(Default/fallback OG image 1200×630 exists: public/images/default-og.png, checked 2026-10-02.)</t>
         </is>
       </c>
       <c r="E305" s="14" t="inlineStr">
@@ -7855,7 +7855,7 @@
       <c r="A306" s="4" t="n"/>
       <c r="B306" s="4" t="inlineStr">
         <is>
-          <t>Blog hero images</t>
+          <t>Author photo(s) for blog author schema (Tony Greenberg headshot at minimum)</t>
         </is>
       </c>
       <c r="C306" s="13" t="inlineStr">
@@ -7865,7 +7865,7 @@
       </c>
       <c r="D306" s="4" t="inlineStr">
         <is>
-          <t>audited, then migrated. Final state:</t>
+          <t>2026-10-02: the rescued headshot is already the author avatar in Sanity; now also in every post's Article JSON-LD (author image + url /about). The JSON-LD publisher logo pointed at /favicon.ico, a 404 here; now /icon.</t>
         </is>
       </c>
       <c r="E306" s="14" t="inlineStr">
@@ -7878,7 +7878,7 @@
       <c r="A307" s="4" t="n"/>
       <c r="B307" s="4" t="inlineStr">
         <is>
-          <t>22 posts have a real hero image, now live in Sanity (17 already on RampRate's own CloudFront + 4 rescued from the legacy /api/img/ proxy + 1…</t>
+          <t>Blog hero images</t>
         </is>
       </c>
       <c r="C307" s="13" t="inlineStr">
@@ -7888,7 +7888,7 @@
       </c>
       <c r="D307" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> rescued from /manus-storage/, all pulled over by migrate-blog-posts.ts before Manus is decommissioned)</t>
+          <t>audited, then migrated. Final state:</t>
         </is>
       </c>
       <c r="E307" s="14" t="inlineStr">
@@ -7901,7 +7901,7 @@
       <c r="A308" s="4" t="n"/>
       <c r="B308" s="4" t="inlineStr">
         <is>
-          <t>7 more posts got a real, unique hero image rescued from the live legacy site's newly-added art this pass (scripts/rescue-2026-09-blog-images…</t>
+          <t>22 posts have a real hero image, now live in Sanity (17 already on RampRate's own CloudFront + 4 rescued from the legacy /api/img/ proxy + 1…</t>
         </is>
       </c>
       <c r="C308" s="13" t="inlineStr">
@@ -7911,7 +7911,7 @@
       </c>
       <c r="D308" s="4" t="inlineStr">
         <is>
-          <t>.ts — see the correction note above): california-toll-roads-legalized-scam, the-1000-hour-hold, conscious-capital-partnership-ecosystem, the-peptide-truth-65m-fraud-industry-vs-life-changing-medicine, clear-communication, building-services-market-transhuman-era, heart-protocol-addendum.</t>
+          <t xml:space="preserve"> rescued from /manus-storage/, all pulled over by migrate-blog-posts.ts before Manus is decommissioned)</t>
         </is>
       </c>
       <c r="E308" s="14" t="inlineStr">
@@ -7924,17 +7924,17 @@
       <c r="A309" s="4" t="n"/>
       <c r="B309" s="4" t="inlineStr">
         <is>
-          <t>92 posts still need a real, unique hero image</t>
-        </is>
-      </c>
-      <c r="C309" s="15" t="inlineStr">
-        <is>
-          <t>Remaining</t>
+          <t>7 more posts got a real, unique hero image rescued from the live legacy site's newly-added art this pass (scripts/rescue-2026-09-blog-images…</t>
+        </is>
+      </c>
+      <c r="C309" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D309" s="4" t="inlineStr">
         <is>
-          <t>(down from 99). Tracked one row per post, with a suggested image-generation prompt, in BLOG-IMAGE-BRIEFS.md — work through that file and check items off there, not here. No image-generation tool was connected in this environment as of this writing; either connect one (e.g. an MCP image-gen extension), source these manually/with a designer then upload via Sanity Studio (/studio), or re-check the live legacy site periodically per the correction note above.</t>
+          <t>.ts — see the correction note above): california-toll-roads-legalized-scam, the-1000-hour-hold, conscious-capital-partnership-ecosystem, the-peptide-truth-65m-fraud-industry-vs-life-changing-medicine, clear-communication, building-services-market-transhuman-era, heart-protocol-addendum.</t>
         </is>
       </c>
       <c r="E309" s="14" t="inlineStr">
@@ -7947,17 +7947,17 @@
       <c r="A310" s="4" t="n"/>
       <c r="B310" s="4" t="inlineStr">
         <is>
-          <t>Blog: per-post OG image if different from hero (many posts can reuse hero as OG)</t>
-        </is>
-      </c>
-      <c r="C310" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>92 posts still need a real, unique hero image</t>
+        </is>
+      </c>
+      <c r="C310" s="15" t="inlineStr">
+        <is>
+          <t>Remaining</t>
         </is>
       </c>
       <c r="D310" s="4" t="inlineStr">
         <is>
-          <t>Confirmed 2026-10-02: generateMetadata uses seo.ogImage, else the hero, else the default OG image.</t>
+          <t>(down from 99). Tracked one row per post, with a suggested image-generation prompt, in BLOG-IMAGE-BRIEFS.md — work through that file and check items off there, not here. No image-generation tool was connected in this environment as of this writing; either connect one (e.g. an MCP image-gen extension), source these manually/with a designer then upload via Sanity Studio (/studio), or re-check the live legacy site periodically per the correction note above.</t>
         </is>
       </c>
       <c r="E310" s="14" t="inlineStr">
@@ -7970,7 +7970,7 @@
       <c r="A311" s="4" t="n"/>
       <c r="B311" s="4" t="inlineStr">
         <is>
-          <t>Marketing pages</t>
+          <t>Blog: per-post OG image if different from hero (many posts can reuse hero as OG)</t>
         </is>
       </c>
       <c r="C311" s="13" t="inlineStr">
@@ -7980,7 +7980,7 @@
       </c>
       <c r="D311" s="4" t="inlineStr">
         <is>
-          <t>hero/section images for /the-letter, /the-territory, /engine-room, /the-body, /the-nightstand, /recent-creations (portfolio thumbnails), /published (publication logos), /clients (client logos — confirm licensing before re-hosting). Checked against live 2026-10-02: same image count on every one; /the-territory, /engine-room, /recent-creations, /published, /clients have no images on live either.</t>
+          <t>Confirmed 2026-10-02: generateMetadata uses seo.ogImage, else the hero, else the default OG image.</t>
         </is>
       </c>
       <c r="E311" s="14" t="inlineStr">
@@ -7993,7 +7993,7 @@
       <c r="A312" s="4" t="n"/>
       <c r="B312" s="4" t="inlineStr">
         <is>
-          <t>/akbar essay images</t>
+          <t>Marketing pages</t>
         </is>
       </c>
       <c r="C312" s="13" t="inlineStr">
@@ -8003,7 +8003,7 @@
       </c>
       <c r="D312" s="4" t="inlineStr">
         <is>
-          <t>not lost after all: 20 of the 21 were rescued into Sanity by scripts/rescue-manus-media.ts (2026-09-28) and are wired back in legacy's layout (hero mosaic, JC portrait, 2x2 grid, 3 full-bleeds, 3-up strip, footer gallery) as of 2026-09-29. Only slider-3 was gone (HTTP 502); the hero mosaic is 4 tiles instead of 5.</t>
+          <t>hero/section images for /the-letter, /the-territory, /engine-room, /the-body, /the-nightstand, /recent-creations (portfolio thumbnails), /published (publication logos), /clients (client logos — confirm licensing before re-hosting). Checked against live 2026-10-02: same image count on every one; /the-territory, /engine-room, /recent-creations, /published, /clients have no images on live either.</t>
         </is>
       </c>
       <c r="E312" s="14" t="inlineStr">
@@ -8016,7 +8016,7 @@
       <c r="A313" s="4" t="n"/>
       <c r="B313" s="4" t="inlineStr">
         <is>
-          <t>Rescued page images wired back in (2026-09-29)</t>
+          <t>/akbar essay images</t>
         </is>
       </c>
       <c r="C313" s="13" t="inlineStr">
@@ -8026,7 +8026,7 @@
       </c>
       <c r="D313" s="4" t="inlineStr">
         <is>
-          <t>/living-declaration hero, hand image and Clarisse Abelarde artwork; /impact-dashboard earth hero; /find-my banner; /find-your-coffee dark photo landing (legacy copy restored, replacing an intro that wasn't in legacy). Also wired (second pass): /consciousness-scale (legacy's hero-first flow restored, the invented intro screen removed), /find-your-me hero, /humanos hero, the HumanOS nav logo, and all 12 HumanOS people headshots (/humanos/ecosystem, /humanos/philosophy). Blog-body images (2026-09-29): all 19 the migration dropped are restored by scripts/restore-blog-body-images.ts as Sanity drafts on 4 posts (Clarisse Abelarde 7, You Are the Moat 4, FRQNCY 6, Energy Is Money 2), waiting to be published in Studio; the other blog-listed assets were heroes already set. Still unwired from docs/ai/manus-media-rescue.md: and /alex-azzi's subject photo (a photo of a real person on an accusation page: needs Tony's yes first).</t>
+          <t>not lost after all: 20 of the 21 were rescued into Sanity by scripts/rescue-manus-media.ts (2026-09-28) and are wired back in legacy's layout (hero mosaic, JC portrait, 2x2 grid, 3 full-bleeds, 3-up strip, footer gallery) as of 2026-09-29. Only slider-3 was gone (HTTP 502); the hero mosaic is 4 tiles instead of 5.</t>
         </is>
       </c>
       <c r="E313" s="14" t="inlineStr">
@@ -8039,7 +8039,7 @@
       <c r="A314" s="4" t="n"/>
       <c r="B314" s="4" t="inlineStr">
         <is>
-          <t>BrewSoul: coffee/product images (brewsoul-coffees-expanded.ts likely has image refs</t>
+          <t>Rescued page images wired back in (2026-09-29)</t>
         </is>
       </c>
       <c r="C314" s="13" t="inlineStr">
@@ -8049,7 +8049,7 @@
       </c>
       <c r="D314" s="4" t="inlineStr">
         <is>
-          <t>audit), city guide header images, roaster directory photos. Audited 2026-09-09 (status spreadsheet), confirmed 2026-10-02: city guides already have photos; coffees, chains and roasters have no image field in legacy or here (text-only by design); farms got real photos.</t>
+          <t>/living-declaration hero, hand image and Clarisse Abelarde artwork; /impact-dashboard earth hero; /find-my banner; /find-your-coffee dark photo landing (legacy copy restored, replacing an intro that wasn't in legacy). Also wired (second pass): /consciousness-scale (legacy's hero-first flow restored, the invented intro screen removed), /find-your-me hero, /humanos hero, the HumanOS nav logo, and all 12 HumanOS people headshots (/humanos/ecosystem, /humanos/philosophy). Blog-body images (2026-09-29): all 19 the migration dropped are restored by scripts/restore-blog-body-images.ts as Sanity drafts on 4 posts (Clarisse Abelarde 7, You Are the Moat 4, FRQNCY 6, Energy Is Money 2), waiting to be published in Studio; the other blog-listed assets were heroes already set. Still unwired from docs/ai/manus-media-rescue.md: and /alex-azzi's subject photo (a photo of a real person on an accusation page: needs Tony's yes first).</t>
         </is>
       </c>
       <c r="E314" s="14" t="inlineStr">
@@ -8062,7 +8062,7 @@
       <c r="A315" s="4" t="n"/>
       <c r="B315" s="4" t="inlineStr">
         <is>
-          <t>65 page images moved off the Manus storage copy into Sanity (2026-10-02)</t>
+          <t>BrewSoul: coffee/product images (brewsoul-coffees-expanded.ts likely has image refs</t>
         </is>
       </c>
       <c r="C315" s="13" t="inlineStr">
@@ -8072,7 +8072,7 @@
       </c>
       <c r="D315" s="4" t="inlineStr">
         <is>
-          <t>every image the code loaded from d2xsxph8kpxj0f.cloudfront.net (PRI medicine images, Iboga module, facilitator index, /attention-theft, /alex-azzi, /protecting-your-business, /peyote-mescaline, HumanOS, the peptide quiz). Notes called it "RampRate's own CloudFront", but every file sits in the legacy Manus project's folder and its owner couldn't be confirmed. All 65 uploaded (scripts/rescue-cloudfront-images.ts), code rewritten, host removed from images.remotePatterns, no Sanity document used it. Table in docs/ai/manus-media-rescue.md.</t>
+          <t>audit), city guide header images, roaster directory photos. Audited 2026-09-09 (status spreadsheet), confirmed 2026-10-02: city guides already have photos; coffees, chains and roasters have no image field in legacy or here (text-only by design); farms got real photos.</t>
         </is>
       </c>
       <c r="E315" s="14" t="inlineStr">
@@ -8085,7 +8085,7 @@
       <c r="A316" s="4" t="n"/>
       <c r="B316" s="4" t="inlineStr">
         <is>
-          <t>PRI/Kava: medicine reference images (medicine-images.ts), facility images for /facilitator-index</t>
+          <t>65 page images moved off the Manus storage copy into Sanity (2026-10-02)</t>
         </is>
       </c>
       <c r="C316" s="13" t="inlineStr">
@@ -8095,7 +8095,7 @@
       </c>
       <c r="D316" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02: all in Sanity; image counts match live on PRI, Kava, Iboga, Peyote, facilitator pages.</t>
+          <t>every image the code loaded from d2xsxph8kpxj0f.cloudfront.net (PRI medicine images, Iboga module, facilitator index, /attention-theft, /alex-azzi, /protecting-your-business, /peyote-mescaline, HumanOS, the peptide quiz). Notes called it "RampRate's own CloudFront", but every file sits in the legacy Manus project's folder and its owner couldn't be confirmed. All 65 uploaded (scripts/rescue-cloudfront-images.ts), code rewritten, host removed from images.remotePatterns, no Sanity document used it. Table in docs/ai/manus-media-rescue.md.</t>
         </is>
       </c>
       <c r="E316" s="14" t="inlineStr">
@@ -8108,7 +8108,7 @@
       <c r="A317" s="4" t="n"/>
       <c r="B317" s="4" t="inlineStr">
         <is>
-          <t>Manifesto/Attention Theft: any diagram/illustration assets used on the mega-page</t>
+          <t>PRI/Kava: medicine reference images (medicine-images.ts), facility images for /facilitator-index</t>
         </is>
       </c>
       <c r="C317" s="13" t="inlineStr">
@@ -8118,7 +8118,7 @@
       </c>
       <c r="D317" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02: 6 of live's 7 are in (now in Sanity); the 7th belongs to the Wall of Shame section left out on purpose.</t>
+          <t>2026-10-02: all in Sanity; image counts match live on PRI, Kava, Iboga, Peyote, facilitator pages.</t>
         </is>
       </c>
       <c r="E317" s="14" t="inlineStr">
@@ -8131,17 +8131,17 @@
       <c r="A318" s="4" t="n"/>
       <c r="B318" s="4" t="inlineStr">
         <is>
-          <t>Assessment result-screen background art (flagged in STATUS.md as a known gap</t>
-        </is>
-      </c>
-      <c r="C318" s="15" t="inlineStr">
-        <is>
-          <t>Remaining</t>
+          <t>Manifesto/Attention Theft: any diagram/illustration assets used on the mega-page</t>
+        </is>
+      </c>
+      <c r="C318" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D318" s="4" t="inlineStr">
         <is>
-          <t>18/20 assessments currently have plain black backgrounds; sourcing themed art here also closes that gap)</t>
+          <t>2026-10-02: 6 of live's 7 are in (now in Sanity); the 7th belongs to the Wall of Shame section left out on purpose.</t>
         </is>
       </c>
       <c r="E318" s="14" t="inlineStr">
@@ -8154,17 +8154,17 @@
       <c r="A319" s="4" t="n"/>
       <c r="B319" s="4" t="inlineStr">
         <is>
-          <t>Chatbot: FauxTony avatar/icon</t>
-        </is>
-      </c>
-      <c r="C319" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Assessment result-screen background art (flagged in STATUS.md as a known gap</t>
+        </is>
+      </c>
+      <c r="C319" s="15" t="inlineStr">
+        <is>
+          <t>Remaining</t>
         </is>
       </c>
       <c r="D319" s="4" t="inlineStr">
         <is>
-          <t>Not needed (2026-10-02): the chatbot phase (Phase 10) was cancelled.</t>
+          <t>18/20 assessments currently have plain black backgrounds; sourcing themed art here also closes that gap)</t>
         </is>
       </c>
       <c r="E319" s="14" t="inlineStr">
@@ -8177,73 +8177,73 @@
       <c r="A320" s="4" t="n"/>
       <c r="B320" s="4" t="inlineStr">
         <is>
+          <t>Chatbot: FauxTony avatar/icon</t>
+        </is>
+      </c>
+      <c r="C320" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D320" s="4" t="inlineStr">
+        <is>
+          <t>Not needed (2026-10-02): the chatbot phase (Phase 10) was cancelled.</t>
+        </is>
+      </c>
+      <c r="E320" s="14" t="inlineStr">
+        <is>
+          <t>Phase 13 — Images Needed in Sanity</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" s="4" t="n"/>
+      <c r="B321" s="4" t="inlineStr">
+        <is>
           <t>Audit client/public/ (including alex-azzi/, brewsoul/ subfolders) for any static assets already sitting there unused that should be pulled i…</t>
         </is>
       </c>
-      <c r="C320" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D320" s="4" t="inlineStr">
+      <c r="C321" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D321" s="4" t="inlineStr">
         <is>
           <t>n rather than re-created. Done 2026-10-02: no images there at all (only llms.txt, a BrewSoul catalog, Manus debug files, design-options.html). Found and fixed a cutover risk instead: live serves two Google site-verification files (/google6881a0411c48b301.html, /alex-azzi/googleedff0185753a4a1f.html) that the new site returned 404 for, so Search Console could lose verification at DNS cutover. Both copied to public/ byte for byte. Not copied: site.webmanifest (its icons don't exist here; Next's app/icon.tsx covers the favicon).</t>
         </is>
       </c>
-      <c r="E320" s="14" t="inlineStr">
+      <c r="E321" s="14" t="inlineStr">
         <is>
           <t>Phase 13 — Images Needed in Sanity</t>
         </is>
       </c>
     </row>
-    <row r="321">
-      <c r="A321" s="10" t="inlineStr">
+    <row r="322">
+      <c r="A322" s="10" t="inlineStr">
         <is>
           <t>Phase 14 — QA &amp; Launch</t>
         </is>
       </c>
-      <c r="B321" s="11" t="n"/>
-      <c r="C321" s="11" t="n"/>
-      <c r="D321" s="12" t="n"/>
-    </row>
-    <row r="322">
-      <c r="A322" s="4" t="n"/>
-      <c r="B322" s="4" t="inlineStr">
-        <is>
-          <t>Mobile responsive pass on every ported section</t>
-        </is>
-      </c>
-      <c r="C322" s="15" t="inlineStr">
-        <is>
-          <t>Remaining</t>
-        </is>
-      </c>
-      <c r="D322" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-29: no page scrolls sideways at 375px any more (114 pages checked in Chrome: every unique page plus 3 of each templated set like blog posts and coffees). Fixed: BrewSoul NextSteps forced 3 columns (and used an inline style), charity-scorecard tab row, /brewsoul/browse filter dropdowns, /the-philosophy hero glow. Still to check by hand: 44px tap targets and Safari iOS. 2026-09-30: 44px tap targets on phones for the shared header, footer, BrewSoul/Kava/HumanOS menus and ~100 standalone links (undersized targets 1,904 → 578; the rest are 24-43px pills/chips that meet WCAG 2.2 AA). axe target-size (WCAG 2.2 AA, with its spacing exception): 0 failures on 114 pages. Safari/iPhone (WebKit, iPhone 14 emulation): all 114 pages load, no sideways scroll, no JS errors; form fields under 16px (iOS zoom-on-tap) fixed site-wide in globals.css. Still to check on a real iPhone: BrewSoul's bottom journey bar showed page text through it in headless WebKit only (taps hit the bar correctly; Chrome renders it solid). Fixed 2026-10-09: the bar is now solid (bg-[#2C1810], was 92% plus backdrop-blur-md), so nothing can show through even where the blur isn't drawn; checked in WebKit (iPhone 13 profile) and Chrome: background rgb(44, 24, 16), no text behind the buttons. A real iPhone check is still part of Phase 14.</t>
-        </is>
-      </c>
-      <c r="E322" s="14" t="inlineStr">
-        <is>
-          <t>Phase 14 — QA &amp; Launch</t>
-        </is>
-      </c>
+      <c r="B322" s="11" t="n"/>
+      <c r="C322" s="11" t="n"/>
+      <c r="D322" s="12" t="n"/>
     </row>
     <row r="323">
       <c r="A323" s="4" t="n"/>
       <c r="B323" s="4" t="inlineStr">
         <is>
-          <t>Accessibility pass (WCAG AA contrast, 44px touch targets, keyboard nav)</t>
-        </is>
-      </c>
-      <c r="C323" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Mobile responsive pass on every ported section</t>
+        </is>
+      </c>
+      <c r="C323" s="15" t="inlineStr">
+        <is>
+          <t>Remaining</t>
         </is>
       </c>
       <c r="D323" s="4" t="inlineStr">
         <is>
-          <t>same bar as legacy QA_MASTER_PROMPT.md. 2026-09-29 axe-core pass (WCAG 2.1 AA, same 114 pages, production build): all unlabeled dropdowns/inputs and unnamed links fixed; contrast down from 1,453 failing items on 106 pages to 1,038 on 70 (43 pages fully clean). Shared fixes: brand gold #8b6914 → #836311 site-wide (was 4.3:1 on cream, AA needs 4.5), header "⌘K"/social icons, BrewSoul nav and footer, HumanOS footer, Kava footer, assessment intro footnote, post-card image links. 2026-09-30: contrast finished, 0 axe color-contrast failures left on the same 114 pages (production build). Token changes: --kava-saffron #b86a28 → #8e521f, --pri-purple-light #a855f7 → #b87bf9 (on-dark purple only), --crusade-teal #0e7c7c → #0d7373; PriEyebrow goes light purple inside a dark PriSection via group-data-dark/pri; /find-your-me and the journey tracker's dark glass panels 60-70% → 90% (legacy's own 60% glass on beige rendered gray, cream text failed). Everything else: nearest passing shade of the same hue, or gold ↔ gold-light on the wrong background. Left: 18 links inside text marked only by color (need an underline), 44px tap targets, keyboard nav. 2026-09-30: 18 color-only in-text links underlined (axe link-in-text-block: 0 left); keyboard focus visible on every focusable item on 8 sampled pages (two form fields had none, fixed). 2026-10-02 re-run (axe WCAG 2.2 AA, 142 pages × 375/1280px, production build, plus Tab through 40 stops per page): found 1,370 contrast failures (mostly BrewSoul'</t>
+          <t>2026-09-29: no page scrolls sideways at 375px any more (114 pages checked in Chrome: every unique page plus 3 of each templated set like blog posts and coffees). Fixed: BrewSoul NextSteps forced 3 columns (and used an inline style), charity-scorecard tab row, /brewsoul/browse filter dropdowns, /the-philosophy hero glow. Still to check by hand: 44px tap targets and Safari iOS. 2026-09-30: 44px tap targets on phones for the shared header, footer, BrewSoul/Kava/HumanOS menus and ~100 standalone links (undersized targets 1,904 → 578; the rest are 24-43px pills/chips that meet WCAG 2.2 AA). axe target-size (WCAG 2.2 AA, with its spacing exception): 0 failures on 114 pages. Safari/iPhone (WebKit, iPhone 14 emulation): all 114 pages load, no sideways scroll, no JS errors; form fields under 16px (iOS zoom-on-tap) fixed site-wide in globals.css. Still to check on a real iPhone: BrewSoul's bottom journey bar showed page text through it in headless WebKit only (taps hit the bar correctly; Chrome renders it solid). Fixed 2026-10-09: the bar is now solid (bg-[#2C1810], was 92% plus backdrop-blur-md), so nothing can show through even where the blur isn't drawn; checked in WebKit (iPhone 13 profile) and Chrome: background rgb(44, 24, 16), no text behind the buttons. A real iPhone check is still part of Phase 14.</t>
         </is>
       </c>
       <c r="E323" s="14" t="inlineStr">
@@ -8256,17 +8256,17 @@
       <c r="A324" s="4" t="n"/>
       <c r="B324" s="4" t="inlineStr">
         <is>
-          <t>No dead-end pages (every page links to 2+ others)</t>
-        </is>
-      </c>
-      <c r="C324" s="15" t="inlineStr">
-        <is>
-          <t>Remaining</t>
+          <t>Accessibility pass (WCAG AA contrast, 44px touch targets, keyboard nav)</t>
+        </is>
+      </c>
+      <c r="C324" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D324" s="4" t="inlineStr">
         <is>
-          <t>same bar as legacy MASTER_QUALITY_PROMPT.md 2026-09-30 scan (496 sitemap pages, header/footer links not counted): every page has a way home (the 6 HumanOS pages had none, in legacy too; added a "← TonyGreenberg.com" footer link). ~17 quiz pages only look like dead ends on their intro screen; their result screens link to related assessments. Left for a content decision: ~20 marketing pages (/akbar, /amplifier, /diamond-cut, /ecosystem, /engage, /engine-room, /intel, /invest, /pick-up-the-phone, /protecting-your-business, /published, /speaking, /the-nightstand, /the-territory, /the-web, /under-nda, /pri-calibration, /charity-scorecard and its detail pages) link to only 0-1 other page in their content. The port matches legacy there (legacy was just as sparse), so adding related links is new content and needs the owner's yes.</t>
+          <t>same bar as legacy QA_MASTER_PROMPT.md. 2026-09-29 axe-core pass (WCAG 2.1 AA, same 114 pages, production build): all unlabeled dropdowns/inputs and unnamed links fixed; contrast down from 1,453 failing items on 106 pages to 1,038 on 70 (43 pages fully clean). Shared fixes: brand gold #8b6914 → #836311 site-wide (was 4.3:1 on cream, AA needs 4.5), header "⌘K"/social icons, BrewSoul nav and footer, HumanOS footer, Kava footer, assessment intro footnote, post-card image links. 2026-09-30: contrast finished, 0 axe color-contrast failures left on the same 114 pages (production build). Token changes: --kava-saffron #b86a28 → #8e521f, --pri-purple-light #a855f7 → #b87bf9 (on-dark purple only), --crusade-teal #0e7c7c → #0d7373; PriEyebrow goes light purple inside a dark PriSection via group-data-dark/pri; /find-your-me and the journey tracker's dark glass panels 60-70% → 90% (legacy's own 60% glass on beige rendered gray, cream text failed). Everything else: nearest passing shade of the same hue, or gold ↔ gold-light on the wrong background. Left: 18 links inside text marked only by color (need an underline), 44px tap targets, keyboard nav. 2026-09-30: 18 color-only in-text links underlined (axe link-in-text-block: 0 left); keyboard focus visible on every focusable item on 8 sampled pages (two form fields had none, fixed). 2026-10-02 re-run (axe WCAG 2.2 AA, 142 pages × 375/1280px, production build, plus Tab through 40 stops per page): found 1,370 contrast failures (mostly BrewSoul'</t>
         </is>
       </c>
       <c r="E324" s="14" t="inlineStr">
@@ -8279,7 +8279,7 @@
       <c r="A325" s="4" t="n"/>
       <c r="B325" s="4" t="inlineStr">
         <is>
-          <t>Cross-browser check (Safari iOS in particular, per legacy performance notes) 2026-10-06 WebKit pass (Playwright WebKit, iPhone 13 profile, 1…</t>
+          <t>No dead-end pages (every page links to 2+ others)</t>
         </is>
       </c>
       <c r="C325" s="15" t="inlineStr">
@@ -8289,7 +8289,7 @@
       </c>
       <c r="D325" s="4" t="inlineStr">
         <is>
-          <t>52 pages: every unique page plus 3 of each templated set, production build): no page pans sideways, no failed requests, no JS errors. Found and fixed on the way: upgrade-insecure-requests in the new CSP made Safari fetch every stylesheet and font over https on localhost (dropped; the site is HTTPS-only via HSTS anyway), and .toLocaleString() without a locale caused a hydration error on /brewsoul/chains in Safari (all number formatting now en-US). Left: a check on a real iPhone (Phase 14).</t>
+          <t>same bar as legacy MASTER_QUALITY_PROMPT.md 2026-09-30 scan (496 sitemap pages, header/footer links not counted): every page has a way home (the 6 HumanOS pages had none, in legacy too; added a "← TonyGreenberg.com" footer link). ~17 quiz pages only look like dead ends on their intro screen; their result screens link to related assessments. Left for a content decision: ~20 marketing pages (/akbar, /amplifier, /diamond-cut, /ecosystem, /engage, /engine-room, /intel, /invest, /pick-up-the-phone, /protecting-your-business, /published, /speaking, /the-nightstand, /the-territory, /the-web, /under-nda, /pri-calibration, /charity-scorecard and its detail pages) link to only 0-1 other page in their content. The port matches legacy there (legacy was just as sparse), so adding related links is new content and needs the owner's yes.</t>
         </is>
       </c>
       <c r="E325" s="14" t="inlineStr">
@@ -8302,7 +8302,7 @@
       <c r="A326" s="4" t="n"/>
       <c r="B326" s="4" t="inlineStr">
         <is>
-          <t>Remove noindex only when sign-off is given</t>
+          <t>Cross-browser check (Safari iOS in particular, per legacy performance notes) 2026-10-06 WebKit pass (Playwright WebKit, iPhone 13 profile, 1…</t>
         </is>
       </c>
       <c r="C326" s="15" t="inlineStr">
@@ -8312,7 +8312,7 @@
       </c>
       <c r="D326" s="4" t="inlineStr">
         <is>
-          <t>do not launch indexable by accident (The only noindex is the host-based one for *.netlify.app above, so the real domain is indexable as soon as DNS points at it: sign-off must come before DNS.)</t>
+          <t>52 pages: every unique page plus 3 of each templated set, production build): no page pans sideways, no failed requests, no JS errors. Found and fixed on the way: upgrade-insecure-requests in the new CSP made Safari fetch every stylesheet and font over https on localhost (dropped; the site is HTTPS-only via HSTS anyway), and .toLocaleString() without a locale caused a hydration error on /brewsoul/chains in Safari (all number formatting now en-US). Left: a check on a real iPhone (Phase 14).</t>
         </is>
       </c>
       <c r="E326" s="14" t="inlineStr">
@@ -8325,7 +8325,7 @@
       <c r="A327" s="4" t="n"/>
       <c r="B327" s="4" t="inlineStr">
         <is>
-          <t>Final stakeholder sign-off (Tony/Darryl/Kimberly) on the ported site before DNS cutover</t>
+          <t>Remove noindex only when sign-off is given</t>
         </is>
       </c>
       <c r="C327" s="15" t="inlineStr">
@@ -8333,7 +8333,11 @@
           <t>Remaining</t>
         </is>
       </c>
-      <c r="D327" s="4" t="inlineStr"/>
+      <c r="D327" s="4" t="inlineStr">
+        <is>
+          <t>do not launch indexable by accident (The only noindex is the host-based one for *.netlify.app above, so the real domain is indexable as soon as DNS points at it: sign-off must come before DNS.)</t>
+        </is>
+      </c>
       <c r="E327" s="14" t="inlineStr">
         <is>
           <t>Phase 14 — QA &amp; Launch</t>
@@ -8344,7 +8348,7 @@
       <c r="A328" s="4" t="n"/>
       <c r="B328" s="4" t="inlineStr">
         <is>
-          <t>DNS cutover, legacy app decommissioned only after a stable overlap window</t>
+          <t>Final stakeholder sign-off (Tony/Darryl/Kimberly) on the ported site before DNS cutover</t>
         </is>
       </c>
       <c r="C328" s="15" t="inlineStr">
@@ -8359,18 +8363,37 @@
         </is>
       </c>
     </row>
+    <row r="329">
+      <c r="A329" s="4" t="n"/>
+      <c r="B329" s="4" t="inlineStr">
+        <is>
+          <t>DNS cutover, legacy app decommissioned only after a stable overlap window</t>
+        </is>
+      </c>
+      <c r="C329" s="15" t="inlineStr">
+        <is>
+          <t>Remaining</t>
+        </is>
+      </c>
+      <c r="D329" s="4" t="inlineStr"/>
+      <c r="E329" s="14" t="inlineStr">
+        <is>
+          <t>Phase 14 — QA &amp; Launch</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D328"/>
+  <autoFilter ref="A1:D329"/>
   <mergeCells count="14">
     <mergeCell ref="A150:D150"/>
-    <mergeCell ref="A321:D321"/>
+    <mergeCell ref="A322:D322"/>
     <mergeCell ref="A237:D237"/>
     <mergeCell ref="A58:D58"/>
     <mergeCell ref="A258:D258"/>
     <mergeCell ref="A209:D209"/>
     <mergeCell ref="A205:D205"/>
     <mergeCell ref="A15:D15"/>
-    <mergeCell ref="A301:D301"/>
+    <mergeCell ref="A302:D302"/>
     <mergeCell ref="A43:D43"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A183:D183"/>

</xml_diff>

<commit_message>
Old site's database: short share links carried over; findings documented
- Read-only check of the legacy Manus/TiDB database (56 tables): most rows
  are the Manus agent's automated tests. Full private backup kept outside
  the repo (personal data; never committed). Findings, without personal
  data: docs/ai/project_legacy_database.md.
- The old site's 198 short share links /s/<code> now 308 to their page
  (src/lib/content/short-links.ts, read by next.config.ts). 196 land on a
  working page; 2 targets don't exist on live either.
- Restoration-branch note says where its backup is now that it's deleted.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Migration-Status-Report.xlsx
+++ b/Migration-Status-Report.xlsx
@@ -1953,7 +1953,7 @@
       <c r="A42" s="4" t="n"/>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>Copy the old site's visitor data from the Manus database (owner asked, 2026-10-09)</t>
+          <t>Old site's visitor data from the Manus database (owner asked, 2026-10-09)</t>
         </is>
       </c>
       <c r="C42" s="15" t="inlineStr">
@@ -1963,7 +1963,7 @@
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>The legacy app keeps ~55 MySQL tables on Manus (_legacy-manus-app/drizzle/schema.ts); they go away with Manus. Owner has the connection details: put them in .env.local as LEGACY_DATABASE_URL (never in chat or a commit). Plan: (1) read row counts for every table (read-only, a throwaway pymysql reader outside the project, no new package); (2) after the two Supabase scripts below are run, copy the 12 tables that already have a home: blog_comments, blog_ratings, post_reactions → blog_reactions, micro_commitments → blog_commitments, highlights, referral_codes, referrals, clock_keeper_responses, post_intervention_assessments, friend_gate_sessions, friend_gate_slots, pri_calibrations (account-linked rows can only be matched to new accounts by email); (3) email_subscribers go to Kit, not Supabase; (4) owner picks which of the rest need new tables (facilitator submissions/votes, assessment results, journey progress, community, vendor intake, page views...). Billing (purchases, subscriptions) and spam tracking stay out of scope. Blocked on: LEGACY_DATABASE_URL, and the Supabase scripts being run.</t>
+          <t>Connection details in .env.local (LEGACY_DATABASE_URL). Done: read-only check of all 56 tables and a full private backup (75,128 rows) to ~/Desktop/tonyg-site-backups/legacy-db-export-2026-10-09/ on the webmaster's Mac (personal data: never commit); most rows are the Manus agent's automated tests (details: docs/ai/project_legacy_database.md); the 198 short share links /s/&lt;code&gt; now redirect (src/lib/content/short-links.ts; 196 land on a page, 2 targets don't exist on live either). Left (needs a yes): add the 36 real email subscribers to Kit (may send Kit's confirmation email); copy the handful of real reactions/ratings/commitment into Supabase after the scripts below are run; decide whether the ~24 real assessment results, ~17 PRI consents, 2 manifesto responses, 8 supplier forms and 1 Cheshire submission stay in the backup only. Then rotate the database password (it was pasted in a chat) and remove LEGACY_DATABASE_URL.</t>
         </is>
       </c>
       <c r="E42" s="14" t="inlineStr">
@@ -8530,7 +8530,7 @@
       <c r="A4" s="4" t="n"/>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Copy the old site's visitor data from the Manus database (owner asked, 2026-10-09)</t>
+          <t>Old site's visitor data from the Manus database (owner asked, 2026-10-09)</t>
         </is>
       </c>
       <c r="C4" s="15" t="inlineStr">
@@ -8540,7 +8540,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>The legacy app keeps ~55 MySQL tables on Manus (_legacy-manus-app/drizzle/schema.ts); they go away with Manus. Owner has the connection details: put them in .env.local as LEGACY_DATABASE_URL (never in chat or a commit). Plan: (1) read row counts for every table (read-only, a throwaway pymysql reader outside the project, no new package); (2) after the two Supabase scripts below are run, copy the 12 tables that already have a home: blog_comments, blog_ratings, post_reactions → blog_reactions, micro_commitments → blog_commitments, highlights, referral_codes, referrals, clock_keeper_responses, post_intervention_assessments, friend_gate_sessions, friend_gate_slots, pri_calibrations (account-linked rows can only be matched to new accounts by email); (3) email_subscribers go to Kit, not Supabase; (4) owner picks which of the rest need new tables (facilitator submissions/votes, assessment results, journey progress, community, vendor intake, page views...). Billing (purchases, subscriptions) and spam tracking stay out of scope. Blocked on: LEGACY_DATABASE_URL, and the Supabase scripts being run.</t>
+          <t>Connection details in .env.local (LEGACY_DATABASE_URL). Done: read-only check of all 56 tables and a full private backup (75,128 rows) to ~/Desktop/tonyg-site-backups/legacy-db-export-2026-10-09/ on the webmaster's Mac (personal data: never commit); most rows are the Manus agent's automated tests (details: docs/ai/project_legacy_database.md); the 198 short share links /s/&lt;code&gt; now redirect (src/lib/content/short-links.ts; 196 land on a page, 2 targets don't exist on live either). Left (needs a yes): add the 36 real email subscribers to Kit (may send Kit's confirmation email); copy the handful of real reactions/ratings/commitment into Supabase after the scripts below are run; decide whether the ~24 real assessment results, ~17 PRI consents, 2 manifesto responses, 8 supplier forms and 1 Cheshire submission stay in the backup only. Then rotate the database password (it was pasted in a chat) and remove LEGACY_DATABASE_URL.</t>
         </is>
       </c>
       <c r="E4" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Old site's data: subscribers in Kit, supplier-form archive scripts, launch facts
- Kit: 5 of 36 legacy subscribers already there; 31 added quietly via a
  new tag (Kit accepted 27, suppressed 4). No emails sent.
- supabase/migrations/0003_legacy_vendor_intake.sql + scripts/import-
  legacy-vendor-intake.ts: archive the 8 old supplier forms (owner's
  choice). Not run: the Supabase project is paused (address no longer
  resolves); restore it, run 0001-0003, then the script.
- Daily Provocations: the missing 2026-10-07 line from the legacy DB.
- Project file: Supabase pause, DNS at Hostinger (www -> Manus), Netlify
  has no custom domain yet; go-live steps in Phase 14.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Migration-Status-Report.xlsx
+++ b/Migration-Status-Report.xlsx
@@ -1963,7 +1963,7 @@
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Connection details in .env.local (LEGACY_DATABASE_URL). Done: read-only check of all 56 tables and a full private backup (75,128 rows) to ~/Desktop/tonyg-site-backups/legacy-db-export-2026-10-09/ on the webmaster's Mac (personal data: never commit); most rows are the Manus agent's automated tests (details: docs/ai/project_legacy_database.md); the 198 short share links /s/&lt;code&gt; now redirect (src/lib/content/short-links.ts; 196 land on a page, 2 targets don't exist on live either). Left (needs a yes): add the 36 real email subscribers to Kit (may send Kit's confirmation email); copy the handful of real reactions/ratings/commitment into Supabase after the scripts below are run; decide whether the ~24 real assessment results, ~17 PRI consents, 2 manifesto responses, 8 supplier forms and 1 Cheshire submission stay in the backup only. Then rotate the database password (it was pasted in a chat) and remove LEGACY_DATABASE_URL.</t>
+          <t>Connection details in .env.local (LEGACY_DATABASE_URL). Done: read-only check of all 56 tables and a full private backup (75,128 rows) to ~/Desktop/tonyg-site-backups/legacy-db-export-2026-10-09/ on the webmaster's Mac (personal data: never commit); most rows are the Manus agent's automated tests (details: docs/ai/project_legacy_database.md); the 198 short share links /s/&lt;code&gt; now redirect (src/lib/content/short-links.ts; 196 land on a page, 2 targets don't exist on live either). Done 2026-10-09 (owner said yes): email subscribers in Kit with no email sent (5 already there, 27 added on the new tag "Legacy site import 2026-10-09", 4 refused by Kit's suppression list); the missing 2026-10-07 Daily Provocation added; supplier forms: table script supabase/migrations/0003_legacy_vendor_intake.sql and scripts/import-legacy-vendor-intake.ts ready (owner: supplier forms to Supabase, everything else stays in the backup). Left: restore the paused Supabase project, run 0001 to 0003, run the import; the few reactions/ratings (optional). Then rotate the database password (it was pasted in a chat) and remove LEGACY_DATABASE_URL.</t>
         </is>
       </c>
       <c r="E42" s="14" t="inlineStr">
@@ -1976,7 +1976,7 @@
       <c r="A43" s="4" t="n"/>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>Run the database scripts once, in order</t>
+          <t>Restore the Supabase project first: it was paused (2026-10-09, its address no longer resolves), so every member feature, comment and reaction is off until someone with the Supabase account clicks "Restore project"</t>
         </is>
       </c>
       <c r="C43" s="15" t="inlineStr">
@@ -1986,7 +1986,7 @@
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>(supabase/migrations/0001_member_features.sql, then 0002_blog_engagement.sql for essay comments, reactions, ratings and micro-commitments; 0001: highlights, referral codes/referrals, Clock Keeper responses, post-intervention, friend gate, PRI calibrations, all with row-level security) in Supabase: SQL Editor &gt; New query &gt; paste &gt; Run. Also in Supabase: Authentication &gt; URL Configuration &gt; Site URL https://tonygreenberg.com and Redirect URLs https://tonygreenberg.com/auth/callback, https://*--tonygreenberg-website.netlify.app/auth/callback, http://localhost:3000/auth/callback. Then set NEXT_PUBLIC_SUPABASE_URL, NEXT_PUBLIC_SUPABASE_ANON_KEY, SUPABASE_SERVICE_ROLE_KEY, ADMIN_EMAILS in Netlify.</t>
+          <t>Then run the database scripts once, in order (supabase/migrations/0001_member_features.sql, then 0002_blog_engagement.sql, then 0003_legacy_vendor_intake.sql for essay comments, reactions, ratings and micro-commitments; 0001: highlights, referral codes/referrals, Clock Keeper responses, post-intervention, friend gate, PRI calibrations, all with row-level security) in Supabase: SQL Editor &gt; New query &gt; paste &gt; Run. Also in Supabase: Authentication &gt; URL Configuration &gt; Site URL https://tonygreenberg.com and Redirect URLs https://tonygreenberg.com/auth/callback, https://*--tonygreenberg-website.netlify.app/auth/callback, http://localhost:3000/auth/callback. Then set NEXT_PUBLIC_SUPABASE_URL, NEXT_PUBLIC_SUPABASE_ANON_KEY, SUPABASE_SERVICE_ROLE_KEY, ADMIN_EMAILS in Netlify.</t>
         </is>
       </c>
       <c r="E43" s="14" t="inlineStr">
@@ -8413,7 +8413,7 @@
       <c r="A331" s="4" t="n"/>
       <c r="B331" s="4" t="inlineStr">
         <is>
-          <t>DNS cutover, legacy app decommissioned only after a stable overlap window</t>
+          <t>DNS cutover, legacy app decommissioned only after a stable overlap window Checked 2026-10-09 (owner wants to go live and switch off Manus)</t>
         </is>
       </c>
       <c r="C331" s="15" t="inlineStr">
@@ -8421,7 +8421,11 @@
           <t>Remaining</t>
         </is>
       </c>
-      <c r="D331" s="4" t="inlineStr"/>
+      <c r="D331" s="4" t="inlineStr">
+        <is>
+          <t>DNS for tonygreenberg.com is at Hostinger (name servers ns1/ns2.dns-parking.com); www is a CNAME to cname.manus.space, the bare domain points at Manus's addresses (104.19.168.112 / .169.112); the Netlify site tonygreenberg-website has no custom domain yet (production branch main). Order: (1) merge the three open pull requests into main and check the Netlify copy; (2) restore Supabase and run 0001 to 0003, or launch without member features (they say "isn't available just now"); (3) owner sign-off; (4) add tonygreenberg.com + www in Netlify (Domain management), then at Hostinger point the bare domain at Netlify (A record 75.2.60.5, or Netlify DNS) and www CNAME at tonygreenberg-website.netlify.app; Netlify issues the HTTPS certificate; (5) re-run scripts/check-search-console-urls.ts https://tonygreenberg.com and submit the sitemap in Search Console; (6) only after a few stable days: switch off the Manus site (the database is already backed up, docs/ai/project_legacy_database.md) and rotate the old database password.</t>
+        </is>
+      </c>
       <c r="E331" s="14" t="inlineStr">
         <is>
           <t>Phase 14 — QA &amp; Launch</t>
@@ -8540,7 +8544,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Connection details in .env.local (LEGACY_DATABASE_URL). Done: read-only check of all 56 tables and a full private backup (75,128 rows) to ~/Desktop/tonyg-site-backups/legacy-db-export-2026-10-09/ on the webmaster's Mac (personal data: never commit); most rows are the Manus agent's automated tests (details: docs/ai/project_legacy_database.md); the 198 short share links /s/&lt;code&gt; now redirect (src/lib/content/short-links.ts; 196 land on a page, 2 targets don't exist on live either). Left (needs a yes): add the 36 real email subscribers to Kit (may send Kit's confirmation email); copy the handful of real reactions/ratings/commitment into Supabase after the scripts below are run; decide whether the ~24 real assessment results, ~17 PRI consents, 2 manifesto responses, 8 supplier forms and 1 Cheshire submission stay in the backup only. Then rotate the database password (it was pasted in a chat) and remove LEGACY_DATABASE_URL.</t>
+          <t>Connection details in .env.local (LEGACY_DATABASE_URL). Done: read-only check of all 56 tables and a full private backup (75,128 rows) to ~/Desktop/tonyg-site-backups/legacy-db-export-2026-10-09/ on the webmaster's Mac (personal data: never commit); most rows are the Manus agent's automated tests (details: docs/ai/project_legacy_database.md); the 198 short share links /s/&lt;code&gt; now redirect (src/lib/content/short-links.ts; 196 land on a page, 2 targets don't exist on live either). Done 2026-10-09 (owner said yes): email subscribers in Kit with no email sent (5 already there, 27 added on the new tag "Legacy site import 2026-10-09", 4 refused by Kit's suppression list); the missing 2026-10-07 Daily Provocation added; supplier forms: table script supabase/migrations/0003_legacy_vendor_intake.sql and scripts/import-legacy-vendor-intake.ts ready (owner: supplier forms to Supabase, everything else stays in the backup). Left: restore the paused Supabase project, run 0001 to 0003, run the import; the few reactions/ratings (optional). Then rotate the database password (it was pasted in a chat) and remove LEGACY_DATABASE_URL.</t>
         </is>
       </c>
       <c r="E4" s="14" t="inlineStr">
@@ -8553,7 +8557,7 @@
       <c r="A5" s="4" t="n"/>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Run the database scripts once, in order</t>
+          <t>Restore the Supabase project first: it was paused (2026-10-09, its address no longer resolves), so every member feature, comment and reaction is off until someone with the Supabase account clicks "Restore project"</t>
         </is>
       </c>
       <c r="C5" s="15" t="inlineStr">
@@ -8563,7 +8567,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>(supabase/migrations/0001_member_features.sql, then 0002_blog_engagement.sql for essay comments, reactions, ratings and micro-commitments; 0001: highlights, referral codes/referrals, Clock Keeper responses, post-intervention, friend gate, PRI calibrations, all with row-level security) in Supabase: SQL Editor &gt; New query &gt; paste &gt; Run. Also in Supabase: Authentication &gt; URL Configuration &gt; Site URL https://tonygreenberg.com and Redirect URLs https://tonygreenberg.com/auth/callback, https://*--tonygreenberg-website.netlify.app/auth/callback, http://localhost:3000/auth/callback. Then set NEXT_PUBLIC_SUPABASE_URL, NEXT_PUBLIC_SUPABASE_ANON_KEY, SUPABASE_SERVICE_ROLE_KEY, ADMIN_EMAILS in Netlify.</t>
+          <t>Then run the database scripts once, in order (supabase/migrations/0001_member_features.sql, then 0002_blog_engagement.sql, then 0003_legacy_vendor_intake.sql for essay comments, reactions, ratings and micro-commitments; 0001: highlights, referral codes/referrals, Clock Keeper responses, post-intervention, friend gate, PRI calibrations, all with row-level security) in Supabase: SQL Editor &gt; New query &gt; paste &gt; Run. Also in Supabase: Authentication &gt; URL Configuration &gt; Site URL https://tonygreenberg.com and Redirect URLs https://tonygreenberg.com/auth/callback, https://*--tonygreenberg-website.netlify.app/auth/callback, http://localhost:3000/auth/callback. Then set NEXT_PUBLIC_SUPABASE_URL, NEXT_PUBLIC_SUPABASE_ANON_KEY, SUPABASE_SERVICE_ROLE_KEY, ADMIN_EMAILS in Netlify.</t>
         </is>
       </c>
       <c r="E5" s="14" t="inlineStr">
@@ -8982,7 +8986,7 @@
       <c r="A27" s="4" t="n"/>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>DNS cutover, legacy app decommissioned only after a stable overlap window</t>
+          <t>DNS cutover, legacy app decommissioned only after a stable overlap window Checked 2026-10-09 (owner wants to go live and switch off Manus)</t>
         </is>
       </c>
       <c r="C27" s="15" t="inlineStr">
@@ -8990,7 +8994,11 @@
           <t>Remaining</t>
         </is>
       </c>
-      <c r="D27" s="4" t="inlineStr"/>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>DNS for tonygreenberg.com is at Hostinger (name servers ns1/ns2.dns-parking.com); www is a CNAME to cname.manus.space, the bare domain points at Manus's addresses (104.19.168.112 / .169.112); the Netlify site tonygreenberg-website has no custom domain yet (production branch main). Order: (1) merge the three open pull requests into main and check the Netlify copy; (2) restore Supabase and run 0001 to 0003, or launch without member features (they say "isn't available just now"); (3) owner sign-off; (4) add tonygreenberg.com + www in Netlify (Domain management), then at Hostinger point the bare domain at Netlify (A record 75.2.60.5, or Netlify DNS) and www CNAME at tonygreenberg-website.netlify.app; Netlify issues the HTTPS certificate; (5) re-run scripts/check-search-console-urls.ts https://tonygreenberg.com and submit the sitemap in Search Console; (6) only after a few stable days: switch off the Manus site (the database is already backed up, docs/ai/project_legacy_database.md) and rotate the old database password.</t>
+        </is>
+      </c>
       <c r="E27" s="14" t="inlineStr">
         <is>
           <t>Phase 14 — QA &amp; Launch</t>

</xml_diff>

<commit_message>
Project file: Sanity webhook live, members' cross-device progress tested, PRs 7 and 8 merged
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Migration-Status-Report.xlsx
+++ b/Migration-Status-Report.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Full Detail'!$A$1:$D$337</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Remaining Work'!$A$1:$D$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Remaining Work'!$A$1:$D$25</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1953,17 +1953,17 @@
       <c r="A42" s="4" t="n"/>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>Set SANITY_WEBHOOK_SECRET (found 2026-10-09)</t>
-        </is>
-      </c>
-      <c r="C42" s="15" t="inlineStr">
-        <is>
-          <t>Remaining</t>
+          <t>Set SANITY_WEBHOOK_SECRET (found 2026-10-09, done 2026-10-10)</t>
+        </is>
+      </c>
+      <c r="C42" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>missing in Netlify and .env.local, so Sanity's publish webhook to /api/revalidate is refused and edits appear only after the 60-second refresh. Create the webhook secret in Sanity (manage &gt; API &gt; Webhooks) and add it to Netlify. 2026-10-10: a random 64-character secret is now in .env.local and in Netlify (secret; production, deploy previews, branch deploys). /api/revalidate checked on a local production build: correctly signed request 200 revalidated, wrong signature 401. Left (Sanity dashboard, the site's Sanity token can't manage webhooks): sanity.io/manage &gt; project a3q1cyqs &gt; API &gt; Webhooks &gt; Create: URL https://tonygreenberg-website.netlify.app/api/revalidate (switch to https://tonygreenberg.com/api/revalidate at cutover), dataset production, trigger on create/update/delete, HTTP method POST, secret = the SANITY_WEBHOOK_SECRET value in .env.local.</t>
+          <t>missing in Netlify and .env.local, so Sanity's publish webhook to /api/revalidate is refused and edits appear only after the 60-second refresh. Create the webhook secret in Sanity (manage &gt; API &gt; Webhooks) and add it to Netlify. 2026-10-10: a random 64-character secret is now in .env.local and in Netlify (secret; production, deploy previews, branch deploys). /api/revalidate checked on a local production build: correctly signed request 200 revalidated, wrong signature 401. Left (Sanity dashboard, the site's Sanity token can't manage webhooks): sanity.io/manage &gt; project a3q1cyqs &gt; API &gt; Webhooks &gt; Create: URL https://tonygreenberg-website.netlify.app/api/revalidate (switch to https://tonygreenberg.com/api/revalidate at cutover), dataset production, trigger on create/update/delete, HTTP method POST, secret = the SANITY_WEBHOOK_SECRET value in .env.local. Done 2026-10-10: the owner created the webhook in Sanity (name tonygreenberg, URL https://tonygreenberg-website.netlify.app/api/revalidate, dataset production, enabled), with the secret from .env.local. At cutover: change its URL to https://tonygreenberg.com/api/revalidate.</t>
         </is>
       </c>
       <c r="E42" s="14" t="inlineStr">
@@ -2055,7 +2055,7 @@
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>Built: tables assessment_results and journey_progress (supabase/migrations/0005_assessments.sql, which also copies the old site's 24 real quiz results; its 1,008 test rows are skipped), server actions src/app/assessments/actions.ts, wired into the shared quiz-finish helpers so every quiz's finish and result is saved, and signed-in members' Journey Tracker progress follows them across devices. Checked: type check, lint, build. Left: run 0005 in Supabase &gt; SQL Editor (after 0004), then finish one quiz on a deploy preview and see the row in the Table Editor (needs the secret key fixed). Done 2026-10-10: 0005 run (tables created, 24 real old results copied: the-mirror 10, dharma-finder 6, consciousness-scale 4, grant-study 2, find-your-therapy 2). Tested in Chromium on a local production build: finishing /find-your-me saved one row with its result ("The Systems Architect"). Found and fixed on the way: the two save calls per finish ran one after another (~2.7 s each), so leaving within ~5 s lost the result text; now merged in the browser into one call (src/lib/assessments/record-finish.ts, 1.5 s window) and the server does one read instead of two (1.5 s). Test rows deleted. Not yet: the journey sync for a signed-in member (needs a real account).</t>
+          <t>Built: tables assessment_results and journey_progress (supabase/migrations/0005_assessments.sql, which also copies the old site's 24 real quiz results; its 1,008 test rows are skipped), server actions src/app/assessments/actions.ts, wired into the shared quiz-finish helpers so every quiz's finish and result is saved, and signed-in members' Journey Tracker progress follows them across devices. Checked: type check, lint, build. Left: run 0005 in Supabase &gt; SQL Editor (after 0004), then finish one quiz on a deploy preview and see the row in the Table Editor (needs the secret key fixed). Done 2026-10-10: 0005 run (tables created, 24 real old results copied: the-mirror 10, dharma-finder 6, consciousness-scale 4, grant-study 2, find-your-therapy 2). Tested in Chromium on a local production build: finishing /find-your-me saved one row with its result ("The Systems Architect"). Found and fixed on the way: the two save calls per finish ran one after another (~2.7 s each), so leaving within ~5 s lost the result text; now merged in the browser into one call (src/lib/assessments/record-finish.ts, 1.5 s window) and the server does one read instead of two (1.5 s). Test rows deleted. Signed-in sync tested 2026-10-10 with a temporary account (created and deleted through the admin API): device A finished /find-your-me, the account got the journey_progress row and its result; a fresh browser (device B) signed in and its Journey list showed find-your-me.</t>
         </is>
       </c>
       <c r="E46" s="14" t="inlineStr">
@@ -8598,7 +8598,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -8649,7 +8649,7 @@
       <c r="A3" s="4" t="n"/>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Set SANITY_WEBHOOK_SECRET (found 2026-10-09)</t>
+          <t>Old site's forms still simplified (decision, 2026-10-10)</t>
         </is>
       </c>
       <c r="C3" s="15" t="inlineStr">
@@ -8659,7 +8659,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>missing in Netlify and .env.local, so Sanity's publish webhook to /api/revalidate is refused and edits appear only after the 60-second refresh. Create the webhook secret in Sanity (manage &gt; API &gt; Webhooks) and add it to Netlify. 2026-10-10: a random 64-character secret is now in .env.local and in Netlify (secret; production, deploy previews, branch deploys). /api/revalidate checked on a local production build: correctly signed request 200 revalidated, wrong signature 401. Left (Sanity dashboard, the site's Sanity token can't manage webhooks): sanity.io/manage &gt; project a3q1cyqs &gt; API &gt; Webhooks &gt; Create: URL https://tonygreenberg-website.netlify.app/api/revalidate (switch to https://tonygreenberg.com/api/revalidate at cutover), dataset production, trigger on create/update/delete, HTTP method POST, secret = the SANITY_WEBHOOK_SECRET value in .env.local.</t>
+          <t>Full map in docs/ai/project_legacy_database.md ("Everything the old database did"). These now open an email or stay in the browser instead of saving: PRI consent (~17 real rows on the old site, the biggest gap), Living Declaration, PRI corrections, Cheshire stories, Facilitator Index, spam reports. Owner chose not to change them for now; each can save to Supabase the same way if wanted.</t>
         </is>
       </c>
       <c r="E3" s="14" t="inlineStr">
@@ -8669,76 +8669,76 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="n"/>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Old site's forms still simplified (decision, 2026-10-10)</t>
-        </is>
-      </c>
-      <c r="C4" s="15" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>Phase 4 — Marketing Core Pages (30 routes)</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="n"/>
+      <c r="C4" s="11" t="n"/>
+      <c r="D4" s="12" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="n"/>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>/shop, /payment-success, /payment-cancel</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>defer: these are Stripe-backed; flag for the later billing-migration phase, do not port checkout logic yet, static/informational content only if ported now</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="inlineStr">
+        <is>
+          <t>Phase 4 — Marketing Core Pages (30 routes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Phase 11 — Code MCP Server — REBUILT (2026-09-29)</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="n"/>
+      <c r="C6" s="11" t="n"/>
+      <c r="D6" s="12" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="n"/>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Set GITHUB_TOKEN, MCP_ADMIN_USERS, MCP_LOGIN_PASSWORD, MCP_OAUTH_SECRET, MCP_SITE_ORIGIN, MCP_PUBLIC_ORIGIN in Netlify (done) (checked 2026-…</t>
+        </is>
+      </c>
+      <c r="C7" s="15" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Full map in docs/ai/project_legacy_database.md ("Everything the old database did"). These now open an email or stay in the browser instead of saving: PRI consent (~17 real rows on the old site, the biggest gap), Living Declaration, PRI corrections, Cheshire stories, Facilitator Index, spam reports. Owner chose not to change them for now; each can save to Supabase the same way if wanted.</t>
-        </is>
-      </c>
-      <c r="E4" s="14" t="inlineStr">
-        <is>
-          <t>Phase 2 — Supabase</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="10" t="inlineStr">
-        <is>
-          <t>Phase 4 — Marketing Core Pages (30 routes)</t>
-        </is>
-      </c>
-      <c r="B5" s="11" t="n"/>
-      <c r="C5" s="11" t="n"/>
-      <c r="D5" s="12" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="n"/>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>/shop, /payment-success, /payment-cancel</t>
-        </is>
-      </c>
-      <c r="C6" s="16" t="inlineStr">
-        <is>
-          <t>Deferred</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>defer: these are Stripe-backed; flag for the later billing-migration phase, do not port checkout logic yet, static/informational content only if ported now</t>
-        </is>
-      </c>
-      <c r="E6" s="14" t="inlineStr">
-        <is>
-          <t>Phase 4 — Marketing Core Pages (30 routes)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>10-07: all already set in Netlify). Left: connect Claude.ai to /api/mcp for real, and verify the GitHub flow end to end (branch → PR → deploy preview → publish_changes) against a real PR.</t>
+        </is>
+      </c>
+      <c r="E7" s="14" t="inlineStr">
         <is>
           <t>Phase 11 — Code MCP Server — REBUILT (2026-09-29)</t>
         </is>
       </c>
-      <c r="B7" s="11" t="n"/>
-      <c r="C7" s="11" t="n"/>
-      <c r="D7" s="12" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n"/>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Set GITHUB_TOKEN, MCP_ADMIN_USERS, MCP_LOGIN_PASSWORD, MCP_OAUTH_SECRET, MCP_SITE_ORIGIN, MCP_PUBLIC_ORIGIN in Netlify (done) (checked 2026-…</t>
+          <t>Commit a team-wide .mcp.json (URL only) once the production URL is settled.</t>
         </is>
       </c>
       <c r="C8" s="15" t="inlineStr">
@@ -8746,11 +8746,7 @@
           <t>Remaining</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>10-07: all already set in Netlify). Left: connect Claude.ai to /api/mcp for real, and verify the GitHub flow end to end (branch → PR → deploy preview → publish_changes) against a real PR.</t>
-        </is>
-      </c>
+      <c r="D8" s="4" t="inlineStr"/>
       <c r="E8" s="14" t="inlineStr">
         <is>
           <t>Phase 11 — Code MCP Server — REBUILT (2026-09-29)</t>
@@ -8761,7 +8757,7 @@
       <c r="A9" s="4" t="n"/>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Commit a team-wide .mcp.json (URL only) once the production URL is settled.</t>
+          <t>Blocked on you (Google)</t>
         </is>
       </c>
       <c r="C9" s="15" t="inlineStr">
@@ -8769,7 +8765,11 @@
           <t>Remaining</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr"/>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>create a GOOGLE_API_KEY in Google Cloud (project of the vcos-ga4-reader service account, where the PageSpeed Insights API is already on), restricted to the PageSpeed Insights API, then add it to .env.local and Netlify. Creating it from here was blocked by the session's safety check (it would use the service account's credentials to change the Cloud project). Note lighthouse_check_page may time out on Netlify (10 s function limit on the free plan).</t>
+        </is>
+      </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
           <t>Phase 11 — Code MCP Server — REBUILT (2026-09-29)</t>
@@ -8780,7 +8780,7 @@
       <c r="A10" s="4" t="n"/>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Blocked on you (Google)</t>
+          <t>Test the new review end to end on a deploy preview</t>
         </is>
       </c>
       <c r="C10" s="15" t="inlineStr">
@@ -8790,7 +8790,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>create a GOOGLE_API_KEY in Google Cloud (project of the vcos-ga4-reader service account, where the PageSpeed Insights API is already on), restricted to the PageSpeed Insights API, then add it to .env.local and Netlify. Creating it from here was blocked by the session's safety check (it would use the service account's credentials to change the Cloud project). Note lighthouse_check_page may time out on Netlify (10 s function limit on the free plan).</t>
+          <t>(needs a yes, it opens a real pull request): one throwaway change from Claude.ai or ChatGPT: start (unclear request, so the confirm step shows), confirm, edit, review card, screenshots, upload link, then discard.</t>
         </is>
       </c>
       <c r="E10" s="14" t="inlineStr">
@@ -8800,43 +8800,43 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="n"/>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>Test the new review end to end on a deploy preview</t>
-        </is>
-      </c>
-      <c r="C11" s="15" t="inlineStr">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="n"/>
+      <c r="C11" s="11" t="n"/>
+      <c r="D11" s="12" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="n"/>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Lighthouse pass (performance/accessibility/SEO) on top 20 pages by traffic 2026-09-30, 20 key pages (no traffic data yet), local production …</t>
+        </is>
+      </c>
+      <c r="C12" s="15" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>(needs a yes, it opens a real pull request): one throwaway change from Claude.ai or ChatGPT: start (unclear request, so the confirm step shows), confirm, edit, review card, screenshots, upload link, then discard.</t>
-        </is>
-      </c>
-      <c r="E11" s="14" t="inlineStr">
-        <is>
-          <t>Phase 11 — Code MCP Server — REBUILT (2026-09-29)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="10" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>build, mobile: averages performance 87, accessibility 99→100, best practices 100, SEO 92→100, CLS 0 everywhere. Fixed: public/robots.txt had an LLMs: line (not a real directive) that made Google treat the whole file as invalid, now a comment; h3/h4 headings skipping a level on /assessments, /kava, /peptide-watch (same look, right tag); the Kava and /attention-theft back-arrow links had no accessible name on phones; two small phone-width contrast misses. Left: performance is local-machine only (±10-15 points, see CONTRIBUTING.md); the slowest were / 76 (LCP 5.2 s), /psychedelic-readiness-index 82, /iboga-ibogaine 83. Re-run against the Netlify deploy before launch. 2026-10-06 re-run against the Netlify deploy (14 key pages, mobile): accessibility 100 and CLS 0 on every page, SEO clean (only the expected netlify.app noindex), performance 77-97 held back by 3-4 s LCP. Fixed: all 21 hero images moved off the deprecated priority prop to fetchPriority="high" + loading="eager" (Next 16); /iboga-ibogaine hero and the first card on /blog and category pages no longer lazy-loaded; sizes on the Four Doors cards (~150 KiB per page), /humanos diagram (~100 KiB) and /about headshot; urlFor no longer imports the Sanity client, so ~115 KB of Sanity client code stopped loading on / and /blog; React hydration error #418 on / and /blog (post dates) gone, checked in two time zones; /blog is static again; empty icon &lt;th&gt;s on /iboga-ibogaine labelled; category page reads use sanityFetch(). Left: se</t>
+        </is>
+      </c>
+      <c r="E12" s="14" t="inlineStr">
         <is>
           <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n"/>
-      <c r="C12" s="11" t="n"/>
-      <c r="D12" s="12" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n"/>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Lighthouse pass (performance/accessibility/SEO) on top 20 pages by traffic 2026-09-30, 20 key pages (no traffic data yet), local production …</t>
+          <t>SEO audit items needing a yes (2026-10-06)</t>
         </is>
       </c>
       <c r="C13" s="15" t="inlineStr">
@@ -8846,7 +8846,7 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>build, mobile: averages performance 87, accessibility 99→100, best practices 100, SEO 92→100, CLS 0 everywhere. Fixed: public/robots.txt had an LLMs: line (not a real directive) that made Google treat the whole file as invalid, now a comment; h3/h4 headings skipping a level on /assessments, /kava, /peptide-watch (same look, right tag); the Kava and /attention-theft back-arrow links had no accessible name on phones; two small phone-width contrast misses. Left: performance is local-machine only (±10-15 points, see CONTRIBUTING.md); the slowest were / 76 (LCP 5.2 s), /psychedelic-readiness-index 82, /iboga-ibogaine 83. Re-run against the Netlify deploy before launch. 2026-10-06 re-run against the Netlify deploy (14 key pages, mobile): accessibility 100 and CLS 0 on every page, SEO clean (only the expected netlify.app noindex), performance 77-97 held back by 3-4 s LCP. Fixed: all 21 hero images moved off the deprecated priority prop to fetchPriority="high" + loading="eager" (Next 16); /iboga-ibogaine hero and the first card on /blog and category pages no longer lazy-loaded; sizes on the Four Doors cards (~150 KiB per page), /humanos diagram (~100 KiB) and /about headshot; urlFor no longer imports the Sanity client, so ~115 KB of Sanity client code stopped loading on / and /blog; React hydration error #418 on / and /blog (post dates) gone, checked in two time zones; /blog is static again; empty icon &lt;th&gt;s on /iboga-ibogaine labelled; category page reads use sanityFetch(). Left: se</t>
+          <t>the pack's new copy (homepage title/description, five-cups title, description, short answer, FAQ, heading rewrites, entity statement, newsletter block, author box, health disclaimer, COA wording); "Further Reading" shown twice on posts (merge the lists?); long post title (84 chars), homepage description length and obsolete keywords tag, slugs (/blog/five-cups, the -2 slug; would need redirects), "Six lenses" over four cards, sources for health claims and proof for "$10B+", "Certified B Corp", "Validity: 91", legal review of the homepage Case File banner, ABIT waitlist disclosures, one contact email, the two one-post categories, fewer homepage CTAs / email signup / table of contents / explaining "COA".</t>
         </is>
       </c>
       <c r="E13" s="14" t="inlineStr">
@@ -8859,7 +8859,7 @@
       <c r="A14" s="4" t="n"/>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>SEO audit items needing a yes (2026-10-06)</t>
+          <t>Connect Google Search Console + GA4 to the new deployment on day one of cutover</t>
         </is>
       </c>
       <c r="C14" s="15" t="inlineStr">
@@ -8867,11 +8867,7 @@
           <t>Remaining</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>the pack's new copy (homepage title/description, five-cups title, description, short answer, FAQ, heading rewrites, entity statement, newsletter block, author box, health disclaimer, COA wording); "Further Reading" shown twice on posts (merge the lists?); long post title (84 chars), homepage description length and obsolete keywords tag, slugs (/blog/five-cups, the -2 slug; would need redirects), "Six lenses" over four cards, sources for health claims and proof for "$10B+", "Certified B Corp", "Validity: 91", legal review of the homepage Case File banner, ABIT waitlist disclosures, one contact email, the two one-post categories, fewer homepage CTAs / email signup / table of contents / explaining "COA".</t>
-        </is>
-      </c>
+      <c r="D14" s="4" t="inlineStr"/>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
@@ -8879,39 +8875,43 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="n"/>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>Connect Google Search Console + GA4 to the new deployment on day one of cutover</t>
-        </is>
-      </c>
-      <c r="C15" s="15" t="inlineStr">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>Phase 13 — Images Needed in Sanity</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="n"/>
+      <c r="C15" s="11" t="n"/>
+      <c r="D15" s="12" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="n"/>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Site-wide: logo (light + dark) beyond the current text wordmark</t>
+        </is>
+      </c>
+      <c r="C16" s="15" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr"/>
-      <c r="E15" s="14" t="inlineStr">
-        <is>
-          <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="10" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>(Default/fallback OG image 1200×630 exists: public/images/default-og.png, checked 2026-10-02.)</t>
+        </is>
+      </c>
+      <c r="E16" s="14" t="inlineStr">
         <is>
           <t>Phase 13 — Images Needed in Sanity</t>
         </is>
       </c>
-      <c r="B16" s="11" t="n"/>
-      <c r="C16" s="11" t="n"/>
-      <c r="D16" s="12" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n"/>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Site-wide: logo (light + dark) beyond the current text wordmark</t>
+          <t>92 posts still need a real, unique hero image</t>
         </is>
       </c>
       <c r="C17" s="15" t="inlineStr">
@@ -8921,7 +8921,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>(Default/fallback OG image 1200×630 exists: public/images/default-og.png, checked 2026-10-02.)</t>
+          <t>(down from 99). Tracked one row per post, with a suggested image-generation prompt, in BLOG-IMAGE-BRIEFS.md — work through that file and check items off there, not here. No image-generation tool was connected in this environment as of this writing; either connect one (e.g. an MCP image-gen extension), source these manually/with a designer then upload via Sanity Studio (/studio), or re-check the live legacy site periodically per the correction note above.</t>
         </is>
       </c>
       <c r="E17" s="14" t="inlineStr">
@@ -8934,7 +8934,7 @@
       <c r="A18" s="4" t="n"/>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>92 posts still need a real, unique hero image</t>
+          <t>Assessment result-screen background art (flagged in STATUS.md as a known gap</t>
         </is>
       </c>
       <c r="C18" s="15" t="inlineStr">
@@ -8944,7 +8944,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>(down from 99). Tracked one row per post, with a suggested image-generation prompt, in BLOG-IMAGE-BRIEFS.md — work through that file and check items off there, not here. No image-generation tool was connected in this environment as of this writing; either connect one (e.g. an MCP image-gen extension), source these manually/with a designer then upload via Sanity Studio (/studio), or re-check the live legacy site periodically per the correction note above.</t>
+          <t>18/20 assessments currently have plain black backgrounds; sourcing themed art here also closes that gap)</t>
         </is>
       </c>
       <c r="E18" s="14" t="inlineStr">
@@ -8954,43 +8954,43 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="n"/>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>Assessment result-screen background art (flagged in STATUS.md as a known gap</t>
-        </is>
-      </c>
-      <c r="C19" s="15" t="inlineStr">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>Phase 14 — QA &amp; Launch</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="n"/>
+      <c r="C19" s="11" t="n"/>
+      <c r="D19" s="12" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="n"/>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Mobile responsive pass on every ported section</t>
+        </is>
+      </c>
+      <c r="C20" s="15" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>18/20 assessments currently have plain black backgrounds; sourcing themed art here also closes that gap)</t>
-        </is>
-      </c>
-      <c r="E19" s="14" t="inlineStr">
-        <is>
-          <t>Phase 13 — Images Needed in Sanity</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="10" t="inlineStr">
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-29: no page scrolls sideways at 375px any more (114 pages checked in Chrome: every unique page plus 3 of each templated set like blog posts and coffees). Fixed: BrewSoul NextSteps forced 3 columns (and used an inline style), charity-scorecard tab row, /brewsoul/browse filter dropdowns, /the-philosophy hero glow. Still to check by hand: 44px tap targets and Safari iOS. 2026-09-30: 44px tap targets on phones for the shared header, footer, BrewSoul/Kava/HumanOS menus and ~100 standalone links (undersized targets 1,904 → 578; the rest are 24-43px pills/chips that meet WCAG 2.2 AA). axe target-size (WCAG 2.2 AA, with its spacing exception): 0 failures on 114 pages. Safari/iPhone (WebKit, iPhone 14 emulation): all 114 pages load, no sideways scroll, no JS errors; form fields under 16px (iOS zoom-on-tap) fixed site-wide in globals.css. Still to check on a real iPhone: BrewSoul's bottom journey bar showed page text through it in headless WebKit only (taps hit the bar correctly; Chrome renders it solid). Fixed 2026-10-09: the bar is now solid (bg-[#2C1810], was 92% plus backdrop-blur-md), so nothing can show through even where the blur isn't drawn; checked in WebKit (iPhone 13 profile) and Chrome: background rgb(44, 24, 16), no text behind the buttons. A real iPhone check is still part of Phase 14.</t>
+        </is>
+      </c>
+      <c r="E20" s="14" t="inlineStr">
         <is>
           <t>Phase 14 — QA &amp; Launch</t>
         </is>
       </c>
-      <c r="B20" s="11" t="n"/>
-      <c r="C20" s="11" t="n"/>
-      <c r="D20" s="12" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n"/>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Mobile responsive pass on every ported section</t>
+          <t>No dead-end pages (every page links to 2+ others)</t>
         </is>
       </c>
       <c r="C21" s="15" t="inlineStr">
@@ -9000,7 +9000,7 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>2026-09-29: no page scrolls sideways at 375px any more (114 pages checked in Chrome: every unique page plus 3 of each templated set like blog posts and coffees). Fixed: BrewSoul NextSteps forced 3 columns (and used an inline style), charity-scorecard tab row, /brewsoul/browse filter dropdowns, /the-philosophy hero glow. Still to check by hand: 44px tap targets and Safari iOS. 2026-09-30: 44px tap targets on phones for the shared header, footer, BrewSoul/Kava/HumanOS menus and ~100 standalone links (undersized targets 1,904 → 578; the rest are 24-43px pills/chips that meet WCAG 2.2 AA). axe target-size (WCAG 2.2 AA, with its spacing exception): 0 failures on 114 pages. Safari/iPhone (WebKit, iPhone 14 emulation): all 114 pages load, no sideways scroll, no JS errors; form fields under 16px (iOS zoom-on-tap) fixed site-wide in globals.css. Still to check on a real iPhone: BrewSoul's bottom journey bar showed page text through it in headless WebKit only (taps hit the bar correctly; Chrome renders it solid). Fixed 2026-10-09: the bar is now solid (bg-[#2C1810], was 92% plus backdrop-blur-md), so nothing can show through even where the blur isn't drawn; checked in WebKit (iPhone 13 profile) and Chrome: background rgb(44, 24, 16), no text behind the buttons. A real iPhone check is still part of Phase 14.</t>
+          <t>same bar as legacy MASTER_QUALITY_PROMPT.md 2026-09-30 scan (496 sitemap pages, header/footer links not counted): every page has a way home (the 6 HumanOS pages had none, in legacy too; added a "← TonyGreenberg.com" footer link). ~17 quiz pages only look like dead ends on their intro screen; their result screens link to related assessments. Left for a content decision: ~20 marketing pages (/akbar, /amplifier, /diamond-cut, /ecosystem, /engage, /engine-room, /intel, /invest, /pick-up-the-phone, /protecting-your-business, /published, /speaking, /the-nightstand, /the-territory, /the-web, /under-nda, /pri-calibration, /charity-scorecard and its detail pages) link to only 0-1 other page in their content. The port matches legacy there (legacy was just as sparse), so adding related links is new content and needs the owner's yes.</t>
         </is>
       </c>
       <c r="E21" s="14" t="inlineStr">
@@ -9013,7 +9013,7 @@
       <c r="A22" s="4" t="n"/>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>No dead-end pages (every page links to 2+ others)</t>
+          <t>Cross-browser check (Safari iOS in particular, per legacy performance notes) 2026-10-06 WebKit pass (Playwright WebKit, iPhone 13 profile, 1…</t>
         </is>
       </c>
       <c r="C22" s="15" t="inlineStr">
@@ -9023,7 +9023,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>same bar as legacy MASTER_QUALITY_PROMPT.md 2026-09-30 scan (496 sitemap pages, header/footer links not counted): every page has a way home (the 6 HumanOS pages had none, in legacy too; added a "← TonyGreenberg.com" footer link). ~17 quiz pages only look like dead ends on their intro screen; their result screens link to related assessments. Left for a content decision: ~20 marketing pages (/akbar, /amplifier, /diamond-cut, /ecosystem, /engage, /engine-room, /intel, /invest, /pick-up-the-phone, /protecting-your-business, /published, /speaking, /the-nightstand, /the-territory, /the-web, /under-nda, /pri-calibration, /charity-scorecard and its detail pages) link to only 0-1 other page in their content. The port matches legacy there (legacy was just as sparse), so adding related links is new content and needs the owner's yes.</t>
+          <t>52 pages: every unique page plus 3 of each templated set, production build): no page pans sideways, no failed requests, no JS errors. Found and fixed on the way: upgrade-insecure-requests in the new CSP made Safari fetch every stylesheet and font over https on localhost (dropped; the site is HTTPS-only via HSTS anyway), and .toLocaleString() without a locale caused a hydration error on /brewsoul/chains in Safari (all number formatting now en-US). Left: a check on a real iPhone (Phase 14).</t>
         </is>
       </c>
       <c r="E22" s="14" t="inlineStr">
@@ -9036,7 +9036,7 @@
       <c r="A23" s="4" t="n"/>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Cross-browser check (Safari iOS in particular, per legacy performance notes) 2026-10-06 WebKit pass (Playwright WebKit, iPhone 13 profile, 1…</t>
+          <t>Remove noindex only when sign-off is given</t>
         </is>
       </c>
       <c r="C23" s="15" t="inlineStr">
@@ -9046,7 +9046,7 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>52 pages: every unique page plus 3 of each templated set, production build): no page pans sideways, no failed requests, no JS errors. Found and fixed on the way: upgrade-insecure-requests in the new CSP made Safari fetch every stylesheet and font over https on localhost (dropped; the site is HTTPS-only via HSTS anyway), and .toLocaleString() without a locale caused a hydration error on /brewsoul/chains in Safari (all number formatting now en-US). Left: a check on a real iPhone (Phase 14).</t>
+          <t>do not launch indexable by accident (The only noindex is the host-based one for *.netlify.app above, so the real domain is indexable as soon as DNS points at it: sign-off must come before DNS.)</t>
         </is>
       </c>
       <c r="E23" s="14" t="inlineStr">
@@ -9059,7 +9059,7 @@
       <c r="A24" s="4" t="n"/>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Remove noindex only when sign-off is given</t>
+          <t>Final stakeholder sign-off (Tony/Darryl/Kimberly) on the ported site before DNS cutover</t>
         </is>
       </c>
       <c r="C24" s="15" t="inlineStr">
@@ -9067,11 +9067,7 @@
           <t>Remaining</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>do not launch indexable by accident (The only noindex is the host-based one for *.netlify.app above, so the real domain is indexable as soon as DNS points at it: sign-off must come before DNS.)</t>
-        </is>
-      </c>
+      <c r="D24" s="4" t="inlineStr"/>
       <c r="E24" s="14" t="inlineStr">
         <is>
           <t>Phase 14 — QA &amp; Launch</t>
@@ -9082,7 +9078,7 @@
       <c r="A25" s="4" t="n"/>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Final stakeholder sign-off (Tony/Darryl/Kimberly) on the ported site before DNS cutover</t>
+          <t>DNS cutover, legacy app decommissioned only after a stable overlap window Checked 2026-10-09 (owner wants to go live and switch off Manus)</t>
         </is>
       </c>
       <c r="C25" s="15" t="inlineStr">
@@ -9090,45 +9086,26 @@
           <t>Remaining</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr"/>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>DNS for tonygreenberg.com is at Hostinger (name servers ns1/ns2.dns-parking.com); www is a CNAME to cname.manus.space, the bare domain points at Manus's addresses (104.19.168.112 / .169.112); the Netlify site tonygreenberg-website has no custom domain yet (production branch main). Order: (1) merge the three open pull requests into main and check the Netlify copy; (2) restore Supabase and run 0001 to 0003, or launch without member features (they say "isn't available just now"); (3) owner sign-off; (4) add tonygreenberg.com + www in Netlify (Domain management), then at Hostinger point the bare domain at Netlify (A record 75.2.60.5, or Netlify DNS) and www CNAME at tonygreenberg-website.netlify.app; Netlify issues the HTTPS certificate; (5) re-run scripts/check-search-console-urls.ts https://tonygreenberg.com and submit the sitemap in Search Console; (6) only after a few stable days: switch off the Manus site (the database is already backed up, docs/ai/project_legacy_database.md) and rotate the old database password.</t>
+        </is>
+      </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
           <t>Phase 14 — QA &amp; Launch</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="4" t="n"/>
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>DNS cutover, legacy app decommissioned only after a stable overlap window Checked 2026-10-09 (owner wants to go live and switch off Manus)</t>
-        </is>
-      </c>
-      <c r="C26" s="15" t="inlineStr">
-        <is>
-          <t>Remaining</t>
-        </is>
-      </c>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
-          <t>DNS for tonygreenberg.com is at Hostinger (name servers ns1/ns2.dns-parking.com); www is a CNAME to cname.manus.space, the bare domain points at Manus's addresses (104.19.168.112 / .169.112); the Netlify site tonygreenberg-website has no custom domain yet (production branch main). Order: (1) merge the three open pull requests into main and check the Netlify copy; (2) restore Supabase and run 0001 to 0003, or launch without member features (they say "isn't available just now"); (3) owner sign-off; (4) add tonygreenberg.com + www in Netlify (Domain management), then at Hostinger point the bare domain at Netlify (A record 75.2.60.5, or Netlify DNS) and www CNAME at tonygreenberg-website.netlify.app; Netlify issues the HTTPS certificate; (5) re-run scripts/check-search-console-urls.ts https://tonygreenberg.com and submit the sitemap in Search Console; (6) only after a few stable days: switch off the Manus site (the database is already backed up, docs/ai/project_legacy_database.md) and rotate the old database password.</t>
-        </is>
-      </c>
-      <c r="E26" s="14" t="inlineStr">
-        <is>
-          <t>Phase 14 — QA &amp; Launch</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:D26"/>
+  <autoFilter ref="A1:D25"/>
   <mergeCells count="6">
-    <mergeCell ref="A5:D5"/>
-    <mergeCell ref="A12:D12"/>
-    <mergeCell ref="A20:D20"/>
-    <mergeCell ref="A7:D7"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A15:D15"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="A19:D19"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Owner yes: old forms save to Supabase, SEO pack copy, Related links, shared SEO defaults
- Seven old-site forms (PRI consent/corrections, Living Declaration,
  Cheshire story, Facilitator Index, spam report, BrewSoul) save to
  Supabase (migration 0006, run) and email Tony; mailto fallback on error.
- SEO pack copy: homepage title/description/entity statement/newsletter,
  COA wording, Four lenses; essays get author line, one Further Reading,
  optional Updated date, health disclaimer; Five Cups SEO fields, short
  answer, FAQ and headings (Sanity, published, backup kept).
- Related section with 3 links on 19 sparse pages and charity profiles.
- Shared share image/X card for every page (165 of 171 had none);
  meta keywords removed; essay date line wraps on phones.
- Project file, notes, CONTRIBUTING SEO rule.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Migration-Status-Report.xlsx
+++ b/Migration-Status-Report.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Full Detail'!$A$1:$D$337</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Remaining Work'!$A$1:$D$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Remaining Work'!$A$1:$D$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -86,12 +86,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FDE2E2"/>
+        <fgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEF3C7"/>
+        <fgColor rgb="00FDE2E2"/>
       </patternFill>
     </fill>
   </fills>
@@ -2068,17 +2068,17 @@
       <c r="A47" s="4" t="n"/>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>Old site's forms still simplified (decision, 2026-10-10)</t>
-        </is>
-      </c>
-      <c r="C47" s="15" t="inlineStr">
-        <is>
-          <t>Remaining</t>
+          <t>Old site's forms still simplified (decision, 2026-10-10; owner said yes the same day, done)</t>
+        </is>
+      </c>
+      <c r="C47" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>Full map in docs/ai/project_legacy_database.md ("Everything the old database did"). These now open an email or stay in the browser instead of saving: PRI consent (~17 real rows on the old site, the biggest gap), Living Declaration, PRI corrections, Cheshire stories, Facilitator Index, spam reports. Owner chose not to change them for now; each can save to Supabase the same way if wanted.</t>
+          <t>Full map in docs/ai/project_legacy_database.md ("Everything the old database did"). These now open an email or stay in the browser instead of saving: PRI consent (~17 real rows on the old site, the biggest gap), Living Declaration, PRI corrections, Cheshire stories, Facilitator Index, spam reports. Owner chose not to change them for now; each can save to Supabase the same way if wanted. Done 2026-10-10: all seven save to Supabase and email Tony (Resend), like the old site: PRI consent (disclaimer-gate.tsx, never blocks the visitor, no email, as legacy), PRI corrections, Living Declaration, Cheshire story (legacy's full form is back on /protecting-your-business and /alex-azzi, components/cheshire/story-form.tsx), Facilitator Index full form and Quick Intake, spam reports, BrewSoul suggestions. Tables in supabase/migrations/0006_site_forms.sql (run; 7 tables, row-level security on, no public policies); actions src/app/forms/actions.ts (server validation, flood guard per visitor, honeypot). A failed save shows the error plus "Or email Tony directly" with the old pre-filled email, so nothing is lost. Tested in a browser on a production build with email off: the BrewSoul and spam forms saved a row each (deleted afterwards). Left: the PRI results "Want a personal introduction?" card still opens an email (it wasn't one of the old site's saved forms).</t>
         </is>
       </c>
       <c r="E47" s="14" t="inlineStr">
@@ -3823,7 +3823,7 @@
           <t>/shop, /payment-success, /payment-cancel</t>
         </is>
       </c>
-      <c r="C125" s="16" t="inlineStr">
+      <c r="C125" s="15" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
@@ -6650,7 +6650,7 @@
           <t>Set GITHUB_TOKEN, MCP_ADMIN_USERS, MCP_LOGIN_PASSWORD, MCP_OAUTH_SECRET, MCP_SITE_ORIGIN, MCP_PUBLIC_ORIGIN in Netlify (done) (checked 2026-…</t>
         </is>
       </c>
-      <c r="C252" s="15" t="inlineStr">
+      <c r="C252" s="16" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
@@ -6673,7 +6673,7 @@
           <t>Commit a team-wide .mcp.json (URL only) once the production URL is settled.</t>
         </is>
       </c>
-      <c r="C253" s="15" t="inlineStr">
+      <c r="C253" s="16" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
@@ -6853,7 +6853,7 @@
           <t>Blocked on you (Google)</t>
         </is>
       </c>
-      <c r="C261" s="15" t="inlineStr">
+      <c r="C261" s="16" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
@@ -6899,7 +6899,7 @@
           <t>Test the new review end to end on a deploy preview</t>
         </is>
       </c>
-      <c r="C263" s="15" t="inlineStr">
+      <c r="C263" s="16" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
@@ -7484,7 +7484,7 @@
           <t>Lighthouse pass (performance/accessibility/SEO) on top 20 pages by traffic 2026-09-30, 20 key pages (no traffic data yet), local production …</t>
         </is>
       </c>
-      <c r="C289" s="15" t="inlineStr">
+      <c r="C289" s="16" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
@@ -7642,17 +7642,17 @@
       <c r="A296" s="4" t="n"/>
       <c r="B296" s="4" t="inlineStr">
         <is>
-          <t>SEO audit items needing a yes (2026-10-06)</t>
-        </is>
-      </c>
-      <c r="C296" s="15" t="inlineStr">
-        <is>
-          <t>Remaining</t>
+          <t>SEO audit items needing a yes (2026-10-06; owner said yes to the copy 2026-10-10, done)</t>
+        </is>
+      </c>
+      <c r="C296" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D296" s="4" t="inlineStr">
         <is>
-          <t>the pack's new copy (homepage title/description, five-cups title, description, short answer, FAQ, heading rewrites, entity statement, newsletter block, author box, health disclaimer, COA wording); "Further Reading" shown twice on posts (merge the lists?); long post title (84 chars), homepage description length and obsolete keywords tag, slugs (/blog/five-cups, the -2 slug; would need redirects), "Six lenses" over four cards, sources for health claims and proof for "$10B+", "Certified B Corp", "Validity: 91", legal review of the homepage Case File banner, ABIT waitlist disclosures, one contact email, the two one-post categories, fewer homepage CTAs / email signup / table of contents / explaining "COA".</t>
+          <t xml:space="preserve">the pack's new copy (homepage title/description, five-cups title, description, short answer, FAQ, heading rewrites, entity statement, newsletter block, author box, health disclaimer, COA wording); "Further Reading" shown twice on posts (merge the lists?); long post title (84 chars), homepage description length and obsolete keywords tag, slugs (/blog/five-cups, the -2 slug; would need redirects), "Six lenses" over four cards, sources for health claims and proof for "$10B+", "Certified B Corp", "Validity: 91", legal review of the homepage Case File banner, ABIT waitlist disclosures, one contact email, the two one-post categories, fewer homepage CTAs / email signup / table of contents / explaining "COA". Done 2026-10-10: homepage title "Tony Greenberg | Strategist, Author &amp; CEO of RampRate" and description (essay count computed: 123); entity statement under the hero (107 coffees / 100 chains computed from the data) with a link to /ecosystem; door 4 "Certificate of Analysis (COA) checks, lab testing and vendor scoring"; "Four lenses" (computed); newsletter box after Editor's Picks (existing Kit form); meta keywords removed site-wide; every essay: author line + "About Tony", one merged "Further Reading", optional lastUpdated field shown as "Updated &lt;date&gt;" (not set on any post yet: every _updatedAt is the import date), health disclaimer on 20 personal-health essays (chosen by Sanity tag); Five Cups (Sanity, published, backup kept): SEO title/description, short answer, visible FAQ </t>
         </is>
       </c>
       <c r="E296" s="14" t="inlineStr">
@@ -7691,7 +7691,7 @@
           <t>Connect Google Search Console + GA4 to the new deployment on day one of cutover</t>
         </is>
       </c>
-      <c r="C298" s="15" t="inlineStr">
+      <c r="C298" s="16" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
@@ -8019,7 +8019,7 @@
           <t>Site-wide: logo (light + dark) beyond the current text wordmark</t>
         </is>
       </c>
-      <c r="C313" s="15" t="inlineStr">
+      <c r="C313" s="16" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
@@ -8134,7 +8134,7 @@
           <t>92 posts still need a real, unique hero image</t>
         </is>
       </c>
-      <c r="C318" s="15" t="inlineStr">
+      <c r="C318" s="16" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
@@ -8341,7 +8341,7 @@
           <t>Assessment result-screen background art (flagged in STATUS.md as a known gap</t>
         </is>
       </c>
-      <c r="C327" s="15" t="inlineStr">
+      <c r="C327" s="16" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
@@ -8420,7 +8420,7 @@
           <t>Mobile responsive pass on every ported section</t>
         </is>
       </c>
-      <c r="C331" s="15" t="inlineStr">
+      <c r="C331" s="16" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
@@ -8466,14 +8466,14 @@
           <t>No dead-end pages (every page links to 2+ others)</t>
         </is>
       </c>
-      <c r="C333" s="15" t="inlineStr">
-        <is>
-          <t>Remaining</t>
+      <c r="C333" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D333" s="4" t="inlineStr">
         <is>
-          <t>same bar as legacy MASTER_QUALITY_PROMPT.md 2026-09-30 scan (496 sitemap pages, header/footer links not counted): every page has a way home (the 6 HumanOS pages had none, in legacy too; added a "← TonyGreenberg.com" footer link). ~17 quiz pages only look like dead ends on their intro screen; their result screens link to related assessments. Left for a content decision: ~20 marketing pages (/akbar, /amplifier, /diamond-cut, /ecosystem, /engage, /engine-room, /intel, /invest, /pick-up-the-phone, /protecting-your-business, /published, /speaking, /the-nightstand, /the-territory, /the-web, /under-nda, /pri-calibration, /charity-scorecard and its detail pages) link to only 0-1 other page in their content. The port matches legacy there (legacy was just as sparse), so adding related links is new content and needs the owner's yes.</t>
+          <t>same bar as legacy MASTER_QUALITY_PROMPT.md 2026-09-30 scan (496 sitemap pages, header/footer links not counted): every page has a way home (the 6 HumanOS pages had none, in legacy too; added a "← TonyGreenberg.com" footer link). ~17 quiz pages only look like dead ends on their intro screen; their result screens link to related assessments. Left for a content decision: ~20 marketing pages (/akbar, /amplifier, /diamond-cut, /ecosystem, /engage, /engine-room, /intel, /invest, /pick-up-the-phone, /protecting-your-business, /published, /speaking, /the-nightstand, /the-territory, /the-web, /under-nda, /pri-calibration, /charity-scorecard and its detail pages) link to only 0-1 other page in their content. The port matches legacy there (legacy was just as sparse), so adding related links is new content and needs the owner's yes. Done 2026-10-10 (owner said yes): a "Related" section with 3 real links (no redirects, titles and blurbs from each target's own copy) on all 19 sparse pages and every charity profile: data src/lib/content/related-pages.ts, component src/components/marketing/related-pages.tsx (light/dark). Checked at 375/820/1280px with no sideways scroll; found and fixed on the way: the essay date line couldn't wrap on phones (21px sideways on long category names).</t>
         </is>
       </c>
       <c r="E333" s="14" t="inlineStr">
@@ -8489,7 +8489,7 @@
           <t>Cross-browser check (Safari iOS in particular, per legacy performance notes) 2026-10-06 WebKit pass (Playwright WebKit, iPhone 13 profile, 1…</t>
         </is>
       </c>
-      <c r="C334" s="15" t="inlineStr">
+      <c r="C334" s="16" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
@@ -8512,7 +8512,7 @@
           <t>Remove noindex only when sign-off is given</t>
         </is>
       </c>
-      <c r="C335" s="15" t="inlineStr">
+      <c r="C335" s="16" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
@@ -8535,7 +8535,7 @@
           <t>Final stakeholder sign-off (Tony/Darryl/Kimberly) on the ported site before DNS cutover</t>
         </is>
       </c>
-      <c r="C336" s="15" t="inlineStr">
+      <c r="C336" s="16" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
@@ -8554,7 +8554,7 @@
           <t>DNS cutover, legacy app decommissioned only after a stable overlap window Checked 2026-10-09 (owner wants to go live and switch off Manus)</t>
         </is>
       </c>
-      <c r="C337" s="15" t="inlineStr">
+      <c r="C337" s="16" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
@@ -8598,7 +8598,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -8638,7 +8638,7 @@
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t>Phase 2 — Supabase</t>
+          <t>Phase 4 — Marketing Core Pages (30 routes)</t>
         </is>
       </c>
       <c r="B2" s="11" t="n"/>
@@ -8649,29 +8649,29 @@
       <c r="A3" s="4" t="n"/>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Old site's forms still simplified (decision, 2026-10-10)</t>
+          <t>/shop, /payment-success, /payment-cancel</t>
         </is>
       </c>
       <c r="C3" s="15" t="inlineStr">
         <is>
-          <t>Remaining</t>
+          <t>Deferred</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Full map in docs/ai/project_legacy_database.md ("Everything the old database did"). These now open an email or stay in the browser instead of saving: PRI consent (~17 real rows on the old site, the biggest gap), Living Declaration, PRI corrections, Cheshire stories, Facilitator Index, spam reports. Owner chose not to change them for now; each can save to Supabase the same way if wanted.</t>
+          <t>defer: these are Stripe-backed; flag for the later billing-migration phase, do not port checkout logic yet, static/informational content only if ported now</t>
         </is>
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>Phase 2 — Supabase</t>
+          <t>Phase 4 — Marketing Core Pages (30 routes)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
-          <t>Phase 4 — Marketing Core Pages (30 routes)</t>
+          <t>Phase 11 — Code MCP Server — REBUILT (2026-09-29)</t>
         </is>
       </c>
       <c r="B4" s="11" t="n"/>
@@ -8682,50 +8682,59 @@
       <c r="A5" s="4" t="n"/>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>/shop, /payment-success, /payment-cancel</t>
+          <t>Set GITHUB_TOKEN, MCP_ADMIN_USERS, MCP_LOGIN_PASSWORD, MCP_OAUTH_SECRET, MCP_SITE_ORIGIN, MCP_PUBLIC_ORIGIN in Netlify (done) (checked 2026-…</t>
         </is>
       </c>
       <c r="C5" s="16" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Remaining</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>defer: these are Stripe-backed; flag for the later billing-migration phase, do not port checkout logic yet, static/informational content only if ported now</t>
+          <t>10-07: all already set in Netlify). Left: connect Claude.ai to /api/mcp for real, and verify the GitHub flow end to end (branch → PR → deploy preview → publish_changes) against a real PR.</t>
         </is>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>Phase 4 — Marketing Core Pages (30 routes)</t>
+          <t>Phase 11 — Code MCP Server — REBUILT (2026-09-29)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="4" t="n"/>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Commit a team-wide .mcp.json (URL only) once the production URL is settled.</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>Remaining</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr"/>
+      <c r="E6" s="14" t="inlineStr">
         <is>
           <t>Phase 11 — Code MCP Server — REBUILT (2026-09-29)</t>
         </is>
       </c>
-      <c r="B6" s="11" t="n"/>
-      <c r="C6" s="11" t="n"/>
-      <c r="D6" s="12" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n"/>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Set GITHUB_TOKEN, MCP_ADMIN_USERS, MCP_LOGIN_PASSWORD, MCP_OAUTH_SECRET, MCP_SITE_ORIGIN, MCP_PUBLIC_ORIGIN in Netlify (done) (checked 2026-…</t>
-        </is>
-      </c>
-      <c r="C7" s="15" t="inlineStr">
+          <t>Blocked on you (Google)</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>10-07: all already set in Netlify). Left: connect Claude.ai to /api/mcp for real, and verify the GitHub flow end to end (branch → PR → deploy preview → publish_changes) against a real PR.</t>
+          <t>create a GOOGLE_API_KEY in Google Cloud (project of the vcos-ga4-reader service account, where the PageSpeed Insights API is already on), restricted to the PageSpeed Insights API, then add it to .env.local and Netlify. Creating it from here was blocked by the session's safety check (it would use the service account's credentials to change the Cloud project). Note lighthouse_check_page may time out on Netlify (10 s function limit on the free plan).</t>
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr">
@@ -8738,15 +8747,19 @@
       <c r="A8" s="4" t="n"/>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Commit a team-wide .mcp.json (URL only) once the production URL is settled.</t>
-        </is>
-      </c>
-      <c r="C8" s="15" t="inlineStr">
+          <t>Test the new review end to end on a deploy preview</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr"/>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>(needs a yes, it opens a real pull request): one throwaway change from Claude.ai or ChatGPT: start (unclear request, so the confirm step shows), confirm, edit, review card, screenshots, upload link, then discard.</t>
+        </is>
+      </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
           <t>Phase 11 — Code MCP Server — REBUILT (2026-09-29)</t>
@@ -8754,104 +8767,87 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="n"/>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>Blocked on you (Google)</t>
-        </is>
-      </c>
-      <c r="C9" s="15" t="inlineStr">
-        <is>
-          <t>Remaining</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>create a GOOGLE_API_KEY in Google Cloud (project of the vcos-ga4-reader service account, where the PageSpeed Insights API is already on), restricted to the PageSpeed Insights API, then add it to .env.local and Netlify. Creating it from here was blocked by the session's safety check (it would use the service account's credentials to change the Cloud project). Note lighthouse_check_page may time out on Netlify (10 s function limit on the free plan).</t>
-        </is>
-      </c>
-      <c r="E9" s="14" t="inlineStr">
-        <is>
-          <t>Phase 11 — Code MCP Server — REBUILT (2026-09-29)</t>
-        </is>
-      </c>
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="n"/>
+      <c r="C9" s="11" t="n"/>
+      <c r="D9" s="12" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n"/>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Test the new review end to end on a deploy preview</t>
-        </is>
-      </c>
-      <c r="C10" s="15" t="inlineStr">
+          <t>Lighthouse pass (performance/accessibility/SEO) on top 20 pages by traffic 2026-09-30, 20 key pages (no traffic data yet), local production …</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>(needs a yes, it opens a real pull request): one throwaway change from Claude.ai or ChatGPT: start (unclear request, so the confirm step shows), confirm, edit, review card, screenshots, upload link, then discard.</t>
+          <t>build, mobile: averages performance 87, accessibility 99→100, best practices 100, SEO 92→100, CLS 0 everywhere. Fixed: public/robots.txt had an LLMs: line (not a real directive) that made Google treat the whole file as invalid, now a comment; h3/h4 headings skipping a level on /assessments, /kava, /peptide-watch (same look, right tag); the Kava and /attention-theft back-arrow links had no accessible name on phones; two small phone-width contrast misses. Left: performance is local-machine only (±10-15 points, see CONTRIBUTING.md); the slowest were / 76 (LCP 5.2 s), /psychedelic-readiness-index 82, /iboga-ibogaine 83. Re-run against the Netlify deploy before launch. 2026-10-06 re-run against the Netlify deploy (14 key pages, mobile): accessibility 100 and CLS 0 on every page, SEO clean (only the expected netlify.app noindex), performance 77-97 held back by 3-4 s LCP. Fixed: all 21 hero images moved off the deprecated priority prop to fetchPriority="high" + loading="eager" (Next 16); /iboga-ibogaine hero and the first card on /blog and category pages no longer lazy-loaded; sizes on the Four Doors cards (~150 KiB per page), /humanos diagram (~100 KiB) and /about headshot; urlFor no longer imports the Sanity client, so ~115 KB of Sanity client code stopped loading on / and /blog; React hydration error #418 on / and /blog (post dates) gone, checked in two time zones; /blog is static again; empty icon &lt;th&gt;s on /iboga-ibogaine labelled; category page reads use sanityFetch(). Left: se</t>
         </is>
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
-          <t>Phase 11 — Code MCP Server — REBUILT (2026-09-29)</t>
+          <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="A11" s="4" t="n"/>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Connect Google Search Console + GA4 to the new deployment on day one of cutover</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Remaining</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr"/>
+      <c r="E11" s="14" t="inlineStr">
         <is>
           <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
         </is>
       </c>
-      <c r="B11" s="11" t="n"/>
-      <c r="C11" s="11" t="n"/>
-      <c r="D11" s="12" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="n"/>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>Lighthouse pass (performance/accessibility/SEO) on top 20 pages by traffic 2026-09-30, 20 key pages (no traffic data yet), local production …</t>
-        </is>
-      </c>
-      <c r="C12" s="15" t="inlineStr">
-        <is>
-          <t>Remaining</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>build, mobile: averages performance 87, accessibility 99→100, best practices 100, SEO 92→100, CLS 0 everywhere. Fixed: public/robots.txt had an LLMs: line (not a real directive) that made Google treat the whole file as invalid, now a comment; h3/h4 headings skipping a level on /assessments, /kava, /peptide-watch (same look, right tag); the Kava and /attention-theft back-arrow links had no accessible name on phones; two small phone-width contrast misses. Left: performance is local-machine only (±10-15 points, see CONTRIBUTING.md); the slowest were / 76 (LCP 5.2 s), /psychedelic-readiness-index 82, /iboga-ibogaine 83. Re-run against the Netlify deploy before launch. 2026-10-06 re-run against the Netlify deploy (14 key pages, mobile): accessibility 100 and CLS 0 on every page, SEO clean (only the expected netlify.app noindex), performance 77-97 held back by 3-4 s LCP. Fixed: all 21 hero images moved off the deprecated priority prop to fetchPriority="high" + loading="eager" (Next 16); /iboga-ibogaine hero and the first card on /blog and category pages no longer lazy-loaded; sizes on the Four Doors cards (~150 KiB per page), /humanos diagram (~100 KiB) and /about headshot; urlFor no longer imports the Sanity client, so ~115 KB of Sanity client code stopped loading on / and /blog; React hydration error #418 on / and /blog (post dates) gone, checked in two time zones; /blog is static again; empty icon &lt;th&gt;s on /iboga-ibogaine labelled; category page reads use sanityFetch(). Left: se</t>
-        </is>
-      </c>
-      <c r="E12" s="14" t="inlineStr">
-        <is>
-          <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
-        </is>
-      </c>
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>Phase 13 — Images Needed in Sanity</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="n"/>
+      <c r="C12" s="11" t="n"/>
+      <c r="D12" s="12" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n"/>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>SEO audit items needing a yes (2026-10-06)</t>
-        </is>
-      </c>
-      <c r="C13" s="15" t="inlineStr">
+          <t>Site-wide: logo (light + dark) beyond the current text wordmark</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>the pack's new copy (homepage title/description, five-cups title, description, short answer, FAQ, heading rewrites, entity statement, newsletter block, author box, health disclaimer, COA wording); "Further Reading" shown twice on posts (merge the lists?); long post title (84 chars), homepage description length and obsolete keywords tag, slugs (/blog/five-cups, the -2 slug; would need redirects), "Six lenses" over four cards, sources for health claims and proof for "$10B+", "Certified B Corp", "Validity: 91", legal review of the homepage Case File banner, ABIT waitlist disclosures, one contact email, the two one-post categories, fewer homepage CTAs / email signup / table of contents / explaining "COA".</t>
+          <t>(Default/fallback OG image 1200×630 exists: public/images/default-og.png, checked 2026-10-02.)</t>
         </is>
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
+          <t>Phase 13 — Images Needed in Sanity</t>
         </is>
       </c>
     </row>
@@ -8859,74 +8855,78 @@
       <c r="A14" s="4" t="n"/>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Connect Google Search Console + GA4 to the new deployment on day one of cutover</t>
-        </is>
-      </c>
-      <c r="C14" s="15" t="inlineStr">
+          <t>92 posts still need a real, unique hero image</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr"/>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>(down from 99). Tracked one row per post, with a suggested image-generation prompt, in BLOG-IMAGE-BRIEFS.md — work through that file and check items off there, not here. No image-generation tool was connected in this environment as of this writing; either connect one (e.g. an MCP image-gen extension), source these manually/with a designer then upload via Sanity Studio (/studio), or re-check the live legacy site periodically per the correction note above.</t>
+        </is>
+      </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
-          <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
+          <t>Phase 13 — Images Needed in Sanity</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="inlineStr">
+      <c r="A15" s="4" t="n"/>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Assessment result-screen background art (flagged in STATUS.md as a known gap</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>Remaining</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>18/20 assessments currently have plain black backgrounds; sourcing themed art here also closes that gap)</t>
+        </is>
+      </c>
+      <c r="E15" s="14" t="inlineStr">
         <is>
           <t>Phase 13 — Images Needed in Sanity</t>
         </is>
       </c>
-      <c r="B15" s="11" t="n"/>
-      <c r="C15" s="11" t="n"/>
-      <c r="D15" s="12" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="n"/>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>Site-wide: logo (light + dark) beyond the current text wordmark</t>
-        </is>
-      </c>
-      <c r="C16" s="15" t="inlineStr">
-        <is>
-          <t>Remaining</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>(Default/fallback OG image 1200×630 exists: public/images/default-og.png, checked 2026-10-02.)</t>
-        </is>
-      </c>
-      <c r="E16" s="14" t="inlineStr">
-        <is>
-          <t>Phase 13 — Images Needed in Sanity</t>
-        </is>
-      </c>
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>Phase 14 — QA &amp; Launch</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="n"/>
+      <c r="C16" s="11" t="n"/>
+      <c r="D16" s="12" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n"/>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>92 posts still need a real, unique hero image</t>
-        </is>
-      </c>
-      <c r="C17" s="15" t="inlineStr">
+          <t>Mobile responsive pass on every ported section</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>(down from 99). Tracked one row per post, with a suggested image-generation prompt, in BLOG-IMAGE-BRIEFS.md — work through that file and check items off there, not here. No image-generation tool was connected in this environment as of this writing; either connect one (e.g. an MCP image-gen extension), source these manually/with a designer then upload via Sanity Studio (/studio), or re-check the live legacy site periodically per the correction note above.</t>
+          <t>2026-09-29: no page scrolls sideways at 375px any more (114 pages checked in Chrome: every unique page plus 3 of each templated set like blog posts and coffees). Fixed: BrewSoul NextSteps forced 3 columns (and used an inline style), charity-scorecard tab row, /brewsoul/browse filter dropdowns, /the-philosophy hero glow. Still to check by hand: 44px tap targets and Safari iOS. 2026-09-30: 44px tap targets on phones for the shared header, footer, BrewSoul/Kava/HumanOS menus and ~100 standalone links (undersized targets 1,904 → 578; the rest are 24-43px pills/chips that meet WCAG 2.2 AA). axe target-size (WCAG 2.2 AA, with its spacing exception): 0 failures on 114 pages. Safari/iPhone (WebKit, iPhone 14 emulation): all 114 pages load, no sideways scroll, no JS errors; form fields under 16px (iOS zoom-on-tap) fixed site-wide in globals.css. Still to check on a real iPhone: BrewSoul's bottom journey bar showed page text through it in headless WebKit only (taps hit the bar correctly; Chrome renders it solid). Fixed 2026-10-09: the bar is now solid (bg-[#2C1810], was 92% plus backdrop-blur-md), so nothing can show through even where the blur isn't drawn; checked in WebKit (iPhone 13 profile) and Chrome: background rgb(44, 24, 16), no text behind the buttons. A real iPhone check is still part of Phase 14.</t>
         </is>
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
-          <t>Phase 13 — Images Needed in Sanity</t>
+          <t>Phase 14 — QA &amp; Launch</t>
         </is>
       </c>
     </row>
@@ -8934,52 +8934,61 @@
       <c r="A18" s="4" t="n"/>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Assessment result-screen background art (flagged in STATUS.md as a known gap</t>
-        </is>
-      </c>
-      <c r="C18" s="15" t="inlineStr">
+          <t>Cross-browser check (Safari iOS in particular, per legacy performance notes) 2026-10-06 WebKit pass (Playwright WebKit, iPhone 13 profile, 1…</t>
+        </is>
+      </c>
+      <c r="C18" s="16" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>18/20 assessments currently have plain black backgrounds; sourcing themed art here also closes that gap)</t>
+          <t>52 pages: every unique page plus 3 of each templated set, production build): no page pans sideways, no failed requests, no JS errors. Found and fixed on the way: upgrade-insecure-requests in the new CSP made Safari fetch every stylesheet and font over https on localhost (dropped; the site is HTTPS-only via HSTS anyway), and .toLocaleString() without a locale caused a hydration error on /brewsoul/chains in Safari (all number formatting now en-US). Left: a check on a real iPhone (Phase 14).</t>
         </is>
       </c>
       <c r="E18" s="14" t="inlineStr">
         <is>
-          <t>Phase 13 — Images Needed in Sanity</t>
+          <t>Phase 14 — QA &amp; Launch</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="inlineStr">
+      <c r="A19" s="4" t="n"/>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Remove noindex only when sign-off is given</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>Remaining</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>do not launch indexable by accident (The only noindex is the host-based one for *.netlify.app above, so the real domain is indexable as soon as DNS points at it: sign-off must come before DNS.)</t>
+        </is>
+      </c>
+      <c r="E19" s="14" t="inlineStr">
         <is>
           <t>Phase 14 — QA &amp; Launch</t>
         </is>
       </c>
-      <c r="B19" s="11" t="n"/>
-      <c r="C19" s="11" t="n"/>
-      <c r="D19" s="12" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n"/>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Mobile responsive pass on every ported section</t>
-        </is>
-      </c>
-      <c r="C20" s="15" t="inlineStr">
+          <t>Final stakeholder sign-off (Tony/Darryl/Kimberly) on the ported site before DNS cutover</t>
+        </is>
+      </c>
+      <c r="C20" s="16" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-29: no page scrolls sideways at 375px any more (114 pages checked in Chrome: every unique page plus 3 of each templated set like blog posts and coffees). Fixed: BrewSoul NextSteps forced 3 columns (and used an inline style), charity-scorecard tab row, /brewsoul/browse filter dropdowns, /the-philosophy hero glow. Still to check by hand: 44px tap targets and Safari iOS. 2026-09-30: 44px tap targets on phones for the shared header, footer, BrewSoul/Kava/HumanOS menus and ~100 standalone links (undersized targets 1,904 → 578; the rest are 24-43px pills/chips that meet WCAG 2.2 AA). axe target-size (WCAG 2.2 AA, with its spacing exception): 0 failures on 114 pages. Safari/iPhone (WebKit, iPhone 14 emulation): all 114 pages load, no sideways scroll, no JS errors; form fields under 16px (iOS zoom-on-tap) fixed site-wide in globals.css. Still to check on a real iPhone: BrewSoul's bottom journey bar showed page text through it in headless WebKit only (taps hit the bar correctly; Chrome renders it solid). Fixed 2026-10-09: the bar is now solid (bg-[#2C1810], was 92% plus backdrop-blur-md), so nothing can show through even where the blur isn't drawn; checked in WebKit (iPhone 13 profile) and Chrome: background rgb(44, 24, 16), no text behind the buttons. A real iPhone check is still part of Phase 14.</t>
-        </is>
-      </c>
+      <c r="D20" s="4" t="inlineStr"/>
       <c r="E20" s="14" t="inlineStr">
         <is>
           <t>Phase 14 — QA &amp; Launch</t>
@@ -8990,17 +8999,17 @@
       <c r="A21" s="4" t="n"/>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>No dead-end pages (every page links to 2+ others)</t>
-        </is>
-      </c>
-      <c r="C21" s="15" t="inlineStr">
+          <t>DNS cutover, legacy app decommissioned only after a stable overlap window Checked 2026-10-09 (owner wants to go live and switch off Manus)</t>
+        </is>
+      </c>
+      <c r="C21" s="16" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>same bar as legacy MASTER_QUALITY_PROMPT.md 2026-09-30 scan (496 sitemap pages, header/footer links not counted): every page has a way home (the 6 HumanOS pages had none, in legacy too; added a "← TonyGreenberg.com" footer link). ~17 quiz pages only look like dead ends on their intro screen; their result screens link to related assessments. Left for a content decision: ~20 marketing pages (/akbar, /amplifier, /diamond-cut, /ecosystem, /engage, /engine-room, /intel, /invest, /pick-up-the-phone, /protecting-your-business, /published, /speaking, /the-nightstand, /the-territory, /the-web, /under-nda, /pri-calibration, /charity-scorecard and its detail pages) link to only 0-1 other page in their content. The port matches legacy there (legacy was just as sparse), so adding related links is new content and needs the owner's yes.</t>
+          <t>DNS for tonygreenberg.com is at Hostinger (name servers ns1/ns2.dns-parking.com); www is a CNAME to cname.manus.space, the bare domain points at Manus's addresses (104.19.168.112 / .169.112); the Netlify site tonygreenberg-website has no custom domain yet (production branch main). Order: (1) merge the three open pull requests into main and check the Netlify copy; (2) restore Supabase and run 0001 to 0003, or launch without member features (they say "isn't available just now"); (3) owner sign-off; (4) add tonygreenberg.com + www in Netlify (Domain management), then at Hostinger point the bare domain at Netlify (A record 75.2.60.5, or Netlify DNS) and www CNAME at tonygreenberg-website.netlify.app; Netlify issues the HTTPS certificate; (5) re-run scripts/check-search-console-urls.ts https://tonygreenberg.com and submit the sitemap in Search Console; (6) only after a few stable days: switch off the Manus site (the database is already backed up, docs/ai/project_legacy_database.md) and rotate the old database password.</t>
         </is>
       </c>
       <c r="E21" s="14" t="inlineStr">
@@ -9009,103 +9018,14 @@
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="4" t="n"/>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>Cross-browser check (Safari iOS in particular, per legacy performance notes) 2026-10-06 WebKit pass (Playwright WebKit, iPhone 13 profile, 1…</t>
-        </is>
-      </c>
-      <c r="C22" s="15" t="inlineStr">
-        <is>
-          <t>Remaining</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t>52 pages: every unique page plus 3 of each templated set, production build): no page pans sideways, no failed requests, no JS errors. Found and fixed on the way: upgrade-insecure-requests in the new CSP made Safari fetch every stylesheet and font over https on localhost (dropped; the site is HTTPS-only via HSTS anyway), and .toLocaleString() without a locale caused a hydration error on /brewsoul/chains in Safari (all number formatting now en-US). Left: a check on a real iPhone (Phase 14).</t>
-        </is>
-      </c>
-      <c r="E22" s="14" t="inlineStr">
-        <is>
-          <t>Phase 14 — QA &amp; Launch</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="n"/>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>Remove noindex only when sign-off is given</t>
-        </is>
-      </c>
-      <c r="C23" s="15" t="inlineStr">
-        <is>
-          <t>Remaining</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>do not launch indexable by accident (The only noindex is the host-based one for *.netlify.app above, so the real domain is indexable as soon as DNS points at it: sign-off must come before DNS.)</t>
-        </is>
-      </c>
-      <c r="E23" s="14" t="inlineStr">
-        <is>
-          <t>Phase 14 — QA &amp; Launch</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="n"/>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>Final stakeholder sign-off (Tony/Darryl/Kimberly) on the ported site before DNS cutover</t>
-        </is>
-      </c>
-      <c r="C24" s="15" t="inlineStr">
-        <is>
-          <t>Remaining</t>
-        </is>
-      </c>
-      <c r="D24" s="4" t="inlineStr"/>
-      <c r="E24" s="14" t="inlineStr">
-        <is>
-          <t>Phase 14 — QA &amp; Launch</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="n"/>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>DNS cutover, legacy app decommissioned only after a stable overlap window Checked 2026-10-09 (owner wants to go live and switch off Manus)</t>
-        </is>
-      </c>
-      <c r="C25" s="15" t="inlineStr">
-        <is>
-          <t>Remaining</t>
-        </is>
-      </c>
-      <c r="D25" s="4" t="inlineStr">
-        <is>
-          <t>DNS for tonygreenberg.com is at Hostinger (name servers ns1/ns2.dns-parking.com); www is a CNAME to cname.manus.space, the bare domain points at Manus's addresses (104.19.168.112 / .169.112); the Netlify site tonygreenberg-website has no custom domain yet (production branch main). Order: (1) merge the three open pull requests into main and check the Netlify copy; (2) restore Supabase and run 0001 to 0003, or launch without member features (they say "isn't available just now"); (3) owner sign-off; (4) add tonygreenberg.com + www in Netlify (Domain management), then at Hostinger point the bare domain at Netlify (A record 75.2.60.5, or Netlify DNS) and www CNAME at tonygreenberg-website.netlify.app; Netlify issues the HTTPS certificate; (5) re-run scripts/check-search-console-urls.ts https://tonygreenberg.com and submit the sitemap in Search Console; (6) only after a few stable days: switch off the Manus site (the database is already backed up, docs/ai/project_legacy_database.md) and rotate the old database password.</t>
-        </is>
-      </c>
-      <c r="E25" s="14" t="inlineStr">
-        <is>
-          <t>Phase 14 — QA &amp; Launch</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:D25"/>
-  <mergeCells count="6">
-    <mergeCell ref="A6:D6"/>
+  <autoFilter ref="A1:D21"/>
+  <mergeCells count="5">
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="A12:D12"/>
     <mergeCell ref="A4:D4"/>
-    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A16:D16"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="A19:D19"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
GA4 custom events from the old site (scroll depth, 45s engaged, second page view, homepage paths)
Same event names as legacy ConversionMechanics.tsx AnalyticsTracker, so
existing GA4 reports keep working; only fires where gtag loads
(tonygreenberg.com). Legacy's duplicate history page_view not ported.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Migration-Status-Report.xlsx
+++ b/Migration-Status-Report.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Remaining Work" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Full Detail'!$A$1:$D$337</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Full Detail'!$A$1:$D$338</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Remaining Work'!$A$1:$D$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -639,15 +639,15 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$337,$A5,'Full Detail'!$C$2:$C$337,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A5,'Full Detail'!$C$2:$C$338,"Done")</f>
         <v/>
       </c>
       <c r="C5" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$337,$A5,'Full Detail'!$C$2:$C$337,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A5,'Full Detail'!$C$2:$C$338,"Remaining")</f>
         <v/>
       </c>
       <c r="D5" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$337,$A5,'Full Detail'!$C$2:$C$337,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A5,'Full Detail'!$C$2:$C$338,"Deferred")</f>
         <v/>
       </c>
       <c r="E5" s="5">
@@ -666,15 +666,15 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$337,$A6,'Full Detail'!$C$2:$C$337,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A6,'Full Detail'!$C$2:$C$338,"Done")</f>
         <v/>
       </c>
       <c r="C6" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$337,$A6,'Full Detail'!$C$2:$C$337,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A6,'Full Detail'!$C$2:$C$338,"Remaining")</f>
         <v/>
       </c>
       <c r="D6" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$337,$A6,'Full Detail'!$C$2:$C$337,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A6,'Full Detail'!$C$2:$C$338,"Deferred")</f>
         <v/>
       </c>
       <c r="E6" s="5">
@@ -693,15 +693,15 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$337,$A7,'Full Detail'!$C$2:$C$337,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A7,'Full Detail'!$C$2:$C$338,"Done")</f>
         <v/>
       </c>
       <c r="C7" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$337,$A7,'Full Detail'!$C$2:$C$337,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A7,'Full Detail'!$C$2:$C$338,"Remaining")</f>
         <v/>
       </c>
       <c r="D7" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$337,$A7,'Full Detail'!$C$2:$C$337,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A7,'Full Detail'!$C$2:$C$338,"Deferred")</f>
         <v/>
       </c>
       <c r="E7" s="5">
@@ -720,15 +720,15 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$337,$A8,'Full Detail'!$C$2:$C$337,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A8,'Full Detail'!$C$2:$C$338,"Done")</f>
         <v/>
       </c>
       <c r="C8" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$337,$A8,'Full Detail'!$C$2:$C$337,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A8,'Full Detail'!$C$2:$C$338,"Remaining")</f>
         <v/>
       </c>
       <c r="D8" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$337,$A8,'Full Detail'!$C$2:$C$337,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A8,'Full Detail'!$C$2:$C$338,"Deferred")</f>
         <v/>
       </c>
       <c r="E8" s="5">
@@ -747,15 +747,15 @@
         </is>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$337,$A9,'Full Detail'!$C$2:$C$337,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A9,'Full Detail'!$C$2:$C$338,"Done")</f>
         <v/>
       </c>
       <c r="C9" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$337,$A9,'Full Detail'!$C$2:$C$337,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A9,'Full Detail'!$C$2:$C$338,"Remaining")</f>
         <v/>
       </c>
       <c r="D9" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$337,$A9,'Full Detail'!$C$2:$C$337,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A9,'Full Detail'!$C$2:$C$338,"Deferred")</f>
         <v/>
       </c>
       <c r="E9" s="5">
@@ -774,15 +774,15 @@
         </is>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$337,$A10,'Full Detail'!$C$2:$C$337,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A10,'Full Detail'!$C$2:$C$338,"Done")</f>
         <v/>
       </c>
       <c r="C10" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$337,$A10,'Full Detail'!$C$2:$C$337,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A10,'Full Detail'!$C$2:$C$338,"Remaining")</f>
         <v/>
       </c>
       <c r="D10" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$337,$A10,'Full Detail'!$C$2:$C$337,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A10,'Full Detail'!$C$2:$C$338,"Deferred")</f>
         <v/>
       </c>
       <c r="E10" s="5">
@@ -801,15 +801,15 @@
         </is>
       </c>
       <c r="B11" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$337,$A11,'Full Detail'!$C$2:$C$337,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A11,'Full Detail'!$C$2:$C$338,"Done")</f>
         <v/>
       </c>
       <c r="C11" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$337,$A11,'Full Detail'!$C$2:$C$337,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A11,'Full Detail'!$C$2:$C$338,"Remaining")</f>
         <v/>
       </c>
       <c r="D11" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$337,$A11,'Full Detail'!$C$2:$C$337,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A11,'Full Detail'!$C$2:$C$338,"Deferred")</f>
         <v/>
       </c>
       <c r="E11" s="5">
@@ -828,15 +828,15 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$337,$A12,'Full Detail'!$C$2:$C$337,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A12,'Full Detail'!$C$2:$C$338,"Done")</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$337,$A12,'Full Detail'!$C$2:$C$337,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A12,'Full Detail'!$C$2:$C$338,"Remaining")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$337,$A12,'Full Detail'!$C$2:$C$337,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A12,'Full Detail'!$C$2:$C$338,"Deferred")</f>
         <v/>
       </c>
       <c r="E12" s="5">
@@ -855,15 +855,15 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$337,$A13,'Full Detail'!$C$2:$C$337,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A13,'Full Detail'!$C$2:$C$338,"Done")</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$337,$A13,'Full Detail'!$C$2:$C$337,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A13,'Full Detail'!$C$2:$C$338,"Remaining")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$337,$A13,'Full Detail'!$C$2:$C$337,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A13,'Full Detail'!$C$2:$C$338,"Deferred")</f>
         <v/>
       </c>
       <c r="E13" s="5">
@@ -882,15 +882,15 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$337,$A14,'Full Detail'!$C$2:$C$337,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A14,'Full Detail'!$C$2:$C$338,"Done")</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$337,$A14,'Full Detail'!$C$2:$C$337,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A14,'Full Detail'!$C$2:$C$338,"Remaining")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$337,$A14,'Full Detail'!$C$2:$C$337,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A14,'Full Detail'!$C$2:$C$338,"Deferred")</f>
         <v/>
       </c>
       <c r="E14" s="5">
@@ -909,15 +909,15 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$337,$A15,'Full Detail'!$C$2:$C$337,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A15,'Full Detail'!$C$2:$C$338,"Done")</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$337,$A15,'Full Detail'!$C$2:$C$337,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A15,'Full Detail'!$C$2:$C$338,"Remaining")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$337,$A15,'Full Detail'!$C$2:$C$337,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A15,'Full Detail'!$C$2:$C$338,"Deferred")</f>
         <v/>
       </c>
       <c r="E15" s="5">
@@ -936,15 +936,15 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$337,$A16,'Full Detail'!$C$2:$C$337,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A16,'Full Detail'!$C$2:$C$338,"Done")</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$337,$A16,'Full Detail'!$C$2:$C$337,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A16,'Full Detail'!$C$2:$C$338,"Remaining")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$337,$A16,'Full Detail'!$C$2:$C$337,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A16,'Full Detail'!$C$2:$C$338,"Deferred")</f>
         <v/>
       </c>
       <c r="E16" s="5">
@@ -963,15 +963,15 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$337,$A17,'Full Detail'!$C$2:$C$337,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A17,'Full Detail'!$C$2:$C$338,"Done")</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$337,$A17,'Full Detail'!$C$2:$C$337,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A17,'Full Detail'!$C$2:$C$338,"Remaining")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$337,$A17,'Full Detail'!$C$2:$C$337,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A17,'Full Detail'!$C$2:$C$338,"Deferred")</f>
         <v/>
       </c>
       <c r="E17" s="5">
@@ -990,15 +990,15 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$337,$A18,'Full Detail'!$C$2:$C$337,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A18,'Full Detail'!$C$2:$C$338,"Done")</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$337,$A18,'Full Detail'!$C$2:$C$337,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A18,'Full Detail'!$C$2:$C$338,"Remaining")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$337,$A18,'Full Detail'!$C$2:$C$337,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A18,'Full Detail'!$C$2:$C$338,"Deferred")</f>
         <v/>
       </c>
       <c r="E18" s="5">
@@ -1017,15 +1017,15 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$337,$A19,'Full Detail'!$C$2:$C$337,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A19,'Full Detail'!$C$2:$C$338,"Done")</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$337,$A19,'Full Detail'!$C$2:$C$337,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A19,'Full Detail'!$C$2:$C$338,"Remaining")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$337,$A19,'Full Detail'!$C$2:$C$337,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A19,'Full Detail'!$C$2:$C$338,"Deferred")</f>
         <v/>
       </c>
       <c r="E19" s="5">
@@ -1075,7 +1075,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E337"/>
+  <dimension ref="A1:E338"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -7688,15 +7688,19 @@
       <c r="A298" s="4" t="n"/>
       <c r="B298" s="4" t="inlineStr">
         <is>
-          <t>Connect Google Search Console + GA4 to the new deployment on day one of cutover</t>
-        </is>
-      </c>
-      <c r="C298" s="16" t="inlineStr">
-        <is>
-          <t>Remaining</t>
-        </is>
-      </c>
-      <c r="D298" s="4" t="inlineStr"/>
+          <t>Old site's custom GA4 events ported (2026-10-10, owner asked to match legacy's Google tags)</t>
+        </is>
+      </c>
+      <c r="C298" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D298" s="4" t="inlineStr">
+        <is>
+          <t>Legacy loaded GA4 G-4GVW40S47N (already on the new site), Manus's own Umami counter (gone with Manus, not portable) and custom events from ConversionMechanics.tsx's AnalyticsTracker. Now src/components/ga-events.tsx (root layout) sends the same names: article_/page_25/50/75/90_scroll, engaged_45_seconds, second_page_view, homepage_path_work/_thinking/_building, start_here_open. Legacy's extra page_view on every history change is not ported (GA4 Enhanced measurement already counts in-site page changes; it would double-count). Tested in Chromium with Google's requests blocked: tonygreenberg.com (mapped to a local build) fired the homepage path and all four essay scroll events plus second_page_view; localhost loads no tag. A RampRate-style weekly report / hourly alert email and an admin analytics page were built the same day and removed at the owner's request (they use the Looker Studio report instead); the empty report_runs table and CRON_SECRET were removed too.</t>
+        </is>
+      </c>
       <c r="E298" s="14" t="inlineStr">
         <is>
           <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
@@ -7707,19 +7711,15 @@
       <c r="A299" s="4" t="n"/>
       <c r="B299" s="4" t="inlineStr">
         <is>
-          <t>Restore/adapt the manus.space triple-layer noindex lockdown pattern for any remaining staging URLs</t>
-        </is>
-      </c>
-      <c r="C299" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D299" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-01: the Netlify copy (tonygreenberg-website.netlify.app) and every deploy preview had no noindex at all, so Google could index a duplicate of the site. next.config.ts headers() now sends X-Robots-Tag: noindex, nofollow on any *.netlify.app host only; tonygreenberg.com is unaffected, so nothing to remove at cutover. Tested with Host headers on a production build.</t>
-        </is>
-      </c>
+          <t>Connect Google Search Console + GA4 to the new deployment on day one of cutover</t>
+        </is>
+      </c>
+      <c r="C299" s="16" t="inlineStr">
+        <is>
+          <t>Remaining</t>
+        </is>
+      </c>
+      <c r="D299" s="4" t="inlineStr"/>
       <c r="E299" s="14" t="inlineStr">
         <is>
           <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
@@ -7730,7 +7730,7 @@
       <c r="A300" s="4" t="n"/>
       <c r="B300" s="4" t="inlineStr">
         <is>
-          <t>"Keep going" strip above the footer on every page (2026-10-07)</t>
+          <t>Restore/adapt the manus.space triple-layer noindex lockdown pattern for any remaining staging URLs</t>
         </is>
       </c>
       <c r="C300" s="13" t="inlineStr">
@@ -7740,7 +7740,7 @@
       </c>
       <c r="D300" s="4" t="inlineStr">
         <is>
-          <t>legacy's WhereNext (deferred in Phase 3, never picked up) with its per-page suggestions, Home · Site Index · All Assessments; links pointed at current routes.</t>
+          <t>2026-10-01: the Netlify copy (tonygreenberg-website.netlify.app) and every deploy preview had no noindex at all, so Google could index a duplicate of the site. next.config.ts headers() now sends X-Robots-Tag: noindex, nofollow on any *.netlify.app host only; tonygreenberg.com is unaffected, so nothing to remove at cutover. Tested with Host headers on a production build.</t>
         </is>
       </c>
       <c r="E300" s="14" t="inlineStr">
@@ -7753,7 +7753,7 @@
       <c r="A301" s="4" t="n"/>
       <c r="B301" s="4" t="inlineStr">
         <is>
-          <t>Live-only and redesigned pages from the 2026-10-07 page sweep (188 pages compared with live)</t>
+          <t>"Keep going" strip above the footer on every page (2026-10-07)</t>
         </is>
       </c>
       <c r="C301" s="13" t="inlineStr">
@@ -7763,7 +7763,7 @@
       </c>
       <c r="D301" s="4" t="inlineStr">
         <is>
-          <t>/the-index rebuilt from live's code (20 concepts, related-word search across essays and site pages, full-text search on the server, "three related places to go next"; the old redirect to /search removed and its links, including the "Site Index" link in "Keep going", point at it again); /the-mirror (and /life-assessment) opens on live's intro (dark hero, "What We Measure" with the six areas, "The Ecosystem"), rebuilt as a step registry (rule 19); /essays header, order and column like live; /about "What They Say" styled like live (live picks 3 of the same 19 quotes at random; ours shows a fixed 3 so they're in the server HTML); /impact-futurism list titles and subtitles; /supplier-intake is a real page again with live's Stage 1 form; /seven-doors and /projects redirect home like live; /impact, /health, /library, /built-on-manus, /heroes are 404 on live too. Left as is on purpose: /blog stays our archive page (on live it repeats the homepage), the email gates on /framework and /peptide-supply-chain, the attention-theft Wall of Shame.</t>
+          <t>legacy's WhereNext (deferred in Phase 3, never picked up) with its per-page suggestions, Home · Site Index · All Assessments; links pointed at current routes.</t>
         </is>
       </c>
       <c r="E301" s="14" t="inlineStr">
@@ -7776,7 +7776,7 @@
       <c r="A302" s="4" t="n"/>
       <c r="B302" s="4" t="inlineStr">
         <is>
-          <t>/alex-azzi locked like live (2026-10-07, owner said match it)</t>
+          <t>Live-only and redesigned pages from the 2026-10-07 page sweep (188 pages compared with live)</t>
         </is>
       </c>
       <c r="C302" s="13" t="inlineStr">
@@ -7786,7 +7786,7 @@
       </c>
       <c r="D302" s="4" t="inlineStr">
         <is>
-          <t>same server-checked password as the locked essay (GATED_POST_PASSWORD, now also set in Netlify), live's "Restricted Access" screen, the report not in the page until unlocked, out of search and the sitemap.</t>
+          <t>/the-index rebuilt from live's code (20 concepts, related-word search across essays and site pages, full-text search on the server, "three related places to go next"; the old redirect to /search removed and its links, including the "Site Index" link in "Keep going", point at it again); /the-mirror (and /life-assessment) opens on live's intro (dark hero, "What We Measure" with the six areas, "The Ecosystem"), rebuilt as a step registry (rule 19); /essays header, order and column like live; /about "What They Say" styled like live (live picks 3 of the same 19 quotes at random; ours shows a fixed 3 so they're in the server HTML); /impact-futurism list titles and subtitles; /supplier-intake is a real page again with live's Stage 1 form; /seven-doors and /projects redirect home like live; /impact, /health, /library, /built-on-manus, /heroes are 404 on live too. Left as is on purpose: /blog stays our archive page (on live it repeats the homepage), the email gates on /framework and /peptide-supply-chain, the attention-theft Wall of Shame.</t>
         </is>
       </c>
       <c r="E302" s="14" t="inlineStr">
@@ -7799,7 +7799,7 @@
       <c r="A303" s="4" t="n"/>
       <c r="B303" s="4" t="inlineStr">
         <is>
-          <t>Live's title fonts and sizes (2026-10-07, "fix the style")</t>
+          <t>/alex-azzi locked like live (2026-10-07, owner said match it)</t>
         </is>
       </c>
       <c r="C303" s="13" t="inlineStr">
@@ -7809,7 +7809,7 @@
       </c>
       <c r="D303" s="4" t="inlineStr">
         <is>
-          <t>measured every page's title font, weight, size and label colour on live vs ours (136 pages). Now like live: Kava headings in Fraunces, HumanOS in Space Grotesk, the peptide tools / charity scorecard / thesis threads in the system serif, America Unbundled in the Iowan Old Style stack at live's size, /akbar in Fraunces 900, friend-gate and post-intervention in Georgia, and live's title sizes on peptide-matrix, peptide-supply-chain, rip-peptide-sciences and the HumanOS pages. Fonts load only on the pages that use them (src/lib/fonts/page-fonts.ts). Label colours stay the darker AA-contrast versions where live's lighter ones fail on a light background.</t>
+          <t>same server-checked password as the locked essay (GATED_POST_PASSWORD, now also set in Netlify), live's "Restricted Access" screen, the report not in the page until unlocked, out of search and the sitemap.</t>
         </is>
       </c>
       <c r="E303" s="14" t="inlineStr">
@@ -7822,7 +7822,7 @@
       <c r="A304" s="4" t="n"/>
       <c r="B304" s="4" t="inlineStr">
         <is>
-          <t>Peptide page images rescued into Sanity and wired (2026-10-07)</t>
+          <t>Live's title fonts and sizes (2026-10-07, "fix the style")</t>
         </is>
       </c>
       <c r="C304" s="13" t="inlineStr">
@@ -7832,7 +7832,7 @@
       </c>
       <c r="D304" s="4" t="inlineStr">
         <is>
-          <t>/peptide-watch hero plus its 11 section banners, /peptide-matrix and /peptide-supply-chain heroes, the /peptide-hall-of-shame hero (scripts/rescue-2026-10-07-peptide-images.ts, logged in docs/ai/manus-media-rescue.md).</t>
+          <t>measured every page's title font, weight, size and label colour on live vs ours (136 pages). Now like live: Kava headings in Fraunces, HumanOS in Space Grotesk, the peptide tools / charity scorecard / thesis threads in the system serif, America Unbundled in the Iowan Old Style stack at live's size, /akbar in Fraunces 900, friend-gate and post-intervention in Georgia, and live's title sizes on peptide-matrix, peptide-supply-chain, rip-peptide-sciences and the HumanOS pages. Fonts load only on the pages that use them (src/lib/fonts/page-fonts.ts). Label colours stay the darker AA-contrast versions where live's lighter ones fail on a light background.</t>
         </is>
       </c>
       <c r="E304" s="14" t="inlineStr">
@@ -7845,7 +7845,7 @@
       <c r="A305" s="4" t="n"/>
       <c r="B305" s="4" t="inlineStr">
         <is>
-          <t>Live's editorial redesign, first group (2026-10-07)</t>
+          <t>Peptide page images rescued into Sanity and wired (2026-10-07)</t>
         </is>
       </c>
       <c r="C305" s="13" t="inlineStr">
@@ -7855,7 +7855,7 @@
       </c>
       <c r="D305" s="4" t="inlineStr">
         <is>
-          <t>dark top sections, narrow single text column, short red section rules and dark call-to-action bands on /invest, /amplifier, /community (now "Sign In to Join the Community", linking our real sign-in; live's made-up counters left out), /framework, /the-letter (daily provocation with "Share this thought" and "Search past provocations"), /engage, /diamond-cut, /ecosystem and the homepage's "The thinking doesn't stop here" band. Kept on purpose: AA-contrast colours where live's fail, "Enter the Gate" instead of live's $5,000 checkout on /diamond-cut.</t>
+          <t>/peptide-watch hero plus its 11 section banners, /peptide-matrix and /peptide-supply-chain heroes, the /peptide-hall-of-shame hero (scripts/rescue-2026-10-07-peptide-images.ts, logged in docs/ai/manus-media-rescue.md).</t>
         </is>
       </c>
       <c r="E305" s="14" t="inlineStr">
@@ -7868,7 +7868,7 @@
       <c r="A306" s="4" t="n"/>
       <c r="B306" s="4" t="inlineStr">
         <is>
-          <t>Live's redesign, second group (done 2026-10-08)</t>
+          <t>Live's editorial redesign, first group (2026-10-07)</t>
         </is>
       </c>
       <c r="C306" s="13" t="inlineStr">
@@ -7878,7 +7878,7 @@
       </c>
       <c r="D306" s="4" t="inlineStr">
         <is>
-          <t>re-measured all 18 pages on live vs a fresh production build (title font/size/weight/colour, labels, hero images). Already matching from 2026-10-07: /the-web, /spirits, /iboga-ibogaine (weight 800), /living-declaration, BrewSoul photo on /brewsoul, /brewsoul/browse, /brewsoul/first-sip (live has none there either), /quiz_25q, /recent-creations. Fixed today: /find-your-journey (64px title, red label), /impact-dashboard (64px title in essay ink, label spacing), red labels on /published and /speaking (plus its "rooms" chips), /soulscore "by ImpactSoul" label, /pri-calibration title (weight 900, solid cream, was a purple gradient), /clients (live's narrow 546px column for the whole page, 56px title, roomier stats band, cards 2 per row; two static inline styles moved to classes), /brewsoul/guest (live's BrewSoul photo on the guest card instead of "SN" initials, labels in capitals), /humanos/connect (cards line up with the title), /peptide-hall-of-shame (stats and label readable light gold; were dark gold on dark). Typed arrows on the touched links are icons now (rule 18). Deliberately not copied from live (new CONTRIBUTING rule 20, owner 2026-10-08): red labels on dark bands use #E07A80 (live's #8E1E25 on black is about 2:1, unreadable); /recent-creations keeps our darker label colours (live's fail contrast on white); /humanos/connect keeps "Start Reading" (that card links to the philosophy page, the quiz live's "Start the Assessment" implies doesn't exist). Checked: type check, l</t>
+          <t>dark top sections, narrow single text column, short red section rules and dark call-to-action bands on /invest, /amplifier, /community (now "Sign In to Join the Community", linking our real sign-in; live's made-up counters left out), /framework, /the-letter (daily provocation with "Share this thought" and "Search past provocations"), /engage, /diamond-cut, /ecosystem and the homepage's "The thinking doesn't stop here" band. Kept on purpose: AA-contrast colours where live's fail, "Enter the Gate" instead of live's $5,000 checkout on /diamond-cut.</t>
         </is>
       </c>
       <c r="E306" s="14" t="inlineStr">
@@ -7891,7 +7891,7 @@
       <c r="A307" s="4" t="n"/>
       <c r="B307" s="4" t="inlineStr">
         <is>
-          <t>BrewSoul top of page (2026-10-08, owner: "button in the center at the top doesn't look good")</t>
+          <t>Live's redesign, second group (done 2026-10-08)</t>
         </is>
       </c>
       <c r="C307" s="13" t="inlineStr">
@@ -7901,7 +7901,7 @@
       </c>
       <c r="D307" s="4" t="inlineStr">
         <is>
-          <t>the category badge ("Deep Research" etc.) sat centred in an empty strip, squeezed against the hero, because we copied live's doubled 52px top gap. Now one gap everywhere and the badge floats in the top-left corner, lined up with the BrewSoul logo (brewsoul-main.tsx, category-badge.tsx); checked on all 26 badge pages at 3 widths that it covers nothing. BrewSoul menu: on tablets (768-1023px) the links were cut off and "More" was hidden with no menu button at all; now the menu button shows below 1024px, 5 links + "More" from 1024px, all 8 from 1280px, "More" always visible.</t>
+          <t>re-measured all 18 pages on live vs a fresh production build (title font/size/weight/colour, labels, hero images). Already matching from 2026-10-07: /the-web, /spirits, /iboga-ibogaine (weight 800), /living-declaration, BrewSoul photo on /brewsoul, /brewsoul/browse, /brewsoul/first-sip (live has none there either), /quiz_25q, /recent-creations. Fixed today: /find-your-journey (64px title, red label), /impact-dashboard (64px title in essay ink, label spacing), red labels on /published and /speaking (plus its "rooms" chips), /soulscore "by ImpactSoul" label, /pri-calibration title (weight 900, solid cream, was a purple gradient), /clients (live's narrow 546px column for the whole page, 56px title, roomier stats band, cards 2 per row; two static inline styles moved to classes), /brewsoul/guest (live's BrewSoul photo on the guest card instead of "SN" initials, labels in capitals), /humanos/connect (cards line up with the title), /peptide-hall-of-shame (stats and label readable light gold; were dark gold on dark). Typed arrows on the touched links are icons now (rule 18). Deliberately not copied from live (new CONTRIBUTING rule 20, owner 2026-10-08): red labels on dark bands use #E07A80 (live's #8E1E25 on black is about 2:1, unreadable); /recent-creations keeps our darker label colours (live's fail contrast on white); /humanos/connect keeps "Start Reading" (that card links to the philosophy page, the quiz live's "Start the Assessment" implies doesn't exist). Checked: type check, l</t>
         </is>
       </c>
       <c r="E307" s="14" t="inlineStr">
@@ -7914,7 +7914,7 @@
       <c r="A308" s="4" t="n"/>
       <c r="B308" s="4" t="inlineStr">
         <is>
-          <t>/pri-efficacy's "Simulation / Live Calibrations" switch like live (2026-10-08)</t>
+          <t>BrewSoul top of page (2026-10-08, owner: "button in the center at the top doesn't look good")</t>
         </is>
       </c>
       <c r="C308" s="13" t="inlineStr">
@@ -7924,7 +7924,7 @@
       </c>
       <c r="D308" s="4" t="inlineStr">
         <is>
-          <t>shadcn Tabs, both panels in the server HTML (forceMount). The Live tab reads real aggregate numbers from pri_calibrations (getPriLiveStats() in src/lib/pri-research.ts: totals, opt-ins, average score per dimension; no rows leave the server), page stays static and refreshes every 10 minutes. Until the Supabase scripts are run (Phase 2) it says the numbers "aren't available just now" instead of a fake zero. Checked: build (○, 10m), server HTML has both tabs, tab switch at 390/1280px, no JS errors. Re-check with real numbers once the table exists.</t>
+          <t>the category badge ("Deep Research" etc.) sat centred in an empty strip, squeezed against the hero, because we copied live's doubled 52px top gap. Now one gap everywhere and the badge floats in the top-left corner, lined up with the BrewSoul logo (brewsoul-main.tsx, category-badge.tsx); checked on all 26 badge pages at 3 widths that it covers nothing. BrewSoul menu: on tablets (768-1023px) the links were cut off and "More" was hidden with no menu button at all; now the menu button shows below 1024px, 5 links + "More" from 1024px, all 8 from 1280px, "More" always visible.</t>
         </is>
       </c>
       <c r="E308" s="14" t="inlineStr">
@@ -7937,63 +7937,63 @@
       <c r="A309" s="4" t="n"/>
       <c r="B309" s="4" t="inlineStr">
         <is>
+          <t>/pri-efficacy's "Simulation / Live Calibrations" switch like live (2026-10-08)</t>
+        </is>
+      </c>
+      <c r="C309" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D309" s="4" t="inlineStr">
+        <is>
+          <t>shadcn Tabs, both panels in the server HTML (forceMount). The Live tab reads real aggregate numbers from pri_calibrations (getPriLiveStats() in src/lib/pri-research.ts: totals, opt-ins, average score per dimension; no rows leave the server), page stays static and refreshes every 10 minutes. Until the Supabase scripts are run (Phase 2) it says the numbers "aren't available just now" instead of a fake zero. Checked: build (○, 10m), server HTML has both tabs, tab switch at 390/1280px, no JS errors. Re-check with real numbers once the table exists.</t>
+        </is>
+      </c>
+      <c r="E309" s="14" t="inlineStr">
+        <is>
+          <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" s="4" t="n"/>
+      <c r="B310" s="4" t="inlineStr">
+        <is>
           <t>/brewsoul/browse hero readable (2026-10-08, owner said go ahead)</t>
         </is>
       </c>
-      <c r="C309" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D309" s="4" t="inlineStr">
+      <c r="C310" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D310" s="4" t="inlineStr">
         <is>
           <t>a soft cream glow behind the title block so "The Catalog", the subtitle and the stat labels read clearly over the coffee photo (live is hard to read there too; rule 20). Photo still shows around the edges. Checked at 390/1280px.</t>
         </is>
       </c>
-      <c r="E309" s="14" t="inlineStr">
+      <c r="E310" s="14" t="inlineStr">
         <is>
           <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
         </is>
       </c>
     </row>
-    <row r="310">
-      <c r="A310" s="10" t="inlineStr">
+    <row r="311">
+      <c r="A311" s="10" t="inlineStr">
         <is>
           <t>Phase 13 — Images Needed in Sanity</t>
         </is>
       </c>
-      <c r="B310" s="11" t="n"/>
-      <c r="C310" s="11" t="n"/>
-      <c r="D310" s="12" t="n"/>
-    </row>
-    <row r="311">
-      <c r="A311" s="4" t="n"/>
-      <c r="B311" s="4" t="inlineStr">
-        <is>
-          <t>Manus media rescue (2026-09-29)</t>
-        </is>
-      </c>
-      <c r="C311" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D311" s="4" t="inlineStr">
-        <is>
-          <t>all 94 Manus-hosted image/video references in the legacy source (/api/img/, /manus-storage/) were checked live. 91 were still downloadable, including the /akbar photos the entry below calls "permanently lost", and all 91 are now Sanity assets (scripts/rescue-manus-media.ts; Sanity dedupes by SHA-1). 3 were gone (HTTP 502). The manifest docs/ai/manus-media-rescue.md maps each one to the legacy files that used it and its Sanity URL. They are not wired into pages yet: go page by page, with real alt text. /facilitator-index's two diagrams are done (scripts/rescue-facilitator-images.ts).</t>
-        </is>
-      </c>
-      <c r="E311" s="14" t="inlineStr">
-        <is>
-          <t>Phase 13 — Images Needed in Sanity</t>
-        </is>
-      </c>
+      <c r="B311" s="11" t="n"/>
+      <c r="C311" s="11" t="n"/>
+      <c r="D311" s="12" t="n"/>
     </row>
     <row r="312">
       <c r="A312" s="4" t="n"/>
       <c r="B312" s="4" t="inlineStr">
         <is>
-          <t>Favicon</t>
+          <t>Manus media rescue (2026-09-29)</t>
         </is>
       </c>
       <c r="C312" s="13" t="inlineStr">
@@ -8003,7 +8003,7 @@
       </c>
       <c r="D312" s="4" t="inlineStr">
         <is>
-          <t>real "G" brand mark generated from the header's actual wordmark treatment (src/app/icon.tsx), see Phase 3</t>
+          <t>all 94 Manus-hosted image/video references in the legacy source (/api/img/, /manus-storage/) were checked live. 91 were still downloadable, including the /akbar photos the entry below calls "permanently lost", and all 91 are now Sanity assets (scripts/rescue-manus-media.ts; Sanity dedupes by SHA-1). 3 were gone (HTTP 502). The manifest docs/ai/manus-media-rescue.md maps each one to the legacy files that used it and its Sanity URL. They are not wired into pages yet: go page by page, with real alt text. /facilitator-index's two diagrams are done (scripts/rescue-facilitator-images.ts).</t>
         </is>
       </c>
       <c r="E312" s="14" t="inlineStr">
@@ -8016,17 +8016,17 @@
       <c r="A313" s="4" t="n"/>
       <c r="B313" s="4" t="inlineStr">
         <is>
-          <t>Site-wide: logo (light + dark) beyond the current text wordmark</t>
-        </is>
-      </c>
-      <c r="C313" s="16" t="inlineStr">
-        <is>
-          <t>Remaining</t>
+          <t>Favicon</t>
+        </is>
+      </c>
+      <c r="C313" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D313" s="4" t="inlineStr">
         <is>
-          <t>(Default/fallback OG image 1200×630 exists: public/images/default-og.png, checked 2026-10-02.)</t>
+          <t>real "G" brand mark generated from the header's actual wordmark treatment (src/app/icon.tsx), see Phase 3</t>
         </is>
       </c>
       <c r="E313" s="14" t="inlineStr">
@@ -8039,17 +8039,17 @@
       <c r="A314" s="4" t="n"/>
       <c r="B314" s="4" t="inlineStr">
         <is>
-          <t>Author photo(s) for blog author schema (Tony Greenberg headshot at minimum)</t>
-        </is>
-      </c>
-      <c r="C314" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Site-wide: logo (light + dark) beyond the current text wordmark</t>
+        </is>
+      </c>
+      <c r="C314" s="16" t="inlineStr">
+        <is>
+          <t>Remaining</t>
         </is>
       </c>
       <c r="D314" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02: the rescued headshot is already the author avatar in Sanity; now also in every post's Article JSON-LD (author image + url /about). The JSON-LD publisher logo pointed at /favicon.ico, a 404 here; now /icon.</t>
+          <t>(Default/fallback OG image 1200×630 exists: public/images/default-og.png, checked 2026-10-02.)</t>
         </is>
       </c>
       <c r="E314" s="14" t="inlineStr">
@@ -8062,7 +8062,7 @@
       <c r="A315" s="4" t="n"/>
       <c r="B315" s="4" t="inlineStr">
         <is>
-          <t>Blog hero images</t>
+          <t>Author photo(s) for blog author schema (Tony Greenberg headshot at minimum)</t>
         </is>
       </c>
       <c r="C315" s="13" t="inlineStr">
@@ -8072,7 +8072,7 @@
       </c>
       <c r="D315" s="4" t="inlineStr">
         <is>
-          <t>audited, then migrated. Final state:</t>
+          <t>2026-10-02: the rescued headshot is already the author avatar in Sanity; now also in every post's Article JSON-LD (author image + url /about). The JSON-LD publisher logo pointed at /favicon.ico, a 404 here; now /icon.</t>
         </is>
       </c>
       <c r="E315" s="14" t="inlineStr">
@@ -8085,7 +8085,7 @@
       <c r="A316" s="4" t="n"/>
       <c r="B316" s="4" t="inlineStr">
         <is>
-          <t>22 posts have a real hero image, now live in Sanity (17 already on RampRate's own CloudFront + 4 rescued from the legacy /api/img/ proxy + 1…</t>
+          <t>Blog hero images</t>
         </is>
       </c>
       <c r="C316" s="13" t="inlineStr">
@@ -8095,7 +8095,7 @@
       </c>
       <c r="D316" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> rescued from /manus-storage/, all pulled over by migrate-blog-posts.ts before Manus is decommissioned)</t>
+          <t>audited, then migrated. Final state:</t>
         </is>
       </c>
       <c r="E316" s="14" t="inlineStr">
@@ -8108,7 +8108,7 @@
       <c r="A317" s="4" t="n"/>
       <c r="B317" s="4" t="inlineStr">
         <is>
-          <t>7 more posts got a real, unique hero image rescued from the live legacy site's newly-added art this pass (scripts/rescue-2026-09-blog-images…</t>
+          <t>22 posts have a real hero image, now live in Sanity (17 already on RampRate's own CloudFront + 4 rescued from the legacy /api/img/ proxy + 1…</t>
         </is>
       </c>
       <c r="C317" s="13" t="inlineStr">
@@ -8118,7 +8118,7 @@
       </c>
       <c r="D317" s="4" t="inlineStr">
         <is>
-          <t>.ts — see the correction note above): california-toll-roads-legalized-scam, the-1000-hour-hold, conscious-capital-partnership-ecosystem, the-peptide-truth-65m-fraud-industry-vs-life-changing-medicine, clear-communication, building-services-market-transhuman-era, heart-protocol-addendum.</t>
+          <t xml:space="preserve"> rescued from /manus-storage/, all pulled over by migrate-blog-posts.ts before Manus is decommissioned)</t>
         </is>
       </c>
       <c r="E317" s="14" t="inlineStr">
@@ -8131,17 +8131,17 @@
       <c r="A318" s="4" t="n"/>
       <c r="B318" s="4" t="inlineStr">
         <is>
-          <t>92 posts still need a real, unique hero image</t>
-        </is>
-      </c>
-      <c r="C318" s="16" t="inlineStr">
-        <is>
-          <t>Remaining</t>
+          <t>7 more posts got a real, unique hero image rescued from the live legacy site's newly-added art this pass (scripts/rescue-2026-09-blog-images…</t>
+        </is>
+      </c>
+      <c r="C318" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D318" s="4" t="inlineStr">
         <is>
-          <t>(down from 99). Tracked one row per post, with a suggested image-generation prompt, in BLOG-IMAGE-BRIEFS.md — work through that file and check items off there, not here. No image-generation tool was connected in this environment as of this writing; either connect one (e.g. an MCP image-gen extension), source these manually/with a designer then upload via Sanity Studio (/studio), or re-check the live legacy site periodically per the correction note above.</t>
+          <t>.ts — see the correction note above): california-toll-roads-legalized-scam, the-1000-hour-hold, conscious-capital-partnership-ecosystem, the-peptide-truth-65m-fraud-industry-vs-life-changing-medicine, clear-communication, building-services-market-transhuman-era, heart-protocol-addendum.</t>
         </is>
       </c>
       <c r="E318" s="14" t="inlineStr">
@@ -8154,17 +8154,17 @@
       <c r="A319" s="4" t="n"/>
       <c r="B319" s="4" t="inlineStr">
         <is>
-          <t>Blog: per-post OG image if different from hero (many posts can reuse hero as OG)</t>
-        </is>
-      </c>
-      <c r="C319" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>92 posts still need a real, unique hero image</t>
+        </is>
+      </c>
+      <c r="C319" s="16" t="inlineStr">
+        <is>
+          <t>Remaining</t>
         </is>
       </c>
       <c r="D319" s="4" t="inlineStr">
         <is>
-          <t>Confirmed 2026-10-02: generateMetadata uses seo.ogImage, else the hero, else the default OG image.</t>
+          <t>(down from 99). Tracked one row per post, with a suggested image-generation prompt, in BLOG-IMAGE-BRIEFS.md — work through that file and check items off there, not here. No image-generation tool was connected in this environment as of this writing; either connect one (e.g. an MCP image-gen extension), source these manually/with a designer then upload via Sanity Studio (/studio), or re-check the live legacy site periodically per the correction note above.</t>
         </is>
       </c>
       <c r="E319" s="14" t="inlineStr">
@@ -8177,7 +8177,7 @@
       <c r="A320" s="4" t="n"/>
       <c r="B320" s="4" t="inlineStr">
         <is>
-          <t>Marketing pages</t>
+          <t>Blog: per-post OG image if different from hero (many posts can reuse hero as OG)</t>
         </is>
       </c>
       <c r="C320" s="13" t="inlineStr">
@@ -8187,7 +8187,7 @@
       </c>
       <c r="D320" s="4" t="inlineStr">
         <is>
-          <t>hero/section images for /the-letter, /the-territory, /engine-room, /the-body, /the-nightstand, /recent-creations (portfolio thumbnails), /published (publication logos), /clients (client logos — confirm licensing before re-hosting). Checked against live 2026-10-02: same image count on every one; /the-territory, /engine-room, /recent-creations, /published, /clients have no images on live either.</t>
+          <t>Confirmed 2026-10-02: generateMetadata uses seo.ogImage, else the hero, else the default OG image.</t>
         </is>
       </c>
       <c r="E320" s="14" t="inlineStr">
@@ -8200,7 +8200,7 @@
       <c r="A321" s="4" t="n"/>
       <c r="B321" s="4" t="inlineStr">
         <is>
-          <t>/akbar essay images</t>
+          <t>Marketing pages</t>
         </is>
       </c>
       <c r="C321" s="13" t="inlineStr">
@@ -8210,7 +8210,7 @@
       </c>
       <c r="D321" s="4" t="inlineStr">
         <is>
-          <t>not lost after all: 20 of the 21 were rescued into Sanity by scripts/rescue-manus-media.ts (2026-09-28) and are wired back in legacy's layout (hero mosaic, JC portrait, 2x2 grid, 3 full-bleeds, 3-up strip, footer gallery) as of 2026-09-29. Only slider-3 was gone (HTTP 502); the hero mosaic is 4 tiles instead of 5.</t>
+          <t>hero/section images for /the-letter, /the-territory, /engine-room, /the-body, /the-nightstand, /recent-creations (portfolio thumbnails), /published (publication logos), /clients (client logos — confirm licensing before re-hosting). Checked against live 2026-10-02: same image count on every one; /the-territory, /engine-room, /recent-creations, /published, /clients have no images on live either.</t>
         </is>
       </c>
       <c r="E321" s="14" t="inlineStr">
@@ -8223,7 +8223,7 @@
       <c r="A322" s="4" t="n"/>
       <c r="B322" s="4" t="inlineStr">
         <is>
-          <t>Rescued page images wired back in (2026-09-29)</t>
+          <t>/akbar essay images</t>
         </is>
       </c>
       <c r="C322" s="13" t="inlineStr">
@@ -8233,7 +8233,7 @@
       </c>
       <c r="D322" s="4" t="inlineStr">
         <is>
-          <t>/living-declaration hero, hand image and Clarisse Abelarde artwork; /impact-dashboard earth hero; /find-my banner; /find-your-coffee dark photo landing (legacy copy restored, replacing an intro that wasn't in legacy). Also wired (second pass): /consciousness-scale (legacy's hero-first flow restored, the invented intro screen removed), /find-your-me hero, /humanos hero, the HumanOS nav logo, and all 12 HumanOS people headshots (/humanos/ecosystem, /humanos/philosophy). Blog-body images (2026-09-29): all 19 the migration dropped are restored by scripts/restore-blog-body-images.ts as Sanity drafts on 4 posts (Clarisse Abelarde 7, You Are the Moat 4, FRQNCY 6, Energy Is Money 2), waiting to be published in Studio; the other blog-listed assets were heroes already set. Still unwired from docs/ai/manus-media-rescue.md: and /alex-azzi's subject photo (a photo of a real person on an accusation page: needs Tony's yes first).</t>
+          <t>not lost after all: 20 of the 21 were rescued into Sanity by scripts/rescue-manus-media.ts (2026-09-28) and are wired back in legacy's layout (hero mosaic, JC portrait, 2x2 grid, 3 full-bleeds, 3-up strip, footer gallery) as of 2026-09-29. Only slider-3 was gone (HTTP 502); the hero mosaic is 4 tiles instead of 5.</t>
         </is>
       </c>
       <c r="E322" s="14" t="inlineStr">
@@ -8246,7 +8246,7 @@
       <c r="A323" s="4" t="n"/>
       <c r="B323" s="4" t="inlineStr">
         <is>
-          <t>BrewSoul: coffee/product images (brewsoul-coffees-expanded.ts likely has image refs</t>
+          <t>Rescued page images wired back in (2026-09-29)</t>
         </is>
       </c>
       <c r="C323" s="13" t="inlineStr">
@@ -8256,7 +8256,7 @@
       </c>
       <c r="D323" s="4" t="inlineStr">
         <is>
-          <t>audit), city guide header images, roaster directory photos. Audited 2026-09-09 (status spreadsheet), confirmed 2026-10-02: city guides already have photos; coffees, chains and roasters have no image field in legacy or here (text-only by design); farms got real photos.</t>
+          <t>/living-declaration hero, hand image and Clarisse Abelarde artwork; /impact-dashboard earth hero; /find-my banner; /find-your-coffee dark photo landing (legacy copy restored, replacing an intro that wasn't in legacy). Also wired (second pass): /consciousness-scale (legacy's hero-first flow restored, the invented intro screen removed), /find-your-me hero, /humanos hero, the HumanOS nav logo, and all 12 HumanOS people headshots (/humanos/ecosystem, /humanos/philosophy). Blog-body images (2026-09-29): all 19 the migration dropped are restored by scripts/restore-blog-body-images.ts as Sanity drafts on 4 posts (Clarisse Abelarde 7, You Are the Moat 4, FRQNCY 6, Energy Is Money 2), waiting to be published in Studio; the other blog-listed assets were heroes already set. Still unwired from docs/ai/manus-media-rescue.md: and /alex-azzi's subject photo (a photo of a real person on an accusation page: needs Tony's yes first).</t>
         </is>
       </c>
       <c r="E323" s="14" t="inlineStr">
@@ -8269,7 +8269,7 @@
       <c r="A324" s="4" t="n"/>
       <c r="B324" s="4" t="inlineStr">
         <is>
-          <t>65 page images moved off the Manus storage copy into Sanity (2026-10-02)</t>
+          <t>BrewSoul: coffee/product images (brewsoul-coffees-expanded.ts likely has image refs</t>
         </is>
       </c>
       <c r="C324" s="13" t="inlineStr">
@@ -8279,7 +8279,7 @@
       </c>
       <c r="D324" s="4" t="inlineStr">
         <is>
-          <t>every image the code loaded from d2xsxph8kpxj0f.cloudfront.net (PRI medicine images, Iboga module, facilitator index, /attention-theft, /alex-azzi, /protecting-your-business, /peyote-mescaline, HumanOS, the peptide quiz). Notes called it "RampRate's own CloudFront", but every file sits in the legacy Manus project's folder and its owner couldn't be confirmed. All 65 uploaded (scripts/rescue-cloudfront-images.ts), code rewritten, host removed from images.remotePatterns, no Sanity document used it. Table in docs/ai/manus-media-rescue.md.</t>
+          <t>audit), city guide header images, roaster directory photos. Audited 2026-09-09 (status spreadsheet), confirmed 2026-10-02: city guides already have photos; coffees, chains and roasters have no image field in legacy or here (text-only by design); farms got real photos.</t>
         </is>
       </c>
       <c r="E324" s="14" t="inlineStr">
@@ -8292,7 +8292,7 @@
       <c r="A325" s="4" t="n"/>
       <c r="B325" s="4" t="inlineStr">
         <is>
-          <t>PRI/Kava: medicine reference images (medicine-images.ts), facility images for /facilitator-index</t>
+          <t>65 page images moved off the Manus storage copy into Sanity (2026-10-02)</t>
         </is>
       </c>
       <c r="C325" s="13" t="inlineStr">
@@ -8302,7 +8302,7 @@
       </c>
       <c r="D325" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02: all in Sanity; image counts match live on PRI, Kava, Iboga, Peyote, facilitator pages.</t>
+          <t>every image the code loaded from d2xsxph8kpxj0f.cloudfront.net (PRI medicine images, Iboga module, facilitator index, /attention-theft, /alex-azzi, /protecting-your-business, /peyote-mescaline, HumanOS, the peptide quiz). Notes called it "RampRate's own CloudFront", but every file sits in the legacy Manus project's folder and its owner couldn't be confirmed. All 65 uploaded (scripts/rescue-cloudfront-images.ts), code rewritten, host removed from images.remotePatterns, no Sanity document used it. Table in docs/ai/manus-media-rescue.md.</t>
         </is>
       </c>
       <c r="E325" s="14" t="inlineStr">
@@ -8315,7 +8315,7 @@
       <c r="A326" s="4" t="n"/>
       <c r="B326" s="4" t="inlineStr">
         <is>
-          <t>Manifesto/Attention Theft: any diagram/illustration assets used on the mega-page</t>
+          <t>PRI/Kava: medicine reference images (medicine-images.ts), facility images for /facilitator-index</t>
         </is>
       </c>
       <c r="C326" s="13" t="inlineStr">
@@ -8325,7 +8325,7 @@
       </c>
       <c r="D326" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02: 6 of live's 7 are in (now in Sanity); the 7th belongs to the Wall of Shame section left out on purpose.</t>
+          <t>2026-10-02: all in Sanity; image counts match live on PRI, Kava, Iboga, Peyote, facilitator pages.</t>
         </is>
       </c>
       <c r="E326" s="14" t="inlineStr">
@@ -8338,17 +8338,17 @@
       <c r="A327" s="4" t="n"/>
       <c r="B327" s="4" t="inlineStr">
         <is>
-          <t>Assessment result-screen background art (flagged in STATUS.md as a known gap</t>
-        </is>
-      </c>
-      <c r="C327" s="16" t="inlineStr">
-        <is>
-          <t>Remaining</t>
+          <t>Manifesto/Attention Theft: any diagram/illustration assets used on the mega-page</t>
+        </is>
+      </c>
+      <c r="C327" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D327" s="4" t="inlineStr">
         <is>
-          <t>18/20 assessments currently have plain black backgrounds; sourcing themed art here also closes that gap)</t>
+          <t>2026-10-02: 6 of live's 7 are in (now in Sanity); the 7th belongs to the Wall of Shame section left out on purpose.</t>
         </is>
       </c>
       <c r="E327" s="14" t="inlineStr">
@@ -8361,17 +8361,17 @@
       <c r="A328" s="4" t="n"/>
       <c r="B328" s="4" t="inlineStr">
         <is>
-          <t>Chatbot: FauxTony avatar/icon</t>
-        </is>
-      </c>
-      <c r="C328" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Assessment result-screen background art (flagged in STATUS.md as a known gap</t>
+        </is>
+      </c>
+      <c r="C328" s="16" t="inlineStr">
+        <is>
+          <t>Remaining</t>
         </is>
       </c>
       <c r="D328" s="4" t="inlineStr">
         <is>
-          <t>Not needed (2026-10-02): the chatbot phase (Phase 10) was cancelled.</t>
+          <t>18/20 assessments currently have plain black backgrounds; sourcing themed art here also closes that gap)</t>
         </is>
       </c>
       <c r="E328" s="14" t="inlineStr">
@@ -8384,73 +8384,73 @@
       <c r="A329" s="4" t="n"/>
       <c r="B329" s="4" t="inlineStr">
         <is>
+          <t>Chatbot: FauxTony avatar/icon</t>
+        </is>
+      </c>
+      <c r="C329" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D329" s="4" t="inlineStr">
+        <is>
+          <t>Not needed (2026-10-02): the chatbot phase (Phase 10) was cancelled.</t>
+        </is>
+      </c>
+      <c r="E329" s="14" t="inlineStr">
+        <is>
+          <t>Phase 13 — Images Needed in Sanity</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" s="4" t="n"/>
+      <c r="B330" s="4" t="inlineStr">
+        <is>
           <t>Audit client/public/ (including alex-azzi/, brewsoul/ subfolders) for any static assets already sitting there unused that should be pulled i…</t>
         </is>
       </c>
-      <c r="C329" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D329" s="4" t="inlineStr">
+      <c r="C330" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D330" s="4" t="inlineStr">
         <is>
           <t>n rather than re-created. Done 2026-10-02: no images there at all (only llms.txt, a BrewSoul catalog, Manus debug files, design-options.html). Found and fixed a cutover risk instead: live serves two Google site-verification files (/google6881a0411c48b301.html, /alex-azzi/googleedff0185753a4a1f.html) that the new site returned 404 for, so Search Console could lose verification at DNS cutover. Both copied to public/ byte for byte. Not copied: site.webmanifest (its icons don't exist here; Next's app/icon.tsx covers the favicon).</t>
         </is>
       </c>
-      <c r="E329" s="14" t="inlineStr">
+      <c r="E330" s="14" t="inlineStr">
         <is>
           <t>Phase 13 — Images Needed in Sanity</t>
         </is>
       </c>
     </row>
-    <row r="330">
-      <c r="A330" s="10" t="inlineStr">
+    <row r="331">
+      <c r="A331" s="10" t="inlineStr">
         <is>
           <t>Phase 14 — QA &amp; Launch</t>
         </is>
       </c>
-      <c r="B330" s="11" t="n"/>
-      <c r="C330" s="11" t="n"/>
-      <c r="D330" s="12" t="n"/>
-    </row>
-    <row r="331">
-      <c r="A331" s="4" t="n"/>
-      <c r="B331" s="4" t="inlineStr">
-        <is>
-          <t>Mobile responsive pass on every ported section</t>
-        </is>
-      </c>
-      <c r="C331" s="16" t="inlineStr">
-        <is>
-          <t>Remaining</t>
-        </is>
-      </c>
-      <c r="D331" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-29: no page scrolls sideways at 375px any more (114 pages checked in Chrome: every unique page plus 3 of each templated set like blog posts and coffees). Fixed: BrewSoul NextSteps forced 3 columns (and used an inline style), charity-scorecard tab row, /brewsoul/browse filter dropdowns, /the-philosophy hero glow. Still to check by hand: 44px tap targets and Safari iOS. 2026-09-30: 44px tap targets on phones for the shared header, footer, BrewSoul/Kava/HumanOS menus and ~100 standalone links (undersized targets 1,904 → 578; the rest are 24-43px pills/chips that meet WCAG 2.2 AA). axe target-size (WCAG 2.2 AA, with its spacing exception): 0 failures on 114 pages. Safari/iPhone (WebKit, iPhone 14 emulation): all 114 pages load, no sideways scroll, no JS errors; form fields under 16px (iOS zoom-on-tap) fixed site-wide in globals.css. Still to check on a real iPhone: BrewSoul's bottom journey bar showed page text through it in headless WebKit only (taps hit the bar correctly; Chrome renders it solid). Fixed 2026-10-09: the bar is now solid (bg-[#2C1810], was 92% plus backdrop-blur-md), so nothing can show through even where the blur isn't drawn; checked in WebKit (iPhone 13 profile) and Chrome: background rgb(44, 24, 16), no text behind the buttons. A real iPhone check is still part of Phase 14.</t>
-        </is>
-      </c>
-      <c r="E331" s="14" t="inlineStr">
-        <is>
-          <t>Phase 14 — QA &amp; Launch</t>
-        </is>
-      </c>
+      <c r="B331" s="11" t="n"/>
+      <c r="C331" s="11" t="n"/>
+      <c r="D331" s="12" t="n"/>
     </row>
     <row r="332">
       <c r="A332" s="4" t="n"/>
       <c r="B332" s="4" t="inlineStr">
         <is>
-          <t>Accessibility pass (WCAG AA contrast, 44px touch targets, keyboard nav)</t>
-        </is>
-      </c>
-      <c r="C332" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Mobile responsive pass on every ported section</t>
+        </is>
+      </c>
+      <c r="C332" s="16" t="inlineStr">
+        <is>
+          <t>Remaining</t>
         </is>
       </c>
       <c r="D332" s="4" t="inlineStr">
         <is>
-          <t>same bar as legacy QA_MASTER_PROMPT.md. 2026-09-29 axe-core pass (WCAG 2.1 AA, same 114 pages, production build): all unlabeled dropdowns/inputs and unnamed links fixed; contrast down from 1,453 failing items on 106 pages to 1,038 on 70 (43 pages fully clean). Shared fixes: brand gold #8b6914 → #836311 site-wide (was 4.3:1 on cream, AA needs 4.5), header "⌘K"/social icons, BrewSoul nav and footer, HumanOS footer, Kava footer, assessment intro footnote, post-card image links. 2026-09-30: contrast finished, 0 axe color-contrast failures left on the same 114 pages (production build). Token changes: --kava-saffron #b86a28 → #8e521f, --pri-purple-light #a855f7 → #b87bf9 (on-dark purple only), --crusade-teal #0e7c7c → #0d7373; PriEyebrow goes light purple inside a dark PriSection via group-data-dark/pri; /find-your-me and the journey tracker's dark glass panels 60-70% → 90% (legacy's own 60% glass on beige rendered gray, cream text failed). Everything else: nearest passing shade of the same hue, or gold ↔ gold-light on the wrong background. Left: 18 links inside text marked only by color (need an underline), 44px tap targets, keyboard nav. 2026-09-30: 18 color-only in-text links underlined (axe link-in-text-block: 0 left); keyboard focus visible on every focusable item on 8 sampled pages (two form fields had none, fixed). 2026-10-02 re-run (axe WCAG 2.2 AA, 142 pages × 375/1280px, production build, plus Tab through 40 stops per page): found 1,370 contrast failures (mostly BrewSoul'</t>
+          <t>2026-09-29: no page scrolls sideways at 375px any more (114 pages checked in Chrome: every unique page plus 3 of each templated set like blog posts and coffees). Fixed: BrewSoul NextSteps forced 3 columns (and used an inline style), charity-scorecard tab row, /brewsoul/browse filter dropdowns, /the-philosophy hero glow. Still to check by hand: 44px tap targets and Safari iOS. 2026-09-30: 44px tap targets on phones for the shared header, footer, BrewSoul/Kava/HumanOS menus and ~100 standalone links (undersized targets 1,904 → 578; the rest are 24-43px pills/chips that meet WCAG 2.2 AA). axe target-size (WCAG 2.2 AA, with its spacing exception): 0 failures on 114 pages. Safari/iPhone (WebKit, iPhone 14 emulation): all 114 pages load, no sideways scroll, no JS errors; form fields under 16px (iOS zoom-on-tap) fixed site-wide in globals.css. Still to check on a real iPhone: BrewSoul's bottom journey bar showed page text through it in headless WebKit only (taps hit the bar correctly; Chrome renders it solid). Fixed 2026-10-09: the bar is now solid (bg-[#2C1810], was 92% plus backdrop-blur-md), so nothing can show through even where the blur isn't drawn; checked in WebKit (iPhone 13 profile) and Chrome: background rgb(44, 24, 16), no text behind the buttons. A real iPhone check is still part of Phase 14.</t>
         </is>
       </c>
       <c r="E332" s="14" t="inlineStr">
@@ -8463,7 +8463,7 @@
       <c r="A333" s="4" t="n"/>
       <c r="B333" s="4" t="inlineStr">
         <is>
-          <t>No dead-end pages (every page links to 2+ others)</t>
+          <t>Accessibility pass (WCAG AA contrast, 44px touch targets, keyboard nav)</t>
         </is>
       </c>
       <c r="C333" s="13" t="inlineStr">
@@ -8473,7 +8473,7 @@
       </c>
       <c r="D333" s="4" t="inlineStr">
         <is>
-          <t>same bar as legacy MASTER_QUALITY_PROMPT.md 2026-09-30 scan (496 sitemap pages, header/footer links not counted): every page has a way home (the 6 HumanOS pages had none, in legacy too; added a "← TonyGreenberg.com" footer link). ~17 quiz pages only look like dead ends on their intro screen; their result screens link to related assessments. Left for a content decision: ~20 marketing pages (/akbar, /amplifier, /diamond-cut, /ecosystem, /engage, /engine-room, /intel, /invest, /pick-up-the-phone, /protecting-your-business, /published, /speaking, /the-nightstand, /the-territory, /the-web, /under-nda, /pri-calibration, /charity-scorecard and its detail pages) link to only 0-1 other page in their content. The port matches legacy there (legacy was just as sparse), so adding related links is new content and needs the owner's yes. Done 2026-10-10 (owner said yes): a "Related" section with 3 real links (no redirects, titles and blurbs from each target's own copy) on all 19 sparse pages and every charity profile: data src/lib/content/related-pages.ts, component src/components/marketing/related-pages.tsx (light/dark). Checked at 375/820/1280px with no sideways scroll; found and fixed on the way: the essay date line couldn't wrap on phones (21px sideways on long category names).</t>
+          <t>same bar as legacy QA_MASTER_PROMPT.md. 2026-09-29 axe-core pass (WCAG 2.1 AA, same 114 pages, production build): all unlabeled dropdowns/inputs and unnamed links fixed; contrast down from 1,453 failing items on 106 pages to 1,038 on 70 (43 pages fully clean). Shared fixes: brand gold #8b6914 → #836311 site-wide (was 4.3:1 on cream, AA needs 4.5), header "⌘K"/social icons, BrewSoul nav and footer, HumanOS footer, Kava footer, assessment intro footnote, post-card image links. 2026-09-30: contrast finished, 0 axe color-contrast failures left on the same 114 pages (production build). Token changes: --kava-saffron #b86a28 → #8e521f, --pri-purple-light #a855f7 → #b87bf9 (on-dark purple only), --crusade-teal #0e7c7c → #0d7373; PriEyebrow goes light purple inside a dark PriSection via group-data-dark/pri; /find-your-me and the journey tracker's dark glass panels 60-70% → 90% (legacy's own 60% glass on beige rendered gray, cream text failed). Everything else: nearest passing shade of the same hue, or gold ↔ gold-light on the wrong background. Left: 18 links inside text marked only by color (need an underline), 44px tap targets, keyboard nav. 2026-09-30: 18 color-only in-text links underlined (axe link-in-text-block: 0 left); keyboard focus visible on every focusable item on 8 sampled pages (two form fields had none, fixed). 2026-10-02 re-run (axe WCAG 2.2 AA, 142 pages × 375/1280px, production build, plus Tab through 40 stops per page): found 1,370 contrast failures (mostly BrewSoul'</t>
         </is>
       </c>
       <c r="E333" s="14" t="inlineStr">
@@ -8486,17 +8486,17 @@
       <c r="A334" s="4" t="n"/>
       <c r="B334" s="4" t="inlineStr">
         <is>
-          <t>Cross-browser check (Safari iOS in particular, per legacy performance notes) 2026-10-06 WebKit pass (Playwright WebKit, iPhone 13 profile, 1…</t>
-        </is>
-      </c>
-      <c r="C334" s="16" t="inlineStr">
-        <is>
-          <t>Remaining</t>
+          <t>No dead-end pages (every page links to 2+ others)</t>
+        </is>
+      </c>
+      <c r="C334" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D334" s="4" t="inlineStr">
         <is>
-          <t>52 pages: every unique page plus 3 of each templated set, production build): no page pans sideways, no failed requests, no JS errors. Found and fixed on the way: upgrade-insecure-requests in the new CSP made Safari fetch every stylesheet and font over https on localhost (dropped; the site is HTTPS-only via HSTS anyway), and .toLocaleString() without a locale caused a hydration error on /brewsoul/chains in Safari (all number formatting now en-US). Left: a check on a real iPhone (Phase 14).</t>
+          <t>same bar as legacy MASTER_QUALITY_PROMPT.md 2026-09-30 scan (496 sitemap pages, header/footer links not counted): every page has a way home (the 6 HumanOS pages had none, in legacy too; added a "← TonyGreenberg.com" footer link). ~17 quiz pages only look like dead ends on their intro screen; their result screens link to related assessments. Left for a content decision: ~20 marketing pages (/akbar, /amplifier, /diamond-cut, /ecosystem, /engage, /engine-room, /intel, /invest, /pick-up-the-phone, /protecting-your-business, /published, /speaking, /the-nightstand, /the-territory, /the-web, /under-nda, /pri-calibration, /charity-scorecard and its detail pages) link to only 0-1 other page in their content. The port matches legacy there (legacy was just as sparse), so adding related links is new content and needs the owner's yes. Done 2026-10-10 (owner said yes): a "Related" section with 3 real links (no redirects, titles and blurbs from each target's own copy) on all 19 sparse pages and every charity profile: data src/lib/content/related-pages.ts, component src/components/marketing/related-pages.tsx (light/dark). Checked at 375/820/1280px with no sideways scroll; found and fixed on the way: the essay date line couldn't wrap on phones (21px sideways on long category names).</t>
         </is>
       </c>
       <c r="E334" s="14" t="inlineStr">
@@ -8509,7 +8509,7 @@
       <c r="A335" s="4" t="n"/>
       <c r="B335" s="4" t="inlineStr">
         <is>
-          <t>Remove noindex only when sign-off is given</t>
+          <t>Cross-browser check (Safari iOS in particular, per legacy performance notes) 2026-10-06 WebKit pass (Playwright WebKit, iPhone 13 profile, 1…</t>
         </is>
       </c>
       <c r="C335" s="16" t="inlineStr">
@@ -8519,7 +8519,7 @@
       </c>
       <c r="D335" s="4" t="inlineStr">
         <is>
-          <t>do not launch indexable by accident (The only noindex is the host-based one for *.netlify.app above, so the real domain is indexable as soon as DNS points at it: sign-off must come before DNS.)</t>
+          <t>52 pages: every unique page plus 3 of each templated set, production build): no page pans sideways, no failed requests, no JS errors. Found and fixed on the way: upgrade-insecure-requests in the new CSP made Safari fetch every stylesheet and font over https on localhost (dropped; the site is HTTPS-only via HSTS anyway), and .toLocaleString() without a locale caused a hydration error on /brewsoul/chains in Safari (all number formatting now en-US). Left: a check on a real iPhone (Phase 14).</t>
         </is>
       </c>
       <c r="E335" s="14" t="inlineStr">
@@ -8532,7 +8532,7 @@
       <c r="A336" s="4" t="n"/>
       <c r="B336" s="4" t="inlineStr">
         <is>
-          <t>Final stakeholder sign-off (Tony/Darryl/Kimberly) on the ported site before DNS cutover</t>
+          <t>Remove noindex only when sign-off is given</t>
         </is>
       </c>
       <c r="C336" s="16" t="inlineStr">
@@ -8540,7 +8540,11 @@
           <t>Remaining</t>
         </is>
       </c>
-      <c r="D336" s="4" t="inlineStr"/>
+      <c r="D336" s="4" t="inlineStr">
+        <is>
+          <t>do not launch indexable by accident (The only noindex is the host-based one for *.netlify.app above, so the real domain is indexable as soon as DNS points at it: sign-off must come before DNS.)</t>
+        </is>
+      </c>
       <c r="E336" s="14" t="inlineStr">
         <is>
           <t>Phase 14 — QA &amp; Launch</t>
@@ -8551,40 +8555,59 @@
       <c r="A337" s="4" t="n"/>
       <c r="B337" s="4" t="inlineStr">
         <is>
+          <t>Final stakeholder sign-off (Tony/Darryl/Kimberly) on the ported site before DNS cutover</t>
+        </is>
+      </c>
+      <c r="C337" s="16" t="inlineStr">
+        <is>
+          <t>Remaining</t>
+        </is>
+      </c>
+      <c r="D337" s="4" t="inlineStr"/>
+      <c r="E337" s="14" t="inlineStr">
+        <is>
+          <t>Phase 14 — QA &amp; Launch</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" s="4" t="n"/>
+      <c r="B338" s="4" t="inlineStr">
+        <is>
           <t>DNS cutover, legacy app decommissioned only after a stable overlap window Checked 2026-10-09 (owner wants to go live and switch off Manus)</t>
         </is>
       </c>
-      <c r="C337" s="16" t="inlineStr">
+      <c r="C338" s="16" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
       </c>
-      <c r="D337" s="4" t="inlineStr">
+      <c r="D338" s="4" t="inlineStr">
         <is>
           <t>DNS for tonygreenberg.com is at Hostinger (name servers ns1/ns2.dns-parking.com); www is a CNAME to cname.manus.space, the bare domain points at Manus's addresses (104.19.168.112 / .169.112); the Netlify site tonygreenberg-website has no custom domain yet (production branch main). Order: (1) merge the three open pull requests into main and check the Netlify copy; (2) restore Supabase and run 0001 to 0003, or launch without member features (they say "isn't available just now"); (3) owner sign-off; (4) add tonygreenberg.com + www in Netlify (Domain management), then at Hostinger point the bare domain at Netlify (A record 75.2.60.5, or Netlify DNS) and www CNAME at tonygreenberg-website.netlify.app; Netlify issues the HTTPS certificate; (5) re-run scripts/check-search-console-urls.ts https://tonygreenberg.com and submit the sitemap in Search Console; (6) only after a few stable days: switch off the Manus site (the database is already backed up, docs/ai/project_legacy_database.md) and rotate the old database password.</t>
         </is>
       </c>
-      <c r="E337" s="14" t="inlineStr">
+      <c r="E338" s="14" t="inlineStr">
         <is>
           <t>Phase 14 — QA &amp; Launch</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D337"/>
+  <autoFilter ref="A1:D338"/>
   <mergeCells count="14">
     <mergeCell ref="A211:D211"/>
     <mergeCell ref="A189:D189"/>
     <mergeCell ref="A243:D243"/>
     <mergeCell ref="A215:D215"/>
-    <mergeCell ref="A310:D310"/>
+    <mergeCell ref="A311:D311"/>
     <mergeCell ref="A15:D15"/>
     <mergeCell ref="A64:D64"/>
     <mergeCell ref="A156:D156"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A49:D49"/>
     <mergeCell ref="A129:D129"/>
-    <mergeCell ref="A330:D330"/>
+    <mergeCell ref="A331:D331"/>
     <mergeCell ref="A32:D32"/>
     <mergeCell ref="A264:D264"/>
   </mergeCells>

</xml_diff>

<commit_message>
Email post-intervention check-ins to Tony; logo and launch checks
/post-intervention says "Results go to tony@tonygreenberg.com", so every
saved check-in is now emailed there too (sendEmail, as the site forms do;
a failed email never fails the submission). Status file: logo decided
(keep the text logo), noindex and DNS re-checked before cutover.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Migration-Status-Report.xlsx
+++ b/Migration-Status-Report.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Full Detail'!$A$1:$D$338</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Remaining Work'!$A$1:$D$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Remaining Work'!$A$1:$D$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -596,7 +596,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated from NEXTJS-MIGRATION-TODO.md on 2026-10-10 by scripts/build-migration-status-report.py — a living document; re-run the script after updating the todo file. Counts are formulas over the Full Detail tab.</t>
+          <t>Generated from NEXTJS-MIGRATION-TODO.md on 2026-10-13 by scripts/build-migration-status-report.py — a living document; re-run the script after updating the todo file. Counts are formulas over the Full Detail tab.</t>
         </is>
       </c>
     </row>
@@ -3738,7 +3738,7 @@
       </c>
       <c r="D121" s="4" t="inlineStr">
         <is>
-          <t>PostIntervention.tsx. Built 2026-10-06 as a step registry (day, type, survey, done); saves to Supabase post_intervention_assessments, server-validated. Live's copy says results "go to tony@tonygreenberg.com"; that needs an email service (none connected yet), so for now they are only saved in Supabase. Saving works once the database script is run. Was: Deferred, not skipped. Unlike other single-tRPC-call pages in this migration, this one can't be honestly reduced to a mailto: fallback: the page's entire value proposition, stated three times in its own copy ("Anonymous", "No one can see your name. No one can see your email.", results routed anonymously), is that the facilitator never sees who submitted it. A mailto: would expose the visitor's own email address the moment they hit send in their mail client — actively contradicting the one promise the page makes, not just a missing nice-to-have. Blocked on a real anonymous-submission backend (Phase 5+).</t>
+          <t>PostIntervention.tsx. Built 2026-10-06 as a step registry (day, type, survey, done); saves to Supabase post_intervention_assessments, server-validated. Live's copy says results "go to tony@tonygreenberg.com": since 2026-10-13 every saved check-in is also emailed there (sendEmail, same as the site forms; a failed email never fails the submission). Not yet tried with a real submission, since that emails Tony. Was: Deferred, not skipped. Unlike other single-tRPC-call pages in this migration, this one can't be honestly reduced to a mailto: fallback: the page's entire value proposition, stated three times in its own copy ("Anonymous", "No one can see your name. No one can see your email.", results routed anonymously), is that the facilitator never sees who submitted it. A mailto: would expose the visitor's own email address the moment they hit send in their mail client — actively contradicting the one promise the page makes, not just a missing nice-to-have. Blocked on a real anonymous-submission backend (Phase 5+).</t>
         </is>
       </c>
       <c r="E121" s="14" t="inlineStr">
@@ -8042,14 +8042,14 @@
           <t>Site-wide: logo (light + dark) beyond the current text wordmark</t>
         </is>
       </c>
-      <c r="C314" s="16" t="inlineStr">
-        <is>
-          <t>Remaining</t>
+      <c r="C314" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D314" s="4" t="inlineStr">
         <is>
-          <t>(Default/fallback OG image 1200×630 exists: public/images/default-og.png, checked 2026-10-02.)</t>
+          <t>Decided 2026-10-13 (owner): keep the text logo. The header's "TonyG" wordmark (site-header.tsx, gold G) already has light and dark colours, so no change. (Default/fallback OG image 1200×630 exists: public/images/default-og.png, checked 2026-10-02.)</t>
         </is>
       </c>
       <c r="E314" s="14" t="inlineStr">
@@ -8542,7 +8542,7 @@
       </c>
       <c r="D336" s="4" t="inlineStr">
         <is>
-          <t>do not launch indexable by accident (The only noindex is the host-based one for *.netlify.app above, so the real domain is indexable as soon as DNS points at it: sign-off must come before DNS.)</t>
+          <t>do not launch indexable by accident (The only noindex is the host-based one for *.netlify.app above, so the real domain is indexable as soon as DNS points at it: sign-off must come before DNS.) Re-checked 2026-10-13 on a fresh production build: tonygreenberg.com and www get no X-Robots-Tag and no robots meta (/, /blog, /about, /post-intervention), *.netlify.app gets noindex, nofollow; robots.txt allows crawlers, sitemap 200, missing pages 404, /manifesto 308. Ready; still waits on sign-off.</t>
         </is>
       </c>
       <c r="E336" s="14" t="inlineStr">
@@ -8574,7 +8574,7 @@
       <c r="A338" s="4" t="n"/>
       <c r="B338" s="4" t="inlineStr">
         <is>
-          <t>DNS cutover, legacy app decommissioned only after a stable overlap window Checked 2026-10-09 (owner wants to go live and switch off Manus)</t>
+          <t>DNS cutover, legacy app decommissioned only after a stable overlap window Re-checked 2026-10-13</t>
         </is>
       </c>
       <c r="C338" s="16" t="inlineStr">
@@ -8584,7 +8584,7 @@
       </c>
       <c r="D338" s="4" t="inlineStr">
         <is>
-          <t>DNS for tonygreenberg.com is at Hostinger (name servers ns1/ns2.dns-parking.com); www is a CNAME to cname.manus.space, the bare domain points at Manus's addresses (104.19.168.112 / .169.112); the Netlify site tonygreenberg-website has no custom domain yet (production branch main). Order: (1) merge the three open pull requests into main and check the Netlify copy; (2) restore Supabase and run 0001 to 0003, or launch without member features (they say "isn't available just now"); (3) owner sign-off; (4) add tonygreenberg.com + www in Netlify (Domain management), then at Hostinger point the bare domain at Netlify (A record 75.2.60.5, or Netlify DNS) and www CNAME at tonygreenberg-website.netlify.app; Netlify issues the HTTPS certificate; (5) re-run scripts/check-search-console-urls.ts https://tonygreenberg.com and submit the sitemap in Search Console; (6) only after a few stable days: switch off the Manus site (the database is already backed up, docs/ai/project_legacy_database.md) and rotate the old database password.</t>
+          <t>unchanged (Hostinger name servers, bare domain on Manus 104.19.168/169.112, www CNAME cname.manus.space). Checked 2026-10-09 (owner wants to go live and switch off Manus): DNS for tonygreenberg.com is at Hostinger (name servers ns1/ns2.dns-parking.com); www is a CNAME to cname.manus.space, the bare domain points at Manus's addresses (104.19.168.112 / .169.112); the Netlify site tonygreenberg-website has no custom domain yet (production branch main). Order: (1) merge the three open pull requests into main and check the Netlify copy; (2) restore Supabase and run 0001 to 0003, or launch without member features (they say "isn't available just now"); (3) owner sign-off; (4) add tonygreenberg.com + www in Netlify (Domain management), then at Hostinger point the bare domain at Netlify (A record 75.2.60.5, or Netlify DNS) and www CNAME at tonygreenberg-website.netlify.app; Netlify issues the HTTPS certificate; (5) re-run scripts/check-search-console-urls.ts https://tonygreenberg.com and submit the sitemap in Search Console; (6) only after a few stable days: switch off the Manus site (the database is already backed up, docs/ai/project_legacy_database.md) and rotate the old database password.</t>
         </is>
       </c>
       <c r="E338" s="14" t="inlineStr">
@@ -8621,7 +8621,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -8855,7 +8855,7 @@
       <c r="A13" s="4" t="n"/>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Site-wide: logo (light + dark) beyond the current text wordmark</t>
+          <t>92 posts still need a real, unique hero image</t>
         </is>
       </c>
       <c r="C13" s="16" t="inlineStr">
@@ -8865,7 +8865,7 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>(Default/fallback OG image 1200×630 exists: public/images/default-og.png, checked 2026-10-02.)</t>
+          <t>(down from 99). Tracked one row per post, with a suggested image-generation prompt, in BLOG-IMAGE-BRIEFS.md — work through that file and check items off there, not here. No image-generation tool was connected in this environment as of this writing; either connect one (e.g. an MCP image-gen extension), source these manually/with a designer then upload via Sanity Studio (/studio), or re-check the live legacy site periodically per the correction note above.</t>
         </is>
       </c>
       <c r="E13" s="14" t="inlineStr">
@@ -8878,7 +8878,7 @@
       <c r="A14" s="4" t="n"/>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>92 posts still need a real, unique hero image</t>
+          <t>Assessment result-screen background art (flagged in STATUS.md as a known gap</t>
         </is>
       </c>
       <c r="C14" s="16" t="inlineStr">
@@ -8888,7 +8888,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>(down from 99). Tracked one row per post, with a suggested image-generation prompt, in BLOG-IMAGE-BRIEFS.md — work through that file and check items off there, not here. No image-generation tool was connected in this environment as of this writing; either connect one (e.g. an MCP image-gen extension), source these manually/with a designer then upload via Sanity Studio (/studio), or re-check the live legacy site periodically per the correction note above.</t>
+          <t>18/20 assessments currently have plain black backgrounds; sourcing themed art here also closes that gap)</t>
         </is>
       </c>
       <c r="E14" s="14" t="inlineStr">
@@ -8898,43 +8898,43 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="n"/>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>Assessment result-screen background art (flagged in STATUS.md as a known gap</t>
-        </is>
-      </c>
-      <c r="C15" s="16" t="inlineStr">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>Phase 14 — QA &amp; Launch</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="n"/>
+      <c r="C15" s="11" t="n"/>
+      <c r="D15" s="12" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="n"/>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Mobile responsive pass on every ported section</t>
+        </is>
+      </c>
+      <c r="C16" s="16" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>18/20 assessments currently have plain black backgrounds; sourcing themed art here also closes that gap)</t>
-        </is>
-      </c>
-      <c r="E15" s="14" t="inlineStr">
-        <is>
-          <t>Phase 13 — Images Needed in Sanity</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="10" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-29: no page scrolls sideways at 375px any more (114 pages checked in Chrome: every unique page plus 3 of each templated set like blog posts and coffees). Fixed: BrewSoul NextSteps forced 3 columns (and used an inline style), charity-scorecard tab row, /brewsoul/browse filter dropdowns, /the-philosophy hero glow. Still to check by hand: 44px tap targets and Safari iOS. 2026-09-30: 44px tap targets on phones for the shared header, footer, BrewSoul/Kava/HumanOS menus and ~100 standalone links (undersized targets 1,904 → 578; the rest are 24-43px pills/chips that meet WCAG 2.2 AA). axe target-size (WCAG 2.2 AA, with its spacing exception): 0 failures on 114 pages. Safari/iPhone (WebKit, iPhone 14 emulation): all 114 pages load, no sideways scroll, no JS errors; form fields under 16px (iOS zoom-on-tap) fixed site-wide in globals.css. Still to check on a real iPhone: BrewSoul's bottom journey bar showed page text through it in headless WebKit only (taps hit the bar correctly; Chrome renders it solid). Fixed 2026-10-09: the bar is now solid (bg-[#2C1810], was 92% plus backdrop-blur-md), so nothing can show through even where the blur isn't drawn; checked in WebKit (iPhone 13 profile) and Chrome: background rgb(44, 24, 16), no text behind the buttons. A real iPhone check is still part of Phase 14.</t>
+        </is>
+      </c>
+      <c r="E16" s="14" t="inlineStr">
         <is>
           <t>Phase 14 — QA &amp; Launch</t>
         </is>
       </c>
-      <c r="B16" s="11" t="n"/>
-      <c r="C16" s="11" t="n"/>
-      <c r="D16" s="12" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n"/>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Mobile responsive pass on every ported section</t>
+          <t>Cross-browser check (Safari iOS in particular, per legacy performance notes) 2026-10-06 WebKit pass (Playwright WebKit, iPhone 13 profile, 1…</t>
         </is>
       </c>
       <c r="C17" s="16" t="inlineStr">
@@ -8944,7 +8944,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>2026-09-29: no page scrolls sideways at 375px any more (114 pages checked in Chrome: every unique page plus 3 of each templated set like blog posts and coffees). Fixed: BrewSoul NextSteps forced 3 columns (and used an inline style), charity-scorecard tab row, /brewsoul/browse filter dropdowns, /the-philosophy hero glow. Still to check by hand: 44px tap targets and Safari iOS. 2026-09-30: 44px tap targets on phones for the shared header, footer, BrewSoul/Kava/HumanOS menus and ~100 standalone links (undersized targets 1,904 → 578; the rest are 24-43px pills/chips that meet WCAG 2.2 AA). axe target-size (WCAG 2.2 AA, with its spacing exception): 0 failures on 114 pages. Safari/iPhone (WebKit, iPhone 14 emulation): all 114 pages load, no sideways scroll, no JS errors; form fields under 16px (iOS zoom-on-tap) fixed site-wide in globals.css. Still to check on a real iPhone: BrewSoul's bottom journey bar showed page text through it in headless WebKit only (taps hit the bar correctly; Chrome renders it solid). Fixed 2026-10-09: the bar is now solid (bg-[#2C1810], was 92% plus backdrop-blur-md), so nothing can show through even where the blur isn't drawn; checked in WebKit (iPhone 13 profile) and Chrome: background rgb(44, 24, 16), no text behind the buttons. A real iPhone check is still part of Phase 14.</t>
+          <t>52 pages: every unique page plus 3 of each templated set, production build): no page pans sideways, no failed requests, no JS errors. Found and fixed on the way: upgrade-insecure-requests in the new CSP made Safari fetch every stylesheet and font over https on localhost (dropped; the site is HTTPS-only via HSTS anyway), and .toLocaleString() without a locale caused a hydration error on /brewsoul/chains in Safari (all number formatting now en-US). Left: a check on a real iPhone (Phase 14).</t>
         </is>
       </c>
       <c r="E17" s="14" t="inlineStr">
@@ -8957,7 +8957,7 @@
       <c r="A18" s="4" t="n"/>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Cross-browser check (Safari iOS in particular, per legacy performance notes) 2026-10-06 WebKit pass (Playwright WebKit, iPhone 13 profile, 1…</t>
+          <t>Remove noindex only when sign-off is given</t>
         </is>
       </c>
       <c r="C18" s="16" t="inlineStr">
@@ -8967,7 +8967,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>52 pages: every unique page plus 3 of each templated set, production build): no page pans sideways, no failed requests, no JS errors. Found and fixed on the way: upgrade-insecure-requests in the new CSP made Safari fetch every stylesheet and font over https on localhost (dropped; the site is HTTPS-only via HSTS anyway), and .toLocaleString() without a locale caused a hydration error on /brewsoul/chains in Safari (all number formatting now en-US). Left: a check on a real iPhone (Phase 14).</t>
+          <t>do not launch indexable by accident (The only noindex is the host-based one for *.netlify.app above, so the real domain is indexable as soon as DNS points at it: sign-off must come before DNS.) Re-checked 2026-10-13 on a fresh production build: tonygreenberg.com and www get no X-Robots-Tag and no robots meta (/, /blog, /about, /post-intervention), *.netlify.app gets noindex, nofollow; robots.txt allows crawlers, sitemap 200, missing pages 404, /manifesto 308. Ready; still waits on sign-off.</t>
         </is>
       </c>
       <c r="E18" s="14" t="inlineStr">
@@ -8980,7 +8980,7 @@
       <c r="A19" s="4" t="n"/>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Remove noindex only when sign-off is given</t>
+          <t>Final stakeholder sign-off (Tony/Darryl/Kimberly) on the ported site before DNS cutover</t>
         </is>
       </c>
       <c r="C19" s="16" t="inlineStr">
@@ -8988,11 +8988,7 @@
           <t>Remaining</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>do not launch indexable by accident (The only noindex is the host-based one for *.netlify.app above, so the real domain is indexable as soon as DNS points at it: sign-off must come before DNS.)</t>
-        </is>
-      </c>
+      <c r="D19" s="4" t="inlineStr"/>
       <c r="E19" s="14" t="inlineStr">
         <is>
           <t>Phase 14 — QA &amp; Launch</t>
@@ -9003,7 +8999,7 @@
       <c r="A20" s="4" t="n"/>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Final stakeholder sign-off (Tony/Darryl/Kimberly) on the ported site before DNS cutover</t>
+          <t>DNS cutover, legacy app decommissioned only after a stable overlap window Re-checked 2026-10-13</t>
         </is>
       </c>
       <c r="C20" s="16" t="inlineStr">
@@ -9011,43 +9007,24 @@
           <t>Remaining</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr"/>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>unchanged (Hostinger name servers, bare domain on Manus 104.19.168/169.112, www CNAME cname.manus.space). Checked 2026-10-09 (owner wants to go live and switch off Manus): DNS for tonygreenberg.com is at Hostinger (name servers ns1/ns2.dns-parking.com); www is a CNAME to cname.manus.space, the bare domain points at Manus's addresses (104.19.168.112 / .169.112); the Netlify site tonygreenberg-website has no custom domain yet (production branch main). Order: (1) merge the three open pull requests into main and check the Netlify copy; (2) restore Supabase and run 0001 to 0003, or launch without member features (they say "isn't available just now"); (3) owner sign-off; (4) add tonygreenberg.com + www in Netlify (Domain management), then at Hostinger point the bare domain at Netlify (A record 75.2.60.5, or Netlify DNS) and www CNAME at tonygreenberg-website.netlify.app; Netlify issues the HTTPS certificate; (5) re-run scripts/check-search-console-urls.ts https://tonygreenberg.com and submit the sitemap in Search Console; (6) only after a few stable days: switch off the Manus site (the database is already backed up, docs/ai/project_legacy_database.md) and rotate the old database password.</t>
+        </is>
+      </c>
       <c r="E20" s="14" t="inlineStr">
         <is>
           <t>Phase 14 — QA &amp; Launch</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="4" t="n"/>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>DNS cutover, legacy app decommissioned only after a stable overlap window Checked 2026-10-09 (owner wants to go live and switch off Manus)</t>
-        </is>
-      </c>
-      <c r="C21" s="16" t="inlineStr">
-        <is>
-          <t>Remaining</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>DNS for tonygreenberg.com is at Hostinger (name servers ns1/ns2.dns-parking.com); www is a CNAME to cname.manus.space, the bare domain points at Manus's addresses (104.19.168.112 / .169.112); the Netlify site tonygreenberg-website has no custom domain yet (production branch main). Order: (1) merge the three open pull requests into main and check the Netlify copy; (2) restore Supabase and run 0001 to 0003, or launch without member features (they say "isn't available just now"); (3) owner sign-off; (4) add tonygreenberg.com + www in Netlify (Domain management), then at Hostinger point the bare domain at Netlify (A record 75.2.60.5, or Netlify DNS) and www CNAME at tonygreenberg-website.netlify.app; Netlify issues the HTTPS certificate; (5) re-run scripts/check-search-console-urls.ts https://tonygreenberg.com and submit the sitemap in Search Console; (6) only after a few stable days: switch off the Manus site (the database is already backed up, docs/ai/project_legacy_database.md) and rotate the old database password.</t>
-        </is>
-      </c>
-      <c r="E21" s="14" t="inlineStr">
-        <is>
-          <t>Phase 14 — QA &amp; Launch</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:D21"/>
+  <autoFilter ref="A1:D20"/>
   <mergeCells count="5">
     <mergeCell ref="A9:D9"/>
     <mergeCell ref="A12:D12"/>
     <mergeCell ref="A4:D4"/>
-    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="A15:D15"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Colour backgrounds on dark quiz results; generated hero art for 92 essays
- /find-your-journey result, /my-journey, /pri-calibration and the PRI
  assessment section: dark colour gradients instead of flat black (owner
  said yes; text stays light, axe contrast 0 at 375/1280).
- Essay heroes: scripts to generate text-free art in the default arch's
  family and set it on the 92 posts without their own picture (owner said
  yes; published, only drafts whose sole change was the picture).
- Status file and spreadsheet updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Migration-Status-Report.xlsx
+++ b/Migration-Status-Report.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Full Detail'!$A$1:$D$338</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Remaining Work'!$A$1:$D$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Remaining Work'!$A$1:$D$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -8157,14 +8157,14 @@
           <t>92 posts still need a real, unique hero image</t>
         </is>
       </c>
-      <c r="C319" s="16" t="inlineStr">
-        <is>
-          <t>Remaining</t>
+      <c r="C319" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D319" s="4" t="inlineStr">
         <is>
-          <t>(down from 99). Tracked one row per post, with a suggested image-generation prompt, in BLOG-IMAGE-BRIEFS.md — work through that file and check items off there, not here. No image-generation tool was connected in this environment as of this writing; either connect one (e.g. an MCP image-gen extension), source these manually/with a designer then upload via Sanity Studio (/studio), or re-check the live legacy site periodically per the correction note above.</t>
+          <t>(down from 99). 2026-10-13 (owner: "image you can add in Sanity"): generated a unique, text-free picture for each of the 92 (live's default-arch family: cream over a deep colour, gold line geometry, colour and motif by category, layout from the slug; scripts/generate-essay-hero-art.mjs) and set it as each post's heroImage draft (scripts/upload-essay-hero-art-2026-10-13.ts; dry run first: 92 found, none had art, nothing replaced). Checked in Sanity: 92 drafts carry the new image, 0 published posts changed. Published 2026-10-13 (owner: yes) with the script's --publish (only drafts whose sole change was the picture; 92 of 92). Checked: the Netlify copy's essay page now serves the new image (webhook refresh). Real photography can still replace any of them later. Tracked one row per post, with a suggested image-generation prompt, in BLOG-IMAGE-BRIEFS.md — work through that file and check items off there, not here. No image-generation tool was connected in this environment as of this writing; either connect one (e.g. an MCP image-gen extension), source these manually/with a designer then upload via Sanity Studio (/studio), or re-check the live legacy site periodically per the correction note above.</t>
         </is>
       </c>
       <c r="E319" s="14" t="inlineStr">
@@ -8364,14 +8364,14 @@
           <t>Assessment result-screen background art (flagged in STATUS.md as a known gap</t>
         </is>
       </c>
-      <c r="C328" s="16" t="inlineStr">
-        <is>
-          <t>Remaining</t>
+      <c r="C328" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D328" s="4" t="inlineStr">
         <is>
-          <t>18/20 assessments currently have plain black backgrounds; sourcing themed art here also closes that gap)</t>
+          <t>18/20 assessments currently have plain black backgrounds; sourcing themed art here also closes that gap) Done 2026-10-13 with colour instead of art (owner: "yes" to colour backgrounds). About 20 quizzes already had a coloured background (ThemedBackground, light per-theme gradients). The 4 still flat dark now have a dark colour gradient, kept dark so their light text stays readable: /find-your-journey result (purple to teal), /my-journey (its black layer hid the gradient; now green to purple), /pri-calibration and the /psychedelic-readiness-index assessment section (PRI ink to amber to plum, starting at ink so the photo band's fade still meets it). Checked: type check, lint, build (all 8 colours in the compiled CSS), screenshots at 375/820/1280 (quiz completed for the journey result), no sideways scroll or JS errors, axe colour-contrast 0 at 375 and 1280.</t>
         </is>
       </c>
       <c r="E328" s="14" t="inlineStr">
@@ -8621,7 +8621,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -8844,7 +8844,7 @@
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>Phase 13 — Images Needed in Sanity</t>
+          <t>Phase 14 — QA &amp; Launch</t>
         </is>
       </c>
       <c r="B12" s="11" t="n"/>
@@ -8855,7 +8855,7 @@
       <c r="A13" s="4" t="n"/>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>92 posts still need a real, unique hero image</t>
+          <t>Mobile responsive pass on every ported section</t>
         </is>
       </c>
       <c r="C13" s="16" t="inlineStr">
@@ -8865,12 +8865,12 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>(down from 99). Tracked one row per post, with a suggested image-generation prompt, in BLOG-IMAGE-BRIEFS.md — work through that file and check items off there, not here. No image-generation tool was connected in this environment as of this writing; either connect one (e.g. an MCP image-gen extension), source these manually/with a designer then upload via Sanity Studio (/studio), or re-check the live legacy site periodically per the correction note above.</t>
+          <t>2026-09-29: no page scrolls sideways at 375px any more (114 pages checked in Chrome: every unique page plus 3 of each templated set like blog posts and coffees). Fixed: BrewSoul NextSteps forced 3 columns (and used an inline style), charity-scorecard tab row, /brewsoul/browse filter dropdowns, /the-philosophy hero glow. Still to check by hand: 44px tap targets and Safari iOS. 2026-09-30: 44px tap targets on phones for the shared header, footer, BrewSoul/Kava/HumanOS menus and ~100 standalone links (undersized targets 1,904 → 578; the rest are 24-43px pills/chips that meet WCAG 2.2 AA). axe target-size (WCAG 2.2 AA, with its spacing exception): 0 failures on 114 pages. Safari/iPhone (WebKit, iPhone 14 emulation): all 114 pages load, no sideways scroll, no JS errors; form fields under 16px (iOS zoom-on-tap) fixed site-wide in globals.css. Still to check on a real iPhone: BrewSoul's bottom journey bar showed page text through it in headless WebKit only (taps hit the bar correctly; Chrome renders it solid). Fixed 2026-10-09: the bar is now solid (bg-[#2C1810], was 92% plus backdrop-blur-md), so nothing can show through even where the blur isn't drawn; checked in WebKit (iPhone 13 profile) and Chrome: background rgb(44, 24, 16), no text behind the buttons. A real iPhone check is still part of Phase 14.</t>
         </is>
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>Phase 13 — Images Needed in Sanity</t>
+          <t>Phase 14 — QA &amp; Launch</t>
         </is>
       </c>
     </row>
@@ -8878,7 +8878,7 @@
       <c r="A14" s="4" t="n"/>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Assessment result-screen background art (flagged in STATUS.md as a known gap</t>
+          <t>Cross-browser check (Safari iOS in particular, per legacy performance notes) 2026-10-06 WebKit pass (Playwright WebKit, iPhone 13 profile, 1…</t>
         </is>
       </c>
       <c r="C14" s="16" t="inlineStr">
@@ -8888,30 +8888,43 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>18/20 assessments currently have plain black backgrounds; sourcing themed art here also closes that gap)</t>
+          <t>52 pages: every unique page plus 3 of each templated set, production build): no page pans sideways, no failed requests, no JS errors. Found and fixed on the way: upgrade-insecure-requests in the new CSP made Safari fetch every stylesheet and font over https on localhost (dropped; the site is HTTPS-only via HSTS anyway), and .toLocaleString() without a locale caused a hydration error on /brewsoul/chains in Safari (all number formatting now en-US). Left: a check on a real iPhone (Phase 14).</t>
         </is>
       </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
-          <t>Phase 13 — Images Needed in Sanity</t>
+          <t>Phase 14 — QA &amp; Launch</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="inlineStr">
+      <c r="A15" s="4" t="n"/>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Remove noindex only when sign-off is given</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>Remaining</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>do not launch indexable by accident (The only noindex is the host-based one for *.netlify.app above, so the real domain is indexable as soon as DNS points at it: sign-off must come before DNS.) Re-checked 2026-10-13 on a fresh production build: tonygreenberg.com and www get no X-Robots-Tag and no robots meta (/, /blog, /about, /post-intervention), *.netlify.app gets noindex, nofollow; robots.txt allows crawlers, sitemap 200, missing pages 404, /manifesto 308. Ready; still waits on sign-off.</t>
+        </is>
+      </c>
+      <c r="E15" s="14" t="inlineStr">
         <is>
           <t>Phase 14 — QA &amp; Launch</t>
         </is>
       </c>
-      <c r="B15" s="11" t="n"/>
-      <c r="C15" s="11" t="n"/>
-      <c r="D15" s="12" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n"/>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Mobile responsive pass on every ported section</t>
+          <t>Final stakeholder sign-off (Tony/Darryl/Kimberly) on the ported site before DNS cutover</t>
         </is>
       </c>
       <c r="C16" s="16" t="inlineStr">
@@ -8919,11 +8932,7 @@
           <t>Remaining</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-29: no page scrolls sideways at 375px any more (114 pages checked in Chrome: every unique page plus 3 of each templated set like blog posts and coffees). Fixed: BrewSoul NextSteps forced 3 columns (and used an inline style), charity-scorecard tab row, /brewsoul/browse filter dropdowns, /the-philosophy hero glow. Still to check by hand: 44px tap targets and Safari iOS. 2026-09-30: 44px tap targets on phones for the shared header, footer, BrewSoul/Kava/HumanOS menus and ~100 standalone links (undersized targets 1,904 → 578; the rest are 24-43px pills/chips that meet WCAG 2.2 AA). axe target-size (WCAG 2.2 AA, with its spacing exception): 0 failures on 114 pages. Safari/iPhone (WebKit, iPhone 14 emulation): all 114 pages load, no sideways scroll, no JS errors; form fields under 16px (iOS zoom-on-tap) fixed site-wide in globals.css. Still to check on a real iPhone: BrewSoul's bottom journey bar showed page text through it in headless WebKit only (taps hit the bar correctly; Chrome renders it solid). Fixed 2026-10-09: the bar is now solid (bg-[#2C1810], was 92% plus backdrop-blur-md), so nothing can show through even where the blur isn't drawn; checked in WebKit (iPhone 13 profile) and Chrome: background rgb(44, 24, 16), no text behind the buttons. A real iPhone check is still part of Phase 14.</t>
-        </is>
-      </c>
+      <c r="D16" s="4" t="inlineStr"/>
       <c r="E16" s="14" t="inlineStr">
         <is>
           <t>Phase 14 — QA &amp; Launch</t>
@@ -8934,7 +8943,7 @@
       <c r="A17" s="4" t="n"/>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Cross-browser check (Safari iOS in particular, per legacy performance notes) 2026-10-06 WebKit pass (Playwright WebKit, iPhone 13 profile, 1…</t>
+          <t>DNS cutover, legacy app decommissioned only after a stable overlap window Re-checked 2026-10-13</t>
         </is>
       </c>
       <c r="C17" s="16" t="inlineStr">
@@ -8944,7 +8953,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>52 pages: every unique page plus 3 of each templated set, production build): no page pans sideways, no failed requests, no JS errors. Found and fixed on the way: upgrade-insecure-requests in the new CSP made Safari fetch every stylesheet and font over https on localhost (dropped; the site is HTTPS-only via HSTS anyway), and .toLocaleString() without a locale caused a hydration error on /brewsoul/chains in Safari (all number formatting now en-US). Left: a check on a real iPhone (Phase 14).</t>
+          <t>unchanged (Hostinger name servers, bare domain on Manus 104.19.168/169.112, www CNAME cname.manus.space). Checked 2026-10-09 (owner wants to go live and switch off Manus): DNS for tonygreenberg.com is at Hostinger (name servers ns1/ns2.dns-parking.com); www is a CNAME to cname.manus.space, the bare domain points at Manus's addresses (104.19.168.112 / .169.112); the Netlify site tonygreenberg-website has no custom domain yet (production branch main). Order: (1) merge the three open pull requests into main and check the Netlify copy; (2) restore Supabase and run 0001 to 0003, or launch without member features (they say "isn't available just now"); (3) owner sign-off; (4) add tonygreenberg.com + www in Netlify (Domain management), then at Hostinger point the bare domain at Netlify (A record 75.2.60.5, or Netlify DNS) and www CNAME at tonygreenberg-website.netlify.app; Netlify issues the HTTPS certificate; (5) re-run scripts/check-search-console-urls.ts https://tonygreenberg.com and submit the sitemap in Search Console; (6) only after a few stable days: switch off the Manus site (the database is already backed up, docs/ai/project_legacy_database.md) and rotate the old database password.</t>
         </is>
       </c>
       <c r="E17" s="14" t="inlineStr">
@@ -8953,78 +8962,12 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="4" t="n"/>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>Remove noindex only when sign-off is given</t>
-        </is>
-      </c>
-      <c r="C18" s="16" t="inlineStr">
-        <is>
-          <t>Remaining</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>do not launch indexable by accident (The only noindex is the host-based one for *.netlify.app above, so the real domain is indexable as soon as DNS points at it: sign-off must come before DNS.) Re-checked 2026-10-13 on a fresh production build: tonygreenberg.com and www get no X-Robots-Tag and no robots meta (/, /blog, /about, /post-intervention), *.netlify.app gets noindex, nofollow; robots.txt allows crawlers, sitemap 200, missing pages 404, /manifesto 308. Ready; still waits on sign-off.</t>
-        </is>
-      </c>
-      <c r="E18" s="14" t="inlineStr">
-        <is>
-          <t>Phase 14 — QA &amp; Launch</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="n"/>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>Final stakeholder sign-off (Tony/Darryl/Kimberly) on the ported site before DNS cutover</t>
-        </is>
-      </c>
-      <c r="C19" s="16" t="inlineStr">
-        <is>
-          <t>Remaining</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="inlineStr"/>
-      <c r="E19" s="14" t="inlineStr">
-        <is>
-          <t>Phase 14 — QA &amp; Launch</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="n"/>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>DNS cutover, legacy app decommissioned only after a stable overlap window Re-checked 2026-10-13</t>
-        </is>
-      </c>
-      <c r="C20" s="16" t="inlineStr">
-        <is>
-          <t>Remaining</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>unchanged (Hostinger name servers, bare domain on Manus 104.19.168/169.112, www CNAME cname.manus.space). Checked 2026-10-09 (owner wants to go live and switch off Manus): DNS for tonygreenberg.com is at Hostinger (name servers ns1/ns2.dns-parking.com); www is a CNAME to cname.manus.space, the bare domain points at Manus's addresses (104.19.168.112 / .169.112); the Netlify site tonygreenberg-website has no custom domain yet (production branch main). Order: (1) merge the three open pull requests into main and check the Netlify copy; (2) restore Supabase and run 0001 to 0003, or launch without member features (they say "isn't available just now"); (3) owner sign-off; (4) add tonygreenberg.com + www in Netlify (Domain management), then at Hostinger point the bare domain at Netlify (A record 75.2.60.5, or Netlify DNS) and www CNAME at tonygreenberg-website.netlify.app; Netlify issues the HTTPS certificate; (5) re-run scripts/check-search-console-urls.ts https://tonygreenberg.com and submit the sitemap in Search Console; (6) only after a few stable days: switch off the Manus site (the database is already backed up, docs/ai/project_legacy_database.md) and rotate the old database password.</t>
-        </is>
-      </c>
-      <c r="E20" s="14" t="inlineStr">
-        <is>
-          <t>Phase 14 — QA &amp; Launch</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:D20"/>
-  <mergeCells count="5">
-    <mergeCell ref="A9:D9"/>
+  <autoFilter ref="A1:D17"/>
+  <mergeCells count="4">
     <mergeCell ref="A12:D12"/>
     <mergeCell ref="A4:D4"/>
-    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A9:D9"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Status: iPhone check done in the iOS Simulator; Google speed test dropped
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Migration-Status-Report.xlsx
+++ b/Migration-Status-Report.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Full Detail'!$A$1:$D$338</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Remaining Work'!$A$1:$D$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Remaining Work'!$A$1:$D$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -6853,14 +6853,14 @@
           <t>Blocked on you (Google)</t>
         </is>
       </c>
-      <c r="C261" s="16" t="inlineStr">
-        <is>
-          <t>Remaining</t>
+      <c r="C261" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D261" s="4" t="inlineStr">
         <is>
-          <t>create a GOOGLE_API_KEY in Google Cloud (project of the vcos-ga4-reader service account, where the PageSpeed Insights API is already on), restricted to the PageSpeed Insights API, then add it to .env.local and Netlify. Creating it from here was blocked by the session's safety check (it would use the service account's credentials to change the Cloud project). Note lighthouse_check_page may time out on Netlify (10 s function limit on the free plan).</t>
+          <t>create a GOOGLE_API_KEY in Google Cloud (project of the vcos-ga4-reader service account, where the PageSpeed Insights API is already on), restricted to the PageSpeed Insights API, then add it to .env.local and Netlify. Creating it from here was blocked by the session's safety check (it would use the service account's credentials to change the Cloud project). Note lighthouse_check_page may time out on Netlify (10 s function limit on the free plan). Dropped 2026-10-13 (owner: "pagespeed.web.dev you can remove"): no Google key or US PageSpeed run needed.</t>
         </is>
       </c>
       <c r="E261" s="14" t="inlineStr">
@@ -7484,9 +7484,9 @@
           <t>Lighthouse pass (performance/accessibility/SEO) on top 20 pages by traffic 2026-09-30, 20 key pages (no traffic data yet), local production …</t>
         </is>
       </c>
-      <c r="C289" s="16" t="inlineStr">
-        <is>
-          <t>Remaining</t>
+      <c r="C289" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D289" s="4" t="inlineStr">
@@ -8443,14 +8443,14 @@
           <t>Mobile responsive pass on every ported section</t>
         </is>
       </c>
-      <c r="C332" s="16" t="inlineStr">
-        <is>
-          <t>Remaining</t>
+      <c r="C332" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D332" s="4" t="inlineStr">
         <is>
-          <t>2026-09-29: no page scrolls sideways at 375px any more (114 pages checked in Chrome: every unique page plus 3 of each templated set like blog posts and coffees). Fixed: BrewSoul NextSteps forced 3 columns (and used an inline style), charity-scorecard tab row, /brewsoul/browse filter dropdowns, /the-philosophy hero glow. Still to check by hand: 44px tap targets and Safari iOS. 2026-09-30: 44px tap targets on phones for the shared header, footer, BrewSoul/Kava/HumanOS menus and ~100 standalone links (undersized targets 1,904 → 578; the rest are 24-43px pills/chips that meet WCAG 2.2 AA). axe target-size (WCAG 2.2 AA, with its spacing exception): 0 failures on 114 pages. Safari/iPhone (WebKit, iPhone 14 emulation): all 114 pages load, no sideways scroll, no JS errors; form fields under 16px (iOS zoom-on-tap) fixed site-wide in globals.css. Still to check on a real iPhone: BrewSoul's bottom journey bar showed page text through it in headless WebKit only (taps hit the bar correctly; Chrome renders it solid). Fixed 2026-10-09: the bar is now solid (bg-[#2C1810], was 92% plus backdrop-blur-md), so nothing can show through even where the blur isn't drawn; checked in WebKit (iPhone 13 profile) and Chrome: background rgb(44, 24, 16), no text behind the buttons. A real iPhone check is still part of Phase 14.</t>
+          <t>2026-09-29: no page scrolls sideways at 375px any more (114 pages checked in Chrome: every unique page plus 3 of each templated set like blog posts and coffees). Fixed: BrewSoul NextSteps forced 3 columns (and used an inline style), charity-scorecard tab row, /brewsoul/browse filter dropdowns, /the-philosophy hero glow. Still to check by hand: 44px tap targets and Safari iOS. 2026-09-30: 44px tap targets on phones for the shared header, footer, BrewSoul/Kava/HumanOS menus and ~100 standalone links (undersized targets 1,904 → 578; the rest are 24-43px pills/chips that meet WCAG 2.2 AA). axe target-size (WCAG 2.2 AA, with its spacing exception): 0 failures on 114 pages. Safari/iPhone (WebKit, iPhone 14 emulation): all 114 pages load, no sideways scroll, no JS errors; form fields under 16px (iOS zoom-on-tap) fixed site-wide in globals.css. Still to check on a real iPhone: BrewSoul's bottom journey bar showed page text through it in headless WebKit only (taps hit the bar correctly; Chrome renders it solid). Fixed 2026-10-09: the bar is now solid (bg-[#2C1810], was 92% plus backdrop-blur-md), so nothing can show through even where the blur isn't drawn; checked in WebKit (iPhone 13 profile) and Chrome: background rgb(44, 24, 16), no text behind the buttons. A real iPhone check is still part of Phase 14. Checked 2026-10-13 in Apple's iPhone Simulator (iPhone 16, iOS 26.5, real Mobile Safari; not a physical phone, owner accepted this as the iPhone check): 14 key pages on a fresh prod</t>
         </is>
       </c>
       <c r="E332" s="14" t="inlineStr">
@@ -8512,14 +8512,14 @@
           <t>Cross-browser check (Safari iOS in particular, per legacy performance notes) 2026-10-06 WebKit pass (Playwright WebKit, iPhone 13 profile, 1…</t>
         </is>
       </c>
-      <c r="C335" s="16" t="inlineStr">
-        <is>
-          <t>Remaining</t>
+      <c r="C335" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D335" s="4" t="inlineStr">
         <is>
-          <t>52 pages: every unique page plus 3 of each templated set, production build): no page pans sideways, no failed requests, no JS errors. Found and fixed on the way: upgrade-insecure-requests in the new CSP made Safari fetch every stylesheet and font over https on localhost (dropped; the site is HTTPS-only via HSTS anyway), and .toLocaleString() without a locale caused a hydration error on /brewsoul/chains in Safari (all number formatting now en-US). Left: a check on a real iPhone (Phase 14).</t>
+          <t>52 pages: every unique page plus 3 of each templated set, production build): no page pans sideways, no failed requests, no JS errors. Found and fixed on the way: upgrade-insecure-requests in the new CSP made Safari fetch every stylesheet and font over https on localhost (dropped; the site is HTTPS-only via HSTS anyway), and .toLocaleString() without a locale caused a hydration error on /brewsoul/chains in Safari (all number formatting now en-US). Left: a check on a real iPhone (Phase 14). Checked 2026-10-13 in Apple's iPhone Simulator (iPhone 16, iOS 26.5, real Mobile Safari; not a physical phone, owner accepted this as the iPhone check): 14 key pages on a fresh production build (/, /blog, an essay, /brewsoul, /brewsoul/browse, /find-your-journey, /psychedelic-readiness-index, /kava, /humanos, /about, /iboga-ibogaine, /peptide-hall-of-shame, /my-journey, /pri-calibration): all render, no sideways pan, header and menus in place, BrewSoul's bottom bar solid. / and /blog showed blank on the very first cold load, then load within 3 s on every later visit.</t>
         </is>
       </c>
       <c r="E335" s="14" t="inlineStr">
@@ -8621,7 +8621,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -8747,7 +8747,7 @@
       <c r="A7" s="4" t="n"/>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Blocked on you (Google)</t>
+          <t>Test the new review end to end on a deploy preview</t>
         </is>
       </c>
       <c r="C7" s="16" t="inlineStr">
@@ -8757,7 +8757,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>create a GOOGLE_API_KEY in Google Cloud (project of the vcos-ga4-reader service account, where the PageSpeed Insights API is already on), restricted to the PageSpeed Insights API, then add it to .env.local and Netlify. Creating it from here was blocked by the session's safety check (it would use the service account's credentials to change the Cloud project). Note lighthouse_check_page may time out on Netlify (10 s function limit on the free plan).</t>
+          <t>(needs a yes, it opens a real pull request): one throwaway change from Claude.ai or ChatGPT: start (unclear request, so the confirm step shows), confirm, edit, review card, screenshots, upload link, then discard.</t>
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr">
@@ -8767,66 +8767,49 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="n"/>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>Test the new review end to end on a deploy preview</t>
-        </is>
-      </c>
-      <c r="C8" s="16" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="n"/>
+      <c r="C8" s="11" t="n"/>
+      <c r="D8" s="12" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n"/>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Connect Google Search Console + GA4 to the new deployment on day one of cutover</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>(needs a yes, it opens a real pull request): one throwaway change from Claude.ai or ChatGPT: start (unclear request, so the confirm step shows), confirm, edit, review card, screenshots, upload link, then discard.</t>
-        </is>
-      </c>
-      <c r="E8" s="14" t="inlineStr">
-        <is>
-          <t>Phase 11 — Code MCP Server — REBUILT (2026-09-29)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr"/>
+      <c r="E9" s="14" t="inlineStr">
         <is>
           <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
         </is>
       </c>
-      <c r="B9" s="11" t="n"/>
-      <c r="C9" s="11" t="n"/>
-      <c r="D9" s="12" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="n"/>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>Lighthouse pass (performance/accessibility/SEO) on top 20 pages by traffic 2026-09-30, 20 key pages (no traffic data yet), local production …</t>
-        </is>
-      </c>
-      <c r="C10" s="16" t="inlineStr">
-        <is>
-          <t>Remaining</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>build, mobile: averages performance 87, accessibility 99→100, best practices 100, SEO 92→100, CLS 0 everywhere. Fixed: public/robots.txt had an LLMs: line (not a real directive) that made Google treat the whole file as invalid, now a comment; h3/h4 headings skipping a level on /assessments, /kava, /peptide-watch (same look, right tag); the Kava and /attention-theft back-arrow links had no accessible name on phones; two small phone-width contrast misses. Left: performance is local-machine only (±10-15 points, see CONTRIBUTING.md); the slowest were / 76 (LCP 5.2 s), /psychedelic-readiness-index 82, /iboga-ibogaine 83. Re-run against the Netlify deploy before launch. 2026-10-06 re-run against the Netlify deploy (14 key pages, mobile): accessibility 100 and CLS 0 on every page, SEO clean (only the expected netlify.app noindex), performance 77-97 held back by 3-4 s LCP. Fixed: all 21 hero images moved off the deprecated priority prop to fetchPriority="high" + loading="eager" (Next 16); /iboga-ibogaine hero and the first card on /blog and category pages no longer lazy-loaded; sizes on the Four Doors cards (~150 KiB per page), /humanos diagram (~100 KiB) and /about headshot; urlFor no longer imports the Sanity client, so ~115 KB of Sanity client code stopped loading on / and /blog; React hydration error #418 on / and /blog (post dates) gone, checked in two time zones; /blog is static again; empty icon &lt;th&gt;s on /iboga-ibogaine labelled; category page reads use sanityFetch(). Left: se</t>
-        </is>
-      </c>
-      <c r="E10" s="14" t="inlineStr">
-        <is>
-          <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
-        </is>
-      </c>
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>Phase 14 — QA &amp; Launch</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="n"/>
+      <c r="C10" s="11" t="n"/>
+      <c r="D10" s="12" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n"/>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Connect Google Search Console + GA4 to the new deployment on day one of cutover</t>
+          <t>Remove noindex only when sign-off is given</t>
         </is>
       </c>
       <c r="C11" s="16" t="inlineStr">
@@ -8834,28 +8817,41 @@
           <t>Remaining</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr"/>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>do not launch indexable by accident (The only noindex is the host-based one for *.netlify.app above, so the real domain is indexable as soon as DNS points at it: sign-off must come before DNS.) Re-checked 2026-10-13 on a fresh production build: tonygreenberg.com and www get no X-Robots-Tag and no robots meta (/, /blog, /about, /post-intervention), *.netlify.app gets noindex, nofollow; robots.txt allows crawlers, sitemap 200, missing pages 404, /manifesto 308. Ready; still waits on sign-off.</t>
+        </is>
+      </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
+          <t>Phase 14 — QA &amp; Launch</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="inlineStr">
+      <c r="A12" s="4" t="n"/>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Final stakeholder sign-off (Tony/Darryl/Kimberly) on the ported site before DNS cutover</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>Remaining</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr"/>
+      <c r="E12" s="14" t="inlineStr">
         <is>
           <t>Phase 14 — QA &amp; Launch</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n"/>
-      <c r="C12" s="11" t="n"/>
-      <c r="D12" s="12" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n"/>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Mobile responsive pass on every ported section</t>
+          <t>DNS cutover, legacy app decommissioned only after a stable overlap window Re-checked 2026-10-13</t>
         </is>
       </c>
       <c r="C13" s="16" t="inlineStr">
@@ -8865,7 +8861,7 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>2026-09-29: no page scrolls sideways at 375px any more (114 pages checked in Chrome: every unique page plus 3 of each templated set like blog posts and coffees). Fixed: BrewSoul NextSteps forced 3 columns (and used an inline style), charity-scorecard tab row, /brewsoul/browse filter dropdowns, /the-philosophy hero glow. Still to check by hand: 44px tap targets and Safari iOS. 2026-09-30: 44px tap targets on phones for the shared header, footer, BrewSoul/Kava/HumanOS menus and ~100 standalone links (undersized targets 1,904 → 578; the rest are 24-43px pills/chips that meet WCAG 2.2 AA). axe target-size (WCAG 2.2 AA, with its spacing exception): 0 failures on 114 pages. Safari/iPhone (WebKit, iPhone 14 emulation): all 114 pages load, no sideways scroll, no JS errors; form fields under 16px (iOS zoom-on-tap) fixed site-wide in globals.css. Still to check on a real iPhone: BrewSoul's bottom journey bar showed page text through it in headless WebKit only (taps hit the bar correctly; Chrome renders it solid). Fixed 2026-10-09: the bar is now solid (bg-[#2C1810], was 92% plus backdrop-blur-md), so nothing can show through even where the blur isn't drawn; checked in WebKit (iPhone 13 profile) and Chrome: background rgb(44, 24, 16), no text behind the buttons. A real iPhone check is still part of Phase 14.</t>
+          <t>unchanged (Hostinger name servers, bare domain on Manus 104.19.168/169.112, www CNAME cname.manus.space). Checked 2026-10-09 (owner wants to go live and switch off Manus): DNS for tonygreenberg.com is at Hostinger (name servers ns1/ns2.dns-parking.com); www is a CNAME to cname.manus.space, the bare domain points at Manus's addresses (104.19.168.112 / .169.112); the Netlify site tonygreenberg-website has no custom domain yet (production branch main). Order: (1) merge the three open pull requests into main and check the Netlify copy; (2) restore Supabase and run 0001 to 0003, or launch without member features (they say "isn't available just now"); (3) owner sign-off; (4) add tonygreenberg.com + www in Netlify (Domain management), then at Hostinger point the bare domain at Netlify (A record 75.2.60.5, or Netlify DNS) and www CNAME at tonygreenberg-website.netlify.app; Netlify issues the HTTPS certificate; (5) re-run scripts/check-search-console-urls.ts https://tonygreenberg.com and submit the sitemap in Search Console; (6) only after a few stable days: switch off the Manus site (the database is already backed up, docs/ai/project_legacy_database.md) and rotate the old database password.</t>
         </is>
       </c>
       <c r="E13" s="14" t="inlineStr">
@@ -8874,100 +8870,12 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="4" t="n"/>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>Cross-browser check (Safari iOS in particular, per legacy performance notes) 2026-10-06 WebKit pass (Playwright WebKit, iPhone 13 profile, 1…</t>
-        </is>
-      </c>
-      <c r="C14" s="16" t="inlineStr">
-        <is>
-          <t>Remaining</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>52 pages: every unique page plus 3 of each templated set, production build): no page pans sideways, no failed requests, no JS errors. Found and fixed on the way: upgrade-insecure-requests in the new CSP made Safari fetch every stylesheet and font over https on localhost (dropped; the site is HTTPS-only via HSTS anyway), and .toLocaleString() without a locale caused a hydration error on /brewsoul/chains in Safari (all number formatting now en-US). Left: a check on a real iPhone (Phase 14).</t>
-        </is>
-      </c>
-      <c r="E14" s="14" t="inlineStr">
-        <is>
-          <t>Phase 14 — QA &amp; Launch</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="n"/>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>Remove noindex only when sign-off is given</t>
-        </is>
-      </c>
-      <c r="C15" s="16" t="inlineStr">
-        <is>
-          <t>Remaining</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>do not launch indexable by accident (The only noindex is the host-based one for *.netlify.app above, so the real domain is indexable as soon as DNS points at it: sign-off must come before DNS.) Re-checked 2026-10-13 on a fresh production build: tonygreenberg.com and www get no X-Robots-Tag and no robots meta (/, /blog, /about, /post-intervention), *.netlify.app gets noindex, nofollow; robots.txt allows crawlers, sitemap 200, missing pages 404, /manifesto 308. Ready; still waits on sign-off.</t>
-        </is>
-      </c>
-      <c r="E15" s="14" t="inlineStr">
-        <is>
-          <t>Phase 14 — QA &amp; Launch</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="n"/>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>Final stakeholder sign-off (Tony/Darryl/Kimberly) on the ported site before DNS cutover</t>
-        </is>
-      </c>
-      <c r="C16" s="16" t="inlineStr">
-        <is>
-          <t>Remaining</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr"/>
-      <c r="E16" s="14" t="inlineStr">
-        <is>
-          <t>Phase 14 — QA &amp; Launch</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="n"/>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>DNS cutover, legacy app decommissioned only after a stable overlap window Re-checked 2026-10-13</t>
-        </is>
-      </c>
-      <c r="C17" s="16" t="inlineStr">
-        <is>
-          <t>Remaining</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>unchanged (Hostinger name servers, bare domain on Manus 104.19.168/169.112, www CNAME cname.manus.space). Checked 2026-10-09 (owner wants to go live and switch off Manus): DNS for tonygreenberg.com is at Hostinger (name servers ns1/ns2.dns-parking.com); www is a CNAME to cname.manus.space, the bare domain points at Manus's addresses (104.19.168.112 / .169.112); the Netlify site tonygreenberg-website has no custom domain yet (production branch main). Order: (1) merge the three open pull requests into main and check the Netlify copy; (2) restore Supabase and run 0001 to 0003, or launch without member features (they say "isn't available just now"); (3) owner sign-off; (4) add tonygreenberg.com + www in Netlify (Domain management), then at Hostinger point the bare domain at Netlify (A record 75.2.60.5, or Netlify DNS) and www CNAME at tonygreenberg-website.netlify.app; Netlify issues the HTTPS certificate; (5) re-run scripts/check-search-console-urls.ts https://tonygreenberg.com and submit the sitemap in Search Console; (6) only after a few stable days: switch off the Manus site (the database is already backed up, docs/ai/project_legacy_database.md) and rotate the old database password.</t>
-        </is>
-      </c>
-      <c r="E17" s="14" t="inlineStr">
-        <is>
-          <t>Phase 14 — QA &amp; Launch</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:D17"/>
+  <autoFilter ref="A1:D13"/>
   <mergeCells count="4">
-    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A10:D10"/>
     <mergeCell ref="A4:D4"/>
-    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="A8:D8"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Status: sign-off given; Google indexing turns on with the DNS switch
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Migration-Status-Report.xlsx
+++ b/Migration-Status-Report.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Full Detail'!$A$1:$D$338</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Remaining Work'!$A$1:$D$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Remaining Work'!$A$1:$D$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -8535,14 +8535,14 @@
           <t>Remove noindex only when sign-off is given</t>
         </is>
       </c>
-      <c r="C336" s="16" t="inlineStr">
-        <is>
-          <t>Remaining</t>
+      <c r="C336" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D336" s="4" t="inlineStr">
         <is>
-          <t>do not launch indexable by accident (The only noindex is the host-based one for *.netlify.app above, so the real domain is indexable as soon as DNS points at it: sign-off must come before DNS.) Re-checked 2026-10-13 on a fresh production build: tonygreenberg.com and www get no X-Robots-Tag and no robots meta (/, /blog, /about, /post-intervention), *.netlify.app gets noindex, nofollow; robots.txt allows crawlers, sitemap 200, missing pages 404, /manifesto 308. Ready; still waits on sign-off.</t>
+          <t>do not launch indexable by accident (The only noindex is the host-based one for .netlify.app above, so the real domain is indexable as soon as DNS points at it: sign-off must come before DNS.) Re-checked 2026-10-13 on a fresh production build: tonygreenberg.com and www get no X-Robots-Tag and no robots meta (/, /blog, /about, /post-intervention), *.netlify.app gets noindex, nofollow; robots.txt allows crawlers, sitemap 200, missing pages 404, /manifesto 308. Ready; still waits on sign-off. Done 2026-10-13 (sign-off given): nothing to switch off. The only noindex is host-based (.netlify.app), so tonygreenberg.com becomes indexable by Google the moment DNS points at Netlify (re-checked on today's build: no X-Robots-Tag or robots meta for the real domain).</t>
         </is>
       </c>
       <c r="E336" s="14" t="inlineStr">
@@ -8555,15 +8555,19 @@
       <c r="A337" s="4" t="n"/>
       <c r="B337" s="4" t="inlineStr">
         <is>
-          <t>Final stakeholder sign-off (Tony/Darryl/Kimberly) on the ported site before DNS cutover</t>
-        </is>
-      </c>
-      <c r="C337" s="16" t="inlineStr">
-        <is>
-          <t>Remaining</t>
-        </is>
-      </c>
-      <c r="D337" s="4" t="inlineStr"/>
+          <t>Final stakeholder sign-off (Tony/Darryl/Kimberly) on the ported site before DNS cutover Given 2026-10-13 by the webmaster (web.master@rampra…</t>
+        </is>
+      </c>
+      <c r="C337" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D337" s="4" t="inlineStr">
+        <is>
+          <t>te.com) in a Claude Code session, answering "Tony's team sign-off, then turning on Google indexing" with yes. If Tony, Darryl or Kimberly haven't seen the Netlify copy themselves, get their yes before the DNS switch.</t>
+        </is>
+      </c>
       <c r="E337" s="14" t="inlineStr">
         <is>
           <t>Phase 14 — QA &amp; Launch</t>
@@ -8621,7 +8625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -8809,7 +8813,7 @@
       <c r="A11" s="4" t="n"/>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Remove noindex only when sign-off is given</t>
+          <t>DNS cutover, legacy app decommissioned only after a stable overlap window Re-checked 2026-10-13</t>
         </is>
       </c>
       <c r="C11" s="16" t="inlineStr">
@@ -8819,7 +8823,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>do not launch indexable by accident (The only noindex is the host-based one for *.netlify.app above, so the real domain is indexable as soon as DNS points at it: sign-off must come before DNS.) Re-checked 2026-10-13 on a fresh production build: tonygreenberg.com and www get no X-Robots-Tag and no robots meta (/, /blog, /about, /post-intervention), *.netlify.app gets noindex, nofollow; robots.txt allows crawlers, sitemap 200, missing pages 404, /manifesto 308. Ready; still waits on sign-off.</t>
+          <t>unchanged (Hostinger name servers, bare domain on Manus 104.19.168/169.112, www CNAME cname.manus.space). Checked 2026-10-09 (owner wants to go live and switch off Manus): DNS for tonygreenberg.com is at Hostinger (name servers ns1/ns2.dns-parking.com); www is a CNAME to cname.manus.space, the bare domain points at Manus's addresses (104.19.168.112 / .169.112); the Netlify site tonygreenberg-website has no custom domain yet (production branch main). Order: (1) merge the three open pull requests into main and check the Netlify copy; (2) restore Supabase and run 0001 to 0003, or launch without member features (they say "isn't available just now"); (3) owner sign-off; (4) add tonygreenberg.com + www in Netlify (Domain management), then at Hostinger point the bare domain at Netlify (A record 75.2.60.5, or Netlify DNS) and www CNAME at tonygreenberg-website.netlify.app; Netlify issues the HTTPS certificate; (5) re-run scripts/check-search-console-urls.ts https://tonygreenberg.com and submit the sitemap in Search Console; (6) only after a few stable days: switch off the Manus site (the database is already backed up, docs/ai/project_legacy_database.md) and rotate the old database password.</t>
         </is>
       </c>
       <c r="E11" s="14" t="inlineStr">
@@ -8828,50 +8832,8 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="4" t="n"/>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>Final stakeholder sign-off (Tony/Darryl/Kimberly) on the ported site before DNS cutover</t>
-        </is>
-      </c>
-      <c r="C12" s="16" t="inlineStr">
-        <is>
-          <t>Remaining</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr"/>
-      <c r="E12" s="14" t="inlineStr">
-        <is>
-          <t>Phase 14 — QA &amp; Launch</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="n"/>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>DNS cutover, legacy app decommissioned only after a stable overlap window Re-checked 2026-10-13</t>
-        </is>
-      </c>
-      <c r="C13" s="16" t="inlineStr">
-        <is>
-          <t>Remaining</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>unchanged (Hostinger name servers, bare domain on Manus 104.19.168/169.112, www CNAME cname.manus.space). Checked 2026-10-09 (owner wants to go live and switch off Manus): DNS for tonygreenberg.com is at Hostinger (name servers ns1/ns2.dns-parking.com); www is a CNAME to cname.manus.space, the bare domain points at Manus's addresses (104.19.168.112 / .169.112); the Netlify site tonygreenberg-website has no custom domain yet (production branch main). Order: (1) merge the three open pull requests into main and check the Netlify copy; (2) restore Supabase and run 0001 to 0003, or launch without member features (they say "isn't available just now"); (3) owner sign-off; (4) add tonygreenberg.com + www in Netlify (Domain management), then at Hostinger point the bare domain at Netlify (A record 75.2.60.5, or Netlify DNS) and www CNAME at tonygreenberg-website.netlify.app; Netlify issues the HTTPS certificate; (5) re-run scripts/check-search-console-urls.ts https://tonygreenberg.com and submit the sitemap in Search Console; (6) only after a few stable days: switch off the Manus site (the database is already backed up, docs/ai/project_legacy_database.md) and rotate the old database password.</t>
-        </is>
-      </c>
-      <c r="E13" s="14" t="inlineStr">
-        <is>
-          <t>Phase 14 — QA &amp; Launch</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:D13"/>
+  <autoFilter ref="A1:D11"/>
   <mergeCells count="4">
     <mergeCell ref="A10:D10"/>
     <mergeCell ref="A4:D4"/>

</xml_diff>

<commit_message>
Redirect the old Google addresses that were 404 (owner asked)
423 of 430 Search Console addresses now reach a working page (was 410):
/library, /impact, /members, /the-right-numbers-supplier, /portfolio,
/fauxtony, /health(/page/n), /request-a-password and /built-on-manus go to
the closest real page; /shop -> /subscribe is temporary (307) until the
shop exists. /terms, the removed Dr. Lee case file and two stray script
addresses stay 404 on purpose.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Migration-Status-Report.xlsx
+++ b/Migration-Status-Report.xlsx
@@ -3830,7 +3830,7 @@
       </c>
       <c r="D125" s="4" t="inlineStr">
         <is>
-          <t>defer: these are Stripe-backed; flag for the later billing-migration phase, do not port checkout logic yet, static/informational content only if ported now</t>
+          <t>defer: (2026-10-13: /shop temporarily redirects to /subscribe; delete that entry in SEARCH_CONSOLE_TEMPORARY_REDIRECTS when this is built) these are Stripe-backed; flag for the later billing-migration phase, do not port checkout logic yet, static/informational content only if ported now</t>
         </is>
       </c>
       <c r="E125" s="14" t="inlineStr">
@@ -8686,7 +8686,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>defer: these are Stripe-backed; flag for the later billing-migration phase, do not port checkout logic yet, static/informational content only if ported now</t>
+          <t>defer: (2026-10-13: /shop temporarily redirects to /subscribe; delete that entry in SEARCH_CONSOLE_TEMPORARY_REDIRECTS when this is built) these are Stripe-backed; flag for the later billing-migration phase, do not port checkout logic yet, static/informational content only if ported now</t>
         </is>
       </c>
       <c r="E3" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Team review fixes: essay counts, Contact/Privacy/Terms pages, 404 titles
- Essay count comes from Sanity everywhere: homepage Read card, /subscribe,
  /the-letter, and Ask Tony / /search / /the-index (was a hardcoded "92").
- New /contact, /privacy and /terms pages, linked from the footer; footer
  email is now a mailto link. Policy wording drafted from what the site
  collects, for Josh (legal) to review before launch.
- Missing essays and categories use the "Page not found" tab title.
- Explore menu's three Attention Theft links point straight at the page
  sections instead of through a redirect.
- NEXTJS-MIGRATION-TODO.md, ROUTES-INVENTORY.md, PROJECT_STRUCTURE.md and
  the status spreadsheet updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Migration-Status-Report.xlsx
+++ b/Migration-Status-Report.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Remaining Work" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Full Detail'!$A$1:$D$338</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Full Detail'!$A$1:$D$343</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Remaining Work'!$A$1:$D$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -596,7 +596,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated from NEXTJS-MIGRATION-TODO.md on 2026-10-13 by scripts/build-migration-status-report.py — a living document; re-run the script after updating the todo file. Counts are formulas over the Full Detail tab.</t>
+          <t>Generated from NEXTJS-MIGRATION-TODO.md on 2026-10-14 by scripts/build-migration-status-report.py — a living document; re-run the script after updating the todo file. Counts are formulas over the Full Detail tab.</t>
         </is>
       </c>
     </row>
@@ -639,15 +639,15 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A5,'Full Detail'!$C$2:$C$338,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A5,'Full Detail'!$C$2:$C$343,"Done")</f>
         <v/>
       </c>
       <c r="C5" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A5,'Full Detail'!$C$2:$C$338,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A5,'Full Detail'!$C$2:$C$343,"Remaining")</f>
         <v/>
       </c>
       <c r="D5" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A5,'Full Detail'!$C$2:$C$338,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A5,'Full Detail'!$C$2:$C$343,"Deferred")</f>
         <v/>
       </c>
       <c r="E5" s="5">
@@ -666,15 +666,15 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A6,'Full Detail'!$C$2:$C$338,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A6,'Full Detail'!$C$2:$C$343,"Done")</f>
         <v/>
       </c>
       <c r="C6" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A6,'Full Detail'!$C$2:$C$338,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A6,'Full Detail'!$C$2:$C$343,"Remaining")</f>
         <v/>
       </c>
       <c r="D6" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A6,'Full Detail'!$C$2:$C$338,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A6,'Full Detail'!$C$2:$C$343,"Deferred")</f>
         <v/>
       </c>
       <c r="E6" s="5">
@@ -693,15 +693,15 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A7,'Full Detail'!$C$2:$C$338,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A7,'Full Detail'!$C$2:$C$343,"Done")</f>
         <v/>
       </c>
       <c r="C7" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A7,'Full Detail'!$C$2:$C$338,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A7,'Full Detail'!$C$2:$C$343,"Remaining")</f>
         <v/>
       </c>
       <c r="D7" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A7,'Full Detail'!$C$2:$C$338,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A7,'Full Detail'!$C$2:$C$343,"Deferred")</f>
         <v/>
       </c>
       <c r="E7" s="5">
@@ -720,15 +720,15 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A8,'Full Detail'!$C$2:$C$338,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A8,'Full Detail'!$C$2:$C$343,"Done")</f>
         <v/>
       </c>
       <c r="C8" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A8,'Full Detail'!$C$2:$C$338,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A8,'Full Detail'!$C$2:$C$343,"Remaining")</f>
         <v/>
       </c>
       <c r="D8" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A8,'Full Detail'!$C$2:$C$338,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A8,'Full Detail'!$C$2:$C$343,"Deferred")</f>
         <v/>
       </c>
       <c r="E8" s="5">
@@ -747,15 +747,15 @@
         </is>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A9,'Full Detail'!$C$2:$C$338,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A9,'Full Detail'!$C$2:$C$343,"Done")</f>
         <v/>
       </c>
       <c r="C9" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A9,'Full Detail'!$C$2:$C$338,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A9,'Full Detail'!$C$2:$C$343,"Remaining")</f>
         <v/>
       </c>
       <c r="D9" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A9,'Full Detail'!$C$2:$C$338,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A9,'Full Detail'!$C$2:$C$343,"Deferred")</f>
         <v/>
       </c>
       <c r="E9" s="5">
@@ -774,15 +774,15 @@
         </is>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A10,'Full Detail'!$C$2:$C$338,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A10,'Full Detail'!$C$2:$C$343,"Done")</f>
         <v/>
       </c>
       <c r="C10" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A10,'Full Detail'!$C$2:$C$338,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A10,'Full Detail'!$C$2:$C$343,"Remaining")</f>
         <v/>
       </c>
       <c r="D10" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A10,'Full Detail'!$C$2:$C$338,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A10,'Full Detail'!$C$2:$C$343,"Deferred")</f>
         <v/>
       </c>
       <c r="E10" s="5">
@@ -801,15 +801,15 @@
         </is>
       </c>
       <c r="B11" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A11,'Full Detail'!$C$2:$C$338,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A11,'Full Detail'!$C$2:$C$343,"Done")</f>
         <v/>
       </c>
       <c r="C11" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A11,'Full Detail'!$C$2:$C$338,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A11,'Full Detail'!$C$2:$C$343,"Remaining")</f>
         <v/>
       </c>
       <c r="D11" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A11,'Full Detail'!$C$2:$C$338,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A11,'Full Detail'!$C$2:$C$343,"Deferred")</f>
         <v/>
       </c>
       <c r="E11" s="5">
@@ -828,15 +828,15 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A12,'Full Detail'!$C$2:$C$338,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A12,'Full Detail'!$C$2:$C$343,"Done")</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A12,'Full Detail'!$C$2:$C$338,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A12,'Full Detail'!$C$2:$C$343,"Remaining")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A12,'Full Detail'!$C$2:$C$338,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A12,'Full Detail'!$C$2:$C$343,"Deferred")</f>
         <v/>
       </c>
       <c r="E12" s="5">
@@ -855,15 +855,15 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A13,'Full Detail'!$C$2:$C$338,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A13,'Full Detail'!$C$2:$C$343,"Done")</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A13,'Full Detail'!$C$2:$C$338,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A13,'Full Detail'!$C$2:$C$343,"Remaining")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A13,'Full Detail'!$C$2:$C$338,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A13,'Full Detail'!$C$2:$C$343,"Deferred")</f>
         <v/>
       </c>
       <c r="E13" s="5">
@@ -882,15 +882,15 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A14,'Full Detail'!$C$2:$C$338,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A14,'Full Detail'!$C$2:$C$343,"Done")</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A14,'Full Detail'!$C$2:$C$338,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A14,'Full Detail'!$C$2:$C$343,"Remaining")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A14,'Full Detail'!$C$2:$C$338,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A14,'Full Detail'!$C$2:$C$343,"Deferred")</f>
         <v/>
       </c>
       <c r="E14" s="5">
@@ -909,15 +909,15 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A15,'Full Detail'!$C$2:$C$338,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A15,'Full Detail'!$C$2:$C$343,"Done")</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A15,'Full Detail'!$C$2:$C$338,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A15,'Full Detail'!$C$2:$C$343,"Remaining")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A15,'Full Detail'!$C$2:$C$338,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A15,'Full Detail'!$C$2:$C$343,"Deferred")</f>
         <v/>
       </c>
       <c r="E15" s="5">
@@ -936,15 +936,15 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A16,'Full Detail'!$C$2:$C$338,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A16,'Full Detail'!$C$2:$C$343,"Done")</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A16,'Full Detail'!$C$2:$C$338,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A16,'Full Detail'!$C$2:$C$343,"Remaining")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A16,'Full Detail'!$C$2:$C$338,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A16,'Full Detail'!$C$2:$C$343,"Deferred")</f>
         <v/>
       </c>
       <c r="E16" s="5">
@@ -963,15 +963,15 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A17,'Full Detail'!$C$2:$C$338,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A17,'Full Detail'!$C$2:$C$343,"Done")</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A17,'Full Detail'!$C$2:$C$338,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A17,'Full Detail'!$C$2:$C$343,"Remaining")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A17,'Full Detail'!$C$2:$C$338,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A17,'Full Detail'!$C$2:$C$343,"Deferred")</f>
         <v/>
       </c>
       <c r="E17" s="5">
@@ -990,15 +990,15 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A18,'Full Detail'!$C$2:$C$338,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A18,'Full Detail'!$C$2:$C$343,"Done")</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A18,'Full Detail'!$C$2:$C$338,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A18,'Full Detail'!$C$2:$C$343,"Remaining")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A18,'Full Detail'!$C$2:$C$338,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A18,'Full Detail'!$C$2:$C$343,"Deferred")</f>
         <v/>
       </c>
       <c r="E18" s="5">
@@ -1017,15 +1017,15 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A19,'Full Detail'!$C$2:$C$338,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A19,'Full Detail'!$C$2:$C$343,"Done")</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A19,'Full Detail'!$C$2:$C$338,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A19,'Full Detail'!$C$2:$C$343,"Remaining")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$338,$A19,'Full Detail'!$C$2:$C$338,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A19,'Full Detail'!$C$2:$C$343,"Deferred")</f>
         <v/>
       </c>
       <c r="E19" s="5">
@@ -1075,7 +1075,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E338"/>
+  <dimension ref="A1:E343"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -8578,27 +8578,142 @@
       <c r="A338" s="4" t="n"/>
       <c r="B338" s="4" t="inlineStr">
         <is>
+          <t>Privacy Policy page (/privacy) + footer link</t>
+        </is>
+      </c>
+      <c r="C338" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D338" s="4" t="inlineStr">
+        <is>
+          <t>(team review 2026-10-14; owner: "create any page that isn't there"). Neither live nor the old app has one, so it's a new page. Wording drafted from what the code really does: newsletter (Kit), member accounts, quiz results (sexuality/religion save only "finished"), comments/reactions/highlights, the site's forms (Supabase, emailed to Tony via Resend), supplier intake to RampRate, Google Analytics, the sign-in, tg_visit_count and visitor-session cookies, browser storage. Contact for requests: t@ramprate.com (the footer's address). Josh (legal) to review the wording before launch.</t>
+        </is>
+      </c>
+      <c r="E338" s="14" t="inlineStr">
+        <is>
+          <t>Phase 14 — QA &amp; Launch</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" s="4" t="n"/>
+      <c r="B339" s="4" t="inlineStr">
+        <is>
+          <t>Terms of Use page (/terms) + footer link</t>
+        </is>
+      </c>
+      <c r="C339" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D339" s="4" t="inlineStr">
+        <is>
+          <t>(team review 2026-10-14). Not-medical-advice (peptides, diet, therapy, kava, psychedelics, ibogaine) and not-investment-advice (waitlists are not offers) sections, ownership matching the footer notice, user content, liability, California law. /terms was one of the intentional 404s; now a real page (ROUTES-INVENTORY.md updated). Josh (legal) to review before launch.</t>
+        </is>
+      </c>
+      <c r="E339" s="14" t="inlineStr">
+        <is>
+          <t>Phase 14 — QA &amp; Launch</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" s="4" t="n"/>
+      <c r="B340" s="4" t="inlineStr">
+        <is>
+          <t>Contact page (/contact) + footer link</t>
+        </is>
+      </c>
+      <c r="C340" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D340" s="4" t="inlineStr">
+        <is>
+          <t>(team review 2026-10-14). Gathers details already on the site: email t@ramprate.com (now also a clickable link in the footer, where it was plain text), booking link, the Engagement Audit (/pick-up-the-phone), RampRate supplier intake, Santa Monica, X and LinkedIn. No form (none needed: every option already exists). Checked 2026-10-14 for all three: type check, lint, Manus grep, build (all ○ static), fresh server: 200, one H1, title, canonical, share image, in the sitemap and Ask Tony search, footer links on every page; browser at 375/820/1280 light and 375/1280 dark: no sideways scroll, no JS errors.</t>
+        </is>
+      </c>
+      <c r="E340" s="14" t="inlineStr">
+        <is>
+          <t>Phase 14 — QA &amp; Launch</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" s="4" t="n"/>
+      <c r="B341" s="4" t="inlineStr">
+        <is>
+          <t>Essay counts match</t>
+        </is>
+      </c>
+      <c r="C341" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D341" s="4" t="inlineStr">
+        <is>
+          <t>(team review 2026-10-14). Ask Tony's Blog entry said "92 essays" (copied from the old app), the homepage Read card "118", /subscribe and /the-letter's Read card "121", while the homepage and /search count 123 from Sanity. All now use Sanity's count ({count} in home-doors.ts and /the-letter's doors, /subscribe fetches it). Ask Tony (owner: show the number): the root layout fetches the count and passes it to SiteHeader → SearchModal; withEssayCount() in search-directory.ts fills {count} for Ask Tony, /search and /the-index too. Checked in a browser: Ask Tony shows "123 essays spanning 15 years", build still 150 static / 28 dynamic pages as before. Left alone: /living-declaration's "QPR Index scores intellectual rigor across 91 essays" (a claim about that tool, Tony's copy). Checked 2026-10-14: type check, lint, build (/, /subscribe, /the-letter still static), fresh server: all three show 123, no "92 essays" in the built browser code.</t>
+        </is>
+      </c>
+      <c r="E341" s="14" t="inlineStr">
+        <is>
+          <t>Phase 14 — QA &amp; Launch</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" s="4" t="n"/>
+      <c r="B342" s="4" t="inlineStr">
+        <is>
+          <t>Team review's "everything else looks fine" re-checked</t>
+        </is>
+      </c>
+      <c r="C342" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D342" s="4" t="inlineStr">
+        <is>
+          <t>(2026-10-14, owner: "you can check"). Fresh production build: all 60 menu pages (main menu, Fix Myself, Explore...) at 1280px and 375px: 200, one H1, no sideways scroll, no JS errors. All 130 blog links on them (122 posts, 8 categories): 200, no redirects. 404 page: 404 for a missing page, essay and category. Dark mode: switches and stays on across pages; 10 essays checked on a phone in dark mode. Phone menu shows every section; Ask Tony works on a phone. Netlify test site: the same 60 menu pages answer. Two small fixes: a missing essay or category showed the homepage's tab title on its 404 page (now "Page not found"); three Explore links (/attention-theft/weapons, /report, /legal) went through a redirect, now link straight to /attention-theft#weapons etc. Checked: type check, lint, build, clicked "Legal Database" in the menu.</t>
+        </is>
+      </c>
+      <c r="E342" s="14" t="inlineStr">
+        <is>
+          <t>Phase 14 — QA &amp; Launch</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" s="4" t="n"/>
+      <c r="B343" s="4" t="inlineStr">
+        <is>
           <t>DNS cutover, legacy app decommissioned only after a stable overlap window Re-checked 2026-10-13</t>
         </is>
       </c>
-      <c r="C338" s="16" t="inlineStr">
+      <c r="C343" s="16" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
       </c>
-      <c r="D338" s="4" t="inlineStr">
+      <c r="D343" s="4" t="inlineStr">
         <is>
           <t>unchanged (Hostinger name servers, bare domain on Manus 104.19.168/169.112, www CNAME cname.manus.space). Checked 2026-10-09 (owner wants to go live and switch off Manus): DNS for tonygreenberg.com is at Hostinger (name servers ns1/ns2.dns-parking.com); www is a CNAME to cname.manus.space, the bare domain points at Manus's addresses (104.19.168.112 / .169.112); the Netlify site tonygreenberg-website has no custom domain yet (production branch main). Order: (1) merge the three open pull requests into main and check the Netlify copy; (2) restore Supabase and run 0001 to 0003, or launch without member features (they say "isn't available just now"); (3) owner sign-off; (4) add tonygreenberg.com + www in Netlify (Domain management), then at Hostinger point the bare domain at Netlify (A record 75.2.60.5, or Netlify DNS) and www CNAME at tonygreenberg-website.netlify.app; Netlify issues the HTTPS certificate; (5) re-run scripts/check-search-console-urls.ts https://tonygreenberg.com and submit the sitemap in Search Console; (6) only after a few stable days: switch off the Manus site (the database is already backed up, docs/ai/project_legacy_database.md) and rotate the old database password.</t>
         </is>
       </c>
-      <c r="E338" s="14" t="inlineStr">
+      <c r="E343" s="14" t="inlineStr">
         <is>
           <t>Phase 14 — QA &amp; Launch</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D338"/>
+  <autoFilter ref="A1:D343"/>
   <mergeCells count="14">
     <mergeCell ref="A211:D211"/>
     <mergeCell ref="A189:D189"/>

</xml_diff>

<commit_message>
Essay archive: search suggestions and sort/year/reading-time/topic filters
The archive on "/" and "/blog" gets a suggestions dropdown while typing
(matching categories and topics, plus essays from /api/search, which also
matches words inside the essay text) and four filters: newest/oldest,
year, reading time and topic (tags used by 3+ essays). Reading time falls
back to a word-count estimate from Sanity, since only 34 of 123 posts set
one. On phones the filters fold behind a "Filters" button.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Migration-Status-Report.xlsx
+++ b/Migration-Status-Report.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Remaining Work" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Full Detail'!$A$1:$D$343</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Full Detail'!$A$1:$D$344</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Remaining Work'!$A$1:$D$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -639,15 +639,15 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A5,'Full Detail'!$C$2:$C$343,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A5,'Full Detail'!$C$2:$C$344,"Done")</f>
         <v/>
       </c>
       <c r="C5" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A5,'Full Detail'!$C$2:$C$343,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A5,'Full Detail'!$C$2:$C$344,"Remaining")</f>
         <v/>
       </c>
       <c r="D5" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A5,'Full Detail'!$C$2:$C$343,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A5,'Full Detail'!$C$2:$C$344,"Deferred")</f>
         <v/>
       </c>
       <c r="E5" s="5">
@@ -666,15 +666,15 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A6,'Full Detail'!$C$2:$C$343,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A6,'Full Detail'!$C$2:$C$344,"Done")</f>
         <v/>
       </c>
       <c r="C6" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A6,'Full Detail'!$C$2:$C$343,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A6,'Full Detail'!$C$2:$C$344,"Remaining")</f>
         <v/>
       </c>
       <c r="D6" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A6,'Full Detail'!$C$2:$C$343,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A6,'Full Detail'!$C$2:$C$344,"Deferred")</f>
         <v/>
       </c>
       <c r="E6" s="5">
@@ -693,15 +693,15 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A7,'Full Detail'!$C$2:$C$343,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A7,'Full Detail'!$C$2:$C$344,"Done")</f>
         <v/>
       </c>
       <c r="C7" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A7,'Full Detail'!$C$2:$C$343,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A7,'Full Detail'!$C$2:$C$344,"Remaining")</f>
         <v/>
       </c>
       <c r="D7" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A7,'Full Detail'!$C$2:$C$343,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A7,'Full Detail'!$C$2:$C$344,"Deferred")</f>
         <v/>
       </c>
       <c r="E7" s="5">
@@ -720,15 +720,15 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A8,'Full Detail'!$C$2:$C$343,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A8,'Full Detail'!$C$2:$C$344,"Done")</f>
         <v/>
       </c>
       <c r="C8" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A8,'Full Detail'!$C$2:$C$343,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A8,'Full Detail'!$C$2:$C$344,"Remaining")</f>
         <v/>
       </c>
       <c r="D8" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A8,'Full Detail'!$C$2:$C$343,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A8,'Full Detail'!$C$2:$C$344,"Deferred")</f>
         <v/>
       </c>
       <c r="E8" s="5">
@@ -747,15 +747,15 @@
         </is>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A9,'Full Detail'!$C$2:$C$343,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A9,'Full Detail'!$C$2:$C$344,"Done")</f>
         <v/>
       </c>
       <c r="C9" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A9,'Full Detail'!$C$2:$C$343,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A9,'Full Detail'!$C$2:$C$344,"Remaining")</f>
         <v/>
       </c>
       <c r="D9" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A9,'Full Detail'!$C$2:$C$343,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A9,'Full Detail'!$C$2:$C$344,"Deferred")</f>
         <v/>
       </c>
       <c r="E9" s="5">
@@ -774,15 +774,15 @@
         </is>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A10,'Full Detail'!$C$2:$C$343,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A10,'Full Detail'!$C$2:$C$344,"Done")</f>
         <v/>
       </c>
       <c r="C10" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A10,'Full Detail'!$C$2:$C$343,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A10,'Full Detail'!$C$2:$C$344,"Remaining")</f>
         <v/>
       </c>
       <c r="D10" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A10,'Full Detail'!$C$2:$C$343,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A10,'Full Detail'!$C$2:$C$344,"Deferred")</f>
         <v/>
       </c>
       <c r="E10" s="5">
@@ -801,15 +801,15 @@
         </is>
       </c>
       <c r="B11" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A11,'Full Detail'!$C$2:$C$343,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A11,'Full Detail'!$C$2:$C$344,"Done")</f>
         <v/>
       </c>
       <c r="C11" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A11,'Full Detail'!$C$2:$C$343,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A11,'Full Detail'!$C$2:$C$344,"Remaining")</f>
         <v/>
       </c>
       <c r="D11" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A11,'Full Detail'!$C$2:$C$343,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A11,'Full Detail'!$C$2:$C$344,"Deferred")</f>
         <v/>
       </c>
       <c r="E11" s="5">
@@ -828,15 +828,15 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A12,'Full Detail'!$C$2:$C$343,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A12,'Full Detail'!$C$2:$C$344,"Done")</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A12,'Full Detail'!$C$2:$C$343,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A12,'Full Detail'!$C$2:$C$344,"Remaining")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A12,'Full Detail'!$C$2:$C$343,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A12,'Full Detail'!$C$2:$C$344,"Deferred")</f>
         <v/>
       </c>
       <c r="E12" s="5">
@@ -855,15 +855,15 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A13,'Full Detail'!$C$2:$C$343,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A13,'Full Detail'!$C$2:$C$344,"Done")</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A13,'Full Detail'!$C$2:$C$343,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A13,'Full Detail'!$C$2:$C$344,"Remaining")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A13,'Full Detail'!$C$2:$C$343,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A13,'Full Detail'!$C$2:$C$344,"Deferred")</f>
         <v/>
       </c>
       <c r="E13" s="5">
@@ -882,15 +882,15 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A14,'Full Detail'!$C$2:$C$343,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A14,'Full Detail'!$C$2:$C$344,"Done")</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A14,'Full Detail'!$C$2:$C$343,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A14,'Full Detail'!$C$2:$C$344,"Remaining")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A14,'Full Detail'!$C$2:$C$343,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A14,'Full Detail'!$C$2:$C$344,"Deferred")</f>
         <v/>
       </c>
       <c r="E14" s="5">
@@ -909,15 +909,15 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A15,'Full Detail'!$C$2:$C$343,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A15,'Full Detail'!$C$2:$C$344,"Done")</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A15,'Full Detail'!$C$2:$C$343,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A15,'Full Detail'!$C$2:$C$344,"Remaining")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A15,'Full Detail'!$C$2:$C$343,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A15,'Full Detail'!$C$2:$C$344,"Deferred")</f>
         <v/>
       </c>
       <c r="E15" s="5">
@@ -936,15 +936,15 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A16,'Full Detail'!$C$2:$C$343,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A16,'Full Detail'!$C$2:$C$344,"Done")</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A16,'Full Detail'!$C$2:$C$343,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A16,'Full Detail'!$C$2:$C$344,"Remaining")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A16,'Full Detail'!$C$2:$C$343,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A16,'Full Detail'!$C$2:$C$344,"Deferred")</f>
         <v/>
       </c>
       <c r="E16" s="5">
@@ -963,15 +963,15 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A17,'Full Detail'!$C$2:$C$343,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A17,'Full Detail'!$C$2:$C$344,"Done")</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A17,'Full Detail'!$C$2:$C$343,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A17,'Full Detail'!$C$2:$C$344,"Remaining")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A17,'Full Detail'!$C$2:$C$343,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A17,'Full Detail'!$C$2:$C$344,"Deferred")</f>
         <v/>
       </c>
       <c r="E17" s="5">
@@ -990,15 +990,15 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A18,'Full Detail'!$C$2:$C$343,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A18,'Full Detail'!$C$2:$C$344,"Done")</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A18,'Full Detail'!$C$2:$C$343,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A18,'Full Detail'!$C$2:$C$344,"Remaining")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A18,'Full Detail'!$C$2:$C$343,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A18,'Full Detail'!$C$2:$C$344,"Deferred")</f>
         <v/>
       </c>
       <c r="E18" s="5">
@@ -1017,15 +1017,15 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A19,'Full Detail'!$C$2:$C$343,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A19,'Full Detail'!$C$2:$C$344,"Done")</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A19,'Full Detail'!$C$2:$C$343,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A19,'Full Detail'!$C$2:$C$344,"Remaining")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$343,$A19,'Full Detail'!$C$2:$C$343,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A19,'Full Detail'!$C$2:$C$344,"Deferred")</f>
         <v/>
       </c>
       <c r="E19" s="5">
@@ -1075,7 +1075,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E343"/>
+  <dimension ref="A1:E344"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -4513,43 +4513,43 @@
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="10" t="inlineStr">
+      <c r="A156" s="4" t="n"/>
+      <c r="B156" s="4" t="inlineStr">
+        <is>
+          <t>Essay archive: search suggestions + more filters</t>
+        </is>
+      </c>
+      <c r="C156" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D156" s="4" t="inlineStr">
+        <is>
+          <t>(owner asked 2026-10-14, chose: search-as-you-type, and sort, year, reading time, topic). The archive at the bottom of / (and on /blog) was already live data (Sanity, newest first, refreshed within 60s or by the webhook; every essay on live's sitemap is in Sanity). Added: archive-search-box.tsx, a dropdown while typing with matching categories and topics (instant) and essays from /api/search (also matches words inside the essay text); arrow keys + Enter, Escape. Filters: Newest/Oldest, Year, Reading time (under 5, 5 to 10, over 10 min) and Topic (tags used by 3+ essays, about 30 of 874), with "Clear filters"; on phones they fold behind a "Filters" button. Reading time uses the editor's value or a word-count estimate (minutes in allPostsForArchiveQuery; only 34 of 123 posts had one). Checked: type check, lint, build (150 static / 28 dynamic, unchanged), browser on a fresh server: every filter count matches the data (year 2010: 21, neuroscience: 13, 5 to 10 min: 52...), "kurzweil" suggests the H+ essays and Enter opens one, picking a topic suggestion sets the Topic filter; 375 light/dark, 820, 1280: no sideways scroll, no JS errors.</t>
+        </is>
+      </c>
+      <c r="E156" s="14" t="inlineStr">
+        <is>
+          <t>Phase 5 — Blog Engine (Sanity-backed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="10" t="inlineStr">
         <is>
           <t>Phase 6 — BrewSoul (28 routes)</t>
         </is>
       </c>
-      <c r="B156" s="11" t="n"/>
-      <c r="C156" s="11" t="n"/>
-      <c r="D156" s="12" t="n"/>
-    </row>
-    <row r="157">
-      <c r="A157" s="4" t="n"/>
-      <c r="B157" s="4" t="inlineStr">
-        <is>
-          <t>/brewsoul</t>
-        </is>
-      </c>
-      <c r="C157" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D157" s="4" t="inlineStr">
-        <is>
-          <t>welcome/landing gate (built, not yet pushed — pending local review), along with the shared foundation the rest of Phase 6 depends on. Ported BrewSoulLayout.tsx → app/brewsoul/layout.tsx + components/brewsoul/brewsoul-nav.tsx (BrewSoulNav/BrewSoulFooter), CategoryBadge.tsx → components/brewsoul/category-badge.tsx, brewsoul-config.ts → lib/content/brewsoul-config.ts, and BrewSoulDirectory.tsx's CATEGORIES/PAGE_CATEGORY_MAP data (not the page itself yet) → lib/content/brewsoul-directory.ts. Real architecture decision: BrewSoul is a self-contained sub-site with its own nav/footer/coffee-brown palette, same as legacy — but this app has one flat root layout with no route groups, so the main site's SiteHeader/SiteFooter needed to be suppressed for this one subtree without restructuring every existing route. Added components/site-chrome.tsx (SiteChrome, a small client wrapper checking pathname.startsWith("/brewsoul")) around both in app/layout.tsx — verified via literal &lt;header&gt;/&lt;footer&gt;/&lt;nav&gt; tag counts in real SSR HTML (not text search, which false-positives on Next dev mode's RSC debug payload) that /brewsoul gets zero main-site chrome and its own real nav+footer, while / still gets exactly one of each. Dropped TonyAvatarTrigger (FauxTony chatbot widget — Phase 10, no backend yet, same "don't fake it" call made elsewhere) from the nav. Ported BrewSoulWelcome.tsx → components/brewsoul/brewsoul-welcome-quiz.tsx (8-screen onboarding quiz, real identity-scoring logic, palate questions</t>
-        </is>
-      </c>
-      <c r="E157" s="14" t="inlineStr">
-        <is>
-          <t>Phase 6 — BrewSoul (28 routes)</t>
-        </is>
-      </c>
+      <c r="B157" s="11" t="n"/>
+      <c r="C157" s="11" t="n"/>
+      <c r="D157" s="12" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="4" t="n"/>
       <c r="B158" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/first-sip</t>
+          <t>/brewsoul</t>
         </is>
       </c>
       <c r="C158" s="13" t="inlineStr">
@@ -4559,7 +4559,7 @@
       </c>
       <c r="D158" s="4" t="inlineStr">
         <is>
-          <t>onboarding intro (built, not yet pushed — pending local review). Ported "The First Sip Is a Vote" in full — the complete manifesto essay (5 sections, 3 pullquotes, the couplets block, the disclosure-demands grid), the 5-tool journey map, 6 related-essay links (real slugs, cross-checked against this session's already-verified corpus), the closing + sources, and the email capture. Built as a Server Component (all static except the email form) + components/brewsoul/next-steps.tsx (shared "what's next" CTA, itself a Server Component — legacy's hover effects were plain CSS-able, no JS state needed) + components/brewsoul/first-sip-email-capture.tsx (client island, mailto: fallback since no subscribe backend exists, same pattern as newsletter-popup.tsx). Dropped the canvas CoffeeDust decoration and the confirmed-dead hero photo (/api/img/brewsoul-orig_84eb4bc9.jpg, 404, same Manus proxy) — with no image left, the scroll-linked parallax that moved it went too. The 5 tool-card links (prescription/health/pairings/economics/compare) point at later Phase 6 routes not built yet — same forward-reference pattern as /find-my. Verified live: 200 OK, full essay text present, CategoryBadge correctly shows "Start Here" (from PAGE_CATEGORY_MAP), zero main-site chrome leaking in, typecheck/lint clean.</t>
+          <t>welcome/landing gate (built, not yet pushed — pending local review), along with the shared foundation the rest of Phase 6 depends on. Ported BrewSoulLayout.tsx → app/brewsoul/layout.tsx + components/brewsoul/brewsoul-nav.tsx (BrewSoulNav/BrewSoulFooter), CategoryBadge.tsx → components/brewsoul/category-badge.tsx, brewsoul-config.ts → lib/content/brewsoul-config.ts, and BrewSoulDirectory.tsx's CATEGORIES/PAGE_CATEGORY_MAP data (not the page itself yet) → lib/content/brewsoul-directory.ts. Real architecture decision: BrewSoul is a self-contained sub-site with its own nav/footer/coffee-brown palette, same as legacy — but this app has one flat root layout with no route groups, so the main site's SiteHeader/SiteFooter needed to be suppressed for this one subtree without restructuring every existing route. Added components/site-chrome.tsx (SiteChrome, a small client wrapper checking pathname.startsWith("/brewsoul")) around both in app/layout.tsx — verified via literal &lt;header&gt;/&lt;footer&gt;/&lt;nav&gt; tag counts in real SSR HTML (not text search, which false-positives on Next dev mode's RSC debug payload) that /brewsoul gets zero main-site chrome and its own real nav+footer, while / still gets exactly one of each. Dropped TonyAvatarTrigger (FauxTony chatbot widget — Phase 10, no backend yet, same "don't fake it" call made elsewhere) from the nav. Ported BrewSoulWelcome.tsx → components/brewsoul/brewsoul-welcome-quiz.tsx (8-screen onboarding quiz, real identity-scoring logic, palate questions</t>
         </is>
       </c>
       <c r="E158" s="14" t="inlineStr">
@@ -4572,7 +4572,7 @@
       <c r="A159" s="4" t="n"/>
       <c r="B159" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/home</t>
+          <t>/brewsoul/first-sip</t>
         </is>
       </c>
       <c r="C159" s="13" t="inlineStr">
@@ -4582,7 +4582,7 @@
       </c>
       <c r="D159" s="4" t="inlineStr">
         <is>
-          <t>the real BrewSoul dashboard (distinct from /brewsoul's identity-quiz welcome gate and /brewsoul/first-sip's manifesto): hero + stats, Follow the Dollar teaser, Top QPR coffees (computed live via computeQPR), the 2025 crisis callout, New Drops, a Wall of Shame preview (SHAME_ENTRIES), the research-hub card grid, and a cyclable health-fact ticker (components/brewsoul/health-ticker.tsx, its own small client island so the rest of the page stays a Server Component). Canvas WarmParticles/ParallaxBg decorations and the dead hero photo (/api/img/brewsoul-orig_84eb4bc9.jpg, same confirmed-404 Manus proxy used elsewhere in Phase 6) dropped for CSS gradients. Stats use the real live BREWSOUL_COFFEES.length (107) in place of legacy's stale "103". Verified live: 200 OK.</t>
+          <t>onboarding intro (built, not yet pushed — pending local review). Ported "The First Sip Is a Vote" in full — the complete manifesto essay (5 sections, 3 pullquotes, the couplets block, the disclosure-demands grid), the 5-tool journey map, 6 related-essay links (real slugs, cross-checked against this session's already-verified corpus), the closing + sources, and the email capture. Built as a Server Component (all static except the email form) + components/brewsoul/next-steps.tsx (shared "what's next" CTA, itself a Server Component — legacy's hover effects were plain CSS-able, no JS state needed) + components/brewsoul/first-sip-email-capture.tsx (client island, mailto: fallback since no subscribe backend exists, same pattern as newsletter-popup.tsx). Dropped the canvas CoffeeDust decoration and the confirmed-dead hero photo (/api/img/brewsoul-orig_84eb4bc9.jpg, 404, same Manus proxy) — with no image left, the scroll-linked parallax that moved it went too. The 5 tool-card links (prescription/health/pairings/economics/compare) point at later Phase 6 routes not built yet — same forward-reference pattern as /find-my. Verified live: 200 OK, full essay text present, CategoryBadge correctly shows "Start Here" (from PAGE_CATEGORY_MAP), zero main-site chrome leaking in, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E159" s="14" t="inlineStr">
@@ -4595,7 +4595,7 @@
       <c r="A160" s="4" t="n"/>
       <c r="B160" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/browse</t>
+          <t>/brewsoul/home</t>
         </is>
       </c>
       <c r="C160" s="13" t="inlineStr">
@@ -4605,7 +4605,7 @@
       </c>
       <c r="D160" s="4" t="inlineStr">
         <is>
-          <t>coffee listing (components/brewsoul/browse-explorer.tsx), real filter/search over the full BREWSOUL_COFFEES catalog. Verified live: 200 OK.</t>
+          <t>the real BrewSoul dashboard (distinct from /brewsoul's identity-quiz welcome gate and /brewsoul/first-sip's manifesto): hero + stats, Follow the Dollar teaser, Top QPR coffees (computed live via computeQPR), the 2025 crisis callout, New Drops, a Wall of Shame preview (SHAME_ENTRIES), the research-hub card grid, and a cyclable health-fact ticker (components/brewsoul/health-ticker.tsx, its own small client island so the rest of the page stays a Server Component). Canvas WarmParticles/ParallaxBg decorations and the dead hero photo (/api/img/brewsoul-orig_84eb4bc9.jpg, same confirmed-404 Manus proxy used elsewhere in Phase 6) dropped for CSS gradients. Stats use the real live BREWSOUL_COFFEES.length (107) in place of legacy's stale "103". Verified live: 200 OK.</t>
         </is>
       </c>
       <c r="E160" s="14" t="inlineStr">
@@ -4618,7 +4618,7 @@
       <c r="A161" s="4" t="n"/>
       <c r="B161" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/coffee/[id]</t>
+          <t>/brewsoul/browse</t>
         </is>
       </c>
       <c r="C161" s="13" t="inlineStr">
@@ -4628,7 +4628,7 @@
       </c>
       <c r="D161" s="4" t="inlineStr">
         <is>
-          <t>coffee detail page (breadcrumb, QPR + tier header, quick stats, tasting notes, flavor-profile bars, the 4 intelligence scores, transparency/ethics data, buy links, competition wins, similar-coffees cross-links, journey CTAs), server-rendered with generateStaticParams over all 107 real coffees (this repo's bounded-dynamic-route convention, same as /blog/[slug]) instead of legacy's client-side useParams lookup. Verified live: 200 OK.</t>
+          <t>coffee listing (components/brewsoul/browse-explorer.tsx), real filter/search over the full BREWSOUL_COFFEES catalog. Verified live: 200 OK.</t>
         </is>
       </c>
       <c r="E161" s="14" t="inlineStr">
@@ -4641,7 +4641,7 @@
       <c r="A162" s="4" t="n"/>
       <c r="B162" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/quiz</t>
+          <t>/brewsoul/coffee/[id]</t>
         </is>
       </c>
       <c r="C162" s="13" t="inlineStr">
@@ -4651,7 +4651,7 @@
       </c>
       <c r="D162" s="4" t="inlineStr">
         <is>
-          <t>matching quiz (built, not yet pushed — pending local review), along with the real data/engine foundation most of the rest of Phase 6 depends on. Ported lib/intelligence-engine/{types,scoring}.ts verbatim (generic scoring engine — QPR/availability/scarcity/wow/tier/freshness — reusable beyond BrewSoul) and the full coffee catalog (legacy's 3 files: brewsoul-coffees.ts + -expanded.ts + -expanded2.ts, merged at import time) → one lib/content/brewsoul-coffees.ts, extracted via tsx (not hand-typed — 107 real entries, ~6.5K lines). Caught a real stale count: legacy's own file header claimed "105" and its UI copy said "103", but the actual merged arrays contain 107 — this migration shows the live BREWSOUL_COFFEES.length everywhere instead of a repeated hardcoded number. Ported JourneyBar.tsx (components/brewsoul/journey-bar.tsx) — the fixed bottom "what's next" bar shown on every BrewSoul content page except the identity quiz — and retrofitted it onto /brewsoul/first-sip too (built before JourneyBar existed). Built components/brewsoul/brewsoul-quiz.tsx: real 7-question taste quiz scored against each coffee's real flavorProfile via the real scoring engine, ranking the full catalog by match. Legacy's useMarkVisited was renamed to markVisited (it's a plain localStorage write, not a hook — its old use-prefixed name tripped React's rules-of-hooks lint when called from inside a useEffect). Dropped the canvas WarmParticles decoration and the dead hero photo (same confirmed-404 Manus proxy,</t>
+          <t>coffee detail page (breadcrumb, QPR + tier header, quick stats, tasting notes, flavor-profile bars, the 4 intelligence scores, transparency/ethics data, buy links, competition wins, similar-coffees cross-links, journey CTAs), server-rendered with generateStaticParams over all 107 real coffees (this repo's bounded-dynamic-route convention, same as /blog/[slug]) instead of legacy's client-side useParams lookup. Verified live: 200 OK.</t>
         </is>
       </c>
       <c r="E162" s="14" t="inlineStr">
@@ -4664,7 +4664,7 @@
       <c r="A163" s="4" t="n"/>
       <c r="B163" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/wall-of-shame</t>
+          <t>/brewsoul/quiz</t>
         </is>
       </c>
       <c r="C163" s="13" t="inlineStr">
@@ -4674,7 +4674,7 @@
       </c>
       <c r="D163" s="4" t="inlineStr">
         <is>
-          <t>content page. Real 13 entries (brand/category/evidence/severity/response) from SHAME_ENTRIES, unchanged. Category filter buttons extracted into components/brewsoul/shame-explorer.tsx (the only interactive piece) so the page itself stays a Server Component. Verified live: 200 OK.</t>
+          <t>matching quiz (built, not yet pushed — pending local review), along with the real data/engine foundation most of the rest of Phase 6 depends on. Ported lib/intelligence-engine/{types,scoring}.ts verbatim (generic scoring engine — QPR/availability/scarcity/wow/tier/freshness — reusable beyond BrewSoul) and the full coffee catalog (legacy's 3 files: brewsoul-coffees.ts + -expanded.ts + -expanded2.ts, merged at import time) → one lib/content/brewsoul-coffees.ts, extracted via tsx (not hand-typed — 107 real entries, ~6.5K lines). Caught a real stale count: legacy's own file header claimed "105" and its UI copy said "103", but the actual merged arrays contain 107 — this migration shows the live BREWSOUL_COFFEES.length everywhere instead of a repeated hardcoded number. Ported JourneyBar.tsx (components/brewsoul/journey-bar.tsx) — the fixed bottom "what's next" bar shown on every BrewSoul content page except the identity quiz — and retrofitted it onto /brewsoul/first-sip too (built before JourneyBar existed). Built components/brewsoul/brewsoul-quiz.tsx: real 7-question taste quiz scored against each coffee's real flavorProfile via the real scoring engine, ranking the full catalog by match. Legacy's useMarkVisited was renamed to markVisited (it's a plain localStorage write, not a hook — its old use-prefixed name tripped React's rules-of-hooks lint when called from inside a useEffect). Dropped the canvas WarmParticles decoration and the dead hero photo (same confirmed-404 Manus proxy,</t>
         </is>
       </c>
       <c r="E163" s="14" t="inlineStr">
@@ -4687,7 +4687,7 @@
       <c r="A164" s="4" t="n"/>
       <c r="B164" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/follow-the-dollar</t>
+          <t>/brewsoul/wall-of-shame</t>
         </is>
       </c>
       <c r="C164" s="13" t="inlineStr">
@@ -4697,7 +4697,7 @@
       </c>
       <c r="D164" s="4" t="inlineStr">
         <is>
-          <t>supply-chain essay. Real DOLLAR_BREAKDOWNS segment bars (farmer/exporter/importer/roaster/retailer %, real commentary), unchanged. The farmer-segment bar's data-driven color (green/gold/red by threshold) is a small known set of variants — precomposed as 3 literal Tailwind classes rather than an inline style background, per this repo's dynamic-class rule; only the genuinely per-item width stays as style. Fully static, Server Component. Verified live: 200 OK.</t>
+          <t>content page. Real 13 entries (brand/category/evidence/severity/response) from SHAME_ENTRIES, unchanged. Category filter buttons extracted into components/brewsoul/shame-explorer.tsx (the only interactive piece) so the page itself stays a Server Component. Verified live: 200 OK.</t>
         </is>
       </c>
       <c r="E164" s="14" t="inlineStr">
@@ -4710,7 +4710,7 @@
       <c r="A165" s="4" t="n"/>
       <c r="B165" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/farms</t>
+          <t>/brewsoul/follow-the-dollar</t>
         </is>
       </c>
       <c r="C165" s="13" t="inlineStr">
@@ -4720,7 +4720,7 @@
       </c>
       <c r="D165" s="4" t="inlineStr">
         <is>
-          <t>sourcing content ("Farm Passports"). Real FARMS entries (country/region/producer/altitude/story/varieties/certifications), unchanged. Fully static. Verified live: 200 OK.</t>
+          <t>supply-chain essay. Real DOLLAR_BREAKDOWNS segment bars (farmer/exporter/importer/roaster/retailer %, real commentary), unchanged. The farmer-segment bar's data-driven color (green/gold/red by threshold) is a small known set of variants — precomposed as 3 literal Tailwind classes rather than an inline style background, per this repo's dynamic-class rule; only the genuinely per-item width stays as style. Fully static, Server Component. Verified live: 200 OK.</t>
         </is>
       </c>
       <c r="E165" s="14" t="inlineStr">
@@ -4733,7 +4733,7 @@
       <c r="A166" s="4" t="n"/>
       <c r="B166" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/mold-free</t>
+          <t>/brewsoul/farms</t>
         </is>
       </c>
       <c r="C166" s="13" t="inlineStr">
@@ -4743,7 +4743,7 @@
       </c>
       <c r="D166" s="4" t="inlineStr">
         <is>
-          <t>mycotoxin content. Real verified/claims/untested split computed live over the full BREWSOUL_COFFEES catalog by moldTestStatus. Fully static. Verified live: 200 OK.</t>
+          <t>sourcing content ("Farm Passports"). Real FARMS entries (country/region/producer/altitude/story/varieties/certifications), unchanged. Fully static. Verified live: 200 OK.</t>
         </is>
       </c>
       <c r="E166" s="14" t="inlineStr">
@@ -4756,7 +4756,7 @@
       <c r="A167" s="4" t="n"/>
       <c r="B167" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/experiences</t>
+          <t>/brewsoul/mold-free</t>
         </is>
       </c>
       <c r="C167" s="13" t="inlineStr">
@@ -4766,7 +4766,7 @@
       </c>
       <c r="D167" s="4" t="inlineStr">
         <is>
-          <t>experiential content ("Experience Map"). Real EXPERIENCES entries (farm tours, cafés, cupping labs, roastery visits), unchanged. Country filter buttons extracted into components/brewsoul/experiences-explorer.tsx, same split-out-the-interactive-bit pattern as wall-of-shame. Verified live: 200 OK.</t>
+          <t>mycotoxin content. Real verified/claims/untested split computed live over the full BREWSOUL_COFFEES catalog by moldTestStatus. Fully static. Verified live: 200 OK.</t>
         </is>
       </c>
       <c r="E167" s="14" t="inlineStr">
@@ -4779,7 +4779,7 @@
       <c r="A168" s="4" t="n"/>
       <c r="B168" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/health</t>
+          <t>/brewsoul/experiences</t>
         </is>
       </c>
       <c r="C168" s="13" t="inlineStr">
@@ -4789,7 +4789,7 @@
       </c>
       <c r="D168" s="4" t="inlineStr">
         <is>
-          <t>health deep-dive, ported from BrewSoulHealthFull.tsx (the file legacy's own router actually uses for this route — BrewSoulContent.tsx's same-named BrewSoulHealth export is real but genuinely dead/unrouted code in legacy, shadowed by this one). Real 8 longevity findings with real citations/participant counts, 7 real risks with severity ratings, CYP1A2 caffeine-metabolism genetics, a 6-step chronobiology timing schedule, 8 real bioactive compounds, 3 real mycotoxin threats, and a 3-step "simplification protocol," all ported unchanged and verbatim. Dead Manus hero image dropped for a CSS gradient. Legacy's own redundant BrewSoulLayout wrapper dropped — app/brewsoul/layout.tsx already wraps every route. The two real interactive pieces (show-all-risks toggle, per-compound click-to-expand) split into components/brewsoul/health-{risks,compounds}.tsx client islands so the rest stays a Server Component. Legacy's bespoke earthy "science" palette (soil/clay/sage/moss — distinct from the rest of BrewSoul's amber/gold commercial palette) kept as a deliberate one-off sub-identity for this one page, same reasoning as /attention-theft's own "crusade" palette elsewhere in this migration. Verified live: 200 OK, typecheck/lint clean.</t>
+          <t>experiential content ("Experience Map"). Real EXPERIENCES entries (farm tours, cafés, cupping labs, roastery visits), unchanged. Country filter buttons extracted into components/brewsoul/experiences-explorer.tsx, same split-out-the-interactive-bit pattern as wall-of-shame. Verified live: 200 OK.</t>
         </is>
       </c>
       <c r="E168" s="14" t="inlineStr">
@@ -4802,7 +4802,7 @@
       <c r="A169" s="4" t="n"/>
       <c r="B169" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/varieties</t>
+          <t>/brewsoul/health</t>
         </is>
       </c>
       <c r="C169" s="13" t="inlineStr">
@@ -4812,7 +4812,7 @@
       </c>
       <c r="D169" s="4" t="inlineStr">
         <is>
-          <t>reference: varieties. Real VARIETIES encyclopedia entries (species/origin/genetics/cup profile/yield/disease resistance), unchanged. Search extracted into components/brewsoul/varieties-explorer.tsx. Verified live: 200 OK.</t>
+          <t>health deep-dive, ported from BrewSoulHealthFull.tsx (the file legacy's own router actually uses for this route — BrewSoulContent.tsx's same-named BrewSoulHealth export is real but genuinely dead/unrouted code in legacy, shadowed by this one). Real 8 longevity findings with real citations/participant counts, 7 real risks with severity ratings, CYP1A2 caffeine-metabolism genetics, a 6-step chronobiology timing schedule, 8 real bioactive compounds, 3 real mycotoxin threats, and a 3-step "simplification protocol," all ported unchanged and verbatim. Dead Manus hero image dropped for a CSS gradient. Legacy's own redundant BrewSoulLayout wrapper dropped — app/brewsoul/layout.tsx already wraps every route. The two real interactive pieces (show-all-risks toggle, per-compound click-to-expand) split into components/brewsoul/health-{risks,compounds}.tsx client islands so the rest stays a Server Component. Legacy's bespoke earthy "science" palette (soil/clay/sage/moss — distinct from the rest of BrewSoul's amber/gold commercial palette) kept as a deliberate one-off sub-identity for this one page, same reasoning as /attention-theft's own "crusade" palette elsewhere in this migration. Verified live: 200 OK, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E169" s="14" t="inlineStr">
@@ -4825,7 +4825,7 @@
       <c r="A170" s="4" t="n"/>
       <c r="B170" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/processing</t>
+          <t>/brewsoul/varieties</t>
         </is>
       </c>
       <c r="C170" s="13" t="inlineStr">
@@ -4835,7 +4835,7 @@
       </c>
       <c r="D170" s="4" t="inlineStr">
         <is>
-          <t>reference: processing. Real PROCESSING_METHODS entries (description/flavor impact/complexity/controversy), unchanged. Fully static. Verified live: 200 OK.</t>
+          <t>reference: varieties. Real VARIETIES encyclopedia entries (species/origin/genetics/cup profile/yield/disease resistance), unchanged. Search extracted into components/brewsoul/varieties-explorer.tsx. Verified live: 200 OK.</t>
         </is>
       </c>
       <c r="E170" s="14" t="inlineStr">
@@ -4848,7 +4848,7 @@
       <c r="A171" s="4" t="n"/>
       <c r="B171" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/roasters</t>
+          <t>/brewsoul/processing</t>
         </is>
       </c>
       <c r="C171" s="13" t="inlineStr">
@@ -4858,7 +4858,7 @@
       </c>
       <c r="D171" s="4" t="inlineStr">
         <is>
-          <t>reference: roaster directory. Real ROASTERS entries (philosophy/quality/transparency/farmer-equity scores), unchanged. Search + tier filter extracted into components/brewsoul/roasters-explorer.tsx. Verified live: 200 OK.</t>
+          <t>reference: processing. Real PROCESSING_METHODS entries (description/flavor impact/complexity/controversy), unchanged. Fully static. Verified live: 200 OK.</t>
         </is>
       </c>
       <c r="E171" s="14" t="inlineStr">
@@ -4871,7 +4871,7 @@
       <c r="A172" s="4" t="n"/>
       <c r="B172" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/glossary</t>
+          <t>/brewsoul/roasters</t>
         </is>
       </c>
       <c r="C172" s="13" t="inlineStr">
@@ -4881,7 +4881,7 @@
       </c>
       <c r="D172" s="4" t="inlineStr">
         <is>
-          <t>reference: glossary. Real GLOSSARY terms, unchanged. Search + alphabetical grouping extracted into components/brewsoul/glossary-explorer.tsx. Verified live: 200 OK.</t>
+          <t>reference: roaster directory. Real ROASTERS entries (philosophy/quality/transparency/farmer-equity scores), unchanged. Search + tier filter extracted into components/brewsoul/roasters-explorer.tsx. Verified live: 200 OK.</t>
         </is>
       </c>
       <c r="E172" s="14" t="inlineStr">
@@ -4894,7 +4894,7 @@
       <c r="A173" s="4" t="n"/>
       <c r="B173" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/pairings</t>
+          <t>/brewsoul/glossary</t>
         </is>
       </c>
       <c r="C173" s="13" t="inlineStr">
@@ -4904,7 +4904,7 @@
       </c>
       <c r="D173" s="4" t="inlineStr">
         <is>
-          <t>reference: pairings. Real PAIRINGS (food/drink pairings by origin) and 3 real curated FLIGHTS (each linking to real coffees in the catalog), unchanged. Fully static. Verified live: 200 OK.</t>
+          <t>reference: glossary. Real GLOSSARY terms, unchanged. Search + alphabetical grouping extracted into components/brewsoul/glossary-explorer.tsx. Verified live: 200 OK.</t>
         </is>
       </c>
       <c r="E173" s="14" t="inlineStr">
@@ -4917,7 +4917,7 @@
       <c r="A174" s="4" t="n"/>
       <c r="B174" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/economics</t>
+          <t>/brewsoul/pairings</t>
         </is>
       </c>
       <c r="C174" s="13" t="inlineStr">
@@ -4927,7 +4927,7 @@
       </c>
       <c r="D174" s="4" t="inlineStr">
         <is>
-          <t>reference: economics. Real live-computed stats (coffee/origin/roaster/variety counts, average price, average farmer share via DOLLAR_BREAKDOWNS), a real price-distribution histogram, and a real top-origins ranking — all computed directly from BREWSOUL_COFFEES at render time, unchanged. Fully static. Verified live: 200 OK.</t>
+          <t>reference: pairings. Real PAIRINGS (food/drink pairings by origin) and 3 real curated FLIGHTS (each linking to real coffees in the catalog), unchanged. Fully static. Verified live: 200 OK.</t>
         </is>
       </c>
       <c r="E174" s="14" t="inlineStr">
@@ -4940,7 +4940,7 @@
       <c r="A175" s="4" t="n"/>
       <c r="B175" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/compare</t>
+          <t>/brewsoul/economics</t>
         </is>
       </c>
       <c r="C175" s="13" t="inlineStr">
@@ -4950,7 +4950,7 @@
       </c>
       <c r="D175" s="4" t="inlineStr">
         <is>
-          <t>tool: compare coffees. Real side-by-side comparison of up to 4 coffees across origin/producer/variety/process/price/cupping and the 4 intelligence scores (QPR/availability/wow/overall), unchanged. Interactivity in components/brewsoul/compare-explorer.tsx. Verified live: 200 OK.</t>
+          <t>reference: economics. Real live-computed stats (coffee/origin/roaster/variety counts, average price, average farmer share via DOLLAR_BREAKDOWNS), a real price-distribution histogram, and a real top-origins ranking — all computed directly from BREWSOUL_COFFEES at render time, unchanged. Fully static. Verified live: 200 OK.</t>
         </is>
       </c>
       <c r="E175" s="14" t="inlineStr">
@@ -4963,7 +4963,7 @@
       <c r="A176" s="4" t="n"/>
       <c r="B176" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/blend-builder</t>
+          <t>/brewsoul/compare</t>
         </is>
       </c>
       <c r="C176" s="13" t="inlineStr">
@@ -4973,7 +4973,7 @@
       </c>
       <c r="D176" s="4" t="inlineStr">
         <is>
-          <t>tool: blend builder. Real combine-up-to-5-coffees ratio calculator with weighted-average QPR/Wow/Overall scores via range sliders, unchanged (never persisted anywhere in legacy either — a pure in-session calculator). Interactivity in components/brewsoul/blend-builder-explorer.tsx. Verified live: 200 OK.</t>
+          <t>tool: compare coffees. Real side-by-side comparison of up to 4 coffees across origin/producer/variety/process/price/cupping and the 4 intelligence scores (QPR/availability/wow/overall), unchanged. Interactivity in components/brewsoul/compare-explorer.tsx. Verified live: 200 OK.</t>
         </is>
       </c>
       <c r="E176" s="14" t="inlineStr">
@@ -4986,7 +4986,7 @@
       <c r="A177" s="4" t="n"/>
       <c r="B177" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/drops</t>
+          <t>/brewsoul/blend-builder</t>
         </is>
       </c>
       <c r="C177" s="13" t="inlineStr">
@@ -4996,7 +4996,7 @@
       </c>
       <c r="D177" s="4" t="inlineStr">
         <is>
-          <t>tool: product drops ("Latest Drops"). Real top-12-by-overall-score coffees. No client-side state at all (legacy's own useMemo had no changing dependencies — a pure derived list), so this ships as a plain Server Component. Verified live: 200 OK.</t>
+          <t>tool: blend builder. Real combine-up-to-5-coffees ratio calculator with weighted-average QPR/Wow/Overall scores via range sliders, unchanged (never persisted anywhere in legacy either — a pure in-session calculator). Interactivity in components/brewsoul/blend-builder-explorer.tsx. Verified live: 200 OK.</t>
         </is>
       </c>
       <c r="E177" s="14" t="inlineStr">
@@ -5009,7 +5009,7 @@
       <c r="A178" s="4" t="n"/>
       <c r="B178" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/collection</t>
+          <t>/brewsoul/drops</t>
         </is>
       </c>
       <c r="C178" s="13" t="inlineStr">
@@ -5019,7 +5019,7 @@
       </c>
       <c r="D178" s="4" t="inlineStr">
         <is>
-          <t>tool: personal collection tracker ("My Collection"). Real save/toggle-to-collection behavior, unchanged. Real bug found and fixed: legacy read localStorage directly inside a useState initializer — unsafe during SSR, same hydration-mismatch class already fixed in journey-bar.tsx/journey-tracker.tsx — rebuilt around a module-level external store fed through useSyncExternalStore in components/brewsoul/collection-explorer.tsx. Also found and fixed: the already-ported brewsoul-directory.ts listed this page's path as /brewsoul/my-coffees — a real dead link in legacy's own directory (legacy's actual router only ever served this at /brewsoul/collection, /brewsoul/my-coffees never existed) — corrected to the real path. Verified live: 200 OK.</t>
+          <t>tool: product drops ("Latest Drops"). Real top-12-by-overall-score coffees. No client-side state at all (legacy's own useMemo had no changing dependencies — a pure derived list), so this ships as a plain Server Component. Verified live: 200 OK.</t>
         </is>
       </c>
       <c r="E178" s="14" t="inlineStr">
@@ -5032,7 +5032,7 @@
       <c r="A179" s="4" t="n"/>
       <c r="B179" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/submit</t>
+          <t>/brewsoul/collection</t>
         </is>
       </c>
       <c r="C179" s="13" t="inlineStr">
@@ -5042,7 +5042,7 @@
       </c>
       <c r="D179" s="4" t="inlineStr">
         <is>
-          <t>tool: submit a coffee ("Submit or Appeal"). Real submit-a-coffee / appeal-a-score form, unchanged in structure. Real bug found and fixed: legacy's own comment admitted "In production this would POST to a tRPC endpoint" but in the meantime wrote the submission to localStorage and showed "Received. We'll review your submission" regardless — actively misleading, since nobody would ever see a localStorage-only write. Replaced with a real mailto: fallback pre-filled with the form fields, same honest-degradation pattern as first-sip-email-capture.tsx — no fake success state. Verified live: 200 OK.</t>
+          <t>tool: personal collection tracker ("My Collection"). Real save/toggle-to-collection behavior, unchanged. Real bug found and fixed: legacy read localStorage directly inside a useState initializer — unsafe during SSR, same hydration-mismatch class already fixed in journey-bar.tsx/journey-tracker.tsx — rebuilt around a module-level external store fed through useSyncExternalStore in components/brewsoul/collection-explorer.tsx. Also found and fixed: the already-ported brewsoul-directory.ts listed this page's path as /brewsoul/my-coffees — a real dead link in legacy's own directory (legacy's actual router only ever served this at /brewsoul/collection, /brewsoul/my-coffees never existed) — corrected to the real path. Verified live: 200 OK.</t>
         </is>
       </c>
       <c r="E179" s="14" t="inlineStr">
@@ -5055,7 +5055,7 @@
       <c r="A180" s="4" t="n"/>
       <c r="B180" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/prescription</t>
+          <t>/brewsoul/submit</t>
         </is>
       </c>
       <c r="C180" s="13" t="inlineStr">
@@ -5065,7 +5065,7 @@
       </c>
       <c r="D180" s="4" t="inlineStr">
         <is>
-          <t>personalized "prescription", ported from BrewSoulPrescriptionFull.tsx (the file legacy's router actually uses — BrewSoulTools.tsx's same-named export is dead/unrouted, same shadowed-file trap as /brewsoul/health). Real 5-step questionnaire (genetics/timing/health/flavor/budget) generating a real, deterministic prescription (generatePrescription — real roast/cup-count/brand/pricing/warning logic), all ported unchanged and verbatim. Legacy's trpc.coffeePrescription.generate AI-enhancement mutation doesn't exist in this migration — dropped along with its "AI ANALYSIS LOADING..." block, which would otherwise spin forever and never resolve; the real prescription itself never depended on that call, it's already fully computed client-side. Same bespoke earthy "science" palette as /brewsoul/health kept as the same deliberate sub-identity. Verified live: 200 OK, typecheck/lint clean.</t>
+          <t>tool: submit a coffee ("Submit or Appeal"). Real submit-a-coffee / appeal-a-score form, unchanged in structure. Real bug found and fixed: legacy's own comment admitted "In production this would POST to a tRPC endpoint" but in the meantime wrote the submission to localStorage and showed "Received. We'll review your submission" regardless — actively misleading, since nobody would ever see a localStorage-only write. Replaced with a real mailto: fallback pre-filled with the form fields, same honest-degradation pattern as first-sip-email-capture.tsx — no fake success state. Verified live: 200 OK.</t>
         </is>
       </c>
       <c r="E180" s="14" t="inlineStr">
@@ -5078,7 +5078,7 @@
       <c r="A181" s="4" t="n"/>
       <c r="B181" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/chains</t>
+          <t>/brewsoul/prescription</t>
         </is>
       </c>
       <c r="C181" s="13" t="inlineStr">
@@ -5088,7 +5088,7 @@
       </c>
       <c r="D181" s="4" t="inlineStr">
         <is>
-          <t>"Top 100 Coffee Chains" ranking (not supply-chain visualization — that's /brewsoul/economics//brewsoul/follow-the-dollar; this is chain rankings). Real 100-chain dataset extracted from legacy's computed CHAIN_RANKINGS export (5 real weighted dimensions → aggregate → S-F tier) via a one-off tsx script (same approach as brewsoul-coffees.ts) into lib/content/brewsoul-chains.ts, with a new ChainEntry type added to intelligence-engine/types.ts. Real tier/type filters, search, and per-chain expand, unchanged, extracted into components/brewsoul/chains-explorer.tsx. Verified live: 200 OK, typecheck/lint clean.</t>
+          <t>personalized "prescription", ported from BrewSoulPrescriptionFull.tsx (the file legacy's router actually uses — BrewSoulTools.tsx's same-named export is dead/unrouted, same shadowed-file trap as /brewsoul/health). Real 5-step questionnaire (genetics/timing/health/flavor/budget) generating a real, deterministic prescription (generatePrescription — real roast/cup-count/brand/pricing/warning logic), all ported unchanged and verbatim. Legacy's trpc.coffeePrescription.generate AI-enhancement mutation doesn't exist in this migration — dropped along with its "AI ANALYSIS LOADING..." block, which would otherwise spin forever and never resolve; the real prescription itself never depended on that call, it's already fully computed client-side. Same bespoke earthy "science" palette as /brewsoul/health kept as the same deliberate sub-identity. Verified live: 200 OK, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E181" s="14" t="inlineStr">
@@ -5101,7 +5101,7 @@
       <c r="A182" s="4" t="n"/>
       <c r="B182" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/biodynamic</t>
+          <t>/brewsoul/chains</t>
         </is>
       </c>
       <c r="C182" s="13" t="inlineStr">
@@ -5111,7 +5111,7 @@
       </c>
       <c r="D182" s="4" t="inlineStr">
         <is>
-          <t>biodynamic content. The complete real census of Demeter-certified biodynamic coffee: 3 real source farms, 6 real roasters/brands with real product tables and pricing, real nutritional-science compounds, a real cost calculator, and a real impact/tokenization section, all ported unchanged and verbatim. Dead Manus hero image dropped for a CSS gradient. The 3 genuinely interactive pieces (click-to-expand farms/roasters, cups-per-day cost slider) split into components/brewsoul/{biodynamic-farms,biodynamic-roasters,cost-calculator}.tsx client islands so the rest stays a Server Component. Same bespoke earthy "science" palette as /brewsoul/health and /brewsoul/prescription kept as the same deliberate sub-identity. Verified live: 200 OK, typecheck/lint clean.</t>
+          <t>"Top 100 Coffee Chains" ranking (not supply-chain visualization — that's /brewsoul/economics//brewsoul/follow-the-dollar; this is chain rankings). Real 100-chain dataset extracted from legacy's computed CHAIN_RANKINGS export (5 real weighted dimensions → aggregate → S-F tier) via a one-off tsx script (same approach as brewsoul-coffees.ts) into lib/content/brewsoul-chains.ts, with a new ChainEntry type added to intelligence-engine/types.ts. Real tier/type filters, search, and per-chain expand, unchanged, extracted into components/brewsoul/chains-explorer.tsx. Verified live: 200 OK, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E182" s="14" t="inlineStr">
@@ -5124,7 +5124,7 @@
       <c r="A183" s="4" t="n"/>
       <c r="B183" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/decaf</t>
+          <t>/brewsoul/biodynamic</t>
         </is>
       </c>
       <c r="C183" s="13" t="inlineStr">
@@ -5134,7 +5134,7 @@
       </c>
       <c r="D183" s="4" t="inlineStr">
         <is>
-          <t>decaf content ("Paint Stripper or Pure Water?"). Real 3-process breakdown (methylene chloride/Swiss Water/supercritical CO₂), 13 real clean-decaf brands ("Hall of Fame"), 10 real methylene-chloride brands ("Wall of Shame," with real Clean Label Project lawsuit citations), a real carbon footprint comparison, real decaf health science, and a real price-comparison table, all ported unchanged and verbatim. Legacy's manual document.title/&lt;meta keywords&gt; mutation in a useEffect (a real anti-pattern — Next's generateMetadata already owns the head) dropped for the real metadata export. Real bug found and fixed: the 13-brand FAME dataset was initially exported from the "use client" decaf-fame.tsx component file and imported into the Server Component page for its price-comparison table — non-component exports from a client module aren't available across the RSC boundary, which threw FAME is not iterable at runtime (only caught by live verification, not typecheck/lint). Moved the data to a plain lib/content/brewsoul-decaf.ts module instead. The 2 genuinely interactive pieces (click-to-expand Hall of Fame, reveal-toggle Wall of Shame) split into components/brewsoul/decaf-{fame,shame}.tsx client islands. Same bespoke earthy "science" palette as the other /brewsoul deep-dive pages kept as the same deliberate sub-identity. Verified live: 200 OK, typecheck/lint clean.</t>
+          <t>biodynamic content. The complete real census of Demeter-certified biodynamic coffee: 3 real source farms, 6 real roasters/brands with real product tables and pricing, real nutritional-science compounds, a real cost calculator, and a real impact/tokenization section, all ported unchanged and verbatim. Dead Manus hero image dropped for a CSS gradient. The 3 genuinely interactive pieces (click-to-expand farms/roasters, cups-per-day cost slider) split into components/brewsoul/{biodynamic-farms,biodynamic-roasters,cost-calculator}.tsx client islands so the rest stays a Server Component. Same bespoke earthy "science" palette as /brewsoul/health and /brewsoul/prescription kept as the same deliberate sub-identity. Verified live: 200 OK, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E183" s="14" t="inlineStr">
@@ -5147,7 +5147,7 @@
       <c r="A184" s="4" t="n"/>
       <c r="B184" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/esoteric</t>
+          <t>/brewsoul/decaf</t>
         </is>
       </c>
       <c r="C184" s="13" t="inlineStr">
@@ -5157,7 +5157,7 @@
       </c>
       <c r="D184" s="4" t="inlineStr">
         <is>
-          <t>rare-coffee content ("Esoteric Coffee Index"). Real 9-coffee index across 2 tiers (Panama Geisha, Yemen Mokha, Liberica, Eugenioides, Wush Wush, Sidra, Pink Bourbon, Bourbon Aji, Sudan Rume) with real tasting notes, rarity scores, and real named buy sources, plus a real acquisition-priority list and explorer scorecard, all ported unchanged and verbatim. Real content gap found, not fixed: legacy's own "Top 10 Acquisition Priority" list and scorecard table both reference "Laurina" as a 10th entry, but no coffee card for it exists anywhere in the source dataset — ported as-is rather than inventing card content that was never written. Zero client-side state anywhere in this page (only CSS-able hover) — ships entirely as a Server Component. Verified live: 200 OK, typecheck/lint clean.</t>
+          <t>decaf content ("Paint Stripper or Pure Water?"). Real 3-process breakdown (methylene chloride/Swiss Water/supercritical CO₂), 13 real clean-decaf brands ("Hall of Fame"), 10 real methylene-chloride brands ("Wall of Shame," with real Clean Label Project lawsuit citations), a real carbon footprint comparison, real decaf health science, and a real price-comparison table, all ported unchanged and verbatim. Legacy's manual document.title/&lt;meta keywords&gt; mutation in a useEffect (a real anti-pattern — Next's generateMetadata already owns the head) dropped for the real metadata export. Real bug found and fixed: the 13-brand FAME dataset was initially exported from the "use client" decaf-fame.tsx component file and imported into the Server Component page for its price-comparison table — non-component exports from a client module aren't available across the RSC boundary, which threw FAME is not iterable at runtime (only caught by live verification, not typecheck/lint). Moved the data to a plain lib/content/brewsoul-decaf.ts module instead. The 2 genuinely interactive pieces (click-to-expand Hall of Fame, reveal-toggle Wall of Shame) split into components/brewsoul/decaf-{fame,shame}.tsx client islands. Same bespoke earthy "science" palette as the other /brewsoul deep-dive pages kept as the same deliberate sub-identity. Verified live: 200 OK, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E184" s="14" t="inlineStr">
@@ -5170,7 +5170,7 @@
       <c r="A185" s="4" t="n"/>
       <c r="B185" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/cities + /brewsoul/cities/[slug]</t>
+          <t>/brewsoul/esoteric</t>
         </is>
       </c>
       <c r="C185" s="13" t="inlineStr">
@@ -5180,7 +5180,7 @@
       </c>
       <c r="D185" s="4" t="inlineStr">
         <is>
-          <t>city directory + detail ("City Intelligence Module"). Real 25-city leaderboard (name/state/grade/score/tagline/verdict/live stats), a real 7-dimension scoring methodology, and real national + universal/nuanced chain report cards, all ported unchanged and verbatim into lib/content/brewsoul-cities.ts. Real data-completeness note, not a bug: legacy's own comment admits only Portland has full shop-by-shop data (25 real best + 5 real worst shops with real blurbs/scores/order-this/skip-this) — the other 24 cities have real city-level stats but empty shop/chain/bridge-drink/non-coffee arrays; legacy's own UI already handles this honestly (a real "Full data coming soon" state on both the card and detail page, not fake data) — preserved exactly, verified for both Portland (full tabs) and Seattle (coming-soon state). Grade filter, methodology modal, and chain-toggle interactivity in components/brewsoul/cities-explorer.tsx; per-city tab switching and per-shop expand in components/brewsoul/city-detail-tabs.tsx. Detail route uses generateStaticParams over all 25 real slugs. Scroll-linked parallax and floating-particle backgrounds dropped, same decoration call made throughout this migration. Real image-hosting gap flagged, not silently worked around: the 25 city hero photos are real, live Unsplash URLs (not a dead Manus proxy) but aren't yet uploaded to Sanity per this repo's own image convention — added images.unsplash.com to next.config.ts's remotePatterns as an interim measure rather th</t>
+          <t>rare-coffee content ("Esoteric Coffee Index"). Real 9-coffee index across 2 tiers (Panama Geisha, Yemen Mokha, Liberica, Eugenioides, Wush Wush, Sidra, Pink Bourbon, Bourbon Aji, Sudan Rume) with real tasting notes, rarity scores, and real named buy sources, plus a real acquisition-priority list and explorer scorecard, all ported unchanged and verbatim. Real content gap found, not fixed: legacy's own "Top 10 Acquisition Priority" list and scorecard table both reference "Laurina" as a 10th entry, but no coffee card for it exists anywhere in the source dataset — ported as-is rather than inventing card content that was never written. Zero client-side state anywhere in this page (only CSS-able hover) — ships entirely as a Server Component. Verified live: 200 OK, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E185" s="14" t="inlineStr">
@@ -5193,7 +5193,7 @@
       <c r="A186" s="4" t="n"/>
       <c r="B186" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/directory</t>
+          <t>/brewsoul/cities + /brewsoul/cities/[slug]</t>
         </is>
       </c>
       <c r="C186" s="13" t="inlineStr">
@@ -5203,7 +5203,7 @@
       </c>
       <c r="D186" s="4" t="inlineStr">
         <is>
-          <t>real master page index ("Everything Inside BrewSoul," not a roaster directory — that's /brewsoul/roasters). Real 6 categories with real page descriptions/icons, unchanged; the underlying data already lived in lib/content/brewsoul-directory.ts (built earlier this phase to power CategoryBadge) — this route is where it finally becomes a real browsable page. Category filter extracted into components/brewsoul/directory-explorer.tsx. Fixed the stale "Browse All 103 Coffees" label (real count is 107) by dropping the hardcoded number from the shared data module — benefits every other consumer of that module too. Verified live: 200 OK, typecheck/lint clean.</t>
+          <t>city directory + detail ("City Intelligence Module"). Real 25-city leaderboard (name/state/grade/score/tagline/verdict/live stats), a real 7-dimension scoring methodology, and real national + universal/nuanced chain report cards, all ported unchanged and verbatim into lib/content/brewsoul-cities.ts. Real data-completeness note, not a bug: legacy's own comment admits only Portland has full shop-by-shop data (25 real best + 5 real worst shops with real blurbs/scores/order-this/skip-this) — the other 24 cities have real city-level stats but empty shop/chain/bridge-drink/non-coffee arrays; legacy's own UI already handles this honestly (a real "Full data coming soon" state on both the card and detail page, not fake data) — preserved exactly, verified for both Portland (full tabs) and Seattle (coming-soon state). Grade filter, methodology modal, and chain-toggle interactivity in components/brewsoul/cities-explorer.tsx; per-city tab switching and per-shop expand in components/brewsoul/city-detail-tabs.tsx. Detail route uses generateStaticParams over all 25 real slugs. Scroll-linked parallax and floating-particle backgrounds dropped, same decoration call made throughout this migration. Real image-hosting gap flagged, not silently worked around: the 25 city hero photos are real, live Unsplash URLs (not a dead Manus proxy) but aren't yet uploaded to Sanity per this repo's own image convention — added images.unsplash.com to next.config.ts's remotePatterns as an interim measure rather th</t>
         </is>
       </c>
       <c r="E186" s="14" t="inlineStr">
@@ -5216,7 +5216,7 @@
       <c r="A187" s="4" t="n"/>
       <c r="B187" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/guest + /brewsoul/guest/shanita-nicholas</t>
+          <t>/brewsoul/directory</t>
         </is>
       </c>
       <c r="C187" s="13" t="inlineStr">
@@ -5226,7 +5226,7 @@
       </c>
       <c r="D187" s="4" t="inlineStr">
         <is>
-          <t>guest series index + profile ("Tony G Guest Series"). Real single guest entry (Shanita Nicholas — real headline/teaser/tags) on the index, and the real 10-question interview on the detail page (Fair Trade economics, roasting mythology, the C Market, regenerative vs. sustainable, origin-roasting economics vs. Fair Trade, blockchain traceability, pre-harvest financing — real substantive answers with real citations), all ported unchanged and verbatim into components/brewsoul/shanita-interview.tsx. Legacy's guest photo (/api/img/brewsoul-orig_84eb4bc9.jpg) was the same dead Manus proxy confirmed 404 throughout this migration — dropped for a plain initial avatar on both pages rather than a broken headshot. Per-question expand/collapse, "Expand/Collapse All," and the real Twitter/LinkedIn/copy-link share row are genuinely interactive, split into client islands. Verified live: 200 OK on both, typecheck/lint clean.</t>
+          <t>real master page index ("Everything Inside BrewSoul," not a roaster directory — that's /brewsoul/roasters). Real 6 categories with real page descriptions/icons, unchanged; the underlying data already lived in lib/content/brewsoul-directory.ts (built earlier this phase to power CategoryBadge) — this route is where it finally becomes a real browsable page. Category filter extracted into components/brewsoul/directory-explorer.tsx. Fixed the stale "Browse All 103 Coffees" label (real count is 107) by dropping the hardcoded number from the shared data module — benefits every other consumer of that module too. Verified live: 200 OK, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E187" s="14" t="inlineStr">
@@ -5239,63 +5239,63 @@
       <c r="A188" s="4" t="n"/>
       <c r="B188" s="4" t="inlineStr">
         <is>
+          <t>/brewsoul/guest + /brewsoul/guest/shanita-nicholas</t>
+        </is>
+      </c>
+      <c r="C188" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D188" s="4" t="inlineStr">
+        <is>
+          <t>guest series index + profile ("Tony G Guest Series"). Real single guest entry (Shanita Nicholas — real headline/teaser/tags) on the index, and the real 10-question interview on the detail page (Fair Trade economics, roasting mythology, the C Market, regenerative vs. sustainable, origin-roasting economics vs. Fair Trade, blockchain traceability, pre-harvest financing — real substantive answers with real citations), all ported unchanged and verbatim into components/brewsoul/shanita-interview.tsx. Legacy's guest photo (/api/img/brewsoul-orig_84eb4bc9.jpg) was the same dead Manus proxy confirmed 404 throughout this migration — dropped for a plain initial avatar on both pages rather than a broken headshot. Per-question expand/collapse, "Expand/Collapse All," and the real Twitter/LinkedIn/copy-link share row are genuinely interactive, split into client islands. Verified live: 200 OK on both, typecheck/lint clean.</t>
+        </is>
+      </c>
+      <c r="E188" s="14" t="inlineStr">
+        <is>
+          <t>Phase 6 — BrewSoul (28 routes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="4" t="n"/>
+      <c r="B189" s="4" t="inlineStr">
+        <is>
           <t>Shared: port BrewSoulLayout, CategoryBadge, JourneyBar, NextSteps as Next.js layout/components</t>
         </is>
       </c>
-      <c r="C188" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D188" s="4" t="inlineStr">
+      <c r="C189" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D189" s="4" t="inlineStr">
         <is>
           <t>app/brewsoul/layout.tsx + components/brewsoul/{brewsoul-nav,category-badge,journey-bar,next-steps}.tsx, all built and reused by every /brewsoul/* route above.</t>
         </is>
       </c>
-      <c r="E188" s="14" t="inlineStr">
+      <c r="E189" s="14" t="inlineStr">
         <is>
           <t>Phase 6 — BrewSoul (28 routes)</t>
         </is>
       </c>
     </row>
-    <row r="189">
-      <c r="A189" s="10" t="inlineStr">
+    <row r="190">
+      <c r="A190" s="10" t="inlineStr">
         <is>
           <t>Phase 7 — PRI &amp; Kava Encyclopedias (19 routes)</t>
         </is>
       </c>
-      <c r="B189" s="11" t="n"/>
-      <c r="C189" s="11" t="n"/>
-      <c r="D189" s="12" t="n"/>
-    </row>
-    <row r="190">
-      <c r="A190" s="4" t="n"/>
-      <c r="B190" s="4" t="inlineStr">
-        <is>
-          <t>Kava shared foundation</t>
-        </is>
-      </c>
-      <c r="C190" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D190" s="4" t="inlineStr">
-        <is>
-          <t>app/kava/layout.tsx + components/kava/kava-nav.tsx (KavaNav/KavaFooter, 10 real nav items) + components/kava/kava-ui.tsx (KavaHero/KavaSection/KavaSectionTitle/KavaCard/KavaBadge/KavaDivider/KavaDisclaimer, converted from legacy inline style={} to Tailwind + new --kava-* tokens in globals.css). Added /kava to site-chrome.tsx's SUPPRESSED_PREFIXES (self-contained sub-site, same pattern as BrewSoul and /attention-theft). Real dead link fixed: legacy nav pointed at /pri, which legacy's own App.tsx never routed (only /psychedelic-readiness-index exists) — corrected.</t>
-        </is>
-      </c>
-      <c r="E190" s="14" t="inlineStr">
-        <is>
-          <t>Phase 7 — PRI &amp; Kava Encyclopedias (19 routes)</t>
-        </is>
-      </c>
+      <c r="B190" s="11" t="n"/>
+      <c r="C190" s="11" t="n"/>
+      <c r="D190" s="12" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="4" t="n"/>
       <c r="B191" s="4" t="inlineStr">
         <is>
-          <t>/kava (home)</t>
+          <t>Kava shared foundation</t>
         </is>
       </c>
       <c r="C191" s="13" t="inlineStr">
@@ -5305,7 +5305,7 @@
       </c>
       <c r="D191" s="4" t="inlineStr">
         <is>
-          <t>9 module cards, "Threshold Doctrine," "Sacred Masculine Triad" (Mezcal/Kava/Peyote), 4 market stats, all ported unchanged. Verified live: 200 OK, exactly 1 header/1 footer (chrome suppression confirmed), typecheck/lint clean.</t>
+          <t>app/kava/layout.tsx + components/kava/kava-nav.tsx (KavaNav/KavaFooter, 10 real nav items) + components/kava/kava-ui.tsx (KavaHero/KavaSection/KavaSectionTitle/KavaCard/KavaBadge/KavaDivider/KavaDisclaimer, converted from legacy inline style={} to Tailwind + new --kava-* tokens in globals.css). Added /kava to site-chrome.tsx's SUPPRESSED_PREFIXES (self-contained sub-site, same pattern as BrewSoul and /attention-theft). Real dead link fixed: legacy nav pointed at /pri, which legacy's own App.tsx never routed (only /psychedelic-readiness-index exists) — corrected.</t>
         </is>
       </c>
       <c r="E191" s="14" t="inlineStr">
@@ -5318,7 +5318,7 @@
       <c r="A192" s="4" t="n"/>
       <c r="B192" s="4" t="inlineStr">
         <is>
-          <t>/kava/origins</t>
+          <t>/kava (home)</t>
         </is>
       </c>
       <c r="C192" s="13" t="inlineStr">
@@ -5328,7 +5328,7 @@
       </c>
       <c r="D192" s="4" t="inlineStr">
         <is>
-          <t>real migration timeline (6 Pacific nations, ~3000 BCE–1000 CE), real 6-island selector (Vanuatu/Fiji/Tonga/Samoa/Hawaii/Pohnpei, each with real facts/ceremony/cultivar/safety content), and the real Noble vs. Tudei safety comparison, all ported unchanged and verbatim. Island-selector interactivity in components/kava/origins-explorer.tsx. Verified live: 200 OK, typecheck/lint clean.</t>
+          <t>9 module cards, "Threshold Doctrine," "Sacred Masculine Triad" (Mezcal/Kava/Peyote), 4 market stats, all ported unchanged. Verified live: 200 OK, exactly 1 header/1 footer (chrome suppression confirmed), typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E192" s="14" t="inlineStr">
@@ -5341,7 +5341,7 @@
       <c r="A193" s="4" t="n"/>
       <c r="B193" s="4" t="inlineStr">
         <is>
-          <t>/kava/interactions</t>
+          <t>/kava/origins</t>
         </is>
       </c>
       <c r="C193" s="13" t="inlineStr">
@@ -5351,7 +5351,7 @@
       </c>
       <c r="D193" s="4" t="inlineStr">
         <is>
-          <t>real 24-substance drug interaction database (real severity ratings across an 11-value scale, real pharmacological mechanisms, real PRI protocol guidance) and real 5-enzyme CYP450 inhibition profile, ported unchanged and verbatim. Search + severity-filter interactivity in components/kava/interactions-explorer.tsx, using a precomposed SEVERITY_CONFIG class lookup (not string-built classes — same Tailwind static-scanner rule enforced elsewhere this migration). Legacy's unused Download icon import (dead code, no export feature attached to it) not ported. Verified live: 200 OK, typecheck/lint clean.</t>
+          <t>real migration timeline (6 Pacific nations, ~3000 BCE–1000 CE), real 6-island selector (Vanuatu/Fiji/Tonga/Samoa/Hawaii/Pohnpei, each with real facts/ceremony/cultivar/safety content), and the real Noble vs. Tudei safety comparison, all ported unchanged and verbatim. Island-selector interactivity in components/kava/origins-explorer.tsx. Verified live: 200 OK, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E193" s="14" t="inlineStr">
@@ -5364,7 +5364,7 @@
       <c r="A194" s="4" t="n"/>
       <c r="B194" s="4" t="inlineStr">
         <is>
-          <t>/kava/science</t>
+          <t>/kava/interactions</t>
         </is>
       </c>
       <c r="C194" s="13" t="inlineStr">
@@ -5374,7 +5374,7 @@
       </c>
       <c r="D194" s="4" t="inlineStr">
         <is>
-          <t>real 6 major kavalactones (real receptor mechanisms, real PRI relevance) and real 11-item combined pharmacological profile, ported unchanged into lib/content/kava-science.ts. RSC-boundary bug caught proactively before shipping: initially drafted KAVALACTONES as an export of the "use client" chemotype-decoder.tsx, which would have thrown the same TypeError: X is not iterable already hit once this migration on /brewsoul/decaf when the Server Component page tried to import it — moved to the plain data module before ever running it. Chemotype decoder tool (enter e.g. 4-2-6-5-3-1, see dominant kavalactones) kept as the real interactive client island. Verified live: 200 OK, typecheck/lint clean.</t>
+          <t>real 24-substance drug interaction database (real severity ratings across an 11-value scale, real pharmacological mechanisms, real PRI protocol guidance) and real 5-enzyme CYP450 inhibition profile, ported unchanged and verbatim. Search + severity-filter interactivity in components/kava/interactions-explorer.tsx, using a precomposed SEVERITY_CONFIG class lookup (not string-built classes — same Tailwind static-scanner rule enforced elsewhere this migration). Legacy's unused Download icon import (dead code, no export feature attached to it) not ported. Verified live: 200 OK, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E194" s="14" t="inlineStr">
@@ -5387,7 +5387,7 @@
       <c r="A195" s="4" t="n"/>
       <c r="B195" s="4" t="inlineStr">
         <is>
-          <t>/kava/assessment</t>
+          <t>/kava/science</t>
         </is>
       </c>
       <c r="C195" s="13" t="inlineStr">
@@ -5397,7 +5397,7 @@
       </c>
       <c r="D195" s="4" t="inlineStr">
         <is>
-          <t>real 5-domain, 20-question PRI readiness assessment (somatic/psychological/relational/cultural/integration), real per-domain point weights, and real 4-band recommendation scoring (CLEARED/CONDITIONAL/DEFER/NOT READY), all ported unchanged into components/kava/assessment-quiz.tsx. Fully stateful (domain navigation, per-question answers, results view), so kept as a single client island per this migration's established pattern for multi-step assessments. Domain and recommendation accent colors (5 + 4 distinct hexes, none matching the --kava-* brand palette) precomposed into literal DOMAIN_STYLES/RECOMMENDATION_STYLES lookup objects rather than style={}, avoiding the dynamic-class bug already caught twice this migration (chains-explorer.tsx, biodynamic/page.tsx). Real backend gap, handled honestly: legacy's AssessmentResultActions took sessionId/serialized-answers props feeding a trpc.assessments.submit mutation this migration never built — used the already-simplified, print-only AssessmentResultActions (components/assessments/result-actions.tsx, built during Phase 9) instead of reproducing a submit call with no backend. Verified live: 200 OK, real domain/question content confirmed in rendered HTML, typecheck/lint clean.</t>
+          <t>real 6 major kavalactones (real receptor mechanisms, real PRI relevance) and real 11-item combined pharmacological profile, ported unchanged into lib/content/kava-science.ts. RSC-boundary bug caught proactively before shipping: initially drafted KAVALACTONES as an export of the "use client" chemotype-decoder.tsx, which would have thrown the same TypeError: X is not iterable already hit once this migration on /brewsoul/decaf when the Server Component page tried to import it — moved to the plain data module before ever running it. Chemotype decoder tool (enter e.g. 4-2-6-5-3-1, see dominant kavalactones) kept as the real interactive client island. Verified live: 200 OK, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E195" s="14" t="inlineStr">
@@ -5410,7 +5410,7 @@
       <c r="A196" s="4" t="n"/>
       <c r="B196" s="4" t="inlineStr">
         <is>
-          <t>/kava/hawaii</t>
+          <t>/kava/assessment</t>
         </is>
       </c>
       <c r="C196" s="13" t="inlineStr">
@@ -5420,7 +5420,7 @@
       </c>
       <c r="D196" s="4" t="inlineStr">
         <is>
-          <t>real ICE/meth crisis statistics (Quest Diagnostics 410% figure, Hawaii DOH conviction rates, law enforcement seizure data), real dual crisis/revival timeline (1985–present), the real (explicitly-labeled hypothesis, not proven) pharmacological alignment table, and real recovery resource listings, all ported unchanged and verbatim. Fully static, no client island needed. Verified live: 200 OK, typecheck/lint clean.</t>
+          <t>real 5-domain, 20-question PRI readiness assessment (somatic/psychological/relational/cultural/integration), real per-domain point weights, and real 4-band recommendation scoring (CLEARED/CONDITIONAL/DEFER/NOT READY), all ported unchanged into components/kava/assessment-quiz.tsx. Fully stateful (domain navigation, per-question answers, results view), so kept as a single client island per this migration's established pattern for multi-step assessments. Domain and recommendation accent colors (5 + 4 distinct hexes, none matching the --kava-* brand palette) precomposed into literal DOMAIN_STYLES/RECOMMENDATION_STYLES lookup objects rather than style={}, avoiding the dynamic-class bug already caught twice this migration (chains-explorer.tsx, biodynamic/page.tsx). Real backend gap, handled honestly: legacy's AssessmentResultActions took sessionId/serialized-answers props feeding a trpc.assessments.submit mutation this migration never built — used the already-simplified, print-only AssessmentResultActions (components/assessments/result-actions.tsx, built during Phase 9) instead of reproducing a submit call with no backend. Verified live: 200 OK, real domain/question content confirmed in rendered HTML, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E196" s="14" t="inlineStr">
@@ -5433,7 +5433,7 @@
       <c r="A197" s="4" t="n"/>
       <c r="B197" s="4" t="inlineStr">
         <is>
-          <t>/kava/myths</t>
+          <t>/kava/hawaii</t>
         </is>
       </c>
       <c r="C197" s="13" t="inlineStr">
@@ -5443,7 +5443,7 @@
       </c>
       <c r="D197" s="4" t="inlineStr">
         <is>
-          <t>real 7-myth evidence review (2002/2014 European kava ban and reversal, WHO findings, CYP2D6 metabolism differences by population, chemotype/preparation distinctions) and the real closing takeaway, ported unchanged. Expand/collapse interactivity in components/kava/myths-explorer.tsx, verdict colors (3-value enum) precomposed into a literal VERDICT_CLASS lookup. Extended shared KavaCard (kava-ui.tsx) with an optional onClick prop to support this — first Kava page needing a clickable card. Verified live: 200 OK, typecheck/lint clean.</t>
+          <t>real ICE/meth crisis statistics (Quest Diagnostics 410% figure, Hawaii DOH conviction rates, law enforcement seizure data), real dual crisis/revival timeline (1985–present), the real (explicitly-labeled hypothesis, not proven) pharmacological alignment table, and real recovery resource listings, all ported unchanged and verbatim. Fully static, no client island needed. Verified live: 200 OK, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E197" s="14" t="inlineStr">
@@ -5456,7 +5456,7 @@
       <c r="A198" s="4" t="n"/>
       <c r="B198" s="4" t="inlineStr">
         <is>
-          <t>/kava/caffeine</t>
+          <t>/kava/myths</t>
         </is>
       </c>
       <c r="C198" s="13" t="inlineStr">
@@ -5466,7 +5466,7 @@
       </c>
       <c r="D198" s="4" t="inlineStr">
         <is>
-          <t>real CYP1A2 inhibition mechanism (56%, the same pathway grapefruit juice uses on medications), real caffeine cutoff protocol, and the real kava-vs-coffee comparison table, ported unchanged. Fully static, no client island needed. Verified live: 200 OK, typecheck/lint clean.</t>
+          <t>real 7-myth evidence review (2002/2014 European kava ban and reversal, WHO findings, CYP2D6 metabolism differences by population, chemotype/preparation distinctions) and the real closing takeaway, ported unchanged. Expand/collapse interactivity in components/kava/myths-explorer.tsx, verdict colors (3-value enum) precomposed into a literal VERDICT_CLASS lookup. Extended shared KavaCard (kava-ui.tsx) with an optional onClick prop to support this — first Kava page needing a clickable card. Verified live: 200 OK, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E198" s="14" t="inlineStr">
@@ -5479,7 +5479,7 @@
       <c r="A199" s="4" t="n"/>
       <c r="B199" s="4" t="inlineStr">
         <is>
-          <t>/kava/products</t>
+          <t>/kava/caffeine</t>
         </is>
       </c>
       <c r="C199" s="13" t="inlineStr">
@@ -5489,7 +5489,7 @@
       </c>
       <c r="D199" s="4" t="inlineStr">
         <is>
-          <t>real 5-category product index (ceremonial powder, fresh frozen, RTD beverages, supplements, kava bars) with real named vendors/cultivars/chemotypes/pricing/PRI ratings and real outbound buy links (all live vendor domains, not Manus proxies — no image assets on this page to check), ported unchanged into components/kava/products-explorer.tsx. Category-tab interactivity kept as the client island. Verified live: 200 OK, typecheck/lint clean.</t>
+          <t>real CYP1A2 inhibition mechanism (56%, the same pathway grapefruit juice uses on medications), real caffeine cutoff protocol, and the real kava-vs-coffee comparison table, ported unchanged. Fully static, no client island needed. Verified live: 200 OK, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E199" s="14" t="inlineStr">
@@ -5502,7 +5502,7 @@
       <c r="A200" s="4" t="n"/>
       <c r="B200" s="4" t="inlineStr">
         <is>
-          <t>/kava/certification</t>
+          <t>/kava/products</t>
         </is>
       </c>
       <c r="C200" s="13" t="inlineStr">
@@ -5512,7 +5512,7 @@
       </c>
       <c r="D200" s="4" t="inlineStr">
         <is>
-          <t>real 12-module, 80-hour facilitator curriculum, real 3-tier certification structure (Practitioner/Threshold Facilitator/Master Facilitator), and real prerequisites list, ported unchanged. Fully static, no client island needed; legacy's wouter cross-links replaced with next/link. Verified live: 200 OK, typecheck/lint clean.</t>
+          <t>real 5-category product index (ceremonial powder, fresh frozen, RTD beverages, supplements, kava bars) with real named vendors/cultivars/chemotypes/pricing/PRI ratings and real outbound buy links (all live vendor domains, not Manus proxies — no image assets on this page to check), ported unchanged into components/kava/products-explorer.tsx. Category-tab interactivity kept as the client island. Verified live: 200 OK, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E200" s="14" t="inlineStr">
@@ -5525,7 +5525,7 @@
       <c r="A201" s="4" t="n"/>
       <c r="B201" s="4" t="inlineStr">
         <is>
-          <t>PRI shared data: lib/content/pri-data.ts (copied verbatim from legacy pri/data.ts</t>
+          <t>/kava/certification</t>
         </is>
       </c>
       <c r="C201" s="13" t="inlineStr">
@@ -5535,7 +5535,7 @@
       </c>
       <c r="D201" s="4" t="inlineStr">
         <is>
-          <t>real 39-medicine pharmacopoeia, 50+ questions across 6 domains, MAO-B interaction matrix, medication interaction guide, crisis/integration resources, pathway questions), lib/content/pri-safety-data.ts (verbatim safety data merge source), lib/content/pri-medicine-images.ts (verbatim real CloudFront hero-image map, all spot-checked 200 OK — RampRate's own CDN, already whitelisted, not Manus), lib/content/pri-shared.ts (the real scoring engine — computeScores/READINESS_LEVELS/getMedicineWithSafety — extracted to a plain module per the RSC-boundary lesson from /brewsoul/decaf and /kava/science). Added --pri-* CSS custom properties to globals.css (this subsystem's own purple/parchment/near-black palette, same pattern as --kava-/--crusade-) since Phase 7's PRI section spans 9 more routes.</t>
+          <t>real 12-module, 80-hour facilitator curriculum, real 3-tier certification structure (Practitioner/Threshold Facilitator/Master Facilitator), and real prerequisites list, ported unchanged. Fully static, no client island needed; legacy's wouter cross-links replaced with next/link. Verified live: 200 OK, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E201" s="14" t="inlineStr">
@@ -5548,7 +5548,7 @@
       <c r="A202" s="4" t="n"/>
       <c r="B202" s="4" t="inlineStr">
         <is>
-          <t>/psychedelic-readiness-index (core tool)</t>
+          <t>PRI shared data: lib/content/pri-data.ts (copied verbatim from legacy pri/data.ts</t>
         </is>
       </c>
       <c r="C202" s="13" t="inlineStr">
@@ -5558,7 +5558,7 @@
       </c>
       <c r="D202" s="4" t="inlineStr">
         <is>
-          <t>the real hero, 39-medicine grid with compare/save/bookmark tooling, MAO-B interaction matrix, medication interaction guide, crisis resources, the real 5-state assessment flow (philosophy intro → readiness quiz → pathway &amp; access questions → legal disclaimer gate → results), medicine detail modal (overview/safety/correction tabs), testimonials, and ImpactSoul cross-promotion, all ported unchanged and verbatim into components/pri/psychedelic-readiness-index.tsx plus supporting client islands (disclaimer-gate.tsx, medicine-modal.tsx, safety-section.tsx, correction-form.tsx, share-bar.tsx, cinematic-band.tsx). Kept as one client island — a single state machine drives which section renders, same call made for other large multi-step assessments this migration. Real hero/section photography (8 CloudFront images) kept via next/image; legacy's purely decorative glitch-scanline overlay divs and CSS shimmer/glow @keyframes dropped (no framer-motion — CONTRIBUTING.md rule 5 — and "decoration not worth the cost," same call made throughout this migration).</t>
+          <t>real 39-medicine pharmacopoeia, 50+ questions across 6 domains, MAO-B interaction matrix, medication interaction guide, crisis/integration resources, pathway questions), lib/content/pri-safety-data.ts (verbatim safety data merge source), lib/content/pri-medicine-images.ts (verbatim real CloudFront hero-image map, all spot-checked 200 OK — RampRate's own CDN, already whitelisted, not Manus), lib/content/pri-shared.ts (the real scoring engine — computeScores/READINESS_LEVELS/getMedicineWithSafety — extracted to a plain module per the RSC-boundary lesson from /brewsoul/decaf and /kava/science). Added --pri-* CSS custom properties to globals.css (this subsystem's own purple/parchment/near-black palette, same pattern as --kava-/--crusade-) since Phase 7's PRI section spans 9 more routes.</t>
         </is>
       </c>
       <c r="E202" s="14" t="inlineStr">
@@ -5571,7 +5571,7 @@
       <c r="A203" s="4" t="n"/>
       <c r="B203" s="4" t="inlineStr">
         <is>
-          <t>PRI: /peyote-mescaline</t>
+          <t>/psychedelic-readiness-index (core tool)</t>
         </is>
       </c>
       <c r="C203" s="13" t="inlineStr">
@@ -5581,7 +5581,7 @@
       </c>
       <c r="D203" s="4" t="inlineStr">
         <is>
-          <t>MescalineDeepDive, real receptor pharmacology table, the real "Latuda Mirror" same-target-opposite-action comparison, real clinical outcomes (Agin-Liebes et al. 2021, n=452), the real 16-row pharma-to-plant alternatives table, real supplement protocol (pre/day-of/post-integration), real mescaline-specific PRI dimension scores, the real medicine-selector comparison table, and real sources, all ported unchanged and verbatim into lib/content/pri-mescaline-module.ts (copied verbatim) + app/peyote-mescaline/page.tsx. Fully static except the pharma-table expand toggle, extracted into components/pri/pharma-table.tsx; shared PriSection/PriEyebrow wrapper (components/pri/pri-section.tsx) introduced here for reuse by the remaining PRI deep-dive modules. All 8 real section photos (CloudFront) spot-checked live before use; legacy's purely decorative glitch-scanline overlays dropped. Verified live: 200 OK, real content confirmed in rendered HTML, exactly 1 header/1 footer, typecheck/lint clean.</t>
+          <t>the real hero, 39-medicine grid with compare/save/bookmark tooling, MAO-B interaction matrix, medication interaction guide, crisis resources, the real 5-state assessment flow (philosophy intro → readiness quiz → pathway &amp; access questions → legal disclaimer gate → results), medicine detail modal (overview/safety/correction tabs), testimonials, and ImpactSoul cross-promotion, all ported unchanged and verbatim into components/pri/psychedelic-readiness-index.tsx plus supporting client islands (disclaimer-gate.tsx, medicine-modal.tsx, safety-section.tsx, correction-form.tsx, share-bar.tsx, cinematic-band.tsx). Kept as one client island — a single state machine drives which section renders, same call made for other large multi-step assessments this migration. Real hero/section photography (8 CloudFront images) kept via next/image; legacy's purely decorative glitch-scanline overlay divs and CSS shimmer/glow @keyframes dropped (no framer-motion — CONTRIBUTING.md rule 5 — and "decoration not worth the cost," same call made throughout this migration).</t>
         </is>
       </c>
       <c r="E203" s="14" t="inlineStr">
@@ -5594,7 +5594,7 @@
       <c r="A204" s="4" t="n"/>
       <c r="B204" s="4" t="inlineStr">
         <is>
-          <t>PRI: /iboga-ibogaine</t>
+          <t>PRI: /peyote-mescaline</t>
         </is>
       </c>
       <c r="C204" s="13" t="inlineStr">
@@ -5604,7 +5604,7 @@
       </c>
       <c r="D204" s="4" t="inlineStr">
         <is>
-          <t>IbogaDeepDive, "The Plant vs The Isolate": real alkaloid-profile comparison, real receptor pharmacology, real head-to-head iboga-vs-ibogaine table, real clinical outcomes (Mash/Noller/Schenberg/Brown &amp; Alper/Cherian/Williams — including the 2024 Stanford Nature Medicine SOF-veteran data and the 2026 19,071-patient safety analysis), real pharma-to-plant alternatives, real supplement protocol, real dimension thresholds, real medicine selector, Tony's real first-hand account of sitting ibogaine at The Mission Within, real hard-stop contraindications, a real 9-facility directory (with the 2 facilities legacy explicitly removed and why), real Nagoya Protocol / extractive-capitalism argument, real 2026 US legal-status rundown, the embedded Iboga Compass v2 documentation section (components/pri/iboga-compass-section.tsx, its own client island for the question-group toggles), and real sources — all ported unchanged and verbatim into lib/content/pri-iboga-module.ts + lib/content/pri-iboga-compass-data.ts (both copied verbatim) + app/iboga-ibogaine/page.tsx. Fully static except the pharma-table expand toggle (components/pri/iboga-pharma-table.tsx) and the compass section's toggles; reused the shared PriSection/PriEyebrow wrapper from the mescaline module. All 5 real hero/section photos (CloudFront) spot-checked live before use. Verified live: 200 OK, real content confirmed in rendered HTML, exactly 1 header/1 footer, typecheck/lint clean.</t>
+          <t>MescalineDeepDive, real receptor pharmacology table, the real "Latuda Mirror" same-target-opposite-action comparison, real clinical outcomes (Agin-Liebes et al. 2021, n=452), the real 16-row pharma-to-plant alternatives table, real supplement protocol (pre/day-of/post-integration), real mescaline-specific PRI dimension scores, the real medicine-selector comparison table, and real sources, all ported unchanged and verbatim into lib/content/pri-mescaline-module.ts (copied verbatim) + app/peyote-mescaline/page.tsx. Fully static except the pharma-table expand toggle, extracted into components/pri/pharma-table.tsx; shared PriSection/PriEyebrow wrapper (components/pri/pri-section.tsx) introduced here for reuse by the remaining PRI deep-dive modules. All 8 real section photos (CloudFront) spot-checked live before use; legacy's purely decorative glitch-scanline overlays dropped. Verified live: 200 OK, real content confirmed in rendered HTML, exactly 1 header/1 footer, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E204" s="14" t="inlineStr">
@@ -5617,7 +5617,7 @@
       <c r="A205" s="4" t="n"/>
       <c r="B205" s="4" t="inlineStr">
         <is>
-          <t>PRI: /iboga-compass</t>
+          <t>PRI: /iboga-ibogaine</t>
         </is>
       </c>
       <c r="C205" s="13" t="inlineStr">
@@ -5627,7 +5627,7 @@
       </c>
       <c r="D205" s="4" t="inlineStr">
         <is>
-          <t>IbogaCompassAssessment, the real interactive 28-question / 7-section compass (outcome/medical/approach/logistics/geography/personal/aftercare), the real drag-or-arrow priority-rank step (top dimension ×2.0, bottom ×0.5), the real facility-scoring engine, and the real results view (matched facilities with real "why this matched" reasoning and real elimination reasons), all ported unchanged and verbatim. lib/content/pri-iboga-compass-engine.ts (real scoring logic — weight deltas, hard filters, substance bonuses, priority-rank application, facility scoring) and lib/content/pri-iboga-facility-data.ts (real facility directory + substance-bonus data) both copied verbatim from legacy rather than hand-transcribed, given this is the actual matching algorithm — correctness matters more here than anywhere else in this migration. Uses this site's own brand-gold/foreground/muted-foreground design tokens rather than the pri-* palette — legacy's own hex here (#8B6914) is an exact match for brand-gold, confirming this one page always used the main site identity, not a PRI-specific one. Real backend gap handled honestly: legacy's lead-capture gate posted a rich structured payload (question-by-question answers, top facility matches, primary goal, budget range) to trpc.assessments.submit (no backend built for this migration) — replaced with a mailto: to Tony carrying the same structured summary, same pattern used throughout this migration; the meaningless "Submitting..." pending state and its e</t>
+          <t>IbogaDeepDive, "The Plant vs The Isolate": real alkaloid-profile comparison, real receptor pharmacology, real head-to-head iboga-vs-ibogaine table, real clinical outcomes (Mash/Noller/Schenberg/Brown &amp; Alper/Cherian/Williams — including the 2024 Stanford Nature Medicine SOF-veteran data and the 2026 19,071-patient safety analysis), real pharma-to-plant alternatives, real supplement protocol, real dimension thresholds, real medicine selector, Tony's real first-hand account of sitting ibogaine at The Mission Within, real hard-stop contraindications, a real 9-facility directory (with the 2 facilities legacy explicitly removed and why), real Nagoya Protocol / extractive-capitalism argument, real 2026 US legal-status rundown, the embedded Iboga Compass v2 documentation section (components/pri/iboga-compass-section.tsx, its own client island for the question-group toggles), and real sources — all ported unchanged and verbatim into lib/content/pri-iboga-module.ts + lib/content/pri-iboga-compass-data.ts (both copied verbatim) + app/iboga-ibogaine/page.tsx. Fully static except the pharma-table expand toggle (components/pri/iboga-pharma-table.tsx) and the compass section's toggles; reused the shared PriSection/PriEyebrow wrapper from the mescaline module. All 5 real hero/section photos (CloudFront) spot-checked live before use. Verified live: 200 OK, real content confirmed in rendered HTML, exactly 1 header/1 footer, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E205" s="14" t="inlineStr">
@@ -5640,7 +5640,7 @@
       <c r="A206" s="4" t="n"/>
       <c r="B206" s="4" t="inlineStr">
         <is>
-          <t>PRI: /pri-calibration</t>
+          <t>PRI: /iboga-compass</t>
         </is>
       </c>
       <c r="C206" s="13" t="inlineStr">
@@ -5650,7 +5650,7 @@
       </c>
       <c r="D206" s="4" t="inlineStr">
         <is>
-          <t>forced-rank calibration study, the real Bradley-Terry pairwise-comparison model (all 15 unique pairs of the 6 PRI dimensions), the real drag-or-arrow full ranking step, real methodology copy (acquiescence-bias explanation, the 4 headline validation stats), and the real Monte Carlo validation metrics (lib/content/pri-efficacy-data.json, copied verbatim from legacy — also feeds /pri-efficacy below), all ported unchanged into components/pri/calibration-assessment.tsx. Real backend gap, handled honestly: legacy's "Contribute to Research?" opt-in phase posted to trpc.priCalibration.submit (no backend built for this migration), and the results view's "Community Data" section read a live trpc.priCalibration.stats aggregate query showing other users' scores — neither has an honest backend-free equivalent (a cross-user aggregate can't be faked locally, and a research opt-in toggle with nothing behind it would be dishonest UI, the same call already made dropping the main PRI results page's inert research-pool checkbox). Both dropped; the flow goes straight from ranking to results. Verified live: 200 OK, real content confirmed in rendered HTML, exactly 1 header/1 footer, typecheck/lint clean.</t>
+          <t>IbogaCompassAssessment, the real interactive 28-question / 7-section compass (outcome/medical/approach/logistics/geography/personal/aftercare), the real drag-or-arrow priority-rank step (top dimension ×2.0, bottom ×0.5), the real facility-scoring engine, and the real results view (matched facilities with real "why this matched" reasoning and real elimination reasons), all ported unchanged and verbatim. lib/content/pri-iboga-compass-engine.ts (real scoring logic — weight deltas, hard filters, substance bonuses, priority-rank application, facility scoring) and lib/content/pri-iboga-facility-data.ts (real facility directory + substance-bonus data) both copied verbatim from legacy rather than hand-transcribed, given this is the actual matching algorithm — correctness matters more here than anywhere else in this migration. Uses this site's own brand-gold/foreground/muted-foreground design tokens rather than the pri-* palette — legacy's own hex here (#8B6914) is an exact match for brand-gold, confirming this one page always used the main site identity, not a PRI-specific one. Real backend gap handled honestly: legacy's lead-capture gate posted a rich structured payload (question-by-question answers, top facility matches, primary goal, budget range) to trpc.assessments.submit (no backend built for this migration) — replaced with a mailto: to Tony carrying the same structured summary, same pattern used throughout this migration; the meaningless "Submitting..." pending state and its e</t>
         </is>
       </c>
       <c r="E206" s="14" t="inlineStr">
@@ -5663,7 +5663,7 @@
       <c r="A207" s="4" t="n"/>
       <c r="B207" s="4" t="inlineStr">
         <is>
-          <t>PRI: /pri-efficacy</t>
+          <t>PRI: /pri-calibration</t>
         </is>
       </c>
       <c r="C207" s="13" t="inlineStr">
@@ -5673,7 +5673,7 @@
       </c>
       <c r="D207" s="4" t="inlineStr">
         <is>
-          <t>psychometric validation dashboard, the real Monte Carlo simulation results (10,000 synthetic respondents), real classification-accuracy comparison, real dimension-priority distribution (the real first-dimension-inflation finding), real test-retest reliability and entropy metrics, and the real methodology writeup, all ported unchanged into app/pri-efficacy/page.tsx, reading the same lib/content/pri-efficacy-data.json also used by /pri-calibration. Real backend gap, handled honestly: legacy's "Live Calibrations" tab read a live trpc.priCalibration.stats query — since /pri-calibration's own submit call was already dropped (no backend, see that page's port note), this tab would permanently render "0 total calibrations, no data yet," a dead feature masquerading as a live one. Dropped entirely rather than ship a perpetually-empty tab; only the real, fully-populated Simulation view ships — which also means this page has no state left at all, so it's a plain Server Component now instead of a client one. Verified live: 200 OK, real content confirmed in rendered HTML, exactly 1 header/1 footer, typecheck/lint clean.</t>
+          <t>forced-rank calibration study, the real Bradley-Terry pairwise-comparison model (all 15 unique pairs of the 6 PRI dimensions), the real drag-or-arrow full ranking step, real methodology copy (acquiescence-bias explanation, the 4 headline validation stats), and the real Monte Carlo validation metrics (lib/content/pri-efficacy-data.json, copied verbatim from legacy — also feeds /pri-efficacy below), all ported unchanged into components/pri/calibration-assessment.tsx. Real backend gap, handled honestly: legacy's "Contribute to Research?" opt-in phase posted to trpc.priCalibration.submit (no backend built for this migration), and the results view's "Community Data" section read a live trpc.priCalibration.stats aggregate query showing other users' scores — neither has an honest backend-free equivalent (a cross-user aggregate can't be faked locally, and a research opt-in toggle with nothing behind it would be dishonest UI, the same call already made dropping the main PRI results page's inert research-pool checkbox). Both dropped; the flow goes straight from ranking to results. Verified live: 200 OK, real content confirmed in rendered HTML, exactly 1 header/1 footer, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E207" s="14" t="inlineStr">
@@ -5686,7 +5686,7 @@
       <c r="A208" s="4" t="n"/>
       <c r="B208" s="4" t="inlineStr">
         <is>
-          <t>PRI: /pri-research Built 2026-10-06 behind the login: admins are the emails in ADMIN_EMAILS; everyone else gets live's "Access Denied"</t>
+          <t>PRI: /pri-efficacy</t>
         </is>
       </c>
       <c r="C208" s="13" t="inlineStr">
@@ -5696,7 +5696,7 @@
       </c>
       <c r="D208" s="4" t="inlineStr">
         <is>
-          <t>Totals, anonymized opt-in table, admin-only CSV export (/pri-research/export). /pri-calibration regained legacy's "Contribute to Research?" step and now saves every calibration anonymously to pri_calibrations (opt-ins flagged). Was: — Deferred, not skipped (access-model question resolved by inspection). Read the real legacy source: this is a genuine admin-only dashboard (useAuth() gated to role === "admin") showing trpc.priCalibration.researchData — the same calibration-submission backend already confirmed absent and intentionally not built for /pri-calibration and /pri-efficacy (see their port notes). No admin-auth system exists anywhere in this Next.js migration yet either. So this isn't just an access-control decision — even fully wired up, the page would have zero real data to show, forever. Not worth building an admin dashboard against a backend this migration has twice already decided not to build. Added to "Explicitly deferred" below alongside the other admin dashboards; revisit only if/when both a real admin-auth system and a real calibration-submission backend exist.</t>
+          <t>psychometric validation dashboard, the real Monte Carlo simulation results (10,000 synthetic respondents), real classification-accuracy comparison, real dimension-priority distribution (the real first-dimension-inflation finding), real test-retest reliability and entropy metrics, and the real methodology writeup, all ported unchanged into app/pri-efficacy/page.tsx, reading the same lib/content/pri-efficacy-data.json also used by /pri-calibration. Real backend gap, handled honestly: legacy's "Live Calibrations" tab read a live trpc.priCalibration.stats query — since /pri-calibration's own submit call was already dropped (no backend, see that page's port note), this tab would permanently render "0 total calibrations, no data yet," a dead feature masquerading as a live one. Dropped entirely rather than ship a perpetually-empty tab; only the real, fully-populated Simulation view ships — which also means this page has no state left at all, so it's a plain Server Component now instead of a client one. Verified live: 200 OK, real content confirmed in rendered HTML, exactly 1 header/1 footer, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E208" s="14" t="inlineStr">
@@ -5709,7 +5709,7 @@
       <c r="A209" s="4" t="n"/>
       <c r="B209" s="4" t="inlineStr">
         <is>
-          <t>PRI: /facilitator-index</t>
+          <t>PRI: /pri-research Built 2026-10-06 behind the login: admins are the emails in ADMIN_EMAILS; everyone else gets live's "Access Denied"</t>
         </is>
       </c>
       <c r="C209" s="13" t="inlineStr">
@@ -5719,7 +5719,7 @@
       </c>
       <c r="D209" s="4" t="inlineStr">
         <is>
-          <t>"The Facilitator Index: Know Who You Go With," the real 15-question quick-intake archetype quiz (real Bradley-Terry-style axis derivation, fully client-computed via deriveArchetype()), the real 108-item, 12-band (plus Band 0) practitioner self-assessment instrument, and the real methodology prose (rationale, code/tier system, data-handling policy, Reciprocity Gate, Corroboration token system), all ported unchanged and verbatim into lib/content/facilitator-index-data.ts (single authoritative content source) + components/facilitator/* + app/facilitator-index/page.tsx. Real content-drift bug found and fixed: legacy shipped two divergent copies of the same "108 items" — the on-page JSX and a separate printFacilitatorQuestions() print/PDF export using an older, different set of item numbers and band groupings (missing the on-page "Twenty-Five Traditions and Protocols" band entirely) — the print export was never updated when the on-page instrument was revised. Used the on-page version (the one actually shown to visitors) as the single source of truth and rebuilt the print export to generate from that same data, so the two can never diverge again. Real fake-data found and dropped: legacy's PeerStats component's own comment admits its numbers ("163 practitioners mapped so far," etc.) are "seeded, realistic-feeling" — fabricated, not real — dropped entirely, same principle as BrewSoul's stale "reads" counts; UsageCounter's hardcoded 160-practitioner fallback (shown forever since no ba</t>
+          <t>Totals, anonymized opt-in table, admin-only CSV export (/pri-research/export). /pri-calibration regained legacy's "Contribute to Research?" step and now saves every calibration anonymously to pri_calibrations (opt-ins flagged). Was: — Deferred, not skipped (access-model question resolved by inspection). Read the real legacy source: this is a genuine admin-only dashboard (useAuth() gated to role === "admin") showing trpc.priCalibration.researchData — the same calibration-submission backend already confirmed absent and intentionally not built for /pri-calibration and /pri-efficacy (see their port notes). No admin-auth system exists anywhere in this Next.js migration yet either. So this isn't just an access-control decision — even fully wired up, the page would have zero real data to show, forever. Not worth building an admin dashboard against a backend this migration has twice already decided not to build. Added to "Explicitly deferred" below alongside the other admin dashboards; revisit only if/when both a real admin-auth system and a real calibration-submission backend exist.</t>
         </is>
       </c>
       <c r="E209" s="14" t="inlineStr">
@@ -5732,63 +5732,63 @@
       <c r="A210" s="4" t="n"/>
       <c r="B210" s="4" t="inlineStr">
         <is>
+          <t>PRI: /facilitator-index</t>
+        </is>
+      </c>
+      <c r="C210" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D210" s="4" t="inlineStr">
+        <is>
+          <t>"The Facilitator Index: Know Who You Go With," the real 15-question quick-intake archetype quiz (real Bradley-Terry-style axis derivation, fully client-computed via deriveArchetype()), the real 108-item, 12-band (plus Band 0) practitioner self-assessment instrument, and the real methodology prose (rationale, code/tier system, data-handling policy, Reciprocity Gate, Corroboration token system), all ported unchanged and verbatim into lib/content/facilitator-index-data.ts (single authoritative content source) + components/facilitator/* + app/facilitator-index/page.tsx. Real content-drift bug found and fixed: legacy shipped two divergent copies of the same "108 items" — the on-page JSX and a separate printFacilitatorQuestions() print/PDF export using an older, different set of item numbers and band groupings (missing the on-page "Twenty-Five Traditions and Protocols" band entirely) — the print export was never updated when the on-page instrument was revised. Used the on-page version (the one actually shown to visitors) as the single source of truth and rebuilt the print export to generate from that same data, so the two can never diverge again. Real fake-data found and dropped: legacy's PeerStats component's own comment admits its numbers ("163 practitioners mapped so far," etc.) are "seeded, realistic-feeling" — fabricated, not real — dropped entirely, same principle as BrewSoul's stale "reads" counts; UsageCounter's hardcoded 160-practitioner fallback (shown forever since no ba</t>
+        </is>
+      </c>
+      <c r="E210" s="14" t="inlineStr">
+        <is>
+          <t>Phase 7 — PRI &amp; Kava Encyclopedias (19 routes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="4" t="n"/>
+      <c r="B211" s="4" t="inlineStr">
+        <is>
           <t>Port shared safety/medicine data modules (safety-data.ts, medicine-images.ts) as typed .ts content in the new codebase</t>
         </is>
       </c>
-      <c r="C210" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D210" s="4" t="inlineStr">
+      <c r="C211" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D211" s="4" t="inlineStr">
         <is>
           <t>done as part of the main PRI page above (lib/content/pri-safety-data.ts, lib/content/pri-medicine-images.ts, both copied verbatim).</t>
         </is>
       </c>
-      <c r="E210" s="14" t="inlineStr">
+      <c r="E211" s="14" t="inlineStr">
         <is>
           <t>Phase 7 — PRI &amp; Kava Encyclopedias (19 routes)</t>
         </is>
       </c>
     </row>
-    <row r="211">
-      <c r="A211" s="10" t="inlineStr">
+    <row r="212">
+      <c r="A212" s="10" t="inlineStr">
         <is>
           <t>Phase 8 — Attention Theft Manifesto (7 routes)</t>
         </is>
       </c>
-      <c r="B211" s="11" t="n"/>
-      <c r="C211" s="11" t="n"/>
-      <c r="D211" s="12" t="n"/>
-    </row>
-    <row r="212">
-      <c r="A212" s="4" t="n"/>
-      <c r="B212" s="4" t="inlineStr">
-        <is>
-          <t>/attention-theft</t>
-        </is>
-      </c>
-      <c r="C212" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D212" s="4" t="inlineStr">
-        <is>
-          <t>consolidated mega-page. Real content ported in full across all 9 sections (hero, The Sacred, The Heresy economics data + full breakdown table + sources, the 10 Weapons, Legal Arsenal w/ filter + letter template, AI Blocker Finder quiz, Report a Spammer, closing vow + related reading) — AttentionTheft.tsx used as the single source, the 5 pre-consolidation sub-pages not resurrected (they never existed in this codebase anyway). Section "glamour" photography is real, live imagery on RampRate's own CloudFront (already whitelisted in next.config.ts as a non-Manus, permanent host — confirmed all 7 URLs 200 before using them), rendered via next/image. Real backend gap found and handled honestly: legacy's Wall of Shame (a live trpc.spam.wallOfShame ranked list) and the Report form's trpc.spam.submit both depended on a spam-tracking backend that this migration explicitly defers (see "Explicitly deferred" list below: "/youve-been-reported, /spamtoast, admin spam tooling") — rather than fake a public database with no real data behind it, the report form now composes a mailto: to Tony (same honest non-fake-success pattern as newsletter-popup.tsx), and the ranked Wall of Shame list isn't reproduced. Two simplifications matching precedent set elsewhere in this migration: legacy's "Fraunces" serif (loaded for this one page only) was dropped for font-heading (Playfair Display, already loaded — same call made on /akbar), and the glitch/VHS/ember-particle/shattered-glass decoration layer was dr</t>
-        </is>
-      </c>
-      <c r="E212" s="14" t="inlineStr">
-        <is>
-          <t>Phase 8 — Attention Theft Manifesto (7 routes)</t>
-        </is>
-      </c>
+      <c r="B212" s="11" t="n"/>
+      <c r="C212" s="11" t="n"/>
+      <c r="D212" s="12" t="n"/>
     </row>
     <row r="213">
       <c r="A213" s="4" t="n"/>
       <c r="B213" s="4" t="inlineStr">
         <is>
-          <t>Legacy anchor redirects</t>
+          <t>/attention-theft</t>
         </is>
       </c>
       <c r="C213" s="13" t="inlineStr">
@@ -5798,7 +5798,7 @@
       </c>
       <c r="D213" s="4" t="inlineStr">
         <is>
-          <t>/attention-theft/economics, /blocker-finder, /legal, /weapons, /report → /attention-theft#&lt;anchor&gt; via next.config.ts redirects(). Verified live: all return real 308s to the correct anchor.</t>
+          <t>consolidated mega-page. Real content ported in full across all 9 sections (hero, The Sacred, The Heresy economics data + full breakdown table + sources, the 10 Weapons, Legal Arsenal w/ filter + letter template, AI Blocker Finder quiz, Report a Spammer, closing vow + related reading) — AttentionTheft.tsx used as the single source, the 5 pre-consolidation sub-pages not resurrected (they never existed in this codebase anyway). Section "glamour" photography is real, live imagery on RampRate's own CloudFront (already whitelisted in next.config.ts as a non-Manus, permanent host — confirmed all 7 URLs 200 before using them), rendered via next/image. Real backend gap found and handled honestly: legacy's Wall of Shame (a live trpc.spam.wallOfShame ranked list) and the Report form's trpc.spam.submit both depended on a spam-tracking backend that this migration explicitly defers (see "Explicitly deferred" list below: "/youve-been-reported, /spamtoast, admin spam tooling") — rather than fake a public database with no real data behind it, the report form now composes a mailto: to Tony (same honest non-fake-success pattern as newsletter-popup.tsx), and the ranked Wall of Shame list isn't reproduced. Two simplifications matching precedent set elsewhere in this migration: legacy's "Fraunces" serif (loaded for this one page only) was dropped for font-heading (Playfair Display, already loaded — same call made on /akbar), and the glitch/VHS/ember-particle/shattered-glass decoration layer was dr</t>
         </is>
       </c>
       <c r="E213" s="14" t="inlineStr">
@@ -5811,63 +5811,63 @@
       <c r="A214" s="4" t="n"/>
       <c r="B214" s="4" t="inlineStr">
         <is>
+          <t>Legacy anchor redirects</t>
+        </is>
+      </c>
+      <c r="C214" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D214" s="4" t="inlineStr">
+        <is>
+          <t>/attention-theft/economics, /blocker-finder, /legal, /weapons, /report → /attention-theft#&lt;anchor&gt; via next.config.ts redirects(). Verified live: all return real 308s to the correct anchor.</t>
+        </is>
+      </c>
+      <c r="E214" s="14" t="inlineStr">
+        <is>
+          <t>Phase 8 — Attention Theft Manifesto (7 routes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="4" t="n"/>
+      <c r="B215" s="4" t="inlineStr">
+        <is>
           <t>Port ManifestoLayout scroll-tracking wrapper behavior</t>
         </is>
       </c>
-      <c r="C214" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D214" s="4" t="inlineStr">
+      <c r="C215" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D215" s="4" t="inlineStr">
         <is>
           <t>components/manifesto/manifesto-nav.tsx tracks which section is in view on scroll and highlights the matching nav pill (desktop + mobile), real behavior kept per this line item rather than simplified away.</t>
         </is>
       </c>
-      <c r="E214" s="14" t="inlineStr">
+      <c r="E215" s="14" t="inlineStr">
         <is>
           <t>Phase 8 — Attention Theft Manifesto (7 routes)</t>
         </is>
       </c>
     </row>
-    <row r="215">
-      <c r="A215" s="10" t="inlineStr">
+    <row r="216">
+      <c r="A216" s="10" t="inlineStr">
         <is>
           <t>Phase 9 — Assessments (33 routes)</t>
         </is>
       </c>
-      <c r="B215" s="11" t="n"/>
-      <c r="C215" s="11" t="n"/>
-      <c r="D215" s="12" t="n"/>
-    </row>
-    <row r="216">
-      <c r="A216" s="4" t="n"/>
-      <c r="B216" s="4" t="inlineStr">
-        <is>
-          <t>HumanOS section</t>
-        </is>
-      </c>
-      <c r="C216" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D216" s="4" t="inlineStr">
-        <is>
-          <t>/humanos, /humanos/philosophy, /humanos/ecosystem, /humanos/resources, /humanos/connect, /humanos/path-to-here, ported from _legacy-manus-app/client/src/pages/HumanOS.tsx + humanos/*.tsx. The top-level HumanOS.tsx (an iframe embed of an external manus.space site) turned out to be dead code, never wired into legacy's router — the real, routed implementation is HumanosHome/HumanosPhilosophy/HumanosEcosystem/HumanosResources/HumanosConnect/HumanosPathToHere behind HumanosLayout, which is what got ported, with its own nested layout.tsx (route now added to site-chrome.tsx's SUPPRESSED_PREFIXES so the main SiteHeader/SiteFooter don't double up around HumanOS's own nav/footer). Real content in full: the Maximizer-vs-Satisficer framework and "Boiling the Human"/"Maximizer Trap"/"Conscious Satisficer" philosophy sections, the full ecosystem roster (1 mentor, 8 advisors, 3 partners, 29 clients), all 4 transformation playbooks + 3 daily-practice protocols + 8-book reading list, all 4 connect channels, and the 6-entry "Path to Here" timeline (2010 H+ Summit through 2025). Real bugs fixed: every "Take the Diagnostic" CTA site-wide pointed at /assessment, an 8-question Maximizer/Satisficer quiz that was never actually built anywhere (legacy's real /assessment and /assessments routes are two different, unrelated quiz sets) — redirected to /humanos/philosophy, which delivers the actual promised content; Connect's "Read the Living Declaration" pointed at /manifesto, a dead redirect stub in le</t>
-        </is>
-      </c>
-      <c r="E216" s="14" t="inlineStr">
-        <is>
-          <t>Phase 9 — Assessments (33 routes)</t>
-        </is>
-      </c>
+      <c r="B216" s="11" t="n"/>
+      <c r="C216" s="11" t="n"/>
+      <c r="D216" s="12" t="n"/>
     </row>
     <row r="217">
       <c r="A217" s="4" t="n"/>
       <c r="B217" s="4" t="inlineStr">
         <is>
-          <t>/find-your-me (+ /find-my-me, /discover)</t>
+          <t>HumanOS section</t>
         </is>
       </c>
       <c r="C217" s="13" t="inlineStr">
@@ -5877,7 +5877,7 @@
       </c>
       <c r="D217" s="4" t="inlineStr">
         <is>
-          <t>"Find My — To Find Your We," the ecosystem hub assessment and by far the largest page in Phase 9. Real 5 NLP-driven questions, 6 dimensions (relationships/purpose/body/truth/tribe/consciousness), and 6 real archetypes (each with a real description, real blog article links, real satellite-site links, real "go deeper" forward-references, and a real share text) ported unchanged and verbatim into a new lib/content/find-your-me.ts data module (kept separate from the component given the file's exceptional size, same pattern as brewsoul-directory.ts). All 17 unique blog article slugs referenced across the 6 archetypes were individually verified live (200 OK) against this migration's real Sanity blog before porting — zero dead article links. Real accuracy fix: legacy's "Full Ecosystem Directory" (26 items across 5 categories, with a real LIVE/COMING pill UI already built for exactly this purpose) marked everything "live," including several routes that don't exist anywhere in this migration yet (/find-my, /the-mirror, /assessments/dharma-finder, /assessments/consciousness-scale, /assessments/grant-study, /flow-circuit) — corrected each item's status to this app's actual current build state rather than shipping false LIVE labels on what would be 404s. Real completeness fix: added Find Your Peptide and Find Your Sexuality to the directory (Body &amp; Temple and Love &amp; Belonging) — both are real, fully-built assessments elsewhere in this migration that didn't exist yet when legacy was writte</t>
+          <t>/humanos, /humanos/philosophy, /humanos/ecosystem, /humanos/resources, /humanos/connect, /humanos/path-to-here, ported from _legacy-manus-app/client/src/pages/HumanOS.tsx + humanos/*.tsx. The top-level HumanOS.tsx (an iframe embed of an external manus.space site) turned out to be dead code, never wired into legacy's router — the real, routed implementation is HumanosHome/HumanosPhilosophy/HumanosEcosystem/HumanosResources/HumanosConnect/HumanosPathToHere behind HumanosLayout, which is what got ported, with its own nested layout.tsx (route now added to site-chrome.tsx's SUPPRESSED_PREFIXES so the main SiteHeader/SiteFooter don't double up around HumanOS's own nav/footer). Real content in full: the Maximizer-vs-Satisficer framework and "Boiling the Human"/"Maximizer Trap"/"Conscious Satisficer" philosophy sections, the full ecosystem roster (1 mentor, 8 advisors, 3 partners, 29 clients), all 4 transformation playbooks + 3 daily-practice protocols + 8-book reading list, all 4 connect channels, and the 6-entry "Path to Here" timeline (2010 H+ Summit through 2025). Real bugs fixed: every "Take the Diagnostic" CTA site-wide pointed at /assessment, an 8-question Maximizer/Satisficer quiz that was never actually built anywhere (legacy's real /assessment and /assessments routes are two different, unrelated quiz sets) — redirected to /humanos/philosophy, which delivers the actual promised content; Connect's "Read the Living Declaration" pointed at /manifesto, a dead redirect stub in le</t>
         </is>
       </c>
       <c r="E217" s="14" t="inlineStr">
@@ -5890,7 +5890,7 @@
       <c r="A218" s="4" t="n"/>
       <c r="B218" s="4" t="inlineStr">
         <is>
-          <t>/find-your-therapy (+ /find-my-therapy)</t>
+          <t>/find-your-me (+ /find-my-me, /discover)</t>
         </is>
       </c>
       <c r="C218" s="13" t="inlineStr">
@@ -5900,7 +5900,7 @@
       </c>
       <c r="D218" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Real 25 questions across 6 dimensions (Cognitive/Somatic/Relational/Depth-Unconscious/Altered States/Integrative), 6 real therapeutic modalities (each with a real description, "how it works," best-for/not-ideal-for lists, real named pioneers, and real book/directory resources), and the real archetype-matching logic (highest-scoring dimension wins) ported unchanged and verbatim. Three real stale-count bugs found and fixed: legacy's own file-header comment claimed "10 questions," its AssessmentIntro stats prop claimed 20 — neither matches the real 25-item array (the scoring code's own maxPossible = 30 // rough max per dimension with 25 questions comment confirms 25 is correct) — replaced both with live QUESTIONS.length. Real dead-link bug fixed: legacy's "Journey Continues" grid linked "Find Your Spirit"/"Find Your Religion" to external findmyassess-9eekxcob.manus.space stub URLs (dead Manus domain) despite this migration already having real, fully-built internal pages at /find-your-spirit and /find-your-religion — repointed to the real internal routes, and corrected Religion's stale "15 Questions" badge to the real 20. Real accent-color inconsistency fixed: legacy passed accentColor="#7B1FA2" only to the landing screen, then hardcoded brand-gold everywhere on the results screen instead — threaded one ACCENT constant through intro/radar/result-actions consistently, matching every other assessment in this migration. The "Also Worth Exploring" related-modality cards were dropped </t>
+          <t>"Find My — To Find Your We," the ecosystem hub assessment and by far the largest page in Phase 9. Real 5 NLP-driven questions, 6 dimensions (relationships/purpose/body/truth/tribe/consciousness), and 6 real archetypes (each with a real description, real blog article links, real satellite-site links, real "go deeper" forward-references, and a real share text) ported unchanged and verbatim into a new lib/content/find-your-me.ts data module (kept separate from the component given the file's exceptional size, same pattern as brewsoul-directory.ts). All 17 unique blog article slugs referenced across the 6 archetypes were individually verified live (200 OK) against this migration's real Sanity blog before porting — zero dead article links. Real accuracy fix: legacy's "Full Ecosystem Directory" (26 items across 5 categories, with a real LIVE/COMING pill UI already built for exactly this purpose) marked everything "live," including several routes that don't exist anywhere in this migration yet (/find-my, /the-mirror, /assessments/dharma-finder, /assessments/consciousness-scale, /assessments/grant-study, /flow-circuit) — corrected each item's status to this app's actual current build state rather than shipping false LIVE labels on what would be 404s. Real completeness fix: added Find Your Peptide and Find Your Sexuality to the directory (Body &amp; Temple and Love &amp; Belonging) — both are real, fully-built assessments elsewhere in this migration that didn't exist yet when legacy was writte</t>
         </is>
       </c>
       <c r="E218" s="14" t="inlineStr">
@@ -5913,7 +5913,7 @@
       <c r="A219" s="4" t="n"/>
       <c r="B219" s="4" t="inlineStr">
         <is>
-          <t>/find-your-sake</t>
+          <t>/find-your-therapy (+ /find-my-therapy)</t>
         </is>
       </c>
       <c r="C219" s="13" t="inlineStr">
@@ -5923,7 +5923,7 @@
       </c>
       <c r="D219" s="4" t="inlineStr">
         <is>
-          <t>Real 20 questions across 5 dimensions (Palate/Ritual/Terroir/Philosophy/Season) and the real 5 sake profiles (each with real Japanese name, tasting notes, food pairings, serving temperature, named producers with region/note, and further-reading resources) ported unchanged and verbatim. Legacy's own AssessmentIntro stats prop claimed "15 questions, 6 dimensions" — didn't match the real 20/5 implementation — replaced with live QUESTIONS.length/DIMENSIONS.length counts, same fix pattern already applied on /find-your-attachment-style and /find-your-sexuality. Two real bugs found and fixed: (1) legacy's "Journey Continues" list read "Find Myzcal" — a literal typo for "Find Your Mezcal" — corrected. (2) legacy's JSX rendered &lt;WhatsNext /&gt; (a full page section) nested inside the small "Retake the Tasting" &lt;button&gt; element — moved to a proper top-level section, same class of nested-interactive-content bug already fixed on /find-your-religion. The dark GlassPanel treatment (near-black translucent cards with light cream text, sitting on the page's own light parchment ThemedBackground) was kept as a real, intentional design choice rather than "fixed" to this migration's usual light-card convention — unlike the light-text-directly-on-light-background contrast bugs found on Style/Sexuality/Peptide/Religion, the text here sits inside its own correctly-contrasted dark card. SacredGeometryBg's canvas-based floating rice-grain particles dropped (same decoration-not-worth-the-JS-cost call made</t>
+          <t xml:space="preserve">Real 25 questions across 6 dimensions (Cognitive/Somatic/Relational/Depth-Unconscious/Altered States/Integrative), 6 real therapeutic modalities (each with a real description, "how it works," best-for/not-ideal-for lists, real named pioneers, and real book/directory resources), and the real archetype-matching logic (highest-scoring dimension wins) ported unchanged and verbatim. Three real stale-count bugs found and fixed: legacy's own file-header comment claimed "10 questions," its AssessmentIntro stats prop claimed 20 — neither matches the real 25-item array (the scoring code's own maxPossible = 30 // rough max per dimension with 25 questions comment confirms 25 is correct) — replaced both with live QUESTIONS.length. Real dead-link bug fixed: legacy's "Journey Continues" grid linked "Find Your Spirit"/"Find Your Religion" to external findmyassess-9eekxcob.manus.space stub URLs (dead Manus domain) despite this migration already having real, fully-built internal pages at /find-your-spirit and /find-your-religion — repointed to the real internal routes, and corrected Religion's stale "15 Questions" badge to the real 20. Real accent-color inconsistency fixed: legacy passed accentColor="#7B1FA2" only to the landing screen, then hardcoded brand-gold everywhere on the results screen instead — threaded one ACCENT constant through intro/radar/result-actions consistently, matching every other assessment in this migration. The "Also Worth Exploring" related-modality cards were dropped </t>
         </is>
       </c>
       <c r="E219" s="14" t="inlineStr">
@@ -5936,7 +5936,7 @@
       <c r="A220" s="4" t="n"/>
       <c r="B220" s="4" t="inlineStr">
         <is>
-          <t>/find-your-spirit (+ /find-my-spirit), along with a shared PDF-export component the rest of Phase 9 can reuse</t>
+          <t>/find-your-sake</t>
         </is>
       </c>
       <c r="C220" s="13" t="inlineStr">
@@ -5946,7 +5946,7 @@
       </c>
       <c r="D220" s="4" t="inlineStr">
         <is>
-          <t>Real 35 questions, 10 dimensions, and the 6 real spiritual traditions (each with real description/practices/key texts/figures/modern expressions/growth edge) ported unchanged and verbatim — legacy's own file-header comment claimed "12 archetypes," but only 6 TRADITIONS actually exist in the code; ported the real 6, not the stale doc comment. The real weighted tradition-matching logic (top 3 dimensions per tradition, weighted 3/2/1) is unchanged. Ported components/assessments/result-actions.tsx from legacy's AssessmentResultActions — kept only the real, backend-free "Download PDF" action (browser print); the "Send to Tony"/"Keep Private" buttons posted to an unbuilt trpc.assessments.submit and weren't reproduced, same honest-degradation pattern used throughout this migration. Verified live: 200 OK, redirect confirmed 308, typecheck/lint clean.</t>
+          <t>Real 20 questions across 5 dimensions (Palate/Ritual/Terroir/Philosophy/Season) and the real 5 sake profiles (each with real Japanese name, tasting notes, food pairings, serving temperature, named producers with region/note, and further-reading resources) ported unchanged and verbatim. Legacy's own AssessmentIntro stats prop claimed "15 questions, 6 dimensions" — didn't match the real 20/5 implementation — replaced with live QUESTIONS.length/DIMENSIONS.length counts, same fix pattern already applied on /find-your-attachment-style and /find-your-sexuality. Two real bugs found and fixed: (1) legacy's "Journey Continues" list read "Find Myzcal" — a literal typo for "Find Your Mezcal" — corrected. (2) legacy's JSX rendered &lt;WhatsNext /&gt; (a full page section) nested inside the small "Retake the Tasting" &lt;button&gt; element — moved to a proper top-level section, same class of nested-interactive-content bug already fixed on /find-your-religion. The dark GlassPanel treatment (near-black translucent cards with light cream text, sitting on the page's own light parchment ThemedBackground) was kept as a real, intentional design choice rather than "fixed" to this migration's usual light-card convention — unlike the light-text-directly-on-light-background contrast bugs found on Style/Sexuality/Peptide/Religion, the text here sits inside its own correctly-contrasted dark card. SacredGeometryBg's canvas-based floating rice-grain particles dropped (same decoration-not-worth-the-JS-cost call made</t>
         </is>
       </c>
       <c r="E220" s="14" t="inlineStr">
@@ -5959,7 +5959,7 @@
       <c r="A221" s="4" t="n"/>
       <c r="B221" s="4" t="inlineStr">
         <is>
-          <t>/find-your-religion</t>
+          <t>/find-your-spirit (+ /find-my-spirit), along with a shared PDF-export component the rest of Phase 9 can reuse</t>
         </is>
       </c>
       <c r="C221" s="13" t="inlineStr">
@@ -5969,7 +5969,7 @@
       </c>
       <c r="D221" s="4" t="inlineStr">
         <is>
-          <t>Real 20 questions across 8 dimensions, 8 real spiritual/philosophical archetypes (each with real description/practices/key texts/figures/resonant traditions/growth-edge tensions), and the real scoring/matching logic ported unchanged and verbatim. Real bug found and fixed: legacy's own JSX rendered &lt;AssessmentResultActions&gt; nested inside the "Retake Assessment" &lt;button&gt; element — a button inside a button, invalid HTML — fixed by rendering it as a sibling instead, same fix pattern already applied on /find-your-spirit. Verified live: 200 OK, typecheck/lint clean.</t>
+          <t>Real 35 questions, 10 dimensions, and the 6 real spiritual traditions (each with real description/practices/key texts/figures/modern expressions/growth edge) ported unchanged and verbatim — legacy's own file-header comment claimed "12 archetypes," but only 6 TRADITIONS actually exist in the code; ported the real 6, not the stale doc comment. The real weighted tradition-matching logic (top 3 dimensions per tradition, weighted 3/2/1) is unchanged. Ported components/assessments/result-actions.tsx from legacy's AssessmentResultActions — kept only the real, backend-free "Download PDF" action (browser print); the "Send to Tony"/"Keep Private" buttons posted to an unbuilt trpc.assessments.submit and weren't reproduced, same honest-degradation pattern used throughout this migration. Verified live: 200 OK, redirect confirmed 308, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E221" s="14" t="inlineStr">
@@ -5982,7 +5982,7 @@
       <c r="A222" s="4" t="n"/>
       <c r="B222" s="4" t="inlineStr">
         <is>
-          <t>/find-your-diet (+ /find-my-diet)</t>
+          <t>/find-your-religion</t>
         </is>
       </c>
       <c r="C222" s="13" t="inlineStr">
@@ -5992,7 +5992,7 @@
       </c>
       <c r="D222" s="4" t="inlineStr">
         <is>
-          <t>Real 15 questions, 6 real archetypes (with descriptions), and the real nearest-neighbor archetype-matching logic ported unchanged. Legacy's dead JourneyTracker import wired in for real (see journey-tracker.tsx). /find-my-diet → /find-your-diet redirect added. Verified live: 200 OK, full quiz flow, redirect confirmed 308, typecheck/lint clean.</t>
+          <t>Real 20 questions across 8 dimensions, 8 real spiritual/philosophical archetypes (each with real description/practices/key texts/figures/resonant traditions/growth-edge tensions), and the real scoring/matching logic ported unchanged and verbatim. Real bug found and fixed: legacy's own JSX rendered &lt;AssessmentResultActions&gt; nested inside the "Retake Assessment" &lt;button&gt; element — a button inside a button, invalid HTML — fixed by rendering it as a sibling instead, same fix pattern already applied on /find-your-spirit. Verified live: 200 OK, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E222" s="14" t="inlineStr">
@@ -6005,7 +6005,7 @@
       <c r="A223" s="4" t="n"/>
       <c r="B223" s="4" t="inlineStr">
         <is>
-          <t>/find-your-movement (+ /find-my-movement), along with the shared assessment foundation the rest of Phase 9 depends on</t>
+          <t>/find-your-diet (+ /find-my-diet)</t>
         </is>
       </c>
       <c r="C223" s="13" t="inlineStr">
@@ -6015,7 +6015,7 @@
       </c>
       <c r="D223" s="4" t="inlineStr">
         <is>
-          <t>Ported components/assessments/{themed-background,assessment-intro,email-gate,whats-next}.tsx from legacy's ThemedBackground/AssessmentIntro/EmailGate/WhatsNext — real content/behavior unchanged, with 2 real fixes along the way: (1) EmailGate now posts to the real /api/subscribe Route Handler (built earlier this migration) using the exact find-your-&lt;slug&gt; source keys already defined in lib/content/kit-source-tags.ts's KIT_TAG_MAP — legacy's own assessment-gate:&lt;slug&gt; prefix didn't match any tag in that map, so this is a genuine improvement, not just a port. (2) ThemedBackground's per-theme decorative particle field + SVG sacred-geometry overlay + 2 extra radial-glow layers dropped (same "not worth the cost" call made repeatedly elsewhere) — the real per-theme base gradient (16 themes) is kept, precomposed as one literal Tailwind class per theme rather than assembled from fragments. find-your-movement-quiz.tsx ports all 15 real questions and the real 6-dimension (Strength/Flexibility/Endurance/Mindfulness/Community/Adventure) scoring unchanged; the legacy JourneyTracker/useJourneyProgress import in the source file was dead code (imported, never rendered) and not ported. /find-my-movement → /find-your-movement redirect added (next.config.ts), same duplicate-route pattern as /find-my-tribe. Verified live: 200 OK, full quiz flow renders, redirect confirmed 308, typecheck/lint clean.</t>
+          <t>Real 15 questions, 6 real archetypes (with descriptions), and the real nearest-neighbor archetype-matching logic ported unchanged. Legacy's dead JourneyTracker import wired in for real (see journey-tracker.tsx). /find-my-diet → /find-your-diet redirect added. Verified live: 200 OK, full quiz flow, redirect confirmed 308, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E223" s="14" t="inlineStr">
@@ -6028,7 +6028,7 @@
       <c r="A224" s="4" t="n"/>
       <c r="B224" s="4" t="inlineStr">
         <is>
-          <t>/find-your-sleep (+ /find-my-sleep)</t>
+          <t>/find-your-movement (+ /find-my-movement), along with the shared assessment foundation the rest of Phase 9 depends on</t>
         </is>
       </c>
       <c r="C224" s="13" t="inlineStr">
@@ -6038,7 +6038,7 @@
       </c>
       <c r="D224" s="4" t="inlineStr">
         <is>
-          <t>Real 15 questions, 6 real archetypes, and the real cascading archetype-match logic ported unchanged, including legacy's own real behavioral quirk of rendering JourneyTracker on every phase (not just results). One real duplicate-destination "Journey Continues" link pair dropped (see file's own port note), the one real distinct link (Find Your Diet) kept. /find-my-sleep → /find-your-sleep redirect added. Verified live: 200 OK, redirect confirmed 308, typecheck/lint clean.</t>
+          <t>Ported components/assessments/{themed-background,assessment-intro,email-gate,whats-next}.tsx from legacy's ThemedBackground/AssessmentIntro/EmailGate/WhatsNext — real content/behavior unchanged, with 2 real fixes along the way: (1) EmailGate now posts to the real /api/subscribe Route Handler (built earlier this migration) using the exact find-your-&lt;slug&gt; source keys already defined in lib/content/kit-source-tags.ts's KIT_TAG_MAP — legacy's own assessment-gate:&lt;slug&gt; prefix didn't match any tag in that map, so this is a genuine improvement, not just a port. (2) ThemedBackground's per-theme decorative particle field + SVG sacred-geometry overlay + 2 extra radial-glow layers dropped (same "not worth the cost" call made repeatedly elsewhere) — the real per-theme base gradient (16 themes) is kept, precomposed as one literal Tailwind class per theme rather than assembled from fragments. find-your-movement-quiz.tsx ports all 15 real questions and the real 6-dimension (Strength/Flexibility/Endurance/Mindfulness/Community/Adventure) scoring unchanged; the legacy JourneyTracker/useJourneyProgress import in the source file was dead code (imported, never rendered) and not ported. /find-my-movement → /find-your-movement redirect added (next.config.ts), same duplicate-route pattern as /find-my-tribe. Verified live: 200 OK, full quiz flow renders, redirect confirmed 308, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E224" s="14" t="inlineStr">
@@ -6051,7 +6051,7 @@
       <c r="A225" s="4" t="n"/>
       <c r="B225" s="4" t="inlineStr">
         <is>
-          <t>/find-your-coffee (+ /find-my-coffee)</t>
+          <t>/find-your-sleep (+ /find-my-sleep)</t>
         </is>
       </c>
       <c r="C225" s="13" t="inlineStr">
@@ -6061,7 +6061,7 @@
       </c>
       <c r="D225" s="4" t="inlineStr">
         <is>
-          <t>Real 15 questions, 6 dimensions (Roast Preference/Origin Curiosity/Brewing Ritual/Social Context/Caffeine Sensitivity/Flavor Complexity), 6 real archetypes (each with a real description and 5 real named coffee recommendations — roaster, origin, roast level, tasting notes, real "why" rationale), and the real archetype-matching logic (sum of each archetype's 2 primary dimensions, highest wins) ported unchanged and verbatim. This legacy page predates the shared ThemedBackground/AssessmentIntro component system the rest of Phase 9 is built on — it hand-rolled its own hero-image page shell — so it needed more normalization than most: its hero image (/api/img/coffee-orig_a935f111.jpg) was a dead Manus asset, dropped for the standard ThemedBackground light theme (added a new "coffee" warm-cream entry) instead of reproducing a broken background; the canvas bean-particle field, floating steam-wisp divs, and SVG sacred-geometry overlay all dropped (same decoration-not-worth-the-JS-cost call made repeatedly elsewhere). Real bug found and fixed: legacy read window.innerWidth directly during render (twice — to pick grid columns and flex direction), unsafe during SSR and a real hydration-mismatch source — replaced with responsive Tailwind classes. EmailGate's prop was legacy's assessmentName; ported using this repo's real assessmentSlug="coffee" to match find-your-coffee in KIT_TAG_MAP. Legacy imported useJourneyProgress for markComplete but never rendered a visible JourneyTracker, and nev</t>
+          <t>Real 15 questions, 6 real archetypes, and the real cascading archetype-match logic ported unchanged, including legacy's own real behavioral quirk of rendering JourneyTracker on every phase (not just results). One real duplicate-destination "Journey Continues" link pair dropped (see file's own port note), the one real distinct link (Find Your Diet) kept. /find-my-sleep → /find-your-sleep redirect added. Verified live: 200 OK, redirect confirmed 308, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E225" s="14" t="inlineStr">
@@ -6074,7 +6074,7 @@
       <c r="A226" s="4" t="n"/>
       <c r="B226" s="4" t="inlineStr">
         <is>
-          <t>/find-your-kitchen. Real 15 questions (all rendered on one page at once</t>
+          <t>/find-your-coffee (+ /find-my-coffee)</t>
         </is>
       </c>
       <c r="C226" s="13" t="inlineStr">
@@ -6084,7 +6084,7 @@
       </c>
       <c r="D226" s="4" t="inlineStr">
         <is>
-          <t>a genuinely different, legacy-intentional UX from the other paginated quizzes, kept as-is) and the real dual-tracking scoring (answer score keys split into archetype tallies vs. 6 separate radar-chart dimensions) ported unchanged, including the 3 real "Journey Continues" links (one to already-built /find-your-diet, one forward-reference to /find-your-style). Verified live: 200 OK, typecheck/lint clean.</t>
+          <t>Real 15 questions, 6 dimensions (Roast Preference/Origin Curiosity/Brewing Ritual/Social Context/Caffeine Sensitivity/Flavor Complexity), 6 real archetypes (each with a real description and 5 real named coffee recommendations — roaster, origin, roast level, tasting notes, real "why" rationale), and the real archetype-matching logic (sum of each archetype's 2 primary dimensions, highest wins) ported unchanged and verbatim. This legacy page predates the shared ThemedBackground/AssessmentIntro component system the rest of Phase 9 is built on — it hand-rolled its own hero-image page shell — so it needed more normalization than most: its hero image (/api/img/coffee-orig_a935f111.jpg) was a dead Manus asset, dropped for the standard ThemedBackground light theme (added a new "coffee" warm-cream entry) instead of reproducing a broken background; the canvas bean-particle field, floating steam-wisp divs, and SVG sacred-geometry overlay all dropped (same decoration-not-worth-the-JS-cost call made repeatedly elsewhere). Real bug found and fixed: legacy read window.innerWidth directly during render (twice — to pick grid columns and flex direction), unsafe during SSR and a real hydration-mismatch source — replaced with responsive Tailwind classes. EmailGate's prop was legacy's assessmentName; ported using this repo's real assessmentSlug="coffee" to match find-your-coffee in KIT_TAG_MAP. Legacy imported useJourneyProgress for markComplete but never rendered a visible JourneyTracker, and nev</t>
         </is>
       </c>
       <c r="E226" s="14" t="inlineStr">
@@ -6097,7 +6097,7 @@
       <c r="A227" s="4" t="n"/>
       <c r="B227" s="4" t="inlineStr">
         <is>
-          <t>/find-your-style. Real 15 questions, 6 real archetypes, and the real (if crude</t>
+          <t>/find-your-kitchen. Real 15 questions (all rendered on one page at once</t>
         </is>
       </c>
       <c r="C227" s="13" t="inlineStr">
@@ -6107,7 +6107,7 @@
       </c>
       <c r="D227" s="4" t="inlineStr">
         <is>
-          <t>legacy's own comment admits "Simple mapping for demonstration") threshold-based archetype match ported unchanged. Two real inconsistencies found and normalized: legacy's own inline styles used near-illegible light text on ThemedBackground's actual light pastel "style" theme (inconsistent with every other assessment in this migration); and legacy rendered &lt;JourneyTracker /&gt; defaulting to variant="dark" on a light results screen instead of the variant="light" every other assessment passes. Verified live: 200 OK, typecheck/lint clean.</t>
+          <t>a genuinely different, legacy-intentional UX from the other paginated quizzes, kept as-is) and the real dual-tracking scoring (answer score keys split into archetype tallies vs. 6 separate radar-chart dimensions) ported unchanged, including the 3 real "Journey Continues" links (one to already-built /find-your-diet, one forward-reference to /find-your-style). Verified live: 200 OK, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E227" s="14" t="inlineStr">
@@ -6120,7 +6120,7 @@
       <c r="A228" s="4" t="n"/>
       <c r="B228" s="4" t="inlineStr">
         <is>
-          <t>/find-your-attachment-style (+ /find-my-attachment-style, /find-my-we)</t>
+          <t>/find-your-style. Real 15 questions, 6 real archetypes, and the real (if crude</t>
         </is>
       </c>
       <c r="C228" s="13" t="inlineStr">
@@ -6130,7 +6130,7 @@
       </c>
       <c r="D228" s="4" t="inlineStr">
         <is>
-          <t>Real 18 questions (legacy's own AssessmentIntro stats prop under-reported this as "15" — used the live QUESTIONS.length instead of repeating the stale number, same live-count discipline used elsewhere in this migration), the 4 real archetypes, and the real scoring/selection logic all ported unchanged, including the real closing note on attachment theory. Both alt-path redirects added. Verified live: 200 OK, both redirects confirmed 308, typecheck/lint clean.</t>
+          <t>legacy's own comment admits "Simple mapping for demonstration") threshold-based archetype match ported unchanged. Two real inconsistencies found and normalized: legacy's own inline styles used near-illegible light text on ThemedBackground's actual light pastel "style" theme (inconsistent with every other assessment in this migration); and legacy rendered &lt;JourneyTracker /&gt; defaulting to variant="dark" on a light results screen instead of the variant="light" every other assessment passes. Verified live: 200 OK, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E228" s="14" t="inlineStr">
@@ -6143,7 +6143,7 @@
       <c r="A229" s="4" t="n"/>
       <c r="B229" s="4" t="inlineStr">
         <is>
-          <t>/find-your-love-language</t>
+          <t>/find-your-attachment-style (+ /find-my-attachment-style, /find-my-we)</t>
         </is>
       </c>
       <c r="C229" s="13" t="inlineStr">
@@ -6153,7 +6153,7 @@
       </c>
       <c r="D229" s="4" t="inlineStr">
         <is>
-          <t>Real 15 questions (incl. the negative-score "disconnect" question), 5 real archetypes with descriptions/tips, and Dr. Gary Chapman's real attribution note all ported unchanged. Verified live: 200 OK, full quiz flow, typecheck/lint clean.</t>
+          <t>Real 18 questions (legacy's own AssessmentIntro stats prop under-reported this as "15" — used the live QUESTIONS.length instead of repeating the stale number, same live-count discipline used elsewhere in this migration), the 4 real archetypes, and the real scoring/selection logic all ported unchanged, including the real closing note on attachment theory. Both alt-path redirects added. Verified live: 200 OK, both redirects confirmed 308, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E229" s="14" t="inlineStr">
@@ -6166,7 +6166,7 @@
       <c r="A230" s="4" t="n"/>
       <c r="B230" s="4" t="inlineStr">
         <is>
-          <t>/find-your-peptide (+ /find-my-peptide)</t>
+          <t>/find-your-love-language</t>
         </is>
       </c>
       <c r="C230" s="13" t="inlineStr">
@@ -6176,7 +6176,7 @@
       </c>
       <c r="D230" s="4" t="inlineStr">
         <is>
-          <t>"The Peptide Clarity Index™." A real, evidence-cited 10-question assessment across 7 clinical axes, mapping to 16 real peptide archetype profiles — every question (with its real PubMed/journal citation), every profile's real primary/secondary peptides with mechanisms and evidence, suggested lab work, red flags, and stacking notes ported unchanged and verbatim (clinical-adjacent content, not paraphrased). The real Peptide Readiness Score, contraindication-flag screening, share buttons (Twitter/LinkedIn/email/copy — real, backend-free), and the real medical disclaimer are all preserved. Real hero image (CloudFront, confirmed live) kept via next/image. Reused the simplified AssessmentResultActions (PDF-only) built for /find-your-spirit. Same light-text-on-light-background contrast bug already caught elsewhere was fixed here too. Verified live: 200 OK, redirect confirmed 308, typecheck/lint clean.</t>
+          <t>Real 15 questions (incl. the negative-score "disconnect" question), 5 real archetypes with descriptions/tips, and Dr. Gary Chapman's real attribution note all ported unchanged. Verified live: 200 OK, full quiz flow, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E230" s="14" t="inlineStr">
@@ -6189,7 +6189,7 @@
       <c r="A231" s="4" t="n"/>
       <c r="B231" s="4" t="inlineStr">
         <is>
-          <t>/find-your-sexuality (+ /find-my-sexuality)</t>
+          <t>/find-your-peptide (+ /find-my-peptide)</t>
         </is>
       </c>
       <c r="C231" s="13" t="inlineStr">
@@ -6199,7 +6199,7 @@
       </c>
       <c r="D231" s="4" t="inlineStr">
         <is>
-          <t>A research-informed assessment across 6 real dimensions, grounded in real cited research (Klein Sexual Orientation Grid 1978, Kinsey Scale 1948, Lisa Diamond 2008, Sari van Anders 2015) — real 16 questions (with per-question research context notes), real 12 archetypes (each with a real description + research note), and the real scoring/selection logic all ported unchanged and verbatim, including the real closing disclaimer. Legacy's own AssessmentIntro stats prop claimed "20 questions, 7 dimensions" — didn't match the real 16/6 implementation, used the live counts instead. Legacy's results screen also used light grey text on the real light pastel theme background (same low-contrast bug already caught on /find-your-style) — normalized to dark ink. Verified live: 200 OK, redirect confirmed 308, typecheck/lint clean.</t>
+          <t>"The Peptide Clarity Index™." A real, evidence-cited 10-question assessment across 7 clinical axes, mapping to 16 real peptide archetype profiles — every question (with its real PubMed/journal citation), every profile's real primary/secondary peptides with mechanisms and evidence, suggested lab work, red flags, and stacking notes ported unchanged and verbatim (clinical-adjacent content, not paraphrased). The real Peptide Readiness Score, contraindication-flag screening, share buttons (Twitter/LinkedIn/email/copy — real, backend-free), and the real medical disclaimer are all preserved. Real hero image (CloudFront, confirmed live) kept via next/image. Reused the simplified AssessmentResultActions (PDF-only) built for /find-your-spirit. Same light-text-on-light-background contrast bug already caught elsewhere was fixed here too. Verified live: 200 OK, redirect confirmed 308, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E231" s="14" t="inlineStr">
@@ -6212,7 +6212,7 @@
       <c r="A232" s="4" t="n"/>
       <c r="B232" s="4" t="inlineStr">
         <is>
-          <t>/find-my</t>
+          <t>/find-your-sexuality (+ /find-my-sexuality)</t>
         </is>
       </c>
       <c r="C232" s="13" t="inlineStr">
@@ -6222,7 +6222,7 @@
       </c>
       <c r="D232" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Find What's Yours," the real destination of the homepage's "Diagnose" door (confirmed by grepping lib/content/home-doors.ts's /find-my href) and of whats-next.tsx's "Take Another Assessment" link, both already pointing here as forward-references before this page existed. Legacy's 26-item ALL_LINKS directory (Featured + 6 categories) ported unchanged and verbatim into lib/content/find-my-directory.ts. Real accuracy fix, same pattern as /find-your-me's own port note: cross-checked all 26 destinations against the real route list — /find-your-ev, /life-assessment, and /soulscore (at the time) didn't exist yet, rendered as real "Coming Soon" cards instead of links that would 404 (dharma-finder/consciousness-scale/grant-study have since shipped and now flip to live — see below). Real reuse, not re-derivation: every item whose destination already exists in find-your-me.ts's audited DIRECTORY pulls that entry's real hook text and status at build time via a lookup helper, instead of hand-copying a second, driftable copy of the same facts. Two real live destinations added that legacy linked but find-your-me.ts's directory didn't track: /brewsoul (confirmed 200) and the external findmystem-s3lknc4h.manus.space sibling tool (confirmed live), both using the same "real external sibling product" trust already established for the other manus.space tools. Legacy's dead Manus hero image dropped for ThemedBackground (theme="ecosystem"), same call as /find-your-me. AssessmentProgressBar (never </t>
+          <t>A research-informed assessment across 6 real dimensions, grounded in real cited research (Klein Sexual Orientation Grid 1978, Kinsey Scale 1948, Lisa Diamond 2008, Sari van Anders 2015) — real 16 questions (with per-question research context notes), real 12 archetypes (each with a real description + research note), and the real scoring/selection logic all ported unchanged and verbatim, including the real closing disclaimer. Legacy's own AssessmentIntro stats prop claimed "20 questions, 7 dimensions" — didn't match the real 16/6 implementation, used the live counts instead. Legacy's results screen also used light grey text on the real light pastel theme background (same low-contrast bug already caught on /find-your-style) — normalized to dark ink. Verified live: 200 OK, redirect confirmed 308, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E232" s="14" t="inlineStr">
@@ -6235,7 +6235,7 @@
       <c r="A233" s="4" t="n"/>
       <c r="B233" s="4" t="inlineStr">
         <is>
-          <t>/assessments</t>
+          <t>/find-my</t>
         </is>
       </c>
       <c r="C233" s="13" t="inlineStr">
@@ -6245,7 +6245,7 @@
       </c>
       <c r="D233" s="4" t="inlineStr">
         <is>
-          <t>"Three Maps. One Journey," confirmed genuinely distinct from /find-my rather than a duplicate: /find-my is the wide 26-item ecosystem directory, /assessments is its own page for exactly 3 long research-grounded instruments (Dharma Finder / Consciousness Scale / Grant Study) that also happen to appear as one category inside /find-my's directory — legacy kept these as two separate pages, so the port does too. Real title/subtitle/description/time/icon/accent content for all 3 instruments ported unchanged and verbatim into lib/content/assessments-hub.ts, including the full "Why These Three" closing essay (Schmachtenberger/Hawkins/Harvard Grant Study triangulation). All 3 instrument cards now link live (dharma-finder/consciousness-scale/grant-study shipped alongside this page). Legacy's footer claim "Results saved for your return" was dropped — replaced with an honest line since nothing persists results yet. Added a real cross-link to /find-my. JourneyTracker reused unchanged; no EmailGate/AssessmentResultActions — pure preview/hub page with no quiz or results step of its own. Verified live: 200 OK, exactly 1 header/footer, real content in all 3 cards, typecheck/lint clean.</t>
+          <t xml:space="preserve">"Find What's Yours," the real destination of the homepage's "Diagnose" door (confirmed by grepping lib/content/home-doors.ts's /find-my href) and of whats-next.tsx's "Take Another Assessment" link, both already pointing here as forward-references before this page existed. Legacy's 26-item ALL_LINKS directory (Featured + 6 categories) ported unchanged and verbatim into lib/content/find-my-directory.ts. Real accuracy fix, same pattern as /find-your-me's own port note: cross-checked all 26 destinations against the real route list — /find-your-ev, /life-assessment, and /soulscore (at the time) didn't exist yet, rendered as real "Coming Soon" cards instead of links that would 404 (dharma-finder/consciousness-scale/grant-study have since shipped and now flip to live — see below). Real reuse, not re-derivation: every item whose destination already exists in find-your-me.ts's audited DIRECTORY pulls that entry's real hook text and status at build time via a lookup helper, instead of hand-copying a second, driftable copy of the same facts. Two real live destinations added that legacy linked but find-your-me.ts's directory didn't track: /brewsoul (confirmed 200) and the external findmystem-s3lknc4h.manus.space sibling tool (confirmed live), both using the same "real external sibling product" trust already established for the other manus.space tools. Legacy's dead Manus hero image dropped for ThemedBackground (theme="ecosystem"), same call as /find-your-me. AssessmentProgressBar (never </t>
         </is>
       </c>
       <c r="E233" s="14" t="inlineStr">
@@ -6258,7 +6258,7 @@
       <c r="A234" s="4" t="n"/>
       <c r="B234" s="4" t="inlineStr">
         <is>
-          <t>/dharma-finder (+ /assessments/dharma-finder redirect). Structurally different from every other Phase 9 quiz</t>
+          <t>/assessments</t>
         </is>
       </c>
       <c r="C234" s="13" t="inlineStr">
@@ -6268,7 +6268,7 @@
       </c>
       <c r="D234" s="4" t="inlineStr">
         <is>
-          <t>legacy's real 25 questions are open-text reflection prompts, not multiple choice, distilled from Daniel Schmachtenberger's Dharma Inquiry and grouped into 4 real sections (Capacities/Values/Propensities/The Shadow Inquiry), each with a real framing quote, plus 3 real interstitial quotes shown between sections with the original 4-second auto-advance. All 25 questions, all quotes, and legacy's own keyword-matching generateDharmaProfile (deriving up to 3 archetypal roles and up to 4 core values from free-text answers, plus a completion-depth percentage) are ported unchanged and verbatim into a new dharma-finder-quiz.tsx. Real bug found and fixed: legacy's result-screen JSX rendered &lt;AssessmentResultActions&gt; nested inside the "Retake Assessment" &lt;button&gt; element — a button inside a button, invalid HTML — fixed the same way as /find-your-religion. Real dead-link bug fixed: "Journey Continues" linked to /assessments/consciousness-scale (repointed to the real /consciousness-scale) and /assessments/grant-study (dropped at the time, now live too). EmailGate (new here; legacy had none) is a real ecosystem-consistency addition. find-your-me.ts's ecosystem-directory status flipped from "coming" to "live" now that this page ships. Verified live: 200 OK, typecheck/lint clean.</t>
+          <t>"Three Maps. One Journey," confirmed genuinely distinct from /find-my rather than a duplicate: /find-my is the wide 26-item ecosystem directory, /assessments is its own page for exactly 3 long research-grounded instruments (Dharma Finder / Consciousness Scale / Grant Study) that also happen to appear as one category inside /find-my's directory — legacy kept these as two separate pages, so the port does too. Real title/subtitle/description/time/icon/accent content for all 3 instruments ported unchanged and verbatim into lib/content/assessments-hub.ts, including the full "Why These Three" closing essay (Schmachtenberger/Hawkins/Harvard Grant Study triangulation). All 3 instrument cards now link live (dharma-finder/consciousness-scale/grant-study shipped alongside this page). Legacy's footer claim "Results saved for your return" was dropped — replaced with an honest line since nothing persists results yet. Added a real cross-link to /find-my. JourneyTracker reused unchanged; no EmailGate/AssessmentResultActions — pure preview/hub page with no quiz or results step of its own. Verified live: 200 OK, exactly 1 header/footer, real content in all 3 cards, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E234" s="14" t="inlineStr">
@@ -6281,7 +6281,7 @@
       <c r="A235" s="4" t="n"/>
       <c r="B235" s="4" t="inlineStr">
         <is>
-          <t>/consciousness-scale (+ /assessments/consciousness-scale redirect)</t>
+          <t>/dharma-finder (+ /assessments/dharma-finder redirect). Structurally different from every other Phase 9 quiz</t>
         </is>
       </c>
       <c r="C235" s="13" t="inlineStr">
@@ -6291,7 +6291,7 @@
       </c>
       <c r="D235" s="4" t="inlineStr">
         <is>
-          <t>Real 25 questions, each scored against David R. Hawkins' real 17-level Map of Consciousness (Shame 20 through Enlightenment 700+, final score = average of all 25 answers) — every question/option, every level's name/emotion/threshold, and getInsight's exact 6 tiers of interpretive copy ported unchanged and verbatim into a new consciousness-scale-quiz.tsx, along with the real live running-average indicator, visual scale gauge, full 17-level map, 6-month reminder, and X/LinkedIn/copy share. Since this assessment produces one composite score on a single axis rather than independent dimensions, a bespoke single-axis gauge replaces AssessmentRadarChart; per-level colors (17 known-at-build-time values) are precomposed literal Tailwind classes rather than assembled from hex fragments. Real Manus-dependency bug found and fixed: legacy's cinematic Q1 hero used a /api/img/consciousness-scale-hero-v2_085e0746.jpg Manus-proxied image — forbidden even temporarily per this migration's Zero-Manus rule — dropped for the plain question-card layout every other assessment uses; a real Sanity-hosted replacement is a tracked follow-up (see BLOG-IMAGE-BRIEFS.md-style tracking). find-your-me.ts's ecosystem-directory status flipped from "coming" to "live" now that this page ships. Verified live: 200 OK, typecheck/lint clean.</t>
+          <t>legacy's real 25 questions are open-text reflection prompts, not multiple choice, distilled from Daniel Schmachtenberger's Dharma Inquiry and grouped into 4 real sections (Capacities/Values/Propensities/The Shadow Inquiry), each with a real framing quote, plus 3 real interstitial quotes shown between sections with the original 4-second auto-advance. All 25 questions, all quotes, and legacy's own keyword-matching generateDharmaProfile (deriving up to 3 archetypal roles and up to 4 core values from free-text answers, plus a completion-depth percentage) are ported unchanged and verbatim into a new dharma-finder-quiz.tsx. Real bug found and fixed: legacy's result-screen JSX rendered &lt;AssessmentResultActions&gt; nested inside the "Retake Assessment" &lt;button&gt; element — a button inside a button, invalid HTML — fixed the same way as /find-your-religion. Real dead-link bug fixed: "Journey Continues" linked to /assessments/consciousness-scale (repointed to the real /consciousness-scale) and /assessments/grant-study (dropped at the time, now live too). EmailGate (new here; legacy had none) is a real ecosystem-consistency addition. find-your-me.ts's ecosystem-directory status flipped from "coming" to "live" now that this page ships. Verified live: 200 OK, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E235" s="14" t="inlineStr">
@@ -6304,7 +6304,7 @@
       <c r="A236" s="4" t="n"/>
       <c r="B236" s="4" t="inlineStr">
         <is>
-          <t>/grant-study (+ /assessments/grant-study redirect)</t>
+          <t>/consciousness-scale (+ /assessments/consciousness-scale redirect)</t>
         </is>
       </c>
       <c r="C236" s="13" t="inlineStr">
@@ -6314,7 +6314,7 @@
       </c>
       <c r="D236" s="4" t="inlineStr">
         <is>
-          <t>"Find Your Score," the real 25-question (5 per factor), 5-factor Harvard Grant Study life-satisfaction assessment (724 men, 1938–present, 85+ years — the longest-running study of human happiness). Every question, the 5 real factors (Warm Relationships/Adaptive Coping/Generativity/Career Satisfaction/Physical Vitality), every per-factor/per-tier insight (real named findings — Vaillant's "mature defenses," Erikson's generativity, Waldinger's quote), and the closing "Tony's Note" (Vaillant's "Happiness is love. Full stop." + Waldinger's "good relationships keep us happier and healthier") all ported unchanged and verbatim. Real nested-interactive-element bug found and fixed: legacy rendered &lt;AssessmentResultActions&gt; (its own &lt;button&gt;) literally inside the "Retake Assessment" &lt;button&gt; — same bug class already caught on /find-your-religion//find-your-sake — split into siblings. Real dead-link fix: "Journey Continues" pointed "Find Your Spirit" at a dead external Manus stub despite the real internal /find-your-spirit existing — repointed. Real ecosystem-consistency normalization: unlike every sibling "Find Your X" quiz, legacy skipped EmailGate entirely and went straight to results — added for consistency, plus new find-your-grant-study/find-your-dharma-finder/find-your-consciousness-scale alias keys in kit-source-tags.ts's KIT_TAG_MAP so EmailGate's fixed find-your-&lt;slug&gt; source prefix actually resolves to the intended tag instead of a generic fallback. resultSlug="grant-study" pas</t>
+          <t>Real 25 questions, each scored against David R. Hawkins' real 17-level Map of Consciousness (Shame 20 through Enlightenment 700+, final score = average of all 25 answers) — every question/option, every level's name/emotion/threshold, and getInsight's exact 6 tiers of interpretive copy ported unchanged and verbatim into a new consciousness-scale-quiz.tsx, along with the real live running-average indicator, visual scale gauge, full 17-level map, 6-month reminder, and X/LinkedIn/copy share. Since this assessment produces one composite score on a single axis rather than independent dimensions, a bespoke single-axis gauge replaces AssessmentRadarChart; per-level colors (17 known-at-build-time values) are precomposed literal Tailwind classes rather than assembled from hex fragments. Real Manus-dependency bug found and fixed: legacy's cinematic Q1 hero used a /api/img/consciousness-scale-hero-v2_085e0746.jpg Manus-proxied image — forbidden even temporarily per this migration's Zero-Manus rule — dropped for the plain question-card layout every other assessment uses; a real Sanity-hosted replacement is a tracked follow-up (see BLOG-IMAGE-BRIEFS.md-style tracking). find-your-me.ts's ecosystem-directory status flipped from "coming" to "live" now that this page ships. Verified live: 200 OK, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E236" s="14" t="inlineStr">
@@ -6327,7 +6327,7 @@
       <c r="A237" s="4" t="n"/>
       <c r="B237" s="4" t="inlineStr">
         <is>
-          <t>/soulscore</t>
+          <t>/grant-study (+ /assessments/grant-study redirect)</t>
         </is>
       </c>
       <c r="C237" s="13" t="inlineStr">
@@ -6337,7 +6337,7 @@
       </c>
       <c r="D237" s="4" t="inlineStr">
         <is>
-          <t>SoulScore™, ImpactSoul's 12-dimension impact measurement engine (1231-line legacy file, the largest remaining port). Unlike the quiz-style "Find Your X" assessments, this is a live interactive calculator, not a Q&amp;A flow: entity-type picker, 12 weighted dimension sliders (Hawkins-scale Consciousness + 11 others), real-time score/grade/radar/auto-diagnosis, a benchmark table against 7 real entities (Patagonia, BP, Fortune 500 Avg, etc.), a 6-tier/30-factor supply chain drill-down, 20 "why every impact system failed" entries, a real Consciousness-Adjusted NPV calculator, and the gig-economy 5-layer stack comparison — all real content/formulas ported verbatim. Fixed: legacy's own SEO block described an unrelated assessment (stale copy-paste, replaced with real metadata); a div-pretending-to-be-a-button wrapping 30 nested range-input sliders (fixed to a real &lt;button&gt; + sibling content div); hardcoded intro/tab counts now read off real array lengths. No EmailGate (legacy never had one here — it's an open calculator, not a report unlock), matching /find-your-peptide's precedent. AssessmentResultActions wired with resultSlug="soulscore". journey-tracker.tsx's JOURNEY_MAP and /impact-dashboard's "Launch SoulScore Engine"/"Launch C-NPV Calculator" links (previously a disabled "Coming Soon" note) now point at the real page. This closes the real dead-end referenced from site-nav-data.ts (/soulscore appears twice in nav) and from /impact-dashboard — the last item in the STATUS.md dead-end</t>
+          <t>"Find Your Score," the real 25-question (5 per factor), 5-factor Harvard Grant Study life-satisfaction assessment (724 men, 1938–present, 85+ years — the longest-running study of human happiness). Every question, the 5 real factors (Warm Relationships/Adaptive Coping/Generativity/Career Satisfaction/Physical Vitality), every per-factor/per-tier insight (real named findings — Vaillant's "mature defenses," Erikson's generativity, Waldinger's quote), and the closing "Tony's Note" (Vaillant's "Happiness is love. Full stop." + Waldinger's "good relationships keep us happier and healthier") all ported unchanged and verbatim. Real nested-interactive-element bug found and fixed: legacy rendered &lt;AssessmentResultActions&gt; (its own &lt;button&gt;) literally inside the "Retake Assessment" &lt;button&gt; — same bug class already caught on /find-your-religion//find-your-sake — split into siblings. Real dead-link fix: "Journey Continues" pointed "Find Your Spirit" at a dead external Manus stub despite the real internal /find-your-spirit existing — repointed. Real ecosystem-consistency normalization: unlike every sibling "Find Your X" quiz, legacy skipped EmailGate entirely and went straight to results — added for consistency, plus new find-your-grant-study/find-your-dharma-finder/find-your-consciousness-scale alias keys in kit-source-tags.ts's KIT_TAG_MAP so EmailGate's fixed find-your-&lt;slug&gt; source prefix actually resolves to the intended tag instead of a generic fallback. resultSlug="grant-study" pas</t>
         </is>
       </c>
       <c r="E237" s="14" t="inlineStr">
@@ -6350,7 +6350,7 @@
       <c r="A238" s="4" t="n"/>
       <c r="B238" s="4" t="inlineStr">
         <is>
-          <t>/self-portrait</t>
+          <t>/soulscore</t>
         </is>
       </c>
       <c r="C238" s="13" t="inlineStr">
@@ -6360,7 +6360,7 @@
       </c>
       <c r="D238" s="4" t="inlineStr">
         <is>
-          <t>composite of completed assessments. Decision made: local-only (a real cookie, not Supabase — Phase 2 isn't provisioned yet). AssessmentResultActions (components/assessments/result-actions.tsx) takes an optional resultSlug and logs completions to a tg_assessment_results cookie via lib/assessments/result-log.ts, the same real-cookie-read-via-next/headers pattern already established by returning-visitor-hero.tsx/track-last-blog-visit.tsx — the page itself is a Server Component reading that cookie with zero client hydration step. Real, deliberate scope cut, not a silent one: legacy's SelfPortrait.tsx combined each assessment's own per-dimension scores (16 separate localStorage keys) into one composite radar chart across 15 unified dimensions, gated behind "5+ completed." This migration's result log only ever records that an assessment was completed, not its actual scored answers — building the real composite radar would mean threading a second, much larger data channel through every quiz. Shipped the honest subset instead: a real completed-assessments list (title, real completion date, retake link) plus a real "X of N completed" count and a "Still to Explore" section for the rest, via a new lib/content/self-portrait-catalog.ts. Wired resultSlug into the 7 remaining older "Find Your X" quizzes that already call AssessmentResultActions but hadn't been threaded yet (spirit/therapy/religion/sake/coffee/peptide/me) — /self-portrait now tracks 13 real assessments total. /find-my's "Sel</t>
+          <t>SoulScore™, ImpactSoul's 12-dimension impact measurement engine (1231-line legacy file, the largest remaining port). Unlike the quiz-style "Find Your X" assessments, this is a live interactive calculator, not a Q&amp;A flow: entity-type picker, 12 weighted dimension sliders (Hawkins-scale Consciousness + 11 others), real-time score/grade/radar/auto-diagnosis, a benchmark table against 7 real entities (Patagonia, BP, Fortune 500 Avg, etc.), a 6-tier/30-factor supply chain drill-down, 20 "why every impact system failed" entries, a real Consciousness-Adjusted NPV calculator, and the gig-economy 5-layer stack comparison — all real content/formulas ported verbatim. Fixed: legacy's own SEO block described an unrelated assessment (stale copy-paste, replaced with real metadata); a div-pretending-to-be-a-button wrapping 30 nested range-input sliders (fixed to a real &lt;button&gt; + sibling content div); hardcoded intro/tab counts now read off real array lengths. No EmailGate (legacy never had one here — it's an open calculator, not a report unlock), matching /find-your-peptide's precedent. AssessmentResultActions wired with resultSlug="soulscore". journey-tracker.tsx's JOURNEY_MAP and /impact-dashboard's "Launch SoulScore Engine"/"Launch C-NPV Calculator" links (previously a disabled "Coming Soon" note) now point at the real page. This closes the real dead-end referenced from site-nav-data.ts (/soulscore appears twice in nav) and from /impact-dashboard — the last item in the STATUS.md dead-end</t>
         </is>
       </c>
       <c r="E238" s="14" t="inlineStr">
@@ -6373,7 +6373,7 @@
       <c r="A239" s="4" t="n"/>
       <c r="B239" s="4" t="inlineStr">
         <is>
-          <t>/the-mirror (+ /life-assessment)</t>
+          <t>/self-portrait</t>
         </is>
       </c>
       <c r="C239" s="13" t="inlineStr">
@@ -6383,7 +6383,7 @@
       </c>
       <c r="D239" s="4" t="inlineStr">
         <is>
-          <t>uses mirrorData.json, real 6-dimension/18-question life assessment ("The Mirror") ported into a typed lib/content/mirror-data.ts. Legacy served the identical component at both paths; /the-mirror is canonical (it's the only URL every existing internal link already pointed to — nav, journey tracker, Find Your Me), /life-assessment permanently redirects there. Real dimension-averaged scoring, radar chart via the shared AssessmentRadarChart, and weakest-dimension article/satellite-site recommendations ported unchanged. A live Sanity check found only 27 of 85 legacy article slugs still resolve; recommendations now resolve server-side and defensively skip missing ones, matching legacy's own behavior. Fixed: a hydration-unsafe typeof window branch computing the share URL, three stale manus.space satellite URLs superseded by their current live counterparts already used elsewhere in this migration, and dead /assessments/*/external-stub links in the "Journey Continues" grid. Added find-your-mirror to kit-source-tags.ts's KIT_TAG_MAP and reconciled journey-tracker.tsx's stale 10-minute estimate to legacy's real "~4 minutes" claim. find-your-me.ts's ecosystem-directory status flipped to "live." Verified live: 200 OK on both paths, redirect confirmed, typecheck/lint clean.</t>
+          <t>composite of completed assessments. Decision made: local-only (a real cookie, not Supabase — Phase 2 isn't provisioned yet). AssessmentResultActions (components/assessments/result-actions.tsx) takes an optional resultSlug and logs completions to a tg_assessment_results cookie via lib/assessments/result-log.ts, the same real-cookie-read-via-next/headers pattern already established by returning-visitor-hero.tsx/track-last-blog-visit.tsx — the page itself is a Server Component reading that cookie with zero client hydration step. Real, deliberate scope cut, not a silent one: legacy's SelfPortrait.tsx combined each assessment's own per-dimension scores (16 separate localStorage keys) into one composite radar chart across 15 unified dimensions, gated behind "5+ completed." This migration's result log only ever records that an assessment was completed, not its actual scored answers — building the real composite radar would mean threading a second, much larger data channel through every quiz. Shipped the honest subset instead: a real completed-assessments list (title, real completion date, retake link) plus a real "X of N completed" count and a "Still to Explore" section for the rest, via a new lib/content/self-portrait-catalog.ts. Wired resultSlug into the 7 remaining older "Find Your X" quizzes that already call AssessmentResultActions but hadn't been threaded yet (spirit/therapy/religion/sake/coffee/peptide/me) — /self-portrait now tracks 13 real assessments total. /find-my's "Sel</t>
         </is>
       </c>
       <c r="E239" s="14" t="inlineStr">
@@ -6396,7 +6396,7 @@
       <c r="A240" s="4" t="n"/>
       <c r="B240" s="4" t="inlineStr">
         <is>
-          <t>/assessment</t>
+          <t>/the-mirror (+ /life-assessment)</t>
         </is>
       </c>
       <c r="C240" s="13" t="inlineStr">
@@ -6406,7 +6406,7 @@
       </c>
       <c r="D240" s="4" t="inlineStr">
         <is>
-          <t>confirmed via full legacy read this is not a "Find Your X" quiz (it predates that convention): it's Tony's own 3-way reader-path diagnostic — Builder / Crusader / Investor — 5 real questions, one point per matching answer, highest tally wins. Real questions and real archetype copy ported unchanged, reused from lib/content/archetypes.ts (already ported for /essays's archetype filter) rather than duplicated — added the page's ASSESSMENT_QUESTIONS to that same module since both come from the identical legacy source file. Preserved the real, distinct UX (no landing screen, no ThemedBackground/JourneyTracker — this page sits outside that ecosystem). Real bugs fixed: JS onMouseEnter/onMouseLeave inline-style hover hack replaced with Tailwind hover: classes; literal "..." pending-state text replaced with a real Loader2 spinner per house rule; dead trpc.subscribe.add replaced with a real POST /api/subscribe call. Real link audit: kept /impact-dashboard, /find-your-me, /living-declaration, and the real /blog/boiling-the-human-summit-harvard-kurzweil article as live links; /soulscore and /humanos are established forward-references used repeatedly elsewhere in this migration and both now ship too. The Human OS CTA reuses the border-red-800/30 text-red-800 treatment /living-declaration already established for the identical button instead of a new one-off raw-hex pair. AssessmentResultActions resultSlug="assessment" added (didn't exist when legacy was written). Added assessment-builder/as</t>
+          <t>uses mirrorData.json, real 6-dimension/18-question life assessment ("The Mirror") ported into a typed lib/content/mirror-data.ts. Legacy served the identical component at both paths; /the-mirror is canonical (it's the only URL every existing internal link already pointed to — nav, journey tracker, Find Your Me), /life-assessment permanently redirects there. Real dimension-averaged scoring, radar chart via the shared AssessmentRadarChart, and weakest-dimension article/satellite-site recommendations ported unchanged. A live Sanity check found only 27 of 85 legacy article slugs still resolve; recommendations now resolve server-side and defensively skip missing ones, matching legacy's own behavior. Fixed: a hydration-unsafe typeof window branch computing the share URL, three stale manus.space satellite URLs superseded by their current live counterparts already used elsewhere in this migration, and dead /assessments/*/external-stub links in the "Journey Continues" grid. Added find-your-mirror to kit-source-tags.ts's KIT_TAG_MAP and reconciled journey-tracker.tsx's stale 10-minute estimate to legacy's real "~4 minutes" claim. find-your-me.ts's ecosystem-directory status flipped to "live." Verified live: 200 OK on both paths, redirect confirmed, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E240" s="14" t="inlineStr">
@@ -6419,7 +6419,7 @@
       <c r="A241" s="4" t="n"/>
       <c r="B241" s="4" t="inlineStr">
         <is>
-          <t>Fix dead-end pages flagged in STATUS.md</t>
+          <t>/assessment</t>
         </is>
       </c>
       <c r="C241" s="13" t="inlineStr">
@@ -6429,7 +6429,7 @@
       </c>
       <c r="D241" s="4" t="inlineStr">
         <is>
-          <t>sake, therapy, and love-language all got real next-step navigation (WhatsNext + real "Journey Continues" links) during their ports — the last remaining one, soulscore, is now built (see above), closing this out.</t>
+          <t>confirmed via full legacy read this is not a "Find Your X" quiz (it predates that convention): it's Tony's own 3-way reader-path diagnostic — Builder / Crusader / Investor — 5 real questions, one point per matching answer, highest tally wins. Real questions and real archetype copy ported unchanged, reused from lib/content/archetypes.ts (already ported for /essays's archetype filter) rather than duplicated — added the page's ASSESSMENT_QUESTIONS to that same module since both come from the identical legacy source file. Preserved the real, distinct UX (no landing screen, no ThemedBackground/JourneyTracker — this page sits outside that ecosystem). Real bugs fixed: JS onMouseEnter/onMouseLeave inline-style hover hack replaced with Tailwind hover: classes; literal "..." pending-state text replaced with a real Loader2 spinner per house rule; dead trpc.subscribe.add replaced with a real POST /api/subscribe call. Real link audit: kept /impact-dashboard, /find-your-me, /living-declaration, and the real /blog/boiling-the-human-summit-harvard-kurzweil article as live links; /soulscore and /humanos are established forward-references used repeatedly elsewhere in this migration and both now ship too. The Human OS CTA reuses the border-red-800/30 text-red-800 treatment /living-declaration already established for the identical button instead of a new one-off raw-hex pair. AssessmentResultActions resultSlug="assessment" added (didn't exist when legacy was written). Added assessment-builder/as</t>
         </is>
       </c>
       <c r="E241" s="14" t="inlineStr">
@@ -6442,63 +6442,63 @@
       <c r="A242" s="4" t="n"/>
       <c r="B242" s="4" t="inlineStr">
         <is>
+          <t>Fix dead-end pages flagged in STATUS.md</t>
+        </is>
+      </c>
+      <c r="C242" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D242" s="4" t="inlineStr">
+        <is>
+          <t>sake, therapy, and love-language all got real next-step navigation (WhatsNext + real "Journey Continues" links) during their ports — the last remaining one, soulscore, is now built (see above), closing this out.</t>
+        </is>
+      </c>
+      <c r="E242" s="14" t="inlineStr">
+        <is>
+          <t>Phase 9 — Assessments (33 routes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="4" t="n"/>
+      <c r="B243" s="4" t="inlineStr">
+        <is>
           <t>Port shared radar-chart / PDF-export / email-gate components used across assessments</t>
         </is>
       </c>
-      <c r="C242" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D242" s="4" t="inlineStr">
+      <c r="C243" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D243" s="4" t="inlineStr">
         <is>
           <t>components/assessments/{radar-chart,result-actions,email-gate}.tsx, built during Phase 9 and reused unchanged by all 15 "Find Your X" quizzes plus /find-your-me.</t>
         </is>
       </c>
-      <c r="E242" s="14" t="inlineStr">
+      <c r="E243" s="14" t="inlineStr">
         <is>
           <t>Phase 9 — Assessments (33 routes)</t>
         </is>
       </c>
     </row>
-    <row r="243">
-      <c r="A243" s="10" t="inlineStr">
+    <row r="244">
+      <c r="A244" s="10" t="inlineStr">
         <is>
           <t>Phase 11 — Code MCP Server — REBUILT (2026-09-29)</t>
         </is>
       </c>
-      <c r="B243" s="11" t="n"/>
-      <c r="C243" s="11" t="n"/>
-      <c r="D243" s="12" t="n"/>
-    </row>
-    <row r="244">
-      <c r="A244" s="4" t="n"/>
-      <c r="B244" s="4" t="inlineStr">
-        <is>
-          <t>src/lib/admin/</t>
-        </is>
-      </c>
-      <c r="C244" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D244" s="4" t="inlineStr">
-        <is>
-          <t>guardrails (fixes the removed version's proxy.ts pattern, which missed the real src/proxy.ts), GitHub client (RRTONY/tonygreenberg-website), Sanity draft helpers, code-check.ts (ESLint + CONTRIBUTING.md house-rule patterns, now also Manus URLs and ellipsis loading text), seo-check.ts, tools.ts, mcp-server.ts, mcp-handler.ts, mcp-tool-context.ts (GitHub looked up lazily, so Sanity/SEO/code-check tools work without GITHUB_TOKEN).</t>
-        </is>
-      </c>
-      <c r="E244" s="14" t="inlineStr">
-        <is>
-          <t>Phase 11 — Code MCP Server — REBUILT (2026-09-29)</t>
-        </is>
-      </c>
+      <c r="B244" s="11" t="n"/>
+      <c r="C244" s="11" t="n"/>
+      <c r="D244" s="12" t="n"/>
     </row>
     <row r="245">
       <c r="A245" s="4" t="n"/>
       <c r="B245" s="4" t="inlineStr">
         <is>
-          <t>Per-person access via MCP_ADMIN_USERS (read/edit/write roles, tools filtered per role, calls logged, commits stamped [by &lt;name&gt;])</t>
+          <t>src/lib/admin/</t>
         </is>
       </c>
       <c r="C245" s="13" t="inlineStr">
@@ -6508,7 +6508,7 @@
       </c>
       <c r="D245" s="4" t="inlineStr">
         <is>
-          <t>mcp-auth.ts.</t>
+          <t>guardrails (fixes the removed version's proxy.ts pattern, which missed the real src/proxy.ts), GitHub client (RRTONY/tonygreenberg-website), Sanity draft helpers, code-check.ts (ESLint + CONTRIBUTING.md house-rule patterns, now also Manus URLs and ellipsis loading text), seo-check.ts, tools.ts, mcp-server.ts, mcp-handler.ts, mcp-tool-context.ts (GitHub looked up lazily, so Sanity/SEO/code-check tools work without GITHUB_TOKEN).</t>
         </is>
       </c>
       <c r="E245" s="14" t="inlineStr">
@@ -6521,7 +6521,7 @@
       <c r="A246" s="4" t="n"/>
       <c r="B246" s="4" t="inlineStr">
         <is>
-          <t>Rules gate: get_project_rules serves CONTRIBUTING.md + AGENTS.md + docs/ai/ guides with a rulesVersion; all 6 write tools require it</t>
+          <t>Per-person access via MCP_ADMIN_USERS (read/edit/write roles, tools filtered per role, calls logged, commits stamped [by &lt;name&gt;])</t>
         </is>
       </c>
       <c r="C246" s="13" t="inlineStr">
@@ -6531,7 +6531,7 @@
       </c>
       <c r="D246" s="4" t="inlineStr">
         <is>
-          <t>project-rules.ts.</t>
+          <t>mcp-auth.ts.</t>
         </is>
       </c>
       <c r="E246" s="14" t="inlineStr">
@@ -6544,7 +6544,7 @@
       <c r="A247" s="4" t="n"/>
       <c r="B247" s="4" t="inlineStr">
         <is>
-          <t>src/app/api/mcp/route.ts (header auth) + src/app/api/mcp/[token]/route.ts (token in URL).</t>
+          <t>Rules gate: get_project_rules serves CONTRIBUTING.md + AGENTS.md + docs/ai/ guides with a rulesVersion; all 6 write tools require it</t>
         </is>
       </c>
       <c r="C247" s="13" t="inlineStr">
@@ -6552,7 +6552,11 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="D247" s="4" t="inlineStr"/>
+      <c r="D247" s="4" t="inlineStr">
+        <is>
+          <t>project-rules.ts.</t>
+        </is>
+      </c>
       <c r="E247" s="14" t="inlineStr">
         <is>
           <t>Phase 11 — Code MCP Server — REBUILT (2026-09-29)</t>
@@ -6563,7 +6567,7 @@
       <c r="A248" s="4" t="n"/>
       <c r="B248" s="4" t="inlineStr">
         <is>
-          <t>docs/ai/ knowledge base (README, TASK_GUIDE, PROJECT_STRUCTURE, project_mcp_server), linked from CONTRIBUTING.md.</t>
+          <t>src/app/api/mcp/route.ts (header auth) + src/app/api/mcp/[token]/route.ts (token in URL).</t>
         </is>
       </c>
       <c r="C248" s="13" t="inlineStr">
@@ -6582,7 +6586,7 @@
       <c r="A249" s="4" t="n"/>
       <c r="B249" s="4" t="inlineStr">
         <is>
-          <t>@modelcontextprotocol/sdk ^1.30.0 re-added (approved 2026-09-29); GITHUB_TOKEN/MCP_ADMIN_USERS/MCP_SITE_ORIGIN documented in .env.local.example.</t>
+          <t>docs/ai/ knowledge base (README, TASK_GUIDE, PROJECT_STRUCTURE, project_mcp_server), linked from CONTRIBUTING.md.</t>
         </is>
       </c>
       <c r="C249" s="13" t="inlineStr">
@@ -6601,7 +6605,7 @@
       <c r="A250" s="4" t="n"/>
       <c r="B250" s="4" t="inlineStr">
         <is>
-          <t>Verified locally</t>
+          <t>@modelcontextprotocol/sdk ^1.30.0 re-added (approved 2026-09-29); GITHUB_TOKEN/MCP_ADMIN_USERS/MCP_SITE_ORIGIN documented in .env.local.example.</t>
         </is>
       </c>
       <c r="C250" s="13" t="inlineStr">
@@ -6609,11 +6613,7 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="D250" s="4" t="inlineStr">
-        <is>
-          <t>auth (401/405), role filtering, rules-gate markers, token-in-URL route, code check, Sanity query, SEO check.</t>
-        </is>
-      </c>
+      <c r="D250" s="4" t="inlineStr"/>
       <c r="E250" s="14" t="inlineStr">
         <is>
           <t>Phase 11 — Code MCP Server — REBUILT (2026-09-29)</t>
@@ -6624,7 +6624,7 @@
       <c r="A251" s="4" t="n"/>
       <c r="B251" s="4" t="inlineStr">
         <is>
-          <t>Sign-in for the MCP server (OAuth 2.1, ported from ramprate-ui, 2026-09-30)</t>
+          <t>Verified locally</t>
         </is>
       </c>
       <c r="C251" s="13" t="inlineStr">
@@ -6634,7 +6634,7 @@
       </c>
       <c r="D251" s="4" t="inlineStr">
         <is>
-          <t>/oauth/authorize sign-in page + /.well-known metadata + register/authorize/token endpoints, stateless (signed tokens, no database), no new dependency. Verified end to end on a local production build. See docs/ai/project_mcp_server.md.</t>
+          <t>auth (401/405), role filtering, rules-gate markers, token-in-URL route, code check, Sanity query, SEO check.</t>
         </is>
       </c>
       <c r="E251" s="14" t="inlineStr">
@@ -6647,17 +6647,17 @@
       <c r="A252" s="4" t="n"/>
       <c r="B252" s="4" t="inlineStr">
         <is>
-          <t>Set GITHUB_TOKEN, MCP_ADMIN_USERS, MCP_LOGIN_PASSWORD, MCP_OAUTH_SECRET, MCP_SITE_ORIGIN, MCP_PUBLIC_ORIGIN in Netlify (done) (checked 2026-…</t>
-        </is>
-      </c>
-      <c r="C252" s="16" t="inlineStr">
-        <is>
-          <t>Remaining</t>
+          <t>Sign-in for the MCP server (OAuth 2.1, ported from ramprate-ui, 2026-09-30)</t>
+        </is>
+      </c>
+      <c r="C252" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D252" s="4" t="inlineStr">
         <is>
-          <t>10-07: all already set in Netlify). Left: connect Claude.ai to /api/mcp for real, and verify the GitHub flow end to end (branch → PR → deploy preview → publish_changes) against a real PR.</t>
+          <t>/oauth/authorize sign-in page + /.well-known metadata + register/authorize/token endpoints, stateless (signed tokens, no database), no new dependency. Verified end to end on a local production build. See docs/ai/project_mcp_server.md.</t>
         </is>
       </c>
       <c r="E252" s="14" t="inlineStr">
@@ -6670,7 +6670,7 @@
       <c r="A253" s="4" t="n"/>
       <c r="B253" s="4" t="inlineStr">
         <is>
-          <t>Commit a team-wide .mcp.json (URL only) once the production URL is settled.</t>
+          <t>Set GITHUB_TOKEN, MCP_ADMIN_USERS, MCP_LOGIN_PASSWORD, MCP_OAUTH_SECRET, MCP_SITE_ORIGIN, MCP_PUBLIC_ORIGIN in Netlify (done) (checked 2026-…</t>
         </is>
       </c>
       <c r="C253" s="16" t="inlineStr">
@@ -6678,7 +6678,11 @@
           <t>Remaining</t>
         </is>
       </c>
-      <c r="D253" s="4" t="inlineStr"/>
+      <c r="D253" s="4" t="inlineStr">
+        <is>
+          <t>10-07: all already set in Netlify). Left: connect Claude.ai to /api/mcp for real, and verify the GitHub flow end to end (branch → PR → deploy preview → publish_changes) against a real PR.</t>
+        </is>
+      </c>
       <c r="E253" s="14" t="inlineStr">
         <is>
           <t>Phase 11 — Code MCP Server — REBUILT (2026-09-29)</t>
@@ -6689,19 +6693,15 @@
       <c r="A254" s="4" t="n"/>
       <c r="B254" s="4" t="inlineStr">
         <is>
-          <t>Google read-only tools added (2026-10-02)</t>
-        </is>
-      </c>
-      <c r="C254" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D254" s="4" t="inlineStr">
-        <is>
-          <t>check_analytics (GA4), search_console_sites / _performance / _inspect_url / _sitemaps (list only, no submit or delete), lighthouse_check_page (PageSpeed Insights). New files google-auth.ts, ga4-client.ts, gsc-client.ts, lighthouse-check.ts; no new dependency. Verified on a local production build through /api/mcp: 22 tools listed, GA4 returns real numbers (1,233 sessions in 7 days), the others return a clear "what's missing" error. Env vars added to .env.local.example.</t>
-        </is>
-      </c>
+          <t>Commit a team-wide .mcp.json (URL only) once the production URL is settled.</t>
+        </is>
+      </c>
+      <c r="C254" s="16" t="inlineStr">
+        <is>
+          <t>Remaining</t>
+        </is>
+      </c>
+      <c r="D254" s="4" t="inlineStr"/>
       <c r="E254" s="14" t="inlineStr">
         <is>
           <t>Phase 11 — Code MCP Server — REBUILT (2026-09-29)</t>
@@ -6712,7 +6712,7 @@
       <c r="A255" s="4" t="n"/>
       <c r="B255" s="4" t="inlineStr">
         <is>
-          <t>publish_changes fixed (2026-10-02)</t>
+          <t>Google read-only tools added (2026-10-02)</t>
         </is>
       </c>
       <c r="C255" s="13" t="inlineStr">
@@ -6722,7 +6722,7 @@
       </c>
       <c r="D255" s="4" t="inlineStr">
         <is>
-          <t>it published every draft in Sanity (31 waiting for review today), so any one-line fix would have pushed them all live. Now it publishes only the drafts named in draft_ids; unknown ids are refused before anything happens (verified).</t>
+          <t>check_analytics (GA4), search_console_sites / _performance / _inspect_url / _sitemaps (list only, no submit or delete), lighthouse_check_page (PageSpeed Insights). New files google-auth.ts, ga4-client.ts, gsc-client.ts, lighthouse-check.ts; no new dependency. Verified on a local production build through /api/mcp: 22 tools listed, GA4 returns real numbers (1,233 sessions in 7 days), the others return a clear "what's missing" error. Env vars added to .env.local.example.</t>
         </is>
       </c>
       <c r="E255" s="14" t="inlineStr">
@@ -6735,7 +6735,7 @@
       <c r="A256" s="4" t="n"/>
       <c r="B256" s="4" t="inlineStr">
         <is>
-          <t>seo_check_page decoded &amp;#39; but not React's &amp;#x27;, so descriptions showed Tony Greenberg&amp;#x27;s and the length was off</t>
+          <t>publish_changes fixed (2026-10-02)</t>
         </is>
       </c>
       <c r="C256" s="13" t="inlineStr">
@@ -6745,7 +6745,7 @@
       </c>
       <c r="D256" s="4" t="inlineStr">
         <is>
-          <t>Fixed and verified (2026-10-02).</t>
+          <t>it published every draft in Sanity (31 waiting for review today), so any one-line fix would have pushed them all live. Now it publishes only the drafts named in draft_ids; unknown ids are refused before anything happens (verified).</t>
         </is>
       </c>
       <c r="E256" s="14" t="inlineStr">
@@ -6758,7 +6758,7 @@
       <c r="A257" s="4" t="n"/>
       <c r="B257" s="4" t="inlineStr">
         <is>
-          <t>Search Console access for the service account added by the team (2026-10-02); all four search_console_* tools verified with real tonygreenbe…</t>
+          <t>seo_check_page decoded &amp;#39; but not React's &amp;#x27;, so descriptions showed Tony Greenberg&amp;#x27;s and the length was off</t>
         </is>
       </c>
       <c r="C257" s="13" t="inlineStr">
@@ -6768,7 +6768,7 @@
       </c>
       <c r="D257" s="4" t="inlineStr">
         <is>
-          <t>rg.com data (99 clicks / 1,663 impressions in 28 days, homepage indexed, sitemap 284 URLs, 0 errors, 82 warnings).</t>
+          <t>Fixed and verified (2026-10-02).</t>
         </is>
       </c>
       <c r="E257" s="14" t="inlineStr">
@@ -6781,7 +6781,7 @@
       <c r="A258" s="4" t="n"/>
       <c r="B258" s="4" t="inlineStr">
         <is>
-          <t>GOOGLE_GA_CLIENT_EMAIL, GOOGLE_GA_PRIVATE_KEY, GA4_PROPERTY_ID_TONYGREENBERG set in Netlify (2026-10-02, via the Netlify API, values checked…</t>
+          <t>Search Console access for the service account added by the team (2026-10-02); all four search_console_* tools verified with real tonygreenbe…</t>
         </is>
       </c>
       <c r="C258" s="13" t="inlineStr">
@@ -6791,7 +6791,7 @@
       </c>
       <c r="D258" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> equal to .env.local; this plan can't limit a variable's scopes, so they're available to builds and functions). Used from the next deploy.</t>
+          <t>rg.com data (99 clicks / 1,663 impressions in 28 days, homepage indexed, sitemap 284 URLs, 0 errors, 82 warnings).</t>
         </is>
       </c>
       <c r="E258" s="14" t="inlineStr">
@@ -6804,7 +6804,7 @@
       <c r="A259" s="4" t="n"/>
       <c r="B259" s="4" t="inlineStr">
         <is>
-          <t>Per-request change system ported from ramprate-ui (2026-10-02, owner said yes)</t>
+          <t>GOOGLE_GA_CLIENT_EMAIL, GOOGLE_GA_PRIVATE_KEY, GA4_PROPERTY_ID_TONYGREENBERG set in Netlify (2026-10-02, via the Netlify API, values checked…</t>
         </is>
       </c>
       <c r="C259" s="13" t="inlineStr">
@@ -6814,7 +6814,7 @@
       </c>
       <c r="D259" s="4" t="inlineStr">
         <is>
-          <t>, covering the 10 review points the team raised for RampRate's setup: (1) discard_change; (2) one request = one change with its own branch, PR and drafts, so publishing never takes another request live; (3) a review with pages affected, a server-written "what's included" line and preview links; (4) publish needs the review's reviewToken, and the rules make the AI ask "You are about to publish these changes to the live tonygreenberg.com website. Are you sure you want to continue?"; (5) list_change_history, also visible read-only in Studio under "Website change history" (new adminChange type); (6) undo_change; (7) before/after (automatic for Sanity, given by the AI for code); (8) preview_on_devices phone + laptop screenshots (needs GOOGLE_API_KEY); (9) the AI's plain summary plus the server's facts line; (10) Draft → Ready for review → Published / Discarded. Files: change-sets.ts, change-describe.ts, device-preview.ts, mcp-tool-context.ts, mcp-server.ts, github-client.ts (RampRate's full version), src/sanity/schemas/adminChange.ts, sanity.config.ts. Tested end to end with a real throwaway change, then discarded (see docs/ai/project_mcp_server.md).</t>
+          <t xml:space="preserve"> equal to .env.local; this plan can't limit a variable's scopes, so they're available to builds and functions). Used from the next deploy.</t>
         </is>
       </c>
       <c r="E259" s="14" t="inlineStr">
@@ -6827,7 +6827,7 @@
       <c r="A260" s="4" t="n"/>
       <c r="B260" s="4" t="inlineStr">
         <is>
-          <t>Merge the CI fix into main</t>
+          <t>Per-request change system ported from ramprate-ui (2026-10-02, owner said yes)</t>
         </is>
       </c>
       <c r="C260" s="13" t="inlineStr">
@@ -6837,7 +6837,7 @@
       </c>
       <c r="D260" s="4" t="inlineStr">
         <is>
-          <t>(done with PR #3; checked 2026-10-06: main's pr-lint.yml runs Node 22 and next typegen before the type check). The test change's GitHub check failed because main still has the old pr-lint.yml (Node 20 crash). Every MCP change will fail its site check, and so can't be published, until this branch's work (or at least .github/workflows/pr-lint.yml) is on main. Then test a real publish and undo_change.</t>
+          <t>, covering the 10 review points the team raised for RampRate's setup: (1) discard_change; (2) one request = one change with its own branch, PR and drafts, so publishing never takes another request live; (3) a review with pages affected, a server-written "what's included" line and preview links; (4) publish needs the review's reviewToken, and the rules make the AI ask "You are about to publish these changes to the live tonygreenberg.com website. Are you sure you want to continue?"; (5) list_change_history, also visible read-only in Studio under "Website change history" (new adminChange type); (6) undo_change; (7) before/after (automatic for Sanity, given by the AI for code); (8) preview_on_devices phone + laptop screenshots (needs GOOGLE_API_KEY); (9) the AI's plain summary plus the server's facts line; (10) Draft → Ready for review → Published / Discarded. Files: change-sets.ts, change-describe.ts, device-preview.ts, mcp-tool-context.ts, mcp-server.ts, github-client.ts (RampRate's full version), src/sanity/schemas/adminChange.ts, sanity.config.ts. Tested end to end with a real throwaway change, then discarded (see docs/ai/project_mcp_server.md).</t>
         </is>
       </c>
       <c r="E260" s="14" t="inlineStr">
@@ -6850,7 +6850,7 @@
       <c r="A261" s="4" t="n"/>
       <c r="B261" s="4" t="inlineStr">
         <is>
-          <t>Blocked on you (Google)</t>
+          <t>Merge the CI fix into main</t>
         </is>
       </c>
       <c r="C261" s="13" t="inlineStr">
@@ -6860,7 +6860,7 @@
       </c>
       <c r="D261" s="4" t="inlineStr">
         <is>
-          <t>create a GOOGLE_API_KEY in Google Cloud (project of the vcos-ga4-reader service account, where the PageSpeed Insights API is already on), restricted to the PageSpeed Insights API, then add it to .env.local and Netlify. Creating it from here was blocked by the session's safety check (it would use the service account's credentials to change the Cloud project). Note lighthouse_check_page may time out on Netlify (10 s function limit on the free plan). Dropped 2026-10-13 (owner: "pagespeed.web.dev you can remove"): no Google key or US PageSpeed run needed.</t>
+          <t>(done with PR #3; checked 2026-10-06: main's pr-lint.yml runs Node 22 and next typegen before the type check). The test change's GitHub check failed because main still has the old pr-lint.yml (Node 20 crash). Every MCP change will fail its site check, and so can't be published, until this branch's work (or at least .github/workflows/pr-lint.yml) is on main. Then test a real publish and undo_change.</t>
         </is>
       </c>
       <c r="E261" s="14" t="inlineStr">
@@ -6873,7 +6873,7 @@
       <c r="A262" s="4" t="n"/>
       <c r="B262" s="4" t="inlineStr">
         <is>
-          <t>Synced with ramprate-ui's MCP server (2026-10-09, owner asked; card included by their choice)</t>
+          <t>Blocked on you (Google)</t>
         </is>
       </c>
       <c r="C262" s="13" t="inlineStr">
@@ -6883,7 +6883,7 @@
       </c>
       <c r="D262" s="4" t="inlineStr">
         <is>
-          <t>the review card for ChatGPT/Claude (one status and next step, Build / Type check / Lint / GitHub / phone-and-laptop checks, "what goes live" and what doesn't, Preview / Discard / Publish / Retry, history with Restore); start_change restates the request (understood_as) and unclear ones wait for the person's OK (confirm_change); before (live) / after (preview) screenshots on phone and laptop; attached images and files (ChatGPT file, or request_upload_link, a private 30-minute upload page at /api/mcp/upload, size and real-type checked); every change result lists the other waiting changes and the AI ends its reply with them (new Status Report line); the server lints changed files itself; ESLint now traced into the deployed function (serverExternalPackages; ramprate's tracing globs crash Turbopack under pnpm, left out). Everything named for tonygreenberg.com only (Netlify tonygreenberg-website, live tonygreenberg.com, card ui://tonygreenberg-admin/...). Verified on a local production build: type check, lint, build; 30 tools listed; card served and its script valid; rules include migrationStatus; list_pending_changes returns other pending changes; check_code_quality runs ESLint; upload page refuses bad links (401). See docs/ai/project_mcp_server.md.</t>
+          <t>create a GOOGLE_API_KEY in Google Cloud (project of the vcos-ga4-reader service account, where the PageSpeed Insights API is already on), restricted to the PageSpeed Insights API, then add it to .env.local and Netlify. Creating it from here was blocked by the session's safety check (it would use the service account's credentials to change the Cloud project). Note lighthouse_check_page may time out on Netlify (10 s function limit on the free plan). Dropped 2026-10-13 (owner: "pagespeed.web.dev you can remove"): no Google key or US PageSpeed run needed.</t>
         </is>
       </c>
       <c r="E262" s="14" t="inlineStr">
@@ -6896,63 +6896,63 @@
       <c r="A263" s="4" t="n"/>
       <c r="B263" s="4" t="inlineStr">
         <is>
+          <t>Synced with ramprate-ui's MCP server (2026-10-09, owner asked; card included by their choice)</t>
+        </is>
+      </c>
+      <c r="C263" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D263" s="4" t="inlineStr">
+        <is>
+          <t>the review card for ChatGPT/Claude (one status and next step, Build / Type check / Lint / GitHub / phone-and-laptop checks, "what goes live" and what doesn't, Preview / Discard / Publish / Retry, history with Restore); start_change restates the request (understood_as) and unclear ones wait for the person's OK (confirm_change); before (live) / after (preview) screenshots on phone and laptop; attached images and files (ChatGPT file, or request_upload_link, a private 30-minute upload page at /api/mcp/upload, size and real-type checked); every change result lists the other waiting changes and the AI ends its reply with them (new Status Report line); the server lints changed files itself; ESLint now traced into the deployed function (serverExternalPackages; ramprate's tracing globs crash Turbopack under pnpm, left out). Everything named for tonygreenberg.com only (Netlify tonygreenberg-website, live tonygreenberg.com, card ui://tonygreenberg-admin/...). Verified on a local production build: type check, lint, build; 30 tools listed; card served and its script valid; rules include migrationStatus; list_pending_changes returns other pending changes; check_code_quality runs ESLint; upload page refuses bad links (401). See docs/ai/project_mcp_server.md.</t>
+        </is>
+      </c>
+      <c r="E263" s="14" t="inlineStr">
+        <is>
+          <t>Phase 11 — Code MCP Server — REBUILT (2026-09-29)</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="4" t="n"/>
+      <c r="B264" s="4" t="inlineStr">
+        <is>
           <t>Test the new review end to end on a deploy preview</t>
         </is>
       </c>
-      <c r="C263" s="16" t="inlineStr">
+      <c r="C264" s="16" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
       </c>
-      <c r="D263" s="4" t="inlineStr">
+      <c r="D264" s="4" t="inlineStr">
         <is>
           <t>(needs a yes, it opens a real pull request): one throwaway change from Claude.ai or ChatGPT: start (unclear request, so the confirm step shows), confirm, edit, review card, screenshots, upload link, then discard.</t>
         </is>
       </c>
-      <c r="E263" s="14" t="inlineStr">
+      <c r="E264" s="14" t="inlineStr">
         <is>
           <t>Phase 11 — Code MCP Server — REBUILT (2026-09-29)</t>
         </is>
       </c>
     </row>
-    <row r="264">
-      <c r="A264" s="10" t="inlineStr">
+    <row r="265">
+      <c r="A265" s="10" t="inlineStr">
         <is>
           <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
         </is>
       </c>
-      <c r="B264" s="11" t="n"/>
-      <c r="C264" s="11" t="n"/>
-      <c r="D264" s="12" t="n"/>
-    </row>
-    <row r="265">
-      <c r="A265" s="4" t="n"/>
-      <c r="B265" s="4" t="inlineStr">
-        <is>
-          <t>Per-page generateMetadata (title, description, OG, Twitter Card, canonical) for every ported route, sourced from Sanity seo object where con…</t>
-        </is>
-      </c>
-      <c r="C265" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D265" s="4" t="inlineStr">
-        <is>
-          <t>tent is CMS-backed, static otherwise. Audited all 140 page.tsx files: only /studio has none (correct — it's robots.txt-disallowed, not public content). Real gap found and fixed: /blog/category/[slug] had no alternates.canonical at all, and no page-aware title for its own real pagination (?page=N) — every paginated page was serving an identical title with no canonical, a real duplicate-content signal. Fixed: generateMetadata now reads searchParams too, self-canonicals each page (?page=N pages canonical to themselves, not consolidated to page 1 — genuinely different posts per page, matching Google's current pagination guidance) and appends "— Page N" to the title past page 1. Verified live: page 1 canonicals to the bare URL, ?page=2 canonicals to ?page=2 with a distinct title.</t>
-        </is>
-      </c>
-      <c r="E265" s="14" t="inlineStr">
-        <is>
-          <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
-        </is>
-      </c>
+      <c r="B265" s="11" t="n"/>
+      <c r="C265" s="11" t="n"/>
+      <c r="D265" s="12" t="n"/>
     </row>
     <row r="266">
       <c r="A266" s="4" t="n"/>
       <c r="B266" s="4" t="inlineStr">
         <is>
-          <t>sitemap.ts generated from real Sanity content + static route list, auto-updates on publish</t>
+          <t>Per-page generateMetadata (title, description, OG, Twitter Card, canonical) for every ported route, sourced from Sanity seo object where con…</t>
         </is>
       </c>
       <c r="C266" s="13" t="inlineStr">
@@ -6962,7 +6962,7 @@
       </c>
       <c r="D266" s="4" t="inlineStr">
         <is>
-          <t>Extended from the Phase 5-era version (homepage + blog posts only, 122 URLs) to every real route: the full static route list (130 routes, generated from find src/app -name page.tsx, excluding /studio (robots.txt-disallowed), /(auth)/login (noindex via its own metadata), and /life-assessment (a pure redirect, not distinct content)) plus all 5 real dynamic sources — blog categories (allCategorySlugsQuery), BrewSoul cities (25), BrewSoul coffees (107), and charity-scorecard entries (103) — each pulled from the exact same data source its own page's generateStaticParams already uses, not re-derived. Auto-updates on publish for anything Sanity-backed (blog posts/categories) since it's a live client.fetch on every build; the static route list itself needs a one-line addition whenever a new page ships (same as any other route-registration step). Verified live: 496 real &lt;loc&gt; entries, spot-checked a coffee/city/charity/category URL each, typecheck/lint clean.</t>
+          <t>tent is CMS-backed, static otherwise. Audited all 140 page.tsx files: only /studio has none (correct — it's robots.txt-disallowed, not public content). Real gap found and fixed: /blog/category/[slug] had no alternates.canonical at all, and no page-aware title for its own real pagination (?page=N) — every paginated page was serving an identical title with no canonical, a real duplicate-content signal. Fixed: generateMetadata now reads searchParams too, self-canonicals each page (?page=N pages canonical to themselves, not consolidated to page 1 — genuinely different posts per page, matching Google's current pagination guidance) and appends "— Page N" to the title past page 1. Verified live: page 1 canonicals to the bare URL, ?page=2 canonicals to ?page=2 with a distinct title.</t>
         </is>
       </c>
       <c r="E266" s="14" t="inlineStr">
@@ -6975,7 +6975,7 @@
       <c r="A267" s="4" t="n"/>
       <c r="B267" s="4" t="inlineStr">
         <is>
-          <t>llms.txt</t>
+          <t>sitemap.ts generated from real Sanity content + static route list, auto-updates on publish</t>
         </is>
       </c>
       <c r="C267" s="13" t="inlineStr">
@@ -6985,7 +6985,7 @@
       </c>
       <c r="D267" s="4" t="inlineStr">
         <is>
-          <t>fetched verbatim from the still-live site and saved to web/public/llms.txt (real content: Tony's bio, expertise, full article index by category, every product/tool section) — do this before Manus goes away, it won't be recoverable after</t>
+          <t>Extended from the Phase 5-era version (homepage + blog posts only, 122 URLs) to every real route: the full static route list (130 routes, generated from find src/app -name page.tsx, excluding /studio (robots.txt-disallowed), /(auth)/login (noindex via its own metadata), and /life-assessment (a pure redirect, not distinct content)) plus all 5 real dynamic sources — blog categories (allCategorySlugsQuery), BrewSoul cities (25), BrewSoul coffees (107), and charity-scorecard entries (103) — each pulled from the exact same data source its own page's generateStaticParams already uses, not re-derived. Auto-updates on publish for anything Sanity-backed (blog posts/categories) since it's a live client.fetch on every build; the static route list itself needs a one-line addition whenever a new page ships (same as any other route-registration step). Verified live: 496 real &lt;loc&gt; entries, spot-checked a coffee/city/charity/category URL each, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E267" s="14" t="inlineStr">
@@ -6998,7 +6998,7 @@
       <c r="A268" s="4" t="n"/>
       <c r="B268" s="4" t="inlineStr">
         <is>
-          <t>robots.txt</t>
+          <t>llms.txt</t>
         </is>
       </c>
       <c r="C268" s="13" t="inlineStr">
@@ -7008,7 +7008,7 @@
       </c>
       <c r="D268" s="4" t="inlineStr">
         <is>
-          <t>same approach: fetched the real live file (not my earlier guessed robots.ts, which has been removed) and saved verbatim to web/public/robots.txt, plus added Disallow: /studio for the new Sanity Studio route. Confirmed live: real AI-crawler allowlist (GPTBot, Claude-Web, PerplexityBot, etc.), scraper blocklist, and the site's non-standard LLMs: directive all intact</t>
+          <t>fetched verbatim from the still-live site and saved to web/public/llms.txt (real content: Tony's bio, expertise, full article index by category, every product/tool section) — do this before Manus goes away, it won't be recoverable after</t>
         </is>
       </c>
       <c r="E268" s="14" t="inlineStr">
@@ -7021,7 +7021,7 @@
       <c r="A269" s="4" t="n"/>
       <c r="B269" s="4" t="inlineStr">
         <is>
-          <t>JSON-LD</t>
+          <t>robots.txt</t>
         </is>
       </c>
       <c r="C269" s="13" t="inlineStr">
@@ -7031,7 +7031,7 @@
       </c>
       <c r="D269" s="4" t="inlineStr">
         <is>
-          <t>WebSite + Person schema ported verbatim from the live homepage's actual &lt;script type="application/ld+json"&gt; tags (not reconstructed from memory) — rendered site-wide from src/lib/structured-data.ts in the root layout. The Person image was hardcoded to a /api/img/... legacy proxy path on the live site — rescued that headshot (downloaded it while still live, uploaded to Sanity as the author-tony-greenberg document's avatar) so the new site's JSON-LD has zero Manus dependency instead of just copying the fragile path forward</t>
+          <t>same approach: fetched the real live file (not my earlier guessed robots.ts, which has been removed) and saved verbatim to web/public/robots.txt, plus added Disallow: /studio for the new Sanity Studio route. Confirmed live: real AI-crawler allowlist (GPTBot, Claude-Web, PerplexityBot, etc.), scraper blocklist, and the site's non-standard LLMs: directive all intact</t>
         </is>
       </c>
       <c r="E269" s="14" t="inlineStr">
@@ -7044,7 +7044,7 @@
       <c r="A270" s="4" t="n"/>
       <c r="B270" s="4" t="inlineStr">
         <is>
-          <t>Article JSON-LD on /blog/[slug], built from real per-post Sanity data (headline, image, datePublished/dateModified, author, canonical URL)</t>
+          <t>JSON-LD</t>
         </is>
       </c>
       <c r="C270" s="13" t="inlineStr">
@@ -7054,7 +7054,7 @@
       </c>
       <c r="D270" s="4" t="inlineStr">
         <is>
-          <t>verified live on a real post</t>
+          <t>WebSite + Person schema ported verbatim from the live homepage's actual &lt;script type="application/ld+json"&gt; tags (not reconstructed from memory) — rendered site-wide from src/lib/structured-data.ts in the root layout. The Person image was hardcoded to a /api/img/... legacy proxy path on the live site — rescued that headshot (downloaded it while still live, uploaded to Sanity as the author-tony-greenberg document's avatar) so the new site's JSON-LD has zero Manus dependency instead of just copying the fragile path forward</t>
         </is>
       </c>
       <c r="E270" s="14" t="inlineStr">
@@ -7067,7 +7067,7 @@
       <c r="A271" s="4" t="n"/>
       <c r="B271" s="4" t="inlineStr">
         <is>
-          <t>Build the full Manus/legacy-URL → Next.js-URL 301 redirect map (next.config.ts redirects() or Sanity redirect documents)</t>
+          <t>Article JSON-LD on /blog/[slug], built from real per-post Sanity data (headline, image, datePublished/dateModified, author, canonical URL)</t>
         </is>
       </c>
       <c r="C271" s="13" t="inlineStr">
@@ -7077,7 +7077,7 @@
       </c>
       <c r="D271" s="4" t="inlineStr">
         <is>
-          <t>hard QA gate, nothing proceeds to DNS cutover until this is complete and tested. First real pass done: extracted all 197 real path= routes from legacy's App.tsx router (not guessed — the actual route table), diffed against this app's real current routes (find src/app -maxdepth 1 -name page.tsx) + next.config.ts's existing redirect sources, normalizing :param/[param] syntax to compare like-for-like. Started at 41 real gaps, closed 10 with new redirects: /attention-theft/{blocker-finder,legal,report,weapons} (legacy registered both a bare AND a /attention-theft/-nested path for each, only the bare ones had redirects before), /find-my-car → /find-my, /the-index → /search (matching the fix already applied to other pages' dead links to it), /supplier-intake-long (bare) + /vendor-intake + /vendor-intake-long (+/:token) → the same real ramprate.com/biochain/supplier-intake destination the token'd path already redirected to, and /spamtoast + /youve-been-reported → / (the live half of legacy's "report a spammer" confrontation flow — a fake IP-fingerprinting/countdown-timer page; the other half, ReportSpammer.tsx, was already a documented drop in Phase 4, this is the same call for its sequel). 21 of the remaining 31 gaps need no redirect — they're /admin/*//analytics//edit/frqncy (internal tools never meant for public discovery) or already-documented intentional defers from Phase 4/7/10 (/clock-keeper-part-2, /ecosystem-map, /friend-gate, /friend-survey/:token, /medicine-sequencing, /m</t>
+          <t>verified live on a real post</t>
         </is>
       </c>
       <c r="E271" s="14" t="inlineStr">
@@ -7090,7 +7090,7 @@
       <c r="A272" s="4" t="n"/>
       <c r="B272" s="4" t="inlineStr">
         <is>
-          <t>/path/:archetype (src/app/path/[archetype]/page.tsx)</t>
+          <t>Build the full Manus/legacy-URL → Next.js-URL 301 redirect map (next.config.ts redirects() or Sanity redirect documents)</t>
         </is>
       </c>
       <c r="C272" s="13" t="inlineStr">
@@ -7100,7 +7100,7 @@
       </c>
       <c r="D272" s="4" t="inlineStr">
         <is>
-          <t>per-archetype landing page for /assessment's Builder/Crusader/Investor result, reusing lib/content/archetypes.ts. Real content ported in full (top-5 essential-reading list per archetype via allPostsForArchiveQuery, real PathSubscribeForm posting to /api/subscribe, AUTHORITY_ITEMS strip). Real bug fixed vs. legacy: replaced a hand-rolled inline-styled "Path not found" div with a real notFound() (this route's generateStaticParams only ever produces the 3 real keys). Verified live: all 3 archetype routes 200 OK, typecheck/lint clean.</t>
+          <t>hard QA gate, nothing proceeds to DNS cutover until this is complete and tested. First real pass done: extracted all 197 real path= routes from legacy's App.tsx router (not guessed — the actual route table), diffed against this app's real current routes (find src/app -maxdepth 1 -name page.tsx) + next.config.ts's existing redirect sources, normalizing :param/[param] syntax to compare like-for-like. Started at 41 real gaps, closed 10 with new redirects: /attention-theft/{blocker-finder,legal,report,weapons} (legacy registered both a bare AND a /attention-theft/-nested path for each, only the bare ones had redirects before), /find-my-car → /find-my, /the-index → /search (matching the fix already applied to other pages' dead links to it), /supplier-intake-long (bare) + /vendor-intake + /vendor-intake-long (+/:token) → the same real ramprate.com/biochain/supplier-intake destination the token'd path already redirected to, and /spamtoast + /youve-been-reported → / (the live half of legacy's "report a spammer" confrontation flow — a fake IP-fingerprinting/countdown-timer page; the other half, ReportSpammer.tsx, was already a documented drop in Phase 4, this is the same call for its sequel). 21 of the remaining 31 gaps need no redirect — they're /admin/*//analytics//edit/frqncy (internal tools never meant for public discovery) or already-documented intentional defers from Phase 4/7/10 (/clock-keeper-part-2, /ecosystem-map, /friend-gate, /friend-survey/:token, /medicine-sequencing, /m</t>
         </is>
       </c>
       <c r="E272" s="14" t="inlineStr">
@@ -7113,7 +7113,7 @@
       <c r="A273" s="4" t="n"/>
       <c r="B273" s="4" t="inlineStr">
         <is>
-          <t>/my-journey (src/app/my-journey/page.tsx + components/assessments/my-journey-dashboard.tsx)</t>
+          <t>/path/:archetype (src/app/path/[archetype]/page.tsx)</t>
         </is>
       </c>
       <c r="C273" s="13" t="inlineStr">
@@ -7123,7 +7123,7 @@
       </c>
       <c r="D273" s="4" t="inlineStr">
         <is>
-          <t>"My Journey Dashboard," real grid/timeline views across all 28 JOURNEY_MAP experiences, category/status filters, phase progress ring, recommended-next card, using the same real useJourneyProgress/JOURNEY_MAP completion tracking every "Find Your X" quiz already writes to (not the narrower tg_assessment_results cookie built for /self-portrait). Legacy's per-quiz scored-result caching (RESULT_KEYS, feeding a mini radar chart) was not ported — no quiz in this migration writes that data either, same honest-degradation call already made for /self-portrait's own composite radar. Fixed a real legacy dead link (/ecosystem-map, a still-unbuilt page) to /self-portrait. Verified live: 200 OK, real content confirmed, typecheck/lint clean.</t>
+          <t>per-archetype landing page for /assessment's Builder/Crusader/Investor result, reusing lib/content/archetypes.ts. Real content ported in full (top-5 essential-reading list per archetype via allPostsForArchiveQuery, real PathSubscribeForm posting to /api/subscribe, AUTHORITY_ITEMS strip). Real bug fixed vs. legacy: replaced a hand-rolled inline-styled "Path not found" div with a real notFound() (this route's generateStaticParams only ever produces the 3 real keys). Verified live: all 3 archetype routes 200 OK, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E273" s="14" t="inlineStr">
@@ -7136,7 +7136,7 @@
       <c r="A274" s="4" t="n"/>
       <c r="B274" s="4" t="inlineStr">
         <is>
-          <t>/the-open-door (src/app/the-open-door/page.tsx)</t>
+          <t>/my-journey (src/app/my-journey/page.tsx + components/assessments/my-journey-dashboard.tsx)</t>
         </is>
       </c>
       <c r="C274" s="13" t="inlineStr">
@@ -7146,7 +7146,7 @@
       </c>
       <c r="D274" s="4" t="inlineStr">
         <is>
-          <t>real press/credibility content: all 10 "Magic Genie" client-pitch prompts (real named targets — Marco Argenti/Goldman Sachs, Adam Smith/Disney, etc.), 18 real client testimonials, all 8 explicitly-labeled satirical "parody" quotes (kept with disclaimers, not presented as real). Real overlap found and reconciled: this page's publications/speaking/podcasts arrays substantially duplicate the already-shipped /published's fuller bibliography — kept only what /published doesn't cover (Forbes + Business Insider bylines, the Clinton Global Initiative keynote, 4 of 5 podcast appearances) and cross-linked to /published for the rest, same reconciliation pattern as /assessments vs /find-my. Real bugs fixed: 3 genie/keynote links pointed externally at tonygreenberg.com/&lt;slug&gt; for posts that are real internal posts in this migration — relinked to /blog/psychedelics-could-become-extractive-capitalism, /blog/boiling-the-human-summit-harvard-kurzweil, /blog/return-on-investment-going-green-going-green-2 (all verified 200); a bare self-link to tonygreenberg.com remapped to /. Ships as a pure Server Component (legacy's FadeIn/Section/editorial-component dependencies don't exist here and weren't needed). Verified live: 200 OK, real content in raw SSR HTML, typecheck/lint clean.</t>
+          <t>"My Journey Dashboard," real grid/timeline views across all 28 JOURNEY_MAP experiences, category/status filters, phase progress ring, recommended-next card, using the same real useJourneyProgress/JOURNEY_MAP completion tracking every "Find Your X" quiz already writes to (not the narrower tg_assessment_results cookie built for /self-portrait). Legacy's per-quiz scored-result caching (RESULT_KEYS, feeding a mini radar chart) was not ported — no quiz in this migration writes that data either, same honest-degradation call already made for /self-portrait's own composite radar. Fixed a real legacy dead link (/ecosystem-map, a still-unbuilt page) to /self-portrait. Verified live: 200 OK, real content confirmed, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E274" s="14" t="inlineStr">
@@ -7159,7 +7159,7 @@
       <c r="A275" s="4" t="n"/>
       <c r="B275" s="4" t="inlineStr">
         <is>
-          <t>Homepage "Recent Updates" band (2026-09-29)</t>
+          <t>/the-open-door (src/app/the-open-door/page.tsx)</t>
         </is>
       </c>
       <c r="C275" s="13" t="inlineStr">
@@ -7169,7 +7169,7 @@
       </c>
       <c r="D275" s="4" t="inlineStr">
         <is>
-          <t>on the live site (a newer Blog.tsx than _legacy-manus-app/, so rebuilt from the live page's markup), replacing the older "Latest Thinking" pair. Found while doing it: two live essays are missing from Sanity, the-tollbooth-and-the-alternative (Aug 18, 2026, the live site's newest) and what-quest-could-fix. Both were published on live after the legacy snapshot and need importing.</t>
+          <t>real press/credibility content: all 10 "Magic Genie" client-pitch prompts (real named targets — Marco Argenti/Goldman Sachs, Adam Smith/Disney, etc.), 18 real client testimonials, all 8 explicitly-labeled satirical "parody" quotes (kept with disclaimers, not presented as real). Real overlap found and reconciled: this page's publications/speaking/podcasts arrays substantially duplicate the already-shipped /published's fuller bibliography — kept only what /published doesn't cover (Forbes + Business Insider bylines, the Clinton Global Initiative keynote, 4 of 5 podcast appearances) and cross-linked to /published for the rest, same reconciliation pattern as /assessments vs /find-my. Real bugs fixed: 3 genie/keynote links pointed externally at tonygreenberg.com/&lt;slug&gt; for posts that are real internal posts in this migration — relinked to /blog/psychedelics-could-become-extractive-capitalism, /blog/boiling-the-human-summit-harvard-kurzweil, /blog/return-on-investment-going-green-going-green-2 (all verified 200); a bare self-link to tonygreenberg.com remapped to /. Ships as a pure Server Component (legacy's FadeIn/Section/editorial-component dependencies don't exist here and weren't needed). Verified live: 200 OK, real content in raw SSR HTML, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E275" s="14" t="inlineStr">
@@ -7182,7 +7182,7 @@
       <c r="A276" s="4" t="n"/>
       <c r="B276" s="4" t="inlineStr">
         <is>
-          <t>Re-sync the legacy reference</t>
+          <t>Homepage "Recent Updates" band (2026-09-29)</t>
         </is>
       </c>
       <c r="C276" s="13" t="inlineStr">
@@ -7192,7 +7192,7 @@
       </c>
       <c r="D276" s="4" t="inlineStr">
         <is>
-          <t>_legacy-manus-app/ is older than what's live (Recent Updates proves it), so visual diffs should be against the live site, not only that folder. Closed 2026-10-08: done the way this item suggests: every comparison since 2026-10-01 is against the live site itself (163 pages + 121 posts on 2026-10-01, 188 pages on 2026-10-07, 18 redesigned pages on 2026-10-08), with _legacy-manus-app/ used only as the code reference.</t>
+          <t>on the live site (a newer Blog.tsx than _legacy-manus-app/, so rebuilt from the live page's markup), replacing the older "Latest Thinking" pair. Found while doing it: two live essays are missing from Sanity, the-tollbooth-and-the-alternative (Aug 18, 2026, the live site's newest) and what-quest-could-fix. Both were published on live after the legacy snapshot and need importing.</t>
         </is>
       </c>
       <c r="E276" s="14" t="inlineStr">
@@ -7205,7 +7205,7 @@
       <c r="A277" s="4" t="n"/>
       <c r="B277" s="4" t="inlineStr">
         <is>
-          <t>Visual diff pass: every ported page vs</t>
+          <t>Re-sync the legacy reference</t>
         </is>
       </c>
       <c r="C277" s="13" t="inlineStr">
@@ -7215,7 +7215,7 @@
       </c>
       <c r="D277" s="4" t="inlineStr">
         <is>
-          <t>legacy page Closed 2026-10-08: covered by the live-site sweeps above (screenshots and measured title/label/spacing per page, see the 2026-10-01, 10-02, 10-07 and 10-08 entries in this phase). Remaining differences are listed as decisions (Cormorant titles, /find-my header) or deliberate (CONTRIBUTING rule 20).</t>
+          <t>_legacy-manus-app/ is older than what's live (Recent Updates proves it), so visual diffs should be against the live site, not only that folder. Closed 2026-10-08: done the way this item suggests: every comparison since 2026-10-01 is against the live site itself (163 pages + 121 posts on 2026-10-01, 188 pages on 2026-10-07, 18 redesigned pages on 2026-10-08), with _legacy-manus-app/ used only as the code reference.</t>
         </is>
       </c>
       <c r="E277" s="14" t="inlineStr">
@@ -7228,7 +7228,7 @@
       <c r="A278" s="4" t="n"/>
       <c r="B278" s="4" t="inlineStr">
         <is>
-          <t>Padding / spacing on the story pages matched to live (2026-10-01)</t>
+          <t>Visual diff pass: every ported page vs</t>
         </is>
       </c>
       <c r="C278" s="13" t="inlineStr">
@@ -7238,7 +7238,7 @@
       </c>
       <c r="D278" s="4" t="inlineStr">
         <is>
-          <t>Measured margins, text column and spacing on 31 pages, live vs a production build, at 375px and 1280px. The "door" story pages were the clear mismatch: live's text column is ~546px (ours was 720px), 20px side margins on phones / 40px on desktop, body text 19px/1.8 on phones and 18px/1.85 on desktop (ours 16px/1.5). Fixed on /the-body, /engine-room, /under-nda, /the-nightstand, /the-web, /the-territory, /about, /intel (Intel uses live's 16.8px/1.9; About's hero line 480px max, 18.4px/1.8). Re-measured: all 8 match live to within 2px (About's column 28px narrower), no sideways scroll at 375px.</t>
+          <t>legacy page Closed 2026-10-08: covered by the live-site sweeps above (screenshots and measured title/label/spacing per page, see the 2026-10-01, 10-02, 10-07 and 10-08 entries in this phase). Remaining differences are listed as decisions (Cormorant titles, /find-my header) or deliberate (CONTRIBUTING rule 20).</t>
         </is>
       </c>
       <c r="E278" s="14" t="inlineStr">
@@ -7251,7 +7251,7 @@
       <c r="A279" s="4" t="n"/>
       <c r="B279" s="4" t="inlineStr">
         <is>
-          <t>Header-to-title spacing re-checked (2026-10-02)</t>
+          <t>Padding / spacing on the story pages matched to live (2026-10-01)</t>
         </is>
       </c>
       <c r="C279" s="13" t="inlineStr">
@@ -7261,7 +7261,7 @@
       </c>
       <c r="D279" s="4" t="inlineStr">
         <is>
-          <t>The 2026-10-01 note compared different things: live's header wasn't measured (it showed 0), so "96px vs 168px" was really 161px vs 168px from the top of the page. Measured again from the top of the page, live vs a production build, at 375px and 1280px: most pages were already within 10px. Fixed the real gaps: /the-open-door (now live's dark centered hero band, 56px title, 546px text column; title was 72px too high), /start-here (live's 48px/96px top padding; 25px too high on desktop), /invest and /engage (label spacing and live's 32px/51px title; /invest's desktop title was 36px), /impact-dashboard on phones (card edge to edge under the header like live; title was 89px too low). Re-measured: all within 8px of live, no sideways scroll at 375px, no JS errors.</t>
+          <t>Measured margins, text column and spacing on 31 pages, live vs a production build, at 375px and 1280px. The "door" story pages were the clear mismatch: live's text column is ~546px (ours was 720px), 20px side margins on phones / 40px on desktop, body text 19px/1.8 on phones and 18px/1.85 on desktop (ours 16px/1.5). Fixed on /the-body, /engine-room, /under-nda, /the-nightstand, /the-web, /the-territory, /about, /intel (Intel uses live's 16.8px/1.9; About's hero line 480px max, 18.4px/1.8). Re-measured: all 8 match live to within 2px (About's column 28px narrower), no sideways scroll at 375px.</t>
         </is>
       </c>
       <c r="E279" s="14" t="inlineStr">
@@ -7274,7 +7274,7 @@
       <c r="A280" s="4" t="n"/>
       <c r="B280" s="4" t="inlineStr">
         <is>
-          <t>HumanOS headings in capitals like live (2026-10-02, owner said yes)</t>
+          <t>Header-to-title spacing re-checked (2026-10-02)</t>
         </is>
       </c>
       <c r="C280" s="13" t="inlineStr">
@@ -7284,7 +7284,7 @@
       </c>
       <c r="D280" s="4" t="inlineStr">
         <is>
-          <t>the 4 headings live capitalises on /humanos (title, "Are you a Maximizer...", "Take the Diagnostic", "The Diagnostic") get uppercase; the words are unchanged. The subpages already matched.</t>
+          <t>The 2026-10-01 note compared different things: live's header wasn't measured (it showed 0), so "96px vs 168px" was really 161px vs 168px from the top of the page. Measured again from the top of the page, live vs a production build, at 375px and 1280px: most pages were already within 10px. Fixed the real gaps: /the-open-door (now live's dark centered hero band, 56px title, 546px text column; title was 72px too high), /start-here (live's 48px/96px top padding; 25px too high on desktop), /invest and /engage (label spacing and live's 32px/51px title; /invest's desktop title was 36px), /impact-dashboard on phones (card edge to edge under the header like live; title was 89px too low). Re-measured: all within 8px of live, no sideways scroll at 375px, no JS errors.</t>
         </is>
       </c>
       <c r="E280" s="14" t="inlineStr">
@@ -7297,7 +7297,7 @@
       <c r="A281" s="4" t="n"/>
       <c r="B281" s="4" t="inlineStr">
         <is>
-          <t>More layout gaps matched to live (2026-10-02)</t>
+          <t>HumanOS headings in capitals like live (2026-10-02, owner said yes)</t>
         </is>
       </c>
       <c r="C281" s="13" t="inlineStr">
@@ -7307,7 +7307,7 @@
       </c>
       <c r="D281" s="4" t="inlineStr">
         <is>
-          <t>/series (live's centered 546px column, and a bug fixed: every card kept an empty 240px picture column, squeezing the text; live's per-series picture is one generic placeholder on the Manus proxy, so not copied), /humanos (middle section 900px like live), homepage desktop widths (hero text 804px, Four Doors 1000px, Editor's Picks 1168px, GemSpark edge, section title sizes; live's /blog now shows the homepage), /find-my (photo undimmed and plain background, like live; our site header kept). Re-measured: headings within 3px (/series) to 20px (homepage) of live, no sideways scroll, no JS errors. Note: live's "New here?" tour bar sits over its header and doesn't move the page, so it doesn't affect these numbers.</t>
+          <t>the 4 headings live capitalises on /humanos (title, "Are you a Maximizer...", "Take the Diagnostic", "The Diagnostic") get uppercase; the words are unchanged. The subpages already matched.</t>
         </is>
       </c>
       <c r="E281" s="14" t="inlineStr">
@@ -7320,7 +7320,7 @@
       <c r="A282" s="4" t="n"/>
       <c r="B282" s="4" t="inlineStr">
         <is>
-          <t>Full sweep vs live (2026-10-02)</t>
+          <t>More layout gaps matched to live (2026-10-02)</t>
         </is>
       </c>
       <c r="C282" s="13" t="inlineStr">
@@ -7330,7 +7330,7 @@
       </c>
       <c r="D282" s="4" t="inlineStr">
         <is>
-          <t>142 pages (every non-blog page, 3 of each templated set) at 375px and 1280px, title position, text column, title size. Fixed the shared causes: BrewSoul (live wraps most pages in its frame twice, so a second 52px offset plus the category badge; the landing, cities, directory and quiz pages have neither: src/components/brewsoul/brewsoul-main.tsx; intro paragraphs uncapped like live; 38px titles), Kava (live's extra 52px offset), /the-body, /the-nightstand, /the-web (405px top photo like live), the 6 peptide pages (live's 768/896px intro column), /journeys, /pick-up-the-phone, /published, /ecosystem (546px story column and live's text size). Re-measured: 110 of 120 within 40px / 60px of live.</t>
+          <t>/series (live's centered 546px column, and a bug fixed: every card kept an empty 240px picture column, squeezing the text; live's per-series picture is one generic placeholder on the Manus proxy, so not copied), /humanos (middle section 900px like live), homepage desktop widths (hero text 804px, Four Doors 1000px, Editor's Picks 1168px, GemSpark edge, section title sizes; live's /blog now shows the homepage), /find-my (photo undimmed and plain background, like live; our site header kept). Re-measured: headings within 3px (/series) to 20px (homepage) of live, no sideways scroll, no JS errors. Note: live's "New here?" tour bar sits over its header and doesn't move the page, so it doesn't affect these numbers.</t>
         </is>
       </c>
       <c r="E282" s="14" t="inlineStr">
@@ -7343,7 +7343,7 @@
       <c r="A283" s="4" t="n"/>
       <c r="B283" s="4" t="inlineStr">
         <is>
-          <t>Sweep leftovers fixed (2026-10-06)</t>
+          <t>Full sweep vs live (2026-10-02)</t>
         </is>
       </c>
       <c r="C283" s="13" t="inlineStr">
@@ -7353,7 +7353,7 @@
       </c>
       <c r="D283" s="4" t="inlineStr">
         <is>
-          <t>Ported legacy's exact title sizes, margins and column widths. Measured live vs a production build at 375px and 1280px (H1 distance from the top, H1 size, intro and table widths). Now within 8px and the same title size on /published, /brewsoul/first-sip, /brewsoul/home, /brewsoul/chains (intro 912px like live), /brewsoul/browse, /brewsoul/directory (3-column 952px grid like live), /brewsoul and /brewsoul/quiz (intro 520px), /amplifier (546px column), /diamond-cut, /speaking, /living-declaration, /spirits, /protecting-your-business (tables 730px), and the 5 HumanOS subpages (titles smaller like live, 752px column). No sideways scroll at 375px. Left on purpose: /self-portrait (font matches; our page has a different title and no back link, so it sits 23-57px higher), BrewSoul pages 3-6px off (the shared journey bar row), and the different-layout pages /dharma-finder, /grant-study, /search, /quiz_25q, /soulscore. Also: /brewsoul/quiz rebuilt as a step registry (src/components/brewsoul/brewsoul-quiz/: parent + hook/ + components/step-* + data/), same questions, scoring and look; Back/Skip/Retake use lucide icons. New CONTRIBUTING rule 19 (multi-step flows, FydoPartner pattern). brewsoul-welcome-quiz.tsx (/brewsoul) still has the old shape and text arrows.</t>
+          <t>142 pages (every non-blog page, 3 of each templated set) at 375px and 1280px, title position, text column, title size. Fixed the shared causes: BrewSoul (live wraps most pages in its frame twice, so a second 52px offset plus the category badge; the landing, cities, directory and quiz pages have neither: src/components/brewsoul/brewsoul-main.tsx; intro paragraphs uncapped like live; 38px titles), Kava (live's extra 52px offset), /the-body, /the-nightstand, /the-web (405px top photo like live), the 6 peptide pages (live's 768/896px intro column), /journeys, /pick-up-the-phone, /published, /ecosystem (546px story column and live's text size). Re-measured: 110 of 120 within 40px / 60px of live.</t>
         </is>
       </c>
       <c r="E283" s="14" t="inlineStr">
@@ -7366,7 +7366,7 @@
       <c r="A284" s="4" t="n"/>
       <c r="B284" s="4" t="inlineStr">
         <is>
-          <t>Match live's redesigned pages (2026-10-06, owner said go)</t>
+          <t>Sweep leftovers fixed (2026-10-06)</t>
         </is>
       </c>
       <c r="C284" s="13" t="inlineStr">
@@ -7376,7 +7376,7 @@
       </c>
       <c r="D284" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">/self-portrait (live: dark page, progress ring, "N more brushstrokes" lock until 5 assessments), /grant-study and /dharma-finder (live opens straight on question 1, no intro screen), /quiz_25q (live adds a hero picture above the title; rescue it into Sanity first), /search (live: one search box across essays, BrewSoul, peptides, HumanOS, assessments, kava and pages with filter chips). Measure live vs a production build at 375px and 1280px when done. Done 2026-10-06: /grant-study and /dharma-finder open straight on question 1 like live (title block / part header above the first question, live's 546px column, plain page, credit under every question), both rebuilt as step registries (rule 19); measured within 3px of live at the top (dharma's question block within 7px). /quiz_25q's hero rescued into Sanity and placed like live (within 2px). Found and fixed on the way: on the deployed copy /grant-study's answer buttons could not be clicked (the themed page background was fixed z-0, painted over the quiz); ThemedBackground is now -z-10 pointer-events-none (backgrounds unchanged on all 21 pages that use it), and the shared email gate no longer scrolls sideways on phones. Both quizzes clicked through to results in Chrome and Safari. /self-portrait restyled to live (dark page, "The Composite You", progress ring, "N More Brushstrokes Needed" lock until 5 done, live's copy) on our real cookie data; within 3px of live at both widths; tested with 0, 2 and 6 completed. Counts are ours (13 </t>
+          <t>Ported legacy's exact title sizes, margins and column widths. Measured live vs a production build at 375px and 1280px (H1 distance from the top, H1 size, intro and table widths). Now within 8px and the same title size on /published, /brewsoul/first-sip, /brewsoul/home, /brewsoul/chains (intro 912px like live), /brewsoul/browse, /brewsoul/directory (3-column 952px grid like live), /brewsoul and /brewsoul/quiz (intro 520px), /amplifier (546px column), /diamond-cut, /speaking, /living-declaration, /spirits, /protecting-your-business (tables 730px), and the 5 HumanOS subpages (titles smaller like live, 752px column). No sideways scroll at 375px. Left on purpose: /self-portrait (font matches; our page has a different title and no back link, so it sits 23-57px higher), BrewSoul pages 3-6px off (the shared journey bar row), and the different-layout pages /dharma-finder, /grant-study, /search, /quiz_25q, /soulscore. Also: /brewsoul/quiz rebuilt as a step registry (src/components/brewsoul/brewsoul-quiz/: parent + hook/ + components/step-* + data/), same questions, scoring and look; Back/Skip/Retake use lucide icons. New CONTRIBUTING rule 19 (multi-step flows, FydoPartner pattern). brewsoul-welcome-quiz.tsx (/brewsoul) still has the old shape and text arrows.</t>
         </is>
       </c>
       <c r="E284" s="14" t="inlineStr">
@@ -7389,7 +7389,7 @@
       <c r="A285" s="4" t="n"/>
       <c r="B285" s="4" t="inlineStr">
         <is>
-          <t>Still different from live (decided 2026-10-09)</t>
+          <t>Match live's redesigned pages (2026-10-06, owner said go)</t>
         </is>
       </c>
       <c r="C285" s="13" t="inlineStr">
@@ -7399,7 +7399,7 @@
       </c>
       <c r="D285" s="4" t="inlineStr">
         <is>
-          <t>blog posts (done) (done 2026-10-07, see Phase 5); /find-my on live hides the site header. /walk-through is a 404 on live now. Owner: keep our site menu on /find-my (visitors can still reach the rest of the site); nothing left to change.</t>
+          <t xml:space="preserve">/self-portrait (live: dark page, progress ring, "N more brushstrokes" lock until 5 assessments), /grant-study and /dharma-finder (live opens straight on question 1, no intro screen), /quiz_25q (live adds a hero picture above the title; rescue it into Sanity first), /search (live: one search box across essays, BrewSoul, peptides, HumanOS, assessments, kava and pages with filter chips). Measure live vs a production build at 375px and 1280px when done. Done 2026-10-06: /grant-study and /dharma-finder open straight on question 1 like live (title block / part header above the first question, live's 546px column, plain page, credit under every question), both rebuilt as step registries (rule 19); measured within 3px of live at the top (dharma's question block within 7px). /quiz_25q's hero rescued into Sanity and placed like live (within 2px). Found and fixed on the way: on the deployed copy /grant-study's answer buttons could not be clicked (the themed page background was fixed z-0, painted over the quiz); ThemedBackground is now -z-10 pointer-events-none (backgrounds unchanged on all 21 pages that use it), and the shared email gate no longer scrolls sideways on phones. Both quizzes clicked through to results in Chrome and Safari. /self-portrait restyled to live (dark page, "The Composite You", progress ring, "N More Brushstrokes Needed" lock until 5 done, live's copy) on our real cookie data; within 3px of live at both widths; tested with 0, 2 and 6 completed. Counts are ours (13 </t>
         </is>
       </c>
       <c r="E285" s="14" t="inlineStr">
@@ -7412,7 +7412,7 @@
       <c r="A286" s="4" t="n"/>
       <c r="B286" s="4" t="inlineStr">
         <is>
-          <t>Design change on live (owner: "match live", 2026-10-09)</t>
+          <t>Still different from live (decided 2026-10-09)</t>
         </is>
       </c>
       <c r="C286" s="13" t="inlineStr">
@@ -7422,7 +7422,7 @@
       </c>
       <c r="D286" s="4" t="inlineStr">
         <is>
-          <t>live's story pages now use Cormorant Garamond for titles (ours: Playfair Display), a lighter title weight (400 vs our 700), and a red eyebrow label (#8E1E25, wider letter spacing) instead of our gold. A site-wide font swap is a design call, so not done. Done 2026-10-09: a fresh sweep of 163 live pages found live has since dropped Cormorant from the story pages (only /living-declaration uses it, ours already matched) and mostly uses Playfair; the real differences were fixed: every heading on /attention-theft in Fraunces 700 (section-wide, like Kava), /supplier-intake title in the system serif, and live's fluid title sizes on /about, /articles, /the-letter, /the-philosophy, /clock-keeper-part-2, /living-declaration (measured at 375/640/820/1024/1280, now identical). Label colours stay darker than live on purpose (contrast, rule 20).</t>
+          <t>blog posts (done) (done 2026-10-07, see Phase 5); /find-my on live hides the site header. /walk-through is a 404 on live now. Owner: keep our site menu on /find-my (visitors can still reach the rest of the site); nothing left to change.</t>
         </is>
       </c>
       <c r="E286" s="14" t="inlineStr">
@@ -7435,7 +7435,7 @@
       <c r="A287" s="4" t="n"/>
       <c r="B287" s="4" t="inlineStr">
         <is>
-          <t>Link check across all ported pages (no 404s, no broken internal cross-references)</t>
+          <t>Design change on live (owner: "match live", 2026-10-09)</t>
         </is>
       </c>
       <c r="C287" s="13" t="inlineStr">
@@ -7445,7 +7445,7 @@
       </c>
       <c r="D287" s="4" t="inlineStr">
         <is>
-          <t>First full pass done 2026-09-29 (510 pages crawled from the sitemap plus every internal link, on a production build). Fixed in code: /brewsoul/coffee/…-tarrazú 404 (the route got the id still percent-encoded), 30+ links that went through the /assessments/* redirects, /find-your-me's dead Homeaglow link, the two root-level Iboga essay links, and the dead FauxTony nav item. Fixed as Sanity drafts (scripts/fix-blog-body-links.ts, 14 posts): broken post links, leaked !… placeholder text, Energy Is Money's split author bio, and scraped WordPress furniture ("Share this / Related / You Might Also Like / Copyright", "Show More / Top News", [mc4wp_form]). Left for a decision: /framework's "Ask FauxTony" button, when-healing-becomes-extraction's two links to a Dr. Lee case file that doesn't exist, and the-clock-keeper-chronicles-part-1's link to the deferred /clock-keeper-part-2. Re-run after the drafts are published. 2026-10-01 re-run (local production build, all 498 sitemap URLs load; 440 unique internal links): 5 broken. Fixed as a Sanity draft: molecule-as-mirror-10-what-the-pioneers-know's "Final installment" link pointed at a non-existent part-10 slug (now part 11; live also shows that line twice, kept). Already fixed in a waiting draft: forever-chemicals-... → /blog/psychedelic-readiness-index. Still the 3 known decisions: /fauxtony (from /framework), /clock-keeper-part-2, /blog/the-case-file-dr-samuel-lee. 2026-10-08 re-run (production build, all 497 sitemap pages, 453 unique i</t>
+          <t>live's story pages now use Cormorant Garamond for titles (ours: Playfair Display), a lighter title weight (400 vs our 700), and a red eyebrow label (#8E1E25, wider letter spacing) instead of our gold. A site-wide font swap is a design call, so not done. Done 2026-10-09: a fresh sweep of 163 live pages found live has since dropped Cormorant from the story pages (only /living-declaration uses it, ours already matched) and mostly uses Playfair; the real differences were fixed: every heading on /attention-theft in Fraunces 700 (section-wide, like Kava), /supplier-intake title in the system serif, and live's fluid title sizes on /about, /articles, /the-letter, /the-philosophy, /clock-keeper-part-2, /living-declaration (measured at 375/640/820/1024/1280, now identical). Label colours stay darker than live on purpose (contrast, rule 20).</t>
         </is>
       </c>
       <c r="E287" s="14" t="inlineStr">
@@ -7458,7 +7458,7 @@
       <c r="A288" s="4" t="n"/>
       <c r="B288" s="4" t="inlineStr">
         <is>
-          <t>Sitemap: no noindex pages (2026-10-08)</t>
+          <t>Link check across all ported pages (no 404s, no broken internal cross-references)</t>
         </is>
       </c>
       <c r="C288" s="13" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="D288" s="4" t="inlineStr">
         <is>
-          <t>the password-locked /blog/you-are-the-moat was in the sitemap while telling Google not to index it (a Search Console sitemap warning). Gated posts and posts that redirect are now left out (src/app/sitemap.ts); all 497 sitemap addresses return 200 with a matching canonical and no noindex. The 82 warnings Search Console shows are for the old live sitemap, so re-check them after cutover.</t>
+          <t>First full pass done 2026-09-29 (510 pages crawled from the sitemap plus every internal link, on a production build). Fixed in code: /brewsoul/coffee/…-tarrazú 404 (the route got the id still percent-encoded), 30+ links that went through the /assessments/* redirects, /find-your-me's dead Homeaglow link, the two root-level Iboga essay links, and the dead FauxTony nav item. Fixed as Sanity drafts (scripts/fix-blog-body-links.ts, 14 posts): broken post links, leaked !… placeholder text, Energy Is Money's split author bio, and scraped WordPress furniture ("Share this / Related / You Might Also Like / Copyright", "Show More / Top News", [mc4wp_form]). Left for a decision: /framework's "Ask FauxTony" button, when-healing-becomes-extraction's two links to a Dr. Lee case file that doesn't exist, and the-clock-keeper-chronicles-part-1's link to the deferred /clock-keeper-part-2. Re-run after the drafts are published. 2026-10-01 re-run (local production build, all 498 sitemap URLs load; 440 unique internal links): 5 broken. Fixed as a Sanity draft: molecule-as-mirror-10-what-the-pioneers-know's "Final installment" link pointed at a non-existent part-10 slug (now part 11; live also shows that line twice, kept). Already fixed in a waiting draft: forever-chemicals-... → /blog/psychedelic-readiness-index. Still the 3 known decisions: /fauxtony (from /framework), /clock-keeper-part-2, /blog/the-case-file-dr-samuel-lee. 2026-10-08 re-run (production build, all 497 sitemap pages, 453 unique i</t>
         </is>
       </c>
       <c r="E288" s="14" t="inlineStr">
@@ -7481,7 +7481,7 @@
       <c r="A289" s="4" t="n"/>
       <c r="B289" s="4" t="inlineStr">
         <is>
-          <t>Lighthouse pass (performance/accessibility/SEO) on top 20 pages by traffic 2026-09-30, 20 key pages (no traffic data yet), local production …</t>
+          <t>Sitemap: no noindex pages (2026-10-08)</t>
         </is>
       </c>
       <c r="C289" s="13" t="inlineStr">
@@ -7491,7 +7491,7 @@
       </c>
       <c r="D289" s="4" t="inlineStr">
         <is>
-          <t>build, mobile: averages performance 87, accessibility 99→100, best practices 100, SEO 92→100, CLS 0 everywhere. Fixed: public/robots.txt had an LLMs: line (not a real directive) that made Google treat the whole file as invalid, now a comment; h3/h4 headings skipping a level on /assessments, /kava, /peptide-watch (same look, right tag); the Kava and /attention-theft back-arrow links had no accessible name on phones; two small phone-width contrast misses. Left: performance is local-machine only (±10-15 points, see CONTRIBUTING.md); the slowest were / 76 (LCP 5.2 s), /psychedelic-readiness-index 82, /iboga-ibogaine 83. Re-run against the Netlify deploy before launch. 2026-10-06 re-run against the Netlify deploy (14 key pages, mobile): accessibility 100 and CLS 0 on every page, SEO clean (only the expected netlify.app noindex), performance 77-97 held back by 3-4 s LCP. Fixed: all 21 hero images moved off the deprecated priority prop to fetchPriority="high" + loading="eager" (Next 16); /iboga-ibogaine hero and the first card on /blog and category pages no longer lazy-loaded; sizes on the Four Doors cards (~150 KiB per page), /humanos diagram (~100 KiB) and /about headshot; urlFor no longer imports the Sanity client, so ~115 KB of Sanity client code stopped loading on / and /blog; React hydration error #418 on / and /blog (post dates) gone, checked in two time zones; /blog is static again; empty icon &lt;th&gt;s on /iboga-ibogaine labelled; category page reads use sanityFetch(). Left: se</t>
+          <t>the password-locked /blog/you-are-the-moat was in the sitemap while telling Google not to index it (a Search Console sitemap warning). Gated posts and posts that redirect are now left out (src/app/sitemap.ts); all 497 sitemap addresses return 200 with a matching canonical and no noindex. The 82 warnings Search Console shows are for the old live sitemap, so re-check them after cutover.</t>
         </is>
       </c>
       <c r="E289" s="14" t="inlineStr">
@@ -7504,7 +7504,7 @@
       <c r="A290" s="4" t="n"/>
       <c r="B290" s="4" t="inlineStr">
         <is>
-          <t>No Manus links anywhere (2026-10-09, owner: "drop them everywhere")</t>
+          <t>Lighthouse pass (performance/accessibility/SEO) on top 20 pages by traffic 2026-09-30, 20 key pages (no traffic data yet), local production …</t>
         </is>
       </c>
       <c r="C290" s="13" t="inlineStr">
@@ -7514,7 +7514,7 @@
       </c>
       <c r="D290" s="4" t="inlineStr">
         <is>
-          <t>every *.manus.space link removed from code and essays. Lists of "try this next" apps lose those entries (journey tracker, Find Your Me results and next steps, /find-my, search directory, Sake and Grant Study results, BrewSoul footer, The Mirror); The Magnetic Partner's and The Temple Keeper's next step now go to their first in-site assessment (/grant-study, /consciousness-scale); their empty "Find Your _" section hides itself; /recent-creations, /spirits and /ecosystem-map keep the cards, unlinked. Clarisse Abelarde now links to her own site clarisseartist.com (owner gave it) on /about and in essays. Essays: lib/sanity/portable-text.tsx rewrites tonygreenberg.manus.space/&lt;path&gt; to /&lt;path&gt;, clarisseart.manus.space to clarisseartist.com (same paths), and renders other Manus app links as plain text (no Sanity drafts). Verified on a production build: no clickable *.manus.space link in any page, no manus.space in any browser script; 13 affected pages load (200).</t>
+          <t>build, mobile: averages performance 87, accessibility 99→100, best practices 100, SEO 92→100, CLS 0 everywhere. Fixed: public/robots.txt had an LLMs: line (not a real directive) that made Google treat the whole file as invalid, now a comment; h3/h4 headings skipping a level on /assessments, /kava, /peptide-watch (same look, right tag); the Kava and /attention-theft back-arrow links had no accessible name on phones; two small phone-width contrast misses. Left: performance is local-machine only (±10-15 points, see CONTRIBUTING.md); the slowest were / 76 (LCP 5.2 s), /psychedelic-readiness-index 82, /iboga-ibogaine 83. Re-run against the Netlify deploy before launch. 2026-10-06 re-run against the Netlify deploy (14 key pages, mobile): accessibility 100 and CLS 0 on every page, SEO clean (only the expected netlify.app noindex), performance 77-97 held back by 3-4 s LCP. Fixed: all 21 hero images moved off the deprecated priority prop to fetchPriority="high" + loading="eager" (Next 16); /iboga-ibogaine hero and the first card on /blog and category pages no longer lazy-loaded; sizes on the Four Doors cards (~150 KiB per page), /humanos diagram (~100 KiB) and /about headshot; urlFor no longer imports the Sanity client, so ~115 KB of Sanity client code stopped loading on / and /blog; React hydration error #418 on / and /blog (post dates) gone, checked in two time zones; /blog is static again; empty icon &lt;th&gt;s on /iboga-ibogaine labelled; category page reads use sanityFetch(). Left: se</t>
         </is>
       </c>
       <c r="E290" s="14" t="inlineStr">
@@ -7527,7 +7527,7 @@
       <c r="A291" s="4" t="n"/>
       <c r="B291" s="4" t="inlineStr">
         <is>
-          <t>Owner answers, round 2 (2026-10-09)</t>
+          <t>No Manus links anywhere (2026-10-09, owner: "drop them everywhere")</t>
         </is>
       </c>
       <c r="C291" s="13" t="inlineStr">
@@ -7537,7 +7537,7 @@
       </c>
       <c r="D291" s="4" t="inlineStr">
         <is>
-          <t>(1) real counts instead of live's typed numbers: /charity-scorecard intro and description ("98"/"Ninety-eight" → STATS.totalCharities = 103), /impact-dashboard ("100" → passed in from the page so the browser doesn't load the charity list), /the-index (prop), search directory coffees 103 → 107 (typed, with a note, since it ships to the search pop-up); (2) The Mirror results no longer list the 4 *.manus.space apps (the "Explore further" section hides when empty); (3) /framework's "Ask FauxTony" button and its lead-in line removed; the Dr. Lee case-file link (4 places in when-healing-becomes-extraction, original and updated versions) renders as plain text through a DEAD_INTERNAL_LINKS list in lib/sanity/portable-text.tsx (no Sanity draft needed); (4) B Corp: checked live, nothing shown on either site, no change. Verified on a production build: the counts read 103, /framework has no FauxTony block, the essay has 0 links to the case file and keeps the words, /the-index shows "103 charities" when searching "charity".</t>
+          <t>every *.manus.space link removed from code and essays. Lists of "try this next" apps lose those entries (journey tracker, Find Your Me results and next steps, /find-my, search directory, Sake and Grant Study results, BrewSoul footer, The Mirror); The Magnetic Partner's and The Temple Keeper's next step now go to their first in-site assessment (/grant-study, /consciousness-scale); their empty "Find Your _" section hides itself; /recent-creations, /spirits and /ecosystem-map keep the cards, unlinked. Clarisse Abelarde now links to her own site clarisseartist.com (owner gave it) on /about and in essays. Essays: lib/sanity/portable-text.tsx rewrites tonygreenberg.manus.space/&lt;path&gt; to /&lt;path&gt;, clarisseart.manus.space to clarisseartist.com (same paths), and renders other Manus app links as plain text (no Sanity drafts). Verified on a production build: no clickable *.manus.space link in any page, no manus.space in any browser script; 13 affected pages load (200).</t>
         </is>
       </c>
       <c r="E291" s="14" t="inlineStr">
@@ -7550,7 +7550,7 @@
       <c r="A292" s="4" t="n"/>
       <c r="B292" s="4" t="inlineStr">
         <is>
-          <t>Arrows in buttons and links are icons (2026-10-09, owner said yes)</t>
+          <t>Owner answers, round 2 (2026-10-09)</t>
         </is>
       </c>
       <c r="C292" s="13" t="inlineStr">
@@ -7560,7 +7560,7 @@
       </c>
       <c r="D292" s="4" t="inlineStr">
         <is>
-          <t>113 typed arrows in 52 files (button and link labels, "Next"/"See My Results" toggles, decorative arrow spans, the walk-through "See the..." labels, the Letter's "I'm in" button) replaced with lucide ArrowRight/ArrowLeft (size-[1em], inside inline-flex items-center gap-1.5, so the parent layout is untouched). Left as content on purpose: arrows inside Tony's text and data (health findings, origins, iboga compass options, process flows like "Inherit → Wake → Choose → Act", share text), the "← you" marker on the consciousness scale, and &lt;option&gt; sort labels (an option can't hold an icon). Checked on 16 pages at 375 and 1280: no typed arrow left in any link or button, no sideways scroll, no JS errors; close-up screenshots of the new icons.</t>
+          <t>(1) real counts instead of live's typed numbers: /charity-scorecard intro and description ("98"/"Ninety-eight" → STATS.totalCharities = 103), /impact-dashboard ("100" → passed in from the page so the browser doesn't load the charity list), /the-index (prop), search directory coffees 103 → 107 (typed, with a note, since it ships to the search pop-up); (2) The Mirror results no longer list the 4 *.manus.space apps (the "Explore further" section hides when empty); (3) /framework's "Ask FauxTony" button and its lead-in line removed; the Dr. Lee case-file link (4 places in when-healing-becomes-extraction, original and updated versions) renders as plain text through a DEAD_INTERNAL_LINKS list in lib/sanity/portable-text.tsx (no Sanity draft needed); (4) B Corp: checked live, nothing shown on either site, no change. Verified on a production build: the counts read 103, /framework has no FauxTony block, the essay has 0 links to the case file and keeps the words, /the-index shows "103 charities" when searching "charity".</t>
         </is>
       </c>
       <c r="E292" s="14" t="inlineStr">
@@ -7573,7 +7573,7 @@
       <c r="A293" s="4" t="n"/>
       <c r="B293" s="4" t="inlineStr">
         <is>
-          <t>Category pages pre-built (2026-10-09)</t>
+          <t>Arrows in buttons and links are icons (2026-10-09, owner said yes)</t>
         </is>
       </c>
       <c r="C293" s="13" t="inlineStr">
@@ -7583,7 +7583,7 @@
       </c>
       <c r="D293" s="4" t="inlineStr">
         <is>
-          <t>/blog/category/[slug] read ?page=N, so every category page was rendered on each request (slower first byte, flagged in the Lighthouse notes). Page numbers are now part of the address (/blog/category/&lt;slug&gt;/page/&lt;n&gt;, generateStaticParams, dynamicParams = false), shared code in src/components/blog/category-listing.tsx; old ?page=N links 308 to the new address (pages 2+ only, so no loop), /page/1 308s to the plain address, a page past the end is a 404; "All essays" back link uses an icon. Verified on a production build: route table shows every category page as pre-built (9 page-1s, 7 later pages), titles and canonicals per page, Previous/Next links, the redirects and the 404s.</t>
+          <t>113 typed arrows in 52 files (button and link labels, "Next"/"See My Results" toggles, decorative arrow spans, the walk-through "See the..." labels, the Letter's "I'm in" button) replaced with lucide ArrowRight/ArrowLeft (size-[1em], inside inline-flex items-center gap-1.5, so the parent layout is untouched). Left as content on purpose: arrows inside Tony's text and data (health findings, origins, iboga compass options, process flows like "Inherit → Wake → Choose → Act", share text), the "← you" marker on the consciousness scale, and &lt;option&gt; sort labels (an option can't hold an icon). Checked on 16 pages at 375 and 1280: no typed arrow left in any link or button, no sideways scroll, no JS errors; close-up screenshots of the new icons.</t>
         </is>
       </c>
       <c r="E293" s="14" t="inlineStr">
@@ -7596,7 +7596,7 @@
       <c r="A294" s="4" t="n"/>
       <c r="B294" s="4" t="inlineStr">
         <is>
-          <t>Error pages (2026-10-09, owner asked)</t>
+          <t>Category pages pre-built (2026-10-09)</t>
         </is>
       </c>
       <c r="C294" s="13" t="inlineStr">
@@ -7606,7 +7606,7 @@
       </c>
       <c r="D294" s="4" t="inlineStr">
         <is>
-          <t>404 page now sets its own title ("Page not found") as a server page around live's 3-second redirect (not-found.tsx + components/not-found-redirect.tsx), arrow as an icon; page error screen (error.tsx) uses Next 16's retry (re-fetches), shows a reference code for the server logs, links home and to the site index; new global-error.tsx for failures in the root layout itself (own &lt;html&gt;, plain links). Verified on a production build: missing page, missing essay and missing Kava page return 404 with the right title; a test page that throws returns 500 with the error screen, "Try again" re-fetches; phone and laptop, no sideways scroll (test page removed).</t>
+          <t>/blog/category/[slug] read ?page=N, so every category page was rendered on each request (slower first byte, flagged in the Lighthouse notes). Page numbers are now part of the address (/blog/category/&lt;slug&gt;/page/&lt;n&gt;, generateStaticParams, dynamicParams = false), shared code in src/components/blog/category-listing.tsx; old ?page=N links 308 to the new address (pages 2+ only, so no loop), /page/1 308s to the plain address, a page past the end is a 404; "All essays" back link uses an icon. Verified on a production build: route table shows every category page as pre-built (9 page-1s, 7 later pages), titles and canonicals per page, Previous/Next links, the redirects and the 404s.</t>
         </is>
       </c>
       <c r="E294" s="14" t="inlineStr">
@@ -7619,7 +7619,7 @@
       <c r="A295" s="4" t="n"/>
       <c r="B295" s="4" t="inlineStr">
         <is>
-          <t>SEO audit fixes (2026-10-06)</t>
+          <t>Error pages (2026-10-09, owner asked)</t>
         </is>
       </c>
       <c r="C295" s="13" t="inlineStr">
@@ -7629,7 +7629,7 @@
       </c>
       <c r="D295" s="4" t="inlineStr">
         <is>
-          <t>Checked an outside audit point by point against the code. Fixed: Core Themes cards linked to /?theme=…#essays-archive (not crawlable, counts from a stale hand-kept list) and now link to /blog/category/&lt;slug&gt; with real counts (21/25/20/14, matching the archive pills; THEME_MAP and the ?theme= filter removed); Four Doors cards were &lt;button&gt;s, now real links that still open the modal on a plain click; "DIAGNOSE · ENGAGE" now link to /find-my and /engage; one shared formatPostDate (Asia/Kolkata, src/lib/format-post-date.ts) so a post no longer shows two different dates; the title repeated as the first body paragraph is dropped at render time (legacyBodyLayout); essay cards are h3 under a section h2 (archive, Read next), h2 only on category/search; heading glyphs (◆ ✦) hidden from screen readers; posts send BlogPosting with the author tied to the site Person (@id) plus a BreadcrumbList; descriptive alt on the homepage and BrewSoul heroes; homepage OG image cropped to 1200x630 JPEG. Already fine (audit could not see it): Person/Article schema, Netlify noindex, robots.txt, sitemap, header nav and search, Amazon links carry no affiliate tag. Checked on a production build: type check, lint, build, status codes, browser click test at 375px, no console errors. Implementation pack (Mohammad Danish, 2026-10-05) checked the same day: added og:type/og:site_name back on the 6 pages with their own openGraph (a page-level openGraph replaces the layout one), twitter:creator, and on posts og:url</t>
+          <t>404 page now sets its own title ("Page not found") as a server page around live's 3-second redirect (not-found.tsx + components/not-found-redirect.tsx), arrow as an icon; page error screen (error.tsx) uses Next 16's retry (re-fetches), shows a reference code for the server logs, links home and to the site index; new global-error.tsx for failures in the root layout itself (own &lt;html&gt;, plain links). Verified on a production build: missing page, missing essay and missing Kava page return 404 with the right title; a test page that throws returns 500 with the error screen, "Try again" re-fetches; phone and laptop, no sideways scroll (test page removed).</t>
         </is>
       </c>
       <c r="E295" s="14" t="inlineStr">
@@ -7642,7 +7642,7 @@
       <c r="A296" s="4" t="n"/>
       <c r="B296" s="4" t="inlineStr">
         <is>
-          <t>SEO audit items needing a yes (2026-10-06; owner said yes to the copy 2026-10-10, done)</t>
+          <t>SEO audit fixes (2026-10-06)</t>
         </is>
       </c>
       <c r="C296" s="13" t="inlineStr">
@@ -7652,7 +7652,7 @@
       </c>
       <c r="D296" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">the pack's new copy (homepage title/description, five-cups title, description, short answer, FAQ, heading rewrites, entity statement, newsletter block, author box, health disclaimer, COA wording); "Further Reading" shown twice on posts (merge the lists?); long post title (84 chars), homepage description length and obsolete keywords tag, slugs (/blog/five-cups, the -2 slug; would need redirects), "Six lenses" over four cards, sources for health claims and proof for "$10B+", "Certified B Corp", "Validity: 91", legal review of the homepage Case File banner, ABIT waitlist disclosures, one contact email, the two one-post categories, fewer homepage CTAs / email signup / table of contents / explaining "COA". Done 2026-10-10: homepage title "Tony Greenberg | Strategist, Author &amp; CEO of RampRate" and description (essay count computed: 123); entity statement under the hero (107 coffees / 100 chains computed from the data) with a link to /ecosystem; door 4 "Certificate of Analysis (COA) checks, lab testing and vendor scoring"; "Four lenses" (computed); newsletter box after Editor's Picks (existing Kit form); meta keywords removed site-wide; every essay: author line + "About Tony", one merged "Further Reading", optional lastUpdated field shown as "Updated &lt;date&gt;" (not set on any post yet: every _updatedAt is the import date), health disclaimer on 20 personal-health essays (chosen by Sanity tag); Five Cups (Sanity, published, backup kept): SEO title/description, short answer, visible FAQ </t>
+          <t>Checked an outside audit point by point against the code. Fixed: Core Themes cards linked to /?theme=…#essays-archive (not crawlable, counts from a stale hand-kept list) and now link to /blog/category/&lt;slug&gt; with real counts (21/25/20/14, matching the archive pills; THEME_MAP and the ?theme= filter removed); Four Doors cards were &lt;button&gt;s, now real links that still open the modal on a plain click; "DIAGNOSE · ENGAGE" now link to /find-my and /engage; one shared formatPostDate (Asia/Kolkata, src/lib/format-post-date.ts) so a post no longer shows two different dates; the title repeated as the first body paragraph is dropped at render time (legacyBodyLayout); essay cards are h3 under a section h2 (archive, Read next), h2 only on category/search; heading glyphs (◆ ✦) hidden from screen readers; posts send BlogPosting with the author tied to the site Person (@id) plus a BreadcrumbList; descriptive alt on the homepage and BrewSoul heroes; homepage OG image cropped to 1200x630 JPEG. Already fine (audit could not see it): Person/Article schema, Netlify noindex, robots.txt, sitemap, header nav and search, Amazon links carry no affiliate tag. Checked on a production build: type check, lint, build, status codes, browser click test at 375px, no console errors. Implementation pack (Mohammad Danish, 2026-10-05) checked the same day: added og:type/og:site_name back on the 6 pages with their own openGraph (a page-level openGraph replaces the layout one), twitter:creator, and on posts og:url</t>
         </is>
       </c>
       <c r="E296" s="14" t="inlineStr">
@@ -7665,7 +7665,7 @@
       <c r="A297" s="4" t="n"/>
       <c r="B297" s="4" t="inlineStr">
         <is>
-          <t>Google Analytics tag (found missing 2026-10-10, added the same day)</t>
+          <t>SEO audit items needing a yes (2026-10-06; owner said yes to the copy 2026-10-10, done)</t>
         </is>
       </c>
       <c r="C297" s="13" t="inlineStr">
@@ -7675,7 +7675,7 @@
       </c>
       <c r="D297" s="4" t="inlineStr">
         <is>
-          <t>Live loads GA4 G-4GVW40S47N; the new site sent nothing, so stats would have stopped at cutover. Added src/components/google-analytics.tsx (plain next/script, no new package) in the root layout; it only runs on tonygreenberg.com / www, so Netlify previews and localhost never reach the real reports. Checked: type check, lint, build; in Chromium with Google's requests blocked: localhost sends nothing, tonygreenberg.com (mapped to a local production build) loads the tag on / and /find-your-coffee, no JS errors. In-site page changes are counted by GA4's Enhanced measurement (on by default; confirm in GA4 &gt; Admin &gt; Data streams on launch day).</t>
+          <t xml:space="preserve">the pack's new copy (homepage title/description, five-cups title, description, short answer, FAQ, heading rewrites, entity statement, newsletter block, author box, health disclaimer, COA wording); "Further Reading" shown twice on posts (merge the lists?); long post title (84 chars), homepage description length and obsolete keywords tag, slugs (/blog/five-cups, the -2 slug; would need redirects), "Six lenses" over four cards, sources for health claims and proof for "$10B+", "Certified B Corp", "Validity: 91", legal review of the homepage Case File banner, ABIT waitlist disclosures, one contact email, the two one-post categories, fewer homepage CTAs / email signup / table of contents / explaining "COA". Done 2026-10-10: homepage title "Tony Greenberg | Strategist, Author &amp; CEO of RampRate" and description (essay count computed: 123); entity statement under the hero (107 coffees / 100 chains computed from the data) with a link to /ecosystem; door 4 "Certificate of Analysis (COA) checks, lab testing and vendor scoring"; "Four lenses" (computed); newsletter box after Editor's Picks (existing Kit form); meta keywords removed site-wide; every essay: author line + "About Tony", one merged "Further Reading", optional lastUpdated field shown as "Updated &lt;date&gt;" (not set on any post yet: every _updatedAt is the import date), health disclaimer on 20 personal-health essays (chosen by Sanity tag); Five Cups (Sanity, published, backup kept): SEO title/description, short answer, visible FAQ </t>
         </is>
       </c>
       <c r="E297" s="14" t="inlineStr">
@@ -7688,7 +7688,7 @@
       <c r="A298" s="4" t="n"/>
       <c r="B298" s="4" t="inlineStr">
         <is>
-          <t>Old site's custom GA4 events ported (2026-10-10, owner asked to match legacy's Google tags)</t>
+          <t>Google Analytics tag (found missing 2026-10-10, added the same day)</t>
         </is>
       </c>
       <c r="C298" s="13" t="inlineStr">
@@ -7698,7 +7698,7 @@
       </c>
       <c r="D298" s="4" t="inlineStr">
         <is>
-          <t>Legacy loaded GA4 G-4GVW40S47N (already on the new site), Manus's own Umami counter (gone with Manus, not portable) and custom events from ConversionMechanics.tsx's AnalyticsTracker. Now src/components/ga-events.tsx (root layout) sends the same names: article_/page_25/50/75/90_scroll, engaged_45_seconds, second_page_view, homepage_path_work/_thinking/_building, start_here_open. Legacy's extra page_view on every history change is not ported (GA4 Enhanced measurement already counts in-site page changes; it would double-count). Tested in Chromium with Google's requests blocked: tonygreenberg.com (mapped to a local build) fired the homepage path and all four essay scroll events plus second_page_view; localhost loads no tag. A RampRate-style weekly report / hourly alert email and an admin analytics page were built the same day and removed at the owner's request (they use the Looker Studio report instead); the empty report_runs table and CRON_SECRET were removed too.</t>
+          <t>Live loads GA4 G-4GVW40S47N; the new site sent nothing, so stats would have stopped at cutover. Added src/components/google-analytics.tsx (plain next/script, no new package) in the root layout; it only runs on tonygreenberg.com / www, so Netlify previews and localhost never reach the real reports. Checked: type check, lint, build; in Chromium with Google's requests blocked: localhost sends nothing, tonygreenberg.com (mapped to a local production build) loads the tag on / and /find-your-coffee, no JS errors. In-site page changes are counted by GA4's Enhanced measurement (on by default; confirm in GA4 &gt; Admin &gt; Data streams on launch day).</t>
         </is>
       </c>
       <c r="E298" s="14" t="inlineStr">
@@ -7711,15 +7711,19 @@
       <c r="A299" s="4" t="n"/>
       <c r="B299" s="4" t="inlineStr">
         <is>
-          <t>Connect Google Search Console + GA4 to the new deployment on day one of cutover</t>
-        </is>
-      </c>
-      <c r="C299" s="16" t="inlineStr">
-        <is>
-          <t>Remaining</t>
-        </is>
-      </c>
-      <c r="D299" s="4" t="inlineStr"/>
+          <t>Old site's custom GA4 events ported (2026-10-10, owner asked to match legacy's Google tags)</t>
+        </is>
+      </c>
+      <c r="C299" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D299" s="4" t="inlineStr">
+        <is>
+          <t>Legacy loaded GA4 G-4GVW40S47N (already on the new site), Manus's own Umami counter (gone with Manus, not portable) and custom events from ConversionMechanics.tsx's AnalyticsTracker. Now src/components/ga-events.tsx (root layout) sends the same names: article_/page_25/50/75/90_scroll, engaged_45_seconds, second_page_view, homepage_path_work/_thinking/_building, start_here_open. Legacy's extra page_view on every history change is not ported (GA4 Enhanced measurement already counts in-site page changes; it would double-count). Tested in Chromium with Google's requests blocked: tonygreenberg.com (mapped to a local build) fired the homepage path and all four essay scroll events plus second_page_view; localhost loads no tag. A RampRate-style weekly report / hourly alert email and an admin analytics page were built the same day and removed at the owner's request (they use the Looker Studio report instead); the empty report_runs table and CRON_SECRET were removed too.</t>
+        </is>
+      </c>
       <c r="E299" s="14" t="inlineStr">
         <is>
           <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
@@ -7730,19 +7734,15 @@
       <c r="A300" s="4" t="n"/>
       <c r="B300" s="4" t="inlineStr">
         <is>
-          <t>Restore/adapt the manus.space triple-layer noindex lockdown pattern for any remaining staging URLs</t>
-        </is>
-      </c>
-      <c r="C300" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D300" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-01: the Netlify copy (tonygreenberg-website.netlify.app) and every deploy preview had no noindex at all, so Google could index a duplicate of the site. next.config.ts headers() now sends X-Robots-Tag: noindex, nofollow on any *.netlify.app host only; tonygreenberg.com is unaffected, so nothing to remove at cutover. Tested with Host headers on a production build.</t>
-        </is>
-      </c>
+          <t>Connect Google Search Console + GA4 to the new deployment on day one of cutover</t>
+        </is>
+      </c>
+      <c r="C300" s="16" t="inlineStr">
+        <is>
+          <t>Remaining</t>
+        </is>
+      </c>
+      <c r="D300" s="4" t="inlineStr"/>
       <c r="E300" s="14" t="inlineStr">
         <is>
           <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
@@ -7753,7 +7753,7 @@
       <c r="A301" s="4" t="n"/>
       <c r="B301" s="4" t="inlineStr">
         <is>
-          <t>"Keep going" strip above the footer on every page (2026-10-07)</t>
+          <t>Restore/adapt the manus.space triple-layer noindex lockdown pattern for any remaining staging URLs</t>
         </is>
       </c>
       <c r="C301" s="13" t="inlineStr">
@@ -7763,7 +7763,7 @@
       </c>
       <c r="D301" s="4" t="inlineStr">
         <is>
-          <t>legacy's WhereNext (deferred in Phase 3, never picked up) with its per-page suggestions, Home · Site Index · All Assessments; links pointed at current routes.</t>
+          <t>2026-10-01: the Netlify copy (tonygreenberg-website.netlify.app) and every deploy preview had no noindex at all, so Google could index a duplicate of the site. next.config.ts headers() now sends X-Robots-Tag: noindex, nofollow on any *.netlify.app host only; tonygreenberg.com is unaffected, so nothing to remove at cutover. Tested with Host headers on a production build.</t>
         </is>
       </c>
       <c r="E301" s="14" t="inlineStr">
@@ -7776,7 +7776,7 @@
       <c r="A302" s="4" t="n"/>
       <c r="B302" s="4" t="inlineStr">
         <is>
-          <t>Live-only and redesigned pages from the 2026-10-07 page sweep (188 pages compared with live)</t>
+          <t>"Keep going" strip above the footer on every page (2026-10-07)</t>
         </is>
       </c>
       <c r="C302" s="13" t="inlineStr">
@@ -7786,7 +7786,7 @@
       </c>
       <c r="D302" s="4" t="inlineStr">
         <is>
-          <t>/the-index rebuilt from live's code (20 concepts, related-word search across essays and site pages, full-text search on the server, "three related places to go next"; the old redirect to /search removed and its links, including the "Site Index" link in "Keep going", point at it again); /the-mirror (and /life-assessment) opens on live's intro (dark hero, "What We Measure" with the six areas, "The Ecosystem"), rebuilt as a step registry (rule 19); /essays header, order and column like live; /about "What They Say" styled like live (live picks 3 of the same 19 quotes at random; ours shows a fixed 3 so they're in the server HTML); /impact-futurism list titles and subtitles; /supplier-intake is a real page again with live's Stage 1 form; /seven-doors and /projects redirect home like live; /impact, /health, /library, /built-on-manus, /heroes are 404 on live too. Left as is on purpose: /blog stays our archive page (on live it repeats the homepage), the email gates on /framework and /peptide-supply-chain, the attention-theft Wall of Shame.</t>
+          <t>legacy's WhereNext (deferred in Phase 3, never picked up) with its per-page suggestions, Home · Site Index · All Assessments; links pointed at current routes.</t>
         </is>
       </c>
       <c r="E302" s="14" t="inlineStr">
@@ -7799,7 +7799,7 @@
       <c r="A303" s="4" t="n"/>
       <c r="B303" s="4" t="inlineStr">
         <is>
-          <t>/alex-azzi locked like live (2026-10-07, owner said match it)</t>
+          <t>Live-only and redesigned pages from the 2026-10-07 page sweep (188 pages compared with live)</t>
         </is>
       </c>
       <c r="C303" s="13" t="inlineStr">
@@ -7809,7 +7809,7 @@
       </c>
       <c r="D303" s="4" t="inlineStr">
         <is>
-          <t>same server-checked password as the locked essay (GATED_POST_PASSWORD, now also set in Netlify), live's "Restricted Access" screen, the report not in the page until unlocked, out of search and the sitemap.</t>
+          <t>/the-index rebuilt from live's code (20 concepts, related-word search across essays and site pages, full-text search on the server, "three related places to go next"; the old redirect to /search removed and its links, including the "Site Index" link in "Keep going", point at it again); /the-mirror (and /life-assessment) opens on live's intro (dark hero, "What We Measure" with the six areas, "The Ecosystem"), rebuilt as a step registry (rule 19); /essays header, order and column like live; /about "What They Say" styled like live (live picks 3 of the same 19 quotes at random; ours shows a fixed 3 so they're in the server HTML); /impact-futurism list titles and subtitles; /supplier-intake is a real page again with live's Stage 1 form; /seven-doors and /projects redirect home like live; /impact, /health, /library, /built-on-manus, /heroes are 404 on live too. Left as is on purpose: /blog stays our archive page (on live it repeats the homepage), the email gates on /framework and /peptide-supply-chain, the attention-theft Wall of Shame.</t>
         </is>
       </c>
       <c r="E303" s="14" t="inlineStr">
@@ -7822,7 +7822,7 @@
       <c r="A304" s="4" t="n"/>
       <c r="B304" s="4" t="inlineStr">
         <is>
-          <t>Live's title fonts and sizes (2026-10-07, "fix the style")</t>
+          <t>/alex-azzi locked like live (2026-10-07, owner said match it)</t>
         </is>
       </c>
       <c r="C304" s="13" t="inlineStr">
@@ -7832,7 +7832,7 @@
       </c>
       <c r="D304" s="4" t="inlineStr">
         <is>
-          <t>measured every page's title font, weight, size and label colour on live vs ours (136 pages). Now like live: Kava headings in Fraunces, HumanOS in Space Grotesk, the peptide tools / charity scorecard / thesis threads in the system serif, America Unbundled in the Iowan Old Style stack at live's size, /akbar in Fraunces 900, friend-gate and post-intervention in Georgia, and live's title sizes on peptide-matrix, peptide-supply-chain, rip-peptide-sciences and the HumanOS pages. Fonts load only on the pages that use them (src/lib/fonts/page-fonts.ts). Label colours stay the darker AA-contrast versions where live's lighter ones fail on a light background.</t>
+          <t>same server-checked password as the locked essay (GATED_POST_PASSWORD, now also set in Netlify), live's "Restricted Access" screen, the report not in the page until unlocked, out of search and the sitemap.</t>
         </is>
       </c>
       <c r="E304" s="14" t="inlineStr">
@@ -7845,7 +7845,7 @@
       <c r="A305" s="4" t="n"/>
       <c r="B305" s="4" t="inlineStr">
         <is>
-          <t>Peptide page images rescued into Sanity and wired (2026-10-07)</t>
+          <t>Live's title fonts and sizes (2026-10-07, "fix the style")</t>
         </is>
       </c>
       <c r="C305" s="13" t="inlineStr">
@@ -7855,7 +7855,7 @@
       </c>
       <c r="D305" s="4" t="inlineStr">
         <is>
-          <t>/peptide-watch hero plus its 11 section banners, /peptide-matrix and /peptide-supply-chain heroes, the /peptide-hall-of-shame hero (scripts/rescue-2026-10-07-peptide-images.ts, logged in docs/ai/manus-media-rescue.md).</t>
+          <t>measured every page's title font, weight, size and label colour on live vs ours (136 pages). Now like live: Kava headings in Fraunces, HumanOS in Space Grotesk, the peptide tools / charity scorecard / thesis threads in the system serif, America Unbundled in the Iowan Old Style stack at live's size, /akbar in Fraunces 900, friend-gate and post-intervention in Georgia, and live's title sizes on peptide-matrix, peptide-supply-chain, rip-peptide-sciences and the HumanOS pages. Fonts load only on the pages that use them (src/lib/fonts/page-fonts.ts). Label colours stay the darker AA-contrast versions where live's lighter ones fail on a light background.</t>
         </is>
       </c>
       <c r="E305" s="14" t="inlineStr">
@@ -7868,7 +7868,7 @@
       <c r="A306" s="4" t="n"/>
       <c r="B306" s="4" t="inlineStr">
         <is>
-          <t>Live's editorial redesign, first group (2026-10-07)</t>
+          <t>Peptide page images rescued into Sanity and wired (2026-10-07)</t>
         </is>
       </c>
       <c r="C306" s="13" t="inlineStr">
@@ -7878,7 +7878,7 @@
       </c>
       <c r="D306" s="4" t="inlineStr">
         <is>
-          <t>dark top sections, narrow single text column, short red section rules and dark call-to-action bands on /invest, /amplifier, /community (now "Sign In to Join the Community", linking our real sign-in; live's made-up counters left out), /framework, /the-letter (daily provocation with "Share this thought" and "Search past provocations"), /engage, /diamond-cut, /ecosystem and the homepage's "The thinking doesn't stop here" band. Kept on purpose: AA-contrast colours where live's fail, "Enter the Gate" instead of live's $5,000 checkout on /diamond-cut.</t>
+          <t>/peptide-watch hero plus its 11 section banners, /peptide-matrix and /peptide-supply-chain heroes, the /peptide-hall-of-shame hero (scripts/rescue-2026-10-07-peptide-images.ts, logged in docs/ai/manus-media-rescue.md).</t>
         </is>
       </c>
       <c r="E306" s="14" t="inlineStr">
@@ -7891,7 +7891,7 @@
       <c r="A307" s="4" t="n"/>
       <c r="B307" s="4" t="inlineStr">
         <is>
-          <t>Live's redesign, second group (done 2026-10-08)</t>
+          <t>Live's editorial redesign, first group (2026-10-07)</t>
         </is>
       </c>
       <c r="C307" s="13" t="inlineStr">
@@ -7901,7 +7901,7 @@
       </c>
       <c r="D307" s="4" t="inlineStr">
         <is>
-          <t>re-measured all 18 pages on live vs a fresh production build (title font/size/weight/colour, labels, hero images). Already matching from 2026-10-07: /the-web, /spirits, /iboga-ibogaine (weight 800), /living-declaration, BrewSoul photo on /brewsoul, /brewsoul/browse, /brewsoul/first-sip (live has none there either), /quiz_25q, /recent-creations. Fixed today: /find-your-journey (64px title, red label), /impact-dashboard (64px title in essay ink, label spacing), red labels on /published and /speaking (plus its "rooms" chips), /soulscore "by ImpactSoul" label, /pri-calibration title (weight 900, solid cream, was a purple gradient), /clients (live's narrow 546px column for the whole page, 56px title, roomier stats band, cards 2 per row; two static inline styles moved to classes), /brewsoul/guest (live's BrewSoul photo on the guest card instead of "SN" initials, labels in capitals), /humanos/connect (cards line up with the title), /peptide-hall-of-shame (stats and label readable light gold; were dark gold on dark). Typed arrows on the touched links are icons now (rule 18). Deliberately not copied from live (new CONTRIBUTING rule 20, owner 2026-10-08): red labels on dark bands use #E07A80 (live's #8E1E25 on black is about 2:1, unreadable); /recent-creations keeps our darker label colours (live's fail contrast on white); /humanos/connect keeps "Start Reading" (that card links to the philosophy page, the quiz live's "Start the Assessment" implies doesn't exist). Checked: type check, l</t>
+          <t>dark top sections, narrow single text column, short red section rules and dark call-to-action bands on /invest, /amplifier, /community (now "Sign In to Join the Community", linking our real sign-in; live's made-up counters left out), /framework, /the-letter (daily provocation with "Share this thought" and "Search past provocations"), /engage, /diamond-cut, /ecosystem and the homepage's "The thinking doesn't stop here" band. Kept on purpose: AA-contrast colours where live's fail, "Enter the Gate" instead of live's $5,000 checkout on /diamond-cut.</t>
         </is>
       </c>
       <c r="E307" s="14" t="inlineStr">
@@ -7914,7 +7914,7 @@
       <c r="A308" s="4" t="n"/>
       <c r="B308" s="4" t="inlineStr">
         <is>
-          <t>BrewSoul top of page (2026-10-08, owner: "button in the center at the top doesn't look good")</t>
+          <t>Live's redesign, second group (done 2026-10-08)</t>
         </is>
       </c>
       <c r="C308" s="13" t="inlineStr">
@@ -7924,7 +7924,7 @@
       </c>
       <c r="D308" s="4" t="inlineStr">
         <is>
-          <t>the category badge ("Deep Research" etc.) sat centred in an empty strip, squeezed against the hero, because we copied live's doubled 52px top gap. Now one gap everywhere and the badge floats in the top-left corner, lined up with the BrewSoul logo (brewsoul-main.tsx, category-badge.tsx); checked on all 26 badge pages at 3 widths that it covers nothing. BrewSoul menu: on tablets (768-1023px) the links were cut off and "More" was hidden with no menu button at all; now the menu button shows below 1024px, 5 links + "More" from 1024px, all 8 from 1280px, "More" always visible.</t>
+          <t>re-measured all 18 pages on live vs a fresh production build (title font/size/weight/colour, labels, hero images). Already matching from 2026-10-07: /the-web, /spirits, /iboga-ibogaine (weight 800), /living-declaration, BrewSoul photo on /brewsoul, /brewsoul/browse, /brewsoul/first-sip (live has none there either), /quiz_25q, /recent-creations. Fixed today: /find-your-journey (64px title, red label), /impact-dashboard (64px title in essay ink, label spacing), red labels on /published and /speaking (plus its "rooms" chips), /soulscore "by ImpactSoul" label, /pri-calibration title (weight 900, solid cream, was a purple gradient), /clients (live's narrow 546px column for the whole page, 56px title, roomier stats band, cards 2 per row; two static inline styles moved to classes), /brewsoul/guest (live's BrewSoul photo on the guest card instead of "SN" initials, labels in capitals), /humanos/connect (cards line up with the title), /peptide-hall-of-shame (stats and label readable light gold; were dark gold on dark). Typed arrows on the touched links are icons now (rule 18). Deliberately not copied from live (new CONTRIBUTING rule 20, owner 2026-10-08): red labels on dark bands use #E07A80 (live's #8E1E25 on black is about 2:1, unreadable); /recent-creations keeps our darker label colours (live's fail contrast on white); /humanos/connect keeps "Start Reading" (that card links to the philosophy page, the quiz live's "Start the Assessment" implies doesn't exist). Checked: type check, l</t>
         </is>
       </c>
       <c r="E308" s="14" t="inlineStr">
@@ -7937,7 +7937,7 @@
       <c r="A309" s="4" t="n"/>
       <c r="B309" s="4" t="inlineStr">
         <is>
-          <t>/pri-efficacy's "Simulation / Live Calibrations" switch like live (2026-10-08)</t>
+          <t>BrewSoul top of page (2026-10-08, owner: "button in the center at the top doesn't look good")</t>
         </is>
       </c>
       <c r="C309" s="13" t="inlineStr">
@@ -7947,7 +7947,7 @@
       </c>
       <c r="D309" s="4" t="inlineStr">
         <is>
-          <t>shadcn Tabs, both panels in the server HTML (forceMount). The Live tab reads real aggregate numbers from pri_calibrations (getPriLiveStats() in src/lib/pri-research.ts: totals, opt-ins, average score per dimension; no rows leave the server), page stays static and refreshes every 10 minutes. Until the Supabase scripts are run (Phase 2) it says the numbers "aren't available just now" instead of a fake zero. Checked: build (○, 10m), server HTML has both tabs, tab switch at 390/1280px, no JS errors. Re-check with real numbers once the table exists.</t>
+          <t>the category badge ("Deep Research" etc.) sat centred in an empty strip, squeezed against the hero, because we copied live's doubled 52px top gap. Now one gap everywhere and the badge floats in the top-left corner, lined up with the BrewSoul logo (brewsoul-main.tsx, category-badge.tsx); checked on all 26 badge pages at 3 widths that it covers nothing. BrewSoul menu: on tablets (768-1023px) the links were cut off and "More" was hidden with no menu button at all; now the menu button shows below 1024px, 5 links + "More" from 1024px, all 8 from 1280px, "More" always visible.</t>
         </is>
       </c>
       <c r="E309" s="14" t="inlineStr">
@@ -7960,63 +7960,63 @@
       <c r="A310" s="4" t="n"/>
       <c r="B310" s="4" t="inlineStr">
         <is>
+          <t>/pri-efficacy's "Simulation / Live Calibrations" switch like live (2026-10-08)</t>
+        </is>
+      </c>
+      <c r="C310" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D310" s="4" t="inlineStr">
+        <is>
+          <t>shadcn Tabs, both panels in the server HTML (forceMount). The Live tab reads real aggregate numbers from pri_calibrations (getPriLiveStats() in src/lib/pri-research.ts: totals, opt-ins, average score per dimension; no rows leave the server), page stays static and refreshes every 10 minutes. Until the Supabase scripts are run (Phase 2) it says the numbers "aren't available just now" instead of a fake zero. Checked: build (○, 10m), server HTML has both tabs, tab switch at 390/1280px, no JS errors. Re-check with real numbers once the table exists.</t>
+        </is>
+      </c>
+      <c r="E310" s="14" t="inlineStr">
+        <is>
+          <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" s="4" t="n"/>
+      <c r="B311" s="4" t="inlineStr">
+        <is>
           <t>/brewsoul/browse hero readable (2026-10-08, owner said go ahead)</t>
         </is>
       </c>
-      <c r="C310" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D310" s="4" t="inlineStr">
+      <c r="C311" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D311" s="4" t="inlineStr">
         <is>
           <t>a soft cream glow behind the title block so "The Catalog", the subtitle and the stat labels read clearly over the coffee photo (live is hard to read there too; rule 20). Photo still shows around the edges. Checked at 390/1280px.</t>
         </is>
       </c>
-      <c r="E310" s="14" t="inlineStr">
+      <c r="E311" s="14" t="inlineStr">
         <is>
           <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
         </is>
       </c>
     </row>
-    <row r="311">
-      <c r="A311" s="10" t="inlineStr">
+    <row r="312">
+      <c r="A312" s="10" t="inlineStr">
         <is>
           <t>Phase 13 — Images Needed in Sanity</t>
         </is>
       </c>
-      <c r="B311" s="11" t="n"/>
-      <c r="C311" s="11" t="n"/>
-      <c r="D311" s="12" t="n"/>
-    </row>
-    <row r="312">
-      <c r="A312" s="4" t="n"/>
-      <c r="B312" s="4" t="inlineStr">
-        <is>
-          <t>Manus media rescue (2026-09-29)</t>
-        </is>
-      </c>
-      <c r="C312" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D312" s="4" t="inlineStr">
-        <is>
-          <t>all 94 Manus-hosted image/video references in the legacy source (/api/img/, /manus-storage/) were checked live. 91 were still downloadable, including the /akbar photos the entry below calls "permanently lost", and all 91 are now Sanity assets (scripts/rescue-manus-media.ts; Sanity dedupes by SHA-1). 3 were gone (HTTP 502). The manifest docs/ai/manus-media-rescue.md maps each one to the legacy files that used it and its Sanity URL. They are not wired into pages yet: go page by page, with real alt text. /facilitator-index's two diagrams are done (scripts/rescue-facilitator-images.ts).</t>
-        </is>
-      </c>
-      <c r="E312" s="14" t="inlineStr">
-        <is>
-          <t>Phase 13 — Images Needed in Sanity</t>
-        </is>
-      </c>
+      <c r="B312" s="11" t="n"/>
+      <c r="C312" s="11" t="n"/>
+      <c r="D312" s="12" t="n"/>
     </row>
     <row r="313">
       <c r="A313" s="4" t="n"/>
       <c r="B313" s="4" t="inlineStr">
         <is>
-          <t>Favicon</t>
+          <t>Manus media rescue (2026-09-29)</t>
         </is>
       </c>
       <c r="C313" s="13" t="inlineStr">
@@ -8026,7 +8026,7 @@
       </c>
       <c r="D313" s="4" t="inlineStr">
         <is>
-          <t>real "G" brand mark generated from the header's actual wordmark treatment (src/app/icon.tsx), see Phase 3</t>
+          <t>all 94 Manus-hosted image/video references in the legacy source (/api/img/, /manus-storage/) were checked live. 91 were still downloadable, including the /akbar photos the entry below calls "permanently lost", and all 91 are now Sanity assets (scripts/rescue-manus-media.ts; Sanity dedupes by SHA-1). 3 were gone (HTTP 502). The manifest docs/ai/manus-media-rescue.md maps each one to the legacy files that used it and its Sanity URL. They are not wired into pages yet: go page by page, with real alt text. /facilitator-index's two diagrams are done (scripts/rescue-facilitator-images.ts).</t>
         </is>
       </c>
       <c r="E313" s="14" t="inlineStr">
@@ -8039,7 +8039,7 @@
       <c r="A314" s="4" t="n"/>
       <c r="B314" s="4" t="inlineStr">
         <is>
-          <t>Site-wide: logo (light + dark) beyond the current text wordmark</t>
+          <t>Favicon</t>
         </is>
       </c>
       <c r="C314" s="13" t="inlineStr">
@@ -8049,7 +8049,7 @@
       </c>
       <c r="D314" s="4" t="inlineStr">
         <is>
-          <t>Decided 2026-10-13 (owner): keep the text logo. The header's "TonyG" wordmark (site-header.tsx, gold G) already has light and dark colours, so no change. (Default/fallback OG image 1200×630 exists: public/images/default-og.png, checked 2026-10-02.)</t>
+          <t>real "G" brand mark generated from the header's actual wordmark treatment (src/app/icon.tsx), see Phase 3</t>
         </is>
       </c>
       <c r="E314" s="14" t="inlineStr">
@@ -8062,7 +8062,7 @@
       <c r="A315" s="4" t="n"/>
       <c r="B315" s="4" t="inlineStr">
         <is>
-          <t>Author photo(s) for blog author schema (Tony Greenberg headshot at minimum)</t>
+          <t>Site-wide: logo (light + dark) beyond the current text wordmark</t>
         </is>
       </c>
       <c r="C315" s="13" t="inlineStr">
@@ -8072,7 +8072,7 @@
       </c>
       <c r="D315" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02: the rescued headshot is already the author avatar in Sanity; now also in every post's Article JSON-LD (author image + url /about). The JSON-LD publisher logo pointed at /favicon.ico, a 404 here; now /icon.</t>
+          <t>Decided 2026-10-13 (owner): keep the text logo. The header's "TonyG" wordmark (site-header.tsx, gold G) already has light and dark colours, so no change. (Default/fallback OG image 1200×630 exists: public/images/default-og.png, checked 2026-10-02.)</t>
         </is>
       </c>
       <c r="E315" s="14" t="inlineStr">
@@ -8085,7 +8085,7 @@
       <c r="A316" s="4" t="n"/>
       <c r="B316" s="4" t="inlineStr">
         <is>
-          <t>Blog hero images</t>
+          <t>Author photo(s) for blog author schema (Tony Greenberg headshot at minimum)</t>
         </is>
       </c>
       <c r="C316" s="13" t="inlineStr">
@@ -8095,7 +8095,7 @@
       </c>
       <c r="D316" s="4" t="inlineStr">
         <is>
-          <t>audited, then migrated. Final state:</t>
+          <t>2026-10-02: the rescued headshot is already the author avatar in Sanity; now also in every post's Article JSON-LD (author image + url /about). The JSON-LD publisher logo pointed at /favicon.ico, a 404 here; now /icon.</t>
         </is>
       </c>
       <c r="E316" s="14" t="inlineStr">
@@ -8108,7 +8108,7 @@
       <c r="A317" s="4" t="n"/>
       <c r="B317" s="4" t="inlineStr">
         <is>
-          <t>22 posts have a real hero image, now live in Sanity (17 already on RampRate's own CloudFront + 4 rescued from the legacy /api/img/ proxy + 1…</t>
+          <t>Blog hero images</t>
         </is>
       </c>
       <c r="C317" s="13" t="inlineStr">
@@ -8118,7 +8118,7 @@
       </c>
       <c r="D317" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> rescued from /manus-storage/, all pulled over by migrate-blog-posts.ts before Manus is decommissioned)</t>
+          <t>audited, then migrated. Final state:</t>
         </is>
       </c>
       <c r="E317" s="14" t="inlineStr">
@@ -8131,7 +8131,7 @@
       <c r="A318" s="4" t="n"/>
       <c r="B318" s="4" t="inlineStr">
         <is>
-          <t>7 more posts got a real, unique hero image rescued from the live legacy site's newly-added art this pass (scripts/rescue-2026-09-blog-images…</t>
+          <t>22 posts have a real hero image, now live in Sanity (17 already on RampRate's own CloudFront + 4 rescued from the legacy /api/img/ proxy + 1…</t>
         </is>
       </c>
       <c r="C318" s="13" t="inlineStr">
@@ -8141,7 +8141,7 @@
       </c>
       <c r="D318" s="4" t="inlineStr">
         <is>
-          <t>.ts — see the correction note above): california-toll-roads-legalized-scam, the-1000-hour-hold, conscious-capital-partnership-ecosystem, the-peptide-truth-65m-fraud-industry-vs-life-changing-medicine, clear-communication, building-services-market-transhuman-era, heart-protocol-addendum.</t>
+          <t xml:space="preserve"> rescued from /manus-storage/, all pulled over by migrate-blog-posts.ts before Manus is decommissioned)</t>
         </is>
       </c>
       <c r="E318" s="14" t="inlineStr">
@@ -8154,7 +8154,7 @@
       <c r="A319" s="4" t="n"/>
       <c r="B319" s="4" t="inlineStr">
         <is>
-          <t>92 posts still need a real, unique hero image</t>
+          <t>7 more posts got a real, unique hero image rescued from the live legacy site's newly-added art this pass (scripts/rescue-2026-09-blog-images…</t>
         </is>
       </c>
       <c r="C319" s="13" t="inlineStr">
@@ -8164,7 +8164,7 @@
       </c>
       <c r="D319" s="4" t="inlineStr">
         <is>
-          <t>(down from 99). 2026-10-13 (owner: "image you can add in Sanity"): generated a unique, text-free picture for each of the 92 (live's default-arch family: cream over a deep colour, gold line geometry, colour and motif by category, layout from the slug; scripts/generate-essay-hero-art.mjs) and set it as each post's heroImage draft (scripts/upload-essay-hero-art-2026-10-13.ts; dry run first: 92 found, none had art, nothing replaced). Checked in Sanity: 92 drafts carry the new image, 0 published posts changed. Published 2026-10-13 (owner: yes) with the script's --publish (only drafts whose sole change was the picture; 92 of 92). Checked: the Netlify copy's essay page now serves the new image (webhook refresh). Real photography can still replace any of them later. Tracked one row per post, with a suggested image-generation prompt, in BLOG-IMAGE-BRIEFS.md — work through that file and check items off there, not here. No image-generation tool was connected in this environment as of this writing; either connect one (e.g. an MCP image-gen extension), source these manually/with a designer then upload via Sanity Studio (/studio), or re-check the live legacy site periodically per the correction note above.</t>
+          <t>.ts — see the correction note above): california-toll-roads-legalized-scam, the-1000-hour-hold, conscious-capital-partnership-ecosystem, the-peptide-truth-65m-fraud-industry-vs-life-changing-medicine, clear-communication, building-services-market-transhuman-era, heart-protocol-addendum.</t>
         </is>
       </c>
       <c r="E319" s="14" t="inlineStr">
@@ -8177,7 +8177,7 @@
       <c r="A320" s="4" t="n"/>
       <c r="B320" s="4" t="inlineStr">
         <is>
-          <t>Blog: per-post OG image if different from hero (many posts can reuse hero as OG)</t>
+          <t>92 posts still need a real, unique hero image</t>
         </is>
       </c>
       <c r="C320" s="13" t="inlineStr">
@@ -8187,7 +8187,7 @@
       </c>
       <c r="D320" s="4" t="inlineStr">
         <is>
-          <t>Confirmed 2026-10-02: generateMetadata uses seo.ogImage, else the hero, else the default OG image.</t>
+          <t>(down from 99). 2026-10-13 (owner: "image you can add in Sanity"): generated a unique, text-free picture for each of the 92 (live's default-arch family: cream over a deep colour, gold line geometry, colour and motif by category, layout from the slug; scripts/generate-essay-hero-art.mjs) and set it as each post's heroImage draft (scripts/upload-essay-hero-art-2026-10-13.ts; dry run first: 92 found, none had art, nothing replaced). Checked in Sanity: 92 drafts carry the new image, 0 published posts changed. Published 2026-10-13 (owner: yes) with the script's --publish (only drafts whose sole change was the picture; 92 of 92). Checked: the Netlify copy's essay page now serves the new image (webhook refresh). Real photography can still replace any of them later. Tracked one row per post, with a suggested image-generation prompt, in BLOG-IMAGE-BRIEFS.md — work through that file and check items off there, not here. No image-generation tool was connected in this environment as of this writing; either connect one (e.g. an MCP image-gen extension), source these manually/with a designer then upload via Sanity Studio (/studio), or re-check the live legacy site periodically per the correction note above.</t>
         </is>
       </c>
       <c r="E320" s="14" t="inlineStr">
@@ -8200,7 +8200,7 @@
       <c r="A321" s="4" t="n"/>
       <c r="B321" s="4" t="inlineStr">
         <is>
-          <t>Marketing pages</t>
+          <t>Blog: per-post OG image if different from hero (many posts can reuse hero as OG)</t>
         </is>
       </c>
       <c r="C321" s="13" t="inlineStr">
@@ -8210,7 +8210,7 @@
       </c>
       <c r="D321" s="4" t="inlineStr">
         <is>
-          <t>hero/section images for /the-letter, /the-territory, /engine-room, /the-body, /the-nightstand, /recent-creations (portfolio thumbnails), /published (publication logos), /clients (client logos — confirm licensing before re-hosting). Checked against live 2026-10-02: same image count on every one; /the-territory, /engine-room, /recent-creations, /published, /clients have no images on live either.</t>
+          <t>Confirmed 2026-10-02: generateMetadata uses seo.ogImage, else the hero, else the default OG image.</t>
         </is>
       </c>
       <c r="E321" s="14" t="inlineStr">
@@ -8223,7 +8223,7 @@
       <c r="A322" s="4" t="n"/>
       <c r="B322" s="4" t="inlineStr">
         <is>
-          <t>/akbar essay images</t>
+          <t>Marketing pages</t>
         </is>
       </c>
       <c r="C322" s="13" t="inlineStr">
@@ -8233,7 +8233,7 @@
       </c>
       <c r="D322" s="4" t="inlineStr">
         <is>
-          <t>not lost after all: 20 of the 21 were rescued into Sanity by scripts/rescue-manus-media.ts (2026-09-28) and are wired back in legacy's layout (hero mosaic, JC portrait, 2x2 grid, 3 full-bleeds, 3-up strip, footer gallery) as of 2026-09-29. Only slider-3 was gone (HTTP 502); the hero mosaic is 4 tiles instead of 5.</t>
+          <t>hero/section images for /the-letter, /the-territory, /engine-room, /the-body, /the-nightstand, /recent-creations (portfolio thumbnails), /published (publication logos), /clients (client logos — confirm licensing before re-hosting). Checked against live 2026-10-02: same image count on every one; /the-territory, /engine-room, /recent-creations, /published, /clients have no images on live either.</t>
         </is>
       </c>
       <c r="E322" s="14" t="inlineStr">
@@ -8246,7 +8246,7 @@
       <c r="A323" s="4" t="n"/>
       <c r="B323" s="4" t="inlineStr">
         <is>
-          <t>Rescued page images wired back in (2026-09-29)</t>
+          <t>/akbar essay images</t>
         </is>
       </c>
       <c r="C323" s="13" t="inlineStr">
@@ -8256,7 +8256,7 @@
       </c>
       <c r="D323" s="4" t="inlineStr">
         <is>
-          <t>/living-declaration hero, hand image and Clarisse Abelarde artwork; /impact-dashboard earth hero; /find-my banner; /find-your-coffee dark photo landing (legacy copy restored, replacing an intro that wasn't in legacy). Also wired (second pass): /consciousness-scale (legacy's hero-first flow restored, the invented intro screen removed), /find-your-me hero, /humanos hero, the HumanOS nav logo, and all 12 HumanOS people headshots (/humanos/ecosystem, /humanos/philosophy). Blog-body images (2026-09-29): all 19 the migration dropped are restored by scripts/restore-blog-body-images.ts as Sanity drafts on 4 posts (Clarisse Abelarde 7, You Are the Moat 4, FRQNCY 6, Energy Is Money 2), waiting to be published in Studio; the other blog-listed assets were heroes already set. Still unwired from docs/ai/manus-media-rescue.md: and /alex-azzi's subject photo (a photo of a real person on an accusation page: needs Tony's yes first).</t>
+          <t>not lost after all: 20 of the 21 were rescued into Sanity by scripts/rescue-manus-media.ts (2026-09-28) and are wired back in legacy's layout (hero mosaic, JC portrait, 2x2 grid, 3 full-bleeds, 3-up strip, footer gallery) as of 2026-09-29. Only slider-3 was gone (HTTP 502); the hero mosaic is 4 tiles instead of 5.</t>
         </is>
       </c>
       <c r="E323" s="14" t="inlineStr">
@@ -8269,7 +8269,7 @@
       <c r="A324" s="4" t="n"/>
       <c r="B324" s="4" t="inlineStr">
         <is>
-          <t>BrewSoul: coffee/product images (brewsoul-coffees-expanded.ts likely has image refs</t>
+          <t>Rescued page images wired back in (2026-09-29)</t>
         </is>
       </c>
       <c r="C324" s="13" t="inlineStr">
@@ -8279,7 +8279,7 @@
       </c>
       <c r="D324" s="4" t="inlineStr">
         <is>
-          <t>audit), city guide header images, roaster directory photos. Audited 2026-09-09 (status spreadsheet), confirmed 2026-10-02: city guides already have photos; coffees, chains and roasters have no image field in legacy or here (text-only by design); farms got real photos.</t>
+          <t>/living-declaration hero, hand image and Clarisse Abelarde artwork; /impact-dashboard earth hero; /find-my banner; /find-your-coffee dark photo landing (legacy copy restored, replacing an intro that wasn't in legacy). Also wired (second pass): /consciousness-scale (legacy's hero-first flow restored, the invented intro screen removed), /find-your-me hero, /humanos hero, the HumanOS nav logo, and all 12 HumanOS people headshots (/humanos/ecosystem, /humanos/philosophy). Blog-body images (2026-09-29): all 19 the migration dropped are restored by scripts/restore-blog-body-images.ts as Sanity drafts on 4 posts (Clarisse Abelarde 7, You Are the Moat 4, FRQNCY 6, Energy Is Money 2), waiting to be published in Studio; the other blog-listed assets were heroes already set. Still unwired from docs/ai/manus-media-rescue.md: and /alex-azzi's subject photo (a photo of a real person on an accusation page: needs Tony's yes first).</t>
         </is>
       </c>
       <c r="E324" s="14" t="inlineStr">
@@ -8292,7 +8292,7 @@
       <c r="A325" s="4" t="n"/>
       <c r="B325" s="4" t="inlineStr">
         <is>
-          <t>65 page images moved off the Manus storage copy into Sanity (2026-10-02)</t>
+          <t>BrewSoul: coffee/product images (brewsoul-coffees-expanded.ts likely has image refs</t>
         </is>
       </c>
       <c r="C325" s="13" t="inlineStr">
@@ -8302,7 +8302,7 @@
       </c>
       <c r="D325" s="4" t="inlineStr">
         <is>
-          <t>every image the code loaded from d2xsxph8kpxj0f.cloudfront.net (PRI medicine images, Iboga module, facilitator index, /attention-theft, /alex-azzi, /protecting-your-business, /peyote-mescaline, HumanOS, the peptide quiz). Notes called it "RampRate's own CloudFront", but every file sits in the legacy Manus project's folder and its owner couldn't be confirmed. All 65 uploaded (scripts/rescue-cloudfront-images.ts), code rewritten, host removed from images.remotePatterns, no Sanity document used it. Table in docs/ai/manus-media-rescue.md.</t>
+          <t>audit), city guide header images, roaster directory photos. Audited 2026-09-09 (status spreadsheet), confirmed 2026-10-02: city guides already have photos; coffees, chains and roasters have no image field in legacy or here (text-only by design); farms got real photos.</t>
         </is>
       </c>
       <c r="E325" s="14" t="inlineStr">
@@ -8315,7 +8315,7 @@
       <c r="A326" s="4" t="n"/>
       <c r="B326" s="4" t="inlineStr">
         <is>
-          <t>PRI/Kava: medicine reference images (medicine-images.ts), facility images for /facilitator-index</t>
+          <t>65 page images moved off the Manus storage copy into Sanity (2026-10-02)</t>
         </is>
       </c>
       <c r="C326" s="13" t="inlineStr">
@@ -8325,7 +8325,7 @@
       </c>
       <c r="D326" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02: all in Sanity; image counts match live on PRI, Kava, Iboga, Peyote, facilitator pages.</t>
+          <t>every image the code loaded from d2xsxph8kpxj0f.cloudfront.net (PRI medicine images, Iboga module, facilitator index, /attention-theft, /alex-azzi, /protecting-your-business, /peyote-mescaline, HumanOS, the peptide quiz). Notes called it "RampRate's own CloudFront", but every file sits in the legacy Manus project's folder and its owner couldn't be confirmed. All 65 uploaded (scripts/rescue-cloudfront-images.ts), code rewritten, host removed from images.remotePatterns, no Sanity document used it. Table in docs/ai/manus-media-rescue.md.</t>
         </is>
       </c>
       <c r="E326" s="14" t="inlineStr">
@@ -8338,7 +8338,7 @@
       <c r="A327" s="4" t="n"/>
       <c r="B327" s="4" t="inlineStr">
         <is>
-          <t>Manifesto/Attention Theft: any diagram/illustration assets used on the mega-page</t>
+          <t>PRI/Kava: medicine reference images (medicine-images.ts), facility images for /facilitator-index</t>
         </is>
       </c>
       <c r="C327" s="13" t="inlineStr">
@@ -8348,7 +8348,7 @@
       </c>
       <c r="D327" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02: 6 of live's 7 are in (now in Sanity); the 7th belongs to the Wall of Shame section left out on purpose.</t>
+          <t>2026-10-02: all in Sanity; image counts match live on PRI, Kava, Iboga, Peyote, facilitator pages.</t>
         </is>
       </c>
       <c r="E327" s="14" t="inlineStr">
@@ -8361,7 +8361,7 @@
       <c r="A328" s="4" t="n"/>
       <c r="B328" s="4" t="inlineStr">
         <is>
-          <t>Assessment result-screen background art (flagged in STATUS.md as a known gap</t>
+          <t>Manifesto/Attention Theft: any diagram/illustration assets used on the mega-page</t>
         </is>
       </c>
       <c r="C328" s="13" t="inlineStr">
@@ -8371,7 +8371,7 @@
       </c>
       <c r="D328" s="4" t="inlineStr">
         <is>
-          <t>18/20 assessments currently have plain black backgrounds; sourcing themed art here also closes that gap) Done 2026-10-13 with colour instead of art (owner: "yes" to colour backgrounds). About 20 quizzes already had a coloured background (ThemedBackground, light per-theme gradients). The 4 still flat dark now have a dark colour gradient, kept dark so their light text stays readable: /find-your-journey result (purple to teal), /my-journey (its black layer hid the gradient; now green to purple), /pri-calibration and the /psychedelic-readiness-index assessment section (PRI ink to amber to plum, starting at ink so the photo band's fade still meets it). Checked: type check, lint, build (all 8 colours in the compiled CSS), screenshots at 375/820/1280 (quiz completed for the journey result), no sideways scroll or JS errors, axe colour-contrast 0 at 375 and 1280.</t>
+          <t>2026-10-02: 6 of live's 7 are in (now in Sanity); the 7th belongs to the Wall of Shame section left out on purpose.</t>
         </is>
       </c>
       <c r="E328" s="14" t="inlineStr">
@@ -8384,7 +8384,7 @@
       <c r="A329" s="4" t="n"/>
       <c r="B329" s="4" t="inlineStr">
         <is>
-          <t>Chatbot: FauxTony avatar/icon</t>
+          <t>Assessment result-screen background art (flagged in STATUS.md as a known gap</t>
         </is>
       </c>
       <c r="C329" s="13" t="inlineStr">
@@ -8394,7 +8394,7 @@
       </c>
       <c r="D329" s="4" t="inlineStr">
         <is>
-          <t>Not needed (2026-10-02): the chatbot phase (Phase 10) was cancelled.</t>
+          <t>18/20 assessments currently have plain black backgrounds; sourcing themed art here also closes that gap) Done 2026-10-13 with colour instead of art (owner: "yes" to colour backgrounds). About 20 quizzes already had a coloured background (ThemedBackground, light per-theme gradients). The 4 still flat dark now have a dark colour gradient, kept dark so their light text stays readable: /find-your-journey result (purple to teal), /my-journey (its black layer hid the gradient; now green to purple), /pri-calibration and the /psychedelic-readiness-index assessment section (PRI ink to amber to plum, starting at ink so the photo band's fade still meets it). Checked: type check, lint, build (all 8 colours in the compiled CSS), screenshots at 375/820/1280 (quiz completed for the journey result), no sideways scroll or JS errors, axe colour-contrast 0 at 375 and 1280.</t>
         </is>
       </c>
       <c r="E329" s="14" t="inlineStr">
@@ -8407,63 +8407,63 @@
       <c r="A330" s="4" t="n"/>
       <c r="B330" s="4" t="inlineStr">
         <is>
+          <t>Chatbot: FauxTony avatar/icon</t>
+        </is>
+      </c>
+      <c r="C330" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D330" s="4" t="inlineStr">
+        <is>
+          <t>Not needed (2026-10-02): the chatbot phase (Phase 10) was cancelled.</t>
+        </is>
+      </c>
+      <c r="E330" s="14" t="inlineStr">
+        <is>
+          <t>Phase 13 — Images Needed in Sanity</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" s="4" t="n"/>
+      <c r="B331" s="4" t="inlineStr">
+        <is>
           <t>Audit client/public/ (including alex-azzi/, brewsoul/ subfolders) for any static assets already sitting there unused that should be pulled i…</t>
         </is>
       </c>
-      <c r="C330" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D330" s="4" t="inlineStr">
+      <c r="C331" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D331" s="4" t="inlineStr">
         <is>
           <t>n rather than re-created. Done 2026-10-02: no images there at all (only llms.txt, a BrewSoul catalog, Manus debug files, design-options.html). Found and fixed a cutover risk instead: live serves two Google site-verification files (/google6881a0411c48b301.html, /alex-azzi/googleedff0185753a4a1f.html) that the new site returned 404 for, so Search Console could lose verification at DNS cutover. Both copied to public/ byte for byte. Not copied: site.webmanifest (its icons don't exist here; Next's app/icon.tsx covers the favicon).</t>
         </is>
       </c>
-      <c r="E330" s="14" t="inlineStr">
+      <c r="E331" s="14" t="inlineStr">
         <is>
           <t>Phase 13 — Images Needed in Sanity</t>
         </is>
       </c>
     </row>
-    <row r="331">
-      <c r="A331" s="10" t="inlineStr">
+    <row r="332">
+      <c r="A332" s="10" t="inlineStr">
         <is>
           <t>Phase 14 — QA &amp; Launch</t>
         </is>
       </c>
-      <c r="B331" s="11" t="n"/>
-      <c r="C331" s="11" t="n"/>
-      <c r="D331" s="12" t="n"/>
-    </row>
-    <row r="332">
-      <c r="A332" s="4" t="n"/>
-      <c r="B332" s="4" t="inlineStr">
-        <is>
-          <t>Mobile responsive pass on every ported section</t>
-        </is>
-      </c>
-      <c r="C332" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D332" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-29: no page scrolls sideways at 375px any more (114 pages checked in Chrome: every unique page plus 3 of each templated set like blog posts and coffees). Fixed: BrewSoul NextSteps forced 3 columns (and used an inline style), charity-scorecard tab row, /brewsoul/browse filter dropdowns, /the-philosophy hero glow. Still to check by hand: 44px tap targets and Safari iOS. 2026-09-30: 44px tap targets on phones for the shared header, footer, BrewSoul/Kava/HumanOS menus and ~100 standalone links (undersized targets 1,904 → 578; the rest are 24-43px pills/chips that meet WCAG 2.2 AA). axe target-size (WCAG 2.2 AA, with its spacing exception): 0 failures on 114 pages. Safari/iPhone (WebKit, iPhone 14 emulation): all 114 pages load, no sideways scroll, no JS errors; form fields under 16px (iOS zoom-on-tap) fixed site-wide in globals.css. Still to check on a real iPhone: BrewSoul's bottom journey bar showed page text through it in headless WebKit only (taps hit the bar correctly; Chrome renders it solid). Fixed 2026-10-09: the bar is now solid (bg-[#2C1810], was 92% plus backdrop-blur-md), so nothing can show through even where the blur isn't drawn; checked in WebKit (iPhone 13 profile) and Chrome: background rgb(44, 24, 16), no text behind the buttons. A real iPhone check is still part of Phase 14. Checked 2026-10-13 in Apple's iPhone Simulator (iPhone 16, iOS 26.5, real Mobile Safari; not a physical phone, owner accepted this as the iPhone check): 14 key pages on a fresh prod</t>
-        </is>
-      </c>
-      <c r="E332" s="14" t="inlineStr">
-        <is>
-          <t>Phase 14 — QA &amp; Launch</t>
-        </is>
-      </c>
+      <c r="B332" s="11" t="n"/>
+      <c r="C332" s="11" t="n"/>
+      <c r="D332" s="12" t="n"/>
     </row>
     <row r="333">
       <c r="A333" s="4" t="n"/>
       <c r="B333" s="4" t="inlineStr">
         <is>
-          <t>Accessibility pass (WCAG AA contrast, 44px touch targets, keyboard nav)</t>
+          <t>Mobile responsive pass on every ported section</t>
         </is>
       </c>
       <c r="C333" s="13" t="inlineStr">
@@ -8473,7 +8473,7 @@
       </c>
       <c r="D333" s="4" t="inlineStr">
         <is>
-          <t>same bar as legacy QA_MASTER_PROMPT.md. 2026-09-29 axe-core pass (WCAG 2.1 AA, same 114 pages, production build): all unlabeled dropdowns/inputs and unnamed links fixed; contrast down from 1,453 failing items on 106 pages to 1,038 on 70 (43 pages fully clean). Shared fixes: brand gold #8b6914 → #836311 site-wide (was 4.3:1 on cream, AA needs 4.5), header "⌘K"/social icons, BrewSoul nav and footer, HumanOS footer, Kava footer, assessment intro footnote, post-card image links. 2026-09-30: contrast finished, 0 axe color-contrast failures left on the same 114 pages (production build). Token changes: --kava-saffron #b86a28 → #8e521f, --pri-purple-light #a855f7 → #b87bf9 (on-dark purple only), --crusade-teal #0e7c7c → #0d7373; PriEyebrow goes light purple inside a dark PriSection via group-data-dark/pri; /find-your-me and the journey tracker's dark glass panels 60-70% → 90% (legacy's own 60% glass on beige rendered gray, cream text failed). Everything else: nearest passing shade of the same hue, or gold ↔ gold-light on the wrong background. Left: 18 links inside text marked only by color (need an underline), 44px tap targets, keyboard nav. 2026-09-30: 18 color-only in-text links underlined (axe link-in-text-block: 0 left); keyboard focus visible on every focusable item on 8 sampled pages (two form fields had none, fixed). 2026-10-02 re-run (axe WCAG 2.2 AA, 142 pages × 375/1280px, production build, plus Tab through 40 stops per page): found 1,370 contrast failures (mostly BrewSoul'</t>
+          <t>2026-09-29: no page scrolls sideways at 375px any more (114 pages checked in Chrome: every unique page plus 3 of each templated set like blog posts and coffees). Fixed: BrewSoul NextSteps forced 3 columns (and used an inline style), charity-scorecard tab row, /brewsoul/browse filter dropdowns, /the-philosophy hero glow. Still to check by hand: 44px tap targets and Safari iOS. 2026-09-30: 44px tap targets on phones for the shared header, footer, BrewSoul/Kava/HumanOS menus and ~100 standalone links (undersized targets 1,904 → 578; the rest are 24-43px pills/chips that meet WCAG 2.2 AA). axe target-size (WCAG 2.2 AA, with its spacing exception): 0 failures on 114 pages. Safari/iPhone (WebKit, iPhone 14 emulation): all 114 pages load, no sideways scroll, no JS errors; form fields under 16px (iOS zoom-on-tap) fixed site-wide in globals.css. Still to check on a real iPhone: BrewSoul's bottom journey bar showed page text through it in headless WebKit only (taps hit the bar correctly; Chrome renders it solid). Fixed 2026-10-09: the bar is now solid (bg-[#2C1810], was 92% plus backdrop-blur-md), so nothing can show through even where the blur isn't drawn; checked in WebKit (iPhone 13 profile) and Chrome: background rgb(44, 24, 16), no text behind the buttons. A real iPhone check is still part of Phase 14. Checked 2026-10-13 in Apple's iPhone Simulator (iPhone 16, iOS 26.5, real Mobile Safari; not a physical phone, owner accepted this as the iPhone check): 14 key pages on a fresh prod</t>
         </is>
       </c>
       <c r="E333" s="14" t="inlineStr">
@@ -8486,7 +8486,7 @@
       <c r="A334" s="4" t="n"/>
       <c r="B334" s="4" t="inlineStr">
         <is>
-          <t>No dead-end pages (every page links to 2+ others)</t>
+          <t>Accessibility pass (WCAG AA contrast, 44px touch targets, keyboard nav)</t>
         </is>
       </c>
       <c r="C334" s="13" t="inlineStr">
@@ -8496,7 +8496,7 @@
       </c>
       <c r="D334" s="4" t="inlineStr">
         <is>
-          <t>same bar as legacy MASTER_QUALITY_PROMPT.md 2026-09-30 scan (496 sitemap pages, header/footer links not counted): every page has a way home (the 6 HumanOS pages had none, in legacy too; added a "← TonyGreenberg.com" footer link). ~17 quiz pages only look like dead ends on their intro screen; their result screens link to related assessments. Left for a content decision: ~20 marketing pages (/akbar, /amplifier, /diamond-cut, /ecosystem, /engage, /engine-room, /intel, /invest, /pick-up-the-phone, /protecting-your-business, /published, /speaking, /the-nightstand, /the-territory, /the-web, /under-nda, /pri-calibration, /charity-scorecard and its detail pages) link to only 0-1 other page in their content. The port matches legacy there (legacy was just as sparse), so adding related links is new content and needs the owner's yes. Done 2026-10-10 (owner said yes): a "Related" section with 3 real links (no redirects, titles and blurbs from each target's own copy) on all 19 sparse pages and every charity profile: data src/lib/content/related-pages.ts, component src/components/marketing/related-pages.tsx (light/dark). Checked at 375/820/1280px with no sideways scroll; found and fixed on the way: the essay date line couldn't wrap on phones (21px sideways on long category names).</t>
+          <t>same bar as legacy QA_MASTER_PROMPT.md. 2026-09-29 axe-core pass (WCAG 2.1 AA, same 114 pages, production build): all unlabeled dropdowns/inputs and unnamed links fixed; contrast down from 1,453 failing items on 106 pages to 1,038 on 70 (43 pages fully clean). Shared fixes: brand gold #8b6914 → #836311 site-wide (was 4.3:1 on cream, AA needs 4.5), header "⌘K"/social icons, BrewSoul nav and footer, HumanOS footer, Kava footer, assessment intro footnote, post-card image links. 2026-09-30: contrast finished, 0 axe color-contrast failures left on the same 114 pages (production build). Token changes: --kava-saffron #b86a28 → #8e521f, --pri-purple-light #a855f7 → #b87bf9 (on-dark purple only), --crusade-teal #0e7c7c → #0d7373; PriEyebrow goes light purple inside a dark PriSection via group-data-dark/pri; /find-your-me and the journey tracker's dark glass panels 60-70% → 90% (legacy's own 60% glass on beige rendered gray, cream text failed). Everything else: nearest passing shade of the same hue, or gold ↔ gold-light on the wrong background. Left: 18 links inside text marked only by color (need an underline), 44px tap targets, keyboard nav. 2026-09-30: 18 color-only in-text links underlined (axe link-in-text-block: 0 left); keyboard focus visible on every focusable item on 8 sampled pages (two form fields had none, fixed). 2026-10-02 re-run (axe WCAG 2.2 AA, 142 pages × 375/1280px, production build, plus Tab through 40 stops per page): found 1,370 contrast failures (mostly BrewSoul'</t>
         </is>
       </c>
       <c r="E334" s="14" t="inlineStr">
@@ -8509,7 +8509,7 @@
       <c r="A335" s="4" t="n"/>
       <c r="B335" s="4" t="inlineStr">
         <is>
-          <t>Cross-browser check (Safari iOS in particular, per legacy performance notes) 2026-10-06 WebKit pass (Playwright WebKit, iPhone 13 profile, 1…</t>
+          <t>No dead-end pages (every page links to 2+ others)</t>
         </is>
       </c>
       <c r="C335" s="13" t="inlineStr">
@@ -8519,7 +8519,7 @@
       </c>
       <c r="D335" s="4" t="inlineStr">
         <is>
-          <t>52 pages: every unique page plus 3 of each templated set, production build): no page pans sideways, no failed requests, no JS errors. Found and fixed on the way: upgrade-insecure-requests in the new CSP made Safari fetch every stylesheet and font over https on localhost (dropped; the site is HTTPS-only via HSTS anyway), and .toLocaleString() without a locale caused a hydration error on /brewsoul/chains in Safari (all number formatting now en-US). Left: a check on a real iPhone (Phase 14). Checked 2026-10-13 in Apple's iPhone Simulator (iPhone 16, iOS 26.5, real Mobile Safari; not a physical phone, owner accepted this as the iPhone check): 14 key pages on a fresh production build (/, /blog, an essay, /brewsoul, /brewsoul/browse, /find-your-journey, /psychedelic-readiness-index, /kava, /humanos, /about, /iboga-ibogaine, /peptide-hall-of-shame, /my-journey, /pri-calibration): all render, no sideways pan, header and menus in place, BrewSoul's bottom bar solid. / and /blog showed blank on the very first cold load, then load within 3 s on every later visit.</t>
+          <t>same bar as legacy MASTER_QUALITY_PROMPT.md 2026-09-30 scan (496 sitemap pages, header/footer links not counted): every page has a way home (the 6 HumanOS pages had none, in legacy too; added a "← TonyGreenberg.com" footer link). ~17 quiz pages only look like dead ends on their intro screen; their result screens link to related assessments. Left for a content decision: ~20 marketing pages (/akbar, /amplifier, /diamond-cut, /ecosystem, /engage, /engine-room, /intel, /invest, /pick-up-the-phone, /protecting-your-business, /published, /speaking, /the-nightstand, /the-territory, /the-web, /under-nda, /pri-calibration, /charity-scorecard and its detail pages) link to only 0-1 other page in their content. The port matches legacy there (legacy was just as sparse), so adding related links is new content and needs the owner's yes. Done 2026-10-10 (owner said yes): a "Related" section with 3 real links (no redirects, titles and blurbs from each target's own copy) on all 19 sparse pages and every charity profile: data src/lib/content/related-pages.ts, component src/components/marketing/related-pages.tsx (light/dark). Checked at 375/820/1280px with no sideways scroll; found and fixed on the way: the essay date line couldn't wrap on phones (21px sideways on long category names).</t>
         </is>
       </c>
       <c r="E335" s="14" t="inlineStr">
@@ -8532,7 +8532,7 @@
       <c r="A336" s="4" t="n"/>
       <c r="B336" s="4" t="inlineStr">
         <is>
-          <t>Remove noindex only when sign-off is given</t>
+          <t>Cross-browser check (Safari iOS in particular, per legacy performance notes) 2026-10-06 WebKit pass (Playwright WebKit, iPhone 13 profile, 1…</t>
         </is>
       </c>
       <c r="C336" s="13" t="inlineStr">
@@ -8542,7 +8542,7 @@
       </c>
       <c r="D336" s="4" t="inlineStr">
         <is>
-          <t>do not launch indexable by accident (The only noindex is the host-based one for .netlify.app above, so the real domain is indexable as soon as DNS points at it: sign-off must come before DNS.) Re-checked 2026-10-13 on a fresh production build: tonygreenberg.com and www get no X-Robots-Tag and no robots meta (/, /blog, /about, /post-intervention), *.netlify.app gets noindex, nofollow; robots.txt allows crawlers, sitemap 200, missing pages 404, /manifesto 308. Ready; still waits on sign-off. Done 2026-10-13 (sign-off given): nothing to switch off. The only noindex is host-based (.netlify.app), so tonygreenberg.com becomes indexable by Google the moment DNS points at Netlify (re-checked on today's build: no X-Robots-Tag or robots meta for the real domain).</t>
+          <t>52 pages: every unique page plus 3 of each templated set, production build): no page pans sideways, no failed requests, no JS errors. Found and fixed on the way: upgrade-insecure-requests in the new CSP made Safari fetch every stylesheet and font over https on localhost (dropped; the site is HTTPS-only via HSTS anyway), and .toLocaleString() without a locale caused a hydration error on /brewsoul/chains in Safari (all number formatting now en-US). Left: a check on a real iPhone (Phase 14). Checked 2026-10-13 in Apple's iPhone Simulator (iPhone 16, iOS 26.5, real Mobile Safari; not a physical phone, owner accepted this as the iPhone check): 14 key pages on a fresh production build (/, /blog, an essay, /brewsoul, /brewsoul/browse, /find-your-journey, /psychedelic-readiness-index, /kava, /humanos, /about, /iboga-ibogaine, /peptide-hall-of-shame, /my-journey, /pri-calibration): all render, no sideways pan, header and menus in place, BrewSoul's bottom bar solid. / and /blog showed blank on the very first cold load, then load within 3 s on every later visit.</t>
         </is>
       </c>
       <c r="E336" s="14" t="inlineStr">
@@ -8555,7 +8555,7 @@
       <c r="A337" s="4" t="n"/>
       <c r="B337" s="4" t="inlineStr">
         <is>
-          <t>Final stakeholder sign-off (Tony/Darryl/Kimberly) on the ported site before DNS cutover Given 2026-10-13 by the webmaster (web.master@rampra…</t>
+          <t>Remove noindex only when sign-off is given</t>
         </is>
       </c>
       <c r="C337" s="13" t="inlineStr">
@@ -8565,7 +8565,7 @@
       </c>
       <c r="D337" s="4" t="inlineStr">
         <is>
-          <t>te.com) in a Claude Code session, answering "Tony's team sign-off, then turning on Google indexing" with yes. If Tony, Darryl or Kimberly haven't seen the Netlify copy themselves, get their yes before the DNS switch.</t>
+          <t>do not launch indexable by accident (The only noindex is the host-based one for .netlify.app above, so the real domain is indexable as soon as DNS points at it: sign-off must come before DNS.) Re-checked 2026-10-13 on a fresh production build: tonygreenberg.com and www get no X-Robots-Tag and no robots meta (/, /blog, /about, /post-intervention), *.netlify.app gets noindex, nofollow; robots.txt allows crawlers, sitemap 200, missing pages 404, /manifesto 308. Ready; still waits on sign-off. Done 2026-10-13 (sign-off given): nothing to switch off. The only noindex is host-based (.netlify.app), so tonygreenberg.com becomes indexable by Google the moment DNS points at Netlify (re-checked on today's build: no X-Robots-Tag or robots meta for the real domain).</t>
         </is>
       </c>
       <c r="E337" s="14" t="inlineStr">
@@ -8578,7 +8578,7 @@
       <c r="A338" s="4" t="n"/>
       <c r="B338" s="4" t="inlineStr">
         <is>
-          <t>Privacy Policy page (/privacy) + footer link</t>
+          <t>Final stakeholder sign-off (Tony/Darryl/Kimberly) on the ported site before DNS cutover Given 2026-10-13 by the webmaster (web.master@rampra…</t>
         </is>
       </c>
       <c r="C338" s="13" t="inlineStr">
@@ -8588,7 +8588,7 @@
       </c>
       <c r="D338" s="4" t="inlineStr">
         <is>
-          <t>(team review 2026-10-14; owner: "create any page that isn't there"). Neither live nor the old app has one, so it's a new page. Wording drafted from what the code really does: newsletter (Kit), member accounts, quiz results (sexuality/religion save only "finished"), comments/reactions/highlights, the site's forms (Supabase, emailed to Tony via Resend), supplier intake to RampRate, Google Analytics, the sign-in, tg_visit_count and visitor-session cookies, browser storage. Contact for requests: t@ramprate.com (the footer's address). Josh (legal) to review the wording before launch.</t>
+          <t>te.com) in a Claude Code session, answering "Tony's team sign-off, then turning on Google indexing" with yes. If Tony, Darryl or Kimberly haven't seen the Netlify copy themselves, get their yes before the DNS switch.</t>
         </is>
       </c>
       <c r="E338" s="14" t="inlineStr">
@@ -8601,7 +8601,7 @@
       <c r="A339" s="4" t="n"/>
       <c r="B339" s="4" t="inlineStr">
         <is>
-          <t>Terms of Use page (/terms) + footer link</t>
+          <t>Privacy Policy page (/privacy) + footer link</t>
         </is>
       </c>
       <c r="C339" s="13" t="inlineStr">
@@ -8611,7 +8611,7 @@
       </c>
       <c r="D339" s="4" t="inlineStr">
         <is>
-          <t>(team review 2026-10-14). Not-medical-advice (peptides, diet, therapy, kava, psychedelics, ibogaine) and not-investment-advice (waitlists are not offers) sections, ownership matching the footer notice, user content, liability, California law. /terms was one of the intentional 404s; now a real page (ROUTES-INVENTORY.md updated). Josh (legal) to review before launch.</t>
+          <t>(team review 2026-10-14; owner: "create any page that isn't there"). Neither live nor the old app has one, so it's a new page. Wording drafted from what the code really does: newsletter (Kit), member accounts, quiz results (sexuality/religion save only "finished"), comments/reactions/highlights, the site's forms (Supabase, emailed to Tony via Resend), supplier intake to RampRate, Google Analytics, the sign-in, tg_visit_count and visitor-session cookies, browser storage. Contact for requests: t@ramprate.com (the footer's address). Josh (legal) to review the wording before launch.</t>
         </is>
       </c>
       <c r="E339" s="14" t="inlineStr">
@@ -8624,7 +8624,7 @@
       <c r="A340" s="4" t="n"/>
       <c r="B340" s="4" t="inlineStr">
         <is>
-          <t>Contact page (/contact) + footer link</t>
+          <t>Terms of Use page (/terms) + footer link</t>
         </is>
       </c>
       <c r="C340" s="13" t="inlineStr">
@@ -8634,7 +8634,7 @@
       </c>
       <c r="D340" s="4" t="inlineStr">
         <is>
-          <t>(team review 2026-10-14). Gathers details already on the site: email t@ramprate.com (now also a clickable link in the footer, where it was plain text), booking link, the Engagement Audit (/pick-up-the-phone), RampRate supplier intake, Santa Monica, X and LinkedIn. No form (none needed: every option already exists). Checked 2026-10-14 for all three: type check, lint, Manus grep, build (all ○ static), fresh server: 200, one H1, title, canonical, share image, in the sitemap and Ask Tony search, footer links on every page; browser at 375/820/1280 light and 375/1280 dark: no sideways scroll, no JS errors.</t>
+          <t>(team review 2026-10-14). Not-medical-advice (peptides, diet, therapy, kava, psychedelics, ibogaine) and not-investment-advice (waitlists are not offers) sections, ownership matching the footer notice, user content, liability, California law. /terms was one of the intentional 404s; now a real page (ROUTES-INVENTORY.md updated). Josh (legal) to review before launch.</t>
         </is>
       </c>
       <c r="E340" s="14" t="inlineStr">
@@ -8647,7 +8647,7 @@
       <c r="A341" s="4" t="n"/>
       <c r="B341" s="4" t="inlineStr">
         <is>
-          <t>Essay counts match</t>
+          <t>Contact page (/contact) + footer link</t>
         </is>
       </c>
       <c r="C341" s="13" t="inlineStr">
@@ -8657,7 +8657,7 @@
       </c>
       <c r="D341" s="4" t="inlineStr">
         <is>
-          <t>(team review 2026-10-14). Ask Tony's Blog entry said "92 essays" (copied from the old app), the homepage Read card "118", /subscribe and /the-letter's Read card "121", while the homepage and /search count 123 from Sanity. All now use Sanity's count ({count} in home-doors.ts and /the-letter's doors, /subscribe fetches it). Ask Tony (owner: show the number): the root layout fetches the count and passes it to SiteHeader → SearchModal; withEssayCount() in search-directory.ts fills {count} for Ask Tony, /search and /the-index too. Checked in a browser: Ask Tony shows "123 essays spanning 15 years", build still 150 static / 28 dynamic pages as before. Left alone: /living-declaration's "QPR Index scores intellectual rigor across 91 essays" (a claim about that tool, Tony's copy). Checked 2026-10-14: type check, lint, build (/, /subscribe, /the-letter still static), fresh server: all three show 123, no "92 essays" in the built browser code.</t>
+          <t>(team review 2026-10-14). Gathers details already on the site: email t@ramprate.com (now also a clickable link in the footer, where it was plain text), booking link, the Engagement Audit (/pick-up-the-phone), RampRate supplier intake, Santa Monica, X and LinkedIn. No form (none needed: every option already exists). Checked 2026-10-14 for all three: type check, lint, Manus grep, build (all ○ static), fresh server: 200, one H1, title, canonical, share image, in the sitemap and Ask Tony search, footer links on every page; browser at 375/820/1280 light and 375/1280 dark: no sideways scroll, no JS errors.</t>
         </is>
       </c>
       <c r="E341" s="14" t="inlineStr">
@@ -8670,7 +8670,7 @@
       <c r="A342" s="4" t="n"/>
       <c r="B342" s="4" t="inlineStr">
         <is>
-          <t>Team review's "everything else looks fine" re-checked</t>
+          <t>Essay counts match</t>
         </is>
       </c>
       <c r="C342" s="13" t="inlineStr">
@@ -8680,7 +8680,7 @@
       </c>
       <c r="D342" s="4" t="inlineStr">
         <is>
-          <t>(2026-10-14, owner: "you can check"). Fresh production build: all 60 menu pages (main menu, Fix Myself, Explore...) at 1280px and 375px: 200, one H1, no sideways scroll, no JS errors. All 130 blog links on them (122 posts, 8 categories): 200, no redirects. 404 page: 404 for a missing page, essay and category. Dark mode: switches and stays on across pages; 10 essays checked on a phone in dark mode. Phone menu shows every section; Ask Tony works on a phone. Netlify test site: the same 60 menu pages answer. Two small fixes: a missing essay or category showed the homepage's tab title on its 404 page (now "Page not found"); three Explore links (/attention-theft/weapons, /report, /legal) went through a redirect, now link straight to /attention-theft#weapons etc. Checked: type check, lint, build, clicked "Legal Database" in the menu.</t>
+          <t>(team review 2026-10-14). Ask Tony's Blog entry said "92 essays" (copied from the old app), the homepage Read card "118", /subscribe and /the-letter's Read card "121", while the homepage and /search count 123 from Sanity. All now use Sanity's count ({count} in home-doors.ts and /the-letter's doors, /subscribe fetches it). Ask Tony (owner: show the number): the root layout fetches the count and passes it to SiteHeader → SearchModal; withEssayCount() in search-directory.ts fills {count} for Ask Tony, /search and /the-index too. Checked in a browser: Ask Tony shows "123 essays spanning 15 years", build still 150 static / 28 dynamic pages as before. Left alone: /living-declaration's "QPR Index scores intellectual rigor across 91 essays" (a claim about that tool, Tony's copy). Checked 2026-10-14: type check, lint, build (/, /subscribe, /the-letter still static), fresh server: all three show 123, no "92 essays" in the built browser code.</t>
         </is>
       </c>
       <c r="E342" s="14" t="inlineStr">
@@ -8693,42 +8693,65 @@
       <c r="A343" s="4" t="n"/>
       <c r="B343" s="4" t="inlineStr">
         <is>
+          <t>Team review's "everything else looks fine" re-checked</t>
+        </is>
+      </c>
+      <c r="C343" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D343" s="4" t="inlineStr">
+        <is>
+          <t>(2026-10-14, owner: "you can check"). Fresh production build: all 60 menu pages (main menu, Fix Myself, Explore...) at 1280px and 375px: 200, one H1, no sideways scroll, no JS errors. All 130 blog links on them (122 posts, 8 categories): 200, no redirects. 404 page: 404 for a missing page, essay and category. Dark mode: switches and stays on across pages; 10 essays checked on a phone in dark mode. Phone menu shows every section; Ask Tony works on a phone. Netlify test site: the same 60 menu pages answer. Two small fixes: a missing essay or category showed the homepage's tab title on its 404 page (now "Page not found"); three Explore links (/attention-theft/weapons, /report, /legal) went through a redirect, now link straight to /attention-theft#weapons etc. Checked: type check, lint, build, clicked "Legal Database" in the menu.</t>
+        </is>
+      </c>
+      <c r="E343" s="14" t="inlineStr">
+        <is>
+          <t>Phase 14 — QA &amp; Launch</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" s="4" t="n"/>
+      <c r="B344" s="4" t="inlineStr">
+        <is>
           <t>DNS cutover, legacy app decommissioned only after a stable overlap window Re-checked 2026-10-13</t>
         </is>
       </c>
-      <c r="C343" s="16" t="inlineStr">
+      <c r="C344" s="16" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
       </c>
-      <c r="D343" s="4" t="inlineStr">
+      <c r="D344" s="4" t="inlineStr">
         <is>
           <t>unchanged (Hostinger name servers, bare domain on Manus 104.19.168/169.112, www CNAME cname.manus.space). Checked 2026-10-09 (owner wants to go live and switch off Manus): DNS for tonygreenberg.com is at Hostinger (name servers ns1/ns2.dns-parking.com); www is a CNAME to cname.manus.space, the bare domain points at Manus's addresses (104.19.168.112 / .169.112); the Netlify site tonygreenberg-website has no custom domain yet (production branch main). Order: (1) merge the three open pull requests into main and check the Netlify copy; (2) restore Supabase and run 0001 to 0003, or launch without member features (they say "isn't available just now"); (3) owner sign-off; (4) add tonygreenberg.com + www in Netlify (Domain management), then at Hostinger point the bare domain at Netlify (A record 75.2.60.5, or Netlify DNS) and www CNAME at tonygreenberg-website.netlify.app; Netlify issues the HTTPS certificate; (5) re-run scripts/check-search-console-urls.ts https://tonygreenberg.com and submit the sitemap in Search Console; (6) only after a few stable days: switch off the Manus site (the database is already backed up, docs/ai/project_legacy_database.md) and rotate the old database password.</t>
         </is>
       </c>
-      <c r="E343" s="14" t="inlineStr">
+      <c r="E344" s="14" t="inlineStr">
         <is>
           <t>Phase 14 — QA &amp; Launch</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D343"/>
+  <autoFilter ref="A1:D344"/>
   <mergeCells count="14">
-    <mergeCell ref="A211:D211"/>
-    <mergeCell ref="A189:D189"/>
-    <mergeCell ref="A243:D243"/>
-    <mergeCell ref="A215:D215"/>
-    <mergeCell ref="A311:D311"/>
+    <mergeCell ref="A312:D312"/>
+    <mergeCell ref="A244:D244"/>
+    <mergeCell ref="A157:D157"/>
     <mergeCell ref="A15:D15"/>
     <mergeCell ref="A64:D64"/>
-    <mergeCell ref="A156:D156"/>
+    <mergeCell ref="A332:D332"/>
+    <mergeCell ref="A212:D212"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A49:D49"/>
     <mergeCell ref="A129:D129"/>
-    <mergeCell ref="A331:D331"/>
+    <mergeCell ref="A190:D190"/>
+    <mergeCell ref="A216:D216"/>
+    <mergeCell ref="A265:D265"/>
     <mergeCell ref="A32:D32"/>
-    <mergeCell ref="A264:D264"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Curated Journeys filter the essay archive instead of a dead-end link
Every journey linked to /journeys, where 5 of the 7 don't exist. A click
now filters the archive on "/" and "/blog" to that journey's essays and
scrolls to them; counts are the published essays in each journey.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Migration-Status-Report.xlsx
+++ b/Migration-Status-Report.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Remaining Work" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Full Detail'!$A$1:$D$344</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Full Detail'!$A$1:$D$345</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Remaining Work'!$A$1:$D$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -639,15 +639,15 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A5,'Full Detail'!$C$2:$C$344,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$345,$A5,'Full Detail'!$C$2:$C$345,"Done")</f>
         <v/>
       </c>
       <c r="C5" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A5,'Full Detail'!$C$2:$C$344,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$345,$A5,'Full Detail'!$C$2:$C$345,"Remaining")</f>
         <v/>
       </c>
       <c r="D5" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A5,'Full Detail'!$C$2:$C$344,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$345,$A5,'Full Detail'!$C$2:$C$345,"Deferred")</f>
         <v/>
       </c>
       <c r="E5" s="5">
@@ -666,15 +666,15 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A6,'Full Detail'!$C$2:$C$344,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$345,$A6,'Full Detail'!$C$2:$C$345,"Done")</f>
         <v/>
       </c>
       <c r="C6" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A6,'Full Detail'!$C$2:$C$344,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$345,$A6,'Full Detail'!$C$2:$C$345,"Remaining")</f>
         <v/>
       </c>
       <c r="D6" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A6,'Full Detail'!$C$2:$C$344,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$345,$A6,'Full Detail'!$C$2:$C$345,"Deferred")</f>
         <v/>
       </c>
       <c r="E6" s="5">
@@ -693,15 +693,15 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A7,'Full Detail'!$C$2:$C$344,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$345,$A7,'Full Detail'!$C$2:$C$345,"Done")</f>
         <v/>
       </c>
       <c r="C7" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A7,'Full Detail'!$C$2:$C$344,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$345,$A7,'Full Detail'!$C$2:$C$345,"Remaining")</f>
         <v/>
       </c>
       <c r="D7" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A7,'Full Detail'!$C$2:$C$344,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$345,$A7,'Full Detail'!$C$2:$C$345,"Deferred")</f>
         <v/>
       </c>
       <c r="E7" s="5">
@@ -720,15 +720,15 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A8,'Full Detail'!$C$2:$C$344,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$345,$A8,'Full Detail'!$C$2:$C$345,"Done")</f>
         <v/>
       </c>
       <c r="C8" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A8,'Full Detail'!$C$2:$C$344,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$345,$A8,'Full Detail'!$C$2:$C$345,"Remaining")</f>
         <v/>
       </c>
       <c r="D8" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A8,'Full Detail'!$C$2:$C$344,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$345,$A8,'Full Detail'!$C$2:$C$345,"Deferred")</f>
         <v/>
       </c>
       <c r="E8" s="5">
@@ -747,15 +747,15 @@
         </is>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A9,'Full Detail'!$C$2:$C$344,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$345,$A9,'Full Detail'!$C$2:$C$345,"Done")</f>
         <v/>
       </c>
       <c r="C9" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A9,'Full Detail'!$C$2:$C$344,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$345,$A9,'Full Detail'!$C$2:$C$345,"Remaining")</f>
         <v/>
       </c>
       <c r="D9" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A9,'Full Detail'!$C$2:$C$344,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$345,$A9,'Full Detail'!$C$2:$C$345,"Deferred")</f>
         <v/>
       </c>
       <c r="E9" s="5">
@@ -774,15 +774,15 @@
         </is>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A10,'Full Detail'!$C$2:$C$344,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$345,$A10,'Full Detail'!$C$2:$C$345,"Done")</f>
         <v/>
       </c>
       <c r="C10" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A10,'Full Detail'!$C$2:$C$344,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$345,$A10,'Full Detail'!$C$2:$C$345,"Remaining")</f>
         <v/>
       </c>
       <c r="D10" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A10,'Full Detail'!$C$2:$C$344,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$345,$A10,'Full Detail'!$C$2:$C$345,"Deferred")</f>
         <v/>
       </c>
       <c r="E10" s="5">
@@ -801,15 +801,15 @@
         </is>
       </c>
       <c r="B11" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A11,'Full Detail'!$C$2:$C$344,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$345,$A11,'Full Detail'!$C$2:$C$345,"Done")</f>
         <v/>
       </c>
       <c r="C11" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A11,'Full Detail'!$C$2:$C$344,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$345,$A11,'Full Detail'!$C$2:$C$345,"Remaining")</f>
         <v/>
       </c>
       <c r="D11" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A11,'Full Detail'!$C$2:$C$344,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$345,$A11,'Full Detail'!$C$2:$C$345,"Deferred")</f>
         <v/>
       </c>
       <c r="E11" s="5">
@@ -828,15 +828,15 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A12,'Full Detail'!$C$2:$C$344,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$345,$A12,'Full Detail'!$C$2:$C$345,"Done")</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A12,'Full Detail'!$C$2:$C$344,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$345,$A12,'Full Detail'!$C$2:$C$345,"Remaining")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A12,'Full Detail'!$C$2:$C$344,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$345,$A12,'Full Detail'!$C$2:$C$345,"Deferred")</f>
         <v/>
       </c>
       <c r="E12" s="5">
@@ -855,15 +855,15 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A13,'Full Detail'!$C$2:$C$344,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$345,$A13,'Full Detail'!$C$2:$C$345,"Done")</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A13,'Full Detail'!$C$2:$C$344,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$345,$A13,'Full Detail'!$C$2:$C$345,"Remaining")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A13,'Full Detail'!$C$2:$C$344,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$345,$A13,'Full Detail'!$C$2:$C$345,"Deferred")</f>
         <v/>
       </c>
       <c r="E13" s="5">
@@ -882,15 +882,15 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A14,'Full Detail'!$C$2:$C$344,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$345,$A14,'Full Detail'!$C$2:$C$345,"Done")</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A14,'Full Detail'!$C$2:$C$344,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$345,$A14,'Full Detail'!$C$2:$C$345,"Remaining")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A14,'Full Detail'!$C$2:$C$344,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$345,$A14,'Full Detail'!$C$2:$C$345,"Deferred")</f>
         <v/>
       </c>
       <c r="E14" s="5">
@@ -909,15 +909,15 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A15,'Full Detail'!$C$2:$C$344,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$345,$A15,'Full Detail'!$C$2:$C$345,"Done")</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A15,'Full Detail'!$C$2:$C$344,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$345,$A15,'Full Detail'!$C$2:$C$345,"Remaining")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A15,'Full Detail'!$C$2:$C$344,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$345,$A15,'Full Detail'!$C$2:$C$345,"Deferred")</f>
         <v/>
       </c>
       <c r="E15" s="5">
@@ -936,15 +936,15 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A16,'Full Detail'!$C$2:$C$344,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$345,$A16,'Full Detail'!$C$2:$C$345,"Done")</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A16,'Full Detail'!$C$2:$C$344,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$345,$A16,'Full Detail'!$C$2:$C$345,"Remaining")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A16,'Full Detail'!$C$2:$C$344,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$345,$A16,'Full Detail'!$C$2:$C$345,"Deferred")</f>
         <v/>
       </c>
       <c r="E16" s="5">
@@ -963,15 +963,15 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A17,'Full Detail'!$C$2:$C$344,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$345,$A17,'Full Detail'!$C$2:$C$345,"Done")</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A17,'Full Detail'!$C$2:$C$344,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$345,$A17,'Full Detail'!$C$2:$C$345,"Remaining")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A17,'Full Detail'!$C$2:$C$344,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$345,$A17,'Full Detail'!$C$2:$C$345,"Deferred")</f>
         <v/>
       </c>
       <c r="E17" s="5">
@@ -990,15 +990,15 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A18,'Full Detail'!$C$2:$C$344,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$345,$A18,'Full Detail'!$C$2:$C$345,"Done")</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A18,'Full Detail'!$C$2:$C$344,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$345,$A18,'Full Detail'!$C$2:$C$345,"Remaining")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A18,'Full Detail'!$C$2:$C$344,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$345,$A18,'Full Detail'!$C$2:$C$345,"Deferred")</f>
         <v/>
       </c>
       <c r="E18" s="5">
@@ -1017,15 +1017,15 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A19,'Full Detail'!$C$2:$C$344,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$345,$A19,'Full Detail'!$C$2:$C$345,"Done")</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A19,'Full Detail'!$C$2:$C$344,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$345,$A19,'Full Detail'!$C$2:$C$345,"Remaining")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$344,$A19,'Full Detail'!$C$2:$C$344,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$345,$A19,'Full Detail'!$C$2:$C$345,"Deferred")</f>
         <v/>
       </c>
       <c r="E19" s="5">
@@ -1075,7 +1075,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E344"/>
+  <dimension ref="A1:E345"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -4516,63 +4516,63 @@
       <c r="A156" s="4" t="n"/>
       <c r="B156" s="4" t="inlineStr">
         <is>
+          <t>Curated Journeys sidebar checked and fixed</t>
+        </is>
+      </c>
+      <c r="C156" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D156" s="4" t="inlineStr">
+        <is>
+          <t>(owner, 2026-10-14: "check it's real data"). All 29 essays in the 7 journeys exist in Sanity and the counts match live (5, 4, 4, 4, 4, 4, 4). But every journey linked to /journeys, where 5 of the 7 don't exist (dead end, same on live). Now a click filters the archive to that journey's essays ("Curated Journey: ..." heading, "Show all essays" to clear) and scrolls to them; counts come from published essays (journeyCounts in summarizeArchive). Checked in a browser on / and /blog: all 7 journeys show exactly their essays, no JS errors. Also found: Most Read / Most Provocative match live's lists, but live's "19,694 reads" are numbers typed into the old site's data file, not real. GA4 works from this repo and shows a very different real top list (When Healing Becomes Extraction 690 views in 12 months, Your Blood Lies Without Your DNA 222, The 1000-Hour Hold 196...); there is no real data for "Most Provocative" (4 reactions, 0 comments in Supabase). Owner to decide whether Most Read should switch to real Google Analytics data.</t>
+        </is>
+      </c>
+      <c r="E156" s="14" t="inlineStr">
+        <is>
+          <t>Phase 5 — Blog Engine (Sanity-backed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="4" t="n"/>
+      <c r="B157" s="4" t="inlineStr">
+        <is>
           <t>Essay archive: search suggestions + more filters</t>
         </is>
       </c>
-      <c r="C156" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D156" s="4" t="inlineStr">
+      <c r="C157" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D157" s="4" t="inlineStr">
         <is>
           <t>(owner asked 2026-10-14, chose: search-as-you-type, and sort, year, reading time, topic). The archive at the bottom of / (and on /blog) was already live data (Sanity, newest first, refreshed within 60s or by the webhook; every essay on live's sitemap is in Sanity). Added: archive-search-box.tsx, a dropdown while typing with matching categories and topics (instant) and essays from /api/search (also matches words inside the essay text); arrow keys + Enter, Escape. Filters: Newest/Oldest, Year, Reading time (under 5, 5 to 10, over 10 min) and Topic (tags used by 3+ essays, about 30 of 874), with "Clear filters"; on phones they fold behind a "Filters" button. Reading time uses the editor's value or a word-count estimate (minutes in allPostsForArchiveQuery; only 34 of 123 posts had one). Checked: type check, lint, build (150 static / 28 dynamic, unchanged), browser on a fresh server: every filter count matches the data (year 2010: 21, neuroscience: 13, 5 to 10 min: 52...), "kurzweil" suggests the H+ essays and Enter opens one, picking a topic suggestion sets the Topic filter; 375 light/dark, 820, 1280: no sideways scroll, no JS errors.</t>
         </is>
       </c>
-      <c r="E156" s="14" t="inlineStr">
+      <c r="E157" s="14" t="inlineStr">
         <is>
           <t>Phase 5 — Blog Engine (Sanity-backed)</t>
         </is>
       </c>
     </row>
-    <row r="157">
-      <c r="A157" s="10" t="inlineStr">
+    <row r="158">
+      <c r="A158" s="10" t="inlineStr">
         <is>
           <t>Phase 6 — BrewSoul (28 routes)</t>
         </is>
       </c>
-      <c r="B157" s="11" t="n"/>
-      <c r="C157" s="11" t="n"/>
-      <c r="D157" s="12" t="n"/>
-    </row>
-    <row r="158">
-      <c r="A158" s="4" t="n"/>
-      <c r="B158" s="4" t="inlineStr">
-        <is>
-          <t>/brewsoul</t>
-        </is>
-      </c>
-      <c r="C158" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D158" s="4" t="inlineStr">
-        <is>
-          <t>welcome/landing gate (built, not yet pushed — pending local review), along with the shared foundation the rest of Phase 6 depends on. Ported BrewSoulLayout.tsx → app/brewsoul/layout.tsx + components/brewsoul/brewsoul-nav.tsx (BrewSoulNav/BrewSoulFooter), CategoryBadge.tsx → components/brewsoul/category-badge.tsx, brewsoul-config.ts → lib/content/brewsoul-config.ts, and BrewSoulDirectory.tsx's CATEGORIES/PAGE_CATEGORY_MAP data (not the page itself yet) → lib/content/brewsoul-directory.ts. Real architecture decision: BrewSoul is a self-contained sub-site with its own nav/footer/coffee-brown palette, same as legacy — but this app has one flat root layout with no route groups, so the main site's SiteHeader/SiteFooter needed to be suppressed for this one subtree without restructuring every existing route. Added components/site-chrome.tsx (SiteChrome, a small client wrapper checking pathname.startsWith("/brewsoul")) around both in app/layout.tsx — verified via literal &lt;header&gt;/&lt;footer&gt;/&lt;nav&gt; tag counts in real SSR HTML (not text search, which false-positives on Next dev mode's RSC debug payload) that /brewsoul gets zero main-site chrome and its own real nav+footer, while / still gets exactly one of each. Dropped TonyAvatarTrigger (FauxTony chatbot widget — Phase 10, no backend yet, same "don't fake it" call made elsewhere) from the nav. Ported BrewSoulWelcome.tsx → components/brewsoul/brewsoul-welcome-quiz.tsx (8-screen onboarding quiz, real identity-scoring logic, palate questions</t>
-        </is>
-      </c>
-      <c r="E158" s="14" t="inlineStr">
-        <is>
-          <t>Phase 6 — BrewSoul (28 routes)</t>
-        </is>
-      </c>
+      <c r="B158" s="11" t="n"/>
+      <c r="C158" s="11" t="n"/>
+      <c r="D158" s="12" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="4" t="n"/>
       <c r="B159" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/first-sip</t>
+          <t>/brewsoul</t>
         </is>
       </c>
       <c r="C159" s="13" t="inlineStr">
@@ -4582,7 +4582,7 @@
       </c>
       <c r="D159" s="4" t="inlineStr">
         <is>
-          <t>onboarding intro (built, not yet pushed — pending local review). Ported "The First Sip Is a Vote" in full — the complete manifesto essay (5 sections, 3 pullquotes, the couplets block, the disclosure-demands grid), the 5-tool journey map, 6 related-essay links (real slugs, cross-checked against this session's already-verified corpus), the closing + sources, and the email capture. Built as a Server Component (all static except the email form) + components/brewsoul/next-steps.tsx (shared "what's next" CTA, itself a Server Component — legacy's hover effects were plain CSS-able, no JS state needed) + components/brewsoul/first-sip-email-capture.tsx (client island, mailto: fallback since no subscribe backend exists, same pattern as newsletter-popup.tsx). Dropped the canvas CoffeeDust decoration and the confirmed-dead hero photo (/api/img/brewsoul-orig_84eb4bc9.jpg, 404, same Manus proxy) — with no image left, the scroll-linked parallax that moved it went too. The 5 tool-card links (prescription/health/pairings/economics/compare) point at later Phase 6 routes not built yet — same forward-reference pattern as /find-my. Verified live: 200 OK, full essay text present, CategoryBadge correctly shows "Start Here" (from PAGE_CATEGORY_MAP), zero main-site chrome leaking in, typecheck/lint clean.</t>
+          <t>welcome/landing gate (built, not yet pushed — pending local review), along with the shared foundation the rest of Phase 6 depends on. Ported BrewSoulLayout.tsx → app/brewsoul/layout.tsx + components/brewsoul/brewsoul-nav.tsx (BrewSoulNav/BrewSoulFooter), CategoryBadge.tsx → components/brewsoul/category-badge.tsx, brewsoul-config.ts → lib/content/brewsoul-config.ts, and BrewSoulDirectory.tsx's CATEGORIES/PAGE_CATEGORY_MAP data (not the page itself yet) → lib/content/brewsoul-directory.ts. Real architecture decision: BrewSoul is a self-contained sub-site with its own nav/footer/coffee-brown palette, same as legacy — but this app has one flat root layout with no route groups, so the main site's SiteHeader/SiteFooter needed to be suppressed for this one subtree without restructuring every existing route. Added components/site-chrome.tsx (SiteChrome, a small client wrapper checking pathname.startsWith("/brewsoul")) around both in app/layout.tsx — verified via literal &lt;header&gt;/&lt;footer&gt;/&lt;nav&gt; tag counts in real SSR HTML (not text search, which false-positives on Next dev mode's RSC debug payload) that /brewsoul gets zero main-site chrome and its own real nav+footer, while / still gets exactly one of each. Dropped TonyAvatarTrigger (FauxTony chatbot widget — Phase 10, no backend yet, same "don't fake it" call made elsewhere) from the nav. Ported BrewSoulWelcome.tsx → components/brewsoul/brewsoul-welcome-quiz.tsx (8-screen onboarding quiz, real identity-scoring logic, palate questions</t>
         </is>
       </c>
       <c r="E159" s="14" t="inlineStr">
@@ -4595,7 +4595,7 @@
       <c r="A160" s="4" t="n"/>
       <c r="B160" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/home</t>
+          <t>/brewsoul/first-sip</t>
         </is>
       </c>
       <c r="C160" s="13" t="inlineStr">
@@ -4605,7 +4605,7 @@
       </c>
       <c r="D160" s="4" t="inlineStr">
         <is>
-          <t>the real BrewSoul dashboard (distinct from /brewsoul's identity-quiz welcome gate and /brewsoul/first-sip's manifesto): hero + stats, Follow the Dollar teaser, Top QPR coffees (computed live via computeQPR), the 2025 crisis callout, New Drops, a Wall of Shame preview (SHAME_ENTRIES), the research-hub card grid, and a cyclable health-fact ticker (components/brewsoul/health-ticker.tsx, its own small client island so the rest of the page stays a Server Component). Canvas WarmParticles/ParallaxBg decorations and the dead hero photo (/api/img/brewsoul-orig_84eb4bc9.jpg, same confirmed-404 Manus proxy used elsewhere in Phase 6) dropped for CSS gradients. Stats use the real live BREWSOUL_COFFEES.length (107) in place of legacy's stale "103". Verified live: 200 OK.</t>
+          <t>onboarding intro (built, not yet pushed — pending local review). Ported "The First Sip Is a Vote" in full — the complete manifesto essay (5 sections, 3 pullquotes, the couplets block, the disclosure-demands grid), the 5-tool journey map, 6 related-essay links (real slugs, cross-checked against this session's already-verified corpus), the closing + sources, and the email capture. Built as a Server Component (all static except the email form) + components/brewsoul/next-steps.tsx (shared "what's next" CTA, itself a Server Component — legacy's hover effects were plain CSS-able, no JS state needed) + components/brewsoul/first-sip-email-capture.tsx (client island, mailto: fallback since no subscribe backend exists, same pattern as newsletter-popup.tsx). Dropped the canvas CoffeeDust decoration and the confirmed-dead hero photo (/api/img/brewsoul-orig_84eb4bc9.jpg, 404, same Manus proxy) — with no image left, the scroll-linked parallax that moved it went too. The 5 tool-card links (prescription/health/pairings/economics/compare) point at later Phase 6 routes not built yet — same forward-reference pattern as /find-my. Verified live: 200 OK, full essay text present, CategoryBadge correctly shows "Start Here" (from PAGE_CATEGORY_MAP), zero main-site chrome leaking in, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E160" s="14" t="inlineStr">
@@ -4618,7 +4618,7 @@
       <c r="A161" s="4" t="n"/>
       <c r="B161" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/browse</t>
+          <t>/brewsoul/home</t>
         </is>
       </c>
       <c r="C161" s="13" t="inlineStr">
@@ -4628,7 +4628,7 @@
       </c>
       <c r="D161" s="4" t="inlineStr">
         <is>
-          <t>coffee listing (components/brewsoul/browse-explorer.tsx), real filter/search over the full BREWSOUL_COFFEES catalog. Verified live: 200 OK.</t>
+          <t>the real BrewSoul dashboard (distinct from /brewsoul's identity-quiz welcome gate and /brewsoul/first-sip's manifesto): hero + stats, Follow the Dollar teaser, Top QPR coffees (computed live via computeQPR), the 2025 crisis callout, New Drops, a Wall of Shame preview (SHAME_ENTRIES), the research-hub card grid, and a cyclable health-fact ticker (components/brewsoul/health-ticker.tsx, its own small client island so the rest of the page stays a Server Component). Canvas WarmParticles/ParallaxBg decorations and the dead hero photo (/api/img/brewsoul-orig_84eb4bc9.jpg, same confirmed-404 Manus proxy used elsewhere in Phase 6) dropped for CSS gradients. Stats use the real live BREWSOUL_COFFEES.length (107) in place of legacy's stale "103". Verified live: 200 OK.</t>
         </is>
       </c>
       <c r="E161" s="14" t="inlineStr">
@@ -4641,7 +4641,7 @@
       <c r="A162" s="4" t="n"/>
       <c r="B162" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/coffee/[id]</t>
+          <t>/brewsoul/browse</t>
         </is>
       </c>
       <c r="C162" s="13" t="inlineStr">
@@ -4651,7 +4651,7 @@
       </c>
       <c r="D162" s="4" t="inlineStr">
         <is>
-          <t>coffee detail page (breadcrumb, QPR + tier header, quick stats, tasting notes, flavor-profile bars, the 4 intelligence scores, transparency/ethics data, buy links, competition wins, similar-coffees cross-links, journey CTAs), server-rendered with generateStaticParams over all 107 real coffees (this repo's bounded-dynamic-route convention, same as /blog/[slug]) instead of legacy's client-side useParams lookup. Verified live: 200 OK.</t>
+          <t>coffee listing (components/brewsoul/browse-explorer.tsx), real filter/search over the full BREWSOUL_COFFEES catalog. Verified live: 200 OK.</t>
         </is>
       </c>
       <c r="E162" s="14" t="inlineStr">
@@ -4664,7 +4664,7 @@
       <c r="A163" s="4" t="n"/>
       <c r="B163" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/quiz</t>
+          <t>/brewsoul/coffee/[id]</t>
         </is>
       </c>
       <c r="C163" s="13" t="inlineStr">
@@ -4674,7 +4674,7 @@
       </c>
       <c r="D163" s="4" t="inlineStr">
         <is>
-          <t>matching quiz (built, not yet pushed — pending local review), along with the real data/engine foundation most of the rest of Phase 6 depends on. Ported lib/intelligence-engine/{types,scoring}.ts verbatim (generic scoring engine — QPR/availability/scarcity/wow/tier/freshness — reusable beyond BrewSoul) and the full coffee catalog (legacy's 3 files: brewsoul-coffees.ts + -expanded.ts + -expanded2.ts, merged at import time) → one lib/content/brewsoul-coffees.ts, extracted via tsx (not hand-typed — 107 real entries, ~6.5K lines). Caught a real stale count: legacy's own file header claimed "105" and its UI copy said "103", but the actual merged arrays contain 107 — this migration shows the live BREWSOUL_COFFEES.length everywhere instead of a repeated hardcoded number. Ported JourneyBar.tsx (components/brewsoul/journey-bar.tsx) — the fixed bottom "what's next" bar shown on every BrewSoul content page except the identity quiz — and retrofitted it onto /brewsoul/first-sip too (built before JourneyBar existed). Built components/brewsoul/brewsoul-quiz.tsx: real 7-question taste quiz scored against each coffee's real flavorProfile via the real scoring engine, ranking the full catalog by match. Legacy's useMarkVisited was renamed to markVisited (it's a plain localStorage write, not a hook — its old use-prefixed name tripped React's rules-of-hooks lint when called from inside a useEffect). Dropped the canvas WarmParticles decoration and the dead hero photo (same confirmed-404 Manus proxy,</t>
+          <t>coffee detail page (breadcrumb, QPR + tier header, quick stats, tasting notes, flavor-profile bars, the 4 intelligence scores, transparency/ethics data, buy links, competition wins, similar-coffees cross-links, journey CTAs), server-rendered with generateStaticParams over all 107 real coffees (this repo's bounded-dynamic-route convention, same as /blog/[slug]) instead of legacy's client-side useParams lookup. Verified live: 200 OK.</t>
         </is>
       </c>
       <c r="E163" s="14" t="inlineStr">
@@ -4687,7 +4687,7 @@
       <c r="A164" s="4" t="n"/>
       <c r="B164" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/wall-of-shame</t>
+          <t>/brewsoul/quiz</t>
         </is>
       </c>
       <c r="C164" s="13" t="inlineStr">
@@ -4697,7 +4697,7 @@
       </c>
       <c r="D164" s="4" t="inlineStr">
         <is>
-          <t>content page. Real 13 entries (brand/category/evidence/severity/response) from SHAME_ENTRIES, unchanged. Category filter buttons extracted into components/brewsoul/shame-explorer.tsx (the only interactive piece) so the page itself stays a Server Component. Verified live: 200 OK.</t>
+          <t>matching quiz (built, not yet pushed — pending local review), along with the real data/engine foundation most of the rest of Phase 6 depends on. Ported lib/intelligence-engine/{types,scoring}.ts verbatim (generic scoring engine — QPR/availability/scarcity/wow/tier/freshness — reusable beyond BrewSoul) and the full coffee catalog (legacy's 3 files: brewsoul-coffees.ts + -expanded.ts + -expanded2.ts, merged at import time) → one lib/content/brewsoul-coffees.ts, extracted via tsx (not hand-typed — 107 real entries, ~6.5K lines). Caught a real stale count: legacy's own file header claimed "105" and its UI copy said "103", but the actual merged arrays contain 107 — this migration shows the live BREWSOUL_COFFEES.length everywhere instead of a repeated hardcoded number. Ported JourneyBar.tsx (components/brewsoul/journey-bar.tsx) — the fixed bottom "what's next" bar shown on every BrewSoul content page except the identity quiz — and retrofitted it onto /brewsoul/first-sip too (built before JourneyBar existed). Built components/brewsoul/brewsoul-quiz.tsx: real 7-question taste quiz scored against each coffee's real flavorProfile via the real scoring engine, ranking the full catalog by match. Legacy's useMarkVisited was renamed to markVisited (it's a plain localStorage write, not a hook — its old use-prefixed name tripped React's rules-of-hooks lint when called from inside a useEffect). Dropped the canvas WarmParticles decoration and the dead hero photo (same confirmed-404 Manus proxy,</t>
         </is>
       </c>
       <c r="E164" s="14" t="inlineStr">
@@ -4710,7 +4710,7 @@
       <c r="A165" s="4" t="n"/>
       <c r="B165" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/follow-the-dollar</t>
+          <t>/brewsoul/wall-of-shame</t>
         </is>
       </c>
       <c r="C165" s="13" t="inlineStr">
@@ -4720,7 +4720,7 @@
       </c>
       <c r="D165" s="4" t="inlineStr">
         <is>
-          <t>supply-chain essay. Real DOLLAR_BREAKDOWNS segment bars (farmer/exporter/importer/roaster/retailer %, real commentary), unchanged. The farmer-segment bar's data-driven color (green/gold/red by threshold) is a small known set of variants — precomposed as 3 literal Tailwind classes rather than an inline style background, per this repo's dynamic-class rule; only the genuinely per-item width stays as style. Fully static, Server Component. Verified live: 200 OK.</t>
+          <t>content page. Real 13 entries (brand/category/evidence/severity/response) from SHAME_ENTRIES, unchanged. Category filter buttons extracted into components/brewsoul/shame-explorer.tsx (the only interactive piece) so the page itself stays a Server Component. Verified live: 200 OK.</t>
         </is>
       </c>
       <c r="E165" s="14" t="inlineStr">
@@ -4733,7 +4733,7 @@
       <c r="A166" s="4" t="n"/>
       <c r="B166" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/farms</t>
+          <t>/brewsoul/follow-the-dollar</t>
         </is>
       </c>
       <c r="C166" s="13" t="inlineStr">
@@ -4743,7 +4743,7 @@
       </c>
       <c r="D166" s="4" t="inlineStr">
         <is>
-          <t>sourcing content ("Farm Passports"). Real FARMS entries (country/region/producer/altitude/story/varieties/certifications), unchanged. Fully static. Verified live: 200 OK.</t>
+          <t>supply-chain essay. Real DOLLAR_BREAKDOWNS segment bars (farmer/exporter/importer/roaster/retailer %, real commentary), unchanged. The farmer-segment bar's data-driven color (green/gold/red by threshold) is a small known set of variants — precomposed as 3 literal Tailwind classes rather than an inline style background, per this repo's dynamic-class rule; only the genuinely per-item width stays as style. Fully static, Server Component. Verified live: 200 OK.</t>
         </is>
       </c>
       <c r="E166" s="14" t="inlineStr">
@@ -4756,7 +4756,7 @@
       <c r="A167" s="4" t="n"/>
       <c r="B167" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/mold-free</t>
+          <t>/brewsoul/farms</t>
         </is>
       </c>
       <c r="C167" s="13" t="inlineStr">
@@ -4766,7 +4766,7 @@
       </c>
       <c r="D167" s="4" t="inlineStr">
         <is>
-          <t>mycotoxin content. Real verified/claims/untested split computed live over the full BREWSOUL_COFFEES catalog by moldTestStatus. Fully static. Verified live: 200 OK.</t>
+          <t>sourcing content ("Farm Passports"). Real FARMS entries (country/region/producer/altitude/story/varieties/certifications), unchanged. Fully static. Verified live: 200 OK.</t>
         </is>
       </c>
       <c r="E167" s="14" t="inlineStr">
@@ -4779,7 +4779,7 @@
       <c r="A168" s="4" t="n"/>
       <c r="B168" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/experiences</t>
+          <t>/brewsoul/mold-free</t>
         </is>
       </c>
       <c r="C168" s="13" t="inlineStr">
@@ -4789,7 +4789,7 @@
       </c>
       <c r="D168" s="4" t="inlineStr">
         <is>
-          <t>experiential content ("Experience Map"). Real EXPERIENCES entries (farm tours, cafés, cupping labs, roastery visits), unchanged. Country filter buttons extracted into components/brewsoul/experiences-explorer.tsx, same split-out-the-interactive-bit pattern as wall-of-shame. Verified live: 200 OK.</t>
+          <t>mycotoxin content. Real verified/claims/untested split computed live over the full BREWSOUL_COFFEES catalog by moldTestStatus. Fully static. Verified live: 200 OK.</t>
         </is>
       </c>
       <c r="E168" s="14" t="inlineStr">
@@ -4802,7 +4802,7 @@
       <c r="A169" s="4" t="n"/>
       <c r="B169" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/health</t>
+          <t>/brewsoul/experiences</t>
         </is>
       </c>
       <c r="C169" s="13" t="inlineStr">
@@ -4812,7 +4812,7 @@
       </c>
       <c r="D169" s="4" t="inlineStr">
         <is>
-          <t>health deep-dive, ported from BrewSoulHealthFull.tsx (the file legacy's own router actually uses for this route — BrewSoulContent.tsx's same-named BrewSoulHealth export is real but genuinely dead/unrouted code in legacy, shadowed by this one). Real 8 longevity findings with real citations/participant counts, 7 real risks with severity ratings, CYP1A2 caffeine-metabolism genetics, a 6-step chronobiology timing schedule, 8 real bioactive compounds, 3 real mycotoxin threats, and a 3-step "simplification protocol," all ported unchanged and verbatim. Dead Manus hero image dropped for a CSS gradient. Legacy's own redundant BrewSoulLayout wrapper dropped — app/brewsoul/layout.tsx already wraps every route. The two real interactive pieces (show-all-risks toggle, per-compound click-to-expand) split into components/brewsoul/health-{risks,compounds}.tsx client islands so the rest stays a Server Component. Legacy's bespoke earthy "science" palette (soil/clay/sage/moss — distinct from the rest of BrewSoul's amber/gold commercial palette) kept as a deliberate one-off sub-identity for this one page, same reasoning as /attention-theft's own "crusade" palette elsewhere in this migration. Verified live: 200 OK, typecheck/lint clean.</t>
+          <t>experiential content ("Experience Map"). Real EXPERIENCES entries (farm tours, cafés, cupping labs, roastery visits), unchanged. Country filter buttons extracted into components/brewsoul/experiences-explorer.tsx, same split-out-the-interactive-bit pattern as wall-of-shame. Verified live: 200 OK.</t>
         </is>
       </c>
       <c r="E169" s="14" t="inlineStr">
@@ -4825,7 +4825,7 @@
       <c r="A170" s="4" t="n"/>
       <c r="B170" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/varieties</t>
+          <t>/brewsoul/health</t>
         </is>
       </c>
       <c r="C170" s="13" t="inlineStr">
@@ -4835,7 +4835,7 @@
       </c>
       <c r="D170" s="4" t="inlineStr">
         <is>
-          <t>reference: varieties. Real VARIETIES encyclopedia entries (species/origin/genetics/cup profile/yield/disease resistance), unchanged. Search extracted into components/brewsoul/varieties-explorer.tsx. Verified live: 200 OK.</t>
+          <t>health deep-dive, ported from BrewSoulHealthFull.tsx (the file legacy's own router actually uses for this route — BrewSoulContent.tsx's same-named BrewSoulHealth export is real but genuinely dead/unrouted code in legacy, shadowed by this one). Real 8 longevity findings with real citations/participant counts, 7 real risks with severity ratings, CYP1A2 caffeine-metabolism genetics, a 6-step chronobiology timing schedule, 8 real bioactive compounds, 3 real mycotoxin threats, and a 3-step "simplification protocol," all ported unchanged and verbatim. Dead Manus hero image dropped for a CSS gradient. Legacy's own redundant BrewSoulLayout wrapper dropped — app/brewsoul/layout.tsx already wraps every route. The two real interactive pieces (show-all-risks toggle, per-compound click-to-expand) split into components/brewsoul/health-{risks,compounds}.tsx client islands so the rest stays a Server Component. Legacy's bespoke earthy "science" palette (soil/clay/sage/moss — distinct from the rest of BrewSoul's amber/gold commercial palette) kept as a deliberate one-off sub-identity for this one page, same reasoning as /attention-theft's own "crusade" palette elsewhere in this migration. Verified live: 200 OK, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E170" s="14" t="inlineStr">
@@ -4848,7 +4848,7 @@
       <c r="A171" s="4" t="n"/>
       <c r="B171" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/processing</t>
+          <t>/brewsoul/varieties</t>
         </is>
       </c>
       <c r="C171" s="13" t="inlineStr">
@@ -4858,7 +4858,7 @@
       </c>
       <c r="D171" s="4" t="inlineStr">
         <is>
-          <t>reference: processing. Real PROCESSING_METHODS entries (description/flavor impact/complexity/controversy), unchanged. Fully static. Verified live: 200 OK.</t>
+          <t>reference: varieties. Real VARIETIES encyclopedia entries (species/origin/genetics/cup profile/yield/disease resistance), unchanged. Search extracted into components/brewsoul/varieties-explorer.tsx. Verified live: 200 OK.</t>
         </is>
       </c>
       <c r="E171" s="14" t="inlineStr">
@@ -4871,7 +4871,7 @@
       <c r="A172" s="4" t="n"/>
       <c r="B172" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/roasters</t>
+          <t>/brewsoul/processing</t>
         </is>
       </c>
       <c r="C172" s="13" t="inlineStr">
@@ -4881,7 +4881,7 @@
       </c>
       <c r="D172" s="4" t="inlineStr">
         <is>
-          <t>reference: roaster directory. Real ROASTERS entries (philosophy/quality/transparency/farmer-equity scores), unchanged. Search + tier filter extracted into components/brewsoul/roasters-explorer.tsx. Verified live: 200 OK.</t>
+          <t>reference: processing. Real PROCESSING_METHODS entries (description/flavor impact/complexity/controversy), unchanged. Fully static. Verified live: 200 OK.</t>
         </is>
       </c>
       <c r="E172" s="14" t="inlineStr">
@@ -4894,7 +4894,7 @@
       <c r="A173" s="4" t="n"/>
       <c r="B173" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/glossary</t>
+          <t>/brewsoul/roasters</t>
         </is>
       </c>
       <c r="C173" s="13" t="inlineStr">
@@ -4904,7 +4904,7 @@
       </c>
       <c r="D173" s="4" t="inlineStr">
         <is>
-          <t>reference: glossary. Real GLOSSARY terms, unchanged. Search + alphabetical grouping extracted into components/brewsoul/glossary-explorer.tsx. Verified live: 200 OK.</t>
+          <t>reference: roaster directory. Real ROASTERS entries (philosophy/quality/transparency/farmer-equity scores), unchanged. Search + tier filter extracted into components/brewsoul/roasters-explorer.tsx. Verified live: 200 OK.</t>
         </is>
       </c>
       <c r="E173" s="14" t="inlineStr">
@@ -4917,7 +4917,7 @@
       <c r="A174" s="4" t="n"/>
       <c r="B174" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/pairings</t>
+          <t>/brewsoul/glossary</t>
         </is>
       </c>
       <c r="C174" s="13" t="inlineStr">
@@ -4927,7 +4927,7 @@
       </c>
       <c r="D174" s="4" t="inlineStr">
         <is>
-          <t>reference: pairings. Real PAIRINGS (food/drink pairings by origin) and 3 real curated FLIGHTS (each linking to real coffees in the catalog), unchanged. Fully static. Verified live: 200 OK.</t>
+          <t>reference: glossary. Real GLOSSARY terms, unchanged. Search + alphabetical grouping extracted into components/brewsoul/glossary-explorer.tsx. Verified live: 200 OK.</t>
         </is>
       </c>
       <c r="E174" s="14" t="inlineStr">
@@ -4940,7 +4940,7 @@
       <c r="A175" s="4" t="n"/>
       <c r="B175" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/economics</t>
+          <t>/brewsoul/pairings</t>
         </is>
       </c>
       <c r="C175" s="13" t="inlineStr">
@@ -4950,7 +4950,7 @@
       </c>
       <c r="D175" s="4" t="inlineStr">
         <is>
-          <t>reference: economics. Real live-computed stats (coffee/origin/roaster/variety counts, average price, average farmer share via DOLLAR_BREAKDOWNS), a real price-distribution histogram, and a real top-origins ranking — all computed directly from BREWSOUL_COFFEES at render time, unchanged. Fully static. Verified live: 200 OK.</t>
+          <t>reference: pairings. Real PAIRINGS (food/drink pairings by origin) and 3 real curated FLIGHTS (each linking to real coffees in the catalog), unchanged. Fully static. Verified live: 200 OK.</t>
         </is>
       </c>
       <c r="E175" s="14" t="inlineStr">
@@ -4963,7 +4963,7 @@
       <c r="A176" s="4" t="n"/>
       <c r="B176" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/compare</t>
+          <t>/brewsoul/economics</t>
         </is>
       </c>
       <c r="C176" s="13" t="inlineStr">
@@ -4973,7 +4973,7 @@
       </c>
       <c r="D176" s="4" t="inlineStr">
         <is>
-          <t>tool: compare coffees. Real side-by-side comparison of up to 4 coffees across origin/producer/variety/process/price/cupping and the 4 intelligence scores (QPR/availability/wow/overall), unchanged. Interactivity in components/brewsoul/compare-explorer.tsx. Verified live: 200 OK.</t>
+          <t>reference: economics. Real live-computed stats (coffee/origin/roaster/variety counts, average price, average farmer share via DOLLAR_BREAKDOWNS), a real price-distribution histogram, and a real top-origins ranking — all computed directly from BREWSOUL_COFFEES at render time, unchanged. Fully static. Verified live: 200 OK.</t>
         </is>
       </c>
       <c r="E176" s="14" t="inlineStr">
@@ -4986,7 +4986,7 @@
       <c r="A177" s="4" t="n"/>
       <c r="B177" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/blend-builder</t>
+          <t>/brewsoul/compare</t>
         </is>
       </c>
       <c r="C177" s="13" t="inlineStr">
@@ -4996,7 +4996,7 @@
       </c>
       <c r="D177" s="4" t="inlineStr">
         <is>
-          <t>tool: blend builder. Real combine-up-to-5-coffees ratio calculator with weighted-average QPR/Wow/Overall scores via range sliders, unchanged (never persisted anywhere in legacy either — a pure in-session calculator). Interactivity in components/brewsoul/blend-builder-explorer.tsx. Verified live: 200 OK.</t>
+          <t>tool: compare coffees. Real side-by-side comparison of up to 4 coffees across origin/producer/variety/process/price/cupping and the 4 intelligence scores (QPR/availability/wow/overall), unchanged. Interactivity in components/brewsoul/compare-explorer.tsx. Verified live: 200 OK.</t>
         </is>
       </c>
       <c r="E177" s="14" t="inlineStr">
@@ -5009,7 +5009,7 @@
       <c r="A178" s="4" t="n"/>
       <c r="B178" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/drops</t>
+          <t>/brewsoul/blend-builder</t>
         </is>
       </c>
       <c r="C178" s="13" t="inlineStr">
@@ -5019,7 +5019,7 @@
       </c>
       <c r="D178" s="4" t="inlineStr">
         <is>
-          <t>tool: product drops ("Latest Drops"). Real top-12-by-overall-score coffees. No client-side state at all (legacy's own useMemo had no changing dependencies — a pure derived list), so this ships as a plain Server Component. Verified live: 200 OK.</t>
+          <t>tool: blend builder. Real combine-up-to-5-coffees ratio calculator with weighted-average QPR/Wow/Overall scores via range sliders, unchanged (never persisted anywhere in legacy either — a pure in-session calculator). Interactivity in components/brewsoul/blend-builder-explorer.tsx. Verified live: 200 OK.</t>
         </is>
       </c>
       <c r="E178" s="14" t="inlineStr">
@@ -5032,7 +5032,7 @@
       <c r="A179" s="4" t="n"/>
       <c r="B179" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/collection</t>
+          <t>/brewsoul/drops</t>
         </is>
       </c>
       <c r="C179" s="13" t="inlineStr">
@@ -5042,7 +5042,7 @@
       </c>
       <c r="D179" s="4" t="inlineStr">
         <is>
-          <t>tool: personal collection tracker ("My Collection"). Real save/toggle-to-collection behavior, unchanged. Real bug found and fixed: legacy read localStorage directly inside a useState initializer — unsafe during SSR, same hydration-mismatch class already fixed in journey-bar.tsx/journey-tracker.tsx — rebuilt around a module-level external store fed through useSyncExternalStore in components/brewsoul/collection-explorer.tsx. Also found and fixed: the already-ported brewsoul-directory.ts listed this page's path as /brewsoul/my-coffees — a real dead link in legacy's own directory (legacy's actual router only ever served this at /brewsoul/collection, /brewsoul/my-coffees never existed) — corrected to the real path. Verified live: 200 OK.</t>
+          <t>tool: product drops ("Latest Drops"). Real top-12-by-overall-score coffees. No client-side state at all (legacy's own useMemo had no changing dependencies — a pure derived list), so this ships as a plain Server Component. Verified live: 200 OK.</t>
         </is>
       </c>
       <c r="E179" s="14" t="inlineStr">
@@ -5055,7 +5055,7 @@
       <c r="A180" s="4" t="n"/>
       <c r="B180" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/submit</t>
+          <t>/brewsoul/collection</t>
         </is>
       </c>
       <c r="C180" s="13" t="inlineStr">
@@ -5065,7 +5065,7 @@
       </c>
       <c r="D180" s="4" t="inlineStr">
         <is>
-          <t>tool: submit a coffee ("Submit or Appeal"). Real submit-a-coffee / appeal-a-score form, unchanged in structure. Real bug found and fixed: legacy's own comment admitted "In production this would POST to a tRPC endpoint" but in the meantime wrote the submission to localStorage and showed "Received. We'll review your submission" regardless — actively misleading, since nobody would ever see a localStorage-only write. Replaced with a real mailto: fallback pre-filled with the form fields, same honest-degradation pattern as first-sip-email-capture.tsx — no fake success state. Verified live: 200 OK.</t>
+          <t>tool: personal collection tracker ("My Collection"). Real save/toggle-to-collection behavior, unchanged. Real bug found and fixed: legacy read localStorage directly inside a useState initializer — unsafe during SSR, same hydration-mismatch class already fixed in journey-bar.tsx/journey-tracker.tsx — rebuilt around a module-level external store fed through useSyncExternalStore in components/brewsoul/collection-explorer.tsx. Also found and fixed: the already-ported brewsoul-directory.ts listed this page's path as /brewsoul/my-coffees — a real dead link in legacy's own directory (legacy's actual router only ever served this at /brewsoul/collection, /brewsoul/my-coffees never existed) — corrected to the real path. Verified live: 200 OK.</t>
         </is>
       </c>
       <c r="E180" s="14" t="inlineStr">
@@ -5078,7 +5078,7 @@
       <c r="A181" s="4" t="n"/>
       <c r="B181" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/prescription</t>
+          <t>/brewsoul/submit</t>
         </is>
       </c>
       <c r="C181" s="13" t="inlineStr">
@@ -5088,7 +5088,7 @@
       </c>
       <c r="D181" s="4" t="inlineStr">
         <is>
-          <t>personalized "prescription", ported from BrewSoulPrescriptionFull.tsx (the file legacy's router actually uses — BrewSoulTools.tsx's same-named export is dead/unrouted, same shadowed-file trap as /brewsoul/health). Real 5-step questionnaire (genetics/timing/health/flavor/budget) generating a real, deterministic prescription (generatePrescription — real roast/cup-count/brand/pricing/warning logic), all ported unchanged and verbatim. Legacy's trpc.coffeePrescription.generate AI-enhancement mutation doesn't exist in this migration — dropped along with its "AI ANALYSIS LOADING..." block, which would otherwise spin forever and never resolve; the real prescription itself never depended on that call, it's already fully computed client-side. Same bespoke earthy "science" palette as /brewsoul/health kept as the same deliberate sub-identity. Verified live: 200 OK, typecheck/lint clean.</t>
+          <t>tool: submit a coffee ("Submit or Appeal"). Real submit-a-coffee / appeal-a-score form, unchanged in structure. Real bug found and fixed: legacy's own comment admitted "In production this would POST to a tRPC endpoint" but in the meantime wrote the submission to localStorage and showed "Received. We'll review your submission" regardless — actively misleading, since nobody would ever see a localStorage-only write. Replaced with a real mailto: fallback pre-filled with the form fields, same honest-degradation pattern as first-sip-email-capture.tsx — no fake success state. Verified live: 200 OK.</t>
         </is>
       </c>
       <c r="E181" s="14" t="inlineStr">
@@ -5101,7 +5101,7 @@
       <c r="A182" s="4" t="n"/>
       <c r="B182" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/chains</t>
+          <t>/brewsoul/prescription</t>
         </is>
       </c>
       <c r="C182" s="13" t="inlineStr">
@@ -5111,7 +5111,7 @@
       </c>
       <c r="D182" s="4" t="inlineStr">
         <is>
-          <t>"Top 100 Coffee Chains" ranking (not supply-chain visualization — that's /brewsoul/economics//brewsoul/follow-the-dollar; this is chain rankings). Real 100-chain dataset extracted from legacy's computed CHAIN_RANKINGS export (5 real weighted dimensions → aggregate → S-F tier) via a one-off tsx script (same approach as brewsoul-coffees.ts) into lib/content/brewsoul-chains.ts, with a new ChainEntry type added to intelligence-engine/types.ts. Real tier/type filters, search, and per-chain expand, unchanged, extracted into components/brewsoul/chains-explorer.tsx. Verified live: 200 OK, typecheck/lint clean.</t>
+          <t>personalized "prescription", ported from BrewSoulPrescriptionFull.tsx (the file legacy's router actually uses — BrewSoulTools.tsx's same-named export is dead/unrouted, same shadowed-file trap as /brewsoul/health). Real 5-step questionnaire (genetics/timing/health/flavor/budget) generating a real, deterministic prescription (generatePrescription — real roast/cup-count/brand/pricing/warning logic), all ported unchanged and verbatim. Legacy's trpc.coffeePrescription.generate AI-enhancement mutation doesn't exist in this migration — dropped along with its "AI ANALYSIS LOADING..." block, which would otherwise spin forever and never resolve; the real prescription itself never depended on that call, it's already fully computed client-side. Same bespoke earthy "science" palette as /brewsoul/health kept as the same deliberate sub-identity. Verified live: 200 OK, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E182" s="14" t="inlineStr">
@@ -5124,7 +5124,7 @@
       <c r="A183" s="4" t="n"/>
       <c r="B183" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/biodynamic</t>
+          <t>/brewsoul/chains</t>
         </is>
       </c>
       <c r="C183" s="13" t="inlineStr">
@@ -5134,7 +5134,7 @@
       </c>
       <c r="D183" s="4" t="inlineStr">
         <is>
-          <t>biodynamic content. The complete real census of Demeter-certified biodynamic coffee: 3 real source farms, 6 real roasters/brands with real product tables and pricing, real nutritional-science compounds, a real cost calculator, and a real impact/tokenization section, all ported unchanged and verbatim. Dead Manus hero image dropped for a CSS gradient. The 3 genuinely interactive pieces (click-to-expand farms/roasters, cups-per-day cost slider) split into components/brewsoul/{biodynamic-farms,biodynamic-roasters,cost-calculator}.tsx client islands so the rest stays a Server Component. Same bespoke earthy "science" palette as /brewsoul/health and /brewsoul/prescription kept as the same deliberate sub-identity. Verified live: 200 OK, typecheck/lint clean.</t>
+          <t>"Top 100 Coffee Chains" ranking (not supply-chain visualization — that's /brewsoul/economics//brewsoul/follow-the-dollar; this is chain rankings). Real 100-chain dataset extracted from legacy's computed CHAIN_RANKINGS export (5 real weighted dimensions → aggregate → S-F tier) via a one-off tsx script (same approach as brewsoul-coffees.ts) into lib/content/brewsoul-chains.ts, with a new ChainEntry type added to intelligence-engine/types.ts. Real tier/type filters, search, and per-chain expand, unchanged, extracted into components/brewsoul/chains-explorer.tsx. Verified live: 200 OK, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E183" s="14" t="inlineStr">
@@ -5147,7 +5147,7 @@
       <c r="A184" s="4" t="n"/>
       <c r="B184" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/decaf</t>
+          <t>/brewsoul/biodynamic</t>
         </is>
       </c>
       <c r="C184" s="13" t="inlineStr">
@@ -5157,7 +5157,7 @@
       </c>
       <c r="D184" s="4" t="inlineStr">
         <is>
-          <t>decaf content ("Paint Stripper or Pure Water?"). Real 3-process breakdown (methylene chloride/Swiss Water/supercritical CO₂), 13 real clean-decaf brands ("Hall of Fame"), 10 real methylene-chloride brands ("Wall of Shame," with real Clean Label Project lawsuit citations), a real carbon footprint comparison, real decaf health science, and a real price-comparison table, all ported unchanged and verbatim. Legacy's manual document.title/&lt;meta keywords&gt; mutation in a useEffect (a real anti-pattern — Next's generateMetadata already owns the head) dropped for the real metadata export. Real bug found and fixed: the 13-brand FAME dataset was initially exported from the "use client" decaf-fame.tsx component file and imported into the Server Component page for its price-comparison table — non-component exports from a client module aren't available across the RSC boundary, which threw FAME is not iterable at runtime (only caught by live verification, not typecheck/lint). Moved the data to a plain lib/content/brewsoul-decaf.ts module instead. The 2 genuinely interactive pieces (click-to-expand Hall of Fame, reveal-toggle Wall of Shame) split into components/brewsoul/decaf-{fame,shame}.tsx client islands. Same bespoke earthy "science" palette as the other /brewsoul deep-dive pages kept as the same deliberate sub-identity. Verified live: 200 OK, typecheck/lint clean.</t>
+          <t>biodynamic content. The complete real census of Demeter-certified biodynamic coffee: 3 real source farms, 6 real roasters/brands with real product tables and pricing, real nutritional-science compounds, a real cost calculator, and a real impact/tokenization section, all ported unchanged and verbatim. Dead Manus hero image dropped for a CSS gradient. The 3 genuinely interactive pieces (click-to-expand farms/roasters, cups-per-day cost slider) split into components/brewsoul/{biodynamic-farms,biodynamic-roasters,cost-calculator}.tsx client islands so the rest stays a Server Component. Same bespoke earthy "science" palette as /brewsoul/health and /brewsoul/prescription kept as the same deliberate sub-identity. Verified live: 200 OK, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E184" s="14" t="inlineStr">
@@ -5170,7 +5170,7 @@
       <c r="A185" s="4" t="n"/>
       <c r="B185" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/esoteric</t>
+          <t>/brewsoul/decaf</t>
         </is>
       </c>
       <c r="C185" s="13" t="inlineStr">
@@ -5180,7 +5180,7 @@
       </c>
       <c r="D185" s="4" t="inlineStr">
         <is>
-          <t>rare-coffee content ("Esoteric Coffee Index"). Real 9-coffee index across 2 tiers (Panama Geisha, Yemen Mokha, Liberica, Eugenioides, Wush Wush, Sidra, Pink Bourbon, Bourbon Aji, Sudan Rume) with real tasting notes, rarity scores, and real named buy sources, plus a real acquisition-priority list and explorer scorecard, all ported unchanged and verbatim. Real content gap found, not fixed: legacy's own "Top 10 Acquisition Priority" list and scorecard table both reference "Laurina" as a 10th entry, but no coffee card for it exists anywhere in the source dataset — ported as-is rather than inventing card content that was never written. Zero client-side state anywhere in this page (only CSS-able hover) — ships entirely as a Server Component. Verified live: 200 OK, typecheck/lint clean.</t>
+          <t>decaf content ("Paint Stripper or Pure Water?"). Real 3-process breakdown (methylene chloride/Swiss Water/supercritical CO₂), 13 real clean-decaf brands ("Hall of Fame"), 10 real methylene-chloride brands ("Wall of Shame," with real Clean Label Project lawsuit citations), a real carbon footprint comparison, real decaf health science, and a real price-comparison table, all ported unchanged and verbatim. Legacy's manual document.title/&lt;meta keywords&gt; mutation in a useEffect (a real anti-pattern — Next's generateMetadata already owns the head) dropped for the real metadata export. Real bug found and fixed: the 13-brand FAME dataset was initially exported from the "use client" decaf-fame.tsx component file and imported into the Server Component page for its price-comparison table — non-component exports from a client module aren't available across the RSC boundary, which threw FAME is not iterable at runtime (only caught by live verification, not typecheck/lint). Moved the data to a plain lib/content/brewsoul-decaf.ts module instead. The 2 genuinely interactive pieces (click-to-expand Hall of Fame, reveal-toggle Wall of Shame) split into components/brewsoul/decaf-{fame,shame}.tsx client islands. Same bespoke earthy "science" palette as the other /brewsoul deep-dive pages kept as the same deliberate sub-identity. Verified live: 200 OK, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E185" s="14" t="inlineStr">
@@ -5193,7 +5193,7 @@
       <c r="A186" s="4" t="n"/>
       <c r="B186" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/cities + /brewsoul/cities/[slug]</t>
+          <t>/brewsoul/esoteric</t>
         </is>
       </c>
       <c r="C186" s="13" t="inlineStr">
@@ -5203,7 +5203,7 @@
       </c>
       <c r="D186" s="4" t="inlineStr">
         <is>
-          <t>city directory + detail ("City Intelligence Module"). Real 25-city leaderboard (name/state/grade/score/tagline/verdict/live stats), a real 7-dimension scoring methodology, and real national + universal/nuanced chain report cards, all ported unchanged and verbatim into lib/content/brewsoul-cities.ts. Real data-completeness note, not a bug: legacy's own comment admits only Portland has full shop-by-shop data (25 real best + 5 real worst shops with real blurbs/scores/order-this/skip-this) — the other 24 cities have real city-level stats but empty shop/chain/bridge-drink/non-coffee arrays; legacy's own UI already handles this honestly (a real "Full data coming soon" state on both the card and detail page, not fake data) — preserved exactly, verified for both Portland (full tabs) and Seattle (coming-soon state). Grade filter, methodology modal, and chain-toggle interactivity in components/brewsoul/cities-explorer.tsx; per-city tab switching and per-shop expand in components/brewsoul/city-detail-tabs.tsx. Detail route uses generateStaticParams over all 25 real slugs. Scroll-linked parallax and floating-particle backgrounds dropped, same decoration call made throughout this migration. Real image-hosting gap flagged, not silently worked around: the 25 city hero photos are real, live Unsplash URLs (not a dead Manus proxy) but aren't yet uploaded to Sanity per this repo's own image convention — added images.unsplash.com to next.config.ts's remotePatterns as an interim measure rather th</t>
+          <t>rare-coffee content ("Esoteric Coffee Index"). Real 9-coffee index across 2 tiers (Panama Geisha, Yemen Mokha, Liberica, Eugenioides, Wush Wush, Sidra, Pink Bourbon, Bourbon Aji, Sudan Rume) with real tasting notes, rarity scores, and real named buy sources, plus a real acquisition-priority list and explorer scorecard, all ported unchanged and verbatim. Real content gap found, not fixed: legacy's own "Top 10 Acquisition Priority" list and scorecard table both reference "Laurina" as a 10th entry, but no coffee card for it exists anywhere in the source dataset — ported as-is rather than inventing card content that was never written. Zero client-side state anywhere in this page (only CSS-able hover) — ships entirely as a Server Component. Verified live: 200 OK, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E186" s="14" t="inlineStr">
@@ -5216,7 +5216,7 @@
       <c r="A187" s="4" t="n"/>
       <c r="B187" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/directory</t>
+          <t>/brewsoul/cities + /brewsoul/cities/[slug]</t>
         </is>
       </c>
       <c r="C187" s="13" t="inlineStr">
@@ -5226,7 +5226,7 @@
       </c>
       <c r="D187" s="4" t="inlineStr">
         <is>
-          <t>real master page index ("Everything Inside BrewSoul," not a roaster directory — that's /brewsoul/roasters). Real 6 categories with real page descriptions/icons, unchanged; the underlying data already lived in lib/content/brewsoul-directory.ts (built earlier this phase to power CategoryBadge) — this route is where it finally becomes a real browsable page. Category filter extracted into components/brewsoul/directory-explorer.tsx. Fixed the stale "Browse All 103 Coffees" label (real count is 107) by dropping the hardcoded number from the shared data module — benefits every other consumer of that module too. Verified live: 200 OK, typecheck/lint clean.</t>
+          <t>city directory + detail ("City Intelligence Module"). Real 25-city leaderboard (name/state/grade/score/tagline/verdict/live stats), a real 7-dimension scoring methodology, and real national + universal/nuanced chain report cards, all ported unchanged and verbatim into lib/content/brewsoul-cities.ts. Real data-completeness note, not a bug: legacy's own comment admits only Portland has full shop-by-shop data (25 real best + 5 real worst shops with real blurbs/scores/order-this/skip-this) — the other 24 cities have real city-level stats but empty shop/chain/bridge-drink/non-coffee arrays; legacy's own UI already handles this honestly (a real "Full data coming soon" state on both the card and detail page, not fake data) — preserved exactly, verified for both Portland (full tabs) and Seattle (coming-soon state). Grade filter, methodology modal, and chain-toggle interactivity in components/brewsoul/cities-explorer.tsx; per-city tab switching and per-shop expand in components/brewsoul/city-detail-tabs.tsx. Detail route uses generateStaticParams over all 25 real slugs. Scroll-linked parallax and floating-particle backgrounds dropped, same decoration call made throughout this migration. Real image-hosting gap flagged, not silently worked around: the 25 city hero photos are real, live Unsplash URLs (not a dead Manus proxy) but aren't yet uploaded to Sanity per this repo's own image convention — added images.unsplash.com to next.config.ts's remotePatterns as an interim measure rather th</t>
         </is>
       </c>
       <c r="E187" s="14" t="inlineStr">
@@ -5239,7 +5239,7 @@
       <c r="A188" s="4" t="n"/>
       <c r="B188" s="4" t="inlineStr">
         <is>
-          <t>/brewsoul/guest + /brewsoul/guest/shanita-nicholas</t>
+          <t>/brewsoul/directory</t>
         </is>
       </c>
       <c r="C188" s="13" t="inlineStr">
@@ -5249,7 +5249,7 @@
       </c>
       <c r="D188" s="4" t="inlineStr">
         <is>
-          <t>guest series index + profile ("Tony G Guest Series"). Real single guest entry (Shanita Nicholas — real headline/teaser/tags) on the index, and the real 10-question interview on the detail page (Fair Trade economics, roasting mythology, the C Market, regenerative vs. sustainable, origin-roasting economics vs. Fair Trade, blockchain traceability, pre-harvest financing — real substantive answers with real citations), all ported unchanged and verbatim into components/brewsoul/shanita-interview.tsx. Legacy's guest photo (/api/img/brewsoul-orig_84eb4bc9.jpg) was the same dead Manus proxy confirmed 404 throughout this migration — dropped for a plain initial avatar on both pages rather than a broken headshot. Per-question expand/collapse, "Expand/Collapse All," and the real Twitter/LinkedIn/copy-link share row are genuinely interactive, split into client islands. Verified live: 200 OK on both, typecheck/lint clean.</t>
+          <t>real master page index ("Everything Inside BrewSoul," not a roaster directory — that's /brewsoul/roasters). Real 6 categories with real page descriptions/icons, unchanged; the underlying data already lived in lib/content/brewsoul-directory.ts (built earlier this phase to power CategoryBadge) — this route is where it finally becomes a real browsable page. Category filter extracted into components/brewsoul/directory-explorer.tsx. Fixed the stale "Browse All 103 Coffees" label (real count is 107) by dropping the hardcoded number from the shared data module — benefits every other consumer of that module too. Verified live: 200 OK, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E188" s="14" t="inlineStr">
@@ -5262,63 +5262,63 @@
       <c r="A189" s="4" t="n"/>
       <c r="B189" s="4" t="inlineStr">
         <is>
+          <t>/brewsoul/guest + /brewsoul/guest/shanita-nicholas</t>
+        </is>
+      </c>
+      <c r="C189" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D189" s="4" t="inlineStr">
+        <is>
+          <t>guest series index + profile ("Tony G Guest Series"). Real single guest entry (Shanita Nicholas — real headline/teaser/tags) on the index, and the real 10-question interview on the detail page (Fair Trade economics, roasting mythology, the C Market, regenerative vs. sustainable, origin-roasting economics vs. Fair Trade, blockchain traceability, pre-harvest financing — real substantive answers with real citations), all ported unchanged and verbatim into components/brewsoul/shanita-interview.tsx. Legacy's guest photo (/api/img/brewsoul-orig_84eb4bc9.jpg) was the same dead Manus proxy confirmed 404 throughout this migration — dropped for a plain initial avatar on both pages rather than a broken headshot. Per-question expand/collapse, "Expand/Collapse All," and the real Twitter/LinkedIn/copy-link share row are genuinely interactive, split into client islands. Verified live: 200 OK on both, typecheck/lint clean.</t>
+        </is>
+      </c>
+      <c r="E189" s="14" t="inlineStr">
+        <is>
+          <t>Phase 6 — BrewSoul (28 routes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="4" t="n"/>
+      <c r="B190" s="4" t="inlineStr">
+        <is>
           <t>Shared: port BrewSoulLayout, CategoryBadge, JourneyBar, NextSteps as Next.js layout/components</t>
         </is>
       </c>
-      <c r="C189" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D189" s="4" t="inlineStr">
+      <c r="C190" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D190" s="4" t="inlineStr">
         <is>
           <t>app/brewsoul/layout.tsx + components/brewsoul/{brewsoul-nav,category-badge,journey-bar,next-steps}.tsx, all built and reused by every /brewsoul/* route above.</t>
         </is>
       </c>
-      <c r="E189" s="14" t="inlineStr">
+      <c r="E190" s="14" t="inlineStr">
         <is>
           <t>Phase 6 — BrewSoul (28 routes)</t>
         </is>
       </c>
     </row>
-    <row r="190">
-      <c r="A190" s="10" t="inlineStr">
+    <row r="191">
+      <c r="A191" s="10" t="inlineStr">
         <is>
           <t>Phase 7 — PRI &amp; Kava Encyclopedias (19 routes)</t>
         </is>
       </c>
-      <c r="B190" s="11" t="n"/>
-      <c r="C190" s="11" t="n"/>
-      <c r="D190" s="12" t="n"/>
-    </row>
-    <row r="191">
-      <c r="A191" s="4" t="n"/>
-      <c r="B191" s="4" t="inlineStr">
-        <is>
-          <t>Kava shared foundation</t>
-        </is>
-      </c>
-      <c r="C191" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D191" s="4" t="inlineStr">
-        <is>
-          <t>app/kava/layout.tsx + components/kava/kava-nav.tsx (KavaNav/KavaFooter, 10 real nav items) + components/kava/kava-ui.tsx (KavaHero/KavaSection/KavaSectionTitle/KavaCard/KavaBadge/KavaDivider/KavaDisclaimer, converted from legacy inline style={} to Tailwind + new --kava-* tokens in globals.css). Added /kava to site-chrome.tsx's SUPPRESSED_PREFIXES (self-contained sub-site, same pattern as BrewSoul and /attention-theft). Real dead link fixed: legacy nav pointed at /pri, which legacy's own App.tsx never routed (only /psychedelic-readiness-index exists) — corrected.</t>
-        </is>
-      </c>
-      <c r="E191" s="14" t="inlineStr">
-        <is>
-          <t>Phase 7 — PRI &amp; Kava Encyclopedias (19 routes)</t>
-        </is>
-      </c>
+      <c r="B191" s="11" t="n"/>
+      <c r="C191" s="11" t="n"/>
+      <c r="D191" s="12" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="4" t="n"/>
       <c r="B192" s="4" t="inlineStr">
         <is>
-          <t>/kava (home)</t>
+          <t>Kava shared foundation</t>
         </is>
       </c>
       <c r="C192" s="13" t="inlineStr">
@@ -5328,7 +5328,7 @@
       </c>
       <c r="D192" s="4" t="inlineStr">
         <is>
-          <t>9 module cards, "Threshold Doctrine," "Sacred Masculine Triad" (Mezcal/Kava/Peyote), 4 market stats, all ported unchanged. Verified live: 200 OK, exactly 1 header/1 footer (chrome suppression confirmed), typecheck/lint clean.</t>
+          <t>app/kava/layout.tsx + components/kava/kava-nav.tsx (KavaNav/KavaFooter, 10 real nav items) + components/kava/kava-ui.tsx (KavaHero/KavaSection/KavaSectionTitle/KavaCard/KavaBadge/KavaDivider/KavaDisclaimer, converted from legacy inline style={} to Tailwind + new --kava-* tokens in globals.css). Added /kava to site-chrome.tsx's SUPPRESSED_PREFIXES (self-contained sub-site, same pattern as BrewSoul and /attention-theft). Real dead link fixed: legacy nav pointed at /pri, which legacy's own App.tsx never routed (only /psychedelic-readiness-index exists) — corrected.</t>
         </is>
       </c>
       <c r="E192" s="14" t="inlineStr">
@@ -5341,7 +5341,7 @@
       <c r="A193" s="4" t="n"/>
       <c r="B193" s="4" t="inlineStr">
         <is>
-          <t>/kava/origins</t>
+          <t>/kava (home)</t>
         </is>
       </c>
       <c r="C193" s="13" t="inlineStr">
@@ -5351,7 +5351,7 @@
       </c>
       <c r="D193" s="4" t="inlineStr">
         <is>
-          <t>real migration timeline (6 Pacific nations, ~3000 BCE–1000 CE), real 6-island selector (Vanuatu/Fiji/Tonga/Samoa/Hawaii/Pohnpei, each with real facts/ceremony/cultivar/safety content), and the real Noble vs. Tudei safety comparison, all ported unchanged and verbatim. Island-selector interactivity in components/kava/origins-explorer.tsx. Verified live: 200 OK, typecheck/lint clean.</t>
+          <t>9 module cards, "Threshold Doctrine," "Sacred Masculine Triad" (Mezcal/Kava/Peyote), 4 market stats, all ported unchanged. Verified live: 200 OK, exactly 1 header/1 footer (chrome suppression confirmed), typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E193" s="14" t="inlineStr">
@@ -5364,7 +5364,7 @@
       <c r="A194" s="4" t="n"/>
       <c r="B194" s="4" t="inlineStr">
         <is>
-          <t>/kava/interactions</t>
+          <t>/kava/origins</t>
         </is>
       </c>
       <c r="C194" s="13" t="inlineStr">
@@ -5374,7 +5374,7 @@
       </c>
       <c r="D194" s="4" t="inlineStr">
         <is>
-          <t>real 24-substance drug interaction database (real severity ratings across an 11-value scale, real pharmacological mechanisms, real PRI protocol guidance) and real 5-enzyme CYP450 inhibition profile, ported unchanged and verbatim. Search + severity-filter interactivity in components/kava/interactions-explorer.tsx, using a precomposed SEVERITY_CONFIG class lookup (not string-built classes — same Tailwind static-scanner rule enforced elsewhere this migration). Legacy's unused Download icon import (dead code, no export feature attached to it) not ported. Verified live: 200 OK, typecheck/lint clean.</t>
+          <t>real migration timeline (6 Pacific nations, ~3000 BCE–1000 CE), real 6-island selector (Vanuatu/Fiji/Tonga/Samoa/Hawaii/Pohnpei, each with real facts/ceremony/cultivar/safety content), and the real Noble vs. Tudei safety comparison, all ported unchanged and verbatim. Island-selector interactivity in components/kava/origins-explorer.tsx. Verified live: 200 OK, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E194" s="14" t="inlineStr">
@@ -5387,7 +5387,7 @@
       <c r="A195" s="4" t="n"/>
       <c r="B195" s="4" t="inlineStr">
         <is>
-          <t>/kava/science</t>
+          <t>/kava/interactions</t>
         </is>
       </c>
       <c r="C195" s="13" t="inlineStr">
@@ -5397,7 +5397,7 @@
       </c>
       <c r="D195" s="4" t="inlineStr">
         <is>
-          <t>real 6 major kavalactones (real receptor mechanisms, real PRI relevance) and real 11-item combined pharmacological profile, ported unchanged into lib/content/kava-science.ts. RSC-boundary bug caught proactively before shipping: initially drafted KAVALACTONES as an export of the "use client" chemotype-decoder.tsx, which would have thrown the same TypeError: X is not iterable already hit once this migration on /brewsoul/decaf when the Server Component page tried to import it — moved to the plain data module before ever running it. Chemotype decoder tool (enter e.g. 4-2-6-5-3-1, see dominant kavalactones) kept as the real interactive client island. Verified live: 200 OK, typecheck/lint clean.</t>
+          <t>real 24-substance drug interaction database (real severity ratings across an 11-value scale, real pharmacological mechanisms, real PRI protocol guidance) and real 5-enzyme CYP450 inhibition profile, ported unchanged and verbatim. Search + severity-filter interactivity in components/kava/interactions-explorer.tsx, using a precomposed SEVERITY_CONFIG class lookup (not string-built classes — same Tailwind static-scanner rule enforced elsewhere this migration). Legacy's unused Download icon import (dead code, no export feature attached to it) not ported. Verified live: 200 OK, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E195" s="14" t="inlineStr">
@@ -5410,7 +5410,7 @@
       <c r="A196" s="4" t="n"/>
       <c r="B196" s="4" t="inlineStr">
         <is>
-          <t>/kava/assessment</t>
+          <t>/kava/science</t>
         </is>
       </c>
       <c r="C196" s="13" t="inlineStr">
@@ -5420,7 +5420,7 @@
       </c>
       <c r="D196" s="4" t="inlineStr">
         <is>
-          <t>real 5-domain, 20-question PRI readiness assessment (somatic/psychological/relational/cultural/integration), real per-domain point weights, and real 4-band recommendation scoring (CLEARED/CONDITIONAL/DEFER/NOT READY), all ported unchanged into components/kava/assessment-quiz.tsx. Fully stateful (domain navigation, per-question answers, results view), so kept as a single client island per this migration's established pattern for multi-step assessments. Domain and recommendation accent colors (5 + 4 distinct hexes, none matching the --kava-* brand palette) precomposed into literal DOMAIN_STYLES/RECOMMENDATION_STYLES lookup objects rather than style={}, avoiding the dynamic-class bug already caught twice this migration (chains-explorer.tsx, biodynamic/page.tsx). Real backend gap, handled honestly: legacy's AssessmentResultActions took sessionId/serialized-answers props feeding a trpc.assessments.submit mutation this migration never built — used the already-simplified, print-only AssessmentResultActions (components/assessments/result-actions.tsx, built during Phase 9) instead of reproducing a submit call with no backend. Verified live: 200 OK, real domain/question content confirmed in rendered HTML, typecheck/lint clean.</t>
+          <t>real 6 major kavalactones (real receptor mechanisms, real PRI relevance) and real 11-item combined pharmacological profile, ported unchanged into lib/content/kava-science.ts. RSC-boundary bug caught proactively before shipping: initially drafted KAVALACTONES as an export of the "use client" chemotype-decoder.tsx, which would have thrown the same TypeError: X is not iterable already hit once this migration on /brewsoul/decaf when the Server Component page tried to import it — moved to the plain data module before ever running it. Chemotype decoder tool (enter e.g. 4-2-6-5-3-1, see dominant kavalactones) kept as the real interactive client island. Verified live: 200 OK, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E196" s="14" t="inlineStr">
@@ -5433,7 +5433,7 @@
       <c r="A197" s="4" t="n"/>
       <c r="B197" s="4" t="inlineStr">
         <is>
-          <t>/kava/hawaii</t>
+          <t>/kava/assessment</t>
         </is>
       </c>
       <c r="C197" s="13" t="inlineStr">
@@ -5443,7 +5443,7 @@
       </c>
       <c r="D197" s="4" t="inlineStr">
         <is>
-          <t>real ICE/meth crisis statistics (Quest Diagnostics 410% figure, Hawaii DOH conviction rates, law enforcement seizure data), real dual crisis/revival timeline (1985–present), the real (explicitly-labeled hypothesis, not proven) pharmacological alignment table, and real recovery resource listings, all ported unchanged and verbatim. Fully static, no client island needed. Verified live: 200 OK, typecheck/lint clean.</t>
+          <t>real 5-domain, 20-question PRI readiness assessment (somatic/psychological/relational/cultural/integration), real per-domain point weights, and real 4-band recommendation scoring (CLEARED/CONDITIONAL/DEFER/NOT READY), all ported unchanged into components/kava/assessment-quiz.tsx. Fully stateful (domain navigation, per-question answers, results view), so kept as a single client island per this migration's established pattern for multi-step assessments. Domain and recommendation accent colors (5 + 4 distinct hexes, none matching the --kava-* brand palette) precomposed into literal DOMAIN_STYLES/RECOMMENDATION_STYLES lookup objects rather than style={}, avoiding the dynamic-class bug already caught twice this migration (chains-explorer.tsx, biodynamic/page.tsx). Real backend gap, handled honestly: legacy's AssessmentResultActions took sessionId/serialized-answers props feeding a trpc.assessments.submit mutation this migration never built — used the already-simplified, print-only AssessmentResultActions (components/assessments/result-actions.tsx, built during Phase 9) instead of reproducing a submit call with no backend. Verified live: 200 OK, real domain/question content confirmed in rendered HTML, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E197" s="14" t="inlineStr">
@@ -5456,7 +5456,7 @@
       <c r="A198" s="4" t="n"/>
       <c r="B198" s="4" t="inlineStr">
         <is>
-          <t>/kava/myths</t>
+          <t>/kava/hawaii</t>
         </is>
       </c>
       <c r="C198" s="13" t="inlineStr">
@@ -5466,7 +5466,7 @@
       </c>
       <c r="D198" s="4" t="inlineStr">
         <is>
-          <t>real 7-myth evidence review (2002/2014 European kava ban and reversal, WHO findings, CYP2D6 metabolism differences by population, chemotype/preparation distinctions) and the real closing takeaway, ported unchanged. Expand/collapse interactivity in components/kava/myths-explorer.tsx, verdict colors (3-value enum) precomposed into a literal VERDICT_CLASS lookup. Extended shared KavaCard (kava-ui.tsx) with an optional onClick prop to support this — first Kava page needing a clickable card. Verified live: 200 OK, typecheck/lint clean.</t>
+          <t>real ICE/meth crisis statistics (Quest Diagnostics 410% figure, Hawaii DOH conviction rates, law enforcement seizure data), real dual crisis/revival timeline (1985–present), the real (explicitly-labeled hypothesis, not proven) pharmacological alignment table, and real recovery resource listings, all ported unchanged and verbatim. Fully static, no client island needed. Verified live: 200 OK, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E198" s="14" t="inlineStr">
@@ -5479,7 +5479,7 @@
       <c r="A199" s="4" t="n"/>
       <c r="B199" s="4" t="inlineStr">
         <is>
-          <t>/kava/caffeine</t>
+          <t>/kava/myths</t>
         </is>
       </c>
       <c r="C199" s="13" t="inlineStr">
@@ -5489,7 +5489,7 @@
       </c>
       <c r="D199" s="4" t="inlineStr">
         <is>
-          <t>real CYP1A2 inhibition mechanism (56%, the same pathway grapefruit juice uses on medications), real caffeine cutoff protocol, and the real kava-vs-coffee comparison table, ported unchanged. Fully static, no client island needed. Verified live: 200 OK, typecheck/lint clean.</t>
+          <t>real 7-myth evidence review (2002/2014 European kava ban and reversal, WHO findings, CYP2D6 metabolism differences by population, chemotype/preparation distinctions) and the real closing takeaway, ported unchanged. Expand/collapse interactivity in components/kava/myths-explorer.tsx, verdict colors (3-value enum) precomposed into a literal VERDICT_CLASS lookup. Extended shared KavaCard (kava-ui.tsx) with an optional onClick prop to support this — first Kava page needing a clickable card. Verified live: 200 OK, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E199" s="14" t="inlineStr">
@@ -5502,7 +5502,7 @@
       <c r="A200" s="4" t="n"/>
       <c r="B200" s="4" t="inlineStr">
         <is>
-          <t>/kava/products</t>
+          <t>/kava/caffeine</t>
         </is>
       </c>
       <c r="C200" s="13" t="inlineStr">
@@ -5512,7 +5512,7 @@
       </c>
       <c r="D200" s="4" t="inlineStr">
         <is>
-          <t>real 5-category product index (ceremonial powder, fresh frozen, RTD beverages, supplements, kava bars) with real named vendors/cultivars/chemotypes/pricing/PRI ratings and real outbound buy links (all live vendor domains, not Manus proxies — no image assets on this page to check), ported unchanged into components/kava/products-explorer.tsx. Category-tab interactivity kept as the client island. Verified live: 200 OK, typecheck/lint clean.</t>
+          <t>real CYP1A2 inhibition mechanism (56%, the same pathway grapefruit juice uses on medications), real caffeine cutoff protocol, and the real kava-vs-coffee comparison table, ported unchanged. Fully static, no client island needed. Verified live: 200 OK, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E200" s="14" t="inlineStr">
@@ -5525,7 +5525,7 @@
       <c r="A201" s="4" t="n"/>
       <c r="B201" s="4" t="inlineStr">
         <is>
-          <t>/kava/certification</t>
+          <t>/kava/products</t>
         </is>
       </c>
       <c r="C201" s="13" t="inlineStr">
@@ -5535,7 +5535,7 @@
       </c>
       <c r="D201" s="4" t="inlineStr">
         <is>
-          <t>real 12-module, 80-hour facilitator curriculum, real 3-tier certification structure (Practitioner/Threshold Facilitator/Master Facilitator), and real prerequisites list, ported unchanged. Fully static, no client island needed; legacy's wouter cross-links replaced with next/link. Verified live: 200 OK, typecheck/lint clean.</t>
+          <t>real 5-category product index (ceremonial powder, fresh frozen, RTD beverages, supplements, kava bars) with real named vendors/cultivars/chemotypes/pricing/PRI ratings and real outbound buy links (all live vendor domains, not Manus proxies — no image assets on this page to check), ported unchanged into components/kava/products-explorer.tsx. Category-tab interactivity kept as the client island. Verified live: 200 OK, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E201" s="14" t="inlineStr">
@@ -5548,7 +5548,7 @@
       <c r="A202" s="4" t="n"/>
       <c r="B202" s="4" t="inlineStr">
         <is>
-          <t>PRI shared data: lib/content/pri-data.ts (copied verbatim from legacy pri/data.ts</t>
+          <t>/kava/certification</t>
         </is>
       </c>
       <c r="C202" s="13" t="inlineStr">
@@ -5558,7 +5558,7 @@
       </c>
       <c r="D202" s="4" t="inlineStr">
         <is>
-          <t>real 39-medicine pharmacopoeia, 50+ questions across 6 domains, MAO-B interaction matrix, medication interaction guide, crisis/integration resources, pathway questions), lib/content/pri-safety-data.ts (verbatim safety data merge source), lib/content/pri-medicine-images.ts (verbatim real CloudFront hero-image map, all spot-checked 200 OK — RampRate's own CDN, already whitelisted, not Manus), lib/content/pri-shared.ts (the real scoring engine — computeScores/READINESS_LEVELS/getMedicineWithSafety — extracted to a plain module per the RSC-boundary lesson from /brewsoul/decaf and /kava/science). Added --pri-* CSS custom properties to globals.css (this subsystem's own purple/parchment/near-black palette, same pattern as --kava-/--crusade-) since Phase 7's PRI section spans 9 more routes.</t>
+          <t>real 12-module, 80-hour facilitator curriculum, real 3-tier certification structure (Practitioner/Threshold Facilitator/Master Facilitator), and real prerequisites list, ported unchanged. Fully static, no client island needed; legacy's wouter cross-links replaced with next/link. Verified live: 200 OK, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E202" s="14" t="inlineStr">
@@ -5571,7 +5571,7 @@
       <c r="A203" s="4" t="n"/>
       <c r="B203" s="4" t="inlineStr">
         <is>
-          <t>/psychedelic-readiness-index (core tool)</t>
+          <t>PRI shared data: lib/content/pri-data.ts (copied verbatim from legacy pri/data.ts</t>
         </is>
       </c>
       <c r="C203" s="13" t="inlineStr">
@@ -5581,7 +5581,7 @@
       </c>
       <c r="D203" s="4" t="inlineStr">
         <is>
-          <t>the real hero, 39-medicine grid with compare/save/bookmark tooling, MAO-B interaction matrix, medication interaction guide, crisis resources, the real 5-state assessment flow (philosophy intro → readiness quiz → pathway &amp; access questions → legal disclaimer gate → results), medicine detail modal (overview/safety/correction tabs), testimonials, and ImpactSoul cross-promotion, all ported unchanged and verbatim into components/pri/psychedelic-readiness-index.tsx plus supporting client islands (disclaimer-gate.tsx, medicine-modal.tsx, safety-section.tsx, correction-form.tsx, share-bar.tsx, cinematic-band.tsx). Kept as one client island — a single state machine drives which section renders, same call made for other large multi-step assessments this migration. Real hero/section photography (8 CloudFront images) kept via next/image; legacy's purely decorative glitch-scanline overlay divs and CSS shimmer/glow @keyframes dropped (no framer-motion — CONTRIBUTING.md rule 5 — and "decoration not worth the cost," same call made throughout this migration).</t>
+          <t>real 39-medicine pharmacopoeia, 50+ questions across 6 domains, MAO-B interaction matrix, medication interaction guide, crisis/integration resources, pathway questions), lib/content/pri-safety-data.ts (verbatim safety data merge source), lib/content/pri-medicine-images.ts (verbatim real CloudFront hero-image map, all spot-checked 200 OK — RampRate's own CDN, already whitelisted, not Manus), lib/content/pri-shared.ts (the real scoring engine — computeScores/READINESS_LEVELS/getMedicineWithSafety — extracted to a plain module per the RSC-boundary lesson from /brewsoul/decaf and /kava/science). Added --pri-* CSS custom properties to globals.css (this subsystem's own purple/parchment/near-black palette, same pattern as --kava-/--crusade-) since Phase 7's PRI section spans 9 more routes.</t>
         </is>
       </c>
       <c r="E203" s="14" t="inlineStr">
@@ -5594,7 +5594,7 @@
       <c r="A204" s="4" t="n"/>
       <c r="B204" s="4" t="inlineStr">
         <is>
-          <t>PRI: /peyote-mescaline</t>
+          <t>/psychedelic-readiness-index (core tool)</t>
         </is>
       </c>
       <c r="C204" s="13" t="inlineStr">
@@ -5604,7 +5604,7 @@
       </c>
       <c r="D204" s="4" t="inlineStr">
         <is>
-          <t>MescalineDeepDive, real receptor pharmacology table, the real "Latuda Mirror" same-target-opposite-action comparison, real clinical outcomes (Agin-Liebes et al. 2021, n=452), the real 16-row pharma-to-plant alternatives table, real supplement protocol (pre/day-of/post-integration), real mescaline-specific PRI dimension scores, the real medicine-selector comparison table, and real sources, all ported unchanged and verbatim into lib/content/pri-mescaline-module.ts (copied verbatim) + app/peyote-mescaline/page.tsx. Fully static except the pharma-table expand toggle, extracted into components/pri/pharma-table.tsx; shared PriSection/PriEyebrow wrapper (components/pri/pri-section.tsx) introduced here for reuse by the remaining PRI deep-dive modules. All 8 real section photos (CloudFront) spot-checked live before use; legacy's purely decorative glitch-scanline overlays dropped. Verified live: 200 OK, real content confirmed in rendered HTML, exactly 1 header/1 footer, typecheck/lint clean.</t>
+          <t>the real hero, 39-medicine grid with compare/save/bookmark tooling, MAO-B interaction matrix, medication interaction guide, crisis resources, the real 5-state assessment flow (philosophy intro → readiness quiz → pathway &amp; access questions → legal disclaimer gate → results), medicine detail modal (overview/safety/correction tabs), testimonials, and ImpactSoul cross-promotion, all ported unchanged and verbatim into components/pri/psychedelic-readiness-index.tsx plus supporting client islands (disclaimer-gate.tsx, medicine-modal.tsx, safety-section.tsx, correction-form.tsx, share-bar.tsx, cinematic-band.tsx). Kept as one client island — a single state machine drives which section renders, same call made for other large multi-step assessments this migration. Real hero/section photography (8 CloudFront images) kept via next/image; legacy's purely decorative glitch-scanline overlay divs and CSS shimmer/glow @keyframes dropped (no framer-motion — CONTRIBUTING.md rule 5 — and "decoration not worth the cost," same call made throughout this migration).</t>
         </is>
       </c>
       <c r="E204" s="14" t="inlineStr">
@@ -5617,7 +5617,7 @@
       <c r="A205" s="4" t="n"/>
       <c r="B205" s="4" t="inlineStr">
         <is>
-          <t>PRI: /iboga-ibogaine</t>
+          <t>PRI: /peyote-mescaline</t>
         </is>
       </c>
       <c r="C205" s="13" t="inlineStr">
@@ -5627,7 +5627,7 @@
       </c>
       <c r="D205" s="4" t="inlineStr">
         <is>
-          <t>IbogaDeepDive, "The Plant vs The Isolate": real alkaloid-profile comparison, real receptor pharmacology, real head-to-head iboga-vs-ibogaine table, real clinical outcomes (Mash/Noller/Schenberg/Brown &amp; Alper/Cherian/Williams — including the 2024 Stanford Nature Medicine SOF-veteran data and the 2026 19,071-patient safety analysis), real pharma-to-plant alternatives, real supplement protocol, real dimension thresholds, real medicine selector, Tony's real first-hand account of sitting ibogaine at The Mission Within, real hard-stop contraindications, a real 9-facility directory (with the 2 facilities legacy explicitly removed and why), real Nagoya Protocol / extractive-capitalism argument, real 2026 US legal-status rundown, the embedded Iboga Compass v2 documentation section (components/pri/iboga-compass-section.tsx, its own client island for the question-group toggles), and real sources — all ported unchanged and verbatim into lib/content/pri-iboga-module.ts + lib/content/pri-iboga-compass-data.ts (both copied verbatim) + app/iboga-ibogaine/page.tsx. Fully static except the pharma-table expand toggle (components/pri/iboga-pharma-table.tsx) and the compass section's toggles; reused the shared PriSection/PriEyebrow wrapper from the mescaline module. All 5 real hero/section photos (CloudFront) spot-checked live before use. Verified live: 200 OK, real content confirmed in rendered HTML, exactly 1 header/1 footer, typecheck/lint clean.</t>
+          <t>MescalineDeepDive, real receptor pharmacology table, the real "Latuda Mirror" same-target-opposite-action comparison, real clinical outcomes (Agin-Liebes et al. 2021, n=452), the real 16-row pharma-to-plant alternatives table, real supplement protocol (pre/day-of/post-integration), real mescaline-specific PRI dimension scores, the real medicine-selector comparison table, and real sources, all ported unchanged and verbatim into lib/content/pri-mescaline-module.ts (copied verbatim) + app/peyote-mescaline/page.tsx. Fully static except the pharma-table expand toggle, extracted into components/pri/pharma-table.tsx; shared PriSection/PriEyebrow wrapper (components/pri/pri-section.tsx) introduced here for reuse by the remaining PRI deep-dive modules. All 8 real section photos (CloudFront) spot-checked live before use; legacy's purely decorative glitch-scanline overlays dropped. Verified live: 200 OK, real content confirmed in rendered HTML, exactly 1 header/1 footer, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E205" s="14" t="inlineStr">
@@ -5640,7 +5640,7 @@
       <c r="A206" s="4" t="n"/>
       <c r="B206" s="4" t="inlineStr">
         <is>
-          <t>PRI: /iboga-compass</t>
+          <t>PRI: /iboga-ibogaine</t>
         </is>
       </c>
       <c r="C206" s="13" t="inlineStr">
@@ -5650,7 +5650,7 @@
       </c>
       <c r="D206" s="4" t="inlineStr">
         <is>
-          <t>IbogaCompassAssessment, the real interactive 28-question / 7-section compass (outcome/medical/approach/logistics/geography/personal/aftercare), the real drag-or-arrow priority-rank step (top dimension ×2.0, bottom ×0.5), the real facility-scoring engine, and the real results view (matched facilities with real "why this matched" reasoning and real elimination reasons), all ported unchanged and verbatim. lib/content/pri-iboga-compass-engine.ts (real scoring logic — weight deltas, hard filters, substance bonuses, priority-rank application, facility scoring) and lib/content/pri-iboga-facility-data.ts (real facility directory + substance-bonus data) both copied verbatim from legacy rather than hand-transcribed, given this is the actual matching algorithm — correctness matters more here than anywhere else in this migration. Uses this site's own brand-gold/foreground/muted-foreground design tokens rather than the pri-* palette — legacy's own hex here (#8B6914) is an exact match for brand-gold, confirming this one page always used the main site identity, not a PRI-specific one. Real backend gap handled honestly: legacy's lead-capture gate posted a rich structured payload (question-by-question answers, top facility matches, primary goal, budget range) to trpc.assessments.submit (no backend built for this migration) — replaced with a mailto: to Tony carrying the same structured summary, same pattern used throughout this migration; the meaningless "Submitting..." pending state and its e</t>
+          <t>IbogaDeepDive, "The Plant vs The Isolate": real alkaloid-profile comparison, real receptor pharmacology, real head-to-head iboga-vs-ibogaine table, real clinical outcomes (Mash/Noller/Schenberg/Brown &amp; Alper/Cherian/Williams — including the 2024 Stanford Nature Medicine SOF-veteran data and the 2026 19,071-patient safety analysis), real pharma-to-plant alternatives, real supplement protocol, real dimension thresholds, real medicine selector, Tony's real first-hand account of sitting ibogaine at The Mission Within, real hard-stop contraindications, a real 9-facility directory (with the 2 facilities legacy explicitly removed and why), real Nagoya Protocol / extractive-capitalism argument, real 2026 US legal-status rundown, the embedded Iboga Compass v2 documentation section (components/pri/iboga-compass-section.tsx, its own client island for the question-group toggles), and real sources — all ported unchanged and verbatim into lib/content/pri-iboga-module.ts + lib/content/pri-iboga-compass-data.ts (both copied verbatim) + app/iboga-ibogaine/page.tsx. Fully static except the pharma-table expand toggle (components/pri/iboga-pharma-table.tsx) and the compass section's toggles; reused the shared PriSection/PriEyebrow wrapper from the mescaline module. All 5 real hero/section photos (CloudFront) spot-checked live before use. Verified live: 200 OK, real content confirmed in rendered HTML, exactly 1 header/1 footer, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E206" s="14" t="inlineStr">
@@ -5663,7 +5663,7 @@
       <c r="A207" s="4" t="n"/>
       <c r="B207" s="4" t="inlineStr">
         <is>
-          <t>PRI: /pri-calibration</t>
+          <t>PRI: /iboga-compass</t>
         </is>
       </c>
       <c r="C207" s="13" t="inlineStr">
@@ -5673,7 +5673,7 @@
       </c>
       <c r="D207" s="4" t="inlineStr">
         <is>
-          <t>forced-rank calibration study, the real Bradley-Terry pairwise-comparison model (all 15 unique pairs of the 6 PRI dimensions), the real drag-or-arrow full ranking step, real methodology copy (acquiescence-bias explanation, the 4 headline validation stats), and the real Monte Carlo validation metrics (lib/content/pri-efficacy-data.json, copied verbatim from legacy — also feeds /pri-efficacy below), all ported unchanged into components/pri/calibration-assessment.tsx. Real backend gap, handled honestly: legacy's "Contribute to Research?" opt-in phase posted to trpc.priCalibration.submit (no backend built for this migration), and the results view's "Community Data" section read a live trpc.priCalibration.stats aggregate query showing other users' scores — neither has an honest backend-free equivalent (a cross-user aggregate can't be faked locally, and a research opt-in toggle with nothing behind it would be dishonest UI, the same call already made dropping the main PRI results page's inert research-pool checkbox). Both dropped; the flow goes straight from ranking to results. Verified live: 200 OK, real content confirmed in rendered HTML, exactly 1 header/1 footer, typecheck/lint clean.</t>
+          <t>IbogaCompassAssessment, the real interactive 28-question / 7-section compass (outcome/medical/approach/logistics/geography/personal/aftercare), the real drag-or-arrow priority-rank step (top dimension ×2.0, bottom ×0.5), the real facility-scoring engine, and the real results view (matched facilities with real "why this matched" reasoning and real elimination reasons), all ported unchanged and verbatim. lib/content/pri-iboga-compass-engine.ts (real scoring logic — weight deltas, hard filters, substance bonuses, priority-rank application, facility scoring) and lib/content/pri-iboga-facility-data.ts (real facility directory + substance-bonus data) both copied verbatim from legacy rather than hand-transcribed, given this is the actual matching algorithm — correctness matters more here than anywhere else in this migration. Uses this site's own brand-gold/foreground/muted-foreground design tokens rather than the pri-* palette — legacy's own hex here (#8B6914) is an exact match for brand-gold, confirming this one page always used the main site identity, not a PRI-specific one. Real backend gap handled honestly: legacy's lead-capture gate posted a rich structured payload (question-by-question answers, top facility matches, primary goal, budget range) to trpc.assessments.submit (no backend built for this migration) — replaced with a mailto: to Tony carrying the same structured summary, same pattern used throughout this migration; the meaningless "Submitting..." pending state and its e</t>
         </is>
       </c>
       <c r="E207" s="14" t="inlineStr">
@@ -5686,7 +5686,7 @@
       <c r="A208" s="4" t="n"/>
       <c r="B208" s="4" t="inlineStr">
         <is>
-          <t>PRI: /pri-efficacy</t>
+          <t>PRI: /pri-calibration</t>
         </is>
       </c>
       <c r="C208" s="13" t="inlineStr">
@@ -5696,7 +5696,7 @@
       </c>
       <c r="D208" s="4" t="inlineStr">
         <is>
-          <t>psychometric validation dashboard, the real Monte Carlo simulation results (10,000 synthetic respondents), real classification-accuracy comparison, real dimension-priority distribution (the real first-dimension-inflation finding), real test-retest reliability and entropy metrics, and the real methodology writeup, all ported unchanged into app/pri-efficacy/page.tsx, reading the same lib/content/pri-efficacy-data.json also used by /pri-calibration. Real backend gap, handled honestly: legacy's "Live Calibrations" tab read a live trpc.priCalibration.stats query — since /pri-calibration's own submit call was already dropped (no backend, see that page's port note), this tab would permanently render "0 total calibrations, no data yet," a dead feature masquerading as a live one. Dropped entirely rather than ship a perpetually-empty tab; only the real, fully-populated Simulation view ships — which also means this page has no state left at all, so it's a plain Server Component now instead of a client one. Verified live: 200 OK, real content confirmed in rendered HTML, exactly 1 header/1 footer, typecheck/lint clean.</t>
+          <t>forced-rank calibration study, the real Bradley-Terry pairwise-comparison model (all 15 unique pairs of the 6 PRI dimensions), the real drag-or-arrow full ranking step, real methodology copy (acquiescence-bias explanation, the 4 headline validation stats), and the real Monte Carlo validation metrics (lib/content/pri-efficacy-data.json, copied verbatim from legacy — also feeds /pri-efficacy below), all ported unchanged into components/pri/calibration-assessment.tsx. Real backend gap, handled honestly: legacy's "Contribute to Research?" opt-in phase posted to trpc.priCalibration.submit (no backend built for this migration), and the results view's "Community Data" section read a live trpc.priCalibration.stats aggregate query showing other users' scores — neither has an honest backend-free equivalent (a cross-user aggregate can't be faked locally, and a research opt-in toggle with nothing behind it would be dishonest UI, the same call already made dropping the main PRI results page's inert research-pool checkbox). Both dropped; the flow goes straight from ranking to results. Verified live: 200 OK, real content confirmed in rendered HTML, exactly 1 header/1 footer, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E208" s="14" t="inlineStr">
@@ -5709,7 +5709,7 @@
       <c r="A209" s="4" t="n"/>
       <c r="B209" s="4" t="inlineStr">
         <is>
-          <t>PRI: /pri-research Built 2026-10-06 behind the login: admins are the emails in ADMIN_EMAILS; everyone else gets live's "Access Denied"</t>
+          <t>PRI: /pri-efficacy</t>
         </is>
       </c>
       <c r="C209" s="13" t="inlineStr">
@@ -5719,7 +5719,7 @@
       </c>
       <c r="D209" s="4" t="inlineStr">
         <is>
-          <t>Totals, anonymized opt-in table, admin-only CSV export (/pri-research/export). /pri-calibration regained legacy's "Contribute to Research?" step and now saves every calibration anonymously to pri_calibrations (opt-ins flagged). Was: — Deferred, not skipped (access-model question resolved by inspection). Read the real legacy source: this is a genuine admin-only dashboard (useAuth() gated to role === "admin") showing trpc.priCalibration.researchData — the same calibration-submission backend already confirmed absent and intentionally not built for /pri-calibration and /pri-efficacy (see their port notes). No admin-auth system exists anywhere in this Next.js migration yet either. So this isn't just an access-control decision — even fully wired up, the page would have zero real data to show, forever. Not worth building an admin dashboard against a backend this migration has twice already decided not to build. Added to "Explicitly deferred" below alongside the other admin dashboards; revisit only if/when both a real admin-auth system and a real calibration-submission backend exist.</t>
+          <t>psychometric validation dashboard, the real Monte Carlo simulation results (10,000 synthetic respondents), real classification-accuracy comparison, real dimension-priority distribution (the real first-dimension-inflation finding), real test-retest reliability and entropy metrics, and the real methodology writeup, all ported unchanged into app/pri-efficacy/page.tsx, reading the same lib/content/pri-efficacy-data.json also used by /pri-calibration. Real backend gap, handled honestly: legacy's "Live Calibrations" tab read a live trpc.priCalibration.stats query — since /pri-calibration's own submit call was already dropped (no backend, see that page's port note), this tab would permanently render "0 total calibrations, no data yet," a dead feature masquerading as a live one. Dropped entirely rather than ship a perpetually-empty tab; only the real, fully-populated Simulation view ships — which also means this page has no state left at all, so it's a plain Server Component now instead of a client one. Verified live: 200 OK, real content confirmed in rendered HTML, exactly 1 header/1 footer, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E209" s="14" t="inlineStr">
@@ -5732,7 +5732,7 @@
       <c r="A210" s="4" t="n"/>
       <c r="B210" s="4" t="inlineStr">
         <is>
-          <t>PRI: /facilitator-index</t>
+          <t>PRI: /pri-research Built 2026-10-06 behind the login: admins are the emails in ADMIN_EMAILS; everyone else gets live's "Access Denied"</t>
         </is>
       </c>
       <c r="C210" s="13" t="inlineStr">
@@ -5742,7 +5742,7 @@
       </c>
       <c r="D210" s="4" t="inlineStr">
         <is>
-          <t>"The Facilitator Index: Know Who You Go With," the real 15-question quick-intake archetype quiz (real Bradley-Terry-style axis derivation, fully client-computed via deriveArchetype()), the real 108-item, 12-band (plus Band 0) practitioner self-assessment instrument, and the real methodology prose (rationale, code/tier system, data-handling policy, Reciprocity Gate, Corroboration token system), all ported unchanged and verbatim into lib/content/facilitator-index-data.ts (single authoritative content source) + components/facilitator/* + app/facilitator-index/page.tsx. Real content-drift bug found and fixed: legacy shipped two divergent copies of the same "108 items" — the on-page JSX and a separate printFacilitatorQuestions() print/PDF export using an older, different set of item numbers and band groupings (missing the on-page "Twenty-Five Traditions and Protocols" band entirely) — the print export was never updated when the on-page instrument was revised. Used the on-page version (the one actually shown to visitors) as the single source of truth and rebuilt the print export to generate from that same data, so the two can never diverge again. Real fake-data found and dropped: legacy's PeerStats component's own comment admits its numbers ("163 practitioners mapped so far," etc.) are "seeded, realistic-feeling" — fabricated, not real — dropped entirely, same principle as BrewSoul's stale "reads" counts; UsageCounter's hardcoded 160-practitioner fallback (shown forever since no ba</t>
+          <t>Totals, anonymized opt-in table, admin-only CSV export (/pri-research/export). /pri-calibration regained legacy's "Contribute to Research?" step and now saves every calibration anonymously to pri_calibrations (opt-ins flagged). Was: — Deferred, not skipped (access-model question resolved by inspection). Read the real legacy source: this is a genuine admin-only dashboard (useAuth() gated to role === "admin") showing trpc.priCalibration.researchData — the same calibration-submission backend already confirmed absent and intentionally not built for /pri-calibration and /pri-efficacy (see their port notes). No admin-auth system exists anywhere in this Next.js migration yet either. So this isn't just an access-control decision — even fully wired up, the page would have zero real data to show, forever. Not worth building an admin dashboard against a backend this migration has twice already decided not to build. Added to "Explicitly deferred" below alongside the other admin dashboards; revisit only if/when both a real admin-auth system and a real calibration-submission backend exist.</t>
         </is>
       </c>
       <c r="E210" s="14" t="inlineStr">
@@ -5755,63 +5755,63 @@
       <c r="A211" s="4" t="n"/>
       <c r="B211" s="4" t="inlineStr">
         <is>
+          <t>PRI: /facilitator-index</t>
+        </is>
+      </c>
+      <c r="C211" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D211" s="4" t="inlineStr">
+        <is>
+          <t>"The Facilitator Index: Know Who You Go With," the real 15-question quick-intake archetype quiz (real Bradley-Terry-style axis derivation, fully client-computed via deriveArchetype()), the real 108-item, 12-band (plus Band 0) practitioner self-assessment instrument, and the real methodology prose (rationale, code/tier system, data-handling policy, Reciprocity Gate, Corroboration token system), all ported unchanged and verbatim into lib/content/facilitator-index-data.ts (single authoritative content source) + components/facilitator/* + app/facilitator-index/page.tsx. Real content-drift bug found and fixed: legacy shipped two divergent copies of the same "108 items" — the on-page JSX and a separate printFacilitatorQuestions() print/PDF export using an older, different set of item numbers and band groupings (missing the on-page "Twenty-Five Traditions and Protocols" band entirely) — the print export was never updated when the on-page instrument was revised. Used the on-page version (the one actually shown to visitors) as the single source of truth and rebuilt the print export to generate from that same data, so the two can never diverge again. Real fake-data found and dropped: legacy's PeerStats component's own comment admits its numbers ("163 practitioners mapped so far," etc.) are "seeded, realistic-feeling" — fabricated, not real — dropped entirely, same principle as BrewSoul's stale "reads" counts; UsageCounter's hardcoded 160-practitioner fallback (shown forever since no ba</t>
+        </is>
+      </c>
+      <c r="E211" s="14" t="inlineStr">
+        <is>
+          <t>Phase 7 — PRI &amp; Kava Encyclopedias (19 routes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="4" t="n"/>
+      <c r="B212" s="4" t="inlineStr">
+        <is>
           <t>Port shared safety/medicine data modules (safety-data.ts, medicine-images.ts) as typed .ts content in the new codebase</t>
         </is>
       </c>
-      <c r="C211" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D211" s="4" t="inlineStr">
+      <c r="C212" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D212" s="4" t="inlineStr">
         <is>
           <t>done as part of the main PRI page above (lib/content/pri-safety-data.ts, lib/content/pri-medicine-images.ts, both copied verbatim).</t>
         </is>
       </c>
-      <c r="E211" s="14" t="inlineStr">
+      <c r="E212" s="14" t="inlineStr">
         <is>
           <t>Phase 7 — PRI &amp; Kava Encyclopedias (19 routes)</t>
         </is>
       </c>
     </row>
-    <row r="212">
-      <c r="A212" s="10" t="inlineStr">
+    <row r="213">
+      <c r="A213" s="10" t="inlineStr">
         <is>
           <t>Phase 8 — Attention Theft Manifesto (7 routes)</t>
         </is>
       </c>
-      <c r="B212" s="11" t="n"/>
-      <c r="C212" s="11" t="n"/>
-      <c r="D212" s="12" t="n"/>
-    </row>
-    <row r="213">
-      <c r="A213" s="4" t="n"/>
-      <c r="B213" s="4" t="inlineStr">
-        <is>
-          <t>/attention-theft</t>
-        </is>
-      </c>
-      <c r="C213" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D213" s="4" t="inlineStr">
-        <is>
-          <t>consolidated mega-page. Real content ported in full across all 9 sections (hero, The Sacred, The Heresy economics data + full breakdown table + sources, the 10 Weapons, Legal Arsenal w/ filter + letter template, AI Blocker Finder quiz, Report a Spammer, closing vow + related reading) — AttentionTheft.tsx used as the single source, the 5 pre-consolidation sub-pages not resurrected (they never existed in this codebase anyway). Section "glamour" photography is real, live imagery on RampRate's own CloudFront (already whitelisted in next.config.ts as a non-Manus, permanent host — confirmed all 7 URLs 200 before using them), rendered via next/image. Real backend gap found and handled honestly: legacy's Wall of Shame (a live trpc.spam.wallOfShame ranked list) and the Report form's trpc.spam.submit both depended on a spam-tracking backend that this migration explicitly defers (see "Explicitly deferred" list below: "/youve-been-reported, /spamtoast, admin spam tooling") — rather than fake a public database with no real data behind it, the report form now composes a mailto: to Tony (same honest non-fake-success pattern as newsletter-popup.tsx), and the ranked Wall of Shame list isn't reproduced. Two simplifications matching precedent set elsewhere in this migration: legacy's "Fraunces" serif (loaded for this one page only) was dropped for font-heading (Playfair Display, already loaded — same call made on /akbar), and the glitch/VHS/ember-particle/shattered-glass decoration layer was dr</t>
-        </is>
-      </c>
-      <c r="E213" s="14" t="inlineStr">
-        <is>
-          <t>Phase 8 — Attention Theft Manifesto (7 routes)</t>
-        </is>
-      </c>
+      <c r="B213" s="11" t="n"/>
+      <c r="C213" s="11" t="n"/>
+      <c r="D213" s="12" t="n"/>
     </row>
     <row r="214">
       <c r="A214" s="4" t="n"/>
       <c r="B214" s="4" t="inlineStr">
         <is>
-          <t>Legacy anchor redirects</t>
+          <t>/attention-theft</t>
         </is>
       </c>
       <c r="C214" s="13" t="inlineStr">
@@ -5821,7 +5821,7 @@
       </c>
       <c r="D214" s="4" t="inlineStr">
         <is>
-          <t>/attention-theft/economics, /blocker-finder, /legal, /weapons, /report → /attention-theft#&lt;anchor&gt; via next.config.ts redirects(). Verified live: all return real 308s to the correct anchor.</t>
+          <t>consolidated mega-page. Real content ported in full across all 9 sections (hero, The Sacred, The Heresy economics data + full breakdown table + sources, the 10 Weapons, Legal Arsenal w/ filter + letter template, AI Blocker Finder quiz, Report a Spammer, closing vow + related reading) — AttentionTheft.tsx used as the single source, the 5 pre-consolidation sub-pages not resurrected (they never existed in this codebase anyway). Section "glamour" photography is real, live imagery on RampRate's own CloudFront (already whitelisted in next.config.ts as a non-Manus, permanent host — confirmed all 7 URLs 200 before using them), rendered via next/image. Real backend gap found and handled honestly: legacy's Wall of Shame (a live trpc.spam.wallOfShame ranked list) and the Report form's trpc.spam.submit both depended on a spam-tracking backend that this migration explicitly defers (see "Explicitly deferred" list below: "/youve-been-reported, /spamtoast, admin spam tooling") — rather than fake a public database with no real data behind it, the report form now composes a mailto: to Tony (same honest non-fake-success pattern as newsletter-popup.tsx), and the ranked Wall of Shame list isn't reproduced. Two simplifications matching precedent set elsewhere in this migration: legacy's "Fraunces" serif (loaded for this one page only) was dropped for font-heading (Playfair Display, already loaded — same call made on /akbar), and the glitch/VHS/ember-particle/shattered-glass decoration layer was dr</t>
         </is>
       </c>
       <c r="E214" s="14" t="inlineStr">
@@ -5834,63 +5834,63 @@
       <c r="A215" s="4" t="n"/>
       <c r="B215" s="4" t="inlineStr">
         <is>
+          <t>Legacy anchor redirects</t>
+        </is>
+      </c>
+      <c r="C215" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D215" s="4" t="inlineStr">
+        <is>
+          <t>/attention-theft/economics, /blocker-finder, /legal, /weapons, /report → /attention-theft#&lt;anchor&gt; via next.config.ts redirects(). Verified live: all return real 308s to the correct anchor.</t>
+        </is>
+      </c>
+      <c r="E215" s="14" t="inlineStr">
+        <is>
+          <t>Phase 8 — Attention Theft Manifesto (7 routes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="4" t="n"/>
+      <c r="B216" s="4" t="inlineStr">
+        <is>
           <t>Port ManifestoLayout scroll-tracking wrapper behavior</t>
         </is>
       </c>
-      <c r="C215" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D215" s="4" t="inlineStr">
+      <c r="C216" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D216" s="4" t="inlineStr">
         <is>
           <t>components/manifesto/manifesto-nav.tsx tracks which section is in view on scroll and highlights the matching nav pill (desktop + mobile), real behavior kept per this line item rather than simplified away.</t>
         </is>
       </c>
-      <c r="E215" s="14" t="inlineStr">
+      <c r="E216" s="14" t="inlineStr">
         <is>
           <t>Phase 8 — Attention Theft Manifesto (7 routes)</t>
         </is>
       </c>
     </row>
-    <row r="216">
-      <c r="A216" s="10" t="inlineStr">
+    <row r="217">
+      <c r="A217" s="10" t="inlineStr">
         <is>
           <t>Phase 9 — Assessments (33 routes)</t>
         </is>
       </c>
-      <c r="B216" s="11" t="n"/>
-      <c r="C216" s="11" t="n"/>
-      <c r="D216" s="12" t="n"/>
-    </row>
-    <row r="217">
-      <c r="A217" s="4" t="n"/>
-      <c r="B217" s="4" t="inlineStr">
-        <is>
-          <t>HumanOS section</t>
-        </is>
-      </c>
-      <c r="C217" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D217" s="4" t="inlineStr">
-        <is>
-          <t>/humanos, /humanos/philosophy, /humanos/ecosystem, /humanos/resources, /humanos/connect, /humanos/path-to-here, ported from _legacy-manus-app/client/src/pages/HumanOS.tsx + humanos/*.tsx. The top-level HumanOS.tsx (an iframe embed of an external manus.space site) turned out to be dead code, never wired into legacy's router — the real, routed implementation is HumanosHome/HumanosPhilosophy/HumanosEcosystem/HumanosResources/HumanosConnect/HumanosPathToHere behind HumanosLayout, which is what got ported, with its own nested layout.tsx (route now added to site-chrome.tsx's SUPPRESSED_PREFIXES so the main SiteHeader/SiteFooter don't double up around HumanOS's own nav/footer). Real content in full: the Maximizer-vs-Satisficer framework and "Boiling the Human"/"Maximizer Trap"/"Conscious Satisficer" philosophy sections, the full ecosystem roster (1 mentor, 8 advisors, 3 partners, 29 clients), all 4 transformation playbooks + 3 daily-practice protocols + 8-book reading list, all 4 connect channels, and the 6-entry "Path to Here" timeline (2010 H+ Summit through 2025). Real bugs fixed: every "Take the Diagnostic" CTA site-wide pointed at /assessment, an 8-question Maximizer/Satisficer quiz that was never actually built anywhere (legacy's real /assessment and /assessments routes are two different, unrelated quiz sets) — redirected to /humanos/philosophy, which delivers the actual promised content; Connect's "Read the Living Declaration" pointed at /manifesto, a dead redirect stub in le</t>
-        </is>
-      </c>
-      <c r="E217" s="14" t="inlineStr">
-        <is>
-          <t>Phase 9 — Assessments (33 routes)</t>
-        </is>
-      </c>
+      <c r="B217" s="11" t="n"/>
+      <c r="C217" s="11" t="n"/>
+      <c r="D217" s="12" t="n"/>
     </row>
     <row r="218">
       <c r="A218" s="4" t="n"/>
       <c r="B218" s="4" t="inlineStr">
         <is>
-          <t>/find-your-me (+ /find-my-me, /discover)</t>
+          <t>HumanOS section</t>
         </is>
       </c>
       <c r="C218" s="13" t="inlineStr">
@@ -5900,7 +5900,7 @@
       </c>
       <c r="D218" s="4" t="inlineStr">
         <is>
-          <t>"Find My — To Find Your We," the ecosystem hub assessment and by far the largest page in Phase 9. Real 5 NLP-driven questions, 6 dimensions (relationships/purpose/body/truth/tribe/consciousness), and 6 real archetypes (each with a real description, real blog article links, real satellite-site links, real "go deeper" forward-references, and a real share text) ported unchanged and verbatim into a new lib/content/find-your-me.ts data module (kept separate from the component given the file's exceptional size, same pattern as brewsoul-directory.ts). All 17 unique blog article slugs referenced across the 6 archetypes were individually verified live (200 OK) against this migration's real Sanity blog before porting — zero dead article links. Real accuracy fix: legacy's "Full Ecosystem Directory" (26 items across 5 categories, with a real LIVE/COMING pill UI already built for exactly this purpose) marked everything "live," including several routes that don't exist anywhere in this migration yet (/find-my, /the-mirror, /assessments/dharma-finder, /assessments/consciousness-scale, /assessments/grant-study, /flow-circuit) — corrected each item's status to this app's actual current build state rather than shipping false LIVE labels on what would be 404s. Real completeness fix: added Find Your Peptide and Find Your Sexuality to the directory (Body &amp; Temple and Love &amp; Belonging) — both are real, fully-built assessments elsewhere in this migration that didn't exist yet when legacy was writte</t>
+          <t>/humanos, /humanos/philosophy, /humanos/ecosystem, /humanos/resources, /humanos/connect, /humanos/path-to-here, ported from _legacy-manus-app/client/src/pages/HumanOS.tsx + humanos/*.tsx. The top-level HumanOS.tsx (an iframe embed of an external manus.space site) turned out to be dead code, never wired into legacy's router — the real, routed implementation is HumanosHome/HumanosPhilosophy/HumanosEcosystem/HumanosResources/HumanosConnect/HumanosPathToHere behind HumanosLayout, which is what got ported, with its own nested layout.tsx (route now added to site-chrome.tsx's SUPPRESSED_PREFIXES so the main SiteHeader/SiteFooter don't double up around HumanOS's own nav/footer). Real content in full: the Maximizer-vs-Satisficer framework and "Boiling the Human"/"Maximizer Trap"/"Conscious Satisficer" philosophy sections, the full ecosystem roster (1 mentor, 8 advisors, 3 partners, 29 clients), all 4 transformation playbooks + 3 daily-practice protocols + 8-book reading list, all 4 connect channels, and the 6-entry "Path to Here" timeline (2010 H+ Summit through 2025). Real bugs fixed: every "Take the Diagnostic" CTA site-wide pointed at /assessment, an 8-question Maximizer/Satisficer quiz that was never actually built anywhere (legacy's real /assessment and /assessments routes are two different, unrelated quiz sets) — redirected to /humanos/philosophy, which delivers the actual promised content; Connect's "Read the Living Declaration" pointed at /manifesto, a dead redirect stub in le</t>
         </is>
       </c>
       <c r="E218" s="14" t="inlineStr">
@@ -5913,7 +5913,7 @@
       <c r="A219" s="4" t="n"/>
       <c r="B219" s="4" t="inlineStr">
         <is>
-          <t>/find-your-therapy (+ /find-my-therapy)</t>
+          <t>/find-your-me (+ /find-my-me, /discover)</t>
         </is>
       </c>
       <c r="C219" s="13" t="inlineStr">
@@ -5923,7 +5923,7 @@
       </c>
       <c r="D219" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Real 25 questions across 6 dimensions (Cognitive/Somatic/Relational/Depth-Unconscious/Altered States/Integrative), 6 real therapeutic modalities (each with a real description, "how it works," best-for/not-ideal-for lists, real named pioneers, and real book/directory resources), and the real archetype-matching logic (highest-scoring dimension wins) ported unchanged and verbatim. Three real stale-count bugs found and fixed: legacy's own file-header comment claimed "10 questions," its AssessmentIntro stats prop claimed 20 — neither matches the real 25-item array (the scoring code's own maxPossible = 30 // rough max per dimension with 25 questions comment confirms 25 is correct) — replaced both with live QUESTIONS.length. Real dead-link bug fixed: legacy's "Journey Continues" grid linked "Find Your Spirit"/"Find Your Religion" to external findmyassess-9eekxcob.manus.space stub URLs (dead Manus domain) despite this migration already having real, fully-built internal pages at /find-your-spirit and /find-your-religion — repointed to the real internal routes, and corrected Religion's stale "15 Questions" badge to the real 20. Real accent-color inconsistency fixed: legacy passed accentColor="#7B1FA2" only to the landing screen, then hardcoded brand-gold everywhere on the results screen instead — threaded one ACCENT constant through intro/radar/result-actions consistently, matching every other assessment in this migration. The "Also Worth Exploring" related-modality cards were dropped </t>
+          <t>"Find My — To Find Your We," the ecosystem hub assessment and by far the largest page in Phase 9. Real 5 NLP-driven questions, 6 dimensions (relationships/purpose/body/truth/tribe/consciousness), and 6 real archetypes (each with a real description, real blog article links, real satellite-site links, real "go deeper" forward-references, and a real share text) ported unchanged and verbatim into a new lib/content/find-your-me.ts data module (kept separate from the component given the file's exceptional size, same pattern as brewsoul-directory.ts). All 17 unique blog article slugs referenced across the 6 archetypes were individually verified live (200 OK) against this migration's real Sanity blog before porting — zero dead article links. Real accuracy fix: legacy's "Full Ecosystem Directory" (26 items across 5 categories, with a real LIVE/COMING pill UI already built for exactly this purpose) marked everything "live," including several routes that don't exist anywhere in this migration yet (/find-my, /the-mirror, /assessments/dharma-finder, /assessments/consciousness-scale, /assessments/grant-study, /flow-circuit) — corrected each item's status to this app's actual current build state rather than shipping false LIVE labels on what would be 404s. Real completeness fix: added Find Your Peptide and Find Your Sexuality to the directory (Body &amp; Temple and Love &amp; Belonging) — both are real, fully-built assessments elsewhere in this migration that didn't exist yet when legacy was writte</t>
         </is>
       </c>
       <c r="E219" s="14" t="inlineStr">
@@ -5936,7 +5936,7 @@
       <c r="A220" s="4" t="n"/>
       <c r="B220" s="4" t="inlineStr">
         <is>
-          <t>/find-your-sake</t>
+          <t>/find-your-therapy (+ /find-my-therapy)</t>
         </is>
       </c>
       <c r="C220" s="13" t="inlineStr">
@@ -5946,7 +5946,7 @@
       </c>
       <c r="D220" s="4" t="inlineStr">
         <is>
-          <t>Real 20 questions across 5 dimensions (Palate/Ritual/Terroir/Philosophy/Season) and the real 5 sake profiles (each with real Japanese name, tasting notes, food pairings, serving temperature, named producers with region/note, and further-reading resources) ported unchanged and verbatim. Legacy's own AssessmentIntro stats prop claimed "15 questions, 6 dimensions" — didn't match the real 20/5 implementation — replaced with live QUESTIONS.length/DIMENSIONS.length counts, same fix pattern already applied on /find-your-attachment-style and /find-your-sexuality. Two real bugs found and fixed: (1) legacy's "Journey Continues" list read "Find Myzcal" — a literal typo for "Find Your Mezcal" — corrected. (2) legacy's JSX rendered &lt;WhatsNext /&gt; (a full page section) nested inside the small "Retake the Tasting" &lt;button&gt; element — moved to a proper top-level section, same class of nested-interactive-content bug already fixed on /find-your-religion. The dark GlassPanel treatment (near-black translucent cards with light cream text, sitting on the page's own light parchment ThemedBackground) was kept as a real, intentional design choice rather than "fixed" to this migration's usual light-card convention — unlike the light-text-directly-on-light-background contrast bugs found on Style/Sexuality/Peptide/Religion, the text here sits inside its own correctly-contrasted dark card. SacredGeometryBg's canvas-based floating rice-grain particles dropped (same decoration-not-worth-the-JS-cost call made</t>
+          <t xml:space="preserve">Real 25 questions across 6 dimensions (Cognitive/Somatic/Relational/Depth-Unconscious/Altered States/Integrative), 6 real therapeutic modalities (each with a real description, "how it works," best-for/not-ideal-for lists, real named pioneers, and real book/directory resources), and the real archetype-matching logic (highest-scoring dimension wins) ported unchanged and verbatim. Three real stale-count bugs found and fixed: legacy's own file-header comment claimed "10 questions," its AssessmentIntro stats prop claimed 20 — neither matches the real 25-item array (the scoring code's own maxPossible = 30 // rough max per dimension with 25 questions comment confirms 25 is correct) — replaced both with live QUESTIONS.length. Real dead-link bug fixed: legacy's "Journey Continues" grid linked "Find Your Spirit"/"Find Your Religion" to external findmyassess-9eekxcob.manus.space stub URLs (dead Manus domain) despite this migration already having real, fully-built internal pages at /find-your-spirit and /find-your-religion — repointed to the real internal routes, and corrected Religion's stale "15 Questions" badge to the real 20. Real accent-color inconsistency fixed: legacy passed accentColor="#7B1FA2" only to the landing screen, then hardcoded brand-gold everywhere on the results screen instead — threaded one ACCENT constant through intro/radar/result-actions consistently, matching every other assessment in this migration. The "Also Worth Exploring" related-modality cards were dropped </t>
         </is>
       </c>
       <c r="E220" s="14" t="inlineStr">
@@ -5959,7 +5959,7 @@
       <c r="A221" s="4" t="n"/>
       <c r="B221" s="4" t="inlineStr">
         <is>
-          <t>/find-your-spirit (+ /find-my-spirit), along with a shared PDF-export component the rest of Phase 9 can reuse</t>
+          <t>/find-your-sake</t>
         </is>
       </c>
       <c r="C221" s="13" t="inlineStr">
@@ -5969,7 +5969,7 @@
       </c>
       <c r="D221" s="4" t="inlineStr">
         <is>
-          <t>Real 35 questions, 10 dimensions, and the 6 real spiritual traditions (each with real description/practices/key texts/figures/modern expressions/growth edge) ported unchanged and verbatim — legacy's own file-header comment claimed "12 archetypes," but only 6 TRADITIONS actually exist in the code; ported the real 6, not the stale doc comment. The real weighted tradition-matching logic (top 3 dimensions per tradition, weighted 3/2/1) is unchanged. Ported components/assessments/result-actions.tsx from legacy's AssessmentResultActions — kept only the real, backend-free "Download PDF" action (browser print); the "Send to Tony"/"Keep Private" buttons posted to an unbuilt trpc.assessments.submit and weren't reproduced, same honest-degradation pattern used throughout this migration. Verified live: 200 OK, redirect confirmed 308, typecheck/lint clean.</t>
+          <t>Real 20 questions across 5 dimensions (Palate/Ritual/Terroir/Philosophy/Season) and the real 5 sake profiles (each with real Japanese name, tasting notes, food pairings, serving temperature, named producers with region/note, and further-reading resources) ported unchanged and verbatim. Legacy's own AssessmentIntro stats prop claimed "15 questions, 6 dimensions" — didn't match the real 20/5 implementation — replaced with live QUESTIONS.length/DIMENSIONS.length counts, same fix pattern already applied on /find-your-attachment-style and /find-your-sexuality. Two real bugs found and fixed: (1) legacy's "Journey Continues" list read "Find Myzcal" — a literal typo for "Find Your Mezcal" — corrected. (2) legacy's JSX rendered &lt;WhatsNext /&gt; (a full page section) nested inside the small "Retake the Tasting" &lt;button&gt; element — moved to a proper top-level section, same class of nested-interactive-content bug already fixed on /find-your-religion. The dark GlassPanel treatment (near-black translucent cards with light cream text, sitting on the page's own light parchment ThemedBackground) was kept as a real, intentional design choice rather than "fixed" to this migration's usual light-card convention — unlike the light-text-directly-on-light-background contrast bugs found on Style/Sexuality/Peptide/Religion, the text here sits inside its own correctly-contrasted dark card. SacredGeometryBg's canvas-based floating rice-grain particles dropped (same decoration-not-worth-the-JS-cost call made</t>
         </is>
       </c>
       <c r="E221" s="14" t="inlineStr">
@@ -5982,7 +5982,7 @@
       <c r="A222" s="4" t="n"/>
       <c r="B222" s="4" t="inlineStr">
         <is>
-          <t>/find-your-religion</t>
+          <t>/find-your-spirit (+ /find-my-spirit), along with a shared PDF-export component the rest of Phase 9 can reuse</t>
         </is>
       </c>
       <c r="C222" s="13" t="inlineStr">
@@ -5992,7 +5992,7 @@
       </c>
       <c r="D222" s="4" t="inlineStr">
         <is>
-          <t>Real 20 questions across 8 dimensions, 8 real spiritual/philosophical archetypes (each with real description/practices/key texts/figures/resonant traditions/growth-edge tensions), and the real scoring/matching logic ported unchanged and verbatim. Real bug found and fixed: legacy's own JSX rendered &lt;AssessmentResultActions&gt; nested inside the "Retake Assessment" &lt;button&gt; element — a button inside a button, invalid HTML — fixed by rendering it as a sibling instead, same fix pattern already applied on /find-your-spirit. Verified live: 200 OK, typecheck/lint clean.</t>
+          <t>Real 35 questions, 10 dimensions, and the 6 real spiritual traditions (each with real description/practices/key texts/figures/modern expressions/growth edge) ported unchanged and verbatim — legacy's own file-header comment claimed "12 archetypes," but only 6 TRADITIONS actually exist in the code; ported the real 6, not the stale doc comment. The real weighted tradition-matching logic (top 3 dimensions per tradition, weighted 3/2/1) is unchanged. Ported components/assessments/result-actions.tsx from legacy's AssessmentResultActions — kept only the real, backend-free "Download PDF" action (browser print); the "Send to Tony"/"Keep Private" buttons posted to an unbuilt trpc.assessments.submit and weren't reproduced, same honest-degradation pattern used throughout this migration. Verified live: 200 OK, redirect confirmed 308, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E222" s="14" t="inlineStr">
@@ -6005,7 +6005,7 @@
       <c r="A223" s="4" t="n"/>
       <c r="B223" s="4" t="inlineStr">
         <is>
-          <t>/find-your-diet (+ /find-my-diet)</t>
+          <t>/find-your-religion</t>
         </is>
       </c>
       <c r="C223" s="13" t="inlineStr">
@@ -6015,7 +6015,7 @@
       </c>
       <c r="D223" s="4" t="inlineStr">
         <is>
-          <t>Real 15 questions, 6 real archetypes (with descriptions), and the real nearest-neighbor archetype-matching logic ported unchanged. Legacy's dead JourneyTracker import wired in for real (see journey-tracker.tsx). /find-my-diet → /find-your-diet redirect added. Verified live: 200 OK, full quiz flow, redirect confirmed 308, typecheck/lint clean.</t>
+          <t>Real 20 questions across 8 dimensions, 8 real spiritual/philosophical archetypes (each with real description/practices/key texts/figures/resonant traditions/growth-edge tensions), and the real scoring/matching logic ported unchanged and verbatim. Real bug found and fixed: legacy's own JSX rendered &lt;AssessmentResultActions&gt; nested inside the "Retake Assessment" &lt;button&gt; element — a button inside a button, invalid HTML — fixed by rendering it as a sibling instead, same fix pattern already applied on /find-your-spirit. Verified live: 200 OK, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E223" s="14" t="inlineStr">
@@ -6028,7 +6028,7 @@
       <c r="A224" s="4" t="n"/>
       <c r="B224" s="4" t="inlineStr">
         <is>
-          <t>/find-your-movement (+ /find-my-movement), along with the shared assessment foundation the rest of Phase 9 depends on</t>
+          <t>/find-your-diet (+ /find-my-diet)</t>
         </is>
       </c>
       <c r="C224" s="13" t="inlineStr">
@@ -6038,7 +6038,7 @@
       </c>
       <c r="D224" s="4" t="inlineStr">
         <is>
-          <t>Ported components/assessments/{themed-background,assessment-intro,email-gate,whats-next}.tsx from legacy's ThemedBackground/AssessmentIntro/EmailGate/WhatsNext — real content/behavior unchanged, with 2 real fixes along the way: (1) EmailGate now posts to the real /api/subscribe Route Handler (built earlier this migration) using the exact find-your-&lt;slug&gt; source keys already defined in lib/content/kit-source-tags.ts's KIT_TAG_MAP — legacy's own assessment-gate:&lt;slug&gt; prefix didn't match any tag in that map, so this is a genuine improvement, not just a port. (2) ThemedBackground's per-theme decorative particle field + SVG sacred-geometry overlay + 2 extra radial-glow layers dropped (same "not worth the cost" call made repeatedly elsewhere) — the real per-theme base gradient (16 themes) is kept, precomposed as one literal Tailwind class per theme rather than assembled from fragments. find-your-movement-quiz.tsx ports all 15 real questions and the real 6-dimension (Strength/Flexibility/Endurance/Mindfulness/Community/Adventure) scoring unchanged; the legacy JourneyTracker/useJourneyProgress import in the source file was dead code (imported, never rendered) and not ported. /find-my-movement → /find-your-movement redirect added (next.config.ts), same duplicate-route pattern as /find-my-tribe. Verified live: 200 OK, full quiz flow renders, redirect confirmed 308, typecheck/lint clean.</t>
+          <t>Real 15 questions, 6 real archetypes (with descriptions), and the real nearest-neighbor archetype-matching logic ported unchanged. Legacy's dead JourneyTracker import wired in for real (see journey-tracker.tsx). /find-my-diet → /find-your-diet redirect added. Verified live: 200 OK, full quiz flow, redirect confirmed 308, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E224" s="14" t="inlineStr">
@@ -6051,7 +6051,7 @@
       <c r="A225" s="4" t="n"/>
       <c r="B225" s="4" t="inlineStr">
         <is>
-          <t>/find-your-sleep (+ /find-my-sleep)</t>
+          <t>/find-your-movement (+ /find-my-movement), along with the shared assessment foundation the rest of Phase 9 depends on</t>
         </is>
       </c>
       <c r="C225" s="13" t="inlineStr">
@@ -6061,7 +6061,7 @@
       </c>
       <c r="D225" s="4" t="inlineStr">
         <is>
-          <t>Real 15 questions, 6 real archetypes, and the real cascading archetype-match logic ported unchanged, including legacy's own real behavioral quirk of rendering JourneyTracker on every phase (not just results). One real duplicate-destination "Journey Continues" link pair dropped (see file's own port note), the one real distinct link (Find Your Diet) kept. /find-my-sleep → /find-your-sleep redirect added. Verified live: 200 OK, redirect confirmed 308, typecheck/lint clean.</t>
+          <t>Ported components/assessments/{themed-background,assessment-intro,email-gate,whats-next}.tsx from legacy's ThemedBackground/AssessmentIntro/EmailGate/WhatsNext — real content/behavior unchanged, with 2 real fixes along the way: (1) EmailGate now posts to the real /api/subscribe Route Handler (built earlier this migration) using the exact find-your-&lt;slug&gt; source keys already defined in lib/content/kit-source-tags.ts's KIT_TAG_MAP — legacy's own assessment-gate:&lt;slug&gt; prefix didn't match any tag in that map, so this is a genuine improvement, not just a port. (2) ThemedBackground's per-theme decorative particle field + SVG sacred-geometry overlay + 2 extra radial-glow layers dropped (same "not worth the cost" call made repeatedly elsewhere) — the real per-theme base gradient (16 themes) is kept, precomposed as one literal Tailwind class per theme rather than assembled from fragments. find-your-movement-quiz.tsx ports all 15 real questions and the real 6-dimension (Strength/Flexibility/Endurance/Mindfulness/Community/Adventure) scoring unchanged; the legacy JourneyTracker/useJourneyProgress import in the source file was dead code (imported, never rendered) and not ported. /find-my-movement → /find-your-movement redirect added (next.config.ts), same duplicate-route pattern as /find-my-tribe. Verified live: 200 OK, full quiz flow renders, redirect confirmed 308, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E225" s="14" t="inlineStr">
@@ -6074,7 +6074,7 @@
       <c r="A226" s="4" t="n"/>
       <c r="B226" s="4" t="inlineStr">
         <is>
-          <t>/find-your-coffee (+ /find-my-coffee)</t>
+          <t>/find-your-sleep (+ /find-my-sleep)</t>
         </is>
       </c>
       <c r="C226" s="13" t="inlineStr">
@@ -6084,7 +6084,7 @@
       </c>
       <c r="D226" s="4" t="inlineStr">
         <is>
-          <t>Real 15 questions, 6 dimensions (Roast Preference/Origin Curiosity/Brewing Ritual/Social Context/Caffeine Sensitivity/Flavor Complexity), 6 real archetypes (each with a real description and 5 real named coffee recommendations — roaster, origin, roast level, tasting notes, real "why" rationale), and the real archetype-matching logic (sum of each archetype's 2 primary dimensions, highest wins) ported unchanged and verbatim. This legacy page predates the shared ThemedBackground/AssessmentIntro component system the rest of Phase 9 is built on — it hand-rolled its own hero-image page shell — so it needed more normalization than most: its hero image (/api/img/coffee-orig_a935f111.jpg) was a dead Manus asset, dropped for the standard ThemedBackground light theme (added a new "coffee" warm-cream entry) instead of reproducing a broken background; the canvas bean-particle field, floating steam-wisp divs, and SVG sacred-geometry overlay all dropped (same decoration-not-worth-the-JS-cost call made repeatedly elsewhere). Real bug found and fixed: legacy read window.innerWidth directly during render (twice — to pick grid columns and flex direction), unsafe during SSR and a real hydration-mismatch source — replaced with responsive Tailwind classes. EmailGate's prop was legacy's assessmentName; ported using this repo's real assessmentSlug="coffee" to match find-your-coffee in KIT_TAG_MAP. Legacy imported useJourneyProgress for markComplete but never rendered a visible JourneyTracker, and nev</t>
+          <t>Real 15 questions, 6 real archetypes, and the real cascading archetype-match logic ported unchanged, including legacy's own real behavioral quirk of rendering JourneyTracker on every phase (not just results). One real duplicate-destination "Journey Continues" link pair dropped (see file's own port note), the one real distinct link (Find Your Diet) kept. /find-my-sleep → /find-your-sleep redirect added. Verified live: 200 OK, redirect confirmed 308, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E226" s="14" t="inlineStr">
@@ -6097,7 +6097,7 @@
       <c r="A227" s="4" t="n"/>
       <c r="B227" s="4" t="inlineStr">
         <is>
-          <t>/find-your-kitchen. Real 15 questions (all rendered on one page at once</t>
+          <t>/find-your-coffee (+ /find-my-coffee)</t>
         </is>
       </c>
       <c r="C227" s="13" t="inlineStr">
@@ -6107,7 +6107,7 @@
       </c>
       <c r="D227" s="4" t="inlineStr">
         <is>
-          <t>a genuinely different, legacy-intentional UX from the other paginated quizzes, kept as-is) and the real dual-tracking scoring (answer score keys split into archetype tallies vs. 6 separate radar-chart dimensions) ported unchanged, including the 3 real "Journey Continues" links (one to already-built /find-your-diet, one forward-reference to /find-your-style). Verified live: 200 OK, typecheck/lint clean.</t>
+          <t>Real 15 questions, 6 dimensions (Roast Preference/Origin Curiosity/Brewing Ritual/Social Context/Caffeine Sensitivity/Flavor Complexity), 6 real archetypes (each with a real description and 5 real named coffee recommendations — roaster, origin, roast level, tasting notes, real "why" rationale), and the real archetype-matching logic (sum of each archetype's 2 primary dimensions, highest wins) ported unchanged and verbatim. This legacy page predates the shared ThemedBackground/AssessmentIntro component system the rest of Phase 9 is built on — it hand-rolled its own hero-image page shell — so it needed more normalization than most: its hero image (/api/img/coffee-orig_a935f111.jpg) was a dead Manus asset, dropped for the standard ThemedBackground light theme (added a new "coffee" warm-cream entry) instead of reproducing a broken background; the canvas bean-particle field, floating steam-wisp divs, and SVG sacred-geometry overlay all dropped (same decoration-not-worth-the-JS-cost call made repeatedly elsewhere). Real bug found and fixed: legacy read window.innerWidth directly during render (twice — to pick grid columns and flex direction), unsafe during SSR and a real hydration-mismatch source — replaced with responsive Tailwind classes. EmailGate's prop was legacy's assessmentName; ported using this repo's real assessmentSlug="coffee" to match find-your-coffee in KIT_TAG_MAP. Legacy imported useJourneyProgress for markComplete but never rendered a visible JourneyTracker, and nev</t>
         </is>
       </c>
       <c r="E227" s="14" t="inlineStr">
@@ -6120,7 +6120,7 @@
       <c r="A228" s="4" t="n"/>
       <c r="B228" s="4" t="inlineStr">
         <is>
-          <t>/find-your-style. Real 15 questions, 6 real archetypes, and the real (if crude</t>
+          <t>/find-your-kitchen. Real 15 questions (all rendered on one page at once</t>
         </is>
       </c>
       <c r="C228" s="13" t="inlineStr">
@@ -6130,7 +6130,7 @@
       </c>
       <c r="D228" s="4" t="inlineStr">
         <is>
-          <t>legacy's own comment admits "Simple mapping for demonstration") threshold-based archetype match ported unchanged. Two real inconsistencies found and normalized: legacy's own inline styles used near-illegible light text on ThemedBackground's actual light pastel "style" theme (inconsistent with every other assessment in this migration); and legacy rendered &lt;JourneyTracker /&gt; defaulting to variant="dark" on a light results screen instead of the variant="light" every other assessment passes. Verified live: 200 OK, typecheck/lint clean.</t>
+          <t>a genuinely different, legacy-intentional UX from the other paginated quizzes, kept as-is) and the real dual-tracking scoring (answer score keys split into archetype tallies vs. 6 separate radar-chart dimensions) ported unchanged, including the 3 real "Journey Continues" links (one to already-built /find-your-diet, one forward-reference to /find-your-style). Verified live: 200 OK, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E228" s="14" t="inlineStr">
@@ -6143,7 +6143,7 @@
       <c r="A229" s="4" t="n"/>
       <c r="B229" s="4" t="inlineStr">
         <is>
-          <t>/find-your-attachment-style (+ /find-my-attachment-style, /find-my-we)</t>
+          <t>/find-your-style. Real 15 questions, 6 real archetypes, and the real (if crude</t>
         </is>
       </c>
       <c r="C229" s="13" t="inlineStr">
@@ -6153,7 +6153,7 @@
       </c>
       <c r="D229" s="4" t="inlineStr">
         <is>
-          <t>Real 18 questions (legacy's own AssessmentIntro stats prop under-reported this as "15" — used the live QUESTIONS.length instead of repeating the stale number, same live-count discipline used elsewhere in this migration), the 4 real archetypes, and the real scoring/selection logic all ported unchanged, including the real closing note on attachment theory. Both alt-path redirects added. Verified live: 200 OK, both redirects confirmed 308, typecheck/lint clean.</t>
+          <t>legacy's own comment admits "Simple mapping for demonstration") threshold-based archetype match ported unchanged. Two real inconsistencies found and normalized: legacy's own inline styles used near-illegible light text on ThemedBackground's actual light pastel "style" theme (inconsistent with every other assessment in this migration); and legacy rendered &lt;JourneyTracker /&gt; defaulting to variant="dark" on a light results screen instead of the variant="light" every other assessment passes. Verified live: 200 OK, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E229" s="14" t="inlineStr">
@@ -6166,7 +6166,7 @@
       <c r="A230" s="4" t="n"/>
       <c r="B230" s="4" t="inlineStr">
         <is>
-          <t>/find-your-love-language</t>
+          <t>/find-your-attachment-style (+ /find-my-attachment-style, /find-my-we)</t>
         </is>
       </c>
       <c r="C230" s="13" t="inlineStr">
@@ -6176,7 +6176,7 @@
       </c>
       <c r="D230" s="4" t="inlineStr">
         <is>
-          <t>Real 15 questions (incl. the negative-score "disconnect" question), 5 real archetypes with descriptions/tips, and Dr. Gary Chapman's real attribution note all ported unchanged. Verified live: 200 OK, full quiz flow, typecheck/lint clean.</t>
+          <t>Real 18 questions (legacy's own AssessmentIntro stats prop under-reported this as "15" — used the live QUESTIONS.length instead of repeating the stale number, same live-count discipline used elsewhere in this migration), the 4 real archetypes, and the real scoring/selection logic all ported unchanged, including the real closing note on attachment theory. Both alt-path redirects added. Verified live: 200 OK, both redirects confirmed 308, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E230" s="14" t="inlineStr">
@@ -6189,7 +6189,7 @@
       <c r="A231" s="4" t="n"/>
       <c r="B231" s="4" t="inlineStr">
         <is>
-          <t>/find-your-peptide (+ /find-my-peptide)</t>
+          <t>/find-your-love-language</t>
         </is>
       </c>
       <c r="C231" s="13" t="inlineStr">
@@ -6199,7 +6199,7 @@
       </c>
       <c r="D231" s="4" t="inlineStr">
         <is>
-          <t>"The Peptide Clarity Index™." A real, evidence-cited 10-question assessment across 7 clinical axes, mapping to 16 real peptide archetype profiles — every question (with its real PubMed/journal citation), every profile's real primary/secondary peptides with mechanisms and evidence, suggested lab work, red flags, and stacking notes ported unchanged and verbatim (clinical-adjacent content, not paraphrased). The real Peptide Readiness Score, contraindication-flag screening, share buttons (Twitter/LinkedIn/email/copy — real, backend-free), and the real medical disclaimer are all preserved. Real hero image (CloudFront, confirmed live) kept via next/image. Reused the simplified AssessmentResultActions (PDF-only) built for /find-your-spirit. Same light-text-on-light-background contrast bug already caught elsewhere was fixed here too. Verified live: 200 OK, redirect confirmed 308, typecheck/lint clean.</t>
+          <t>Real 15 questions (incl. the negative-score "disconnect" question), 5 real archetypes with descriptions/tips, and Dr. Gary Chapman's real attribution note all ported unchanged. Verified live: 200 OK, full quiz flow, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E231" s="14" t="inlineStr">
@@ -6212,7 +6212,7 @@
       <c r="A232" s="4" t="n"/>
       <c r="B232" s="4" t="inlineStr">
         <is>
-          <t>/find-your-sexuality (+ /find-my-sexuality)</t>
+          <t>/find-your-peptide (+ /find-my-peptide)</t>
         </is>
       </c>
       <c r="C232" s="13" t="inlineStr">
@@ -6222,7 +6222,7 @@
       </c>
       <c r="D232" s="4" t="inlineStr">
         <is>
-          <t>A research-informed assessment across 6 real dimensions, grounded in real cited research (Klein Sexual Orientation Grid 1978, Kinsey Scale 1948, Lisa Diamond 2008, Sari van Anders 2015) — real 16 questions (with per-question research context notes), real 12 archetypes (each with a real description + research note), and the real scoring/selection logic all ported unchanged and verbatim, including the real closing disclaimer. Legacy's own AssessmentIntro stats prop claimed "20 questions, 7 dimensions" — didn't match the real 16/6 implementation, used the live counts instead. Legacy's results screen also used light grey text on the real light pastel theme background (same low-contrast bug already caught on /find-your-style) — normalized to dark ink. Verified live: 200 OK, redirect confirmed 308, typecheck/lint clean.</t>
+          <t>"The Peptide Clarity Index™." A real, evidence-cited 10-question assessment across 7 clinical axes, mapping to 16 real peptide archetype profiles — every question (with its real PubMed/journal citation), every profile's real primary/secondary peptides with mechanisms and evidence, suggested lab work, red flags, and stacking notes ported unchanged and verbatim (clinical-adjacent content, not paraphrased). The real Peptide Readiness Score, contraindication-flag screening, share buttons (Twitter/LinkedIn/email/copy — real, backend-free), and the real medical disclaimer are all preserved. Real hero image (CloudFront, confirmed live) kept via next/image. Reused the simplified AssessmentResultActions (PDF-only) built for /find-your-spirit. Same light-text-on-light-background contrast bug already caught elsewhere was fixed here too. Verified live: 200 OK, redirect confirmed 308, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E232" s="14" t="inlineStr">
@@ -6235,7 +6235,7 @@
       <c r="A233" s="4" t="n"/>
       <c r="B233" s="4" t="inlineStr">
         <is>
-          <t>/find-my</t>
+          <t>/find-your-sexuality (+ /find-my-sexuality)</t>
         </is>
       </c>
       <c r="C233" s="13" t="inlineStr">
@@ -6245,7 +6245,7 @@
       </c>
       <c r="D233" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Find What's Yours," the real destination of the homepage's "Diagnose" door (confirmed by grepping lib/content/home-doors.ts's /find-my href) and of whats-next.tsx's "Take Another Assessment" link, both already pointing here as forward-references before this page existed. Legacy's 26-item ALL_LINKS directory (Featured + 6 categories) ported unchanged and verbatim into lib/content/find-my-directory.ts. Real accuracy fix, same pattern as /find-your-me's own port note: cross-checked all 26 destinations against the real route list — /find-your-ev, /life-assessment, and /soulscore (at the time) didn't exist yet, rendered as real "Coming Soon" cards instead of links that would 404 (dharma-finder/consciousness-scale/grant-study have since shipped and now flip to live — see below). Real reuse, not re-derivation: every item whose destination already exists in find-your-me.ts's audited DIRECTORY pulls that entry's real hook text and status at build time via a lookup helper, instead of hand-copying a second, driftable copy of the same facts. Two real live destinations added that legacy linked but find-your-me.ts's directory didn't track: /brewsoul (confirmed 200) and the external findmystem-s3lknc4h.manus.space sibling tool (confirmed live), both using the same "real external sibling product" trust already established for the other manus.space tools. Legacy's dead Manus hero image dropped for ThemedBackground (theme="ecosystem"), same call as /find-your-me. AssessmentProgressBar (never </t>
+          <t>A research-informed assessment across 6 real dimensions, grounded in real cited research (Klein Sexual Orientation Grid 1978, Kinsey Scale 1948, Lisa Diamond 2008, Sari van Anders 2015) — real 16 questions (with per-question research context notes), real 12 archetypes (each with a real description + research note), and the real scoring/selection logic all ported unchanged and verbatim, including the real closing disclaimer. Legacy's own AssessmentIntro stats prop claimed "20 questions, 7 dimensions" — didn't match the real 16/6 implementation, used the live counts instead. Legacy's results screen also used light grey text on the real light pastel theme background (same low-contrast bug already caught on /find-your-style) — normalized to dark ink. Verified live: 200 OK, redirect confirmed 308, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E233" s="14" t="inlineStr">
@@ -6258,7 +6258,7 @@
       <c r="A234" s="4" t="n"/>
       <c r="B234" s="4" t="inlineStr">
         <is>
-          <t>/assessments</t>
+          <t>/find-my</t>
         </is>
       </c>
       <c r="C234" s="13" t="inlineStr">
@@ -6268,7 +6268,7 @@
       </c>
       <c r="D234" s="4" t="inlineStr">
         <is>
-          <t>"Three Maps. One Journey," confirmed genuinely distinct from /find-my rather than a duplicate: /find-my is the wide 26-item ecosystem directory, /assessments is its own page for exactly 3 long research-grounded instruments (Dharma Finder / Consciousness Scale / Grant Study) that also happen to appear as one category inside /find-my's directory — legacy kept these as two separate pages, so the port does too. Real title/subtitle/description/time/icon/accent content for all 3 instruments ported unchanged and verbatim into lib/content/assessments-hub.ts, including the full "Why These Three" closing essay (Schmachtenberger/Hawkins/Harvard Grant Study triangulation). All 3 instrument cards now link live (dharma-finder/consciousness-scale/grant-study shipped alongside this page). Legacy's footer claim "Results saved for your return" was dropped — replaced with an honest line since nothing persists results yet. Added a real cross-link to /find-my. JourneyTracker reused unchanged; no EmailGate/AssessmentResultActions — pure preview/hub page with no quiz or results step of its own. Verified live: 200 OK, exactly 1 header/footer, real content in all 3 cards, typecheck/lint clean.</t>
+          <t xml:space="preserve">"Find What's Yours," the real destination of the homepage's "Diagnose" door (confirmed by grepping lib/content/home-doors.ts's /find-my href) and of whats-next.tsx's "Take Another Assessment" link, both already pointing here as forward-references before this page existed. Legacy's 26-item ALL_LINKS directory (Featured + 6 categories) ported unchanged and verbatim into lib/content/find-my-directory.ts. Real accuracy fix, same pattern as /find-your-me's own port note: cross-checked all 26 destinations against the real route list — /find-your-ev, /life-assessment, and /soulscore (at the time) didn't exist yet, rendered as real "Coming Soon" cards instead of links that would 404 (dharma-finder/consciousness-scale/grant-study have since shipped and now flip to live — see below). Real reuse, not re-derivation: every item whose destination already exists in find-your-me.ts's audited DIRECTORY pulls that entry's real hook text and status at build time via a lookup helper, instead of hand-copying a second, driftable copy of the same facts. Two real live destinations added that legacy linked but find-your-me.ts's directory didn't track: /brewsoul (confirmed 200) and the external findmystem-s3lknc4h.manus.space sibling tool (confirmed live), both using the same "real external sibling product" trust already established for the other manus.space tools. Legacy's dead Manus hero image dropped for ThemedBackground (theme="ecosystem"), same call as /find-your-me. AssessmentProgressBar (never </t>
         </is>
       </c>
       <c r="E234" s="14" t="inlineStr">
@@ -6281,7 +6281,7 @@
       <c r="A235" s="4" t="n"/>
       <c r="B235" s="4" t="inlineStr">
         <is>
-          <t>/dharma-finder (+ /assessments/dharma-finder redirect). Structurally different from every other Phase 9 quiz</t>
+          <t>/assessments</t>
         </is>
       </c>
       <c r="C235" s="13" t="inlineStr">
@@ -6291,7 +6291,7 @@
       </c>
       <c r="D235" s="4" t="inlineStr">
         <is>
-          <t>legacy's real 25 questions are open-text reflection prompts, not multiple choice, distilled from Daniel Schmachtenberger's Dharma Inquiry and grouped into 4 real sections (Capacities/Values/Propensities/The Shadow Inquiry), each with a real framing quote, plus 3 real interstitial quotes shown between sections with the original 4-second auto-advance. All 25 questions, all quotes, and legacy's own keyword-matching generateDharmaProfile (deriving up to 3 archetypal roles and up to 4 core values from free-text answers, plus a completion-depth percentage) are ported unchanged and verbatim into a new dharma-finder-quiz.tsx. Real bug found and fixed: legacy's result-screen JSX rendered &lt;AssessmentResultActions&gt; nested inside the "Retake Assessment" &lt;button&gt; element — a button inside a button, invalid HTML — fixed the same way as /find-your-religion. Real dead-link bug fixed: "Journey Continues" linked to /assessments/consciousness-scale (repointed to the real /consciousness-scale) and /assessments/grant-study (dropped at the time, now live too). EmailGate (new here; legacy had none) is a real ecosystem-consistency addition. find-your-me.ts's ecosystem-directory status flipped from "coming" to "live" now that this page ships. Verified live: 200 OK, typecheck/lint clean.</t>
+          <t>"Three Maps. One Journey," confirmed genuinely distinct from /find-my rather than a duplicate: /find-my is the wide 26-item ecosystem directory, /assessments is its own page for exactly 3 long research-grounded instruments (Dharma Finder / Consciousness Scale / Grant Study) that also happen to appear as one category inside /find-my's directory — legacy kept these as two separate pages, so the port does too. Real title/subtitle/description/time/icon/accent content for all 3 instruments ported unchanged and verbatim into lib/content/assessments-hub.ts, including the full "Why These Three" closing essay (Schmachtenberger/Hawkins/Harvard Grant Study triangulation). All 3 instrument cards now link live (dharma-finder/consciousness-scale/grant-study shipped alongside this page). Legacy's footer claim "Results saved for your return" was dropped — replaced with an honest line since nothing persists results yet. Added a real cross-link to /find-my. JourneyTracker reused unchanged; no EmailGate/AssessmentResultActions — pure preview/hub page with no quiz or results step of its own. Verified live: 200 OK, exactly 1 header/footer, real content in all 3 cards, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E235" s="14" t="inlineStr">
@@ -6304,7 +6304,7 @@
       <c r="A236" s="4" t="n"/>
       <c r="B236" s="4" t="inlineStr">
         <is>
-          <t>/consciousness-scale (+ /assessments/consciousness-scale redirect)</t>
+          <t>/dharma-finder (+ /assessments/dharma-finder redirect). Structurally different from every other Phase 9 quiz</t>
         </is>
       </c>
       <c r="C236" s="13" t="inlineStr">
@@ -6314,7 +6314,7 @@
       </c>
       <c r="D236" s="4" t="inlineStr">
         <is>
-          <t>Real 25 questions, each scored against David R. Hawkins' real 17-level Map of Consciousness (Shame 20 through Enlightenment 700+, final score = average of all 25 answers) — every question/option, every level's name/emotion/threshold, and getInsight's exact 6 tiers of interpretive copy ported unchanged and verbatim into a new consciousness-scale-quiz.tsx, along with the real live running-average indicator, visual scale gauge, full 17-level map, 6-month reminder, and X/LinkedIn/copy share. Since this assessment produces one composite score on a single axis rather than independent dimensions, a bespoke single-axis gauge replaces AssessmentRadarChart; per-level colors (17 known-at-build-time values) are precomposed literal Tailwind classes rather than assembled from hex fragments. Real Manus-dependency bug found and fixed: legacy's cinematic Q1 hero used a /api/img/consciousness-scale-hero-v2_085e0746.jpg Manus-proxied image — forbidden even temporarily per this migration's Zero-Manus rule — dropped for the plain question-card layout every other assessment uses; a real Sanity-hosted replacement is a tracked follow-up (see BLOG-IMAGE-BRIEFS.md-style tracking). find-your-me.ts's ecosystem-directory status flipped from "coming" to "live" now that this page ships. Verified live: 200 OK, typecheck/lint clean.</t>
+          <t>legacy's real 25 questions are open-text reflection prompts, not multiple choice, distilled from Daniel Schmachtenberger's Dharma Inquiry and grouped into 4 real sections (Capacities/Values/Propensities/The Shadow Inquiry), each with a real framing quote, plus 3 real interstitial quotes shown between sections with the original 4-second auto-advance. All 25 questions, all quotes, and legacy's own keyword-matching generateDharmaProfile (deriving up to 3 archetypal roles and up to 4 core values from free-text answers, plus a completion-depth percentage) are ported unchanged and verbatim into a new dharma-finder-quiz.tsx. Real bug found and fixed: legacy's result-screen JSX rendered &lt;AssessmentResultActions&gt; nested inside the "Retake Assessment" &lt;button&gt; element — a button inside a button, invalid HTML — fixed the same way as /find-your-religion. Real dead-link bug fixed: "Journey Continues" linked to /assessments/consciousness-scale (repointed to the real /consciousness-scale) and /assessments/grant-study (dropped at the time, now live too). EmailGate (new here; legacy had none) is a real ecosystem-consistency addition. find-your-me.ts's ecosystem-directory status flipped from "coming" to "live" now that this page ships. Verified live: 200 OK, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E236" s="14" t="inlineStr">
@@ -6327,7 +6327,7 @@
       <c r="A237" s="4" t="n"/>
       <c r="B237" s="4" t="inlineStr">
         <is>
-          <t>/grant-study (+ /assessments/grant-study redirect)</t>
+          <t>/consciousness-scale (+ /assessments/consciousness-scale redirect)</t>
         </is>
       </c>
       <c r="C237" s="13" t="inlineStr">
@@ -6337,7 +6337,7 @@
       </c>
       <c r="D237" s="4" t="inlineStr">
         <is>
-          <t>"Find Your Score," the real 25-question (5 per factor), 5-factor Harvard Grant Study life-satisfaction assessment (724 men, 1938–present, 85+ years — the longest-running study of human happiness). Every question, the 5 real factors (Warm Relationships/Adaptive Coping/Generativity/Career Satisfaction/Physical Vitality), every per-factor/per-tier insight (real named findings — Vaillant's "mature defenses," Erikson's generativity, Waldinger's quote), and the closing "Tony's Note" (Vaillant's "Happiness is love. Full stop." + Waldinger's "good relationships keep us happier and healthier") all ported unchanged and verbatim. Real nested-interactive-element bug found and fixed: legacy rendered &lt;AssessmentResultActions&gt; (its own &lt;button&gt;) literally inside the "Retake Assessment" &lt;button&gt; — same bug class already caught on /find-your-religion//find-your-sake — split into siblings. Real dead-link fix: "Journey Continues" pointed "Find Your Spirit" at a dead external Manus stub despite the real internal /find-your-spirit existing — repointed. Real ecosystem-consistency normalization: unlike every sibling "Find Your X" quiz, legacy skipped EmailGate entirely and went straight to results — added for consistency, plus new find-your-grant-study/find-your-dharma-finder/find-your-consciousness-scale alias keys in kit-source-tags.ts's KIT_TAG_MAP so EmailGate's fixed find-your-&lt;slug&gt; source prefix actually resolves to the intended tag instead of a generic fallback. resultSlug="grant-study" pas</t>
+          <t>Real 25 questions, each scored against David R. Hawkins' real 17-level Map of Consciousness (Shame 20 through Enlightenment 700+, final score = average of all 25 answers) — every question/option, every level's name/emotion/threshold, and getInsight's exact 6 tiers of interpretive copy ported unchanged and verbatim into a new consciousness-scale-quiz.tsx, along with the real live running-average indicator, visual scale gauge, full 17-level map, 6-month reminder, and X/LinkedIn/copy share. Since this assessment produces one composite score on a single axis rather than independent dimensions, a bespoke single-axis gauge replaces AssessmentRadarChart; per-level colors (17 known-at-build-time values) are precomposed literal Tailwind classes rather than assembled from hex fragments. Real Manus-dependency bug found and fixed: legacy's cinematic Q1 hero used a /api/img/consciousness-scale-hero-v2_085e0746.jpg Manus-proxied image — forbidden even temporarily per this migration's Zero-Manus rule — dropped for the plain question-card layout every other assessment uses; a real Sanity-hosted replacement is a tracked follow-up (see BLOG-IMAGE-BRIEFS.md-style tracking). find-your-me.ts's ecosystem-directory status flipped from "coming" to "live" now that this page ships. Verified live: 200 OK, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E237" s="14" t="inlineStr">
@@ -6350,7 +6350,7 @@
       <c r="A238" s="4" t="n"/>
       <c r="B238" s="4" t="inlineStr">
         <is>
-          <t>/soulscore</t>
+          <t>/grant-study (+ /assessments/grant-study redirect)</t>
         </is>
       </c>
       <c r="C238" s="13" t="inlineStr">
@@ -6360,7 +6360,7 @@
       </c>
       <c r="D238" s="4" t="inlineStr">
         <is>
-          <t>SoulScore™, ImpactSoul's 12-dimension impact measurement engine (1231-line legacy file, the largest remaining port). Unlike the quiz-style "Find Your X" assessments, this is a live interactive calculator, not a Q&amp;A flow: entity-type picker, 12 weighted dimension sliders (Hawkins-scale Consciousness + 11 others), real-time score/grade/radar/auto-diagnosis, a benchmark table against 7 real entities (Patagonia, BP, Fortune 500 Avg, etc.), a 6-tier/30-factor supply chain drill-down, 20 "why every impact system failed" entries, a real Consciousness-Adjusted NPV calculator, and the gig-economy 5-layer stack comparison — all real content/formulas ported verbatim. Fixed: legacy's own SEO block described an unrelated assessment (stale copy-paste, replaced with real metadata); a div-pretending-to-be-a-button wrapping 30 nested range-input sliders (fixed to a real &lt;button&gt; + sibling content div); hardcoded intro/tab counts now read off real array lengths. No EmailGate (legacy never had one here — it's an open calculator, not a report unlock), matching /find-your-peptide's precedent. AssessmentResultActions wired with resultSlug="soulscore". journey-tracker.tsx's JOURNEY_MAP and /impact-dashboard's "Launch SoulScore Engine"/"Launch C-NPV Calculator" links (previously a disabled "Coming Soon" note) now point at the real page. This closes the real dead-end referenced from site-nav-data.ts (/soulscore appears twice in nav) and from /impact-dashboard — the last item in the STATUS.md dead-end</t>
+          <t>"Find Your Score," the real 25-question (5 per factor), 5-factor Harvard Grant Study life-satisfaction assessment (724 men, 1938–present, 85+ years — the longest-running study of human happiness). Every question, the 5 real factors (Warm Relationships/Adaptive Coping/Generativity/Career Satisfaction/Physical Vitality), every per-factor/per-tier insight (real named findings — Vaillant's "mature defenses," Erikson's generativity, Waldinger's quote), and the closing "Tony's Note" (Vaillant's "Happiness is love. Full stop." + Waldinger's "good relationships keep us happier and healthier") all ported unchanged and verbatim. Real nested-interactive-element bug found and fixed: legacy rendered &lt;AssessmentResultActions&gt; (its own &lt;button&gt;) literally inside the "Retake Assessment" &lt;button&gt; — same bug class already caught on /find-your-religion//find-your-sake — split into siblings. Real dead-link fix: "Journey Continues" pointed "Find Your Spirit" at a dead external Manus stub despite the real internal /find-your-spirit existing — repointed. Real ecosystem-consistency normalization: unlike every sibling "Find Your X" quiz, legacy skipped EmailGate entirely and went straight to results — added for consistency, plus new find-your-grant-study/find-your-dharma-finder/find-your-consciousness-scale alias keys in kit-source-tags.ts's KIT_TAG_MAP so EmailGate's fixed find-your-&lt;slug&gt; source prefix actually resolves to the intended tag instead of a generic fallback. resultSlug="grant-study" pas</t>
         </is>
       </c>
       <c r="E238" s="14" t="inlineStr">
@@ -6373,7 +6373,7 @@
       <c r="A239" s="4" t="n"/>
       <c r="B239" s="4" t="inlineStr">
         <is>
-          <t>/self-portrait</t>
+          <t>/soulscore</t>
         </is>
       </c>
       <c r="C239" s="13" t="inlineStr">
@@ -6383,7 +6383,7 @@
       </c>
       <c r="D239" s="4" t="inlineStr">
         <is>
-          <t>composite of completed assessments. Decision made: local-only (a real cookie, not Supabase — Phase 2 isn't provisioned yet). AssessmentResultActions (components/assessments/result-actions.tsx) takes an optional resultSlug and logs completions to a tg_assessment_results cookie via lib/assessments/result-log.ts, the same real-cookie-read-via-next/headers pattern already established by returning-visitor-hero.tsx/track-last-blog-visit.tsx — the page itself is a Server Component reading that cookie with zero client hydration step. Real, deliberate scope cut, not a silent one: legacy's SelfPortrait.tsx combined each assessment's own per-dimension scores (16 separate localStorage keys) into one composite radar chart across 15 unified dimensions, gated behind "5+ completed." This migration's result log only ever records that an assessment was completed, not its actual scored answers — building the real composite radar would mean threading a second, much larger data channel through every quiz. Shipped the honest subset instead: a real completed-assessments list (title, real completion date, retake link) plus a real "X of N completed" count and a "Still to Explore" section for the rest, via a new lib/content/self-portrait-catalog.ts. Wired resultSlug into the 7 remaining older "Find Your X" quizzes that already call AssessmentResultActions but hadn't been threaded yet (spirit/therapy/religion/sake/coffee/peptide/me) — /self-portrait now tracks 13 real assessments total. /find-my's "Sel</t>
+          <t>SoulScore™, ImpactSoul's 12-dimension impact measurement engine (1231-line legacy file, the largest remaining port). Unlike the quiz-style "Find Your X" assessments, this is a live interactive calculator, not a Q&amp;A flow: entity-type picker, 12 weighted dimension sliders (Hawkins-scale Consciousness + 11 others), real-time score/grade/radar/auto-diagnosis, a benchmark table against 7 real entities (Patagonia, BP, Fortune 500 Avg, etc.), a 6-tier/30-factor supply chain drill-down, 20 "why every impact system failed" entries, a real Consciousness-Adjusted NPV calculator, and the gig-economy 5-layer stack comparison — all real content/formulas ported verbatim. Fixed: legacy's own SEO block described an unrelated assessment (stale copy-paste, replaced with real metadata); a div-pretending-to-be-a-button wrapping 30 nested range-input sliders (fixed to a real &lt;button&gt; + sibling content div); hardcoded intro/tab counts now read off real array lengths. No EmailGate (legacy never had one here — it's an open calculator, not a report unlock), matching /find-your-peptide's precedent. AssessmentResultActions wired with resultSlug="soulscore". journey-tracker.tsx's JOURNEY_MAP and /impact-dashboard's "Launch SoulScore Engine"/"Launch C-NPV Calculator" links (previously a disabled "Coming Soon" note) now point at the real page. This closes the real dead-end referenced from site-nav-data.ts (/soulscore appears twice in nav) and from /impact-dashboard — the last item in the STATUS.md dead-end</t>
         </is>
       </c>
       <c r="E239" s="14" t="inlineStr">
@@ -6396,7 +6396,7 @@
       <c r="A240" s="4" t="n"/>
       <c r="B240" s="4" t="inlineStr">
         <is>
-          <t>/the-mirror (+ /life-assessment)</t>
+          <t>/self-portrait</t>
         </is>
       </c>
       <c r="C240" s="13" t="inlineStr">
@@ -6406,7 +6406,7 @@
       </c>
       <c r="D240" s="4" t="inlineStr">
         <is>
-          <t>uses mirrorData.json, real 6-dimension/18-question life assessment ("The Mirror") ported into a typed lib/content/mirror-data.ts. Legacy served the identical component at both paths; /the-mirror is canonical (it's the only URL every existing internal link already pointed to — nav, journey tracker, Find Your Me), /life-assessment permanently redirects there. Real dimension-averaged scoring, radar chart via the shared AssessmentRadarChart, and weakest-dimension article/satellite-site recommendations ported unchanged. A live Sanity check found only 27 of 85 legacy article slugs still resolve; recommendations now resolve server-side and defensively skip missing ones, matching legacy's own behavior. Fixed: a hydration-unsafe typeof window branch computing the share URL, three stale manus.space satellite URLs superseded by their current live counterparts already used elsewhere in this migration, and dead /assessments/*/external-stub links in the "Journey Continues" grid. Added find-your-mirror to kit-source-tags.ts's KIT_TAG_MAP and reconciled journey-tracker.tsx's stale 10-minute estimate to legacy's real "~4 minutes" claim. find-your-me.ts's ecosystem-directory status flipped to "live." Verified live: 200 OK on both paths, redirect confirmed, typecheck/lint clean.</t>
+          <t>composite of completed assessments. Decision made: local-only (a real cookie, not Supabase — Phase 2 isn't provisioned yet). AssessmentResultActions (components/assessments/result-actions.tsx) takes an optional resultSlug and logs completions to a tg_assessment_results cookie via lib/assessments/result-log.ts, the same real-cookie-read-via-next/headers pattern already established by returning-visitor-hero.tsx/track-last-blog-visit.tsx — the page itself is a Server Component reading that cookie with zero client hydration step. Real, deliberate scope cut, not a silent one: legacy's SelfPortrait.tsx combined each assessment's own per-dimension scores (16 separate localStorage keys) into one composite radar chart across 15 unified dimensions, gated behind "5+ completed." This migration's result log only ever records that an assessment was completed, not its actual scored answers — building the real composite radar would mean threading a second, much larger data channel through every quiz. Shipped the honest subset instead: a real completed-assessments list (title, real completion date, retake link) plus a real "X of N completed" count and a "Still to Explore" section for the rest, via a new lib/content/self-portrait-catalog.ts. Wired resultSlug into the 7 remaining older "Find Your X" quizzes that already call AssessmentResultActions but hadn't been threaded yet (spirit/therapy/religion/sake/coffee/peptide/me) — /self-portrait now tracks 13 real assessments total. /find-my's "Sel</t>
         </is>
       </c>
       <c r="E240" s="14" t="inlineStr">
@@ -6419,7 +6419,7 @@
       <c r="A241" s="4" t="n"/>
       <c r="B241" s="4" t="inlineStr">
         <is>
-          <t>/assessment</t>
+          <t>/the-mirror (+ /life-assessment)</t>
         </is>
       </c>
       <c r="C241" s="13" t="inlineStr">
@@ -6429,7 +6429,7 @@
       </c>
       <c r="D241" s="4" t="inlineStr">
         <is>
-          <t>confirmed via full legacy read this is not a "Find Your X" quiz (it predates that convention): it's Tony's own 3-way reader-path diagnostic — Builder / Crusader / Investor — 5 real questions, one point per matching answer, highest tally wins. Real questions and real archetype copy ported unchanged, reused from lib/content/archetypes.ts (already ported for /essays's archetype filter) rather than duplicated — added the page's ASSESSMENT_QUESTIONS to that same module since both come from the identical legacy source file. Preserved the real, distinct UX (no landing screen, no ThemedBackground/JourneyTracker — this page sits outside that ecosystem). Real bugs fixed: JS onMouseEnter/onMouseLeave inline-style hover hack replaced with Tailwind hover: classes; literal "..." pending-state text replaced with a real Loader2 spinner per house rule; dead trpc.subscribe.add replaced with a real POST /api/subscribe call. Real link audit: kept /impact-dashboard, /find-your-me, /living-declaration, and the real /blog/boiling-the-human-summit-harvard-kurzweil article as live links; /soulscore and /humanos are established forward-references used repeatedly elsewhere in this migration and both now ship too. The Human OS CTA reuses the border-red-800/30 text-red-800 treatment /living-declaration already established for the identical button instead of a new one-off raw-hex pair. AssessmentResultActions resultSlug="assessment" added (didn't exist when legacy was written). Added assessment-builder/as</t>
+          <t>uses mirrorData.json, real 6-dimension/18-question life assessment ("The Mirror") ported into a typed lib/content/mirror-data.ts. Legacy served the identical component at both paths; /the-mirror is canonical (it's the only URL every existing internal link already pointed to — nav, journey tracker, Find Your Me), /life-assessment permanently redirects there. Real dimension-averaged scoring, radar chart via the shared AssessmentRadarChart, and weakest-dimension article/satellite-site recommendations ported unchanged. A live Sanity check found only 27 of 85 legacy article slugs still resolve; recommendations now resolve server-side and defensively skip missing ones, matching legacy's own behavior. Fixed: a hydration-unsafe typeof window branch computing the share URL, three stale manus.space satellite URLs superseded by their current live counterparts already used elsewhere in this migration, and dead /assessments/*/external-stub links in the "Journey Continues" grid. Added find-your-mirror to kit-source-tags.ts's KIT_TAG_MAP and reconciled journey-tracker.tsx's stale 10-minute estimate to legacy's real "~4 minutes" claim. find-your-me.ts's ecosystem-directory status flipped to "live." Verified live: 200 OK on both paths, redirect confirmed, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E241" s="14" t="inlineStr">
@@ -6442,7 +6442,7 @@
       <c r="A242" s="4" t="n"/>
       <c r="B242" s="4" t="inlineStr">
         <is>
-          <t>Fix dead-end pages flagged in STATUS.md</t>
+          <t>/assessment</t>
         </is>
       </c>
       <c r="C242" s="13" t="inlineStr">
@@ -6452,7 +6452,7 @@
       </c>
       <c r="D242" s="4" t="inlineStr">
         <is>
-          <t>sake, therapy, and love-language all got real next-step navigation (WhatsNext + real "Journey Continues" links) during their ports — the last remaining one, soulscore, is now built (see above), closing this out.</t>
+          <t>confirmed via full legacy read this is not a "Find Your X" quiz (it predates that convention): it's Tony's own 3-way reader-path diagnostic — Builder / Crusader / Investor — 5 real questions, one point per matching answer, highest tally wins. Real questions and real archetype copy ported unchanged, reused from lib/content/archetypes.ts (already ported for /essays's archetype filter) rather than duplicated — added the page's ASSESSMENT_QUESTIONS to that same module since both come from the identical legacy source file. Preserved the real, distinct UX (no landing screen, no ThemedBackground/JourneyTracker — this page sits outside that ecosystem). Real bugs fixed: JS onMouseEnter/onMouseLeave inline-style hover hack replaced with Tailwind hover: classes; literal "..." pending-state text replaced with a real Loader2 spinner per house rule; dead trpc.subscribe.add replaced with a real POST /api/subscribe call. Real link audit: kept /impact-dashboard, /find-your-me, /living-declaration, and the real /blog/boiling-the-human-summit-harvard-kurzweil article as live links; /soulscore and /humanos are established forward-references used repeatedly elsewhere in this migration and both now ship too. The Human OS CTA reuses the border-red-800/30 text-red-800 treatment /living-declaration already established for the identical button instead of a new one-off raw-hex pair. AssessmentResultActions resultSlug="assessment" added (didn't exist when legacy was written). Added assessment-builder/as</t>
         </is>
       </c>
       <c r="E242" s="14" t="inlineStr">
@@ -6465,63 +6465,63 @@
       <c r="A243" s="4" t="n"/>
       <c r="B243" s="4" t="inlineStr">
         <is>
+          <t>Fix dead-end pages flagged in STATUS.md</t>
+        </is>
+      </c>
+      <c r="C243" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D243" s="4" t="inlineStr">
+        <is>
+          <t>sake, therapy, and love-language all got real next-step navigation (WhatsNext + real "Journey Continues" links) during their ports — the last remaining one, soulscore, is now built (see above), closing this out.</t>
+        </is>
+      </c>
+      <c r="E243" s="14" t="inlineStr">
+        <is>
+          <t>Phase 9 — Assessments (33 routes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="4" t="n"/>
+      <c r="B244" s="4" t="inlineStr">
+        <is>
           <t>Port shared radar-chart / PDF-export / email-gate components used across assessments</t>
         </is>
       </c>
-      <c r="C243" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D243" s="4" t="inlineStr">
+      <c r="C244" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D244" s="4" t="inlineStr">
         <is>
           <t>components/assessments/{radar-chart,result-actions,email-gate}.tsx, built during Phase 9 and reused unchanged by all 15 "Find Your X" quizzes plus /find-your-me.</t>
         </is>
       </c>
-      <c r="E243" s="14" t="inlineStr">
+      <c r="E244" s="14" t="inlineStr">
         <is>
           <t>Phase 9 — Assessments (33 routes)</t>
         </is>
       </c>
     </row>
-    <row r="244">
-      <c r="A244" s="10" t="inlineStr">
+    <row r="245">
+      <c r="A245" s="10" t="inlineStr">
         <is>
           <t>Phase 11 — Code MCP Server — REBUILT (2026-09-29)</t>
         </is>
       </c>
-      <c r="B244" s="11" t="n"/>
-      <c r="C244" s="11" t="n"/>
-      <c r="D244" s="12" t="n"/>
-    </row>
-    <row r="245">
-      <c r="A245" s="4" t="n"/>
-      <c r="B245" s="4" t="inlineStr">
-        <is>
-          <t>src/lib/admin/</t>
-        </is>
-      </c>
-      <c r="C245" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D245" s="4" t="inlineStr">
-        <is>
-          <t>guardrails (fixes the removed version's proxy.ts pattern, which missed the real src/proxy.ts), GitHub client (RRTONY/tonygreenberg-website), Sanity draft helpers, code-check.ts (ESLint + CONTRIBUTING.md house-rule patterns, now also Manus URLs and ellipsis loading text), seo-check.ts, tools.ts, mcp-server.ts, mcp-handler.ts, mcp-tool-context.ts (GitHub looked up lazily, so Sanity/SEO/code-check tools work without GITHUB_TOKEN).</t>
-        </is>
-      </c>
-      <c r="E245" s="14" t="inlineStr">
-        <is>
-          <t>Phase 11 — Code MCP Server — REBUILT (2026-09-29)</t>
-        </is>
-      </c>
+      <c r="B245" s="11" t="n"/>
+      <c r="C245" s="11" t="n"/>
+      <c r="D245" s="12" t="n"/>
     </row>
     <row r="246">
       <c r="A246" s="4" t="n"/>
       <c r="B246" s="4" t="inlineStr">
         <is>
-          <t>Per-person access via MCP_ADMIN_USERS (read/edit/write roles, tools filtered per role, calls logged, commits stamped [by &lt;name&gt;])</t>
+          <t>src/lib/admin/</t>
         </is>
       </c>
       <c r="C246" s="13" t="inlineStr">
@@ -6531,7 +6531,7 @@
       </c>
       <c r="D246" s="4" t="inlineStr">
         <is>
-          <t>mcp-auth.ts.</t>
+          <t>guardrails (fixes the removed version's proxy.ts pattern, which missed the real src/proxy.ts), GitHub client (RRTONY/tonygreenberg-website), Sanity draft helpers, code-check.ts (ESLint + CONTRIBUTING.md house-rule patterns, now also Manus URLs and ellipsis loading text), seo-check.ts, tools.ts, mcp-server.ts, mcp-handler.ts, mcp-tool-context.ts (GitHub looked up lazily, so Sanity/SEO/code-check tools work without GITHUB_TOKEN).</t>
         </is>
       </c>
       <c r="E246" s="14" t="inlineStr">
@@ -6544,7 +6544,7 @@
       <c r="A247" s="4" t="n"/>
       <c r="B247" s="4" t="inlineStr">
         <is>
-          <t>Rules gate: get_project_rules serves CONTRIBUTING.md + AGENTS.md + docs/ai/ guides with a rulesVersion; all 6 write tools require it</t>
+          <t>Per-person access via MCP_ADMIN_USERS (read/edit/write roles, tools filtered per role, calls logged, commits stamped [by &lt;name&gt;])</t>
         </is>
       </c>
       <c r="C247" s="13" t="inlineStr">
@@ -6554,7 +6554,7 @@
       </c>
       <c r="D247" s="4" t="inlineStr">
         <is>
-          <t>project-rules.ts.</t>
+          <t>mcp-auth.ts.</t>
         </is>
       </c>
       <c r="E247" s="14" t="inlineStr">
@@ -6567,7 +6567,7 @@
       <c r="A248" s="4" t="n"/>
       <c r="B248" s="4" t="inlineStr">
         <is>
-          <t>src/app/api/mcp/route.ts (header auth) + src/app/api/mcp/[token]/route.ts (token in URL).</t>
+          <t>Rules gate: get_project_rules serves CONTRIBUTING.md + AGENTS.md + docs/ai/ guides with a rulesVersion; all 6 write tools require it</t>
         </is>
       </c>
       <c r="C248" s="13" t="inlineStr">
@@ -6575,7 +6575,11 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="D248" s="4" t="inlineStr"/>
+      <c r="D248" s="4" t="inlineStr">
+        <is>
+          <t>project-rules.ts.</t>
+        </is>
+      </c>
       <c r="E248" s="14" t="inlineStr">
         <is>
           <t>Phase 11 — Code MCP Server — REBUILT (2026-09-29)</t>
@@ -6586,7 +6590,7 @@
       <c r="A249" s="4" t="n"/>
       <c r="B249" s="4" t="inlineStr">
         <is>
-          <t>docs/ai/ knowledge base (README, TASK_GUIDE, PROJECT_STRUCTURE, project_mcp_server), linked from CONTRIBUTING.md.</t>
+          <t>src/app/api/mcp/route.ts (header auth) + src/app/api/mcp/[token]/route.ts (token in URL).</t>
         </is>
       </c>
       <c r="C249" s="13" t="inlineStr">
@@ -6605,7 +6609,7 @@
       <c r="A250" s="4" t="n"/>
       <c r="B250" s="4" t="inlineStr">
         <is>
-          <t>@modelcontextprotocol/sdk ^1.30.0 re-added (approved 2026-09-29); GITHUB_TOKEN/MCP_ADMIN_USERS/MCP_SITE_ORIGIN documented in .env.local.example.</t>
+          <t>docs/ai/ knowledge base (README, TASK_GUIDE, PROJECT_STRUCTURE, project_mcp_server), linked from CONTRIBUTING.md.</t>
         </is>
       </c>
       <c r="C250" s="13" t="inlineStr">
@@ -6624,7 +6628,7 @@
       <c r="A251" s="4" t="n"/>
       <c r="B251" s="4" t="inlineStr">
         <is>
-          <t>Verified locally</t>
+          <t>@modelcontextprotocol/sdk ^1.30.0 re-added (approved 2026-09-29); GITHUB_TOKEN/MCP_ADMIN_USERS/MCP_SITE_ORIGIN documented in .env.local.example.</t>
         </is>
       </c>
       <c r="C251" s="13" t="inlineStr">
@@ -6632,11 +6636,7 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="D251" s="4" t="inlineStr">
-        <is>
-          <t>auth (401/405), role filtering, rules-gate markers, token-in-URL route, code check, Sanity query, SEO check.</t>
-        </is>
-      </c>
+      <c r="D251" s="4" t="inlineStr"/>
       <c r="E251" s="14" t="inlineStr">
         <is>
           <t>Phase 11 — Code MCP Server — REBUILT (2026-09-29)</t>
@@ -6647,7 +6647,7 @@
       <c r="A252" s="4" t="n"/>
       <c r="B252" s="4" t="inlineStr">
         <is>
-          <t>Sign-in for the MCP server (OAuth 2.1, ported from ramprate-ui, 2026-09-30)</t>
+          <t>Verified locally</t>
         </is>
       </c>
       <c r="C252" s="13" t="inlineStr">
@@ -6657,7 +6657,7 @@
       </c>
       <c r="D252" s="4" t="inlineStr">
         <is>
-          <t>/oauth/authorize sign-in page + /.well-known metadata + register/authorize/token endpoints, stateless (signed tokens, no database), no new dependency. Verified end to end on a local production build. See docs/ai/project_mcp_server.md.</t>
+          <t>auth (401/405), role filtering, rules-gate markers, token-in-URL route, code check, Sanity query, SEO check.</t>
         </is>
       </c>
       <c r="E252" s="14" t="inlineStr">
@@ -6670,17 +6670,17 @@
       <c r="A253" s="4" t="n"/>
       <c r="B253" s="4" t="inlineStr">
         <is>
-          <t>Set GITHUB_TOKEN, MCP_ADMIN_USERS, MCP_LOGIN_PASSWORD, MCP_OAUTH_SECRET, MCP_SITE_ORIGIN, MCP_PUBLIC_ORIGIN in Netlify (done) (checked 2026-…</t>
-        </is>
-      </c>
-      <c r="C253" s="16" t="inlineStr">
-        <is>
-          <t>Remaining</t>
+          <t>Sign-in for the MCP server (OAuth 2.1, ported from ramprate-ui, 2026-09-30)</t>
+        </is>
+      </c>
+      <c r="C253" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D253" s="4" t="inlineStr">
         <is>
-          <t>10-07: all already set in Netlify). Left: connect Claude.ai to /api/mcp for real, and verify the GitHub flow end to end (branch → PR → deploy preview → publish_changes) against a real PR.</t>
+          <t>/oauth/authorize sign-in page + /.well-known metadata + register/authorize/token endpoints, stateless (signed tokens, no database), no new dependency. Verified end to end on a local production build. See docs/ai/project_mcp_server.md.</t>
         </is>
       </c>
       <c r="E253" s="14" t="inlineStr">
@@ -6693,7 +6693,7 @@
       <c r="A254" s="4" t="n"/>
       <c r="B254" s="4" t="inlineStr">
         <is>
-          <t>Commit a team-wide .mcp.json (URL only) once the production URL is settled.</t>
+          <t>Set GITHUB_TOKEN, MCP_ADMIN_USERS, MCP_LOGIN_PASSWORD, MCP_OAUTH_SECRET, MCP_SITE_ORIGIN, MCP_PUBLIC_ORIGIN in Netlify (done) (checked 2026-…</t>
         </is>
       </c>
       <c r="C254" s="16" t="inlineStr">
@@ -6701,7 +6701,11 @@
           <t>Remaining</t>
         </is>
       </c>
-      <c r="D254" s="4" t="inlineStr"/>
+      <c r="D254" s="4" t="inlineStr">
+        <is>
+          <t>10-07: all already set in Netlify). Left: connect Claude.ai to /api/mcp for real, and verify the GitHub flow end to end (branch → PR → deploy preview → publish_changes) against a real PR.</t>
+        </is>
+      </c>
       <c r="E254" s="14" t="inlineStr">
         <is>
           <t>Phase 11 — Code MCP Server — REBUILT (2026-09-29)</t>
@@ -6712,19 +6716,15 @@
       <c r="A255" s="4" t="n"/>
       <c r="B255" s="4" t="inlineStr">
         <is>
-          <t>Google read-only tools added (2026-10-02)</t>
-        </is>
-      </c>
-      <c r="C255" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D255" s="4" t="inlineStr">
-        <is>
-          <t>check_analytics (GA4), search_console_sites / _performance / _inspect_url / _sitemaps (list only, no submit or delete), lighthouse_check_page (PageSpeed Insights). New files google-auth.ts, ga4-client.ts, gsc-client.ts, lighthouse-check.ts; no new dependency. Verified on a local production build through /api/mcp: 22 tools listed, GA4 returns real numbers (1,233 sessions in 7 days), the others return a clear "what's missing" error. Env vars added to .env.local.example.</t>
-        </is>
-      </c>
+          <t>Commit a team-wide .mcp.json (URL only) once the production URL is settled.</t>
+        </is>
+      </c>
+      <c r="C255" s="16" t="inlineStr">
+        <is>
+          <t>Remaining</t>
+        </is>
+      </c>
+      <c r="D255" s="4" t="inlineStr"/>
       <c r="E255" s="14" t="inlineStr">
         <is>
           <t>Phase 11 — Code MCP Server — REBUILT (2026-09-29)</t>
@@ -6735,7 +6735,7 @@
       <c r="A256" s="4" t="n"/>
       <c r="B256" s="4" t="inlineStr">
         <is>
-          <t>publish_changes fixed (2026-10-02)</t>
+          <t>Google read-only tools added (2026-10-02)</t>
         </is>
       </c>
       <c r="C256" s="13" t="inlineStr">
@@ -6745,7 +6745,7 @@
       </c>
       <c r="D256" s="4" t="inlineStr">
         <is>
-          <t>it published every draft in Sanity (31 waiting for review today), so any one-line fix would have pushed them all live. Now it publishes only the drafts named in draft_ids; unknown ids are refused before anything happens (verified).</t>
+          <t>check_analytics (GA4), search_console_sites / _performance / _inspect_url / _sitemaps (list only, no submit or delete), lighthouse_check_page (PageSpeed Insights). New files google-auth.ts, ga4-client.ts, gsc-client.ts, lighthouse-check.ts; no new dependency. Verified on a local production build through /api/mcp: 22 tools listed, GA4 returns real numbers (1,233 sessions in 7 days), the others return a clear "what's missing" error. Env vars added to .env.local.example.</t>
         </is>
       </c>
       <c r="E256" s="14" t="inlineStr">
@@ -6758,7 +6758,7 @@
       <c r="A257" s="4" t="n"/>
       <c r="B257" s="4" t="inlineStr">
         <is>
-          <t>seo_check_page decoded &amp;#39; but not React's &amp;#x27;, so descriptions showed Tony Greenberg&amp;#x27;s and the length was off</t>
+          <t>publish_changes fixed (2026-10-02)</t>
         </is>
       </c>
       <c r="C257" s="13" t="inlineStr">
@@ -6768,7 +6768,7 @@
       </c>
       <c r="D257" s="4" t="inlineStr">
         <is>
-          <t>Fixed and verified (2026-10-02).</t>
+          <t>it published every draft in Sanity (31 waiting for review today), so any one-line fix would have pushed them all live. Now it publishes only the drafts named in draft_ids; unknown ids are refused before anything happens (verified).</t>
         </is>
       </c>
       <c r="E257" s="14" t="inlineStr">
@@ -6781,7 +6781,7 @@
       <c r="A258" s="4" t="n"/>
       <c r="B258" s="4" t="inlineStr">
         <is>
-          <t>Search Console access for the service account added by the team (2026-10-02); all four search_console_* tools verified with real tonygreenbe…</t>
+          <t>seo_check_page decoded &amp;#39; but not React's &amp;#x27;, so descriptions showed Tony Greenberg&amp;#x27;s and the length was off</t>
         </is>
       </c>
       <c r="C258" s="13" t="inlineStr">
@@ -6791,7 +6791,7 @@
       </c>
       <c r="D258" s="4" t="inlineStr">
         <is>
-          <t>rg.com data (99 clicks / 1,663 impressions in 28 days, homepage indexed, sitemap 284 URLs, 0 errors, 82 warnings).</t>
+          <t>Fixed and verified (2026-10-02).</t>
         </is>
       </c>
       <c r="E258" s="14" t="inlineStr">
@@ -6804,7 +6804,7 @@
       <c r="A259" s="4" t="n"/>
       <c r="B259" s="4" t="inlineStr">
         <is>
-          <t>GOOGLE_GA_CLIENT_EMAIL, GOOGLE_GA_PRIVATE_KEY, GA4_PROPERTY_ID_TONYGREENBERG set in Netlify (2026-10-02, via the Netlify API, values checked…</t>
+          <t>Search Console access for the service account added by the team (2026-10-02); all four search_console_* tools verified with real tonygreenbe…</t>
         </is>
       </c>
       <c r="C259" s="13" t="inlineStr">
@@ -6814,7 +6814,7 @@
       </c>
       <c r="D259" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> equal to .env.local; this plan can't limit a variable's scopes, so they're available to builds and functions). Used from the next deploy.</t>
+          <t>rg.com data (99 clicks / 1,663 impressions in 28 days, homepage indexed, sitemap 284 URLs, 0 errors, 82 warnings).</t>
         </is>
       </c>
       <c r="E259" s="14" t="inlineStr">
@@ -6827,7 +6827,7 @@
       <c r="A260" s="4" t="n"/>
       <c r="B260" s="4" t="inlineStr">
         <is>
-          <t>Per-request change system ported from ramprate-ui (2026-10-02, owner said yes)</t>
+          <t>GOOGLE_GA_CLIENT_EMAIL, GOOGLE_GA_PRIVATE_KEY, GA4_PROPERTY_ID_TONYGREENBERG set in Netlify (2026-10-02, via the Netlify API, values checked…</t>
         </is>
       </c>
       <c r="C260" s="13" t="inlineStr">
@@ -6837,7 +6837,7 @@
       </c>
       <c r="D260" s="4" t="inlineStr">
         <is>
-          <t>, covering the 10 review points the team raised for RampRate's setup: (1) discard_change; (2) one request = one change with its own branch, PR and drafts, so publishing never takes another request live; (3) a review with pages affected, a server-written "what's included" line and preview links; (4) publish needs the review's reviewToken, and the rules make the AI ask "You are about to publish these changes to the live tonygreenberg.com website. Are you sure you want to continue?"; (5) list_change_history, also visible read-only in Studio under "Website change history" (new adminChange type); (6) undo_change; (7) before/after (automatic for Sanity, given by the AI for code); (8) preview_on_devices phone + laptop screenshots (needs GOOGLE_API_KEY); (9) the AI's plain summary plus the server's facts line; (10) Draft → Ready for review → Published / Discarded. Files: change-sets.ts, change-describe.ts, device-preview.ts, mcp-tool-context.ts, mcp-server.ts, github-client.ts (RampRate's full version), src/sanity/schemas/adminChange.ts, sanity.config.ts. Tested end to end with a real throwaway change, then discarded (see docs/ai/project_mcp_server.md).</t>
+          <t xml:space="preserve"> equal to .env.local; this plan can't limit a variable's scopes, so they're available to builds and functions). Used from the next deploy.</t>
         </is>
       </c>
       <c r="E260" s="14" t="inlineStr">
@@ -6850,7 +6850,7 @@
       <c r="A261" s="4" t="n"/>
       <c r="B261" s="4" t="inlineStr">
         <is>
-          <t>Merge the CI fix into main</t>
+          <t>Per-request change system ported from ramprate-ui (2026-10-02, owner said yes)</t>
         </is>
       </c>
       <c r="C261" s="13" t="inlineStr">
@@ -6860,7 +6860,7 @@
       </c>
       <c r="D261" s="4" t="inlineStr">
         <is>
-          <t>(done with PR #3; checked 2026-10-06: main's pr-lint.yml runs Node 22 and next typegen before the type check). The test change's GitHub check failed because main still has the old pr-lint.yml (Node 20 crash). Every MCP change will fail its site check, and so can't be published, until this branch's work (or at least .github/workflows/pr-lint.yml) is on main. Then test a real publish and undo_change.</t>
+          <t>, covering the 10 review points the team raised for RampRate's setup: (1) discard_change; (2) one request = one change with its own branch, PR and drafts, so publishing never takes another request live; (3) a review with pages affected, a server-written "what's included" line and preview links; (4) publish needs the review's reviewToken, and the rules make the AI ask "You are about to publish these changes to the live tonygreenberg.com website. Are you sure you want to continue?"; (5) list_change_history, also visible read-only in Studio under "Website change history" (new adminChange type); (6) undo_change; (7) before/after (automatic for Sanity, given by the AI for code); (8) preview_on_devices phone + laptop screenshots (needs GOOGLE_API_KEY); (9) the AI's plain summary plus the server's facts line; (10) Draft → Ready for review → Published / Discarded. Files: change-sets.ts, change-describe.ts, device-preview.ts, mcp-tool-context.ts, mcp-server.ts, github-client.ts (RampRate's full version), src/sanity/schemas/adminChange.ts, sanity.config.ts. Tested end to end with a real throwaway change, then discarded (see docs/ai/project_mcp_server.md).</t>
         </is>
       </c>
       <c r="E261" s="14" t="inlineStr">
@@ -6873,7 +6873,7 @@
       <c r="A262" s="4" t="n"/>
       <c r="B262" s="4" t="inlineStr">
         <is>
-          <t>Blocked on you (Google)</t>
+          <t>Merge the CI fix into main</t>
         </is>
       </c>
       <c r="C262" s="13" t="inlineStr">
@@ -6883,7 +6883,7 @@
       </c>
       <c r="D262" s="4" t="inlineStr">
         <is>
-          <t>create a GOOGLE_API_KEY in Google Cloud (project of the vcos-ga4-reader service account, where the PageSpeed Insights API is already on), restricted to the PageSpeed Insights API, then add it to .env.local and Netlify. Creating it from here was blocked by the session's safety check (it would use the service account's credentials to change the Cloud project). Note lighthouse_check_page may time out on Netlify (10 s function limit on the free plan). Dropped 2026-10-13 (owner: "pagespeed.web.dev you can remove"): no Google key or US PageSpeed run needed.</t>
+          <t>(done with PR #3; checked 2026-10-06: main's pr-lint.yml runs Node 22 and next typegen before the type check). The test change's GitHub check failed because main still has the old pr-lint.yml (Node 20 crash). Every MCP change will fail its site check, and so can't be published, until this branch's work (or at least .github/workflows/pr-lint.yml) is on main. Then test a real publish and undo_change.</t>
         </is>
       </c>
       <c r="E262" s="14" t="inlineStr">
@@ -6896,7 +6896,7 @@
       <c r="A263" s="4" t="n"/>
       <c r="B263" s="4" t="inlineStr">
         <is>
-          <t>Synced with ramprate-ui's MCP server (2026-10-09, owner asked; card included by their choice)</t>
+          <t>Blocked on you (Google)</t>
         </is>
       </c>
       <c r="C263" s="13" t="inlineStr">
@@ -6906,7 +6906,7 @@
       </c>
       <c r="D263" s="4" t="inlineStr">
         <is>
-          <t>the review card for ChatGPT/Claude (one status and next step, Build / Type check / Lint / GitHub / phone-and-laptop checks, "what goes live" and what doesn't, Preview / Discard / Publish / Retry, history with Restore); start_change restates the request (understood_as) and unclear ones wait for the person's OK (confirm_change); before (live) / after (preview) screenshots on phone and laptop; attached images and files (ChatGPT file, or request_upload_link, a private 30-minute upload page at /api/mcp/upload, size and real-type checked); every change result lists the other waiting changes and the AI ends its reply with them (new Status Report line); the server lints changed files itself; ESLint now traced into the deployed function (serverExternalPackages; ramprate's tracing globs crash Turbopack under pnpm, left out). Everything named for tonygreenberg.com only (Netlify tonygreenberg-website, live tonygreenberg.com, card ui://tonygreenberg-admin/...). Verified on a local production build: type check, lint, build; 30 tools listed; card served and its script valid; rules include migrationStatus; list_pending_changes returns other pending changes; check_code_quality runs ESLint; upload page refuses bad links (401). See docs/ai/project_mcp_server.md.</t>
+          <t>create a GOOGLE_API_KEY in Google Cloud (project of the vcos-ga4-reader service account, where the PageSpeed Insights API is already on), restricted to the PageSpeed Insights API, then add it to .env.local and Netlify. Creating it from here was blocked by the session's safety check (it would use the service account's credentials to change the Cloud project). Note lighthouse_check_page may time out on Netlify (10 s function limit on the free plan). Dropped 2026-10-13 (owner: "pagespeed.web.dev you can remove"): no Google key or US PageSpeed run needed.</t>
         </is>
       </c>
       <c r="E263" s="14" t="inlineStr">
@@ -6919,63 +6919,63 @@
       <c r="A264" s="4" t="n"/>
       <c r="B264" s="4" t="inlineStr">
         <is>
+          <t>Synced with ramprate-ui's MCP server (2026-10-09, owner asked; card included by their choice)</t>
+        </is>
+      </c>
+      <c r="C264" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D264" s="4" t="inlineStr">
+        <is>
+          <t>the review card for ChatGPT/Claude (one status and next step, Build / Type check / Lint / GitHub / phone-and-laptop checks, "what goes live" and what doesn't, Preview / Discard / Publish / Retry, history with Restore); start_change restates the request (understood_as) and unclear ones wait for the person's OK (confirm_change); before (live) / after (preview) screenshots on phone and laptop; attached images and files (ChatGPT file, or request_upload_link, a private 30-minute upload page at /api/mcp/upload, size and real-type checked); every change result lists the other waiting changes and the AI ends its reply with them (new Status Report line); the server lints changed files itself; ESLint now traced into the deployed function (serverExternalPackages; ramprate's tracing globs crash Turbopack under pnpm, left out). Everything named for tonygreenberg.com only (Netlify tonygreenberg-website, live tonygreenberg.com, card ui://tonygreenberg-admin/...). Verified on a local production build: type check, lint, build; 30 tools listed; card served and its script valid; rules include migrationStatus; list_pending_changes returns other pending changes; check_code_quality runs ESLint; upload page refuses bad links (401). See docs/ai/project_mcp_server.md.</t>
+        </is>
+      </c>
+      <c r="E264" s="14" t="inlineStr">
+        <is>
+          <t>Phase 11 — Code MCP Server — REBUILT (2026-09-29)</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="4" t="n"/>
+      <c r="B265" s="4" t="inlineStr">
+        <is>
           <t>Test the new review end to end on a deploy preview</t>
         </is>
       </c>
-      <c r="C264" s="16" t="inlineStr">
+      <c r="C265" s="16" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
       </c>
-      <c r="D264" s="4" t="inlineStr">
+      <c r="D265" s="4" t="inlineStr">
         <is>
           <t>(needs a yes, it opens a real pull request): one throwaway change from Claude.ai or ChatGPT: start (unclear request, so the confirm step shows), confirm, edit, review card, screenshots, upload link, then discard.</t>
         </is>
       </c>
-      <c r="E264" s="14" t="inlineStr">
+      <c r="E265" s="14" t="inlineStr">
         <is>
           <t>Phase 11 — Code MCP Server — REBUILT (2026-09-29)</t>
         </is>
       </c>
     </row>
-    <row r="265">
-      <c r="A265" s="10" t="inlineStr">
+    <row r="266">
+      <c r="A266" s="10" t="inlineStr">
         <is>
           <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
         </is>
       </c>
-      <c r="B265" s="11" t="n"/>
-      <c r="C265" s="11" t="n"/>
-      <c r="D265" s="12" t="n"/>
-    </row>
-    <row r="266">
-      <c r="A266" s="4" t="n"/>
-      <c r="B266" s="4" t="inlineStr">
-        <is>
-          <t>Per-page generateMetadata (title, description, OG, Twitter Card, canonical) for every ported route, sourced from Sanity seo object where con…</t>
-        </is>
-      </c>
-      <c r="C266" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D266" s="4" t="inlineStr">
-        <is>
-          <t>tent is CMS-backed, static otherwise. Audited all 140 page.tsx files: only /studio has none (correct — it's robots.txt-disallowed, not public content). Real gap found and fixed: /blog/category/[slug] had no alternates.canonical at all, and no page-aware title for its own real pagination (?page=N) — every paginated page was serving an identical title with no canonical, a real duplicate-content signal. Fixed: generateMetadata now reads searchParams too, self-canonicals each page (?page=N pages canonical to themselves, not consolidated to page 1 — genuinely different posts per page, matching Google's current pagination guidance) and appends "— Page N" to the title past page 1. Verified live: page 1 canonicals to the bare URL, ?page=2 canonicals to ?page=2 with a distinct title.</t>
-        </is>
-      </c>
-      <c r="E266" s="14" t="inlineStr">
-        <is>
-          <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
-        </is>
-      </c>
+      <c r="B266" s="11" t="n"/>
+      <c r="C266" s="11" t="n"/>
+      <c r="D266" s="12" t="n"/>
     </row>
     <row r="267">
       <c r="A267" s="4" t="n"/>
       <c r="B267" s="4" t="inlineStr">
         <is>
-          <t>sitemap.ts generated from real Sanity content + static route list, auto-updates on publish</t>
+          <t>Per-page generateMetadata (title, description, OG, Twitter Card, canonical) for every ported route, sourced from Sanity seo object where con…</t>
         </is>
       </c>
       <c r="C267" s="13" t="inlineStr">
@@ -6985,7 +6985,7 @@
       </c>
       <c r="D267" s="4" t="inlineStr">
         <is>
-          <t>Extended from the Phase 5-era version (homepage + blog posts only, 122 URLs) to every real route: the full static route list (130 routes, generated from find src/app -name page.tsx, excluding /studio (robots.txt-disallowed), /(auth)/login (noindex via its own metadata), and /life-assessment (a pure redirect, not distinct content)) plus all 5 real dynamic sources — blog categories (allCategorySlugsQuery), BrewSoul cities (25), BrewSoul coffees (107), and charity-scorecard entries (103) — each pulled from the exact same data source its own page's generateStaticParams already uses, not re-derived. Auto-updates on publish for anything Sanity-backed (blog posts/categories) since it's a live client.fetch on every build; the static route list itself needs a one-line addition whenever a new page ships (same as any other route-registration step). Verified live: 496 real &lt;loc&gt; entries, spot-checked a coffee/city/charity/category URL each, typecheck/lint clean.</t>
+          <t>tent is CMS-backed, static otherwise. Audited all 140 page.tsx files: only /studio has none (correct — it's robots.txt-disallowed, not public content). Real gap found and fixed: /blog/category/[slug] had no alternates.canonical at all, and no page-aware title for its own real pagination (?page=N) — every paginated page was serving an identical title with no canonical, a real duplicate-content signal. Fixed: generateMetadata now reads searchParams too, self-canonicals each page (?page=N pages canonical to themselves, not consolidated to page 1 — genuinely different posts per page, matching Google's current pagination guidance) and appends "— Page N" to the title past page 1. Verified live: page 1 canonicals to the bare URL, ?page=2 canonicals to ?page=2 with a distinct title.</t>
         </is>
       </c>
       <c r="E267" s="14" t="inlineStr">
@@ -6998,7 +6998,7 @@
       <c r="A268" s="4" t="n"/>
       <c r="B268" s="4" t="inlineStr">
         <is>
-          <t>llms.txt</t>
+          <t>sitemap.ts generated from real Sanity content + static route list, auto-updates on publish</t>
         </is>
       </c>
       <c r="C268" s="13" t="inlineStr">
@@ -7008,7 +7008,7 @@
       </c>
       <c r="D268" s="4" t="inlineStr">
         <is>
-          <t>fetched verbatim from the still-live site and saved to web/public/llms.txt (real content: Tony's bio, expertise, full article index by category, every product/tool section) — do this before Manus goes away, it won't be recoverable after</t>
+          <t>Extended from the Phase 5-era version (homepage + blog posts only, 122 URLs) to every real route: the full static route list (130 routes, generated from find src/app -name page.tsx, excluding /studio (robots.txt-disallowed), /(auth)/login (noindex via its own metadata), and /life-assessment (a pure redirect, not distinct content)) plus all 5 real dynamic sources — blog categories (allCategorySlugsQuery), BrewSoul cities (25), BrewSoul coffees (107), and charity-scorecard entries (103) — each pulled from the exact same data source its own page's generateStaticParams already uses, not re-derived. Auto-updates on publish for anything Sanity-backed (blog posts/categories) since it's a live client.fetch on every build; the static route list itself needs a one-line addition whenever a new page ships (same as any other route-registration step). Verified live: 496 real &lt;loc&gt; entries, spot-checked a coffee/city/charity/category URL each, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E268" s="14" t="inlineStr">
@@ -7021,7 +7021,7 @@
       <c r="A269" s="4" t="n"/>
       <c r="B269" s="4" t="inlineStr">
         <is>
-          <t>robots.txt</t>
+          <t>llms.txt</t>
         </is>
       </c>
       <c r="C269" s="13" t="inlineStr">
@@ -7031,7 +7031,7 @@
       </c>
       <c r="D269" s="4" t="inlineStr">
         <is>
-          <t>same approach: fetched the real live file (not my earlier guessed robots.ts, which has been removed) and saved verbatim to web/public/robots.txt, plus added Disallow: /studio for the new Sanity Studio route. Confirmed live: real AI-crawler allowlist (GPTBot, Claude-Web, PerplexityBot, etc.), scraper blocklist, and the site's non-standard LLMs: directive all intact</t>
+          <t>fetched verbatim from the still-live site and saved to web/public/llms.txt (real content: Tony's bio, expertise, full article index by category, every product/tool section) — do this before Manus goes away, it won't be recoverable after</t>
         </is>
       </c>
       <c r="E269" s="14" t="inlineStr">
@@ -7044,7 +7044,7 @@
       <c r="A270" s="4" t="n"/>
       <c r="B270" s="4" t="inlineStr">
         <is>
-          <t>JSON-LD</t>
+          <t>robots.txt</t>
         </is>
       </c>
       <c r="C270" s="13" t="inlineStr">
@@ -7054,7 +7054,7 @@
       </c>
       <c r="D270" s="4" t="inlineStr">
         <is>
-          <t>WebSite + Person schema ported verbatim from the live homepage's actual &lt;script type="application/ld+json"&gt; tags (not reconstructed from memory) — rendered site-wide from src/lib/structured-data.ts in the root layout. The Person image was hardcoded to a /api/img/... legacy proxy path on the live site — rescued that headshot (downloaded it while still live, uploaded to Sanity as the author-tony-greenberg document's avatar) so the new site's JSON-LD has zero Manus dependency instead of just copying the fragile path forward</t>
+          <t>same approach: fetched the real live file (not my earlier guessed robots.ts, which has been removed) and saved verbatim to web/public/robots.txt, plus added Disallow: /studio for the new Sanity Studio route. Confirmed live: real AI-crawler allowlist (GPTBot, Claude-Web, PerplexityBot, etc.), scraper blocklist, and the site's non-standard LLMs: directive all intact</t>
         </is>
       </c>
       <c r="E270" s="14" t="inlineStr">
@@ -7067,7 +7067,7 @@
       <c r="A271" s="4" t="n"/>
       <c r="B271" s="4" t="inlineStr">
         <is>
-          <t>Article JSON-LD on /blog/[slug], built from real per-post Sanity data (headline, image, datePublished/dateModified, author, canonical URL)</t>
+          <t>JSON-LD</t>
         </is>
       </c>
       <c r="C271" s="13" t="inlineStr">
@@ -7077,7 +7077,7 @@
       </c>
       <c r="D271" s="4" t="inlineStr">
         <is>
-          <t>verified live on a real post</t>
+          <t>WebSite + Person schema ported verbatim from the live homepage's actual &lt;script type="application/ld+json"&gt; tags (not reconstructed from memory) — rendered site-wide from src/lib/structured-data.ts in the root layout. The Person image was hardcoded to a /api/img/... legacy proxy path on the live site — rescued that headshot (downloaded it while still live, uploaded to Sanity as the author-tony-greenberg document's avatar) so the new site's JSON-LD has zero Manus dependency instead of just copying the fragile path forward</t>
         </is>
       </c>
       <c r="E271" s="14" t="inlineStr">
@@ -7090,7 +7090,7 @@
       <c r="A272" s="4" t="n"/>
       <c r="B272" s="4" t="inlineStr">
         <is>
-          <t>Build the full Manus/legacy-URL → Next.js-URL 301 redirect map (next.config.ts redirects() or Sanity redirect documents)</t>
+          <t>Article JSON-LD on /blog/[slug], built from real per-post Sanity data (headline, image, datePublished/dateModified, author, canonical URL)</t>
         </is>
       </c>
       <c r="C272" s="13" t="inlineStr">
@@ -7100,7 +7100,7 @@
       </c>
       <c r="D272" s="4" t="inlineStr">
         <is>
-          <t>hard QA gate, nothing proceeds to DNS cutover until this is complete and tested. First real pass done: extracted all 197 real path= routes from legacy's App.tsx router (not guessed — the actual route table), diffed against this app's real current routes (find src/app -maxdepth 1 -name page.tsx) + next.config.ts's existing redirect sources, normalizing :param/[param] syntax to compare like-for-like. Started at 41 real gaps, closed 10 with new redirects: /attention-theft/{blocker-finder,legal,report,weapons} (legacy registered both a bare AND a /attention-theft/-nested path for each, only the bare ones had redirects before), /find-my-car → /find-my, /the-index → /search (matching the fix already applied to other pages' dead links to it), /supplier-intake-long (bare) + /vendor-intake + /vendor-intake-long (+/:token) → the same real ramprate.com/biochain/supplier-intake destination the token'd path already redirected to, and /spamtoast + /youve-been-reported → / (the live half of legacy's "report a spammer" confrontation flow — a fake IP-fingerprinting/countdown-timer page; the other half, ReportSpammer.tsx, was already a documented drop in Phase 4, this is the same call for its sequel). 21 of the remaining 31 gaps need no redirect — they're /admin/*//analytics//edit/frqncy (internal tools never meant for public discovery) or already-documented intentional defers from Phase 4/7/10 (/clock-keeper-part-2, /ecosystem-map, /friend-gate, /friend-survey/:token, /medicine-sequencing, /m</t>
+          <t>verified live on a real post</t>
         </is>
       </c>
       <c r="E272" s="14" t="inlineStr">
@@ -7113,7 +7113,7 @@
       <c r="A273" s="4" t="n"/>
       <c r="B273" s="4" t="inlineStr">
         <is>
-          <t>/path/:archetype (src/app/path/[archetype]/page.tsx)</t>
+          <t>Build the full Manus/legacy-URL → Next.js-URL 301 redirect map (next.config.ts redirects() or Sanity redirect documents)</t>
         </is>
       </c>
       <c r="C273" s="13" t="inlineStr">
@@ -7123,7 +7123,7 @@
       </c>
       <c r="D273" s="4" t="inlineStr">
         <is>
-          <t>per-archetype landing page for /assessment's Builder/Crusader/Investor result, reusing lib/content/archetypes.ts. Real content ported in full (top-5 essential-reading list per archetype via allPostsForArchiveQuery, real PathSubscribeForm posting to /api/subscribe, AUTHORITY_ITEMS strip). Real bug fixed vs. legacy: replaced a hand-rolled inline-styled "Path not found" div with a real notFound() (this route's generateStaticParams only ever produces the 3 real keys). Verified live: all 3 archetype routes 200 OK, typecheck/lint clean.</t>
+          <t>hard QA gate, nothing proceeds to DNS cutover until this is complete and tested. First real pass done: extracted all 197 real path= routes from legacy's App.tsx router (not guessed — the actual route table), diffed against this app's real current routes (find src/app -maxdepth 1 -name page.tsx) + next.config.ts's existing redirect sources, normalizing :param/[param] syntax to compare like-for-like. Started at 41 real gaps, closed 10 with new redirects: /attention-theft/{blocker-finder,legal,report,weapons} (legacy registered both a bare AND a /attention-theft/-nested path for each, only the bare ones had redirects before), /find-my-car → /find-my, /the-index → /search (matching the fix already applied to other pages' dead links to it), /supplier-intake-long (bare) + /vendor-intake + /vendor-intake-long (+/:token) → the same real ramprate.com/biochain/supplier-intake destination the token'd path already redirected to, and /spamtoast + /youve-been-reported → / (the live half of legacy's "report a spammer" confrontation flow — a fake IP-fingerprinting/countdown-timer page; the other half, ReportSpammer.tsx, was already a documented drop in Phase 4, this is the same call for its sequel). 21 of the remaining 31 gaps need no redirect — they're /admin/*//analytics//edit/frqncy (internal tools never meant for public discovery) or already-documented intentional defers from Phase 4/7/10 (/clock-keeper-part-2, /ecosystem-map, /friend-gate, /friend-survey/:token, /medicine-sequencing, /m</t>
         </is>
       </c>
       <c r="E273" s="14" t="inlineStr">
@@ -7136,7 +7136,7 @@
       <c r="A274" s="4" t="n"/>
       <c r="B274" s="4" t="inlineStr">
         <is>
-          <t>/my-journey (src/app/my-journey/page.tsx + components/assessments/my-journey-dashboard.tsx)</t>
+          <t>/path/:archetype (src/app/path/[archetype]/page.tsx)</t>
         </is>
       </c>
       <c r="C274" s="13" t="inlineStr">
@@ -7146,7 +7146,7 @@
       </c>
       <c r="D274" s="4" t="inlineStr">
         <is>
-          <t>"My Journey Dashboard," real grid/timeline views across all 28 JOURNEY_MAP experiences, category/status filters, phase progress ring, recommended-next card, using the same real useJourneyProgress/JOURNEY_MAP completion tracking every "Find Your X" quiz already writes to (not the narrower tg_assessment_results cookie built for /self-portrait). Legacy's per-quiz scored-result caching (RESULT_KEYS, feeding a mini radar chart) was not ported — no quiz in this migration writes that data either, same honest-degradation call already made for /self-portrait's own composite radar. Fixed a real legacy dead link (/ecosystem-map, a still-unbuilt page) to /self-portrait. Verified live: 200 OK, real content confirmed, typecheck/lint clean.</t>
+          <t>per-archetype landing page for /assessment's Builder/Crusader/Investor result, reusing lib/content/archetypes.ts. Real content ported in full (top-5 essential-reading list per archetype via allPostsForArchiveQuery, real PathSubscribeForm posting to /api/subscribe, AUTHORITY_ITEMS strip). Real bug fixed vs. legacy: replaced a hand-rolled inline-styled "Path not found" div with a real notFound() (this route's generateStaticParams only ever produces the 3 real keys). Verified live: all 3 archetype routes 200 OK, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E274" s="14" t="inlineStr">
@@ -7159,7 +7159,7 @@
       <c r="A275" s="4" t="n"/>
       <c r="B275" s="4" t="inlineStr">
         <is>
-          <t>/the-open-door (src/app/the-open-door/page.tsx)</t>
+          <t>/my-journey (src/app/my-journey/page.tsx + components/assessments/my-journey-dashboard.tsx)</t>
         </is>
       </c>
       <c r="C275" s="13" t="inlineStr">
@@ -7169,7 +7169,7 @@
       </c>
       <c r="D275" s="4" t="inlineStr">
         <is>
-          <t>real press/credibility content: all 10 "Magic Genie" client-pitch prompts (real named targets — Marco Argenti/Goldman Sachs, Adam Smith/Disney, etc.), 18 real client testimonials, all 8 explicitly-labeled satirical "parody" quotes (kept with disclaimers, not presented as real). Real overlap found and reconciled: this page's publications/speaking/podcasts arrays substantially duplicate the already-shipped /published's fuller bibliography — kept only what /published doesn't cover (Forbes + Business Insider bylines, the Clinton Global Initiative keynote, 4 of 5 podcast appearances) and cross-linked to /published for the rest, same reconciliation pattern as /assessments vs /find-my. Real bugs fixed: 3 genie/keynote links pointed externally at tonygreenberg.com/&lt;slug&gt; for posts that are real internal posts in this migration — relinked to /blog/psychedelics-could-become-extractive-capitalism, /blog/boiling-the-human-summit-harvard-kurzweil, /blog/return-on-investment-going-green-going-green-2 (all verified 200); a bare self-link to tonygreenberg.com remapped to /. Ships as a pure Server Component (legacy's FadeIn/Section/editorial-component dependencies don't exist here and weren't needed). Verified live: 200 OK, real content in raw SSR HTML, typecheck/lint clean.</t>
+          <t>"My Journey Dashboard," real grid/timeline views across all 28 JOURNEY_MAP experiences, category/status filters, phase progress ring, recommended-next card, using the same real useJourneyProgress/JOURNEY_MAP completion tracking every "Find Your X" quiz already writes to (not the narrower tg_assessment_results cookie built for /self-portrait). Legacy's per-quiz scored-result caching (RESULT_KEYS, feeding a mini radar chart) was not ported — no quiz in this migration writes that data either, same honest-degradation call already made for /self-portrait's own composite radar. Fixed a real legacy dead link (/ecosystem-map, a still-unbuilt page) to /self-portrait. Verified live: 200 OK, real content confirmed, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E275" s="14" t="inlineStr">
@@ -7182,7 +7182,7 @@
       <c r="A276" s="4" t="n"/>
       <c r="B276" s="4" t="inlineStr">
         <is>
-          <t>Homepage "Recent Updates" band (2026-09-29)</t>
+          <t>/the-open-door (src/app/the-open-door/page.tsx)</t>
         </is>
       </c>
       <c r="C276" s="13" t="inlineStr">
@@ -7192,7 +7192,7 @@
       </c>
       <c r="D276" s="4" t="inlineStr">
         <is>
-          <t>on the live site (a newer Blog.tsx than _legacy-manus-app/, so rebuilt from the live page's markup), replacing the older "Latest Thinking" pair. Found while doing it: two live essays are missing from Sanity, the-tollbooth-and-the-alternative (Aug 18, 2026, the live site's newest) and what-quest-could-fix. Both were published on live after the legacy snapshot and need importing.</t>
+          <t>real press/credibility content: all 10 "Magic Genie" client-pitch prompts (real named targets — Marco Argenti/Goldman Sachs, Adam Smith/Disney, etc.), 18 real client testimonials, all 8 explicitly-labeled satirical "parody" quotes (kept with disclaimers, not presented as real). Real overlap found and reconciled: this page's publications/speaking/podcasts arrays substantially duplicate the already-shipped /published's fuller bibliography — kept only what /published doesn't cover (Forbes + Business Insider bylines, the Clinton Global Initiative keynote, 4 of 5 podcast appearances) and cross-linked to /published for the rest, same reconciliation pattern as /assessments vs /find-my. Real bugs fixed: 3 genie/keynote links pointed externally at tonygreenberg.com/&lt;slug&gt; for posts that are real internal posts in this migration — relinked to /blog/psychedelics-could-become-extractive-capitalism, /blog/boiling-the-human-summit-harvard-kurzweil, /blog/return-on-investment-going-green-going-green-2 (all verified 200); a bare self-link to tonygreenberg.com remapped to /. Ships as a pure Server Component (legacy's FadeIn/Section/editorial-component dependencies don't exist here and weren't needed). Verified live: 200 OK, real content in raw SSR HTML, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E276" s="14" t="inlineStr">
@@ -7205,7 +7205,7 @@
       <c r="A277" s="4" t="n"/>
       <c r="B277" s="4" t="inlineStr">
         <is>
-          <t>Re-sync the legacy reference</t>
+          <t>Homepage "Recent Updates" band (2026-09-29)</t>
         </is>
       </c>
       <c r="C277" s="13" t="inlineStr">
@@ -7215,7 +7215,7 @@
       </c>
       <c r="D277" s="4" t="inlineStr">
         <is>
-          <t>_legacy-manus-app/ is older than what's live (Recent Updates proves it), so visual diffs should be against the live site, not only that folder. Closed 2026-10-08: done the way this item suggests: every comparison since 2026-10-01 is against the live site itself (163 pages + 121 posts on 2026-10-01, 188 pages on 2026-10-07, 18 redesigned pages on 2026-10-08), with _legacy-manus-app/ used only as the code reference.</t>
+          <t>on the live site (a newer Blog.tsx than _legacy-manus-app/, so rebuilt from the live page's markup), replacing the older "Latest Thinking" pair. Found while doing it: two live essays are missing from Sanity, the-tollbooth-and-the-alternative (Aug 18, 2026, the live site's newest) and what-quest-could-fix. Both were published on live after the legacy snapshot and need importing.</t>
         </is>
       </c>
       <c r="E277" s="14" t="inlineStr">
@@ -7228,7 +7228,7 @@
       <c r="A278" s="4" t="n"/>
       <c r="B278" s="4" t="inlineStr">
         <is>
-          <t>Visual diff pass: every ported page vs</t>
+          <t>Re-sync the legacy reference</t>
         </is>
       </c>
       <c r="C278" s="13" t="inlineStr">
@@ -7238,7 +7238,7 @@
       </c>
       <c r="D278" s="4" t="inlineStr">
         <is>
-          <t>legacy page Closed 2026-10-08: covered by the live-site sweeps above (screenshots and measured title/label/spacing per page, see the 2026-10-01, 10-02, 10-07 and 10-08 entries in this phase). Remaining differences are listed as decisions (Cormorant titles, /find-my header) or deliberate (CONTRIBUTING rule 20).</t>
+          <t>_legacy-manus-app/ is older than what's live (Recent Updates proves it), so visual diffs should be against the live site, not only that folder. Closed 2026-10-08: done the way this item suggests: every comparison since 2026-10-01 is against the live site itself (163 pages + 121 posts on 2026-10-01, 188 pages on 2026-10-07, 18 redesigned pages on 2026-10-08), with _legacy-manus-app/ used only as the code reference.</t>
         </is>
       </c>
       <c r="E278" s="14" t="inlineStr">
@@ -7251,7 +7251,7 @@
       <c r="A279" s="4" t="n"/>
       <c r="B279" s="4" t="inlineStr">
         <is>
-          <t>Padding / spacing on the story pages matched to live (2026-10-01)</t>
+          <t>Visual diff pass: every ported page vs</t>
         </is>
       </c>
       <c r="C279" s="13" t="inlineStr">
@@ -7261,7 +7261,7 @@
       </c>
       <c r="D279" s="4" t="inlineStr">
         <is>
-          <t>Measured margins, text column and spacing on 31 pages, live vs a production build, at 375px and 1280px. The "door" story pages were the clear mismatch: live's text column is ~546px (ours was 720px), 20px side margins on phones / 40px on desktop, body text 19px/1.8 on phones and 18px/1.85 on desktop (ours 16px/1.5). Fixed on /the-body, /engine-room, /under-nda, /the-nightstand, /the-web, /the-territory, /about, /intel (Intel uses live's 16.8px/1.9; About's hero line 480px max, 18.4px/1.8). Re-measured: all 8 match live to within 2px (About's column 28px narrower), no sideways scroll at 375px.</t>
+          <t>legacy page Closed 2026-10-08: covered by the live-site sweeps above (screenshots and measured title/label/spacing per page, see the 2026-10-01, 10-02, 10-07 and 10-08 entries in this phase). Remaining differences are listed as decisions (Cormorant titles, /find-my header) or deliberate (CONTRIBUTING rule 20).</t>
         </is>
       </c>
       <c r="E279" s="14" t="inlineStr">
@@ -7274,7 +7274,7 @@
       <c r="A280" s="4" t="n"/>
       <c r="B280" s="4" t="inlineStr">
         <is>
-          <t>Header-to-title spacing re-checked (2026-10-02)</t>
+          <t>Padding / spacing on the story pages matched to live (2026-10-01)</t>
         </is>
       </c>
       <c r="C280" s="13" t="inlineStr">
@@ -7284,7 +7284,7 @@
       </c>
       <c r="D280" s="4" t="inlineStr">
         <is>
-          <t>The 2026-10-01 note compared different things: live's header wasn't measured (it showed 0), so "96px vs 168px" was really 161px vs 168px from the top of the page. Measured again from the top of the page, live vs a production build, at 375px and 1280px: most pages were already within 10px. Fixed the real gaps: /the-open-door (now live's dark centered hero band, 56px title, 546px text column; title was 72px too high), /start-here (live's 48px/96px top padding; 25px too high on desktop), /invest and /engage (label spacing and live's 32px/51px title; /invest's desktop title was 36px), /impact-dashboard on phones (card edge to edge under the header like live; title was 89px too low). Re-measured: all within 8px of live, no sideways scroll at 375px, no JS errors.</t>
+          <t>Measured margins, text column and spacing on 31 pages, live vs a production build, at 375px and 1280px. The "door" story pages were the clear mismatch: live's text column is ~546px (ours was 720px), 20px side margins on phones / 40px on desktop, body text 19px/1.8 on phones and 18px/1.85 on desktop (ours 16px/1.5). Fixed on /the-body, /engine-room, /under-nda, /the-nightstand, /the-web, /the-territory, /about, /intel (Intel uses live's 16.8px/1.9; About's hero line 480px max, 18.4px/1.8). Re-measured: all 8 match live to within 2px (About's column 28px narrower), no sideways scroll at 375px.</t>
         </is>
       </c>
       <c r="E280" s="14" t="inlineStr">
@@ -7297,7 +7297,7 @@
       <c r="A281" s="4" t="n"/>
       <c r="B281" s="4" t="inlineStr">
         <is>
-          <t>HumanOS headings in capitals like live (2026-10-02, owner said yes)</t>
+          <t>Header-to-title spacing re-checked (2026-10-02)</t>
         </is>
       </c>
       <c r="C281" s="13" t="inlineStr">
@@ -7307,7 +7307,7 @@
       </c>
       <c r="D281" s="4" t="inlineStr">
         <is>
-          <t>the 4 headings live capitalises on /humanos (title, "Are you a Maximizer...", "Take the Diagnostic", "The Diagnostic") get uppercase; the words are unchanged. The subpages already matched.</t>
+          <t>The 2026-10-01 note compared different things: live's header wasn't measured (it showed 0), so "96px vs 168px" was really 161px vs 168px from the top of the page. Measured again from the top of the page, live vs a production build, at 375px and 1280px: most pages were already within 10px. Fixed the real gaps: /the-open-door (now live's dark centered hero band, 56px title, 546px text column; title was 72px too high), /start-here (live's 48px/96px top padding; 25px too high on desktop), /invest and /engage (label spacing and live's 32px/51px title; /invest's desktop title was 36px), /impact-dashboard on phones (card edge to edge under the header like live; title was 89px too low). Re-measured: all within 8px of live, no sideways scroll at 375px, no JS errors.</t>
         </is>
       </c>
       <c r="E281" s="14" t="inlineStr">
@@ -7320,7 +7320,7 @@
       <c r="A282" s="4" t="n"/>
       <c r="B282" s="4" t="inlineStr">
         <is>
-          <t>More layout gaps matched to live (2026-10-02)</t>
+          <t>HumanOS headings in capitals like live (2026-10-02, owner said yes)</t>
         </is>
       </c>
       <c r="C282" s="13" t="inlineStr">
@@ -7330,7 +7330,7 @@
       </c>
       <c r="D282" s="4" t="inlineStr">
         <is>
-          <t>/series (live's centered 546px column, and a bug fixed: every card kept an empty 240px picture column, squeezing the text; live's per-series picture is one generic placeholder on the Manus proxy, so not copied), /humanos (middle section 900px like live), homepage desktop widths (hero text 804px, Four Doors 1000px, Editor's Picks 1168px, GemSpark edge, section title sizes; live's /blog now shows the homepage), /find-my (photo undimmed and plain background, like live; our site header kept). Re-measured: headings within 3px (/series) to 20px (homepage) of live, no sideways scroll, no JS errors. Note: live's "New here?" tour bar sits over its header and doesn't move the page, so it doesn't affect these numbers.</t>
+          <t>the 4 headings live capitalises on /humanos (title, "Are you a Maximizer...", "Take the Diagnostic", "The Diagnostic") get uppercase; the words are unchanged. The subpages already matched.</t>
         </is>
       </c>
       <c r="E282" s="14" t="inlineStr">
@@ -7343,7 +7343,7 @@
       <c r="A283" s="4" t="n"/>
       <c r="B283" s="4" t="inlineStr">
         <is>
-          <t>Full sweep vs live (2026-10-02)</t>
+          <t>More layout gaps matched to live (2026-10-02)</t>
         </is>
       </c>
       <c r="C283" s="13" t="inlineStr">
@@ -7353,7 +7353,7 @@
       </c>
       <c r="D283" s="4" t="inlineStr">
         <is>
-          <t>142 pages (every non-blog page, 3 of each templated set) at 375px and 1280px, title position, text column, title size. Fixed the shared causes: BrewSoul (live wraps most pages in its frame twice, so a second 52px offset plus the category badge; the landing, cities, directory and quiz pages have neither: src/components/brewsoul/brewsoul-main.tsx; intro paragraphs uncapped like live; 38px titles), Kava (live's extra 52px offset), /the-body, /the-nightstand, /the-web (405px top photo like live), the 6 peptide pages (live's 768/896px intro column), /journeys, /pick-up-the-phone, /published, /ecosystem (546px story column and live's text size). Re-measured: 110 of 120 within 40px / 60px of live.</t>
+          <t>/series (live's centered 546px column, and a bug fixed: every card kept an empty 240px picture column, squeezing the text; live's per-series picture is one generic placeholder on the Manus proxy, so not copied), /humanos (middle section 900px like live), homepage desktop widths (hero text 804px, Four Doors 1000px, Editor's Picks 1168px, GemSpark edge, section title sizes; live's /blog now shows the homepage), /find-my (photo undimmed and plain background, like live; our site header kept). Re-measured: headings within 3px (/series) to 20px (homepage) of live, no sideways scroll, no JS errors. Note: live's "New here?" tour bar sits over its header and doesn't move the page, so it doesn't affect these numbers.</t>
         </is>
       </c>
       <c r="E283" s="14" t="inlineStr">
@@ -7366,7 +7366,7 @@
       <c r="A284" s="4" t="n"/>
       <c r="B284" s="4" t="inlineStr">
         <is>
-          <t>Sweep leftovers fixed (2026-10-06)</t>
+          <t>Full sweep vs live (2026-10-02)</t>
         </is>
       </c>
       <c r="C284" s="13" t="inlineStr">
@@ -7376,7 +7376,7 @@
       </c>
       <c r="D284" s="4" t="inlineStr">
         <is>
-          <t>Ported legacy's exact title sizes, margins and column widths. Measured live vs a production build at 375px and 1280px (H1 distance from the top, H1 size, intro and table widths). Now within 8px and the same title size on /published, /brewsoul/first-sip, /brewsoul/home, /brewsoul/chains (intro 912px like live), /brewsoul/browse, /brewsoul/directory (3-column 952px grid like live), /brewsoul and /brewsoul/quiz (intro 520px), /amplifier (546px column), /diamond-cut, /speaking, /living-declaration, /spirits, /protecting-your-business (tables 730px), and the 5 HumanOS subpages (titles smaller like live, 752px column). No sideways scroll at 375px. Left on purpose: /self-portrait (font matches; our page has a different title and no back link, so it sits 23-57px higher), BrewSoul pages 3-6px off (the shared journey bar row), and the different-layout pages /dharma-finder, /grant-study, /search, /quiz_25q, /soulscore. Also: /brewsoul/quiz rebuilt as a step registry (src/components/brewsoul/brewsoul-quiz/: parent + hook/ + components/step-* + data/), same questions, scoring and look; Back/Skip/Retake use lucide icons. New CONTRIBUTING rule 19 (multi-step flows, FydoPartner pattern). brewsoul-welcome-quiz.tsx (/brewsoul) still has the old shape and text arrows.</t>
+          <t>142 pages (every non-blog page, 3 of each templated set) at 375px and 1280px, title position, text column, title size. Fixed the shared causes: BrewSoul (live wraps most pages in its frame twice, so a second 52px offset plus the category badge; the landing, cities, directory and quiz pages have neither: src/components/brewsoul/brewsoul-main.tsx; intro paragraphs uncapped like live; 38px titles), Kava (live's extra 52px offset), /the-body, /the-nightstand, /the-web (405px top photo like live), the 6 peptide pages (live's 768/896px intro column), /journeys, /pick-up-the-phone, /published, /ecosystem (546px story column and live's text size). Re-measured: 110 of 120 within 40px / 60px of live.</t>
         </is>
       </c>
       <c r="E284" s="14" t="inlineStr">
@@ -7389,7 +7389,7 @@
       <c r="A285" s="4" t="n"/>
       <c r="B285" s="4" t="inlineStr">
         <is>
-          <t>Match live's redesigned pages (2026-10-06, owner said go)</t>
+          <t>Sweep leftovers fixed (2026-10-06)</t>
         </is>
       </c>
       <c r="C285" s="13" t="inlineStr">
@@ -7399,7 +7399,7 @@
       </c>
       <c r="D285" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">/self-portrait (live: dark page, progress ring, "N more brushstrokes" lock until 5 assessments), /grant-study and /dharma-finder (live opens straight on question 1, no intro screen), /quiz_25q (live adds a hero picture above the title; rescue it into Sanity first), /search (live: one search box across essays, BrewSoul, peptides, HumanOS, assessments, kava and pages with filter chips). Measure live vs a production build at 375px and 1280px when done. Done 2026-10-06: /grant-study and /dharma-finder open straight on question 1 like live (title block / part header above the first question, live's 546px column, plain page, credit under every question), both rebuilt as step registries (rule 19); measured within 3px of live at the top (dharma's question block within 7px). /quiz_25q's hero rescued into Sanity and placed like live (within 2px). Found and fixed on the way: on the deployed copy /grant-study's answer buttons could not be clicked (the themed page background was fixed z-0, painted over the quiz); ThemedBackground is now -z-10 pointer-events-none (backgrounds unchanged on all 21 pages that use it), and the shared email gate no longer scrolls sideways on phones. Both quizzes clicked through to results in Chrome and Safari. /self-portrait restyled to live (dark page, "The Composite You", progress ring, "N More Brushstrokes Needed" lock until 5 done, live's copy) on our real cookie data; within 3px of live at both widths; tested with 0, 2 and 6 completed. Counts are ours (13 </t>
+          <t>Ported legacy's exact title sizes, margins and column widths. Measured live vs a production build at 375px and 1280px (H1 distance from the top, H1 size, intro and table widths). Now within 8px and the same title size on /published, /brewsoul/first-sip, /brewsoul/home, /brewsoul/chains (intro 912px like live), /brewsoul/browse, /brewsoul/directory (3-column 952px grid like live), /brewsoul and /brewsoul/quiz (intro 520px), /amplifier (546px column), /diamond-cut, /speaking, /living-declaration, /spirits, /protecting-your-business (tables 730px), and the 5 HumanOS subpages (titles smaller like live, 752px column). No sideways scroll at 375px. Left on purpose: /self-portrait (font matches; our page has a different title and no back link, so it sits 23-57px higher), BrewSoul pages 3-6px off (the shared journey bar row), and the different-layout pages /dharma-finder, /grant-study, /search, /quiz_25q, /soulscore. Also: /brewsoul/quiz rebuilt as a step registry (src/components/brewsoul/brewsoul-quiz/: parent + hook/ + components/step-* + data/), same questions, scoring and look; Back/Skip/Retake use lucide icons. New CONTRIBUTING rule 19 (multi-step flows, FydoPartner pattern). brewsoul-welcome-quiz.tsx (/brewsoul) still has the old shape and text arrows.</t>
         </is>
       </c>
       <c r="E285" s="14" t="inlineStr">
@@ -7412,7 +7412,7 @@
       <c r="A286" s="4" t="n"/>
       <c r="B286" s="4" t="inlineStr">
         <is>
-          <t>Still different from live (decided 2026-10-09)</t>
+          <t>Match live's redesigned pages (2026-10-06, owner said go)</t>
         </is>
       </c>
       <c r="C286" s="13" t="inlineStr">
@@ -7422,7 +7422,7 @@
       </c>
       <c r="D286" s="4" t="inlineStr">
         <is>
-          <t>blog posts (done) (done 2026-10-07, see Phase 5); /find-my on live hides the site header. /walk-through is a 404 on live now. Owner: keep our site menu on /find-my (visitors can still reach the rest of the site); nothing left to change.</t>
+          <t xml:space="preserve">/self-portrait (live: dark page, progress ring, "N more brushstrokes" lock until 5 assessments), /grant-study and /dharma-finder (live opens straight on question 1, no intro screen), /quiz_25q (live adds a hero picture above the title; rescue it into Sanity first), /search (live: one search box across essays, BrewSoul, peptides, HumanOS, assessments, kava and pages with filter chips). Measure live vs a production build at 375px and 1280px when done. Done 2026-10-06: /grant-study and /dharma-finder open straight on question 1 like live (title block / part header above the first question, live's 546px column, plain page, credit under every question), both rebuilt as step registries (rule 19); measured within 3px of live at the top (dharma's question block within 7px). /quiz_25q's hero rescued into Sanity and placed like live (within 2px). Found and fixed on the way: on the deployed copy /grant-study's answer buttons could not be clicked (the themed page background was fixed z-0, painted over the quiz); ThemedBackground is now -z-10 pointer-events-none (backgrounds unchanged on all 21 pages that use it), and the shared email gate no longer scrolls sideways on phones. Both quizzes clicked through to results in Chrome and Safari. /self-portrait restyled to live (dark page, "The Composite You", progress ring, "N More Brushstrokes Needed" lock until 5 done, live's copy) on our real cookie data; within 3px of live at both widths; tested with 0, 2 and 6 completed. Counts are ours (13 </t>
         </is>
       </c>
       <c r="E286" s="14" t="inlineStr">
@@ -7435,7 +7435,7 @@
       <c r="A287" s="4" t="n"/>
       <c r="B287" s="4" t="inlineStr">
         <is>
-          <t>Design change on live (owner: "match live", 2026-10-09)</t>
+          <t>Still different from live (decided 2026-10-09)</t>
         </is>
       </c>
       <c r="C287" s="13" t="inlineStr">
@@ -7445,7 +7445,7 @@
       </c>
       <c r="D287" s="4" t="inlineStr">
         <is>
-          <t>live's story pages now use Cormorant Garamond for titles (ours: Playfair Display), a lighter title weight (400 vs our 700), and a red eyebrow label (#8E1E25, wider letter spacing) instead of our gold. A site-wide font swap is a design call, so not done. Done 2026-10-09: a fresh sweep of 163 live pages found live has since dropped Cormorant from the story pages (only /living-declaration uses it, ours already matched) and mostly uses Playfair; the real differences were fixed: every heading on /attention-theft in Fraunces 700 (section-wide, like Kava), /supplier-intake title in the system serif, and live's fluid title sizes on /about, /articles, /the-letter, /the-philosophy, /clock-keeper-part-2, /living-declaration (measured at 375/640/820/1024/1280, now identical). Label colours stay darker than live on purpose (contrast, rule 20).</t>
+          <t>blog posts (done) (done 2026-10-07, see Phase 5); /find-my on live hides the site header. /walk-through is a 404 on live now. Owner: keep our site menu on /find-my (visitors can still reach the rest of the site); nothing left to change.</t>
         </is>
       </c>
       <c r="E287" s="14" t="inlineStr">
@@ -7458,7 +7458,7 @@
       <c r="A288" s="4" t="n"/>
       <c r="B288" s="4" t="inlineStr">
         <is>
-          <t>Link check across all ported pages (no 404s, no broken internal cross-references)</t>
+          <t>Design change on live (owner: "match live", 2026-10-09)</t>
         </is>
       </c>
       <c r="C288" s="13" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="D288" s="4" t="inlineStr">
         <is>
-          <t>First full pass done 2026-09-29 (510 pages crawled from the sitemap plus every internal link, on a production build). Fixed in code: /brewsoul/coffee/…-tarrazú 404 (the route got the id still percent-encoded), 30+ links that went through the /assessments/* redirects, /find-your-me's dead Homeaglow link, the two root-level Iboga essay links, and the dead FauxTony nav item. Fixed as Sanity drafts (scripts/fix-blog-body-links.ts, 14 posts): broken post links, leaked !… placeholder text, Energy Is Money's split author bio, and scraped WordPress furniture ("Share this / Related / You Might Also Like / Copyright", "Show More / Top News", [mc4wp_form]). Left for a decision: /framework's "Ask FauxTony" button, when-healing-becomes-extraction's two links to a Dr. Lee case file that doesn't exist, and the-clock-keeper-chronicles-part-1's link to the deferred /clock-keeper-part-2. Re-run after the drafts are published. 2026-10-01 re-run (local production build, all 498 sitemap URLs load; 440 unique internal links): 5 broken. Fixed as a Sanity draft: molecule-as-mirror-10-what-the-pioneers-know's "Final installment" link pointed at a non-existent part-10 slug (now part 11; live also shows that line twice, kept). Already fixed in a waiting draft: forever-chemicals-... → /blog/psychedelic-readiness-index. Still the 3 known decisions: /fauxtony (from /framework), /clock-keeper-part-2, /blog/the-case-file-dr-samuel-lee. 2026-10-08 re-run (production build, all 497 sitemap pages, 453 unique i</t>
+          <t>live's story pages now use Cormorant Garamond for titles (ours: Playfair Display), a lighter title weight (400 vs our 700), and a red eyebrow label (#8E1E25, wider letter spacing) instead of our gold. A site-wide font swap is a design call, so not done. Done 2026-10-09: a fresh sweep of 163 live pages found live has since dropped Cormorant from the story pages (only /living-declaration uses it, ours already matched) and mostly uses Playfair; the real differences were fixed: every heading on /attention-theft in Fraunces 700 (section-wide, like Kava), /supplier-intake title in the system serif, and live's fluid title sizes on /about, /articles, /the-letter, /the-philosophy, /clock-keeper-part-2, /living-declaration (measured at 375/640/820/1024/1280, now identical). Label colours stay darker than live on purpose (contrast, rule 20).</t>
         </is>
       </c>
       <c r="E288" s="14" t="inlineStr">
@@ -7481,7 +7481,7 @@
       <c r="A289" s="4" t="n"/>
       <c r="B289" s="4" t="inlineStr">
         <is>
-          <t>Sitemap: no noindex pages (2026-10-08)</t>
+          <t>Link check across all ported pages (no 404s, no broken internal cross-references)</t>
         </is>
       </c>
       <c r="C289" s="13" t="inlineStr">
@@ -7491,7 +7491,7 @@
       </c>
       <c r="D289" s="4" t="inlineStr">
         <is>
-          <t>the password-locked /blog/you-are-the-moat was in the sitemap while telling Google not to index it (a Search Console sitemap warning). Gated posts and posts that redirect are now left out (src/app/sitemap.ts); all 497 sitemap addresses return 200 with a matching canonical and no noindex. The 82 warnings Search Console shows are for the old live sitemap, so re-check them after cutover.</t>
+          <t>First full pass done 2026-09-29 (510 pages crawled from the sitemap plus every internal link, on a production build). Fixed in code: /brewsoul/coffee/…-tarrazú 404 (the route got the id still percent-encoded), 30+ links that went through the /assessments/* redirects, /find-your-me's dead Homeaglow link, the two root-level Iboga essay links, and the dead FauxTony nav item. Fixed as Sanity drafts (scripts/fix-blog-body-links.ts, 14 posts): broken post links, leaked !… placeholder text, Energy Is Money's split author bio, and scraped WordPress furniture ("Share this / Related / You Might Also Like / Copyright", "Show More / Top News", [mc4wp_form]). Left for a decision: /framework's "Ask FauxTony" button, when-healing-becomes-extraction's two links to a Dr. Lee case file that doesn't exist, and the-clock-keeper-chronicles-part-1's link to the deferred /clock-keeper-part-2. Re-run after the drafts are published. 2026-10-01 re-run (local production build, all 498 sitemap URLs load; 440 unique internal links): 5 broken. Fixed as a Sanity draft: molecule-as-mirror-10-what-the-pioneers-know's "Final installment" link pointed at a non-existent part-10 slug (now part 11; live also shows that line twice, kept). Already fixed in a waiting draft: forever-chemicals-... → /blog/psychedelic-readiness-index. Still the 3 known decisions: /fauxtony (from /framework), /clock-keeper-part-2, /blog/the-case-file-dr-samuel-lee. 2026-10-08 re-run (production build, all 497 sitemap pages, 453 unique i</t>
         </is>
       </c>
       <c r="E289" s="14" t="inlineStr">
@@ -7504,7 +7504,7 @@
       <c r="A290" s="4" t="n"/>
       <c r="B290" s="4" t="inlineStr">
         <is>
-          <t>Lighthouse pass (performance/accessibility/SEO) on top 20 pages by traffic 2026-09-30, 20 key pages (no traffic data yet), local production …</t>
+          <t>Sitemap: no noindex pages (2026-10-08)</t>
         </is>
       </c>
       <c r="C290" s="13" t="inlineStr">
@@ -7514,7 +7514,7 @@
       </c>
       <c r="D290" s="4" t="inlineStr">
         <is>
-          <t>build, mobile: averages performance 87, accessibility 99→100, best practices 100, SEO 92→100, CLS 0 everywhere. Fixed: public/robots.txt had an LLMs: line (not a real directive) that made Google treat the whole file as invalid, now a comment; h3/h4 headings skipping a level on /assessments, /kava, /peptide-watch (same look, right tag); the Kava and /attention-theft back-arrow links had no accessible name on phones; two small phone-width contrast misses. Left: performance is local-machine only (±10-15 points, see CONTRIBUTING.md); the slowest were / 76 (LCP 5.2 s), /psychedelic-readiness-index 82, /iboga-ibogaine 83. Re-run against the Netlify deploy before launch. 2026-10-06 re-run against the Netlify deploy (14 key pages, mobile): accessibility 100 and CLS 0 on every page, SEO clean (only the expected netlify.app noindex), performance 77-97 held back by 3-4 s LCP. Fixed: all 21 hero images moved off the deprecated priority prop to fetchPriority="high" + loading="eager" (Next 16); /iboga-ibogaine hero and the first card on /blog and category pages no longer lazy-loaded; sizes on the Four Doors cards (~150 KiB per page), /humanos diagram (~100 KiB) and /about headshot; urlFor no longer imports the Sanity client, so ~115 KB of Sanity client code stopped loading on / and /blog; React hydration error #418 on / and /blog (post dates) gone, checked in two time zones; /blog is static again; empty icon &lt;th&gt;s on /iboga-ibogaine labelled; category page reads use sanityFetch(). Left: se</t>
+          <t>the password-locked /blog/you-are-the-moat was in the sitemap while telling Google not to index it (a Search Console sitemap warning). Gated posts and posts that redirect are now left out (src/app/sitemap.ts); all 497 sitemap addresses return 200 with a matching canonical and no noindex. The 82 warnings Search Console shows are for the old live sitemap, so re-check them after cutover.</t>
         </is>
       </c>
       <c r="E290" s="14" t="inlineStr">
@@ -7527,7 +7527,7 @@
       <c r="A291" s="4" t="n"/>
       <c r="B291" s="4" t="inlineStr">
         <is>
-          <t>No Manus links anywhere (2026-10-09, owner: "drop them everywhere")</t>
+          <t>Lighthouse pass (performance/accessibility/SEO) on top 20 pages by traffic 2026-09-30, 20 key pages (no traffic data yet), local production …</t>
         </is>
       </c>
       <c r="C291" s="13" t="inlineStr">
@@ -7537,7 +7537,7 @@
       </c>
       <c r="D291" s="4" t="inlineStr">
         <is>
-          <t>every *.manus.space link removed from code and essays. Lists of "try this next" apps lose those entries (journey tracker, Find Your Me results and next steps, /find-my, search directory, Sake and Grant Study results, BrewSoul footer, The Mirror); The Magnetic Partner's and The Temple Keeper's next step now go to their first in-site assessment (/grant-study, /consciousness-scale); their empty "Find Your _" section hides itself; /recent-creations, /spirits and /ecosystem-map keep the cards, unlinked. Clarisse Abelarde now links to her own site clarisseartist.com (owner gave it) on /about and in essays. Essays: lib/sanity/portable-text.tsx rewrites tonygreenberg.manus.space/&lt;path&gt; to /&lt;path&gt;, clarisseart.manus.space to clarisseartist.com (same paths), and renders other Manus app links as plain text (no Sanity drafts). Verified on a production build: no clickable *.manus.space link in any page, no manus.space in any browser script; 13 affected pages load (200).</t>
+          <t>build, mobile: averages performance 87, accessibility 99→100, best practices 100, SEO 92→100, CLS 0 everywhere. Fixed: public/robots.txt had an LLMs: line (not a real directive) that made Google treat the whole file as invalid, now a comment; h3/h4 headings skipping a level on /assessments, /kava, /peptide-watch (same look, right tag); the Kava and /attention-theft back-arrow links had no accessible name on phones; two small phone-width contrast misses. Left: performance is local-machine only (±10-15 points, see CONTRIBUTING.md); the slowest were / 76 (LCP 5.2 s), /psychedelic-readiness-index 82, /iboga-ibogaine 83. Re-run against the Netlify deploy before launch. 2026-10-06 re-run against the Netlify deploy (14 key pages, mobile): accessibility 100 and CLS 0 on every page, SEO clean (only the expected netlify.app noindex), performance 77-97 held back by 3-4 s LCP. Fixed: all 21 hero images moved off the deprecated priority prop to fetchPriority="high" + loading="eager" (Next 16); /iboga-ibogaine hero and the first card on /blog and category pages no longer lazy-loaded; sizes on the Four Doors cards (~150 KiB per page), /humanos diagram (~100 KiB) and /about headshot; urlFor no longer imports the Sanity client, so ~115 KB of Sanity client code stopped loading on / and /blog; React hydration error #418 on / and /blog (post dates) gone, checked in two time zones; /blog is static again; empty icon &lt;th&gt;s on /iboga-ibogaine labelled; category page reads use sanityFetch(). Left: se</t>
         </is>
       </c>
       <c r="E291" s="14" t="inlineStr">
@@ -7550,7 +7550,7 @@
       <c r="A292" s="4" t="n"/>
       <c r="B292" s="4" t="inlineStr">
         <is>
-          <t>Owner answers, round 2 (2026-10-09)</t>
+          <t>No Manus links anywhere (2026-10-09, owner: "drop them everywhere")</t>
         </is>
       </c>
       <c r="C292" s="13" t="inlineStr">
@@ -7560,7 +7560,7 @@
       </c>
       <c r="D292" s="4" t="inlineStr">
         <is>
-          <t>(1) real counts instead of live's typed numbers: /charity-scorecard intro and description ("98"/"Ninety-eight" → STATS.totalCharities = 103), /impact-dashboard ("100" → passed in from the page so the browser doesn't load the charity list), /the-index (prop), search directory coffees 103 → 107 (typed, with a note, since it ships to the search pop-up); (2) The Mirror results no longer list the 4 *.manus.space apps (the "Explore further" section hides when empty); (3) /framework's "Ask FauxTony" button and its lead-in line removed; the Dr. Lee case-file link (4 places in when-healing-becomes-extraction, original and updated versions) renders as plain text through a DEAD_INTERNAL_LINKS list in lib/sanity/portable-text.tsx (no Sanity draft needed); (4) B Corp: checked live, nothing shown on either site, no change. Verified on a production build: the counts read 103, /framework has no FauxTony block, the essay has 0 links to the case file and keeps the words, /the-index shows "103 charities" when searching "charity".</t>
+          <t>every *.manus.space link removed from code and essays. Lists of "try this next" apps lose those entries (journey tracker, Find Your Me results and next steps, /find-my, search directory, Sake and Grant Study results, BrewSoul footer, The Mirror); The Magnetic Partner's and The Temple Keeper's next step now go to their first in-site assessment (/grant-study, /consciousness-scale); their empty "Find Your _" section hides itself; /recent-creations, /spirits and /ecosystem-map keep the cards, unlinked. Clarisse Abelarde now links to her own site clarisseartist.com (owner gave it) on /about and in essays. Essays: lib/sanity/portable-text.tsx rewrites tonygreenberg.manus.space/&lt;path&gt; to /&lt;path&gt;, clarisseart.manus.space to clarisseartist.com (same paths), and renders other Manus app links as plain text (no Sanity drafts). Verified on a production build: no clickable *.manus.space link in any page, no manus.space in any browser script; 13 affected pages load (200).</t>
         </is>
       </c>
       <c r="E292" s="14" t="inlineStr">
@@ -7573,7 +7573,7 @@
       <c r="A293" s="4" t="n"/>
       <c r="B293" s="4" t="inlineStr">
         <is>
-          <t>Arrows in buttons and links are icons (2026-10-09, owner said yes)</t>
+          <t>Owner answers, round 2 (2026-10-09)</t>
         </is>
       </c>
       <c r="C293" s="13" t="inlineStr">
@@ -7583,7 +7583,7 @@
       </c>
       <c r="D293" s="4" t="inlineStr">
         <is>
-          <t>113 typed arrows in 52 files (button and link labels, "Next"/"See My Results" toggles, decorative arrow spans, the walk-through "See the..." labels, the Letter's "I'm in" button) replaced with lucide ArrowRight/ArrowLeft (size-[1em], inside inline-flex items-center gap-1.5, so the parent layout is untouched). Left as content on purpose: arrows inside Tony's text and data (health findings, origins, iboga compass options, process flows like "Inherit → Wake → Choose → Act", share text), the "← you" marker on the consciousness scale, and &lt;option&gt; sort labels (an option can't hold an icon). Checked on 16 pages at 375 and 1280: no typed arrow left in any link or button, no sideways scroll, no JS errors; close-up screenshots of the new icons.</t>
+          <t>(1) real counts instead of live's typed numbers: /charity-scorecard intro and description ("98"/"Ninety-eight" → STATS.totalCharities = 103), /impact-dashboard ("100" → passed in from the page so the browser doesn't load the charity list), /the-index (prop), search directory coffees 103 → 107 (typed, with a note, since it ships to the search pop-up); (2) The Mirror results no longer list the 4 *.manus.space apps (the "Explore further" section hides when empty); (3) /framework's "Ask FauxTony" button and its lead-in line removed; the Dr. Lee case-file link (4 places in when-healing-becomes-extraction, original and updated versions) renders as plain text through a DEAD_INTERNAL_LINKS list in lib/sanity/portable-text.tsx (no Sanity draft needed); (4) B Corp: checked live, nothing shown on either site, no change. Verified on a production build: the counts read 103, /framework has no FauxTony block, the essay has 0 links to the case file and keeps the words, /the-index shows "103 charities" when searching "charity".</t>
         </is>
       </c>
       <c r="E293" s="14" t="inlineStr">
@@ -7596,7 +7596,7 @@
       <c r="A294" s="4" t="n"/>
       <c r="B294" s="4" t="inlineStr">
         <is>
-          <t>Category pages pre-built (2026-10-09)</t>
+          <t>Arrows in buttons and links are icons (2026-10-09, owner said yes)</t>
         </is>
       </c>
       <c r="C294" s="13" t="inlineStr">
@@ -7606,7 +7606,7 @@
       </c>
       <c r="D294" s="4" t="inlineStr">
         <is>
-          <t>/blog/category/[slug] read ?page=N, so every category page was rendered on each request (slower first byte, flagged in the Lighthouse notes). Page numbers are now part of the address (/blog/category/&lt;slug&gt;/page/&lt;n&gt;, generateStaticParams, dynamicParams = false), shared code in src/components/blog/category-listing.tsx; old ?page=N links 308 to the new address (pages 2+ only, so no loop), /page/1 308s to the plain address, a page past the end is a 404; "All essays" back link uses an icon. Verified on a production build: route table shows every category page as pre-built (9 page-1s, 7 later pages), titles and canonicals per page, Previous/Next links, the redirects and the 404s.</t>
+          <t>113 typed arrows in 52 files (button and link labels, "Next"/"See My Results" toggles, decorative arrow spans, the walk-through "See the..." labels, the Letter's "I'm in" button) replaced with lucide ArrowRight/ArrowLeft (size-[1em], inside inline-flex items-center gap-1.5, so the parent layout is untouched). Left as content on purpose: arrows inside Tony's text and data (health findings, origins, iboga compass options, process flows like "Inherit → Wake → Choose → Act", share text), the "← you" marker on the consciousness scale, and &lt;option&gt; sort labels (an option can't hold an icon). Checked on 16 pages at 375 and 1280: no typed arrow left in any link or button, no sideways scroll, no JS errors; close-up screenshots of the new icons.</t>
         </is>
       </c>
       <c r="E294" s="14" t="inlineStr">
@@ -7619,7 +7619,7 @@
       <c r="A295" s="4" t="n"/>
       <c r="B295" s="4" t="inlineStr">
         <is>
-          <t>Error pages (2026-10-09, owner asked)</t>
+          <t>Category pages pre-built (2026-10-09)</t>
         </is>
       </c>
       <c r="C295" s="13" t="inlineStr">
@@ -7629,7 +7629,7 @@
       </c>
       <c r="D295" s="4" t="inlineStr">
         <is>
-          <t>404 page now sets its own title ("Page not found") as a server page around live's 3-second redirect (not-found.tsx + components/not-found-redirect.tsx), arrow as an icon; page error screen (error.tsx) uses Next 16's retry (re-fetches), shows a reference code for the server logs, links home and to the site index; new global-error.tsx for failures in the root layout itself (own &lt;html&gt;, plain links). Verified on a production build: missing page, missing essay and missing Kava page return 404 with the right title; a test page that throws returns 500 with the error screen, "Try again" re-fetches; phone and laptop, no sideways scroll (test page removed).</t>
+          <t>/blog/category/[slug] read ?page=N, so every category page was rendered on each request (slower first byte, flagged in the Lighthouse notes). Page numbers are now part of the address (/blog/category/&lt;slug&gt;/page/&lt;n&gt;, generateStaticParams, dynamicParams = false), shared code in src/components/blog/category-listing.tsx; old ?page=N links 308 to the new address (pages 2+ only, so no loop), /page/1 308s to the plain address, a page past the end is a 404; "All essays" back link uses an icon. Verified on a production build: route table shows every category page as pre-built (9 page-1s, 7 later pages), titles and canonicals per page, Previous/Next links, the redirects and the 404s.</t>
         </is>
       </c>
       <c r="E295" s="14" t="inlineStr">
@@ -7642,7 +7642,7 @@
       <c r="A296" s="4" t="n"/>
       <c r="B296" s="4" t="inlineStr">
         <is>
-          <t>SEO audit fixes (2026-10-06)</t>
+          <t>Error pages (2026-10-09, owner asked)</t>
         </is>
       </c>
       <c r="C296" s="13" t="inlineStr">
@@ -7652,7 +7652,7 @@
       </c>
       <c r="D296" s="4" t="inlineStr">
         <is>
-          <t>Checked an outside audit point by point against the code. Fixed: Core Themes cards linked to /?theme=…#essays-archive (not crawlable, counts from a stale hand-kept list) and now link to /blog/category/&lt;slug&gt; with real counts (21/25/20/14, matching the archive pills; THEME_MAP and the ?theme= filter removed); Four Doors cards were &lt;button&gt;s, now real links that still open the modal on a plain click; "DIAGNOSE · ENGAGE" now link to /find-my and /engage; one shared formatPostDate (Asia/Kolkata, src/lib/format-post-date.ts) so a post no longer shows two different dates; the title repeated as the first body paragraph is dropped at render time (legacyBodyLayout); essay cards are h3 under a section h2 (archive, Read next), h2 only on category/search; heading glyphs (◆ ✦) hidden from screen readers; posts send BlogPosting with the author tied to the site Person (@id) plus a BreadcrumbList; descriptive alt on the homepage and BrewSoul heroes; homepage OG image cropped to 1200x630 JPEG. Already fine (audit could not see it): Person/Article schema, Netlify noindex, robots.txt, sitemap, header nav and search, Amazon links carry no affiliate tag. Checked on a production build: type check, lint, build, status codes, browser click test at 375px, no console errors. Implementation pack (Mohammad Danish, 2026-10-05) checked the same day: added og:type/og:site_name back on the 6 pages with their own openGraph (a page-level openGraph replaces the layout one), twitter:creator, and on posts og:url</t>
+          <t>404 page now sets its own title ("Page not found") as a server page around live's 3-second redirect (not-found.tsx + components/not-found-redirect.tsx), arrow as an icon; page error screen (error.tsx) uses Next 16's retry (re-fetches), shows a reference code for the server logs, links home and to the site index; new global-error.tsx for failures in the root layout itself (own &lt;html&gt;, plain links). Verified on a production build: missing page, missing essay and missing Kava page return 404 with the right title; a test page that throws returns 500 with the error screen, "Try again" re-fetches; phone and laptop, no sideways scroll (test page removed).</t>
         </is>
       </c>
       <c r="E296" s="14" t="inlineStr">
@@ -7665,7 +7665,7 @@
       <c r="A297" s="4" t="n"/>
       <c r="B297" s="4" t="inlineStr">
         <is>
-          <t>SEO audit items needing a yes (2026-10-06; owner said yes to the copy 2026-10-10, done)</t>
+          <t>SEO audit fixes (2026-10-06)</t>
         </is>
       </c>
       <c r="C297" s="13" t="inlineStr">
@@ -7675,7 +7675,7 @@
       </c>
       <c r="D297" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">the pack's new copy (homepage title/description, five-cups title, description, short answer, FAQ, heading rewrites, entity statement, newsletter block, author box, health disclaimer, COA wording); "Further Reading" shown twice on posts (merge the lists?); long post title (84 chars), homepage description length and obsolete keywords tag, slugs (/blog/five-cups, the -2 slug; would need redirects), "Six lenses" over four cards, sources for health claims and proof for "$10B+", "Certified B Corp", "Validity: 91", legal review of the homepage Case File banner, ABIT waitlist disclosures, one contact email, the two one-post categories, fewer homepage CTAs / email signup / table of contents / explaining "COA". Done 2026-10-10: homepage title "Tony Greenberg | Strategist, Author &amp; CEO of RampRate" and description (essay count computed: 123); entity statement under the hero (107 coffees / 100 chains computed from the data) with a link to /ecosystem; door 4 "Certificate of Analysis (COA) checks, lab testing and vendor scoring"; "Four lenses" (computed); newsletter box after Editor's Picks (existing Kit form); meta keywords removed site-wide; every essay: author line + "About Tony", one merged "Further Reading", optional lastUpdated field shown as "Updated &lt;date&gt;" (not set on any post yet: every _updatedAt is the import date), health disclaimer on 20 personal-health essays (chosen by Sanity tag); Five Cups (Sanity, published, backup kept): SEO title/description, short answer, visible FAQ </t>
+          <t>Checked an outside audit point by point against the code. Fixed: Core Themes cards linked to /?theme=…#essays-archive (not crawlable, counts from a stale hand-kept list) and now link to /blog/category/&lt;slug&gt; with real counts (21/25/20/14, matching the archive pills; THEME_MAP and the ?theme= filter removed); Four Doors cards were &lt;button&gt;s, now real links that still open the modal on a plain click; "DIAGNOSE · ENGAGE" now link to /find-my and /engage; one shared formatPostDate (Asia/Kolkata, src/lib/format-post-date.ts) so a post no longer shows two different dates; the title repeated as the first body paragraph is dropped at render time (legacyBodyLayout); essay cards are h3 under a section h2 (archive, Read next), h2 only on category/search; heading glyphs (◆ ✦) hidden from screen readers; posts send BlogPosting with the author tied to the site Person (@id) plus a BreadcrumbList; descriptive alt on the homepage and BrewSoul heroes; homepage OG image cropped to 1200x630 JPEG. Already fine (audit could not see it): Person/Article schema, Netlify noindex, robots.txt, sitemap, header nav and search, Amazon links carry no affiliate tag. Checked on a production build: type check, lint, build, status codes, browser click test at 375px, no console errors. Implementation pack (Mohammad Danish, 2026-10-05) checked the same day: added og:type/og:site_name back on the 6 pages with their own openGraph (a page-level openGraph replaces the layout one), twitter:creator, and on posts og:url</t>
         </is>
       </c>
       <c r="E297" s="14" t="inlineStr">
@@ -7688,7 +7688,7 @@
       <c r="A298" s="4" t="n"/>
       <c r="B298" s="4" t="inlineStr">
         <is>
-          <t>Google Analytics tag (found missing 2026-10-10, added the same day)</t>
+          <t>SEO audit items needing a yes (2026-10-06; owner said yes to the copy 2026-10-10, done)</t>
         </is>
       </c>
       <c r="C298" s="13" t="inlineStr">
@@ -7698,7 +7698,7 @@
       </c>
       <c r="D298" s="4" t="inlineStr">
         <is>
-          <t>Live loads GA4 G-4GVW40S47N; the new site sent nothing, so stats would have stopped at cutover. Added src/components/google-analytics.tsx (plain next/script, no new package) in the root layout; it only runs on tonygreenberg.com / www, so Netlify previews and localhost never reach the real reports. Checked: type check, lint, build; in Chromium with Google's requests blocked: localhost sends nothing, tonygreenberg.com (mapped to a local production build) loads the tag on / and /find-your-coffee, no JS errors. In-site page changes are counted by GA4's Enhanced measurement (on by default; confirm in GA4 &gt; Admin &gt; Data streams on launch day).</t>
+          <t xml:space="preserve">the pack's new copy (homepage title/description, five-cups title, description, short answer, FAQ, heading rewrites, entity statement, newsletter block, author box, health disclaimer, COA wording); "Further Reading" shown twice on posts (merge the lists?); long post title (84 chars), homepage description length and obsolete keywords tag, slugs (/blog/five-cups, the -2 slug; would need redirects), "Six lenses" over four cards, sources for health claims and proof for "$10B+", "Certified B Corp", "Validity: 91", legal review of the homepage Case File banner, ABIT waitlist disclosures, one contact email, the two one-post categories, fewer homepage CTAs / email signup / table of contents / explaining "COA". Done 2026-10-10: homepage title "Tony Greenberg | Strategist, Author &amp; CEO of RampRate" and description (essay count computed: 123); entity statement under the hero (107 coffees / 100 chains computed from the data) with a link to /ecosystem; door 4 "Certificate of Analysis (COA) checks, lab testing and vendor scoring"; "Four lenses" (computed); newsletter box after Editor's Picks (existing Kit form); meta keywords removed site-wide; every essay: author line + "About Tony", one merged "Further Reading", optional lastUpdated field shown as "Updated &lt;date&gt;" (not set on any post yet: every _updatedAt is the import date), health disclaimer on 20 personal-health essays (chosen by Sanity tag); Five Cups (Sanity, published, backup kept): SEO title/description, short answer, visible FAQ </t>
         </is>
       </c>
       <c r="E298" s="14" t="inlineStr">
@@ -7711,7 +7711,7 @@
       <c r="A299" s="4" t="n"/>
       <c r="B299" s="4" t="inlineStr">
         <is>
-          <t>Old site's custom GA4 events ported (2026-10-10, owner asked to match legacy's Google tags)</t>
+          <t>Google Analytics tag (found missing 2026-10-10, added the same day)</t>
         </is>
       </c>
       <c r="C299" s="13" t="inlineStr">
@@ -7721,7 +7721,7 @@
       </c>
       <c r="D299" s="4" t="inlineStr">
         <is>
-          <t>Legacy loaded GA4 G-4GVW40S47N (already on the new site), Manus's own Umami counter (gone with Manus, not portable) and custom events from ConversionMechanics.tsx's AnalyticsTracker. Now src/components/ga-events.tsx (root layout) sends the same names: article_/page_25/50/75/90_scroll, engaged_45_seconds, second_page_view, homepage_path_work/_thinking/_building, start_here_open. Legacy's extra page_view on every history change is not ported (GA4 Enhanced measurement already counts in-site page changes; it would double-count). Tested in Chromium with Google's requests blocked: tonygreenberg.com (mapped to a local build) fired the homepage path and all four essay scroll events plus second_page_view; localhost loads no tag. A RampRate-style weekly report / hourly alert email and an admin analytics page were built the same day and removed at the owner's request (they use the Looker Studio report instead); the empty report_runs table and CRON_SECRET were removed too.</t>
+          <t>Live loads GA4 G-4GVW40S47N; the new site sent nothing, so stats would have stopped at cutover. Added src/components/google-analytics.tsx (plain next/script, no new package) in the root layout; it only runs on tonygreenberg.com / www, so Netlify previews and localhost never reach the real reports. Checked: type check, lint, build; in Chromium with Google's requests blocked: localhost sends nothing, tonygreenberg.com (mapped to a local production build) loads the tag on / and /find-your-coffee, no JS errors. In-site page changes are counted by GA4's Enhanced measurement (on by default; confirm in GA4 &gt; Admin &gt; Data streams on launch day).</t>
         </is>
       </c>
       <c r="E299" s="14" t="inlineStr">
@@ -7734,15 +7734,19 @@
       <c r="A300" s="4" t="n"/>
       <c r="B300" s="4" t="inlineStr">
         <is>
-          <t>Connect Google Search Console + GA4 to the new deployment on day one of cutover</t>
-        </is>
-      </c>
-      <c r="C300" s="16" t="inlineStr">
-        <is>
-          <t>Remaining</t>
-        </is>
-      </c>
-      <c r="D300" s="4" t="inlineStr"/>
+          <t>Old site's custom GA4 events ported (2026-10-10, owner asked to match legacy's Google tags)</t>
+        </is>
+      </c>
+      <c r="C300" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D300" s="4" t="inlineStr">
+        <is>
+          <t>Legacy loaded GA4 G-4GVW40S47N (already on the new site), Manus's own Umami counter (gone with Manus, not portable) and custom events from ConversionMechanics.tsx's AnalyticsTracker. Now src/components/ga-events.tsx (root layout) sends the same names: article_/page_25/50/75/90_scroll, engaged_45_seconds, second_page_view, homepage_path_work/_thinking/_building, start_here_open. Legacy's extra page_view on every history change is not ported (GA4 Enhanced measurement already counts in-site page changes; it would double-count). Tested in Chromium with Google's requests blocked: tonygreenberg.com (mapped to a local build) fired the homepage path and all four essay scroll events plus second_page_view; localhost loads no tag. A RampRate-style weekly report / hourly alert email and an admin analytics page were built the same day and removed at the owner's request (they use the Looker Studio report instead); the empty report_runs table and CRON_SECRET were removed too.</t>
+        </is>
+      </c>
       <c r="E300" s="14" t="inlineStr">
         <is>
           <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
@@ -7753,19 +7757,15 @@
       <c r="A301" s="4" t="n"/>
       <c r="B301" s="4" t="inlineStr">
         <is>
-          <t>Restore/adapt the manus.space triple-layer noindex lockdown pattern for any remaining staging URLs</t>
-        </is>
-      </c>
-      <c r="C301" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D301" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-01: the Netlify copy (tonygreenberg-website.netlify.app) and every deploy preview had no noindex at all, so Google could index a duplicate of the site. next.config.ts headers() now sends X-Robots-Tag: noindex, nofollow on any *.netlify.app host only; tonygreenberg.com is unaffected, so nothing to remove at cutover. Tested with Host headers on a production build.</t>
-        </is>
-      </c>
+          <t>Connect Google Search Console + GA4 to the new deployment on day one of cutover</t>
+        </is>
+      </c>
+      <c r="C301" s="16" t="inlineStr">
+        <is>
+          <t>Remaining</t>
+        </is>
+      </c>
+      <c r="D301" s="4" t="inlineStr"/>
       <c r="E301" s="14" t="inlineStr">
         <is>
           <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
@@ -7776,7 +7776,7 @@
       <c r="A302" s="4" t="n"/>
       <c r="B302" s="4" t="inlineStr">
         <is>
-          <t>"Keep going" strip above the footer on every page (2026-10-07)</t>
+          <t>Restore/adapt the manus.space triple-layer noindex lockdown pattern for any remaining staging URLs</t>
         </is>
       </c>
       <c r="C302" s="13" t="inlineStr">
@@ -7786,7 +7786,7 @@
       </c>
       <c r="D302" s="4" t="inlineStr">
         <is>
-          <t>legacy's WhereNext (deferred in Phase 3, never picked up) with its per-page suggestions, Home · Site Index · All Assessments; links pointed at current routes.</t>
+          <t>2026-10-01: the Netlify copy (tonygreenberg-website.netlify.app) and every deploy preview had no noindex at all, so Google could index a duplicate of the site. next.config.ts headers() now sends X-Robots-Tag: noindex, nofollow on any *.netlify.app host only; tonygreenberg.com is unaffected, so nothing to remove at cutover. Tested with Host headers on a production build.</t>
         </is>
       </c>
       <c r="E302" s="14" t="inlineStr">
@@ -7799,7 +7799,7 @@
       <c r="A303" s="4" t="n"/>
       <c r="B303" s="4" t="inlineStr">
         <is>
-          <t>Live-only and redesigned pages from the 2026-10-07 page sweep (188 pages compared with live)</t>
+          <t>"Keep going" strip above the footer on every page (2026-10-07)</t>
         </is>
       </c>
       <c r="C303" s="13" t="inlineStr">
@@ -7809,7 +7809,7 @@
       </c>
       <c r="D303" s="4" t="inlineStr">
         <is>
-          <t>/the-index rebuilt from live's code (20 concepts, related-word search across essays and site pages, full-text search on the server, "three related places to go next"; the old redirect to /search removed and its links, including the "Site Index" link in "Keep going", point at it again); /the-mirror (and /life-assessment) opens on live's intro (dark hero, "What We Measure" with the six areas, "The Ecosystem"), rebuilt as a step registry (rule 19); /essays header, order and column like live; /about "What They Say" styled like live (live picks 3 of the same 19 quotes at random; ours shows a fixed 3 so they're in the server HTML); /impact-futurism list titles and subtitles; /supplier-intake is a real page again with live's Stage 1 form; /seven-doors and /projects redirect home like live; /impact, /health, /library, /built-on-manus, /heroes are 404 on live too. Left as is on purpose: /blog stays our archive page (on live it repeats the homepage), the email gates on /framework and /peptide-supply-chain, the attention-theft Wall of Shame.</t>
+          <t>legacy's WhereNext (deferred in Phase 3, never picked up) with its per-page suggestions, Home · Site Index · All Assessments; links pointed at current routes.</t>
         </is>
       </c>
       <c r="E303" s="14" t="inlineStr">
@@ -7822,7 +7822,7 @@
       <c r="A304" s="4" t="n"/>
       <c r="B304" s="4" t="inlineStr">
         <is>
-          <t>/alex-azzi locked like live (2026-10-07, owner said match it)</t>
+          <t>Live-only and redesigned pages from the 2026-10-07 page sweep (188 pages compared with live)</t>
         </is>
       </c>
       <c r="C304" s="13" t="inlineStr">
@@ -7832,7 +7832,7 @@
       </c>
       <c r="D304" s="4" t="inlineStr">
         <is>
-          <t>same server-checked password as the locked essay (GATED_POST_PASSWORD, now also set in Netlify), live's "Restricted Access" screen, the report not in the page until unlocked, out of search and the sitemap.</t>
+          <t>/the-index rebuilt from live's code (20 concepts, related-word search across essays and site pages, full-text search on the server, "three related places to go next"; the old redirect to /search removed and its links, including the "Site Index" link in "Keep going", point at it again); /the-mirror (and /life-assessment) opens on live's intro (dark hero, "What We Measure" with the six areas, "The Ecosystem"), rebuilt as a step registry (rule 19); /essays header, order and column like live; /about "What They Say" styled like live (live picks 3 of the same 19 quotes at random; ours shows a fixed 3 so they're in the server HTML); /impact-futurism list titles and subtitles; /supplier-intake is a real page again with live's Stage 1 form; /seven-doors and /projects redirect home like live; /impact, /health, /library, /built-on-manus, /heroes are 404 on live too. Left as is on purpose: /blog stays our archive page (on live it repeats the homepage), the email gates on /framework and /peptide-supply-chain, the attention-theft Wall of Shame.</t>
         </is>
       </c>
       <c r="E304" s="14" t="inlineStr">
@@ -7845,7 +7845,7 @@
       <c r="A305" s="4" t="n"/>
       <c r="B305" s="4" t="inlineStr">
         <is>
-          <t>Live's title fonts and sizes (2026-10-07, "fix the style")</t>
+          <t>/alex-azzi locked like live (2026-10-07, owner said match it)</t>
         </is>
       </c>
       <c r="C305" s="13" t="inlineStr">
@@ -7855,7 +7855,7 @@
       </c>
       <c r="D305" s="4" t="inlineStr">
         <is>
-          <t>measured every page's title font, weight, size and label colour on live vs ours (136 pages). Now like live: Kava headings in Fraunces, HumanOS in Space Grotesk, the peptide tools / charity scorecard / thesis threads in the system serif, America Unbundled in the Iowan Old Style stack at live's size, /akbar in Fraunces 900, friend-gate and post-intervention in Georgia, and live's title sizes on peptide-matrix, peptide-supply-chain, rip-peptide-sciences and the HumanOS pages. Fonts load only on the pages that use them (src/lib/fonts/page-fonts.ts). Label colours stay the darker AA-contrast versions where live's lighter ones fail on a light background.</t>
+          <t>same server-checked password as the locked essay (GATED_POST_PASSWORD, now also set in Netlify), live's "Restricted Access" screen, the report not in the page until unlocked, out of search and the sitemap.</t>
         </is>
       </c>
       <c r="E305" s="14" t="inlineStr">
@@ -7868,7 +7868,7 @@
       <c r="A306" s="4" t="n"/>
       <c r="B306" s="4" t="inlineStr">
         <is>
-          <t>Peptide page images rescued into Sanity and wired (2026-10-07)</t>
+          <t>Live's title fonts and sizes (2026-10-07, "fix the style")</t>
         </is>
       </c>
       <c r="C306" s="13" t="inlineStr">
@@ -7878,7 +7878,7 @@
       </c>
       <c r="D306" s="4" t="inlineStr">
         <is>
-          <t>/peptide-watch hero plus its 11 section banners, /peptide-matrix and /peptide-supply-chain heroes, the /peptide-hall-of-shame hero (scripts/rescue-2026-10-07-peptide-images.ts, logged in docs/ai/manus-media-rescue.md).</t>
+          <t>measured every page's title font, weight, size and label colour on live vs ours (136 pages). Now like live: Kava headings in Fraunces, HumanOS in Space Grotesk, the peptide tools / charity scorecard / thesis threads in the system serif, America Unbundled in the Iowan Old Style stack at live's size, /akbar in Fraunces 900, friend-gate and post-intervention in Georgia, and live's title sizes on peptide-matrix, peptide-supply-chain, rip-peptide-sciences and the HumanOS pages. Fonts load only on the pages that use them (src/lib/fonts/page-fonts.ts). Label colours stay the darker AA-contrast versions where live's lighter ones fail on a light background.</t>
         </is>
       </c>
       <c r="E306" s="14" t="inlineStr">
@@ -7891,7 +7891,7 @@
       <c r="A307" s="4" t="n"/>
       <c r="B307" s="4" t="inlineStr">
         <is>
-          <t>Live's editorial redesign, first group (2026-10-07)</t>
+          <t>Peptide page images rescued into Sanity and wired (2026-10-07)</t>
         </is>
       </c>
       <c r="C307" s="13" t="inlineStr">
@@ -7901,7 +7901,7 @@
       </c>
       <c r="D307" s="4" t="inlineStr">
         <is>
-          <t>dark top sections, narrow single text column, short red section rules and dark call-to-action bands on /invest, /amplifier, /community (now "Sign In to Join the Community", linking our real sign-in; live's made-up counters left out), /framework, /the-letter (daily provocation with "Share this thought" and "Search past provocations"), /engage, /diamond-cut, /ecosystem and the homepage's "The thinking doesn't stop here" band. Kept on purpose: AA-contrast colours where live's fail, "Enter the Gate" instead of live's $5,000 checkout on /diamond-cut.</t>
+          <t>/peptide-watch hero plus its 11 section banners, /peptide-matrix and /peptide-supply-chain heroes, the /peptide-hall-of-shame hero (scripts/rescue-2026-10-07-peptide-images.ts, logged in docs/ai/manus-media-rescue.md).</t>
         </is>
       </c>
       <c r="E307" s="14" t="inlineStr">
@@ -7914,7 +7914,7 @@
       <c r="A308" s="4" t="n"/>
       <c r="B308" s="4" t="inlineStr">
         <is>
-          <t>Live's redesign, second group (done 2026-10-08)</t>
+          <t>Live's editorial redesign, first group (2026-10-07)</t>
         </is>
       </c>
       <c r="C308" s="13" t="inlineStr">
@@ -7924,7 +7924,7 @@
       </c>
       <c r="D308" s="4" t="inlineStr">
         <is>
-          <t>re-measured all 18 pages on live vs a fresh production build (title font/size/weight/colour, labels, hero images). Already matching from 2026-10-07: /the-web, /spirits, /iboga-ibogaine (weight 800), /living-declaration, BrewSoul photo on /brewsoul, /brewsoul/browse, /brewsoul/first-sip (live has none there either), /quiz_25q, /recent-creations. Fixed today: /find-your-journey (64px title, red label), /impact-dashboard (64px title in essay ink, label spacing), red labels on /published and /speaking (plus its "rooms" chips), /soulscore "by ImpactSoul" label, /pri-calibration title (weight 900, solid cream, was a purple gradient), /clients (live's narrow 546px column for the whole page, 56px title, roomier stats band, cards 2 per row; two static inline styles moved to classes), /brewsoul/guest (live's BrewSoul photo on the guest card instead of "SN" initials, labels in capitals), /humanos/connect (cards line up with the title), /peptide-hall-of-shame (stats and label readable light gold; were dark gold on dark). Typed arrows on the touched links are icons now (rule 18). Deliberately not copied from live (new CONTRIBUTING rule 20, owner 2026-10-08): red labels on dark bands use #E07A80 (live's #8E1E25 on black is about 2:1, unreadable); /recent-creations keeps our darker label colours (live's fail contrast on white); /humanos/connect keeps "Start Reading" (that card links to the philosophy page, the quiz live's "Start the Assessment" implies doesn't exist). Checked: type check, l</t>
+          <t>dark top sections, narrow single text column, short red section rules and dark call-to-action bands on /invest, /amplifier, /community (now "Sign In to Join the Community", linking our real sign-in; live's made-up counters left out), /framework, /the-letter (daily provocation with "Share this thought" and "Search past provocations"), /engage, /diamond-cut, /ecosystem and the homepage's "The thinking doesn't stop here" band. Kept on purpose: AA-contrast colours where live's fail, "Enter the Gate" instead of live's $5,000 checkout on /diamond-cut.</t>
         </is>
       </c>
       <c r="E308" s="14" t="inlineStr">
@@ -7937,7 +7937,7 @@
       <c r="A309" s="4" t="n"/>
       <c r="B309" s="4" t="inlineStr">
         <is>
-          <t>BrewSoul top of page (2026-10-08, owner: "button in the center at the top doesn't look good")</t>
+          <t>Live's redesign, second group (done 2026-10-08)</t>
         </is>
       </c>
       <c r="C309" s="13" t="inlineStr">
@@ -7947,7 +7947,7 @@
       </c>
       <c r="D309" s="4" t="inlineStr">
         <is>
-          <t>the category badge ("Deep Research" etc.) sat centred in an empty strip, squeezed against the hero, because we copied live's doubled 52px top gap. Now one gap everywhere and the badge floats in the top-left corner, lined up with the BrewSoul logo (brewsoul-main.tsx, category-badge.tsx); checked on all 26 badge pages at 3 widths that it covers nothing. BrewSoul menu: on tablets (768-1023px) the links were cut off and "More" was hidden with no menu button at all; now the menu button shows below 1024px, 5 links + "More" from 1024px, all 8 from 1280px, "More" always visible.</t>
+          <t>re-measured all 18 pages on live vs a fresh production build (title font/size/weight/colour, labels, hero images). Already matching from 2026-10-07: /the-web, /spirits, /iboga-ibogaine (weight 800), /living-declaration, BrewSoul photo on /brewsoul, /brewsoul/browse, /brewsoul/first-sip (live has none there either), /quiz_25q, /recent-creations. Fixed today: /find-your-journey (64px title, red label), /impact-dashboard (64px title in essay ink, label spacing), red labels on /published and /speaking (plus its "rooms" chips), /soulscore "by ImpactSoul" label, /pri-calibration title (weight 900, solid cream, was a purple gradient), /clients (live's narrow 546px column for the whole page, 56px title, roomier stats band, cards 2 per row; two static inline styles moved to classes), /brewsoul/guest (live's BrewSoul photo on the guest card instead of "SN" initials, labels in capitals), /humanos/connect (cards line up with the title), /peptide-hall-of-shame (stats and label readable light gold; were dark gold on dark). Typed arrows on the touched links are icons now (rule 18). Deliberately not copied from live (new CONTRIBUTING rule 20, owner 2026-10-08): red labels on dark bands use #E07A80 (live's #8E1E25 on black is about 2:1, unreadable); /recent-creations keeps our darker label colours (live's fail contrast on white); /humanos/connect keeps "Start Reading" (that card links to the philosophy page, the quiz live's "Start the Assessment" implies doesn't exist). Checked: type check, l</t>
         </is>
       </c>
       <c r="E309" s="14" t="inlineStr">
@@ -7960,7 +7960,7 @@
       <c r="A310" s="4" t="n"/>
       <c r="B310" s="4" t="inlineStr">
         <is>
-          <t>/pri-efficacy's "Simulation / Live Calibrations" switch like live (2026-10-08)</t>
+          <t>BrewSoul top of page (2026-10-08, owner: "button in the center at the top doesn't look good")</t>
         </is>
       </c>
       <c r="C310" s="13" t="inlineStr">
@@ -7970,7 +7970,7 @@
       </c>
       <c r="D310" s="4" t="inlineStr">
         <is>
-          <t>shadcn Tabs, both panels in the server HTML (forceMount). The Live tab reads real aggregate numbers from pri_calibrations (getPriLiveStats() in src/lib/pri-research.ts: totals, opt-ins, average score per dimension; no rows leave the server), page stays static and refreshes every 10 minutes. Until the Supabase scripts are run (Phase 2) it says the numbers "aren't available just now" instead of a fake zero. Checked: build (○, 10m), server HTML has both tabs, tab switch at 390/1280px, no JS errors. Re-check with real numbers once the table exists.</t>
+          <t>the category badge ("Deep Research" etc.) sat centred in an empty strip, squeezed against the hero, because we copied live's doubled 52px top gap. Now one gap everywhere and the badge floats in the top-left corner, lined up with the BrewSoul logo (brewsoul-main.tsx, category-badge.tsx); checked on all 26 badge pages at 3 widths that it covers nothing. BrewSoul menu: on tablets (768-1023px) the links were cut off and "More" was hidden with no menu button at all; now the menu button shows below 1024px, 5 links + "More" from 1024px, all 8 from 1280px, "More" always visible.</t>
         </is>
       </c>
       <c r="E310" s="14" t="inlineStr">
@@ -7983,63 +7983,63 @@
       <c r="A311" s="4" t="n"/>
       <c r="B311" s="4" t="inlineStr">
         <is>
+          <t>/pri-efficacy's "Simulation / Live Calibrations" switch like live (2026-10-08)</t>
+        </is>
+      </c>
+      <c r="C311" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D311" s="4" t="inlineStr">
+        <is>
+          <t>shadcn Tabs, both panels in the server HTML (forceMount). The Live tab reads real aggregate numbers from pri_calibrations (getPriLiveStats() in src/lib/pri-research.ts: totals, opt-ins, average score per dimension; no rows leave the server), page stays static and refreshes every 10 minutes. Until the Supabase scripts are run (Phase 2) it says the numbers "aren't available just now" instead of a fake zero. Checked: build (○, 10m), server HTML has both tabs, tab switch at 390/1280px, no JS errors. Re-check with real numbers once the table exists.</t>
+        </is>
+      </c>
+      <c r="E311" s="14" t="inlineStr">
+        <is>
+          <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" s="4" t="n"/>
+      <c r="B312" s="4" t="inlineStr">
+        <is>
           <t>/brewsoul/browse hero readable (2026-10-08, owner said go ahead)</t>
         </is>
       </c>
-      <c r="C311" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D311" s="4" t="inlineStr">
+      <c r="C312" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D312" s="4" t="inlineStr">
         <is>
           <t>a soft cream glow behind the title block so "The Catalog", the subtitle and the stat labels read clearly over the coffee photo (live is hard to read there too; rule 20). Photo still shows around the edges. Checked at 390/1280px.</t>
         </is>
       </c>
-      <c r="E311" s="14" t="inlineStr">
+      <c r="E312" s="14" t="inlineStr">
         <is>
           <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
         </is>
       </c>
     </row>
-    <row r="312">
-      <c r="A312" s="10" t="inlineStr">
+    <row r="313">
+      <c r="A313" s="10" t="inlineStr">
         <is>
           <t>Phase 13 — Images Needed in Sanity</t>
         </is>
       </c>
-      <c r="B312" s="11" t="n"/>
-      <c r="C312" s="11" t="n"/>
-      <c r="D312" s="12" t="n"/>
-    </row>
-    <row r="313">
-      <c r="A313" s="4" t="n"/>
-      <c r="B313" s="4" t="inlineStr">
-        <is>
-          <t>Manus media rescue (2026-09-29)</t>
-        </is>
-      </c>
-      <c r="C313" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D313" s="4" t="inlineStr">
-        <is>
-          <t>all 94 Manus-hosted image/video references in the legacy source (/api/img/, /manus-storage/) were checked live. 91 were still downloadable, including the /akbar photos the entry below calls "permanently lost", and all 91 are now Sanity assets (scripts/rescue-manus-media.ts; Sanity dedupes by SHA-1). 3 were gone (HTTP 502). The manifest docs/ai/manus-media-rescue.md maps each one to the legacy files that used it and its Sanity URL. They are not wired into pages yet: go page by page, with real alt text. /facilitator-index's two diagrams are done (scripts/rescue-facilitator-images.ts).</t>
-        </is>
-      </c>
-      <c r="E313" s="14" t="inlineStr">
-        <is>
-          <t>Phase 13 — Images Needed in Sanity</t>
-        </is>
-      </c>
+      <c r="B313" s="11" t="n"/>
+      <c r="C313" s="11" t="n"/>
+      <c r="D313" s="12" t="n"/>
     </row>
     <row r="314">
       <c r="A314" s="4" t="n"/>
       <c r="B314" s="4" t="inlineStr">
         <is>
-          <t>Favicon</t>
+          <t>Manus media rescue (2026-09-29)</t>
         </is>
       </c>
       <c r="C314" s="13" t="inlineStr">
@@ -8049,7 +8049,7 @@
       </c>
       <c r="D314" s="4" t="inlineStr">
         <is>
-          <t>real "G" brand mark generated from the header's actual wordmark treatment (src/app/icon.tsx), see Phase 3</t>
+          <t>all 94 Manus-hosted image/video references in the legacy source (/api/img/, /manus-storage/) were checked live. 91 were still downloadable, including the /akbar photos the entry below calls "permanently lost", and all 91 are now Sanity assets (scripts/rescue-manus-media.ts; Sanity dedupes by SHA-1). 3 were gone (HTTP 502). The manifest docs/ai/manus-media-rescue.md maps each one to the legacy files that used it and its Sanity URL. They are not wired into pages yet: go page by page, with real alt text. /facilitator-index's two diagrams are done (scripts/rescue-facilitator-images.ts).</t>
         </is>
       </c>
       <c r="E314" s="14" t="inlineStr">
@@ -8062,7 +8062,7 @@
       <c r="A315" s="4" t="n"/>
       <c r="B315" s="4" t="inlineStr">
         <is>
-          <t>Site-wide: logo (light + dark) beyond the current text wordmark</t>
+          <t>Favicon</t>
         </is>
       </c>
       <c r="C315" s="13" t="inlineStr">
@@ -8072,7 +8072,7 @@
       </c>
       <c r="D315" s="4" t="inlineStr">
         <is>
-          <t>Decided 2026-10-13 (owner): keep the text logo. The header's "TonyG" wordmark (site-header.tsx, gold G) already has light and dark colours, so no change. (Default/fallback OG image 1200×630 exists: public/images/default-og.png, checked 2026-10-02.)</t>
+          <t>real "G" brand mark generated from the header's actual wordmark treatment (src/app/icon.tsx), see Phase 3</t>
         </is>
       </c>
       <c r="E315" s="14" t="inlineStr">
@@ -8085,7 +8085,7 @@
       <c r="A316" s="4" t="n"/>
       <c r="B316" s="4" t="inlineStr">
         <is>
-          <t>Author photo(s) for blog author schema (Tony Greenberg headshot at minimum)</t>
+          <t>Site-wide: logo (light + dark) beyond the current text wordmark</t>
         </is>
       </c>
       <c r="C316" s="13" t="inlineStr">
@@ -8095,7 +8095,7 @@
       </c>
       <c r="D316" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02: the rescued headshot is already the author avatar in Sanity; now also in every post's Article JSON-LD (author image + url /about). The JSON-LD publisher logo pointed at /favicon.ico, a 404 here; now /icon.</t>
+          <t>Decided 2026-10-13 (owner): keep the text logo. The header's "TonyG" wordmark (site-header.tsx, gold G) already has light and dark colours, so no change. (Default/fallback OG image 1200×630 exists: public/images/default-og.png, checked 2026-10-02.)</t>
         </is>
       </c>
       <c r="E316" s="14" t="inlineStr">
@@ -8108,7 +8108,7 @@
       <c r="A317" s="4" t="n"/>
       <c r="B317" s="4" t="inlineStr">
         <is>
-          <t>Blog hero images</t>
+          <t>Author photo(s) for blog author schema (Tony Greenberg headshot at minimum)</t>
         </is>
       </c>
       <c r="C317" s="13" t="inlineStr">
@@ -8118,7 +8118,7 @@
       </c>
       <c r="D317" s="4" t="inlineStr">
         <is>
-          <t>audited, then migrated. Final state:</t>
+          <t>2026-10-02: the rescued headshot is already the author avatar in Sanity; now also in every post's Article JSON-LD (author image + url /about). The JSON-LD publisher logo pointed at /favicon.ico, a 404 here; now /icon.</t>
         </is>
       </c>
       <c r="E317" s="14" t="inlineStr">
@@ -8131,7 +8131,7 @@
       <c r="A318" s="4" t="n"/>
       <c r="B318" s="4" t="inlineStr">
         <is>
-          <t>22 posts have a real hero image, now live in Sanity (17 already on RampRate's own CloudFront + 4 rescued from the legacy /api/img/ proxy + 1…</t>
+          <t>Blog hero images</t>
         </is>
       </c>
       <c r="C318" s="13" t="inlineStr">
@@ -8141,7 +8141,7 @@
       </c>
       <c r="D318" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> rescued from /manus-storage/, all pulled over by migrate-blog-posts.ts before Manus is decommissioned)</t>
+          <t>audited, then migrated. Final state:</t>
         </is>
       </c>
       <c r="E318" s="14" t="inlineStr">
@@ -8154,7 +8154,7 @@
       <c r="A319" s="4" t="n"/>
       <c r="B319" s="4" t="inlineStr">
         <is>
-          <t>7 more posts got a real, unique hero image rescued from the live legacy site's newly-added art this pass (scripts/rescue-2026-09-blog-images…</t>
+          <t>22 posts have a real hero image, now live in Sanity (17 already on RampRate's own CloudFront + 4 rescued from the legacy /api/img/ proxy + 1…</t>
         </is>
       </c>
       <c r="C319" s="13" t="inlineStr">
@@ -8164,7 +8164,7 @@
       </c>
       <c r="D319" s="4" t="inlineStr">
         <is>
-          <t>.ts — see the correction note above): california-toll-roads-legalized-scam, the-1000-hour-hold, conscious-capital-partnership-ecosystem, the-peptide-truth-65m-fraud-industry-vs-life-changing-medicine, clear-communication, building-services-market-transhuman-era, heart-protocol-addendum.</t>
+          <t xml:space="preserve"> rescued from /manus-storage/, all pulled over by migrate-blog-posts.ts before Manus is decommissioned)</t>
         </is>
       </c>
       <c r="E319" s="14" t="inlineStr">
@@ -8177,7 +8177,7 @@
       <c r="A320" s="4" t="n"/>
       <c r="B320" s="4" t="inlineStr">
         <is>
-          <t>92 posts still need a real, unique hero image</t>
+          <t>7 more posts got a real, unique hero image rescued from the live legacy site's newly-added art this pass (scripts/rescue-2026-09-blog-images…</t>
         </is>
       </c>
       <c r="C320" s="13" t="inlineStr">
@@ -8187,7 +8187,7 @@
       </c>
       <c r="D320" s="4" t="inlineStr">
         <is>
-          <t>(down from 99). 2026-10-13 (owner: "image you can add in Sanity"): generated a unique, text-free picture for each of the 92 (live's default-arch family: cream over a deep colour, gold line geometry, colour and motif by category, layout from the slug; scripts/generate-essay-hero-art.mjs) and set it as each post's heroImage draft (scripts/upload-essay-hero-art-2026-10-13.ts; dry run first: 92 found, none had art, nothing replaced). Checked in Sanity: 92 drafts carry the new image, 0 published posts changed. Published 2026-10-13 (owner: yes) with the script's --publish (only drafts whose sole change was the picture; 92 of 92). Checked: the Netlify copy's essay page now serves the new image (webhook refresh). Real photography can still replace any of them later. Tracked one row per post, with a suggested image-generation prompt, in BLOG-IMAGE-BRIEFS.md — work through that file and check items off there, not here. No image-generation tool was connected in this environment as of this writing; either connect one (e.g. an MCP image-gen extension), source these manually/with a designer then upload via Sanity Studio (/studio), or re-check the live legacy site periodically per the correction note above.</t>
+          <t>.ts — see the correction note above): california-toll-roads-legalized-scam, the-1000-hour-hold, conscious-capital-partnership-ecosystem, the-peptide-truth-65m-fraud-industry-vs-life-changing-medicine, clear-communication, building-services-market-transhuman-era, heart-protocol-addendum.</t>
         </is>
       </c>
       <c r="E320" s="14" t="inlineStr">
@@ -8200,7 +8200,7 @@
       <c r="A321" s="4" t="n"/>
       <c r="B321" s="4" t="inlineStr">
         <is>
-          <t>Blog: per-post OG image if different from hero (many posts can reuse hero as OG)</t>
+          <t>92 posts still need a real, unique hero image</t>
         </is>
       </c>
       <c r="C321" s="13" t="inlineStr">
@@ -8210,7 +8210,7 @@
       </c>
       <c r="D321" s="4" t="inlineStr">
         <is>
-          <t>Confirmed 2026-10-02: generateMetadata uses seo.ogImage, else the hero, else the default OG image.</t>
+          <t>(down from 99). 2026-10-13 (owner: "image you can add in Sanity"): generated a unique, text-free picture for each of the 92 (live's default-arch family: cream over a deep colour, gold line geometry, colour and motif by category, layout from the slug; scripts/generate-essay-hero-art.mjs) and set it as each post's heroImage draft (scripts/upload-essay-hero-art-2026-10-13.ts; dry run first: 92 found, none had art, nothing replaced). Checked in Sanity: 92 drafts carry the new image, 0 published posts changed. Published 2026-10-13 (owner: yes) with the script's --publish (only drafts whose sole change was the picture; 92 of 92). Checked: the Netlify copy's essay page now serves the new image (webhook refresh). Real photography can still replace any of them later. Tracked one row per post, with a suggested image-generation prompt, in BLOG-IMAGE-BRIEFS.md — work through that file and check items off there, not here. No image-generation tool was connected in this environment as of this writing; either connect one (e.g. an MCP image-gen extension), source these manually/with a designer then upload via Sanity Studio (/studio), or re-check the live legacy site periodically per the correction note above.</t>
         </is>
       </c>
       <c r="E321" s="14" t="inlineStr">
@@ -8223,7 +8223,7 @@
       <c r="A322" s="4" t="n"/>
       <c r="B322" s="4" t="inlineStr">
         <is>
-          <t>Marketing pages</t>
+          <t>Blog: per-post OG image if different from hero (many posts can reuse hero as OG)</t>
         </is>
       </c>
       <c r="C322" s="13" t="inlineStr">
@@ -8233,7 +8233,7 @@
       </c>
       <c r="D322" s="4" t="inlineStr">
         <is>
-          <t>hero/section images for /the-letter, /the-territory, /engine-room, /the-body, /the-nightstand, /recent-creations (portfolio thumbnails), /published (publication logos), /clients (client logos — confirm licensing before re-hosting). Checked against live 2026-10-02: same image count on every one; /the-territory, /engine-room, /recent-creations, /published, /clients have no images on live either.</t>
+          <t>Confirmed 2026-10-02: generateMetadata uses seo.ogImage, else the hero, else the default OG image.</t>
         </is>
       </c>
       <c r="E322" s="14" t="inlineStr">
@@ -8246,7 +8246,7 @@
       <c r="A323" s="4" t="n"/>
       <c r="B323" s="4" t="inlineStr">
         <is>
-          <t>/akbar essay images</t>
+          <t>Marketing pages</t>
         </is>
       </c>
       <c r="C323" s="13" t="inlineStr">
@@ -8256,7 +8256,7 @@
       </c>
       <c r="D323" s="4" t="inlineStr">
         <is>
-          <t>not lost after all: 20 of the 21 were rescued into Sanity by scripts/rescue-manus-media.ts (2026-09-28) and are wired back in legacy's layout (hero mosaic, JC portrait, 2x2 grid, 3 full-bleeds, 3-up strip, footer gallery) as of 2026-09-29. Only slider-3 was gone (HTTP 502); the hero mosaic is 4 tiles instead of 5.</t>
+          <t>hero/section images for /the-letter, /the-territory, /engine-room, /the-body, /the-nightstand, /recent-creations (portfolio thumbnails), /published (publication logos), /clients (client logos — confirm licensing before re-hosting). Checked against live 2026-10-02: same image count on every one; /the-territory, /engine-room, /recent-creations, /published, /clients have no images on live either.</t>
         </is>
       </c>
       <c r="E323" s="14" t="inlineStr">
@@ -8269,7 +8269,7 @@
       <c r="A324" s="4" t="n"/>
       <c r="B324" s="4" t="inlineStr">
         <is>
-          <t>Rescued page images wired back in (2026-09-29)</t>
+          <t>/akbar essay images</t>
         </is>
       </c>
       <c r="C324" s="13" t="inlineStr">
@@ -8279,7 +8279,7 @@
       </c>
       <c r="D324" s="4" t="inlineStr">
         <is>
-          <t>/living-declaration hero, hand image and Clarisse Abelarde artwork; /impact-dashboard earth hero; /find-my banner; /find-your-coffee dark photo landing (legacy copy restored, replacing an intro that wasn't in legacy). Also wired (second pass): /consciousness-scale (legacy's hero-first flow restored, the invented intro screen removed), /find-your-me hero, /humanos hero, the HumanOS nav logo, and all 12 HumanOS people headshots (/humanos/ecosystem, /humanos/philosophy). Blog-body images (2026-09-29): all 19 the migration dropped are restored by scripts/restore-blog-body-images.ts as Sanity drafts on 4 posts (Clarisse Abelarde 7, You Are the Moat 4, FRQNCY 6, Energy Is Money 2), waiting to be published in Studio; the other blog-listed assets were heroes already set. Still unwired from docs/ai/manus-media-rescue.md: and /alex-azzi's subject photo (a photo of a real person on an accusation page: needs Tony's yes first).</t>
+          <t>not lost after all: 20 of the 21 were rescued into Sanity by scripts/rescue-manus-media.ts (2026-09-28) and are wired back in legacy's layout (hero mosaic, JC portrait, 2x2 grid, 3 full-bleeds, 3-up strip, footer gallery) as of 2026-09-29. Only slider-3 was gone (HTTP 502); the hero mosaic is 4 tiles instead of 5.</t>
         </is>
       </c>
       <c r="E324" s="14" t="inlineStr">
@@ -8292,7 +8292,7 @@
       <c r="A325" s="4" t="n"/>
       <c r="B325" s="4" t="inlineStr">
         <is>
-          <t>BrewSoul: coffee/product images (brewsoul-coffees-expanded.ts likely has image refs</t>
+          <t>Rescued page images wired back in (2026-09-29)</t>
         </is>
       </c>
       <c r="C325" s="13" t="inlineStr">
@@ -8302,7 +8302,7 @@
       </c>
       <c r="D325" s="4" t="inlineStr">
         <is>
-          <t>audit), city guide header images, roaster directory photos. Audited 2026-09-09 (status spreadsheet), confirmed 2026-10-02: city guides already have photos; coffees, chains and roasters have no image field in legacy or here (text-only by design); farms got real photos.</t>
+          <t>/living-declaration hero, hand image and Clarisse Abelarde artwork; /impact-dashboard earth hero; /find-my banner; /find-your-coffee dark photo landing (legacy copy restored, replacing an intro that wasn't in legacy). Also wired (second pass): /consciousness-scale (legacy's hero-first flow restored, the invented intro screen removed), /find-your-me hero, /humanos hero, the HumanOS nav logo, and all 12 HumanOS people headshots (/humanos/ecosystem, /humanos/philosophy). Blog-body images (2026-09-29): all 19 the migration dropped are restored by scripts/restore-blog-body-images.ts as Sanity drafts on 4 posts (Clarisse Abelarde 7, You Are the Moat 4, FRQNCY 6, Energy Is Money 2), waiting to be published in Studio; the other blog-listed assets were heroes already set. Still unwired from docs/ai/manus-media-rescue.md: and /alex-azzi's subject photo (a photo of a real person on an accusation page: needs Tony's yes first).</t>
         </is>
       </c>
       <c r="E325" s="14" t="inlineStr">
@@ -8315,7 +8315,7 @@
       <c r="A326" s="4" t="n"/>
       <c r="B326" s="4" t="inlineStr">
         <is>
-          <t>65 page images moved off the Manus storage copy into Sanity (2026-10-02)</t>
+          <t>BrewSoul: coffee/product images (brewsoul-coffees-expanded.ts likely has image refs</t>
         </is>
       </c>
       <c r="C326" s="13" t="inlineStr">
@@ -8325,7 +8325,7 @@
       </c>
       <c r="D326" s="4" t="inlineStr">
         <is>
-          <t>every image the code loaded from d2xsxph8kpxj0f.cloudfront.net (PRI medicine images, Iboga module, facilitator index, /attention-theft, /alex-azzi, /protecting-your-business, /peyote-mescaline, HumanOS, the peptide quiz). Notes called it "RampRate's own CloudFront", but every file sits in the legacy Manus project's folder and its owner couldn't be confirmed. All 65 uploaded (scripts/rescue-cloudfront-images.ts), code rewritten, host removed from images.remotePatterns, no Sanity document used it. Table in docs/ai/manus-media-rescue.md.</t>
+          <t>audit), city guide header images, roaster directory photos. Audited 2026-09-09 (status spreadsheet), confirmed 2026-10-02: city guides already have photos; coffees, chains and roasters have no image field in legacy or here (text-only by design); farms got real photos.</t>
         </is>
       </c>
       <c r="E326" s="14" t="inlineStr">
@@ -8338,7 +8338,7 @@
       <c r="A327" s="4" t="n"/>
       <c r="B327" s="4" t="inlineStr">
         <is>
-          <t>PRI/Kava: medicine reference images (medicine-images.ts), facility images for /facilitator-index</t>
+          <t>65 page images moved off the Manus storage copy into Sanity (2026-10-02)</t>
         </is>
       </c>
       <c r="C327" s="13" t="inlineStr">
@@ -8348,7 +8348,7 @@
       </c>
       <c r="D327" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02: all in Sanity; image counts match live on PRI, Kava, Iboga, Peyote, facilitator pages.</t>
+          <t>every image the code loaded from d2xsxph8kpxj0f.cloudfront.net (PRI medicine images, Iboga module, facilitator index, /attention-theft, /alex-azzi, /protecting-your-business, /peyote-mescaline, HumanOS, the peptide quiz). Notes called it "RampRate's own CloudFront", but every file sits in the legacy Manus project's folder and its owner couldn't be confirmed. All 65 uploaded (scripts/rescue-cloudfront-images.ts), code rewritten, host removed from images.remotePatterns, no Sanity document used it. Table in docs/ai/manus-media-rescue.md.</t>
         </is>
       </c>
       <c r="E327" s="14" t="inlineStr">
@@ -8361,7 +8361,7 @@
       <c r="A328" s="4" t="n"/>
       <c r="B328" s="4" t="inlineStr">
         <is>
-          <t>Manifesto/Attention Theft: any diagram/illustration assets used on the mega-page</t>
+          <t>PRI/Kava: medicine reference images (medicine-images.ts), facility images for /facilitator-index</t>
         </is>
       </c>
       <c r="C328" s="13" t="inlineStr">
@@ -8371,7 +8371,7 @@
       </c>
       <c r="D328" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02: 6 of live's 7 are in (now in Sanity); the 7th belongs to the Wall of Shame section left out on purpose.</t>
+          <t>2026-10-02: all in Sanity; image counts match live on PRI, Kava, Iboga, Peyote, facilitator pages.</t>
         </is>
       </c>
       <c r="E328" s="14" t="inlineStr">
@@ -8384,7 +8384,7 @@
       <c r="A329" s="4" t="n"/>
       <c r="B329" s="4" t="inlineStr">
         <is>
-          <t>Assessment result-screen background art (flagged in STATUS.md as a known gap</t>
+          <t>Manifesto/Attention Theft: any diagram/illustration assets used on the mega-page</t>
         </is>
       </c>
       <c r="C329" s="13" t="inlineStr">
@@ -8394,7 +8394,7 @@
       </c>
       <c r="D329" s="4" t="inlineStr">
         <is>
-          <t>18/20 assessments currently have plain black backgrounds; sourcing themed art here also closes that gap) Done 2026-10-13 with colour instead of art (owner: "yes" to colour backgrounds). About 20 quizzes already had a coloured background (ThemedBackground, light per-theme gradients). The 4 still flat dark now have a dark colour gradient, kept dark so their light text stays readable: /find-your-journey result (purple to teal), /my-journey (its black layer hid the gradient; now green to purple), /pri-calibration and the /psychedelic-readiness-index assessment section (PRI ink to amber to plum, starting at ink so the photo band's fade still meets it). Checked: type check, lint, build (all 8 colours in the compiled CSS), screenshots at 375/820/1280 (quiz completed for the journey result), no sideways scroll or JS errors, axe colour-contrast 0 at 375 and 1280.</t>
+          <t>2026-10-02: 6 of live's 7 are in (now in Sanity); the 7th belongs to the Wall of Shame section left out on purpose.</t>
         </is>
       </c>
       <c r="E329" s="14" t="inlineStr">
@@ -8407,7 +8407,7 @@
       <c r="A330" s="4" t="n"/>
       <c r="B330" s="4" t="inlineStr">
         <is>
-          <t>Chatbot: FauxTony avatar/icon</t>
+          <t>Assessment result-screen background art (flagged in STATUS.md as a known gap</t>
         </is>
       </c>
       <c r="C330" s="13" t="inlineStr">
@@ -8417,7 +8417,7 @@
       </c>
       <c r="D330" s="4" t="inlineStr">
         <is>
-          <t>Not needed (2026-10-02): the chatbot phase (Phase 10) was cancelled.</t>
+          <t>18/20 assessments currently have plain black backgrounds; sourcing themed art here also closes that gap) Done 2026-10-13 with colour instead of art (owner: "yes" to colour backgrounds). About 20 quizzes already had a coloured background (ThemedBackground, light per-theme gradients). The 4 still flat dark now have a dark colour gradient, kept dark so their light text stays readable: /find-your-journey result (purple to teal), /my-journey (its black layer hid the gradient; now green to purple), /pri-calibration and the /psychedelic-readiness-index assessment section (PRI ink to amber to plum, starting at ink so the photo band's fade still meets it). Checked: type check, lint, build (all 8 colours in the compiled CSS), screenshots at 375/820/1280 (quiz completed for the journey result), no sideways scroll or JS errors, axe colour-contrast 0 at 375 and 1280.</t>
         </is>
       </c>
       <c r="E330" s="14" t="inlineStr">
@@ -8430,63 +8430,63 @@
       <c r="A331" s="4" t="n"/>
       <c r="B331" s="4" t="inlineStr">
         <is>
+          <t>Chatbot: FauxTony avatar/icon</t>
+        </is>
+      </c>
+      <c r="C331" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D331" s="4" t="inlineStr">
+        <is>
+          <t>Not needed (2026-10-02): the chatbot phase (Phase 10) was cancelled.</t>
+        </is>
+      </c>
+      <c r="E331" s="14" t="inlineStr">
+        <is>
+          <t>Phase 13 — Images Needed in Sanity</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" s="4" t="n"/>
+      <c r="B332" s="4" t="inlineStr">
+        <is>
           <t>Audit client/public/ (including alex-azzi/, brewsoul/ subfolders) for any static assets already sitting there unused that should be pulled i…</t>
         </is>
       </c>
-      <c r="C331" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D331" s="4" t="inlineStr">
+      <c r="C332" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D332" s="4" t="inlineStr">
         <is>
           <t>n rather than re-created. Done 2026-10-02: no images there at all (only llms.txt, a BrewSoul catalog, Manus debug files, design-options.html). Found and fixed a cutover risk instead: live serves two Google site-verification files (/google6881a0411c48b301.html, /alex-azzi/googleedff0185753a4a1f.html) that the new site returned 404 for, so Search Console could lose verification at DNS cutover. Both copied to public/ byte for byte. Not copied: site.webmanifest (its icons don't exist here; Next's app/icon.tsx covers the favicon).</t>
         </is>
       </c>
-      <c r="E331" s="14" t="inlineStr">
+      <c r="E332" s="14" t="inlineStr">
         <is>
           <t>Phase 13 — Images Needed in Sanity</t>
         </is>
       </c>
     </row>
-    <row r="332">
-      <c r="A332" s="10" t="inlineStr">
+    <row r="333">
+      <c r="A333" s="10" t="inlineStr">
         <is>
           <t>Phase 14 — QA &amp; Launch</t>
         </is>
       </c>
-      <c r="B332" s="11" t="n"/>
-      <c r="C332" s="11" t="n"/>
-      <c r="D332" s="12" t="n"/>
-    </row>
-    <row r="333">
-      <c r="A333" s="4" t="n"/>
-      <c r="B333" s="4" t="inlineStr">
-        <is>
-          <t>Mobile responsive pass on every ported section</t>
-        </is>
-      </c>
-      <c r="C333" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D333" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-29: no page scrolls sideways at 375px any more (114 pages checked in Chrome: every unique page plus 3 of each templated set like blog posts and coffees). Fixed: BrewSoul NextSteps forced 3 columns (and used an inline style), charity-scorecard tab row, /brewsoul/browse filter dropdowns, /the-philosophy hero glow. Still to check by hand: 44px tap targets and Safari iOS. 2026-09-30: 44px tap targets on phones for the shared header, footer, BrewSoul/Kava/HumanOS menus and ~100 standalone links (undersized targets 1,904 → 578; the rest are 24-43px pills/chips that meet WCAG 2.2 AA). axe target-size (WCAG 2.2 AA, with its spacing exception): 0 failures on 114 pages. Safari/iPhone (WebKit, iPhone 14 emulation): all 114 pages load, no sideways scroll, no JS errors; form fields under 16px (iOS zoom-on-tap) fixed site-wide in globals.css. Still to check on a real iPhone: BrewSoul's bottom journey bar showed page text through it in headless WebKit only (taps hit the bar correctly; Chrome renders it solid). Fixed 2026-10-09: the bar is now solid (bg-[#2C1810], was 92% plus backdrop-blur-md), so nothing can show through even where the blur isn't drawn; checked in WebKit (iPhone 13 profile) and Chrome: background rgb(44, 24, 16), no text behind the buttons. A real iPhone check is still part of Phase 14. Checked 2026-10-13 in Apple's iPhone Simulator (iPhone 16, iOS 26.5, real Mobile Safari; not a physical phone, owner accepted this as the iPhone check): 14 key pages on a fresh prod</t>
-        </is>
-      </c>
-      <c r="E333" s="14" t="inlineStr">
-        <is>
-          <t>Phase 14 — QA &amp; Launch</t>
-        </is>
-      </c>
+      <c r="B333" s="11" t="n"/>
+      <c r="C333" s="11" t="n"/>
+      <c r="D333" s="12" t="n"/>
     </row>
     <row r="334">
       <c r="A334" s="4" t="n"/>
       <c r="B334" s="4" t="inlineStr">
         <is>
-          <t>Accessibility pass (WCAG AA contrast, 44px touch targets, keyboard nav)</t>
+          <t>Mobile responsive pass on every ported section</t>
         </is>
       </c>
       <c r="C334" s="13" t="inlineStr">
@@ -8496,7 +8496,7 @@
       </c>
       <c r="D334" s="4" t="inlineStr">
         <is>
-          <t>same bar as legacy QA_MASTER_PROMPT.md. 2026-09-29 axe-core pass (WCAG 2.1 AA, same 114 pages, production build): all unlabeled dropdowns/inputs and unnamed links fixed; contrast down from 1,453 failing items on 106 pages to 1,038 on 70 (43 pages fully clean). Shared fixes: brand gold #8b6914 → #836311 site-wide (was 4.3:1 on cream, AA needs 4.5), header "⌘K"/social icons, BrewSoul nav and footer, HumanOS footer, Kava footer, assessment intro footnote, post-card image links. 2026-09-30: contrast finished, 0 axe color-contrast failures left on the same 114 pages (production build). Token changes: --kava-saffron #b86a28 → #8e521f, --pri-purple-light #a855f7 → #b87bf9 (on-dark purple only), --crusade-teal #0e7c7c → #0d7373; PriEyebrow goes light purple inside a dark PriSection via group-data-dark/pri; /find-your-me and the journey tracker's dark glass panels 60-70% → 90% (legacy's own 60% glass on beige rendered gray, cream text failed). Everything else: nearest passing shade of the same hue, or gold ↔ gold-light on the wrong background. Left: 18 links inside text marked only by color (need an underline), 44px tap targets, keyboard nav. 2026-09-30: 18 color-only in-text links underlined (axe link-in-text-block: 0 left); keyboard focus visible on every focusable item on 8 sampled pages (two form fields had none, fixed). 2026-10-02 re-run (axe WCAG 2.2 AA, 142 pages × 375/1280px, production build, plus Tab through 40 stops per page): found 1,370 contrast failures (mostly BrewSoul'</t>
+          <t>2026-09-29: no page scrolls sideways at 375px any more (114 pages checked in Chrome: every unique page plus 3 of each templated set like blog posts and coffees). Fixed: BrewSoul NextSteps forced 3 columns (and used an inline style), charity-scorecard tab row, /brewsoul/browse filter dropdowns, /the-philosophy hero glow. Still to check by hand: 44px tap targets and Safari iOS. 2026-09-30: 44px tap targets on phones for the shared header, footer, BrewSoul/Kava/HumanOS menus and ~100 standalone links (undersized targets 1,904 → 578; the rest are 24-43px pills/chips that meet WCAG 2.2 AA). axe target-size (WCAG 2.2 AA, with its spacing exception): 0 failures on 114 pages. Safari/iPhone (WebKit, iPhone 14 emulation): all 114 pages load, no sideways scroll, no JS errors; form fields under 16px (iOS zoom-on-tap) fixed site-wide in globals.css. Still to check on a real iPhone: BrewSoul's bottom journey bar showed page text through it in headless WebKit only (taps hit the bar correctly; Chrome renders it solid). Fixed 2026-10-09: the bar is now solid (bg-[#2C1810], was 92% plus backdrop-blur-md), so nothing can show through even where the blur isn't drawn; checked in WebKit (iPhone 13 profile) and Chrome: background rgb(44, 24, 16), no text behind the buttons. A real iPhone check is still part of Phase 14. Checked 2026-10-13 in Apple's iPhone Simulator (iPhone 16, iOS 26.5, real Mobile Safari; not a physical phone, owner accepted this as the iPhone check): 14 key pages on a fresh prod</t>
         </is>
       </c>
       <c r="E334" s="14" t="inlineStr">
@@ -8509,7 +8509,7 @@
       <c r="A335" s="4" t="n"/>
       <c r="B335" s="4" t="inlineStr">
         <is>
-          <t>No dead-end pages (every page links to 2+ others)</t>
+          <t>Accessibility pass (WCAG AA contrast, 44px touch targets, keyboard nav)</t>
         </is>
       </c>
       <c r="C335" s="13" t="inlineStr">
@@ -8519,7 +8519,7 @@
       </c>
       <c r="D335" s="4" t="inlineStr">
         <is>
-          <t>same bar as legacy MASTER_QUALITY_PROMPT.md 2026-09-30 scan (496 sitemap pages, header/footer links not counted): every page has a way home (the 6 HumanOS pages had none, in legacy too; added a "← TonyGreenberg.com" footer link). ~17 quiz pages only look like dead ends on their intro screen; their result screens link to related assessments. Left for a content decision: ~20 marketing pages (/akbar, /amplifier, /diamond-cut, /ecosystem, /engage, /engine-room, /intel, /invest, /pick-up-the-phone, /protecting-your-business, /published, /speaking, /the-nightstand, /the-territory, /the-web, /under-nda, /pri-calibration, /charity-scorecard and its detail pages) link to only 0-1 other page in their content. The port matches legacy there (legacy was just as sparse), so adding related links is new content and needs the owner's yes. Done 2026-10-10 (owner said yes): a "Related" section with 3 real links (no redirects, titles and blurbs from each target's own copy) on all 19 sparse pages and every charity profile: data src/lib/content/related-pages.ts, component src/components/marketing/related-pages.tsx (light/dark). Checked at 375/820/1280px with no sideways scroll; found and fixed on the way: the essay date line couldn't wrap on phones (21px sideways on long category names).</t>
+          <t>same bar as legacy QA_MASTER_PROMPT.md. 2026-09-29 axe-core pass (WCAG 2.1 AA, same 114 pages, production build): all unlabeled dropdowns/inputs and unnamed links fixed; contrast down from 1,453 failing items on 106 pages to 1,038 on 70 (43 pages fully clean). Shared fixes: brand gold #8b6914 → #836311 site-wide (was 4.3:1 on cream, AA needs 4.5), header "⌘K"/social icons, BrewSoul nav and footer, HumanOS footer, Kava footer, assessment intro footnote, post-card image links. 2026-09-30: contrast finished, 0 axe color-contrast failures left on the same 114 pages (production build). Token changes: --kava-saffron #b86a28 → #8e521f, --pri-purple-light #a855f7 → #b87bf9 (on-dark purple only), --crusade-teal #0e7c7c → #0d7373; PriEyebrow goes light purple inside a dark PriSection via group-data-dark/pri; /find-your-me and the journey tracker's dark glass panels 60-70% → 90% (legacy's own 60% glass on beige rendered gray, cream text failed). Everything else: nearest passing shade of the same hue, or gold ↔ gold-light on the wrong background. Left: 18 links inside text marked only by color (need an underline), 44px tap targets, keyboard nav. 2026-09-30: 18 color-only in-text links underlined (axe link-in-text-block: 0 left); keyboard focus visible on every focusable item on 8 sampled pages (two form fields had none, fixed). 2026-10-02 re-run (axe WCAG 2.2 AA, 142 pages × 375/1280px, production build, plus Tab through 40 stops per page): found 1,370 contrast failures (mostly BrewSoul'</t>
         </is>
       </c>
       <c r="E335" s="14" t="inlineStr">
@@ -8532,7 +8532,7 @@
       <c r="A336" s="4" t="n"/>
       <c r="B336" s="4" t="inlineStr">
         <is>
-          <t>Cross-browser check (Safari iOS in particular, per legacy performance notes) 2026-10-06 WebKit pass (Playwright WebKit, iPhone 13 profile, 1…</t>
+          <t>No dead-end pages (every page links to 2+ others)</t>
         </is>
       </c>
       <c r="C336" s="13" t="inlineStr">
@@ -8542,7 +8542,7 @@
       </c>
       <c r="D336" s="4" t="inlineStr">
         <is>
-          <t>52 pages: every unique page plus 3 of each templated set, production build): no page pans sideways, no failed requests, no JS errors. Found and fixed on the way: upgrade-insecure-requests in the new CSP made Safari fetch every stylesheet and font over https on localhost (dropped; the site is HTTPS-only via HSTS anyway), and .toLocaleString() without a locale caused a hydration error on /brewsoul/chains in Safari (all number formatting now en-US). Left: a check on a real iPhone (Phase 14). Checked 2026-10-13 in Apple's iPhone Simulator (iPhone 16, iOS 26.5, real Mobile Safari; not a physical phone, owner accepted this as the iPhone check): 14 key pages on a fresh production build (/, /blog, an essay, /brewsoul, /brewsoul/browse, /find-your-journey, /psychedelic-readiness-index, /kava, /humanos, /about, /iboga-ibogaine, /peptide-hall-of-shame, /my-journey, /pri-calibration): all render, no sideways pan, header and menus in place, BrewSoul's bottom bar solid. / and /blog showed blank on the very first cold load, then load within 3 s on every later visit.</t>
+          <t>same bar as legacy MASTER_QUALITY_PROMPT.md 2026-09-30 scan (496 sitemap pages, header/footer links not counted): every page has a way home (the 6 HumanOS pages had none, in legacy too; added a "← TonyGreenberg.com" footer link). ~17 quiz pages only look like dead ends on their intro screen; their result screens link to related assessments. Left for a content decision: ~20 marketing pages (/akbar, /amplifier, /diamond-cut, /ecosystem, /engage, /engine-room, /intel, /invest, /pick-up-the-phone, /protecting-your-business, /published, /speaking, /the-nightstand, /the-territory, /the-web, /under-nda, /pri-calibration, /charity-scorecard and its detail pages) link to only 0-1 other page in their content. The port matches legacy there (legacy was just as sparse), so adding related links is new content and needs the owner's yes. Done 2026-10-10 (owner said yes): a "Related" section with 3 real links (no redirects, titles and blurbs from each target's own copy) on all 19 sparse pages and every charity profile: data src/lib/content/related-pages.ts, component src/components/marketing/related-pages.tsx (light/dark). Checked at 375/820/1280px with no sideways scroll; found and fixed on the way: the essay date line couldn't wrap on phones (21px sideways on long category names).</t>
         </is>
       </c>
       <c r="E336" s="14" t="inlineStr">
@@ -8555,7 +8555,7 @@
       <c r="A337" s="4" t="n"/>
       <c r="B337" s="4" t="inlineStr">
         <is>
-          <t>Remove noindex only when sign-off is given</t>
+          <t>Cross-browser check (Safari iOS in particular, per legacy performance notes) 2026-10-06 WebKit pass (Playwright WebKit, iPhone 13 profile, 1…</t>
         </is>
       </c>
       <c r="C337" s="13" t="inlineStr">
@@ -8565,7 +8565,7 @@
       </c>
       <c r="D337" s="4" t="inlineStr">
         <is>
-          <t>do not launch indexable by accident (The only noindex is the host-based one for .netlify.app above, so the real domain is indexable as soon as DNS points at it: sign-off must come before DNS.) Re-checked 2026-10-13 on a fresh production build: tonygreenberg.com and www get no X-Robots-Tag and no robots meta (/, /blog, /about, /post-intervention), *.netlify.app gets noindex, nofollow; robots.txt allows crawlers, sitemap 200, missing pages 404, /manifesto 308. Ready; still waits on sign-off. Done 2026-10-13 (sign-off given): nothing to switch off. The only noindex is host-based (.netlify.app), so tonygreenberg.com becomes indexable by Google the moment DNS points at Netlify (re-checked on today's build: no X-Robots-Tag or robots meta for the real domain).</t>
+          <t>52 pages: every unique page plus 3 of each templated set, production build): no page pans sideways, no failed requests, no JS errors. Found and fixed on the way: upgrade-insecure-requests in the new CSP made Safari fetch every stylesheet and font over https on localhost (dropped; the site is HTTPS-only via HSTS anyway), and .toLocaleString() without a locale caused a hydration error on /brewsoul/chains in Safari (all number formatting now en-US). Left: a check on a real iPhone (Phase 14). Checked 2026-10-13 in Apple's iPhone Simulator (iPhone 16, iOS 26.5, real Mobile Safari; not a physical phone, owner accepted this as the iPhone check): 14 key pages on a fresh production build (/, /blog, an essay, /brewsoul, /brewsoul/browse, /find-your-journey, /psychedelic-readiness-index, /kava, /humanos, /about, /iboga-ibogaine, /peptide-hall-of-shame, /my-journey, /pri-calibration): all render, no sideways pan, header and menus in place, BrewSoul's bottom bar solid. / and /blog showed blank on the very first cold load, then load within 3 s on every later visit.</t>
         </is>
       </c>
       <c r="E337" s="14" t="inlineStr">
@@ -8578,7 +8578,7 @@
       <c r="A338" s="4" t="n"/>
       <c r="B338" s="4" t="inlineStr">
         <is>
-          <t>Final stakeholder sign-off (Tony/Darryl/Kimberly) on the ported site before DNS cutover Given 2026-10-13 by the webmaster (web.master@rampra…</t>
+          <t>Remove noindex only when sign-off is given</t>
         </is>
       </c>
       <c r="C338" s="13" t="inlineStr">
@@ -8588,7 +8588,7 @@
       </c>
       <c r="D338" s="4" t="inlineStr">
         <is>
-          <t>te.com) in a Claude Code session, answering "Tony's team sign-off, then turning on Google indexing" with yes. If Tony, Darryl or Kimberly haven't seen the Netlify copy themselves, get their yes before the DNS switch.</t>
+          <t>do not launch indexable by accident (The only noindex is the host-based one for .netlify.app above, so the real domain is indexable as soon as DNS points at it: sign-off must come before DNS.) Re-checked 2026-10-13 on a fresh production build: tonygreenberg.com and www get no X-Robots-Tag and no robots meta (/, /blog, /about, /post-intervention), *.netlify.app gets noindex, nofollow; robots.txt allows crawlers, sitemap 200, missing pages 404, /manifesto 308. Ready; still waits on sign-off. Done 2026-10-13 (sign-off given): nothing to switch off. The only noindex is host-based (.netlify.app), so tonygreenberg.com becomes indexable by Google the moment DNS points at Netlify (re-checked on today's build: no X-Robots-Tag or robots meta for the real domain).</t>
         </is>
       </c>
       <c r="E338" s="14" t="inlineStr">
@@ -8601,7 +8601,7 @@
       <c r="A339" s="4" t="n"/>
       <c r="B339" s="4" t="inlineStr">
         <is>
-          <t>Privacy Policy page (/privacy) + footer link</t>
+          <t>Final stakeholder sign-off (Tony/Darryl/Kimberly) on the ported site before DNS cutover Given 2026-10-13 by the webmaster (web.master@rampra…</t>
         </is>
       </c>
       <c r="C339" s="13" t="inlineStr">
@@ -8611,7 +8611,7 @@
       </c>
       <c r="D339" s="4" t="inlineStr">
         <is>
-          <t>(team review 2026-10-14; owner: "create any page that isn't there"). Neither live nor the old app has one, so it's a new page. Wording drafted from what the code really does: newsletter (Kit), member accounts, quiz results (sexuality/religion save only "finished"), comments/reactions/highlights, the site's forms (Supabase, emailed to Tony via Resend), supplier intake to RampRate, Google Analytics, the sign-in, tg_visit_count and visitor-session cookies, browser storage. Contact for requests: t@ramprate.com (the footer's address). Josh (legal) to review the wording before launch.</t>
+          <t>te.com) in a Claude Code session, answering "Tony's team sign-off, then turning on Google indexing" with yes. If Tony, Darryl or Kimberly haven't seen the Netlify copy themselves, get their yes before the DNS switch.</t>
         </is>
       </c>
       <c r="E339" s="14" t="inlineStr">
@@ -8624,7 +8624,7 @@
       <c r="A340" s="4" t="n"/>
       <c r="B340" s="4" t="inlineStr">
         <is>
-          <t>Terms of Use page (/terms) + footer link</t>
+          <t>Privacy Policy page (/privacy) + footer link</t>
         </is>
       </c>
       <c r="C340" s="13" t="inlineStr">
@@ -8634,7 +8634,7 @@
       </c>
       <c r="D340" s="4" t="inlineStr">
         <is>
-          <t>(team review 2026-10-14). Not-medical-advice (peptides, diet, therapy, kava, psychedelics, ibogaine) and not-investment-advice (waitlists are not offers) sections, ownership matching the footer notice, user content, liability, California law. /terms was one of the intentional 404s; now a real page (ROUTES-INVENTORY.md updated). Josh (legal) to review before launch.</t>
+          <t>(team review 2026-10-14; owner: "create any page that isn't there"). Neither live nor the old app has one, so it's a new page. Wording drafted from what the code really does: newsletter (Kit), member accounts, quiz results (sexuality/religion save only "finished"), comments/reactions/highlights, the site's forms (Supabase, emailed to Tony via Resend), supplier intake to RampRate, Google Analytics, the sign-in, tg_visit_count and visitor-session cookies, browser storage. Contact for requests: t@ramprate.com (the footer's address). Josh (legal) to review the wording before launch.</t>
         </is>
       </c>
       <c r="E340" s="14" t="inlineStr">
@@ -8647,7 +8647,7 @@
       <c r="A341" s="4" t="n"/>
       <c r="B341" s="4" t="inlineStr">
         <is>
-          <t>Contact page (/contact) + footer link</t>
+          <t>Terms of Use page (/terms) + footer link</t>
         </is>
       </c>
       <c r="C341" s="13" t="inlineStr">
@@ -8657,7 +8657,7 @@
       </c>
       <c r="D341" s="4" t="inlineStr">
         <is>
-          <t>(team review 2026-10-14). Gathers details already on the site: email t@ramprate.com (now also a clickable link in the footer, where it was plain text), booking link, the Engagement Audit (/pick-up-the-phone), RampRate supplier intake, Santa Monica, X and LinkedIn. No form (none needed: every option already exists). Checked 2026-10-14 for all three: type check, lint, Manus grep, build (all ○ static), fresh server: 200, one H1, title, canonical, share image, in the sitemap and Ask Tony search, footer links on every page; browser at 375/820/1280 light and 375/1280 dark: no sideways scroll, no JS errors.</t>
+          <t>(team review 2026-10-14). Not-medical-advice (peptides, diet, therapy, kava, psychedelics, ibogaine) and not-investment-advice (waitlists are not offers) sections, ownership matching the footer notice, user content, liability, California law. /terms was one of the intentional 404s; now a real page (ROUTES-INVENTORY.md updated). Josh (legal) to review before launch.</t>
         </is>
       </c>
       <c r="E341" s="14" t="inlineStr">
@@ -8670,7 +8670,7 @@
       <c r="A342" s="4" t="n"/>
       <c r="B342" s="4" t="inlineStr">
         <is>
-          <t>Essay counts match</t>
+          <t>Contact page (/contact) + footer link</t>
         </is>
       </c>
       <c r="C342" s="13" t="inlineStr">
@@ -8680,7 +8680,7 @@
       </c>
       <c r="D342" s="4" t="inlineStr">
         <is>
-          <t>(team review 2026-10-14). Ask Tony's Blog entry said "92 essays" (copied from the old app), the homepage Read card "118", /subscribe and /the-letter's Read card "121", while the homepage and /search count 123 from Sanity. All now use Sanity's count ({count} in home-doors.ts and /the-letter's doors, /subscribe fetches it). Ask Tony (owner: show the number): the root layout fetches the count and passes it to SiteHeader → SearchModal; withEssayCount() in search-directory.ts fills {count} for Ask Tony, /search and /the-index too. Checked in a browser: Ask Tony shows "123 essays spanning 15 years", build still 150 static / 28 dynamic pages as before. Left alone: /living-declaration's "QPR Index scores intellectual rigor across 91 essays" (a claim about that tool, Tony's copy). Checked 2026-10-14: type check, lint, build (/, /subscribe, /the-letter still static), fresh server: all three show 123, no "92 essays" in the built browser code.</t>
+          <t>(team review 2026-10-14). Gathers details already on the site: email t@ramprate.com (now also a clickable link in the footer, where it was plain text), booking link, the Engagement Audit (/pick-up-the-phone), RampRate supplier intake, Santa Monica, X and LinkedIn. No form (none needed: every option already exists). Checked 2026-10-14 for all three: type check, lint, Manus grep, build (all ○ static), fresh server: 200, one H1, title, canonical, share image, in the sitemap and Ask Tony search, footer links on every page; browser at 375/820/1280 light and 375/1280 dark: no sideways scroll, no JS errors.</t>
         </is>
       </c>
       <c r="E342" s="14" t="inlineStr">
@@ -8693,7 +8693,7 @@
       <c r="A343" s="4" t="n"/>
       <c r="B343" s="4" t="inlineStr">
         <is>
-          <t>Team review's "everything else looks fine" re-checked</t>
+          <t>Essay counts match</t>
         </is>
       </c>
       <c r="C343" s="13" t="inlineStr">
@@ -8703,7 +8703,7 @@
       </c>
       <c r="D343" s="4" t="inlineStr">
         <is>
-          <t>(2026-10-14, owner: "you can check"). Fresh production build: all 60 menu pages (main menu, Fix Myself, Explore...) at 1280px and 375px: 200, one H1, no sideways scroll, no JS errors. All 130 blog links on them (122 posts, 8 categories): 200, no redirects. 404 page: 404 for a missing page, essay and category. Dark mode: switches and stays on across pages; 10 essays checked on a phone in dark mode. Phone menu shows every section; Ask Tony works on a phone. Netlify test site: the same 60 menu pages answer. Two small fixes: a missing essay or category showed the homepage's tab title on its 404 page (now "Page not found"); three Explore links (/attention-theft/weapons, /report, /legal) went through a redirect, now link straight to /attention-theft#weapons etc. Checked: type check, lint, build, clicked "Legal Database" in the menu.</t>
+          <t>(team review 2026-10-14). Ask Tony's Blog entry said "92 essays" (copied from the old app), the homepage Read card "118", /subscribe and /the-letter's Read card "121", while the homepage and /search count 123 from Sanity. All now use Sanity's count ({count} in home-doors.ts and /the-letter's doors, /subscribe fetches it). Ask Tony (owner: show the number): the root layout fetches the count and passes it to SiteHeader → SearchModal; withEssayCount() in search-directory.ts fills {count} for Ask Tony, /search and /the-index too. Checked in a browser: Ask Tony shows "123 essays spanning 15 years", build still 150 static / 28 dynamic pages as before. Left alone: /living-declaration's "QPR Index scores intellectual rigor across 91 essays" (a claim about that tool, Tony's copy). Checked 2026-10-14: type check, lint, build (/, /subscribe, /the-letter still static), fresh server: all three show 123, no "92 essays" in the built browser code.</t>
         </is>
       </c>
       <c r="E343" s="14" t="inlineStr">
@@ -8716,42 +8716,65 @@
       <c r="A344" s="4" t="n"/>
       <c r="B344" s="4" t="inlineStr">
         <is>
+          <t>Team review's "everything else looks fine" re-checked</t>
+        </is>
+      </c>
+      <c r="C344" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D344" s="4" t="inlineStr">
+        <is>
+          <t>(2026-10-14, owner: "you can check"). Fresh production build: all 60 menu pages (main menu, Fix Myself, Explore...) at 1280px and 375px: 200, one H1, no sideways scroll, no JS errors. All 130 blog links on them (122 posts, 8 categories): 200, no redirects. 404 page: 404 for a missing page, essay and category. Dark mode: switches and stays on across pages; 10 essays checked on a phone in dark mode. Phone menu shows every section; Ask Tony works on a phone. Netlify test site: the same 60 menu pages answer. Two small fixes: a missing essay or category showed the homepage's tab title on its 404 page (now "Page not found"); three Explore links (/attention-theft/weapons, /report, /legal) went through a redirect, now link straight to /attention-theft#weapons etc. Checked: type check, lint, build, clicked "Legal Database" in the menu.</t>
+        </is>
+      </c>
+      <c r="E344" s="14" t="inlineStr">
+        <is>
+          <t>Phase 14 — QA &amp; Launch</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" s="4" t="n"/>
+      <c r="B345" s="4" t="inlineStr">
+        <is>
           <t>DNS cutover, legacy app decommissioned only after a stable overlap window Re-checked 2026-10-13</t>
         </is>
       </c>
-      <c r="C344" s="16" t="inlineStr">
+      <c r="C345" s="16" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
       </c>
-      <c r="D344" s="4" t="inlineStr">
+      <c r="D345" s="4" t="inlineStr">
         <is>
           <t>unchanged (Hostinger name servers, bare domain on Manus 104.19.168/169.112, www CNAME cname.manus.space). Checked 2026-10-09 (owner wants to go live and switch off Manus): DNS for tonygreenberg.com is at Hostinger (name servers ns1/ns2.dns-parking.com); www is a CNAME to cname.manus.space, the bare domain points at Manus's addresses (104.19.168.112 / .169.112); the Netlify site tonygreenberg-website has no custom domain yet (production branch main). Order: (1) merge the three open pull requests into main and check the Netlify copy; (2) restore Supabase and run 0001 to 0003, or launch without member features (they say "isn't available just now"); (3) owner sign-off; (4) add tonygreenberg.com + www in Netlify (Domain management), then at Hostinger point the bare domain at Netlify (A record 75.2.60.5, or Netlify DNS) and www CNAME at tonygreenberg-website.netlify.app; Netlify issues the HTTPS certificate; (5) re-run scripts/check-search-console-urls.ts https://tonygreenberg.com and submit the sitemap in Search Console; (6) only after a few stable days: switch off the Manus site (the database is already backed up, docs/ai/project_legacy_database.md) and rotate the old database password.</t>
         </is>
       </c>
-      <c r="E344" s="14" t="inlineStr">
+      <c r="E345" s="14" t="inlineStr">
         <is>
           <t>Phase 14 — QA &amp; Launch</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D344"/>
+  <autoFilter ref="A1:D345"/>
   <mergeCells count="14">
-    <mergeCell ref="A312:D312"/>
-    <mergeCell ref="A244:D244"/>
-    <mergeCell ref="A157:D157"/>
+    <mergeCell ref="A245:D245"/>
+    <mergeCell ref="A158:D158"/>
+    <mergeCell ref="A333:D333"/>
+    <mergeCell ref="A313:D313"/>
     <mergeCell ref="A15:D15"/>
     <mergeCell ref="A64:D64"/>
-    <mergeCell ref="A332:D332"/>
-    <mergeCell ref="A212:D212"/>
+    <mergeCell ref="A213:D213"/>
+    <mergeCell ref="A266:D266"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A49:D49"/>
     <mergeCell ref="A129:D129"/>
-    <mergeCell ref="A190:D190"/>
-    <mergeCell ref="A216:D216"/>
-    <mergeCell ref="A265:D265"/>
+    <mergeCell ref="A191:D191"/>
     <mergeCell ref="A32:D32"/>
+    <mergeCell ref="A217:D217"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Find Your Me: fix dead essay links, hide never-written picks
Checked all 17 recommended essays against Sanity (123 published): only
3 worked, on live too. 5 were real essays under an old, longer address
and now use the real slug. 9 were never written anywhere; the result
screen now shows only essays Sanity returned and hides "Rabbit Holes"
when none are left, instead of raw slugs linking to a 404. Systems
Architect and Truth Speaker now show no essays: Tony to pick (filed in
Phase 14; the 9 are listed as NEVER_WRITTEN in the data test).

Also: a full test run is ~1.5 minutes; the 10-minute run was slowed by
stuck test processes left over from the helpers.

Checked: full test run 618/618 files, typecheck, lint.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Migration-Status-Report.xlsx
+++ b/Migration-Status-Report.xlsx
@@ -12,8 +12,8 @@
     <sheet name="Remaining Work" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Full Detail'!$A$1:$D$352</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Remaining Work'!$A$1:$D$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Full Detail'!$A$1:$D$354</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Remaining Work'!$A$1:$D$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -639,15 +639,15 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$352,$A5,'Full Detail'!$C$2:$C$352,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$354,$A5,'Full Detail'!$C$2:$C$354,"Done")</f>
         <v/>
       </c>
       <c r="C5" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$352,$A5,'Full Detail'!$C$2:$C$352,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$354,$A5,'Full Detail'!$C$2:$C$354,"Remaining")</f>
         <v/>
       </c>
       <c r="D5" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$352,$A5,'Full Detail'!$C$2:$C$352,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$354,$A5,'Full Detail'!$C$2:$C$354,"Deferred")</f>
         <v/>
       </c>
       <c r="E5" s="5">
@@ -666,15 +666,15 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$352,$A6,'Full Detail'!$C$2:$C$352,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$354,$A6,'Full Detail'!$C$2:$C$354,"Done")</f>
         <v/>
       </c>
       <c r="C6" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$352,$A6,'Full Detail'!$C$2:$C$352,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$354,$A6,'Full Detail'!$C$2:$C$354,"Remaining")</f>
         <v/>
       </c>
       <c r="D6" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$352,$A6,'Full Detail'!$C$2:$C$352,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$354,$A6,'Full Detail'!$C$2:$C$354,"Deferred")</f>
         <v/>
       </c>
       <c r="E6" s="5">
@@ -693,15 +693,15 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$352,$A7,'Full Detail'!$C$2:$C$352,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$354,$A7,'Full Detail'!$C$2:$C$354,"Done")</f>
         <v/>
       </c>
       <c r="C7" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$352,$A7,'Full Detail'!$C$2:$C$352,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$354,$A7,'Full Detail'!$C$2:$C$354,"Remaining")</f>
         <v/>
       </c>
       <c r="D7" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$352,$A7,'Full Detail'!$C$2:$C$352,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$354,$A7,'Full Detail'!$C$2:$C$354,"Deferred")</f>
         <v/>
       </c>
       <c r="E7" s="5">
@@ -720,15 +720,15 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$352,$A8,'Full Detail'!$C$2:$C$352,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$354,$A8,'Full Detail'!$C$2:$C$354,"Done")</f>
         <v/>
       </c>
       <c r="C8" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$352,$A8,'Full Detail'!$C$2:$C$352,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$354,$A8,'Full Detail'!$C$2:$C$354,"Remaining")</f>
         <v/>
       </c>
       <c r="D8" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$352,$A8,'Full Detail'!$C$2:$C$352,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$354,$A8,'Full Detail'!$C$2:$C$354,"Deferred")</f>
         <v/>
       </c>
       <c r="E8" s="5">
@@ -747,15 +747,15 @@
         </is>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$352,$A9,'Full Detail'!$C$2:$C$352,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$354,$A9,'Full Detail'!$C$2:$C$354,"Done")</f>
         <v/>
       </c>
       <c r="C9" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$352,$A9,'Full Detail'!$C$2:$C$352,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$354,$A9,'Full Detail'!$C$2:$C$354,"Remaining")</f>
         <v/>
       </c>
       <c r="D9" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$352,$A9,'Full Detail'!$C$2:$C$352,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$354,$A9,'Full Detail'!$C$2:$C$354,"Deferred")</f>
         <v/>
       </c>
       <c r="E9" s="5">
@@ -774,15 +774,15 @@
         </is>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$352,$A10,'Full Detail'!$C$2:$C$352,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$354,$A10,'Full Detail'!$C$2:$C$354,"Done")</f>
         <v/>
       </c>
       <c r="C10" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$352,$A10,'Full Detail'!$C$2:$C$352,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$354,$A10,'Full Detail'!$C$2:$C$354,"Remaining")</f>
         <v/>
       </c>
       <c r="D10" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$352,$A10,'Full Detail'!$C$2:$C$352,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$354,$A10,'Full Detail'!$C$2:$C$354,"Deferred")</f>
         <v/>
       </c>
       <c r="E10" s="5">
@@ -801,15 +801,15 @@
         </is>
       </c>
       <c r="B11" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$352,$A11,'Full Detail'!$C$2:$C$352,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$354,$A11,'Full Detail'!$C$2:$C$354,"Done")</f>
         <v/>
       </c>
       <c r="C11" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$352,$A11,'Full Detail'!$C$2:$C$352,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$354,$A11,'Full Detail'!$C$2:$C$354,"Remaining")</f>
         <v/>
       </c>
       <c r="D11" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$352,$A11,'Full Detail'!$C$2:$C$352,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$354,$A11,'Full Detail'!$C$2:$C$354,"Deferred")</f>
         <v/>
       </c>
       <c r="E11" s="5">
@@ -828,15 +828,15 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$352,$A12,'Full Detail'!$C$2:$C$352,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$354,$A12,'Full Detail'!$C$2:$C$354,"Done")</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$352,$A12,'Full Detail'!$C$2:$C$352,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$354,$A12,'Full Detail'!$C$2:$C$354,"Remaining")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$352,$A12,'Full Detail'!$C$2:$C$352,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$354,$A12,'Full Detail'!$C$2:$C$354,"Deferred")</f>
         <v/>
       </c>
       <c r="E12" s="5">
@@ -855,15 +855,15 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$352,$A13,'Full Detail'!$C$2:$C$352,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$354,$A13,'Full Detail'!$C$2:$C$354,"Done")</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$352,$A13,'Full Detail'!$C$2:$C$352,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$354,$A13,'Full Detail'!$C$2:$C$354,"Remaining")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$352,$A13,'Full Detail'!$C$2:$C$352,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$354,$A13,'Full Detail'!$C$2:$C$354,"Deferred")</f>
         <v/>
       </c>
       <c r="E13" s="5">
@@ -882,15 +882,15 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$352,$A14,'Full Detail'!$C$2:$C$352,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$354,$A14,'Full Detail'!$C$2:$C$354,"Done")</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$352,$A14,'Full Detail'!$C$2:$C$352,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$354,$A14,'Full Detail'!$C$2:$C$354,"Remaining")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$352,$A14,'Full Detail'!$C$2:$C$352,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$354,$A14,'Full Detail'!$C$2:$C$354,"Deferred")</f>
         <v/>
       </c>
       <c r="E14" s="5">
@@ -909,15 +909,15 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$352,$A15,'Full Detail'!$C$2:$C$352,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$354,$A15,'Full Detail'!$C$2:$C$354,"Done")</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$352,$A15,'Full Detail'!$C$2:$C$352,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$354,$A15,'Full Detail'!$C$2:$C$354,"Remaining")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$352,$A15,'Full Detail'!$C$2:$C$352,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$354,$A15,'Full Detail'!$C$2:$C$354,"Deferred")</f>
         <v/>
       </c>
       <c r="E15" s="5">
@@ -936,15 +936,15 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$352,$A16,'Full Detail'!$C$2:$C$352,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$354,$A16,'Full Detail'!$C$2:$C$354,"Done")</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$352,$A16,'Full Detail'!$C$2:$C$352,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$354,$A16,'Full Detail'!$C$2:$C$354,"Remaining")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$352,$A16,'Full Detail'!$C$2:$C$352,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$354,$A16,'Full Detail'!$C$2:$C$354,"Deferred")</f>
         <v/>
       </c>
       <c r="E16" s="5">
@@ -963,15 +963,15 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$352,$A17,'Full Detail'!$C$2:$C$352,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$354,$A17,'Full Detail'!$C$2:$C$354,"Done")</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$352,$A17,'Full Detail'!$C$2:$C$352,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$354,$A17,'Full Detail'!$C$2:$C$354,"Remaining")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$352,$A17,'Full Detail'!$C$2:$C$352,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$354,$A17,'Full Detail'!$C$2:$C$354,"Deferred")</f>
         <v/>
       </c>
       <c r="E17" s="5">
@@ -990,15 +990,15 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$352,$A18,'Full Detail'!$C$2:$C$352,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$354,$A18,'Full Detail'!$C$2:$C$354,"Done")</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$352,$A18,'Full Detail'!$C$2:$C$352,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$354,$A18,'Full Detail'!$C$2:$C$354,"Remaining")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$352,$A18,'Full Detail'!$C$2:$C$352,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$354,$A18,'Full Detail'!$C$2:$C$354,"Deferred")</f>
         <v/>
       </c>
       <c r="E18" s="5">
@@ -1017,15 +1017,15 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$352,$A19,'Full Detail'!$C$2:$C$352,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$354,$A19,'Full Detail'!$C$2:$C$354,"Done")</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$352,$A19,'Full Detail'!$C$2:$C$352,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$354,$A19,'Full Detail'!$C$2:$C$354,"Remaining")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$352,$A19,'Full Detail'!$C$2:$C$352,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$354,$A19,'Full Detail'!$C$2:$C$354,"Deferred")</f>
         <v/>
       </c>
       <c r="E19" s="5">
@@ -1075,7 +1075,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E352"/>
+  <dimension ref="A1:E354"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -8896,27 +8896,73 @@
       <c r="A352" s="4" t="n"/>
       <c r="B352" s="4" t="inlineStr">
         <is>
+          <t>Find Your Me essay links (2026-10-16, owner: "you can start")</t>
+        </is>
+      </c>
+      <c r="C352" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D352" s="4" t="inlineStr">
+        <is>
+          <t>Checked all 17 against</t>
+        </is>
+      </c>
+      <c r="E352" s="14" t="inlineStr">
+        <is>
+          <t>Phase 14 — QA &amp; Launch</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" s="4" t="n"/>
+      <c r="B353" s="4" t="inlineStr">
+        <is>
+          <t>Find Your Me: pick real essays for two results (2026-10-16), needs Tony</t>
+        </is>
+      </c>
+      <c r="C353" s="16" t="inlineStr">
+        <is>
+          <t>Remaining</t>
+        </is>
+      </c>
+      <c r="D353" s="4" t="inlineStr">
+        <is>
+          <t>The Systems</t>
+        </is>
+      </c>
+      <c r="E353" s="14" t="inlineStr">
+        <is>
+          <t>Phase 14 — QA &amp; Launch</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" s="4" t="n"/>
+      <c r="B354" s="4" t="inlineStr">
+        <is>
           <t>DNS cutover, legacy app decommissioned only after a stable overlap window Re-checked 2026-10-13</t>
         </is>
       </c>
-      <c r="C352" s="16" t="inlineStr">
+      <c r="C354" s="16" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
       </c>
-      <c r="D352" s="4" t="inlineStr">
+      <c r="D354" s="4" t="inlineStr">
         <is>
           <t>unchanged (Hostinger name servers, bare domain on Manus 104.19.168/169.112, www CNAME cname.manus.space). Checked 2026-10-09 (owner wants to go live and switch off Manus): DNS for tonygreenberg.com is at Hostinger (name servers ns1/ns2.dns-parking.com); www is a CNAME to cname.manus.space, the bare domain points at Manus's addresses (104.19.168.112 / .169.112); the Netlify site tonygreenberg-website has no custom domain yet (production branch main). Order: (1) merge the three open pull requests into main and check the Netlify copy; (2) restore Supabase and run 0001 to 0003, or launch without member features (they say "isn't available just now"); (3) owner sign-off; (4) add tonygreenberg.com + www in Netlify (Domain management), then at Hostinger point the bare domain at Netlify (A record 75.2.60.5, or Netlify DNS) and www CNAME at tonygreenberg-website.netlify.app; Netlify issues the HTTPS certificate; (5) re-run scripts/check-search-console-urls.ts https://tonygreenberg.com and submit the sitemap in Search Console; (6) only after a few stable days: switch off the Manus site (the database is already backed up, docs/ai/project_legacy_database.md) and rotate the old database password.</t>
         </is>
       </c>
-      <c r="E352" s="14" t="inlineStr">
+      <c r="E354" s="14" t="inlineStr">
         <is>
           <t>Phase 14 — QA &amp; Launch</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D352"/>
+  <autoFilter ref="A1:D354"/>
   <mergeCells count="14">
     <mergeCell ref="A245:D245"/>
     <mergeCell ref="A158:D158"/>
@@ -8943,7 +8989,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -9265,27 +9311,50 @@
       <c r="A17" s="4" t="n"/>
       <c r="B17" s="4" t="inlineStr">
         <is>
+          <t>Find Your Me: pick real essays for two results (2026-10-16), needs Tony</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>Remaining</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>The Systems</t>
+        </is>
+      </c>
+      <c r="E17" s="14" t="inlineStr">
+        <is>
+          <t>Phase 14 — QA &amp; Launch</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="n"/>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
           <t>DNS cutover, legacy app decommissioned only after a stable overlap window Re-checked 2026-10-13</t>
         </is>
       </c>
-      <c r="C17" s="16" t="inlineStr">
+      <c r="C18" s="16" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>unchanged (Hostinger name servers, bare domain on Manus 104.19.168/169.112, www CNAME cname.manus.space). Checked 2026-10-09 (owner wants to go live and switch off Manus): DNS for tonygreenberg.com is at Hostinger (name servers ns1/ns2.dns-parking.com); www is a CNAME to cname.manus.space, the bare domain points at Manus's addresses (104.19.168.112 / .169.112); the Netlify site tonygreenberg-website has no custom domain yet (production branch main). Order: (1) merge the three open pull requests into main and check the Netlify copy; (2) restore Supabase and run 0001 to 0003, or launch without member features (they say "isn't available just now"); (3) owner sign-off; (4) add tonygreenberg.com + www in Netlify (Domain management), then at Hostinger point the bare domain at Netlify (A record 75.2.60.5, or Netlify DNS) and www CNAME at tonygreenberg-website.netlify.app; Netlify issues the HTTPS certificate; (5) re-run scripts/check-search-console-urls.ts https://tonygreenberg.com and submit the sitemap in Search Console; (6) only after a few stable days: switch off the Manus site (the database is already backed up, docs/ai/project_legacy_database.md) and rotate the old database password.</t>
         </is>
       </c>
-      <c r="E17" s="14" t="inlineStr">
+      <c r="E18" s="14" t="inlineStr">
         <is>
           <t>Phase 14 — QA &amp; Launch</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D17"/>
+  <autoFilter ref="A1:D18"/>
   <mergeCells count="4">
     <mergeCell ref="A10:D10"/>
     <mergeCell ref="A4:D4"/>

</xml_diff>

<commit_message>
MCP: port send_email, create_report and ClickUp task tools from ramprate-ui
- send_email: sends through the site's Resend setup; sendEmail now takes
  several recipients and an optional {text, from, attachments}.
- create_report: builds a PDF report (@react-pdf/renderer) and emails it.
- ClickUp task tools (clickup-client.ts), needs CLICKUP_API_TOKEN.
- Tools classified in mcp-auth.ts and gated in project-rules.ts.
- get_attachment and create_download not ported as separate tools: this
  server has no attachment store or download route; reports go by email.
- Tests for every new/changed file (621 files, 3382 tests, 90%+ coverage).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Migration-Status-Report.xlsx
+++ b/Migration-Status-Report.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Remaining Work" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Full Detail'!$A$1:$D$356</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Full Detail'!$A$1:$D$357</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Remaining Work'!$A$1:$D$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -639,15 +639,15 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$356,$A5,'Full Detail'!$C$2:$C$356,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A5,'Full Detail'!$C$2:$C$357,"Done")</f>
         <v/>
       </c>
       <c r="C5" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$356,$A5,'Full Detail'!$C$2:$C$356,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A5,'Full Detail'!$C$2:$C$357,"Remaining")</f>
         <v/>
       </c>
       <c r="D5" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$356,$A5,'Full Detail'!$C$2:$C$356,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A5,'Full Detail'!$C$2:$C$357,"Deferred")</f>
         <v/>
       </c>
       <c r="E5" s="5">
@@ -666,15 +666,15 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$356,$A6,'Full Detail'!$C$2:$C$356,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A6,'Full Detail'!$C$2:$C$357,"Done")</f>
         <v/>
       </c>
       <c r="C6" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$356,$A6,'Full Detail'!$C$2:$C$356,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A6,'Full Detail'!$C$2:$C$357,"Remaining")</f>
         <v/>
       </c>
       <c r="D6" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$356,$A6,'Full Detail'!$C$2:$C$356,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A6,'Full Detail'!$C$2:$C$357,"Deferred")</f>
         <v/>
       </c>
       <c r="E6" s="5">
@@ -693,15 +693,15 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$356,$A7,'Full Detail'!$C$2:$C$356,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A7,'Full Detail'!$C$2:$C$357,"Done")</f>
         <v/>
       </c>
       <c r="C7" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$356,$A7,'Full Detail'!$C$2:$C$356,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A7,'Full Detail'!$C$2:$C$357,"Remaining")</f>
         <v/>
       </c>
       <c r="D7" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$356,$A7,'Full Detail'!$C$2:$C$356,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A7,'Full Detail'!$C$2:$C$357,"Deferred")</f>
         <v/>
       </c>
       <c r="E7" s="5">
@@ -720,15 +720,15 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$356,$A8,'Full Detail'!$C$2:$C$356,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A8,'Full Detail'!$C$2:$C$357,"Done")</f>
         <v/>
       </c>
       <c r="C8" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$356,$A8,'Full Detail'!$C$2:$C$356,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A8,'Full Detail'!$C$2:$C$357,"Remaining")</f>
         <v/>
       </c>
       <c r="D8" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$356,$A8,'Full Detail'!$C$2:$C$356,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A8,'Full Detail'!$C$2:$C$357,"Deferred")</f>
         <v/>
       </c>
       <c r="E8" s="5">
@@ -747,15 +747,15 @@
         </is>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$356,$A9,'Full Detail'!$C$2:$C$356,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A9,'Full Detail'!$C$2:$C$357,"Done")</f>
         <v/>
       </c>
       <c r="C9" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$356,$A9,'Full Detail'!$C$2:$C$356,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A9,'Full Detail'!$C$2:$C$357,"Remaining")</f>
         <v/>
       </c>
       <c r="D9" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$356,$A9,'Full Detail'!$C$2:$C$356,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A9,'Full Detail'!$C$2:$C$357,"Deferred")</f>
         <v/>
       </c>
       <c r="E9" s="5">
@@ -774,15 +774,15 @@
         </is>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$356,$A10,'Full Detail'!$C$2:$C$356,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A10,'Full Detail'!$C$2:$C$357,"Done")</f>
         <v/>
       </c>
       <c r="C10" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$356,$A10,'Full Detail'!$C$2:$C$356,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A10,'Full Detail'!$C$2:$C$357,"Remaining")</f>
         <v/>
       </c>
       <c r="D10" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$356,$A10,'Full Detail'!$C$2:$C$356,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A10,'Full Detail'!$C$2:$C$357,"Deferred")</f>
         <v/>
       </c>
       <c r="E10" s="5">
@@ -801,15 +801,15 @@
         </is>
       </c>
       <c r="B11" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$356,$A11,'Full Detail'!$C$2:$C$356,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A11,'Full Detail'!$C$2:$C$357,"Done")</f>
         <v/>
       </c>
       <c r="C11" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$356,$A11,'Full Detail'!$C$2:$C$356,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A11,'Full Detail'!$C$2:$C$357,"Remaining")</f>
         <v/>
       </c>
       <c r="D11" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$356,$A11,'Full Detail'!$C$2:$C$356,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A11,'Full Detail'!$C$2:$C$357,"Deferred")</f>
         <v/>
       </c>
       <c r="E11" s="5">
@@ -828,15 +828,15 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$356,$A12,'Full Detail'!$C$2:$C$356,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A12,'Full Detail'!$C$2:$C$357,"Done")</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$356,$A12,'Full Detail'!$C$2:$C$356,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A12,'Full Detail'!$C$2:$C$357,"Remaining")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$356,$A12,'Full Detail'!$C$2:$C$356,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A12,'Full Detail'!$C$2:$C$357,"Deferred")</f>
         <v/>
       </c>
       <c r="E12" s="5">
@@ -855,15 +855,15 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$356,$A13,'Full Detail'!$C$2:$C$356,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A13,'Full Detail'!$C$2:$C$357,"Done")</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$356,$A13,'Full Detail'!$C$2:$C$356,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A13,'Full Detail'!$C$2:$C$357,"Remaining")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$356,$A13,'Full Detail'!$C$2:$C$356,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A13,'Full Detail'!$C$2:$C$357,"Deferred")</f>
         <v/>
       </c>
       <c r="E13" s="5">
@@ -882,15 +882,15 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$356,$A14,'Full Detail'!$C$2:$C$356,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A14,'Full Detail'!$C$2:$C$357,"Done")</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$356,$A14,'Full Detail'!$C$2:$C$356,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A14,'Full Detail'!$C$2:$C$357,"Remaining")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$356,$A14,'Full Detail'!$C$2:$C$356,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A14,'Full Detail'!$C$2:$C$357,"Deferred")</f>
         <v/>
       </c>
       <c r="E14" s="5">
@@ -909,15 +909,15 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$356,$A15,'Full Detail'!$C$2:$C$356,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A15,'Full Detail'!$C$2:$C$357,"Done")</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$356,$A15,'Full Detail'!$C$2:$C$356,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A15,'Full Detail'!$C$2:$C$357,"Remaining")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$356,$A15,'Full Detail'!$C$2:$C$356,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A15,'Full Detail'!$C$2:$C$357,"Deferred")</f>
         <v/>
       </c>
       <c r="E15" s="5">
@@ -936,15 +936,15 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$356,$A16,'Full Detail'!$C$2:$C$356,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A16,'Full Detail'!$C$2:$C$357,"Done")</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$356,$A16,'Full Detail'!$C$2:$C$356,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A16,'Full Detail'!$C$2:$C$357,"Remaining")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$356,$A16,'Full Detail'!$C$2:$C$356,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A16,'Full Detail'!$C$2:$C$357,"Deferred")</f>
         <v/>
       </c>
       <c r="E16" s="5">
@@ -963,15 +963,15 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$356,$A17,'Full Detail'!$C$2:$C$356,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A17,'Full Detail'!$C$2:$C$357,"Done")</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$356,$A17,'Full Detail'!$C$2:$C$356,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A17,'Full Detail'!$C$2:$C$357,"Remaining")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$356,$A17,'Full Detail'!$C$2:$C$356,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A17,'Full Detail'!$C$2:$C$357,"Deferred")</f>
         <v/>
       </c>
       <c r="E17" s="5">
@@ -990,15 +990,15 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$356,$A18,'Full Detail'!$C$2:$C$356,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A18,'Full Detail'!$C$2:$C$357,"Done")</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$356,$A18,'Full Detail'!$C$2:$C$356,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A18,'Full Detail'!$C$2:$C$357,"Remaining")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$356,$A18,'Full Detail'!$C$2:$C$356,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A18,'Full Detail'!$C$2:$C$357,"Deferred")</f>
         <v/>
       </c>
       <c r="E18" s="5">
@@ -1017,15 +1017,15 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$356,$A19,'Full Detail'!$C$2:$C$356,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A19,'Full Detail'!$C$2:$C$357,"Done")</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$356,$A19,'Full Detail'!$C$2:$C$356,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A19,'Full Detail'!$C$2:$C$357,"Remaining")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$356,$A19,'Full Detail'!$C$2:$C$356,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A19,'Full Detail'!$C$2:$C$357,"Deferred")</f>
         <v/>
       </c>
       <c r="E19" s="5">
@@ -1075,7 +1075,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E356"/>
+  <dimension ref="A1:E357"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -6962,43 +6962,43 @@
       </c>
     </row>
     <row r="266">
-      <c r="A266" s="10" t="inlineStr">
+      <c r="A266" s="4" t="n"/>
+      <c r="B266" s="4" t="inlineStr">
+        <is>
+          <t>Email, PDF reports and ClickUp ported from ramprate-ui (2026-10-16, owner said yes, including the one new dependency @react-pdf/renderer ^4.9.0)</t>
+        </is>
+      </c>
+      <c r="C266" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D266" s="4" t="inlineStr">
+        <is>
+          <t>send_email, create_report (Tony Greenberg PDF emailed as an attachment), create_clickup_task, update_clickup_task, delete_clickup_task. Email reuses src/lib/email.ts (extended, site forms unchanged). Sending email and deleting tasks need the write role, creating/updating tasks edit; all five are rules-gated. New files clickup-client.ts, report-pdf.tsx. Checked: full test suite with 90%+ per file (new files 100%; the PDF test renders a real PDF and reads its text), typecheck, lint, build. Not exercised against real Resend or ClickUp (it would send a real email / make a real task). Needs CLICKUP_API_TOKEN set in Netlify; until then the ClickUp tools say ClickUp isn't set up. check_deploy was ported the same day. Not ported: get_attachment / create_download (chat-page-only; ramprate's own MCP server leaves them out), Slack, Prettier (reasons in docs/ai/project_mcp_server.md).</t>
+        </is>
+      </c>
+      <c r="E266" s="14" t="inlineStr">
+        <is>
+          <t>Phase 11 — Code MCP Server — REBUILT (2026-09-29)</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="10" t="inlineStr">
         <is>
           <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
         </is>
       </c>
-      <c r="B266" s="11" t="n"/>
-      <c r="C266" s="11" t="n"/>
-      <c r="D266" s="12" t="n"/>
-    </row>
-    <row r="267">
-      <c r="A267" s="4" t="n"/>
-      <c r="B267" s="4" t="inlineStr">
-        <is>
-          <t>Per-page generateMetadata (title, description, OG, Twitter Card, canonical) for every ported route, sourced from Sanity seo object where con…</t>
-        </is>
-      </c>
-      <c r="C267" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D267" s="4" t="inlineStr">
-        <is>
-          <t>tent is CMS-backed, static otherwise. Audited all 140 page.tsx files: only /studio has none (correct — it's robots.txt-disallowed, not public content). Real gap found and fixed: /blog/category/[slug] had no alternates.canonical at all, and no page-aware title for its own real pagination (?page=N) — every paginated page was serving an identical title with no canonical, a real duplicate-content signal. Fixed: generateMetadata now reads searchParams too, self-canonicals each page (?page=N pages canonical to themselves, not consolidated to page 1 — genuinely different posts per page, matching Google's current pagination guidance) and appends "— Page N" to the title past page 1. Verified live: page 1 canonicals to the bare URL, ?page=2 canonicals to ?page=2 with a distinct title.</t>
-        </is>
-      </c>
-      <c r="E267" s="14" t="inlineStr">
-        <is>
-          <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
-        </is>
-      </c>
+      <c r="B267" s="11" t="n"/>
+      <c r="C267" s="11" t="n"/>
+      <c r="D267" s="12" t="n"/>
     </row>
     <row r="268">
       <c r="A268" s="4" t="n"/>
       <c r="B268" s="4" t="inlineStr">
         <is>
-          <t>sitemap.ts generated from real Sanity content + static route list, auto-updates on publish</t>
+          <t>Per-page generateMetadata (title, description, OG, Twitter Card, canonical) for every ported route, sourced from Sanity seo object where con…</t>
         </is>
       </c>
       <c r="C268" s="13" t="inlineStr">
@@ -7008,7 +7008,7 @@
       </c>
       <c r="D268" s="4" t="inlineStr">
         <is>
-          <t>Extended from the Phase 5-era version (homepage + blog posts only, 122 URLs) to every real route: the full static route list (130 routes, generated from find src/app -name page.tsx, excluding /studio (robots.txt-disallowed), /(auth)/login (noindex via its own metadata), and /life-assessment (a pure redirect, not distinct content)) plus all 5 real dynamic sources — blog categories (allCategorySlugsQuery), BrewSoul cities (25), BrewSoul coffees (107), and charity-scorecard entries (103) — each pulled from the exact same data source its own page's generateStaticParams already uses, not re-derived. Auto-updates on publish for anything Sanity-backed (blog posts/categories) since it's a live client.fetch on every build; the static route list itself needs a one-line addition whenever a new page ships (same as any other route-registration step). Verified live: 496 real &lt;loc&gt; entries, spot-checked a coffee/city/charity/category URL each, typecheck/lint clean.</t>
+          <t>tent is CMS-backed, static otherwise. Audited all 140 page.tsx files: only /studio has none (correct — it's robots.txt-disallowed, not public content). Real gap found and fixed: /blog/category/[slug] had no alternates.canonical at all, and no page-aware title for its own real pagination (?page=N) — every paginated page was serving an identical title with no canonical, a real duplicate-content signal. Fixed: generateMetadata now reads searchParams too, self-canonicals each page (?page=N pages canonical to themselves, not consolidated to page 1 — genuinely different posts per page, matching Google's current pagination guidance) and appends "— Page N" to the title past page 1. Verified live: page 1 canonicals to the bare URL, ?page=2 canonicals to ?page=2 with a distinct title.</t>
         </is>
       </c>
       <c r="E268" s="14" t="inlineStr">
@@ -7021,7 +7021,7 @@
       <c r="A269" s="4" t="n"/>
       <c r="B269" s="4" t="inlineStr">
         <is>
-          <t>llms.txt</t>
+          <t>sitemap.ts generated from real Sanity content + static route list, auto-updates on publish</t>
         </is>
       </c>
       <c r="C269" s="13" t="inlineStr">
@@ -7031,7 +7031,7 @@
       </c>
       <c r="D269" s="4" t="inlineStr">
         <is>
-          <t>fetched verbatim from the still-live site and saved to web/public/llms.txt (real content: Tony's bio, expertise, full article index by category, every product/tool section) — do this before Manus goes away, it won't be recoverable after</t>
+          <t>Extended from the Phase 5-era version (homepage + blog posts only, 122 URLs) to every real route: the full static route list (130 routes, generated from find src/app -name page.tsx, excluding /studio (robots.txt-disallowed), /(auth)/login (noindex via its own metadata), and /life-assessment (a pure redirect, not distinct content)) plus all 5 real dynamic sources — blog categories (allCategorySlugsQuery), BrewSoul cities (25), BrewSoul coffees (107), and charity-scorecard entries (103) — each pulled from the exact same data source its own page's generateStaticParams already uses, not re-derived. Auto-updates on publish for anything Sanity-backed (blog posts/categories) since it's a live client.fetch on every build; the static route list itself needs a one-line addition whenever a new page ships (same as any other route-registration step). Verified live: 496 real &lt;loc&gt; entries, spot-checked a coffee/city/charity/category URL each, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E269" s="14" t="inlineStr">
@@ -7044,7 +7044,7 @@
       <c r="A270" s="4" t="n"/>
       <c r="B270" s="4" t="inlineStr">
         <is>
-          <t>robots.txt</t>
+          <t>llms.txt</t>
         </is>
       </c>
       <c r="C270" s="13" t="inlineStr">
@@ -7054,7 +7054,7 @@
       </c>
       <c r="D270" s="4" t="inlineStr">
         <is>
-          <t>same approach: fetched the real live file (not my earlier guessed robots.ts, which has been removed) and saved verbatim to web/public/robots.txt, plus added Disallow: /studio for the new Sanity Studio route. Confirmed live: real AI-crawler allowlist (GPTBot, Claude-Web, PerplexityBot, etc.), scraper blocklist, and the site's non-standard LLMs: directive all intact</t>
+          <t>fetched verbatim from the still-live site and saved to web/public/llms.txt (real content: Tony's bio, expertise, full article index by category, every product/tool section) — do this before Manus goes away, it won't be recoverable after</t>
         </is>
       </c>
       <c r="E270" s="14" t="inlineStr">
@@ -7067,7 +7067,7 @@
       <c r="A271" s="4" t="n"/>
       <c r="B271" s="4" t="inlineStr">
         <is>
-          <t>JSON-LD</t>
+          <t>robots.txt</t>
         </is>
       </c>
       <c r="C271" s="13" t="inlineStr">
@@ -7077,7 +7077,7 @@
       </c>
       <c r="D271" s="4" t="inlineStr">
         <is>
-          <t>WebSite + Person schema ported verbatim from the live homepage's actual &lt;script type="application/ld+json"&gt; tags (not reconstructed from memory) — rendered site-wide from src/lib/structured-data.ts in the root layout. The Person image was hardcoded to a /api/img/... legacy proxy path on the live site — rescued that headshot (downloaded it while still live, uploaded to Sanity as the author-tony-greenberg document's avatar) so the new site's JSON-LD has zero Manus dependency instead of just copying the fragile path forward</t>
+          <t>same approach: fetched the real live file (not my earlier guessed robots.ts, which has been removed) and saved verbatim to web/public/robots.txt, plus added Disallow: /studio for the new Sanity Studio route. Confirmed live: real AI-crawler allowlist (GPTBot, Claude-Web, PerplexityBot, etc.), scraper blocklist, and the site's non-standard LLMs: directive all intact</t>
         </is>
       </c>
       <c r="E271" s="14" t="inlineStr">
@@ -7090,7 +7090,7 @@
       <c r="A272" s="4" t="n"/>
       <c r="B272" s="4" t="inlineStr">
         <is>
-          <t>Article JSON-LD on /blog/[slug], built from real per-post Sanity data (headline, image, datePublished/dateModified, author, canonical URL)</t>
+          <t>JSON-LD</t>
         </is>
       </c>
       <c r="C272" s="13" t="inlineStr">
@@ -7100,7 +7100,7 @@
       </c>
       <c r="D272" s="4" t="inlineStr">
         <is>
-          <t>verified live on a real post</t>
+          <t>WebSite + Person schema ported verbatim from the live homepage's actual &lt;script type="application/ld+json"&gt; tags (not reconstructed from memory) — rendered site-wide from src/lib/structured-data.ts in the root layout. The Person image was hardcoded to a /api/img/... legacy proxy path on the live site — rescued that headshot (downloaded it while still live, uploaded to Sanity as the author-tony-greenberg document's avatar) so the new site's JSON-LD has zero Manus dependency instead of just copying the fragile path forward</t>
         </is>
       </c>
       <c r="E272" s="14" t="inlineStr">
@@ -7113,7 +7113,7 @@
       <c r="A273" s="4" t="n"/>
       <c r="B273" s="4" t="inlineStr">
         <is>
-          <t>Build the full Manus/legacy-URL → Next.js-URL 301 redirect map (next.config.ts redirects() or Sanity redirect documents)</t>
+          <t>Article JSON-LD on /blog/[slug], built from real per-post Sanity data (headline, image, datePublished/dateModified, author, canonical URL)</t>
         </is>
       </c>
       <c r="C273" s="13" t="inlineStr">
@@ -7123,7 +7123,7 @@
       </c>
       <c r="D273" s="4" t="inlineStr">
         <is>
-          <t>hard QA gate, nothing proceeds to DNS cutover until this is complete and tested. First real pass done: extracted all 197 real path= routes from legacy's App.tsx router (not guessed — the actual route table), diffed against this app's real current routes (find src/app -maxdepth 1 -name page.tsx) + next.config.ts's existing redirect sources, normalizing :param/[param] syntax to compare like-for-like. Started at 41 real gaps, closed 10 with new redirects: /attention-theft/{blocker-finder,legal,report,weapons} (legacy registered both a bare AND a /attention-theft/-nested path for each, only the bare ones had redirects before), /find-my-car → /find-my, /the-index → /search (matching the fix already applied to other pages' dead links to it), /supplier-intake-long (bare) + /vendor-intake + /vendor-intake-long (+/:token) → the same real ramprate.com/biochain/supplier-intake destination the token'd path already redirected to, and /spamtoast + /youve-been-reported → / (the live half of legacy's "report a spammer" confrontation flow — a fake IP-fingerprinting/countdown-timer page; the other half, ReportSpammer.tsx, was already a documented drop in Phase 4, this is the same call for its sequel). 21 of the remaining 31 gaps need no redirect — they're /admin/*//analytics//edit/frqncy (internal tools never meant for public discovery) or already-documented intentional defers from Phase 4/7/10 (/clock-keeper-part-2, /ecosystem-map, /friend-gate, /friend-survey/:token, /medicine-sequencing, /m</t>
+          <t>verified live on a real post</t>
         </is>
       </c>
       <c r="E273" s="14" t="inlineStr">
@@ -7136,7 +7136,7 @@
       <c r="A274" s="4" t="n"/>
       <c r="B274" s="4" t="inlineStr">
         <is>
-          <t>/path/:archetype (src/app/path/[archetype]/page.tsx)</t>
+          <t>Build the full Manus/legacy-URL → Next.js-URL 301 redirect map (next.config.ts redirects() or Sanity redirect documents)</t>
         </is>
       </c>
       <c r="C274" s="13" t="inlineStr">
@@ -7146,7 +7146,7 @@
       </c>
       <c r="D274" s="4" t="inlineStr">
         <is>
-          <t>per-archetype landing page for /assessment's Builder/Crusader/Investor result, reusing lib/content/archetypes.ts. Real content ported in full (top-5 essential-reading list per archetype via allPostsForArchiveQuery, real PathSubscribeForm posting to /api/subscribe, AUTHORITY_ITEMS strip). Real bug fixed vs. legacy: replaced a hand-rolled inline-styled "Path not found" div with a real notFound() (this route's generateStaticParams only ever produces the 3 real keys). Verified live: all 3 archetype routes 200 OK, typecheck/lint clean.</t>
+          <t>hard QA gate, nothing proceeds to DNS cutover until this is complete and tested. First real pass done: extracted all 197 real path= routes from legacy's App.tsx router (not guessed — the actual route table), diffed against this app's real current routes (find src/app -maxdepth 1 -name page.tsx) + next.config.ts's existing redirect sources, normalizing :param/[param] syntax to compare like-for-like. Started at 41 real gaps, closed 10 with new redirects: /attention-theft/{blocker-finder,legal,report,weapons} (legacy registered both a bare AND a /attention-theft/-nested path for each, only the bare ones had redirects before), /find-my-car → /find-my, /the-index → /search (matching the fix already applied to other pages' dead links to it), /supplier-intake-long (bare) + /vendor-intake + /vendor-intake-long (+/:token) → the same real ramprate.com/biochain/supplier-intake destination the token'd path already redirected to, and /spamtoast + /youve-been-reported → / (the live half of legacy's "report a spammer" confrontation flow — a fake IP-fingerprinting/countdown-timer page; the other half, ReportSpammer.tsx, was already a documented drop in Phase 4, this is the same call for its sequel). 21 of the remaining 31 gaps need no redirect — they're /admin/*//analytics//edit/frqncy (internal tools never meant for public discovery) or already-documented intentional defers from Phase 4/7/10 (/clock-keeper-part-2, /ecosystem-map, /friend-gate, /friend-survey/:token, /medicine-sequencing, /m</t>
         </is>
       </c>
       <c r="E274" s="14" t="inlineStr">
@@ -7159,7 +7159,7 @@
       <c r="A275" s="4" t="n"/>
       <c r="B275" s="4" t="inlineStr">
         <is>
-          <t>/my-journey (src/app/my-journey/page.tsx + components/assessments/my-journey-dashboard.tsx)</t>
+          <t>/path/:archetype (src/app/path/[archetype]/page.tsx)</t>
         </is>
       </c>
       <c r="C275" s="13" t="inlineStr">
@@ -7169,7 +7169,7 @@
       </c>
       <c r="D275" s="4" t="inlineStr">
         <is>
-          <t>"My Journey Dashboard," real grid/timeline views across all 28 JOURNEY_MAP experiences, category/status filters, phase progress ring, recommended-next card, using the same real useJourneyProgress/JOURNEY_MAP completion tracking every "Find Your X" quiz already writes to (not the narrower tg_assessment_results cookie built for /self-portrait). Legacy's per-quiz scored-result caching (RESULT_KEYS, feeding a mini radar chart) was not ported — no quiz in this migration writes that data either, same honest-degradation call already made for /self-portrait's own composite radar. Fixed a real legacy dead link (/ecosystem-map, a still-unbuilt page) to /self-portrait. Verified live: 200 OK, real content confirmed, typecheck/lint clean.</t>
+          <t>per-archetype landing page for /assessment's Builder/Crusader/Investor result, reusing lib/content/archetypes.ts. Real content ported in full (top-5 essential-reading list per archetype via allPostsForArchiveQuery, real PathSubscribeForm posting to /api/subscribe, AUTHORITY_ITEMS strip). Real bug fixed vs. legacy: replaced a hand-rolled inline-styled "Path not found" div with a real notFound() (this route's generateStaticParams only ever produces the 3 real keys). Verified live: all 3 archetype routes 200 OK, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E275" s="14" t="inlineStr">
@@ -7182,7 +7182,7 @@
       <c r="A276" s="4" t="n"/>
       <c r="B276" s="4" t="inlineStr">
         <is>
-          <t>/the-open-door (src/app/the-open-door/page.tsx)</t>
+          <t>/my-journey (src/app/my-journey/page.tsx + components/assessments/my-journey-dashboard.tsx)</t>
         </is>
       </c>
       <c r="C276" s="13" t="inlineStr">
@@ -7192,7 +7192,7 @@
       </c>
       <c r="D276" s="4" t="inlineStr">
         <is>
-          <t>real press/credibility content: all 10 "Magic Genie" client-pitch prompts (real named targets — Marco Argenti/Goldman Sachs, Adam Smith/Disney, etc.), 18 real client testimonials, all 8 explicitly-labeled satirical "parody" quotes (kept with disclaimers, not presented as real). Real overlap found and reconciled: this page's publications/speaking/podcasts arrays substantially duplicate the already-shipped /published's fuller bibliography — kept only what /published doesn't cover (Forbes + Business Insider bylines, the Clinton Global Initiative keynote, 4 of 5 podcast appearances) and cross-linked to /published for the rest, same reconciliation pattern as /assessments vs /find-my. Real bugs fixed: 3 genie/keynote links pointed externally at tonygreenberg.com/&lt;slug&gt; for posts that are real internal posts in this migration — relinked to /blog/psychedelics-could-become-extractive-capitalism, /blog/boiling-the-human-summit-harvard-kurzweil, /blog/return-on-investment-going-green-going-green-2 (all verified 200); a bare self-link to tonygreenberg.com remapped to /. Ships as a pure Server Component (legacy's FadeIn/Section/editorial-component dependencies don't exist here and weren't needed). Verified live: 200 OK, real content in raw SSR HTML, typecheck/lint clean.</t>
+          <t>"My Journey Dashboard," real grid/timeline views across all 28 JOURNEY_MAP experiences, category/status filters, phase progress ring, recommended-next card, using the same real useJourneyProgress/JOURNEY_MAP completion tracking every "Find Your X" quiz already writes to (not the narrower tg_assessment_results cookie built for /self-portrait). Legacy's per-quiz scored-result caching (RESULT_KEYS, feeding a mini radar chart) was not ported — no quiz in this migration writes that data either, same honest-degradation call already made for /self-portrait's own composite radar. Fixed a real legacy dead link (/ecosystem-map, a still-unbuilt page) to /self-portrait. Verified live: 200 OK, real content confirmed, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E276" s="14" t="inlineStr">
@@ -7205,7 +7205,7 @@
       <c r="A277" s="4" t="n"/>
       <c r="B277" s="4" t="inlineStr">
         <is>
-          <t>Homepage "Recent Updates" band (2026-09-29)</t>
+          <t>/the-open-door (src/app/the-open-door/page.tsx)</t>
         </is>
       </c>
       <c r="C277" s="13" t="inlineStr">
@@ -7215,7 +7215,7 @@
       </c>
       <c r="D277" s="4" t="inlineStr">
         <is>
-          <t>on the live site (a newer Blog.tsx than _legacy-manus-app/, so rebuilt from the live page's markup), replacing the older "Latest Thinking" pair. Found while doing it: two live essays are missing from Sanity, the-tollbooth-and-the-alternative (Aug 18, 2026, the live site's newest) and what-quest-could-fix. Both were published on live after the legacy snapshot and need importing.</t>
+          <t>real press/credibility content: all 10 "Magic Genie" client-pitch prompts (real named targets — Marco Argenti/Goldman Sachs, Adam Smith/Disney, etc.), 18 real client testimonials, all 8 explicitly-labeled satirical "parody" quotes (kept with disclaimers, not presented as real). Real overlap found and reconciled: this page's publications/speaking/podcasts arrays substantially duplicate the already-shipped /published's fuller bibliography — kept only what /published doesn't cover (Forbes + Business Insider bylines, the Clinton Global Initiative keynote, 4 of 5 podcast appearances) and cross-linked to /published for the rest, same reconciliation pattern as /assessments vs /find-my. Real bugs fixed: 3 genie/keynote links pointed externally at tonygreenberg.com/&lt;slug&gt; for posts that are real internal posts in this migration — relinked to /blog/psychedelics-could-become-extractive-capitalism, /blog/boiling-the-human-summit-harvard-kurzweil, /blog/return-on-investment-going-green-going-green-2 (all verified 200); a bare self-link to tonygreenberg.com remapped to /. Ships as a pure Server Component (legacy's FadeIn/Section/editorial-component dependencies don't exist here and weren't needed). Verified live: 200 OK, real content in raw SSR HTML, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E277" s="14" t="inlineStr">
@@ -7228,7 +7228,7 @@
       <c r="A278" s="4" t="n"/>
       <c r="B278" s="4" t="inlineStr">
         <is>
-          <t>Re-sync the legacy reference</t>
+          <t>Homepage "Recent Updates" band (2026-09-29)</t>
         </is>
       </c>
       <c r="C278" s="13" t="inlineStr">
@@ -7238,7 +7238,7 @@
       </c>
       <c r="D278" s="4" t="inlineStr">
         <is>
-          <t>_legacy-manus-app/ is older than what's live (Recent Updates proves it), so visual diffs should be against the live site, not only that folder. Closed 2026-10-08: done the way this item suggests: every comparison since 2026-10-01 is against the live site itself (163 pages + 121 posts on 2026-10-01, 188 pages on 2026-10-07, 18 redesigned pages on 2026-10-08), with _legacy-manus-app/ used only as the code reference.</t>
+          <t>on the live site (a newer Blog.tsx than _legacy-manus-app/, so rebuilt from the live page's markup), replacing the older "Latest Thinking" pair. Found while doing it: two live essays are missing from Sanity, the-tollbooth-and-the-alternative (Aug 18, 2026, the live site's newest) and what-quest-could-fix. Both were published on live after the legacy snapshot and need importing.</t>
         </is>
       </c>
       <c r="E278" s="14" t="inlineStr">
@@ -7251,7 +7251,7 @@
       <c r="A279" s="4" t="n"/>
       <c r="B279" s="4" t="inlineStr">
         <is>
-          <t>Visual diff pass: every ported page vs</t>
+          <t>Re-sync the legacy reference</t>
         </is>
       </c>
       <c r="C279" s="13" t="inlineStr">
@@ -7261,7 +7261,7 @@
       </c>
       <c r="D279" s="4" t="inlineStr">
         <is>
-          <t>legacy page Closed 2026-10-08: covered by the live-site sweeps above (screenshots and measured title/label/spacing per page, see the 2026-10-01, 10-02, 10-07 and 10-08 entries in this phase). Remaining differences are listed as decisions (Cormorant titles, /find-my header) or deliberate (CONTRIBUTING rule 20).</t>
+          <t>_legacy-manus-app/ is older than what's live (Recent Updates proves it), so visual diffs should be against the live site, not only that folder. Closed 2026-10-08: done the way this item suggests: every comparison since 2026-10-01 is against the live site itself (163 pages + 121 posts on 2026-10-01, 188 pages on 2026-10-07, 18 redesigned pages on 2026-10-08), with _legacy-manus-app/ used only as the code reference.</t>
         </is>
       </c>
       <c r="E279" s="14" t="inlineStr">
@@ -7274,7 +7274,7 @@
       <c r="A280" s="4" t="n"/>
       <c r="B280" s="4" t="inlineStr">
         <is>
-          <t>Padding / spacing on the story pages matched to live (2026-10-01)</t>
+          <t>Visual diff pass: every ported page vs</t>
         </is>
       </c>
       <c r="C280" s="13" t="inlineStr">
@@ -7284,7 +7284,7 @@
       </c>
       <c r="D280" s="4" t="inlineStr">
         <is>
-          <t>Measured margins, text column and spacing on 31 pages, live vs a production build, at 375px and 1280px. The "door" story pages were the clear mismatch: live's text column is ~546px (ours was 720px), 20px side margins on phones / 40px on desktop, body text 19px/1.8 on phones and 18px/1.85 on desktop (ours 16px/1.5). Fixed on /the-body, /engine-room, /under-nda, /the-nightstand, /the-web, /the-territory, /about, /intel (Intel uses live's 16.8px/1.9; About's hero line 480px max, 18.4px/1.8). Re-measured: all 8 match live to within 2px (About's column 28px narrower), no sideways scroll at 375px.</t>
+          <t>legacy page Closed 2026-10-08: covered by the live-site sweeps above (screenshots and measured title/label/spacing per page, see the 2026-10-01, 10-02, 10-07 and 10-08 entries in this phase). Remaining differences are listed as decisions (Cormorant titles, /find-my header) or deliberate (CONTRIBUTING rule 20).</t>
         </is>
       </c>
       <c r="E280" s="14" t="inlineStr">
@@ -7297,7 +7297,7 @@
       <c r="A281" s="4" t="n"/>
       <c r="B281" s="4" t="inlineStr">
         <is>
-          <t>Header-to-title spacing re-checked (2026-10-02)</t>
+          <t>Padding / spacing on the story pages matched to live (2026-10-01)</t>
         </is>
       </c>
       <c r="C281" s="13" t="inlineStr">
@@ -7307,7 +7307,7 @@
       </c>
       <c r="D281" s="4" t="inlineStr">
         <is>
-          <t>The 2026-10-01 note compared different things: live's header wasn't measured (it showed 0), so "96px vs 168px" was really 161px vs 168px from the top of the page. Measured again from the top of the page, live vs a production build, at 375px and 1280px: most pages were already within 10px. Fixed the real gaps: /the-open-door (now live's dark centered hero band, 56px title, 546px text column; title was 72px too high), /start-here (live's 48px/96px top padding; 25px too high on desktop), /invest and /engage (label spacing and live's 32px/51px title; /invest's desktop title was 36px), /impact-dashboard on phones (card edge to edge under the header like live; title was 89px too low). Re-measured: all within 8px of live, no sideways scroll at 375px, no JS errors.</t>
+          <t>Measured margins, text column and spacing on 31 pages, live vs a production build, at 375px and 1280px. The "door" story pages were the clear mismatch: live's text column is ~546px (ours was 720px), 20px side margins on phones / 40px on desktop, body text 19px/1.8 on phones and 18px/1.85 on desktop (ours 16px/1.5). Fixed on /the-body, /engine-room, /under-nda, /the-nightstand, /the-web, /the-territory, /about, /intel (Intel uses live's 16.8px/1.9; About's hero line 480px max, 18.4px/1.8). Re-measured: all 8 match live to within 2px (About's column 28px narrower), no sideways scroll at 375px.</t>
         </is>
       </c>
       <c r="E281" s="14" t="inlineStr">
@@ -7320,7 +7320,7 @@
       <c r="A282" s="4" t="n"/>
       <c r="B282" s="4" t="inlineStr">
         <is>
-          <t>HumanOS headings in capitals like live (2026-10-02, owner said yes)</t>
+          <t>Header-to-title spacing re-checked (2026-10-02)</t>
         </is>
       </c>
       <c r="C282" s="13" t="inlineStr">
@@ -7330,7 +7330,7 @@
       </c>
       <c r="D282" s="4" t="inlineStr">
         <is>
-          <t>the 4 headings live capitalises on /humanos (title, "Are you a Maximizer...", "Take the Diagnostic", "The Diagnostic") get uppercase; the words are unchanged. The subpages already matched.</t>
+          <t>The 2026-10-01 note compared different things: live's header wasn't measured (it showed 0), so "96px vs 168px" was really 161px vs 168px from the top of the page. Measured again from the top of the page, live vs a production build, at 375px and 1280px: most pages were already within 10px. Fixed the real gaps: /the-open-door (now live's dark centered hero band, 56px title, 546px text column; title was 72px too high), /start-here (live's 48px/96px top padding; 25px too high on desktop), /invest and /engage (label spacing and live's 32px/51px title; /invest's desktop title was 36px), /impact-dashboard on phones (card edge to edge under the header like live; title was 89px too low). Re-measured: all within 8px of live, no sideways scroll at 375px, no JS errors.</t>
         </is>
       </c>
       <c r="E282" s="14" t="inlineStr">
@@ -7343,7 +7343,7 @@
       <c r="A283" s="4" t="n"/>
       <c r="B283" s="4" t="inlineStr">
         <is>
-          <t>More layout gaps matched to live (2026-10-02)</t>
+          <t>HumanOS headings in capitals like live (2026-10-02, owner said yes)</t>
         </is>
       </c>
       <c r="C283" s="13" t="inlineStr">
@@ -7353,7 +7353,7 @@
       </c>
       <c r="D283" s="4" t="inlineStr">
         <is>
-          <t>/series (live's centered 546px column, and a bug fixed: every card kept an empty 240px picture column, squeezing the text; live's per-series picture is one generic placeholder on the Manus proxy, so not copied), /humanos (middle section 900px like live), homepage desktop widths (hero text 804px, Four Doors 1000px, Editor's Picks 1168px, GemSpark edge, section title sizes; live's /blog now shows the homepage), /find-my (photo undimmed and plain background, like live; our site header kept). Re-measured: headings within 3px (/series) to 20px (homepage) of live, no sideways scroll, no JS errors. Note: live's "New here?" tour bar sits over its header and doesn't move the page, so it doesn't affect these numbers.</t>
+          <t>the 4 headings live capitalises on /humanos (title, "Are you a Maximizer...", "Take the Diagnostic", "The Diagnostic") get uppercase; the words are unchanged. The subpages already matched.</t>
         </is>
       </c>
       <c r="E283" s="14" t="inlineStr">
@@ -7366,7 +7366,7 @@
       <c r="A284" s="4" t="n"/>
       <c r="B284" s="4" t="inlineStr">
         <is>
-          <t>Full sweep vs live (2026-10-02)</t>
+          <t>More layout gaps matched to live (2026-10-02)</t>
         </is>
       </c>
       <c r="C284" s="13" t="inlineStr">
@@ -7376,7 +7376,7 @@
       </c>
       <c r="D284" s="4" t="inlineStr">
         <is>
-          <t>142 pages (every non-blog page, 3 of each templated set) at 375px and 1280px, title position, text column, title size. Fixed the shared causes: BrewSoul (live wraps most pages in its frame twice, so a second 52px offset plus the category badge; the landing, cities, directory and quiz pages have neither: src/components/brewsoul/brewsoul-main.tsx; intro paragraphs uncapped like live; 38px titles), Kava (live's extra 52px offset), /the-body, /the-nightstand, /the-web (405px top photo like live), the 6 peptide pages (live's 768/896px intro column), /journeys, /pick-up-the-phone, /published, /ecosystem (546px story column and live's text size). Re-measured: 110 of 120 within 40px / 60px of live.</t>
+          <t>/series (live's centered 546px column, and a bug fixed: every card kept an empty 240px picture column, squeezing the text; live's per-series picture is one generic placeholder on the Manus proxy, so not copied), /humanos (middle section 900px like live), homepage desktop widths (hero text 804px, Four Doors 1000px, Editor's Picks 1168px, GemSpark edge, section title sizes; live's /blog now shows the homepage), /find-my (photo undimmed and plain background, like live; our site header kept). Re-measured: headings within 3px (/series) to 20px (homepage) of live, no sideways scroll, no JS errors. Note: live's "New here?" tour bar sits over its header and doesn't move the page, so it doesn't affect these numbers.</t>
         </is>
       </c>
       <c r="E284" s="14" t="inlineStr">
@@ -7389,7 +7389,7 @@
       <c r="A285" s="4" t="n"/>
       <c r="B285" s="4" t="inlineStr">
         <is>
-          <t>Sweep leftovers fixed (2026-10-06)</t>
+          <t>Full sweep vs live (2026-10-02)</t>
         </is>
       </c>
       <c r="C285" s="13" t="inlineStr">
@@ -7399,7 +7399,7 @@
       </c>
       <c r="D285" s="4" t="inlineStr">
         <is>
-          <t>Ported legacy's exact title sizes, margins and column widths. Measured live vs a production build at 375px and 1280px (H1 distance from the top, H1 size, intro and table widths). Now within 8px and the same title size on /published, /brewsoul/first-sip, /brewsoul/home, /brewsoul/chains (intro 912px like live), /brewsoul/browse, /brewsoul/directory (3-column 952px grid like live), /brewsoul and /brewsoul/quiz (intro 520px), /amplifier (546px column), /diamond-cut, /speaking, /living-declaration, /spirits, /protecting-your-business (tables 730px), and the 5 HumanOS subpages (titles smaller like live, 752px column). No sideways scroll at 375px. Left on purpose: /self-portrait (font matches; our page has a different title and no back link, so it sits 23-57px higher), BrewSoul pages 3-6px off (the shared journey bar row), and the different-layout pages /dharma-finder, /grant-study, /search, /quiz_25q, /soulscore. Also: /brewsoul/quiz rebuilt as a step registry (src/components/brewsoul/brewsoul-quiz/: parent + hook/ + components/step-* + data/), same questions, scoring and look; Back/Skip/Retake use lucide icons. New CONTRIBUTING rule 19 (multi-step flows, FydoPartner pattern). brewsoul-welcome-quiz.tsx (/brewsoul) still has the old shape and text arrows.</t>
+          <t>142 pages (every non-blog page, 3 of each templated set) at 375px and 1280px, title position, text column, title size. Fixed the shared causes: BrewSoul (live wraps most pages in its frame twice, so a second 52px offset plus the category badge; the landing, cities, directory and quiz pages have neither: src/components/brewsoul/brewsoul-main.tsx; intro paragraphs uncapped like live; 38px titles), Kava (live's extra 52px offset), /the-body, /the-nightstand, /the-web (405px top photo like live), the 6 peptide pages (live's 768/896px intro column), /journeys, /pick-up-the-phone, /published, /ecosystem (546px story column and live's text size). Re-measured: 110 of 120 within 40px / 60px of live.</t>
         </is>
       </c>
       <c r="E285" s="14" t="inlineStr">
@@ -7412,7 +7412,7 @@
       <c r="A286" s="4" t="n"/>
       <c r="B286" s="4" t="inlineStr">
         <is>
-          <t>Match live's redesigned pages (2026-10-06, owner said go)</t>
+          <t>Sweep leftovers fixed (2026-10-06)</t>
         </is>
       </c>
       <c r="C286" s="13" t="inlineStr">
@@ -7422,7 +7422,7 @@
       </c>
       <c r="D286" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">/self-portrait (live: dark page, progress ring, "N more brushstrokes" lock until 5 assessments), /grant-study and /dharma-finder (live opens straight on question 1, no intro screen), /quiz_25q (live adds a hero picture above the title; rescue it into Sanity first), /search (live: one search box across essays, BrewSoul, peptides, HumanOS, assessments, kava and pages with filter chips). Measure live vs a production build at 375px and 1280px when done. Done 2026-10-06: /grant-study and /dharma-finder open straight on question 1 like live (title block / part header above the first question, live's 546px column, plain page, credit under every question), both rebuilt as step registries (rule 19); measured within 3px of live at the top (dharma's question block within 7px). /quiz_25q's hero rescued into Sanity and placed like live (within 2px). Found and fixed on the way: on the deployed copy /grant-study's answer buttons could not be clicked (the themed page background was fixed z-0, painted over the quiz); ThemedBackground is now -z-10 pointer-events-none (backgrounds unchanged on all 21 pages that use it), and the shared email gate no longer scrolls sideways on phones. Both quizzes clicked through to results in Chrome and Safari. /self-portrait restyled to live (dark page, "The Composite You", progress ring, "N More Brushstrokes Needed" lock until 5 done, live's copy) on our real cookie data; within 3px of live at both widths; tested with 0, 2 and 6 completed. Counts are ours (13 </t>
+          <t>Ported legacy's exact title sizes, margins and column widths. Measured live vs a production build at 375px and 1280px (H1 distance from the top, H1 size, intro and table widths). Now within 8px and the same title size on /published, /brewsoul/first-sip, /brewsoul/home, /brewsoul/chains (intro 912px like live), /brewsoul/browse, /brewsoul/directory (3-column 952px grid like live), /brewsoul and /brewsoul/quiz (intro 520px), /amplifier (546px column), /diamond-cut, /speaking, /living-declaration, /spirits, /protecting-your-business (tables 730px), and the 5 HumanOS subpages (titles smaller like live, 752px column). No sideways scroll at 375px. Left on purpose: /self-portrait (font matches; our page has a different title and no back link, so it sits 23-57px higher), BrewSoul pages 3-6px off (the shared journey bar row), and the different-layout pages /dharma-finder, /grant-study, /search, /quiz_25q, /soulscore. Also: /brewsoul/quiz rebuilt as a step registry (src/components/brewsoul/brewsoul-quiz/: parent + hook/ + components/step-* + data/), same questions, scoring and look; Back/Skip/Retake use lucide icons. New CONTRIBUTING rule 19 (multi-step flows, FydoPartner pattern). brewsoul-welcome-quiz.tsx (/brewsoul) still has the old shape and text arrows.</t>
         </is>
       </c>
       <c r="E286" s="14" t="inlineStr">
@@ -7435,7 +7435,7 @@
       <c r="A287" s="4" t="n"/>
       <c r="B287" s="4" t="inlineStr">
         <is>
-          <t>Still different from live (decided 2026-10-09)</t>
+          <t>Match live's redesigned pages (2026-10-06, owner said go)</t>
         </is>
       </c>
       <c r="C287" s="13" t="inlineStr">
@@ -7445,7 +7445,7 @@
       </c>
       <c r="D287" s="4" t="inlineStr">
         <is>
-          <t>blog posts (done) (done 2026-10-07, see Phase 5); /find-my on live hides the site header. /walk-through is a 404 on live now. Owner: keep our site menu on /find-my (visitors can still reach the rest of the site); nothing left to change.</t>
+          <t xml:space="preserve">/self-portrait (live: dark page, progress ring, "N more brushstrokes" lock until 5 assessments), /grant-study and /dharma-finder (live opens straight on question 1, no intro screen), /quiz_25q (live adds a hero picture above the title; rescue it into Sanity first), /search (live: one search box across essays, BrewSoul, peptides, HumanOS, assessments, kava and pages with filter chips). Measure live vs a production build at 375px and 1280px when done. Done 2026-10-06: /grant-study and /dharma-finder open straight on question 1 like live (title block / part header above the first question, live's 546px column, plain page, credit under every question), both rebuilt as step registries (rule 19); measured within 3px of live at the top (dharma's question block within 7px). /quiz_25q's hero rescued into Sanity and placed like live (within 2px). Found and fixed on the way: on the deployed copy /grant-study's answer buttons could not be clicked (the themed page background was fixed z-0, painted over the quiz); ThemedBackground is now -z-10 pointer-events-none (backgrounds unchanged on all 21 pages that use it), and the shared email gate no longer scrolls sideways on phones. Both quizzes clicked through to results in Chrome and Safari. /self-portrait restyled to live (dark page, "The Composite You", progress ring, "N More Brushstrokes Needed" lock until 5 done, live's copy) on our real cookie data; within 3px of live at both widths; tested with 0, 2 and 6 completed. Counts are ours (13 </t>
         </is>
       </c>
       <c r="E287" s="14" t="inlineStr">
@@ -7458,7 +7458,7 @@
       <c r="A288" s="4" t="n"/>
       <c r="B288" s="4" t="inlineStr">
         <is>
-          <t>Design change on live (owner: "match live", 2026-10-09)</t>
+          <t>Still different from live (decided 2026-10-09)</t>
         </is>
       </c>
       <c r="C288" s="13" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="D288" s="4" t="inlineStr">
         <is>
-          <t>live's story pages now use Cormorant Garamond for titles (ours: Playfair Display), a lighter title weight (400 vs our 700), and a red eyebrow label (#8E1E25, wider letter spacing) instead of our gold. A site-wide font swap is a design call, so not done. Done 2026-10-09: a fresh sweep of 163 live pages found live has since dropped Cormorant from the story pages (only /living-declaration uses it, ours already matched) and mostly uses Playfair; the real differences were fixed: every heading on /attention-theft in Fraunces 700 (section-wide, like Kava), /supplier-intake title in the system serif, and live's fluid title sizes on /about, /articles, /the-letter, /the-philosophy, /clock-keeper-part-2, /living-declaration (measured at 375/640/820/1024/1280, now identical). Label colours stay darker than live on purpose (contrast, rule 20).</t>
+          <t>blog posts (done) (done 2026-10-07, see Phase 5); /find-my on live hides the site header. /walk-through is a 404 on live now. Owner: keep our site menu on /find-my (visitors can still reach the rest of the site); nothing left to change.</t>
         </is>
       </c>
       <c r="E288" s="14" t="inlineStr">
@@ -7481,7 +7481,7 @@
       <c r="A289" s="4" t="n"/>
       <c r="B289" s="4" t="inlineStr">
         <is>
-          <t>Link check across all ported pages (no 404s, no broken internal cross-references)</t>
+          <t>Design change on live (owner: "match live", 2026-10-09)</t>
         </is>
       </c>
       <c r="C289" s="13" t="inlineStr">
@@ -7491,7 +7491,7 @@
       </c>
       <c r="D289" s="4" t="inlineStr">
         <is>
-          <t>First full pass done 2026-09-29 (510 pages crawled from the sitemap plus every internal link, on a production build). Fixed in code: /brewsoul/coffee/…-tarrazú 404 (the route got the id still percent-encoded), 30+ links that went through the /assessments/* redirects, /find-your-me's dead Homeaglow link, the two root-level Iboga essay links, and the dead FauxTony nav item. Fixed as Sanity drafts (scripts/fix-blog-body-links.ts, 14 posts): broken post links, leaked !… placeholder text, Energy Is Money's split author bio, and scraped WordPress furniture ("Share this / Related / You Might Also Like / Copyright", "Show More / Top News", [mc4wp_form]). Left for a decision: /framework's "Ask FauxTony" button, when-healing-becomes-extraction's two links to a Dr. Lee case file that doesn't exist, and the-clock-keeper-chronicles-part-1's link to the deferred /clock-keeper-part-2. Re-run after the drafts are published. 2026-10-01 re-run (local production build, all 498 sitemap URLs load; 440 unique internal links): 5 broken. Fixed as a Sanity draft: molecule-as-mirror-10-what-the-pioneers-know's "Final installment" link pointed at a non-existent part-10 slug (now part 11; live also shows that line twice, kept). Already fixed in a waiting draft: forever-chemicals-... → /blog/psychedelic-readiness-index. Still the 3 known decisions: /fauxtony (from /framework), /clock-keeper-part-2, /blog/the-case-file-dr-samuel-lee. 2026-10-08 re-run (production build, all 497 sitemap pages, 453 unique i</t>
+          <t>live's story pages now use Cormorant Garamond for titles (ours: Playfair Display), a lighter title weight (400 vs our 700), and a red eyebrow label (#8E1E25, wider letter spacing) instead of our gold. A site-wide font swap is a design call, so not done. Done 2026-10-09: a fresh sweep of 163 live pages found live has since dropped Cormorant from the story pages (only /living-declaration uses it, ours already matched) and mostly uses Playfair; the real differences were fixed: every heading on /attention-theft in Fraunces 700 (section-wide, like Kava), /supplier-intake title in the system serif, and live's fluid title sizes on /about, /articles, /the-letter, /the-philosophy, /clock-keeper-part-2, /living-declaration (measured at 375/640/820/1024/1280, now identical). Label colours stay darker than live on purpose (contrast, rule 20).</t>
         </is>
       </c>
       <c r="E289" s="14" t="inlineStr">
@@ -7504,7 +7504,7 @@
       <c r="A290" s="4" t="n"/>
       <c r="B290" s="4" t="inlineStr">
         <is>
-          <t>Sitemap: no noindex pages (2026-10-08)</t>
+          <t>Link check across all ported pages (no 404s, no broken internal cross-references)</t>
         </is>
       </c>
       <c r="C290" s="13" t="inlineStr">
@@ -7514,7 +7514,7 @@
       </c>
       <c r="D290" s="4" t="inlineStr">
         <is>
-          <t>the password-locked /blog/you-are-the-moat was in the sitemap while telling Google not to index it (a Search Console sitemap warning). Gated posts and posts that redirect are now left out (src/app/sitemap.ts); all 497 sitemap addresses return 200 with a matching canonical and no noindex. The 82 warnings Search Console shows are for the old live sitemap, so re-check them after cutover.</t>
+          <t>First full pass done 2026-09-29 (510 pages crawled from the sitemap plus every internal link, on a production build). Fixed in code: /brewsoul/coffee/…-tarrazú 404 (the route got the id still percent-encoded), 30+ links that went through the /assessments/* redirects, /find-your-me's dead Homeaglow link, the two root-level Iboga essay links, and the dead FauxTony nav item. Fixed as Sanity drafts (scripts/fix-blog-body-links.ts, 14 posts): broken post links, leaked !… placeholder text, Energy Is Money's split author bio, and scraped WordPress furniture ("Share this / Related / You Might Also Like / Copyright", "Show More / Top News", [mc4wp_form]). Left for a decision: /framework's "Ask FauxTony" button, when-healing-becomes-extraction's two links to a Dr. Lee case file that doesn't exist, and the-clock-keeper-chronicles-part-1's link to the deferred /clock-keeper-part-2. Re-run after the drafts are published. 2026-10-01 re-run (local production build, all 498 sitemap URLs load; 440 unique internal links): 5 broken. Fixed as a Sanity draft: molecule-as-mirror-10-what-the-pioneers-know's "Final installment" link pointed at a non-existent part-10 slug (now part 11; live also shows that line twice, kept). Already fixed in a waiting draft: forever-chemicals-... → /blog/psychedelic-readiness-index. Still the 3 known decisions: /fauxtony (from /framework), /clock-keeper-part-2, /blog/the-case-file-dr-samuel-lee. 2026-10-08 re-run (production build, all 497 sitemap pages, 453 unique i</t>
         </is>
       </c>
       <c r="E290" s="14" t="inlineStr">
@@ -7527,7 +7527,7 @@
       <c r="A291" s="4" t="n"/>
       <c r="B291" s="4" t="inlineStr">
         <is>
-          <t>Lighthouse pass (performance/accessibility/SEO) on top 20 pages by traffic 2026-09-30, 20 key pages (no traffic data yet), local production …</t>
+          <t>Sitemap: no noindex pages (2026-10-08)</t>
         </is>
       </c>
       <c r="C291" s="13" t="inlineStr">
@@ -7537,7 +7537,7 @@
       </c>
       <c r="D291" s="4" t="inlineStr">
         <is>
-          <t>build, mobile: averages performance 87, accessibility 99→100, best practices 100, SEO 92→100, CLS 0 everywhere. Fixed: public/robots.txt had an LLMs: line (not a real directive) that made Google treat the whole file as invalid, now a comment; h3/h4 headings skipping a level on /assessments, /kava, /peptide-watch (same look, right tag); the Kava and /attention-theft back-arrow links had no accessible name on phones; two small phone-width contrast misses. Left: performance is local-machine only (±10-15 points, see CONTRIBUTING.md); the slowest were / 76 (LCP 5.2 s), /psychedelic-readiness-index 82, /iboga-ibogaine 83. Re-run against the Netlify deploy before launch. 2026-10-06 re-run against the Netlify deploy (14 key pages, mobile): accessibility 100 and CLS 0 on every page, SEO clean (only the expected netlify.app noindex), performance 77-97 held back by 3-4 s LCP. Fixed: all 21 hero images moved off the deprecated priority prop to fetchPriority="high" + loading="eager" (Next 16); /iboga-ibogaine hero and the first card on /blog and category pages no longer lazy-loaded; sizes on the Four Doors cards (~150 KiB per page), /humanos diagram (~100 KiB) and /about headshot; urlFor no longer imports the Sanity client, so ~115 KB of Sanity client code stopped loading on / and /blog; React hydration error #418 on / and /blog (post dates) gone, checked in two time zones; /blog is static again; empty icon &lt;th&gt;s on /iboga-ibogaine labelled; category page reads use sanityFetch(). Left: se</t>
+          <t>the password-locked /blog/you-are-the-moat was in the sitemap while telling Google not to index it (a Search Console sitemap warning). Gated posts and posts that redirect are now left out (src/app/sitemap.ts); all 497 sitemap addresses return 200 with a matching canonical and no noindex. The 82 warnings Search Console shows are for the old live sitemap, so re-check them after cutover.</t>
         </is>
       </c>
       <c r="E291" s="14" t="inlineStr">
@@ -7550,7 +7550,7 @@
       <c r="A292" s="4" t="n"/>
       <c r="B292" s="4" t="inlineStr">
         <is>
-          <t>No Manus links anywhere (2026-10-09, owner: "drop them everywhere")</t>
+          <t>Lighthouse pass (performance/accessibility/SEO) on top 20 pages by traffic 2026-09-30, 20 key pages (no traffic data yet), local production …</t>
         </is>
       </c>
       <c r="C292" s="13" t="inlineStr">
@@ -7560,7 +7560,7 @@
       </c>
       <c r="D292" s="4" t="inlineStr">
         <is>
-          <t>every *.manus.space link removed from code and essays. Lists of "try this next" apps lose those entries (journey tracker, Find Your Me results and next steps, /find-my, search directory, Sake and Grant Study results, BrewSoul footer, The Mirror); The Magnetic Partner's and The Temple Keeper's next step now go to their first in-site assessment (/grant-study, /consciousness-scale); their empty "Find Your _" section hides itself; /recent-creations, /spirits and /ecosystem-map keep the cards, unlinked. Clarisse Abelarde now links to her own site clarisseartist.com (owner gave it) on /about and in essays. Essays: lib/sanity/portable-text.tsx rewrites tonygreenberg.manus.space/&lt;path&gt; to /&lt;path&gt;, clarisseart.manus.space to clarisseartist.com (same paths), and renders other Manus app links as plain text (no Sanity drafts). Verified on a production build: no clickable *.manus.space link in any page, no manus.space in any browser script; 13 affected pages load (200).</t>
+          <t>build, mobile: averages performance 87, accessibility 99→100, best practices 100, SEO 92→100, CLS 0 everywhere. Fixed: public/robots.txt had an LLMs: line (not a real directive) that made Google treat the whole file as invalid, now a comment; h3/h4 headings skipping a level on /assessments, /kava, /peptide-watch (same look, right tag); the Kava and /attention-theft back-arrow links had no accessible name on phones; two small phone-width contrast misses. Left: performance is local-machine only (±10-15 points, see CONTRIBUTING.md); the slowest were / 76 (LCP 5.2 s), /psychedelic-readiness-index 82, /iboga-ibogaine 83. Re-run against the Netlify deploy before launch. 2026-10-06 re-run against the Netlify deploy (14 key pages, mobile): accessibility 100 and CLS 0 on every page, SEO clean (only the expected netlify.app noindex), performance 77-97 held back by 3-4 s LCP. Fixed: all 21 hero images moved off the deprecated priority prop to fetchPriority="high" + loading="eager" (Next 16); /iboga-ibogaine hero and the first card on /blog and category pages no longer lazy-loaded; sizes on the Four Doors cards (~150 KiB per page), /humanos diagram (~100 KiB) and /about headshot; urlFor no longer imports the Sanity client, so ~115 KB of Sanity client code stopped loading on / and /blog; React hydration error #418 on / and /blog (post dates) gone, checked in two time zones; /blog is static again; empty icon &lt;th&gt;s on /iboga-ibogaine labelled; category page reads use sanityFetch(). Left: se</t>
         </is>
       </c>
       <c r="E292" s="14" t="inlineStr">
@@ -7573,7 +7573,7 @@
       <c r="A293" s="4" t="n"/>
       <c r="B293" s="4" t="inlineStr">
         <is>
-          <t>Owner answers, round 2 (2026-10-09)</t>
+          <t>No Manus links anywhere (2026-10-09, owner: "drop them everywhere")</t>
         </is>
       </c>
       <c r="C293" s="13" t="inlineStr">
@@ -7583,7 +7583,7 @@
       </c>
       <c r="D293" s="4" t="inlineStr">
         <is>
-          <t>(1) real counts instead of live's typed numbers: /charity-scorecard intro and description ("98"/"Ninety-eight" → STATS.totalCharities = 103), /impact-dashboard ("100" → passed in from the page so the browser doesn't load the charity list), /the-index (prop), search directory coffees 103 → 107 (typed, with a note, since it ships to the search pop-up); (2) The Mirror results no longer list the 4 *.manus.space apps (the "Explore further" section hides when empty); (3) /framework's "Ask FauxTony" button and its lead-in line removed; the Dr. Lee case-file link (4 places in when-healing-becomes-extraction, original and updated versions) renders as plain text through a DEAD_INTERNAL_LINKS list in lib/sanity/portable-text.tsx (no Sanity draft needed); (4) B Corp: checked live, nothing shown on either site, no change. Verified on a production build: the counts read 103, /framework has no FauxTony block, the essay has 0 links to the case file and keeps the words, /the-index shows "103 charities" when searching "charity".</t>
+          <t>every *.manus.space link removed from code and essays. Lists of "try this next" apps lose those entries (journey tracker, Find Your Me results and next steps, /find-my, search directory, Sake and Grant Study results, BrewSoul footer, The Mirror); The Magnetic Partner's and The Temple Keeper's next step now go to their first in-site assessment (/grant-study, /consciousness-scale); their empty "Find Your _" section hides itself; /recent-creations, /spirits and /ecosystem-map keep the cards, unlinked. Clarisse Abelarde now links to her own site clarisseartist.com (owner gave it) on /about and in essays. Essays: lib/sanity/portable-text.tsx rewrites tonygreenberg.manus.space/&lt;path&gt; to /&lt;path&gt;, clarisseart.manus.space to clarisseartist.com (same paths), and renders other Manus app links as plain text (no Sanity drafts). Verified on a production build: no clickable *.manus.space link in any page, no manus.space in any browser script; 13 affected pages load (200).</t>
         </is>
       </c>
       <c r="E293" s="14" t="inlineStr">
@@ -7596,7 +7596,7 @@
       <c r="A294" s="4" t="n"/>
       <c r="B294" s="4" t="inlineStr">
         <is>
-          <t>Arrows in buttons and links are icons (2026-10-09, owner said yes)</t>
+          <t>Owner answers, round 2 (2026-10-09)</t>
         </is>
       </c>
       <c r="C294" s="13" t="inlineStr">
@@ -7606,7 +7606,7 @@
       </c>
       <c r="D294" s="4" t="inlineStr">
         <is>
-          <t>113 typed arrows in 52 files (button and link labels, "Next"/"See My Results" toggles, decorative arrow spans, the walk-through "See the..." labels, the Letter's "I'm in" button) replaced with lucide ArrowRight/ArrowLeft (size-[1em], inside inline-flex items-center gap-1.5, so the parent layout is untouched). Left as content on purpose: arrows inside Tony's text and data (health findings, origins, iboga compass options, process flows like "Inherit → Wake → Choose → Act", share text), the "← you" marker on the consciousness scale, and &lt;option&gt; sort labels (an option can't hold an icon). Checked on 16 pages at 375 and 1280: no typed arrow left in any link or button, no sideways scroll, no JS errors; close-up screenshots of the new icons.</t>
+          <t>(1) real counts instead of live's typed numbers: /charity-scorecard intro and description ("98"/"Ninety-eight" → STATS.totalCharities = 103), /impact-dashboard ("100" → passed in from the page so the browser doesn't load the charity list), /the-index (prop), search directory coffees 103 → 107 (typed, with a note, since it ships to the search pop-up); (2) The Mirror results no longer list the 4 *.manus.space apps (the "Explore further" section hides when empty); (3) /framework's "Ask FauxTony" button and its lead-in line removed; the Dr. Lee case-file link (4 places in when-healing-becomes-extraction, original and updated versions) renders as plain text through a DEAD_INTERNAL_LINKS list in lib/sanity/portable-text.tsx (no Sanity draft needed); (4) B Corp: checked live, nothing shown on either site, no change. Verified on a production build: the counts read 103, /framework has no FauxTony block, the essay has 0 links to the case file and keeps the words, /the-index shows "103 charities" when searching "charity".</t>
         </is>
       </c>
       <c r="E294" s="14" t="inlineStr">
@@ -7619,7 +7619,7 @@
       <c r="A295" s="4" t="n"/>
       <c r="B295" s="4" t="inlineStr">
         <is>
-          <t>Category pages pre-built (2026-10-09)</t>
+          <t>Arrows in buttons and links are icons (2026-10-09, owner said yes)</t>
         </is>
       </c>
       <c r="C295" s="13" t="inlineStr">
@@ -7629,7 +7629,7 @@
       </c>
       <c r="D295" s="4" t="inlineStr">
         <is>
-          <t>/blog/category/[slug] read ?page=N, so every category page was rendered on each request (slower first byte, flagged in the Lighthouse notes). Page numbers are now part of the address (/blog/category/&lt;slug&gt;/page/&lt;n&gt;, generateStaticParams, dynamicParams = false), shared code in src/components/blog/category-listing.tsx; old ?page=N links 308 to the new address (pages 2+ only, so no loop), /page/1 308s to the plain address, a page past the end is a 404; "All essays" back link uses an icon. Verified on a production build: route table shows every category page as pre-built (9 page-1s, 7 later pages), titles and canonicals per page, Previous/Next links, the redirects and the 404s.</t>
+          <t>113 typed arrows in 52 files (button and link labels, "Next"/"See My Results" toggles, decorative arrow spans, the walk-through "See the..." labels, the Letter's "I'm in" button) replaced with lucide ArrowRight/ArrowLeft (size-[1em], inside inline-flex items-center gap-1.5, so the parent layout is untouched). Left as content on purpose: arrows inside Tony's text and data (health findings, origins, iboga compass options, process flows like "Inherit → Wake → Choose → Act", share text), the "← you" marker on the consciousness scale, and &lt;option&gt; sort labels (an option can't hold an icon). Checked on 16 pages at 375 and 1280: no typed arrow left in any link or button, no sideways scroll, no JS errors; close-up screenshots of the new icons.</t>
         </is>
       </c>
       <c r="E295" s="14" t="inlineStr">
@@ -7642,7 +7642,7 @@
       <c r="A296" s="4" t="n"/>
       <c r="B296" s="4" t="inlineStr">
         <is>
-          <t>Error pages (2026-10-09, owner asked)</t>
+          <t>Category pages pre-built (2026-10-09)</t>
         </is>
       </c>
       <c r="C296" s="13" t="inlineStr">
@@ -7652,7 +7652,7 @@
       </c>
       <c r="D296" s="4" t="inlineStr">
         <is>
-          <t>404 page now sets its own title ("Page not found") as a server page around live's 3-second redirect (not-found.tsx + components/not-found-redirect.tsx), arrow as an icon; page error screen (error.tsx) uses Next 16's retry (re-fetches), shows a reference code for the server logs, links home and to the site index; new global-error.tsx for failures in the root layout itself (own &lt;html&gt;, plain links). Verified on a production build: missing page, missing essay and missing Kava page return 404 with the right title; a test page that throws returns 500 with the error screen, "Try again" re-fetches; phone and laptop, no sideways scroll (test page removed).</t>
+          <t>/blog/category/[slug] read ?page=N, so every category page was rendered on each request (slower first byte, flagged in the Lighthouse notes). Page numbers are now part of the address (/blog/category/&lt;slug&gt;/page/&lt;n&gt;, generateStaticParams, dynamicParams = false), shared code in src/components/blog/category-listing.tsx; old ?page=N links 308 to the new address (pages 2+ only, so no loop), /page/1 308s to the plain address, a page past the end is a 404; "All essays" back link uses an icon. Verified on a production build: route table shows every category page as pre-built (9 page-1s, 7 later pages), titles and canonicals per page, Previous/Next links, the redirects and the 404s.</t>
         </is>
       </c>
       <c r="E296" s="14" t="inlineStr">
@@ -7665,7 +7665,7 @@
       <c r="A297" s="4" t="n"/>
       <c r="B297" s="4" t="inlineStr">
         <is>
-          <t>SEO audit fixes (2026-10-06)</t>
+          <t>Error pages (2026-10-09, owner asked)</t>
         </is>
       </c>
       <c r="C297" s="13" t="inlineStr">
@@ -7675,7 +7675,7 @@
       </c>
       <c r="D297" s="4" t="inlineStr">
         <is>
-          <t>Checked an outside audit point by point against the code. Fixed: Core Themes cards linked to /?theme=…#essays-archive (not crawlable, counts from a stale hand-kept list) and now link to /blog/category/&lt;slug&gt; with real counts (21/25/20/14, matching the archive pills; THEME_MAP and the ?theme= filter removed); Four Doors cards were &lt;button&gt;s, now real links that still open the modal on a plain click; "DIAGNOSE · ENGAGE" now link to /find-my and /engage; one shared formatPostDate (Asia/Kolkata, src/lib/format-post-date.ts) so a post no longer shows two different dates; the title repeated as the first body paragraph is dropped at render time (legacyBodyLayout); essay cards are h3 under a section h2 (archive, Read next), h2 only on category/search; heading glyphs (◆ ✦) hidden from screen readers; posts send BlogPosting with the author tied to the site Person (@id) plus a BreadcrumbList; descriptive alt on the homepage and BrewSoul heroes; homepage OG image cropped to 1200x630 JPEG. Already fine (audit could not see it): Person/Article schema, Netlify noindex, robots.txt, sitemap, header nav and search, Amazon links carry no affiliate tag. Checked on a production build: type check, lint, build, status codes, browser click test at 375px, no console errors. Implementation pack (Mohammad Danish, 2026-10-05) checked the same day: added og:type/og:site_name back on the 6 pages with their own openGraph (a page-level openGraph replaces the layout one), twitter:creator, and on posts og:url</t>
+          <t>404 page now sets its own title ("Page not found") as a server page around live's 3-second redirect (not-found.tsx + components/not-found-redirect.tsx), arrow as an icon; page error screen (error.tsx) uses Next 16's retry (re-fetches), shows a reference code for the server logs, links home and to the site index; new global-error.tsx for failures in the root layout itself (own &lt;html&gt;, plain links). Verified on a production build: missing page, missing essay and missing Kava page return 404 with the right title; a test page that throws returns 500 with the error screen, "Try again" re-fetches; phone and laptop, no sideways scroll (test page removed).</t>
         </is>
       </c>
       <c r="E297" s="14" t="inlineStr">
@@ -7688,7 +7688,7 @@
       <c r="A298" s="4" t="n"/>
       <c r="B298" s="4" t="inlineStr">
         <is>
-          <t>SEO audit items needing a yes (2026-10-06; owner said yes to the copy 2026-10-10, done)</t>
+          <t>SEO audit fixes (2026-10-06)</t>
         </is>
       </c>
       <c r="C298" s="13" t="inlineStr">
@@ -7698,7 +7698,7 @@
       </c>
       <c r="D298" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">the pack's new copy (homepage title/description, five-cups title, description, short answer, FAQ, heading rewrites, entity statement, newsletter block, author box, health disclaimer, COA wording); "Further Reading" shown twice on posts (merge the lists?); long post title (84 chars), homepage description length and obsolete keywords tag, slugs (/blog/five-cups, the -2 slug; would need redirects), "Six lenses" over four cards, sources for health claims and proof for "$10B+", "Certified B Corp", "Validity: 91", legal review of the homepage Case File banner, ABIT waitlist disclosures, one contact email, the two one-post categories, fewer homepage CTAs / email signup / table of contents / explaining "COA". Done 2026-10-10: homepage title "Tony Greenberg | Strategist, Author &amp; CEO of RampRate" and description (essay count computed: 123); entity statement under the hero (107 coffees / 100 chains computed from the data) with a link to /ecosystem; door 4 "Certificate of Analysis (COA) checks, lab testing and vendor scoring"; "Four lenses" (computed); newsletter box after Editor's Picks (existing Kit form); meta keywords removed site-wide; every essay: author line + "About Tony", one merged "Further Reading", optional lastUpdated field shown as "Updated &lt;date&gt;" (not set on any post yet: every _updatedAt is the import date), health disclaimer on 20 personal-health essays (chosen by Sanity tag); Five Cups (Sanity, published, backup kept): SEO title/description, short answer, visible FAQ </t>
+          <t>Checked an outside audit point by point against the code. Fixed: Core Themes cards linked to /?theme=…#essays-archive (not crawlable, counts from a stale hand-kept list) and now link to /blog/category/&lt;slug&gt; with real counts (21/25/20/14, matching the archive pills; THEME_MAP and the ?theme= filter removed); Four Doors cards were &lt;button&gt;s, now real links that still open the modal on a plain click; "DIAGNOSE · ENGAGE" now link to /find-my and /engage; one shared formatPostDate (Asia/Kolkata, src/lib/format-post-date.ts) so a post no longer shows two different dates; the title repeated as the first body paragraph is dropped at render time (legacyBodyLayout); essay cards are h3 under a section h2 (archive, Read next), h2 only on category/search; heading glyphs (◆ ✦) hidden from screen readers; posts send BlogPosting with the author tied to the site Person (@id) plus a BreadcrumbList; descriptive alt on the homepage and BrewSoul heroes; homepage OG image cropped to 1200x630 JPEG. Already fine (audit could not see it): Person/Article schema, Netlify noindex, robots.txt, sitemap, header nav and search, Amazon links carry no affiliate tag. Checked on a production build: type check, lint, build, status codes, browser click test at 375px, no console errors. Implementation pack (Mohammad Danish, 2026-10-05) checked the same day: added og:type/og:site_name back on the 6 pages with their own openGraph (a page-level openGraph replaces the layout one), twitter:creator, and on posts og:url</t>
         </is>
       </c>
       <c r="E298" s="14" t="inlineStr">
@@ -7711,7 +7711,7 @@
       <c r="A299" s="4" t="n"/>
       <c r="B299" s="4" t="inlineStr">
         <is>
-          <t>Google Analytics tag (found missing 2026-10-10, added the same day)</t>
+          <t>SEO audit items needing a yes (2026-10-06; owner said yes to the copy 2026-10-10, done)</t>
         </is>
       </c>
       <c r="C299" s="13" t="inlineStr">
@@ -7721,7 +7721,7 @@
       </c>
       <c r="D299" s="4" t="inlineStr">
         <is>
-          <t>Live loads GA4 G-4GVW40S47N; the new site sent nothing, so stats would have stopped at cutover. Added src/components/google-analytics.tsx (plain next/script, no new package) in the root layout; it only runs on tonygreenberg.com / www, so Netlify previews and localhost never reach the real reports. Checked: type check, lint, build; in Chromium with Google's requests blocked: localhost sends nothing, tonygreenberg.com (mapped to a local production build) loads the tag on / and /find-your-coffee, no JS errors. In-site page changes are counted by GA4's Enhanced measurement (on by default; confirm in GA4 &gt; Admin &gt; Data streams on launch day).</t>
+          <t xml:space="preserve">the pack's new copy (homepage title/description, five-cups title, description, short answer, FAQ, heading rewrites, entity statement, newsletter block, author box, health disclaimer, COA wording); "Further Reading" shown twice on posts (merge the lists?); long post title (84 chars), homepage description length and obsolete keywords tag, slugs (/blog/five-cups, the -2 slug; would need redirects), "Six lenses" over four cards, sources for health claims and proof for "$10B+", "Certified B Corp", "Validity: 91", legal review of the homepage Case File banner, ABIT waitlist disclosures, one contact email, the two one-post categories, fewer homepage CTAs / email signup / table of contents / explaining "COA". Done 2026-10-10: homepage title "Tony Greenberg | Strategist, Author &amp; CEO of RampRate" and description (essay count computed: 123); entity statement under the hero (107 coffees / 100 chains computed from the data) with a link to /ecosystem; door 4 "Certificate of Analysis (COA) checks, lab testing and vendor scoring"; "Four lenses" (computed); newsletter box after Editor's Picks (existing Kit form); meta keywords removed site-wide; every essay: author line + "About Tony", one merged "Further Reading", optional lastUpdated field shown as "Updated &lt;date&gt;" (not set on any post yet: every _updatedAt is the import date), health disclaimer on 20 personal-health essays (chosen by Sanity tag); Five Cups (Sanity, published, backup kept): SEO title/description, short answer, visible FAQ </t>
         </is>
       </c>
       <c r="E299" s="14" t="inlineStr">
@@ -7734,7 +7734,7 @@
       <c r="A300" s="4" t="n"/>
       <c r="B300" s="4" t="inlineStr">
         <is>
-          <t>Old site's custom GA4 events ported (2026-10-10, owner asked to match legacy's Google tags)</t>
+          <t>Google Analytics tag (found missing 2026-10-10, added the same day)</t>
         </is>
       </c>
       <c r="C300" s="13" t="inlineStr">
@@ -7744,7 +7744,7 @@
       </c>
       <c r="D300" s="4" t="inlineStr">
         <is>
-          <t>Legacy loaded GA4 G-4GVW40S47N (already on the new site), Manus's own Umami counter (gone with Manus, not portable) and custom events from ConversionMechanics.tsx's AnalyticsTracker. Now src/components/ga-events.tsx (root layout) sends the same names: article_/page_25/50/75/90_scroll, engaged_45_seconds, second_page_view, homepage_path_work/_thinking/_building, start_here_open. Legacy's extra page_view on every history change is not ported (GA4 Enhanced measurement already counts in-site page changes; it would double-count). Tested in Chromium with Google's requests blocked: tonygreenberg.com (mapped to a local build) fired the homepage path and all four essay scroll events plus second_page_view; localhost loads no tag. A RampRate-style weekly report / hourly alert email and an admin analytics page were built the same day and removed at the owner's request (they use the Looker Studio report instead); the empty report_runs table and CRON_SECRET were removed too.</t>
+          <t>Live loads GA4 G-4GVW40S47N; the new site sent nothing, so stats would have stopped at cutover. Added src/components/google-analytics.tsx (plain next/script, no new package) in the root layout; it only runs on tonygreenberg.com / www, so Netlify previews and localhost never reach the real reports. Checked: type check, lint, build; in Chromium with Google's requests blocked: localhost sends nothing, tonygreenberg.com (mapped to a local production build) loads the tag on / and /find-your-coffee, no JS errors. In-site page changes are counted by GA4's Enhanced measurement (on by default; confirm in GA4 &gt; Admin &gt; Data streams on launch day).</t>
         </is>
       </c>
       <c r="E300" s="14" t="inlineStr">
@@ -7757,15 +7757,19 @@
       <c r="A301" s="4" t="n"/>
       <c r="B301" s="4" t="inlineStr">
         <is>
-          <t>Connect Google Search Console + GA4 to the new deployment on day one of cutover</t>
-        </is>
-      </c>
-      <c r="C301" s="16" t="inlineStr">
-        <is>
-          <t>Remaining</t>
-        </is>
-      </c>
-      <c r="D301" s="4" t="inlineStr"/>
+          <t>Old site's custom GA4 events ported (2026-10-10, owner asked to match legacy's Google tags)</t>
+        </is>
+      </c>
+      <c r="C301" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D301" s="4" t="inlineStr">
+        <is>
+          <t>Legacy loaded GA4 G-4GVW40S47N (already on the new site), Manus's own Umami counter (gone with Manus, not portable) and custom events from ConversionMechanics.tsx's AnalyticsTracker. Now src/components/ga-events.tsx (root layout) sends the same names: article_/page_25/50/75/90_scroll, engaged_45_seconds, second_page_view, homepage_path_work/_thinking/_building, start_here_open. Legacy's extra page_view on every history change is not ported (GA4 Enhanced measurement already counts in-site page changes; it would double-count). Tested in Chromium with Google's requests blocked: tonygreenberg.com (mapped to a local build) fired the homepage path and all four essay scroll events plus second_page_view; localhost loads no tag. A RampRate-style weekly report / hourly alert email and an admin analytics page were built the same day and removed at the owner's request (they use the Looker Studio report instead); the empty report_runs table and CRON_SECRET were removed too.</t>
+        </is>
+      </c>
       <c r="E301" s="14" t="inlineStr">
         <is>
           <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
@@ -7776,19 +7780,15 @@
       <c r="A302" s="4" t="n"/>
       <c r="B302" s="4" t="inlineStr">
         <is>
-          <t>Restore/adapt the manus.space triple-layer noindex lockdown pattern for any remaining staging URLs</t>
-        </is>
-      </c>
-      <c r="C302" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D302" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-01: the Netlify copy (tonygreenberg-website.netlify.app) and every deploy preview had no noindex at all, so Google could index a duplicate of the site. next.config.ts headers() now sends X-Robots-Tag: noindex, nofollow on any *.netlify.app host only; tonygreenberg.com is unaffected, so nothing to remove at cutover. Tested with Host headers on a production build.</t>
-        </is>
-      </c>
+          <t>Connect Google Search Console + GA4 to the new deployment on day one of cutover</t>
+        </is>
+      </c>
+      <c r="C302" s="16" t="inlineStr">
+        <is>
+          <t>Remaining</t>
+        </is>
+      </c>
+      <c r="D302" s="4" t="inlineStr"/>
       <c r="E302" s="14" t="inlineStr">
         <is>
           <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
@@ -7799,7 +7799,7 @@
       <c r="A303" s="4" t="n"/>
       <c r="B303" s="4" t="inlineStr">
         <is>
-          <t>"Keep going" strip above the footer on every page (2026-10-07)</t>
+          <t>Restore/adapt the manus.space triple-layer noindex lockdown pattern for any remaining staging URLs</t>
         </is>
       </c>
       <c r="C303" s="13" t="inlineStr">
@@ -7809,7 +7809,7 @@
       </c>
       <c r="D303" s="4" t="inlineStr">
         <is>
-          <t>legacy's WhereNext (deferred in Phase 3, never picked up) with its per-page suggestions, Home · Site Index · All Assessments; links pointed at current routes.</t>
+          <t>2026-10-01: the Netlify copy (tonygreenberg-website.netlify.app) and every deploy preview had no noindex at all, so Google could index a duplicate of the site. next.config.ts headers() now sends X-Robots-Tag: noindex, nofollow on any *.netlify.app host only; tonygreenberg.com is unaffected, so nothing to remove at cutover. Tested with Host headers on a production build.</t>
         </is>
       </c>
       <c r="E303" s="14" t="inlineStr">
@@ -7822,7 +7822,7 @@
       <c r="A304" s="4" t="n"/>
       <c r="B304" s="4" t="inlineStr">
         <is>
-          <t>Live-only and redesigned pages from the 2026-10-07 page sweep (188 pages compared with live)</t>
+          <t>"Keep going" strip above the footer on every page (2026-10-07)</t>
         </is>
       </c>
       <c r="C304" s="13" t="inlineStr">
@@ -7832,7 +7832,7 @@
       </c>
       <c r="D304" s="4" t="inlineStr">
         <is>
-          <t>/the-index rebuilt from live's code (20 concepts, related-word search across essays and site pages, full-text search on the server, "three related places to go next"; the old redirect to /search removed and its links, including the "Site Index" link in "Keep going", point at it again); /the-mirror (and /life-assessment) opens on live's intro (dark hero, "What We Measure" with the six areas, "The Ecosystem"), rebuilt as a step registry (rule 19); /essays header, order and column like live; /about "What They Say" styled like live (live picks 3 of the same 19 quotes at random; ours shows a fixed 3 so they're in the server HTML); /impact-futurism list titles and subtitles; /supplier-intake is a real page again with live's Stage 1 form; /seven-doors and /projects redirect home like live; /impact, /health, /library, /built-on-manus, /heroes are 404 on live too. Left as is on purpose: /blog stays our archive page (on live it repeats the homepage), the email gates on /framework and /peptide-supply-chain, the attention-theft Wall of Shame.</t>
+          <t>legacy's WhereNext (deferred in Phase 3, never picked up) with its per-page suggestions, Home · Site Index · All Assessments; links pointed at current routes.</t>
         </is>
       </c>
       <c r="E304" s="14" t="inlineStr">
@@ -7845,7 +7845,7 @@
       <c r="A305" s="4" t="n"/>
       <c r="B305" s="4" t="inlineStr">
         <is>
-          <t>/alex-azzi locked like live (2026-10-07, owner said match it)</t>
+          <t>Live-only and redesigned pages from the 2026-10-07 page sweep (188 pages compared with live)</t>
         </is>
       </c>
       <c r="C305" s="13" t="inlineStr">
@@ -7855,7 +7855,7 @@
       </c>
       <c r="D305" s="4" t="inlineStr">
         <is>
-          <t>same server-checked password as the locked essay (GATED_POST_PASSWORD, now also set in Netlify), live's "Restricted Access" screen, the report not in the page until unlocked, out of search and the sitemap.</t>
+          <t>/the-index rebuilt from live's code (20 concepts, related-word search across essays and site pages, full-text search on the server, "three related places to go next"; the old redirect to /search removed and its links, including the "Site Index" link in "Keep going", point at it again); /the-mirror (and /life-assessment) opens on live's intro (dark hero, "What We Measure" with the six areas, "The Ecosystem"), rebuilt as a step registry (rule 19); /essays header, order and column like live; /about "What They Say" styled like live (live picks 3 of the same 19 quotes at random; ours shows a fixed 3 so they're in the server HTML); /impact-futurism list titles and subtitles; /supplier-intake is a real page again with live's Stage 1 form; /seven-doors and /projects redirect home like live; /impact, /health, /library, /built-on-manus, /heroes are 404 on live too. Left as is on purpose: /blog stays our archive page (on live it repeats the homepage), the email gates on /framework and /peptide-supply-chain, the attention-theft Wall of Shame.</t>
         </is>
       </c>
       <c r="E305" s="14" t="inlineStr">
@@ -7868,7 +7868,7 @@
       <c r="A306" s="4" t="n"/>
       <c r="B306" s="4" t="inlineStr">
         <is>
-          <t>Live's title fonts and sizes (2026-10-07, "fix the style")</t>
+          <t>/alex-azzi locked like live (2026-10-07, owner said match it)</t>
         </is>
       </c>
       <c r="C306" s="13" t="inlineStr">
@@ -7878,7 +7878,7 @@
       </c>
       <c r="D306" s="4" t="inlineStr">
         <is>
-          <t>measured every page's title font, weight, size and label colour on live vs ours (136 pages). Now like live: Kava headings in Fraunces, HumanOS in Space Grotesk, the peptide tools / charity scorecard / thesis threads in the system serif, America Unbundled in the Iowan Old Style stack at live's size, /akbar in Fraunces 900, friend-gate and post-intervention in Georgia, and live's title sizes on peptide-matrix, peptide-supply-chain, rip-peptide-sciences and the HumanOS pages. Fonts load only on the pages that use them (src/lib/fonts/page-fonts.ts). Label colours stay the darker AA-contrast versions where live's lighter ones fail on a light background.</t>
+          <t>same server-checked password as the locked essay (GATED_POST_PASSWORD, now also set in Netlify), live's "Restricted Access" screen, the report not in the page until unlocked, out of search and the sitemap.</t>
         </is>
       </c>
       <c r="E306" s="14" t="inlineStr">
@@ -7891,7 +7891,7 @@
       <c r="A307" s="4" t="n"/>
       <c r="B307" s="4" t="inlineStr">
         <is>
-          <t>Peptide page images rescued into Sanity and wired (2026-10-07)</t>
+          <t>Live's title fonts and sizes (2026-10-07, "fix the style")</t>
         </is>
       </c>
       <c r="C307" s="13" t="inlineStr">
@@ -7901,7 +7901,7 @@
       </c>
       <c r="D307" s="4" t="inlineStr">
         <is>
-          <t>/peptide-watch hero plus its 11 section banners, /peptide-matrix and /peptide-supply-chain heroes, the /peptide-hall-of-shame hero (scripts/rescue-2026-10-07-peptide-images.ts, logged in docs/ai/manus-media-rescue.md).</t>
+          <t>measured every page's title font, weight, size and label colour on live vs ours (136 pages). Now like live: Kava headings in Fraunces, HumanOS in Space Grotesk, the peptide tools / charity scorecard / thesis threads in the system serif, America Unbundled in the Iowan Old Style stack at live's size, /akbar in Fraunces 900, friend-gate and post-intervention in Georgia, and live's title sizes on peptide-matrix, peptide-supply-chain, rip-peptide-sciences and the HumanOS pages. Fonts load only on the pages that use them (src/lib/fonts/page-fonts.ts). Label colours stay the darker AA-contrast versions where live's lighter ones fail on a light background.</t>
         </is>
       </c>
       <c r="E307" s="14" t="inlineStr">
@@ -7914,7 +7914,7 @@
       <c r="A308" s="4" t="n"/>
       <c r="B308" s="4" t="inlineStr">
         <is>
-          <t>Live's editorial redesign, first group (2026-10-07)</t>
+          <t>Peptide page images rescued into Sanity and wired (2026-10-07)</t>
         </is>
       </c>
       <c r="C308" s="13" t="inlineStr">
@@ -7924,7 +7924,7 @@
       </c>
       <c r="D308" s="4" t="inlineStr">
         <is>
-          <t>dark top sections, narrow single text column, short red section rules and dark call-to-action bands on /invest, /amplifier, /community (now "Sign In to Join the Community", linking our real sign-in; live's made-up counters left out), /framework, /the-letter (daily provocation with "Share this thought" and "Search past provocations"), /engage, /diamond-cut, /ecosystem and the homepage's "The thinking doesn't stop here" band. Kept on purpose: AA-contrast colours where live's fail, "Enter the Gate" instead of live's $5,000 checkout on /diamond-cut.</t>
+          <t>/peptide-watch hero plus its 11 section banners, /peptide-matrix and /peptide-supply-chain heroes, the /peptide-hall-of-shame hero (scripts/rescue-2026-10-07-peptide-images.ts, logged in docs/ai/manus-media-rescue.md).</t>
         </is>
       </c>
       <c r="E308" s="14" t="inlineStr">
@@ -7937,7 +7937,7 @@
       <c r="A309" s="4" t="n"/>
       <c r="B309" s="4" t="inlineStr">
         <is>
-          <t>Live's redesign, second group (done 2026-10-08)</t>
+          <t>Live's editorial redesign, first group (2026-10-07)</t>
         </is>
       </c>
       <c r="C309" s="13" t="inlineStr">
@@ -7947,7 +7947,7 @@
       </c>
       <c r="D309" s="4" t="inlineStr">
         <is>
-          <t>re-measured all 18 pages on live vs a fresh production build (title font/size/weight/colour, labels, hero images). Already matching from 2026-10-07: /the-web, /spirits, /iboga-ibogaine (weight 800), /living-declaration, BrewSoul photo on /brewsoul, /brewsoul/browse, /brewsoul/first-sip (live has none there either), /quiz_25q, /recent-creations. Fixed today: /find-your-journey (64px title, red label), /impact-dashboard (64px title in essay ink, label spacing), red labels on /published and /speaking (plus its "rooms" chips), /soulscore "by ImpactSoul" label, /pri-calibration title (weight 900, solid cream, was a purple gradient), /clients (live's narrow 546px column for the whole page, 56px title, roomier stats band, cards 2 per row; two static inline styles moved to classes), /brewsoul/guest (live's BrewSoul photo on the guest card instead of "SN" initials, labels in capitals), /humanos/connect (cards line up with the title), /peptide-hall-of-shame (stats and label readable light gold; were dark gold on dark). Typed arrows on the touched links are icons now (rule 18). Deliberately not copied from live (new CONTRIBUTING rule 20, owner 2026-10-08): red labels on dark bands use #E07A80 (live's #8E1E25 on black is about 2:1, unreadable); /recent-creations keeps our darker label colours (live's fail contrast on white); /humanos/connect keeps "Start Reading" (that card links to the philosophy page, the quiz live's "Start the Assessment" implies doesn't exist). Checked: type check, l</t>
+          <t>dark top sections, narrow single text column, short red section rules and dark call-to-action bands on /invest, /amplifier, /community (now "Sign In to Join the Community", linking our real sign-in; live's made-up counters left out), /framework, /the-letter (daily provocation with "Share this thought" and "Search past provocations"), /engage, /diamond-cut, /ecosystem and the homepage's "The thinking doesn't stop here" band. Kept on purpose: AA-contrast colours where live's fail, "Enter the Gate" instead of live's $5,000 checkout on /diamond-cut.</t>
         </is>
       </c>
       <c r="E309" s="14" t="inlineStr">
@@ -7960,7 +7960,7 @@
       <c r="A310" s="4" t="n"/>
       <c r="B310" s="4" t="inlineStr">
         <is>
-          <t>BrewSoul top of page (2026-10-08, owner: "button in the center at the top doesn't look good")</t>
+          <t>Live's redesign, second group (done 2026-10-08)</t>
         </is>
       </c>
       <c r="C310" s="13" t="inlineStr">
@@ -7970,7 +7970,7 @@
       </c>
       <c r="D310" s="4" t="inlineStr">
         <is>
-          <t>the category badge ("Deep Research" etc.) sat centred in an empty strip, squeezed against the hero, because we copied live's doubled 52px top gap. Now one gap everywhere and the badge floats in the top-left corner, lined up with the BrewSoul logo (brewsoul-main.tsx, category-badge.tsx); checked on all 26 badge pages at 3 widths that it covers nothing. BrewSoul menu: on tablets (768-1023px) the links were cut off and "More" was hidden with no menu button at all; now the menu button shows below 1024px, 5 links + "More" from 1024px, all 8 from 1280px, "More" always visible.</t>
+          <t>re-measured all 18 pages on live vs a fresh production build (title font/size/weight/colour, labels, hero images). Already matching from 2026-10-07: /the-web, /spirits, /iboga-ibogaine (weight 800), /living-declaration, BrewSoul photo on /brewsoul, /brewsoul/browse, /brewsoul/first-sip (live has none there either), /quiz_25q, /recent-creations. Fixed today: /find-your-journey (64px title, red label), /impact-dashboard (64px title in essay ink, label spacing), red labels on /published and /speaking (plus its "rooms" chips), /soulscore "by ImpactSoul" label, /pri-calibration title (weight 900, solid cream, was a purple gradient), /clients (live's narrow 546px column for the whole page, 56px title, roomier stats band, cards 2 per row; two static inline styles moved to classes), /brewsoul/guest (live's BrewSoul photo on the guest card instead of "SN" initials, labels in capitals), /humanos/connect (cards line up with the title), /peptide-hall-of-shame (stats and label readable light gold; were dark gold on dark). Typed arrows on the touched links are icons now (rule 18). Deliberately not copied from live (new CONTRIBUTING rule 20, owner 2026-10-08): red labels on dark bands use #E07A80 (live's #8E1E25 on black is about 2:1, unreadable); /recent-creations keeps our darker label colours (live's fail contrast on white); /humanos/connect keeps "Start Reading" (that card links to the philosophy page, the quiz live's "Start the Assessment" implies doesn't exist). Checked: type check, l</t>
         </is>
       </c>
       <c r="E310" s="14" t="inlineStr">
@@ -7983,7 +7983,7 @@
       <c r="A311" s="4" t="n"/>
       <c r="B311" s="4" t="inlineStr">
         <is>
-          <t>/pri-efficacy's "Simulation / Live Calibrations" switch like live (2026-10-08)</t>
+          <t>BrewSoul top of page (2026-10-08, owner: "button in the center at the top doesn't look good")</t>
         </is>
       </c>
       <c r="C311" s="13" t="inlineStr">
@@ -7993,7 +7993,7 @@
       </c>
       <c r="D311" s="4" t="inlineStr">
         <is>
-          <t>shadcn Tabs, both panels in the server HTML (forceMount). The Live tab reads real aggregate numbers from pri_calibrations (getPriLiveStats() in src/lib/pri-research.ts: totals, opt-ins, average score per dimension; no rows leave the server), page stays static and refreshes every 10 minutes. Until the Supabase scripts are run (Phase 2) it says the numbers "aren't available just now" instead of a fake zero. Checked: build (○, 10m), server HTML has both tabs, tab switch at 390/1280px, no JS errors. Re-check with real numbers once the table exists.</t>
+          <t>the category badge ("Deep Research" etc.) sat centred in an empty strip, squeezed against the hero, because we copied live's doubled 52px top gap. Now one gap everywhere and the badge floats in the top-left corner, lined up with the BrewSoul logo (brewsoul-main.tsx, category-badge.tsx); checked on all 26 badge pages at 3 widths that it covers nothing. BrewSoul menu: on tablets (768-1023px) the links were cut off and "More" was hidden with no menu button at all; now the menu button shows below 1024px, 5 links + "More" from 1024px, all 8 from 1280px, "More" always visible.</t>
         </is>
       </c>
       <c r="E311" s="14" t="inlineStr">
@@ -8006,63 +8006,63 @@
       <c r="A312" s="4" t="n"/>
       <c r="B312" s="4" t="inlineStr">
         <is>
+          <t>/pri-efficacy's "Simulation / Live Calibrations" switch like live (2026-10-08)</t>
+        </is>
+      </c>
+      <c r="C312" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D312" s="4" t="inlineStr">
+        <is>
+          <t>shadcn Tabs, both panels in the server HTML (forceMount). The Live tab reads real aggregate numbers from pri_calibrations (getPriLiveStats() in src/lib/pri-research.ts: totals, opt-ins, average score per dimension; no rows leave the server), page stays static and refreshes every 10 minutes. Until the Supabase scripts are run (Phase 2) it says the numbers "aren't available just now" instead of a fake zero. Checked: build (○, 10m), server HTML has both tabs, tab switch at 390/1280px, no JS errors. Re-check with real numbers once the table exists.</t>
+        </is>
+      </c>
+      <c r="E312" s="14" t="inlineStr">
+        <is>
+          <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" s="4" t="n"/>
+      <c r="B313" s="4" t="inlineStr">
+        <is>
           <t>/brewsoul/browse hero readable (2026-10-08, owner said go ahead)</t>
         </is>
       </c>
-      <c r="C312" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D312" s="4" t="inlineStr">
+      <c r="C313" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D313" s="4" t="inlineStr">
         <is>
           <t>a soft cream glow behind the title block so "The Catalog", the subtitle and the stat labels read clearly over the coffee photo (live is hard to read there too; rule 20). Photo still shows around the edges. Checked at 390/1280px.</t>
         </is>
       </c>
-      <c r="E312" s="14" t="inlineStr">
+      <c r="E313" s="14" t="inlineStr">
         <is>
           <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
         </is>
       </c>
     </row>
-    <row r="313">
-      <c r="A313" s="10" t="inlineStr">
+    <row r="314">
+      <c r="A314" s="10" t="inlineStr">
         <is>
           <t>Phase 13 — Images Needed in Sanity</t>
         </is>
       </c>
-      <c r="B313" s="11" t="n"/>
-      <c r="C313" s="11" t="n"/>
-      <c r="D313" s="12" t="n"/>
-    </row>
-    <row r="314">
-      <c r="A314" s="4" t="n"/>
-      <c r="B314" s="4" t="inlineStr">
-        <is>
-          <t>Manus media rescue (2026-09-29)</t>
-        </is>
-      </c>
-      <c r="C314" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D314" s="4" t="inlineStr">
-        <is>
-          <t>all 94 Manus-hosted image/video references in the legacy source (/api/img/, /manus-storage/) were checked live. 91 were still downloadable, including the /akbar photos the entry below calls "permanently lost", and all 91 are now Sanity assets (scripts/rescue-manus-media.ts; Sanity dedupes by SHA-1). 3 were gone (HTTP 502). The manifest docs/ai/manus-media-rescue.md maps each one to the legacy files that used it and its Sanity URL. They are not wired into pages yet: go page by page, with real alt text. /facilitator-index's two diagrams are done (scripts/rescue-facilitator-images.ts).</t>
-        </is>
-      </c>
-      <c r="E314" s="14" t="inlineStr">
-        <is>
-          <t>Phase 13 — Images Needed in Sanity</t>
-        </is>
-      </c>
+      <c r="B314" s="11" t="n"/>
+      <c r="C314" s="11" t="n"/>
+      <c r="D314" s="12" t="n"/>
     </row>
     <row r="315">
       <c r="A315" s="4" t="n"/>
       <c r="B315" s="4" t="inlineStr">
         <is>
-          <t>Favicon</t>
+          <t>Manus media rescue (2026-09-29)</t>
         </is>
       </c>
       <c r="C315" s="13" t="inlineStr">
@@ -8072,7 +8072,7 @@
       </c>
       <c r="D315" s="4" t="inlineStr">
         <is>
-          <t>real "G" brand mark generated from the header's actual wordmark treatment (src/app/icon.tsx), see Phase 3</t>
+          <t>all 94 Manus-hosted image/video references in the legacy source (/api/img/, /manus-storage/) were checked live. 91 were still downloadable, including the /akbar photos the entry below calls "permanently lost", and all 91 are now Sanity assets (scripts/rescue-manus-media.ts; Sanity dedupes by SHA-1). 3 were gone (HTTP 502). The manifest docs/ai/manus-media-rescue.md maps each one to the legacy files that used it and its Sanity URL. They are not wired into pages yet: go page by page, with real alt text. /facilitator-index's two diagrams are done (scripts/rescue-facilitator-images.ts).</t>
         </is>
       </c>
       <c r="E315" s="14" t="inlineStr">
@@ -8085,7 +8085,7 @@
       <c r="A316" s="4" t="n"/>
       <c r="B316" s="4" t="inlineStr">
         <is>
-          <t>Site-wide: logo (light + dark) beyond the current text wordmark</t>
+          <t>Favicon</t>
         </is>
       </c>
       <c r="C316" s="13" t="inlineStr">
@@ -8095,7 +8095,7 @@
       </c>
       <c r="D316" s="4" t="inlineStr">
         <is>
-          <t>Decided 2026-10-13 (owner): keep the text logo. The header's "TonyG" wordmark (site-header.tsx, gold G) already has light and dark colours, so no change. (Default/fallback OG image 1200×630 exists: public/images/default-og.png, checked 2026-10-02.)</t>
+          <t>real "G" brand mark generated from the header's actual wordmark treatment (src/app/icon.tsx), see Phase 3</t>
         </is>
       </c>
       <c r="E316" s="14" t="inlineStr">
@@ -8108,7 +8108,7 @@
       <c r="A317" s="4" t="n"/>
       <c r="B317" s="4" t="inlineStr">
         <is>
-          <t>Author photo(s) for blog author schema (Tony Greenberg headshot at minimum)</t>
+          <t>Site-wide: logo (light + dark) beyond the current text wordmark</t>
         </is>
       </c>
       <c r="C317" s="13" t="inlineStr">
@@ -8118,7 +8118,7 @@
       </c>
       <c r="D317" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02: the rescued headshot is already the author avatar in Sanity; now also in every post's Article JSON-LD (author image + url /about). The JSON-LD publisher logo pointed at /favicon.ico, a 404 here; now /icon.</t>
+          <t>Decided 2026-10-13 (owner): keep the text logo. The header's "TonyG" wordmark (site-header.tsx, gold G) already has light and dark colours, so no change. (Default/fallback OG image 1200×630 exists: public/images/default-og.png, checked 2026-10-02.)</t>
         </is>
       </c>
       <c r="E317" s="14" t="inlineStr">
@@ -8131,7 +8131,7 @@
       <c r="A318" s="4" t="n"/>
       <c r="B318" s="4" t="inlineStr">
         <is>
-          <t>Blog hero images</t>
+          <t>Author photo(s) for blog author schema (Tony Greenberg headshot at minimum)</t>
         </is>
       </c>
       <c r="C318" s="13" t="inlineStr">
@@ -8141,7 +8141,7 @@
       </c>
       <c r="D318" s="4" t="inlineStr">
         <is>
-          <t>audited, then migrated. Final state:</t>
+          <t>2026-10-02: the rescued headshot is already the author avatar in Sanity; now also in every post's Article JSON-LD (author image + url /about). The JSON-LD publisher logo pointed at /favicon.ico, a 404 here; now /icon.</t>
         </is>
       </c>
       <c r="E318" s="14" t="inlineStr">
@@ -8154,7 +8154,7 @@
       <c r="A319" s="4" t="n"/>
       <c r="B319" s="4" t="inlineStr">
         <is>
-          <t>22 posts have a real hero image, now live in Sanity (17 already on RampRate's own CloudFront + 4 rescued from the legacy /api/img/ proxy + 1…</t>
+          <t>Blog hero images</t>
         </is>
       </c>
       <c r="C319" s="13" t="inlineStr">
@@ -8164,7 +8164,7 @@
       </c>
       <c r="D319" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> rescued from /manus-storage/, all pulled over by migrate-blog-posts.ts before Manus is decommissioned)</t>
+          <t>audited, then migrated. Final state:</t>
         </is>
       </c>
       <c r="E319" s="14" t="inlineStr">
@@ -8177,7 +8177,7 @@
       <c r="A320" s="4" t="n"/>
       <c r="B320" s="4" t="inlineStr">
         <is>
-          <t>7 more posts got a real, unique hero image rescued from the live legacy site's newly-added art this pass (scripts/rescue-2026-09-blog-images…</t>
+          <t>22 posts have a real hero image, now live in Sanity (17 already on RampRate's own CloudFront + 4 rescued from the legacy /api/img/ proxy + 1…</t>
         </is>
       </c>
       <c r="C320" s="13" t="inlineStr">
@@ -8187,7 +8187,7 @@
       </c>
       <c r="D320" s="4" t="inlineStr">
         <is>
-          <t>.ts — see the correction note above): california-toll-roads-legalized-scam, the-1000-hour-hold, conscious-capital-partnership-ecosystem, the-peptide-truth-65m-fraud-industry-vs-life-changing-medicine, clear-communication, building-services-market-transhuman-era, heart-protocol-addendum.</t>
+          <t xml:space="preserve"> rescued from /manus-storage/, all pulled over by migrate-blog-posts.ts before Manus is decommissioned)</t>
         </is>
       </c>
       <c r="E320" s="14" t="inlineStr">
@@ -8200,7 +8200,7 @@
       <c r="A321" s="4" t="n"/>
       <c r="B321" s="4" t="inlineStr">
         <is>
-          <t>92 posts still need a real, unique hero image</t>
+          <t>7 more posts got a real, unique hero image rescued from the live legacy site's newly-added art this pass (scripts/rescue-2026-09-blog-images…</t>
         </is>
       </c>
       <c r="C321" s="13" t="inlineStr">
@@ -8210,7 +8210,7 @@
       </c>
       <c r="D321" s="4" t="inlineStr">
         <is>
-          <t>(down from 99). 2026-10-13 (owner: "image you can add in Sanity"): generated a unique, text-free picture for each of the 92 (live's default-arch family: cream over a deep colour, gold line geometry, colour and motif by category, layout from the slug; scripts/generate-essay-hero-art.mjs) and set it as each post's heroImage draft (scripts/upload-essay-hero-art-2026-10-13.ts; dry run first: 92 found, none had art, nothing replaced). Checked in Sanity: 92 drafts carry the new image, 0 published posts changed. Published 2026-10-13 (owner: yes) with the script's --publish (only drafts whose sole change was the picture; 92 of 92). Checked: the Netlify copy's essay page now serves the new image (webhook refresh). Real photography can still replace any of them later. Tracked one row per post, with a suggested image-generation prompt, in BLOG-IMAGE-BRIEFS.md — work through that file and check items off there, not here. No image-generation tool was connected in this environment as of this writing; either connect one (e.g. an MCP image-gen extension), source these manually/with a designer then upload via Sanity Studio (/studio), or re-check the live legacy site periodically per the correction note above.</t>
+          <t>.ts — see the correction note above): california-toll-roads-legalized-scam, the-1000-hour-hold, conscious-capital-partnership-ecosystem, the-peptide-truth-65m-fraud-industry-vs-life-changing-medicine, clear-communication, building-services-market-transhuman-era, heart-protocol-addendum.</t>
         </is>
       </c>
       <c r="E321" s="14" t="inlineStr">
@@ -8223,7 +8223,7 @@
       <c r="A322" s="4" t="n"/>
       <c r="B322" s="4" t="inlineStr">
         <is>
-          <t>Blog: per-post OG image if different from hero (many posts can reuse hero as OG)</t>
+          <t>92 posts still need a real, unique hero image</t>
         </is>
       </c>
       <c r="C322" s="13" t="inlineStr">
@@ -8233,7 +8233,7 @@
       </c>
       <c r="D322" s="4" t="inlineStr">
         <is>
-          <t>Confirmed 2026-10-02: generateMetadata uses seo.ogImage, else the hero, else the default OG image.</t>
+          <t>(down from 99). 2026-10-13 (owner: "image you can add in Sanity"): generated a unique, text-free picture for each of the 92 (live's default-arch family: cream over a deep colour, gold line geometry, colour and motif by category, layout from the slug; scripts/generate-essay-hero-art.mjs) and set it as each post's heroImage draft (scripts/upload-essay-hero-art-2026-10-13.ts; dry run first: 92 found, none had art, nothing replaced). Checked in Sanity: 92 drafts carry the new image, 0 published posts changed. Published 2026-10-13 (owner: yes) with the script's --publish (only drafts whose sole change was the picture; 92 of 92). Checked: the Netlify copy's essay page now serves the new image (webhook refresh). Real photography can still replace any of them later. Tracked one row per post, with a suggested image-generation prompt, in BLOG-IMAGE-BRIEFS.md — work through that file and check items off there, not here. No image-generation tool was connected in this environment as of this writing; either connect one (e.g. an MCP image-gen extension), source these manually/with a designer then upload via Sanity Studio (/studio), or re-check the live legacy site periodically per the correction note above.</t>
         </is>
       </c>
       <c r="E322" s="14" t="inlineStr">
@@ -8246,7 +8246,7 @@
       <c r="A323" s="4" t="n"/>
       <c r="B323" s="4" t="inlineStr">
         <is>
-          <t>Marketing pages</t>
+          <t>Blog: per-post OG image if different from hero (many posts can reuse hero as OG)</t>
         </is>
       </c>
       <c r="C323" s="13" t="inlineStr">
@@ -8256,7 +8256,7 @@
       </c>
       <c r="D323" s="4" t="inlineStr">
         <is>
-          <t>hero/section images for /the-letter, /the-territory, /engine-room, /the-body, /the-nightstand, /recent-creations (portfolio thumbnails), /published (publication logos), /clients (client logos — confirm licensing before re-hosting). Checked against live 2026-10-02: same image count on every one; /the-territory, /engine-room, /recent-creations, /published, /clients have no images on live either.</t>
+          <t>Confirmed 2026-10-02: generateMetadata uses seo.ogImage, else the hero, else the default OG image.</t>
         </is>
       </c>
       <c r="E323" s="14" t="inlineStr">
@@ -8269,7 +8269,7 @@
       <c r="A324" s="4" t="n"/>
       <c r="B324" s="4" t="inlineStr">
         <is>
-          <t>/akbar essay images</t>
+          <t>Marketing pages</t>
         </is>
       </c>
       <c r="C324" s="13" t="inlineStr">
@@ -8279,7 +8279,7 @@
       </c>
       <c r="D324" s="4" t="inlineStr">
         <is>
-          <t>not lost after all: 20 of the 21 were rescued into Sanity by scripts/rescue-manus-media.ts (2026-09-28) and are wired back in legacy's layout (hero mosaic, JC portrait, 2x2 grid, 3 full-bleeds, 3-up strip, footer gallery) as of 2026-09-29. Only slider-3 was gone (HTTP 502); the hero mosaic is 4 tiles instead of 5.</t>
+          <t>hero/section images for /the-letter, /the-territory, /engine-room, /the-body, /the-nightstand, /recent-creations (portfolio thumbnails), /published (publication logos), /clients (client logos — confirm licensing before re-hosting). Checked against live 2026-10-02: same image count on every one; /the-territory, /engine-room, /recent-creations, /published, /clients have no images on live either.</t>
         </is>
       </c>
       <c r="E324" s="14" t="inlineStr">
@@ -8292,7 +8292,7 @@
       <c r="A325" s="4" t="n"/>
       <c r="B325" s="4" t="inlineStr">
         <is>
-          <t>Rescued page images wired back in (2026-09-29)</t>
+          <t>/akbar essay images</t>
         </is>
       </c>
       <c r="C325" s="13" t="inlineStr">
@@ -8302,7 +8302,7 @@
       </c>
       <c r="D325" s="4" t="inlineStr">
         <is>
-          <t>/living-declaration hero, hand image and Clarisse Abelarde artwork; /impact-dashboard earth hero; /find-my banner; /find-your-coffee dark photo landing (legacy copy restored, replacing an intro that wasn't in legacy). Also wired (second pass): /consciousness-scale (legacy's hero-first flow restored, the invented intro screen removed), /find-your-me hero, /humanos hero, the HumanOS nav logo, and all 12 HumanOS people headshots (/humanos/ecosystem, /humanos/philosophy). Blog-body images (2026-09-29): all 19 the migration dropped are restored by scripts/restore-blog-body-images.ts as Sanity drafts on 4 posts (Clarisse Abelarde 7, You Are the Moat 4, FRQNCY 6, Energy Is Money 2), waiting to be published in Studio; the other blog-listed assets were heroes already set. Still unwired from docs/ai/manus-media-rescue.md: and /alex-azzi's subject photo (a photo of a real person on an accusation page: needs Tony's yes first).</t>
+          <t>not lost after all: 20 of the 21 were rescued into Sanity by scripts/rescue-manus-media.ts (2026-09-28) and are wired back in legacy's layout (hero mosaic, JC portrait, 2x2 grid, 3 full-bleeds, 3-up strip, footer gallery) as of 2026-09-29. Only slider-3 was gone (HTTP 502); the hero mosaic is 4 tiles instead of 5.</t>
         </is>
       </c>
       <c r="E325" s="14" t="inlineStr">
@@ -8315,7 +8315,7 @@
       <c r="A326" s="4" t="n"/>
       <c r="B326" s="4" t="inlineStr">
         <is>
-          <t>BrewSoul: coffee/product images (brewsoul-coffees-expanded.ts likely has image refs</t>
+          <t>Rescued page images wired back in (2026-09-29)</t>
         </is>
       </c>
       <c r="C326" s="13" t="inlineStr">
@@ -8325,7 +8325,7 @@
       </c>
       <c r="D326" s="4" t="inlineStr">
         <is>
-          <t>audit), city guide header images, roaster directory photos. Audited 2026-09-09 (status spreadsheet), confirmed 2026-10-02: city guides already have photos; coffees, chains and roasters have no image field in legacy or here (text-only by design); farms got real photos.</t>
+          <t>/living-declaration hero, hand image and Clarisse Abelarde artwork; /impact-dashboard earth hero; /find-my banner; /find-your-coffee dark photo landing (legacy copy restored, replacing an intro that wasn't in legacy). Also wired (second pass): /consciousness-scale (legacy's hero-first flow restored, the invented intro screen removed), /find-your-me hero, /humanos hero, the HumanOS nav logo, and all 12 HumanOS people headshots (/humanos/ecosystem, /humanos/philosophy). Blog-body images (2026-09-29): all 19 the migration dropped are restored by scripts/restore-blog-body-images.ts as Sanity drafts on 4 posts (Clarisse Abelarde 7, You Are the Moat 4, FRQNCY 6, Energy Is Money 2), waiting to be published in Studio; the other blog-listed assets were heroes already set. Still unwired from docs/ai/manus-media-rescue.md: and /alex-azzi's subject photo (a photo of a real person on an accusation page: needs Tony's yes first).</t>
         </is>
       </c>
       <c r="E326" s="14" t="inlineStr">
@@ -8338,7 +8338,7 @@
       <c r="A327" s="4" t="n"/>
       <c r="B327" s="4" t="inlineStr">
         <is>
-          <t>65 page images moved off the Manus storage copy into Sanity (2026-10-02)</t>
+          <t>BrewSoul: coffee/product images (brewsoul-coffees-expanded.ts likely has image refs</t>
         </is>
       </c>
       <c r="C327" s="13" t="inlineStr">
@@ -8348,7 +8348,7 @@
       </c>
       <c r="D327" s="4" t="inlineStr">
         <is>
-          <t>every image the code loaded from d2xsxph8kpxj0f.cloudfront.net (PRI medicine images, Iboga module, facilitator index, /attention-theft, /alex-azzi, /protecting-your-business, /peyote-mescaline, HumanOS, the peptide quiz). Notes called it "RampRate's own CloudFront", but every file sits in the legacy Manus project's folder and its owner couldn't be confirmed. All 65 uploaded (scripts/rescue-cloudfront-images.ts), code rewritten, host removed from images.remotePatterns, no Sanity document used it. Table in docs/ai/manus-media-rescue.md.</t>
+          <t>audit), city guide header images, roaster directory photos. Audited 2026-09-09 (status spreadsheet), confirmed 2026-10-02: city guides already have photos; coffees, chains and roasters have no image field in legacy or here (text-only by design); farms got real photos.</t>
         </is>
       </c>
       <c r="E327" s="14" t="inlineStr">
@@ -8361,7 +8361,7 @@
       <c r="A328" s="4" t="n"/>
       <c r="B328" s="4" t="inlineStr">
         <is>
-          <t>PRI/Kava: medicine reference images (medicine-images.ts), facility images for /facilitator-index</t>
+          <t>65 page images moved off the Manus storage copy into Sanity (2026-10-02)</t>
         </is>
       </c>
       <c r="C328" s="13" t="inlineStr">
@@ -8371,7 +8371,7 @@
       </c>
       <c r="D328" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02: all in Sanity; image counts match live on PRI, Kava, Iboga, Peyote, facilitator pages.</t>
+          <t>every image the code loaded from d2xsxph8kpxj0f.cloudfront.net (PRI medicine images, Iboga module, facilitator index, /attention-theft, /alex-azzi, /protecting-your-business, /peyote-mescaline, HumanOS, the peptide quiz). Notes called it "RampRate's own CloudFront", but every file sits in the legacy Manus project's folder and its owner couldn't be confirmed. All 65 uploaded (scripts/rescue-cloudfront-images.ts), code rewritten, host removed from images.remotePatterns, no Sanity document used it. Table in docs/ai/manus-media-rescue.md.</t>
         </is>
       </c>
       <c r="E328" s="14" t="inlineStr">
@@ -8384,7 +8384,7 @@
       <c r="A329" s="4" t="n"/>
       <c r="B329" s="4" t="inlineStr">
         <is>
-          <t>Manifesto/Attention Theft: any diagram/illustration assets used on the mega-page</t>
+          <t>PRI/Kava: medicine reference images (medicine-images.ts), facility images for /facilitator-index</t>
         </is>
       </c>
       <c r="C329" s="13" t="inlineStr">
@@ -8394,7 +8394,7 @@
       </c>
       <c r="D329" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02: 6 of live's 7 are in (now in Sanity); the 7th belongs to the Wall of Shame section left out on purpose.</t>
+          <t>2026-10-02: all in Sanity; image counts match live on PRI, Kava, Iboga, Peyote, facilitator pages.</t>
         </is>
       </c>
       <c r="E329" s="14" t="inlineStr">
@@ -8407,7 +8407,7 @@
       <c r="A330" s="4" t="n"/>
       <c r="B330" s="4" t="inlineStr">
         <is>
-          <t>Assessment result-screen background art (flagged in STATUS.md as a known gap</t>
+          <t>Manifesto/Attention Theft: any diagram/illustration assets used on the mega-page</t>
         </is>
       </c>
       <c r="C330" s="13" t="inlineStr">
@@ -8417,7 +8417,7 @@
       </c>
       <c r="D330" s="4" t="inlineStr">
         <is>
-          <t>18/20 assessments currently have plain black backgrounds; sourcing themed art here also closes that gap) Done 2026-10-13 with colour instead of art (owner: "yes" to colour backgrounds). About 20 quizzes already had a coloured background (ThemedBackground, light per-theme gradients). The 4 still flat dark now have a dark colour gradient, kept dark so their light text stays readable: /find-your-journey result (purple to teal), /my-journey (its black layer hid the gradient; now green to purple), /pri-calibration and the /psychedelic-readiness-index assessment section (PRI ink to amber to plum, starting at ink so the photo band's fade still meets it). Checked: type check, lint, build (all 8 colours in the compiled CSS), screenshots at 375/820/1280 (quiz completed for the journey result), no sideways scroll or JS errors, axe colour-contrast 0 at 375 and 1280.</t>
+          <t>2026-10-02: 6 of live's 7 are in (now in Sanity); the 7th belongs to the Wall of Shame section left out on purpose.</t>
         </is>
       </c>
       <c r="E330" s="14" t="inlineStr">
@@ -8430,7 +8430,7 @@
       <c r="A331" s="4" t="n"/>
       <c r="B331" s="4" t="inlineStr">
         <is>
-          <t>Chatbot: FauxTony avatar/icon</t>
+          <t>Assessment result-screen background art (flagged in STATUS.md as a known gap</t>
         </is>
       </c>
       <c r="C331" s="13" t="inlineStr">
@@ -8440,7 +8440,7 @@
       </c>
       <c r="D331" s="4" t="inlineStr">
         <is>
-          <t>Not needed (2026-10-02): the chatbot phase (Phase 10) was cancelled.</t>
+          <t>18/20 assessments currently have plain black backgrounds; sourcing themed art here also closes that gap) Done 2026-10-13 with colour instead of art (owner: "yes" to colour backgrounds). About 20 quizzes already had a coloured background (ThemedBackground, light per-theme gradients). The 4 still flat dark now have a dark colour gradient, kept dark so their light text stays readable: /find-your-journey result (purple to teal), /my-journey (its black layer hid the gradient; now green to purple), /pri-calibration and the /psychedelic-readiness-index assessment section (PRI ink to amber to plum, starting at ink so the photo band's fade still meets it). Checked: type check, lint, build (all 8 colours in the compiled CSS), screenshots at 375/820/1280 (quiz completed for the journey result), no sideways scroll or JS errors, axe colour-contrast 0 at 375 and 1280.</t>
         </is>
       </c>
       <c r="E331" s="14" t="inlineStr">
@@ -8453,63 +8453,63 @@
       <c r="A332" s="4" t="n"/>
       <c r="B332" s="4" t="inlineStr">
         <is>
+          <t>Chatbot: FauxTony avatar/icon</t>
+        </is>
+      </c>
+      <c r="C332" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D332" s="4" t="inlineStr">
+        <is>
+          <t>Not needed (2026-10-02): the chatbot phase (Phase 10) was cancelled.</t>
+        </is>
+      </c>
+      <c r="E332" s="14" t="inlineStr">
+        <is>
+          <t>Phase 13 — Images Needed in Sanity</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" s="4" t="n"/>
+      <c r="B333" s="4" t="inlineStr">
+        <is>
           <t>Audit client/public/ (including alex-azzi/, brewsoul/ subfolders) for any static assets already sitting there unused that should be pulled i…</t>
         </is>
       </c>
-      <c r="C332" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D332" s="4" t="inlineStr">
+      <c r="C333" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D333" s="4" t="inlineStr">
         <is>
           <t>n rather than re-created. Done 2026-10-02: no images there at all (only llms.txt, a BrewSoul catalog, Manus debug files, design-options.html). Found and fixed a cutover risk instead: live serves two Google site-verification files (/google6881a0411c48b301.html, /alex-azzi/googleedff0185753a4a1f.html) that the new site returned 404 for, so Search Console could lose verification at DNS cutover. Both copied to public/ byte for byte. Not copied: site.webmanifest (its icons don't exist here; Next's app/icon.tsx covers the favicon).</t>
         </is>
       </c>
-      <c r="E332" s="14" t="inlineStr">
+      <c r="E333" s="14" t="inlineStr">
         <is>
           <t>Phase 13 — Images Needed in Sanity</t>
         </is>
       </c>
     </row>
-    <row r="333">
-      <c r="A333" s="10" t="inlineStr">
+    <row r="334">
+      <c r="A334" s="10" t="inlineStr">
         <is>
           <t>Phase 14 — QA &amp; Launch</t>
         </is>
       </c>
-      <c r="B333" s="11" t="n"/>
-      <c r="C333" s="11" t="n"/>
-      <c r="D333" s="12" t="n"/>
-    </row>
-    <row r="334">
-      <c r="A334" s="4" t="n"/>
-      <c r="B334" s="4" t="inlineStr">
-        <is>
-          <t>Mobile responsive pass on every ported section</t>
-        </is>
-      </c>
-      <c r="C334" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D334" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-29: no page scrolls sideways at 375px any more (114 pages checked in Chrome: every unique page plus 3 of each templated set like blog posts and coffees). Fixed: BrewSoul NextSteps forced 3 columns (and used an inline style), charity-scorecard tab row, /brewsoul/browse filter dropdowns, /the-philosophy hero glow. Still to check by hand: 44px tap targets and Safari iOS. 2026-09-30: 44px tap targets on phones for the shared header, footer, BrewSoul/Kava/HumanOS menus and ~100 standalone links (undersized targets 1,904 → 578; the rest are 24-43px pills/chips that meet WCAG 2.2 AA). axe target-size (WCAG 2.2 AA, with its spacing exception): 0 failures on 114 pages. Safari/iPhone (WebKit, iPhone 14 emulation): all 114 pages load, no sideways scroll, no JS errors; form fields under 16px (iOS zoom-on-tap) fixed site-wide in globals.css. Still to check on a real iPhone: BrewSoul's bottom journey bar showed page text through it in headless WebKit only (taps hit the bar correctly; Chrome renders it solid). Fixed 2026-10-09: the bar is now solid (bg-[#2C1810], was 92% plus backdrop-blur-md), so nothing can show through even where the blur isn't drawn; checked in WebKit (iPhone 13 profile) and Chrome: background rgb(44, 24, 16), no text behind the buttons. A real iPhone check is still part of Phase 14. Checked 2026-10-13 in Apple's iPhone Simulator (iPhone 16, iOS 26.5, real Mobile Safari; not a physical phone, owner accepted this as the iPhone check): 14 key pages on a fresh prod</t>
-        </is>
-      </c>
-      <c r="E334" s="14" t="inlineStr">
-        <is>
-          <t>Phase 14 — QA &amp; Launch</t>
-        </is>
-      </c>
+      <c r="B334" s="11" t="n"/>
+      <c r="C334" s="11" t="n"/>
+      <c r="D334" s="12" t="n"/>
     </row>
     <row r="335">
       <c r="A335" s="4" t="n"/>
       <c r="B335" s="4" t="inlineStr">
         <is>
-          <t>Accessibility pass (WCAG AA contrast, 44px touch targets, keyboard nav)</t>
+          <t>Mobile responsive pass on every ported section</t>
         </is>
       </c>
       <c r="C335" s="13" t="inlineStr">
@@ -8519,7 +8519,7 @@
       </c>
       <c r="D335" s="4" t="inlineStr">
         <is>
-          <t>same bar as legacy QA_MASTER_PROMPT.md. 2026-09-29 axe-core pass (WCAG 2.1 AA, same 114 pages, production build): all unlabeled dropdowns/inputs and unnamed links fixed; contrast down from 1,453 failing items on 106 pages to 1,038 on 70 (43 pages fully clean). Shared fixes: brand gold #8b6914 → #836311 site-wide (was 4.3:1 on cream, AA needs 4.5), header "⌘K"/social icons, BrewSoul nav and footer, HumanOS footer, Kava footer, assessment intro footnote, post-card image links. 2026-09-30: contrast finished, 0 axe color-contrast failures left on the same 114 pages (production build). Token changes: --kava-saffron #b86a28 → #8e521f, --pri-purple-light #a855f7 → #b87bf9 (on-dark purple only), --crusade-teal #0e7c7c → #0d7373; PriEyebrow goes light purple inside a dark PriSection via group-data-dark/pri; /find-your-me and the journey tracker's dark glass panels 60-70% → 90% (legacy's own 60% glass on beige rendered gray, cream text failed). Everything else: nearest passing shade of the same hue, or gold ↔ gold-light on the wrong background. Left: 18 links inside text marked only by color (need an underline), 44px tap targets, keyboard nav. 2026-09-30: 18 color-only in-text links underlined (axe link-in-text-block: 0 left); keyboard focus visible on every focusable item on 8 sampled pages (two form fields had none, fixed). 2026-10-02 re-run (axe WCAG 2.2 AA, 142 pages × 375/1280px, production build, plus Tab through 40 stops per page): found 1,370 contrast failures (mostly BrewSoul'</t>
+          <t>2026-09-29: no page scrolls sideways at 375px any more (114 pages checked in Chrome: every unique page plus 3 of each templated set like blog posts and coffees). Fixed: BrewSoul NextSteps forced 3 columns (and used an inline style), charity-scorecard tab row, /brewsoul/browse filter dropdowns, /the-philosophy hero glow. Still to check by hand: 44px tap targets and Safari iOS. 2026-09-30: 44px tap targets on phones for the shared header, footer, BrewSoul/Kava/HumanOS menus and ~100 standalone links (undersized targets 1,904 → 578; the rest are 24-43px pills/chips that meet WCAG 2.2 AA). axe target-size (WCAG 2.2 AA, with its spacing exception): 0 failures on 114 pages. Safari/iPhone (WebKit, iPhone 14 emulation): all 114 pages load, no sideways scroll, no JS errors; form fields under 16px (iOS zoom-on-tap) fixed site-wide in globals.css. Still to check on a real iPhone: BrewSoul's bottom journey bar showed page text through it in headless WebKit only (taps hit the bar correctly; Chrome renders it solid). Fixed 2026-10-09: the bar is now solid (bg-[#2C1810], was 92% plus backdrop-blur-md), so nothing can show through even where the blur isn't drawn; checked in WebKit (iPhone 13 profile) and Chrome: background rgb(44, 24, 16), no text behind the buttons. A real iPhone check is still part of Phase 14. Checked 2026-10-13 in Apple's iPhone Simulator (iPhone 16, iOS 26.5, real Mobile Safari; not a physical phone, owner accepted this as the iPhone check): 14 key pages on a fresh prod</t>
         </is>
       </c>
       <c r="E335" s="14" t="inlineStr">
@@ -8532,7 +8532,7 @@
       <c r="A336" s="4" t="n"/>
       <c r="B336" s="4" t="inlineStr">
         <is>
-          <t>No dead-end pages (every page links to 2+ others)</t>
+          <t>Accessibility pass (WCAG AA contrast, 44px touch targets, keyboard nav)</t>
         </is>
       </c>
       <c r="C336" s="13" t="inlineStr">
@@ -8542,7 +8542,7 @@
       </c>
       <c r="D336" s="4" t="inlineStr">
         <is>
-          <t>same bar as legacy MASTER_QUALITY_PROMPT.md 2026-09-30 scan (496 sitemap pages, header/footer links not counted): every page has a way home (the 6 HumanOS pages had none, in legacy too; added a "← TonyGreenberg.com" footer link). ~17 quiz pages only look like dead ends on their intro screen; their result screens link to related assessments. Left for a content decision: ~20 marketing pages (/akbar, /amplifier, /diamond-cut, /ecosystem, /engage, /engine-room, /intel, /invest, /pick-up-the-phone, /protecting-your-business, /published, /speaking, /the-nightstand, /the-territory, /the-web, /under-nda, /pri-calibration, /charity-scorecard and its detail pages) link to only 0-1 other page in their content. The port matches legacy there (legacy was just as sparse), so adding related links is new content and needs the owner's yes. Done 2026-10-10 (owner said yes): a "Related" section with 3 real links (no redirects, titles and blurbs from each target's own copy) on all 19 sparse pages and every charity profile: data src/lib/content/related-pages.ts, component src/components/marketing/related-pages.tsx (light/dark). Checked at 375/820/1280px with no sideways scroll; found and fixed on the way: the essay date line couldn't wrap on phones (21px sideways on long category names).</t>
+          <t>same bar as legacy QA_MASTER_PROMPT.md. 2026-09-29 axe-core pass (WCAG 2.1 AA, same 114 pages, production build): all unlabeled dropdowns/inputs and unnamed links fixed; contrast down from 1,453 failing items on 106 pages to 1,038 on 70 (43 pages fully clean). Shared fixes: brand gold #8b6914 → #836311 site-wide (was 4.3:1 on cream, AA needs 4.5), header "⌘K"/social icons, BrewSoul nav and footer, HumanOS footer, Kava footer, assessment intro footnote, post-card image links. 2026-09-30: contrast finished, 0 axe color-contrast failures left on the same 114 pages (production build). Token changes: --kava-saffron #b86a28 → #8e521f, --pri-purple-light #a855f7 → #b87bf9 (on-dark purple only), --crusade-teal #0e7c7c → #0d7373; PriEyebrow goes light purple inside a dark PriSection via group-data-dark/pri; /find-your-me and the journey tracker's dark glass panels 60-70% → 90% (legacy's own 60% glass on beige rendered gray, cream text failed). Everything else: nearest passing shade of the same hue, or gold ↔ gold-light on the wrong background. Left: 18 links inside text marked only by color (need an underline), 44px tap targets, keyboard nav. 2026-09-30: 18 color-only in-text links underlined (axe link-in-text-block: 0 left); keyboard focus visible on every focusable item on 8 sampled pages (two form fields had none, fixed). 2026-10-02 re-run (axe WCAG 2.2 AA, 142 pages × 375/1280px, production build, plus Tab through 40 stops per page): found 1,370 contrast failures (mostly BrewSoul'</t>
         </is>
       </c>
       <c r="E336" s="14" t="inlineStr">
@@ -8555,7 +8555,7 @@
       <c r="A337" s="4" t="n"/>
       <c r="B337" s="4" t="inlineStr">
         <is>
-          <t>Cross-browser check (Safari iOS in particular, per legacy performance notes) 2026-10-06 WebKit pass (Playwright WebKit, iPhone 13 profile, 1…</t>
+          <t>No dead-end pages (every page links to 2+ others)</t>
         </is>
       </c>
       <c r="C337" s="13" t="inlineStr">
@@ -8565,7 +8565,7 @@
       </c>
       <c r="D337" s="4" t="inlineStr">
         <is>
-          <t>52 pages: every unique page plus 3 of each templated set, production build): no page pans sideways, no failed requests, no JS errors. Found and fixed on the way: upgrade-insecure-requests in the new CSP made Safari fetch every stylesheet and font over https on localhost (dropped; the site is HTTPS-only via HSTS anyway), and .toLocaleString() without a locale caused a hydration error on /brewsoul/chains in Safari (all number formatting now en-US). Left: a check on a real iPhone (Phase 14). Checked 2026-10-13 in Apple's iPhone Simulator (iPhone 16, iOS 26.5, real Mobile Safari; not a physical phone, owner accepted this as the iPhone check): 14 key pages on a fresh production build (/, /blog, an essay, /brewsoul, /brewsoul/browse, /find-your-journey, /psychedelic-readiness-index, /kava, /humanos, /about, /iboga-ibogaine, /peptide-hall-of-shame, /my-journey, /pri-calibration): all render, no sideways pan, header and menus in place, BrewSoul's bottom bar solid. / and /blog showed blank on the very first cold load, then load within 3 s on every later visit.</t>
+          <t>same bar as legacy MASTER_QUALITY_PROMPT.md 2026-09-30 scan (496 sitemap pages, header/footer links not counted): every page has a way home (the 6 HumanOS pages had none, in legacy too; added a "← TonyGreenberg.com" footer link). ~17 quiz pages only look like dead ends on their intro screen; their result screens link to related assessments. Left for a content decision: ~20 marketing pages (/akbar, /amplifier, /diamond-cut, /ecosystem, /engage, /engine-room, /intel, /invest, /pick-up-the-phone, /protecting-your-business, /published, /speaking, /the-nightstand, /the-territory, /the-web, /under-nda, /pri-calibration, /charity-scorecard and its detail pages) link to only 0-1 other page in their content. The port matches legacy there (legacy was just as sparse), so adding related links is new content and needs the owner's yes. Done 2026-10-10 (owner said yes): a "Related" section with 3 real links (no redirects, titles and blurbs from each target's own copy) on all 19 sparse pages and every charity profile: data src/lib/content/related-pages.ts, component src/components/marketing/related-pages.tsx (light/dark). Checked at 375/820/1280px with no sideways scroll; found and fixed on the way: the essay date line couldn't wrap on phones (21px sideways on long category names).</t>
         </is>
       </c>
       <c r="E337" s="14" t="inlineStr">
@@ -8578,7 +8578,7 @@
       <c r="A338" s="4" t="n"/>
       <c r="B338" s="4" t="inlineStr">
         <is>
-          <t>Remove noindex only when sign-off is given</t>
+          <t>Cross-browser check (Safari iOS in particular, per legacy performance notes) 2026-10-06 WebKit pass (Playwright WebKit, iPhone 13 profile, 1…</t>
         </is>
       </c>
       <c r="C338" s="13" t="inlineStr">
@@ -8588,7 +8588,7 @@
       </c>
       <c r="D338" s="4" t="inlineStr">
         <is>
-          <t>do not launch indexable by accident (The only noindex is the host-based one for .netlify.app above, so the real domain is indexable as soon as DNS points at it: sign-off must come before DNS.) Re-checked 2026-10-13 on a fresh production build: tonygreenberg.com and www get no X-Robots-Tag and no robots meta (/, /blog, /about, /post-intervention), *.netlify.app gets noindex, nofollow; robots.txt allows crawlers, sitemap 200, missing pages 404, /manifesto 308. Ready; still waits on sign-off. Done 2026-10-13 (sign-off given): nothing to switch off. The only noindex is host-based (.netlify.app), so tonygreenberg.com becomes indexable by Google the moment DNS points at Netlify (re-checked on today's build: no X-Robots-Tag or robots meta for the real domain).</t>
+          <t>52 pages: every unique page plus 3 of each templated set, production build): no page pans sideways, no failed requests, no JS errors. Found and fixed on the way: upgrade-insecure-requests in the new CSP made Safari fetch every stylesheet and font over https on localhost (dropped; the site is HTTPS-only via HSTS anyway), and .toLocaleString() without a locale caused a hydration error on /brewsoul/chains in Safari (all number formatting now en-US). Left: a check on a real iPhone (Phase 14). Checked 2026-10-13 in Apple's iPhone Simulator (iPhone 16, iOS 26.5, real Mobile Safari; not a physical phone, owner accepted this as the iPhone check): 14 key pages on a fresh production build (/, /blog, an essay, /brewsoul, /brewsoul/browse, /find-your-journey, /psychedelic-readiness-index, /kava, /humanos, /about, /iboga-ibogaine, /peptide-hall-of-shame, /my-journey, /pri-calibration): all render, no sideways pan, header and menus in place, BrewSoul's bottom bar solid. / and /blog showed blank on the very first cold load, then load within 3 s on every later visit.</t>
         </is>
       </c>
       <c r="E338" s="14" t="inlineStr">
@@ -8601,7 +8601,7 @@
       <c r="A339" s="4" t="n"/>
       <c r="B339" s="4" t="inlineStr">
         <is>
-          <t>Final stakeholder sign-off (Tony/Darryl/Kimberly) on the ported site before DNS cutover Given 2026-10-13 by the webmaster (web.master@rampra…</t>
+          <t>Remove noindex only when sign-off is given</t>
         </is>
       </c>
       <c r="C339" s="13" t="inlineStr">
@@ -8611,7 +8611,7 @@
       </c>
       <c r="D339" s="4" t="inlineStr">
         <is>
-          <t>te.com) in a Claude Code session, answering "Tony's team sign-off, then turning on Google indexing" with yes. If Tony, Darryl or Kimberly haven't seen the Netlify copy themselves, get their yes before the DNS switch.</t>
+          <t>do not launch indexable by accident (The only noindex is the host-based one for .netlify.app above, so the real domain is indexable as soon as DNS points at it: sign-off must come before DNS.) Re-checked 2026-10-13 on a fresh production build: tonygreenberg.com and www get no X-Robots-Tag and no robots meta (/, /blog, /about, /post-intervention), *.netlify.app gets noindex, nofollow; robots.txt allows crawlers, sitemap 200, missing pages 404, /manifesto 308. Ready; still waits on sign-off. Done 2026-10-13 (sign-off given): nothing to switch off. The only noindex is host-based (.netlify.app), so tonygreenberg.com becomes indexable by Google the moment DNS points at Netlify (re-checked on today's build: no X-Robots-Tag or robots meta for the real domain).</t>
         </is>
       </c>
       <c r="E339" s="14" t="inlineStr">
@@ -8624,7 +8624,7 @@
       <c r="A340" s="4" t="n"/>
       <c r="B340" s="4" t="inlineStr">
         <is>
-          <t>Privacy Policy page (/privacy) + footer link</t>
+          <t>Final stakeholder sign-off (Tony/Darryl/Kimberly) on the ported site before DNS cutover Given 2026-10-13 by the webmaster (web.master@rampra…</t>
         </is>
       </c>
       <c r="C340" s="13" t="inlineStr">
@@ -8634,7 +8634,7 @@
       </c>
       <c r="D340" s="4" t="inlineStr">
         <is>
-          <t>(team review 2026-10-14; owner: "create any page that isn't there"). Neither live nor the old app has one, so it's a new page. Wording drafted from what the code really does: newsletter (Kit), member accounts, quiz results (sexuality/religion save only "finished"), comments/reactions/highlights, the site's forms (Supabase, emailed to Tony via Resend), supplier intake to RampRate, Google Analytics, the sign-in, tg_visit_count and visitor-session cookies, browser storage. Contact for requests: t@ramprate.com (the footer's address). Josh (legal) to review the wording before launch.</t>
+          <t>te.com) in a Claude Code session, answering "Tony's team sign-off, then turning on Google indexing" with yes. If Tony, Darryl or Kimberly haven't seen the Netlify copy themselves, get their yes before the DNS switch.</t>
         </is>
       </c>
       <c r="E340" s="14" t="inlineStr">
@@ -8647,7 +8647,7 @@
       <c r="A341" s="4" t="n"/>
       <c r="B341" s="4" t="inlineStr">
         <is>
-          <t>Terms of Use page (/terms) + footer link</t>
+          <t>Privacy Policy page (/privacy) + footer link</t>
         </is>
       </c>
       <c r="C341" s="13" t="inlineStr">
@@ -8657,7 +8657,7 @@
       </c>
       <c r="D341" s="4" t="inlineStr">
         <is>
-          <t>(team review 2026-10-14). Not-medical-advice (peptides, diet, therapy, kava, psychedelics, ibogaine) and not-investment-advice (waitlists are not offers) sections, ownership matching the footer notice, user content, liability, California law. /terms was one of the intentional 404s; now a real page (ROUTES-INVENTORY.md updated). Josh (legal) to review before launch.</t>
+          <t>(team review 2026-10-14; owner: "create any page that isn't there"). Neither live nor the old app has one, so it's a new page. Wording drafted from what the code really does: newsletter (Kit), member accounts, quiz results (sexuality/religion save only "finished"), comments/reactions/highlights, the site's forms (Supabase, emailed to Tony via Resend), supplier intake to RampRate, Google Analytics, the sign-in, tg_visit_count and visitor-session cookies, browser storage. Contact for requests: t@ramprate.com (the footer's address). Josh (legal) to review the wording before launch.</t>
         </is>
       </c>
       <c r="E341" s="14" t="inlineStr">
@@ -8670,7 +8670,7 @@
       <c r="A342" s="4" t="n"/>
       <c r="B342" s="4" t="inlineStr">
         <is>
-          <t>Contact page (/contact) + footer link</t>
+          <t>Terms of Use page (/terms) + footer link</t>
         </is>
       </c>
       <c r="C342" s="13" t="inlineStr">
@@ -8680,7 +8680,7 @@
       </c>
       <c r="D342" s="4" t="inlineStr">
         <is>
-          <t>(team review 2026-10-14). Gathers details already on the site: email t@ramprate.com (now also a clickable link in the footer, where it was plain text), booking link, the Engagement Audit (/pick-up-the-phone), RampRate supplier intake, Santa Monica, X and LinkedIn. No form (none needed: every option already exists). Checked 2026-10-14 for all three: type check, lint, Manus grep, build (all ○ static), fresh server: 200, one H1, title, canonical, share image, in the sitemap and Ask Tony search, footer links on every page; browser at 375/820/1280 light and 375/1280 dark: no sideways scroll, no JS errors.</t>
+          <t>(team review 2026-10-14). Not-medical-advice (peptides, diet, therapy, kava, psychedelics, ibogaine) and not-investment-advice (waitlists are not offers) sections, ownership matching the footer notice, user content, liability, California law. /terms was one of the intentional 404s; now a real page (ROUTES-INVENTORY.md updated). Josh (legal) to review before launch.</t>
         </is>
       </c>
       <c r="E342" s="14" t="inlineStr">
@@ -8693,7 +8693,7 @@
       <c r="A343" s="4" t="n"/>
       <c r="B343" s="4" t="inlineStr">
         <is>
-          <t>Essay counts match</t>
+          <t>Contact page (/contact) + footer link</t>
         </is>
       </c>
       <c r="C343" s="13" t="inlineStr">
@@ -8703,7 +8703,7 @@
       </c>
       <c r="D343" s="4" t="inlineStr">
         <is>
-          <t>(team review 2026-10-14). Ask Tony's Blog entry said "92 essays" (copied from the old app), the homepage Read card "118", /subscribe and /the-letter's Read card "121", while the homepage and /search count 123 from Sanity. All now use Sanity's count ({count} in home-doors.ts and /the-letter's doors, /subscribe fetches it). Ask Tony (owner: show the number): the root layout fetches the count and passes it to SiteHeader → SearchModal; withEssayCount() in search-directory.ts fills {count} for Ask Tony, /search and /the-index too. Checked in a browser: Ask Tony shows "123 essays spanning 15 years", build still 150 static / 28 dynamic pages as before. Left alone: /living-declaration's "QPR Index scores intellectual rigor across 91 essays" (a claim about that tool, Tony's copy). Checked 2026-10-14: type check, lint, build (/, /subscribe, /the-letter still static), fresh server: all three show 123, no "92 essays" in the built browser code.</t>
+          <t>(team review 2026-10-14). Gathers details already on the site: email t@ramprate.com (now also a clickable link in the footer, where it was plain text), booking link, the Engagement Audit (/pick-up-the-phone), RampRate supplier intake, Santa Monica, X and LinkedIn. No form (none needed: every option already exists). Checked 2026-10-14 for all three: type check, lint, Manus grep, build (all ○ static), fresh server: 200, one H1, title, canonical, share image, in the sitemap and Ask Tony search, footer links on every page; browser at 375/820/1280 light and 375/1280 dark: no sideways scroll, no JS errors.</t>
         </is>
       </c>
       <c r="E343" s="14" t="inlineStr">
@@ -8716,7 +8716,7 @@
       <c r="A344" s="4" t="n"/>
       <c r="B344" s="4" t="inlineStr">
         <is>
-          <t>Team review's "everything else looks fine" re-checked</t>
+          <t>Essay counts match</t>
         </is>
       </c>
       <c r="C344" s="13" t="inlineStr">
@@ -8726,7 +8726,7 @@
       </c>
       <c r="D344" s="4" t="inlineStr">
         <is>
-          <t>(2026-10-14, owner: "you can check"). Fresh production build: all 60 menu pages (main menu, Fix Myself, Explore...) at 1280px and 375px: 200, one H1, no sideways scroll, no JS errors. All 130 blog links on them (122 posts, 8 categories): 200, no redirects. 404 page: 404 for a missing page, essay and category. Dark mode: switches and stays on across pages; 10 essays checked on a phone in dark mode. Phone menu shows every section; Ask Tony works on a phone. Netlify test site: the same 60 menu pages answer. Two small fixes: a missing essay or category showed the homepage's tab title on its 404 page (now "Page not found"); three Explore links (/attention-theft/weapons, /report, /legal) went through a redirect, now link straight to /attention-theft#weapons etc. Checked: type check, lint, build, clicked "Legal Database" in the menu.</t>
+          <t>(team review 2026-10-14). Ask Tony's Blog entry said "92 essays" (copied from the old app), the homepage Read card "118", /subscribe and /the-letter's Read card "121", while the homepage and /search count 123 from Sanity. All now use Sanity's count ({count} in home-doors.ts and /the-letter's doors, /subscribe fetches it). Ask Tony (owner: show the number): the root layout fetches the count and passes it to SiteHeader → SearchModal; withEssayCount() in search-directory.ts fills {count} for Ask Tony, /search and /the-index too. Checked in a browser: Ask Tony shows "123 essays spanning 15 years", build still 150 static / 28 dynamic pages as before. Left alone: /living-declaration's "QPR Index scores intellectual rigor across 91 essays" (a claim about that tool, Tony's copy). Checked 2026-10-14: type check, lint, build (/, /subscribe, /the-letter still static), fresh server: all three show 123, no "92 essays" in the built browser code.</t>
         </is>
       </c>
       <c r="E344" s="14" t="inlineStr">
@@ -8739,7 +8739,7 @@
       <c r="A345" s="4" t="n"/>
       <c r="B345" s="4" t="inlineStr">
         <is>
-          <t>Automated tests for every file (2026-10-16, owner</t>
+          <t>Team review's "everything else looks fine" re-checked</t>
         </is>
       </c>
       <c r="C345" s="13" t="inlineStr">
@@ -8749,7 +8749,7 @@
       </c>
       <c r="D345" s="4" t="inlineStr">
         <is>
-          <t>"write a test case for the full project</t>
+          <t>(2026-10-14, owner: "you can check"). Fresh production build: all 60 menu pages (main menu, Fix Myself, Explore...) at 1280px and 375px: 200, one H1, no sideways scroll, no JS errors. All 130 blog links on them (122 posts, 8 categories): 200, no redirects. 404 page: 404 for a missing page, essay and category. Dark mode: switches and stays on across pages; 10 essays checked on a phone in dark mode. Phone menu shows every section; Ask Tony works on a phone. Netlify test site: the same 60 menu pages answer. Two small fixes: a missing essay or category showed the homepage's tab title on its 404 page (now "Page not found"); three Explore links (/attention-theft/weapons, /report, /legal) went through a redirect, now link straight to /attention-theft#weapons etc. Checked: type check, lint, build, clicked "Legal Database" in the menu.</t>
         </is>
       </c>
       <c r="E345" s="14" t="inlineStr">
@@ -8762,7 +8762,7 @@
       <c r="A346" s="4" t="n"/>
       <c r="B346" s="4" t="inlineStr">
         <is>
-          <t>Security: two holes found by the tests (2026-10-16), fix before launch</t>
+          <t>Automated tests for every file (2026-10-16, owner</t>
         </is>
       </c>
       <c r="C346" s="13" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="D346" s="4" t="inlineStr">
         <is>
-          <t>Fixed 2026-10-16 (owner: "you can try to pass all"): safeNext now reads the path the way a browser does and refuses anything that leaves the site (backslash, and also tab/newline tricks like /&lt;tab&gt;/evil.com, found while checking the first fix); upload links re-check the admin list. Checked: tests, real server (/login?next=/%5Cevil.com and /%09/evil.com fall back to /my-highlights). (1)</t>
+          <t>"write a test case for the full project</t>
         </is>
       </c>
       <c r="E346" s="14" t="inlineStr">
@@ -8785,7 +8785,7 @@
       <c r="A347" s="4" t="n"/>
       <c r="B347" s="4" t="inlineStr">
         <is>
-          <t>PRI results: safety and scoring (2026-10-16), needs a yes</t>
+          <t>Security: two holes found by the tests (2026-10-16), fix before launch</t>
         </is>
       </c>
       <c r="C347" s="13" t="inlineStr">
@@ -8795,7 +8795,7 @@
       </c>
       <c r="D347" s="4" t="inlineStr">
         <is>
-          <t>Fixed 2026-10-16: Hard Stop medicines are filtered out before matching; the match score is a real 0-100% (labels can show); missing answers no longer give NaN. src/lib/content/pri-shared.ts:</t>
+          <t>Fixed 2026-10-16 (owner: "you can try to pass all"): safeNext now reads the path the way a browser does and refuses anything that leaves the site (backslash, and also tab/newline tricks like /&lt;tab&gt;/evil.com, found while checking the first fix); upload links re-check the admin list. Checked: tests, real server (/login?next=/%5Cevil.com and /%09/evil.com fall back to /my-highlights). (1)</t>
         </is>
       </c>
       <c r="E347" s="14" t="inlineStr">
@@ -8808,7 +8808,7 @@
       <c r="A348" s="4" t="n"/>
       <c r="B348" s="4" t="inlineStr">
         <is>
-          <t>Quiz results that come out wrong (2026-10-16), copied from live, needs the owner's</t>
+          <t>PRI results: safety and scoring (2026-10-16), needs a yes</t>
         </is>
       </c>
       <c r="C348" s="13" t="inlineStr">
@@ -8816,7 +8816,11 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="D348" s="4" t="inlineStr"/>
+      <c r="D348" s="4" t="inlineStr">
+        <is>
+          <t>Fixed 2026-10-16: Hard Stop medicines are filtered out before matching; the match score is a real 0-100% (labels can show); missing answers no longer give NaN. src/lib/content/pri-shared.ts:</t>
+        </is>
+      </c>
       <c r="E348" s="14" t="inlineStr">
         <is>
           <t>Phase 14 — QA &amp; Launch</t>
@@ -8827,7 +8831,7 @@
       <c r="A349" s="4" t="n"/>
       <c r="B349" s="4" t="inlineStr">
         <is>
-          <t>Wrong or broken information (2026-10-16)</t>
+          <t>Quiz results that come out wrong (2026-10-16), copied from live, needs the owner's</t>
         </is>
       </c>
       <c r="C349" s="13" t="inlineStr">
@@ -8835,11 +8839,7 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="D349" s="4" t="inlineStr">
-        <is>
-          <t>Fixed 2026-10-16: all of these. BrewSoul grades now follow one rule (owner): the GRADE_SCALE table shown on the site, worked out from each score (some letters changed, e.g. Starbucks D+ to D, Seattle A- to A); /clients keeps "90+" (owner: real total, the page shows a selection); hall of shame average worked out from the clinics (95); /the-philosophy count from the data (39); short link jwd9jx to the restaurant AI-ethics essay (the only place the old sign-up box lived). BrewSoul "My Collection" links to</t>
-        </is>
-      </c>
+      <c r="D349" s="4" t="inlineStr"/>
       <c r="E349" s="14" t="inlineStr">
         <is>
           <t>Phase 14 — QA &amp; Launch</t>
@@ -8850,7 +8850,7 @@
       <c r="A350" s="4" t="n"/>
       <c r="B350" s="4" t="inlineStr">
         <is>
-          <t>Content Google can't see, and missing tags (2026-10-16)</t>
+          <t>Wrong or broken information (2026-10-16)</t>
         </is>
       </c>
       <c r="C350" s="13" t="inlineStr">
@@ -8860,7 +8860,7 @@
       </c>
       <c r="D350" s="4" t="inlineStr">
         <is>
-          <t>Fixed 2026-10-16: all three are in the server HTML now (hidden until opened); /assessment and /iboga-compass have exactly one H1 per screen; both America Unbundled pages keep @ThinkTony. Checked on a fresh pnpm start: 23 changed pages 200 with one H1. Only shown after a click, so not</t>
+          <t>Fixed 2026-10-16: all of these. BrewSoul grades now follow one rule (owner): the GRADE_SCALE table shown on the site, worked out from each score (some letters changed, e.g. Starbucks D+ to D, Seattle A- to A); /clients keeps "90+" (owner: real total, the page shows a selection); hall of shame average worked out from the clinics (95); /the-philosophy count from the data (39); short link jwd9jx to the restaurant AI-ethics essay (the only place the old sign-up box lived). BrewSoul "My Collection" links to</t>
         </is>
       </c>
       <c r="E350" s="14" t="inlineStr">
@@ -8873,7 +8873,7 @@
       <c r="A351" s="4" t="n"/>
       <c r="B351" s="4" t="inlineStr">
         <is>
-          <t>Keyboard and screen-reader fixes (2026-10-16)</t>
+          <t>Content Google can't see, and missing tags (2026-10-16)</t>
         </is>
       </c>
       <c r="C351" s="13" t="inlineStr">
@@ -8883,7 +8883,7 @@
       </c>
       <c r="D351" s="4" t="inlineStr">
         <is>
-          <t>Fixed 2026-10-16: every item, plus the compact journey tracker (it looked clickable and did nothing: now opens the full list) and typed ▲▼↑↓ arrows swapped for icons in 8 places (rule 18). Checked in Chrome at 375 and 1280: Kava myths, BrewSoul chains, roasters, decaf, peptide fraud patterns, Shanita interview open by click and by keyboard, no sideways scroll, no errors. Clickable &lt;div&gt;s with no button</t>
+          <t>Fixed 2026-10-16: all three are in the server HTML now (hidden until opened); /assessment and /iboga-compass have exactly one H1 per screen; both America Unbundled pages keep @ThinkTony. Checked on a fresh pnpm start: 23 changed pages 200 with one H1. Only shown after a click, so not</t>
         </is>
       </c>
       <c r="E351" s="14" t="inlineStr">
@@ -8896,7 +8896,7 @@
       <c r="A352" s="4" t="n"/>
       <c r="B352" s="4" t="inlineStr">
         <is>
-          <t>Find Your Me essay links (2026-10-16, owner: "you can start")</t>
+          <t>Keyboard and screen-reader fixes (2026-10-16)</t>
         </is>
       </c>
       <c r="C352" s="13" t="inlineStr">
@@ -8906,7 +8906,7 @@
       </c>
       <c r="D352" s="4" t="inlineStr">
         <is>
-          <t>Checked all 17 against</t>
+          <t>Fixed 2026-10-16: every item, plus the compact journey tracker (it looked clickable and did nothing: now opens the full list) and typed ▲▼↑↓ arrows swapped for icons in 8 places (rule 18). Checked in Chrome at 375 and 1280: Kava myths, BrewSoul chains, roasters, decaf, peptide fraud patterns, Shanita interview open by click and by keyboard, no sideways scroll, no errors. Clickable &lt;div&gt;s with no button</t>
         </is>
       </c>
       <c r="E352" s="14" t="inlineStr">
@@ -8919,17 +8919,17 @@
       <c r="A353" s="4" t="n"/>
       <c r="B353" s="4" t="inlineStr">
         <is>
-          <t>Find Your Me: pick real essays for two results (2026-10-16), needs Tony</t>
-        </is>
-      </c>
-      <c r="C353" s="16" t="inlineStr">
-        <is>
-          <t>Remaining</t>
+          <t>Find Your Me essay links (2026-10-16, owner: "you can start")</t>
+        </is>
+      </c>
+      <c r="C353" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D353" s="4" t="inlineStr">
         <is>
-          <t>The Systems</t>
+          <t>Checked all 17 against</t>
         </is>
       </c>
       <c r="E353" s="14" t="inlineStr">
@@ -8942,15 +8942,19 @@
       <c r="A354" s="4" t="n"/>
       <c r="B354" s="4" t="inlineStr">
         <is>
-          <t>Every file at 90%+ test coverage (2026-10-16, owner: "90+ for all file")</t>
-        </is>
-      </c>
-      <c r="C354" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D354" s="4" t="inlineStr"/>
+          <t>Find Your Me: pick real essays for two results (2026-10-16), needs Tony</t>
+        </is>
+      </c>
+      <c r="C354" s="16" t="inlineStr">
+        <is>
+          <t>Remaining</t>
+        </is>
+      </c>
+      <c r="D354" s="4" t="inlineStr">
+        <is>
+          <t>The Systems</t>
+        </is>
+      </c>
       <c r="E354" s="14" t="inlineStr">
         <is>
           <t>Phase 14 — QA &amp; Launch</t>
@@ -8961,19 +8965,15 @@
       <c r="A355" s="4" t="n"/>
       <c r="B355" s="4" t="inlineStr">
         <is>
-          <t>Quiz content questions for Tony (2026-10-16)</t>
-        </is>
-      </c>
-      <c r="C355" s="16" t="inlineStr">
-        <is>
-          <t>Remaining</t>
-        </is>
-      </c>
-      <c r="D355" s="4" t="inlineStr">
-        <is>
-          <t>Consciousness Scale: the answer scores only</t>
-        </is>
-      </c>
+          <t>Every file at 90%+ test coverage (2026-10-16, owner: "90+ for all file")</t>
+        </is>
+      </c>
+      <c r="C355" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D355" s="4" t="inlineStr"/>
       <c r="E355" s="14" t="inlineStr">
         <is>
           <t>Phase 14 — QA &amp; Launch</t>
@@ -8984,36 +8984,59 @@
       <c r="A356" s="4" t="n"/>
       <c r="B356" s="4" t="inlineStr">
         <is>
+          <t>Quiz content questions for Tony (2026-10-16)</t>
+        </is>
+      </c>
+      <c r="C356" s="16" t="inlineStr">
+        <is>
+          <t>Remaining</t>
+        </is>
+      </c>
+      <c r="D356" s="4" t="inlineStr">
+        <is>
+          <t>Consciousness Scale: the answer scores only</t>
+        </is>
+      </c>
+      <c r="E356" s="14" t="inlineStr">
+        <is>
+          <t>Phase 14 — QA &amp; Launch</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" s="4" t="n"/>
+      <c r="B357" s="4" t="inlineStr">
+        <is>
           <t>DNS cutover, legacy app decommissioned only after a stable overlap window Re-checked 2026-10-13</t>
         </is>
       </c>
-      <c r="C356" s="16" t="inlineStr">
+      <c r="C357" s="16" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
       </c>
-      <c r="D356" s="4" t="inlineStr">
+      <c r="D357" s="4" t="inlineStr">
         <is>
           <t>unchanged (Hostinger name servers, bare domain on Manus 104.19.168/169.112, www CNAME cname.manus.space). Checked 2026-10-09 (owner wants to go live and switch off Manus): DNS for tonygreenberg.com is at Hostinger (name servers ns1/ns2.dns-parking.com); www is a CNAME to cname.manus.space, the bare domain points at Manus's addresses (104.19.168.112 / .169.112); the Netlify site tonygreenberg-website has no custom domain yet (production branch main). Order: (1) merge the three open pull requests into main and check the Netlify copy; (2) restore Supabase and run 0001 to 0003, or launch without member features (they say "isn't available just now"); (3) owner sign-off; (4) add tonygreenberg.com + www in Netlify (Domain management), then at Hostinger point the bare domain at Netlify (A record 75.2.60.5, or Netlify DNS) and www CNAME at tonygreenberg-website.netlify.app; Netlify issues the HTTPS certificate; (5) re-run scripts/check-search-console-urls.ts https://tonygreenberg.com and submit the sitemap in Search Console; (6) only after a few stable days: switch off the Manus site (the database is already backed up, docs/ai/project_legacy_database.md) and rotate the old database password.</t>
         </is>
       </c>
-      <c r="E356" s="14" t="inlineStr">
+      <c r="E357" s="14" t="inlineStr">
         <is>
           <t>Phase 14 — QA &amp; Launch</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D356"/>
+  <autoFilter ref="A1:D357"/>
   <mergeCells count="14">
+    <mergeCell ref="A334:D334"/>
     <mergeCell ref="A245:D245"/>
     <mergeCell ref="A158:D158"/>
-    <mergeCell ref="A333:D333"/>
-    <mergeCell ref="A313:D313"/>
+    <mergeCell ref="A267:D267"/>
+    <mergeCell ref="A314:D314"/>
     <mergeCell ref="A15:D15"/>
     <mergeCell ref="A64:D64"/>
     <mergeCell ref="A213:D213"/>
-    <mergeCell ref="A266:D266"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A49:D49"/>
     <mergeCell ref="A129:D129"/>

</xml_diff>

<commit_message>
Status: go-live (DNS cutover), MCP on live address, PR #18 merged
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Migration-Status-Report.xlsx
+++ b/Migration-Status-Report.xlsx
@@ -9017,7 +9017,7 @@
       </c>
       <c r="D357" s="4" t="inlineStr">
         <is>
-          <t>unchanged (Hostinger name servers, bare domain on Manus 104.19.168/169.112, www CNAME cname.manus.space). Checked 2026-10-09 (owner wants to go live and switch off Manus): DNS for tonygreenberg.com is at Hostinger (name servers ns1/ns2.dns-parking.com); www is a CNAME to cname.manus.space, the bare domain points at Manus's addresses (104.19.168.112 / .169.112); the Netlify site tonygreenberg-website has no custom domain yet (production branch main). Order: (1) merge the three open pull requests into main and check the Netlify copy; (2) restore Supabase and run 0001 to 0003, or launch without member features (they say "isn't available just now"); (3) owner sign-off; (4) add tonygreenberg.com + www in Netlify (Domain management), then at Hostinger point the bare domain at Netlify (A record 75.2.60.5, or Netlify DNS) and www CNAME at tonygreenberg-website.netlify.app; Netlify issues the HTTPS certificate; (5) re-run scripts/check-search-console-urls.ts https://tonygreenberg.com and submit the sitemap in Search Console; (6) only after a few stable days: switch off the Manus site (the database is already backed up, docs/ai/project_legacy_database.md) and rotate the old database password.</t>
+          <t>unchanged (Hostinger name servers, bare domain on Manus 104.19.168/169.112, www CNAME cname.manus.space). Checked 2026-10-09 (owner wants to go live and switch off Manus): DNS for tonygreenberg.com is at Hostinger (name servers ns1/ns2.dns-parking.com); www is a CNAME to cname.manus.space, the bare domain points at Manus's addresses (104.19.168.112 / .169.112); the Netlify site tonygreenberg-website has no custom domain yet (production branch main). Order: (1) merge the three open pull requests into main and check the Netlify copy; (2) restore Supabase and run 0001 to 0003, or launch without member features (they say "isn't available just now"); (3) owner sign-off; (4) add tonygreenberg.com + www in Netlify (Domain management), then at Hostinger point the bare domain at Netlify (A record 75.2.60.5, or Netlify DNS) and www CNAME at tonygreenberg-website.netlify.app; Netlify issues the HTTPS certificate; (5) re-run scripts/check-search-console-urls.ts https://tonygreenberg.com and submit the sitemap in Search Console; (6) only after a few stable days: switch off the Manus site (the database is already backed up, docs/ai/project_legacy_database.md) and rotate the old database password. 2026-10-16: steps 1 to 4 done (owner added the domains in Netlify and the A/CNAME records at Hostinger; both resolve to Netlify, HTTPS works, email records untouched). Left: step 5 (Search Console re-check and sitemap), change the Sanity webhook URL to https://tonygreenberg.com/api/revalidate, the</t>
         </is>
       </c>
       <c r="E357" s="14" t="inlineStr">
@@ -9298,7 +9298,7 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>unchanged (Hostinger name servers, bare domain on Manus 104.19.168/169.112, www CNAME cname.manus.space). Checked 2026-10-09 (owner wants to go live and switch off Manus): DNS for tonygreenberg.com is at Hostinger (name servers ns1/ns2.dns-parking.com); www is a CNAME to cname.manus.space, the bare domain points at Manus's addresses (104.19.168.112 / .169.112); the Netlify site tonygreenberg-website has no custom domain yet (production branch main). Order: (1) merge the three open pull requests into main and check the Netlify copy; (2) restore Supabase and run 0001 to 0003, or launch without member features (they say "isn't available just now"); (3) owner sign-off; (4) add tonygreenberg.com + www in Netlify (Domain management), then at Hostinger point the bare domain at Netlify (A record 75.2.60.5, or Netlify DNS) and www CNAME at tonygreenberg-website.netlify.app; Netlify issues the HTTPS certificate; (5) re-run scripts/check-search-console-urls.ts https://tonygreenberg.com and submit the sitemap in Search Console; (6) only after a few stable days: switch off the Manus site (the database is already backed up, docs/ai/project_legacy_database.md) and rotate the old database password.</t>
+          <t>unchanged (Hostinger name servers, bare domain on Manus 104.19.168/169.112, www CNAME cname.manus.space). Checked 2026-10-09 (owner wants to go live and switch off Manus): DNS for tonygreenberg.com is at Hostinger (name servers ns1/ns2.dns-parking.com); www is a CNAME to cname.manus.space, the bare domain points at Manus's addresses (104.19.168.112 / .169.112); the Netlify site tonygreenberg-website has no custom domain yet (production branch main). Order: (1) merge the three open pull requests into main and check the Netlify copy; (2) restore Supabase and run 0001 to 0003, or launch without member features (they say "isn't available just now"); (3) owner sign-off; (4) add tonygreenberg.com + www in Netlify (Domain management), then at Hostinger point the bare domain at Netlify (A record 75.2.60.5, or Netlify DNS) and www CNAME at tonygreenberg-website.netlify.app; Netlify issues the HTTPS certificate; (5) re-run scripts/check-search-console-urls.ts https://tonygreenberg.com and submit the sitemap in Search Console; (6) only after a few stable days: switch off the Manus site (the database is already backed up, docs/ai/project_legacy_database.md) and rotate the old database password. 2026-10-16: steps 1 to 4 done (owner added the domains in Netlify and the A/CNAME records at Hostinger; both resolve to Netlify, HTTPS works, email records untouched). Left: step 5 (Search Console re-check and sitemap), change the Sanity webhook URL to https://tonygreenberg.com/api/revalidate, the</t>
         </is>
       </c>
       <c r="E13" s="14" t="inlineStr">

</xml_diff>

<commit_message>
MCP server: fix duplicate required key that made ChatGPT drop every tool
request_upload_link listed change_id in its own required list and
withChangeIdParam appended it again. Claude tolerates the invalid schema;
ChatGPT drops the whole app ("TonyWeb editing tools aren't available").
Same bug ramprate-ui fixed 2026-10-08. The param helpers now never add a
key twice, and a test checks every tool schema for every role.

Also: PR checks run the full Vitest suite (like ramprate-ui), and the
ES2018-only regex flag in github-client.ts that failed tsc is replaced.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Migration-Status-Report.xlsx
+++ b/Migration-Status-Report.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Remaining Work" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Full Detail'!$A$1:$D$357</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Full Detail'!$A$1:$D$358</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Remaining Work'!$A$1:$D$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -596,7 +596,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated from NEXTJS-MIGRATION-TODO.md on 2026-10-16 by scripts/build-migration-status-report.py — a living document; re-run the script after updating the todo file. Counts are formulas over the Full Detail tab.</t>
+          <t>Generated from NEXTJS-MIGRATION-TODO.md on 2026-10-17 by scripts/build-migration-status-report.py — a living document; re-run the script after updating the todo file. Counts are formulas over the Full Detail tab.</t>
         </is>
       </c>
     </row>
@@ -639,15 +639,15 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A5,'Full Detail'!$C$2:$C$357,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$358,$A5,'Full Detail'!$C$2:$C$358,"Done")</f>
         <v/>
       </c>
       <c r="C5" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A5,'Full Detail'!$C$2:$C$357,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$358,$A5,'Full Detail'!$C$2:$C$358,"Remaining")</f>
         <v/>
       </c>
       <c r="D5" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A5,'Full Detail'!$C$2:$C$357,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$358,$A5,'Full Detail'!$C$2:$C$358,"Deferred")</f>
         <v/>
       </c>
       <c r="E5" s="5">
@@ -666,15 +666,15 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A6,'Full Detail'!$C$2:$C$357,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$358,$A6,'Full Detail'!$C$2:$C$358,"Done")</f>
         <v/>
       </c>
       <c r="C6" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A6,'Full Detail'!$C$2:$C$357,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$358,$A6,'Full Detail'!$C$2:$C$358,"Remaining")</f>
         <v/>
       </c>
       <c r="D6" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A6,'Full Detail'!$C$2:$C$357,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$358,$A6,'Full Detail'!$C$2:$C$358,"Deferred")</f>
         <v/>
       </c>
       <c r="E6" s="5">
@@ -693,15 +693,15 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A7,'Full Detail'!$C$2:$C$357,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$358,$A7,'Full Detail'!$C$2:$C$358,"Done")</f>
         <v/>
       </c>
       <c r="C7" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A7,'Full Detail'!$C$2:$C$357,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$358,$A7,'Full Detail'!$C$2:$C$358,"Remaining")</f>
         <v/>
       </c>
       <c r="D7" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A7,'Full Detail'!$C$2:$C$357,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$358,$A7,'Full Detail'!$C$2:$C$358,"Deferred")</f>
         <v/>
       </c>
       <c r="E7" s="5">
@@ -720,15 +720,15 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A8,'Full Detail'!$C$2:$C$357,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$358,$A8,'Full Detail'!$C$2:$C$358,"Done")</f>
         <v/>
       </c>
       <c r="C8" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A8,'Full Detail'!$C$2:$C$357,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$358,$A8,'Full Detail'!$C$2:$C$358,"Remaining")</f>
         <v/>
       </c>
       <c r="D8" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A8,'Full Detail'!$C$2:$C$357,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$358,$A8,'Full Detail'!$C$2:$C$358,"Deferred")</f>
         <v/>
       </c>
       <c r="E8" s="5">
@@ -747,15 +747,15 @@
         </is>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A9,'Full Detail'!$C$2:$C$357,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$358,$A9,'Full Detail'!$C$2:$C$358,"Done")</f>
         <v/>
       </c>
       <c r="C9" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A9,'Full Detail'!$C$2:$C$357,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$358,$A9,'Full Detail'!$C$2:$C$358,"Remaining")</f>
         <v/>
       </c>
       <c r="D9" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A9,'Full Detail'!$C$2:$C$357,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$358,$A9,'Full Detail'!$C$2:$C$358,"Deferred")</f>
         <v/>
       </c>
       <c r="E9" s="5">
@@ -774,15 +774,15 @@
         </is>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A10,'Full Detail'!$C$2:$C$357,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$358,$A10,'Full Detail'!$C$2:$C$358,"Done")</f>
         <v/>
       </c>
       <c r="C10" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A10,'Full Detail'!$C$2:$C$357,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$358,$A10,'Full Detail'!$C$2:$C$358,"Remaining")</f>
         <v/>
       </c>
       <c r="D10" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A10,'Full Detail'!$C$2:$C$357,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$358,$A10,'Full Detail'!$C$2:$C$358,"Deferred")</f>
         <v/>
       </c>
       <c r="E10" s="5">
@@ -801,15 +801,15 @@
         </is>
       </c>
       <c r="B11" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A11,'Full Detail'!$C$2:$C$357,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$358,$A11,'Full Detail'!$C$2:$C$358,"Done")</f>
         <v/>
       </c>
       <c r="C11" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A11,'Full Detail'!$C$2:$C$357,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$358,$A11,'Full Detail'!$C$2:$C$358,"Remaining")</f>
         <v/>
       </c>
       <c r="D11" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A11,'Full Detail'!$C$2:$C$357,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$358,$A11,'Full Detail'!$C$2:$C$358,"Deferred")</f>
         <v/>
       </c>
       <c r="E11" s="5">
@@ -828,15 +828,15 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A12,'Full Detail'!$C$2:$C$357,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$358,$A12,'Full Detail'!$C$2:$C$358,"Done")</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A12,'Full Detail'!$C$2:$C$357,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$358,$A12,'Full Detail'!$C$2:$C$358,"Remaining")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A12,'Full Detail'!$C$2:$C$357,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$358,$A12,'Full Detail'!$C$2:$C$358,"Deferred")</f>
         <v/>
       </c>
       <c r="E12" s="5">
@@ -855,15 +855,15 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A13,'Full Detail'!$C$2:$C$357,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$358,$A13,'Full Detail'!$C$2:$C$358,"Done")</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A13,'Full Detail'!$C$2:$C$357,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$358,$A13,'Full Detail'!$C$2:$C$358,"Remaining")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A13,'Full Detail'!$C$2:$C$357,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$358,$A13,'Full Detail'!$C$2:$C$358,"Deferred")</f>
         <v/>
       </c>
       <c r="E13" s="5">
@@ -882,15 +882,15 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A14,'Full Detail'!$C$2:$C$357,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$358,$A14,'Full Detail'!$C$2:$C$358,"Done")</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A14,'Full Detail'!$C$2:$C$357,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$358,$A14,'Full Detail'!$C$2:$C$358,"Remaining")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A14,'Full Detail'!$C$2:$C$357,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$358,$A14,'Full Detail'!$C$2:$C$358,"Deferred")</f>
         <v/>
       </c>
       <c r="E14" s="5">
@@ -909,15 +909,15 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A15,'Full Detail'!$C$2:$C$357,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$358,$A15,'Full Detail'!$C$2:$C$358,"Done")</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A15,'Full Detail'!$C$2:$C$357,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$358,$A15,'Full Detail'!$C$2:$C$358,"Remaining")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A15,'Full Detail'!$C$2:$C$357,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$358,$A15,'Full Detail'!$C$2:$C$358,"Deferred")</f>
         <v/>
       </c>
       <c r="E15" s="5">
@@ -936,15 +936,15 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A16,'Full Detail'!$C$2:$C$357,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$358,$A16,'Full Detail'!$C$2:$C$358,"Done")</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A16,'Full Detail'!$C$2:$C$357,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$358,$A16,'Full Detail'!$C$2:$C$358,"Remaining")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A16,'Full Detail'!$C$2:$C$357,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$358,$A16,'Full Detail'!$C$2:$C$358,"Deferred")</f>
         <v/>
       </c>
       <c r="E16" s="5">
@@ -963,15 +963,15 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A17,'Full Detail'!$C$2:$C$357,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$358,$A17,'Full Detail'!$C$2:$C$358,"Done")</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A17,'Full Detail'!$C$2:$C$357,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$358,$A17,'Full Detail'!$C$2:$C$358,"Remaining")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A17,'Full Detail'!$C$2:$C$357,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$358,$A17,'Full Detail'!$C$2:$C$358,"Deferred")</f>
         <v/>
       </c>
       <c r="E17" s="5">
@@ -990,15 +990,15 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A18,'Full Detail'!$C$2:$C$357,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$358,$A18,'Full Detail'!$C$2:$C$358,"Done")</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A18,'Full Detail'!$C$2:$C$357,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$358,$A18,'Full Detail'!$C$2:$C$358,"Remaining")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A18,'Full Detail'!$C$2:$C$357,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$358,$A18,'Full Detail'!$C$2:$C$358,"Deferred")</f>
         <v/>
       </c>
       <c r="E18" s="5">
@@ -1017,15 +1017,15 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A19,'Full Detail'!$C$2:$C$357,"Done")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$358,$A19,'Full Detail'!$C$2:$C$358,"Done")</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A19,'Full Detail'!$C$2:$C$357,"Remaining")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$358,$A19,'Full Detail'!$C$2:$C$358,"Remaining")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('Full Detail'!$E$2:$E$357,$A19,'Full Detail'!$C$2:$C$357,"Deferred")</f>
+        <f>COUNTIFS('Full Detail'!$E$2:$E$358,$A19,'Full Detail'!$C$2:$C$358,"Deferred")</f>
         <v/>
       </c>
       <c r="E19" s="5">
@@ -1075,7 +1075,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E357"/>
+  <dimension ref="A1:E358"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -6942,17 +6942,17 @@
       <c r="A265" s="4" t="n"/>
       <c r="B265" s="4" t="inlineStr">
         <is>
-          <t>Test the new review end to end on a deploy preview</t>
-        </is>
-      </c>
-      <c r="C265" s="16" t="inlineStr">
-        <is>
-          <t>Remaining</t>
+          <t>ChatGPT couldn't see any TonyWeb tools (fixed 2026-10-17)</t>
+        </is>
+      </c>
+      <c r="C265" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D265" s="4" t="inlineStr">
         <is>
-          <t>(needs a yes, it opens a real pull request): one throwaway change from Claude.ai or ChatGPT: start (unclear request, so the confirm step shows), confirm, edit, review card, screenshots, upload link, then discard.</t>
+          <t>one tool's settings listed the same field twice; Claude ignored it, ChatGPT drops every tool when it sees that. Fixed the same way ramprate-ui did on 2026-10-08, plus a test that checks every tool for every role, and the test suite now runs on every pull request (like ramprate-ui). Also fixed a type error from the 2026-10-16 "bug fix" commit that would have failed the Netlify build. Checked: test fails on the old code and passes now, full suite (3,385), typecheck, lint, build, and a fresh pnpm start returning all 38 tools. Left: deploy, then refresh the app in ChatGPT (Settings, Apps and Connectors, TonyWeb, Refresh) and try in a new chat.</t>
         </is>
       </c>
       <c r="E265" s="14" t="inlineStr">
@@ -6965,63 +6965,63 @@
       <c r="A266" s="4" t="n"/>
       <c r="B266" s="4" t="inlineStr">
         <is>
+          <t>Test the new review end to end on a deploy preview</t>
+        </is>
+      </c>
+      <c r="C266" s="16" t="inlineStr">
+        <is>
+          <t>Remaining</t>
+        </is>
+      </c>
+      <c r="D266" s="4" t="inlineStr">
+        <is>
+          <t>(needs a yes, it opens a real pull request): one throwaway change from Claude.ai or ChatGPT: start (unclear request, so the confirm step shows), confirm, edit, review card, screenshots, upload link, then discard.</t>
+        </is>
+      </c>
+      <c r="E266" s="14" t="inlineStr">
+        <is>
+          <t>Phase 11 — Code MCP Server — REBUILT (2026-09-29)</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="4" t="n"/>
+      <c r="B267" s="4" t="inlineStr">
+        <is>
           <t>Email, PDF reports and ClickUp ported from ramprate-ui (2026-10-16, owner said yes, including the one new dependency @react-pdf/renderer ^4.9.0)</t>
         </is>
       </c>
-      <c r="C266" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D266" s="4" t="inlineStr">
+      <c r="C267" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D267" s="4" t="inlineStr">
         <is>
           <t>send_email, create_report (Tony Greenberg PDF emailed as an attachment), create_clickup_task, update_clickup_task, delete_clickup_task. Email reuses src/lib/email.ts (extended, site forms unchanged). Sending email and deleting tasks need the write role, creating/updating tasks edit; all five are rules-gated. New files clickup-client.ts, report-pdf.tsx. Checked: full test suite with 90%+ per file (new files 100%; the PDF test renders a real PDF and reads its text), typecheck, lint, build. Not exercised against real Resend or ClickUp (it would send a real email / make a real task). Needs CLICKUP_API_TOKEN set in Netlify; until then the ClickUp tools say ClickUp isn't set up. check_deploy was ported the same day. Not ported: get_attachment / create_download (chat-page-only; ramprate's own MCP server leaves them out), Slack, Prettier (reasons in docs/ai/project_mcp_server.md).</t>
         </is>
       </c>
-      <c r="E266" s="14" t="inlineStr">
+      <c r="E267" s="14" t="inlineStr">
         <is>
           <t>Phase 11 — Code MCP Server — REBUILT (2026-09-29)</t>
         </is>
       </c>
     </row>
-    <row r="267">
-      <c r="A267" s="10" t="inlineStr">
+    <row r="268">
+      <c r="A268" s="10" t="inlineStr">
         <is>
           <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
         </is>
       </c>
-      <c r="B267" s="11" t="n"/>
-      <c r="C267" s="11" t="n"/>
-      <c r="D267" s="12" t="n"/>
-    </row>
-    <row r="268">
-      <c r="A268" s="4" t="n"/>
-      <c r="B268" s="4" t="inlineStr">
-        <is>
-          <t>Per-page generateMetadata (title, description, OG, Twitter Card, canonical) for every ported route, sourced from Sanity seo object where con…</t>
-        </is>
-      </c>
-      <c r="C268" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D268" s="4" t="inlineStr">
-        <is>
-          <t>tent is CMS-backed, static otherwise. Audited all 140 page.tsx files: only /studio has none (correct — it's robots.txt-disallowed, not public content). Real gap found and fixed: /blog/category/[slug] had no alternates.canonical at all, and no page-aware title for its own real pagination (?page=N) — every paginated page was serving an identical title with no canonical, a real duplicate-content signal. Fixed: generateMetadata now reads searchParams too, self-canonicals each page (?page=N pages canonical to themselves, not consolidated to page 1 — genuinely different posts per page, matching Google's current pagination guidance) and appends "— Page N" to the title past page 1. Verified live: page 1 canonicals to the bare URL, ?page=2 canonicals to ?page=2 with a distinct title.</t>
-        </is>
-      </c>
-      <c r="E268" s="14" t="inlineStr">
-        <is>
-          <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
-        </is>
-      </c>
+      <c r="B268" s="11" t="n"/>
+      <c r="C268" s="11" t="n"/>
+      <c r="D268" s="12" t="n"/>
     </row>
     <row r="269">
       <c r="A269" s="4" t="n"/>
       <c r="B269" s="4" t="inlineStr">
         <is>
-          <t>sitemap.ts generated from real Sanity content + static route list, auto-updates on publish</t>
+          <t>Per-page generateMetadata (title, description, OG, Twitter Card, canonical) for every ported route, sourced from Sanity seo object where con…</t>
         </is>
       </c>
       <c r="C269" s="13" t="inlineStr">
@@ -7031,7 +7031,7 @@
       </c>
       <c r="D269" s="4" t="inlineStr">
         <is>
-          <t>Extended from the Phase 5-era version (homepage + blog posts only, 122 URLs) to every real route: the full static route list (130 routes, generated from find src/app -name page.tsx, excluding /studio (robots.txt-disallowed), /(auth)/login (noindex via its own metadata), and /life-assessment (a pure redirect, not distinct content)) plus all 5 real dynamic sources — blog categories (allCategorySlugsQuery), BrewSoul cities (25), BrewSoul coffees (107), and charity-scorecard entries (103) — each pulled from the exact same data source its own page's generateStaticParams already uses, not re-derived. Auto-updates on publish for anything Sanity-backed (blog posts/categories) since it's a live client.fetch on every build; the static route list itself needs a one-line addition whenever a new page ships (same as any other route-registration step). Verified live: 496 real &lt;loc&gt; entries, spot-checked a coffee/city/charity/category URL each, typecheck/lint clean.</t>
+          <t>tent is CMS-backed, static otherwise. Audited all 140 page.tsx files: only /studio has none (correct — it's robots.txt-disallowed, not public content). Real gap found and fixed: /blog/category/[slug] had no alternates.canonical at all, and no page-aware title for its own real pagination (?page=N) — every paginated page was serving an identical title with no canonical, a real duplicate-content signal. Fixed: generateMetadata now reads searchParams too, self-canonicals each page (?page=N pages canonical to themselves, not consolidated to page 1 — genuinely different posts per page, matching Google's current pagination guidance) and appends "— Page N" to the title past page 1. Verified live: page 1 canonicals to the bare URL, ?page=2 canonicals to ?page=2 with a distinct title.</t>
         </is>
       </c>
       <c r="E269" s="14" t="inlineStr">
@@ -7044,7 +7044,7 @@
       <c r="A270" s="4" t="n"/>
       <c r="B270" s="4" t="inlineStr">
         <is>
-          <t>llms.txt</t>
+          <t>sitemap.ts generated from real Sanity content + static route list, auto-updates on publish</t>
         </is>
       </c>
       <c r="C270" s="13" t="inlineStr">
@@ -7054,7 +7054,7 @@
       </c>
       <c r="D270" s="4" t="inlineStr">
         <is>
-          <t>fetched verbatim from the still-live site and saved to web/public/llms.txt (real content: Tony's bio, expertise, full article index by category, every product/tool section) — do this before Manus goes away, it won't be recoverable after</t>
+          <t>Extended from the Phase 5-era version (homepage + blog posts only, 122 URLs) to every real route: the full static route list (130 routes, generated from find src/app -name page.tsx, excluding /studio (robots.txt-disallowed), /(auth)/login (noindex via its own metadata), and /life-assessment (a pure redirect, not distinct content)) plus all 5 real dynamic sources — blog categories (allCategorySlugsQuery), BrewSoul cities (25), BrewSoul coffees (107), and charity-scorecard entries (103) — each pulled from the exact same data source its own page's generateStaticParams already uses, not re-derived. Auto-updates on publish for anything Sanity-backed (blog posts/categories) since it's a live client.fetch on every build; the static route list itself needs a one-line addition whenever a new page ships (same as any other route-registration step). Verified live: 496 real &lt;loc&gt; entries, spot-checked a coffee/city/charity/category URL each, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E270" s="14" t="inlineStr">
@@ -7067,7 +7067,7 @@
       <c r="A271" s="4" t="n"/>
       <c r="B271" s="4" t="inlineStr">
         <is>
-          <t>robots.txt</t>
+          <t>llms.txt</t>
         </is>
       </c>
       <c r="C271" s="13" t="inlineStr">
@@ -7077,7 +7077,7 @@
       </c>
       <c r="D271" s="4" t="inlineStr">
         <is>
-          <t>same approach: fetched the real live file (not my earlier guessed robots.ts, which has been removed) and saved verbatim to web/public/robots.txt, plus added Disallow: /studio for the new Sanity Studio route. Confirmed live: real AI-crawler allowlist (GPTBot, Claude-Web, PerplexityBot, etc.), scraper blocklist, and the site's non-standard LLMs: directive all intact</t>
+          <t>fetched verbatim from the still-live site and saved to web/public/llms.txt (real content: Tony's bio, expertise, full article index by category, every product/tool section) — do this before Manus goes away, it won't be recoverable after</t>
         </is>
       </c>
       <c r="E271" s="14" t="inlineStr">
@@ -7090,7 +7090,7 @@
       <c r="A272" s="4" t="n"/>
       <c r="B272" s="4" t="inlineStr">
         <is>
-          <t>JSON-LD</t>
+          <t>robots.txt</t>
         </is>
       </c>
       <c r="C272" s="13" t="inlineStr">
@@ -7100,7 +7100,7 @@
       </c>
       <c r="D272" s="4" t="inlineStr">
         <is>
-          <t>WebSite + Person schema ported verbatim from the live homepage's actual &lt;script type="application/ld+json"&gt; tags (not reconstructed from memory) — rendered site-wide from src/lib/structured-data.ts in the root layout. The Person image was hardcoded to a /api/img/... legacy proxy path on the live site — rescued that headshot (downloaded it while still live, uploaded to Sanity as the author-tony-greenberg document's avatar) so the new site's JSON-LD has zero Manus dependency instead of just copying the fragile path forward</t>
+          <t>same approach: fetched the real live file (not my earlier guessed robots.ts, which has been removed) and saved verbatim to web/public/robots.txt, plus added Disallow: /studio for the new Sanity Studio route. Confirmed live: real AI-crawler allowlist (GPTBot, Claude-Web, PerplexityBot, etc.), scraper blocklist, and the site's non-standard LLMs: directive all intact</t>
         </is>
       </c>
       <c r="E272" s="14" t="inlineStr">
@@ -7113,7 +7113,7 @@
       <c r="A273" s="4" t="n"/>
       <c r="B273" s="4" t="inlineStr">
         <is>
-          <t>Article JSON-LD on /blog/[slug], built from real per-post Sanity data (headline, image, datePublished/dateModified, author, canonical URL)</t>
+          <t>JSON-LD</t>
         </is>
       </c>
       <c r="C273" s="13" t="inlineStr">
@@ -7123,7 +7123,7 @@
       </c>
       <c r="D273" s="4" t="inlineStr">
         <is>
-          <t>verified live on a real post</t>
+          <t>WebSite + Person schema ported verbatim from the live homepage's actual &lt;script type="application/ld+json"&gt; tags (not reconstructed from memory) — rendered site-wide from src/lib/structured-data.ts in the root layout. The Person image was hardcoded to a /api/img/... legacy proxy path on the live site — rescued that headshot (downloaded it while still live, uploaded to Sanity as the author-tony-greenberg document's avatar) so the new site's JSON-LD has zero Manus dependency instead of just copying the fragile path forward</t>
         </is>
       </c>
       <c r="E273" s="14" t="inlineStr">
@@ -7136,7 +7136,7 @@
       <c r="A274" s="4" t="n"/>
       <c r="B274" s="4" t="inlineStr">
         <is>
-          <t>Build the full Manus/legacy-URL → Next.js-URL 301 redirect map (next.config.ts redirects() or Sanity redirect documents)</t>
+          <t>Article JSON-LD on /blog/[slug], built from real per-post Sanity data (headline, image, datePublished/dateModified, author, canonical URL)</t>
         </is>
       </c>
       <c r="C274" s="13" t="inlineStr">
@@ -7146,7 +7146,7 @@
       </c>
       <c r="D274" s="4" t="inlineStr">
         <is>
-          <t>hard QA gate, nothing proceeds to DNS cutover until this is complete and tested. First real pass done: extracted all 197 real path= routes from legacy's App.tsx router (not guessed — the actual route table), diffed against this app's real current routes (find src/app -maxdepth 1 -name page.tsx) + next.config.ts's existing redirect sources, normalizing :param/[param] syntax to compare like-for-like. Started at 41 real gaps, closed 10 with new redirects: /attention-theft/{blocker-finder,legal,report,weapons} (legacy registered both a bare AND a /attention-theft/-nested path for each, only the bare ones had redirects before), /find-my-car → /find-my, /the-index → /search (matching the fix already applied to other pages' dead links to it), /supplier-intake-long (bare) + /vendor-intake + /vendor-intake-long (+/:token) → the same real ramprate.com/biochain/supplier-intake destination the token'd path already redirected to, and /spamtoast + /youve-been-reported → / (the live half of legacy's "report a spammer" confrontation flow — a fake IP-fingerprinting/countdown-timer page; the other half, ReportSpammer.tsx, was already a documented drop in Phase 4, this is the same call for its sequel). 21 of the remaining 31 gaps need no redirect — they're /admin/*//analytics//edit/frqncy (internal tools never meant for public discovery) or already-documented intentional defers from Phase 4/7/10 (/clock-keeper-part-2, /ecosystem-map, /friend-gate, /friend-survey/:token, /medicine-sequencing, /m</t>
+          <t>verified live on a real post</t>
         </is>
       </c>
       <c r="E274" s="14" t="inlineStr">
@@ -7159,7 +7159,7 @@
       <c r="A275" s="4" t="n"/>
       <c r="B275" s="4" t="inlineStr">
         <is>
-          <t>/path/:archetype (src/app/path/[archetype]/page.tsx)</t>
+          <t>Build the full Manus/legacy-URL → Next.js-URL 301 redirect map (next.config.ts redirects() or Sanity redirect documents)</t>
         </is>
       </c>
       <c r="C275" s="13" t="inlineStr">
@@ -7169,7 +7169,7 @@
       </c>
       <c r="D275" s="4" t="inlineStr">
         <is>
-          <t>per-archetype landing page for /assessment's Builder/Crusader/Investor result, reusing lib/content/archetypes.ts. Real content ported in full (top-5 essential-reading list per archetype via allPostsForArchiveQuery, real PathSubscribeForm posting to /api/subscribe, AUTHORITY_ITEMS strip). Real bug fixed vs. legacy: replaced a hand-rolled inline-styled "Path not found" div with a real notFound() (this route's generateStaticParams only ever produces the 3 real keys). Verified live: all 3 archetype routes 200 OK, typecheck/lint clean.</t>
+          <t>hard QA gate, nothing proceeds to DNS cutover until this is complete and tested. First real pass done: extracted all 197 real path= routes from legacy's App.tsx router (not guessed — the actual route table), diffed against this app's real current routes (find src/app -maxdepth 1 -name page.tsx) + next.config.ts's existing redirect sources, normalizing :param/[param] syntax to compare like-for-like. Started at 41 real gaps, closed 10 with new redirects: /attention-theft/{blocker-finder,legal,report,weapons} (legacy registered both a bare AND a /attention-theft/-nested path for each, only the bare ones had redirects before), /find-my-car → /find-my, /the-index → /search (matching the fix already applied to other pages' dead links to it), /supplier-intake-long (bare) + /vendor-intake + /vendor-intake-long (+/:token) → the same real ramprate.com/biochain/supplier-intake destination the token'd path already redirected to, and /spamtoast + /youve-been-reported → / (the live half of legacy's "report a spammer" confrontation flow — a fake IP-fingerprinting/countdown-timer page; the other half, ReportSpammer.tsx, was already a documented drop in Phase 4, this is the same call for its sequel). 21 of the remaining 31 gaps need no redirect — they're /admin/*//analytics//edit/frqncy (internal tools never meant for public discovery) or already-documented intentional defers from Phase 4/7/10 (/clock-keeper-part-2, /ecosystem-map, /friend-gate, /friend-survey/:token, /medicine-sequencing, /m</t>
         </is>
       </c>
       <c r="E275" s="14" t="inlineStr">
@@ -7182,7 +7182,7 @@
       <c r="A276" s="4" t="n"/>
       <c r="B276" s="4" t="inlineStr">
         <is>
-          <t>/my-journey (src/app/my-journey/page.tsx + components/assessments/my-journey-dashboard.tsx)</t>
+          <t>/path/:archetype (src/app/path/[archetype]/page.tsx)</t>
         </is>
       </c>
       <c r="C276" s="13" t="inlineStr">
@@ -7192,7 +7192,7 @@
       </c>
       <c r="D276" s="4" t="inlineStr">
         <is>
-          <t>"My Journey Dashboard," real grid/timeline views across all 28 JOURNEY_MAP experiences, category/status filters, phase progress ring, recommended-next card, using the same real useJourneyProgress/JOURNEY_MAP completion tracking every "Find Your X" quiz already writes to (not the narrower tg_assessment_results cookie built for /self-portrait). Legacy's per-quiz scored-result caching (RESULT_KEYS, feeding a mini radar chart) was not ported — no quiz in this migration writes that data either, same honest-degradation call already made for /self-portrait's own composite radar. Fixed a real legacy dead link (/ecosystem-map, a still-unbuilt page) to /self-portrait. Verified live: 200 OK, real content confirmed, typecheck/lint clean.</t>
+          <t>per-archetype landing page for /assessment's Builder/Crusader/Investor result, reusing lib/content/archetypes.ts. Real content ported in full (top-5 essential-reading list per archetype via allPostsForArchiveQuery, real PathSubscribeForm posting to /api/subscribe, AUTHORITY_ITEMS strip). Real bug fixed vs. legacy: replaced a hand-rolled inline-styled "Path not found" div with a real notFound() (this route's generateStaticParams only ever produces the 3 real keys). Verified live: all 3 archetype routes 200 OK, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E276" s="14" t="inlineStr">
@@ -7205,7 +7205,7 @@
       <c r="A277" s="4" t="n"/>
       <c r="B277" s="4" t="inlineStr">
         <is>
-          <t>/the-open-door (src/app/the-open-door/page.tsx)</t>
+          <t>/my-journey (src/app/my-journey/page.tsx + components/assessments/my-journey-dashboard.tsx)</t>
         </is>
       </c>
       <c r="C277" s="13" t="inlineStr">
@@ -7215,7 +7215,7 @@
       </c>
       <c r="D277" s="4" t="inlineStr">
         <is>
-          <t>real press/credibility content: all 10 "Magic Genie" client-pitch prompts (real named targets — Marco Argenti/Goldman Sachs, Adam Smith/Disney, etc.), 18 real client testimonials, all 8 explicitly-labeled satirical "parody" quotes (kept with disclaimers, not presented as real). Real overlap found and reconciled: this page's publications/speaking/podcasts arrays substantially duplicate the already-shipped /published's fuller bibliography — kept only what /published doesn't cover (Forbes + Business Insider bylines, the Clinton Global Initiative keynote, 4 of 5 podcast appearances) and cross-linked to /published for the rest, same reconciliation pattern as /assessments vs /find-my. Real bugs fixed: 3 genie/keynote links pointed externally at tonygreenberg.com/&lt;slug&gt; for posts that are real internal posts in this migration — relinked to /blog/psychedelics-could-become-extractive-capitalism, /blog/boiling-the-human-summit-harvard-kurzweil, /blog/return-on-investment-going-green-going-green-2 (all verified 200); a bare self-link to tonygreenberg.com remapped to /. Ships as a pure Server Component (legacy's FadeIn/Section/editorial-component dependencies don't exist here and weren't needed). Verified live: 200 OK, real content in raw SSR HTML, typecheck/lint clean.</t>
+          <t>"My Journey Dashboard," real grid/timeline views across all 28 JOURNEY_MAP experiences, category/status filters, phase progress ring, recommended-next card, using the same real useJourneyProgress/JOURNEY_MAP completion tracking every "Find Your X" quiz already writes to (not the narrower tg_assessment_results cookie built for /self-portrait). Legacy's per-quiz scored-result caching (RESULT_KEYS, feeding a mini radar chart) was not ported — no quiz in this migration writes that data either, same honest-degradation call already made for /self-portrait's own composite radar. Fixed a real legacy dead link (/ecosystem-map, a still-unbuilt page) to /self-portrait. Verified live: 200 OK, real content confirmed, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E277" s="14" t="inlineStr">
@@ -7228,7 +7228,7 @@
       <c r="A278" s="4" t="n"/>
       <c r="B278" s="4" t="inlineStr">
         <is>
-          <t>Homepage "Recent Updates" band (2026-09-29)</t>
+          <t>/the-open-door (src/app/the-open-door/page.tsx)</t>
         </is>
       </c>
       <c r="C278" s="13" t="inlineStr">
@@ -7238,7 +7238,7 @@
       </c>
       <c r="D278" s="4" t="inlineStr">
         <is>
-          <t>on the live site (a newer Blog.tsx than _legacy-manus-app/, so rebuilt from the live page's markup), replacing the older "Latest Thinking" pair. Found while doing it: two live essays are missing from Sanity, the-tollbooth-and-the-alternative (Aug 18, 2026, the live site's newest) and what-quest-could-fix. Both were published on live after the legacy snapshot and need importing.</t>
+          <t>real press/credibility content: all 10 "Magic Genie" client-pitch prompts (real named targets — Marco Argenti/Goldman Sachs, Adam Smith/Disney, etc.), 18 real client testimonials, all 8 explicitly-labeled satirical "parody" quotes (kept with disclaimers, not presented as real). Real overlap found and reconciled: this page's publications/speaking/podcasts arrays substantially duplicate the already-shipped /published's fuller bibliography — kept only what /published doesn't cover (Forbes + Business Insider bylines, the Clinton Global Initiative keynote, 4 of 5 podcast appearances) and cross-linked to /published for the rest, same reconciliation pattern as /assessments vs /find-my. Real bugs fixed: 3 genie/keynote links pointed externally at tonygreenberg.com/&lt;slug&gt; for posts that are real internal posts in this migration — relinked to /blog/psychedelics-could-become-extractive-capitalism, /blog/boiling-the-human-summit-harvard-kurzweil, /blog/return-on-investment-going-green-going-green-2 (all verified 200); a bare self-link to tonygreenberg.com remapped to /. Ships as a pure Server Component (legacy's FadeIn/Section/editorial-component dependencies don't exist here and weren't needed). Verified live: 200 OK, real content in raw SSR HTML, typecheck/lint clean.</t>
         </is>
       </c>
       <c r="E278" s="14" t="inlineStr">
@@ -7251,7 +7251,7 @@
       <c r="A279" s="4" t="n"/>
       <c r="B279" s="4" t="inlineStr">
         <is>
-          <t>Re-sync the legacy reference</t>
+          <t>Homepage "Recent Updates" band (2026-09-29)</t>
         </is>
       </c>
       <c r="C279" s="13" t="inlineStr">
@@ -7261,7 +7261,7 @@
       </c>
       <c r="D279" s="4" t="inlineStr">
         <is>
-          <t>_legacy-manus-app/ is older than what's live (Recent Updates proves it), so visual diffs should be against the live site, not only that folder. Closed 2026-10-08: done the way this item suggests: every comparison since 2026-10-01 is against the live site itself (163 pages + 121 posts on 2026-10-01, 188 pages on 2026-10-07, 18 redesigned pages on 2026-10-08), with _legacy-manus-app/ used only as the code reference.</t>
+          <t>on the live site (a newer Blog.tsx than _legacy-manus-app/, so rebuilt from the live page's markup), replacing the older "Latest Thinking" pair. Found while doing it: two live essays are missing from Sanity, the-tollbooth-and-the-alternative (Aug 18, 2026, the live site's newest) and what-quest-could-fix. Both were published on live after the legacy snapshot and need importing.</t>
         </is>
       </c>
       <c r="E279" s="14" t="inlineStr">
@@ -7274,7 +7274,7 @@
       <c r="A280" s="4" t="n"/>
       <c r="B280" s="4" t="inlineStr">
         <is>
-          <t>Visual diff pass: every ported page vs</t>
+          <t>Re-sync the legacy reference</t>
         </is>
       </c>
       <c r="C280" s="13" t="inlineStr">
@@ -7284,7 +7284,7 @@
       </c>
       <c r="D280" s="4" t="inlineStr">
         <is>
-          <t>legacy page Closed 2026-10-08: covered by the live-site sweeps above (screenshots and measured title/label/spacing per page, see the 2026-10-01, 10-02, 10-07 and 10-08 entries in this phase). Remaining differences are listed as decisions (Cormorant titles, /find-my header) or deliberate (CONTRIBUTING rule 20).</t>
+          <t>_legacy-manus-app/ is older than what's live (Recent Updates proves it), so visual diffs should be against the live site, not only that folder. Closed 2026-10-08: done the way this item suggests: every comparison since 2026-10-01 is against the live site itself (163 pages + 121 posts on 2026-10-01, 188 pages on 2026-10-07, 18 redesigned pages on 2026-10-08), with _legacy-manus-app/ used only as the code reference.</t>
         </is>
       </c>
       <c r="E280" s="14" t="inlineStr">
@@ -7297,7 +7297,7 @@
       <c r="A281" s="4" t="n"/>
       <c r="B281" s="4" t="inlineStr">
         <is>
-          <t>Padding / spacing on the story pages matched to live (2026-10-01)</t>
+          <t>Visual diff pass: every ported page vs</t>
         </is>
       </c>
       <c r="C281" s="13" t="inlineStr">
@@ -7307,7 +7307,7 @@
       </c>
       <c r="D281" s="4" t="inlineStr">
         <is>
-          <t>Measured margins, text column and spacing on 31 pages, live vs a production build, at 375px and 1280px. The "door" story pages were the clear mismatch: live's text column is ~546px (ours was 720px), 20px side margins on phones / 40px on desktop, body text 19px/1.8 on phones and 18px/1.85 on desktop (ours 16px/1.5). Fixed on /the-body, /engine-room, /under-nda, /the-nightstand, /the-web, /the-territory, /about, /intel (Intel uses live's 16.8px/1.9; About's hero line 480px max, 18.4px/1.8). Re-measured: all 8 match live to within 2px (About's column 28px narrower), no sideways scroll at 375px.</t>
+          <t>legacy page Closed 2026-10-08: covered by the live-site sweeps above (screenshots and measured title/label/spacing per page, see the 2026-10-01, 10-02, 10-07 and 10-08 entries in this phase). Remaining differences are listed as decisions (Cormorant titles, /find-my header) or deliberate (CONTRIBUTING rule 20).</t>
         </is>
       </c>
       <c r="E281" s="14" t="inlineStr">
@@ -7320,7 +7320,7 @@
       <c r="A282" s="4" t="n"/>
       <c r="B282" s="4" t="inlineStr">
         <is>
-          <t>Header-to-title spacing re-checked (2026-10-02)</t>
+          <t>Padding / spacing on the story pages matched to live (2026-10-01)</t>
         </is>
       </c>
       <c r="C282" s="13" t="inlineStr">
@@ -7330,7 +7330,7 @@
       </c>
       <c r="D282" s="4" t="inlineStr">
         <is>
-          <t>The 2026-10-01 note compared different things: live's header wasn't measured (it showed 0), so "96px vs 168px" was really 161px vs 168px from the top of the page. Measured again from the top of the page, live vs a production build, at 375px and 1280px: most pages were already within 10px. Fixed the real gaps: /the-open-door (now live's dark centered hero band, 56px title, 546px text column; title was 72px too high), /start-here (live's 48px/96px top padding; 25px too high on desktop), /invest and /engage (label spacing and live's 32px/51px title; /invest's desktop title was 36px), /impact-dashboard on phones (card edge to edge under the header like live; title was 89px too low). Re-measured: all within 8px of live, no sideways scroll at 375px, no JS errors.</t>
+          <t>Measured margins, text column and spacing on 31 pages, live vs a production build, at 375px and 1280px. The "door" story pages were the clear mismatch: live's text column is ~546px (ours was 720px), 20px side margins on phones / 40px on desktop, body text 19px/1.8 on phones and 18px/1.85 on desktop (ours 16px/1.5). Fixed on /the-body, /engine-room, /under-nda, /the-nightstand, /the-web, /the-territory, /about, /intel (Intel uses live's 16.8px/1.9; About's hero line 480px max, 18.4px/1.8). Re-measured: all 8 match live to within 2px (About's column 28px narrower), no sideways scroll at 375px.</t>
         </is>
       </c>
       <c r="E282" s="14" t="inlineStr">
@@ -7343,7 +7343,7 @@
       <c r="A283" s="4" t="n"/>
       <c r="B283" s="4" t="inlineStr">
         <is>
-          <t>HumanOS headings in capitals like live (2026-10-02, owner said yes)</t>
+          <t>Header-to-title spacing re-checked (2026-10-02)</t>
         </is>
       </c>
       <c r="C283" s="13" t="inlineStr">
@@ -7353,7 +7353,7 @@
       </c>
       <c r="D283" s="4" t="inlineStr">
         <is>
-          <t>the 4 headings live capitalises on /humanos (title, "Are you a Maximizer...", "Take the Diagnostic", "The Diagnostic") get uppercase; the words are unchanged. The subpages already matched.</t>
+          <t>The 2026-10-01 note compared different things: live's header wasn't measured (it showed 0), so "96px vs 168px" was really 161px vs 168px from the top of the page. Measured again from the top of the page, live vs a production build, at 375px and 1280px: most pages were already within 10px. Fixed the real gaps: /the-open-door (now live's dark centered hero band, 56px title, 546px text column; title was 72px too high), /start-here (live's 48px/96px top padding; 25px too high on desktop), /invest and /engage (label spacing and live's 32px/51px title; /invest's desktop title was 36px), /impact-dashboard on phones (card edge to edge under the header like live; title was 89px too low). Re-measured: all within 8px of live, no sideways scroll at 375px, no JS errors.</t>
         </is>
       </c>
       <c r="E283" s="14" t="inlineStr">
@@ -7366,7 +7366,7 @@
       <c r="A284" s="4" t="n"/>
       <c r="B284" s="4" t="inlineStr">
         <is>
-          <t>More layout gaps matched to live (2026-10-02)</t>
+          <t>HumanOS headings in capitals like live (2026-10-02, owner said yes)</t>
         </is>
       </c>
       <c r="C284" s="13" t="inlineStr">
@@ -7376,7 +7376,7 @@
       </c>
       <c r="D284" s="4" t="inlineStr">
         <is>
-          <t>/series (live's centered 546px column, and a bug fixed: every card kept an empty 240px picture column, squeezing the text; live's per-series picture is one generic placeholder on the Manus proxy, so not copied), /humanos (middle section 900px like live), homepage desktop widths (hero text 804px, Four Doors 1000px, Editor's Picks 1168px, GemSpark edge, section title sizes; live's /blog now shows the homepage), /find-my (photo undimmed and plain background, like live; our site header kept). Re-measured: headings within 3px (/series) to 20px (homepage) of live, no sideways scroll, no JS errors. Note: live's "New here?" tour bar sits over its header and doesn't move the page, so it doesn't affect these numbers.</t>
+          <t>the 4 headings live capitalises on /humanos (title, "Are you a Maximizer...", "Take the Diagnostic", "The Diagnostic") get uppercase; the words are unchanged. The subpages already matched.</t>
         </is>
       </c>
       <c r="E284" s="14" t="inlineStr">
@@ -7389,7 +7389,7 @@
       <c r="A285" s="4" t="n"/>
       <c r="B285" s="4" t="inlineStr">
         <is>
-          <t>Full sweep vs live (2026-10-02)</t>
+          <t>More layout gaps matched to live (2026-10-02)</t>
         </is>
       </c>
       <c r="C285" s="13" t="inlineStr">
@@ -7399,7 +7399,7 @@
       </c>
       <c r="D285" s="4" t="inlineStr">
         <is>
-          <t>142 pages (every non-blog page, 3 of each templated set) at 375px and 1280px, title position, text column, title size. Fixed the shared causes: BrewSoul (live wraps most pages in its frame twice, so a second 52px offset plus the category badge; the landing, cities, directory and quiz pages have neither: src/components/brewsoul/brewsoul-main.tsx; intro paragraphs uncapped like live; 38px titles), Kava (live's extra 52px offset), /the-body, /the-nightstand, /the-web (405px top photo like live), the 6 peptide pages (live's 768/896px intro column), /journeys, /pick-up-the-phone, /published, /ecosystem (546px story column and live's text size). Re-measured: 110 of 120 within 40px / 60px of live.</t>
+          <t>/series (live's centered 546px column, and a bug fixed: every card kept an empty 240px picture column, squeezing the text; live's per-series picture is one generic placeholder on the Manus proxy, so not copied), /humanos (middle section 900px like live), homepage desktop widths (hero text 804px, Four Doors 1000px, Editor's Picks 1168px, GemSpark edge, section title sizes; live's /blog now shows the homepage), /find-my (photo undimmed and plain background, like live; our site header kept). Re-measured: headings within 3px (/series) to 20px (homepage) of live, no sideways scroll, no JS errors. Note: live's "New here?" tour bar sits over its header and doesn't move the page, so it doesn't affect these numbers.</t>
         </is>
       </c>
       <c r="E285" s="14" t="inlineStr">
@@ -7412,7 +7412,7 @@
       <c r="A286" s="4" t="n"/>
       <c r="B286" s="4" t="inlineStr">
         <is>
-          <t>Sweep leftovers fixed (2026-10-06)</t>
+          <t>Full sweep vs live (2026-10-02)</t>
         </is>
       </c>
       <c r="C286" s="13" t="inlineStr">
@@ -7422,7 +7422,7 @@
       </c>
       <c r="D286" s="4" t="inlineStr">
         <is>
-          <t>Ported legacy's exact title sizes, margins and column widths. Measured live vs a production build at 375px and 1280px (H1 distance from the top, H1 size, intro and table widths). Now within 8px and the same title size on /published, /brewsoul/first-sip, /brewsoul/home, /brewsoul/chains (intro 912px like live), /brewsoul/browse, /brewsoul/directory (3-column 952px grid like live), /brewsoul and /brewsoul/quiz (intro 520px), /amplifier (546px column), /diamond-cut, /speaking, /living-declaration, /spirits, /protecting-your-business (tables 730px), and the 5 HumanOS subpages (titles smaller like live, 752px column). No sideways scroll at 375px. Left on purpose: /self-portrait (font matches; our page has a different title and no back link, so it sits 23-57px higher), BrewSoul pages 3-6px off (the shared journey bar row), and the different-layout pages /dharma-finder, /grant-study, /search, /quiz_25q, /soulscore. Also: /brewsoul/quiz rebuilt as a step registry (src/components/brewsoul/brewsoul-quiz/: parent + hook/ + components/step-* + data/), same questions, scoring and look; Back/Skip/Retake use lucide icons. New CONTRIBUTING rule 19 (multi-step flows, FydoPartner pattern). brewsoul-welcome-quiz.tsx (/brewsoul) still has the old shape and text arrows.</t>
+          <t>142 pages (every non-blog page, 3 of each templated set) at 375px and 1280px, title position, text column, title size. Fixed the shared causes: BrewSoul (live wraps most pages in its frame twice, so a second 52px offset plus the category badge; the landing, cities, directory and quiz pages have neither: src/components/brewsoul/brewsoul-main.tsx; intro paragraphs uncapped like live; 38px titles), Kava (live's extra 52px offset), /the-body, /the-nightstand, /the-web (405px top photo like live), the 6 peptide pages (live's 768/896px intro column), /journeys, /pick-up-the-phone, /published, /ecosystem (546px story column and live's text size). Re-measured: 110 of 120 within 40px / 60px of live.</t>
         </is>
       </c>
       <c r="E286" s="14" t="inlineStr">
@@ -7435,7 +7435,7 @@
       <c r="A287" s="4" t="n"/>
       <c r="B287" s="4" t="inlineStr">
         <is>
-          <t>Match live's redesigned pages (2026-10-06, owner said go)</t>
+          <t>Sweep leftovers fixed (2026-10-06)</t>
         </is>
       </c>
       <c r="C287" s="13" t="inlineStr">
@@ -7445,7 +7445,7 @@
       </c>
       <c r="D287" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">/self-portrait (live: dark page, progress ring, "N more brushstrokes" lock until 5 assessments), /grant-study and /dharma-finder (live opens straight on question 1, no intro screen), /quiz_25q (live adds a hero picture above the title; rescue it into Sanity first), /search (live: one search box across essays, BrewSoul, peptides, HumanOS, assessments, kava and pages with filter chips). Measure live vs a production build at 375px and 1280px when done. Done 2026-10-06: /grant-study and /dharma-finder open straight on question 1 like live (title block / part header above the first question, live's 546px column, plain page, credit under every question), both rebuilt as step registries (rule 19); measured within 3px of live at the top (dharma's question block within 7px). /quiz_25q's hero rescued into Sanity and placed like live (within 2px). Found and fixed on the way: on the deployed copy /grant-study's answer buttons could not be clicked (the themed page background was fixed z-0, painted over the quiz); ThemedBackground is now -z-10 pointer-events-none (backgrounds unchanged on all 21 pages that use it), and the shared email gate no longer scrolls sideways on phones. Both quizzes clicked through to results in Chrome and Safari. /self-portrait restyled to live (dark page, "The Composite You", progress ring, "N More Brushstrokes Needed" lock until 5 done, live's copy) on our real cookie data; within 3px of live at both widths; tested with 0, 2 and 6 completed. Counts are ours (13 </t>
+          <t>Ported legacy's exact title sizes, margins and column widths. Measured live vs a production build at 375px and 1280px (H1 distance from the top, H1 size, intro and table widths). Now within 8px and the same title size on /published, /brewsoul/first-sip, /brewsoul/home, /brewsoul/chains (intro 912px like live), /brewsoul/browse, /brewsoul/directory (3-column 952px grid like live), /brewsoul and /brewsoul/quiz (intro 520px), /amplifier (546px column), /diamond-cut, /speaking, /living-declaration, /spirits, /protecting-your-business (tables 730px), and the 5 HumanOS subpages (titles smaller like live, 752px column). No sideways scroll at 375px. Left on purpose: /self-portrait (font matches; our page has a different title and no back link, so it sits 23-57px higher), BrewSoul pages 3-6px off (the shared journey bar row), and the different-layout pages /dharma-finder, /grant-study, /search, /quiz_25q, /soulscore. Also: /brewsoul/quiz rebuilt as a step registry (src/components/brewsoul/brewsoul-quiz/: parent + hook/ + components/step-* + data/), same questions, scoring and look; Back/Skip/Retake use lucide icons. New CONTRIBUTING rule 19 (multi-step flows, FydoPartner pattern). brewsoul-welcome-quiz.tsx (/brewsoul) still has the old shape and text arrows.</t>
         </is>
       </c>
       <c r="E287" s="14" t="inlineStr">
@@ -7458,7 +7458,7 @@
       <c r="A288" s="4" t="n"/>
       <c r="B288" s="4" t="inlineStr">
         <is>
-          <t>Still different from live (decided 2026-10-09)</t>
+          <t>Match live's redesigned pages (2026-10-06, owner said go)</t>
         </is>
       </c>
       <c r="C288" s="13" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="D288" s="4" t="inlineStr">
         <is>
-          <t>blog posts (done) (done 2026-10-07, see Phase 5); /find-my on live hides the site header. /walk-through is a 404 on live now. Owner: keep our site menu on /find-my (visitors can still reach the rest of the site); nothing left to change.</t>
+          <t xml:space="preserve">/self-portrait (live: dark page, progress ring, "N more brushstrokes" lock until 5 assessments), /grant-study and /dharma-finder (live opens straight on question 1, no intro screen), /quiz_25q (live adds a hero picture above the title; rescue it into Sanity first), /search (live: one search box across essays, BrewSoul, peptides, HumanOS, assessments, kava and pages with filter chips). Measure live vs a production build at 375px and 1280px when done. Done 2026-10-06: /grant-study and /dharma-finder open straight on question 1 like live (title block / part header above the first question, live's 546px column, plain page, credit under every question), both rebuilt as step registries (rule 19); measured within 3px of live at the top (dharma's question block within 7px). /quiz_25q's hero rescued into Sanity and placed like live (within 2px). Found and fixed on the way: on the deployed copy /grant-study's answer buttons could not be clicked (the themed page background was fixed z-0, painted over the quiz); ThemedBackground is now -z-10 pointer-events-none (backgrounds unchanged on all 21 pages that use it), and the shared email gate no longer scrolls sideways on phones. Both quizzes clicked through to results in Chrome and Safari. /self-portrait restyled to live (dark page, "The Composite You", progress ring, "N More Brushstrokes Needed" lock until 5 done, live's copy) on our real cookie data; within 3px of live at both widths; tested with 0, 2 and 6 completed. Counts are ours (13 </t>
         </is>
       </c>
       <c r="E288" s="14" t="inlineStr">
@@ -7481,7 +7481,7 @@
       <c r="A289" s="4" t="n"/>
       <c r="B289" s="4" t="inlineStr">
         <is>
-          <t>Design change on live (owner: "match live", 2026-10-09)</t>
+          <t>Still different from live (decided 2026-10-09)</t>
         </is>
       </c>
       <c r="C289" s="13" t="inlineStr">
@@ -7491,7 +7491,7 @@
       </c>
       <c r="D289" s="4" t="inlineStr">
         <is>
-          <t>live's story pages now use Cormorant Garamond for titles (ours: Playfair Display), a lighter title weight (400 vs our 700), and a red eyebrow label (#8E1E25, wider letter spacing) instead of our gold. A site-wide font swap is a design call, so not done. Done 2026-10-09: a fresh sweep of 163 live pages found live has since dropped Cormorant from the story pages (only /living-declaration uses it, ours already matched) and mostly uses Playfair; the real differences were fixed: every heading on /attention-theft in Fraunces 700 (section-wide, like Kava), /supplier-intake title in the system serif, and live's fluid title sizes on /about, /articles, /the-letter, /the-philosophy, /clock-keeper-part-2, /living-declaration (measured at 375/640/820/1024/1280, now identical). Label colours stay darker than live on purpose (contrast, rule 20).</t>
+          <t>blog posts (done) (done 2026-10-07, see Phase 5); /find-my on live hides the site header. /walk-through is a 404 on live now. Owner: keep our site menu on /find-my (visitors can still reach the rest of the site); nothing left to change.</t>
         </is>
       </c>
       <c r="E289" s="14" t="inlineStr">
@@ -7504,7 +7504,7 @@
       <c r="A290" s="4" t="n"/>
       <c r="B290" s="4" t="inlineStr">
         <is>
-          <t>Link check across all ported pages (no 404s, no broken internal cross-references)</t>
+          <t>Design change on live (owner: "match live", 2026-10-09)</t>
         </is>
       </c>
       <c r="C290" s="13" t="inlineStr">
@@ -7514,7 +7514,7 @@
       </c>
       <c r="D290" s="4" t="inlineStr">
         <is>
-          <t>First full pass done 2026-09-29 (510 pages crawled from the sitemap plus every internal link, on a production build). Fixed in code: /brewsoul/coffee/…-tarrazú 404 (the route got the id still percent-encoded), 30+ links that went through the /assessments/* redirects, /find-your-me's dead Homeaglow link, the two root-level Iboga essay links, and the dead FauxTony nav item. Fixed as Sanity drafts (scripts/fix-blog-body-links.ts, 14 posts): broken post links, leaked !… placeholder text, Energy Is Money's split author bio, and scraped WordPress furniture ("Share this / Related / You Might Also Like / Copyright", "Show More / Top News", [mc4wp_form]). Left for a decision: /framework's "Ask FauxTony" button, when-healing-becomes-extraction's two links to a Dr. Lee case file that doesn't exist, and the-clock-keeper-chronicles-part-1's link to the deferred /clock-keeper-part-2. Re-run after the drafts are published. 2026-10-01 re-run (local production build, all 498 sitemap URLs load; 440 unique internal links): 5 broken. Fixed as a Sanity draft: molecule-as-mirror-10-what-the-pioneers-know's "Final installment" link pointed at a non-existent part-10 slug (now part 11; live also shows that line twice, kept). Already fixed in a waiting draft: forever-chemicals-... → /blog/psychedelic-readiness-index. Still the 3 known decisions: /fauxtony (from /framework), /clock-keeper-part-2, /blog/the-case-file-dr-samuel-lee. 2026-10-08 re-run (production build, all 497 sitemap pages, 453 unique i</t>
+          <t>live's story pages now use Cormorant Garamond for titles (ours: Playfair Display), a lighter title weight (400 vs our 700), and a red eyebrow label (#8E1E25, wider letter spacing) instead of our gold. A site-wide font swap is a design call, so not done. Done 2026-10-09: a fresh sweep of 163 live pages found live has since dropped Cormorant from the story pages (only /living-declaration uses it, ours already matched) and mostly uses Playfair; the real differences were fixed: every heading on /attention-theft in Fraunces 700 (section-wide, like Kava), /supplier-intake title in the system serif, and live's fluid title sizes on /about, /articles, /the-letter, /the-philosophy, /clock-keeper-part-2, /living-declaration (measured at 375/640/820/1024/1280, now identical). Label colours stay darker than live on purpose (contrast, rule 20).</t>
         </is>
       </c>
       <c r="E290" s="14" t="inlineStr">
@@ -7527,7 +7527,7 @@
       <c r="A291" s="4" t="n"/>
       <c r="B291" s="4" t="inlineStr">
         <is>
-          <t>Sitemap: no noindex pages (2026-10-08)</t>
+          <t>Link check across all ported pages (no 404s, no broken internal cross-references)</t>
         </is>
       </c>
       <c r="C291" s="13" t="inlineStr">
@@ -7537,7 +7537,7 @@
       </c>
       <c r="D291" s="4" t="inlineStr">
         <is>
-          <t>the password-locked /blog/you-are-the-moat was in the sitemap while telling Google not to index it (a Search Console sitemap warning). Gated posts and posts that redirect are now left out (src/app/sitemap.ts); all 497 sitemap addresses return 200 with a matching canonical and no noindex. The 82 warnings Search Console shows are for the old live sitemap, so re-check them after cutover.</t>
+          <t>First full pass done 2026-09-29 (510 pages crawled from the sitemap plus every internal link, on a production build). Fixed in code: /brewsoul/coffee/…-tarrazú 404 (the route got the id still percent-encoded), 30+ links that went through the /assessments/* redirects, /find-your-me's dead Homeaglow link, the two root-level Iboga essay links, and the dead FauxTony nav item. Fixed as Sanity drafts (scripts/fix-blog-body-links.ts, 14 posts): broken post links, leaked !… placeholder text, Energy Is Money's split author bio, and scraped WordPress furniture ("Share this / Related / You Might Also Like / Copyright", "Show More / Top News", [mc4wp_form]). Left for a decision: /framework's "Ask FauxTony" button, when-healing-becomes-extraction's two links to a Dr. Lee case file that doesn't exist, and the-clock-keeper-chronicles-part-1's link to the deferred /clock-keeper-part-2. Re-run after the drafts are published. 2026-10-01 re-run (local production build, all 498 sitemap URLs load; 440 unique internal links): 5 broken. Fixed as a Sanity draft: molecule-as-mirror-10-what-the-pioneers-know's "Final installment" link pointed at a non-existent part-10 slug (now part 11; live also shows that line twice, kept). Already fixed in a waiting draft: forever-chemicals-... → /blog/psychedelic-readiness-index. Still the 3 known decisions: /fauxtony (from /framework), /clock-keeper-part-2, /blog/the-case-file-dr-samuel-lee. 2026-10-08 re-run (production build, all 497 sitemap pages, 453 unique i</t>
         </is>
       </c>
       <c r="E291" s="14" t="inlineStr">
@@ -7550,7 +7550,7 @@
       <c r="A292" s="4" t="n"/>
       <c r="B292" s="4" t="inlineStr">
         <is>
-          <t>Lighthouse pass (performance/accessibility/SEO) on top 20 pages by traffic 2026-09-30, 20 key pages (no traffic data yet), local production …</t>
+          <t>Sitemap: no noindex pages (2026-10-08)</t>
         </is>
       </c>
       <c r="C292" s="13" t="inlineStr">
@@ -7560,7 +7560,7 @@
       </c>
       <c r="D292" s="4" t="inlineStr">
         <is>
-          <t>build, mobile: averages performance 87, accessibility 99→100, best practices 100, SEO 92→100, CLS 0 everywhere. Fixed: public/robots.txt had an LLMs: line (not a real directive) that made Google treat the whole file as invalid, now a comment; h3/h4 headings skipping a level on /assessments, /kava, /peptide-watch (same look, right tag); the Kava and /attention-theft back-arrow links had no accessible name on phones; two small phone-width contrast misses. Left: performance is local-machine only (±10-15 points, see CONTRIBUTING.md); the slowest were / 76 (LCP 5.2 s), /psychedelic-readiness-index 82, /iboga-ibogaine 83. Re-run against the Netlify deploy before launch. 2026-10-06 re-run against the Netlify deploy (14 key pages, mobile): accessibility 100 and CLS 0 on every page, SEO clean (only the expected netlify.app noindex), performance 77-97 held back by 3-4 s LCP. Fixed: all 21 hero images moved off the deprecated priority prop to fetchPriority="high" + loading="eager" (Next 16); /iboga-ibogaine hero and the first card on /blog and category pages no longer lazy-loaded; sizes on the Four Doors cards (~150 KiB per page), /humanos diagram (~100 KiB) and /about headshot; urlFor no longer imports the Sanity client, so ~115 KB of Sanity client code stopped loading on / and /blog; React hydration error #418 on / and /blog (post dates) gone, checked in two time zones; /blog is static again; empty icon &lt;th&gt;s on /iboga-ibogaine labelled; category page reads use sanityFetch(). Left: se</t>
+          <t>the password-locked /blog/you-are-the-moat was in the sitemap while telling Google not to index it (a Search Console sitemap warning). Gated posts and posts that redirect are now left out (src/app/sitemap.ts); all 497 sitemap addresses return 200 with a matching canonical and no noindex. The 82 warnings Search Console shows are for the old live sitemap, so re-check them after cutover.</t>
         </is>
       </c>
       <c r="E292" s="14" t="inlineStr">
@@ -7573,7 +7573,7 @@
       <c r="A293" s="4" t="n"/>
       <c r="B293" s="4" t="inlineStr">
         <is>
-          <t>No Manus links anywhere (2026-10-09, owner: "drop them everywhere")</t>
+          <t>Lighthouse pass (performance/accessibility/SEO) on top 20 pages by traffic 2026-09-30, 20 key pages (no traffic data yet), local production …</t>
         </is>
       </c>
       <c r="C293" s="13" t="inlineStr">
@@ -7583,7 +7583,7 @@
       </c>
       <c r="D293" s="4" t="inlineStr">
         <is>
-          <t>every *.manus.space link removed from code and essays. Lists of "try this next" apps lose those entries (journey tracker, Find Your Me results and next steps, /find-my, search directory, Sake and Grant Study results, BrewSoul footer, The Mirror); The Magnetic Partner's and The Temple Keeper's next step now go to their first in-site assessment (/grant-study, /consciousness-scale); their empty "Find Your _" section hides itself; /recent-creations, /spirits and /ecosystem-map keep the cards, unlinked. Clarisse Abelarde now links to her own site clarisseartist.com (owner gave it) on /about and in essays. Essays: lib/sanity/portable-text.tsx rewrites tonygreenberg.manus.space/&lt;path&gt; to /&lt;path&gt;, clarisseart.manus.space to clarisseartist.com (same paths), and renders other Manus app links as plain text (no Sanity drafts). Verified on a production build: no clickable *.manus.space link in any page, no manus.space in any browser script; 13 affected pages load (200).</t>
+          <t>build, mobile: averages performance 87, accessibility 99→100, best practices 100, SEO 92→100, CLS 0 everywhere. Fixed: public/robots.txt had an LLMs: line (not a real directive) that made Google treat the whole file as invalid, now a comment; h3/h4 headings skipping a level on /assessments, /kava, /peptide-watch (same look, right tag); the Kava and /attention-theft back-arrow links had no accessible name on phones; two small phone-width contrast misses. Left: performance is local-machine only (±10-15 points, see CONTRIBUTING.md); the slowest were / 76 (LCP 5.2 s), /psychedelic-readiness-index 82, /iboga-ibogaine 83. Re-run against the Netlify deploy before launch. 2026-10-06 re-run against the Netlify deploy (14 key pages, mobile): accessibility 100 and CLS 0 on every page, SEO clean (only the expected netlify.app noindex), performance 77-97 held back by 3-4 s LCP. Fixed: all 21 hero images moved off the deprecated priority prop to fetchPriority="high" + loading="eager" (Next 16); /iboga-ibogaine hero and the first card on /blog and category pages no longer lazy-loaded; sizes on the Four Doors cards (~150 KiB per page), /humanos diagram (~100 KiB) and /about headshot; urlFor no longer imports the Sanity client, so ~115 KB of Sanity client code stopped loading on / and /blog; React hydration error #418 on / and /blog (post dates) gone, checked in two time zones; /blog is static again; empty icon &lt;th&gt;s on /iboga-ibogaine labelled; category page reads use sanityFetch(). Left: se</t>
         </is>
       </c>
       <c r="E293" s="14" t="inlineStr">
@@ -7596,7 +7596,7 @@
       <c r="A294" s="4" t="n"/>
       <c r="B294" s="4" t="inlineStr">
         <is>
-          <t>Owner answers, round 2 (2026-10-09)</t>
+          <t>No Manus links anywhere (2026-10-09, owner: "drop them everywhere")</t>
         </is>
       </c>
       <c r="C294" s="13" t="inlineStr">
@@ -7606,7 +7606,7 @@
       </c>
       <c r="D294" s="4" t="inlineStr">
         <is>
-          <t>(1) real counts instead of live's typed numbers: /charity-scorecard intro and description ("98"/"Ninety-eight" → STATS.totalCharities = 103), /impact-dashboard ("100" → passed in from the page so the browser doesn't load the charity list), /the-index (prop), search directory coffees 103 → 107 (typed, with a note, since it ships to the search pop-up); (2) The Mirror results no longer list the 4 *.manus.space apps (the "Explore further" section hides when empty); (3) /framework's "Ask FauxTony" button and its lead-in line removed; the Dr. Lee case-file link (4 places in when-healing-becomes-extraction, original and updated versions) renders as plain text through a DEAD_INTERNAL_LINKS list in lib/sanity/portable-text.tsx (no Sanity draft needed); (4) B Corp: checked live, nothing shown on either site, no change. Verified on a production build: the counts read 103, /framework has no FauxTony block, the essay has 0 links to the case file and keeps the words, /the-index shows "103 charities" when searching "charity".</t>
+          <t>every *.manus.space link removed from code and essays. Lists of "try this next" apps lose those entries (journey tracker, Find Your Me results and next steps, /find-my, search directory, Sake and Grant Study results, BrewSoul footer, The Mirror); The Magnetic Partner's and The Temple Keeper's next step now go to their first in-site assessment (/grant-study, /consciousness-scale); their empty "Find Your _" section hides itself; /recent-creations, /spirits and /ecosystem-map keep the cards, unlinked. Clarisse Abelarde now links to her own site clarisseartist.com (owner gave it) on /about and in essays. Essays: lib/sanity/portable-text.tsx rewrites tonygreenberg.manus.space/&lt;path&gt; to /&lt;path&gt;, clarisseart.manus.space to clarisseartist.com (same paths), and renders other Manus app links as plain text (no Sanity drafts). Verified on a production build: no clickable *.manus.space link in any page, no manus.space in any browser script; 13 affected pages load (200).</t>
         </is>
       </c>
       <c r="E294" s="14" t="inlineStr">
@@ -7619,7 +7619,7 @@
       <c r="A295" s="4" t="n"/>
       <c r="B295" s="4" t="inlineStr">
         <is>
-          <t>Arrows in buttons and links are icons (2026-10-09, owner said yes)</t>
+          <t>Owner answers, round 2 (2026-10-09)</t>
         </is>
       </c>
       <c r="C295" s="13" t="inlineStr">
@@ -7629,7 +7629,7 @@
       </c>
       <c r="D295" s="4" t="inlineStr">
         <is>
-          <t>113 typed arrows in 52 files (button and link labels, "Next"/"See My Results" toggles, decorative arrow spans, the walk-through "See the..." labels, the Letter's "I'm in" button) replaced with lucide ArrowRight/ArrowLeft (size-[1em], inside inline-flex items-center gap-1.5, so the parent layout is untouched). Left as content on purpose: arrows inside Tony's text and data (health findings, origins, iboga compass options, process flows like "Inherit → Wake → Choose → Act", share text), the "← you" marker on the consciousness scale, and &lt;option&gt; sort labels (an option can't hold an icon). Checked on 16 pages at 375 and 1280: no typed arrow left in any link or button, no sideways scroll, no JS errors; close-up screenshots of the new icons.</t>
+          <t>(1) real counts instead of live's typed numbers: /charity-scorecard intro and description ("98"/"Ninety-eight" → STATS.totalCharities = 103), /impact-dashboard ("100" → passed in from the page so the browser doesn't load the charity list), /the-index (prop), search directory coffees 103 → 107 (typed, with a note, since it ships to the search pop-up); (2) The Mirror results no longer list the 4 *.manus.space apps (the "Explore further" section hides when empty); (3) /framework's "Ask FauxTony" button and its lead-in line removed; the Dr. Lee case-file link (4 places in when-healing-becomes-extraction, original and updated versions) renders as plain text through a DEAD_INTERNAL_LINKS list in lib/sanity/portable-text.tsx (no Sanity draft needed); (4) B Corp: checked live, nothing shown on either site, no change. Verified on a production build: the counts read 103, /framework has no FauxTony block, the essay has 0 links to the case file and keeps the words, /the-index shows "103 charities" when searching "charity".</t>
         </is>
       </c>
       <c r="E295" s="14" t="inlineStr">
@@ -7642,7 +7642,7 @@
       <c r="A296" s="4" t="n"/>
       <c r="B296" s="4" t="inlineStr">
         <is>
-          <t>Category pages pre-built (2026-10-09)</t>
+          <t>Arrows in buttons and links are icons (2026-10-09, owner said yes)</t>
         </is>
       </c>
       <c r="C296" s="13" t="inlineStr">
@@ -7652,7 +7652,7 @@
       </c>
       <c r="D296" s="4" t="inlineStr">
         <is>
-          <t>/blog/category/[slug] read ?page=N, so every category page was rendered on each request (slower first byte, flagged in the Lighthouse notes). Page numbers are now part of the address (/blog/category/&lt;slug&gt;/page/&lt;n&gt;, generateStaticParams, dynamicParams = false), shared code in src/components/blog/category-listing.tsx; old ?page=N links 308 to the new address (pages 2+ only, so no loop), /page/1 308s to the plain address, a page past the end is a 404; "All essays" back link uses an icon. Verified on a production build: route table shows every category page as pre-built (9 page-1s, 7 later pages), titles and canonicals per page, Previous/Next links, the redirects and the 404s.</t>
+          <t>113 typed arrows in 52 files (button and link labels, "Next"/"See My Results" toggles, decorative arrow spans, the walk-through "See the..." labels, the Letter's "I'm in" button) replaced with lucide ArrowRight/ArrowLeft (size-[1em], inside inline-flex items-center gap-1.5, so the parent layout is untouched). Left as content on purpose: arrows inside Tony's text and data (health findings, origins, iboga compass options, process flows like "Inherit → Wake → Choose → Act", share text), the "← you" marker on the consciousness scale, and &lt;option&gt; sort labels (an option can't hold an icon). Checked on 16 pages at 375 and 1280: no typed arrow left in any link or button, no sideways scroll, no JS errors; close-up screenshots of the new icons.</t>
         </is>
       </c>
       <c r="E296" s="14" t="inlineStr">
@@ -7665,7 +7665,7 @@
       <c r="A297" s="4" t="n"/>
       <c r="B297" s="4" t="inlineStr">
         <is>
-          <t>Error pages (2026-10-09, owner asked)</t>
+          <t>Category pages pre-built (2026-10-09)</t>
         </is>
       </c>
       <c r="C297" s="13" t="inlineStr">
@@ -7675,7 +7675,7 @@
       </c>
       <c r="D297" s="4" t="inlineStr">
         <is>
-          <t>404 page now sets its own title ("Page not found") as a server page around live's 3-second redirect (not-found.tsx + components/not-found-redirect.tsx), arrow as an icon; page error screen (error.tsx) uses Next 16's retry (re-fetches), shows a reference code for the server logs, links home and to the site index; new global-error.tsx for failures in the root layout itself (own &lt;html&gt;, plain links). Verified on a production build: missing page, missing essay and missing Kava page return 404 with the right title; a test page that throws returns 500 with the error screen, "Try again" re-fetches; phone and laptop, no sideways scroll (test page removed).</t>
+          <t>/blog/category/[slug] read ?page=N, so every category page was rendered on each request (slower first byte, flagged in the Lighthouse notes). Page numbers are now part of the address (/blog/category/&lt;slug&gt;/page/&lt;n&gt;, generateStaticParams, dynamicParams = false), shared code in src/components/blog/category-listing.tsx; old ?page=N links 308 to the new address (pages 2+ only, so no loop), /page/1 308s to the plain address, a page past the end is a 404; "All essays" back link uses an icon. Verified on a production build: route table shows every category page as pre-built (9 page-1s, 7 later pages), titles and canonicals per page, Previous/Next links, the redirects and the 404s.</t>
         </is>
       </c>
       <c r="E297" s="14" t="inlineStr">
@@ -7688,7 +7688,7 @@
       <c r="A298" s="4" t="n"/>
       <c r="B298" s="4" t="inlineStr">
         <is>
-          <t>SEO audit fixes (2026-10-06)</t>
+          <t>Error pages (2026-10-09, owner asked)</t>
         </is>
       </c>
       <c r="C298" s="13" t="inlineStr">
@@ -7698,7 +7698,7 @@
       </c>
       <c r="D298" s="4" t="inlineStr">
         <is>
-          <t>Checked an outside audit point by point against the code. Fixed: Core Themes cards linked to /?theme=…#essays-archive (not crawlable, counts from a stale hand-kept list) and now link to /blog/category/&lt;slug&gt; with real counts (21/25/20/14, matching the archive pills; THEME_MAP and the ?theme= filter removed); Four Doors cards were &lt;button&gt;s, now real links that still open the modal on a plain click; "DIAGNOSE · ENGAGE" now link to /find-my and /engage; one shared formatPostDate (Asia/Kolkata, src/lib/format-post-date.ts) so a post no longer shows two different dates; the title repeated as the first body paragraph is dropped at render time (legacyBodyLayout); essay cards are h3 under a section h2 (archive, Read next), h2 only on category/search; heading glyphs (◆ ✦) hidden from screen readers; posts send BlogPosting with the author tied to the site Person (@id) plus a BreadcrumbList; descriptive alt on the homepage and BrewSoul heroes; homepage OG image cropped to 1200x630 JPEG. Already fine (audit could not see it): Person/Article schema, Netlify noindex, robots.txt, sitemap, header nav and search, Amazon links carry no affiliate tag. Checked on a production build: type check, lint, build, status codes, browser click test at 375px, no console errors. Implementation pack (Mohammad Danish, 2026-10-05) checked the same day: added og:type/og:site_name back on the 6 pages with their own openGraph (a page-level openGraph replaces the layout one), twitter:creator, and on posts og:url</t>
+          <t>404 page now sets its own title ("Page not found") as a server page around live's 3-second redirect (not-found.tsx + components/not-found-redirect.tsx), arrow as an icon; page error screen (error.tsx) uses Next 16's retry (re-fetches), shows a reference code for the server logs, links home and to the site index; new global-error.tsx for failures in the root layout itself (own &lt;html&gt;, plain links). Verified on a production build: missing page, missing essay and missing Kava page return 404 with the right title; a test page that throws returns 500 with the error screen, "Try again" re-fetches; phone and laptop, no sideways scroll (test page removed).</t>
         </is>
       </c>
       <c r="E298" s="14" t="inlineStr">
@@ -7711,7 +7711,7 @@
       <c r="A299" s="4" t="n"/>
       <c r="B299" s="4" t="inlineStr">
         <is>
-          <t>SEO audit items needing a yes (2026-10-06; owner said yes to the copy 2026-10-10, done)</t>
+          <t>SEO audit fixes (2026-10-06)</t>
         </is>
       </c>
       <c r="C299" s="13" t="inlineStr">
@@ -7721,7 +7721,7 @@
       </c>
       <c r="D299" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">the pack's new copy (homepage title/description, five-cups title, description, short answer, FAQ, heading rewrites, entity statement, newsletter block, author box, health disclaimer, COA wording); "Further Reading" shown twice on posts (merge the lists?); long post title (84 chars), homepage description length and obsolete keywords tag, slugs (/blog/five-cups, the -2 slug; would need redirects), "Six lenses" over four cards, sources for health claims and proof for "$10B+", "Certified B Corp", "Validity: 91", legal review of the homepage Case File banner, ABIT waitlist disclosures, one contact email, the two one-post categories, fewer homepage CTAs / email signup / table of contents / explaining "COA". Done 2026-10-10: homepage title "Tony Greenberg | Strategist, Author &amp; CEO of RampRate" and description (essay count computed: 123); entity statement under the hero (107 coffees / 100 chains computed from the data) with a link to /ecosystem; door 4 "Certificate of Analysis (COA) checks, lab testing and vendor scoring"; "Four lenses" (computed); newsletter box after Editor's Picks (existing Kit form); meta keywords removed site-wide; every essay: author line + "About Tony", one merged "Further Reading", optional lastUpdated field shown as "Updated &lt;date&gt;" (not set on any post yet: every _updatedAt is the import date), health disclaimer on 20 personal-health essays (chosen by Sanity tag); Five Cups (Sanity, published, backup kept): SEO title/description, short answer, visible FAQ </t>
+          <t>Checked an outside audit point by point against the code. Fixed: Core Themes cards linked to /?theme=…#essays-archive (not crawlable, counts from a stale hand-kept list) and now link to /blog/category/&lt;slug&gt; with real counts (21/25/20/14, matching the archive pills; THEME_MAP and the ?theme= filter removed); Four Doors cards were &lt;button&gt;s, now real links that still open the modal on a plain click; "DIAGNOSE · ENGAGE" now link to /find-my and /engage; one shared formatPostDate (Asia/Kolkata, src/lib/format-post-date.ts) so a post no longer shows two different dates; the title repeated as the first body paragraph is dropped at render time (legacyBodyLayout); essay cards are h3 under a section h2 (archive, Read next), h2 only on category/search; heading glyphs (◆ ✦) hidden from screen readers; posts send BlogPosting with the author tied to the site Person (@id) plus a BreadcrumbList; descriptive alt on the homepage and BrewSoul heroes; homepage OG image cropped to 1200x630 JPEG. Already fine (audit could not see it): Person/Article schema, Netlify noindex, robots.txt, sitemap, header nav and search, Amazon links carry no affiliate tag. Checked on a production build: type check, lint, build, status codes, browser click test at 375px, no console errors. Implementation pack (Mohammad Danish, 2026-10-05) checked the same day: added og:type/og:site_name back on the 6 pages with their own openGraph (a page-level openGraph replaces the layout one), twitter:creator, and on posts og:url</t>
         </is>
       </c>
       <c r="E299" s="14" t="inlineStr">
@@ -7734,7 +7734,7 @@
       <c r="A300" s="4" t="n"/>
       <c r="B300" s="4" t="inlineStr">
         <is>
-          <t>Google Analytics tag (found missing 2026-10-10, added the same day)</t>
+          <t>SEO audit items needing a yes (2026-10-06; owner said yes to the copy 2026-10-10, done)</t>
         </is>
       </c>
       <c r="C300" s="13" t="inlineStr">
@@ -7744,7 +7744,7 @@
       </c>
       <c r="D300" s="4" t="inlineStr">
         <is>
-          <t>Live loads GA4 G-4GVW40S47N; the new site sent nothing, so stats would have stopped at cutover. Added src/components/google-analytics.tsx (plain next/script, no new package) in the root layout; it only runs on tonygreenberg.com / www, so Netlify previews and localhost never reach the real reports. Checked: type check, lint, build; in Chromium with Google's requests blocked: localhost sends nothing, tonygreenberg.com (mapped to a local production build) loads the tag on / and /find-your-coffee, no JS errors. In-site page changes are counted by GA4's Enhanced measurement (on by default; confirm in GA4 &gt; Admin &gt; Data streams on launch day).</t>
+          <t xml:space="preserve">the pack's new copy (homepage title/description, five-cups title, description, short answer, FAQ, heading rewrites, entity statement, newsletter block, author box, health disclaimer, COA wording); "Further Reading" shown twice on posts (merge the lists?); long post title (84 chars), homepage description length and obsolete keywords tag, slugs (/blog/five-cups, the -2 slug; would need redirects), "Six lenses" over four cards, sources for health claims and proof for "$10B+", "Certified B Corp", "Validity: 91", legal review of the homepage Case File banner, ABIT waitlist disclosures, one contact email, the two one-post categories, fewer homepage CTAs / email signup / table of contents / explaining "COA". Done 2026-10-10: homepage title "Tony Greenberg | Strategist, Author &amp; CEO of RampRate" and description (essay count computed: 123); entity statement under the hero (107 coffees / 100 chains computed from the data) with a link to /ecosystem; door 4 "Certificate of Analysis (COA) checks, lab testing and vendor scoring"; "Four lenses" (computed); newsletter box after Editor's Picks (existing Kit form); meta keywords removed site-wide; every essay: author line + "About Tony", one merged "Further Reading", optional lastUpdated field shown as "Updated &lt;date&gt;" (not set on any post yet: every _updatedAt is the import date), health disclaimer on 20 personal-health essays (chosen by Sanity tag); Five Cups (Sanity, published, backup kept): SEO title/description, short answer, visible FAQ </t>
         </is>
       </c>
       <c r="E300" s="14" t="inlineStr">
@@ -7757,7 +7757,7 @@
       <c r="A301" s="4" t="n"/>
       <c r="B301" s="4" t="inlineStr">
         <is>
-          <t>Old site's custom GA4 events ported (2026-10-10, owner asked to match legacy's Google tags)</t>
+          <t>Google Analytics tag (found missing 2026-10-10, added the same day)</t>
         </is>
       </c>
       <c r="C301" s="13" t="inlineStr">
@@ -7767,7 +7767,7 @@
       </c>
       <c r="D301" s="4" t="inlineStr">
         <is>
-          <t>Legacy loaded GA4 G-4GVW40S47N (already on the new site), Manus's own Umami counter (gone with Manus, not portable) and custom events from ConversionMechanics.tsx's AnalyticsTracker. Now src/components/ga-events.tsx (root layout) sends the same names: article_/page_25/50/75/90_scroll, engaged_45_seconds, second_page_view, homepage_path_work/_thinking/_building, start_here_open. Legacy's extra page_view on every history change is not ported (GA4 Enhanced measurement already counts in-site page changes; it would double-count). Tested in Chromium with Google's requests blocked: tonygreenberg.com (mapped to a local build) fired the homepage path and all four essay scroll events plus second_page_view; localhost loads no tag. A RampRate-style weekly report / hourly alert email and an admin analytics page were built the same day and removed at the owner's request (they use the Looker Studio report instead); the empty report_runs table and CRON_SECRET were removed too.</t>
+          <t>Live loads GA4 G-4GVW40S47N; the new site sent nothing, so stats would have stopped at cutover. Added src/components/google-analytics.tsx (plain next/script, no new package) in the root layout; it only runs on tonygreenberg.com / www, so Netlify previews and localhost never reach the real reports. Checked: type check, lint, build; in Chromium with Google's requests blocked: localhost sends nothing, tonygreenberg.com (mapped to a local production build) loads the tag on / and /find-your-coffee, no JS errors. In-site page changes are counted by GA4's Enhanced measurement (on by default; confirm in GA4 &gt; Admin &gt; Data streams on launch day).</t>
         </is>
       </c>
       <c r="E301" s="14" t="inlineStr">
@@ -7780,15 +7780,19 @@
       <c r="A302" s="4" t="n"/>
       <c r="B302" s="4" t="inlineStr">
         <is>
-          <t>Connect Google Search Console + GA4 to the new deployment on day one of cutover</t>
-        </is>
-      </c>
-      <c r="C302" s="16" t="inlineStr">
-        <is>
-          <t>Remaining</t>
-        </is>
-      </c>
-      <c r="D302" s="4" t="inlineStr"/>
+          <t>Old site's custom GA4 events ported (2026-10-10, owner asked to match legacy's Google tags)</t>
+        </is>
+      </c>
+      <c r="C302" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D302" s="4" t="inlineStr">
+        <is>
+          <t>Legacy loaded GA4 G-4GVW40S47N (already on the new site), Manus's own Umami counter (gone with Manus, not portable) and custom events from ConversionMechanics.tsx's AnalyticsTracker. Now src/components/ga-events.tsx (root layout) sends the same names: article_/page_25/50/75/90_scroll, engaged_45_seconds, second_page_view, homepage_path_work/_thinking/_building, start_here_open. Legacy's extra page_view on every history change is not ported (GA4 Enhanced measurement already counts in-site page changes; it would double-count). Tested in Chromium with Google's requests blocked: tonygreenberg.com (mapped to a local build) fired the homepage path and all four essay scroll events plus second_page_view; localhost loads no tag. A RampRate-style weekly report / hourly alert email and an admin analytics page were built the same day and removed at the owner's request (they use the Looker Studio report instead); the empty report_runs table and CRON_SECRET were removed too.</t>
+        </is>
+      </c>
       <c r="E302" s="14" t="inlineStr">
         <is>
           <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
@@ -7799,19 +7803,15 @@
       <c r="A303" s="4" t="n"/>
       <c r="B303" s="4" t="inlineStr">
         <is>
-          <t>Restore/adapt the manus.space triple-layer noindex lockdown pattern for any remaining staging URLs</t>
-        </is>
-      </c>
-      <c r="C303" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D303" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-01: the Netlify copy (tonygreenberg-website.netlify.app) and every deploy preview had no noindex at all, so Google could index a duplicate of the site. next.config.ts headers() now sends X-Robots-Tag: noindex, nofollow on any *.netlify.app host only; tonygreenberg.com is unaffected, so nothing to remove at cutover. Tested with Host headers on a production build.</t>
-        </is>
-      </c>
+          <t>Connect Google Search Console + GA4 to the new deployment on day one of cutover</t>
+        </is>
+      </c>
+      <c r="C303" s="16" t="inlineStr">
+        <is>
+          <t>Remaining</t>
+        </is>
+      </c>
+      <c r="D303" s="4" t="inlineStr"/>
       <c r="E303" s="14" t="inlineStr">
         <is>
           <t>Phase 12 — SEO Hardening, Redirects &amp; Cutover Prep</t>
@@ -7822,7 +7822,7 @@
       <c r="A304" s="4" t="n"/>
       <c r="B304" s="4" t="inlineStr">
         <is>
-          <t>"Keep going" strip above the footer on every page (2026-10-07)</t>
+          <t>Restore/adapt the manus.space triple-layer noindex lockdown pattern for any remaining staging URLs</t>
         </is>
       </c>
       <c r="C304" s="13" t="inlineStr">
@@ -7832,7 +7832,7 @@
       </c>
       <c r="D304" s="4" t="inlineStr">
         <is>
-          <t>legacy's WhereNext (deferred in Phase 3, never picked up) with its per-page suggestions, Home · Site Index · All Assessments; links pointed at current routes.</t>
+          <t>2026-10-01: the Netlify copy (tonygreenberg-website.netlify.app) and every deploy preview had no noindex at all, so Google could index a duplicate of the site. next.config.ts headers() now sends X-Robots-Tag: noindex, nofollow on any *.netlify.app host only; tonygreenberg.com is unaffected, so nothing to remove at cutover. Tested with Host headers on a production build.</t>
         </is>
       </c>
       <c r="E304" s="14" t="inlineStr">
@@ -7845,7 +7845,7 @@
       <c r="A305" s="4" t="n"/>
       <c r="B305" s="4" t="inlineStr">
         <is>
-          <t>Live-only and redesigned pages from the 2026-10-07 page sweep (188 pages compared with live)</t>
+          <t>"Keep going" strip above the footer on every page (2026-10-07)</t>
         </is>
       </c>
       <c r="C305" s="13" t="inlineStr">
@@ -7855,7 +7855,7 @@
       </c>
       <c r="D305" s="4" t="inlineStr">
         <is>
-          <t>/the-index rebuilt from live's code (20 concepts, related-word search across essays and site pages, full-text search on the server, "three related places to go next"; the old redirect to /search removed and its links, including the "Site Index" link in "Keep going", point at it again); /the-mirror (and /life-assessment) opens on live's intro (dark hero, "What We Measure" with the six areas, "The Ecosystem"), rebuilt as a step registry (rule 19); /essays header, order and column like live; /about "What They Say" styled like live (live picks 3 of the same 19 quotes at random; ours shows a fixed 3 so they're in the server HTML); /impact-futurism list titles and subtitles; /supplier-intake is a real page again with live's Stage 1 form; /seven-doors and /projects redirect home like live; /impact, /health, /library, /built-on-manus, /heroes are 404 on live too. Left as is on purpose: /blog stays our archive page (on live it repeats the homepage), the email gates on /framework and /peptide-supply-chain, the attention-theft Wall of Shame.</t>
+          <t>legacy's WhereNext (deferred in Phase 3, never picked up) with its per-page suggestions, Home · Site Index · All Assessments; links pointed at current routes.</t>
         </is>
       </c>
       <c r="E305" s="14" t="inlineStr">
@@ -7868,7 +7868,7 @@
       <c r="A306" s="4" t="n"/>
       <c r="B306" s="4" t="inlineStr">
         <is>
-          <t>/alex-azzi locked like live (2026-10-07, owner said match it)</t>
+          <t>Live-only and redesigned pages from the 2026-10-07 page sweep (188 pages compared with live)</t>
         </is>
       </c>
       <c r="C306" s="13" t="inlineStr">
@@ -7878,7 +7878,7 @@
       </c>
       <c r="D306" s="4" t="inlineStr">
         <is>
-          <t>same server-checked password as the locked essay (GATED_POST_PASSWORD, now also set in Netlify), live's "Restricted Access" screen, the report not in the page until unlocked, out of search and the sitemap.</t>
+          <t>/the-index rebuilt from live's code (20 concepts, related-word search across essays and site pages, full-text search on the server, "three related places to go next"; the old redirect to /search removed and its links, including the "Site Index" link in "Keep going", point at it again); /the-mirror (and /life-assessment) opens on live's intro (dark hero, "What We Measure" with the six areas, "The Ecosystem"), rebuilt as a step registry (rule 19); /essays header, order and column like live; /about "What They Say" styled like live (live picks 3 of the same 19 quotes at random; ours shows a fixed 3 so they're in the server HTML); /impact-futurism list titles and subtitles; /supplier-intake is a real page again with live's Stage 1 form; /seven-doors and /projects redirect home like live; /impact, /health, /library, /built-on-manus, /heroes are 404 on live too. Left as is on purpose: /blog stays our archive page (on live it repeats the homepage), the email gates on /framework and /peptide-supply-chain, the attention-theft Wall of Shame.</t>
         </is>
       </c>
       <c r="E306" s="14" t="inlineStr">
@@ -7891,7 +7891,7 @@
       <c r="A307" s="4" t="n"/>
       <c r="B307" s="4" t="inlineStr">
         <is>
-          <t>Live's title fonts and sizes (2026-10-07, "fix the style")</t>
+          <t>/alex-azzi locked like live (2026-10-07, owner said match it)</t>
         </is>
       </c>
       <c r="C307" s="13" t="inlineStr">
@@ -7901,7 +7901,7 @@
       </c>
       <c r="D307" s="4" t="inlineStr">
         <is>
-          <t>measured every page's title font, weight, size and label colour on live vs ours (136 pages). Now like live: Kava headings in Fraunces, HumanOS in Space Grotesk, the peptide tools / charity scorecard / thesis threads in the system serif, America Unbundled in the Iowan Old Style stack at live's size, /akbar in Fraunces 900, friend-gate and post-intervention in Georgia, and live's title sizes on peptide-matrix, peptide-supply-chain, rip-peptide-sciences and the HumanOS pages. Fonts load only on the pages that use them (src/lib/fonts/page-fonts.ts). Label colours stay the darker AA-contrast versions where live's lighter ones fail on a light background.</t>
+          <t>same server-checked password as the locked essay (GATED_POST_PASSWORD, now also set in Netlify), live's "Restricted Access" screen, the report not in the page until unlocked, out of search and the sitemap.</t>
         </is>
       </c>
       <c r="E307" s="14" t="inlineStr">
@@ -7914,7 +7914,7 @@
       <c r="A308" s="4" t="n"/>
       <c r="B308" s="4" t="inlineStr">
         <is>
-          <t>Peptide page images rescued into Sanity and wired (2026-10-07)</t>
+          <t>Live's title fonts and sizes (2026-10-07, "fix the style")</t>
         </is>
       </c>
       <c r="C308" s="13" t="inlineStr">
@@ -7924,7 +7924,7 @@
       </c>
       <c r="D308" s="4" t="inlineStr">
         <is>
-          <t>/peptide-watch hero plus its 11 section banners, /peptide-matrix and /peptide-supply-chain heroes, the /peptide-hall-of-shame hero (scripts/rescue-2026-10-07-peptide-images.ts, logged in docs/ai/manus-media-rescue.md).</t>
+          <t>measured every page's title f